<commit_message>
Atualização automática: mta (14/09/2026 13:57)
</commit_message>
<xml_diff>
--- a/Projetos/02_Dados_Tratados/base_mta_tratada.xlsx
+++ b/Projetos/02_Dados_Tratados/base_mta_tratada.xlsx
@@ -14,7 +14,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1131" uniqueCount="181">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1141" uniqueCount="181">
   <si>
     <t>linha</t>
   </si>
@@ -202,6 +202,9 @@
     <t>C26363</t>
   </si>
   <si>
+    <t>2026-09-11 00:00:00</t>
+  </si>
+  <si>
     <t>1</t>
   </si>
   <si>
@@ -220,13 +223,10 @@
     <t>email do dia 24/04</t>
   </si>
   <si>
-    <t>2026-09-09 00:00:00</t>
-  </si>
-  <si>
     <t>e-mail 12/08</t>
   </si>
   <si>
-    <t>ATENDER E REMANEJAR P/ CABW 30</t>
+    <t>Atender; Alterar a tarefa para "Requisição Consumíveis". Alterar a ND para 339030</t>
   </si>
   <si>
     <t>ATENDER</t>
@@ -238,7 +238,7 @@
     <t>Atender SET</t>
   </si>
   <si>
-    <t>Atender OUT</t>
+    <t>Atender</t>
   </si>
   <si>
     <t>Atender NOV</t>
@@ -247,7 +247,7 @@
     <t>ATENDER com 20XV</t>
   </si>
   <si>
-    <t>Remanejar tarefa módulo extra ctt 005 e Atender</t>
+    <t>Atender; Alterar a tarefa para "Módulo Extra - Sob demanda"</t>
   </si>
   <si>
     <t>LIVRE</t>
@@ -982,6 +982,9 @@
       <c r="F2" t="s">
         <v>30</v>
       </c>
+      <c r="J2" t="s">
+        <v>62</v>
+      </c>
       <c r="K2" t="s">
         <v>70</v>
       </c>
@@ -1480,7 +1483,7 @@
         <v>46</v>
       </c>
       <c r="J12" t="s">
-        <v>62</v>
+        <v>63</v>
       </c>
       <c r="N12" t="s">
         <v>79</v>
@@ -1529,6 +1532,9 @@
       <c r="F13" t="s">
         <v>30</v>
       </c>
+      <c r="J13" t="s">
+        <v>62</v>
+      </c>
       <c r="K13" t="s">
         <v>71</v>
       </c>
@@ -1579,6 +1585,9 @@
       <c r="F14" t="s">
         <v>30</v>
       </c>
+      <c r="J14" t="s">
+        <v>62</v>
+      </c>
       <c r="K14" t="s">
         <v>71</v>
       </c>
@@ -1629,6 +1638,9 @@
       <c r="F15" t="s">
         <v>30</v>
       </c>
+      <c r="J15" t="s">
+        <v>62</v>
+      </c>
       <c r="K15" t="s">
         <v>71</v>
       </c>
@@ -1679,6 +1691,9 @@
       <c r="F16" t="s">
         <v>30</v>
       </c>
+      <c r="J16" t="s">
+        <v>62</v>
+      </c>
       <c r="K16" t="s">
         <v>71</v>
       </c>
@@ -1739,7 +1754,7 @@
         <v>47</v>
       </c>
       <c r="J17" t="s">
-        <v>62</v>
+        <v>63</v>
       </c>
       <c r="N17" t="s">
         <v>84</v>
@@ -2098,7 +2113,7 @@
         <v>49</v>
       </c>
       <c r="J24" t="s">
-        <v>63</v>
+        <v>64</v>
       </c>
       <c r="N24" t="s">
         <v>84</v>
@@ -2259,6 +2274,9 @@
       <c r="F27" t="s">
         <v>30</v>
       </c>
+      <c r="J27" t="s">
+        <v>62</v>
+      </c>
       <c r="K27" t="s">
         <v>71</v>
       </c>
@@ -2319,7 +2337,7 @@
         <v>52</v>
       </c>
       <c r="J28" t="s">
-        <v>64</v>
+        <v>65</v>
       </c>
       <c r="N28" t="s">
         <v>84</v>
@@ -2378,7 +2396,7 @@
         <v>52</v>
       </c>
       <c r="J29" t="s">
-        <v>64</v>
+        <v>65</v>
       </c>
       <c r="N29" t="s">
         <v>84</v>
@@ -2437,7 +2455,7 @@
         <v>53</v>
       </c>
       <c r="J30" t="s">
-        <v>64</v>
+        <v>65</v>
       </c>
       <c r="N30" t="s">
         <v>84</v>
@@ -2496,7 +2514,7 @@
         <v>52</v>
       </c>
       <c r="J31" t="s">
-        <v>64</v>
+        <v>65</v>
       </c>
       <c r="N31" t="s">
         <v>84</v>
@@ -2605,7 +2623,7 @@
         <v>54</v>
       </c>
       <c r="J33" t="s">
-        <v>65</v>
+        <v>66</v>
       </c>
       <c r="N33" t="s">
         <v>84</v>
@@ -3268,7 +3286,7 @@
         <v>54</v>
       </c>
       <c r="J45" t="s">
-        <v>66</v>
+        <v>67</v>
       </c>
       <c r="N45" t="s">
         <v>84</v>
@@ -3420,6 +3438,9 @@
       <c r="F48" t="s">
         <v>30</v>
       </c>
+      <c r="J48" t="s">
+        <v>62</v>
+      </c>
       <c r="K48" t="s">
         <v>71</v>
       </c>
@@ -3480,7 +3501,7 @@
         <v>60</v>
       </c>
       <c r="J49" t="s">
-        <v>67</v>
+        <v>68</v>
       </c>
       <c r="N49" t="s">
         <v>79</v>
@@ -3530,7 +3551,7 @@
         <v>30</v>
       </c>
       <c r="J50" t="s">
-        <v>66</v>
+        <v>67</v>
       </c>
       <c r="K50" t="s">
         <v>73</v>
@@ -3583,10 +3604,10 @@
         <v>30</v>
       </c>
       <c r="J51" t="s">
-        <v>66</v>
+        <v>67</v>
       </c>
       <c r="K51" t="s">
-        <v>72</v>
+        <v>74</v>
       </c>
       <c r="N51" t="s">
         <v>84</v>
@@ -3636,7 +3657,7 @@
         <v>30</v>
       </c>
       <c r="K52" t="s">
-        <v>74</v>
+        <v>72</v>
       </c>
       <c r="N52" t="s">
         <v>84</v>
@@ -3741,6 +3762,9 @@
       <c r="F54" t="s">
         <v>30</v>
       </c>
+      <c r="J54" t="s">
+        <v>62</v>
+      </c>
       <c r="K54" t="s">
         <v>75</v>
       </c>
@@ -3792,10 +3816,10 @@
         <v>39</v>
       </c>
       <c r="J55" t="s">
-        <v>68</v>
+        <v>62</v>
       </c>
       <c r="K55" t="s">
-        <v>75</v>
+        <v>74</v>
       </c>
       <c r="N55" t="s">
         <v>88</v>
@@ -4375,6 +4399,9 @@
       <c r="F68" t="s">
         <v>30</v>
       </c>
+      <c r="J68" t="s">
+        <v>62</v>
+      </c>
       <c r="K68" t="s">
         <v>71</v>
       </c>
@@ -5029,6 +5056,9 @@
       </c>
       <c r="F82" t="s">
         <v>30</v>
+      </c>
+      <c r="J82" t="s">
+        <v>62</v>
       </c>
       <c r="K82" t="s">
         <v>77</v>

</xml_diff>

<commit_message>
Atualização automática: mta (15/09/2026 08:55)
</commit_message>
<xml_diff>
--- a/Projetos/02_Dados_Tratados/base_mta_tratada.xlsx
+++ b/Projetos/02_Dados_Tratados/base_mta_tratada.xlsx
@@ -566,8 +566,16 @@
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="YYYY-MM-DD HH:MM:SS"/>
   </numFmts>
-  <fonts count="1">
+  <fonts count="2">
     <font>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
       <sz val="11"/>
       <color theme="1"/>
       <name val="Calibri"/>
@@ -583,7 +591,7 @@
       <patternFill patternType="gray125"/>
     </fill>
   </fills>
-  <borders count="1">
+  <borders count="2">
     <border>
       <left/>
       <right/>
@@ -591,12 +599,30 @@
       <bottom/>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin">
+        <color auto="1"/>
+      </left>
+      <right style="thin">
+        <color auto="1"/>
+      </right>
+      <top style="thin">
+        <color auto="1"/>
+      </top>
+      <bottom style="thin">
+        <color auto="1"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="3">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
   </cellXfs>
   <cellStyles count="1">
@@ -896,70 +922,70 @@
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:22">
-      <c r="A1" t="s">
+      <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
-      <c r="B1" t="s">
+      <c r="B1" s="1" t="s">
         <v>1</v>
       </c>
-      <c r="C1" t="s">
+      <c r="C1" s="1" t="s">
         <v>2</v>
       </c>
-      <c r="D1" t="s">
+      <c r="D1" s="1" t="s">
         <v>3</v>
       </c>
-      <c r="E1" t="s">
+      <c r="E1" s="1" t="s">
         <v>4</v>
       </c>
-      <c r="F1" t="s">
+      <c r="F1" s="1" t="s">
         <v>5</v>
       </c>
-      <c r="G1" t="s">
+      <c r="G1" s="1" t="s">
         <v>6</v>
       </c>
-      <c r="H1" t="s">
+      <c r="H1" s="1" t="s">
         <v>7</v>
       </c>
-      <c r="I1" t="s">
+      <c r="I1" s="1" t="s">
         <v>8</v>
       </c>
-      <c r="J1" t="s">
+      <c r="J1" s="1" t="s">
         <v>9</v>
       </c>
-      <c r="K1" t="s">
+      <c r="K1" s="1" t="s">
         <v>10</v>
       </c>
-      <c r="L1" t="s">
+      <c r="L1" s="1" t="s">
         <v>11</v>
       </c>
-      <c r="M1" t="s">
+      <c r="M1" s="1" t="s">
         <v>12</v>
       </c>
-      <c r="N1" t="s">
+      <c r="N1" s="1" t="s">
         <v>13</v>
       </c>
-      <c r="O1" t="s">
+      <c r="O1" s="1" t="s">
         <v>14</v>
       </c>
-      <c r="P1" t="s">
+      <c r="P1" s="1" t="s">
         <v>15</v>
       </c>
-      <c r="Q1" t="s">
+      <c r="Q1" s="1" t="s">
         <v>16</v>
       </c>
-      <c r="R1" t="s">
+      <c r="R1" s="1" t="s">
         <v>17</v>
       </c>
-      <c r="S1" t="s">
+      <c r="S1" s="1" t="s">
         <v>18</v>
       </c>
-      <c r="T1" t="s">
+      <c r="T1" s="1" t="s">
         <v>19</v>
       </c>
-      <c r="U1" t="s">
+      <c r="U1" s="1" t="s">
         <v>20</v>
       </c>
-      <c r="V1" t="s">
+      <c r="V1" s="1" t="s">
         <v>21</v>
       </c>
     </row>
@@ -1015,7 +1041,7 @@
       <c r="U2" t="s">
         <v>180</v>
       </c>
-      <c r="V2" s="1">
+      <c r="V2" s="2">
         <v>46229</v>
       </c>
     </row>
@@ -1062,7 +1088,7 @@
       <c r="U3" t="s">
         <v>28</v>
       </c>
-      <c r="V3" s="1">
+      <c r="V3" s="2">
         <v>46291</v>
       </c>
     </row>
@@ -1109,7 +1135,7 @@
       <c r="U4" t="s">
         <v>28</v>
       </c>
-      <c r="V4" s="1">
+      <c r="V4" s="2">
         <v>46321</v>
       </c>
     </row>
@@ -1156,7 +1182,7 @@
       <c r="U5" t="s">
         <v>28</v>
       </c>
-      <c r="V5" s="1">
+      <c r="V5" s="2">
         <v>46321</v>
       </c>
     </row>
@@ -1206,7 +1232,7 @@
       <c r="U6" t="s">
         <v>28</v>
       </c>
-      <c r="V6" s="1">
+      <c r="V6" s="2">
         <v>46291</v>
       </c>
     </row>
@@ -1232,7 +1258,7 @@
       <c r="G7" t="s">
         <v>42</v>
       </c>
-      <c r="H7" s="1">
+      <c r="H7" s="2">
         <v>46121</v>
       </c>
       <c r="I7" t="s">
@@ -1262,7 +1288,7 @@
       <c r="U7" t="s">
         <v>28</v>
       </c>
-      <c r="V7" s="1">
+      <c r="V7" s="2">
         <v>46138</v>
       </c>
     </row>
@@ -1309,7 +1335,7 @@
       <c r="U8" t="s">
         <v>28</v>
       </c>
-      <c r="V8" s="1">
+      <c r="V8" s="2">
         <v>46291</v>
       </c>
     </row>
@@ -1356,7 +1382,7 @@
       <c r="U9" t="s">
         <v>28</v>
       </c>
-      <c r="V9" s="1">
+      <c r="V9" s="2">
         <v>46291</v>
       </c>
     </row>
@@ -1403,7 +1429,7 @@
       <c r="U10" t="s">
         <v>28</v>
       </c>
-      <c r="V10" s="1">
+      <c r="V10" s="2">
         <v>46291</v>
       </c>
     </row>
@@ -1450,7 +1476,7 @@
       <c r="U11" t="s">
         <v>28</v>
       </c>
-      <c r="V11" s="1">
+      <c r="V11" s="2">
         <v>46291</v>
       </c>
     </row>
@@ -1476,7 +1502,7 @@
       <c r="G12" t="s">
         <v>42</v>
       </c>
-      <c r="H12" s="1">
+      <c r="H12" s="2">
         <v>46079</v>
       </c>
       <c r="I12" t="s">
@@ -1509,7 +1535,7 @@
       <c r="U12" t="s">
         <v>180</v>
       </c>
-      <c r="V12" s="1">
+      <c r="V12" s="2">
         <v>46079</v>
       </c>
     </row>
@@ -1562,7 +1588,7 @@
       <c r="U13" t="s">
         <v>180</v>
       </c>
-      <c r="V13" s="1">
+      <c r="V13" s="2">
         <v>46352</v>
       </c>
     </row>
@@ -1615,7 +1641,7 @@
       <c r="U14" t="s">
         <v>180</v>
       </c>
-      <c r="V14" s="1">
+      <c r="V14" s="2">
         <v>46352</v>
       </c>
     </row>
@@ -1668,7 +1694,7 @@
       <c r="U15" t="s">
         <v>180</v>
       </c>
-      <c r="V15" s="1">
+      <c r="V15" s="2">
         <v>46352</v>
       </c>
     </row>
@@ -1721,7 +1747,7 @@
       <c r="U16" t="s">
         <v>180</v>
       </c>
-      <c r="V16" s="1">
+      <c r="V16" s="2">
         <v>46229</v>
       </c>
     </row>
@@ -1747,7 +1773,7 @@
       <c r="G17" t="s">
         <v>42</v>
       </c>
-      <c r="H17" s="1">
+      <c r="H17" s="2">
         <v>46098</v>
       </c>
       <c r="I17" t="s">
@@ -1780,7 +1806,7 @@
       <c r="U17" t="s">
         <v>180</v>
       </c>
-      <c r="V17" s="1">
+      <c r="V17" s="2">
         <v>46107</v>
       </c>
     </row>
@@ -1806,7 +1832,7 @@
       <c r="G18" t="s">
         <v>42</v>
       </c>
-      <c r="H18" s="1">
+      <c r="H18" s="2">
         <v>46076</v>
       </c>
       <c r="I18" t="s">
@@ -1836,7 +1862,7 @@
       <c r="U18" t="s">
         <v>28</v>
       </c>
-      <c r="V18" s="1">
+      <c r="V18" s="2">
         <v>46079</v>
       </c>
     </row>
@@ -1862,7 +1888,7 @@
       <c r="G19" t="s">
         <v>42</v>
       </c>
-      <c r="H19" s="1">
+      <c r="H19" s="2">
         <v>46076</v>
       </c>
       <c r="I19" t="s">
@@ -1892,7 +1918,7 @@
       <c r="U19" t="s">
         <v>28</v>
       </c>
-      <c r="V19" s="1">
+      <c r="V19" s="2">
         <v>46079</v>
       </c>
     </row>
@@ -1939,7 +1965,7 @@
       <c r="U20" t="s">
         <v>28</v>
       </c>
-      <c r="V20" s="1">
+      <c r="V20" s="2">
         <v>46321</v>
       </c>
     </row>
@@ -1986,7 +2012,7 @@
       <c r="U21" t="s">
         <v>28</v>
       </c>
-      <c r="V21" s="1">
+      <c r="V21" s="2">
         <v>46321</v>
       </c>
     </row>
@@ -2033,7 +2059,7 @@
       <c r="U22" t="s">
         <v>28</v>
       </c>
-      <c r="V22" s="1">
+      <c r="V22" s="2">
         <v>46321</v>
       </c>
     </row>
@@ -2080,7 +2106,7 @@
       <c r="U23" t="s">
         <v>28</v>
       </c>
-      <c r="V23" s="1">
+      <c r="V23" s="2">
         <v>46321</v>
       </c>
     </row>
@@ -2106,7 +2132,7 @@
       <c r="G24" t="s">
         <v>42</v>
       </c>
-      <c r="H24" s="1">
+      <c r="H24" s="2">
         <v>46119</v>
       </c>
       <c r="I24" t="s">
@@ -2139,7 +2165,7 @@
       <c r="U24" t="s">
         <v>180</v>
       </c>
-      <c r="V24" s="1">
+      <c r="V24" s="2">
         <v>46138</v>
       </c>
     </row>
@@ -2165,7 +2191,7 @@
       <c r="G25" t="s">
         <v>42</v>
       </c>
-      <c r="H25" s="1">
+      <c r="H25" s="2">
         <v>46121</v>
       </c>
       <c r="I25" t="s">
@@ -2195,7 +2221,7 @@
       <c r="U25" t="s">
         <v>28</v>
       </c>
-      <c r="V25" s="1">
+      <c r="V25" s="2">
         <v>46138</v>
       </c>
     </row>
@@ -2221,7 +2247,7 @@
       <c r="G26" t="s">
         <v>42</v>
       </c>
-      <c r="H26" s="1">
+      <c r="H26" s="2">
         <v>46076</v>
       </c>
       <c r="I26" t="s">
@@ -2251,7 +2277,7 @@
       <c r="U26" t="s">
         <v>28</v>
       </c>
-      <c r="V26" s="1">
+      <c r="V26" s="2">
         <v>46079</v>
       </c>
     </row>
@@ -2304,7 +2330,7 @@
       <c r="U27" t="s">
         <v>180</v>
       </c>
-      <c r="V27" s="1">
+      <c r="V27" s="2">
         <v>46291</v>
       </c>
     </row>
@@ -2330,7 +2356,7 @@
       <c r="G28" t="s">
         <v>42</v>
       </c>
-      <c r="H28" s="1">
+      <c r="H28" s="2">
         <v>46199</v>
       </c>
       <c r="I28" t="s">
@@ -2363,7 +2389,7 @@
       <c r="U28" t="s">
         <v>180</v>
       </c>
-      <c r="V28" s="1">
+      <c r="V28" s="2">
         <v>46199</v>
       </c>
     </row>
@@ -2389,7 +2415,7 @@
       <c r="G29" t="s">
         <v>42</v>
       </c>
-      <c r="H29" s="1">
+      <c r="H29" s="2">
         <v>46199</v>
       </c>
       <c r="I29" t="s">
@@ -2422,7 +2448,7 @@
       <c r="U29" t="s">
         <v>180</v>
       </c>
-      <c r="V29" s="1">
+      <c r="V29" s="2">
         <v>46199</v>
       </c>
     </row>
@@ -2448,7 +2474,7 @@
       <c r="G30" t="s">
         <v>42</v>
       </c>
-      <c r="H30" s="1">
+      <c r="H30" s="2">
         <v>46199</v>
       </c>
       <c r="I30" t="s">
@@ -2481,7 +2507,7 @@
       <c r="U30" t="s">
         <v>180</v>
       </c>
-      <c r="V30" s="1">
+      <c r="V30" s="2">
         <v>46199</v>
       </c>
     </row>
@@ -2507,7 +2533,7 @@
       <c r="G31" t="s">
         <v>42</v>
       </c>
-      <c r="H31" s="1">
+      <c r="H31" s="2">
         <v>46199</v>
       </c>
       <c r="I31" t="s">
@@ -2540,7 +2566,7 @@
       <c r="U31" t="s">
         <v>180</v>
       </c>
-      <c r="V31" s="1">
+      <c r="V31" s="2">
         <v>46199</v>
       </c>
     </row>
@@ -2590,7 +2616,7 @@
       <c r="U32" t="s">
         <v>180</v>
       </c>
-      <c r="V32" s="1">
+      <c r="V32" s="2">
         <v>46291</v>
       </c>
     </row>
@@ -2616,7 +2642,7 @@
       <c r="G33" t="s">
         <v>42</v>
       </c>
-      <c r="H33" s="1">
+      <c r="H33" s="2">
         <v>46191</v>
       </c>
       <c r="I33" t="s">
@@ -2649,7 +2675,7 @@
       <c r="U33" t="s">
         <v>180</v>
       </c>
-      <c r="V33" s="1">
+      <c r="V33" s="2">
         <v>46199</v>
       </c>
     </row>
@@ -2675,7 +2701,7 @@
       <c r="G34" t="s">
         <v>42</v>
       </c>
-      <c r="H34" s="1">
+      <c r="H34" s="2">
         <v>46119</v>
       </c>
       <c r="I34" t="s">
@@ -2705,7 +2731,7 @@
       <c r="U34" t="s">
         <v>180</v>
       </c>
-      <c r="V34" s="1">
+      <c r="V34" s="2">
         <v>46138</v>
       </c>
     </row>
@@ -2731,7 +2757,7 @@
       <c r="G35" t="s">
         <v>42</v>
       </c>
-      <c r="H35" s="1">
+      <c r="H35" s="2">
         <v>46213</v>
       </c>
       <c r="I35" t="s">
@@ -2761,7 +2787,7 @@
       <c r="U35" t="s">
         <v>28</v>
       </c>
-      <c r="V35" s="1">
+      <c r="V35" s="2">
         <v>46229</v>
       </c>
     </row>
@@ -2787,7 +2813,7 @@
       <c r="G36" t="s">
         <v>42</v>
       </c>
-      <c r="H36" s="1">
+      <c r="H36" s="2">
         <v>46175</v>
       </c>
       <c r="I36" t="s">
@@ -2817,7 +2843,7 @@
       <c r="U36" t="s">
         <v>28</v>
       </c>
-      <c r="V36" s="1">
+      <c r="V36" s="2">
         <v>46199</v>
       </c>
     </row>
@@ -2843,7 +2869,7 @@
       <c r="G37" t="s">
         <v>42</v>
       </c>
-      <c r="H37" s="1">
+      <c r="H37" s="2">
         <v>46213</v>
       </c>
       <c r="I37" t="s">
@@ -2873,7 +2899,7 @@
       <c r="U37" t="s">
         <v>28</v>
       </c>
-      <c r="V37" s="1">
+      <c r="V37" s="2">
         <v>46229</v>
       </c>
     </row>
@@ -2899,7 +2925,7 @@
       <c r="G38" t="s">
         <v>42</v>
       </c>
-      <c r="H38" s="1">
+      <c r="H38" s="2">
         <v>46199</v>
       </c>
       <c r="I38" t="s">
@@ -2929,7 +2955,7 @@
       <c r="U38" t="s">
         <v>28</v>
       </c>
-      <c r="V38" s="1">
+      <c r="V38" s="2">
         <v>46199</v>
       </c>
     </row>
@@ -2955,7 +2981,7 @@
       <c r="G39" t="s">
         <v>42</v>
       </c>
-      <c r="H39" s="1">
+      <c r="H39" s="2">
         <v>46199</v>
       </c>
       <c r="I39" t="s">
@@ -2985,7 +3011,7 @@
       <c r="U39" t="s">
         <v>28</v>
       </c>
-      <c r="V39" s="1">
+      <c r="V39" s="2">
         <v>46199</v>
       </c>
     </row>
@@ -3011,7 +3037,7 @@
       <c r="G40" t="s">
         <v>42</v>
       </c>
-      <c r="H40" s="1">
+      <c r="H40" s="2">
         <v>46204</v>
       </c>
       <c r="I40" t="s">
@@ -3041,7 +3067,7 @@
       <c r="U40" t="s">
         <v>28</v>
       </c>
-      <c r="V40" s="1">
+      <c r="V40" s="2">
         <v>46229</v>
       </c>
     </row>
@@ -3067,7 +3093,7 @@
       <c r="G41" t="s">
         <v>42</v>
       </c>
-      <c r="H41" s="1">
+      <c r="H41" s="2">
         <v>46244</v>
       </c>
       <c r="I41" t="s">
@@ -3097,7 +3123,7 @@
       <c r="U41" t="s">
         <v>28</v>
       </c>
-      <c r="V41" s="1">
+      <c r="V41" s="2">
         <v>46199</v>
       </c>
     </row>
@@ -3141,7 +3167,7 @@
       <c r="U42" t="s">
         <v>28</v>
       </c>
-      <c r="V42" s="1">
+      <c r="V42" s="2">
         <v>46260</v>
       </c>
     </row>
@@ -3167,7 +3193,7 @@
       <c r="G43" t="s">
         <v>42</v>
       </c>
-      <c r="H43" s="1">
+      <c r="H43" s="2">
         <v>46191</v>
       </c>
       <c r="I43" t="s">
@@ -3197,7 +3223,7 @@
       <c r="U43" t="s">
         <v>28</v>
       </c>
-      <c r="V43" s="1">
+      <c r="V43" s="2">
         <v>46199</v>
       </c>
     </row>
@@ -3223,7 +3249,7 @@
       <c r="G44" t="s">
         <v>42</v>
       </c>
-      <c r="H44" s="1">
+      <c r="H44" s="2">
         <v>46191</v>
       </c>
       <c r="I44" t="s">
@@ -3253,7 +3279,7 @@
       <c r="U44" t="s">
         <v>28</v>
       </c>
-      <c r="V44" s="1">
+      <c r="V44" s="2">
         <v>46199</v>
       </c>
     </row>
@@ -3279,7 +3305,7 @@
       <c r="G45" t="s">
         <v>42</v>
       </c>
-      <c r="H45" s="1">
+      <c r="H45" s="2">
         <v>46213</v>
       </c>
       <c r="I45" t="s">
@@ -3312,7 +3338,7 @@
       <c r="U45" t="s">
         <v>180</v>
       </c>
-      <c r="V45" s="1">
+      <c r="V45" s="2">
         <v>46229</v>
       </c>
     </row>
@@ -3338,7 +3364,7 @@
       <c r="G46" t="s">
         <v>42</v>
       </c>
-      <c r="H46" s="1">
+      <c r="H46" s="2">
         <v>46210</v>
       </c>
       <c r="I46" t="s">
@@ -3368,7 +3394,7 @@
       <c r="U46" t="s">
         <v>180</v>
       </c>
-      <c r="V46" s="1">
+      <c r="V46" s="2">
         <v>46229</v>
       </c>
     </row>
@@ -3415,7 +3441,7 @@
       <c r="U47" t="s">
         <v>28</v>
       </c>
-      <c r="V47" s="1">
+      <c r="V47" s="2">
         <v>46321</v>
       </c>
     </row>
@@ -3468,7 +3494,7 @@
       <c r="U48" t="s">
         <v>180</v>
       </c>
-      <c r="V48" s="1">
+      <c r="V48" s="2">
         <v>46291</v>
       </c>
     </row>
@@ -3494,7 +3520,7 @@
       <c r="G49" t="s">
         <v>42</v>
       </c>
-      <c r="H49" s="1">
+      <c r="H49" s="2">
         <v>46176</v>
       </c>
       <c r="I49" t="s">
@@ -3527,7 +3553,7 @@
       <c r="U49" t="s">
         <v>180</v>
       </c>
-      <c r="V49" s="1">
+      <c r="V49" s="2">
         <v>46199</v>
       </c>
     </row>
@@ -3580,7 +3606,7 @@
       <c r="U50" t="s">
         <v>180</v>
       </c>
-      <c r="V50" s="1">
+      <c r="V50" s="2">
         <v>46260</v>
       </c>
     </row>
@@ -3633,7 +3659,7 @@
       <c r="U51" t="s">
         <v>180</v>
       </c>
-      <c r="V51" s="1">
+      <c r="V51" s="2">
         <v>46291</v>
       </c>
     </row>
@@ -3683,7 +3709,7 @@
       <c r="U52" t="s">
         <v>180</v>
       </c>
-      <c r="V52" s="1">
+      <c r="V52" s="2">
         <v>46321</v>
       </c>
     </row>
@@ -3709,7 +3735,7 @@
       <c r="G53" t="s">
         <v>42</v>
       </c>
-      <c r="H53" s="1">
+      <c r="H53" s="2">
         <v>46227</v>
       </c>
       <c r="I53" t="s">
@@ -3739,7 +3765,7 @@
       <c r="U53" t="s">
         <v>180</v>
       </c>
-      <c r="V53" s="1">
+      <c r="V53" s="2">
         <v>46229</v>
       </c>
     </row>
@@ -3792,7 +3818,7 @@
       <c r="U54" t="s">
         <v>180</v>
       </c>
-      <c r="V54" s="1">
+      <c r="V54" s="2">
         <v>46352</v>
       </c>
     </row>
@@ -3819,7 +3845,7 @@
         <v>62</v>
       </c>
       <c r="K55" t="s">
-        <v>74</v>
+        <v>71</v>
       </c>
       <c r="N55" t="s">
         <v>88</v>
@@ -3845,7 +3871,7 @@
       <c r="U55" t="s">
         <v>180</v>
       </c>
-      <c r="V55" s="1">
+      <c r="V55" s="2">
         <v>46321</v>
       </c>
     </row>
@@ -3895,7 +3921,7 @@
       <c r="U56" t="s">
         <v>180</v>
       </c>
-      <c r="V56" s="1">
+      <c r="V56" s="2">
         <v>46321</v>
       </c>
     </row>
@@ -3939,7 +3965,7 @@
       <c r="U57" t="s">
         <v>180</v>
       </c>
-      <c r="V57" s="1">
+      <c r="V57" s="2">
         <v>46049</v>
       </c>
     </row>
@@ -4065,7 +4091,7 @@
       <c r="U60" t="s">
         <v>180</v>
       </c>
-      <c r="V60" s="1">
+      <c r="V60" s="2">
         <v>46107</v>
       </c>
     </row>
@@ -4109,7 +4135,7 @@
       <c r="U61" t="s">
         <v>180</v>
       </c>
-      <c r="V61" s="1">
+      <c r="V61" s="2">
         <v>46107</v>
       </c>
     </row>
@@ -4153,7 +4179,7 @@
       <c r="U62" t="s">
         <v>180</v>
       </c>
-      <c r="V62" s="1">
+      <c r="V62" s="2">
         <v>46107</v>
       </c>
     </row>
@@ -4197,7 +4223,7 @@
       <c r="U63" t="s">
         <v>180</v>
       </c>
-      <c r="V63" s="1">
+      <c r="V63" s="2">
         <v>46107</v>
       </c>
     </row>
@@ -4241,7 +4267,7 @@
       <c r="U64" t="s">
         <v>180</v>
       </c>
-      <c r="V64" s="1">
+      <c r="V64" s="2">
         <v>46107</v>
       </c>
     </row>
@@ -4285,7 +4311,7 @@
       <c r="U65" t="s">
         <v>180</v>
       </c>
-      <c r="V65" s="1">
+      <c r="V65" s="2">
         <v>46107</v>
       </c>
     </row>
@@ -4329,7 +4355,7 @@
       <c r="U66" t="s">
         <v>28</v>
       </c>
-      <c r="V66" s="1">
+      <c r="V66" s="2">
         <v>46168</v>
       </c>
     </row>
@@ -4376,7 +4402,7 @@
       <c r="U67" t="s">
         <v>28</v>
       </c>
-      <c r="V67" s="1">
+      <c r="V67" s="2">
         <v>46291</v>
       </c>
     </row>
@@ -4429,7 +4455,7 @@
       <c r="U68" t="s">
         <v>180</v>
       </c>
-      <c r="V68" s="1">
+      <c r="V68" s="2">
         <v>46229</v>
       </c>
     </row>
@@ -4473,7 +4499,7 @@
       <c r="U69" t="s">
         <v>28</v>
       </c>
-      <c r="V69" s="1">
+      <c r="V69" s="2">
         <v>46260</v>
       </c>
     </row>
@@ -4517,7 +4543,7 @@
       <c r="U70" t="s">
         <v>180</v>
       </c>
-      <c r="V70" s="1">
+      <c r="V70" s="2">
         <v>46291</v>
       </c>
     </row>
@@ -4561,7 +4587,7 @@
       <c r="U71" t="s">
         <v>180</v>
       </c>
-      <c r="V71" s="1">
+      <c r="V71" s="2">
         <v>46168</v>
       </c>
     </row>
@@ -4605,7 +4631,7 @@
       <c r="U72" t="s">
         <v>180</v>
       </c>
-      <c r="V72" s="1">
+      <c r="V72" s="2">
         <v>46291</v>
       </c>
     </row>
@@ -4649,7 +4675,7 @@
       <c r="U73" t="s">
         <v>180</v>
       </c>
-      <c r="V73" s="1">
+      <c r="V73" s="2">
         <v>46291</v>
       </c>
     </row>
@@ -4693,7 +4719,7 @@
       <c r="U74" t="s">
         <v>180</v>
       </c>
-      <c r="V74" s="1">
+      <c r="V74" s="2">
         <v>46291</v>
       </c>
     </row>
@@ -4740,7 +4766,7 @@
       <c r="U75" t="s">
         <v>28</v>
       </c>
-      <c r="V75" s="1">
+      <c r="V75" s="2">
         <v>46321</v>
       </c>
     </row>
@@ -4790,7 +4816,7 @@
       <c r="U76" t="s">
         <v>180</v>
       </c>
-      <c r="V76" s="1">
+      <c r="V76" s="2">
         <v>46381</v>
       </c>
     </row>
@@ -4840,7 +4866,7 @@
       <c r="U77" t="s">
         <v>180</v>
       </c>
-      <c r="V77" s="1">
+      <c r="V77" s="2">
         <v>46381</v>
       </c>
     </row>
@@ -4890,7 +4916,7 @@
       <c r="U78" t="s">
         <v>28</v>
       </c>
-      <c r="V78" s="1">
+      <c r="V78" s="2">
         <v>46381</v>
       </c>
     </row>
@@ -4940,7 +4966,7 @@
       <c r="U79" t="s">
         <v>28</v>
       </c>
-      <c r="V79" s="1">
+      <c r="V79" s="2">
         <v>46381</v>
       </c>
     </row>
@@ -4990,7 +5016,7 @@
       <c r="U80" t="s">
         <v>28</v>
       </c>
-      <c r="V80" s="1">
+      <c r="V80" s="2">
         <v>46382</v>
       </c>
     </row>
@@ -5034,7 +5060,7 @@
       <c r="U81" t="s">
         <v>28</v>
       </c>
-      <c r="V81" s="1">
+      <c r="V81" s="2">
         <v>46382</v>
       </c>
     </row>
@@ -5087,7 +5113,7 @@
       <c r="U82" t="s">
         <v>180</v>
       </c>
-      <c r="V82" s="1">
+      <c r="V82" s="2">
         <v>46382</v>
       </c>
     </row>
@@ -5131,7 +5157,7 @@
       <c r="U83" t="s">
         <v>28</v>
       </c>
-      <c r="V83" s="1">
+      <c r="V83" s="2">
         <v>46321</v>
       </c>
     </row>
@@ -5175,7 +5201,7 @@
       <c r="U84" t="s">
         <v>28</v>
       </c>
-      <c r="V84" s="1">
+      <c r="V84" s="2">
         <v>46382</v>
       </c>
     </row>
@@ -5316,7 +5342,7 @@
       <c r="U87" t="s">
         <v>28</v>
       </c>
-      <c r="V87" s="1">
+      <c r="V87" s="2">
         <v>46291</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Atualização automática: mta (15/09/2026 12:33)
</commit_message>
<xml_diff>
--- a/Projetos/02_Dados_Tratados/base_mta_tratada.xlsx
+++ b/Projetos/02_Dados_Tratados/base_mta_tratada.xlsx
@@ -566,16 +566,8 @@
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="YYYY-MM-DD HH:MM:SS"/>
   </numFmts>
-  <fonts count="2">
+  <fonts count="1">
     <font>
-      <sz val="11"/>
-      <color theme="1"/>
-      <name val="Calibri"/>
-      <family val="2"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <b/>
       <sz val="11"/>
       <color theme="1"/>
       <name val="Calibri"/>
@@ -591,7 +583,7 @@
       <patternFill patternType="gray125"/>
     </fill>
   </fills>
-  <borders count="2">
+  <borders count="1">
     <border>
       <left/>
       <right/>
@@ -599,30 +591,12 @@
       <bottom/>
       <diagonal/>
     </border>
-    <border>
-      <left style="thin">
-        <color auto="1"/>
-      </left>
-      <right style="thin">
-        <color auto="1"/>
-      </right>
-      <top style="thin">
-        <color auto="1"/>
-      </top>
-      <bottom style="thin">
-        <color auto="1"/>
-      </bottom>
-      <diagonal/>
-    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="3">
+  <cellXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top"/>
-    </xf>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
   </cellXfs>
   <cellStyles count="1">
@@ -922,70 +896,70 @@
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:22">
-      <c r="A1" s="1" t="s">
+      <c r="A1" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="1" t="s">
+      <c r="B1" t="s">
         <v>1</v>
       </c>
-      <c r="C1" s="1" t="s">
+      <c r="C1" t="s">
         <v>2</v>
       </c>
-      <c r="D1" s="1" t="s">
+      <c r="D1" t="s">
         <v>3</v>
       </c>
-      <c r="E1" s="1" t="s">
+      <c r="E1" t="s">
         <v>4</v>
       </c>
-      <c r="F1" s="1" t="s">
+      <c r="F1" t="s">
         <v>5</v>
       </c>
-      <c r="G1" s="1" t="s">
+      <c r="G1" t="s">
         <v>6</v>
       </c>
-      <c r="H1" s="1" t="s">
+      <c r="H1" t="s">
         <v>7</v>
       </c>
-      <c r="I1" s="1" t="s">
+      <c r="I1" t="s">
         <v>8</v>
       </c>
-      <c r="J1" s="1" t="s">
+      <c r="J1" t="s">
         <v>9</v>
       </c>
-      <c r="K1" s="1" t="s">
+      <c r="K1" t="s">
         <v>10</v>
       </c>
-      <c r="L1" s="1" t="s">
+      <c r="L1" t="s">
         <v>11</v>
       </c>
-      <c r="M1" s="1" t="s">
+      <c r="M1" t="s">
         <v>12</v>
       </c>
-      <c r="N1" s="1" t="s">
+      <c r="N1" t="s">
         <v>13</v>
       </c>
-      <c r="O1" s="1" t="s">
+      <c r="O1" t="s">
         <v>14</v>
       </c>
-      <c r="P1" s="1" t="s">
+      <c r="P1" t="s">
         <v>15</v>
       </c>
-      <c r="Q1" s="1" t="s">
+      <c r="Q1" t="s">
         <v>16</v>
       </c>
-      <c r="R1" s="1" t="s">
+      <c r="R1" t="s">
         <v>17</v>
       </c>
-      <c r="S1" s="1" t="s">
+      <c r="S1" t="s">
         <v>18</v>
       </c>
-      <c r="T1" s="1" t="s">
+      <c r="T1" t="s">
         <v>19</v>
       </c>
-      <c r="U1" s="1" t="s">
+      <c r="U1" t="s">
         <v>20</v>
       </c>
-      <c r="V1" s="1" t="s">
+      <c r="V1" t="s">
         <v>21</v>
       </c>
     </row>
@@ -1041,7 +1015,7 @@
       <c r="U2" t="s">
         <v>180</v>
       </c>
-      <c r="V2" s="2">
+      <c r="V2" s="1">
         <v>46229</v>
       </c>
     </row>
@@ -1088,7 +1062,7 @@
       <c r="U3" t="s">
         <v>28</v>
       </c>
-      <c r="V3" s="2">
+      <c r="V3" s="1">
         <v>46291</v>
       </c>
     </row>
@@ -1135,7 +1109,7 @@
       <c r="U4" t="s">
         <v>28</v>
       </c>
-      <c r="V4" s="2">
+      <c r="V4" s="1">
         <v>46321</v>
       </c>
     </row>
@@ -1182,7 +1156,7 @@
       <c r="U5" t="s">
         <v>28</v>
       </c>
-      <c r="V5" s="2">
+      <c r="V5" s="1">
         <v>46321</v>
       </c>
     </row>
@@ -1232,7 +1206,7 @@
       <c r="U6" t="s">
         <v>28</v>
       </c>
-      <c r="V6" s="2">
+      <c r="V6" s="1">
         <v>46291</v>
       </c>
     </row>
@@ -1258,7 +1232,7 @@
       <c r="G7" t="s">
         <v>42</v>
       </c>
-      <c r="H7" s="2">
+      <c r="H7" s="1">
         <v>46121</v>
       </c>
       <c r="I7" t="s">
@@ -1288,7 +1262,7 @@
       <c r="U7" t="s">
         <v>28</v>
       </c>
-      <c r="V7" s="2">
+      <c r="V7" s="1">
         <v>46138</v>
       </c>
     </row>
@@ -1335,7 +1309,7 @@
       <c r="U8" t="s">
         <v>28</v>
       </c>
-      <c r="V8" s="2">
+      <c r="V8" s="1">
         <v>46291</v>
       </c>
     </row>
@@ -1382,7 +1356,7 @@
       <c r="U9" t="s">
         <v>28</v>
       </c>
-      <c r="V9" s="2">
+      <c r="V9" s="1">
         <v>46291</v>
       </c>
     </row>
@@ -1429,7 +1403,7 @@
       <c r="U10" t="s">
         <v>28</v>
       </c>
-      <c r="V10" s="2">
+      <c r="V10" s="1">
         <v>46291</v>
       </c>
     </row>
@@ -1476,7 +1450,7 @@
       <c r="U11" t="s">
         <v>28</v>
       </c>
-      <c r="V11" s="2">
+      <c r="V11" s="1">
         <v>46291</v>
       </c>
     </row>
@@ -1502,7 +1476,7 @@
       <c r="G12" t="s">
         <v>42</v>
       </c>
-      <c r="H12" s="2">
+      <c r="H12" s="1">
         <v>46079</v>
       </c>
       <c r="I12" t="s">
@@ -1535,7 +1509,7 @@
       <c r="U12" t="s">
         <v>180</v>
       </c>
-      <c r="V12" s="2">
+      <c r="V12" s="1">
         <v>46079</v>
       </c>
     </row>
@@ -1588,7 +1562,7 @@
       <c r="U13" t="s">
         <v>180</v>
       </c>
-      <c r="V13" s="2">
+      <c r="V13" s="1">
         <v>46352</v>
       </c>
     </row>
@@ -1641,7 +1615,7 @@
       <c r="U14" t="s">
         <v>180</v>
       </c>
-      <c r="V14" s="2">
+      <c r="V14" s="1">
         <v>46352</v>
       </c>
     </row>
@@ -1694,7 +1668,7 @@
       <c r="U15" t="s">
         <v>180</v>
       </c>
-      <c r="V15" s="2">
+      <c r="V15" s="1">
         <v>46352</v>
       </c>
     </row>
@@ -1747,7 +1721,7 @@
       <c r="U16" t="s">
         <v>180</v>
       </c>
-      <c r="V16" s="2">
+      <c r="V16" s="1">
         <v>46229</v>
       </c>
     </row>
@@ -1773,7 +1747,7 @@
       <c r="G17" t="s">
         <v>42</v>
       </c>
-      <c r="H17" s="2">
+      <c r="H17" s="1">
         <v>46098</v>
       </c>
       <c r="I17" t="s">
@@ -1806,7 +1780,7 @@
       <c r="U17" t="s">
         <v>180</v>
       </c>
-      <c r="V17" s="2">
+      <c r="V17" s="1">
         <v>46107</v>
       </c>
     </row>
@@ -1832,7 +1806,7 @@
       <c r="G18" t="s">
         <v>42</v>
       </c>
-      <c r="H18" s="2">
+      <c r="H18" s="1">
         <v>46076</v>
       </c>
       <c r="I18" t="s">
@@ -1862,7 +1836,7 @@
       <c r="U18" t="s">
         <v>28</v>
       </c>
-      <c r="V18" s="2">
+      <c r="V18" s="1">
         <v>46079</v>
       </c>
     </row>
@@ -1888,7 +1862,7 @@
       <c r="G19" t="s">
         <v>42</v>
       </c>
-      <c r="H19" s="2">
+      <c r="H19" s="1">
         <v>46076</v>
       </c>
       <c r="I19" t="s">
@@ -1918,7 +1892,7 @@
       <c r="U19" t="s">
         <v>28</v>
       </c>
-      <c r="V19" s="2">
+      <c r="V19" s="1">
         <v>46079</v>
       </c>
     </row>
@@ -1965,7 +1939,7 @@
       <c r="U20" t="s">
         <v>28</v>
       </c>
-      <c r="V20" s="2">
+      <c r="V20" s="1">
         <v>46321</v>
       </c>
     </row>
@@ -2012,7 +1986,7 @@
       <c r="U21" t="s">
         <v>28</v>
       </c>
-      <c r="V21" s="2">
+      <c r="V21" s="1">
         <v>46321</v>
       </c>
     </row>
@@ -2059,7 +2033,7 @@
       <c r="U22" t="s">
         <v>28</v>
       </c>
-      <c r="V22" s="2">
+      <c r="V22" s="1">
         <v>46321</v>
       </c>
     </row>
@@ -2106,7 +2080,7 @@
       <c r="U23" t="s">
         <v>28</v>
       </c>
-      <c r="V23" s="2">
+      <c r="V23" s="1">
         <v>46321</v>
       </c>
     </row>
@@ -2132,7 +2106,7 @@
       <c r="G24" t="s">
         <v>42</v>
       </c>
-      <c r="H24" s="2">
+      <c r="H24" s="1">
         <v>46119</v>
       </c>
       <c r="I24" t="s">
@@ -2165,7 +2139,7 @@
       <c r="U24" t="s">
         <v>180</v>
       </c>
-      <c r="V24" s="2">
+      <c r="V24" s="1">
         <v>46138</v>
       </c>
     </row>
@@ -2191,7 +2165,7 @@
       <c r="G25" t="s">
         <v>42</v>
       </c>
-      <c r="H25" s="2">
+      <c r="H25" s="1">
         <v>46121</v>
       </c>
       <c r="I25" t="s">
@@ -2221,7 +2195,7 @@
       <c r="U25" t="s">
         <v>28</v>
       </c>
-      <c r="V25" s="2">
+      <c r="V25" s="1">
         <v>46138</v>
       </c>
     </row>
@@ -2247,7 +2221,7 @@
       <c r="G26" t="s">
         <v>42</v>
       </c>
-      <c r="H26" s="2">
+      <c r="H26" s="1">
         <v>46076</v>
       </c>
       <c r="I26" t="s">
@@ -2277,7 +2251,7 @@
       <c r="U26" t="s">
         <v>28</v>
       </c>
-      <c r="V26" s="2">
+      <c r="V26" s="1">
         <v>46079</v>
       </c>
     </row>
@@ -2330,7 +2304,7 @@
       <c r="U27" t="s">
         <v>180</v>
       </c>
-      <c r="V27" s="2">
+      <c r="V27" s="1">
         <v>46291</v>
       </c>
     </row>
@@ -2356,7 +2330,7 @@
       <c r="G28" t="s">
         <v>42</v>
       </c>
-      <c r="H28" s="2">
+      <c r="H28" s="1">
         <v>46199</v>
       </c>
       <c r="I28" t="s">
@@ -2389,7 +2363,7 @@
       <c r="U28" t="s">
         <v>180</v>
       </c>
-      <c r="V28" s="2">
+      <c r="V28" s="1">
         <v>46199</v>
       </c>
     </row>
@@ -2415,7 +2389,7 @@
       <c r="G29" t="s">
         <v>42</v>
       </c>
-      <c r="H29" s="2">
+      <c r="H29" s="1">
         <v>46199</v>
       </c>
       <c r="I29" t="s">
@@ -2448,7 +2422,7 @@
       <c r="U29" t="s">
         <v>180</v>
       </c>
-      <c r="V29" s="2">
+      <c r="V29" s="1">
         <v>46199</v>
       </c>
     </row>
@@ -2474,7 +2448,7 @@
       <c r="G30" t="s">
         <v>42</v>
       </c>
-      <c r="H30" s="2">
+      <c r="H30" s="1">
         <v>46199</v>
       </c>
       <c r="I30" t="s">
@@ -2507,7 +2481,7 @@
       <c r="U30" t="s">
         <v>180</v>
       </c>
-      <c r="V30" s="2">
+      <c r="V30" s="1">
         <v>46199</v>
       </c>
     </row>
@@ -2533,7 +2507,7 @@
       <c r="G31" t="s">
         <v>42</v>
       </c>
-      <c r="H31" s="2">
+      <c r="H31" s="1">
         <v>46199</v>
       </c>
       <c r="I31" t="s">
@@ -2566,7 +2540,7 @@
       <c r="U31" t="s">
         <v>180</v>
       </c>
-      <c r="V31" s="2">
+      <c r="V31" s="1">
         <v>46199</v>
       </c>
     </row>
@@ -2616,7 +2590,7 @@
       <c r="U32" t="s">
         <v>180</v>
       </c>
-      <c r="V32" s="2">
+      <c r="V32" s="1">
         <v>46291</v>
       </c>
     </row>
@@ -2642,7 +2616,7 @@
       <c r="G33" t="s">
         <v>42</v>
       </c>
-      <c r="H33" s="2">
+      <c r="H33" s="1">
         <v>46191</v>
       </c>
       <c r="I33" t="s">
@@ -2675,7 +2649,7 @@
       <c r="U33" t="s">
         <v>180</v>
       </c>
-      <c r="V33" s="2">
+      <c r="V33" s="1">
         <v>46199</v>
       </c>
     </row>
@@ -2701,7 +2675,7 @@
       <c r="G34" t="s">
         <v>42</v>
       </c>
-      <c r="H34" s="2">
+      <c r="H34" s="1">
         <v>46119</v>
       </c>
       <c r="I34" t="s">
@@ -2731,7 +2705,7 @@
       <c r="U34" t="s">
         <v>180</v>
       </c>
-      <c r="V34" s="2">
+      <c r="V34" s="1">
         <v>46138</v>
       </c>
     </row>
@@ -2757,7 +2731,7 @@
       <c r="G35" t="s">
         <v>42</v>
       </c>
-      <c r="H35" s="2">
+      <c r="H35" s="1">
         <v>46213</v>
       </c>
       <c r="I35" t="s">
@@ -2787,7 +2761,7 @@
       <c r="U35" t="s">
         <v>28</v>
       </c>
-      <c r="V35" s="2">
+      <c r="V35" s="1">
         <v>46229</v>
       </c>
     </row>
@@ -2813,7 +2787,7 @@
       <c r="G36" t="s">
         <v>42</v>
       </c>
-      <c r="H36" s="2">
+      <c r="H36" s="1">
         <v>46175</v>
       </c>
       <c r="I36" t="s">
@@ -2843,7 +2817,7 @@
       <c r="U36" t="s">
         <v>28</v>
       </c>
-      <c r="V36" s="2">
+      <c r="V36" s="1">
         <v>46199</v>
       </c>
     </row>
@@ -2869,7 +2843,7 @@
       <c r="G37" t="s">
         <v>42</v>
       </c>
-      <c r="H37" s="2">
+      <c r="H37" s="1">
         <v>46213</v>
       </c>
       <c r="I37" t="s">
@@ -2899,7 +2873,7 @@
       <c r="U37" t="s">
         <v>28</v>
       </c>
-      <c r="V37" s="2">
+      <c r="V37" s="1">
         <v>46229</v>
       </c>
     </row>
@@ -2925,7 +2899,7 @@
       <c r="G38" t="s">
         <v>42</v>
       </c>
-      <c r="H38" s="2">
+      <c r="H38" s="1">
         <v>46199</v>
       </c>
       <c r="I38" t="s">
@@ -2955,7 +2929,7 @@
       <c r="U38" t="s">
         <v>28</v>
       </c>
-      <c r="V38" s="2">
+      <c r="V38" s="1">
         <v>46199</v>
       </c>
     </row>
@@ -2981,7 +2955,7 @@
       <c r="G39" t="s">
         <v>42</v>
       </c>
-      <c r="H39" s="2">
+      <c r="H39" s="1">
         <v>46199</v>
       </c>
       <c r="I39" t="s">
@@ -3011,7 +2985,7 @@
       <c r="U39" t="s">
         <v>28</v>
       </c>
-      <c r="V39" s="2">
+      <c r="V39" s="1">
         <v>46199</v>
       </c>
     </row>
@@ -3037,7 +3011,7 @@
       <c r="G40" t="s">
         <v>42</v>
       </c>
-      <c r="H40" s="2">
+      <c r="H40" s="1">
         <v>46204</v>
       </c>
       <c r="I40" t="s">
@@ -3067,7 +3041,7 @@
       <c r="U40" t="s">
         <v>28</v>
       </c>
-      <c r="V40" s="2">
+      <c r="V40" s="1">
         <v>46229</v>
       </c>
     </row>
@@ -3093,7 +3067,7 @@
       <c r="G41" t="s">
         <v>42</v>
       </c>
-      <c r="H41" s="2">
+      <c r="H41" s="1">
         <v>46244</v>
       </c>
       <c r="I41" t="s">
@@ -3123,7 +3097,7 @@
       <c r="U41" t="s">
         <v>28</v>
       </c>
-      <c r="V41" s="2">
+      <c r="V41" s="1">
         <v>46199</v>
       </c>
     </row>
@@ -3167,7 +3141,7 @@
       <c r="U42" t="s">
         <v>28</v>
       </c>
-      <c r="V42" s="2">
+      <c r="V42" s="1">
         <v>46260</v>
       </c>
     </row>
@@ -3193,7 +3167,7 @@
       <c r="G43" t="s">
         <v>42</v>
       </c>
-      <c r="H43" s="2">
+      <c r="H43" s="1">
         <v>46191</v>
       </c>
       <c r="I43" t="s">
@@ -3223,7 +3197,7 @@
       <c r="U43" t="s">
         <v>28</v>
       </c>
-      <c r="V43" s="2">
+      <c r="V43" s="1">
         <v>46199</v>
       </c>
     </row>
@@ -3249,7 +3223,7 @@
       <c r="G44" t="s">
         <v>42</v>
       </c>
-      <c r="H44" s="2">
+      <c r="H44" s="1">
         <v>46191</v>
       </c>
       <c r="I44" t="s">
@@ -3279,7 +3253,7 @@
       <c r="U44" t="s">
         <v>28</v>
       </c>
-      <c r="V44" s="2">
+      <c r="V44" s="1">
         <v>46199</v>
       </c>
     </row>
@@ -3305,7 +3279,7 @@
       <c r="G45" t="s">
         <v>42</v>
       </c>
-      <c r="H45" s="2">
+      <c r="H45" s="1">
         <v>46213</v>
       </c>
       <c r="I45" t="s">
@@ -3338,7 +3312,7 @@
       <c r="U45" t="s">
         <v>180</v>
       </c>
-      <c r="V45" s="2">
+      <c r="V45" s="1">
         <v>46229</v>
       </c>
     </row>
@@ -3364,7 +3338,7 @@
       <c r="G46" t="s">
         <v>42</v>
       </c>
-      <c r="H46" s="2">
+      <c r="H46" s="1">
         <v>46210</v>
       </c>
       <c r="I46" t="s">
@@ -3394,7 +3368,7 @@
       <c r="U46" t="s">
         <v>180</v>
       </c>
-      <c r="V46" s="2">
+      <c r="V46" s="1">
         <v>46229</v>
       </c>
     </row>
@@ -3441,7 +3415,7 @@
       <c r="U47" t="s">
         <v>28</v>
       </c>
-      <c r="V47" s="2">
+      <c r="V47" s="1">
         <v>46321</v>
       </c>
     </row>
@@ -3494,7 +3468,7 @@
       <c r="U48" t="s">
         <v>180</v>
       </c>
-      <c r="V48" s="2">
+      <c r="V48" s="1">
         <v>46291</v>
       </c>
     </row>
@@ -3520,7 +3494,7 @@
       <c r="G49" t="s">
         <v>42</v>
       </c>
-      <c r="H49" s="2">
+      <c r="H49" s="1">
         <v>46176</v>
       </c>
       <c r="I49" t="s">
@@ -3553,7 +3527,7 @@
       <c r="U49" t="s">
         <v>180</v>
       </c>
-      <c r="V49" s="2">
+      <c r="V49" s="1">
         <v>46199</v>
       </c>
     </row>
@@ -3606,7 +3580,7 @@
       <c r="U50" t="s">
         <v>180</v>
       </c>
-      <c r="V50" s="2">
+      <c r="V50" s="1">
         <v>46260</v>
       </c>
     </row>
@@ -3659,7 +3633,7 @@
       <c r="U51" t="s">
         <v>180</v>
       </c>
-      <c r="V51" s="2">
+      <c r="V51" s="1">
         <v>46291</v>
       </c>
     </row>
@@ -3709,7 +3683,7 @@
       <c r="U52" t="s">
         <v>180</v>
       </c>
-      <c r="V52" s="2">
+      <c r="V52" s="1">
         <v>46321</v>
       </c>
     </row>
@@ -3735,7 +3709,7 @@
       <c r="G53" t="s">
         <v>42</v>
       </c>
-      <c r="H53" s="2">
+      <c r="H53" s="1">
         <v>46227</v>
       </c>
       <c r="I53" t="s">
@@ -3765,7 +3739,7 @@
       <c r="U53" t="s">
         <v>180</v>
       </c>
-      <c r="V53" s="2">
+      <c r="V53" s="1">
         <v>46229</v>
       </c>
     </row>
@@ -3818,7 +3792,7 @@
       <c r="U54" t="s">
         <v>180</v>
       </c>
-      <c r="V54" s="2">
+      <c r="V54" s="1">
         <v>46352</v>
       </c>
     </row>
@@ -3871,7 +3845,7 @@
       <c r="U55" t="s">
         <v>180</v>
       </c>
-      <c r="V55" s="2">
+      <c r="V55" s="1">
         <v>46321</v>
       </c>
     </row>
@@ -3921,7 +3895,7 @@
       <c r="U56" t="s">
         <v>180</v>
       </c>
-      <c r="V56" s="2">
+      <c r="V56" s="1">
         <v>46321</v>
       </c>
     </row>
@@ -3965,7 +3939,7 @@
       <c r="U57" t="s">
         <v>180</v>
       </c>
-      <c r="V57" s="2">
+      <c r="V57" s="1">
         <v>46049</v>
       </c>
     </row>
@@ -4091,7 +4065,7 @@
       <c r="U60" t="s">
         <v>180</v>
       </c>
-      <c r="V60" s="2">
+      <c r="V60" s="1">
         <v>46107</v>
       </c>
     </row>
@@ -4135,7 +4109,7 @@
       <c r="U61" t="s">
         <v>180</v>
       </c>
-      <c r="V61" s="2">
+      <c r="V61" s="1">
         <v>46107</v>
       </c>
     </row>
@@ -4179,7 +4153,7 @@
       <c r="U62" t="s">
         <v>180</v>
       </c>
-      <c r="V62" s="2">
+      <c r="V62" s="1">
         <v>46107</v>
       </c>
     </row>
@@ -4223,7 +4197,7 @@
       <c r="U63" t="s">
         <v>180</v>
       </c>
-      <c r="V63" s="2">
+      <c r="V63" s="1">
         <v>46107</v>
       </c>
     </row>
@@ -4267,7 +4241,7 @@
       <c r="U64" t="s">
         <v>180</v>
       </c>
-      <c r="V64" s="2">
+      <c r="V64" s="1">
         <v>46107</v>
       </c>
     </row>
@@ -4311,7 +4285,7 @@
       <c r="U65" t="s">
         <v>180</v>
       </c>
-      <c r="V65" s="2">
+      <c r="V65" s="1">
         <v>46107</v>
       </c>
     </row>
@@ -4355,7 +4329,7 @@
       <c r="U66" t="s">
         <v>28</v>
       </c>
-      <c r="V66" s="2">
+      <c r="V66" s="1">
         <v>46168</v>
       </c>
     </row>
@@ -4402,7 +4376,7 @@
       <c r="U67" t="s">
         <v>28</v>
       </c>
-      <c r="V67" s="2">
+      <c r="V67" s="1">
         <v>46291</v>
       </c>
     </row>
@@ -4455,7 +4429,7 @@
       <c r="U68" t="s">
         <v>180</v>
       </c>
-      <c r="V68" s="2">
+      <c r="V68" s="1">
         <v>46229</v>
       </c>
     </row>
@@ -4499,7 +4473,7 @@
       <c r="U69" t="s">
         <v>28</v>
       </c>
-      <c r="V69" s="2">
+      <c r="V69" s="1">
         <v>46260</v>
       </c>
     </row>
@@ -4543,7 +4517,7 @@
       <c r="U70" t="s">
         <v>180</v>
       </c>
-      <c r="V70" s="2">
+      <c r="V70" s="1">
         <v>46291</v>
       </c>
     </row>
@@ -4587,7 +4561,7 @@
       <c r="U71" t="s">
         <v>180</v>
       </c>
-      <c r="V71" s="2">
+      <c r="V71" s="1">
         <v>46168</v>
       </c>
     </row>
@@ -4631,7 +4605,7 @@
       <c r="U72" t="s">
         <v>180</v>
       </c>
-      <c r="V72" s="2">
+      <c r="V72" s="1">
         <v>46291</v>
       </c>
     </row>
@@ -4675,7 +4649,7 @@
       <c r="U73" t="s">
         <v>180</v>
       </c>
-      <c r="V73" s="2">
+      <c r="V73" s="1">
         <v>46291</v>
       </c>
     </row>
@@ -4719,7 +4693,7 @@
       <c r="U74" t="s">
         <v>180</v>
       </c>
-      <c r="V74" s="2">
+      <c r="V74" s="1">
         <v>46291</v>
       </c>
     </row>
@@ -4766,7 +4740,7 @@
       <c r="U75" t="s">
         <v>28</v>
       </c>
-      <c r="V75" s="2">
+      <c r="V75" s="1">
         <v>46321</v>
       </c>
     </row>
@@ -4816,7 +4790,7 @@
       <c r="U76" t="s">
         <v>180</v>
       </c>
-      <c r="V76" s="2">
+      <c r="V76" s="1">
         <v>46381</v>
       </c>
     </row>
@@ -4866,7 +4840,7 @@
       <c r="U77" t="s">
         <v>180</v>
       </c>
-      <c r="V77" s="2">
+      <c r="V77" s="1">
         <v>46381</v>
       </c>
     </row>
@@ -4916,7 +4890,7 @@
       <c r="U78" t="s">
         <v>28</v>
       </c>
-      <c r="V78" s="2">
+      <c r="V78" s="1">
         <v>46381</v>
       </c>
     </row>
@@ -4966,7 +4940,7 @@
       <c r="U79" t="s">
         <v>28</v>
       </c>
-      <c r="V79" s="2">
+      <c r="V79" s="1">
         <v>46381</v>
       </c>
     </row>
@@ -5016,7 +4990,7 @@
       <c r="U80" t="s">
         <v>28</v>
       </c>
-      <c r="V80" s="2">
+      <c r="V80" s="1">
         <v>46382</v>
       </c>
     </row>
@@ -5060,7 +5034,7 @@
       <c r="U81" t="s">
         <v>28</v>
       </c>
-      <c r="V81" s="2">
+      <c r="V81" s="1">
         <v>46382</v>
       </c>
     </row>
@@ -5113,7 +5087,7 @@
       <c r="U82" t="s">
         <v>180</v>
       </c>
-      <c r="V82" s="2">
+      <c r="V82" s="1">
         <v>46382</v>
       </c>
     </row>
@@ -5157,7 +5131,7 @@
       <c r="U83" t="s">
         <v>28</v>
       </c>
-      <c r="V83" s="2">
+      <c r="V83" s="1">
         <v>46321</v>
       </c>
     </row>
@@ -5201,7 +5175,7 @@
       <c r="U84" t="s">
         <v>28</v>
       </c>
-      <c r="V84" s="2">
+      <c r="V84" s="1">
         <v>46382</v>
       </c>
     </row>
@@ -5342,7 +5316,7 @@
       <c r="U87" t="s">
         <v>28</v>
       </c>
-      <c r="V87" s="2">
+      <c r="V87" s="1">
         <v>46291</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Atualização automática: mta (15/09/2026 14:02)
</commit_message>
<xml_diff>
--- a/Projetos/02_Dados_Tratados/base_mta_tratada.xlsx
+++ b/Projetos/02_Dados_Tratados/base_mta_tratada.xlsx
@@ -566,8 +566,16 @@
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="YYYY-MM-DD HH:MM:SS"/>
   </numFmts>
-  <fonts count="1">
+  <fonts count="2">
     <font>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
       <sz val="11"/>
       <color theme="1"/>
       <name val="Calibri"/>
@@ -583,7 +591,7 @@
       <patternFill patternType="gray125"/>
     </fill>
   </fills>
-  <borders count="1">
+  <borders count="2">
     <border>
       <left/>
       <right/>
@@ -591,12 +599,30 @@
       <bottom/>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin">
+        <color auto="1"/>
+      </left>
+      <right style="thin">
+        <color auto="1"/>
+      </right>
+      <top style="thin">
+        <color auto="1"/>
+      </top>
+      <bottom style="thin">
+        <color auto="1"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="3">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
   </cellXfs>
   <cellStyles count="1">
@@ -896,70 +922,70 @@
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:22">
-      <c r="A1" t="s">
+      <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
-      <c r="B1" t="s">
+      <c r="B1" s="1" t="s">
         <v>1</v>
       </c>
-      <c r="C1" t="s">
+      <c r="C1" s="1" t="s">
         <v>2</v>
       </c>
-      <c r="D1" t="s">
+      <c r="D1" s="1" t="s">
         <v>3</v>
       </c>
-      <c r="E1" t="s">
+      <c r="E1" s="1" t="s">
         <v>4</v>
       </c>
-      <c r="F1" t="s">
+      <c r="F1" s="1" t="s">
         <v>5</v>
       </c>
-      <c r="G1" t="s">
+      <c r="G1" s="1" t="s">
         <v>6</v>
       </c>
-      <c r="H1" t="s">
+      <c r="H1" s="1" t="s">
         <v>7</v>
       </c>
-      <c r="I1" t="s">
+      <c r="I1" s="1" t="s">
         <v>8</v>
       </c>
-      <c r="J1" t="s">
+      <c r="J1" s="1" t="s">
         <v>9</v>
       </c>
-      <c r="K1" t="s">
+      <c r="K1" s="1" t="s">
         <v>10</v>
       </c>
-      <c r="L1" t="s">
+      <c r="L1" s="1" t="s">
         <v>11</v>
       </c>
-      <c r="M1" t="s">
+      <c r="M1" s="1" t="s">
         <v>12</v>
       </c>
-      <c r="N1" t="s">
+      <c r="N1" s="1" t="s">
         <v>13</v>
       </c>
-      <c r="O1" t="s">
+      <c r="O1" s="1" t="s">
         <v>14</v>
       </c>
-      <c r="P1" t="s">
+      <c r="P1" s="1" t="s">
         <v>15</v>
       </c>
-      <c r="Q1" t="s">
+      <c r="Q1" s="1" t="s">
         <v>16</v>
       </c>
-      <c r="R1" t="s">
+      <c r="R1" s="1" t="s">
         <v>17</v>
       </c>
-      <c r="S1" t="s">
+      <c r="S1" s="1" t="s">
         <v>18</v>
       </c>
-      <c r="T1" t="s">
+      <c r="T1" s="1" t="s">
         <v>19</v>
       </c>
-      <c r="U1" t="s">
+      <c r="U1" s="1" t="s">
         <v>20</v>
       </c>
-      <c r="V1" t="s">
+      <c r="V1" s="1" t="s">
         <v>21</v>
       </c>
     </row>
@@ -1015,7 +1041,7 @@
       <c r="U2" t="s">
         <v>180</v>
       </c>
-      <c r="V2" s="1">
+      <c r="V2" s="2">
         <v>46229</v>
       </c>
     </row>
@@ -1062,7 +1088,7 @@
       <c r="U3" t="s">
         <v>28</v>
       </c>
-      <c r="V3" s="1">
+      <c r="V3" s="2">
         <v>46291</v>
       </c>
     </row>
@@ -1109,7 +1135,7 @@
       <c r="U4" t="s">
         <v>28</v>
       </c>
-      <c r="V4" s="1">
+      <c r="V4" s="2">
         <v>46321</v>
       </c>
     </row>
@@ -1156,7 +1182,7 @@
       <c r="U5" t="s">
         <v>28</v>
       </c>
-      <c r="V5" s="1">
+      <c r="V5" s="2">
         <v>46321</v>
       </c>
     </row>
@@ -1206,7 +1232,7 @@
       <c r="U6" t="s">
         <v>28</v>
       </c>
-      <c r="V6" s="1">
+      <c r="V6" s="2">
         <v>46291</v>
       </c>
     </row>
@@ -1232,7 +1258,7 @@
       <c r="G7" t="s">
         <v>42</v>
       </c>
-      <c r="H7" s="1">
+      <c r="H7" s="2">
         <v>46121</v>
       </c>
       <c r="I7" t="s">
@@ -1262,7 +1288,7 @@
       <c r="U7" t="s">
         <v>28</v>
       </c>
-      <c r="V7" s="1">
+      <c r="V7" s="2">
         <v>46138</v>
       </c>
     </row>
@@ -1309,7 +1335,7 @@
       <c r="U8" t="s">
         <v>28</v>
       </c>
-      <c r="V8" s="1">
+      <c r="V8" s="2">
         <v>46291</v>
       </c>
     </row>
@@ -1356,7 +1382,7 @@
       <c r="U9" t="s">
         <v>28</v>
       </c>
-      <c r="V9" s="1">
+      <c r="V9" s="2">
         <v>46291</v>
       </c>
     </row>
@@ -1403,7 +1429,7 @@
       <c r="U10" t="s">
         <v>28</v>
       </c>
-      <c r="V10" s="1">
+      <c r="V10" s="2">
         <v>46291</v>
       </c>
     </row>
@@ -1450,7 +1476,7 @@
       <c r="U11" t="s">
         <v>28</v>
       </c>
-      <c r="V11" s="1">
+      <c r="V11" s="2">
         <v>46291</v>
       </c>
     </row>
@@ -1476,7 +1502,7 @@
       <c r="G12" t="s">
         <v>42</v>
       </c>
-      <c r="H12" s="1">
+      <c r="H12" s="2">
         <v>46079</v>
       </c>
       <c r="I12" t="s">
@@ -1509,7 +1535,7 @@
       <c r="U12" t="s">
         <v>180</v>
       </c>
-      <c r="V12" s="1">
+      <c r="V12" s="2">
         <v>46079</v>
       </c>
     </row>
@@ -1562,7 +1588,7 @@
       <c r="U13" t="s">
         <v>180</v>
       </c>
-      <c r="V13" s="1">
+      <c r="V13" s="2">
         <v>46352</v>
       </c>
     </row>
@@ -1615,7 +1641,7 @@
       <c r="U14" t="s">
         <v>180</v>
       </c>
-      <c r="V14" s="1">
+      <c r="V14" s="2">
         <v>46352</v>
       </c>
     </row>
@@ -1668,7 +1694,7 @@
       <c r="U15" t="s">
         <v>180</v>
       </c>
-      <c r="V15" s="1">
+      <c r="V15" s="2">
         <v>46352</v>
       </c>
     </row>
@@ -1721,7 +1747,7 @@
       <c r="U16" t="s">
         <v>180</v>
       </c>
-      <c r="V16" s="1">
+      <c r="V16" s="2">
         <v>46229</v>
       </c>
     </row>
@@ -1747,7 +1773,7 @@
       <c r="G17" t="s">
         <v>42</v>
       </c>
-      <c r="H17" s="1">
+      <c r="H17" s="2">
         <v>46098</v>
       </c>
       <c r="I17" t="s">
@@ -1780,7 +1806,7 @@
       <c r="U17" t="s">
         <v>180</v>
       </c>
-      <c r="V17" s="1">
+      <c r="V17" s="2">
         <v>46107</v>
       </c>
     </row>
@@ -1806,7 +1832,7 @@
       <c r="G18" t="s">
         <v>42</v>
       </c>
-      <c r="H18" s="1">
+      <c r="H18" s="2">
         <v>46076</v>
       </c>
       <c r="I18" t="s">
@@ -1836,7 +1862,7 @@
       <c r="U18" t="s">
         <v>28</v>
       </c>
-      <c r="V18" s="1">
+      <c r="V18" s="2">
         <v>46079</v>
       </c>
     </row>
@@ -1862,7 +1888,7 @@
       <c r="G19" t="s">
         <v>42</v>
       </c>
-      <c r="H19" s="1">
+      <c r="H19" s="2">
         <v>46076</v>
       </c>
       <c r="I19" t="s">
@@ -1892,7 +1918,7 @@
       <c r="U19" t="s">
         <v>28</v>
       </c>
-      <c r="V19" s="1">
+      <c r="V19" s="2">
         <v>46079</v>
       </c>
     </row>
@@ -1939,7 +1965,7 @@
       <c r="U20" t="s">
         <v>28</v>
       </c>
-      <c r="V20" s="1">
+      <c r="V20" s="2">
         <v>46321</v>
       </c>
     </row>
@@ -1986,7 +2012,7 @@
       <c r="U21" t="s">
         <v>28</v>
       </c>
-      <c r="V21" s="1">
+      <c r="V21" s="2">
         <v>46321</v>
       </c>
     </row>
@@ -2033,7 +2059,7 @@
       <c r="U22" t="s">
         <v>28</v>
       </c>
-      <c r="V22" s="1">
+      <c r="V22" s="2">
         <v>46321</v>
       </c>
     </row>
@@ -2080,7 +2106,7 @@
       <c r="U23" t="s">
         <v>28</v>
       </c>
-      <c r="V23" s="1">
+      <c r="V23" s="2">
         <v>46321</v>
       </c>
     </row>
@@ -2106,7 +2132,7 @@
       <c r="G24" t="s">
         <v>42</v>
       </c>
-      <c r="H24" s="1">
+      <c r="H24" s="2">
         <v>46119</v>
       </c>
       <c r="I24" t="s">
@@ -2139,7 +2165,7 @@
       <c r="U24" t="s">
         <v>180</v>
       </c>
-      <c r="V24" s="1">
+      <c r="V24" s="2">
         <v>46138</v>
       </c>
     </row>
@@ -2165,7 +2191,7 @@
       <c r="G25" t="s">
         <v>42</v>
       </c>
-      <c r="H25" s="1">
+      <c r="H25" s="2">
         <v>46121</v>
       </c>
       <c r="I25" t="s">
@@ -2195,7 +2221,7 @@
       <c r="U25" t="s">
         <v>28</v>
       </c>
-      <c r="V25" s="1">
+      <c r="V25" s="2">
         <v>46138</v>
       </c>
     </row>
@@ -2221,7 +2247,7 @@
       <c r="G26" t="s">
         <v>42</v>
       </c>
-      <c r="H26" s="1">
+      <c r="H26" s="2">
         <v>46076</v>
       </c>
       <c r="I26" t="s">
@@ -2251,7 +2277,7 @@
       <c r="U26" t="s">
         <v>28</v>
       </c>
-      <c r="V26" s="1">
+      <c r="V26" s="2">
         <v>46079</v>
       </c>
     </row>
@@ -2304,7 +2330,7 @@
       <c r="U27" t="s">
         <v>180</v>
       </c>
-      <c r="V27" s="1">
+      <c r="V27" s="2">
         <v>46291</v>
       </c>
     </row>
@@ -2330,7 +2356,7 @@
       <c r="G28" t="s">
         <v>42</v>
       </c>
-      <c r="H28" s="1">
+      <c r="H28" s="2">
         <v>46199</v>
       </c>
       <c r="I28" t="s">
@@ -2363,7 +2389,7 @@
       <c r="U28" t="s">
         <v>180</v>
       </c>
-      <c r="V28" s="1">
+      <c r="V28" s="2">
         <v>46199</v>
       </c>
     </row>
@@ -2389,7 +2415,7 @@
       <c r="G29" t="s">
         <v>42</v>
       </c>
-      <c r="H29" s="1">
+      <c r="H29" s="2">
         <v>46199</v>
       </c>
       <c r="I29" t="s">
@@ -2422,7 +2448,7 @@
       <c r="U29" t="s">
         <v>180</v>
       </c>
-      <c r="V29" s="1">
+      <c r="V29" s="2">
         <v>46199</v>
       </c>
     </row>
@@ -2448,7 +2474,7 @@
       <c r="G30" t="s">
         <v>42</v>
       </c>
-      <c r="H30" s="1">
+      <c r="H30" s="2">
         <v>46199</v>
       </c>
       <c r="I30" t="s">
@@ -2481,7 +2507,7 @@
       <c r="U30" t="s">
         <v>180</v>
       </c>
-      <c r="V30" s="1">
+      <c r="V30" s="2">
         <v>46199</v>
       </c>
     </row>
@@ -2507,7 +2533,7 @@
       <c r="G31" t="s">
         <v>42</v>
       </c>
-      <c r="H31" s="1">
+      <c r="H31" s="2">
         <v>46199</v>
       </c>
       <c r="I31" t="s">
@@ -2540,7 +2566,7 @@
       <c r="U31" t="s">
         <v>180</v>
       </c>
-      <c r="V31" s="1">
+      <c r="V31" s="2">
         <v>46199</v>
       </c>
     </row>
@@ -2590,7 +2616,7 @@
       <c r="U32" t="s">
         <v>180</v>
       </c>
-      <c r="V32" s="1">
+      <c r="V32" s="2">
         <v>46291</v>
       </c>
     </row>
@@ -2616,7 +2642,7 @@
       <c r="G33" t="s">
         <v>42</v>
       </c>
-      <c r="H33" s="1">
+      <c r="H33" s="2">
         <v>46191</v>
       </c>
       <c r="I33" t="s">
@@ -2649,7 +2675,7 @@
       <c r="U33" t="s">
         <v>180</v>
       </c>
-      <c r="V33" s="1">
+      <c r="V33" s="2">
         <v>46199</v>
       </c>
     </row>
@@ -2675,7 +2701,7 @@
       <c r="G34" t="s">
         <v>42</v>
       </c>
-      <c r="H34" s="1">
+      <c r="H34" s="2">
         <v>46119</v>
       </c>
       <c r="I34" t="s">
@@ -2705,7 +2731,7 @@
       <c r="U34" t="s">
         <v>180</v>
       </c>
-      <c r="V34" s="1">
+      <c r="V34" s="2">
         <v>46138</v>
       </c>
     </row>
@@ -2731,7 +2757,7 @@
       <c r="G35" t="s">
         <v>42</v>
       </c>
-      <c r="H35" s="1">
+      <c r="H35" s="2">
         <v>46213</v>
       </c>
       <c r="I35" t="s">
@@ -2761,7 +2787,7 @@
       <c r="U35" t="s">
         <v>28</v>
       </c>
-      <c r="V35" s="1">
+      <c r="V35" s="2">
         <v>46229</v>
       </c>
     </row>
@@ -2787,7 +2813,7 @@
       <c r="G36" t="s">
         <v>42</v>
       </c>
-      <c r="H36" s="1">
+      <c r="H36" s="2">
         <v>46175</v>
       </c>
       <c r="I36" t="s">
@@ -2817,7 +2843,7 @@
       <c r="U36" t="s">
         <v>28</v>
       </c>
-      <c r="V36" s="1">
+      <c r="V36" s="2">
         <v>46199</v>
       </c>
     </row>
@@ -2843,7 +2869,7 @@
       <c r="G37" t="s">
         <v>42</v>
       </c>
-      <c r="H37" s="1">
+      <c r="H37" s="2">
         <v>46213</v>
       </c>
       <c r="I37" t="s">
@@ -2873,7 +2899,7 @@
       <c r="U37" t="s">
         <v>28</v>
       </c>
-      <c r="V37" s="1">
+      <c r="V37" s="2">
         <v>46229</v>
       </c>
     </row>
@@ -2899,7 +2925,7 @@
       <c r="G38" t="s">
         <v>42</v>
       </c>
-      <c r="H38" s="1">
+      <c r="H38" s="2">
         <v>46199</v>
       </c>
       <c r="I38" t="s">
@@ -2929,7 +2955,7 @@
       <c r="U38" t="s">
         <v>28</v>
       </c>
-      <c r="V38" s="1">
+      <c r="V38" s="2">
         <v>46199</v>
       </c>
     </row>
@@ -2955,7 +2981,7 @@
       <c r="G39" t="s">
         <v>42</v>
       </c>
-      <c r="H39" s="1">
+      <c r="H39" s="2">
         <v>46199</v>
       </c>
       <c r="I39" t="s">
@@ -2985,7 +3011,7 @@
       <c r="U39" t="s">
         <v>28</v>
       </c>
-      <c r="V39" s="1">
+      <c r="V39" s="2">
         <v>46199</v>
       </c>
     </row>
@@ -3011,7 +3037,7 @@
       <c r="G40" t="s">
         <v>42</v>
       </c>
-      <c r="H40" s="1">
+      <c r="H40" s="2">
         <v>46204</v>
       </c>
       <c r="I40" t="s">
@@ -3041,7 +3067,7 @@
       <c r="U40" t="s">
         <v>28</v>
       </c>
-      <c r="V40" s="1">
+      <c r="V40" s="2">
         <v>46229</v>
       </c>
     </row>
@@ -3067,7 +3093,7 @@
       <c r="G41" t="s">
         <v>42</v>
       </c>
-      <c r="H41" s="1">
+      <c r="H41" s="2">
         <v>46244</v>
       </c>
       <c r="I41" t="s">
@@ -3097,7 +3123,7 @@
       <c r="U41" t="s">
         <v>28</v>
       </c>
-      <c r="V41" s="1">
+      <c r="V41" s="2">
         <v>46199</v>
       </c>
     </row>
@@ -3141,7 +3167,7 @@
       <c r="U42" t="s">
         <v>28</v>
       </c>
-      <c r="V42" s="1">
+      <c r="V42" s="2">
         <v>46260</v>
       </c>
     </row>
@@ -3167,7 +3193,7 @@
       <c r="G43" t="s">
         <v>42</v>
       </c>
-      <c r="H43" s="1">
+      <c r="H43" s="2">
         <v>46191</v>
       </c>
       <c r="I43" t="s">
@@ -3197,7 +3223,7 @@
       <c r="U43" t="s">
         <v>28</v>
       </c>
-      <c r="V43" s="1">
+      <c r="V43" s="2">
         <v>46199</v>
       </c>
     </row>
@@ -3223,7 +3249,7 @@
       <c r="G44" t="s">
         <v>42</v>
       </c>
-      <c r="H44" s="1">
+      <c r="H44" s="2">
         <v>46191</v>
       </c>
       <c r="I44" t="s">
@@ -3253,7 +3279,7 @@
       <c r="U44" t="s">
         <v>28</v>
       </c>
-      <c r="V44" s="1">
+      <c r="V44" s="2">
         <v>46199</v>
       </c>
     </row>
@@ -3279,7 +3305,7 @@
       <c r="G45" t="s">
         <v>42</v>
       </c>
-      <c r="H45" s="1">
+      <c r="H45" s="2">
         <v>46213</v>
       </c>
       <c r="I45" t="s">
@@ -3312,7 +3338,7 @@
       <c r="U45" t="s">
         <v>180</v>
       </c>
-      <c r="V45" s="1">
+      <c r="V45" s="2">
         <v>46229</v>
       </c>
     </row>
@@ -3338,7 +3364,7 @@
       <c r="G46" t="s">
         <v>42</v>
       </c>
-      <c r="H46" s="1">
+      <c r="H46" s="2">
         <v>46210</v>
       </c>
       <c r="I46" t="s">
@@ -3368,7 +3394,7 @@
       <c r="U46" t="s">
         <v>180</v>
       </c>
-      <c r="V46" s="1">
+      <c r="V46" s="2">
         <v>46229</v>
       </c>
     </row>
@@ -3415,7 +3441,7 @@
       <c r="U47" t="s">
         <v>28</v>
       </c>
-      <c r="V47" s="1">
+      <c r="V47" s="2">
         <v>46321</v>
       </c>
     </row>
@@ -3468,7 +3494,7 @@
       <c r="U48" t="s">
         <v>180</v>
       </c>
-      <c r="V48" s="1">
+      <c r="V48" s="2">
         <v>46291</v>
       </c>
     </row>
@@ -3494,7 +3520,7 @@
       <c r="G49" t="s">
         <v>42</v>
       </c>
-      <c r="H49" s="1">
+      <c r="H49" s="2">
         <v>46176</v>
       </c>
       <c r="I49" t="s">
@@ -3527,7 +3553,7 @@
       <c r="U49" t="s">
         <v>180</v>
       </c>
-      <c r="V49" s="1">
+      <c r="V49" s="2">
         <v>46199</v>
       </c>
     </row>
@@ -3580,7 +3606,7 @@
       <c r="U50" t="s">
         <v>180</v>
       </c>
-      <c r="V50" s="1">
+      <c r="V50" s="2">
         <v>46260</v>
       </c>
     </row>
@@ -3633,7 +3659,7 @@
       <c r="U51" t="s">
         <v>180</v>
       </c>
-      <c r="V51" s="1">
+      <c r="V51" s="2">
         <v>46291</v>
       </c>
     </row>
@@ -3683,7 +3709,7 @@
       <c r="U52" t="s">
         <v>180</v>
       </c>
-      <c r="V52" s="1">
+      <c r="V52" s="2">
         <v>46321</v>
       </c>
     </row>
@@ -3709,7 +3735,7 @@
       <c r="G53" t="s">
         <v>42</v>
       </c>
-      <c r="H53" s="1">
+      <c r="H53" s="2">
         <v>46227</v>
       </c>
       <c r="I53" t="s">
@@ -3739,7 +3765,7 @@
       <c r="U53" t="s">
         <v>180</v>
       </c>
-      <c r="V53" s="1">
+      <c r="V53" s="2">
         <v>46229</v>
       </c>
     </row>
@@ -3792,7 +3818,7 @@
       <c r="U54" t="s">
         <v>180</v>
       </c>
-      <c r="V54" s="1">
+      <c r="V54" s="2">
         <v>46352</v>
       </c>
     </row>
@@ -3845,7 +3871,7 @@
       <c r="U55" t="s">
         <v>180</v>
       </c>
-      <c r="V55" s="1">
+      <c r="V55" s="2">
         <v>46321</v>
       </c>
     </row>
@@ -3895,7 +3921,7 @@
       <c r="U56" t="s">
         <v>180</v>
       </c>
-      <c r="V56" s="1">
+      <c r="V56" s="2">
         <v>46321</v>
       </c>
     </row>
@@ -3939,7 +3965,7 @@
       <c r="U57" t="s">
         <v>180</v>
       </c>
-      <c r="V57" s="1">
+      <c r="V57" s="2">
         <v>46049</v>
       </c>
     </row>
@@ -4065,7 +4091,7 @@
       <c r="U60" t="s">
         <v>180</v>
       </c>
-      <c r="V60" s="1">
+      <c r="V60" s="2">
         <v>46107</v>
       </c>
     </row>
@@ -4109,7 +4135,7 @@
       <c r="U61" t="s">
         <v>180</v>
       </c>
-      <c r="V61" s="1">
+      <c r="V61" s="2">
         <v>46107</v>
       </c>
     </row>
@@ -4153,7 +4179,7 @@
       <c r="U62" t="s">
         <v>180</v>
       </c>
-      <c r="V62" s="1">
+      <c r="V62" s="2">
         <v>46107</v>
       </c>
     </row>
@@ -4197,7 +4223,7 @@
       <c r="U63" t="s">
         <v>180</v>
       </c>
-      <c r="V63" s="1">
+      <c r="V63" s="2">
         <v>46107</v>
       </c>
     </row>
@@ -4241,7 +4267,7 @@
       <c r="U64" t="s">
         <v>180</v>
       </c>
-      <c r="V64" s="1">
+      <c r="V64" s="2">
         <v>46107</v>
       </c>
     </row>
@@ -4285,7 +4311,7 @@
       <c r="U65" t="s">
         <v>180</v>
       </c>
-      <c r="V65" s="1">
+      <c r="V65" s="2">
         <v>46107</v>
       </c>
     </row>
@@ -4329,7 +4355,7 @@
       <c r="U66" t="s">
         <v>28</v>
       </c>
-      <c r="V66" s="1">
+      <c r="V66" s="2">
         <v>46168</v>
       </c>
     </row>
@@ -4376,7 +4402,7 @@
       <c r="U67" t="s">
         <v>28</v>
       </c>
-      <c r="V67" s="1">
+      <c r="V67" s="2">
         <v>46291</v>
       </c>
     </row>
@@ -4429,7 +4455,7 @@
       <c r="U68" t="s">
         <v>180</v>
       </c>
-      <c r="V68" s="1">
+      <c r="V68" s="2">
         <v>46229</v>
       </c>
     </row>
@@ -4473,7 +4499,7 @@
       <c r="U69" t="s">
         <v>28</v>
       </c>
-      <c r="V69" s="1">
+      <c r="V69" s="2">
         <v>46260</v>
       </c>
     </row>
@@ -4517,7 +4543,7 @@
       <c r="U70" t="s">
         <v>180</v>
       </c>
-      <c r="V70" s="1">
+      <c r="V70" s="2">
         <v>46291</v>
       </c>
     </row>
@@ -4561,7 +4587,7 @@
       <c r="U71" t="s">
         <v>180</v>
       </c>
-      <c r="V71" s="1">
+      <c r="V71" s="2">
         <v>46168</v>
       </c>
     </row>
@@ -4605,7 +4631,7 @@
       <c r="U72" t="s">
         <v>180</v>
       </c>
-      <c r="V72" s="1">
+      <c r="V72" s="2">
         <v>46291</v>
       </c>
     </row>
@@ -4649,7 +4675,7 @@
       <c r="U73" t="s">
         <v>180</v>
       </c>
-      <c r="V73" s="1">
+      <c r="V73" s="2">
         <v>46291</v>
       </c>
     </row>
@@ -4693,7 +4719,7 @@
       <c r="U74" t="s">
         <v>180</v>
       </c>
-      <c r="V74" s="1">
+      <c r="V74" s="2">
         <v>46291</v>
       </c>
     </row>
@@ -4740,7 +4766,7 @@
       <c r="U75" t="s">
         <v>28</v>
       </c>
-      <c r="V75" s="1">
+      <c r="V75" s="2">
         <v>46321</v>
       </c>
     </row>
@@ -4790,7 +4816,7 @@
       <c r="U76" t="s">
         <v>180</v>
       </c>
-      <c r="V76" s="1">
+      <c r="V76" s="2">
         <v>46381</v>
       </c>
     </row>
@@ -4840,7 +4866,7 @@
       <c r="U77" t="s">
         <v>180</v>
       </c>
-      <c r="V77" s="1">
+      <c r="V77" s="2">
         <v>46381</v>
       </c>
     </row>
@@ -4890,7 +4916,7 @@
       <c r="U78" t="s">
         <v>28</v>
       </c>
-      <c r="V78" s="1">
+      <c r="V78" s="2">
         <v>46381</v>
       </c>
     </row>
@@ -4940,7 +4966,7 @@
       <c r="U79" t="s">
         <v>28</v>
       </c>
-      <c r="V79" s="1">
+      <c r="V79" s="2">
         <v>46381</v>
       </c>
     </row>
@@ -4990,7 +5016,7 @@
       <c r="U80" t="s">
         <v>28</v>
       </c>
-      <c r="V80" s="1">
+      <c r="V80" s="2">
         <v>46382</v>
       </c>
     </row>
@@ -5034,7 +5060,7 @@
       <c r="U81" t="s">
         <v>28</v>
       </c>
-      <c r="V81" s="1">
+      <c r="V81" s="2">
         <v>46382</v>
       </c>
     </row>
@@ -5087,7 +5113,7 @@
       <c r="U82" t="s">
         <v>180</v>
       </c>
-      <c r="V82" s="1">
+      <c r="V82" s="2">
         <v>46382</v>
       </c>
     </row>
@@ -5131,7 +5157,7 @@
       <c r="U83" t="s">
         <v>28</v>
       </c>
-      <c r="V83" s="1">
+      <c r="V83" s="2">
         <v>46321</v>
       </c>
     </row>
@@ -5175,7 +5201,7 @@
       <c r="U84" t="s">
         <v>28</v>
       </c>
-      <c r="V84" s="1">
+      <c r="V84" s="2">
         <v>46382</v>
       </c>
     </row>
@@ -5316,7 +5342,7 @@
       <c r="U87" t="s">
         <v>28</v>
       </c>
-      <c r="V87" s="1">
+      <c r="V87" s="2">
         <v>46291</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Atualização automática: mta (16/09/2026 12:25)
</commit_message>
<xml_diff>
--- a/Projetos/02_Dados_Tratados/base_mta_tratada.xlsx
+++ b/Projetos/02_Dados_Tratados/base_mta_tratada.xlsx
@@ -566,16 +566,8 @@
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="YYYY-MM-DD HH:MM:SS"/>
   </numFmts>
-  <fonts count="2">
+  <fonts count="1">
     <font>
-      <sz val="11"/>
-      <color theme="1"/>
-      <name val="Calibri"/>
-      <family val="2"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <b/>
       <sz val="11"/>
       <color theme="1"/>
       <name val="Calibri"/>
@@ -591,7 +583,7 @@
       <patternFill patternType="gray125"/>
     </fill>
   </fills>
-  <borders count="2">
+  <borders count="1">
     <border>
       <left/>
       <right/>
@@ -599,30 +591,12 @@
       <bottom/>
       <diagonal/>
     </border>
-    <border>
-      <left style="thin">
-        <color auto="1"/>
-      </left>
-      <right style="thin">
-        <color auto="1"/>
-      </right>
-      <top style="thin">
-        <color auto="1"/>
-      </top>
-      <bottom style="thin">
-        <color auto="1"/>
-      </bottom>
-      <diagonal/>
-    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="3">
+  <cellXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top"/>
-    </xf>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
   </cellXfs>
   <cellStyles count="1">
@@ -922,70 +896,70 @@
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:22">
-      <c r="A1" s="1" t="s">
+      <c r="A1" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="1" t="s">
+      <c r="B1" t="s">
         <v>1</v>
       </c>
-      <c r="C1" s="1" t="s">
+      <c r="C1" t="s">
         <v>2</v>
       </c>
-      <c r="D1" s="1" t="s">
+      <c r="D1" t="s">
         <v>3</v>
       </c>
-      <c r="E1" s="1" t="s">
+      <c r="E1" t="s">
         <v>4</v>
       </c>
-      <c r="F1" s="1" t="s">
+      <c r="F1" t="s">
         <v>5</v>
       </c>
-      <c r="G1" s="1" t="s">
+      <c r="G1" t="s">
         <v>6</v>
       </c>
-      <c r="H1" s="1" t="s">
+      <c r="H1" t="s">
         <v>7</v>
       </c>
-      <c r="I1" s="1" t="s">
+      <c r="I1" t="s">
         <v>8</v>
       </c>
-      <c r="J1" s="1" t="s">
+      <c r="J1" t="s">
         <v>9</v>
       </c>
-      <c r="K1" s="1" t="s">
+      <c r="K1" t="s">
         <v>10</v>
       </c>
-      <c r="L1" s="1" t="s">
+      <c r="L1" t="s">
         <v>11</v>
       </c>
-      <c r="M1" s="1" t="s">
+      <c r="M1" t="s">
         <v>12</v>
       </c>
-      <c r="N1" s="1" t="s">
+      <c r="N1" t="s">
         <v>13</v>
       </c>
-      <c r="O1" s="1" t="s">
+      <c r="O1" t="s">
         <v>14</v>
       </c>
-      <c r="P1" s="1" t="s">
+      <c r="P1" t="s">
         <v>15</v>
       </c>
-      <c r="Q1" s="1" t="s">
+      <c r="Q1" t="s">
         <v>16</v>
       </c>
-      <c r="R1" s="1" t="s">
+      <c r="R1" t="s">
         <v>17</v>
       </c>
-      <c r="S1" s="1" t="s">
+      <c r="S1" t="s">
         <v>18</v>
       </c>
-      <c r="T1" s="1" t="s">
+      <c r="T1" t="s">
         <v>19</v>
       </c>
-      <c r="U1" s="1" t="s">
+      <c r="U1" t="s">
         <v>20</v>
       </c>
-      <c r="V1" s="1" t="s">
+      <c r="V1" t="s">
         <v>21</v>
       </c>
     </row>
@@ -1041,7 +1015,7 @@
       <c r="U2" t="s">
         <v>180</v>
       </c>
-      <c r="V2" s="2">
+      <c r="V2" s="1">
         <v>46229</v>
       </c>
     </row>
@@ -1088,7 +1062,7 @@
       <c r="U3" t="s">
         <v>28</v>
       </c>
-      <c r="V3" s="2">
+      <c r="V3" s="1">
         <v>46291</v>
       </c>
     </row>
@@ -1135,7 +1109,7 @@
       <c r="U4" t="s">
         <v>28</v>
       </c>
-      <c r="V4" s="2">
+      <c r="V4" s="1">
         <v>46321</v>
       </c>
     </row>
@@ -1182,7 +1156,7 @@
       <c r="U5" t="s">
         <v>28</v>
       </c>
-      <c r="V5" s="2">
+      <c r="V5" s="1">
         <v>46321</v>
       </c>
     </row>
@@ -1232,7 +1206,7 @@
       <c r="U6" t="s">
         <v>28</v>
       </c>
-      <c r="V6" s="2">
+      <c r="V6" s="1">
         <v>46291</v>
       </c>
     </row>
@@ -1258,7 +1232,7 @@
       <c r="G7" t="s">
         <v>42</v>
       </c>
-      <c r="H7" s="2">
+      <c r="H7" s="1">
         <v>46121</v>
       </c>
       <c r="I7" t="s">
@@ -1288,7 +1262,7 @@
       <c r="U7" t="s">
         <v>28</v>
       </c>
-      <c r="V7" s="2">
+      <c r="V7" s="1">
         <v>46138</v>
       </c>
     </row>
@@ -1335,7 +1309,7 @@
       <c r="U8" t="s">
         <v>28</v>
       </c>
-      <c r="V8" s="2">
+      <c r="V8" s="1">
         <v>46291</v>
       </c>
     </row>
@@ -1382,7 +1356,7 @@
       <c r="U9" t="s">
         <v>28</v>
       </c>
-      <c r="V9" s="2">
+      <c r="V9" s="1">
         <v>46291</v>
       </c>
     </row>
@@ -1429,7 +1403,7 @@
       <c r="U10" t="s">
         <v>28</v>
       </c>
-      <c r="V10" s="2">
+      <c r="V10" s="1">
         <v>46291</v>
       </c>
     </row>
@@ -1476,7 +1450,7 @@
       <c r="U11" t="s">
         <v>28</v>
       </c>
-      <c r="V11" s="2">
+      <c r="V11" s="1">
         <v>46291</v>
       </c>
     </row>
@@ -1502,7 +1476,7 @@
       <c r="G12" t="s">
         <v>42</v>
       </c>
-      <c r="H12" s="2">
+      <c r="H12" s="1">
         <v>46079</v>
       </c>
       <c r="I12" t="s">
@@ -1535,7 +1509,7 @@
       <c r="U12" t="s">
         <v>180</v>
       </c>
-      <c r="V12" s="2">
+      <c r="V12" s="1">
         <v>46079</v>
       </c>
     </row>
@@ -1588,7 +1562,7 @@
       <c r="U13" t="s">
         <v>180</v>
       </c>
-      <c r="V13" s="2">
+      <c r="V13" s="1">
         <v>46352</v>
       </c>
     </row>
@@ -1641,7 +1615,7 @@
       <c r="U14" t="s">
         <v>180</v>
       </c>
-      <c r="V14" s="2">
+      <c r="V14" s="1">
         <v>46352</v>
       </c>
     </row>
@@ -1694,7 +1668,7 @@
       <c r="U15" t="s">
         <v>180</v>
       </c>
-      <c r="V15" s="2">
+      <c r="V15" s="1">
         <v>46352</v>
       </c>
     </row>
@@ -1747,7 +1721,7 @@
       <c r="U16" t="s">
         <v>180</v>
       </c>
-      <c r="V16" s="2">
+      <c r="V16" s="1">
         <v>46229</v>
       </c>
     </row>
@@ -1773,7 +1747,7 @@
       <c r="G17" t="s">
         <v>42</v>
       </c>
-      <c r="H17" s="2">
+      <c r="H17" s="1">
         <v>46098</v>
       </c>
       <c r="I17" t="s">
@@ -1806,7 +1780,7 @@
       <c r="U17" t="s">
         <v>180</v>
       </c>
-      <c r="V17" s="2">
+      <c r="V17" s="1">
         <v>46107</v>
       </c>
     </row>
@@ -1832,7 +1806,7 @@
       <c r="G18" t="s">
         <v>42</v>
       </c>
-      <c r="H18" s="2">
+      <c r="H18" s="1">
         <v>46076</v>
       </c>
       <c r="I18" t="s">
@@ -1862,7 +1836,7 @@
       <c r="U18" t="s">
         <v>28</v>
       </c>
-      <c r="V18" s="2">
+      <c r="V18" s="1">
         <v>46079</v>
       </c>
     </row>
@@ -1888,7 +1862,7 @@
       <c r="G19" t="s">
         <v>42</v>
       </c>
-      <c r="H19" s="2">
+      <c r="H19" s="1">
         <v>46076</v>
       </c>
       <c r="I19" t="s">
@@ -1918,7 +1892,7 @@
       <c r="U19" t="s">
         <v>28</v>
       </c>
-      <c r="V19" s="2">
+      <c r="V19" s="1">
         <v>46079</v>
       </c>
     </row>
@@ -1965,7 +1939,7 @@
       <c r="U20" t="s">
         <v>28</v>
       </c>
-      <c r="V20" s="2">
+      <c r="V20" s="1">
         <v>46321</v>
       </c>
     </row>
@@ -2012,7 +1986,7 @@
       <c r="U21" t="s">
         <v>28</v>
       </c>
-      <c r="V21" s="2">
+      <c r="V21" s="1">
         <v>46321</v>
       </c>
     </row>
@@ -2059,7 +2033,7 @@
       <c r="U22" t="s">
         <v>28</v>
       </c>
-      <c r="V22" s="2">
+      <c r="V22" s="1">
         <v>46321</v>
       </c>
     </row>
@@ -2106,7 +2080,7 @@
       <c r="U23" t="s">
         <v>28</v>
       </c>
-      <c r="V23" s="2">
+      <c r="V23" s="1">
         <v>46321</v>
       </c>
     </row>
@@ -2132,7 +2106,7 @@
       <c r="G24" t="s">
         <v>42</v>
       </c>
-      <c r="H24" s="2">
+      <c r="H24" s="1">
         <v>46119</v>
       </c>
       <c r="I24" t="s">
@@ -2165,7 +2139,7 @@
       <c r="U24" t="s">
         <v>180</v>
       </c>
-      <c r="V24" s="2">
+      <c r="V24" s="1">
         <v>46138</v>
       </c>
     </row>
@@ -2191,7 +2165,7 @@
       <c r="G25" t="s">
         <v>42</v>
       </c>
-      <c r="H25" s="2">
+      <c r="H25" s="1">
         <v>46121</v>
       </c>
       <c r="I25" t="s">
@@ -2221,7 +2195,7 @@
       <c r="U25" t="s">
         <v>28</v>
       </c>
-      <c r="V25" s="2">
+      <c r="V25" s="1">
         <v>46138</v>
       </c>
     </row>
@@ -2247,7 +2221,7 @@
       <c r="G26" t="s">
         <v>42</v>
       </c>
-      <c r="H26" s="2">
+      <c r="H26" s="1">
         <v>46076</v>
       </c>
       <c r="I26" t="s">
@@ -2277,7 +2251,7 @@
       <c r="U26" t="s">
         <v>28</v>
       </c>
-      <c r="V26" s="2">
+      <c r="V26" s="1">
         <v>46079</v>
       </c>
     </row>
@@ -2330,7 +2304,7 @@
       <c r="U27" t="s">
         <v>180</v>
       </c>
-      <c r="V27" s="2">
+      <c r="V27" s="1">
         <v>46291</v>
       </c>
     </row>
@@ -2356,7 +2330,7 @@
       <c r="G28" t="s">
         <v>42</v>
       </c>
-      <c r="H28" s="2">
+      <c r="H28" s="1">
         <v>46199</v>
       </c>
       <c r="I28" t="s">
@@ -2389,7 +2363,7 @@
       <c r="U28" t="s">
         <v>180</v>
       </c>
-      <c r="V28" s="2">
+      <c r="V28" s="1">
         <v>46199</v>
       </c>
     </row>
@@ -2415,7 +2389,7 @@
       <c r="G29" t="s">
         <v>42</v>
       </c>
-      <c r="H29" s="2">
+      <c r="H29" s="1">
         <v>46199</v>
       </c>
       <c r="I29" t="s">
@@ -2448,7 +2422,7 @@
       <c r="U29" t="s">
         <v>180</v>
       </c>
-      <c r="V29" s="2">
+      <c r="V29" s="1">
         <v>46199</v>
       </c>
     </row>
@@ -2474,7 +2448,7 @@
       <c r="G30" t="s">
         <v>42</v>
       </c>
-      <c r="H30" s="2">
+      <c r="H30" s="1">
         <v>46199</v>
       </c>
       <c r="I30" t="s">
@@ -2507,7 +2481,7 @@
       <c r="U30" t="s">
         <v>180</v>
       </c>
-      <c r="V30" s="2">
+      <c r="V30" s="1">
         <v>46199</v>
       </c>
     </row>
@@ -2533,7 +2507,7 @@
       <c r="G31" t="s">
         <v>42</v>
       </c>
-      <c r="H31" s="2">
+      <c r="H31" s="1">
         <v>46199</v>
       </c>
       <c r="I31" t="s">
@@ -2566,7 +2540,7 @@
       <c r="U31" t="s">
         <v>180</v>
       </c>
-      <c r="V31" s="2">
+      <c r="V31" s="1">
         <v>46199</v>
       </c>
     </row>
@@ -2616,7 +2590,7 @@
       <c r="U32" t="s">
         <v>180</v>
       </c>
-      <c r="V32" s="2">
+      <c r="V32" s="1">
         <v>46291</v>
       </c>
     </row>
@@ -2642,7 +2616,7 @@
       <c r="G33" t="s">
         <v>42</v>
       </c>
-      <c r="H33" s="2">
+      <c r="H33" s="1">
         <v>46191</v>
       </c>
       <c r="I33" t="s">
@@ -2675,7 +2649,7 @@
       <c r="U33" t="s">
         <v>180</v>
       </c>
-      <c r="V33" s="2">
+      <c r="V33" s="1">
         <v>46199</v>
       </c>
     </row>
@@ -2701,7 +2675,7 @@
       <c r="G34" t="s">
         <v>42</v>
       </c>
-      <c r="H34" s="2">
+      <c r="H34" s="1">
         <v>46119</v>
       </c>
       <c r="I34" t="s">
@@ -2731,7 +2705,7 @@
       <c r="U34" t="s">
         <v>180</v>
       </c>
-      <c r="V34" s="2">
+      <c r="V34" s="1">
         <v>46138</v>
       </c>
     </row>
@@ -2757,7 +2731,7 @@
       <c r="G35" t="s">
         <v>42</v>
       </c>
-      <c r="H35" s="2">
+      <c r="H35" s="1">
         <v>46213</v>
       </c>
       <c r="I35" t="s">
@@ -2787,7 +2761,7 @@
       <c r="U35" t="s">
         <v>28</v>
       </c>
-      <c r="V35" s="2">
+      <c r="V35" s="1">
         <v>46229</v>
       </c>
     </row>
@@ -2813,7 +2787,7 @@
       <c r="G36" t="s">
         <v>42</v>
       </c>
-      <c r="H36" s="2">
+      <c r="H36" s="1">
         <v>46175</v>
       </c>
       <c r="I36" t="s">
@@ -2843,7 +2817,7 @@
       <c r="U36" t="s">
         <v>28</v>
       </c>
-      <c r="V36" s="2">
+      <c r="V36" s="1">
         <v>46199</v>
       </c>
     </row>
@@ -2869,7 +2843,7 @@
       <c r="G37" t="s">
         <v>42</v>
       </c>
-      <c r="H37" s="2">
+      <c r="H37" s="1">
         <v>46213</v>
       </c>
       <c r="I37" t="s">
@@ -2899,7 +2873,7 @@
       <c r="U37" t="s">
         <v>28</v>
       </c>
-      <c r="V37" s="2">
+      <c r="V37" s="1">
         <v>46229</v>
       </c>
     </row>
@@ -2925,7 +2899,7 @@
       <c r="G38" t="s">
         <v>42</v>
       </c>
-      <c r="H38" s="2">
+      <c r="H38" s="1">
         <v>46199</v>
       </c>
       <c r="I38" t="s">
@@ -2955,7 +2929,7 @@
       <c r="U38" t="s">
         <v>28</v>
       </c>
-      <c r="V38" s="2">
+      <c r="V38" s="1">
         <v>46199</v>
       </c>
     </row>
@@ -2981,7 +2955,7 @@
       <c r="G39" t="s">
         <v>42</v>
       </c>
-      <c r="H39" s="2">
+      <c r="H39" s="1">
         <v>46199</v>
       </c>
       <c r="I39" t="s">
@@ -3011,7 +2985,7 @@
       <c r="U39" t="s">
         <v>28</v>
       </c>
-      <c r="V39" s="2">
+      <c r="V39" s="1">
         <v>46199</v>
       </c>
     </row>
@@ -3037,7 +3011,7 @@
       <c r="G40" t="s">
         <v>42</v>
       </c>
-      <c r="H40" s="2">
+      <c r="H40" s="1">
         <v>46204</v>
       </c>
       <c r="I40" t="s">
@@ -3067,7 +3041,7 @@
       <c r="U40" t="s">
         <v>28</v>
       </c>
-      <c r="V40" s="2">
+      <c r="V40" s="1">
         <v>46229</v>
       </c>
     </row>
@@ -3093,7 +3067,7 @@
       <c r="G41" t="s">
         <v>42</v>
       </c>
-      <c r="H41" s="2">
+      <c r="H41" s="1">
         <v>46244</v>
       </c>
       <c r="I41" t="s">
@@ -3123,7 +3097,7 @@
       <c r="U41" t="s">
         <v>28</v>
       </c>
-      <c r="V41" s="2">
+      <c r="V41" s="1">
         <v>46199</v>
       </c>
     </row>
@@ -3167,7 +3141,7 @@
       <c r="U42" t="s">
         <v>28</v>
       </c>
-      <c r="V42" s="2">
+      <c r="V42" s="1">
         <v>46260</v>
       </c>
     </row>
@@ -3193,7 +3167,7 @@
       <c r="G43" t="s">
         <v>42</v>
       </c>
-      <c r="H43" s="2">
+      <c r="H43" s="1">
         <v>46191</v>
       </c>
       <c r="I43" t="s">
@@ -3223,7 +3197,7 @@
       <c r="U43" t="s">
         <v>28</v>
       </c>
-      <c r="V43" s="2">
+      <c r="V43" s="1">
         <v>46199</v>
       </c>
     </row>
@@ -3249,7 +3223,7 @@
       <c r="G44" t="s">
         <v>42</v>
       </c>
-      <c r="H44" s="2">
+      <c r="H44" s="1">
         <v>46191</v>
       </c>
       <c r="I44" t="s">
@@ -3279,7 +3253,7 @@
       <c r="U44" t="s">
         <v>28</v>
       </c>
-      <c r="V44" s="2">
+      <c r="V44" s="1">
         <v>46199</v>
       </c>
     </row>
@@ -3305,7 +3279,7 @@
       <c r="G45" t="s">
         <v>42</v>
       </c>
-      <c r="H45" s="2">
+      <c r="H45" s="1">
         <v>46213</v>
       </c>
       <c r="I45" t="s">
@@ -3338,7 +3312,7 @@
       <c r="U45" t="s">
         <v>180</v>
       </c>
-      <c r="V45" s="2">
+      <c r="V45" s="1">
         <v>46229</v>
       </c>
     </row>
@@ -3364,7 +3338,7 @@
       <c r="G46" t="s">
         <v>42</v>
       </c>
-      <c r="H46" s="2">
+      <c r="H46" s="1">
         <v>46210</v>
       </c>
       <c r="I46" t="s">
@@ -3394,7 +3368,7 @@
       <c r="U46" t="s">
         <v>180</v>
       </c>
-      <c r="V46" s="2">
+      <c r="V46" s="1">
         <v>46229</v>
       </c>
     </row>
@@ -3441,7 +3415,7 @@
       <c r="U47" t="s">
         <v>28</v>
       </c>
-      <c r="V47" s="2">
+      <c r="V47" s="1">
         <v>46321</v>
       </c>
     </row>
@@ -3494,7 +3468,7 @@
       <c r="U48" t="s">
         <v>180</v>
       </c>
-      <c r="V48" s="2">
+      <c r="V48" s="1">
         <v>46291</v>
       </c>
     </row>
@@ -3520,7 +3494,7 @@
       <c r="G49" t="s">
         <v>42</v>
       </c>
-      <c r="H49" s="2">
+      <c r="H49" s="1">
         <v>46176</v>
       </c>
       <c r="I49" t="s">
@@ -3553,7 +3527,7 @@
       <c r="U49" t="s">
         <v>180</v>
       </c>
-      <c r="V49" s="2">
+      <c r="V49" s="1">
         <v>46199</v>
       </c>
     </row>
@@ -3606,7 +3580,7 @@
       <c r="U50" t="s">
         <v>180</v>
       </c>
-      <c r="V50" s="2">
+      <c r="V50" s="1">
         <v>46260</v>
       </c>
     </row>
@@ -3659,7 +3633,7 @@
       <c r="U51" t="s">
         <v>180</v>
       </c>
-      <c r="V51" s="2">
+      <c r="V51" s="1">
         <v>46291</v>
       </c>
     </row>
@@ -3709,7 +3683,7 @@
       <c r="U52" t="s">
         <v>180</v>
       </c>
-      <c r="V52" s="2">
+      <c r="V52" s="1">
         <v>46321</v>
       </c>
     </row>
@@ -3735,7 +3709,7 @@
       <c r="G53" t="s">
         <v>42</v>
       </c>
-      <c r="H53" s="2">
+      <c r="H53" s="1">
         <v>46227</v>
       </c>
       <c r="I53" t="s">
@@ -3765,7 +3739,7 @@
       <c r="U53" t="s">
         <v>180</v>
       </c>
-      <c r="V53" s="2">
+      <c r="V53" s="1">
         <v>46229</v>
       </c>
     </row>
@@ -3818,7 +3792,7 @@
       <c r="U54" t="s">
         <v>180</v>
       </c>
-      <c r="V54" s="2">
+      <c r="V54" s="1">
         <v>46352</v>
       </c>
     </row>
@@ -3871,7 +3845,7 @@
       <c r="U55" t="s">
         <v>180</v>
       </c>
-      <c r="V55" s="2">
+      <c r="V55" s="1">
         <v>46321</v>
       </c>
     </row>
@@ -3921,7 +3895,7 @@
       <c r="U56" t="s">
         <v>180</v>
       </c>
-      <c r="V56" s="2">
+      <c r="V56" s="1">
         <v>46321</v>
       </c>
     </row>
@@ -3965,7 +3939,7 @@
       <c r="U57" t="s">
         <v>180</v>
       </c>
-      <c r="V57" s="2">
+      <c r="V57" s="1">
         <v>46049</v>
       </c>
     </row>
@@ -4091,7 +4065,7 @@
       <c r="U60" t="s">
         <v>180</v>
       </c>
-      <c r="V60" s="2">
+      <c r="V60" s="1">
         <v>46107</v>
       </c>
     </row>
@@ -4135,7 +4109,7 @@
       <c r="U61" t="s">
         <v>180</v>
       </c>
-      <c r="V61" s="2">
+      <c r="V61" s="1">
         <v>46107</v>
       </c>
     </row>
@@ -4179,7 +4153,7 @@
       <c r="U62" t="s">
         <v>180</v>
       </c>
-      <c r="V62" s="2">
+      <c r="V62" s="1">
         <v>46107</v>
       </c>
     </row>
@@ -4223,7 +4197,7 @@
       <c r="U63" t="s">
         <v>180</v>
       </c>
-      <c r="V63" s="2">
+      <c r="V63" s="1">
         <v>46107</v>
       </c>
     </row>
@@ -4267,7 +4241,7 @@
       <c r="U64" t="s">
         <v>180</v>
       </c>
-      <c r="V64" s="2">
+      <c r="V64" s="1">
         <v>46107</v>
       </c>
     </row>
@@ -4311,7 +4285,7 @@
       <c r="U65" t="s">
         <v>180</v>
       </c>
-      <c r="V65" s="2">
+      <c r="V65" s="1">
         <v>46107</v>
       </c>
     </row>
@@ -4355,7 +4329,7 @@
       <c r="U66" t="s">
         <v>28</v>
       </c>
-      <c r="V66" s="2">
+      <c r="V66" s="1">
         <v>46168</v>
       </c>
     </row>
@@ -4402,7 +4376,7 @@
       <c r="U67" t="s">
         <v>28</v>
       </c>
-      <c r="V67" s="2">
+      <c r="V67" s="1">
         <v>46291</v>
       </c>
     </row>
@@ -4455,7 +4429,7 @@
       <c r="U68" t="s">
         <v>180</v>
       </c>
-      <c r="V68" s="2">
+      <c r="V68" s="1">
         <v>46229</v>
       </c>
     </row>
@@ -4499,7 +4473,7 @@
       <c r="U69" t="s">
         <v>28</v>
       </c>
-      <c r="V69" s="2">
+      <c r="V69" s="1">
         <v>46260</v>
       </c>
     </row>
@@ -4543,7 +4517,7 @@
       <c r="U70" t="s">
         <v>180</v>
       </c>
-      <c r="V70" s="2">
+      <c r="V70" s="1">
         <v>46291</v>
       </c>
     </row>
@@ -4587,7 +4561,7 @@
       <c r="U71" t="s">
         <v>180</v>
       </c>
-      <c r="V71" s="2">
+      <c r="V71" s="1">
         <v>46168</v>
       </c>
     </row>
@@ -4631,7 +4605,7 @@
       <c r="U72" t="s">
         <v>180</v>
       </c>
-      <c r="V72" s="2">
+      <c r="V72" s="1">
         <v>46291</v>
       </c>
     </row>
@@ -4675,7 +4649,7 @@
       <c r="U73" t="s">
         <v>180</v>
       </c>
-      <c r="V73" s="2">
+      <c r="V73" s="1">
         <v>46291</v>
       </c>
     </row>
@@ -4719,7 +4693,7 @@
       <c r="U74" t="s">
         <v>180</v>
       </c>
-      <c r="V74" s="2">
+      <c r="V74" s="1">
         <v>46291</v>
       </c>
     </row>
@@ -4766,7 +4740,7 @@
       <c r="U75" t="s">
         <v>28</v>
       </c>
-      <c r="V75" s="2">
+      <c r="V75" s="1">
         <v>46321</v>
       </c>
     </row>
@@ -4816,7 +4790,7 @@
       <c r="U76" t="s">
         <v>180</v>
       </c>
-      <c r="V76" s="2">
+      <c r="V76" s="1">
         <v>46381</v>
       </c>
     </row>
@@ -4866,7 +4840,7 @@
       <c r="U77" t="s">
         <v>180</v>
       </c>
-      <c r="V77" s="2">
+      <c r="V77" s="1">
         <v>46381</v>
       </c>
     </row>
@@ -4916,7 +4890,7 @@
       <c r="U78" t="s">
         <v>28</v>
       </c>
-      <c r="V78" s="2">
+      <c r="V78" s="1">
         <v>46381</v>
       </c>
     </row>
@@ -4966,7 +4940,7 @@
       <c r="U79" t="s">
         <v>28</v>
       </c>
-      <c r="V79" s="2">
+      <c r="V79" s="1">
         <v>46381</v>
       </c>
     </row>
@@ -5016,7 +4990,7 @@
       <c r="U80" t="s">
         <v>28</v>
       </c>
-      <c r="V80" s="2">
+      <c r="V80" s="1">
         <v>46382</v>
       </c>
     </row>
@@ -5060,7 +5034,7 @@
       <c r="U81" t="s">
         <v>28</v>
       </c>
-      <c r="V81" s="2">
+      <c r="V81" s="1">
         <v>46382</v>
       </c>
     </row>
@@ -5113,7 +5087,7 @@
       <c r="U82" t="s">
         <v>180</v>
       </c>
-      <c r="V82" s="2">
+      <c r="V82" s="1">
         <v>46382</v>
       </c>
     </row>
@@ -5157,7 +5131,7 @@
       <c r="U83" t="s">
         <v>28</v>
       </c>
-      <c r="V83" s="2">
+      <c r="V83" s="1">
         <v>46321</v>
       </c>
     </row>
@@ -5201,7 +5175,7 @@
       <c r="U84" t="s">
         <v>28</v>
       </c>
-      <c r="V84" s="2">
+      <c r="V84" s="1">
         <v>46382</v>
       </c>
     </row>
@@ -5342,7 +5316,7 @@
       <c r="U87" t="s">
         <v>28</v>
       </c>
-      <c r="V87" s="2">
+      <c r="V87" s="1">
         <v>46291</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Atualização automática: mta (16/09/2026 12:40)
</commit_message>
<xml_diff>
--- a/Projetos/02_Dados_Tratados/base_mta_tratada.xlsx
+++ b/Projetos/02_Dados_Tratados/base_mta_tratada.xlsx
@@ -566,8 +566,16 @@
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="YYYY-MM-DD HH:MM:SS"/>
   </numFmts>
-  <fonts count="1">
+  <fonts count="2">
     <font>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
       <sz val="11"/>
       <color theme="1"/>
       <name val="Calibri"/>
@@ -583,7 +591,7 @@
       <patternFill patternType="gray125"/>
     </fill>
   </fills>
-  <borders count="1">
+  <borders count="2">
     <border>
       <left/>
       <right/>
@@ -591,12 +599,30 @@
       <bottom/>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin">
+        <color auto="1"/>
+      </left>
+      <right style="thin">
+        <color auto="1"/>
+      </right>
+      <top style="thin">
+        <color auto="1"/>
+      </top>
+      <bottom style="thin">
+        <color auto="1"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="3">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
   </cellXfs>
   <cellStyles count="1">
@@ -896,70 +922,70 @@
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:22">
-      <c r="A1" t="s">
+      <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
-      <c r="B1" t="s">
+      <c r="B1" s="1" t="s">
         <v>1</v>
       </c>
-      <c r="C1" t="s">
+      <c r="C1" s="1" t="s">
         <v>2</v>
       </c>
-      <c r="D1" t="s">
+      <c r="D1" s="1" t="s">
         <v>3</v>
       </c>
-      <c r="E1" t="s">
+      <c r="E1" s="1" t="s">
         <v>4</v>
       </c>
-      <c r="F1" t="s">
+      <c r="F1" s="1" t="s">
         <v>5</v>
       </c>
-      <c r="G1" t="s">
+      <c r="G1" s="1" t="s">
         <v>6</v>
       </c>
-      <c r="H1" t="s">
+      <c r="H1" s="1" t="s">
         <v>7</v>
       </c>
-      <c r="I1" t="s">
+      <c r="I1" s="1" t="s">
         <v>8</v>
       </c>
-      <c r="J1" t="s">
+      <c r="J1" s="1" t="s">
         <v>9</v>
       </c>
-      <c r="K1" t="s">
+      <c r="K1" s="1" t="s">
         <v>10</v>
       </c>
-      <c r="L1" t="s">
+      <c r="L1" s="1" t="s">
         <v>11</v>
       </c>
-      <c r="M1" t="s">
+      <c r="M1" s="1" t="s">
         <v>12</v>
       </c>
-      <c r="N1" t="s">
+      <c r="N1" s="1" t="s">
         <v>13</v>
       </c>
-      <c r="O1" t="s">
+      <c r="O1" s="1" t="s">
         <v>14</v>
       </c>
-      <c r="P1" t="s">
+      <c r="P1" s="1" t="s">
         <v>15</v>
       </c>
-      <c r="Q1" t="s">
+      <c r="Q1" s="1" t="s">
         <v>16</v>
       </c>
-      <c r="R1" t="s">
+      <c r="R1" s="1" t="s">
         <v>17</v>
       </c>
-      <c r="S1" t="s">
+      <c r="S1" s="1" t="s">
         <v>18</v>
       </c>
-      <c r="T1" t="s">
+      <c r="T1" s="1" t="s">
         <v>19</v>
       </c>
-      <c r="U1" t="s">
+      <c r="U1" s="1" t="s">
         <v>20</v>
       </c>
-      <c r="V1" t="s">
+      <c r="V1" s="1" t="s">
         <v>21</v>
       </c>
     </row>
@@ -1015,7 +1041,7 @@
       <c r="U2" t="s">
         <v>180</v>
       </c>
-      <c r="V2" s="1">
+      <c r="V2" s="2">
         <v>46229</v>
       </c>
     </row>
@@ -1062,7 +1088,7 @@
       <c r="U3" t="s">
         <v>28</v>
       </c>
-      <c r="V3" s="1">
+      <c r="V3" s="2">
         <v>46291</v>
       </c>
     </row>
@@ -1109,7 +1135,7 @@
       <c r="U4" t="s">
         <v>28</v>
       </c>
-      <c r="V4" s="1">
+      <c r="V4" s="2">
         <v>46321</v>
       </c>
     </row>
@@ -1156,7 +1182,7 @@
       <c r="U5" t="s">
         <v>28</v>
       </c>
-      <c r="V5" s="1">
+      <c r="V5" s="2">
         <v>46321</v>
       </c>
     </row>
@@ -1206,7 +1232,7 @@
       <c r="U6" t="s">
         <v>28</v>
       </c>
-      <c r="V6" s="1">
+      <c r="V6" s="2">
         <v>46291</v>
       </c>
     </row>
@@ -1232,7 +1258,7 @@
       <c r="G7" t="s">
         <v>42</v>
       </c>
-      <c r="H7" s="1">
+      <c r="H7" s="2">
         <v>46121</v>
       </c>
       <c r="I7" t="s">
@@ -1262,7 +1288,7 @@
       <c r="U7" t="s">
         <v>28</v>
       </c>
-      <c r="V7" s="1">
+      <c r="V7" s="2">
         <v>46138</v>
       </c>
     </row>
@@ -1309,7 +1335,7 @@
       <c r="U8" t="s">
         <v>28</v>
       </c>
-      <c r="V8" s="1">
+      <c r="V8" s="2">
         <v>46291</v>
       </c>
     </row>
@@ -1356,7 +1382,7 @@
       <c r="U9" t="s">
         <v>28</v>
       </c>
-      <c r="V9" s="1">
+      <c r="V9" s="2">
         <v>46291</v>
       </c>
     </row>
@@ -1403,7 +1429,7 @@
       <c r="U10" t="s">
         <v>28</v>
       </c>
-      <c r="V10" s="1">
+      <c r="V10" s="2">
         <v>46291</v>
       </c>
     </row>
@@ -1450,7 +1476,7 @@
       <c r="U11" t="s">
         <v>28</v>
       </c>
-      <c r="V11" s="1">
+      <c r="V11" s="2">
         <v>46291</v>
       </c>
     </row>
@@ -1476,7 +1502,7 @@
       <c r="G12" t="s">
         <v>42</v>
       </c>
-      <c r="H12" s="1">
+      <c r="H12" s="2">
         <v>46079</v>
       </c>
       <c r="I12" t="s">
@@ -1509,7 +1535,7 @@
       <c r="U12" t="s">
         <v>180</v>
       </c>
-      <c r="V12" s="1">
+      <c r="V12" s="2">
         <v>46079</v>
       </c>
     </row>
@@ -1562,7 +1588,7 @@
       <c r="U13" t="s">
         <v>180</v>
       </c>
-      <c r="V13" s="1">
+      <c r="V13" s="2">
         <v>46352</v>
       </c>
     </row>
@@ -1615,7 +1641,7 @@
       <c r="U14" t="s">
         <v>180</v>
       </c>
-      <c r="V14" s="1">
+      <c r="V14" s="2">
         <v>46352</v>
       </c>
     </row>
@@ -1668,7 +1694,7 @@
       <c r="U15" t="s">
         <v>180</v>
       </c>
-      <c r="V15" s="1">
+      <c r="V15" s="2">
         <v>46352</v>
       </c>
     </row>
@@ -1721,7 +1747,7 @@
       <c r="U16" t="s">
         <v>180</v>
       </c>
-      <c r="V16" s="1">
+      <c r="V16" s="2">
         <v>46229</v>
       </c>
     </row>
@@ -1747,7 +1773,7 @@
       <c r="G17" t="s">
         <v>42</v>
       </c>
-      <c r="H17" s="1">
+      <c r="H17" s="2">
         <v>46098</v>
       </c>
       <c r="I17" t="s">
@@ -1780,7 +1806,7 @@
       <c r="U17" t="s">
         <v>180</v>
       </c>
-      <c r="V17" s="1">
+      <c r="V17" s="2">
         <v>46107</v>
       </c>
     </row>
@@ -1806,7 +1832,7 @@
       <c r="G18" t="s">
         <v>42</v>
       </c>
-      <c r="H18" s="1">
+      <c r="H18" s="2">
         <v>46076</v>
       </c>
       <c r="I18" t="s">
@@ -1836,7 +1862,7 @@
       <c r="U18" t="s">
         <v>28</v>
       </c>
-      <c r="V18" s="1">
+      <c r="V18" s="2">
         <v>46079</v>
       </c>
     </row>
@@ -1862,7 +1888,7 @@
       <c r="G19" t="s">
         <v>42</v>
       </c>
-      <c r="H19" s="1">
+      <c r="H19" s="2">
         <v>46076</v>
       </c>
       <c r="I19" t="s">
@@ -1892,7 +1918,7 @@
       <c r="U19" t="s">
         <v>28</v>
       </c>
-      <c r="V19" s="1">
+      <c r="V19" s="2">
         <v>46079</v>
       </c>
     </row>
@@ -1939,7 +1965,7 @@
       <c r="U20" t="s">
         <v>28</v>
       </c>
-      <c r="V20" s="1">
+      <c r="V20" s="2">
         <v>46321</v>
       </c>
     </row>
@@ -1986,7 +2012,7 @@
       <c r="U21" t="s">
         <v>28</v>
       </c>
-      <c r="V21" s="1">
+      <c r="V21" s="2">
         <v>46321</v>
       </c>
     </row>
@@ -2033,7 +2059,7 @@
       <c r="U22" t="s">
         <v>28</v>
       </c>
-      <c r="V22" s="1">
+      <c r="V22" s="2">
         <v>46321</v>
       </c>
     </row>
@@ -2080,7 +2106,7 @@
       <c r="U23" t="s">
         <v>28</v>
       </c>
-      <c r="V23" s="1">
+      <c r="V23" s="2">
         <v>46321</v>
       </c>
     </row>
@@ -2106,7 +2132,7 @@
       <c r="G24" t="s">
         <v>42</v>
       </c>
-      <c r="H24" s="1">
+      <c r="H24" s="2">
         <v>46119</v>
       </c>
       <c r="I24" t="s">
@@ -2139,7 +2165,7 @@
       <c r="U24" t="s">
         <v>180</v>
       </c>
-      <c r="V24" s="1">
+      <c r="V24" s="2">
         <v>46138</v>
       </c>
     </row>
@@ -2165,7 +2191,7 @@
       <c r="G25" t="s">
         <v>42</v>
       </c>
-      <c r="H25" s="1">
+      <c r="H25" s="2">
         <v>46121</v>
       </c>
       <c r="I25" t="s">
@@ -2195,7 +2221,7 @@
       <c r="U25" t="s">
         <v>28</v>
       </c>
-      <c r="V25" s="1">
+      <c r="V25" s="2">
         <v>46138</v>
       </c>
     </row>
@@ -2221,7 +2247,7 @@
       <c r="G26" t="s">
         <v>42</v>
       </c>
-      <c r="H26" s="1">
+      <c r="H26" s="2">
         <v>46076</v>
       </c>
       <c r="I26" t="s">
@@ -2251,7 +2277,7 @@
       <c r="U26" t="s">
         <v>28</v>
       </c>
-      <c r="V26" s="1">
+      <c r="V26" s="2">
         <v>46079</v>
       </c>
     </row>
@@ -2304,7 +2330,7 @@
       <c r="U27" t="s">
         <v>180</v>
       </c>
-      <c r="V27" s="1">
+      <c r="V27" s="2">
         <v>46291</v>
       </c>
     </row>
@@ -2330,7 +2356,7 @@
       <c r="G28" t="s">
         <v>42</v>
       </c>
-      <c r="H28" s="1">
+      <c r="H28" s="2">
         <v>46199</v>
       </c>
       <c r="I28" t="s">
@@ -2363,7 +2389,7 @@
       <c r="U28" t="s">
         <v>180</v>
       </c>
-      <c r="V28" s="1">
+      <c r="V28" s="2">
         <v>46199</v>
       </c>
     </row>
@@ -2389,7 +2415,7 @@
       <c r="G29" t="s">
         <v>42</v>
       </c>
-      <c r="H29" s="1">
+      <c r="H29" s="2">
         <v>46199</v>
       </c>
       <c r="I29" t="s">
@@ -2422,7 +2448,7 @@
       <c r="U29" t="s">
         <v>180</v>
       </c>
-      <c r="V29" s="1">
+      <c r="V29" s="2">
         <v>46199</v>
       </c>
     </row>
@@ -2448,7 +2474,7 @@
       <c r="G30" t="s">
         <v>42</v>
       </c>
-      <c r="H30" s="1">
+      <c r="H30" s="2">
         <v>46199</v>
       </c>
       <c r="I30" t="s">
@@ -2481,7 +2507,7 @@
       <c r="U30" t="s">
         <v>180</v>
       </c>
-      <c r="V30" s="1">
+      <c r="V30" s="2">
         <v>46199</v>
       </c>
     </row>
@@ -2507,7 +2533,7 @@
       <c r="G31" t="s">
         <v>42</v>
       </c>
-      <c r="H31" s="1">
+      <c r="H31" s="2">
         <v>46199</v>
       </c>
       <c r="I31" t="s">
@@ -2540,7 +2566,7 @@
       <c r="U31" t="s">
         <v>180</v>
       </c>
-      <c r="V31" s="1">
+      <c r="V31" s="2">
         <v>46199</v>
       </c>
     </row>
@@ -2590,7 +2616,7 @@
       <c r="U32" t="s">
         <v>180</v>
       </c>
-      <c r="V32" s="1">
+      <c r="V32" s="2">
         <v>46291</v>
       </c>
     </row>
@@ -2616,7 +2642,7 @@
       <c r="G33" t="s">
         <v>42</v>
       </c>
-      <c r="H33" s="1">
+      <c r="H33" s="2">
         <v>46191</v>
       </c>
       <c r="I33" t="s">
@@ -2649,7 +2675,7 @@
       <c r="U33" t="s">
         <v>180</v>
       </c>
-      <c r="V33" s="1">
+      <c r="V33" s="2">
         <v>46199</v>
       </c>
     </row>
@@ -2675,7 +2701,7 @@
       <c r="G34" t="s">
         <v>42</v>
       </c>
-      <c r="H34" s="1">
+      <c r="H34" s="2">
         <v>46119</v>
       </c>
       <c r="I34" t="s">
@@ -2705,7 +2731,7 @@
       <c r="U34" t="s">
         <v>180</v>
       </c>
-      <c r="V34" s="1">
+      <c r="V34" s="2">
         <v>46138</v>
       </c>
     </row>
@@ -2731,7 +2757,7 @@
       <c r="G35" t="s">
         <v>42</v>
       </c>
-      <c r="H35" s="1">
+      <c r="H35" s="2">
         <v>46213</v>
       </c>
       <c r="I35" t="s">
@@ -2761,7 +2787,7 @@
       <c r="U35" t="s">
         <v>28</v>
       </c>
-      <c r="V35" s="1">
+      <c r="V35" s="2">
         <v>46229</v>
       </c>
     </row>
@@ -2787,7 +2813,7 @@
       <c r="G36" t="s">
         <v>42</v>
       </c>
-      <c r="H36" s="1">
+      <c r="H36" s="2">
         <v>46175</v>
       </c>
       <c r="I36" t="s">
@@ -2817,7 +2843,7 @@
       <c r="U36" t="s">
         <v>28</v>
       </c>
-      <c r="V36" s="1">
+      <c r="V36" s="2">
         <v>46199</v>
       </c>
     </row>
@@ -2843,7 +2869,7 @@
       <c r="G37" t="s">
         <v>42</v>
       </c>
-      <c r="H37" s="1">
+      <c r="H37" s="2">
         <v>46213</v>
       </c>
       <c r="I37" t="s">
@@ -2873,7 +2899,7 @@
       <c r="U37" t="s">
         <v>28</v>
       </c>
-      <c r="V37" s="1">
+      <c r="V37" s="2">
         <v>46229</v>
       </c>
     </row>
@@ -2899,7 +2925,7 @@
       <c r="G38" t="s">
         <v>42</v>
       </c>
-      <c r="H38" s="1">
+      <c r="H38" s="2">
         <v>46199</v>
       </c>
       <c r="I38" t="s">
@@ -2929,7 +2955,7 @@
       <c r="U38" t="s">
         <v>28</v>
       </c>
-      <c r="V38" s="1">
+      <c r="V38" s="2">
         <v>46199</v>
       </c>
     </row>
@@ -2955,7 +2981,7 @@
       <c r="G39" t="s">
         <v>42</v>
       </c>
-      <c r="H39" s="1">
+      <c r="H39" s="2">
         <v>46199</v>
       </c>
       <c r="I39" t="s">
@@ -2985,7 +3011,7 @@
       <c r="U39" t="s">
         <v>28</v>
       </c>
-      <c r="V39" s="1">
+      <c r="V39" s="2">
         <v>46199</v>
       </c>
     </row>
@@ -3011,7 +3037,7 @@
       <c r="G40" t="s">
         <v>42</v>
       </c>
-      <c r="H40" s="1">
+      <c r="H40" s="2">
         <v>46204</v>
       </c>
       <c r="I40" t="s">
@@ -3041,7 +3067,7 @@
       <c r="U40" t="s">
         <v>28</v>
       </c>
-      <c r="V40" s="1">
+      <c r="V40" s="2">
         <v>46229</v>
       </c>
     </row>
@@ -3067,7 +3093,7 @@
       <c r="G41" t="s">
         <v>42</v>
       </c>
-      <c r="H41" s="1">
+      <c r="H41" s="2">
         <v>46244</v>
       </c>
       <c r="I41" t="s">
@@ -3097,7 +3123,7 @@
       <c r="U41" t="s">
         <v>28</v>
       </c>
-      <c r="V41" s="1">
+      <c r="V41" s="2">
         <v>46199</v>
       </c>
     </row>
@@ -3141,7 +3167,7 @@
       <c r="U42" t="s">
         <v>28</v>
       </c>
-      <c r="V42" s="1">
+      <c r="V42" s="2">
         <v>46260</v>
       </c>
     </row>
@@ -3167,7 +3193,7 @@
       <c r="G43" t="s">
         <v>42</v>
       </c>
-      <c r="H43" s="1">
+      <c r="H43" s="2">
         <v>46191</v>
       </c>
       <c r="I43" t="s">
@@ -3197,7 +3223,7 @@
       <c r="U43" t="s">
         <v>28</v>
       </c>
-      <c r="V43" s="1">
+      <c r="V43" s="2">
         <v>46199</v>
       </c>
     </row>
@@ -3223,7 +3249,7 @@
       <c r="G44" t="s">
         <v>42</v>
       </c>
-      <c r="H44" s="1">
+      <c r="H44" s="2">
         <v>46191</v>
       </c>
       <c r="I44" t="s">
@@ -3253,7 +3279,7 @@
       <c r="U44" t="s">
         <v>28</v>
       </c>
-      <c r="V44" s="1">
+      <c r="V44" s="2">
         <v>46199</v>
       </c>
     </row>
@@ -3279,7 +3305,7 @@
       <c r="G45" t="s">
         <v>42</v>
       </c>
-      <c r="H45" s="1">
+      <c r="H45" s="2">
         <v>46213</v>
       </c>
       <c r="I45" t="s">
@@ -3312,7 +3338,7 @@
       <c r="U45" t="s">
         <v>180</v>
       </c>
-      <c r="V45" s="1">
+      <c r="V45" s="2">
         <v>46229</v>
       </c>
     </row>
@@ -3338,7 +3364,7 @@
       <c r="G46" t="s">
         <v>42</v>
       </c>
-      <c r="H46" s="1">
+      <c r="H46" s="2">
         <v>46210</v>
       </c>
       <c r="I46" t="s">
@@ -3368,7 +3394,7 @@
       <c r="U46" t="s">
         <v>180</v>
       </c>
-      <c r="V46" s="1">
+      <c r="V46" s="2">
         <v>46229</v>
       </c>
     </row>
@@ -3415,7 +3441,7 @@
       <c r="U47" t="s">
         <v>28</v>
       </c>
-      <c r="V47" s="1">
+      <c r="V47" s="2">
         <v>46321</v>
       </c>
     </row>
@@ -3468,7 +3494,7 @@
       <c r="U48" t="s">
         <v>180</v>
       </c>
-      <c r="V48" s="1">
+      <c r="V48" s="2">
         <v>46291</v>
       </c>
     </row>
@@ -3494,7 +3520,7 @@
       <c r="G49" t="s">
         <v>42</v>
       </c>
-      <c r="H49" s="1">
+      <c r="H49" s="2">
         <v>46176</v>
       </c>
       <c r="I49" t="s">
@@ -3527,7 +3553,7 @@
       <c r="U49" t="s">
         <v>180</v>
       </c>
-      <c r="V49" s="1">
+      <c r="V49" s="2">
         <v>46199</v>
       </c>
     </row>
@@ -3580,7 +3606,7 @@
       <c r="U50" t="s">
         <v>180</v>
       </c>
-      <c r="V50" s="1">
+      <c r="V50" s="2">
         <v>46260</v>
       </c>
     </row>
@@ -3633,7 +3659,7 @@
       <c r="U51" t="s">
         <v>180</v>
       </c>
-      <c r="V51" s="1">
+      <c r="V51" s="2">
         <v>46291</v>
       </c>
     </row>
@@ -3683,7 +3709,7 @@
       <c r="U52" t="s">
         <v>180</v>
       </c>
-      <c r="V52" s="1">
+      <c r="V52" s="2">
         <v>46321</v>
       </c>
     </row>
@@ -3709,7 +3735,7 @@
       <c r="G53" t="s">
         <v>42</v>
       </c>
-      <c r="H53" s="1">
+      <c r="H53" s="2">
         <v>46227</v>
       </c>
       <c r="I53" t="s">
@@ -3739,7 +3765,7 @@
       <c r="U53" t="s">
         <v>180</v>
       </c>
-      <c r="V53" s="1">
+      <c r="V53" s="2">
         <v>46229</v>
       </c>
     </row>
@@ -3792,7 +3818,7 @@
       <c r="U54" t="s">
         <v>180</v>
       </c>
-      <c r="V54" s="1">
+      <c r="V54" s="2">
         <v>46352</v>
       </c>
     </row>
@@ -3845,7 +3871,7 @@
       <c r="U55" t="s">
         <v>180</v>
       </c>
-      <c r="V55" s="1">
+      <c r="V55" s="2">
         <v>46321</v>
       </c>
     </row>
@@ -3895,7 +3921,7 @@
       <c r="U56" t="s">
         <v>180</v>
       </c>
-      <c r="V56" s="1">
+      <c r="V56" s="2">
         <v>46321</v>
       </c>
     </row>
@@ -3939,7 +3965,7 @@
       <c r="U57" t="s">
         <v>180</v>
       </c>
-      <c r="V57" s="1">
+      <c r="V57" s="2">
         <v>46049</v>
       </c>
     </row>
@@ -4065,7 +4091,7 @@
       <c r="U60" t="s">
         <v>180</v>
       </c>
-      <c r="V60" s="1">
+      <c r="V60" s="2">
         <v>46107</v>
       </c>
     </row>
@@ -4109,7 +4135,7 @@
       <c r="U61" t="s">
         <v>180</v>
       </c>
-      <c r="V61" s="1">
+      <c r="V61" s="2">
         <v>46107</v>
       </c>
     </row>
@@ -4153,7 +4179,7 @@
       <c r="U62" t="s">
         <v>180</v>
       </c>
-      <c r="V62" s="1">
+      <c r="V62" s="2">
         <v>46107</v>
       </c>
     </row>
@@ -4197,7 +4223,7 @@
       <c r="U63" t="s">
         <v>180</v>
       </c>
-      <c r="V63" s="1">
+      <c r="V63" s="2">
         <v>46107</v>
       </c>
     </row>
@@ -4241,7 +4267,7 @@
       <c r="U64" t="s">
         <v>180</v>
       </c>
-      <c r="V64" s="1">
+      <c r="V64" s="2">
         <v>46107</v>
       </c>
     </row>
@@ -4285,7 +4311,7 @@
       <c r="U65" t="s">
         <v>180</v>
       </c>
-      <c r="V65" s="1">
+      <c r="V65" s="2">
         <v>46107</v>
       </c>
     </row>
@@ -4329,7 +4355,7 @@
       <c r="U66" t="s">
         <v>28</v>
       </c>
-      <c r="V66" s="1">
+      <c r="V66" s="2">
         <v>46168</v>
       </c>
     </row>
@@ -4376,7 +4402,7 @@
       <c r="U67" t="s">
         <v>28</v>
       </c>
-      <c r="V67" s="1">
+      <c r="V67" s="2">
         <v>46291</v>
       </c>
     </row>
@@ -4429,7 +4455,7 @@
       <c r="U68" t="s">
         <v>180</v>
       </c>
-      <c r="V68" s="1">
+      <c r="V68" s="2">
         <v>46229</v>
       </c>
     </row>
@@ -4473,7 +4499,7 @@
       <c r="U69" t="s">
         <v>28</v>
       </c>
-      <c r="V69" s="1">
+      <c r="V69" s="2">
         <v>46260</v>
       </c>
     </row>
@@ -4517,7 +4543,7 @@
       <c r="U70" t="s">
         <v>180</v>
       </c>
-      <c r="V70" s="1">
+      <c r="V70" s="2">
         <v>46291</v>
       </c>
     </row>
@@ -4561,7 +4587,7 @@
       <c r="U71" t="s">
         <v>180</v>
       </c>
-      <c r="V71" s="1">
+      <c r="V71" s="2">
         <v>46168</v>
       </c>
     </row>
@@ -4605,7 +4631,7 @@
       <c r="U72" t="s">
         <v>180</v>
       </c>
-      <c r="V72" s="1">
+      <c r="V72" s="2">
         <v>46291</v>
       </c>
     </row>
@@ -4649,7 +4675,7 @@
       <c r="U73" t="s">
         <v>180</v>
       </c>
-      <c r="V73" s="1">
+      <c r="V73" s="2">
         <v>46291</v>
       </c>
     </row>
@@ -4693,7 +4719,7 @@
       <c r="U74" t="s">
         <v>180</v>
       </c>
-      <c r="V74" s="1">
+      <c r="V74" s="2">
         <v>46291</v>
       </c>
     </row>
@@ -4740,7 +4766,7 @@
       <c r="U75" t="s">
         <v>28</v>
       </c>
-      <c r="V75" s="1">
+      <c r="V75" s="2">
         <v>46321</v>
       </c>
     </row>
@@ -4790,7 +4816,7 @@
       <c r="U76" t="s">
         <v>180</v>
       </c>
-      <c r="V76" s="1">
+      <c r="V76" s="2">
         <v>46381</v>
       </c>
     </row>
@@ -4840,7 +4866,7 @@
       <c r="U77" t="s">
         <v>180</v>
       </c>
-      <c r="V77" s="1">
+      <c r="V77" s="2">
         <v>46381</v>
       </c>
     </row>
@@ -4890,7 +4916,7 @@
       <c r="U78" t="s">
         <v>28</v>
       </c>
-      <c r="V78" s="1">
+      <c r="V78" s="2">
         <v>46381</v>
       </c>
     </row>
@@ -4940,7 +4966,7 @@
       <c r="U79" t="s">
         <v>28</v>
       </c>
-      <c r="V79" s="1">
+      <c r="V79" s="2">
         <v>46381</v>
       </c>
     </row>
@@ -4990,7 +5016,7 @@
       <c r="U80" t="s">
         <v>28</v>
       </c>
-      <c r="V80" s="1">
+      <c r="V80" s="2">
         <v>46382</v>
       </c>
     </row>
@@ -5034,7 +5060,7 @@
       <c r="U81" t="s">
         <v>28</v>
       </c>
-      <c r="V81" s="1">
+      <c r="V81" s="2">
         <v>46382</v>
       </c>
     </row>
@@ -5087,7 +5113,7 @@
       <c r="U82" t="s">
         <v>180</v>
       </c>
-      <c r="V82" s="1">
+      <c r="V82" s="2">
         <v>46382</v>
       </c>
     </row>
@@ -5131,7 +5157,7 @@
       <c r="U83" t="s">
         <v>28</v>
       </c>
-      <c r="V83" s="1">
+      <c r="V83" s="2">
         <v>46321</v>
       </c>
     </row>
@@ -5175,7 +5201,7 @@
       <c r="U84" t="s">
         <v>28</v>
       </c>
-      <c r="V84" s="1">
+      <c r="V84" s="2">
         <v>46382</v>
       </c>
     </row>
@@ -5316,7 +5342,7 @@
       <c r="U87" t="s">
         <v>28</v>
       </c>
-      <c r="V87" s="1">
+      <c r="V87" s="2">
         <v>46291</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Atualização automática: mta (17/09/2026 12:32)
</commit_message>
<xml_diff>
--- a/Projetos/02_Dados_Tratados/base_mta_tratada.xlsx
+++ b/Projetos/02_Dados_Tratados/base_mta_tratada.xlsx
@@ -14,7 +14,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1141" uniqueCount="181">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1153" uniqueCount="182">
   <si>
     <t>linha</t>
   </si>
@@ -133,6 +133,9 @@
     <t>20XV</t>
   </si>
   <si>
+    <t>DESTQ50</t>
+  </si>
+  <si>
     <t>20IH</t>
   </si>
   <si>
@@ -310,7 +313,7 @@
     <t>CNT 001/CABW-PAMASP/2025 - EXCHANGE - FLORIDA SUPPLY</t>
   </si>
   <si>
-    <t>Atualização de GPS</t>
+    <t>Requisição Consumíveis</t>
   </si>
   <si>
     <t>Material reparo acessórios PT6A-114A (1/3)</t>
@@ -502,7 +505,7 @@
     <t>Revisão Geral PT6A-114A</t>
   </si>
   <si>
-    <t>Hora de Voo 10/10 - 310 HV</t>
+    <t>MÓDULO EXTRA - SOB DEMANDA</t>
   </si>
   <si>
     <t>Material reparo PT6A-114A (4/4)</t>
@@ -514,16 +517,16 @@
     <t>CABW</t>
   </si>
   <si>
+    <t>CELOG</t>
+  </si>
+  <si>
     <t>FMS</t>
   </si>
   <si>
-    <t>CELOG</t>
+    <t>339030</t>
   </si>
   <si>
     <t>339039</t>
-  </si>
-  <si>
-    <t>339030</t>
   </si>
   <si>
     <t>449052</t>
@@ -566,16 +569,8 @@
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="YYYY-MM-DD HH:MM:SS"/>
   </numFmts>
-  <fonts count="2">
+  <fonts count="1">
     <font>
-      <sz val="11"/>
-      <color theme="1"/>
-      <name val="Calibri"/>
-      <family val="2"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <b/>
       <sz val="11"/>
       <color theme="1"/>
       <name val="Calibri"/>
@@ -591,7 +586,7 @@
       <patternFill patternType="gray125"/>
     </fill>
   </fills>
-  <borders count="2">
+  <borders count="1">
     <border>
       <left/>
       <right/>
@@ -599,30 +594,12 @@
       <bottom/>
       <diagonal/>
     </border>
-    <border>
-      <left style="thin">
-        <color auto="1"/>
-      </left>
-      <right style="thin">
-        <color auto="1"/>
-      </right>
-      <top style="thin">
-        <color auto="1"/>
-      </top>
-      <bottom style="thin">
-        <color auto="1"/>
-      </bottom>
-      <diagonal/>
-    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="3">
+  <cellXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top"/>
-    </xf>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
   </cellXfs>
   <cellStyles count="1">
@@ -918,74 +895,74 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:V87"/>
+  <dimension ref="A1:V88"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:22">
-      <c r="A1" s="1" t="s">
+      <c r="A1" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="1" t="s">
+      <c r="B1" t="s">
         <v>1</v>
       </c>
-      <c r="C1" s="1" t="s">
+      <c r="C1" t="s">
         <v>2</v>
       </c>
-      <c r="D1" s="1" t="s">
+      <c r="D1" t="s">
         <v>3</v>
       </c>
-      <c r="E1" s="1" t="s">
+      <c r="E1" t="s">
         <v>4</v>
       </c>
-      <c r="F1" s="1" t="s">
+      <c r="F1" t="s">
         <v>5</v>
       </c>
-      <c r="G1" s="1" t="s">
+      <c r="G1" t="s">
         <v>6</v>
       </c>
-      <c r="H1" s="1" t="s">
+      <c r="H1" t="s">
         <v>7</v>
       </c>
-      <c r="I1" s="1" t="s">
+      <c r="I1" t="s">
         <v>8</v>
       </c>
-      <c r="J1" s="1" t="s">
+      <c r="J1" t="s">
         <v>9</v>
       </c>
-      <c r="K1" s="1" t="s">
+      <c r="K1" t="s">
         <v>10</v>
       </c>
-      <c r="L1" s="1" t="s">
+      <c r="L1" t="s">
         <v>11</v>
       </c>
-      <c r="M1" s="1" t="s">
+      <c r="M1" t="s">
         <v>12</v>
       </c>
-      <c r="N1" s="1" t="s">
+      <c r="N1" t="s">
         <v>13</v>
       </c>
-      <c r="O1" s="1" t="s">
+      <c r="O1" t="s">
         <v>14</v>
       </c>
-      <c r="P1" s="1" t="s">
+      <c r="P1" t="s">
         <v>15</v>
       </c>
-      <c r="Q1" s="1" t="s">
+      <c r="Q1" t="s">
         <v>16</v>
       </c>
-      <c r="R1" s="1" t="s">
+      <c r="R1" t="s">
         <v>17</v>
       </c>
-      <c r="S1" s="1" t="s">
+      <c r="S1" t="s">
         <v>18</v>
       </c>
-      <c r="T1" s="1" t="s">
+      <c r="T1" t="s">
         <v>19</v>
       </c>
-      <c r="U1" s="1" t="s">
+      <c r="U1" t="s">
         <v>20</v>
       </c>
-      <c r="V1" s="1" t="s">
+      <c r="V1" t="s">
         <v>21</v>
       </c>
     </row>
@@ -1009,39 +986,39 @@
         <v>30</v>
       </c>
       <c r="J2" t="s">
-        <v>62</v>
+        <v>63</v>
       </c>
       <c r="K2" t="s">
-        <v>70</v>
+        <v>71</v>
       </c>
       <c r="L2" t="s">
-        <v>78</v>
+        <v>79</v>
       </c>
       <c r="N2" t="s">
-        <v>79</v>
+        <v>80</v>
       </c>
       <c r="O2" t="s">
-        <v>98</v>
+        <v>99</v>
       </c>
       <c r="P2">
         <v>135000</v>
       </c>
       <c r="Q2" t="s">
-        <v>165</v>
+        <v>166</v>
       </c>
       <c r="R2" t="s">
-        <v>168</v>
+        <v>169</v>
       </c>
       <c r="S2" t="s">
-        <v>171</v>
+        <v>172</v>
       </c>
       <c r="T2" t="s">
-        <v>175</v>
+        <v>176</v>
       </c>
       <c r="U2" t="s">
-        <v>180</v>
-      </c>
-      <c r="V2" s="2">
+        <v>181</v>
+      </c>
+      <c r="V2" s="1">
         <v>46229</v>
       </c>
     </row>
@@ -1065,10 +1042,10 @@
         <v>30</v>
       </c>
       <c r="N3" t="s">
-        <v>79</v>
+        <v>80</v>
       </c>
       <c r="O3" t="s">
-        <v>99</v>
+        <v>100</v>
       </c>
       <c r="P3">
         <v>400000</v>
@@ -1080,15 +1057,15 @@
         <v>169</v>
       </c>
       <c r="S3" t="s">
-        <v>171</v>
+        <v>172</v>
       </c>
       <c r="T3" t="s">
-        <v>175</v>
+        <v>176</v>
       </c>
       <c r="U3" t="s">
         <v>28</v>
       </c>
-      <c r="V3" s="2">
+      <c r="V3" s="1">
         <v>46291</v>
       </c>
     </row>
@@ -1112,30 +1089,30 @@
         <v>30</v>
       </c>
       <c r="G4" t="s">
-        <v>41</v>
+        <v>42</v>
       </c>
       <c r="N4" t="s">
-        <v>80</v>
+        <v>81</v>
       </c>
       <c r="O4" t="s">
-        <v>100</v>
+        <v>101</v>
       </c>
       <c r="Q4" t="s">
-        <v>165</v>
+        <v>166</v>
       </c>
       <c r="R4" t="s">
-        <v>168</v>
+        <v>170</v>
       </c>
       <c r="S4" t="s">
-        <v>171</v>
+        <v>172</v>
       </c>
       <c r="T4" t="s">
-        <v>175</v>
+        <v>176</v>
       </c>
       <c r="U4" t="s">
         <v>28</v>
       </c>
-      <c r="V4" s="2">
+      <c r="V4" s="1">
         <v>46321</v>
       </c>
     </row>
@@ -1159,30 +1136,30 @@
         <v>30</v>
       </c>
       <c r="N5" t="s">
-        <v>80</v>
+        <v>81</v>
       </c>
       <c r="O5" t="s">
-        <v>101</v>
+        <v>102</v>
       </c>
       <c r="P5">
         <v>384180</v>
       </c>
       <c r="Q5" t="s">
-        <v>165</v>
+        <v>166</v>
       </c>
       <c r="R5" t="s">
-        <v>168</v>
+        <v>170</v>
       </c>
       <c r="S5" t="s">
-        <v>171</v>
+        <v>172</v>
       </c>
       <c r="T5" t="s">
-        <v>175</v>
+        <v>176</v>
       </c>
       <c r="U5" t="s">
         <v>28</v>
       </c>
-      <c r="V5" s="2">
+      <c r="V5" s="1">
         <v>46321</v>
       </c>
     </row>
@@ -1206,33 +1183,33 @@
         <v>30</v>
       </c>
       <c r="L6" t="s">
-        <v>78</v>
+        <v>79</v>
       </c>
       <c r="N6" t="s">
-        <v>81</v>
+        <v>82</v>
       </c>
       <c r="O6" t="s">
-        <v>102</v>
+        <v>103</v>
       </c>
       <c r="P6">
         <v>563000</v>
       </c>
       <c r="Q6" t="s">
-        <v>165</v>
+        <v>166</v>
       </c>
       <c r="R6" t="s">
-        <v>168</v>
+        <v>170</v>
       </c>
       <c r="S6" t="s">
-        <v>171</v>
+        <v>172</v>
       </c>
       <c r="T6" t="s">
-        <v>175</v>
+        <v>176</v>
       </c>
       <c r="U6" t="s">
         <v>28</v>
       </c>
-      <c r="V6" s="2">
+      <c r="V6" s="1">
         <v>46291</v>
       </c>
     </row>
@@ -1256,19 +1233,19 @@
         <v>30</v>
       </c>
       <c r="G7" t="s">
-        <v>42</v>
-      </c>
-      <c r="H7" s="2">
+        <v>43</v>
+      </c>
+      <c r="H7" s="1">
         <v>46121</v>
       </c>
       <c r="I7" t="s">
-        <v>45</v>
+        <v>46</v>
       </c>
       <c r="N7" t="s">
-        <v>82</v>
+        <v>83</v>
       </c>
       <c r="O7" t="s">
-        <v>103</v>
+        <v>104</v>
       </c>
       <c r="P7">
         <v>3799999.6</v>
@@ -1277,18 +1254,18 @@
         <v>167</v>
       </c>
       <c r="R7" t="s">
-        <v>168</v>
+        <v>170</v>
       </c>
       <c r="S7" t="s">
-        <v>171</v>
+        <v>172</v>
       </c>
       <c r="T7" t="s">
-        <v>176</v>
+        <v>177</v>
       </c>
       <c r="U7" t="s">
         <v>28</v>
       </c>
-      <c r="V7" s="2">
+      <c r="V7" s="1">
         <v>46138</v>
       </c>
     </row>
@@ -1312,30 +1289,30 @@
         <v>30</v>
       </c>
       <c r="N8" t="s">
-        <v>80</v>
+        <v>81</v>
       </c>
       <c r="O8" t="s">
-        <v>104</v>
+        <v>105</v>
       </c>
       <c r="P8">
         <v>430000</v>
       </c>
       <c r="Q8" t="s">
-        <v>165</v>
+        <v>166</v>
       </c>
       <c r="R8" t="s">
-        <v>168</v>
+        <v>170</v>
       </c>
       <c r="S8" t="s">
-        <v>171</v>
+        <v>172</v>
       </c>
       <c r="T8" t="s">
-        <v>175</v>
+        <v>176</v>
       </c>
       <c r="U8" t="s">
         <v>28</v>
       </c>
-      <c r="V8" s="2">
+      <c r="V8" s="1">
         <v>46291</v>
       </c>
     </row>
@@ -1359,30 +1336,30 @@
         <v>30</v>
       </c>
       <c r="N9" t="s">
-        <v>80</v>
+        <v>81</v>
       </c>
       <c r="O9" t="s">
-        <v>105</v>
+        <v>106</v>
       </c>
       <c r="P9">
         <v>60000</v>
       </c>
       <c r="Q9" t="s">
-        <v>165</v>
+        <v>166</v>
       </c>
       <c r="R9" t="s">
-        <v>168</v>
+        <v>170</v>
       </c>
       <c r="S9" t="s">
-        <v>171</v>
+        <v>172</v>
       </c>
       <c r="T9" t="s">
-        <v>175</v>
+        <v>176</v>
       </c>
       <c r="U9" t="s">
         <v>28</v>
       </c>
-      <c r="V9" s="2">
+      <c r="V9" s="1">
         <v>46291</v>
       </c>
     </row>
@@ -1406,30 +1383,30 @@
         <v>30</v>
       </c>
       <c r="N10" t="s">
-        <v>81</v>
+        <v>82</v>
       </c>
       <c r="O10" t="s">
-        <v>106</v>
+        <v>107</v>
       </c>
       <c r="P10">
         <v>200000</v>
       </c>
       <c r="Q10" t="s">
-        <v>165</v>
+        <v>166</v>
       </c>
       <c r="R10" t="s">
-        <v>168</v>
+        <v>170</v>
       </c>
       <c r="S10" t="s">
-        <v>171</v>
+        <v>172</v>
       </c>
       <c r="T10" t="s">
-        <v>175</v>
+        <v>176</v>
       </c>
       <c r="U10" t="s">
         <v>28</v>
       </c>
-      <c r="V10" s="2">
+      <c r="V10" s="1">
         <v>46291</v>
       </c>
     </row>
@@ -1453,30 +1430,30 @@
         <v>30</v>
       </c>
       <c r="N11" t="s">
-        <v>81</v>
+        <v>82</v>
       </c>
       <c r="O11" t="s">
-        <v>107</v>
+        <v>108</v>
       </c>
       <c r="P11">
         <v>320000</v>
       </c>
       <c r="Q11" t="s">
-        <v>165</v>
+        <v>166</v>
       </c>
       <c r="R11" t="s">
-        <v>168</v>
+        <v>170</v>
       </c>
       <c r="S11" t="s">
-        <v>171</v>
+        <v>172</v>
       </c>
       <c r="T11" t="s">
-        <v>175</v>
+        <v>176</v>
       </c>
       <c r="U11" t="s">
         <v>28</v>
       </c>
-      <c r="V11" s="2">
+      <c r="V11" s="1">
         <v>46291</v>
       </c>
     </row>
@@ -1500,42 +1477,42 @@
         <v>30</v>
       </c>
       <c r="G12" t="s">
-        <v>42</v>
-      </c>
-      <c r="H12" s="2">
+        <v>43</v>
+      </c>
+      <c r="H12" s="1">
         <v>46079</v>
       </c>
       <c r="I12" t="s">
-        <v>46</v>
+        <v>47</v>
       </c>
       <c r="J12" t="s">
-        <v>63</v>
+        <v>64</v>
       </c>
       <c r="N12" t="s">
-        <v>79</v>
+        <v>80</v>
       </c>
       <c r="O12" t="s">
-        <v>108</v>
+        <v>109</v>
       </c>
       <c r="P12">
         <v>1187433.02</v>
       </c>
       <c r="Q12" t="s">
-        <v>165</v>
+        <v>166</v>
       </c>
       <c r="R12" t="s">
         <v>169</v>
       </c>
       <c r="S12" t="s">
-        <v>171</v>
+        <v>172</v>
       </c>
       <c r="T12" t="s">
-        <v>175</v>
+        <v>176</v>
       </c>
       <c r="U12" t="s">
-        <v>180</v>
-      </c>
-      <c r="V12" s="2">
+        <v>181</v>
+      </c>
+      <c r="V12" s="1">
         <v>46079</v>
       </c>
     </row>
@@ -1559,36 +1536,36 @@
         <v>30</v>
       </c>
       <c r="J13" t="s">
-        <v>62</v>
+        <v>63</v>
       </c>
       <c r="K13" t="s">
-        <v>71</v>
+        <v>72</v>
       </c>
       <c r="N13" t="s">
-        <v>79</v>
+        <v>80</v>
       </c>
       <c r="O13" t="s">
-        <v>109</v>
+        <v>110</v>
       </c>
       <c r="P13">
         <v>1000000</v>
       </c>
       <c r="Q13" t="s">
-        <v>165</v>
+        <v>166</v>
       </c>
       <c r="R13" t="s">
         <v>169</v>
       </c>
       <c r="S13" t="s">
-        <v>171</v>
+        <v>172</v>
       </c>
       <c r="T13" t="s">
-        <v>175</v>
+        <v>176</v>
       </c>
       <c r="U13" t="s">
-        <v>180</v>
-      </c>
-      <c r="V13" s="2">
+        <v>181</v>
+      </c>
+      <c r="V13" s="1">
         <v>46352</v>
       </c>
     </row>
@@ -1612,36 +1589,36 @@
         <v>30</v>
       </c>
       <c r="J14" t="s">
-        <v>62</v>
+        <v>63</v>
       </c>
       <c r="K14" t="s">
-        <v>71</v>
+        <v>72</v>
       </c>
       <c r="N14" t="s">
-        <v>79</v>
+        <v>80</v>
       </c>
       <c r="O14" t="s">
-        <v>110</v>
+        <v>111</v>
       </c>
       <c r="P14">
         <v>1000000</v>
       </c>
       <c r="Q14" t="s">
-        <v>165</v>
+        <v>166</v>
       </c>
       <c r="R14" t="s">
         <v>169</v>
       </c>
       <c r="S14" t="s">
-        <v>171</v>
+        <v>172</v>
       </c>
       <c r="T14" t="s">
-        <v>175</v>
+        <v>176</v>
       </c>
       <c r="U14" t="s">
-        <v>180</v>
-      </c>
-      <c r="V14" s="2">
+        <v>181</v>
+      </c>
+      <c r="V14" s="1">
         <v>46352</v>
       </c>
     </row>
@@ -1665,36 +1642,36 @@
         <v>30</v>
       </c>
       <c r="J15" t="s">
-        <v>62</v>
+        <v>63</v>
       </c>
       <c r="K15" t="s">
-        <v>71</v>
+        <v>72</v>
       </c>
       <c r="N15" t="s">
-        <v>79</v>
+        <v>80</v>
       </c>
       <c r="O15" t="s">
-        <v>111</v>
+        <v>112</v>
       </c>
       <c r="P15">
         <v>1000000</v>
       </c>
       <c r="Q15" t="s">
-        <v>165</v>
+        <v>166</v>
       </c>
       <c r="R15" t="s">
         <v>169</v>
       </c>
       <c r="S15" t="s">
-        <v>171</v>
+        <v>172</v>
       </c>
       <c r="T15" t="s">
-        <v>175</v>
+        <v>176</v>
       </c>
       <c r="U15" t="s">
-        <v>180</v>
-      </c>
-      <c r="V15" s="2">
+        <v>181</v>
+      </c>
+      <c r="V15" s="1">
         <v>46352</v>
       </c>
     </row>
@@ -1718,36 +1695,36 @@
         <v>30</v>
       </c>
       <c r="J16" t="s">
-        <v>62</v>
+        <v>63</v>
       </c>
       <c r="K16" t="s">
-        <v>71</v>
+        <v>72</v>
       </c>
       <c r="N16" t="s">
-        <v>83</v>
+        <v>84</v>
       </c>
       <c r="O16" t="s">
-        <v>112</v>
+        <v>113</v>
       </c>
       <c r="P16">
         <v>100000</v>
       </c>
       <c r="Q16" t="s">
-        <v>166</v>
+        <v>168</v>
       </c>
       <c r="R16" t="s">
         <v>169</v>
       </c>
       <c r="S16" t="s">
-        <v>171</v>
+        <v>172</v>
       </c>
       <c r="T16" t="s">
-        <v>175</v>
+        <v>176</v>
       </c>
       <c r="U16" t="s">
-        <v>180</v>
-      </c>
-      <c r="V16" s="2">
+        <v>181</v>
+      </c>
+      <c r="V16" s="1">
         <v>46229</v>
       </c>
     </row>
@@ -1771,22 +1748,22 @@
         <v>30</v>
       </c>
       <c r="G17" t="s">
-        <v>42</v>
-      </c>
-      <c r="H17" s="2">
+        <v>43</v>
+      </c>
+      <c r="H17" s="1">
         <v>46098</v>
       </c>
       <c r="I17" t="s">
-        <v>47</v>
+        <v>48</v>
       </c>
       <c r="J17" t="s">
-        <v>63</v>
+        <v>64</v>
       </c>
       <c r="N17" t="s">
-        <v>84</v>
+        <v>85</v>
       </c>
       <c r="O17" t="s">
-        <v>113</v>
+        <v>114</v>
       </c>
       <c r="P17">
         <v>1770880.5</v>
@@ -1795,18 +1772,18 @@
         <v>167</v>
       </c>
       <c r="R17" t="s">
-        <v>168</v>
+        <v>170</v>
       </c>
       <c r="S17" t="s">
-        <v>171</v>
+        <v>172</v>
       </c>
       <c r="T17" t="s">
-        <v>177</v>
+        <v>178</v>
       </c>
       <c r="U17" t="s">
-        <v>180</v>
-      </c>
-      <c r="V17" s="2">
+        <v>181</v>
+      </c>
+      <c r="V17" s="1">
         <v>46107</v>
       </c>
     </row>
@@ -1830,19 +1807,19 @@
         <v>30</v>
       </c>
       <c r="G18" t="s">
-        <v>42</v>
-      </c>
-      <c r="H18" s="2">
+        <v>43</v>
+      </c>
+      <c r="H18" s="1">
         <v>46076</v>
       </c>
       <c r="I18" t="s">
-        <v>48</v>
+        <v>49</v>
       </c>
       <c r="N18" t="s">
-        <v>85</v>
+        <v>86</v>
       </c>
       <c r="O18" t="s">
-        <v>114</v>
+        <v>115</v>
       </c>
       <c r="P18">
         <v>350000</v>
@@ -1854,15 +1831,15 @@
         <v>169</v>
       </c>
       <c r="S18" t="s">
-        <v>171</v>
+        <v>172</v>
       </c>
       <c r="T18" t="s">
-        <v>176</v>
+        <v>177</v>
       </c>
       <c r="U18" t="s">
         <v>28</v>
       </c>
-      <c r="V18" s="2">
+      <c r="V18" s="1">
         <v>46079</v>
       </c>
     </row>
@@ -1886,19 +1863,19 @@
         <v>30</v>
       </c>
       <c r="G19" t="s">
-        <v>42</v>
-      </c>
-      <c r="H19" s="2">
+        <v>43</v>
+      </c>
+      <c r="H19" s="1">
         <v>46076</v>
       </c>
       <c r="I19" t="s">
-        <v>48</v>
+        <v>49</v>
       </c>
       <c r="N19" t="s">
-        <v>85</v>
+        <v>86</v>
       </c>
       <c r="O19" t="s">
-        <v>115</v>
+        <v>116</v>
       </c>
       <c r="P19">
         <v>350000</v>
@@ -1910,15 +1887,15 @@
         <v>169</v>
       </c>
       <c r="S19" t="s">
-        <v>171</v>
+        <v>172</v>
       </c>
       <c r="T19" t="s">
-        <v>176</v>
+        <v>177</v>
       </c>
       <c r="U19" t="s">
         <v>28</v>
       </c>
-      <c r="V19" s="2">
+      <c r="V19" s="1">
         <v>46079</v>
       </c>
     </row>
@@ -1942,10 +1919,10 @@
         <v>30</v>
       </c>
       <c r="N20" t="s">
-        <v>86</v>
+        <v>87</v>
       </c>
       <c r="O20" t="s">
-        <v>116</v>
+        <v>117</v>
       </c>
       <c r="P20">
         <v>1000000</v>
@@ -1957,15 +1934,15 @@
         <v>169</v>
       </c>
       <c r="S20" t="s">
-        <v>171</v>
+        <v>172</v>
       </c>
       <c r="T20" t="s">
-        <v>176</v>
+        <v>177</v>
       </c>
       <c r="U20" t="s">
         <v>28</v>
       </c>
-      <c r="V20" s="2">
+      <c r="V20" s="1">
         <v>46321</v>
       </c>
     </row>
@@ -1989,10 +1966,10 @@
         <v>30</v>
       </c>
       <c r="N21" t="s">
-        <v>79</v>
+        <v>80</v>
       </c>
       <c r="O21" t="s">
-        <v>117</v>
+        <v>118</v>
       </c>
       <c r="P21">
         <v>400000</v>
@@ -2004,15 +1981,15 @@
         <v>169</v>
       </c>
       <c r="S21" t="s">
-        <v>171</v>
+        <v>172</v>
       </c>
       <c r="T21" t="s">
-        <v>175</v>
+        <v>176</v>
       </c>
       <c r="U21" t="s">
         <v>28</v>
       </c>
-      <c r="V21" s="2">
+      <c r="V21" s="1">
         <v>46321</v>
       </c>
     </row>
@@ -2036,30 +2013,30 @@
         <v>30</v>
       </c>
       <c r="N22" t="s">
-        <v>80</v>
+        <v>81</v>
       </c>
       <c r="O22" t="s">
-        <v>118</v>
+        <v>119</v>
       </c>
       <c r="P22">
         <v>120000</v>
       </c>
       <c r="Q22" t="s">
-        <v>165</v>
+        <v>166</v>
       </c>
       <c r="R22" t="s">
-        <v>168</v>
+        <v>170</v>
       </c>
       <c r="S22" t="s">
-        <v>171</v>
+        <v>172</v>
       </c>
       <c r="T22" t="s">
-        <v>175</v>
+        <v>176</v>
       </c>
       <c r="U22" t="s">
         <v>28</v>
       </c>
-      <c r="V22" s="2">
+      <c r="V22" s="1">
         <v>46321</v>
       </c>
     </row>
@@ -2083,30 +2060,30 @@
         <v>30</v>
       </c>
       <c r="N23" t="s">
-        <v>80</v>
+        <v>81</v>
       </c>
       <c r="O23" t="s">
-        <v>119</v>
+        <v>120</v>
       </c>
       <c r="P23">
         <v>80000</v>
       </c>
       <c r="Q23" t="s">
-        <v>165</v>
+        <v>166</v>
       </c>
       <c r="R23" t="s">
-        <v>168</v>
+        <v>170</v>
       </c>
       <c r="S23" t="s">
-        <v>171</v>
+        <v>172</v>
       </c>
       <c r="T23" t="s">
-        <v>175</v>
+        <v>176</v>
       </c>
       <c r="U23" t="s">
         <v>28</v>
       </c>
-      <c r="V23" s="2">
+      <c r="V23" s="1">
         <v>46321</v>
       </c>
     </row>
@@ -2130,22 +2107,22 @@
         <v>31</v>
       </c>
       <c r="G24" t="s">
-        <v>42</v>
-      </c>
-      <c r="H24" s="2">
+        <v>43</v>
+      </c>
+      <c r="H24" s="1">
         <v>46119</v>
       </c>
       <c r="I24" t="s">
-        <v>49</v>
+        <v>50</v>
       </c>
       <c r="J24" t="s">
-        <v>64</v>
+        <v>65</v>
       </c>
       <c r="N24" t="s">
-        <v>84</v>
+        <v>85</v>
       </c>
       <c r="O24" t="s">
-        <v>120</v>
+        <v>121</v>
       </c>
       <c r="P24">
         <v>1704503</v>
@@ -2154,18 +2131,18 @@
         <v>167</v>
       </c>
       <c r="R24" t="s">
-        <v>168</v>
+        <v>170</v>
       </c>
       <c r="S24" t="s">
-        <v>171</v>
+        <v>172</v>
       </c>
       <c r="T24" t="s">
-        <v>177</v>
+        <v>178</v>
       </c>
       <c r="U24" t="s">
-        <v>180</v>
-      </c>
-      <c r="V24" s="2">
+        <v>181</v>
+      </c>
+      <c r="V24" s="1">
         <v>46138</v>
       </c>
     </row>
@@ -2189,19 +2166,19 @@
         <v>30</v>
       </c>
       <c r="G25" t="s">
-        <v>42</v>
-      </c>
-      <c r="H25" s="2">
+        <v>43</v>
+      </c>
+      <c r="H25" s="1">
         <v>46121</v>
       </c>
       <c r="I25" t="s">
-        <v>50</v>
+        <v>51</v>
       </c>
       <c r="N25" t="s">
-        <v>87</v>
+        <v>88</v>
       </c>
       <c r="O25" t="s">
-        <v>121</v>
+        <v>122</v>
       </c>
       <c r="P25">
         <v>3799000</v>
@@ -2210,18 +2187,18 @@
         <v>167</v>
       </c>
       <c r="R25" t="s">
-        <v>168</v>
+        <v>170</v>
       </c>
       <c r="S25" t="s">
-        <v>171</v>
+        <v>172</v>
       </c>
       <c r="T25" t="s">
-        <v>176</v>
+        <v>177</v>
       </c>
       <c r="U25" t="s">
         <v>28</v>
       </c>
-      <c r="V25" s="2">
+      <c r="V25" s="1">
         <v>46138</v>
       </c>
     </row>
@@ -2245,19 +2222,19 @@
         <v>30</v>
       </c>
       <c r="G26" t="s">
-        <v>42</v>
-      </c>
-      <c r="H26" s="2">
+        <v>43</v>
+      </c>
+      <c r="H26" s="1">
         <v>46076</v>
       </c>
       <c r="I26" t="s">
-        <v>51</v>
+        <v>52</v>
       </c>
       <c r="N26" t="s">
-        <v>87</v>
+        <v>88</v>
       </c>
       <c r="O26" t="s">
-        <v>121</v>
+        <v>122</v>
       </c>
       <c r="P26">
         <v>1000</v>
@@ -2269,15 +2246,15 @@
         <v>169</v>
       </c>
       <c r="S26" t="s">
-        <v>171</v>
+        <v>172</v>
       </c>
       <c r="T26" t="s">
-        <v>176</v>
+        <v>177</v>
       </c>
       <c r="U26" t="s">
         <v>28</v>
       </c>
-      <c r="V26" s="2">
+      <c r="V26" s="1">
         <v>46079</v>
       </c>
     </row>
@@ -2301,36 +2278,36 @@
         <v>30</v>
       </c>
       <c r="J27" t="s">
-        <v>62</v>
+        <v>63</v>
       </c>
       <c r="K27" t="s">
-        <v>71</v>
+        <v>72</v>
       </c>
       <c r="N27" t="s">
-        <v>83</v>
+        <v>84</v>
       </c>
       <c r="O27" t="s">
-        <v>122</v>
+        <v>123</v>
       </c>
       <c r="P27">
         <v>100000</v>
       </c>
       <c r="Q27" t="s">
-        <v>166</v>
+        <v>168</v>
       </c>
       <c r="R27" t="s">
         <v>169</v>
       </c>
       <c r="S27" t="s">
-        <v>171</v>
+        <v>172</v>
       </c>
       <c r="T27" t="s">
-        <v>175</v>
+        <v>176</v>
       </c>
       <c r="U27" t="s">
-        <v>180</v>
-      </c>
-      <c r="V27" s="2">
+        <v>181</v>
+      </c>
+      <c r="V27" s="1">
         <v>46291</v>
       </c>
     </row>
@@ -2354,22 +2331,22 @@
         <v>32</v>
       </c>
       <c r="G28" t="s">
-        <v>42</v>
-      </c>
-      <c r="H28" s="2">
+        <v>43</v>
+      </c>
+      <c r="H28" s="1">
         <v>46199</v>
       </c>
       <c r="I28" t="s">
-        <v>52</v>
+        <v>53</v>
       </c>
       <c r="J28" t="s">
-        <v>65</v>
+        <v>66</v>
       </c>
       <c r="N28" t="s">
-        <v>84</v>
+        <v>85</v>
       </c>
       <c r="O28" t="s">
-        <v>123</v>
+        <v>124</v>
       </c>
       <c r="P28">
         <v>150000</v>
@@ -2378,18 +2355,18 @@
         <v>167</v>
       </c>
       <c r="R28" t="s">
-        <v>168</v>
+        <v>170</v>
       </c>
       <c r="S28" t="s">
-        <v>171</v>
+        <v>172</v>
       </c>
       <c r="T28" t="s">
-        <v>176</v>
+        <v>177</v>
       </c>
       <c r="U28" t="s">
-        <v>180</v>
-      </c>
-      <c r="V28" s="2">
+        <v>181</v>
+      </c>
+      <c r="V28" s="1">
         <v>46199</v>
       </c>
     </row>
@@ -2413,22 +2390,22 @@
         <v>32</v>
       </c>
       <c r="G29" t="s">
-        <v>42</v>
-      </c>
-      <c r="H29" s="2">
+        <v>43</v>
+      </c>
+      <c r="H29" s="1">
         <v>46199</v>
       </c>
       <c r="I29" t="s">
-        <v>52</v>
+        <v>53</v>
       </c>
       <c r="J29" t="s">
-        <v>65</v>
+        <v>66</v>
       </c>
       <c r="N29" t="s">
-        <v>84</v>
+        <v>85</v>
       </c>
       <c r="O29" t="s">
-        <v>124</v>
+        <v>125</v>
       </c>
       <c r="P29">
         <v>150000</v>
@@ -2437,18 +2414,18 @@
         <v>167</v>
       </c>
       <c r="R29" t="s">
-        <v>168</v>
+        <v>170</v>
       </c>
       <c r="S29" t="s">
-        <v>171</v>
+        <v>172</v>
       </c>
       <c r="T29" t="s">
-        <v>176</v>
+        <v>177</v>
       </c>
       <c r="U29" t="s">
-        <v>180</v>
-      </c>
-      <c r="V29" s="2">
+        <v>181</v>
+      </c>
+      <c r="V29" s="1">
         <v>46199</v>
       </c>
     </row>
@@ -2472,22 +2449,22 @@
         <v>33</v>
       </c>
       <c r="G30" t="s">
-        <v>42</v>
-      </c>
-      <c r="H30" s="2">
+        <v>43</v>
+      </c>
+      <c r="H30" s="1">
         <v>46199</v>
       </c>
       <c r="I30" t="s">
-        <v>53</v>
+        <v>54</v>
       </c>
       <c r="J30" t="s">
-        <v>65</v>
+        <v>66</v>
       </c>
       <c r="N30" t="s">
-        <v>84</v>
+        <v>85</v>
       </c>
       <c r="O30" t="s">
-        <v>125</v>
+        <v>126</v>
       </c>
       <c r="P30">
         <v>18462.36</v>
@@ -2496,18 +2473,18 @@
         <v>167</v>
       </c>
       <c r="R30" t="s">
-        <v>168</v>
+        <v>170</v>
       </c>
       <c r="S30" t="s">
-        <v>171</v>
+        <v>172</v>
       </c>
       <c r="T30" t="s">
-        <v>176</v>
+        <v>177</v>
       </c>
       <c r="U30" t="s">
-        <v>180</v>
-      </c>
-      <c r="V30" s="2">
+        <v>181</v>
+      </c>
+      <c r="V30" s="1">
         <v>46199</v>
       </c>
     </row>
@@ -2531,22 +2508,22 @@
         <v>32</v>
       </c>
       <c r="G31" t="s">
-        <v>42</v>
-      </c>
-      <c r="H31" s="2">
+        <v>43</v>
+      </c>
+      <c r="H31" s="1">
         <v>46199</v>
       </c>
       <c r="I31" t="s">
-        <v>52</v>
+        <v>53</v>
       </c>
       <c r="J31" t="s">
-        <v>65</v>
+        <v>66</v>
       </c>
       <c r="N31" t="s">
-        <v>84</v>
+        <v>85</v>
       </c>
       <c r="O31" t="s">
-        <v>125</v>
+        <v>126</v>
       </c>
       <c r="P31">
         <v>324166.14</v>
@@ -2555,18 +2532,18 @@
         <v>167</v>
       </c>
       <c r="R31" t="s">
-        <v>168</v>
+        <v>170</v>
       </c>
       <c r="S31" t="s">
-        <v>171</v>
+        <v>172</v>
       </c>
       <c r="T31" t="s">
-        <v>176</v>
+        <v>177</v>
       </c>
       <c r="U31" t="s">
-        <v>180</v>
-      </c>
-      <c r="V31" s="2">
+        <v>181</v>
+      </c>
+      <c r="V31" s="1">
         <v>46199</v>
       </c>
     </row>
@@ -2590,13 +2567,13 @@
         <v>30</v>
       </c>
       <c r="K32" t="s">
-        <v>72</v>
+        <v>73</v>
       </c>
       <c r="N32" t="s">
-        <v>84</v>
+        <v>85</v>
       </c>
       <c r="O32" t="s">
-        <v>126</v>
+        <v>127</v>
       </c>
       <c r="P32">
         <v>30000</v>
@@ -2605,18 +2582,18 @@
         <v>167</v>
       </c>
       <c r="R32" t="s">
-        <v>168</v>
+        <v>170</v>
       </c>
       <c r="S32" t="s">
-        <v>171</v>
+        <v>172</v>
       </c>
       <c r="T32" t="s">
-        <v>176</v>
+        <v>177</v>
       </c>
       <c r="U32" t="s">
-        <v>180</v>
-      </c>
-      <c r="V32" s="2">
+        <v>181</v>
+      </c>
+      <c r="V32" s="1">
         <v>46291</v>
       </c>
     </row>
@@ -2640,22 +2617,22 @@
         <v>30</v>
       </c>
       <c r="G33" t="s">
-        <v>42</v>
-      </c>
-      <c r="H33" s="2">
+        <v>43</v>
+      </c>
+      <c r="H33" s="1">
         <v>46191</v>
       </c>
       <c r="I33" t="s">
-        <v>54</v>
+        <v>55</v>
       </c>
       <c r="J33" t="s">
-        <v>66</v>
+        <v>67</v>
       </c>
       <c r="N33" t="s">
-        <v>84</v>
+        <v>85</v>
       </c>
       <c r="O33" t="s">
-        <v>127</v>
+        <v>128</v>
       </c>
       <c r="P33">
         <v>1496713.48</v>
@@ -2664,18 +2641,18 @@
         <v>167</v>
       </c>
       <c r="R33" t="s">
-        <v>168</v>
+        <v>170</v>
       </c>
       <c r="S33" t="s">
-        <v>171</v>
+        <v>172</v>
       </c>
       <c r="T33" t="s">
-        <v>177</v>
+        <v>178</v>
       </c>
       <c r="U33" t="s">
-        <v>180</v>
-      </c>
-      <c r="V33" s="2">
+        <v>181</v>
+      </c>
+      <c r="V33" s="1">
         <v>46199</v>
       </c>
     </row>
@@ -2699,19 +2676,19 @@
         <v>31</v>
       </c>
       <c r="G34" t="s">
-        <v>42</v>
-      </c>
-      <c r="H34" s="2">
+        <v>43</v>
+      </c>
+      <c r="H34" s="1">
         <v>46119</v>
       </c>
       <c r="I34" t="s">
-        <v>49</v>
+        <v>50</v>
       </c>
       <c r="N34" t="s">
-        <v>84</v>
+        <v>85</v>
       </c>
       <c r="O34" t="s">
-        <v>127</v>
+        <v>128</v>
       </c>
       <c r="P34">
         <v>207789.52</v>
@@ -2720,18 +2697,18 @@
         <v>167</v>
       </c>
       <c r="R34" t="s">
-        <v>168</v>
+        <v>170</v>
       </c>
       <c r="S34" t="s">
-        <v>171</v>
+        <v>172</v>
       </c>
       <c r="T34" t="s">
-        <v>177</v>
+        <v>178</v>
       </c>
       <c r="U34" t="s">
-        <v>180</v>
-      </c>
-      <c r="V34" s="2">
+        <v>181</v>
+      </c>
+      <c r="V34" s="1">
         <v>46138</v>
       </c>
     </row>
@@ -2755,19 +2732,19 @@
         <v>30</v>
       </c>
       <c r="G35" t="s">
-        <v>42</v>
-      </c>
-      <c r="H35" s="2">
+        <v>43</v>
+      </c>
+      <c r="H35" s="1">
         <v>46213</v>
       </c>
       <c r="I35" t="s">
-        <v>55</v>
+        <v>56</v>
       </c>
       <c r="N35" t="s">
-        <v>87</v>
+        <v>88</v>
       </c>
       <c r="O35" t="s">
-        <v>128</v>
+        <v>129</v>
       </c>
       <c r="P35">
         <v>962290.8</v>
@@ -2779,15 +2756,15 @@
         <v>169</v>
       </c>
       <c r="S35" t="s">
-        <v>171</v>
+        <v>172</v>
       </c>
       <c r="T35" t="s">
-        <v>176</v>
+        <v>177</v>
       </c>
       <c r="U35" t="s">
         <v>28</v>
       </c>
-      <c r="V35" s="2">
+      <c r="V35" s="1">
         <v>46229</v>
       </c>
     </row>
@@ -2811,19 +2788,19 @@
         <v>34</v>
       </c>
       <c r="G36" t="s">
-        <v>42</v>
-      </c>
-      <c r="H36" s="2">
+        <v>43</v>
+      </c>
+      <c r="H36" s="1">
         <v>46175</v>
       </c>
       <c r="I36" t="s">
-        <v>56</v>
+        <v>57</v>
       </c>
       <c r="N36" t="s">
-        <v>87</v>
+        <v>88</v>
       </c>
       <c r="O36" t="s">
-        <v>128</v>
+        <v>129</v>
       </c>
       <c r="P36">
         <v>798776.97</v>
@@ -2832,18 +2809,18 @@
         <v>167</v>
       </c>
       <c r="R36" t="s">
-        <v>168</v>
+        <v>170</v>
       </c>
       <c r="S36" t="s">
-        <v>171</v>
+        <v>172</v>
       </c>
       <c r="T36" t="s">
-        <v>176</v>
+        <v>177</v>
       </c>
       <c r="U36" t="s">
         <v>28</v>
       </c>
-      <c r="V36" s="2">
+      <c r="V36" s="1">
         <v>46199</v>
       </c>
     </row>
@@ -2867,19 +2844,19 @@
         <v>30</v>
       </c>
       <c r="G37" t="s">
-        <v>42</v>
-      </c>
-      <c r="H37" s="2">
+        <v>43</v>
+      </c>
+      <c r="H37" s="1">
         <v>46213</v>
       </c>
       <c r="I37" t="s">
-        <v>55</v>
+        <v>56</v>
       </c>
       <c r="N37" t="s">
-        <v>87</v>
+        <v>88</v>
       </c>
       <c r="O37" t="s">
-        <v>128</v>
+        <v>129</v>
       </c>
       <c r="P37">
         <v>1530656.62</v>
@@ -2891,15 +2868,15 @@
         <v>169</v>
       </c>
       <c r="S37" t="s">
-        <v>171</v>
+        <v>172</v>
       </c>
       <c r="T37" t="s">
-        <v>176</v>
+        <v>177</v>
       </c>
       <c r="U37" t="s">
         <v>28</v>
       </c>
-      <c r="V37" s="2">
+      <c r="V37" s="1">
         <v>46229</v>
       </c>
     </row>
@@ -2923,19 +2900,19 @@
         <v>35</v>
       </c>
       <c r="G38" t="s">
-        <v>42</v>
-      </c>
-      <c r="H38" s="2">
+        <v>43</v>
+      </c>
+      <c r="H38" s="1">
         <v>46199</v>
       </c>
       <c r="I38" t="s">
-        <v>57</v>
+        <v>58</v>
       </c>
       <c r="N38" t="s">
-        <v>87</v>
+        <v>88</v>
       </c>
       <c r="O38" t="s">
-        <v>128</v>
+        <v>129</v>
       </c>
       <c r="P38">
         <v>72958.08</v>
@@ -2947,15 +2924,15 @@
         <v>169</v>
       </c>
       <c r="S38" t="s">
-        <v>171</v>
+        <v>172</v>
       </c>
       <c r="T38" t="s">
-        <v>176</v>
+        <v>177</v>
       </c>
       <c r="U38" t="s">
         <v>28</v>
       </c>
-      <c r="V38" s="2">
+      <c r="V38" s="1">
         <v>46199</v>
       </c>
     </row>
@@ -2979,19 +2956,19 @@
         <v>36</v>
       </c>
       <c r="G39" t="s">
-        <v>42</v>
-      </c>
-      <c r="H39" s="2">
+        <v>43</v>
+      </c>
+      <c r="H39" s="1">
         <v>46199</v>
       </c>
       <c r="I39" t="s">
-        <v>57</v>
+        <v>58</v>
       </c>
       <c r="N39" t="s">
-        <v>87</v>
+        <v>88</v>
       </c>
       <c r="O39" t="s">
-        <v>128</v>
+        <v>129</v>
       </c>
       <c r="P39">
         <v>8916</v>
@@ -3003,15 +2980,15 @@
         <v>169</v>
       </c>
       <c r="S39" t="s">
-        <v>171</v>
+        <v>172</v>
       </c>
       <c r="T39" t="s">
-        <v>176</v>
+        <v>177</v>
       </c>
       <c r="U39" t="s">
         <v>28</v>
       </c>
-      <c r="V39" s="2">
+      <c r="V39" s="1">
         <v>46199</v>
       </c>
     </row>
@@ -3035,19 +3012,19 @@
         <v>37</v>
       </c>
       <c r="G40" t="s">
-        <v>42</v>
-      </c>
-      <c r="H40" s="2">
+        <v>43</v>
+      </c>
+      <c r="H40" s="1">
         <v>46204</v>
       </c>
       <c r="I40" t="s">
-        <v>57</v>
+        <v>58</v>
       </c>
       <c r="N40" t="s">
-        <v>87</v>
+        <v>88</v>
       </c>
       <c r="O40" t="s">
-        <v>128</v>
+        <v>129</v>
       </c>
       <c r="P40">
         <v>425178.5</v>
@@ -3059,15 +3036,15 @@
         <v>169</v>
       </c>
       <c r="S40" t="s">
-        <v>171</v>
+        <v>172</v>
       </c>
       <c r="T40" t="s">
-        <v>176</v>
+        <v>177</v>
       </c>
       <c r="U40" t="s">
         <v>28</v>
       </c>
-      <c r="V40" s="2">
+      <c r="V40" s="1">
         <v>46229</v>
       </c>
     </row>
@@ -3091,19 +3068,19 @@
         <v>34</v>
       </c>
       <c r="G41" t="s">
-        <v>42</v>
-      </c>
-      <c r="H41" s="2">
+        <v>43</v>
+      </c>
+      <c r="H41" s="1">
         <v>46244</v>
       </c>
       <c r="I41" t="s">
-        <v>58</v>
+        <v>59</v>
       </c>
       <c r="N41" t="s">
-        <v>87</v>
+        <v>88</v>
       </c>
       <c r="O41" t="s">
-        <v>128</v>
+        <v>129</v>
       </c>
       <c r="P41">
         <v>1223.03</v>
@@ -3115,15 +3092,15 @@
         <v>169</v>
       </c>
       <c r="S41" t="s">
-        <v>171</v>
+        <v>172</v>
       </c>
       <c r="T41" t="s">
-        <v>176</v>
+        <v>177</v>
       </c>
       <c r="U41" t="s">
         <v>28</v>
       </c>
-      <c r="V41" s="2">
+      <c r="V41" s="1">
         <v>46199</v>
       </c>
     </row>
@@ -3144,13 +3121,13 @@
         <v>29</v>
       </c>
       <c r="G42" t="s">
-        <v>41</v>
+        <v>42</v>
       </c>
       <c r="N42" t="s">
-        <v>87</v>
+        <v>88</v>
       </c>
       <c r="O42" t="s">
-        <v>129</v>
+        <v>130</v>
       </c>
       <c r="Q42" t="s">
         <v>167</v>
@@ -3159,15 +3136,15 @@
         <v>169</v>
       </c>
       <c r="S42" t="s">
-        <v>172</v>
+        <v>173</v>
       </c>
       <c r="T42" t="s">
-        <v>176</v>
+        <v>177</v>
       </c>
       <c r="U42" t="s">
         <v>28</v>
       </c>
-      <c r="V42" s="2">
+      <c r="V42" s="1">
         <v>46260</v>
       </c>
     </row>
@@ -3191,19 +3168,19 @@
         <v>30</v>
       </c>
       <c r="G43" t="s">
-        <v>42</v>
-      </c>
-      <c r="H43" s="2">
+        <v>43</v>
+      </c>
+      <c r="H43" s="1">
         <v>46191</v>
       </c>
       <c r="I43" t="s">
-        <v>59</v>
+        <v>60</v>
       </c>
       <c r="N43" t="s">
-        <v>85</v>
+        <v>86</v>
       </c>
       <c r="O43" t="s">
-        <v>130</v>
+        <v>131</v>
       </c>
       <c r="P43">
         <v>400000</v>
@@ -3215,15 +3192,15 @@
         <v>169</v>
       </c>
       <c r="S43" t="s">
-        <v>171</v>
+        <v>172</v>
       </c>
       <c r="T43" t="s">
-        <v>176</v>
+        <v>177</v>
       </c>
       <c r="U43" t="s">
         <v>28</v>
       </c>
-      <c r="V43" s="2">
+      <c r="V43" s="1">
         <v>46199</v>
       </c>
     </row>
@@ -3247,19 +3224,19 @@
         <v>30</v>
       </c>
       <c r="G44" t="s">
-        <v>42</v>
-      </c>
-      <c r="H44" s="2">
+        <v>43</v>
+      </c>
+      <c r="H44" s="1">
         <v>46191</v>
       </c>
       <c r="I44" t="s">
-        <v>59</v>
+        <v>60</v>
       </c>
       <c r="N44" t="s">
-        <v>85</v>
+        <v>86</v>
       </c>
       <c r="O44" t="s">
-        <v>131</v>
+        <v>132</v>
       </c>
       <c r="P44">
         <v>400000</v>
@@ -3271,15 +3248,15 @@
         <v>169</v>
       </c>
       <c r="S44" t="s">
-        <v>171</v>
+        <v>172</v>
       </c>
       <c r="T44" t="s">
-        <v>176</v>
+        <v>177</v>
       </c>
       <c r="U44" t="s">
         <v>28</v>
       </c>
-      <c r="V44" s="2">
+      <c r="V44" s="1">
         <v>46199</v>
       </c>
     </row>
@@ -3303,22 +3280,22 @@
         <v>30</v>
       </c>
       <c r="G45" t="s">
-        <v>42</v>
-      </c>
-      <c r="H45" s="2">
+        <v>43</v>
+      </c>
+      <c r="H45" s="1">
         <v>46213</v>
       </c>
       <c r="I45" t="s">
-        <v>54</v>
+        <v>55</v>
       </c>
       <c r="J45" t="s">
-        <v>67</v>
+        <v>68</v>
       </c>
       <c r="N45" t="s">
-        <v>84</v>
+        <v>85</v>
       </c>
       <c r="O45" t="s">
-        <v>132</v>
+        <v>133</v>
       </c>
       <c r="P45">
         <v>173846.38</v>
@@ -3327,18 +3304,18 @@
         <v>167</v>
       </c>
       <c r="R45" t="s">
-        <v>168</v>
+        <v>170</v>
       </c>
       <c r="S45" t="s">
-        <v>171</v>
+        <v>172</v>
       </c>
       <c r="T45" t="s">
-        <v>177</v>
+        <v>178</v>
       </c>
       <c r="U45" t="s">
-        <v>180</v>
-      </c>
-      <c r="V45" s="2">
+        <v>181</v>
+      </c>
+      <c r="V45" s="1">
         <v>46229</v>
       </c>
     </row>
@@ -3362,19 +3339,19 @@
         <v>33</v>
       </c>
       <c r="G46" t="s">
-        <v>42</v>
-      </c>
-      <c r="H46" s="2">
+        <v>43</v>
+      </c>
+      <c r="H46" s="1">
         <v>46210</v>
       </c>
       <c r="I46" t="s">
-        <v>53</v>
+        <v>54</v>
       </c>
       <c r="N46" t="s">
-        <v>84</v>
+        <v>85</v>
       </c>
       <c r="O46" t="s">
-        <v>132</v>
+        <v>133</v>
       </c>
       <c r="P46">
         <v>1530656.62</v>
@@ -3383,18 +3360,18 @@
         <v>167</v>
       </c>
       <c r="R46" t="s">
-        <v>168</v>
+        <v>170</v>
       </c>
       <c r="S46" t="s">
-        <v>171</v>
+        <v>172</v>
       </c>
       <c r="T46" t="s">
-        <v>177</v>
+        <v>178</v>
       </c>
       <c r="U46" t="s">
-        <v>180</v>
-      </c>
-      <c r="V46" s="2">
+        <v>181</v>
+      </c>
+      <c r="V46" s="1">
         <v>46229</v>
       </c>
     </row>
@@ -3418,10 +3395,10 @@
         <v>30</v>
       </c>
       <c r="N47" t="s">
-        <v>86</v>
+        <v>87</v>
       </c>
       <c r="O47" t="s">
-        <v>133</v>
+        <v>134</v>
       </c>
       <c r="P47">
         <v>1000000</v>
@@ -3433,15 +3410,15 @@
         <v>169</v>
       </c>
       <c r="S47" t="s">
-        <v>171</v>
+        <v>172</v>
       </c>
       <c r="T47" t="s">
-        <v>176</v>
+        <v>177</v>
       </c>
       <c r="U47" t="s">
         <v>28</v>
       </c>
-      <c r="V47" s="2">
+      <c r="V47" s="1">
         <v>46321</v>
       </c>
     </row>
@@ -3465,36 +3442,36 @@
         <v>30</v>
       </c>
       <c r="J48" t="s">
-        <v>62</v>
+        <v>63</v>
       </c>
       <c r="K48" t="s">
-        <v>71</v>
+        <v>72</v>
       </c>
       <c r="N48" t="s">
-        <v>79</v>
+        <v>80</v>
       </c>
       <c r="O48" t="s">
-        <v>134</v>
+        <v>135</v>
       </c>
       <c r="P48">
         <v>958040</v>
       </c>
       <c r="Q48" t="s">
-        <v>165</v>
+        <v>166</v>
       </c>
       <c r="R48" t="s">
         <v>169</v>
       </c>
       <c r="S48" t="s">
-        <v>171</v>
+        <v>172</v>
       </c>
       <c r="T48" t="s">
-        <v>175</v>
+        <v>176</v>
       </c>
       <c r="U48" t="s">
-        <v>180</v>
-      </c>
-      <c r="V48" s="2">
+        <v>181</v>
+      </c>
+      <c r="V48" s="1">
         <v>46291</v>
       </c>
     </row>
@@ -3518,42 +3495,42 @@
         <v>30</v>
       </c>
       <c r="G49" t="s">
-        <v>42</v>
-      </c>
-      <c r="H49" s="2">
+        <v>43</v>
+      </c>
+      <c r="H49" s="1">
         <v>46176</v>
       </c>
       <c r="I49" t="s">
-        <v>60</v>
+        <v>61</v>
       </c>
       <c r="J49" t="s">
-        <v>68</v>
+        <v>69</v>
       </c>
       <c r="N49" t="s">
-        <v>79</v>
+        <v>80</v>
       </c>
       <c r="O49" t="s">
-        <v>134</v>
+        <v>135</v>
       </c>
       <c r="P49">
         <v>41730.64</v>
       </c>
       <c r="Q49" t="s">
-        <v>165</v>
+        <v>166</v>
       </c>
       <c r="R49" t="s">
-        <v>170</v>
+        <v>171</v>
       </c>
       <c r="S49" t="s">
-        <v>171</v>
+        <v>172</v>
       </c>
       <c r="T49" t="s">
-        <v>175</v>
+        <v>176</v>
       </c>
       <c r="U49" t="s">
-        <v>180</v>
-      </c>
-      <c r="V49" s="2">
+        <v>181</v>
+      </c>
+      <c r="V49" s="1">
         <v>46199</v>
       </c>
     </row>
@@ -3577,16 +3554,16 @@
         <v>30</v>
       </c>
       <c r="J50" t="s">
-        <v>67</v>
+        <v>68</v>
       </c>
       <c r="K50" t="s">
-        <v>73</v>
+        <v>74</v>
       </c>
       <c r="N50" t="s">
-        <v>84</v>
+        <v>85</v>
       </c>
       <c r="O50" t="s">
-        <v>135</v>
+        <v>136</v>
       </c>
       <c r="P50">
         <v>1468159.32</v>
@@ -3595,18 +3572,18 @@
         <v>167</v>
       </c>
       <c r="R50" t="s">
-        <v>168</v>
+        <v>170</v>
       </c>
       <c r="S50" t="s">
-        <v>171</v>
+        <v>172</v>
       </c>
       <c r="T50" t="s">
-        <v>177</v>
+        <v>178</v>
       </c>
       <c r="U50" t="s">
-        <v>180</v>
-      </c>
-      <c r="V50" s="2">
+        <v>181</v>
+      </c>
+      <c r="V50" s="1">
         <v>46260</v>
       </c>
     </row>
@@ -3630,36 +3607,36 @@
         <v>30</v>
       </c>
       <c r="J51" t="s">
-        <v>67</v>
+        <v>68</v>
       </c>
       <c r="K51" t="s">
-        <v>74</v>
+        <v>75</v>
       </c>
       <c r="N51" t="s">
-        <v>84</v>
+        <v>85</v>
       </c>
       <c r="O51" t="s">
-        <v>136</v>
+        <v>137</v>
       </c>
       <c r="P51">
-        <v>1704503</v>
+        <v>559040.0699999999</v>
       </c>
       <c r="Q51" t="s">
         <v>167</v>
       </c>
       <c r="R51" t="s">
-        <v>168</v>
+        <v>170</v>
       </c>
       <c r="S51" t="s">
-        <v>171</v>
+        <v>172</v>
       </c>
       <c r="T51" t="s">
-        <v>177</v>
+        <v>178</v>
       </c>
       <c r="U51" t="s">
-        <v>180</v>
-      </c>
-      <c r="V51" s="2">
+        <v>181</v>
+      </c>
+      <c r="V51" s="1">
         <v>46291</v>
       </c>
     </row>
@@ -3683,13 +3660,13 @@
         <v>30</v>
       </c>
       <c r="K52" t="s">
-        <v>72</v>
+        <v>73</v>
       </c>
       <c r="N52" t="s">
-        <v>84</v>
+        <v>85</v>
       </c>
       <c r="O52" t="s">
-        <v>137</v>
+        <v>138</v>
       </c>
       <c r="P52">
         <v>1704503</v>
@@ -3698,18 +3675,18 @@
         <v>167</v>
       </c>
       <c r="R52" t="s">
-        <v>168</v>
+        <v>170</v>
       </c>
       <c r="S52" t="s">
-        <v>171</v>
+        <v>172</v>
       </c>
       <c r="T52" t="s">
-        <v>177</v>
+        <v>178</v>
       </c>
       <c r="U52" t="s">
-        <v>180</v>
-      </c>
-      <c r="V52" s="2">
+        <v>181</v>
+      </c>
+      <c r="V52" s="1">
         <v>46321</v>
       </c>
     </row>
@@ -3733,19 +3710,19 @@
         <v>38</v>
       </c>
       <c r="G53" t="s">
-        <v>42</v>
-      </c>
-      <c r="H53" s="2">
+        <v>43</v>
+      </c>
+      <c r="H53" s="1">
         <v>46227</v>
       </c>
       <c r="I53" t="s">
-        <v>61</v>
+        <v>62</v>
       </c>
       <c r="N53" t="s">
-        <v>84</v>
+        <v>85</v>
       </c>
       <c r="O53" t="s">
-        <v>135</v>
+        <v>136</v>
       </c>
       <c r="P53">
         <v>236343.68</v>
@@ -3754,80 +3731,80 @@
         <v>167</v>
       </c>
       <c r="R53" t="s">
-        <v>168</v>
+        <v>170</v>
       </c>
       <c r="S53" t="s">
-        <v>171</v>
+        <v>172</v>
       </c>
       <c r="T53" t="s">
-        <v>177</v>
+        <v>178</v>
       </c>
       <c r="U53" t="s">
-        <v>180</v>
-      </c>
-      <c r="V53" s="2">
+        <v>181</v>
+      </c>
+      <c r="V53" s="1">
         <v>46229</v>
       </c>
     </row>
     <row r="54" spans="1:22">
       <c r="A54">
-        <v>18140</v>
+        <v>17764</v>
       </c>
       <c r="B54" t="s">
         <v>22</v>
       </c>
-      <c r="C54" t="s">
-        <v>22</v>
-      </c>
       <c r="D54" t="s">
-        <v>24</v>
+        <v>26</v>
       </c>
       <c r="E54" t="s">
         <v>28</v>
       </c>
       <c r="F54" t="s">
-        <v>30</v>
-      </c>
-      <c r="J54" t="s">
-        <v>62</v>
-      </c>
-      <c r="K54" t="s">
-        <v>75</v>
+        <v>39</v>
+      </c>
+      <c r="G54" t="s">
+        <v>43</v>
+      </c>
+      <c r="H54" s="1">
+        <v>46280</v>
+      </c>
+      <c r="I54" t="s">
+        <v>54</v>
       </c>
       <c r="N54" t="s">
-        <v>84</v>
+        <v>85</v>
       </c>
       <c r="O54" t="s">
-        <v>138</v>
+        <v>137</v>
       </c>
       <c r="P54">
-        <v>1295422.28</v>
+        <v>1145462.93</v>
       </c>
       <c r="Q54" t="s">
         <v>167</v>
       </c>
       <c r="R54" t="s">
-        <v>168</v>
+        <v>170</v>
       </c>
       <c r="S54" t="s">
-        <v>171</v>
+        <v>172</v>
       </c>
       <c r="T54" t="s">
-        <v>177</v>
+        <v>178</v>
       </c>
       <c r="U54" t="s">
-        <v>180</v>
-      </c>
-      <c r="V54" s="2">
-        <v>46352</v>
+        <v>181</v>
+      </c>
+      <c r="V54" s="1">
+        <v>46291</v>
       </c>
     </row>
     <row r="55" spans="1:22">
       <c r="A55">
-        <v>19240</v>
+        <v>18140</v>
       </c>
       <c r="B55" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="C55" t="s">
         <v>22</v>
@@ -3839,45 +3816,45 @@
         <v>28</v>
       </c>
       <c r="F55" t="s">
-        <v>39</v>
+        <v>30</v>
       </c>
       <c r="J55" t="s">
-        <v>62</v>
+        <v>63</v>
       </c>
       <c r="K55" t="s">
-        <v>71</v>
+        <v>76</v>
       </c>
       <c r="N55" t="s">
-        <v>88</v>
+        <v>85</v>
       </c>
       <c r="O55" t="s">
         <v>139</v>
       </c>
       <c r="P55">
-        <v>500000</v>
+        <v>1295422.28</v>
       </c>
       <c r="Q55" t="s">
         <v>167</v>
       </c>
       <c r="R55" t="s">
-        <v>168</v>
+        <v>170</v>
       </c>
       <c r="S55" t="s">
-        <v>173</v>
+        <v>172</v>
       </c>
       <c r="T55" t="s">
         <v>178</v>
       </c>
       <c r="U55" t="s">
-        <v>180</v>
-      </c>
-      <c r="V55" s="2">
-        <v>46321</v>
+        <v>181</v>
+      </c>
+      <c r="V55" s="1">
+        <v>46352</v>
       </c>
     </row>
     <row r="56" spans="1:22">
       <c r="A56">
-        <v>19241</v>
+        <v>19240</v>
       </c>
       <c r="B56" t="s">
         <v>23</v>
@@ -3886,48 +3863,51 @@
         <v>22</v>
       </c>
       <c r="D56" t="s">
-        <v>27</v>
+        <v>24</v>
       </c>
       <c r="E56" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="F56" t="s">
-        <v>39</v>
-      </c>
-      <c r="G56" t="s">
-        <v>43</v>
+        <v>40</v>
+      </c>
+      <c r="J56" t="s">
+        <v>63</v>
+      </c>
+      <c r="K56" t="s">
+        <v>72</v>
       </c>
       <c r="N56" t="s">
-        <v>88</v>
+        <v>89</v>
       </c>
       <c r="O56" t="s">
-        <v>139</v>
+        <v>140</v>
       </c>
       <c r="P56">
-        <v>5000000</v>
+        <v>1962977.67</v>
       </c>
       <c r="Q56" t="s">
         <v>167</v>
       </c>
       <c r="R56" t="s">
-        <v>168</v>
+        <v>170</v>
       </c>
       <c r="S56" t="s">
-        <v>173</v>
+        <v>174</v>
       </c>
       <c r="T56" t="s">
-        <v>178</v>
+        <v>179</v>
       </c>
       <c r="U56" t="s">
-        <v>180</v>
-      </c>
-      <c r="V56" s="2">
+        <v>181</v>
+      </c>
+      <c r="V56" s="1">
         <v>46321</v>
       </c>
     </row>
     <row r="57" spans="1:22">
       <c r="A57">
-        <v>19260</v>
+        <v>19241</v>
       </c>
       <c r="B57" t="s">
         <v>23</v>
@@ -3942,36 +3922,39 @@
         <v>29</v>
       </c>
       <c r="G57" t="s">
-        <v>41</v>
+        <v>44</v>
       </c>
       <c r="N57" t="s">
-        <v>88</v>
+        <v>89</v>
       </c>
       <c r="O57" t="s">
         <v>140</v>
       </c>
+      <c r="P57">
+        <v>2497091</v>
+      </c>
       <c r="Q57" t="s">
         <v>167</v>
       </c>
       <c r="R57" t="s">
-        <v>168</v>
+        <v>170</v>
       </c>
       <c r="S57" t="s">
-        <v>173</v>
+        <v>174</v>
       </c>
       <c r="T57" t="s">
-        <v>178</v>
+        <v>179</v>
       </c>
       <c r="U57" t="s">
-        <v>180</v>
-      </c>
-      <c r="V57" s="2">
-        <v>46049</v>
+        <v>181</v>
+      </c>
+      <c r="V57" s="1">
+        <v>46321</v>
       </c>
     </row>
     <row r="58" spans="1:22">
       <c r="A58">
-        <v>19600</v>
+        <v>19260</v>
       </c>
       <c r="B58" t="s">
         <v>23</v>
@@ -3986,10 +3969,10 @@
         <v>29</v>
       </c>
       <c r="G58" t="s">
-        <v>41</v>
+        <v>42</v>
       </c>
       <c r="N58" t="s">
-        <v>88</v>
+        <v>89</v>
       </c>
       <c r="O58" t="s">
         <v>141</v>
@@ -3998,21 +3981,24 @@
         <v>167</v>
       </c>
       <c r="R58" t="s">
-        <v>168</v>
+        <v>170</v>
       </c>
       <c r="S58" t="s">
-        <v>173</v>
+        <v>174</v>
       </c>
       <c r="T58" t="s">
-        <v>178</v>
+        <v>179</v>
       </c>
       <c r="U58" t="s">
-        <v>180</v>
+        <v>181</v>
+      </c>
+      <c r="V58" s="1">
+        <v>46049</v>
       </c>
     </row>
     <row r="59" spans="1:22">
       <c r="A59">
-        <v>19620</v>
+        <v>19600</v>
       </c>
       <c r="B59" t="s">
         <v>23</v>
@@ -4027,10 +4013,10 @@
         <v>29</v>
       </c>
       <c r="G59" t="s">
-        <v>41</v>
+        <v>42</v>
       </c>
       <c r="N59" t="s">
-        <v>88</v>
+        <v>89</v>
       </c>
       <c r="O59" t="s">
         <v>142</v>
@@ -4039,24 +4025,24 @@
         <v>167</v>
       </c>
       <c r="R59" t="s">
-        <v>168</v>
+        <v>170</v>
       </c>
       <c r="S59" t="s">
-        <v>173</v>
+        <v>174</v>
       </c>
       <c r="T59" t="s">
-        <v>178</v>
+        <v>179</v>
       </c>
       <c r="U59" t="s">
-        <v>180</v>
+        <v>181</v>
       </c>
     </row>
     <row r="60" spans="1:22">
       <c r="A60">
-        <v>23120</v>
+        <v>19620</v>
       </c>
       <c r="B60" t="s">
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="C60" t="s">
         <v>22</v>
@@ -4067,37 +4053,34 @@
       <c r="E60" t="s">
         <v>29</v>
       </c>
+      <c r="G60" t="s">
+        <v>42</v>
+      </c>
       <c r="N60" t="s">
         <v>89</v>
       </c>
       <c r="O60" t="s">
         <v>143</v>
       </c>
-      <c r="P60">
-        <v>9389.959999999999</v>
-      </c>
       <c r="Q60" t="s">
-        <v>165</v>
+        <v>167</v>
       </c>
       <c r="R60" t="s">
         <v>170</v>
       </c>
       <c r="S60" t="s">
-        <v>172</v>
+        <v>174</v>
       </c>
       <c r="T60" t="s">
-        <v>175</v>
+        <v>179</v>
       </c>
       <c r="U60" t="s">
-        <v>180</v>
-      </c>
-      <c r="V60" s="2">
-        <v>46107</v>
+        <v>181</v>
       </c>
     </row>
     <row r="61" spans="1:22">
       <c r="A61">
-        <v>23160</v>
+        <v>23120</v>
       </c>
       <c r="B61" t="s">
         <v>22</v>
@@ -4118,30 +4101,30 @@
         <v>144</v>
       </c>
       <c r="P61">
-        <v>7204.82</v>
+        <v>9389.959999999999</v>
       </c>
       <c r="Q61" t="s">
-        <v>165</v>
+        <v>166</v>
       </c>
       <c r="R61" t="s">
-        <v>170</v>
+        <v>171</v>
       </c>
       <c r="S61" t="s">
-        <v>172</v>
+        <v>173</v>
       </c>
       <c r="T61" t="s">
-        <v>175</v>
+        <v>176</v>
       </c>
       <c r="U61" t="s">
-        <v>180</v>
-      </c>
-      <c r="V61" s="2">
+        <v>181</v>
+      </c>
+      <c r="V61" s="1">
         <v>46107</v>
       </c>
     </row>
     <row r="62" spans="1:22">
       <c r="A62">
-        <v>23100</v>
+        <v>23160</v>
       </c>
       <c r="B62" t="s">
         <v>22</v>
@@ -4162,30 +4145,30 @@
         <v>145</v>
       </c>
       <c r="P62">
-        <v>4227.84</v>
+        <v>7204.82</v>
       </c>
       <c r="Q62" t="s">
-        <v>165</v>
+        <v>166</v>
       </c>
       <c r="R62" t="s">
-        <v>170</v>
+        <v>171</v>
       </c>
       <c r="S62" t="s">
-        <v>172</v>
+        <v>173</v>
       </c>
       <c r="T62" t="s">
-        <v>175</v>
+        <v>176</v>
       </c>
       <c r="U62" t="s">
-        <v>180</v>
-      </c>
-      <c r="V62" s="2">
+        <v>181</v>
+      </c>
+      <c r="V62" s="1">
         <v>46107</v>
       </c>
     </row>
     <row r="63" spans="1:22">
       <c r="A63">
-        <v>23080</v>
+        <v>23100</v>
       </c>
       <c r="B63" t="s">
         <v>22</v>
@@ -4206,30 +4189,30 @@
         <v>146</v>
       </c>
       <c r="P63">
-        <v>4064.54</v>
+        <v>4227.84</v>
       </c>
       <c r="Q63" t="s">
-        <v>167</v>
+        <v>166</v>
       </c>
       <c r="R63" t="s">
-        <v>170</v>
+        <v>171</v>
       </c>
       <c r="S63" t="s">
-        <v>172</v>
+        <v>173</v>
       </c>
       <c r="T63" t="s">
-        <v>175</v>
+        <v>176</v>
       </c>
       <c r="U63" t="s">
-        <v>180</v>
-      </c>
-      <c r="V63" s="2">
+        <v>181</v>
+      </c>
+      <c r="V63" s="1">
         <v>46107</v>
       </c>
     </row>
     <row r="64" spans="1:22">
       <c r="A64">
-        <v>23180</v>
+        <v>23080</v>
       </c>
       <c r="B64" t="s">
         <v>22</v>
@@ -4247,33 +4230,33 @@
         <v>93</v>
       </c>
       <c r="O64" t="s">
-        <v>145</v>
+        <v>147</v>
       </c>
       <c r="P64">
-        <v>3662.66</v>
+        <v>4064.54</v>
       </c>
       <c r="Q64" t="s">
-        <v>165</v>
+        <v>167</v>
       </c>
       <c r="R64" t="s">
-        <v>170</v>
+        <v>171</v>
       </c>
       <c r="S64" t="s">
-        <v>172</v>
+        <v>173</v>
       </c>
       <c r="T64" t="s">
-        <v>175</v>
+        <v>176</v>
       </c>
       <c r="U64" t="s">
-        <v>180</v>
-      </c>
-      <c r="V64" s="2">
+        <v>181</v>
+      </c>
+      <c r="V64" s="1">
         <v>46107</v>
       </c>
     </row>
     <row r="65" spans="1:22">
       <c r="A65">
-        <v>23140</v>
+        <v>23180</v>
       </c>
       <c r="B65" t="s">
         <v>22</v>
@@ -4291,33 +4274,33 @@
         <v>94</v>
       </c>
       <c r="O65" t="s">
-        <v>147</v>
+        <v>146</v>
       </c>
       <c r="P65">
-        <v>1163.64</v>
+        <v>3662.66</v>
       </c>
       <c r="Q65" t="s">
         <v>166</v>
       </c>
       <c r="R65" t="s">
-        <v>170</v>
+        <v>171</v>
       </c>
       <c r="S65" t="s">
-        <v>172</v>
+        <v>173</v>
       </c>
       <c r="T65" t="s">
-        <v>175</v>
+        <v>176</v>
       </c>
       <c r="U65" t="s">
-        <v>180</v>
-      </c>
-      <c r="V65" s="2">
+        <v>181</v>
+      </c>
+      <c r="V65" s="1">
         <v>46107</v>
       </c>
     </row>
     <row r="66" spans="1:22">
       <c r="A66">
-        <v>23640</v>
+        <v>23140</v>
       </c>
       <c r="B66" t="s">
         <v>22</v>
@@ -4332,36 +4315,36 @@
         <v>29</v>
       </c>
       <c r="N66" t="s">
-        <v>80</v>
+        <v>95</v>
       </c>
       <c r="O66" t="s">
         <v>148</v>
       </c>
       <c r="P66">
-        <v>120000</v>
+        <v>1163.64</v>
       </c>
       <c r="Q66" t="s">
-        <v>165</v>
+        <v>168</v>
       </c>
       <c r="R66" t="s">
-        <v>168</v>
+        <v>171</v>
       </c>
       <c r="S66" t="s">
-        <v>172</v>
+        <v>173</v>
       </c>
       <c r="T66" t="s">
-        <v>175</v>
+        <v>176</v>
       </c>
       <c r="U66" t="s">
-        <v>28</v>
-      </c>
-      <c r="V66" s="2">
-        <v>46168</v>
+        <v>181</v>
+      </c>
+      <c r="V66" s="1">
+        <v>46107</v>
       </c>
     </row>
     <row r="67" spans="1:22">
       <c r="A67">
-        <v>23740</v>
+        <v>23640</v>
       </c>
       <c r="B67" t="s">
         <v>22</v>
@@ -4370,45 +4353,42 @@
         <v>22</v>
       </c>
       <c r="D67" t="s">
-        <v>24</v>
+        <v>27</v>
       </c>
       <c r="E67" t="s">
-        <v>28</v>
-      </c>
-      <c r="F67" t="s">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="N67" t="s">
-        <v>79</v>
+        <v>81</v>
       </c>
       <c r="O67" t="s">
         <v>149</v>
       </c>
       <c r="P67">
-        <v>400000</v>
+        <v>120000</v>
       </c>
       <c r="Q67" t="s">
         <v>166</v>
       </c>
       <c r="R67" t="s">
-        <v>169</v>
+        <v>170</v>
       </c>
       <c r="S67" t="s">
-        <v>171</v>
+        <v>173</v>
       </c>
       <c r="T67" t="s">
-        <v>175</v>
+        <v>176</v>
       </c>
       <c r="U67" t="s">
         <v>28</v>
       </c>
-      <c r="V67" s="2">
-        <v>46291</v>
+      <c r="V67" s="1">
+        <v>46168</v>
       </c>
     </row>
     <row r="68" spans="1:22">
       <c r="A68">
-        <v>24180</v>
+        <v>23740</v>
       </c>
       <c r="B68" t="s">
         <v>22</v>
@@ -4425,20 +4405,14 @@
       <c r="F68" t="s">
         <v>30</v>
       </c>
-      <c r="J68" t="s">
-        <v>62</v>
-      </c>
-      <c r="K68" t="s">
-        <v>71</v>
-      </c>
       <c r="N68" t="s">
-        <v>83</v>
+        <v>80</v>
       </c>
       <c r="O68" t="s">
         <v>150</v>
       </c>
       <c r="P68">
-        <v>100000</v>
+        <v>400000</v>
       </c>
       <c r="Q68" t="s">
         <v>166</v>
@@ -4447,21 +4421,21 @@
         <v>169</v>
       </c>
       <c r="S68" t="s">
-        <v>171</v>
+        <v>172</v>
       </c>
       <c r="T68" t="s">
-        <v>175</v>
+        <v>176</v>
       </c>
       <c r="U68" t="s">
-        <v>180</v>
-      </c>
-      <c r="V68" s="2">
-        <v>46229</v>
+        <v>28</v>
+      </c>
+      <c r="V68" s="1">
+        <v>46291</v>
       </c>
     </row>
     <row r="69" spans="1:22">
       <c r="A69">
-        <v>24380</v>
+        <v>24180</v>
       </c>
       <c r="B69" t="s">
         <v>22</v>
@@ -4470,42 +4444,51 @@
         <v>22</v>
       </c>
       <c r="D69" t="s">
-        <v>27</v>
+        <v>24</v>
       </c>
       <c r="E69" t="s">
-        <v>29</v>
+        <v>28</v>
+      </c>
+      <c r="F69" t="s">
+        <v>30</v>
+      </c>
+      <c r="J69" t="s">
+        <v>63</v>
+      </c>
+      <c r="K69" t="s">
+        <v>72</v>
       </c>
       <c r="N69" t="s">
-        <v>80</v>
+        <v>84</v>
       </c>
       <c r="O69" t="s">
         <v>151</v>
       </c>
       <c r="P69">
-        <v>80000</v>
+        <v>100000</v>
       </c>
       <c r="Q69" t="s">
-        <v>165</v>
+        <v>168</v>
       </c>
       <c r="R69" t="s">
-        <v>168</v>
+        <v>169</v>
       </c>
       <c r="S69" t="s">
         <v>172</v>
       </c>
       <c r="T69" t="s">
-        <v>175</v>
+        <v>176</v>
       </c>
       <c r="U69" t="s">
-        <v>28</v>
-      </c>
-      <c r="V69" s="2">
-        <v>46260</v>
+        <v>181</v>
+      </c>
+      <c r="V69" s="1">
+        <v>46229</v>
       </c>
     </row>
     <row r="70" spans="1:22">
       <c r="A70">
-        <v>24660</v>
+        <v>24380</v>
       </c>
       <c r="B70" t="s">
         <v>22</v>
@@ -4520,36 +4503,36 @@
         <v>29</v>
       </c>
       <c r="N70" t="s">
-        <v>79</v>
+        <v>81</v>
       </c>
       <c r="O70" t="s">
         <v>152</v>
       </c>
       <c r="P70">
-        <v>835000</v>
+        <v>80000</v>
       </c>
       <c r="Q70" t="s">
-        <v>165</v>
+        <v>166</v>
       </c>
       <c r="R70" t="s">
-        <v>169</v>
+        <v>170</v>
       </c>
       <c r="S70" t="s">
-        <v>172</v>
+        <v>173</v>
       </c>
       <c r="T70" t="s">
-        <v>175</v>
+        <v>176</v>
       </c>
       <c r="U70" t="s">
-        <v>180</v>
-      </c>
-      <c r="V70" s="2">
-        <v>46291</v>
+        <v>28</v>
+      </c>
+      <c r="V70" s="1">
+        <v>46260</v>
       </c>
     </row>
     <row r="71" spans="1:22">
       <c r="A71">
-        <v>24661</v>
+        <v>24660</v>
       </c>
       <c r="B71" t="s">
         <v>22</v>
@@ -4564,36 +4547,36 @@
         <v>29</v>
       </c>
       <c r="N71" t="s">
-        <v>79</v>
+        <v>80</v>
       </c>
       <c r="O71" t="s">
-        <v>152</v>
+        <v>153</v>
       </c>
       <c r="P71">
-        <v>165000</v>
+        <v>835000</v>
       </c>
       <c r="Q71" t="s">
-        <v>165</v>
+        <v>166</v>
       </c>
       <c r="R71" t="s">
         <v>169</v>
       </c>
       <c r="S71" t="s">
-        <v>172</v>
+        <v>173</v>
       </c>
       <c r="T71" t="s">
-        <v>175</v>
+        <v>176</v>
       </c>
       <c r="U71" t="s">
-        <v>180</v>
-      </c>
-      <c r="V71" s="2">
-        <v>46168</v>
+        <v>181</v>
+      </c>
+      <c r="V71" s="1">
+        <v>46291</v>
       </c>
     </row>
     <row r="72" spans="1:22">
       <c r="A72">
-        <v>24680</v>
+        <v>24661</v>
       </c>
       <c r="B72" t="s">
         <v>22</v>
@@ -4608,36 +4591,36 @@
         <v>29</v>
       </c>
       <c r="N72" t="s">
-        <v>79</v>
+        <v>80</v>
       </c>
       <c r="O72" t="s">
         <v>153</v>
       </c>
       <c r="P72">
-        <v>1000000</v>
+        <v>165000</v>
       </c>
       <c r="Q72" t="s">
-        <v>165</v>
+        <v>166</v>
       </c>
       <c r="R72" t="s">
         <v>169</v>
       </c>
       <c r="S72" t="s">
-        <v>172</v>
+        <v>173</v>
       </c>
       <c r="T72" t="s">
-        <v>175</v>
+        <v>176</v>
       </c>
       <c r="U72" t="s">
-        <v>180</v>
-      </c>
-      <c r="V72" s="2">
-        <v>46291</v>
+        <v>181</v>
+      </c>
+      <c r="V72" s="1">
+        <v>46168</v>
       </c>
     </row>
     <row r="73" spans="1:22">
       <c r="A73">
-        <v>24700</v>
+        <v>24680</v>
       </c>
       <c r="B73" t="s">
         <v>22</v>
@@ -4652,7 +4635,7 @@
         <v>29</v>
       </c>
       <c r="N73" t="s">
-        <v>79</v>
+        <v>80</v>
       </c>
       <c r="O73" t="s">
         <v>154</v>
@@ -4661,27 +4644,27 @@
         <v>1000000</v>
       </c>
       <c r="Q73" t="s">
-        <v>165</v>
+        <v>166</v>
       </c>
       <c r="R73" t="s">
         <v>169</v>
       </c>
       <c r="S73" t="s">
-        <v>172</v>
+        <v>173</v>
       </c>
       <c r="T73" t="s">
-        <v>175</v>
+        <v>176</v>
       </c>
       <c r="U73" t="s">
-        <v>180</v>
-      </c>
-      <c r="V73" s="2">
+        <v>181</v>
+      </c>
+      <c r="V73" s="1">
         <v>46291</v>
       </c>
     </row>
     <row r="74" spans="1:22">
       <c r="A74">
-        <v>24720</v>
+        <v>24700</v>
       </c>
       <c r="B74" t="s">
         <v>22</v>
@@ -4696,13 +4679,13 @@
         <v>29</v>
       </c>
       <c r="N74" t="s">
-        <v>83</v>
+        <v>80</v>
       </c>
       <c r="O74" t="s">
         <v>155</v>
       </c>
       <c r="P74">
-        <v>100000</v>
+        <v>1000000</v>
       </c>
       <c r="Q74" t="s">
         <v>166</v>
@@ -4711,21 +4694,21 @@
         <v>169</v>
       </c>
       <c r="S74" t="s">
-        <v>172</v>
+        <v>173</v>
       </c>
       <c r="T74" t="s">
-        <v>175</v>
+        <v>176</v>
       </c>
       <c r="U74" t="s">
-        <v>180</v>
-      </c>
-      <c r="V74" s="2">
+        <v>181</v>
+      </c>
+      <c r="V74" s="1">
         <v>46291</v>
       </c>
     </row>
     <row r="75" spans="1:22">
       <c r="A75">
-        <v>25180</v>
+        <v>24720</v>
       </c>
       <c r="B75" t="s">
         <v>22</v>
@@ -4734,45 +4717,42 @@
         <v>22</v>
       </c>
       <c r="D75" t="s">
-        <v>24</v>
+        <v>27</v>
       </c>
       <c r="E75" t="s">
-        <v>28</v>
-      </c>
-      <c r="F75" t="s">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="N75" t="s">
-        <v>86</v>
+        <v>84</v>
       </c>
       <c r="O75" t="s">
         <v>156</v>
       </c>
       <c r="P75">
-        <v>1000000</v>
+        <v>100000</v>
       </c>
       <c r="Q75" t="s">
-        <v>167</v>
+        <v>168</v>
       </c>
       <c r="R75" t="s">
         <v>169</v>
       </c>
       <c r="S75" t="s">
-        <v>171</v>
+        <v>173</v>
       </c>
       <c r="T75" t="s">
         <v>176</v>
       </c>
       <c r="U75" t="s">
-        <v>28</v>
-      </c>
-      <c r="V75" s="2">
-        <v>46321</v>
+        <v>181</v>
+      </c>
+      <c r="V75" s="1">
+        <v>46291</v>
       </c>
     </row>
     <row r="76" spans="1:22">
       <c r="A76">
-        <v>25900</v>
+        <v>25180</v>
       </c>
       <c r="B76" t="s">
         <v>22</v>
@@ -4781,48 +4761,45 @@
         <v>22</v>
       </c>
       <c r="D76" t="s">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="E76" t="s">
         <v>28</v>
       </c>
       <c r="F76" t="s">
-        <v>40</v>
-      </c>
-      <c r="G76" t="s">
-        <v>44</v>
+        <v>30</v>
       </c>
       <c r="N76" t="s">
-        <v>84</v>
+        <v>87</v>
       </c>
       <c r="O76" t="s">
         <v>157</v>
       </c>
       <c r="P76">
-        <v>1704503</v>
+        <v>1000000</v>
       </c>
       <c r="Q76" t="s">
         <v>167</v>
       </c>
       <c r="R76" t="s">
-        <v>168</v>
+        <v>169</v>
       </c>
       <c r="S76" t="s">
-        <v>40</v>
+        <v>172</v>
       </c>
       <c r="T76" t="s">
         <v>177</v>
       </c>
       <c r="U76" t="s">
-        <v>180</v>
-      </c>
-      <c r="V76" s="2">
-        <v>46381</v>
+        <v>28</v>
+      </c>
+      <c r="V76" s="1">
+        <v>46321</v>
       </c>
     </row>
     <row r="77" spans="1:22">
       <c r="A77">
-        <v>25920</v>
+        <v>25900</v>
       </c>
       <c r="B77" t="s">
         <v>22</v>
@@ -4837,42 +4814,42 @@
         <v>28</v>
       </c>
       <c r="F77" t="s">
-        <v>40</v>
+        <v>41</v>
       </c>
       <c r="G77" t="s">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="N77" t="s">
-        <v>84</v>
+        <v>85</v>
       </c>
       <c r="O77" t="s">
         <v>158</v>
       </c>
       <c r="P77">
-        <v>1638125.5</v>
+        <v>1704503</v>
       </c>
       <c r="Q77" t="s">
         <v>167</v>
       </c>
       <c r="R77" t="s">
-        <v>168</v>
+        <v>170</v>
       </c>
       <c r="S77" t="s">
-        <v>40</v>
+        <v>41</v>
       </c>
       <c r="T77" t="s">
-        <v>177</v>
+        <v>178</v>
       </c>
       <c r="U77" t="s">
-        <v>180</v>
-      </c>
-      <c r="V77" s="2">
+        <v>181</v>
+      </c>
+      <c r="V77" s="1">
         <v>46381</v>
       </c>
     </row>
     <row r="78" spans="1:22">
       <c r="A78">
-        <v>25940</v>
+        <v>25920</v>
       </c>
       <c r="B78" t="s">
         <v>22</v>
@@ -4887,42 +4864,42 @@
         <v>28</v>
       </c>
       <c r="F78" t="s">
-        <v>40</v>
+        <v>41</v>
       </c>
       <c r="G78" t="s">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="N78" t="s">
-        <v>82</v>
+        <v>85</v>
       </c>
       <c r="O78" t="s">
         <v>159</v>
       </c>
       <c r="P78">
-        <v>3800000</v>
+        <v>1638125.5</v>
       </c>
       <c r="Q78" t="s">
         <v>167</v>
       </c>
       <c r="R78" t="s">
-        <v>168</v>
+        <v>170</v>
       </c>
       <c r="S78" t="s">
-        <v>40</v>
+        <v>41</v>
       </c>
       <c r="T78" t="s">
-        <v>176</v>
+        <v>178</v>
       </c>
       <c r="U78" t="s">
-        <v>28</v>
-      </c>
-      <c r="V78" s="2">
+        <v>181</v>
+      </c>
+      <c r="V78" s="1">
         <v>46381</v>
       </c>
     </row>
     <row r="79" spans="1:22">
       <c r="A79">
-        <v>25960</v>
+        <v>25940</v>
       </c>
       <c r="B79" t="s">
         <v>22</v>
@@ -4937,13 +4914,13 @@
         <v>28</v>
       </c>
       <c r="F79" t="s">
-        <v>40</v>
+        <v>41</v>
       </c>
       <c r="G79" t="s">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="N79" t="s">
-        <v>82</v>
+        <v>83</v>
       </c>
       <c r="O79" t="s">
         <v>160</v>
@@ -4955,24 +4932,24 @@
         <v>167</v>
       </c>
       <c r="R79" t="s">
-        <v>168</v>
+        <v>170</v>
       </c>
       <c r="S79" t="s">
-        <v>40</v>
+        <v>41</v>
       </c>
       <c r="T79" t="s">
-        <v>176</v>
+        <v>177</v>
       </c>
       <c r="U79" t="s">
         <v>28</v>
       </c>
-      <c r="V79" s="2">
+      <c r="V79" s="1">
         <v>46381</v>
       </c>
     </row>
     <row r="80" spans="1:22">
       <c r="A80">
-        <v>63120</v>
+        <v>25960</v>
       </c>
       <c r="B80" t="s">
         <v>22</v>
@@ -4981,19 +4958,19 @@
         <v>22</v>
       </c>
       <c r="D80" t="s">
-        <v>27</v>
+        <v>25</v>
       </c>
       <c r="E80" t="s">
-        <v>29</v>
-      </c>
-      <c r="J80" t="s">
-        <v>69</v>
-      </c>
-      <c r="K80" t="s">
-        <v>76</v>
+        <v>28</v>
+      </c>
+      <c r="F80" t="s">
+        <v>41</v>
+      </c>
+      <c r="G80" t="s">
+        <v>45</v>
       </c>
       <c r="N80" t="s">
-        <v>87</v>
+        <v>83</v>
       </c>
       <c r="O80" t="s">
         <v>161</v>
@@ -5005,24 +4982,24 @@
         <v>167</v>
       </c>
       <c r="R80" t="s">
-        <v>168</v>
+        <v>170</v>
       </c>
       <c r="S80" t="s">
-        <v>172</v>
+        <v>41</v>
       </c>
       <c r="T80" t="s">
-        <v>176</v>
+        <v>177</v>
       </c>
       <c r="U80" t="s">
         <v>28</v>
       </c>
-      <c r="V80" s="2">
-        <v>46382</v>
+      <c r="V80" s="1">
+        <v>46381</v>
       </c>
     </row>
     <row r="81" spans="1:22">
       <c r="A81">
-        <v>63140</v>
+        <v>63120</v>
       </c>
       <c r="B81" t="s">
         <v>22</v>
@@ -5031,42 +5008,48 @@
         <v>22</v>
       </c>
       <c r="D81" t="s">
-        <v>24</v>
+        <v>27</v>
       </c>
       <c r="E81" t="s">
-        <v>28</v>
+        <v>29</v>
+      </c>
+      <c r="J81" t="s">
+        <v>70</v>
+      </c>
+      <c r="K81" t="s">
+        <v>77</v>
       </c>
       <c r="N81" t="s">
-        <v>95</v>
+        <v>88</v>
       </c>
       <c r="O81" t="s">
-        <v>96</v>
+        <v>162</v>
       </c>
       <c r="P81">
-        <v>4394700</v>
+        <v>3800000</v>
       </c>
       <c r="Q81" t="s">
-        <v>165</v>
+        <v>167</v>
       </c>
       <c r="R81" t="s">
-        <v>169</v>
+        <v>170</v>
       </c>
       <c r="S81" t="s">
-        <v>172</v>
+        <v>173</v>
       </c>
       <c r="T81" t="s">
-        <v>176</v>
+        <v>177</v>
       </c>
       <c r="U81" t="s">
         <v>28</v>
       </c>
-      <c r="V81" s="2">
+      <c r="V81" s="1">
         <v>46382</v>
       </c>
     </row>
     <row r="82" spans="1:22">
       <c r="A82">
-        <v>63940</v>
+        <v>63140</v>
       </c>
       <c r="B82" t="s">
         <v>22</v>
@@ -5080,46 +5063,37 @@
       <c r="E82" t="s">
         <v>28</v>
       </c>
-      <c r="F82" t="s">
-        <v>30</v>
-      </c>
-      <c r="J82" t="s">
-        <v>62</v>
-      </c>
-      <c r="K82" t="s">
-        <v>77</v>
-      </c>
       <c r="N82" t="s">
-        <v>84</v>
+        <v>96</v>
       </c>
       <c r="O82" t="s">
-        <v>162</v>
+        <v>97</v>
       </c>
       <c r="P82">
-        <v>528395.9300000001</v>
+        <v>4394700</v>
       </c>
       <c r="Q82" t="s">
-        <v>167</v>
+        <v>166</v>
       </c>
       <c r="R82" t="s">
-        <v>168</v>
+        <v>169</v>
       </c>
       <c r="S82" t="s">
-        <v>171</v>
+        <v>173</v>
       </c>
       <c r="T82" t="s">
         <v>177</v>
       </c>
       <c r="U82" t="s">
-        <v>180</v>
-      </c>
-      <c r="V82" s="2">
+        <v>28</v>
+      </c>
+      <c r="V82" s="1">
         <v>46382</v>
       </c>
     </row>
     <row r="83" spans="1:22">
       <c r="A83">
-        <v>63960</v>
+        <v>63940</v>
       </c>
       <c r="B83" t="s">
         <v>22</v>
@@ -5128,42 +5102,51 @@
         <v>22</v>
       </c>
       <c r="D83" t="s">
-        <v>27</v>
+        <v>24</v>
       </c>
       <c r="E83" t="s">
-        <v>29</v>
+        <v>28</v>
+      </c>
+      <c r="F83" t="s">
+        <v>30</v>
+      </c>
+      <c r="J83" t="s">
+        <v>63</v>
+      </c>
+      <c r="K83" t="s">
+        <v>78</v>
       </c>
       <c r="N83" t="s">
-        <v>86</v>
+        <v>85</v>
       </c>
       <c r="O83" t="s">
         <v>163</v>
       </c>
       <c r="P83">
-        <v>1000000</v>
+        <v>528395.9300000001</v>
       </c>
       <c r="Q83" t="s">
         <v>167</v>
       </c>
       <c r="R83" t="s">
-        <v>169</v>
+        <v>170</v>
       </c>
       <c r="S83" t="s">
-        <v>174</v>
+        <v>172</v>
       </c>
       <c r="T83" t="s">
-        <v>176</v>
+        <v>178</v>
       </c>
       <c r="U83" t="s">
-        <v>28</v>
-      </c>
-      <c r="V83" s="2">
-        <v>46321</v>
+        <v>181</v>
+      </c>
+      <c r="V83" s="1">
+        <v>46382</v>
       </c>
     </row>
     <row r="84" spans="1:22">
       <c r="A84">
-        <v>64340</v>
+        <v>63960</v>
       </c>
       <c r="B84" t="s">
         <v>22</v>
@@ -5172,42 +5155,42 @@
         <v>22</v>
       </c>
       <c r="D84" t="s">
-        <v>24</v>
+        <v>27</v>
       </c>
       <c r="E84" t="s">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="N84" t="s">
-        <v>95</v>
+        <v>87</v>
       </c>
       <c r="O84" t="s">
-        <v>96</v>
+        <v>164</v>
       </c>
       <c r="P84">
-        <v>4394700</v>
+        <v>1000000</v>
       </c>
       <c r="Q84" t="s">
-        <v>165</v>
+        <v>167</v>
       </c>
       <c r="R84" t="s">
         <v>169</v>
       </c>
       <c r="S84" t="s">
-        <v>172</v>
+        <v>175</v>
       </c>
       <c r="T84" t="s">
-        <v>176</v>
+        <v>177</v>
       </c>
       <c r="U84" t="s">
         <v>28</v>
       </c>
-      <c r="V84" s="2">
-        <v>46382</v>
+      <c r="V84" s="1">
+        <v>46321</v>
       </c>
     </row>
     <row r="85" spans="1:22">
       <c r="A85">
-        <v>64760</v>
+        <v>64340</v>
       </c>
       <c r="B85" t="s">
         <v>22</v>
@@ -5216,45 +5199,42 @@
         <v>22</v>
       </c>
       <c r="D85" t="s">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="E85" t="s">
         <v>28</v>
-      </c>
-      <c r="F85" t="s">
-        <v>40</v>
-      </c>
-      <c r="G85" t="s">
-        <v>44</v>
       </c>
       <c r="N85" t="s">
         <v>96</v>
       </c>
       <c r="O85" t="s">
-        <v>96</v>
+        <v>97</v>
       </c>
       <c r="P85">
-        <v>3306000</v>
+        <v>4394700</v>
       </c>
       <c r="Q85" t="s">
-        <v>165</v>
+        <v>166</v>
       </c>
       <c r="R85" t="s">
         <v>169</v>
       </c>
       <c r="S85" t="s">
-        <v>40</v>
+        <v>173</v>
       </c>
       <c r="T85" t="s">
-        <v>176</v>
+        <v>177</v>
       </c>
       <c r="U85" t="s">
         <v>28</v>
+      </c>
+      <c r="V85" s="1">
+        <v>46382</v>
       </c>
     </row>
     <row r="86" spans="1:22">
       <c r="A86">
-        <v>64780</v>
+        <v>64760</v>
       </c>
       <c r="B86" t="s">
         <v>22</v>
@@ -5269,31 +5249,31 @@
         <v>28</v>
       </c>
       <c r="F86" t="s">
-        <v>40</v>
+        <v>41</v>
       </c>
       <c r="G86" t="s">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="N86" t="s">
-        <v>96</v>
+        <v>97</v>
       </c>
       <c r="O86" t="s">
-        <v>96</v>
+        <v>97</v>
       </c>
       <c r="P86">
         <v>3306000</v>
       </c>
       <c r="Q86" t="s">
-        <v>165</v>
+        <v>166</v>
       </c>
       <c r="R86" t="s">
         <v>169</v>
       </c>
       <c r="S86" t="s">
-        <v>40</v>
+        <v>41</v>
       </c>
       <c r="T86" t="s">
-        <v>176</v>
+        <v>177</v>
       </c>
       <c r="U86" t="s">
         <v>28</v>
@@ -5301,7 +5281,7 @@
     </row>
     <row r="87" spans="1:22">
       <c r="A87">
-        <v>64840</v>
+        <v>64780</v>
       </c>
       <c r="B87" t="s">
         <v>22</v>
@@ -5310,39 +5290,86 @@
         <v>22</v>
       </c>
       <c r="D87" t="s">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="E87" t="s">
         <v>28</v>
       </c>
       <c r="F87" t="s">
-        <v>30</v>
+        <v>41</v>
+      </c>
+      <c r="G87" t="s">
+        <v>45</v>
       </c>
       <c r="N87" t="s">
         <v>97</v>
       </c>
       <c r="O87" t="s">
-        <v>164</v>
+        <v>97</v>
       </c>
       <c r="P87">
-        <v>470820</v>
+        <v>3306000</v>
       </c>
       <c r="Q87" t="s">
-        <v>165</v>
+        <v>166</v>
       </c>
       <c r="R87" t="s">
         <v>169</v>
       </c>
       <c r="S87" t="s">
-        <v>171</v>
+        <v>41</v>
       </c>
       <c r="T87" t="s">
-        <v>179</v>
+        <v>177</v>
       </c>
       <c r="U87" t="s">
         <v>28</v>
       </c>
-      <c r="V87" s="2">
+    </row>
+    <row r="88" spans="1:22">
+      <c r="A88">
+        <v>64840</v>
+      </c>
+      <c r="B88" t="s">
+        <v>22</v>
+      </c>
+      <c r="C88" t="s">
+        <v>22</v>
+      </c>
+      <c r="D88" t="s">
+        <v>24</v>
+      </c>
+      <c r="E88" t="s">
+        <v>28</v>
+      </c>
+      <c r="F88" t="s">
+        <v>30</v>
+      </c>
+      <c r="N88" t="s">
+        <v>98</v>
+      </c>
+      <c r="O88" t="s">
+        <v>165</v>
+      </c>
+      <c r="P88">
+        <v>470820</v>
+      </c>
+      <c r="Q88" t="s">
+        <v>166</v>
+      </c>
+      <c r="R88" t="s">
+        <v>169</v>
+      </c>
+      <c r="S88" t="s">
+        <v>172</v>
+      </c>
+      <c r="T88" t="s">
+        <v>180</v>
+      </c>
+      <c r="U88" t="s">
+        <v>28</v>
+      </c>
+      <c r="V88" s="1">
         <v>46291</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Atualização automática: mta (17/09/2026 12:58)
</commit_message>
<xml_diff>
--- a/Projetos/02_Dados_Tratados/base_mta_tratada.xlsx
+++ b/Projetos/02_Dados_Tratados/base_mta_tratada.xlsx
@@ -569,8 +569,16 @@
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="YYYY-MM-DD HH:MM:SS"/>
   </numFmts>
-  <fonts count="1">
+  <fonts count="2">
     <font>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
       <sz val="11"/>
       <color theme="1"/>
       <name val="Calibri"/>
@@ -586,7 +594,7 @@
       <patternFill patternType="gray125"/>
     </fill>
   </fills>
-  <borders count="1">
+  <borders count="2">
     <border>
       <left/>
       <right/>
@@ -594,12 +602,30 @@
       <bottom/>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin">
+        <color auto="1"/>
+      </left>
+      <right style="thin">
+        <color auto="1"/>
+      </right>
+      <top style="thin">
+        <color auto="1"/>
+      </top>
+      <bottom style="thin">
+        <color auto="1"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="3">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
   </cellXfs>
   <cellStyles count="1">
@@ -899,70 +925,70 @@
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:22">
-      <c r="A1" t="s">
+      <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
-      <c r="B1" t="s">
+      <c r="B1" s="1" t="s">
         <v>1</v>
       </c>
-      <c r="C1" t="s">
+      <c r="C1" s="1" t="s">
         <v>2</v>
       </c>
-      <c r="D1" t="s">
+      <c r="D1" s="1" t="s">
         <v>3</v>
       </c>
-      <c r="E1" t="s">
+      <c r="E1" s="1" t="s">
         <v>4</v>
       </c>
-      <c r="F1" t="s">
+      <c r="F1" s="1" t="s">
         <v>5</v>
       </c>
-      <c r="G1" t="s">
+      <c r="G1" s="1" t="s">
         <v>6</v>
       </c>
-      <c r="H1" t="s">
+      <c r="H1" s="1" t="s">
         <v>7</v>
       </c>
-      <c r="I1" t="s">
+      <c r="I1" s="1" t="s">
         <v>8</v>
       </c>
-      <c r="J1" t="s">
+      <c r="J1" s="1" t="s">
         <v>9</v>
       </c>
-      <c r="K1" t="s">
+      <c r="K1" s="1" t="s">
         <v>10</v>
       </c>
-      <c r="L1" t="s">
+      <c r="L1" s="1" t="s">
         <v>11</v>
       </c>
-      <c r="M1" t="s">
+      <c r="M1" s="1" t="s">
         <v>12</v>
       </c>
-      <c r="N1" t="s">
+      <c r="N1" s="1" t="s">
         <v>13</v>
       </c>
-      <c r="O1" t="s">
+      <c r="O1" s="1" t="s">
         <v>14</v>
       </c>
-      <c r="P1" t="s">
+      <c r="P1" s="1" t="s">
         <v>15</v>
       </c>
-      <c r="Q1" t="s">
+      <c r="Q1" s="1" t="s">
         <v>16</v>
       </c>
-      <c r="R1" t="s">
+      <c r="R1" s="1" t="s">
         <v>17</v>
       </c>
-      <c r="S1" t="s">
+      <c r="S1" s="1" t="s">
         <v>18</v>
       </c>
-      <c r="T1" t="s">
+      <c r="T1" s="1" t="s">
         <v>19</v>
       </c>
-      <c r="U1" t="s">
+      <c r="U1" s="1" t="s">
         <v>20</v>
       </c>
-      <c r="V1" t="s">
+      <c r="V1" s="1" t="s">
         <v>21</v>
       </c>
     </row>
@@ -1018,7 +1044,7 @@
       <c r="U2" t="s">
         <v>181</v>
       </c>
-      <c r="V2" s="1">
+      <c r="V2" s="2">
         <v>46229</v>
       </c>
     </row>
@@ -1065,7 +1091,7 @@
       <c r="U3" t="s">
         <v>28</v>
       </c>
-      <c r="V3" s="1">
+      <c r="V3" s="2">
         <v>46291</v>
       </c>
     </row>
@@ -1112,7 +1138,7 @@
       <c r="U4" t="s">
         <v>28</v>
       </c>
-      <c r="V4" s="1">
+      <c r="V4" s="2">
         <v>46321</v>
       </c>
     </row>
@@ -1159,7 +1185,7 @@
       <c r="U5" t="s">
         <v>28</v>
       </c>
-      <c r="V5" s="1">
+      <c r="V5" s="2">
         <v>46321</v>
       </c>
     </row>
@@ -1209,7 +1235,7 @@
       <c r="U6" t="s">
         <v>28</v>
       </c>
-      <c r="V6" s="1">
+      <c r="V6" s="2">
         <v>46291</v>
       </c>
     </row>
@@ -1235,7 +1261,7 @@
       <c r="G7" t="s">
         <v>43</v>
       </c>
-      <c r="H7" s="1">
+      <c r="H7" s="2">
         <v>46121</v>
       </c>
       <c r="I7" t="s">
@@ -1265,7 +1291,7 @@
       <c r="U7" t="s">
         <v>28</v>
       </c>
-      <c r="V7" s="1">
+      <c r="V7" s="2">
         <v>46138</v>
       </c>
     </row>
@@ -1312,7 +1338,7 @@
       <c r="U8" t="s">
         <v>28</v>
       </c>
-      <c r="V8" s="1">
+      <c r="V8" s="2">
         <v>46291</v>
       </c>
     </row>
@@ -1359,7 +1385,7 @@
       <c r="U9" t="s">
         <v>28</v>
       </c>
-      <c r="V9" s="1">
+      <c r="V9" s="2">
         <v>46291</v>
       </c>
     </row>
@@ -1406,7 +1432,7 @@
       <c r="U10" t="s">
         <v>28</v>
       </c>
-      <c r="V10" s="1">
+      <c r="V10" s="2">
         <v>46291</v>
       </c>
     </row>
@@ -1453,7 +1479,7 @@
       <c r="U11" t="s">
         <v>28</v>
       </c>
-      <c r="V11" s="1">
+      <c r="V11" s="2">
         <v>46291</v>
       </c>
     </row>
@@ -1479,7 +1505,7 @@
       <c r="G12" t="s">
         <v>43</v>
       </c>
-      <c r="H12" s="1">
+      <c r="H12" s="2">
         <v>46079</v>
       </c>
       <c r="I12" t="s">
@@ -1512,7 +1538,7 @@
       <c r="U12" t="s">
         <v>181</v>
       </c>
-      <c r="V12" s="1">
+      <c r="V12" s="2">
         <v>46079</v>
       </c>
     </row>
@@ -1565,7 +1591,7 @@
       <c r="U13" t="s">
         <v>181</v>
       </c>
-      <c r="V13" s="1">
+      <c r="V13" s="2">
         <v>46352</v>
       </c>
     </row>
@@ -1618,7 +1644,7 @@
       <c r="U14" t="s">
         <v>181</v>
       </c>
-      <c r="V14" s="1">
+      <c r="V14" s="2">
         <v>46352</v>
       </c>
     </row>
@@ -1671,7 +1697,7 @@
       <c r="U15" t="s">
         <v>181</v>
       </c>
-      <c r="V15" s="1">
+      <c r="V15" s="2">
         <v>46352</v>
       </c>
     </row>
@@ -1724,7 +1750,7 @@
       <c r="U16" t="s">
         <v>181</v>
       </c>
-      <c r="V16" s="1">
+      <c r="V16" s="2">
         <v>46229</v>
       </c>
     </row>
@@ -1750,7 +1776,7 @@
       <c r="G17" t="s">
         <v>43</v>
       </c>
-      <c r="H17" s="1">
+      <c r="H17" s="2">
         <v>46098</v>
       </c>
       <c r="I17" t="s">
@@ -1783,7 +1809,7 @@
       <c r="U17" t="s">
         <v>181</v>
       </c>
-      <c r="V17" s="1">
+      <c r="V17" s="2">
         <v>46107</v>
       </c>
     </row>
@@ -1809,7 +1835,7 @@
       <c r="G18" t="s">
         <v>43</v>
       </c>
-      <c r="H18" s="1">
+      <c r="H18" s="2">
         <v>46076</v>
       </c>
       <c r="I18" t="s">
@@ -1839,7 +1865,7 @@
       <c r="U18" t="s">
         <v>28</v>
       </c>
-      <c r="V18" s="1">
+      <c r="V18" s="2">
         <v>46079</v>
       </c>
     </row>
@@ -1865,7 +1891,7 @@
       <c r="G19" t="s">
         <v>43</v>
       </c>
-      <c r="H19" s="1">
+      <c r="H19" s="2">
         <v>46076</v>
       </c>
       <c r="I19" t="s">
@@ -1895,7 +1921,7 @@
       <c r="U19" t="s">
         <v>28</v>
       </c>
-      <c r="V19" s="1">
+      <c r="V19" s="2">
         <v>46079</v>
       </c>
     </row>
@@ -1942,7 +1968,7 @@
       <c r="U20" t="s">
         <v>28</v>
       </c>
-      <c r="V20" s="1">
+      <c r="V20" s="2">
         <v>46321</v>
       </c>
     </row>
@@ -1989,7 +2015,7 @@
       <c r="U21" t="s">
         <v>28</v>
       </c>
-      <c r="V21" s="1">
+      <c r="V21" s="2">
         <v>46321</v>
       </c>
     </row>
@@ -2036,7 +2062,7 @@
       <c r="U22" t="s">
         <v>28</v>
       </c>
-      <c r="V22" s="1">
+      <c r="V22" s="2">
         <v>46321</v>
       </c>
     </row>
@@ -2083,7 +2109,7 @@
       <c r="U23" t="s">
         <v>28</v>
       </c>
-      <c r="V23" s="1">
+      <c r="V23" s="2">
         <v>46321</v>
       </c>
     </row>
@@ -2109,7 +2135,7 @@
       <c r="G24" t="s">
         <v>43</v>
       </c>
-      <c r="H24" s="1">
+      <c r="H24" s="2">
         <v>46119</v>
       </c>
       <c r="I24" t="s">
@@ -2142,7 +2168,7 @@
       <c r="U24" t="s">
         <v>181</v>
       </c>
-      <c r="V24" s="1">
+      <c r="V24" s="2">
         <v>46138</v>
       </c>
     </row>
@@ -2168,7 +2194,7 @@
       <c r="G25" t="s">
         <v>43</v>
       </c>
-      <c r="H25" s="1">
+      <c r="H25" s="2">
         <v>46121</v>
       </c>
       <c r="I25" t="s">
@@ -2198,7 +2224,7 @@
       <c r="U25" t="s">
         <v>28</v>
       </c>
-      <c r="V25" s="1">
+      <c r="V25" s="2">
         <v>46138</v>
       </c>
     </row>
@@ -2224,7 +2250,7 @@
       <c r="G26" t="s">
         <v>43</v>
       </c>
-      <c r="H26" s="1">
+      <c r="H26" s="2">
         <v>46076</v>
       </c>
       <c r="I26" t="s">
@@ -2254,7 +2280,7 @@
       <c r="U26" t="s">
         <v>28</v>
       </c>
-      <c r="V26" s="1">
+      <c r="V26" s="2">
         <v>46079</v>
       </c>
     </row>
@@ -2307,7 +2333,7 @@
       <c r="U27" t="s">
         <v>181</v>
       </c>
-      <c r="V27" s="1">
+      <c r="V27" s="2">
         <v>46291</v>
       </c>
     </row>
@@ -2333,7 +2359,7 @@
       <c r="G28" t="s">
         <v>43</v>
       </c>
-      <c r="H28" s="1">
+      <c r="H28" s="2">
         <v>46199</v>
       </c>
       <c r="I28" t="s">
@@ -2366,7 +2392,7 @@
       <c r="U28" t="s">
         <v>181</v>
       </c>
-      <c r="V28" s="1">
+      <c r="V28" s="2">
         <v>46199</v>
       </c>
     </row>
@@ -2392,7 +2418,7 @@
       <c r="G29" t="s">
         <v>43</v>
       </c>
-      <c r="H29" s="1">
+      <c r="H29" s="2">
         <v>46199</v>
       </c>
       <c r="I29" t="s">
@@ -2425,7 +2451,7 @@
       <c r="U29" t="s">
         <v>181</v>
       </c>
-      <c r="V29" s="1">
+      <c r="V29" s="2">
         <v>46199</v>
       </c>
     </row>
@@ -2451,7 +2477,7 @@
       <c r="G30" t="s">
         <v>43</v>
       </c>
-      <c r="H30" s="1">
+      <c r="H30" s="2">
         <v>46199</v>
       </c>
       <c r="I30" t="s">
@@ -2484,7 +2510,7 @@
       <c r="U30" t="s">
         <v>181</v>
       </c>
-      <c r="V30" s="1">
+      <c r="V30" s="2">
         <v>46199</v>
       </c>
     </row>
@@ -2510,7 +2536,7 @@
       <c r="G31" t="s">
         <v>43</v>
       </c>
-      <c r="H31" s="1">
+      <c r="H31" s="2">
         <v>46199</v>
       </c>
       <c r="I31" t="s">
@@ -2543,7 +2569,7 @@
       <c r="U31" t="s">
         <v>181</v>
       </c>
-      <c r="V31" s="1">
+      <c r="V31" s="2">
         <v>46199</v>
       </c>
     </row>
@@ -2593,7 +2619,7 @@
       <c r="U32" t="s">
         <v>181</v>
       </c>
-      <c r="V32" s="1">
+      <c r="V32" s="2">
         <v>46291</v>
       </c>
     </row>
@@ -2619,7 +2645,7 @@
       <c r="G33" t="s">
         <v>43</v>
       </c>
-      <c r="H33" s="1">
+      <c r="H33" s="2">
         <v>46191</v>
       </c>
       <c r="I33" t="s">
@@ -2652,7 +2678,7 @@
       <c r="U33" t="s">
         <v>181</v>
       </c>
-      <c r="V33" s="1">
+      <c r="V33" s="2">
         <v>46199</v>
       </c>
     </row>
@@ -2678,7 +2704,7 @@
       <c r="G34" t="s">
         <v>43</v>
       </c>
-      <c r="H34" s="1">
+      <c r="H34" s="2">
         <v>46119</v>
       </c>
       <c r="I34" t="s">
@@ -2708,7 +2734,7 @@
       <c r="U34" t="s">
         <v>181</v>
       </c>
-      <c r="V34" s="1">
+      <c r="V34" s="2">
         <v>46138</v>
       </c>
     </row>
@@ -2734,7 +2760,7 @@
       <c r="G35" t="s">
         <v>43</v>
       </c>
-      <c r="H35" s="1">
+      <c r="H35" s="2">
         <v>46213</v>
       </c>
       <c r="I35" t="s">
@@ -2764,7 +2790,7 @@
       <c r="U35" t="s">
         <v>28</v>
       </c>
-      <c r="V35" s="1">
+      <c r="V35" s="2">
         <v>46229</v>
       </c>
     </row>
@@ -2790,7 +2816,7 @@
       <c r="G36" t="s">
         <v>43</v>
       </c>
-      <c r="H36" s="1">
+      <c r="H36" s="2">
         <v>46175</v>
       </c>
       <c r="I36" t="s">
@@ -2820,7 +2846,7 @@
       <c r="U36" t="s">
         <v>28</v>
       </c>
-      <c r="V36" s="1">
+      <c r="V36" s="2">
         <v>46199</v>
       </c>
     </row>
@@ -2846,7 +2872,7 @@
       <c r="G37" t="s">
         <v>43</v>
       </c>
-      <c r="H37" s="1">
+      <c r="H37" s="2">
         <v>46213</v>
       </c>
       <c r="I37" t="s">
@@ -2876,7 +2902,7 @@
       <c r="U37" t="s">
         <v>28</v>
       </c>
-      <c r="V37" s="1">
+      <c r="V37" s="2">
         <v>46229</v>
       </c>
     </row>
@@ -2902,7 +2928,7 @@
       <c r="G38" t="s">
         <v>43</v>
       </c>
-      <c r="H38" s="1">
+      <c r="H38" s="2">
         <v>46199</v>
       </c>
       <c r="I38" t="s">
@@ -2932,7 +2958,7 @@
       <c r="U38" t="s">
         <v>28</v>
       </c>
-      <c r="V38" s="1">
+      <c r="V38" s="2">
         <v>46199</v>
       </c>
     </row>
@@ -2958,7 +2984,7 @@
       <c r="G39" t="s">
         <v>43</v>
       </c>
-      <c r="H39" s="1">
+      <c r="H39" s="2">
         <v>46199</v>
       </c>
       <c r="I39" t="s">
@@ -2988,7 +3014,7 @@
       <c r="U39" t="s">
         <v>28</v>
       </c>
-      <c r="V39" s="1">
+      <c r="V39" s="2">
         <v>46199</v>
       </c>
     </row>
@@ -3014,7 +3040,7 @@
       <c r="G40" t="s">
         <v>43</v>
       </c>
-      <c r="H40" s="1">
+      <c r="H40" s="2">
         <v>46204</v>
       </c>
       <c r="I40" t="s">
@@ -3044,7 +3070,7 @@
       <c r="U40" t="s">
         <v>28</v>
       </c>
-      <c r="V40" s="1">
+      <c r="V40" s="2">
         <v>46229</v>
       </c>
     </row>
@@ -3070,7 +3096,7 @@
       <c r="G41" t="s">
         <v>43</v>
       </c>
-      <c r="H41" s="1">
+      <c r="H41" s="2">
         <v>46244</v>
       </c>
       <c r="I41" t="s">
@@ -3100,7 +3126,7 @@
       <c r="U41" t="s">
         <v>28</v>
       </c>
-      <c r="V41" s="1">
+      <c r="V41" s="2">
         <v>46199</v>
       </c>
     </row>
@@ -3144,7 +3170,7 @@
       <c r="U42" t="s">
         <v>28</v>
       </c>
-      <c r="V42" s="1">
+      <c r="V42" s="2">
         <v>46260</v>
       </c>
     </row>
@@ -3170,7 +3196,7 @@
       <c r="G43" t="s">
         <v>43</v>
       </c>
-      <c r="H43" s="1">
+      <c r="H43" s="2">
         <v>46191</v>
       </c>
       <c r="I43" t="s">
@@ -3200,7 +3226,7 @@
       <c r="U43" t="s">
         <v>28</v>
       </c>
-      <c r="V43" s="1">
+      <c r="V43" s="2">
         <v>46199</v>
       </c>
     </row>
@@ -3226,7 +3252,7 @@
       <c r="G44" t="s">
         <v>43</v>
       </c>
-      <c r="H44" s="1">
+      <c r="H44" s="2">
         <v>46191</v>
       </c>
       <c r="I44" t="s">
@@ -3256,7 +3282,7 @@
       <c r="U44" t="s">
         <v>28</v>
       </c>
-      <c r="V44" s="1">
+      <c r="V44" s="2">
         <v>46199</v>
       </c>
     </row>
@@ -3282,7 +3308,7 @@
       <c r="G45" t="s">
         <v>43</v>
       </c>
-      <c r="H45" s="1">
+      <c r="H45" s="2">
         <v>46213</v>
       </c>
       <c r="I45" t="s">
@@ -3315,7 +3341,7 @@
       <c r="U45" t="s">
         <v>181</v>
       </c>
-      <c r="V45" s="1">
+      <c r="V45" s="2">
         <v>46229</v>
       </c>
     </row>
@@ -3341,7 +3367,7 @@
       <c r="G46" t="s">
         <v>43</v>
       </c>
-      <c r="H46" s="1">
+      <c r="H46" s="2">
         <v>46210</v>
       </c>
       <c r="I46" t="s">
@@ -3371,7 +3397,7 @@
       <c r="U46" t="s">
         <v>181</v>
       </c>
-      <c r="V46" s="1">
+      <c r="V46" s="2">
         <v>46229</v>
       </c>
     </row>
@@ -3418,7 +3444,7 @@
       <c r="U47" t="s">
         <v>28</v>
       </c>
-      <c r="V47" s="1">
+      <c r="V47" s="2">
         <v>46321</v>
       </c>
     </row>
@@ -3471,7 +3497,7 @@
       <c r="U48" t="s">
         <v>181</v>
       </c>
-      <c r="V48" s="1">
+      <c r="V48" s="2">
         <v>46291</v>
       </c>
     </row>
@@ -3497,7 +3523,7 @@
       <c r="G49" t="s">
         <v>43</v>
       </c>
-      <c r="H49" s="1">
+      <c r="H49" s="2">
         <v>46176</v>
       </c>
       <c r="I49" t="s">
@@ -3530,7 +3556,7 @@
       <c r="U49" t="s">
         <v>181</v>
       </c>
-      <c r="V49" s="1">
+      <c r="V49" s="2">
         <v>46199</v>
       </c>
     </row>
@@ -3583,7 +3609,7 @@
       <c r="U50" t="s">
         <v>181</v>
       </c>
-      <c r="V50" s="1">
+      <c r="V50" s="2">
         <v>46260</v>
       </c>
     </row>
@@ -3636,7 +3662,7 @@
       <c r="U51" t="s">
         <v>181</v>
       </c>
-      <c r="V51" s="1">
+      <c r="V51" s="2">
         <v>46291</v>
       </c>
     </row>
@@ -3686,7 +3712,7 @@
       <c r="U52" t="s">
         <v>181</v>
       </c>
-      <c r="V52" s="1">
+      <c r="V52" s="2">
         <v>46321</v>
       </c>
     </row>
@@ -3712,7 +3738,7 @@
       <c r="G53" t="s">
         <v>43</v>
       </c>
-      <c r="H53" s="1">
+      <c r="H53" s="2">
         <v>46227</v>
       </c>
       <c r="I53" t="s">
@@ -3742,7 +3768,7 @@
       <c r="U53" t="s">
         <v>181</v>
       </c>
-      <c r="V53" s="1">
+      <c r="V53" s="2">
         <v>46229</v>
       </c>
     </row>
@@ -3765,7 +3791,7 @@
       <c r="G54" t="s">
         <v>43</v>
       </c>
-      <c r="H54" s="1">
+      <c r="H54" s="2">
         <v>46280</v>
       </c>
       <c r="I54" t="s">
@@ -3795,7 +3821,7 @@
       <c r="U54" t="s">
         <v>181</v>
       </c>
-      <c r="V54" s="1">
+      <c r="V54" s="2">
         <v>46291</v>
       </c>
     </row>
@@ -3848,7 +3874,7 @@
       <c r="U55" t="s">
         <v>181</v>
       </c>
-      <c r="V55" s="1">
+      <c r="V55" s="2">
         <v>46352</v>
       </c>
     </row>
@@ -3901,7 +3927,7 @@
       <c r="U56" t="s">
         <v>181</v>
       </c>
-      <c r="V56" s="1">
+      <c r="V56" s="2">
         <v>46321</v>
       </c>
     </row>
@@ -3948,7 +3974,7 @@
       <c r="U57" t="s">
         <v>181</v>
       </c>
-      <c r="V57" s="1">
+      <c r="V57" s="2">
         <v>46321</v>
       </c>
     </row>
@@ -3992,7 +4018,7 @@
       <c r="U58" t="s">
         <v>181</v>
       </c>
-      <c r="V58" s="1">
+      <c r="V58" s="2">
         <v>46049</v>
       </c>
     </row>
@@ -4118,7 +4144,7 @@
       <c r="U61" t="s">
         <v>181</v>
       </c>
-      <c r="V61" s="1">
+      <c r="V61" s="2">
         <v>46107</v>
       </c>
     </row>
@@ -4162,7 +4188,7 @@
       <c r="U62" t="s">
         <v>181</v>
       </c>
-      <c r="V62" s="1">
+      <c r="V62" s="2">
         <v>46107</v>
       </c>
     </row>
@@ -4206,7 +4232,7 @@
       <c r="U63" t="s">
         <v>181</v>
       </c>
-      <c r="V63" s="1">
+      <c r="V63" s="2">
         <v>46107</v>
       </c>
     </row>
@@ -4250,7 +4276,7 @@
       <c r="U64" t="s">
         <v>181</v>
       </c>
-      <c r="V64" s="1">
+      <c r="V64" s="2">
         <v>46107</v>
       </c>
     </row>
@@ -4294,7 +4320,7 @@
       <c r="U65" t="s">
         <v>181</v>
       </c>
-      <c r="V65" s="1">
+      <c r="V65" s="2">
         <v>46107</v>
       </c>
     </row>
@@ -4338,7 +4364,7 @@
       <c r="U66" t="s">
         <v>181</v>
       </c>
-      <c r="V66" s="1">
+      <c r="V66" s="2">
         <v>46107</v>
       </c>
     </row>
@@ -4382,7 +4408,7 @@
       <c r="U67" t="s">
         <v>28</v>
       </c>
-      <c r="V67" s="1">
+      <c r="V67" s="2">
         <v>46168</v>
       </c>
     </row>
@@ -4429,7 +4455,7 @@
       <c r="U68" t="s">
         <v>28</v>
       </c>
-      <c r="V68" s="1">
+      <c r="V68" s="2">
         <v>46291</v>
       </c>
     </row>
@@ -4482,7 +4508,7 @@
       <c r="U69" t="s">
         <v>181</v>
       </c>
-      <c r="V69" s="1">
+      <c r="V69" s="2">
         <v>46229</v>
       </c>
     </row>
@@ -4526,7 +4552,7 @@
       <c r="U70" t="s">
         <v>28</v>
       </c>
-      <c r="V70" s="1">
+      <c r="V70" s="2">
         <v>46260</v>
       </c>
     </row>
@@ -4570,7 +4596,7 @@
       <c r="U71" t="s">
         <v>181</v>
       </c>
-      <c r="V71" s="1">
+      <c r="V71" s="2">
         <v>46291</v>
       </c>
     </row>
@@ -4614,7 +4640,7 @@
       <c r="U72" t="s">
         <v>181</v>
       </c>
-      <c r="V72" s="1">
+      <c r="V72" s="2">
         <v>46168</v>
       </c>
     </row>
@@ -4658,7 +4684,7 @@
       <c r="U73" t="s">
         <v>181</v>
       </c>
-      <c r="V73" s="1">
+      <c r="V73" s="2">
         <v>46291</v>
       </c>
     </row>
@@ -4702,7 +4728,7 @@
       <c r="U74" t="s">
         <v>181</v>
       </c>
-      <c r="V74" s="1">
+      <c r="V74" s="2">
         <v>46291</v>
       </c>
     </row>
@@ -4746,7 +4772,7 @@
       <c r="U75" t="s">
         <v>181</v>
       </c>
-      <c r="V75" s="1">
+      <c r="V75" s="2">
         <v>46291</v>
       </c>
     </row>
@@ -4793,7 +4819,7 @@
       <c r="U76" t="s">
         <v>28</v>
       </c>
-      <c r="V76" s="1">
+      <c r="V76" s="2">
         <v>46321</v>
       </c>
     </row>
@@ -4843,7 +4869,7 @@
       <c r="U77" t="s">
         <v>181</v>
       </c>
-      <c r="V77" s="1">
+      <c r="V77" s="2">
         <v>46381</v>
       </c>
     </row>
@@ -4893,7 +4919,7 @@
       <c r="U78" t="s">
         <v>181</v>
       </c>
-      <c r="V78" s="1">
+      <c r="V78" s="2">
         <v>46381</v>
       </c>
     </row>
@@ -4943,7 +4969,7 @@
       <c r="U79" t="s">
         <v>28</v>
       </c>
-      <c r="V79" s="1">
+      <c r="V79" s="2">
         <v>46381</v>
       </c>
     </row>
@@ -4993,7 +5019,7 @@
       <c r="U80" t="s">
         <v>28</v>
       </c>
-      <c r="V80" s="1">
+      <c r="V80" s="2">
         <v>46381</v>
       </c>
     </row>
@@ -5043,7 +5069,7 @@
       <c r="U81" t="s">
         <v>28</v>
       </c>
-      <c r="V81" s="1">
+      <c r="V81" s="2">
         <v>46382</v>
       </c>
     </row>
@@ -5087,7 +5113,7 @@
       <c r="U82" t="s">
         <v>28</v>
       </c>
-      <c r="V82" s="1">
+      <c r="V82" s="2">
         <v>46382</v>
       </c>
     </row>
@@ -5140,7 +5166,7 @@
       <c r="U83" t="s">
         <v>181</v>
       </c>
-      <c r="V83" s="1">
+      <c r="V83" s="2">
         <v>46382</v>
       </c>
     </row>
@@ -5184,7 +5210,7 @@
       <c r="U84" t="s">
         <v>28</v>
       </c>
-      <c r="V84" s="1">
+      <c r="V84" s="2">
         <v>46321</v>
       </c>
     </row>
@@ -5228,7 +5254,7 @@
       <c r="U85" t="s">
         <v>28</v>
       </c>
-      <c r="V85" s="1">
+      <c r="V85" s="2">
         <v>46382</v>
       </c>
     </row>
@@ -5369,7 +5395,7 @@
       <c r="U88" t="s">
         <v>28</v>
       </c>
-      <c r="V88" s="1">
+      <c r="V88" s="2">
         <v>46291</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Atualização automática: mta (18/09/2026 11:56)
</commit_message>
<xml_diff>
--- a/Projetos/02_Dados_Tratados/base_mta_tratada.xlsx
+++ b/Projetos/02_Dados_Tratados/base_mta_tratada.xlsx
@@ -14,7 +14,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1153" uniqueCount="182">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1166" uniqueCount="184">
   <si>
     <t>linha</t>
   </si>
@@ -130,6 +130,9 @@
     <t>DESTQ32</t>
   </si>
   <si>
+    <t>DESTQ51</t>
+  </si>
+  <si>
     <t>20XV</t>
   </si>
   <si>
@@ -245,6 +248,9 @@
   </si>
   <si>
     <t>Atender NOV</t>
+  </si>
+  <si>
+    <t>Remanejar R$ 1.462.977,67 para a linha 19020 e ATENDER R$ 500.000,00</t>
   </si>
   <si>
     <t>ATENDER com 20XV</t>
@@ -569,16 +575,8 @@
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="YYYY-MM-DD HH:MM:SS"/>
   </numFmts>
-  <fonts count="2">
+  <fonts count="1">
     <font>
-      <sz val="11"/>
-      <color theme="1"/>
-      <name val="Calibri"/>
-      <family val="2"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <b/>
       <sz val="11"/>
       <color theme="1"/>
       <name val="Calibri"/>
@@ -594,7 +592,7 @@
       <patternFill patternType="gray125"/>
     </fill>
   </fills>
-  <borders count="2">
+  <borders count="1">
     <border>
       <left/>
       <right/>
@@ -602,30 +600,12 @@
       <bottom/>
       <diagonal/>
     </border>
-    <border>
-      <left style="thin">
-        <color auto="1"/>
-      </left>
-      <right style="thin">
-        <color auto="1"/>
-      </right>
-      <top style="thin">
-        <color auto="1"/>
-      </top>
-      <bottom style="thin">
-        <color auto="1"/>
-      </bottom>
-      <diagonal/>
-    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="3">
+  <cellXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top"/>
-    </xf>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
   </cellXfs>
   <cellStyles count="1">
@@ -921,74 +901,74 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:V88"/>
+  <dimension ref="A1:V89"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:22">
-      <c r="A1" s="1" t="s">
+      <c r="A1" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="1" t="s">
+      <c r="B1" t="s">
         <v>1</v>
       </c>
-      <c r="C1" s="1" t="s">
+      <c r="C1" t="s">
         <v>2</v>
       </c>
-      <c r="D1" s="1" t="s">
+      <c r="D1" t="s">
         <v>3</v>
       </c>
-      <c r="E1" s="1" t="s">
+      <c r="E1" t="s">
         <v>4</v>
       </c>
-      <c r="F1" s="1" t="s">
+      <c r="F1" t="s">
         <v>5</v>
       </c>
-      <c r="G1" s="1" t="s">
+      <c r="G1" t="s">
         <v>6</v>
       </c>
-      <c r="H1" s="1" t="s">
+      <c r="H1" t="s">
         <v>7</v>
       </c>
-      <c r="I1" s="1" t="s">
+      <c r="I1" t="s">
         <v>8</v>
       </c>
-      <c r="J1" s="1" t="s">
+      <c r="J1" t="s">
         <v>9</v>
       </c>
-      <c r="K1" s="1" t="s">
+      <c r="K1" t="s">
         <v>10</v>
       </c>
-      <c r="L1" s="1" t="s">
+      <c r="L1" t="s">
         <v>11</v>
       </c>
-      <c r="M1" s="1" t="s">
+      <c r="M1" t="s">
         <v>12</v>
       </c>
-      <c r="N1" s="1" t="s">
+      <c r="N1" t="s">
         <v>13</v>
       </c>
-      <c r="O1" s="1" t="s">
+      <c r="O1" t="s">
         <v>14</v>
       </c>
-      <c r="P1" s="1" t="s">
+      <c r="P1" t="s">
         <v>15</v>
       </c>
-      <c r="Q1" s="1" t="s">
+      <c r="Q1" t="s">
         <v>16</v>
       </c>
-      <c r="R1" s="1" t="s">
+      <c r="R1" t="s">
         <v>17</v>
       </c>
-      <c r="S1" s="1" t="s">
+      <c r="S1" t="s">
         <v>18</v>
       </c>
-      <c r="T1" s="1" t="s">
+      <c r="T1" t="s">
         <v>19</v>
       </c>
-      <c r="U1" s="1" t="s">
+      <c r="U1" t="s">
         <v>20</v>
       </c>
-      <c r="V1" s="1" t="s">
+      <c r="V1" t="s">
         <v>21</v>
       </c>
     </row>
@@ -1012,39 +992,36 @@
         <v>30</v>
       </c>
       <c r="J2" t="s">
-        <v>63</v>
+        <v>64</v>
       </c>
       <c r="K2" t="s">
-        <v>71</v>
+        <v>72</v>
       </c>
       <c r="L2" t="s">
-        <v>79</v>
+        <v>81</v>
       </c>
       <c r="N2" t="s">
-        <v>80</v>
+        <v>82</v>
       </c>
       <c r="O2" t="s">
-        <v>99</v>
-      </c>
-      <c r="P2">
-        <v>135000</v>
+        <v>101</v>
       </c>
       <c r="Q2" t="s">
-        <v>166</v>
+        <v>168</v>
       </c>
       <c r="R2" t="s">
-        <v>169</v>
+        <v>171</v>
       </c>
       <c r="S2" t="s">
-        <v>172</v>
+        <v>174</v>
       </c>
       <c r="T2" t="s">
-        <v>176</v>
+        <v>178</v>
       </c>
       <c r="U2" t="s">
-        <v>181</v>
-      </c>
-      <c r="V2" s="2">
+        <v>183</v>
+      </c>
+      <c r="V2" s="1">
         <v>46229</v>
       </c>
     </row>
@@ -1068,30 +1045,27 @@
         <v>30</v>
       </c>
       <c r="N3" t="s">
-        <v>80</v>
+        <v>82</v>
       </c>
       <c r="O3" t="s">
-        <v>100</v>
-      </c>
-      <c r="P3">
-        <v>400000</v>
+        <v>102</v>
       </c>
       <c r="Q3" t="s">
-        <v>166</v>
+        <v>168</v>
       </c>
       <c r="R3" t="s">
-        <v>169</v>
+        <v>171</v>
       </c>
       <c r="S3" t="s">
-        <v>172</v>
+        <v>174</v>
       </c>
       <c r="T3" t="s">
-        <v>176</v>
+        <v>178</v>
       </c>
       <c r="U3" t="s">
         <v>28</v>
       </c>
-      <c r="V3" s="2">
+      <c r="V3" s="1">
         <v>46291</v>
       </c>
     </row>
@@ -1115,30 +1089,30 @@
         <v>30</v>
       </c>
       <c r="G4" t="s">
-        <v>42</v>
+        <v>43</v>
       </c>
       <c r="N4" t="s">
-        <v>81</v>
+        <v>83</v>
       </c>
       <c r="O4" t="s">
-        <v>101</v>
+        <v>103</v>
       </c>
       <c r="Q4" t="s">
-        <v>166</v>
+        <v>168</v>
       </c>
       <c r="R4" t="s">
-        <v>170</v>
+        <v>172</v>
       </c>
       <c r="S4" t="s">
-        <v>172</v>
+        <v>174</v>
       </c>
       <c r="T4" t="s">
-        <v>176</v>
+        <v>178</v>
       </c>
       <c r="U4" t="s">
         <v>28</v>
       </c>
-      <c r="V4" s="2">
+      <c r="V4" s="1">
         <v>46321</v>
       </c>
     </row>
@@ -1162,30 +1136,27 @@
         <v>30</v>
       </c>
       <c r="N5" t="s">
-        <v>81</v>
+        <v>83</v>
       </c>
       <c r="O5" t="s">
-        <v>102</v>
-      </c>
-      <c r="P5">
-        <v>384180</v>
+        <v>104</v>
       </c>
       <c r="Q5" t="s">
-        <v>166</v>
+        <v>168</v>
       </c>
       <c r="R5" t="s">
-        <v>170</v>
+        <v>172</v>
       </c>
       <c r="S5" t="s">
-        <v>172</v>
+        <v>174</v>
       </c>
       <c r="T5" t="s">
-        <v>176</v>
+        <v>178</v>
       </c>
       <c r="U5" t="s">
         <v>28</v>
       </c>
-      <c r="V5" s="2">
+      <c r="V5" s="1">
         <v>46321</v>
       </c>
     </row>
@@ -1209,33 +1180,30 @@
         <v>30</v>
       </c>
       <c r="L6" t="s">
-        <v>79</v>
+        <v>81</v>
       </c>
       <c r="N6" t="s">
-        <v>82</v>
+        <v>84</v>
       </c>
       <c r="O6" t="s">
-        <v>103</v>
-      </c>
-      <c r="P6">
-        <v>563000</v>
+        <v>105</v>
       </c>
       <c r="Q6" t="s">
-        <v>166</v>
+        <v>168</v>
       </c>
       <c r="R6" t="s">
-        <v>170</v>
+        <v>172</v>
       </c>
       <c r="S6" t="s">
-        <v>172</v>
+        <v>174</v>
       </c>
       <c r="T6" t="s">
-        <v>176</v>
+        <v>178</v>
       </c>
       <c r="U6" t="s">
         <v>28</v>
       </c>
-      <c r="V6" s="2">
+      <c r="V6" s="1">
         <v>46291</v>
       </c>
     </row>
@@ -1259,39 +1227,36 @@
         <v>30</v>
       </c>
       <c r="G7" t="s">
-        <v>43</v>
-      </c>
-      <c r="H7" s="2">
+        <v>44</v>
+      </c>
+      <c r="H7" s="1">
         <v>46121</v>
       </c>
       <c r="I7" t="s">
-        <v>46</v>
+        <v>47</v>
       </c>
       <c r="N7" t="s">
-        <v>83</v>
+        <v>85</v>
       </c>
       <c r="O7" t="s">
-        <v>104</v>
-      </c>
-      <c r="P7">
-        <v>3799999.6</v>
+        <v>106</v>
       </c>
       <c r="Q7" t="s">
-        <v>167</v>
+        <v>169</v>
       </c>
       <c r="R7" t="s">
-        <v>170</v>
+        <v>172</v>
       </c>
       <c r="S7" t="s">
-        <v>172</v>
+        <v>174</v>
       </c>
       <c r="T7" t="s">
-        <v>177</v>
+        <v>179</v>
       </c>
       <c r="U7" t="s">
         <v>28</v>
       </c>
-      <c r="V7" s="2">
+      <c r="V7" s="1">
         <v>46138</v>
       </c>
     </row>
@@ -1315,30 +1280,27 @@
         <v>30</v>
       </c>
       <c r="N8" t="s">
-        <v>81</v>
+        <v>83</v>
       </c>
       <c r="O8" t="s">
-        <v>105</v>
-      </c>
-      <c r="P8">
-        <v>430000</v>
+        <v>107</v>
       </c>
       <c r="Q8" t="s">
-        <v>166</v>
+        <v>168</v>
       </c>
       <c r="R8" t="s">
-        <v>170</v>
+        <v>172</v>
       </c>
       <c r="S8" t="s">
-        <v>172</v>
+        <v>174</v>
       </c>
       <c r="T8" t="s">
-        <v>176</v>
+        <v>178</v>
       </c>
       <c r="U8" t="s">
         <v>28</v>
       </c>
-      <c r="V8" s="2">
+      <c r="V8" s="1">
         <v>46291</v>
       </c>
     </row>
@@ -1362,30 +1324,27 @@
         <v>30</v>
       </c>
       <c r="N9" t="s">
-        <v>81</v>
+        <v>83</v>
       </c>
       <c r="O9" t="s">
-        <v>106</v>
-      </c>
-      <c r="P9">
-        <v>60000</v>
+        <v>108</v>
       </c>
       <c r="Q9" t="s">
-        <v>166</v>
+        <v>168</v>
       </c>
       <c r="R9" t="s">
-        <v>170</v>
+        <v>172</v>
       </c>
       <c r="S9" t="s">
-        <v>172</v>
+        <v>174</v>
       </c>
       <c r="T9" t="s">
-        <v>176</v>
+        <v>178</v>
       </c>
       <c r="U9" t="s">
         <v>28</v>
       </c>
-      <c r="V9" s="2">
+      <c r="V9" s="1">
         <v>46291</v>
       </c>
     </row>
@@ -1409,30 +1368,27 @@
         <v>30</v>
       </c>
       <c r="N10" t="s">
-        <v>82</v>
+        <v>84</v>
       </c>
       <c r="O10" t="s">
-        <v>107</v>
-      </c>
-      <c r="P10">
-        <v>200000</v>
+        <v>109</v>
       </c>
       <c r="Q10" t="s">
-        <v>166</v>
+        <v>168</v>
       </c>
       <c r="R10" t="s">
-        <v>170</v>
+        <v>172</v>
       </c>
       <c r="S10" t="s">
-        <v>172</v>
+        <v>174</v>
       </c>
       <c r="T10" t="s">
-        <v>176</v>
+        <v>178</v>
       </c>
       <c r="U10" t="s">
         <v>28</v>
       </c>
-      <c r="V10" s="2">
+      <c r="V10" s="1">
         <v>46291</v>
       </c>
     </row>
@@ -1456,30 +1412,27 @@
         <v>30</v>
       </c>
       <c r="N11" t="s">
-        <v>82</v>
+        <v>84</v>
       </c>
       <c r="O11" t="s">
-        <v>108</v>
-      </c>
-      <c r="P11">
-        <v>320000</v>
+        <v>110</v>
       </c>
       <c r="Q11" t="s">
-        <v>166</v>
+        <v>168</v>
       </c>
       <c r="R11" t="s">
-        <v>170</v>
+        <v>172</v>
       </c>
       <c r="S11" t="s">
-        <v>172</v>
+        <v>174</v>
       </c>
       <c r="T11" t="s">
-        <v>176</v>
+        <v>178</v>
       </c>
       <c r="U11" t="s">
         <v>28</v>
       </c>
-      <c r="V11" s="2">
+      <c r="V11" s="1">
         <v>46291</v>
       </c>
     </row>
@@ -1503,42 +1456,39 @@
         <v>30</v>
       </c>
       <c r="G12" t="s">
-        <v>43</v>
-      </c>
-      <c r="H12" s="2">
+        <v>44</v>
+      </c>
+      <c r="H12" s="1">
         <v>46079</v>
       </c>
       <c r="I12" t="s">
-        <v>47</v>
+        <v>48</v>
       </c>
       <c r="J12" t="s">
-        <v>64</v>
+        <v>65</v>
       </c>
       <c r="N12" t="s">
-        <v>80</v>
+        <v>82</v>
       </c>
       <c r="O12" t="s">
-        <v>109</v>
-      </c>
-      <c r="P12">
-        <v>1187433.02</v>
+        <v>111</v>
       </c>
       <c r="Q12" t="s">
-        <v>166</v>
+        <v>168</v>
       </c>
       <c r="R12" t="s">
-        <v>169</v>
+        <v>171</v>
       </c>
       <c r="S12" t="s">
-        <v>172</v>
+        <v>174</v>
       </c>
       <c r="T12" t="s">
-        <v>176</v>
+        <v>178</v>
       </c>
       <c r="U12" t="s">
-        <v>181</v>
-      </c>
-      <c r="V12" s="2">
+        <v>183</v>
+      </c>
+      <c r="V12" s="1">
         <v>46079</v>
       </c>
     </row>
@@ -1562,36 +1512,33 @@
         <v>30</v>
       </c>
       <c r="J13" t="s">
-        <v>63</v>
+        <v>64</v>
       </c>
       <c r="K13" t="s">
-        <v>72</v>
+        <v>73</v>
       </c>
       <c r="N13" t="s">
-        <v>80</v>
+        <v>82</v>
       </c>
       <c r="O13" t="s">
-        <v>110</v>
-      </c>
-      <c r="P13">
-        <v>1000000</v>
+        <v>112</v>
       </c>
       <c r="Q13" t="s">
-        <v>166</v>
+        <v>168</v>
       </c>
       <c r="R13" t="s">
-        <v>169</v>
+        <v>171</v>
       </c>
       <c r="S13" t="s">
-        <v>172</v>
+        <v>174</v>
       </c>
       <c r="T13" t="s">
-        <v>176</v>
+        <v>178</v>
       </c>
       <c r="U13" t="s">
-        <v>181</v>
-      </c>
-      <c r="V13" s="2">
+        <v>183</v>
+      </c>
+      <c r="V13" s="1">
         <v>46352</v>
       </c>
     </row>
@@ -1615,36 +1562,33 @@
         <v>30</v>
       </c>
       <c r="J14" t="s">
-        <v>63</v>
+        <v>64</v>
       </c>
       <c r="K14" t="s">
-        <v>72</v>
+        <v>73</v>
       </c>
       <c r="N14" t="s">
-        <v>80</v>
+        <v>82</v>
       </c>
       <c r="O14" t="s">
-        <v>111</v>
-      </c>
-      <c r="P14">
-        <v>1000000</v>
+        <v>113</v>
       </c>
       <c r="Q14" t="s">
-        <v>166</v>
+        <v>168</v>
       </c>
       <c r="R14" t="s">
-        <v>169</v>
+        <v>171</v>
       </c>
       <c r="S14" t="s">
-        <v>172</v>
+        <v>174</v>
       </c>
       <c r="T14" t="s">
-        <v>176</v>
+        <v>178</v>
       </c>
       <c r="U14" t="s">
-        <v>181</v>
-      </c>
-      <c r="V14" s="2">
+        <v>183</v>
+      </c>
+      <c r="V14" s="1">
         <v>46352</v>
       </c>
     </row>
@@ -1668,36 +1612,33 @@
         <v>30</v>
       </c>
       <c r="J15" t="s">
-        <v>63</v>
+        <v>64</v>
       </c>
       <c r="K15" t="s">
-        <v>72</v>
+        <v>73</v>
       </c>
       <c r="N15" t="s">
-        <v>80</v>
+        <v>82</v>
       </c>
       <c r="O15" t="s">
-        <v>112</v>
-      </c>
-      <c r="P15">
-        <v>1000000</v>
+        <v>114</v>
       </c>
       <c r="Q15" t="s">
-        <v>166</v>
+        <v>168</v>
       </c>
       <c r="R15" t="s">
-        <v>169</v>
+        <v>171</v>
       </c>
       <c r="S15" t="s">
-        <v>172</v>
+        <v>174</v>
       </c>
       <c r="T15" t="s">
-        <v>176</v>
+        <v>178</v>
       </c>
       <c r="U15" t="s">
-        <v>181</v>
-      </c>
-      <c r="V15" s="2">
+        <v>183</v>
+      </c>
+      <c r="V15" s="1">
         <v>46352</v>
       </c>
     </row>
@@ -1721,36 +1662,33 @@
         <v>30</v>
       </c>
       <c r="J16" t="s">
-        <v>63</v>
+        <v>64</v>
       </c>
       <c r="K16" t="s">
-        <v>72</v>
+        <v>73</v>
       </c>
       <c r="N16" t="s">
-        <v>84</v>
+        <v>86</v>
       </c>
       <c r="O16" t="s">
-        <v>113</v>
-      </c>
-      <c r="P16">
-        <v>100000</v>
+        <v>115</v>
       </c>
       <c r="Q16" t="s">
-        <v>168</v>
+        <v>170</v>
       </c>
       <c r="R16" t="s">
-        <v>169</v>
+        <v>171</v>
       </c>
       <c r="S16" t="s">
-        <v>172</v>
+        <v>174</v>
       </c>
       <c r="T16" t="s">
-        <v>176</v>
+        <v>178</v>
       </c>
       <c r="U16" t="s">
-        <v>181</v>
-      </c>
-      <c r="V16" s="2">
+        <v>183</v>
+      </c>
+      <c r="V16" s="1">
         <v>46229</v>
       </c>
     </row>
@@ -1774,42 +1712,39 @@
         <v>30</v>
       </c>
       <c r="G17" t="s">
-        <v>43</v>
-      </c>
-      <c r="H17" s="2">
+        <v>44</v>
+      </c>
+      <c r="H17" s="1">
         <v>46098</v>
       </c>
       <c r="I17" t="s">
-        <v>48</v>
+        <v>49</v>
       </c>
       <c r="J17" t="s">
-        <v>64</v>
+        <v>65</v>
       </c>
       <c r="N17" t="s">
-        <v>85</v>
+        <v>87</v>
       </c>
       <c r="O17" t="s">
-        <v>114</v>
-      </c>
-      <c r="P17">
-        <v>1770880.5</v>
+        <v>116</v>
       </c>
       <c r="Q17" t="s">
-        <v>167</v>
+        <v>169</v>
       </c>
       <c r="R17" t="s">
-        <v>170</v>
+        <v>172</v>
       </c>
       <c r="S17" t="s">
-        <v>172</v>
+        <v>174</v>
       </c>
       <c r="T17" t="s">
-        <v>178</v>
+        <v>180</v>
       </c>
       <c r="U17" t="s">
-        <v>181</v>
-      </c>
-      <c r="V17" s="2">
+        <v>183</v>
+      </c>
+      <c r="V17" s="1">
         <v>46107</v>
       </c>
     </row>
@@ -1833,39 +1768,36 @@
         <v>30</v>
       </c>
       <c r="G18" t="s">
-        <v>43</v>
-      </c>
-      <c r="H18" s="2">
+        <v>44</v>
+      </c>
+      <c r="H18" s="1">
         <v>46076</v>
       </c>
       <c r="I18" t="s">
-        <v>49</v>
+        <v>50</v>
       </c>
       <c r="N18" t="s">
-        <v>86</v>
+        <v>88</v>
       </c>
       <c r="O18" t="s">
-        <v>115</v>
-      </c>
-      <c r="P18">
-        <v>350000</v>
+        <v>117</v>
       </c>
       <c r="Q18" t="s">
-        <v>167</v>
+        <v>169</v>
       </c>
       <c r="R18" t="s">
-        <v>169</v>
+        <v>171</v>
       </c>
       <c r="S18" t="s">
-        <v>172</v>
+        <v>174</v>
       </c>
       <c r="T18" t="s">
-        <v>177</v>
+        <v>179</v>
       </c>
       <c r="U18" t="s">
         <v>28</v>
       </c>
-      <c r="V18" s="2">
+      <c r="V18" s="1">
         <v>46079</v>
       </c>
     </row>
@@ -1889,39 +1821,36 @@
         <v>30</v>
       </c>
       <c r="G19" t="s">
-        <v>43</v>
-      </c>
-      <c r="H19" s="2">
+        <v>44</v>
+      </c>
+      <c r="H19" s="1">
         <v>46076</v>
       </c>
       <c r="I19" t="s">
-        <v>49</v>
+        <v>50</v>
       </c>
       <c r="N19" t="s">
-        <v>86</v>
+        <v>88</v>
       </c>
       <c r="O19" t="s">
-        <v>116</v>
-      </c>
-      <c r="P19">
-        <v>350000</v>
+        <v>118</v>
       </c>
       <c r="Q19" t="s">
-        <v>167</v>
+        <v>169</v>
       </c>
       <c r="R19" t="s">
-        <v>169</v>
+        <v>171</v>
       </c>
       <c r="S19" t="s">
-        <v>172</v>
+        <v>174</v>
       </c>
       <c r="T19" t="s">
-        <v>177</v>
+        <v>179</v>
       </c>
       <c r="U19" t="s">
         <v>28</v>
       </c>
-      <c r="V19" s="2">
+      <c r="V19" s="1">
         <v>46079</v>
       </c>
     </row>
@@ -1945,30 +1874,27 @@
         <v>30</v>
       </c>
       <c r="N20" t="s">
-        <v>87</v>
+        <v>89</v>
       </c>
       <c r="O20" t="s">
-        <v>117</v>
-      </c>
-      <c r="P20">
-        <v>1000000</v>
+        <v>119</v>
       </c>
       <c r="Q20" t="s">
-        <v>167</v>
+        <v>169</v>
       </c>
       <c r="R20" t="s">
-        <v>169</v>
+        <v>171</v>
       </c>
       <c r="S20" t="s">
-        <v>172</v>
+        <v>174</v>
       </c>
       <c r="T20" t="s">
-        <v>177</v>
+        <v>179</v>
       </c>
       <c r="U20" t="s">
         <v>28</v>
       </c>
-      <c r="V20" s="2">
+      <c r="V20" s="1">
         <v>46321</v>
       </c>
     </row>
@@ -1992,30 +1918,27 @@
         <v>30</v>
       </c>
       <c r="N21" t="s">
-        <v>80</v>
+        <v>82</v>
       </c>
       <c r="O21" t="s">
-        <v>118</v>
-      </c>
-      <c r="P21">
-        <v>400000</v>
+        <v>120</v>
       </c>
       <c r="Q21" t="s">
-        <v>166</v>
+        <v>168</v>
       </c>
       <c r="R21" t="s">
-        <v>169</v>
+        <v>171</v>
       </c>
       <c r="S21" t="s">
-        <v>172</v>
+        <v>174</v>
       </c>
       <c r="T21" t="s">
-        <v>176</v>
+        <v>178</v>
       </c>
       <c r="U21" t="s">
         <v>28</v>
       </c>
-      <c r="V21" s="2">
+      <c r="V21" s="1">
         <v>46321</v>
       </c>
     </row>
@@ -2039,30 +1962,27 @@
         <v>30</v>
       </c>
       <c r="N22" t="s">
-        <v>81</v>
+        <v>83</v>
       </c>
       <c r="O22" t="s">
-        <v>119</v>
-      </c>
-      <c r="P22">
-        <v>120000</v>
+        <v>121</v>
       </c>
       <c r="Q22" t="s">
-        <v>166</v>
+        <v>168</v>
       </c>
       <c r="R22" t="s">
-        <v>170</v>
+        <v>172</v>
       </c>
       <c r="S22" t="s">
-        <v>172</v>
+        <v>174</v>
       </c>
       <c r="T22" t="s">
-        <v>176</v>
+        <v>178</v>
       </c>
       <c r="U22" t="s">
         <v>28</v>
       </c>
-      <c r="V22" s="2">
+      <c r="V22" s="1">
         <v>46321</v>
       </c>
     </row>
@@ -2086,30 +2006,27 @@
         <v>30</v>
       </c>
       <c r="N23" t="s">
-        <v>81</v>
+        <v>83</v>
       </c>
       <c r="O23" t="s">
-        <v>120</v>
-      </c>
-      <c r="P23">
-        <v>80000</v>
+        <v>122</v>
       </c>
       <c r="Q23" t="s">
-        <v>166</v>
+        <v>168</v>
       </c>
       <c r="R23" t="s">
-        <v>170</v>
+        <v>172</v>
       </c>
       <c r="S23" t="s">
-        <v>172</v>
+        <v>174</v>
       </c>
       <c r="T23" t="s">
-        <v>176</v>
+        <v>178</v>
       </c>
       <c r="U23" t="s">
         <v>28</v>
       </c>
-      <c r="V23" s="2">
+      <c r="V23" s="1">
         <v>46321</v>
       </c>
     </row>
@@ -2133,42 +2050,39 @@
         <v>31</v>
       </c>
       <c r="G24" t="s">
-        <v>43</v>
-      </c>
-      <c r="H24" s="2">
+        <v>44</v>
+      </c>
+      <c r="H24" s="1">
         <v>46119</v>
       </c>
       <c r="I24" t="s">
-        <v>50</v>
+        <v>51</v>
       </c>
       <c r="J24" t="s">
-        <v>65</v>
+        <v>66</v>
       </c>
       <c r="N24" t="s">
-        <v>85</v>
+        <v>87</v>
       </c>
       <c r="O24" t="s">
-        <v>121</v>
-      </c>
-      <c r="P24">
-        <v>1704503</v>
+        <v>123</v>
       </c>
       <c r="Q24" t="s">
-        <v>167</v>
+        <v>169</v>
       </c>
       <c r="R24" t="s">
-        <v>170</v>
+        <v>172</v>
       </c>
       <c r="S24" t="s">
-        <v>172</v>
+        <v>174</v>
       </c>
       <c r="T24" t="s">
-        <v>178</v>
+        <v>180</v>
       </c>
       <c r="U24" t="s">
-        <v>181</v>
-      </c>
-      <c r="V24" s="2">
+        <v>183</v>
+      </c>
+      <c r="V24" s="1">
         <v>46138</v>
       </c>
     </row>
@@ -2192,39 +2106,36 @@
         <v>30</v>
       </c>
       <c r="G25" t="s">
-        <v>43</v>
-      </c>
-      <c r="H25" s="2">
+        <v>44</v>
+      </c>
+      <c r="H25" s="1">
         <v>46121</v>
       </c>
       <c r="I25" t="s">
-        <v>51</v>
+        <v>52</v>
       </c>
       <c r="N25" t="s">
-        <v>88</v>
+        <v>90</v>
       </c>
       <c r="O25" t="s">
-        <v>122</v>
-      </c>
-      <c r="P25">
-        <v>3799000</v>
+        <v>124</v>
       </c>
       <c r="Q25" t="s">
-        <v>167</v>
+        <v>169</v>
       </c>
       <c r="R25" t="s">
-        <v>170</v>
+        <v>172</v>
       </c>
       <c r="S25" t="s">
-        <v>172</v>
+        <v>174</v>
       </c>
       <c r="T25" t="s">
-        <v>177</v>
+        <v>179</v>
       </c>
       <c r="U25" t="s">
         <v>28</v>
       </c>
-      <c r="V25" s="2">
+      <c r="V25" s="1">
         <v>46138</v>
       </c>
     </row>
@@ -2248,39 +2159,36 @@
         <v>30</v>
       </c>
       <c r="G26" t="s">
-        <v>43</v>
-      </c>
-      <c r="H26" s="2">
+        <v>44</v>
+      </c>
+      <c r="H26" s="1">
         <v>46076</v>
       </c>
       <c r="I26" t="s">
-        <v>52</v>
+        <v>53</v>
       </c>
       <c r="N26" t="s">
-        <v>88</v>
+        <v>90</v>
       </c>
       <c r="O26" t="s">
-        <v>122</v>
-      </c>
-      <c r="P26">
-        <v>1000</v>
+        <v>124</v>
       </c>
       <c r="Q26" t="s">
-        <v>167</v>
+        <v>169</v>
       </c>
       <c r="R26" t="s">
-        <v>169</v>
+        <v>171</v>
       </c>
       <c r="S26" t="s">
-        <v>172</v>
+        <v>174</v>
       </c>
       <c r="T26" t="s">
-        <v>177</v>
+        <v>179</v>
       </c>
       <c r="U26" t="s">
         <v>28</v>
       </c>
-      <c r="V26" s="2">
+      <c r="V26" s="1">
         <v>46079</v>
       </c>
     </row>
@@ -2304,36 +2212,33 @@
         <v>30</v>
       </c>
       <c r="J27" t="s">
-        <v>63</v>
+        <v>64</v>
       </c>
       <c r="K27" t="s">
-        <v>72</v>
+        <v>73</v>
       </c>
       <c r="N27" t="s">
-        <v>84</v>
+        <v>86</v>
       </c>
       <c r="O27" t="s">
-        <v>123</v>
-      </c>
-      <c r="P27">
-        <v>100000</v>
+        <v>125</v>
       </c>
       <c r="Q27" t="s">
-        <v>168</v>
+        <v>170</v>
       </c>
       <c r="R27" t="s">
-        <v>169</v>
+        <v>171</v>
       </c>
       <c r="S27" t="s">
-        <v>172</v>
+        <v>174</v>
       </c>
       <c r="T27" t="s">
-        <v>176</v>
+        <v>178</v>
       </c>
       <c r="U27" t="s">
-        <v>181</v>
-      </c>
-      <c r="V27" s="2">
+        <v>183</v>
+      </c>
+      <c r="V27" s="1">
         <v>46291</v>
       </c>
     </row>
@@ -2357,42 +2262,39 @@
         <v>32</v>
       </c>
       <c r="G28" t="s">
-        <v>43</v>
-      </c>
-      <c r="H28" s="2">
+        <v>44</v>
+      </c>
+      <c r="H28" s="1">
         <v>46199</v>
       </c>
       <c r="I28" t="s">
-        <v>53</v>
+        <v>54</v>
       </c>
       <c r="J28" t="s">
-        <v>66</v>
+        <v>67</v>
       </c>
       <c r="N28" t="s">
-        <v>85</v>
+        <v>87</v>
       </c>
       <c r="O28" t="s">
-        <v>124</v>
-      </c>
-      <c r="P28">
-        <v>150000</v>
+        <v>126</v>
       </c>
       <c r="Q28" t="s">
-        <v>167</v>
+        <v>169</v>
       </c>
       <c r="R28" t="s">
-        <v>170</v>
+        <v>172</v>
       </c>
       <c r="S28" t="s">
-        <v>172</v>
+        <v>174</v>
       </c>
       <c r="T28" t="s">
-        <v>177</v>
+        <v>179</v>
       </c>
       <c r="U28" t="s">
-        <v>181</v>
-      </c>
-      <c r="V28" s="2">
+        <v>183</v>
+      </c>
+      <c r="V28" s="1">
         <v>46199</v>
       </c>
     </row>
@@ -2416,42 +2318,39 @@
         <v>32</v>
       </c>
       <c r="G29" t="s">
-        <v>43</v>
-      </c>
-      <c r="H29" s="2">
+        <v>44</v>
+      </c>
+      <c r="H29" s="1">
         <v>46199</v>
       </c>
       <c r="I29" t="s">
-        <v>53</v>
+        <v>54</v>
       </c>
       <c r="J29" t="s">
-        <v>66</v>
+        <v>67</v>
       </c>
       <c r="N29" t="s">
-        <v>85</v>
+        <v>87</v>
       </c>
       <c r="O29" t="s">
-        <v>125</v>
-      </c>
-      <c r="P29">
-        <v>150000</v>
+        <v>127</v>
       </c>
       <c r="Q29" t="s">
-        <v>167</v>
+        <v>169</v>
       </c>
       <c r="R29" t="s">
-        <v>170</v>
+        <v>172</v>
       </c>
       <c r="S29" t="s">
-        <v>172</v>
+        <v>174</v>
       </c>
       <c r="T29" t="s">
-        <v>177</v>
+        <v>179</v>
       </c>
       <c r="U29" t="s">
-        <v>181</v>
-      </c>
-      <c r="V29" s="2">
+        <v>183</v>
+      </c>
+      <c r="V29" s="1">
         <v>46199</v>
       </c>
     </row>
@@ -2475,42 +2374,39 @@
         <v>33</v>
       </c>
       <c r="G30" t="s">
-        <v>43</v>
-      </c>
-      <c r="H30" s="2">
+        <v>44</v>
+      </c>
+      <c r="H30" s="1">
         <v>46199</v>
       </c>
       <c r="I30" t="s">
-        <v>54</v>
+        <v>55</v>
       </c>
       <c r="J30" t="s">
-        <v>66</v>
+        <v>67</v>
       </c>
       <c r="N30" t="s">
-        <v>85</v>
+        <v>87</v>
       </c>
       <c r="O30" t="s">
-        <v>126</v>
-      </c>
-      <c r="P30">
-        <v>18462.36</v>
+        <v>128</v>
       </c>
       <c r="Q30" t="s">
-        <v>167</v>
+        <v>169</v>
       </c>
       <c r="R30" t="s">
-        <v>170</v>
+        <v>172</v>
       </c>
       <c r="S30" t="s">
-        <v>172</v>
+        <v>174</v>
       </c>
       <c r="T30" t="s">
-        <v>177</v>
+        <v>179</v>
       </c>
       <c r="U30" t="s">
-        <v>181</v>
-      </c>
-      <c r="V30" s="2">
+        <v>183</v>
+      </c>
+      <c r="V30" s="1">
         <v>46199</v>
       </c>
     </row>
@@ -2534,42 +2430,39 @@
         <v>32</v>
       </c>
       <c r="G31" t="s">
-        <v>43</v>
-      </c>
-      <c r="H31" s="2">
+        <v>44</v>
+      </c>
+      <c r="H31" s="1">
         <v>46199</v>
       </c>
       <c r="I31" t="s">
-        <v>53</v>
+        <v>54</v>
       </c>
       <c r="J31" t="s">
-        <v>66</v>
+        <v>67</v>
       </c>
       <c r="N31" t="s">
-        <v>85</v>
+        <v>87</v>
       </c>
       <c r="O31" t="s">
-        <v>126</v>
-      </c>
-      <c r="P31">
-        <v>324166.14</v>
+        <v>128</v>
       </c>
       <c r="Q31" t="s">
-        <v>167</v>
+        <v>169</v>
       </c>
       <c r="R31" t="s">
-        <v>170</v>
+        <v>172</v>
       </c>
       <c r="S31" t="s">
-        <v>172</v>
+        <v>174</v>
       </c>
       <c r="T31" t="s">
-        <v>177</v>
+        <v>179</v>
       </c>
       <c r="U31" t="s">
-        <v>181</v>
-      </c>
-      <c r="V31" s="2">
+        <v>183</v>
+      </c>
+      <c r="V31" s="1">
         <v>46199</v>
       </c>
     </row>
@@ -2593,33 +2486,30 @@
         <v>30</v>
       </c>
       <c r="K32" t="s">
-        <v>73</v>
+        <v>74</v>
       </c>
       <c r="N32" t="s">
-        <v>85</v>
+        <v>87</v>
       </c>
       <c r="O32" t="s">
-        <v>127</v>
-      </c>
-      <c r="P32">
-        <v>30000</v>
+        <v>129</v>
       </c>
       <c r="Q32" t="s">
-        <v>167</v>
+        <v>169</v>
       </c>
       <c r="R32" t="s">
-        <v>170</v>
+        <v>172</v>
       </c>
       <c r="S32" t="s">
-        <v>172</v>
+        <v>174</v>
       </c>
       <c r="T32" t="s">
-        <v>177</v>
+        <v>179</v>
       </c>
       <c r="U32" t="s">
-        <v>181</v>
-      </c>
-      <c r="V32" s="2">
+        <v>183</v>
+      </c>
+      <c r="V32" s="1">
         <v>46291</v>
       </c>
     </row>
@@ -2643,42 +2533,39 @@
         <v>30</v>
       </c>
       <c r="G33" t="s">
-        <v>43</v>
-      </c>
-      <c r="H33" s="2">
+        <v>44</v>
+      </c>
+      <c r="H33" s="1">
         <v>46191</v>
       </c>
       <c r="I33" t="s">
-        <v>55</v>
+        <v>56</v>
       </c>
       <c r="J33" t="s">
-        <v>67</v>
+        <v>68</v>
       </c>
       <c r="N33" t="s">
-        <v>85</v>
+        <v>87</v>
       </c>
       <c r="O33" t="s">
-        <v>128</v>
-      </c>
-      <c r="P33">
-        <v>1496713.48</v>
+        <v>130</v>
       </c>
       <c r="Q33" t="s">
-        <v>167</v>
+        <v>169</v>
       </c>
       <c r="R33" t="s">
-        <v>170</v>
+        <v>172</v>
       </c>
       <c r="S33" t="s">
-        <v>172</v>
+        <v>174</v>
       </c>
       <c r="T33" t="s">
-        <v>178</v>
+        <v>180</v>
       </c>
       <c r="U33" t="s">
-        <v>181</v>
-      </c>
-      <c r="V33" s="2">
+        <v>183</v>
+      </c>
+      <c r="V33" s="1">
         <v>46199</v>
       </c>
     </row>
@@ -2702,39 +2589,36 @@
         <v>31</v>
       </c>
       <c r="G34" t="s">
-        <v>43</v>
-      </c>
-      <c r="H34" s="2">
+        <v>44</v>
+      </c>
+      <c r="H34" s="1">
         <v>46119</v>
       </c>
       <c r="I34" t="s">
-        <v>50</v>
+        <v>51</v>
       </c>
       <c r="N34" t="s">
-        <v>85</v>
+        <v>87</v>
       </c>
       <c r="O34" t="s">
-        <v>128</v>
-      </c>
-      <c r="P34">
-        <v>207789.52</v>
+        <v>130</v>
       </c>
       <c r="Q34" t="s">
-        <v>167</v>
+        <v>169</v>
       </c>
       <c r="R34" t="s">
-        <v>170</v>
+        <v>172</v>
       </c>
       <c r="S34" t="s">
-        <v>172</v>
+        <v>174</v>
       </c>
       <c r="T34" t="s">
-        <v>178</v>
+        <v>180</v>
       </c>
       <c r="U34" t="s">
-        <v>181</v>
-      </c>
-      <c r="V34" s="2">
+        <v>183</v>
+      </c>
+      <c r="V34" s="1">
         <v>46138</v>
       </c>
     </row>
@@ -2758,39 +2642,36 @@
         <v>30</v>
       </c>
       <c r="G35" t="s">
-        <v>43</v>
-      </c>
-      <c r="H35" s="2">
+        <v>44</v>
+      </c>
+      <c r="H35" s="1">
         <v>46213</v>
       </c>
       <c r="I35" t="s">
-        <v>56</v>
+        <v>57</v>
       </c>
       <c r="N35" t="s">
-        <v>88</v>
+        <v>90</v>
       </c>
       <c r="O35" t="s">
-        <v>129</v>
-      </c>
-      <c r="P35">
-        <v>962290.8</v>
+        <v>131</v>
       </c>
       <c r="Q35" t="s">
-        <v>167</v>
+        <v>169</v>
       </c>
       <c r="R35" t="s">
-        <v>169</v>
+        <v>171</v>
       </c>
       <c r="S35" t="s">
-        <v>172</v>
+        <v>174</v>
       </c>
       <c r="T35" t="s">
-        <v>177</v>
+        <v>179</v>
       </c>
       <c r="U35" t="s">
         <v>28</v>
       </c>
-      <c r="V35" s="2">
+      <c r="V35" s="1">
         <v>46229</v>
       </c>
     </row>
@@ -2814,39 +2695,36 @@
         <v>34</v>
       </c>
       <c r="G36" t="s">
-        <v>43</v>
-      </c>
-      <c r="H36" s="2">
+        <v>44</v>
+      </c>
+      <c r="H36" s="1">
         <v>46175</v>
       </c>
       <c r="I36" t="s">
-        <v>57</v>
+        <v>58</v>
       </c>
       <c r="N36" t="s">
-        <v>88</v>
+        <v>90</v>
       </c>
       <c r="O36" t="s">
-        <v>129</v>
-      </c>
-      <c r="P36">
-        <v>798776.97</v>
+        <v>131</v>
       </c>
       <c r="Q36" t="s">
-        <v>167</v>
+        <v>169</v>
       </c>
       <c r="R36" t="s">
-        <v>170</v>
+        <v>172</v>
       </c>
       <c r="S36" t="s">
-        <v>172</v>
+        <v>174</v>
       </c>
       <c r="T36" t="s">
-        <v>177</v>
+        <v>179</v>
       </c>
       <c r="U36" t="s">
         <v>28</v>
       </c>
-      <c r="V36" s="2">
+      <c r="V36" s="1">
         <v>46199</v>
       </c>
     </row>
@@ -2870,39 +2748,36 @@
         <v>30</v>
       </c>
       <c r="G37" t="s">
-        <v>43</v>
-      </c>
-      <c r="H37" s="2">
+        <v>44</v>
+      </c>
+      <c r="H37" s="1">
         <v>46213</v>
       </c>
       <c r="I37" t="s">
-        <v>56</v>
+        <v>57</v>
       </c>
       <c r="N37" t="s">
-        <v>88</v>
+        <v>90</v>
       </c>
       <c r="O37" t="s">
-        <v>129</v>
-      </c>
-      <c r="P37">
-        <v>1530656.62</v>
+        <v>131</v>
       </c>
       <c r="Q37" t="s">
-        <v>167</v>
+        <v>169</v>
       </c>
       <c r="R37" t="s">
-        <v>169</v>
+        <v>171</v>
       </c>
       <c r="S37" t="s">
-        <v>172</v>
+        <v>174</v>
       </c>
       <c r="T37" t="s">
-        <v>177</v>
+        <v>179</v>
       </c>
       <c r="U37" t="s">
         <v>28</v>
       </c>
-      <c r="V37" s="2">
+      <c r="V37" s="1">
         <v>46229</v>
       </c>
     </row>
@@ -2926,39 +2801,36 @@
         <v>35</v>
       </c>
       <c r="G38" t="s">
-        <v>43</v>
-      </c>
-      <c r="H38" s="2">
+        <v>44</v>
+      </c>
+      <c r="H38" s="1">
         <v>46199</v>
       </c>
       <c r="I38" t="s">
-        <v>58</v>
+        <v>59</v>
       </c>
       <c r="N38" t="s">
-        <v>88</v>
+        <v>90</v>
       </c>
       <c r="O38" t="s">
-        <v>129</v>
-      </c>
-      <c r="P38">
-        <v>72958.08</v>
+        <v>131</v>
       </c>
       <c r="Q38" t="s">
-        <v>167</v>
+        <v>169</v>
       </c>
       <c r="R38" t="s">
-        <v>169</v>
+        <v>171</v>
       </c>
       <c r="S38" t="s">
-        <v>172</v>
+        <v>174</v>
       </c>
       <c r="T38" t="s">
-        <v>177</v>
+        <v>179</v>
       </c>
       <c r="U38" t="s">
         <v>28</v>
       </c>
-      <c r="V38" s="2">
+      <c r="V38" s="1">
         <v>46199</v>
       </c>
     </row>
@@ -2982,39 +2854,36 @@
         <v>36</v>
       </c>
       <c r="G39" t="s">
-        <v>43</v>
-      </c>
-      <c r="H39" s="2">
+        <v>44</v>
+      </c>
+      <c r="H39" s="1">
         <v>46199</v>
       </c>
       <c r="I39" t="s">
-        <v>58</v>
+        <v>59</v>
       </c>
       <c r="N39" t="s">
-        <v>88</v>
+        <v>90</v>
       </c>
       <c r="O39" t="s">
-        <v>129</v>
-      </c>
-      <c r="P39">
-        <v>8916</v>
+        <v>131</v>
       </c>
       <c r="Q39" t="s">
-        <v>167</v>
+        <v>169</v>
       </c>
       <c r="R39" t="s">
-        <v>169</v>
+        <v>171</v>
       </c>
       <c r="S39" t="s">
-        <v>172</v>
+        <v>174</v>
       </c>
       <c r="T39" t="s">
-        <v>177</v>
+        <v>179</v>
       </c>
       <c r="U39" t="s">
         <v>28</v>
       </c>
-      <c r="V39" s="2">
+      <c r="V39" s="1">
         <v>46199</v>
       </c>
     </row>
@@ -3038,39 +2907,36 @@
         <v>37</v>
       </c>
       <c r="G40" t="s">
-        <v>43</v>
-      </c>
-      <c r="H40" s="2">
+        <v>44</v>
+      </c>
+      <c r="H40" s="1">
         <v>46204</v>
       </c>
       <c r="I40" t="s">
-        <v>58</v>
+        <v>59</v>
       </c>
       <c r="N40" t="s">
-        <v>88</v>
+        <v>90</v>
       </c>
       <c r="O40" t="s">
-        <v>129</v>
-      </c>
-      <c r="P40">
-        <v>425178.5</v>
+        <v>131</v>
       </c>
       <c r="Q40" t="s">
-        <v>167</v>
+        <v>169</v>
       </c>
       <c r="R40" t="s">
-        <v>169</v>
+        <v>171</v>
       </c>
       <c r="S40" t="s">
-        <v>172</v>
+        <v>174</v>
       </c>
       <c r="T40" t="s">
-        <v>177</v>
+        <v>179</v>
       </c>
       <c r="U40" t="s">
         <v>28</v>
       </c>
-      <c r="V40" s="2">
+      <c r="V40" s="1">
         <v>46229</v>
       </c>
     </row>
@@ -3094,39 +2960,36 @@
         <v>34</v>
       </c>
       <c r="G41" t="s">
-        <v>43</v>
-      </c>
-      <c r="H41" s="2">
+        <v>44</v>
+      </c>
+      <c r="H41" s="1">
         <v>46244</v>
       </c>
       <c r="I41" t="s">
-        <v>59</v>
+        <v>60</v>
       </c>
       <c r="N41" t="s">
-        <v>88</v>
+        <v>90</v>
       </c>
       <c r="O41" t="s">
-        <v>129</v>
-      </c>
-      <c r="P41">
-        <v>1223.03</v>
+        <v>131</v>
       </c>
       <c r="Q41" t="s">
-        <v>167</v>
+        <v>169</v>
       </c>
       <c r="R41" t="s">
-        <v>169</v>
+        <v>171</v>
       </c>
       <c r="S41" t="s">
-        <v>172</v>
+        <v>174</v>
       </c>
       <c r="T41" t="s">
-        <v>177</v>
+        <v>179</v>
       </c>
       <c r="U41" t="s">
         <v>28</v>
       </c>
-      <c r="V41" s="2">
+      <c r="V41" s="1">
         <v>46199</v>
       </c>
     </row>
@@ -3147,30 +3010,30 @@
         <v>29</v>
       </c>
       <c r="G42" t="s">
-        <v>42</v>
+        <v>43</v>
       </c>
       <c r="N42" t="s">
-        <v>88</v>
+        <v>90</v>
       </c>
       <c r="O42" t="s">
-        <v>130</v>
+        <v>132</v>
       </c>
       <c r="Q42" t="s">
-        <v>167</v>
+        <v>169</v>
       </c>
       <c r="R42" t="s">
-        <v>169</v>
+        <v>171</v>
       </c>
       <c r="S42" t="s">
-        <v>173</v>
+        <v>175</v>
       </c>
       <c r="T42" t="s">
-        <v>177</v>
+        <v>179</v>
       </c>
       <c r="U42" t="s">
         <v>28</v>
       </c>
-      <c r="V42" s="2">
+      <c r="V42" s="1">
         <v>46260</v>
       </c>
     </row>
@@ -3194,39 +3057,36 @@
         <v>30</v>
       </c>
       <c r="G43" t="s">
-        <v>43</v>
-      </c>
-      <c r="H43" s="2">
+        <v>44</v>
+      </c>
+      <c r="H43" s="1">
         <v>46191</v>
       </c>
       <c r="I43" t="s">
-        <v>60</v>
+        <v>61</v>
       </c>
       <c r="N43" t="s">
-        <v>86</v>
+        <v>88</v>
       </c>
       <c r="O43" t="s">
-        <v>131</v>
-      </c>
-      <c r="P43">
-        <v>400000</v>
+        <v>133</v>
       </c>
       <c r="Q43" t="s">
-        <v>167</v>
+        <v>169</v>
       </c>
       <c r="R43" t="s">
-        <v>169</v>
+        <v>171</v>
       </c>
       <c r="S43" t="s">
-        <v>172</v>
+        <v>174</v>
       </c>
       <c r="T43" t="s">
-        <v>177</v>
+        <v>179</v>
       </c>
       <c r="U43" t="s">
         <v>28</v>
       </c>
-      <c r="V43" s="2">
+      <c r="V43" s="1">
         <v>46199</v>
       </c>
     </row>
@@ -3250,39 +3110,36 @@
         <v>30</v>
       </c>
       <c r="G44" t="s">
-        <v>43</v>
-      </c>
-      <c r="H44" s="2">
+        <v>44</v>
+      </c>
+      <c r="H44" s="1">
         <v>46191</v>
       </c>
       <c r="I44" t="s">
-        <v>60</v>
+        <v>61</v>
       </c>
       <c r="N44" t="s">
-        <v>86</v>
+        <v>88</v>
       </c>
       <c r="O44" t="s">
-        <v>132</v>
-      </c>
-      <c r="P44">
-        <v>400000</v>
+        <v>134</v>
       </c>
       <c r="Q44" t="s">
-        <v>167</v>
+        <v>169</v>
       </c>
       <c r="R44" t="s">
-        <v>169</v>
+        <v>171</v>
       </c>
       <c r="S44" t="s">
-        <v>172</v>
+        <v>174</v>
       </c>
       <c r="T44" t="s">
-        <v>177</v>
+        <v>179</v>
       </c>
       <c r="U44" t="s">
         <v>28</v>
       </c>
-      <c r="V44" s="2">
+      <c r="V44" s="1">
         <v>46199</v>
       </c>
     </row>
@@ -3306,42 +3163,39 @@
         <v>30</v>
       </c>
       <c r="G45" t="s">
-        <v>43</v>
-      </c>
-      <c r="H45" s="2">
+        <v>44</v>
+      </c>
+      <c r="H45" s="1">
         <v>46213</v>
       </c>
       <c r="I45" t="s">
-        <v>55</v>
+        <v>56</v>
       </c>
       <c r="J45" t="s">
-        <v>68</v>
+        <v>69</v>
       </c>
       <c r="N45" t="s">
-        <v>85</v>
+        <v>87</v>
       </c>
       <c r="O45" t="s">
-        <v>133</v>
-      </c>
-      <c r="P45">
-        <v>173846.38</v>
+        <v>135</v>
       </c>
       <c r="Q45" t="s">
-        <v>167</v>
+        <v>169</v>
       </c>
       <c r="R45" t="s">
-        <v>170</v>
+        <v>172</v>
       </c>
       <c r="S45" t="s">
-        <v>172</v>
+        <v>174</v>
       </c>
       <c r="T45" t="s">
-        <v>178</v>
+        <v>180</v>
       </c>
       <c r="U45" t="s">
-        <v>181</v>
-      </c>
-      <c r="V45" s="2">
+        <v>183</v>
+      </c>
+      <c r="V45" s="1">
         <v>46229</v>
       </c>
     </row>
@@ -3365,39 +3219,36 @@
         <v>33</v>
       </c>
       <c r="G46" t="s">
-        <v>43</v>
-      </c>
-      <c r="H46" s="2">
+        <v>44</v>
+      </c>
+      <c r="H46" s="1">
         <v>46210</v>
       </c>
       <c r="I46" t="s">
-        <v>54</v>
+        <v>55</v>
       </c>
       <c r="N46" t="s">
-        <v>85</v>
+        <v>87</v>
       </c>
       <c r="O46" t="s">
-        <v>133</v>
-      </c>
-      <c r="P46">
-        <v>1530656.62</v>
+        <v>135</v>
       </c>
       <c r="Q46" t="s">
-        <v>167</v>
+        <v>169</v>
       </c>
       <c r="R46" t="s">
-        <v>170</v>
+        <v>172</v>
       </c>
       <c r="S46" t="s">
-        <v>172</v>
+        <v>174</v>
       </c>
       <c r="T46" t="s">
-        <v>178</v>
+        <v>180</v>
       </c>
       <c r="U46" t="s">
-        <v>181</v>
-      </c>
-      <c r="V46" s="2">
+        <v>183</v>
+      </c>
+      <c r="V46" s="1">
         <v>46229</v>
       </c>
     </row>
@@ -3421,30 +3272,27 @@
         <v>30</v>
       </c>
       <c r="N47" t="s">
-        <v>87</v>
+        <v>89</v>
       </c>
       <c r="O47" t="s">
-        <v>134</v>
-      </c>
-      <c r="P47">
-        <v>1000000</v>
+        <v>136</v>
       </c>
       <c r="Q47" t="s">
-        <v>167</v>
+        <v>169</v>
       </c>
       <c r="R47" t="s">
-        <v>169</v>
+        <v>171</v>
       </c>
       <c r="S47" t="s">
-        <v>172</v>
+        <v>174</v>
       </c>
       <c r="T47" t="s">
-        <v>177</v>
+        <v>179</v>
       </c>
       <c r="U47" t="s">
         <v>28</v>
       </c>
-      <c r="V47" s="2">
+      <c r="V47" s="1">
         <v>46321</v>
       </c>
     </row>
@@ -3468,36 +3316,33 @@
         <v>30</v>
       </c>
       <c r="J48" t="s">
-        <v>63</v>
+        <v>64</v>
       </c>
       <c r="K48" t="s">
-        <v>72</v>
+        <v>73</v>
       </c>
       <c r="N48" t="s">
-        <v>80</v>
+        <v>82</v>
       </c>
       <c r="O48" t="s">
-        <v>135</v>
-      </c>
-      <c r="P48">
-        <v>958040</v>
+        <v>137</v>
       </c>
       <c r="Q48" t="s">
-        <v>166</v>
+        <v>168</v>
       </c>
       <c r="R48" t="s">
-        <v>169</v>
+        <v>171</v>
       </c>
       <c r="S48" t="s">
-        <v>172</v>
+        <v>174</v>
       </c>
       <c r="T48" t="s">
-        <v>176</v>
+        <v>178</v>
       </c>
       <c r="U48" t="s">
-        <v>181</v>
-      </c>
-      <c r="V48" s="2">
+        <v>183</v>
+      </c>
+      <c r="V48" s="1">
         <v>46291</v>
       </c>
     </row>
@@ -3521,101 +3366,95 @@
         <v>30</v>
       </c>
       <c r="G49" t="s">
-        <v>43</v>
-      </c>
-      <c r="H49" s="2">
+        <v>44</v>
+      </c>
+      <c r="H49" s="1">
         <v>46176</v>
       </c>
       <c r="I49" t="s">
-        <v>61</v>
+        <v>62</v>
       </c>
       <c r="J49" t="s">
-        <v>69</v>
+        <v>70</v>
       </c>
       <c r="N49" t="s">
-        <v>80</v>
+        <v>82</v>
       </c>
       <c r="O49" t="s">
-        <v>135</v>
-      </c>
-      <c r="P49">
-        <v>41730.64</v>
+        <v>137</v>
       </c>
       <c r="Q49" t="s">
-        <v>166</v>
+        <v>168</v>
       </c>
       <c r="R49" t="s">
-        <v>171</v>
+        <v>173</v>
       </c>
       <c r="S49" t="s">
-        <v>172</v>
+        <v>174</v>
       </c>
       <c r="T49" t="s">
-        <v>176</v>
+        <v>178</v>
       </c>
       <c r="U49" t="s">
-        <v>181</v>
-      </c>
-      <c r="V49" s="2">
+        <v>183</v>
+      </c>
+      <c r="V49" s="1">
         <v>46199</v>
       </c>
     </row>
     <row r="50" spans="1:22">
       <c r="A50">
-        <v>17760</v>
+        <v>17765</v>
       </c>
       <c r="B50" t="s">
         <v>22</v>
       </c>
-      <c r="C50" t="s">
-        <v>22</v>
-      </c>
       <c r="D50" t="s">
-        <v>24</v>
+        <v>26</v>
       </c>
       <c r="E50" t="s">
         <v>28</v>
       </c>
       <c r="F50" t="s">
-        <v>30</v>
-      </c>
-      <c r="J50" t="s">
-        <v>68</v>
-      </c>
-      <c r="K50" t="s">
-        <v>74</v>
+        <v>38</v>
+      </c>
+      <c r="G50" t="s">
+        <v>44</v>
+      </c>
+      <c r="H50" s="1">
+        <v>46280</v>
+      </c>
+      <c r="I50" t="s">
+        <v>55</v>
       </c>
       <c r="N50" t="s">
-        <v>85</v>
+        <v>87</v>
       </c>
       <c r="O50" t="s">
-        <v>136</v>
-      </c>
-      <c r="P50">
-        <v>1468159.32</v>
+        <v>138</v>
       </c>
       <c r="Q50" t="s">
-        <v>167</v>
+        <v>169</v>
       </c>
       <c r="R50" t="s">
-        <v>170</v>
+        <v>172</v>
       </c>
       <c r="S50" t="s">
-        <v>172</v>
+        <v>174</v>
       </c>
       <c r="T50" t="s">
-        <v>178</v>
+        <v>180</v>
       </c>
       <c r="U50" t="s">
-        <v>181</v>
-      </c>
-      <c r="V50" s="2">
+        <v>183</v>
+      </c>
+      <c r="V50" s="1">
         <v>46260</v>
       </c>
     </row>
     <row r="51" spans="1:22">
       <c r="A51">
-        <v>17761</v>
+        <v>17760</v>
       </c>
       <c r="B51" t="s">
         <v>22</v>
@@ -3633,42 +3472,39 @@
         <v>30</v>
       </c>
       <c r="J51" t="s">
-        <v>68</v>
+        <v>69</v>
       </c>
       <c r="K51" t="s">
         <v>75</v>
       </c>
       <c r="N51" t="s">
-        <v>85</v>
+        <v>87</v>
       </c>
       <c r="O51" t="s">
-        <v>137</v>
-      </c>
-      <c r="P51">
-        <v>559040.0699999999</v>
+        <v>138</v>
       </c>
       <c r="Q51" t="s">
-        <v>167</v>
+        <v>169</v>
       </c>
       <c r="R51" t="s">
-        <v>170</v>
+        <v>172</v>
       </c>
       <c r="S51" t="s">
-        <v>172</v>
+        <v>174</v>
       </c>
       <c r="T51" t="s">
-        <v>178</v>
+        <v>180</v>
       </c>
       <c r="U51" t="s">
-        <v>181</v>
-      </c>
-      <c r="V51" s="2">
-        <v>46291</v>
+        <v>183</v>
+      </c>
+      <c r="V51" s="1">
+        <v>46260</v>
       </c>
     </row>
     <row r="52" spans="1:22">
       <c r="A52">
-        <v>17762</v>
+        <v>17761</v>
       </c>
       <c r="B52" t="s">
         <v>22</v>
@@ -3685,40 +3521,40 @@
       <c r="F52" t="s">
         <v>30</v>
       </c>
+      <c r="J52" t="s">
+        <v>69</v>
+      </c>
       <c r="K52" t="s">
-        <v>73</v>
+        <v>76</v>
       </c>
       <c r="N52" t="s">
-        <v>85</v>
+        <v>87</v>
       </c>
       <c r="O52" t="s">
-        <v>138</v>
-      </c>
-      <c r="P52">
-        <v>1704503</v>
+        <v>139</v>
       </c>
       <c r="Q52" t="s">
-        <v>167</v>
+        <v>169</v>
       </c>
       <c r="R52" t="s">
-        <v>170</v>
+        <v>172</v>
       </c>
       <c r="S52" t="s">
-        <v>172</v>
+        <v>174</v>
       </c>
       <c r="T52" t="s">
-        <v>178</v>
+        <v>180</v>
       </c>
       <c r="U52" t="s">
-        <v>181</v>
-      </c>
-      <c r="V52" s="2">
-        <v>46321</v>
+        <v>183</v>
+      </c>
+      <c r="V52" s="1">
+        <v>46291</v>
       </c>
     </row>
     <row r="53" spans="1:22">
       <c r="A53">
-        <v>17763</v>
+        <v>17762</v>
       </c>
       <c r="B53" t="s">
         <v>22</v>
@@ -3727,56 +3563,50 @@
         <v>22</v>
       </c>
       <c r="D53" t="s">
-        <v>26</v>
+        <v>24</v>
       </c>
       <c r="E53" t="s">
         <v>28</v>
       </c>
       <c r="F53" t="s">
-        <v>38</v>
-      </c>
-      <c r="G53" t="s">
-        <v>43</v>
-      </c>
-      <c r="H53" s="2">
-        <v>46227</v>
-      </c>
-      <c r="I53" t="s">
-        <v>62</v>
+        <v>30</v>
+      </c>
+      <c r="K53" t="s">
+        <v>74</v>
       </c>
       <c r="N53" t="s">
-        <v>85</v>
+        <v>87</v>
       </c>
       <c r="O53" t="s">
-        <v>136</v>
-      </c>
-      <c r="P53">
-        <v>236343.68</v>
+        <v>140</v>
       </c>
       <c r="Q53" t="s">
-        <v>167</v>
+        <v>169</v>
       </c>
       <c r="R53" t="s">
-        <v>170</v>
+        <v>172</v>
       </c>
       <c r="S53" t="s">
-        <v>172</v>
+        <v>174</v>
       </c>
       <c r="T53" t="s">
-        <v>178</v>
+        <v>180</v>
       </c>
       <c r="U53" t="s">
-        <v>181</v>
-      </c>
-      <c r="V53" s="2">
-        <v>46229</v>
+        <v>183</v>
+      </c>
+      <c r="V53" s="1">
+        <v>46321</v>
       </c>
     </row>
     <row r="54" spans="1:22">
       <c r="A54">
-        <v>17764</v>
+        <v>17763</v>
       </c>
       <c r="B54" t="s">
+        <v>22</v>
+      </c>
+      <c r="C54" t="s">
         <v>22</v>
       </c>
       <c r="D54" t="s">
@@ -3789,101 +3619,95 @@
         <v>39</v>
       </c>
       <c r="G54" t="s">
-        <v>43</v>
-      </c>
-      <c r="H54" s="2">
-        <v>46280</v>
+        <v>44</v>
+      </c>
+      <c r="H54" s="1">
+        <v>46227</v>
       </c>
       <c r="I54" t="s">
-        <v>54</v>
+        <v>63</v>
       </c>
       <c r="N54" t="s">
-        <v>85</v>
+        <v>87</v>
       </c>
       <c r="O54" t="s">
-        <v>137</v>
-      </c>
-      <c r="P54">
-        <v>1145462.93</v>
+        <v>138</v>
       </c>
       <c r="Q54" t="s">
-        <v>167</v>
+        <v>169</v>
       </c>
       <c r="R54" t="s">
-        <v>170</v>
+        <v>172</v>
       </c>
       <c r="S54" t="s">
-        <v>172</v>
+        <v>174</v>
       </c>
       <c r="T54" t="s">
-        <v>178</v>
+        <v>180</v>
       </c>
       <c r="U54" t="s">
-        <v>181</v>
-      </c>
-      <c r="V54" s="2">
-        <v>46291</v>
+        <v>183</v>
+      </c>
+      <c r="V54" s="1">
+        <v>46229</v>
       </c>
     </row>
     <row r="55" spans="1:22">
       <c r="A55">
-        <v>18140</v>
+        <v>17764</v>
       </c>
       <c r="B55" t="s">
         <v>22</v>
       </c>
-      <c r="C55" t="s">
-        <v>22</v>
-      </c>
       <c r="D55" t="s">
-        <v>24</v>
+        <v>26</v>
       </c>
       <c r="E55" t="s">
         <v>28</v>
       </c>
       <c r="F55" t="s">
-        <v>30</v>
-      </c>
-      <c r="J55" t="s">
-        <v>63</v>
-      </c>
-      <c r="K55" t="s">
-        <v>76</v>
+        <v>40</v>
+      </c>
+      <c r="G55" t="s">
+        <v>44</v>
+      </c>
+      <c r="H55" s="1">
+        <v>46280</v>
+      </c>
+      <c r="I55" t="s">
+        <v>55</v>
       </c>
       <c r="N55" t="s">
-        <v>85</v>
+        <v>87</v>
       </c>
       <c r="O55" t="s">
         <v>139</v>
       </c>
-      <c r="P55">
-        <v>1295422.28</v>
-      </c>
       <c r="Q55" t="s">
-        <v>167</v>
+        <v>169</v>
       </c>
       <c r="R55" t="s">
-        <v>170</v>
+        <v>172</v>
       </c>
       <c r="S55" t="s">
-        <v>172</v>
+        <v>174</v>
       </c>
       <c r="T55" t="s">
-        <v>178</v>
+        <v>180</v>
       </c>
       <c r="U55" t="s">
-        <v>181</v>
-      </c>
-      <c r="V55" s="2">
-        <v>46352</v>
+        <v>183</v>
+      </c>
+      <c r="V55" s="1">
+        <v>46291</v>
       </c>
     </row>
     <row r="56" spans="1:22">
       <c r="A56">
-        <v>19240</v>
+        <v>18140</v>
       </c>
       <c r="B56" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="C56" t="s">
         <v>22</v>
@@ -3895,45 +3719,42 @@
         <v>28</v>
       </c>
       <c r="F56" t="s">
-        <v>40</v>
+        <v>30</v>
       </c>
       <c r="J56" t="s">
-        <v>63</v>
+        <v>64</v>
       </c>
       <c r="K56" t="s">
-        <v>72</v>
+        <v>77</v>
       </c>
       <c r="N56" t="s">
-        <v>89</v>
+        <v>87</v>
       </c>
       <c r="O56" t="s">
-        <v>140</v>
-      </c>
-      <c r="P56">
-        <v>1962977.67</v>
+        <v>141</v>
       </c>
       <c r="Q56" t="s">
-        <v>167</v>
+        <v>169</v>
       </c>
       <c r="R56" t="s">
-        <v>170</v>
+        <v>172</v>
       </c>
       <c r="S56" t="s">
         <v>174</v>
       </c>
       <c r="T56" t="s">
-        <v>179</v>
+        <v>180</v>
       </c>
       <c r="U56" t="s">
-        <v>181</v>
-      </c>
-      <c r="V56" s="2">
-        <v>46321</v>
+        <v>183</v>
+      </c>
+      <c r="V56" s="1">
+        <v>46352</v>
       </c>
     </row>
     <row r="57" spans="1:22">
       <c r="A57">
-        <v>19241</v>
+        <v>19240</v>
       </c>
       <c r="B57" t="s">
         <v>23</v>
@@ -3942,45 +3763,48 @@
         <v>22</v>
       </c>
       <c r="D57" t="s">
-        <v>27</v>
+        <v>24</v>
       </c>
       <c r="E57" t="s">
-        <v>29</v>
-      </c>
-      <c r="G57" t="s">
-        <v>44</v>
+        <v>28</v>
+      </c>
+      <c r="F57" t="s">
+        <v>41</v>
+      </c>
+      <c r="J57" t="s">
+        <v>64</v>
+      </c>
+      <c r="K57" t="s">
+        <v>78</v>
       </c>
       <c r="N57" t="s">
-        <v>89</v>
+        <v>91</v>
       </c>
       <c r="O57" t="s">
-        <v>140</v>
-      </c>
-      <c r="P57">
-        <v>2497091</v>
+        <v>142</v>
       </c>
       <c r="Q57" t="s">
-        <v>167</v>
+        <v>169</v>
       </c>
       <c r="R57" t="s">
-        <v>170</v>
+        <v>172</v>
       </c>
       <c r="S57" t="s">
-        <v>174</v>
+        <v>176</v>
       </c>
       <c r="T57" t="s">
-        <v>179</v>
+        <v>181</v>
       </c>
       <c r="U57" t="s">
-        <v>181</v>
-      </c>
-      <c r="V57" s="2">
+        <v>183</v>
+      </c>
+      <c r="V57" s="1">
         <v>46321</v>
       </c>
     </row>
     <row r="58" spans="1:22">
       <c r="A58">
-        <v>19260</v>
+        <v>19241</v>
       </c>
       <c r="B58" t="s">
         <v>23</v>
@@ -3995,36 +3819,36 @@
         <v>29</v>
       </c>
       <c r="G58" t="s">
-        <v>42</v>
+        <v>45</v>
       </c>
       <c r="N58" t="s">
-        <v>89</v>
+        <v>91</v>
       </c>
       <c r="O58" t="s">
-        <v>141</v>
+        <v>142</v>
       </c>
       <c r="Q58" t="s">
-        <v>167</v>
+        <v>169</v>
       </c>
       <c r="R58" t="s">
-        <v>170</v>
+        <v>172</v>
       </c>
       <c r="S58" t="s">
-        <v>174</v>
+        <v>176</v>
       </c>
       <c r="T58" t="s">
-        <v>179</v>
+        <v>181</v>
       </c>
       <c r="U58" t="s">
-        <v>181</v>
-      </c>
-      <c r="V58" s="2">
-        <v>46049</v>
+        <v>183</v>
+      </c>
+      <c r="V58" s="1">
+        <v>46321</v>
       </c>
     </row>
     <row r="59" spans="1:22">
       <c r="A59">
-        <v>19600</v>
+        <v>19260</v>
       </c>
       <c r="B59" t="s">
         <v>23</v>
@@ -4039,33 +3863,36 @@
         <v>29</v>
       </c>
       <c r="G59" t="s">
-        <v>42</v>
+        <v>43</v>
       </c>
       <c r="N59" t="s">
-        <v>89</v>
+        <v>91</v>
       </c>
       <c r="O59" t="s">
-        <v>142</v>
+        <v>143</v>
       </c>
       <c r="Q59" t="s">
-        <v>167</v>
+        <v>169</v>
       </c>
       <c r="R59" t="s">
-        <v>170</v>
+        <v>172</v>
       </c>
       <c r="S59" t="s">
-        <v>174</v>
+        <v>176</v>
       </c>
       <c r="T59" t="s">
-        <v>179</v>
+        <v>181</v>
       </c>
       <c r="U59" t="s">
-        <v>181</v>
+        <v>183</v>
+      </c>
+      <c r="V59" s="1">
+        <v>46049</v>
       </c>
     </row>
     <row r="60" spans="1:22">
       <c r="A60">
-        <v>19620</v>
+        <v>19600</v>
       </c>
       <c r="B60" t="s">
         <v>23</v>
@@ -4080,36 +3907,36 @@
         <v>29</v>
       </c>
       <c r="G60" t="s">
-        <v>42</v>
+        <v>43</v>
       </c>
       <c r="N60" t="s">
-        <v>89</v>
+        <v>91</v>
       </c>
       <c r="O60" t="s">
-        <v>143</v>
+        <v>144</v>
       </c>
       <c r="Q60" t="s">
-        <v>167</v>
+        <v>169</v>
       </c>
       <c r="R60" t="s">
-        <v>170</v>
+        <v>172</v>
       </c>
       <c r="S60" t="s">
-        <v>174</v>
+        <v>176</v>
       </c>
       <c r="T60" t="s">
-        <v>179</v>
+        <v>181</v>
       </c>
       <c r="U60" t="s">
-        <v>181</v>
+        <v>183</v>
       </c>
     </row>
     <row r="61" spans="1:22">
       <c r="A61">
-        <v>23120</v>
+        <v>19620</v>
       </c>
       <c r="B61" t="s">
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="C61" t="s">
         <v>22</v>
@@ -4120,37 +3947,34 @@
       <c r="E61" t="s">
         <v>29</v>
       </c>
+      <c r="G61" t="s">
+        <v>43</v>
+      </c>
       <c r="N61" t="s">
-        <v>90</v>
+        <v>91</v>
       </c>
       <c r="O61" t="s">
-        <v>144</v>
-      </c>
-      <c r="P61">
-        <v>9389.959999999999</v>
+        <v>145</v>
       </c>
       <c r="Q61" t="s">
-        <v>166</v>
+        <v>169</v>
       </c>
       <c r="R61" t="s">
-        <v>171</v>
+        <v>172</v>
       </c>
       <c r="S61" t="s">
-        <v>173</v>
+        <v>176</v>
       </c>
       <c r="T61" t="s">
-        <v>176</v>
+        <v>181</v>
       </c>
       <c r="U61" t="s">
-        <v>181</v>
-      </c>
-      <c r="V61" s="2">
-        <v>46107</v>
+        <v>183</v>
       </c>
     </row>
     <row r="62" spans="1:22">
       <c r="A62">
-        <v>23160</v>
+        <v>23120</v>
       </c>
       <c r="B62" t="s">
         <v>22</v>
@@ -4165,36 +3989,33 @@
         <v>29</v>
       </c>
       <c r="N62" t="s">
-        <v>91</v>
+        <v>92</v>
       </c>
       <c r="O62" t="s">
-        <v>145</v>
-      </c>
-      <c r="P62">
-        <v>7204.82</v>
+        <v>146</v>
       </c>
       <c r="Q62" t="s">
-        <v>166</v>
+        <v>168</v>
       </c>
       <c r="R62" t="s">
-        <v>171</v>
+        <v>173</v>
       </c>
       <c r="S62" t="s">
-        <v>173</v>
+        <v>175</v>
       </c>
       <c r="T62" t="s">
-        <v>176</v>
+        <v>178</v>
       </c>
       <c r="U62" t="s">
-        <v>181</v>
-      </c>
-      <c r="V62" s="2">
+        <v>183</v>
+      </c>
+      <c r="V62" s="1">
         <v>46107</v>
       </c>
     </row>
     <row r="63" spans="1:22">
       <c r="A63">
-        <v>23100</v>
+        <v>23160</v>
       </c>
       <c r="B63" t="s">
         <v>22</v>
@@ -4209,36 +4030,33 @@
         <v>29</v>
       </c>
       <c r="N63" t="s">
-        <v>92</v>
+        <v>93</v>
       </c>
       <c r="O63" t="s">
-        <v>146</v>
-      </c>
-      <c r="P63">
-        <v>4227.84</v>
+        <v>147</v>
       </c>
       <c r="Q63" t="s">
-        <v>166</v>
+        <v>168</v>
       </c>
       <c r="R63" t="s">
-        <v>171</v>
+        <v>173</v>
       </c>
       <c r="S63" t="s">
-        <v>173</v>
+        <v>175</v>
       </c>
       <c r="T63" t="s">
-        <v>176</v>
+        <v>178</v>
       </c>
       <c r="U63" t="s">
-        <v>181</v>
-      </c>
-      <c r="V63" s="2">
+        <v>183</v>
+      </c>
+      <c r="V63" s="1">
         <v>46107</v>
       </c>
     </row>
     <row r="64" spans="1:22">
       <c r="A64">
-        <v>23080</v>
+        <v>23100</v>
       </c>
       <c r="B64" t="s">
         <v>22</v>
@@ -4253,36 +4071,33 @@
         <v>29</v>
       </c>
       <c r="N64" t="s">
-        <v>93</v>
+        <v>94</v>
       </c>
       <c r="O64" t="s">
-        <v>147</v>
-      </c>
-      <c r="P64">
-        <v>4064.54</v>
+        <v>148</v>
       </c>
       <c r="Q64" t="s">
-        <v>167</v>
+        <v>168</v>
       </c>
       <c r="R64" t="s">
-        <v>171</v>
+        <v>173</v>
       </c>
       <c r="S64" t="s">
-        <v>173</v>
+        <v>175</v>
       </c>
       <c r="T64" t="s">
-        <v>176</v>
+        <v>178</v>
       </c>
       <c r="U64" t="s">
-        <v>181</v>
-      </c>
-      <c r="V64" s="2">
+        <v>183</v>
+      </c>
+      <c r="V64" s="1">
         <v>46107</v>
       </c>
     </row>
     <row r="65" spans="1:22">
       <c r="A65">
-        <v>23180</v>
+        <v>23080</v>
       </c>
       <c r="B65" t="s">
         <v>22</v>
@@ -4297,36 +4112,33 @@
         <v>29</v>
       </c>
       <c r="N65" t="s">
-        <v>94</v>
+        <v>95</v>
       </c>
       <c r="O65" t="s">
-        <v>146</v>
-      </c>
-      <c r="P65">
-        <v>3662.66</v>
+        <v>149</v>
       </c>
       <c r="Q65" t="s">
-        <v>166</v>
+        <v>169</v>
       </c>
       <c r="R65" t="s">
-        <v>171</v>
+        <v>173</v>
       </c>
       <c r="S65" t="s">
-        <v>173</v>
+        <v>175</v>
       </c>
       <c r="T65" t="s">
-        <v>176</v>
+        <v>178</v>
       </c>
       <c r="U65" t="s">
-        <v>181</v>
-      </c>
-      <c r="V65" s="2">
+        <v>183</v>
+      </c>
+      <c r="V65" s="1">
         <v>46107</v>
       </c>
     </row>
     <row r="66" spans="1:22">
       <c r="A66">
-        <v>23140</v>
+        <v>23180</v>
       </c>
       <c r="B66" t="s">
         <v>22</v>
@@ -4341,36 +4153,33 @@
         <v>29</v>
       </c>
       <c r="N66" t="s">
-        <v>95</v>
+        <v>96</v>
       </c>
       <c r="O66" t="s">
         <v>148</v>
       </c>
-      <c r="P66">
-        <v>1163.64</v>
-      </c>
       <c r="Q66" t="s">
         <v>168</v>
       </c>
       <c r="R66" t="s">
-        <v>171</v>
+        <v>173</v>
       </c>
       <c r="S66" t="s">
-        <v>173</v>
+        <v>175</v>
       </c>
       <c r="T66" t="s">
-        <v>176</v>
+        <v>178</v>
       </c>
       <c r="U66" t="s">
-        <v>181</v>
-      </c>
-      <c r="V66" s="2">
+        <v>183</v>
+      </c>
+      <c r="V66" s="1">
         <v>46107</v>
       </c>
     </row>
     <row r="67" spans="1:22">
       <c r="A67">
-        <v>23640</v>
+        <v>23140</v>
       </c>
       <c r="B67" t="s">
         <v>22</v>
@@ -4385,36 +4194,33 @@
         <v>29</v>
       </c>
       <c r="N67" t="s">
-        <v>81</v>
+        <v>97</v>
       </c>
       <c r="O67" t="s">
-        <v>149</v>
-      </c>
-      <c r="P67">
-        <v>120000</v>
+        <v>150</v>
       </c>
       <c r="Q67" t="s">
-        <v>166</v>
+        <v>170</v>
       </c>
       <c r="R67" t="s">
-        <v>170</v>
+        <v>173</v>
       </c>
       <c r="S67" t="s">
-        <v>173</v>
+        <v>175</v>
       </c>
       <c r="T67" t="s">
-        <v>176</v>
+        <v>178</v>
       </c>
       <c r="U67" t="s">
-        <v>28</v>
-      </c>
-      <c r="V67" s="2">
-        <v>46168</v>
+        <v>183</v>
+      </c>
+      <c r="V67" s="1">
+        <v>46107</v>
       </c>
     </row>
     <row r="68" spans="1:22">
       <c r="A68">
-        <v>23740</v>
+        <v>23640</v>
       </c>
       <c r="B68" t="s">
         <v>22</v>
@@ -4423,45 +4229,39 @@
         <v>22</v>
       </c>
       <c r="D68" t="s">
-        <v>24</v>
+        <v>27</v>
       </c>
       <c r="E68" t="s">
-        <v>28</v>
-      </c>
-      <c r="F68" t="s">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="N68" t="s">
-        <v>80</v>
+        <v>83</v>
       </c>
       <c r="O68" t="s">
-        <v>150</v>
-      </c>
-      <c r="P68">
-        <v>400000</v>
+        <v>151</v>
       </c>
       <c r="Q68" t="s">
-        <v>166</v>
+        <v>168</v>
       </c>
       <c r="R68" t="s">
-        <v>169</v>
+        <v>172</v>
       </c>
       <c r="S68" t="s">
-        <v>172</v>
+        <v>175</v>
       </c>
       <c r="T68" t="s">
-        <v>176</v>
+        <v>178</v>
       </c>
       <c r="U68" t="s">
         <v>28</v>
       </c>
-      <c r="V68" s="2">
-        <v>46291</v>
+      <c r="V68" s="1">
+        <v>46168</v>
       </c>
     </row>
     <row r="69" spans="1:22">
       <c r="A69">
-        <v>24180</v>
+        <v>23740</v>
       </c>
       <c r="B69" t="s">
         <v>22</v>
@@ -4478,43 +4278,34 @@
       <c r="F69" t="s">
         <v>30</v>
       </c>
-      <c r="J69" t="s">
-        <v>63</v>
-      </c>
-      <c r="K69" t="s">
-        <v>72</v>
-      </c>
       <c r="N69" t="s">
-        <v>84</v>
+        <v>82</v>
       </c>
       <c r="O69" t="s">
-        <v>151</v>
-      </c>
-      <c r="P69">
-        <v>100000</v>
+        <v>152</v>
       </c>
       <c r="Q69" t="s">
         <v>168</v>
       </c>
       <c r="R69" t="s">
-        <v>169</v>
+        <v>171</v>
       </c>
       <c r="S69" t="s">
-        <v>172</v>
+        <v>174</v>
       </c>
       <c r="T69" t="s">
-        <v>176</v>
+        <v>178</v>
       </c>
       <c r="U69" t="s">
-        <v>181</v>
-      </c>
-      <c r="V69" s="2">
-        <v>46229</v>
+        <v>28</v>
+      </c>
+      <c r="V69" s="1">
+        <v>46291</v>
       </c>
     </row>
     <row r="70" spans="1:22">
       <c r="A70">
-        <v>24380</v>
+        <v>24180</v>
       </c>
       <c r="B70" t="s">
         <v>22</v>
@@ -4523,42 +4314,48 @@
         <v>22</v>
       </c>
       <c r="D70" t="s">
-        <v>27</v>
+        <v>24</v>
       </c>
       <c r="E70" t="s">
-        <v>29</v>
+        <v>28</v>
+      </c>
+      <c r="F70" t="s">
+        <v>30</v>
+      </c>
+      <c r="J70" t="s">
+        <v>64</v>
+      </c>
+      <c r="K70" t="s">
+        <v>73</v>
       </c>
       <c r="N70" t="s">
-        <v>81</v>
+        <v>86</v>
       </c>
       <c r="O70" t="s">
-        <v>152</v>
-      </c>
-      <c r="P70">
-        <v>80000</v>
+        <v>153</v>
       </c>
       <c r="Q70" t="s">
-        <v>166</v>
+        <v>170</v>
       </c>
       <c r="R70" t="s">
-        <v>170</v>
+        <v>171</v>
       </c>
       <c r="S70" t="s">
-        <v>173</v>
+        <v>174</v>
       </c>
       <c r="T70" t="s">
-        <v>176</v>
+        <v>178</v>
       </c>
       <c r="U70" t="s">
-        <v>28</v>
-      </c>
-      <c r="V70" s="2">
-        <v>46260</v>
+        <v>183</v>
+      </c>
+      <c r="V70" s="1">
+        <v>46229</v>
       </c>
     </row>
     <row r="71" spans="1:22">
       <c r="A71">
-        <v>24660</v>
+        <v>24380</v>
       </c>
       <c r="B71" t="s">
         <v>22</v>
@@ -4573,36 +4370,33 @@
         <v>29</v>
       </c>
       <c r="N71" t="s">
-        <v>80</v>
+        <v>83</v>
       </c>
       <c r="O71" t="s">
-        <v>153</v>
-      </c>
-      <c r="P71">
-        <v>835000</v>
+        <v>154</v>
       </c>
       <c r="Q71" t="s">
-        <v>166</v>
+        <v>168</v>
       </c>
       <c r="R71" t="s">
-        <v>169</v>
+        <v>172</v>
       </c>
       <c r="S71" t="s">
-        <v>173</v>
+        <v>175</v>
       </c>
       <c r="T71" t="s">
-        <v>176</v>
+        <v>178</v>
       </c>
       <c r="U71" t="s">
-        <v>181</v>
-      </c>
-      <c r="V71" s="2">
-        <v>46291</v>
+        <v>28</v>
+      </c>
+      <c r="V71" s="1">
+        <v>46260</v>
       </c>
     </row>
     <row r="72" spans="1:22">
       <c r="A72">
-        <v>24661</v>
+        <v>24660</v>
       </c>
       <c r="B72" t="s">
         <v>22</v>
@@ -4617,36 +4411,33 @@
         <v>29</v>
       </c>
       <c r="N72" t="s">
-        <v>80</v>
+        <v>82</v>
       </c>
       <c r="O72" t="s">
-        <v>153</v>
-      </c>
-      <c r="P72">
-        <v>165000</v>
+        <v>155</v>
       </c>
       <c r="Q72" t="s">
-        <v>166</v>
+        <v>168</v>
       </c>
       <c r="R72" t="s">
-        <v>169</v>
+        <v>171</v>
       </c>
       <c r="S72" t="s">
-        <v>173</v>
+        <v>175</v>
       </c>
       <c r="T72" t="s">
-        <v>176</v>
+        <v>178</v>
       </c>
       <c r="U72" t="s">
-        <v>181</v>
-      </c>
-      <c r="V72" s="2">
-        <v>46168</v>
+        <v>183</v>
+      </c>
+      <c r="V72" s="1">
+        <v>46291</v>
       </c>
     </row>
     <row r="73" spans="1:22">
       <c r="A73">
-        <v>24680</v>
+        <v>24661</v>
       </c>
       <c r="B73" t="s">
         <v>22</v>
@@ -4661,36 +4452,33 @@
         <v>29</v>
       </c>
       <c r="N73" t="s">
-        <v>80</v>
+        <v>82</v>
       </c>
       <c r="O73" t="s">
-        <v>154</v>
-      </c>
-      <c r="P73">
-        <v>1000000</v>
+        <v>155</v>
       </c>
       <c r="Q73" t="s">
-        <v>166</v>
+        <v>168</v>
       </c>
       <c r="R73" t="s">
-        <v>169</v>
+        <v>171</v>
       </c>
       <c r="S73" t="s">
-        <v>173</v>
+        <v>175</v>
       </c>
       <c r="T73" t="s">
-        <v>176</v>
+        <v>178</v>
       </c>
       <c r="U73" t="s">
-        <v>181</v>
-      </c>
-      <c r="V73" s="2">
-        <v>46291</v>
+        <v>183</v>
+      </c>
+      <c r="V73" s="1">
+        <v>46168</v>
       </c>
     </row>
     <row r="74" spans="1:22">
       <c r="A74">
-        <v>24700</v>
+        <v>24680</v>
       </c>
       <c r="B74" t="s">
         <v>22</v>
@@ -4705,36 +4493,33 @@
         <v>29</v>
       </c>
       <c r="N74" t="s">
-        <v>80</v>
+        <v>82</v>
       </c>
       <c r="O74" t="s">
-        <v>155</v>
-      </c>
-      <c r="P74">
-        <v>1000000</v>
+        <v>156</v>
       </c>
       <c r="Q74" t="s">
-        <v>166</v>
+        <v>168</v>
       </c>
       <c r="R74" t="s">
-        <v>169</v>
+        <v>171</v>
       </c>
       <c r="S74" t="s">
-        <v>173</v>
+        <v>175</v>
       </c>
       <c r="T74" t="s">
-        <v>176</v>
+        <v>178</v>
       </c>
       <c r="U74" t="s">
-        <v>181</v>
-      </c>
-      <c r="V74" s="2">
+        <v>183</v>
+      </c>
+      <c r="V74" s="1">
         <v>46291</v>
       </c>
     </row>
     <row r="75" spans="1:22">
       <c r="A75">
-        <v>24720</v>
+        <v>24700</v>
       </c>
       <c r="B75" t="s">
         <v>22</v>
@@ -4749,36 +4534,33 @@
         <v>29</v>
       </c>
       <c r="N75" t="s">
-        <v>84</v>
+        <v>82</v>
       </c>
       <c r="O75" t="s">
-        <v>156</v>
-      </c>
-      <c r="P75">
-        <v>100000</v>
+        <v>157</v>
       </c>
       <c r="Q75" t="s">
         <v>168</v>
       </c>
       <c r="R75" t="s">
-        <v>169</v>
+        <v>171</v>
       </c>
       <c r="S75" t="s">
-        <v>173</v>
+        <v>175</v>
       </c>
       <c r="T75" t="s">
-        <v>176</v>
+        <v>178</v>
       </c>
       <c r="U75" t="s">
-        <v>181</v>
-      </c>
-      <c r="V75" s="2">
+        <v>183</v>
+      </c>
+      <c r="V75" s="1">
         <v>46291</v>
       </c>
     </row>
     <row r="76" spans="1:22">
       <c r="A76">
-        <v>25180</v>
+        <v>24720</v>
       </c>
       <c r="B76" t="s">
         <v>22</v>
@@ -4787,45 +4569,39 @@
         <v>22</v>
       </c>
       <c r="D76" t="s">
-        <v>24</v>
+        <v>27</v>
       </c>
       <c r="E76" t="s">
-        <v>28</v>
-      </c>
-      <c r="F76" t="s">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="N76" t="s">
-        <v>87</v>
+        <v>86</v>
       </c>
       <c r="O76" t="s">
-        <v>157</v>
-      </c>
-      <c r="P76">
-        <v>1000000</v>
+        <v>158</v>
       </c>
       <c r="Q76" t="s">
-        <v>167</v>
+        <v>170</v>
       </c>
       <c r="R76" t="s">
-        <v>169</v>
+        <v>171</v>
       </c>
       <c r="S76" t="s">
-        <v>172</v>
+        <v>175</v>
       </c>
       <c r="T76" t="s">
-        <v>177</v>
+        <v>178</v>
       </c>
       <c r="U76" t="s">
-        <v>28</v>
-      </c>
-      <c r="V76" s="2">
-        <v>46321</v>
+        <v>183</v>
+      </c>
+      <c r="V76" s="1">
+        <v>46291</v>
       </c>
     </row>
     <row r="77" spans="1:22">
       <c r="A77">
-        <v>25900</v>
+        <v>25180</v>
       </c>
       <c r="B77" t="s">
         <v>22</v>
@@ -4834,48 +4610,42 @@
         <v>22</v>
       </c>
       <c r="D77" t="s">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="E77" t="s">
         <v>28</v>
       </c>
       <c r="F77" t="s">
-        <v>41</v>
-      </c>
-      <c r="G77" t="s">
-        <v>45</v>
+        <v>30</v>
       </c>
       <c r="N77" t="s">
-        <v>85</v>
+        <v>89</v>
       </c>
       <c r="O77" t="s">
-        <v>158</v>
-      </c>
-      <c r="P77">
-        <v>1704503</v>
+        <v>159</v>
       </c>
       <c r="Q77" t="s">
-        <v>167</v>
+        <v>169</v>
       </c>
       <c r="R77" t="s">
-        <v>170</v>
+        <v>171</v>
       </c>
       <c r="S77" t="s">
-        <v>41</v>
+        <v>174</v>
       </c>
       <c r="T77" t="s">
-        <v>178</v>
+        <v>179</v>
       </c>
       <c r="U77" t="s">
-        <v>181</v>
-      </c>
-      <c r="V77" s="2">
-        <v>46381</v>
+        <v>28</v>
+      </c>
+      <c r="V77" s="1">
+        <v>46321</v>
       </c>
     </row>
     <row r="78" spans="1:22">
       <c r="A78">
-        <v>25920</v>
+        <v>25900</v>
       </c>
       <c r="B78" t="s">
         <v>22</v>
@@ -4890,42 +4660,39 @@
         <v>28</v>
       </c>
       <c r="F78" t="s">
-        <v>41</v>
+        <v>42</v>
       </c>
       <c r="G78" t="s">
-        <v>45</v>
+        <v>46</v>
       </c>
       <c r="N78" t="s">
-        <v>85</v>
+        <v>87</v>
       </c>
       <c r="O78" t="s">
-        <v>159</v>
-      </c>
-      <c r="P78">
-        <v>1638125.5</v>
+        <v>160</v>
       </c>
       <c r="Q78" t="s">
-        <v>167</v>
+        <v>169</v>
       </c>
       <c r="R78" t="s">
-        <v>170</v>
+        <v>172</v>
       </c>
       <c r="S78" t="s">
-        <v>41</v>
+        <v>42</v>
       </c>
       <c r="T78" t="s">
-        <v>178</v>
+        <v>180</v>
       </c>
       <c r="U78" t="s">
-        <v>181</v>
-      </c>
-      <c r="V78" s="2">
+        <v>183</v>
+      </c>
+      <c r="V78" s="1">
         <v>46381</v>
       </c>
     </row>
     <row r="79" spans="1:22">
       <c r="A79">
-        <v>25940</v>
+        <v>25920</v>
       </c>
       <c r="B79" t="s">
         <v>22</v>
@@ -4940,42 +4707,39 @@
         <v>28</v>
       </c>
       <c r="F79" t="s">
-        <v>41</v>
+        <v>42</v>
       </c>
       <c r="G79" t="s">
-        <v>45</v>
+        <v>46</v>
       </c>
       <c r="N79" t="s">
-        <v>83</v>
+        <v>87</v>
       </c>
       <c r="O79" t="s">
-        <v>160</v>
-      </c>
-      <c r="P79">
-        <v>3800000</v>
+        <v>161</v>
       </c>
       <c r="Q79" t="s">
-        <v>167</v>
+        <v>169</v>
       </c>
       <c r="R79" t="s">
-        <v>170</v>
+        <v>172</v>
       </c>
       <c r="S79" t="s">
-        <v>41</v>
+        <v>42</v>
       </c>
       <c r="T79" t="s">
-        <v>177</v>
+        <v>180</v>
       </c>
       <c r="U79" t="s">
-        <v>28</v>
-      </c>
-      <c r="V79" s="2">
+        <v>183</v>
+      </c>
+      <c r="V79" s="1">
         <v>46381</v>
       </c>
     </row>
     <row r="80" spans="1:22">
       <c r="A80">
-        <v>25960</v>
+        <v>25940</v>
       </c>
       <c r="B80" t="s">
         <v>22</v>
@@ -4990,42 +4754,39 @@
         <v>28</v>
       </c>
       <c r="F80" t="s">
-        <v>41</v>
+        <v>42</v>
       </c>
       <c r="G80" t="s">
-        <v>45</v>
+        <v>46</v>
       </c>
       <c r="N80" t="s">
-        <v>83</v>
+        <v>85</v>
       </c>
       <c r="O80" t="s">
-        <v>161</v>
-      </c>
-      <c r="P80">
-        <v>3800000</v>
+        <v>162</v>
       </c>
       <c r="Q80" t="s">
-        <v>167</v>
+        <v>169</v>
       </c>
       <c r="R80" t="s">
-        <v>170</v>
+        <v>172</v>
       </c>
       <c r="S80" t="s">
-        <v>41</v>
+        <v>42</v>
       </c>
       <c r="T80" t="s">
-        <v>177</v>
+        <v>179</v>
       </c>
       <c r="U80" t="s">
         <v>28</v>
       </c>
-      <c r="V80" s="2">
+      <c r="V80" s="1">
         <v>46381</v>
       </c>
     </row>
     <row r="81" spans="1:22">
       <c r="A81">
-        <v>63120</v>
+        <v>25960</v>
       </c>
       <c r="B81" t="s">
         <v>22</v>
@@ -5034,48 +4795,45 @@
         <v>22</v>
       </c>
       <c r="D81" t="s">
-        <v>27</v>
+        <v>25</v>
       </c>
       <c r="E81" t="s">
-        <v>29</v>
-      </c>
-      <c r="J81" t="s">
-        <v>70</v>
-      </c>
-      <c r="K81" t="s">
-        <v>77</v>
+        <v>28</v>
+      </c>
+      <c r="F81" t="s">
+        <v>42</v>
+      </c>
+      <c r="G81" t="s">
+        <v>46</v>
       </c>
       <c r="N81" t="s">
-        <v>88</v>
+        <v>85</v>
       </c>
       <c r="O81" t="s">
-        <v>162</v>
-      </c>
-      <c r="P81">
-        <v>3800000</v>
+        <v>163</v>
       </c>
       <c r="Q81" t="s">
-        <v>167</v>
+        <v>169</v>
       </c>
       <c r="R81" t="s">
-        <v>170</v>
+        <v>172</v>
       </c>
       <c r="S81" t="s">
-        <v>173</v>
+        <v>42</v>
       </c>
       <c r="T81" t="s">
-        <v>177</v>
+        <v>179</v>
       </c>
       <c r="U81" t="s">
         <v>28</v>
       </c>
-      <c r="V81" s="2">
-        <v>46382</v>
+      <c r="V81" s="1">
+        <v>46381</v>
       </c>
     </row>
     <row r="82" spans="1:22">
       <c r="A82">
-        <v>63140</v>
+        <v>63120</v>
       </c>
       <c r="B82" t="s">
         <v>22</v>
@@ -5084,42 +4842,45 @@
         <v>22</v>
       </c>
       <c r="D82" t="s">
-        <v>24</v>
+        <v>27</v>
       </c>
       <c r="E82" t="s">
-        <v>28</v>
+        <v>29</v>
+      </c>
+      <c r="J82" t="s">
+        <v>71</v>
+      </c>
+      <c r="K82" t="s">
+        <v>79</v>
       </c>
       <c r="N82" t="s">
-        <v>96</v>
+        <v>90</v>
       </c>
       <c r="O82" t="s">
-        <v>97</v>
-      </c>
-      <c r="P82">
-        <v>4394700</v>
+        <v>164</v>
       </c>
       <c r="Q82" t="s">
-        <v>166</v>
+        <v>169</v>
       </c>
       <c r="R82" t="s">
-        <v>169</v>
+        <v>172</v>
       </c>
       <c r="S82" t="s">
-        <v>173</v>
+        <v>175</v>
       </c>
       <c r="T82" t="s">
-        <v>177</v>
+        <v>179</v>
       </c>
       <c r="U82" t="s">
         <v>28</v>
       </c>
-      <c r="V82" s="2">
+      <c r="V82" s="1">
         <v>46382</v>
       </c>
     </row>
     <row r="83" spans="1:22">
       <c r="A83">
-        <v>63940</v>
+        <v>63140</v>
       </c>
       <c r="B83" t="s">
         <v>22</v>
@@ -5133,46 +4894,34 @@
       <c r="E83" t="s">
         <v>28</v>
       </c>
-      <c r="F83" t="s">
-        <v>30</v>
-      </c>
-      <c r="J83" t="s">
-        <v>63</v>
-      </c>
-      <c r="K83" t="s">
-        <v>78</v>
-      </c>
       <c r="N83" t="s">
-        <v>85</v>
+        <v>98</v>
       </c>
       <c r="O83" t="s">
-        <v>163</v>
-      </c>
-      <c r="P83">
-        <v>528395.9300000001</v>
+        <v>99</v>
       </c>
       <c r="Q83" t="s">
-        <v>167</v>
+        <v>168</v>
       </c>
       <c r="R83" t="s">
-        <v>170</v>
+        <v>171</v>
       </c>
       <c r="S83" t="s">
-        <v>172</v>
+        <v>175</v>
       </c>
       <c r="T83" t="s">
-        <v>178</v>
+        <v>179</v>
       </c>
       <c r="U83" t="s">
-        <v>181</v>
-      </c>
-      <c r="V83" s="2">
+        <v>28</v>
+      </c>
+      <c r="V83" s="1">
         <v>46382</v>
       </c>
     </row>
     <row r="84" spans="1:22">
       <c r="A84">
-        <v>63960</v>
+        <v>63940</v>
       </c>
       <c r="B84" t="s">
         <v>22</v>
@@ -5181,42 +4930,48 @@
         <v>22</v>
       </c>
       <c r="D84" t="s">
-        <v>27</v>
+        <v>24</v>
       </c>
       <c r="E84" t="s">
-        <v>29</v>
+        <v>28</v>
+      </c>
+      <c r="F84" t="s">
+        <v>30</v>
+      </c>
+      <c r="J84" t="s">
+        <v>64</v>
+      </c>
+      <c r="K84" t="s">
+        <v>80</v>
       </c>
       <c r="N84" t="s">
         <v>87</v>
       </c>
       <c r="O84" t="s">
-        <v>164</v>
-      </c>
-      <c r="P84">
-        <v>1000000</v>
+        <v>165</v>
       </c>
       <c r="Q84" t="s">
-        <v>167</v>
+        <v>169</v>
       </c>
       <c r="R84" t="s">
-        <v>169</v>
+        <v>172</v>
       </c>
       <c r="S84" t="s">
-        <v>175</v>
+        <v>174</v>
       </c>
       <c r="T84" t="s">
-        <v>177</v>
+        <v>180</v>
       </c>
       <c r="U84" t="s">
-        <v>28</v>
-      </c>
-      <c r="V84" s="2">
-        <v>46321</v>
+        <v>183</v>
+      </c>
+      <c r="V84" s="1">
+        <v>46382</v>
       </c>
     </row>
     <row r="85" spans="1:22">
       <c r="A85">
-        <v>64340</v>
+        <v>63960</v>
       </c>
       <c r="B85" t="s">
         <v>22</v>
@@ -5225,42 +4980,39 @@
         <v>22</v>
       </c>
       <c r="D85" t="s">
-        <v>24</v>
+        <v>27</v>
       </c>
       <c r="E85" t="s">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="N85" t="s">
-        <v>96</v>
+        <v>89</v>
       </c>
       <c r="O85" t="s">
-        <v>97</v>
-      </c>
-      <c r="P85">
-        <v>4394700</v>
+        <v>166</v>
       </c>
       <c r="Q85" t="s">
-        <v>166</v>
+        <v>169</v>
       </c>
       <c r="R85" t="s">
-        <v>169</v>
+        <v>171</v>
       </c>
       <c r="S85" t="s">
-        <v>173</v>
+        <v>177</v>
       </c>
       <c r="T85" t="s">
-        <v>177</v>
+        <v>179</v>
       </c>
       <c r="U85" t="s">
         <v>28</v>
       </c>
-      <c r="V85" s="2">
-        <v>46382</v>
+      <c r="V85" s="1">
+        <v>46321</v>
       </c>
     </row>
     <row r="86" spans="1:22">
       <c r="A86">
-        <v>64760</v>
+        <v>64340</v>
       </c>
       <c r="B86" t="s">
         <v>22</v>
@@ -5269,45 +5021,39 @@
         <v>22</v>
       </c>
       <c r="D86" t="s">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="E86" t="s">
         <v>28</v>
       </c>
-      <c r="F86" t="s">
-        <v>41</v>
-      </c>
-      <c r="G86" t="s">
-        <v>45</v>
-      </c>
       <c r="N86" t="s">
-        <v>97</v>
+        <v>98</v>
       </c>
       <c r="O86" t="s">
-        <v>97</v>
-      </c>
-      <c r="P86">
-        <v>3306000</v>
+        <v>99</v>
       </c>
       <c r="Q86" t="s">
-        <v>166</v>
+        <v>168</v>
       </c>
       <c r="R86" t="s">
-        <v>169</v>
+        <v>171</v>
       </c>
       <c r="S86" t="s">
-        <v>41</v>
+        <v>175</v>
       </c>
       <c r="T86" t="s">
-        <v>177</v>
+        <v>179</v>
       </c>
       <c r="U86" t="s">
         <v>28</v>
+      </c>
+      <c r="V86" s="1">
+        <v>46382</v>
       </c>
     </row>
     <row r="87" spans="1:22">
       <c r="A87">
-        <v>64780</v>
+        <v>64760</v>
       </c>
       <c r="B87" t="s">
         <v>22</v>
@@ -5322,31 +5068,28 @@
         <v>28</v>
       </c>
       <c r="F87" t="s">
-        <v>41</v>
+        <v>42</v>
       </c>
       <c r="G87" t="s">
-        <v>45</v>
+        <v>46</v>
       </c>
       <c r="N87" t="s">
-        <v>97</v>
+        <v>99</v>
       </c>
       <c r="O87" t="s">
-        <v>97</v>
-      </c>
-      <c r="P87">
-        <v>3306000</v>
+        <v>99</v>
       </c>
       <c r="Q87" t="s">
-        <v>166</v>
+        <v>168</v>
       </c>
       <c r="R87" t="s">
-        <v>169</v>
+        <v>171</v>
       </c>
       <c r="S87" t="s">
-        <v>41</v>
+        <v>42</v>
       </c>
       <c r="T87" t="s">
-        <v>177</v>
+        <v>179</v>
       </c>
       <c r="U87" t="s">
         <v>28</v>
@@ -5354,48 +5097,89 @@
     </row>
     <row r="88" spans="1:22">
       <c r="A88">
+        <v>64780</v>
+      </c>
+      <c r="B88" t="s">
+        <v>22</v>
+      </c>
+      <c r="C88" t="s">
+        <v>22</v>
+      </c>
+      <c r="D88" t="s">
+        <v>25</v>
+      </c>
+      <c r="E88" t="s">
+        <v>28</v>
+      </c>
+      <c r="F88" t="s">
+        <v>42</v>
+      </c>
+      <c r="G88" t="s">
+        <v>46</v>
+      </c>
+      <c r="N88" t="s">
+        <v>99</v>
+      </c>
+      <c r="O88" t="s">
+        <v>99</v>
+      </c>
+      <c r="Q88" t="s">
+        <v>168</v>
+      </c>
+      <c r="R88" t="s">
+        <v>171</v>
+      </c>
+      <c r="S88" t="s">
+        <v>42</v>
+      </c>
+      <c r="T88" t="s">
+        <v>179</v>
+      </c>
+      <c r="U88" t="s">
+        <v>28</v>
+      </c>
+    </row>
+    <row r="89" spans="1:22">
+      <c r="A89">
         <v>64840</v>
       </c>
-      <c r="B88" t="s">
-        <v>22</v>
-      </c>
-      <c r="C88" t="s">
-        <v>22</v>
-      </c>
-      <c r="D88" t="s">
+      <c r="B89" t="s">
+        <v>22</v>
+      </c>
+      <c r="C89" t="s">
+        <v>22</v>
+      </c>
+      <c r="D89" t="s">
         <v>24</v>
       </c>
-      <c r="E88" t="s">
-        <v>28</v>
-      </c>
-      <c r="F88" t="s">
+      <c r="E89" t="s">
+        <v>28</v>
+      </c>
+      <c r="F89" t="s">
         <v>30</v>
       </c>
-      <c r="N88" t="s">
-        <v>98</v>
-      </c>
-      <c r="O88" t="s">
-        <v>165</v>
-      </c>
-      <c r="P88">
-        <v>470820</v>
-      </c>
-      <c r="Q88" t="s">
-        <v>166</v>
-      </c>
-      <c r="R88" t="s">
-        <v>169</v>
-      </c>
-      <c r="S88" t="s">
-        <v>172</v>
-      </c>
-      <c r="T88" t="s">
-        <v>180</v>
-      </c>
-      <c r="U88" t="s">
-        <v>28</v>
-      </c>
-      <c r="V88" s="2">
+      <c r="N89" t="s">
+        <v>100</v>
+      </c>
+      <c r="O89" t="s">
+        <v>167</v>
+      </c>
+      <c r="Q89" t="s">
+        <v>168</v>
+      </c>
+      <c r="R89" t="s">
+        <v>171</v>
+      </c>
+      <c r="S89" t="s">
+        <v>174</v>
+      </c>
+      <c r="T89" t="s">
+        <v>182</v>
+      </c>
+      <c r="U89" t="s">
+        <v>28</v>
+      </c>
+      <c r="V89" s="1">
         <v>46291</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Atualização automática: mta (18/09/2026 16:37)
</commit_message>
<xml_diff>
--- a/Projetos/02_Dados_Tratados/base_mta_tratada.xlsx
+++ b/Projetos/02_Dados_Tratados/base_mta_tratada.xlsx
@@ -575,8 +575,16 @@
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="YYYY-MM-DD HH:MM:SS"/>
   </numFmts>
-  <fonts count="1">
+  <fonts count="2">
     <font>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
       <sz val="11"/>
       <color theme="1"/>
       <name val="Calibri"/>
@@ -592,7 +600,7 @@
       <patternFill patternType="gray125"/>
     </fill>
   </fills>
-  <borders count="1">
+  <borders count="2">
     <border>
       <left/>
       <right/>
@@ -600,12 +608,30 @@
       <bottom/>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin">
+        <color auto="1"/>
+      </left>
+      <right style="thin">
+        <color auto="1"/>
+      </right>
+      <top style="thin">
+        <color auto="1"/>
+      </top>
+      <bottom style="thin">
+        <color auto="1"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="3">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
   </cellXfs>
   <cellStyles count="1">
@@ -905,70 +931,70 @@
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:22">
-      <c r="A1" t="s">
+      <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
-      <c r="B1" t="s">
+      <c r="B1" s="1" t="s">
         <v>1</v>
       </c>
-      <c r="C1" t="s">
+      <c r="C1" s="1" t="s">
         <v>2</v>
       </c>
-      <c r="D1" t="s">
+      <c r="D1" s="1" t="s">
         <v>3</v>
       </c>
-      <c r="E1" t="s">
+      <c r="E1" s="1" t="s">
         <v>4</v>
       </c>
-      <c r="F1" t="s">
+      <c r="F1" s="1" t="s">
         <v>5</v>
       </c>
-      <c r="G1" t="s">
+      <c r="G1" s="1" t="s">
         <v>6</v>
       </c>
-      <c r="H1" t="s">
+      <c r="H1" s="1" t="s">
         <v>7</v>
       </c>
-      <c r="I1" t="s">
+      <c r="I1" s="1" t="s">
         <v>8</v>
       </c>
-      <c r="J1" t="s">
+      <c r="J1" s="1" t="s">
         <v>9</v>
       </c>
-      <c r="K1" t="s">
+      <c r="K1" s="1" t="s">
         <v>10</v>
       </c>
-      <c r="L1" t="s">
+      <c r="L1" s="1" t="s">
         <v>11</v>
       </c>
-      <c r="M1" t="s">
+      <c r="M1" s="1" t="s">
         <v>12</v>
       </c>
-      <c r="N1" t="s">
+      <c r="N1" s="1" t="s">
         <v>13</v>
       </c>
-      <c r="O1" t="s">
+      <c r="O1" s="1" t="s">
         <v>14</v>
       </c>
-      <c r="P1" t="s">
+      <c r="P1" s="1" t="s">
         <v>15</v>
       </c>
-      <c r="Q1" t="s">
+      <c r="Q1" s="1" t="s">
         <v>16</v>
       </c>
-      <c r="R1" t="s">
+      <c r="R1" s="1" t="s">
         <v>17</v>
       </c>
-      <c r="S1" t="s">
+      <c r="S1" s="1" t="s">
         <v>18</v>
       </c>
-      <c r="T1" t="s">
+      <c r="T1" s="1" t="s">
         <v>19</v>
       </c>
-      <c r="U1" t="s">
+      <c r="U1" s="1" t="s">
         <v>20</v>
       </c>
-      <c r="V1" t="s">
+      <c r="V1" s="1" t="s">
         <v>21</v>
       </c>
     </row>
@@ -1021,7 +1047,7 @@
       <c r="U2" t="s">
         <v>183</v>
       </c>
-      <c r="V2" s="1">
+      <c r="V2" s="2">
         <v>46229</v>
       </c>
     </row>
@@ -1065,7 +1091,7 @@
       <c r="U3" t="s">
         <v>28</v>
       </c>
-      <c r="V3" s="1">
+      <c r="V3" s="2">
         <v>46291</v>
       </c>
     </row>
@@ -1112,7 +1138,7 @@
       <c r="U4" t="s">
         <v>28</v>
       </c>
-      <c r="V4" s="1">
+      <c r="V4" s="2">
         <v>46321</v>
       </c>
     </row>
@@ -1156,7 +1182,7 @@
       <c r="U5" t="s">
         <v>28</v>
       </c>
-      <c r="V5" s="1">
+      <c r="V5" s="2">
         <v>46321</v>
       </c>
     </row>
@@ -1203,7 +1229,7 @@
       <c r="U6" t="s">
         <v>28</v>
       </c>
-      <c r="V6" s="1">
+      <c r="V6" s="2">
         <v>46291</v>
       </c>
     </row>
@@ -1229,7 +1255,7 @@
       <c r="G7" t="s">
         <v>44</v>
       </c>
-      <c r="H7" s="1">
+      <c r="H7" s="2">
         <v>46121</v>
       </c>
       <c r="I7" t="s">
@@ -1256,7 +1282,7 @@
       <c r="U7" t="s">
         <v>28</v>
       </c>
-      <c r="V7" s="1">
+      <c r="V7" s="2">
         <v>46138</v>
       </c>
     </row>
@@ -1300,7 +1326,7 @@
       <c r="U8" t="s">
         <v>28</v>
       </c>
-      <c r="V8" s="1">
+      <c r="V8" s="2">
         <v>46291</v>
       </c>
     </row>
@@ -1344,7 +1370,7 @@
       <c r="U9" t="s">
         <v>28</v>
       </c>
-      <c r="V9" s="1">
+      <c r="V9" s="2">
         <v>46291</v>
       </c>
     </row>
@@ -1388,7 +1414,7 @@
       <c r="U10" t="s">
         <v>28</v>
       </c>
-      <c r="V10" s="1">
+      <c r="V10" s="2">
         <v>46291</v>
       </c>
     </row>
@@ -1432,7 +1458,7 @@
       <c r="U11" t="s">
         <v>28</v>
       </c>
-      <c r="V11" s="1">
+      <c r="V11" s="2">
         <v>46291</v>
       </c>
     </row>
@@ -1458,7 +1484,7 @@
       <c r="G12" t="s">
         <v>44</v>
       </c>
-      <c r="H12" s="1">
+      <c r="H12" s="2">
         <v>46079</v>
       </c>
       <c r="I12" t="s">
@@ -1488,7 +1514,7 @@
       <c r="U12" t="s">
         <v>183</v>
       </c>
-      <c r="V12" s="1">
+      <c r="V12" s="2">
         <v>46079</v>
       </c>
     </row>
@@ -1538,7 +1564,7 @@
       <c r="U13" t="s">
         <v>183</v>
       </c>
-      <c r="V13" s="1">
+      <c r="V13" s="2">
         <v>46352</v>
       </c>
     </row>
@@ -1588,7 +1614,7 @@
       <c r="U14" t="s">
         <v>183</v>
       </c>
-      <c r="V14" s="1">
+      <c r="V14" s="2">
         <v>46352</v>
       </c>
     </row>
@@ -1638,7 +1664,7 @@
       <c r="U15" t="s">
         <v>183</v>
       </c>
-      <c r="V15" s="1">
+      <c r="V15" s="2">
         <v>46352</v>
       </c>
     </row>
@@ -1688,7 +1714,7 @@
       <c r="U16" t="s">
         <v>183</v>
       </c>
-      <c r="V16" s="1">
+      <c r="V16" s="2">
         <v>46229</v>
       </c>
     </row>
@@ -1714,7 +1740,7 @@
       <c r="G17" t="s">
         <v>44</v>
       </c>
-      <c r="H17" s="1">
+      <c r="H17" s="2">
         <v>46098</v>
       </c>
       <c r="I17" t="s">
@@ -1744,7 +1770,7 @@
       <c r="U17" t="s">
         <v>183</v>
       </c>
-      <c r="V17" s="1">
+      <c r="V17" s="2">
         <v>46107</v>
       </c>
     </row>
@@ -1770,7 +1796,7 @@
       <c r="G18" t="s">
         <v>44</v>
       </c>
-      <c r="H18" s="1">
+      <c r="H18" s="2">
         <v>46076</v>
       </c>
       <c r="I18" t="s">
@@ -1797,7 +1823,7 @@
       <c r="U18" t="s">
         <v>28</v>
       </c>
-      <c r="V18" s="1">
+      <c r="V18" s="2">
         <v>46079</v>
       </c>
     </row>
@@ -1823,7 +1849,7 @@
       <c r="G19" t="s">
         <v>44</v>
       </c>
-      <c r="H19" s="1">
+      <c r="H19" s="2">
         <v>46076</v>
       </c>
       <c r="I19" t="s">
@@ -1850,7 +1876,7 @@
       <c r="U19" t="s">
         <v>28</v>
       </c>
-      <c r="V19" s="1">
+      <c r="V19" s="2">
         <v>46079</v>
       </c>
     </row>
@@ -1894,7 +1920,7 @@
       <c r="U20" t="s">
         <v>28</v>
       </c>
-      <c r="V20" s="1">
+      <c r="V20" s="2">
         <v>46321</v>
       </c>
     </row>
@@ -1938,7 +1964,7 @@
       <c r="U21" t="s">
         <v>28</v>
       </c>
-      <c r="V21" s="1">
+      <c r="V21" s="2">
         <v>46321</v>
       </c>
     </row>
@@ -1982,7 +2008,7 @@
       <c r="U22" t="s">
         <v>28</v>
       </c>
-      <c r="V22" s="1">
+      <c r="V22" s="2">
         <v>46321</v>
       </c>
     </row>
@@ -2026,7 +2052,7 @@
       <c r="U23" t="s">
         <v>28</v>
       </c>
-      <c r="V23" s="1">
+      <c r="V23" s="2">
         <v>46321</v>
       </c>
     </row>
@@ -2052,7 +2078,7 @@
       <c r="G24" t="s">
         <v>44</v>
       </c>
-      <c r="H24" s="1">
+      <c r="H24" s="2">
         <v>46119</v>
       </c>
       <c r="I24" t="s">
@@ -2082,7 +2108,7 @@
       <c r="U24" t="s">
         <v>183</v>
       </c>
-      <c r="V24" s="1">
+      <c r="V24" s="2">
         <v>46138</v>
       </c>
     </row>
@@ -2108,7 +2134,7 @@
       <c r="G25" t="s">
         <v>44</v>
       </c>
-      <c r="H25" s="1">
+      <c r="H25" s="2">
         <v>46121</v>
       </c>
       <c r="I25" t="s">
@@ -2135,7 +2161,7 @@
       <c r="U25" t="s">
         <v>28</v>
       </c>
-      <c r="V25" s="1">
+      <c r="V25" s="2">
         <v>46138</v>
       </c>
     </row>
@@ -2161,7 +2187,7 @@
       <c r="G26" t="s">
         <v>44</v>
       </c>
-      <c r="H26" s="1">
+      <c r="H26" s="2">
         <v>46076</v>
       </c>
       <c r="I26" t="s">
@@ -2188,7 +2214,7 @@
       <c r="U26" t="s">
         <v>28</v>
       </c>
-      <c r="V26" s="1">
+      <c r="V26" s="2">
         <v>46079</v>
       </c>
     </row>
@@ -2238,7 +2264,7 @@
       <c r="U27" t="s">
         <v>183</v>
       </c>
-      <c r="V27" s="1">
+      <c r="V27" s="2">
         <v>46291</v>
       </c>
     </row>
@@ -2264,7 +2290,7 @@
       <c r="G28" t="s">
         <v>44</v>
       </c>
-      <c r="H28" s="1">
+      <c r="H28" s="2">
         <v>46199</v>
       </c>
       <c r="I28" t="s">
@@ -2294,7 +2320,7 @@
       <c r="U28" t="s">
         <v>183</v>
       </c>
-      <c r="V28" s="1">
+      <c r="V28" s="2">
         <v>46199</v>
       </c>
     </row>
@@ -2320,7 +2346,7 @@
       <c r="G29" t="s">
         <v>44</v>
       </c>
-      <c r="H29" s="1">
+      <c r="H29" s="2">
         <v>46199</v>
       </c>
       <c r="I29" t="s">
@@ -2350,7 +2376,7 @@
       <c r="U29" t="s">
         <v>183</v>
       </c>
-      <c r="V29" s="1">
+      <c r="V29" s="2">
         <v>46199</v>
       </c>
     </row>
@@ -2376,7 +2402,7 @@
       <c r="G30" t="s">
         <v>44</v>
       </c>
-      <c r="H30" s="1">
+      <c r="H30" s="2">
         <v>46199</v>
       </c>
       <c r="I30" t="s">
@@ -2406,7 +2432,7 @@
       <c r="U30" t="s">
         <v>183</v>
       </c>
-      <c r="V30" s="1">
+      <c r="V30" s="2">
         <v>46199</v>
       </c>
     </row>
@@ -2432,7 +2458,7 @@
       <c r="G31" t="s">
         <v>44</v>
       </c>
-      <c r="H31" s="1">
+      <c r="H31" s="2">
         <v>46199</v>
       </c>
       <c r="I31" t="s">
@@ -2462,7 +2488,7 @@
       <c r="U31" t="s">
         <v>183</v>
       </c>
-      <c r="V31" s="1">
+      <c r="V31" s="2">
         <v>46199</v>
       </c>
     </row>
@@ -2509,7 +2535,7 @@
       <c r="U32" t="s">
         <v>183</v>
       </c>
-      <c r="V32" s="1">
+      <c r="V32" s="2">
         <v>46291</v>
       </c>
     </row>
@@ -2535,7 +2561,7 @@
       <c r="G33" t="s">
         <v>44</v>
       </c>
-      <c r="H33" s="1">
+      <c r="H33" s="2">
         <v>46191</v>
       </c>
       <c r="I33" t="s">
@@ -2565,7 +2591,7 @@
       <c r="U33" t="s">
         <v>183</v>
       </c>
-      <c r="V33" s="1">
+      <c r="V33" s="2">
         <v>46199</v>
       </c>
     </row>
@@ -2591,7 +2617,7 @@
       <c r="G34" t="s">
         <v>44</v>
       </c>
-      <c r="H34" s="1">
+      <c r="H34" s="2">
         <v>46119</v>
       </c>
       <c r="I34" t="s">
@@ -2618,7 +2644,7 @@
       <c r="U34" t="s">
         <v>183</v>
       </c>
-      <c r="V34" s="1">
+      <c r="V34" s="2">
         <v>46138</v>
       </c>
     </row>
@@ -2644,7 +2670,7 @@
       <c r="G35" t="s">
         <v>44</v>
       </c>
-      <c r="H35" s="1">
+      <c r="H35" s="2">
         <v>46213</v>
       </c>
       <c r="I35" t="s">
@@ -2671,7 +2697,7 @@
       <c r="U35" t="s">
         <v>28</v>
       </c>
-      <c r="V35" s="1">
+      <c r="V35" s="2">
         <v>46229</v>
       </c>
     </row>
@@ -2697,7 +2723,7 @@
       <c r="G36" t="s">
         <v>44</v>
       </c>
-      <c r="H36" s="1">
+      <c r="H36" s="2">
         <v>46175</v>
       </c>
       <c r="I36" t="s">
@@ -2724,7 +2750,7 @@
       <c r="U36" t="s">
         <v>28</v>
       </c>
-      <c r="V36" s="1">
+      <c r="V36" s="2">
         <v>46199</v>
       </c>
     </row>
@@ -2750,7 +2776,7 @@
       <c r="G37" t="s">
         <v>44</v>
       </c>
-      <c r="H37" s="1">
+      <c r="H37" s="2">
         <v>46213</v>
       </c>
       <c r="I37" t="s">
@@ -2777,7 +2803,7 @@
       <c r="U37" t="s">
         <v>28</v>
       </c>
-      <c r="V37" s="1">
+      <c r="V37" s="2">
         <v>46229</v>
       </c>
     </row>
@@ -2803,7 +2829,7 @@
       <c r="G38" t="s">
         <v>44</v>
       </c>
-      <c r="H38" s="1">
+      <c r="H38" s="2">
         <v>46199</v>
       </c>
       <c r="I38" t="s">
@@ -2830,7 +2856,7 @@
       <c r="U38" t="s">
         <v>28</v>
       </c>
-      <c r="V38" s="1">
+      <c r="V38" s="2">
         <v>46199</v>
       </c>
     </row>
@@ -2856,7 +2882,7 @@
       <c r="G39" t="s">
         <v>44</v>
       </c>
-      <c r="H39" s="1">
+      <c r="H39" s="2">
         <v>46199</v>
       </c>
       <c r="I39" t="s">
@@ -2883,7 +2909,7 @@
       <c r="U39" t="s">
         <v>28</v>
       </c>
-      <c r="V39" s="1">
+      <c r="V39" s="2">
         <v>46199</v>
       </c>
     </row>
@@ -2909,7 +2935,7 @@
       <c r="G40" t="s">
         <v>44</v>
       </c>
-      <c r="H40" s="1">
+      <c r="H40" s="2">
         <v>46204</v>
       </c>
       <c r="I40" t="s">
@@ -2936,7 +2962,7 @@
       <c r="U40" t="s">
         <v>28</v>
       </c>
-      <c r="V40" s="1">
+      <c r="V40" s="2">
         <v>46229</v>
       </c>
     </row>
@@ -2962,7 +2988,7 @@
       <c r="G41" t="s">
         <v>44</v>
       </c>
-      <c r="H41" s="1">
+      <c r="H41" s="2">
         <v>46244</v>
       </c>
       <c r="I41" t="s">
@@ -2989,7 +3015,7 @@
       <c r="U41" t="s">
         <v>28</v>
       </c>
-      <c r="V41" s="1">
+      <c r="V41" s="2">
         <v>46199</v>
       </c>
     </row>
@@ -3033,7 +3059,7 @@
       <c r="U42" t="s">
         <v>28</v>
       </c>
-      <c r="V42" s="1">
+      <c r="V42" s="2">
         <v>46260</v>
       </c>
     </row>
@@ -3059,7 +3085,7 @@
       <c r="G43" t="s">
         <v>44</v>
       </c>
-      <c r="H43" s="1">
+      <c r="H43" s="2">
         <v>46191</v>
       </c>
       <c r="I43" t="s">
@@ -3086,7 +3112,7 @@
       <c r="U43" t="s">
         <v>28</v>
       </c>
-      <c r="V43" s="1">
+      <c r="V43" s="2">
         <v>46199</v>
       </c>
     </row>
@@ -3112,7 +3138,7 @@
       <c r="G44" t="s">
         <v>44</v>
       </c>
-      <c r="H44" s="1">
+      <c r="H44" s="2">
         <v>46191</v>
       </c>
       <c r="I44" t="s">
@@ -3139,7 +3165,7 @@
       <c r="U44" t="s">
         <v>28</v>
       </c>
-      <c r="V44" s="1">
+      <c r="V44" s="2">
         <v>46199</v>
       </c>
     </row>
@@ -3165,7 +3191,7 @@
       <c r="G45" t="s">
         <v>44</v>
       </c>
-      <c r="H45" s="1">
+      <c r="H45" s="2">
         <v>46213</v>
       </c>
       <c r="I45" t="s">
@@ -3195,7 +3221,7 @@
       <c r="U45" t="s">
         <v>183</v>
       </c>
-      <c r="V45" s="1">
+      <c r="V45" s="2">
         <v>46229</v>
       </c>
     </row>
@@ -3221,7 +3247,7 @@
       <c r="G46" t="s">
         <v>44</v>
       </c>
-      <c r="H46" s="1">
+      <c r="H46" s="2">
         <v>46210</v>
       </c>
       <c r="I46" t="s">
@@ -3248,7 +3274,7 @@
       <c r="U46" t="s">
         <v>183</v>
       </c>
-      <c r="V46" s="1">
+      <c r="V46" s="2">
         <v>46229</v>
       </c>
     </row>
@@ -3292,7 +3318,7 @@
       <c r="U47" t="s">
         <v>28</v>
       </c>
-      <c r="V47" s="1">
+      <c r="V47" s="2">
         <v>46321</v>
       </c>
     </row>
@@ -3342,7 +3368,7 @@
       <c r="U48" t="s">
         <v>183</v>
       </c>
-      <c r="V48" s="1">
+      <c r="V48" s="2">
         <v>46291</v>
       </c>
     </row>
@@ -3368,7 +3394,7 @@
       <c r="G49" t="s">
         <v>44</v>
       </c>
-      <c r="H49" s="1">
+      <c r="H49" s="2">
         <v>46176</v>
       </c>
       <c r="I49" t="s">
@@ -3398,7 +3424,7 @@
       <c r="U49" t="s">
         <v>183</v>
       </c>
-      <c r="V49" s="1">
+      <c r="V49" s="2">
         <v>46199</v>
       </c>
     </row>
@@ -3421,7 +3447,7 @@
       <c r="G50" t="s">
         <v>44</v>
       </c>
-      <c r="H50" s="1">
+      <c r="H50" s="2">
         <v>46280</v>
       </c>
       <c r="I50" t="s">
@@ -3448,7 +3474,7 @@
       <c r="U50" t="s">
         <v>183</v>
       </c>
-      <c r="V50" s="1">
+      <c r="V50" s="2">
         <v>46260</v>
       </c>
     </row>
@@ -3498,7 +3524,7 @@
       <c r="U51" t="s">
         <v>183</v>
       </c>
-      <c r="V51" s="1">
+      <c r="V51" s="2">
         <v>46260</v>
       </c>
     </row>
@@ -3548,7 +3574,7 @@
       <c r="U52" t="s">
         <v>183</v>
       </c>
-      <c r="V52" s="1">
+      <c r="V52" s="2">
         <v>46291</v>
       </c>
     </row>
@@ -3595,7 +3621,7 @@
       <c r="U53" t="s">
         <v>183</v>
       </c>
-      <c r="V53" s="1">
+      <c r="V53" s="2">
         <v>46321</v>
       </c>
     </row>
@@ -3621,7 +3647,7 @@
       <c r="G54" t="s">
         <v>44</v>
       </c>
-      <c r="H54" s="1">
+      <c r="H54" s="2">
         <v>46227</v>
       </c>
       <c r="I54" t="s">
@@ -3648,7 +3674,7 @@
       <c r="U54" t="s">
         <v>183</v>
       </c>
-      <c r="V54" s="1">
+      <c r="V54" s="2">
         <v>46229</v>
       </c>
     </row>
@@ -3671,7 +3697,7 @@
       <c r="G55" t="s">
         <v>44</v>
       </c>
-      <c r="H55" s="1">
+      <c r="H55" s="2">
         <v>46280</v>
       </c>
       <c r="I55" t="s">
@@ -3698,7 +3724,7 @@
       <c r="U55" t="s">
         <v>183</v>
       </c>
-      <c r="V55" s="1">
+      <c r="V55" s="2">
         <v>46291</v>
       </c>
     </row>
@@ -3748,7 +3774,7 @@
       <c r="U56" t="s">
         <v>183</v>
       </c>
-      <c r="V56" s="1">
+      <c r="V56" s="2">
         <v>46352</v>
       </c>
     </row>
@@ -3798,7 +3824,7 @@
       <c r="U57" t="s">
         <v>183</v>
       </c>
-      <c r="V57" s="1">
+      <c r="V57" s="2">
         <v>46321</v>
       </c>
     </row>
@@ -3842,7 +3868,7 @@
       <c r="U58" t="s">
         <v>183</v>
       </c>
-      <c r="V58" s="1">
+      <c r="V58" s="2">
         <v>46321</v>
       </c>
     </row>
@@ -3886,7 +3912,7 @@
       <c r="U59" t="s">
         <v>183</v>
       </c>
-      <c r="V59" s="1">
+      <c r="V59" s="2">
         <v>46049</v>
       </c>
     </row>
@@ -4009,7 +4035,7 @@
       <c r="U62" t="s">
         <v>183</v>
       </c>
-      <c r="V62" s="1">
+      <c r="V62" s="2">
         <v>46107</v>
       </c>
     </row>
@@ -4050,7 +4076,7 @@
       <c r="U63" t="s">
         <v>183</v>
       </c>
-      <c r="V63" s="1">
+      <c r="V63" s="2">
         <v>46107</v>
       </c>
     </row>
@@ -4091,7 +4117,7 @@
       <c r="U64" t="s">
         <v>183</v>
       </c>
-      <c r="V64" s="1">
+      <c r="V64" s="2">
         <v>46107</v>
       </c>
     </row>
@@ -4132,7 +4158,7 @@
       <c r="U65" t="s">
         <v>183</v>
       </c>
-      <c r="V65" s="1">
+      <c r="V65" s="2">
         <v>46107</v>
       </c>
     </row>
@@ -4173,7 +4199,7 @@
       <c r="U66" t="s">
         <v>183</v>
       </c>
-      <c r="V66" s="1">
+      <c r="V66" s="2">
         <v>46107</v>
       </c>
     </row>
@@ -4214,7 +4240,7 @@
       <c r="U67" t="s">
         <v>183</v>
       </c>
-      <c r="V67" s="1">
+      <c r="V67" s="2">
         <v>46107</v>
       </c>
     </row>
@@ -4255,7 +4281,7 @@
       <c r="U68" t="s">
         <v>28</v>
       </c>
-      <c r="V68" s="1">
+      <c r="V68" s="2">
         <v>46168</v>
       </c>
     </row>
@@ -4299,7 +4325,7 @@
       <c r="U69" t="s">
         <v>28</v>
       </c>
-      <c r="V69" s="1">
+      <c r="V69" s="2">
         <v>46291</v>
       </c>
     </row>
@@ -4349,7 +4375,7 @@
       <c r="U70" t="s">
         <v>183</v>
       </c>
-      <c r="V70" s="1">
+      <c r="V70" s="2">
         <v>46229</v>
       </c>
     </row>
@@ -4390,7 +4416,7 @@
       <c r="U71" t="s">
         <v>28</v>
       </c>
-      <c r="V71" s="1">
+      <c r="V71" s="2">
         <v>46260</v>
       </c>
     </row>
@@ -4431,7 +4457,7 @@
       <c r="U72" t="s">
         <v>183</v>
       </c>
-      <c r="V72" s="1">
+      <c r="V72" s="2">
         <v>46291</v>
       </c>
     </row>
@@ -4472,7 +4498,7 @@
       <c r="U73" t="s">
         <v>183</v>
       </c>
-      <c r="V73" s="1">
+      <c r="V73" s="2">
         <v>46168</v>
       </c>
     </row>
@@ -4513,7 +4539,7 @@
       <c r="U74" t="s">
         <v>183</v>
       </c>
-      <c r="V74" s="1">
+      <c r="V74" s="2">
         <v>46291</v>
       </c>
     </row>
@@ -4554,7 +4580,7 @@
       <c r="U75" t="s">
         <v>183</v>
       </c>
-      <c r="V75" s="1">
+      <c r="V75" s="2">
         <v>46291</v>
       </c>
     </row>
@@ -4595,7 +4621,7 @@
       <c r="U76" t="s">
         <v>183</v>
       </c>
-      <c r="V76" s="1">
+      <c r="V76" s="2">
         <v>46291</v>
       </c>
     </row>
@@ -4639,7 +4665,7 @@
       <c r="U77" t="s">
         <v>28</v>
       </c>
-      <c r="V77" s="1">
+      <c r="V77" s="2">
         <v>46321</v>
       </c>
     </row>
@@ -4686,7 +4712,7 @@
       <c r="U78" t="s">
         <v>183</v>
       </c>
-      <c r="V78" s="1">
+      <c r="V78" s="2">
         <v>46381</v>
       </c>
     </row>
@@ -4733,7 +4759,7 @@
       <c r="U79" t="s">
         <v>183</v>
       </c>
-      <c r="V79" s="1">
+      <c r="V79" s="2">
         <v>46381</v>
       </c>
     </row>
@@ -4780,7 +4806,7 @@
       <c r="U80" t="s">
         <v>28</v>
       </c>
-      <c r="V80" s="1">
+      <c r="V80" s="2">
         <v>46381</v>
       </c>
     </row>
@@ -4827,7 +4853,7 @@
       <c r="U81" t="s">
         <v>28</v>
       </c>
-      <c r="V81" s="1">
+      <c r="V81" s="2">
         <v>46381</v>
       </c>
     </row>
@@ -4874,7 +4900,7 @@
       <c r="U82" t="s">
         <v>28</v>
       </c>
-      <c r="V82" s="1">
+      <c r="V82" s="2">
         <v>46382</v>
       </c>
     </row>
@@ -4915,7 +4941,7 @@
       <c r="U83" t="s">
         <v>28</v>
       </c>
-      <c r="V83" s="1">
+      <c r="V83" s="2">
         <v>46382</v>
       </c>
     </row>
@@ -4965,7 +4991,7 @@
       <c r="U84" t="s">
         <v>183</v>
       </c>
-      <c r="V84" s="1">
+      <c r="V84" s="2">
         <v>46382</v>
       </c>
     </row>
@@ -5006,7 +5032,7 @@
       <c r="U85" t="s">
         <v>28</v>
       </c>
-      <c r="V85" s="1">
+      <c r="V85" s="2">
         <v>46321</v>
       </c>
     </row>
@@ -5047,7 +5073,7 @@
       <c r="U86" t="s">
         <v>28</v>
       </c>
-      <c r="V86" s="1">
+      <c r="V86" s="2">
         <v>46382</v>
       </c>
     </row>
@@ -5179,7 +5205,7 @@
       <c r="U89" t="s">
         <v>28</v>
       </c>
-      <c r="V89" s="1">
+      <c r="V89" s="2">
         <v>46291</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Atualização automática: mta (21/09/2026 13:59)
</commit_message>
<xml_diff>
--- a/Projetos/02_Dados_Tratados/base_mta_tratada.xlsx
+++ b/Projetos/02_Dados_Tratados/base_mta_tratada.xlsx
@@ -575,16 +575,8 @@
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="YYYY-MM-DD HH:MM:SS"/>
   </numFmts>
-  <fonts count="2">
+  <fonts count="1">
     <font>
-      <sz val="11"/>
-      <color theme="1"/>
-      <name val="Calibri"/>
-      <family val="2"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <b/>
       <sz val="11"/>
       <color theme="1"/>
       <name val="Calibri"/>
@@ -600,7 +592,7 @@
       <patternFill patternType="gray125"/>
     </fill>
   </fills>
-  <borders count="2">
+  <borders count="1">
     <border>
       <left/>
       <right/>
@@ -608,30 +600,12 @@
       <bottom/>
       <diagonal/>
     </border>
-    <border>
-      <left style="thin">
-        <color auto="1"/>
-      </left>
-      <right style="thin">
-        <color auto="1"/>
-      </right>
-      <top style="thin">
-        <color auto="1"/>
-      </top>
-      <bottom style="thin">
-        <color auto="1"/>
-      </bottom>
-      <diagonal/>
-    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="3">
+  <cellXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top"/>
-    </xf>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
   </cellXfs>
   <cellStyles count="1">
@@ -931,70 +905,70 @@
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:22">
-      <c r="A1" s="1" t="s">
+      <c r="A1" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="1" t="s">
+      <c r="B1" t="s">
         <v>1</v>
       </c>
-      <c r="C1" s="1" t="s">
+      <c r="C1" t="s">
         <v>2</v>
       </c>
-      <c r="D1" s="1" t="s">
+      <c r="D1" t="s">
         <v>3</v>
       </c>
-      <c r="E1" s="1" t="s">
+      <c r="E1" t="s">
         <v>4</v>
       </c>
-      <c r="F1" s="1" t="s">
+      <c r="F1" t="s">
         <v>5</v>
       </c>
-      <c r="G1" s="1" t="s">
+      <c r="G1" t="s">
         <v>6</v>
       </c>
-      <c r="H1" s="1" t="s">
+      <c r="H1" t="s">
         <v>7</v>
       </c>
-      <c r="I1" s="1" t="s">
+      <c r="I1" t="s">
         <v>8</v>
       </c>
-      <c r="J1" s="1" t="s">
+      <c r="J1" t="s">
         <v>9</v>
       </c>
-      <c r="K1" s="1" t="s">
+      <c r="K1" t="s">
         <v>10</v>
       </c>
-      <c r="L1" s="1" t="s">
+      <c r="L1" t="s">
         <v>11</v>
       </c>
-      <c r="M1" s="1" t="s">
+      <c r="M1" t="s">
         <v>12</v>
       </c>
-      <c r="N1" s="1" t="s">
+      <c r="N1" t="s">
         <v>13</v>
       </c>
-      <c r="O1" s="1" t="s">
+      <c r="O1" t="s">
         <v>14</v>
       </c>
-      <c r="P1" s="1" t="s">
+      <c r="P1" t="s">
         <v>15</v>
       </c>
-      <c r="Q1" s="1" t="s">
+      <c r="Q1" t="s">
         <v>16</v>
       </c>
-      <c r="R1" s="1" t="s">
+      <c r="R1" t="s">
         <v>17</v>
       </c>
-      <c r="S1" s="1" t="s">
+      <c r="S1" t="s">
         <v>18</v>
       </c>
-      <c r="T1" s="1" t="s">
+      <c r="T1" t="s">
         <v>19</v>
       </c>
-      <c r="U1" s="1" t="s">
+      <c r="U1" t="s">
         <v>20</v>
       </c>
-      <c r="V1" s="1" t="s">
+      <c r="V1" t="s">
         <v>21</v>
       </c>
     </row>
@@ -1047,7 +1021,7 @@
       <c r="U2" t="s">
         <v>183</v>
       </c>
-      <c r="V2" s="2">
+      <c r="V2" s="1">
         <v>46229</v>
       </c>
     </row>
@@ -1091,7 +1065,7 @@
       <c r="U3" t="s">
         <v>28</v>
       </c>
-      <c r="V3" s="2">
+      <c r="V3" s="1">
         <v>46291</v>
       </c>
     </row>
@@ -1138,7 +1112,7 @@
       <c r="U4" t="s">
         <v>28</v>
       </c>
-      <c r="V4" s="2">
+      <c r="V4" s="1">
         <v>46321</v>
       </c>
     </row>
@@ -1182,7 +1156,7 @@
       <c r="U5" t="s">
         <v>28</v>
       </c>
-      <c r="V5" s="2">
+      <c r="V5" s="1">
         <v>46321</v>
       </c>
     </row>
@@ -1229,7 +1203,7 @@
       <c r="U6" t="s">
         <v>28</v>
       </c>
-      <c r="V6" s="2">
+      <c r="V6" s="1">
         <v>46291</v>
       </c>
     </row>
@@ -1255,7 +1229,7 @@
       <c r="G7" t="s">
         <v>44</v>
       </c>
-      <c r="H7" s="2">
+      <c r="H7" s="1">
         <v>46121</v>
       </c>
       <c r="I7" t="s">
@@ -1282,7 +1256,7 @@
       <c r="U7" t="s">
         <v>28</v>
       </c>
-      <c r="V7" s="2">
+      <c r="V7" s="1">
         <v>46138</v>
       </c>
     </row>
@@ -1326,7 +1300,7 @@
       <c r="U8" t="s">
         <v>28</v>
       </c>
-      <c r="V8" s="2">
+      <c r="V8" s="1">
         <v>46291</v>
       </c>
     </row>
@@ -1370,7 +1344,7 @@
       <c r="U9" t="s">
         <v>28</v>
       </c>
-      <c r="V9" s="2">
+      <c r="V9" s="1">
         <v>46291</v>
       </c>
     </row>
@@ -1414,7 +1388,7 @@
       <c r="U10" t="s">
         <v>28</v>
       </c>
-      <c r="V10" s="2">
+      <c r="V10" s="1">
         <v>46291</v>
       </c>
     </row>
@@ -1458,7 +1432,7 @@
       <c r="U11" t="s">
         <v>28</v>
       </c>
-      <c r="V11" s="2">
+      <c r="V11" s="1">
         <v>46291</v>
       </c>
     </row>
@@ -1484,7 +1458,7 @@
       <c r="G12" t="s">
         <v>44</v>
       </c>
-      <c r="H12" s="2">
+      <c r="H12" s="1">
         <v>46079</v>
       </c>
       <c r="I12" t="s">
@@ -1514,7 +1488,7 @@
       <c r="U12" t="s">
         <v>183</v>
       </c>
-      <c r="V12" s="2">
+      <c r="V12" s="1">
         <v>46079</v>
       </c>
     </row>
@@ -1564,7 +1538,7 @@
       <c r="U13" t="s">
         <v>183</v>
       </c>
-      <c r="V13" s="2">
+      <c r="V13" s="1">
         <v>46352</v>
       </c>
     </row>
@@ -1614,7 +1588,7 @@
       <c r="U14" t="s">
         <v>183</v>
       </c>
-      <c r="V14" s="2">
+      <c r="V14" s="1">
         <v>46352</v>
       </c>
     </row>
@@ -1664,7 +1638,7 @@
       <c r="U15" t="s">
         <v>183</v>
       </c>
-      <c r="V15" s="2">
+      <c r="V15" s="1">
         <v>46352</v>
       </c>
     </row>
@@ -1714,7 +1688,7 @@
       <c r="U16" t="s">
         <v>183</v>
       </c>
-      <c r="V16" s="2">
+      <c r="V16" s="1">
         <v>46229</v>
       </c>
     </row>
@@ -1740,7 +1714,7 @@
       <c r="G17" t="s">
         <v>44</v>
       </c>
-      <c r="H17" s="2">
+      <c r="H17" s="1">
         <v>46098</v>
       </c>
       <c r="I17" t="s">
@@ -1770,7 +1744,7 @@
       <c r="U17" t="s">
         <v>183</v>
       </c>
-      <c r="V17" s="2">
+      <c r="V17" s="1">
         <v>46107</v>
       </c>
     </row>
@@ -1796,7 +1770,7 @@
       <c r="G18" t="s">
         <v>44</v>
       </c>
-      <c r="H18" s="2">
+      <c r="H18" s="1">
         <v>46076</v>
       </c>
       <c r="I18" t="s">
@@ -1823,7 +1797,7 @@
       <c r="U18" t="s">
         <v>28</v>
       </c>
-      <c r="V18" s="2">
+      <c r="V18" s="1">
         <v>46079</v>
       </c>
     </row>
@@ -1849,7 +1823,7 @@
       <c r="G19" t="s">
         <v>44</v>
       </c>
-      <c r="H19" s="2">
+      <c r="H19" s="1">
         <v>46076</v>
       </c>
       <c r="I19" t="s">
@@ -1876,7 +1850,7 @@
       <c r="U19" t="s">
         <v>28</v>
       </c>
-      <c r="V19" s="2">
+      <c r="V19" s="1">
         <v>46079</v>
       </c>
     </row>
@@ -1920,7 +1894,7 @@
       <c r="U20" t="s">
         <v>28</v>
       </c>
-      <c r="V20" s="2">
+      <c r="V20" s="1">
         <v>46321</v>
       </c>
     </row>
@@ -1964,7 +1938,7 @@
       <c r="U21" t="s">
         <v>28</v>
       </c>
-      <c r="V21" s="2">
+      <c r="V21" s="1">
         <v>46321</v>
       </c>
     </row>
@@ -2008,7 +1982,7 @@
       <c r="U22" t="s">
         <v>28</v>
       </c>
-      <c r="V22" s="2">
+      <c r="V22" s="1">
         <v>46321</v>
       </c>
     </row>
@@ -2052,7 +2026,7 @@
       <c r="U23" t="s">
         <v>28</v>
       </c>
-      <c r="V23" s="2">
+      <c r="V23" s="1">
         <v>46321</v>
       </c>
     </row>
@@ -2078,7 +2052,7 @@
       <c r="G24" t="s">
         <v>44</v>
       </c>
-      <c r="H24" s="2">
+      <c r="H24" s="1">
         <v>46119</v>
       </c>
       <c r="I24" t="s">
@@ -2108,7 +2082,7 @@
       <c r="U24" t="s">
         <v>183</v>
       </c>
-      <c r="V24" s="2">
+      <c r="V24" s="1">
         <v>46138</v>
       </c>
     </row>
@@ -2134,7 +2108,7 @@
       <c r="G25" t="s">
         <v>44</v>
       </c>
-      <c r="H25" s="2">
+      <c r="H25" s="1">
         <v>46121</v>
       </c>
       <c r="I25" t="s">
@@ -2161,7 +2135,7 @@
       <c r="U25" t="s">
         <v>28</v>
       </c>
-      <c r="V25" s="2">
+      <c r="V25" s="1">
         <v>46138</v>
       </c>
     </row>
@@ -2187,7 +2161,7 @@
       <c r="G26" t="s">
         <v>44</v>
       </c>
-      <c r="H26" s="2">
+      <c r="H26" s="1">
         <v>46076</v>
       </c>
       <c r="I26" t="s">
@@ -2214,7 +2188,7 @@
       <c r="U26" t="s">
         <v>28</v>
       </c>
-      <c r="V26" s="2">
+      <c r="V26" s="1">
         <v>46079</v>
       </c>
     </row>
@@ -2264,7 +2238,7 @@
       <c r="U27" t="s">
         <v>183</v>
       </c>
-      <c r="V27" s="2">
+      <c r="V27" s="1">
         <v>46291</v>
       </c>
     </row>
@@ -2290,7 +2264,7 @@
       <c r="G28" t="s">
         <v>44</v>
       </c>
-      <c r="H28" s="2">
+      <c r="H28" s="1">
         <v>46199</v>
       </c>
       <c r="I28" t="s">
@@ -2320,7 +2294,7 @@
       <c r="U28" t="s">
         <v>183</v>
       </c>
-      <c r="V28" s="2">
+      <c r="V28" s="1">
         <v>46199</v>
       </c>
     </row>
@@ -2346,7 +2320,7 @@
       <c r="G29" t="s">
         <v>44</v>
       </c>
-      <c r="H29" s="2">
+      <c r="H29" s="1">
         <v>46199</v>
       </c>
       <c r="I29" t="s">
@@ -2376,7 +2350,7 @@
       <c r="U29" t="s">
         <v>183</v>
       </c>
-      <c r="V29" s="2">
+      <c r="V29" s="1">
         <v>46199</v>
       </c>
     </row>
@@ -2402,7 +2376,7 @@
       <c r="G30" t="s">
         <v>44</v>
       </c>
-      <c r="H30" s="2">
+      <c r="H30" s="1">
         <v>46199</v>
       </c>
       <c r="I30" t="s">
@@ -2432,7 +2406,7 @@
       <c r="U30" t="s">
         <v>183</v>
       </c>
-      <c r="V30" s="2">
+      <c r="V30" s="1">
         <v>46199</v>
       </c>
     </row>
@@ -2458,7 +2432,7 @@
       <c r="G31" t="s">
         <v>44</v>
       </c>
-      <c r="H31" s="2">
+      <c r="H31" s="1">
         <v>46199</v>
       </c>
       <c r="I31" t="s">
@@ -2488,7 +2462,7 @@
       <c r="U31" t="s">
         <v>183</v>
       </c>
-      <c r="V31" s="2">
+      <c r="V31" s="1">
         <v>46199</v>
       </c>
     </row>
@@ -2535,7 +2509,7 @@
       <c r="U32" t="s">
         <v>183</v>
       </c>
-      <c r="V32" s="2">
+      <c r="V32" s="1">
         <v>46291</v>
       </c>
     </row>
@@ -2561,7 +2535,7 @@
       <c r="G33" t="s">
         <v>44</v>
       </c>
-      <c r="H33" s="2">
+      <c r="H33" s="1">
         <v>46191</v>
       </c>
       <c r="I33" t="s">
@@ -2591,7 +2565,7 @@
       <c r="U33" t="s">
         <v>183</v>
       </c>
-      <c r="V33" s="2">
+      <c r="V33" s="1">
         <v>46199</v>
       </c>
     </row>
@@ -2617,7 +2591,7 @@
       <c r="G34" t="s">
         <v>44</v>
       </c>
-      <c r="H34" s="2">
+      <c r="H34" s="1">
         <v>46119</v>
       </c>
       <c r="I34" t="s">
@@ -2644,7 +2618,7 @@
       <c r="U34" t="s">
         <v>183</v>
       </c>
-      <c r="V34" s="2">
+      <c r="V34" s="1">
         <v>46138</v>
       </c>
     </row>
@@ -2670,7 +2644,7 @@
       <c r="G35" t="s">
         <v>44</v>
       </c>
-      <c r="H35" s="2">
+      <c r="H35" s="1">
         <v>46213</v>
       </c>
       <c r="I35" t="s">
@@ -2697,7 +2671,7 @@
       <c r="U35" t="s">
         <v>28</v>
       </c>
-      <c r="V35" s="2">
+      <c r="V35" s="1">
         <v>46229</v>
       </c>
     </row>
@@ -2723,7 +2697,7 @@
       <c r="G36" t="s">
         <v>44</v>
       </c>
-      <c r="H36" s="2">
+      <c r="H36" s="1">
         <v>46175</v>
       </c>
       <c r="I36" t="s">
@@ -2750,7 +2724,7 @@
       <c r="U36" t="s">
         <v>28</v>
       </c>
-      <c r="V36" s="2">
+      <c r="V36" s="1">
         <v>46199</v>
       </c>
     </row>
@@ -2776,7 +2750,7 @@
       <c r="G37" t="s">
         <v>44</v>
       </c>
-      <c r="H37" s="2">
+      <c r="H37" s="1">
         <v>46213</v>
       </c>
       <c r="I37" t="s">
@@ -2803,7 +2777,7 @@
       <c r="U37" t="s">
         <v>28</v>
       </c>
-      <c r="V37" s="2">
+      <c r="V37" s="1">
         <v>46229</v>
       </c>
     </row>
@@ -2829,7 +2803,7 @@
       <c r="G38" t="s">
         <v>44</v>
       </c>
-      <c r="H38" s="2">
+      <c r="H38" s="1">
         <v>46199</v>
       </c>
       <c r="I38" t="s">
@@ -2856,7 +2830,7 @@
       <c r="U38" t="s">
         <v>28</v>
       </c>
-      <c r="V38" s="2">
+      <c r="V38" s="1">
         <v>46199</v>
       </c>
     </row>
@@ -2882,7 +2856,7 @@
       <c r="G39" t="s">
         <v>44</v>
       </c>
-      <c r="H39" s="2">
+      <c r="H39" s="1">
         <v>46199</v>
       </c>
       <c r="I39" t="s">
@@ -2909,7 +2883,7 @@
       <c r="U39" t="s">
         <v>28</v>
       </c>
-      <c r="V39" s="2">
+      <c r="V39" s="1">
         <v>46199</v>
       </c>
     </row>
@@ -2935,7 +2909,7 @@
       <c r="G40" t="s">
         <v>44</v>
       </c>
-      <c r="H40" s="2">
+      <c r="H40" s="1">
         <v>46204</v>
       </c>
       <c r="I40" t="s">
@@ -2962,7 +2936,7 @@
       <c r="U40" t="s">
         <v>28</v>
       </c>
-      <c r="V40" s="2">
+      <c r="V40" s="1">
         <v>46229</v>
       </c>
     </row>
@@ -2988,7 +2962,7 @@
       <c r="G41" t="s">
         <v>44</v>
       </c>
-      <c r="H41" s="2">
+      <c r="H41" s="1">
         <v>46244</v>
       </c>
       <c r="I41" t="s">
@@ -3015,7 +2989,7 @@
       <c r="U41" t="s">
         <v>28</v>
       </c>
-      <c r="V41" s="2">
+      <c r="V41" s="1">
         <v>46199</v>
       </c>
     </row>
@@ -3059,7 +3033,7 @@
       <c r="U42" t="s">
         <v>28</v>
       </c>
-      <c r="V42" s="2">
+      <c r="V42" s="1">
         <v>46260</v>
       </c>
     </row>
@@ -3085,7 +3059,7 @@
       <c r="G43" t="s">
         <v>44</v>
       </c>
-      <c r="H43" s="2">
+      <c r="H43" s="1">
         <v>46191</v>
       </c>
       <c r="I43" t="s">
@@ -3112,7 +3086,7 @@
       <c r="U43" t="s">
         <v>28</v>
       </c>
-      <c r="V43" s="2">
+      <c r="V43" s="1">
         <v>46199</v>
       </c>
     </row>
@@ -3138,7 +3112,7 @@
       <c r="G44" t="s">
         <v>44</v>
       </c>
-      <c r="H44" s="2">
+      <c r="H44" s="1">
         <v>46191</v>
       </c>
       <c r="I44" t="s">
@@ -3165,7 +3139,7 @@
       <c r="U44" t="s">
         <v>28</v>
       </c>
-      <c r="V44" s="2">
+      <c r="V44" s="1">
         <v>46199</v>
       </c>
     </row>
@@ -3191,7 +3165,7 @@
       <c r="G45" t="s">
         <v>44</v>
       </c>
-      <c r="H45" s="2">
+      <c r="H45" s="1">
         <v>46213</v>
       </c>
       <c r="I45" t="s">
@@ -3221,7 +3195,7 @@
       <c r="U45" t="s">
         <v>183</v>
       </c>
-      <c r="V45" s="2">
+      <c r="V45" s="1">
         <v>46229</v>
       </c>
     </row>
@@ -3247,7 +3221,7 @@
       <c r="G46" t="s">
         <v>44</v>
       </c>
-      <c r="H46" s="2">
+      <c r="H46" s="1">
         <v>46210</v>
       </c>
       <c r="I46" t="s">
@@ -3274,7 +3248,7 @@
       <c r="U46" t="s">
         <v>183</v>
       </c>
-      <c r="V46" s="2">
+      <c r="V46" s="1">
         <v>46229</v>
       </c>
     </row>
@@ -3318,7 +3292,7 @@
       <c r="U47" t="s">
         <v>28</v>
       </c>
-      <c r="V47" s="2">
+      <c r="V47" s="1">
         <v>46321</v>
       </c>
     </row>
@@ -3368,7 +3342,7 @@
       <c r="U48" t="s">
         <v>183</v>
       </c>
-      <c r="V48" s="2">
+      <c r="V48" s="1">
         <v>46291</v>
       </c>
     </row>
@@ -3394,7 +3368,7 @@
       <c r="G49" t="s">
         <v>44</v>
       </c>
-      <c r="H49" s="2">
+      <c r="H49" s="1">
         <v>46176</v>
       </c>
       <c r="I49" t="s">
@@ -3424,7 +3398,7 @@
       <c r="U49" t="s">
         <v>183</v>
       </c>
-      <c r="V49" s="2">
+      <c r="V49" s="1">
         <v>46199</v>
       </c>
     </row>
@@ -3447,7 +3421,7 @@
       <c r="G50" t="s">
         <v>44</v>
       </c>
-      <c r="H50" s="2">
+      <c r="H50" s="1">
         <v>46280</v>
       </c>
       <c r="I50" t="s">
@@ -3474,7 +3448,7 @@
       <c r="U50" t="s">
         <v>183</v>
       </c>
-      <c r="V50" s="2">
+      <c r="V50" s="1">
         <v>46260</v>
       </c>
     </row>
@@ -3524,7 +3498,7 @@
       <c r="U51" t="s">
         <v>183</v>
       </c>
-      <c r="V51" s="2">
+      <c r="V51" s="1">
         <v>46260</v>
       </c>
     </row>
@@ -3574,7 +3548,7 @@
       <c r="U52" t="s">
         <v>183</v>
       </c>
-      <c r="V52" s="2">
+      <c r="V52" s="1">
         <v>46291</v>
       </c>
     </row>
@@ -3621,7 +3595,7 @@
       <c r="U53" t="s">
         <v>183</v>
       </c>
-      <c r="V53" s="2">
+      <c r="V53" s="1">
         <v>46321</v>
       </c>
     </row>
@@ -3647,7 +3621,7 @@
       <c r="G54" t="s">
         <v>44</v>
       </c>
-      <c r="H54" s="2">
+      <c r="H54" s="1">
         <v>46227</v>
       </c>
       <c r="I54" t="s">
@@ -3674,7 +3648,7 @@
       <c r="U54" t="s">
         <v>183</v>
       </c>
-      <c r="V54" s="2">
+      <c r="V54" s="1">
         <v>46229</v>
       </c>
     </row>
@@ -3697,7 +3671,7 @@
       <c r="G55" t="s">
         <v>44</v>
       </c>
-      <c r="H55" s="2">
+      <c r="H55" s="1">
         <v>46280</v>
       </c>
       <c r="I55" t="s">
@@ -3724,7 +3698,7 @@
       <c r="U55" t="s">
         <v>183</v>
       </c>
-      <c r="V55" s="2">
+      <c r="V55" s="1">
         <v>46291</v>
       </c>
     </row>
@@ -3774,7 +3748,7 @@
       <c r="U56" t="s">
         <v>183</v>
       </c>
-      <c r="V56" s="2">
+      <c r="V56" s="1">
         <v>46352</v>
       </c>
     </row>
@@ -3824,7 +3798,7 @@
       <c r="U57" t="s">
         <v>183</v>
       </c>
-      <c r="V57" s="2">
+      <c r="V57" s="1">
         <v>46321</v>
       </c>
     </row>
@@ -3868,7 +3842,7 @@
       <c r="U58" t="s">
         <v>183</v>
       </c>
-      <c r="V58" s="2">
+      <c r="V58" s="1">
         <v>46321</v>
       </c>
     </row>
@@ -3912,7 +3886,7 @@
       <c r="U59" t="s">
         <v>183</v>
       </c>
-      <c r="V59" s="2">
+      <c r="V59" s="1">
         <v>46049</v>
       </c>
     </row>
@@ -4035,7 +4009,7 @@
       <c r="U62" t="s">
         <v>183</v>
       </c>
-      <c r="V62" s="2">
+      <c r="V62" s="1">
         <v>46107</v>
       </c>
     </row>
@@ -4076,7 +4050,7 @@
       <c r="U63" t="s">
         <v>183</v>
       </c>
-      <c r="V63" s="2">
+      <c r="V63" s="1">
         <v>46107</v>
       </c>
     </row>
@@ -4117,7 +4091,7 @@
       <c r="U64" t="s">
         <v>183</v>
       </c>
-      <c r="V64" s="2">
+      <c r="V64" s="1">
         <v>46107</v>
       </c>
     </row>
@@ -4158,7 +4132,7 @@
       <c r="U65" t="s">
         <v>183</v>
       </c>
-      <c r="V65" s="2">
+      <c r="V65" s="1">
         <v>46107</v>
       </c>
     </row>
@@ -4199,7 +4173,7 @@
       <c r="U66" t="s">
         <v>183</v>
       </c>
-      <c r="V66" s="2">
+      <c r="V66" s="1">
         <v>46107</v>
       </c>
     </row>
@@ -4240,7 +4214,7 @@
       <c r="U67" t="s">
         <v>183</v>
       </c>
-      <c r="V67" s="2">
+      <c r="V67" s="1">
         <v>46107</v>
       </c>
     </row>
@@ -4281,7 +4255,7 @@
       <c r="U68" t="s">
         <v>28</v>
       </c>
-      <c r="V68" s="2">
+      <c r="V68" s="1">
         <v>46168</v>
       </c>
     </row>
@@ -4325,7 +4299,7 @@
       <c r="U69" t="s">
         <v>28</v>
       </c>
-      <c r="V69" s="2">
+      <c r="V69" s="1">
         <v>46291</v>
       </c>
     </row>
@@ -4375,7 +4349,7 @@
       <c r="U70" t="s">
         <v>183</v>
       </c>
-      <c r="V70" s="2">
+      <c r="V70" s="1">
         <v>46229</v>
       </c>
     </row>
@@ -4416,7 +4390,7 @@
       <c r="U71" t="s">
         <v>28</v>
       </c>
-      <c r="V71" s="2">
+      <c r="V71" s="1">
         <v>46260</v>
       </c>
     </row>
@@ -4457,7 +4431,7 @@
       <c r="U72" t="s">
         <v>183</v>
       </c>
-      <c r="V72" s="2">
+      <c r="V72" s="1">
         <v>46291</v>
       </c>
     </row>
@@ -4498,7 +4472,7 @@
       <c r="U73" t="s">
         <v>183</v>
       </c>
-      <c r="V73" s="2">
+      <c r="V73" s="1">
         <v>46168</v>
       </c>
     </row>
@@ -4539,7 +4513,7 @@
       <c r="U74" t="s">
         <v>183</v>
       </c>
-      <c r="V74" s="2">
+      <c r="V74" s="1">
         <v>46291</v>
       </c>
     </row>
@@ -4580,7 +4554,7 @@
       <c r="U75" t="s">
         <v>183</v>
       </c>
-      <c r="V75" s="2">
+      <c r="V75" s="1">
         <v>46291</v>
       </c>
     </row>
@@ -4621,7 +4595,7 @@
       <c r="U76" t="s">
         <v>183</v>
       </c>
-      <c r="V76" s="2">
+      <c r="V76" s="1">
         <v>46291</v>
       </c>
     </row>
@@ -4665,7 +4639,7 @@
       <c r="U77" t="s">
         <v>28</v>
       </c>
-      <c r="V77" s="2">
+      <c r="V77" s="1">
         <v>46321</v>
       </c>
     </row>
@@ -4712,7 +4686,7 @@
       <c r="U78" t="s">
         <v>183</v>
       </c>
-      <c r="V78" s="2">
+      <c r="V78" s="1">
         <v>46381</v>
       </c>
     </row>
@@ -4759,7 +4733,7 @@
       <c r="U79" t="s">
         <v>183</v>
       </c>
-      <c r="V79" s="2">
+      <c r="V79" s="1">
         <v>46381</v>
       </c>
     </row>
@@ -4806,7 +4780,7 @@
       <c r="U80" t="s">
         <v>28</v>
       </c>
-      <c r="V80" s="2">
+      <c r="V80" s="1">
         <v>46381</v>
       </c>
     </row>
@@ -4853,7 +4827,7 @@
       <c r="U81" t="s">
         <v>28</v>
       </c>
-      <c r="V81" s="2">
+      <c r="V81" s="1">
         <v>46381</v>
       </c>
     </row>
@@ -4900,7 +4874,7 @@
       <c r="U82" t="s">
         <v>28</v>
       </c>
-      <c r="V82" s="2">
+      <c r="V82" s="1">
         <v>46382</v>
       </c>
     </row>
@@ -4941,7 +4915,7 @@
       <c r="U83" t="s">
         <v>28</v>
       </c>
-      <c r="V83" s="2">
+      <c r="V83" s="1">
         <v>46382</v>
       </c>
     </row>
@@ -4991,7 +4965,7 @@
       <c r="U84" t="s">
         <v>183</v>
       </c>
-      <c r="V84" s="2">
+      <c r="V84" s="1">
         <v>46382</v>
       </c>
     </row>
@@ -5032,7 +5006,7 @@
       <c r="U85" t="s">
         <v>28</v>
       </c>
-      <c r="V85" s="2">
+      <c r="V85" s="1">
         <v>46321</v>
       </c>
     </row>
@@ -5073,7 +5047,7 @@
       <c r="U86" t="s">
         <v>28</v>
       </c>
-      <c r="V86" s="2">
+      <c r="V86" s="1">
         <v>46382</v>
       </c>
     </row>
@@ -5205,7 +5179,7 @@
       <c r="U89" t="s">
         <v>28</v>
       </c>
-      <c r="V89" s="2">
+      <c r="V89" s="1">
         <v>46291</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Atualização automática: mta (21/09/2026 14:30)
</commit_message>
<xml_diff>
--- a/Projetos/02_Dados_Tratados/base_mta_tratada.xlsx
+++ b/Projetos/02_Dados_Tratados/base_mta_tratada.xlsx
@@ -575,8 +575,16 @@
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="YYYY-MM-DD HH:MM:SS"/>
   </numFmts>
-  <fonts count="1">
+  <fonts count="2">
     <font>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
       <sz val="11"/>
       <color theme="1"/>
       <name val="Calibri"/>
@@ -592,7 +600,7 @@
       <patternFill patternType="gray125"/>
     </fill>
   </fills>
-  <borders count="1">
+  <borders count="2">
     <border>
       <left/>
       <right/>
@@ -600,12 +608,30 @@
       <bottom/>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin">
+        <color auto="1"/>
+      </left>
+      <right style="thin">
+        <color auto="1"/>
+      </right>
+      <top style="thin">
+        <color auto="1"/>
+      </top>
+      <bottom style="thin">
+        <color auto="1"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="3">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
   </cellXfs>
   <cellStyles count="1">
@@ -905,70 +931,70 @@
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:22">
-      <c r="A1" t="s">
+      <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
-      <c r="B1" t="s">
+      <c r="B1" s="1" t="s">
         <v>1</v>
       </c>
-      <c r="C1" t="s">
+      <c r="C1" s="1" t="s">
         <v>2</v>
       </c>
-      <c r="D1" t="s">
+      <c r="D1" s="1" t="s">
         <v>3</v>
       </c>
-      <c r="E1" t="s">
+      <c r="E1" s="1" t="s">
         <v>4</v>
       </c>
-      <c r="F1" t="s">
+      <c r="F1" s="1" t="s">
         <v>5</v>
       </c>
-      <c r="G1" t="s">
+      <c r="G1" s="1" t="s">
         <v>6</v>
       </c>
-      <c r="H1" t="s">
+      <c r="H1" s="1" t="s">
         <v>7</v>
       </c>
-      <c r="I1" t="s">
+      <c r="I1" s="1" t="s">
         <v>8</v>
       </c>
-      <c r="J1" t="s">
+      <c r="J1" s="1" t="s">
         <v>9</v>
       </c>
-      <c r="K1" t="s">
+      <c r="K1" s="1" t="s">
         <v>10</v>
       </c>
-      <c r="L1" t="s">
+      <c r="L1" s="1" t="s">
         <v>11</v>
       </c>
-      <c r="M1" t="s">
+      <c r="M1" s="1" t="s">
         <v>12</v>
       </c>
-      <c r="N1" t="s">
+      <c r="N1" s="1" t="s">
         <v>13</v>
       </c>
-      <c r="O1" t="s">
+      <c r="O1" s="1" t="s">
         <v>14</v>
       </c>
-      <c r="P1" t="s">
+      <c r="P1" s="1" t="s">
         <v>15</v>
       </c>
-      <c r="Q1" t="s">
+      <c r="Q1" s="1" t="s">
         <v>16</v>
       </c>
-      <c r="R1" t="s">
+      <c r="R1" s="1" t="s">
         <v>17</v>
       </c>
-      <c r="S1" t="s">
+      <c r="S1" s="1" t="s">
         <v>18</v>
       </c>
-      <c r="T1" t="s">
+      <c r="T1" s="1" t="s">
         <v>19</v>
       </c>
-      <c r="U1" t="s">
+      <c r="U1" s="1" t="s">
         <v>20</v>
       </c>
-      <c r="V1" t="s">
+      <c r="V1" s="1" t="s">
         <v>21</v>
       </c>
     </row>
@@ -1021,7 +1047,7 @@
       <c r="U2" t="s">
         <v>183</v>
       </c>
-      <c r="V2" s="1">
+      <c r="V2" s="2">
         <v>46229</v>
       </c>
     </row>
@@ -1065,7 +1091,7 @@
       <c r="U3" t="s">
         <v>28</v>
       </c>
-      <c r="V3" s="1">
+      <c r="V3" s="2">
         <v>46291</v>
       </c>
     </row>
@@ -1112,7 +1138,7 @@
       <c r="U4" t="s">
         <v>28</v>
       </c>
-      <c r="V4" s="1">
+      <c r="V4" s="2">
         <v>46321</v>
       </c>
     </row>
@@ -1156,7 +1182,7 @@
       <c r="U5" t="s">
         <v>28</v>
       </c>
-      <c r="V5" s="1">
+      <c r="V5" s="2">
         <v>46321</v>
       </c>
     </row>
@@ -1203,7 +1229,7 @@
       <c r="U6" t="s">
         <v>28</v>
       </c>
-      <c r="V6" s="1">
+      <c r="V6" s="2">
         <v>46291</v>
       </c>
     </row>
@@ -1229,7 +1255,7 @@
       <c r="G7" t="s">
         <v>44</v>
       </c>
-      <c r="H7" s="1">
+      <c r="H7" s="2">
         <v>46121</v>
       </c>
       <c r="I7" t="s">
@@ -1256,7 +1282,7 @@
       <c r="U7" t="s">
         <v>28</v>
       </c>
-      <c r="V7" s="1">
+      <c r="V7" s="2">
         <v>46138</v>
       </c>
     </row>
@@ -1300,7 +1326,7 @@
       <c r="U8" t="s">
         <v>28</v>
       </c>
-      <c r="V8" s="1">
+      <c r="V8" s="2">
         <v>46291</v>
       </c>
     </row>
@@ -1344,7 +1370,7 @@
       <c r="U9" t="s">
         <v>28</v>
       </c>
-      <c r="V9" s="1">
+      <c r="V9" s="2">
         <v>46291</v>
       </c>
     </row>
@@ -1388,7 +1414,7 @@
       <c r="U10" t="s">
         <v>28</v>
       </c>
-      <c r="V10" s="1">
+      <c r="V10" s="2">
         <v>46291</v>
       </c>
     </row>
@@ -1432,7 +1458,7 @@
       <c r="U11" t="s">
         <v>28</v>
       </c>
-      <c r="V11" s="1">
+      <c r="V11" s="2">
         <v>46291</v>
       </c>
     </row>
@@ -1458,7 +1484,7 @@
       <c r="G12" t="s">
         <v>44</v>
       </c>
-      <c r="H12" s="1">
+      <c r="H12" s="2">
         <v>46079</v>
       </c>
       <c r="I12" t="s">
@@ -1488,7 +1514,7 @@
       <c r="U12" t="s">
         <v>183</v>
       </c>
-      <c r="V12" s="1">
+      <c r="V12" s="2">
         <v>46079</v>
       </c>
     </row>
@@ -1538,7 +1564,7 @@
       <c r="U13" t="s">
         <v>183</v>
       </c>
-      <c r="V13" s="1">
+      <c r="V13" s="2">
         <v>46352</v>
       </c>
     </row>
@@ -1588,7 +1614,7 @@
       <c r="U14" t="s">
         <v>183</v>
       </c>
-      <c r="V14" s="1">
+      <c r="V14" s="2">
         <v>46352</v>
       </c>
     </row>
@@ -1638,7 +1664,7 @@
       <c r="U15" t="s">
         <v>183</v>
       </c>
-      <c r="V15" s="1">
+      <c r="V15" s="2">
         <v>46352</v>
       </c>
     </row>
@@ -1688,7 +1714,7 @@
       <c r="U16" t="s">
         <v>183</v>
       </c>
-      <c r="V16" s="1">
+      <c r="V16" s="2">
         <v>46229</v>
       </c>
     </row>
@@ -1714,7 +1740,7 @@
       <c r="G17" t="s">
         <v>44</v>
       </c>
-      <c r="H17" s="1">
+      <c r="H17" s="2">
         <v>46098</v>
       </c>
       <c r="I17" t="s">
@@ -1744,7 +1770,7 @@
       <c r="U17" t="s">
         <v>183</v>
       </c>
-      <c r="V17" s="1">
+      <c r="V17" s="2">
         <v>46107</v>
       </c>
     </row>
@@ -1770,7 +1796,7 @@
       <c r="G18" t="s">
         <v>44</v>
       </c>
-      <c r="H18" s="1">
+      <c r="H18" s="2">
         <v>46076</v>
       </c>
       <c r="I18" t="s">
@@ -1797,7 +1823,7 @@
       <c r="U18" t="s">
         <v>28</v>
       </c>
-      <c r="V18" s="1">
+      <c r="V18" s="2">
         <v>46079</v>
       </c>
     </row>
@@ -1823,7 +1849,7 @@
       <c r="G19" t="s">
         <v>44</v>
       </c>
-      <c r="H19" s="1">
+      <c r="H19" s="2">
         <v>46076</v>
       </c>
       <c r="I19" t="s">
@@ -1850,7 +1876,7 @@
       <c r="U19" t="s">
         <v>28</v>
       </c>
-      <c r="V19" s="1">
+      <c r="V19" s="2">
         <v>46079</v>
       </c>
     </row>
@@ -1894,7 +1920,7 @@
       <c r="U20" t="s">
         <v>28</v>
       </c>
-      <c r="V20" s="1">
+      <c r="V20" s="2">
         <v>46321</v>
       </c>
     </row>
@@ -1938,7 +1964,7 @@
       <c r="U21" t="s">
         <v>28</v>
       </c>
-      <c r="V21" s="1">
+      <c r="V21" s="2">
         <v>46321</v>
       </c>
     </row>
@@ -1982,7 +2008,7 @@
       <c r="U22" t="s">
         <v>28</v>
       </c>
-      <c r="V22" s="1">
+      <c r="V22" s="2">
         <v>46321</v>
       </c>
     </row>
@@ -2026,7 +2052,7 @@
       <c r="U23" t="s">
         <v>28</v>
       </c>
-      <c r="V23" s="1">
+      <c r="V23" s="2">
         <v>46321</v>
       </c>
     </row>
@@ -2052,7 +2078,7 @@
       <c r="G24" t="s">
         <v>44</v>
       </c>
-      <c r="H24" s="1">
+      <c r="H24" s="2">
         <v>46119</v>
       </c>
       <c r="I24" t="s">
@@ -2082,7 +2108,7 @@
       <c r="U24" t="s">
         <v>183</v>
       </c>
-      <c r="V24" s="1">
+      <c r="V24" s="2">
         <v>46138</v>
       </c>
     </row>
@@ -2108,7 +2134,7 @@
       <c r="G25" t="s">
         <v>44</v>
       </c>
-      <c r="H25" s="1">
+      <c r="H25" s="2">
         <v>46121</v>
       </c>
       <c r="I25" t="s">
@@ -2135,7 +2161,7 @@
       <c r="U25" t="s">
         <v>28</v>
       </c>
-      <c r="V25" s="1">
+      <c r="V25" s="2">
         <v>46138</v>
       </c>
     </row>
@@ -2161,7 +2187,7 @@
       <c r="G26" t="s">
         <v>44</v>
       </c>
-      <c r="H26" s="1">
+      <c r="H26" s="2">
         <v>46076</v>
       </c>
       <c r="I26" t="s">
@@ -2188,7 +2214,7 @@
       <c r="U26" t="s">
         <v>28</v>
       </c>
-      <c r="V26" s="1">
+      <c r="V26" s="2">
         <v>46079</v>
       </c>
     </row>
@@ -2238,7 +2264,7 @@
       <c r="U27" t="s">
         <v>183</v>
       </c>
-      <c r="V27" s="1">
+      <c r="V27" s="2">
         <v>46291</v>
       </c>
     </row>
@@ -2264,7 +2290,7 @@
       <c r="G28" t="s">
         <v>44</v>
       </c>
-      <c r="H28" s="1">
+      <c r="H28" s="2">
         <v>46199</v>
       </c>
       <c r="I28" t="s">
@@ -2294,7 +2320,7 @@
       <c r="U28" t="s">
         <v>183</v>
       </c>
-      <c r="V28" s="1">
+      <c r="V28" s="2">
         <v>46199</v>
       </c>
     </row>
@@ -2320,7 +2346,7 @@
       <c r="G29" t="s">
         <v>44</v>
       </c>
-      <c r="H29" s="1">
+      <c r="H29" s="2">
         <v>46199</v>
       </c>
       <c r="I29" t="s">
@@ -2350,7 +2376,7 @@
       <c r="U29" t="s">
         <v>183</v>
       </c>
-      <c r="V29" s="1">
+      <c r="V29" s="2">
         <v>46199</v>
       </c>
     </row>
@@ -2376,7 +2402,7 @@
       <c r="G30" t="s">
         <v>44</v>
       </c>
-      <c r="H30" s="1">
+      <c r="H30" s="2">
         <v>46199</v>
       </c>
       <c r="I30" t="s">
@@ -2406,7 +2432,7 @@
       <c r="U30" t="s">
         <v>183</v>
       </c>
-      <c r="V30" s="1">
+      <c r="V30" s="2">
         <v>46199</v>
       </c>
     </row>
@@ -2432,7 +2458,7 @@
       <c r="G31" t="s">
         <v>44</v>
       </c>
-      <c r="H31" s="1">
+      <c r="H31" s="2">
         <v>46199</v>
       </c>
       <c r="I31" t="s">
@@ -2462,7 +2488,7 @@
       <c r="U31" t="s">
         <v>183</v>
       </c>
-      <c r="V31" s="1">
+      <c r="V31" s="2">
         <v>46199</v>
       </c>
     </row>
@@ -2509,7 +2535,7 @@
       <c r="U32" t="s">
         <v>183</v>
       </c>
-      <c r="V32" s="1">
+      <c r="V32" s="2">
         <v>46291</v>
       </c>
     </row>
@@ -2535,7 +2561,7 @@
       <c r="G33" t="s">
         <v>44</v>
       </c>
-      <c r="H33" s="1">
+      <c r="H33" s="2">
         <v>46191</v>
       </c>
       <c r="I33" t="s">
@@ -2565,7 +2591,7 @@
       <c r="U33" t="s">
         <v>183</v>
       </c>
-      <c r="V33" s="1">
+      <c r="V33" s="2">
         <v>46199</v>
       </c>
     </row>
@@ -2591,7 +2617,7 @@
       <c r="G34" t="s">
         <v>44</v>
       </c>
-      <c r="H34" s="1">
+      <c r="H34" s="2">
         <v>46119</v>
       </c>
       <c r="I34" t="s">
@@ -2618,7 +2644,7 @@
       <c r="U34" t="s">
         <v>183</v>
       </c>
-      <c r="V34" s="1">
+      <c r="V34" s="2">
         <v>46138</v>
       </c>
     </row>
@@ -2644,7 +2670,7 @@
       <c r="G35" t="s">
         <v>44</v>
       </c>
-      <c r="H35" s="1">
+      <c r="H35" s="2">
         <v>46213</v>
       </c>
       <c r="I35" t="s">
@@ -2671,7 +2697,7 @@
       <c r="U35" t="s">
         <v>28</v>
       </c>
-      <c r="V35" s="1">
+      <c r="V35" s="2">
         <v>46229</v>
       </c>
     </row>
@@ -2697,7 +2723,7 @@
       <c r="G36" t="s">
         <v>44</v>
       </c>
-      <c r="H36" s="1">
+      <c r="H36" s="2">
         <v>46175</v>
       </c>
       <c r="I36" t="s">
@@ -2724,7 +2750,7 @@
       <c r="U36" t="s">
         <v>28</v>
       </c>
-      <c r="V36" s="1">
+      <c r="V36" s="2">
         <v>46199</v>
       </c>
     </row>
@@ -2750,7 +2776,7 @@
       <c r="G37" t="s">
         <v>44</v>
       </c>
-      <c r="H37" s="1">
+      <c r="H37" s="2">
         <v>46213</v>
       </c>
       <c r="I37" t="s">
@@ -2777,7 +2803,7 @@
       <c r="U37" t="s">
         <v>28</v>
       </c>
-      <c r="V37" s="1">
+      <c r="V37" s="2">
         <v>46229</v>
       </c>
     </row>
@@ -2803,7 +2829,7 @@
       <c r="G38" t="s">
         <v>44</v>
       </c>
-      <c r="H38" s="1">
+      <c r="H38" s="2">
         <v>46199</v>
       </c>
       <c r="I38" t="s">
@@ -2830,7 +2856,7 @@
       <c r="U38" t="s">
         <v>28</v>
       </c>
-      <c r="V38" s="1">
+      <c r="V38" s="2">
         <v>46199</v>
       </c>
     </row>
@@ -2856,7 +2882,7 @@
       <c r="G39" t="s">
         <v>44</v>
       </c>
-      <c r="H39" s="1">
+      <c r="H39" s="2">
         <v>46199</v>
       </c>
       <c r="I39" t="s">
@@ -2883,7 +2909,7 @@
       <c r="U39" t="s">
         <v>28</v>
       </c>
-      <c r="V39" s="1">
+      <c r="V39" s="2">
         <v>46199</v>
       </c>
     </row>
@@ -2909,7 +2935,7 @@
       <c r="G40" t="s">
         <v>44</v>
       </c>
-      <c r="H40" s="1">
+      <c r="H40" s="2">
         <v>46204</v>
       </c>
       <c r="I40" t="s">
@@ -2936,7 +2962,7 @@
       <c r="U40" t="s">
         <v>28</v>
       </c>
-      <c r="V40" s="1">
+      <c r="V40" s="2">
         <v>46229</v>
       </c>
     </row>
@@ -2962,7 +2988,7 @@
       <c r="G41" t="s">
         <v>44</v>
       </c>
-      <c r="H41" s="1">
+      <c r="H41" s="2">
         <v>46244</v>
       </c>
       <c r="I41" t="s">
@@ -2989,7 +3015,7 @@
       <c r="U41" t="s">
         <v>28</v>
       </c>
-      <c r="V41" s="1">
+      <c r="V41" s="2">
         <v>46199</v>
       </c>
     </row>
@@ -3033,7 +3059,7 @@
       <c r="U42" t="s">
         <v>28</v>
       </c>
-      <c r="V42" s="1">
+      <c r="V42" s="2">
         <v>46260</v>
       </c>
     </row>
@@ -3059,7 +3085,7 @@
       <c r="G43" t="s">
         <v>44</v>
       </c>
-      <c r="H43" s="1">
+      <c r="H43" s="2">
         <v>46191</v>
       </c>
       <c r="I43" t="s">
@@ -3086,7 +3112,7 @@
       <c r="U43" t="s">
         <v>28</v>
       </c>
-      <c r="V43" s="1">
+      <c r="V43" s="2">
         <v>46199</v>
       </c>
     </row>
@@ -3112,7 +3138,7 @@
       <c r="G44" t="s">
         <v>44</v>
       </c>
-      <c r="H44" s="1">
+      <c r="H44" s="2">
         <v>46191</v>
       </c>
       <c r="I44" t="s">
@@ -3139,7 +3165,7 @@
       <c r="U44" t="s">
         <v>28</v>
       </c>
-      <c r="V44" s="1">
+      <c r="V44" s="2">
         <v>46199</v>
       </c>
     </row>
@@ -3165,7 +3191,7 @@
       <c r="G45" t="s">
         <v>44</v>
       </c>
-      <c r="H45" s="1">
+      <c r="H45" s="2">
         <v>46213</v>
       </c>
       <c r="I45" t="s">
@@ -3195,7 +3221,7 @@
       <c r="U45" t="s">
         <v>183</v>
       </c>
-      <c r="V45" s="1">
+      <c r="V45" s="2">
         <v>46229</v>
       </c>
     </row>
@@ -3221,7 +3247,7 @@
       <c r="G46" t="s">
         <v>44</v>
       </c>
-      <c r="H46" s="1">
+      <c r="H46" s="2">
         <v>46210</v>
       </c>
       <c r="I46" t="s">
@@ -3248,7 +3274,7 @@
       <c r="U46" t="s">
         <v>183</v>
       </c>
-      <c r="V46" s="1">
+      <c r="V46" s="2">
         <v>46229</v>
       </c>
     </row>
@@ -3292,7 +3318,7 @@
       <c r="U47" t="s">
         <v>28</v>
       </c>
-      <c r="V47" s="1">
+      <c r="V47" s="2">
         <v>46321</v>
       </c>
     </row>
@@ -3342,7 +3368,7 @@
       <c r="U48" t="s">
         <v>183</v>
       </c>
-      <c r="V48" s="1">
+      <c r="V48" s="2">
         <v>46291</v>
       </c>
     </row>
@@ -3368,7 +3394,7 @@
       <c r="G49" t="s">
         <v>44</v>
       </c>
-      <c r="H49" s="1">
+      <c r="H49" s="2">
         <v>46176</v>
       </c>
       <c r="I49" t="s">
@@ -3398,7 +3424,7 @@
       <c r="U49" t="s">
         <v>183</v>
       </c>
-      <c r="V49" s="1">
+      <c r="V49" s="2">
         <v>46199</v>
       </c>
     </row>
@@ -3421,7 +3447,7 @@
       <c r="G50" t="s">
         <v>44</v>
       </c>
-      <c r="H50" s="1">
+      <c r="H50" s="2">
         <v>46280</v>
       </c>
       <c r="I50" t="s">
@@ -3448,7 +3474,7 @@
       <c r="U50" t="s">
         <v>183</v>
       </c>
-      <c r="V50" s="1">
+      <c r="V50" s="2">
         <v>46260</v>
       </c>
     </row>
@@ -3498,7 +3524,7 @@
       <c r="U51" t="s">
         <v>183</v>
       </c>
-      <c r="V51" s="1">
+      <c r="V51" s="2">
         <v>46260</v>
       </c>
     </row>
@@ -3548,7 +3574,7 @@
       <c r="U52" t="s">
         <v>183</v>
       </c>
-      <c r="V52" s="1">
+      <c r="V52" s="2">
         <v>46291</v>
       </c>
     </row>
@@ -3595,7 +3621,7 @@
       <c r="U53" t="s">
         <v>183</v>
       </c>
-      <c r="V53" s="1">
+      <c r="V53" s="2">
         <v>46321</v>
       </c>
     </row>
@@ -3621,7 +3647,7 @@
       <c r="G54" t="s">
         <v>44</v>
       </c>
-      <c r="H54" s="1">
+      <c r="H54" s="2">
         <v>46227</v>
       </c>
       <c r="I54" t="s">
@@ -3648,7 +3674,7 @@
       <c r="U54" t="s">
         <v>183</v>
       </c>
-      <c r="V54" s="1">
+      <c r="V54" s="2">
         <v>46229</v>
       </c>
     </row>
@@ -3671,7 +3697,7 @@
       <c r="G55" t="s">
         <v>44</v>
       </c>
-      <c r="H55" s="1">
+      <c r="H55" s="2">
         <v>46280</v>
       </c>
       <c r="I55" t="s">
@@ -3698,7 +3724,7 @@
       <c r="U55" t="s">
         <v>183</v>
       </c>
-      <c r="V55" s="1">
+      <c r="V55" s="2">
         <v>46291</v>
       </c>
     </row>
@@ -3748,7 +3774,7 @@
       <c r="U56" t="s">
         <v>183</v>
       </c>
-      <c r="V56" s="1">
+      <c r="V56" s="2">
         <v>46352</v>
       </c>
     </row>
@@ -3798,7 +3824,7 @@
       <c r="U57" t="s">
         <v>183</v>
       </c>
-      <c r="V57" s="1">
+      <c r="V57" s="2">
         <v>46321</v>
       </c>
     </row>
@@ -3842,7 +3868,7 @@
       <c r="U58" t="s">
         <v>183</v>
       </c>
-      <c r="V58" s="1">
+      <c r="V58" s="2">
         <v>46321</v>
       </c>
     </row>
@@ -3886,7 +3912,7 @@
       <c r="U59" t="s">
         <v>183</v>
       </c>
-      <c r="V59" s="1">
+      <c r="V59" s="2">
         <v>46049</v>
       </c>
     </row>
@@ -4009,7 +4035,7 @@
       <c r="U62" t="s">
         <v>183</v>
       </c>
-      <c r="V62" s="1">
+      <c r="V62" s="2">
         <v>46107</v>
       </c>
     </row>
@@ -4050,7 +4076,7 @@
       <c r="U63" t="s">
         <v>183</v>
       </c>
-      <c r="V63" s="1">
+      <c r="V63" s="2">
         <v>46107</v>
       </c>
     </row>
@@ -4091,7 +4117,7 @@
       <c r="U64" t="s">
         <v>183</v>
       </c>
-      <c r="V64" s="1">
+      <c r="V64" s="2">
         <v>46107</v>
       </c>
     </row>
@@ -4132,7 +4158,7 @@
       <c r="U65" t="s">
         <v>183</v>
       </c>
-      <c r="V65" s="1">
+      <c r="V65" s="2">
         <v>46107</v>
       </c>
     </row>
@@ -4173,7 +4199,7 @@
       <c r="U66" t="s">
         <v>183</v>
       </c>
-      <c r="V66" s="1">
+      <c r="V66" s="2">
         <v>46107</v>
       </c>
     </row>
@@ -4214,7 +4240,7 @@
       <c r="U67" t="s">
         <v>183</v>
       </c>
-      <c r="V67" s="1">
+      <c r="V67" s="2">
         <v>46107</v>
       </c>
     </row>
@@ -4255,7 +4281,7 @@
       <c r="U68" t="s">
         <v>28</v>
       </c>
-      <c r="V68" s="1">
+      <c r="V68" s="2">
         <v>46168</v>
       </c>
     </row>
@@ -4299,7 +4325,7 @@
       <c r="U69" t="s">
         <v>28</v>
       </c>
-      <c r="V69" s="1">
+      <c r="V69" s="2">
         <v>46291</v>
       </c>
     </row>
@@ -4349,7 +4375,7 @@
       <c r="U70" t="s">
         <v>183</v>
       </c>
-      <c r="V70" s="1">
+      <c r="V70" s="2">
         <v>46229</v>
       </c>
     </row>
@@ -4390,7 +4416,7 @@
       <c r="U71" t="s">
         <v>28</v>
       </c>
-      <c r="V71" s="1">
+      <c r="V71" s="2">
         <v>46260</v>
       </c>
     </row>
@@ -4431,7 +4457,7 @@
       <c r="U72" t="s">
         <v>183</v>
       </c>
-      <c r="V72" s="1">
+      <c r="V72" s="2">
         <v>46291</v>
       </c>
     </row>
@@ -4472,7 +4498,7 @@
       <c r="U73" t="s">
         <v>183</v>
       </c>
-      <c r="V73" s="1">
+      <c r="V73" s="2">
         <v>46168</v>
       </c>
     </row>
@@ -4513,7 +4539,7 @@
       <c r="U74" t="s">
         <v>183</v>
       </c>
-      <c r="V74" s="1">
+      <c r="V74" s="2">
         <v>46291</v>
       </c>
     </row>
@@ -4554,7 +4580,7 @@
       <c r="U75" t="s">
         <v>183</v>
       </c>
-      <c r="V75" s="1">
+      <c r="V75" s="2">
         <v>46291</v>
       </c>
     </row>
@@ -4595,7 +4621,7 @@
       <c r="U76" t="s">
         <v>183</v>
       </c>
-      <c r="V76" s="1">
+      <c r="V76" s="2">
         <v>46291</v>
       </c>
     </row>
@@ -4639,7 +4665,7 @@
       <c r="U77" t="s">
         <v>28</v>
       </c>
-      <c r="V77" s="1">
+      <c r="V77" s="2">
         <v>46321</v>
       </c>
     </row>
@@ -4686,7 +4712,7 @@
       <c r="U78" t="s">
         <v>183</v>
       </c>
-      <c r="V78" s="1">
+      <c r="V78" s="2">
         <v>46381</v>
       </c>
     </row>
@@ -4733,7 +4759,7 @@
       <c r="U79" t="s">
         <v>183</v>
       </c>
-      <c r="V79" s="1">
+      <c r="V79" s="2">
         <v>46381</v>
       </c>
     </row>
@@ -4780,7 +4806,7 @@
       <c r="U80" t="s">
         <v>28</v>
       </c>
-      <c r="V80" s="1">
+      <c r="V80" s="2">
         <v>46381</v>
       </c>
     </row>
@@ -4827,7 +4853,7 @@
       <c r="U81" t="s">
         <v>28</v>
       </c>
-      <c r="V81" s="1">
+      <c r="V81" s="2">
         <v>46381</v>
       </c>
     </row>
@@ -4874,7 +4900,7 @@
       <c r="U82" t="s">
         <v>28</v>
       </c>
-      <c r="V82" s="1">
+      <c r="V82" s="2">
         <v>46382</v>
       </c>
     </row>
@@ -4915,7 +4941,7 @@
       <c r="U83" t="s">
         <v>28</v>
       </c>
-      <c r="V83" s="1">
+      <c r="V83" s="2">
         <v>46382</v>
       </c>
     </row>
@@ -4965,7 +4991,7 @@
       <c r="U84" t="s">
         <v>183</v>
       </c>
-      <c r="V84" s="1">
+      <c r="V84" s="2">
         <v>46382</v>
       </c>
     </row>
@@ -5006,7 +5032,7 @@
       <c r="U85" t="s">
         <v>28</v>
       </c>
-      <c r="V85" s="1">
+      <c r="V85" s="2">
         <v>46321</v>
       </c>
     </row>
@@ -5047,7 +5073,7 @@
       <c r="U86" t="s">
         <v>28</v>
       </c>
-      <c r="V86" s="1">
+      <c r="V86" s="2">
         <v>46382</v>
       </c>
     </row>
@@ -5179,7 +5205,7 @@
       <c r="U89" t="s">
         <v>28</v>
       </c>
-      <c r="V89" s="1">
+      <c r="V89" s="2">
         <v>46291</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Atualização automática: mta (22/09/2026 12:30)
</commit_message>
<xml_diff>
--- a/Projetos/02_Dados_Tratados/base_mta_tratada.xlsx
+++ b/Projetos/02_Dados_Tratados/base_mta_tratada.xlsx
@@ -14,7 +14,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1166" uniqueCount="184">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1188" uniqueCount="184">
   <si>
     <t>linha</t>
   </si>
@@ -520,6 +520,9 @@
     <t>Pagar avaliação dos cores</t>
   </si>
   <si>
+    <t>Aquisição material</t>
+  </si>
+  <si>
     <t>CABW</t>
   </si>
   <si>
@@ -545,9 +548,6 @@
   </si>
   <si>
     <t>D</t>
-  </si>
-  <si>
-    <t>B</t>
   </si>
   <si>
     <t>REQUISIÇÃO</t>
@@ -575,16 +575,8 @@
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="YYYY-MM-DD HH:MM:SS"/>
   </numFmts>
-  <fonts count="2">
+  <fonts count="1">
     <font>
-      <sz val="11"/>
-      <color theme="1"/>
-      <name val="Calibri"/>
-      <family val="2"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <b/>
       <sz val="11"/>
       <color theme="1"/>
       <name val="Calibri"/>
@@ -600,7 +592,7 @@
       <patternFill patternType="gray125"/>
     </fill>
   </fills>
-  <borders count="2">
+  <borders count="1">
     <border>
       <left/>
       <right/>
@@ -608,30 +600,12 @@
       <bottom/>
       <diagonal/>
     </border>
-    <border>
-      <left style="thin">
-        <color auto="1"/>
-      </left>
-      <right style="thin">
-        <color auto="1"/>
-      </right>
-      <top style="thin">
-        <color auto="1"/>
-      </top>
-      <bottom style="thin">
-        <color auto="1"/>
-      </bottom>
-      <diagonal/>
-    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="3">
+  <cellXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top"/>
-    </xf>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
   </cellXfs>
   <cellStyles count="1">
@@ -927,74 +901,74 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:V89"/>
+  <dimension ref="A1:V90"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:22">
-      <c r="A1" s="1" t="s">
+      <c r="A1" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="1" t="s">
+      <c r="B1" t="s">
         <v>1</v>
       </c>
-      <c r="C1" s="1" t="s">
+      <c r="C1" t="s">
         <v>2</v>
       </c>
-      <c r="D1" s="1" t="s">
+      <c r="D1" t="s">
         <v>3</v>
       </c>
-      <c r="E1" s="1" t="s">
+      <c r="E1" t="s">
         <v>4</v>
       </c>
-      <c r="F1" s="1" t="s">
+      <c r="F1" t="s">
         <v>5</v>
       </c>
-      <c r="G1" s="1" t="s">
+      <c r="G1" t="s">
         <v>6</v>
       </c>
-      <c r="H1" s="1" t="s">
+      <c r="H1" t="s">
         <v>7</v>
       </c>
-      <c r="I1" s="1" t="s">
+      <c r="I1" t="s">
         <v>8</v>
       </c>
-      <c r="J1" s="1" t="s">
+      <c r="J1" t="s">
         <v>9</v>
       </c>
-      <c r="K1" s="1" t="s">
+      <c r="K1" t="s">
         <v>10</v>
       </c>
-      <c r="L1" s="1" t="s">
+      <c r="L1" t="s">
         <v>11</v>
       </c>
-      <c r="M1" s="1" t="s">
+      <c r="M1" t="s">
         <v>12</v>
       </c>
-      <c r="N1" s="1" t="s">
+      <c r="N1" t="s">
         <v>13</v>
       </c>
-      <c r="O1" s="1" t="s">
+      <c r="O1" t="s">
         <v>14</v>
       </c>
-      <c r="P1" s="1" t="s">
+      <c r="P1" t="s">
         <v>15</v>
       </c>
-      <c r="Q1" s="1" t="s">
+      <c r="Q1" t="s">
         <v>16</v>
       </c>
-      <c r="R1" s="1" t="s">
+      <c r="R1" t="s">
         <v>17</v>
       </c>
-      <c r="S1" s="1" t="s">
+      <c r="S1" t="s">
         <v>18</v>
       </c>
-      <c r="T1" s="1" t="s">
+      <c r="T1" t="s">
         <v>19</v>
       </c>
-      <c r="U1" s="1" t="s">
+      <c r="U1" t="s">
         <v>20</v>
       </c>
-      <c r="V1" s="1" t="s">
+      <c r="V1" t="s">
         <v>21</v>
       </c>
     </row>
@@ -1032,14 +1006,17 @@
       <c r="O2" t="s">
         <v>101</v>
       </c>
+      <c r="P2">
+        <v>135000</v>
+      </c>
       <c r="Q2" t="s">
-        <v>168</v>
+        <v>169</v>
       </c>
       <c r="R2" t="s">
-        <v>171</v>
+        <v>172</v>
       </c>
       <c r="S2" t="s">
-        <v>174</v>
+        <v>175</v>
       </c>
       <c r="T2" t="s">
         <v>178</v>
@@ -1047,7 +1024,7 @@
       <c r="U2" t="s">
         <v>183</v>
       </c>
-      <c r="V2" s="2">
+      <c r="V2" s="1">
         <v>46229</v>
       </c>
     </row>
@@ -1062,7 +1039,7 @@
         <v>22</v>
       </c>
       <c r="D3" t="s">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="E3" t="s">
         <v>28</v>
@@ -1070,6 +1047,9 @@
       <c r="F3" t="s">
         <v>30</v>
       </c>
+      <c r="G3" t="s">
+        <v>43</v>
+      </c>
       <c r="N3" t="s">
         <v>82</v>
       </c>
@@ -1077,13 +1057,13 @@
         <v>102</v>
       </c>
       <c r="Q3" t="s">
-        <v>168</v>
+        <v>169</v>
       </c>
       <c r="R3" t="s">
-        <v>171</v>
+        <v>172</v>
       </c>
       <c r="S3" t="s">
-        <v>174</v>
+        <v>175</v>
       </c>
       <c r="T3" t="s">
         <v>178</v>
@@ -1091,7 +1071,7 @@
       <c r="U3" t="s">
         <v>28</v>
       </c>
-      <c r="V3" s="2">
+      <c r="V3" s="1">
         <v>46291</v>
       </c>
     </row>
@@ -1124,13 +1104,13 @@
         <v>103</v>
       </c>
       <c r="Q4" t="s">
-        <v>168</v>
+        <v>169</v>
       </c>
       <c r="R4" t="s">
-        <v>172</v>
+        <v>173</v>
       </c>
       <c r="S4" t="s">
-        <v>174</v>
+        <v>175</v>
       </c>
       <c r="T4" t="s">
         <v>178</v>
@@ -1138,7 +1118,7 @@
       <c r="U4" t="s">
         <v>28</v>
       </c>
-      <c r="V4" s="2">
+      <c r="V4" s="1">
         <v>46321</v>
       </c>
     </row>
@@ -1153,7 +1133,7 @@
         <v>22</v>
       </c>
       <c r="D5" t="s">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="E5" t="s">
         <v>28</v>
@@ -1161,6 +1141,9 @@
       <c r="F5" t="s">
         <v>30</v>
       </c>
+      <c r="G5" t="s">
+        <v>43</v>
+      </c>
       <c r="N5" t="s">
         <v>83</v>
       </c>
@@ -1168,13 +1151,13 @@
         <v>104</v>
       </c>
       <c r="Q5" t="s">
-        <v>168</v>
+        <v>169</v>
       </c>
       <c r="R5" t="s">
-        <v>172</v>
+        <v>173</v>
       </c>
       <c r="S5" t="s">
-        <v>174</v>
+        <v>175</v>
       </c>
       <c r="T5" t="s">
         <v>178</v>
@@ -1182,7 +1165,7 @@
       <c r="U5" t="s">
         <v>28</v>
       </c>
-      <c r="V5" s="2">
+      <c r="V5" s="1">
         <v>46321</v>
       </c>
     </row>
@@ -1197,7 +1180,7 @@
         <v>22</v>
       </c>
       <c r="D6" t="s">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="E6" t="s">
         <v>28</v>
@@ -1205,6 +1188,9 @@
       <c r="F6" t="s">
         <v>30</v>
       </c>
+      <c r="G6" t="s">
+        <v>43</v>
+      </c>
       <c r="L6" t="s">
         <v>81</v>
       </c>
@@ -1215,13 +1201,13 @@
         <v>105</v>
       </c>
       <c r="Q6" t="s">
-        <v>168</v>
+        <v>169</v>
       </c>
       <c r="R6" t="s">
-        <v>172</v>
+        <v>173</v>
       </c>
       <c r="S6" t="s">
-        <v>174</v>
+        <v>175</v>
       </c>
       <c r="T6" t="s">
         <v>178</v>
@@ -1229,7 +1215,7 @@
       <c r="U6" t="s">
         <v>28</v>
       </c>
-      <c r="V6" s="2">
+      <c r="V6" s="1">
         <v>46291</v>
       </c>
     </row>
@@ -1255,7 +1241,7 @@
       <c r="G7" t="s">
         <v>44</v>
       </c>
-      <c r="H7" s="2">
+      <c r="H7" s="1">
         <v>46121</v>
       </c>
       <c r="I7" t="s">
@@ -1267,14 +1253,17 @@
       <c r="O7" t="s">
         <v>106</v>
       </c>
+      <c r="P7">
+        <v>3799999.6</v>
+      </c>
       <c r="Q7" t="s">
-        <v>169</v>
+        <v>170</v>
       </c>
       <c r="R7" t="s">
-        <v>172</v>
+        <v>173</v>
       </c>
       <c r="S7" t="s">
-        <v>174</v>
+        <v>175</v>
       </c>
       <c r="T7" t="s">
         <v>179</v>
@@ -1282,7 +1271,7 @@
       <c r="U7" t="s">
         <v>28</v>
       </c>
-      <c r="V7" s="2">
+      <c r="V7" s="1">
         <v>46138</v>
       </c>
     </row>
@@ -1297,7 +1286,7 @@
         <v>22</v>
       </c>
       <c r="D8" t="s">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="E8" t="s">
         <v>28</v>
@@ -1305,6 +1294,9 @@
       <c r="F8" t="s">
         <v>30</v>
       </c>
+      <c r="G8" t="s">
+        <v>43</v>
+      </c>
       <c r="N8" t="s">
         <v>83</v>
       </c>
@@ -1312,13 +1304,13 @@
         <v>107</v>
       </c>
       <c r="Q8" t="s">
-        <v>168</v>
+        <v>169</v>
       </c>
       <c r="R8" t="s">
-        <v>172</v>
+        <v>173</v>
       </c>
       <c r="S8" t="s">
-        <v>174</v>
+        <v>175</v>
       </c>
       <c r="T8" t="s">
         <v>178</v>
@@ -1326,7 +1318,7 @@
       <c r="U8" t="s">
         <v>28</v>
       </c>
-      <c r="V8" s="2">
+      <c r="V8" s="1">
         <v>46291</v>
       </c>
     </row>
@@ -1355,14 +1347,17 @@
       <c r="O9" t="s">
         <v>108</v>
       </c>
+      <c r="P9">
+        <v>60000</v>
+      </c>
       <c r="Q9" t="s">
-        <v>168</v>
+        <v>169</v>
       </c>
       <c r="R9" t="s">
-        <v>172</v>
+        <v>173</v>
       </c>
       <c r="S9" t="s">
-        <v>174</v>
+        <v>175</v>
       </c>
       <c r="T9" t="s">
         <v>178</v>
@@ -1370,7 +1365,7 @@
       <c r="U9" t="s">
         <v>28</v>
       </c>
-      <c r="V9" s="2">
+      <c r="V9" s="1">
         <v>46291</v>
       </c>
     </row>
@@ -1385,7 +1380,7 @@
         <v>22</v>
       </c>
       <c r="D10" t="s">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="E10" t="s">
         <v>28</v>
@@ -1393,6 +1388,9 @@
       <c r="F10" t="s">
         <v>30</v>
       </c>
+      <c r="G10" t="s">
+        <v>43</v>
+      </c>
       <c r="N10" t="s">
         <v>84</v>
       </c>
@@ -1400,13 +1398,13 @@
         <v>109</v>
       </c>
       <c r="Q10" t="s">
-        <v>168</v>
+        <v>169</v>
       </c>
       <c r="R10" t="s">
-        <v>172</v>
+        <v>173</v>
       </c>
       <c r="S10" t="s">
-        <v>174</v>
+        <v>175</v>
       </c>
       <c r="T10" t="s">
         <v>178</v>
@@ -1414,7 +1412,7 @@
       <c r="U10" t="s">
         <v>28</v>
       </c>
-      <c r="V10" s="2">
+      <c r="V10" s="1">
         <v>46291</v>
       </c>
     </row>
@@ -1429,7 +1427,7 @@
         <v>22</v>
       </c>
       <c r="D11" t="s">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="E11" t="s">
         <v>28</v>
@@ -1437,6 +1435,9 @@
       <c r="F11" t="s">
         <v>30</v>
       </c>
+      <c r="G11" t="s">
+        <v>43</v>
+      </c>
       <c r="N11" t="s">
         <v>84</v>
       </c>
@@ -1444,13 +1445,13 @@
         <v>110</v>
       </c>
       <c r="Q11" t="s">
-        <v>168</v>
+        <v>169</v>
       </c>
       <c r="R11" t="s">
-        <v>172</v>
+        <v>173</v>
       </c>
       <c r="S11" t="s">
-        <v>174</v>
+        <v>175</v>
       </c>
       <c r="T11" t="s">
         <v>178</v>
@@ -1458,7 +1459,7 @@
       <c r="U11" t="s">
         <v>28</v>
       </c>
-      <c r="V11" s="2">
+      <c r="V11" s="1">
         <v>46291</v>
       </c>
     </row>
@@ -1484,7 +1485,7 @@
       <c r="G12" t="s">
         <v>44</v>
       </c>
-      <c r="H12" s="2">
+      <c r="H12" s="1">
         <v>46079</v>
       </c>
       <c r="I12" t="s">
@@ -1499,14 +1500,17 @@
       <c r="O12" t="s">
         <v>111</v>
       </c>
+      <c r="P12">
+        <v>1187433.02</v>
+      </c>
       <c r="Q12" t="s">
-        <v>168</v>
+        <v>169</v>
       </c>
       <c r="R12" t="s">
-        <v>171</v>
+        <v>172</v>
       </c>
       <c r="S12" t="s">
-        <v>174</v>
+        <v>175</v>
       </c>
       <c r="T12" t="s">
         <v>178</v>
@@ -1514,7 +1518,7 @@
       <c r="U12" t="s">
         <v>183</v>
       </c>
-      <c r="V12" s="2">
+      <c r="V12" s="1">
         <v>46079</v>
       </c>
     </row>
@@ -1549,14 +1553,17 @@
       <c r="O13" t="s">
         <v>112</v>
       </c>
+      <c r="P13">
+        <v>1000000</v>
+      </c>
       <c r="Q13" t="s">
-        <v>168</v>
+        <v>169</v>
       </c>
       <c r="R13" t="s">
-        <v>171</v>
+        <v>172</v>
       </c>
       <c r="S13" t="s">
-        <v>174</v>
+        <v>175</v>
       </c>
       <c r="T13" t="s">
         <v>178</v>
@@ -1564,7 +1571,7 @@
       <c r="U13" t="s">
         <v>183</v>
       </c>
-      <c r="V13" s="2">
+      <c r="V13" s="1">
         <v>46352</v>
       </c>
     </row>
@@ -1599,14 +1606,17 @@
       <c r="O14" t="s">
         <v>113</v>
       </c>
+      <c r="P14">
+        <v>1000000</v>
+      </c>
       <c r="Q14" t="s">
-        <v>168</v>
+        <v>169</v>
       </c>
       <c r="R14" t="s">
-        <v>171</v>
+        <v>172</v>
       </c>
       <c r="S14" t="s">
-        <v>174</v>
+        <v>175</v>
       </c>
       <c r="T14" t="s">
         <v>178</v>
@@ -1614,7 +1624,7 @@
       <c r="U14" t="s">
         <v>183</v>
       </c>
-      <c r="V14" s="2">
+      <c r="V14" s="1">
         <v>46352</v>
       </c>
     </row>
@@ -1649,14 +1659,17 @@
       <c r="O15" t="s">
         <v>114</v>
       </c>
+      <c r="P15">
+        <v>1000000</v>
+      </c>
       <c r="Q15" t="s">
-        <v>168</v>
+        <v>169</v>
       </c>
       <c r="R15" t="s">
-        <v>171</v>
+        <v>172</v>
       </c>
       <c r="S15" t="s">
-        <v>174</v>
+        <v>175</v>
       </c>
       <c r="T15" t="s">
         <v>178</v>
@@ -1664,7 +1677,7 @@
       <c r="U15" t="s">
         <v>183</v>
       </c>
-      <c r="V15" s="2">
+      <c r="V15" s="1">
         <v>46352</v>
       </c>
     </row>
@@ -1699,14 +1712,17 @@
       <c r="O16" t="s">
         <v>115</v>
       </c>
+      <c r="P16">
+        <v>100000</v>
+      </c>
       <c r="Q16" t="s">
-        <v>170</v>
+        <v>171</v>
       </c>
       <c r="R16" t="s">
-        <v>171</v>
+        <v>172</v>
       </c>
       <c r="S16" t="s">
-        <v>174</v>
+        <v>175</v>
       </c>
       <c r="T16" t="s">
         <v>178</v>
@@ -1714,7 +1730,7 @@
       <c r="U16" t="s">
         <v>183</v>
       </c>
-      <c r="V16" s="2">
+      <c r="V16" s="1">
         <v>46229</v>
       </c>
     </row>
@@ -1740,7 +1756,7 @@
       <c r="G17" t="s">
         <v>44</v>
       </c>
-      <c r="H17" s="2">
+      <c r="H17" s="1">
         <v>46098</v>
       </c>
       <c r="I17" t="s">
@@ -1755,14 +1771,17 @@
       <c r="O17" t="s">
         <v>116</v>
       </c>
+      <c r="P17">
+        <v>1770880.5</v>
+      </c>
       <c r="Q17" t="s">
-        <v>169</v>
+        <v>170</v>
       </c>
       <c r="R17" t="s">
-        <v>172</v>
+        <v>173</v>
       </c>
       <c r="S17" t="s">
-        <v>174</v>
+        <v>175</v>
       </c>
       <c r="T17" t="s">
         <v>180</v>
@@ -1770,7 +1789,7 @@
       <c r="U17" t="s">
         <v>183</v>
       </c>
-      <c r="V17" s="2">
+      <c r="V17" s="1">
         <v>46107</v>
       </c>
     </row>
@@ -1796,7 +1815,7 @@
       <c r="G18" t="s">
         <v>44</v>
       </c>
-      <c r="H18" s="2">
+      <c r="H18" s="1">
         <v>46076</v>
       </c>
       <c r="I18" t="s">
@@ -1808,14 +1827,17 @@
       <c r="O18" t="s">
         <v>117</v>
       </c>
+      <c r="P18">
+        <v>350000</v>
+      </c>
       <c r="Q18" t="s">
-        <v>169</v>
+        <v>170</v>
       </c>
       <c r="R18" t="s">
-        <v>171</v>
+        <v>172</v>
       </c>
       <c r="S18" t="s">
-        <v>174</v>
+        <v>175</v>
       </c>
       <c r="T18" t="s">
         <v>179</v>
@@ -1823,7 +1845,7 @@
       <c r="U18" t="s">
         <v>28</v>
       </c>
-      <c r="V18" s="2">
+      <c r="V18" s="1">
         <v>46079</v>
       </c>
     </row>
@@ -1849,7 +1871,7 @@
       <c r="G19" t="s">
         <v>44</v>
       </c>
-      <c r="H19" s="2">
+      <c r="H19" s="1">
         <v>46076</v>
       </c>
       <c r="I19" t="s">
@@ -1861,14 +1883,17 @@
       <c r="O19" t="s">
         <v>118</v>
       </c>
+      <c r="P19">
+        <v>350000</v>
+      </c>
       <c r="Q19" t="s">
-        <v>169</v>
+        <v>170</v>
       </c>
       <c r="R19" t="s">
-        <v>171</v>
+        <v>172</v>
       </c>
       <c r="S19" t="s">
-        <v>174</v>
+        <v>175</v>
       </c>
       <c r="T19" t="s">
         <v>179</v>
@@ -1876,7 +1901,7 @@
       <c r="U19" t="s">
         <v>28</v>
       </c>
-      <c r="V19" s="2">
+      <c r="V19" s="1">
         <v>46079</v>
       </c>
     </row>
@@ -1905,14 +1930,17 @@
       <c r="O20" t="s">
         <v>119</v>
       </c>
+      <c r="P20">
+        <v>1000000</v>
+      </c>
       <c r="Q20" t="s">
-        <v>169</v>
+        <v>170</v>
       </c>
       <c r="R20" t="s">
-        <v>171</v>
+        <v>172</v>
       </c>
       <c r="S20" t="s">
-        <v>174</v>
+        <v>175</v>
       </c>
       <c r="T20" t="s">
         <v>179</v>
@@ -1920,7 +1948,7 @@
       <c r="U20" t="s">
         <v>28</v>
       </c>
-      <c r="V20" s="2">
+      <c r="V20" s="1">
         <v>46321</v>
       </c>
     </row>
@@ -1935,7 +1963,7 @@
         <v>22</v>
       </c>
       <c r="D21" t="s">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="E21" t="s">
         <v>28</v>
@@ -1943,6 +1971,9 @@
       <c r="F21" t="s">
         <v>30</v>
       </c>
+      <c r="G21" t="s">
+        <v>43</v>
+      </c>
       <c r="N21" t="s">
         <v>82</v>
       </c>
@@ -1950,13 +1981,13 @@
         <v>120</v>
       </c>
       <c r="Q21" t="s">
-        <v>168</v>
+        <v>169</v>
       </c>
       <c r="R21" t="s">
-        <v>171</v>
+        <v>172</v>
       </c>
       <c r="S21" t="s">
-        <v>174</v>
+        <v>175</v>
       </c>
       <c r="T21" t="s">
         <v>178</v>
@@ -1964,7 +1995,7 @@
       <c r="U21" t="s">
         <v>28</v>
       </c>
-      <c r="V21" s="2">
+      <c r="V21" s="1">
         <v>46321</v>
       </c>
     </row>
@@ -1979,7 +2010,7 @@
         <v>22</v>
       </c>
       <c r="D22" t="s">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="E22" t="s">
         <v>28</v>
@@ -1987,6 +2018,9 @@
       <c r="F22" t="s">
         <v>30</v>
       </c>
+      <c r="G22" t="s">
+        <v>43</v>
+      </c>
       <c r="N22" t="s">
         <v>83</v>
       </c>
@@ -1994,13 +2028,13 @@
         <v>121</v>
       </c>
       <c r="Q22" t="s">
-        <v>168</v>
+        <v>169</v>
       </c>
       <c r="R22" t="s">
-        <v>172</v>
+        <v>173</v>
       </c>
       <c r="S22" t="s">
-        <v>174</v>
+        <v>175</v>
       </c>
       <c r="T22" t="s">
         <v>178</v>
@@ -2008,7 +2042,7 @@
       <c r="U22" t="s">
         <v>28</v>
       </c>
-      <c r="V22" s="2">
+      <c r="V22" s="1">
         <v>46321</v>
       </c>
     </row>
@@ -2023,7 +2057,7 @@
         <v>22</v>
       </c>
       <c r="D23" t="s">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="E23" t="s">
         <v>28</v>
@@ -2031,6 +2065,9 @@
       <c r="F23" t="s">
         <v>30</v>
       </c>
+      <c r="G23" t="s">
+        <v>43</v>
+      </c>
       <c r="N23" t="s">
         <v>83</v>
       </c>
@@ -2038,13 +2075,13 @@
         <v>122</v>
       </c>
       <c r="Q23" t="s">
-        <v>168</v>
+        <v>169</v>
       </c>
       <c r="R23" t="s">
-        <v>172</v>
+        <v>173</v>
       </c>
       <c r="S23" t="s">
-        <v>174</v>
+        <v>175</v>
       </c>
       <c r="T23" t="s">
         <v>178</v>
@@ -2052,7 +2089,7 @@
       <c r="U23" t="s">
         <v>28</v>
       </c>
-      <c r="V23" s="2">
+      <c r="V23" s="1">
         <v>46321</v>
       </c>
     </row>
@@ -2078,7 +2115,7 @@
       <c r="G24" t="s">
         <v>44</v>
       </c>
-      <c r="H24" s="2">
+      <c r="H24" s="1">
         <v>46119</v>
       </c>
       <c r="I24" t="s">
@@ -2093,14 +2130,17 @@
       <c r="O24" t="s">
         <v>123</v>
       </c>
+      <c r="P24">
+        <v>1704503</v>
+      </c>
       <c r="Q24" t="s">
-        <v>169</v>
+        <v>170</v>
       </c>
       <c r="R24" t="s">
-        <v>172</v>
+        <v>173</v>
       </c>
       <c r="S24" t="s">
-        <v>174</v>
+        <v>175</v>
       </c>
       <c r="T24" t="s">
         <v>180</v>
@@ -2108,7 +2148,7 @@
       <c r="U24" t="s">
         <v>183</v>
       </c>
-      <c r="V24" s="2">
+      <c r="V24" s="1">
         <v>46138</v>
       </c>
     </row>
@@ -2134,7 +2174,7 @@
       <c r="G25" t="s">
         <v>44</v>
       </c>
-      <c r="H25" s="2">
+      <c r="H25" s="1">
         <v>46121</v>
       </c>
       <c r="I25" t="s">
@@ -2146,14 +2186,17 @@
       <c r="O25" t="s">
         <v>124</v>
       </c>
+      <c r="P25">
+        <v>3799000</v>
+      </c>
       <c r="Q25" t="s">
-        <v>169</v>
+        <v>170</v>
       </c>
       <c r="R25" t="s">
-        <v>172</v>
+        <v>173</v>
       </c>
       <c r="S25" t="s">
-        <v>174</v>
+        <v>175</v>
       </c>
       <c r="T25" t="s">
         <v>179</v>
@@ -2161,7 +2204,7 @@
       <c r="U25" t="s">
         <v>28</v>
       </c>
-      <c r="V25" s="2">
+      <c r="V25" s="1">
         <v>46138</v>
       </c>
     </row>
@@ -2187,7 +2230,7 @@
       <c r="G26" t="s">
         <v>44</v>
       </c>
-      <c r="H26" s="2">
+      <c r="H26" s="1">
         <v>46076</v>
       </c>
       <c r="I26" t="s">
@@ -2199,14 +2242,17 @@
       <c r="O26" t="s">
         <v>124</v>
       </c>
+      <c r="P26">
+        <v>1000</v>
+      </c>
       <c r="Q26" t="s">
-        <v>169</v>
+        <v>170</v>
       </c>
       <c r="R26" t="s">
-        <v>171</v>
+        <v>172</v>
       </c>
       <c r="S26" t="s">
-        <v>174</v>
+        <v>175</v>
       </c>
       <c r="T26" t="s">
         <v>179</v>
@@ -2214,7 +2260,7 @@
       <c r="U26" t="s">
         <v>28</v>
       </c>
-      <c r="V26" s="2">
+      <c r="V26" s="1">
         <v>46079</v>
       </c>
     </row>
@@ -2249,14 +2295,17 @@
       <c r="O27" t="s">
         <v>125</v>
       </c>
+      <c r="P27">
+        <v>100000</v>
+      </c>
       <c r="Q27" t="s">
-        <v>170</v>
+        <v>171</v>
       </c>
       <c r="R27" t="s">
-        <v>171</v>
+        <v>172</v>
       </c>
       <c r="S27" t="s">
-        <v>174</v>
+        <v>175</v>
       </c>
       <c r="T27" t="s">
         <v>178</v>
@@ -2264,7 +2313,7 @@
       <c r="U27" t="s">
         <v>183</v>
       </c>
-      <c r="V27" s="2">
+      <c r="V27" s="1">
         <v>46291</v>
       </c>
     </row>
@@ -2290,7 +2339,7 @@
       <c r="G28" t="s">
         <v>44</v>
       </c>
-      <c r="H28" s="2">
+      <c r="H28" s="1">
         <v>46199</v>
       </c>
       <c r="I28" t="s">
@@ -2305,14 +2354,17 @@
       <c r="O28" t="s">
         <v>126</v>
       </c>
+      <c r="P28">
+        <v>150000</v>
+      </c>
       <c r="Q28" t="s">
-        <v>169</v>
+        <v>170</v>
       </c>
       <c r="R28" t="s">
-        <v>172</v>
+        <v>173</v>
       </c>
       <c r="S28" t="s">
-        <v>174</v>
+        <v>175</v>
       </c>
       <c r="T28" t="s">
         <v>179</v>
@@ -2320,7 +2372,7 @@
       <c r="U28" t="s">
         <v>183</v>
       </c>
-      <c r="V28" s="2">
+      <c r="V28" s="1">
         <v>46199</v>
       </c>
     </row>
@@ -2346,7 +2398,7 @@
       <c r="G29" t="s">
         <v>44</v>
       </c>
-      <c r="H29" s="2">
+      <c r="H29" s="1">
         <v>46199</v>
       </c>
       <c r="I29" t="s">
@@ -2361,14 +2413,17 @@
       <c r="O29" t="s">
         <v>127</v>
       </c>
+      <c r="P29">
+        <v>150000</v>
+      </c>
       <c r="Q29" t="s">
-        <v>169</v>
+        <v>170</v>
       </c>
       <c r="R29" t="s">
-        <v>172</v>
+        <v>173</v>
       </c>
       <c r="S29" t="s">
-        <v>174</v>
+        <v>175</v>
       </c>
       <c r="T29" t="s">
         <v>179</v>
@@ -2376,7 +2431,7 @@
       <c r="U29" t="s">
         <v>183</v>
       </c>
-      <c r="V29" s="2">
+      <c r="V29" s="1">
         <v>46199</v>
       </c>
     </row>
@@ -2402,7 +2457,7 @@
       <c r="G30" t="s">
         <v>44</v>
       </c>
-      <c r="H30" s="2">
+      <c r="H30" s="1">
         <v>46199</v>
       </c>
       <c r="I30" t="s">
@@ -2417,14 +2472,17 @@
       <c r="O30" t="s">
         <v>128</v>
       </c>
+      <c r="P30">
+        <v>18462.36</v>
+      </c>
       <c r="Q30" t="s">
-        <v>169</v>
+        <v>170</v>
       </c>
       <c r="R30" t="s">
-        <v>172</v>
+        <v>173</v>
       </c>
       <c r="S30" t="s">
-        <v>174</v>
+        <v>175</v>
       </c>
       <c r="T30" t="s">
         <v>179</v>
@@ -2432,7 +2490,7 @@
       <c r="U30" t="s">
         <v>183</v>
       </c>
-      <c r="V30" s="2">
+      <c r="V30" s="1">
         <v>46199</v>
       </c>
     </row>
@@ -2458,7 +2516,7 @@
       <c r="G31" t="s">
         <v>44</v>
       </c>
-      <c r="H31" s="2">
+      <c r="H31" s="1">
         <v>46199</v>
       </c>
       <c r="I31" t="s">
@@ -2473,14 +2531,17 @@
       <c r="O31" t="s">
         <v>128</v>
       </c>
+      <c r="P31">
+        <v>324166.14</v>
+      </c>
       <c r="Q31" t="s">
-        <v>169</v>
+        <v>170</v>
       </c>
       <c r="R31" t="s">
-        <v>172</v>
+        <v>173</v>
       </c>
       <c r="S31" t="s">
-        <v>174</v>
+        <v>175</v>
       </c>
       <c r="T31" t="s">
         <v>179</v>
@@ -2488,7 +2549,7 @@
       <c r="U31" t="s">
         <v>183</v>
       </c>
-      <c r="V31" s="2">
+      <c r="V31" s="1">
         <v>46199</v>
       </c>
     </row>
@@ -2520,14 +2581,17 @@
       <c r="O32" t="s">
         <v>129</v>
       </c>
+      <c r="P32">
+        <v>30000</v>
+      </c>
       <c r="Q32" t="s">
-        <v>169</v>
+        <v>170</v>
       </c>
       <c r="R32" t="s">
-        <v>172</v>
+        <v>173</v>
       </c>
       <c r="S32" t="s">
-        <v>174</v>
+        <v>175</v>
       </c>
       <c r="T32" t="s">
         <v>179</v>
@@ -2535,7 +2599,7 @@
       <c r="U32" t="s">
         <v>183</v>
       </c>
-      <c r="V32" s="2">
+      <c r="V32" s="1">
         <v>46291</v>
       </c>
     </row>
@@ -2561,7 +2625,7 @@
       <c r="G33" t="s">
         <v>44</v>
       </c>
-      <c r="H33" s="2">
+      <c r="H33" s="1">
         <v>46191</v>
       </c>
       <c r="I33" t="s">
@@ -2576,14 +2640,17 @@
       <c r="O33" t="s">
         <v>130</v>
       </c>
+      <c r="P33">
+        <v>1496713.48</v>
+      </c>
       <c r="Q33" t="s">
-        <v>169</v>
+        <v>170</v>
       </c>
       <c r="R33" t="s">
-        <v>172</v>
+        <v>173</v>
       </c>
       <c r="S33" t="s">
-        <v>174</v>
+        <v>175</v>
       </c>
       <c r="T33" t="s">
         <v>180</v>
@@ -2591,7 +2658,7 @@
       <c r="U33" t="s">
         <v>183</v>
       </c>
-      <c r="V33" s="2">
+      <c r="V33" s="1">
         <v>46199</v>
       </c>
     </row>
@@ -2617,7 +2684,7 @@
       <c r="G34" t="s">
         <v>44</v>
       </c>
-      <c r="H34" s="2">
+      <c r="H34" s="1">
         <v>46119</v>
       </c>
       <c r="I34" t="s">
@@ -2629,14 +2696,17 @@
       <c r="O34" t="s">
         <v>130</v>
       </c>
+      <c r="P34">
+        <v>207789.52</v>
+      </c>
       <c r="Q34" t="s">
-        <v>169</v>
+        <v>170</v>
       </c>
       <c r="R34" t="s">
-        <v>172</v>
+        <v>173</v>
       </c>
       <c r="S34" t="s">
-        <v>174</v>
+        <v>175</v>
       </c>
       <c r="T34" t="s">
         <v>180</v>
@@ -2644,7 +2714,7 @@
       <c r="U34" t="s">
         <v>183</v>
       </c>
-      <c r="V34" s="2">
+      <c r="V34" s="1">
         <v>46138</v>
       </c>
     </row>
@@ -2670,7 +2740,7 @@
       <c r="G35" t="s">
         <v>44</v>
       </c>
-      <c r="H35" s="2">
+      <c r="H35" s="1">
         <v>46213</v>
       </c>
       <c r="I35" t="s">
@@ -2682,14 +2752,17 @@
       <c r="O35" t="s">
         <v>131</v>
       </c>
+      <c r="P35">
+        <v>962290.8</v>
+      </c>
       <c r="Q35" t="s">
-        <v>169</v>
+        <v>170</v>
       </c>
       <c r="R35" t="s">
-        <v>171</v>
+        <v>172</v>
       </c>
       <c r="S35" t="s">
-        <v>174</v>
+        <v>175</v>
       </c>
       <c r="T35" t="s">
         <v>179</v>
@@ -2697,7 +2770,7 @@
       <c r="U35" t="s">
         <v>28</v>
       </c>
-      <c r="V35" s="2">
+      <c r="V35" s="1">
         <v>46229</v>
       </c>
     </row>
@@ -2723,7 +2796,7 @@
       <c r="G36" t="s">
         <v>44</v>
       </c>
-      <c r="H36" s="2">
+      <c r="H36" s="1">
         <v>46175</v>
       </c>
       <c r="I36" t="s">
@@ -2735,14 +2808,17 @@
       <c r="O36" t="s">
         <v>131</v>
       </c>
+      <c r="P36">
+        <v>798776.97</v>
+      </c>
       <c r="Q36" t="s">
-        <v>169</v>
+        <v>170</v>
       </c>
       <c r="R36" t="s">
-        <v>172</v>
+        <v>173</v>
       </c>
       <c r="S36" t="s">
-        <v>174</v>
+        <v>175</v>
       </c>
       <c r="T36" t="s">
         <v>179</v>
@@ -2750,7 +2826,7 @@
       <c r="U36" t="s">
         <v>28</v>
       </c>
-      <c r="V36" s="2">
+      <c r="V36" s="1">
         <v>46199</v>
       </c>
     </row>
@@ -2776,7 +2852,7 @@
       <c r="G37" t="s">
         <v>44</v>
       </c>
-      <c r="H37" s="2">
+      <c r="H37" s="1">
         <v>46213</v>
       </c>
       <c r="I37" t="s">
@@ -2788,14 +2864,17 @@
       <c r="O37" t="s">
         <v>131</v>
       </c>
+      <c r="P37">
+        <v>1530656.62</v>
+      </c>
       <c r="Q37" t="s">
-        <v>169</v>
+        <v>170</v>
       </c>
       <c r="R37" t="s">
-        <v>171</v>
+        <v>172</v>
       </c>
       <c r="S37" t="s">
-        <v>174</v>
+        <v>175</v>
       </c>
       <c r="T37" t="s">
         <v>179</v>
@@ -2803,7 +2882,7 @@
       <c r="U37" t="s">
         <v>28</v>
       </c>
-      <c r="V37" s="2">
+      <c r="V37" s="1">
         <v>46229</v>
       </c>
     </row>
@@ -2829,7 +2908,7 @@
       <c r="G38" t="s">
         <v>44</v>
       </c>
-      <c r="H38" s="2">
+      <c r="H38" s="1">
         <v>46199</v>
       </c>
       <c r="I38" t="s">
@@ -2841,14 +2920,17 @@
       <c r="O38" t="s">
         <v>131</v>
       </c>
+      <c r="P38">
+        <v>72958.08</v>
+      </c>
       <c r="Q38" t="s">
-        <v>169</v>
+        <v>170</v>
       </c>
       <c r="R38" t="s">
-        <v>171</v>
+        <v>172</v>
       </c>
       <c r="S38" t="s">
-        <v>174</v>
+        <v>175</v>
       </c>
       <c r="T38" t="s">
         <v>179</v>
@@ -2856,7 +2938,7 @@
       <c r="U38" t="s">
         <v>28</v>
       </c>
-      <c r="V38" s="2">
+      <c r="V38" s="1">
         <v>46199</v>
       </c>
     </row>
@@ -2882,7 +2964,7 @@
       <c r="G39" t="s">
         <v>44</v>
       </c>
-      <c r="H39" s="2">
+      <c r="H39" s="1">
         <v>46199</v>
       </c>
       <c r="I39" t="s">
@@ -2894,14 +2976,17 @@
       <c r="O39" t="s">
         <v>131</v>
       </c>
+      <c r="P39">
+        <v>8916</v>
+      </c>
       <c r="Q39" t="s">
-        <v>169</v>
+        <v>170</v>
       </c>
       <c r="R39" t="s">
-        <v>171</v>
+        <v>172</v>
       </c>
       <c r="S39" t="s">
-        <v>174</v>
+        <v>175</v>
       </c>
       <c r="T39" t="s">
         <v>179</v>
@@ -2909,7 +2994,7 @@
       <c r="U39" t="s">
         <v>28</v>
       </c>
-      <c r="V39" s="2">
+      <c r="V39" s="1">
         <v>46199</v>
       </c>
     </row>
@@ -2935,7 +3020,7 @@
       <c r="G40" t="s">
         <v>44</v>
       </c>
-      <c r="H40" s="2">
+      <c r="H40" s="1">
         <v>46204</v>
       </c>
       <c r="I40" t="s">
@@ -2947,14 +3032,17 @@
       <c r="O40" t="s">
         <v>131</v>
       </c>
+      <c r="P40">
+        <v>425178.5</v>
+      </c>
       <c r="Q40" t="s">
-        <v>169</v>
+        <v>170</v>
       </c>
       <c r="R40" t="s">
-        <v>171</v>
+        <v>172</v>
       </c>
       <c r="S40" t="s">
-        <v>174</v>
+        <v>175</v>
       </c>
       <c r="T40" t="s">
         <v>179</v>
@@ -2962,7 +3050,7 @@
       <c r="U40" t="s">
         <v>28</v>
       </c>
-      <c r="V40" s="2">
+      <c r="V40" s="1">
         <v>46229</v>
       </c>
     </row>
@@ -2988,7 +3076,7 @@
       <c r="G41" t="s">
         <v>44</v>
       </c>
-      <c r="H41" s="2">
+      <c r="H41" s="1">
         <v>46244</v>
       </c>
       <c r="I41" t="s">
@@ -3000,14 +3088,17 @@
       <c r="O41" t="s">
         <v>131</v>
       </c>
+      <c r="P41">
+        <v>1223.03</v>
+      </c>
       <c r="Q41" t="s">
-        <v>169</v>
+        <v>170</v>
       </c>
       <c r="R41" t="s">
-        <v>171</v>
+        <v>172</v>
       </c>
       <c r="S41" t="s">
-        <v>174</v>
+        <v>175</v>
       </c>
       <c r="T41" t="s">
         <v>179</v>
@@ -3015,7 +3106,7 @@
       <c r="U41" t="s">
         <v>28</v>
       </c>
-      <c r="V41" s="2">
+      <c r="V41" s="1">
         <v>46199</v>
       </c>
     </row>
@@ -3045,13 +3136,13 @@
         <v>132</v>
       </c>
       <c r="Q42" t="s">
-        <v>169</v>
+        <v>170</v>
       </c>
       <c r="R42" t="s">
-        <v>171</v>
+        <v>172</v>
       </c>
       <c r="S42" t="s">
-        <v>175</v>
+        <v>176</v>
       </c>
       <c r="T42" t="s">
         <v>179</v>
@@ -3059,7 +3150,7 @@
       <c r="U42" t="s">
         <v>28</v>
       </c>
-      <c r="V42" s="2">
+      <c r="V42" s="1">
         <v>46260</v>
       </c>
     </row>
@@ -3085,7 +3176,7 @@
       <c r="G43" t="s">
         <v>44</v>
       </c>
-      <c r="H43" s="2">
+      <c r="H43" s="1">
         <v>46191</v>
       </c>
       <c r="I43" t="s">
@@ -3097,14 +3188,17 @@
       <c r="O43" t="s">
         <v>133</v>
       </c>
+      <c r="P43">
+        <v>400000</v>
+      </c>
       <c r="Q43" t="s">
-        <v>169</v>
+        <v>170</v>
       </c>
       <c r="R43" t="s">
-        <v>171</v>
+        <v>172</v>
       </c>
       <c r="S43" t="s">
-        <v>174</v>
+        <v>175</v>
       </c>
       <c r="T43" t="s">
         <v>179</v>
@@ -3112,7 +3206,7 @@
       <c r="U43" t="s">
         <v>28</v>
       </c>
-      <c r="V43" s="2">
+      <c r="V43" s="1">
         <v>46199</v>
       </c>
     </row>
@@ -3138,7 +3232,7 @@
       <c r="G44" t="s">
         <v>44</v>
       </c>
-      <c r="H44" s="2">
+      <c r="H44" s="1">
         <v>46191</v>
       </c>
       <c r="I44" t="s">
@@ -3150,14 +3244,17 @@
       <c r="O44" t="s">
         <v>134</v>
       </c>
+      <c r="P44">
+        <v>400000</v>
+      </c>
       <c r="Q44" t="s">
-        <v>169</v>
+        <v>170</v>
       </c>
       <c r="R44" t="s">
-        <v>171</v>
+        <v>172</v>
       </c>
       <c r="S44" t="s">
-        <v>174</v>
+        <v>175</v>
       </c>
       <c r="T44" t="s">
         <v>179</v>
@@ -3165,7 +3262,7 @@
       <c r="U44" t="s">
         <v>28</v>
       </c>
-      <c r="V44" s="2">
+      <c r="V44" s="1">
         <v>46199</v>
       </c>
     </row>
@@ -3191,7 +3288,7 @@
       <c r="G45" t="s">
         <v>44</v>
       </c>
-      <c r="H45" s="2">
+      <c r="H45" s="1">
         <v>46213</v>
       </c>
       <c r="I45" t="s">
@@ -3206,14 +3303,17 @@
       <c r="O45" t="s">
         <v>135</v>
       </c>
+      <c r="P45">
+        <v>173846.38</v>
+      </c>
       <c r="Q45" t="s">
-        <v>169</v>
+        <v>170</v>
       </c>
       <c r="R45" t="s">
-        <v>172</v>
+        <v>173</v>
       </c>
       <c r="S45" t="s">
-        <v>174</v>
+        <v>175</v>
       </c>
       <c r="T45" t="s">
         <v>180</v>
@@ -3221,7 +3321,7 @@
       <c r="U45" t="s">
         <v>183</v>
       </c>
-      <c r="V45" s="2">
+      <c r="V45" s="1">
         <v>46229</v>
       </c>
     </row>
@@ -3247,7 +3347,7 @@
       <c r="G46" t="s">
         <v>44</v>
       </c>
-      <c r="H46" s="2">
+      <c r="H46" s="1">
         <v>46210</v>
       </c>
       <c r="I46" t="s">
@@ -3259,14 +3359,17 @@
       <c r="O46" t="s">
         <v>135</v>
       </c>
+      <c r="P46">
+        <v>1530656.62</v>
+      </c>
       <c r="Q46" t="s">
-        <v>169</v>
+        <v>170</v>
       </c>
       <c r="R46" t="s">
-        <v>172</v>
+        <v>173</v>
       </c>
       <c r="S46" t="s">
-        <v>174</v>
+        <v>175</v>
       </c>
       <c r="T46" t="s">
         <v>180</v>
@@ -3274,7 +3377,7 @@
       <c r="U46" t="s">
         <v>183</v>
       </c>
-      <c r="V46" s="2">
+      <c r="V46" s="1">
         <v>46229</v>
       </c>
     </row>
@@ -3303,14 +3406,17 @@
       <c r="O47" t="s">
         <v>136</v>
       </c>
+      <c r="P47">
+        <v>1000000</v>
+      </c>
       <c r="Q47" t="s">
-        <v>169</v>
+        <v>170</v>
       </c>
       <c r="R47" t="s">
-        <v>171</v>
+        <v>172</v>
       </c>
       <c r="S47" t="s">
-        <v>174</v>
+        <v>175</v>
       </c>
       <c r="T47" t="s">
         <v>179</v>
@@ -3318,7 +3424,7 @@
       <c r="U47" t="s">
         <v>28</v>
       </c>
-      <c r="V47" s="2">
+      <c r="V47" s="1">
         <v>46321</v>
       </c>
     </row>
@@ -3353,14 +3459,17 @@
       <c r="O48" t="s">
         <v>137</v>
       </c>
+      <c r="P48">
+        <v>958040</v>
+      </c>
       <c r="Q48" t="s">
-        <v>168</v>
+        <v>169</v>
       </c>
       <c r="R48" t="s">
-        <v>171</v>
+        <v>172</v>
       </c>
       <c r="S48" t="s">
-        <v>174</v>
+        <v>175</v>
       </c>
       <c r="T48" t="s">
         <v>178</v>
@@ -3368,7 +3477,7 @@
       <c r="U48" t="s">
         <v>183</v>
       </c>
-      <c r="V48" s="2">
+      <c r="V48" s="1">
         <v>46291</v>
       </c>
     </row>
@@ -3394,7 +3503,7 @@
       <c r="G49" t="s">
         <v>44</v>
       </c>
-      <c r="H49" s="2">
+      <c r="H49" s="1">
         <v>46176</v>
       </c>
       <c r="I49" t="s">
@@ -3409,14 +3518,17 @@
       <c r="O49" t="s">
         <v>137</v>
       </c>
+      <c r="P49">
+        <v>41730.64</v>
+      </c>
       <c r="Q49" t="s">
-        <v>168</v>
+        <v>169</v>
       </c>
       <c r="R49" t="s">
-        <v>173</v>
+        <v>174</v>
       </c>
       <c r="S49" t="s">
-        <v>174</v>
+        <v>175</v>
       </c>
       <c r="T49" t="s">
         <v>178</v>
@@ -3424,7 +3536,7 @@
       <c r="U49" t="s">
         <v>183</v>
       </c>
-      <c r="V49" s="2">
+      <c r="V49" s="1">
         <v>46199</v>
       </c>
     </row>
@@ -3447,7 +3559,7 @@
       <c r="G50" t="s">
         <v>44</v>
       </c>
-      <c r="H50" s="2">
+      <c r="H50" s="1">
         <v>46280</v>
       </c>
       <c r="I50" t="s">
@@ -3459,14 +3571,17 @@
       <c r="O50" t="s">
         <v>138</v>
       </c>
+      <c r="P50">
+        <v>859536.0699999999</v>
+      </c>
       <c r="Q50" t="s">
-        <v>169</v>
+        <v>170</v>
       </c>
       <c r="R50" t="s">
-        <v>172</v>
+        <v>173</v>
       </c>
       <c r="S50" t="s">
-        <v>174</v>
+        <v>175</v>
       </c>
       <c r="T50" t="s">
         <v>180</v>
@@ -3474,7 +3589,7 @@
       <c r="U50" t="s">
         <v>183</v>
       </c>
-      <c r="V50" s="2">
+      <c r="V50" s="1">
         <v>46260</v>
       </c>
     </row>
@@ -3509,14 +3624,17 @@
       <c r="O51" t="s">
         <v>138</v>
       </c>
+      <c r="P51">
+        <v>608623.25</v>
+      </c>
       <c r="Q51" t="s">
-        <v>169</v>
+        <v>170</v>
       </c>
       <c r="R51" t="s">
-        <v>172</v>
+        <v>173</v>
       </c>
       <c r="S51" t="s">
-        <v>174</v>
+        <v>175</v>
       </c>
       <c r="T51" t="s">
         <v>180</v>
@@ -3524,7 +3642,7 @@
       <c r="U51" t="s">
         <v>183</v>
       </c>
-      <c r="V51" s="2">
+      <c r="V51" s="1">
         <v>46260</v>
       </c>
     </row>
@@ -3559,14 +3677,17 @@
       <c r="O52" t="s">
         <v>139</v>
       </c>
+      <c r="P52">
+        <v>559040.0699999999</v>
+      </c>
       <c r="Q52" t="s">
-        <v>169</v>
+        <v>170</v>
       </c>
       <c r="R52" t="s">
-        <v>172</v>
+        <v>173</v>
       </c>
       <c r="S52" t="s">
-        <v>174</v>
+        <v>175</v>
       </c>
       <c r="T52" t="s">
         <v>180</v>
@@ -3574,7 +3695,7 @@
       <c r="U52" t="s">
         <v>183</v>
       </c>
-      <c r="V52" s="2">
+      <c r="V52" s="1">
         <v>46291</v>
       </c>
     </row>
@@ -3606,14 +3727,17 @@
       <c r="O53" t="s">
         <v>140</v>
       </c>
+      <c r="P53">
+        <v>1704503</v>
+      </c>
       <c r="Q53" t="s">
-        <v>169</v>
+        <v>170</v>
       </c>
       <c r="R53" t="s">
-        <v>172</v>
+        <v>173</v>
       </c>
       <c r="S53" t="s">
-        <v>174</v>
+        <v>175</v>
       </c>
       <c r="T53" t="s">
         <v>180</v>
@@ -3621,7 +3745,7 @@
       <c r="U53" t="s">
         <v>183</v>
       </c>
-      <c r="V53" s="2">
+      <c r="V53" s="1">
         <v>46321</v>
       </c>
     </row>
@@ -3647,7 +3771,7 @@
       <c r="G54" t="s">
         <v>44</v>
       </c>
-      <c r="H54" s="2">
+      <c r="H54" s="1">
         <v>46227</v>
       </c>
       <c r="I54" t="s">
@@ -3659,14 +3783,17 @@
       <c r="O54" t="s">
         <v>138</v>
       </c>
+      <c r="P54">
+        <v>236343.68</v>
+      </c>
       <c r="Q54" t="s">
-        <v>169</v>
+        <v>170</v>
       </c>
       <c r="R54" t="s">
-        <v>172</v>
+        <v>173</v>
       </c>
       <c r="S54" t="s">
-        <v>174</v>
+        <v>175</v>
       </c>
       <c r="T54" t="s">
         <v>180</v>
@@ -3674,7 +3801,7 @@
       <c r="U54" t="s">
         <v>183</v>
       </c>
-      <c r="V54" s="2">
+      <c r="V54" s="1">
         <v>46229</v>
       </c>
     </row>
@@ -3697,7 +3824,7 @@
       <c r="G55" t="s">
         <v>44</v>
       </c>
-      <c r="H55" s="2">
+      <c r="H55" s="1">
         <v>46280</v>
       </c>
       <c r="I55" t="s">
@@ -3709,14 +3836,17 @@
       <c r="O55" t="s">
         <v>139</v>
       </c>
+      <c r="P55">
+        <v>1145462.93</v>
+      </c>
       <c r="Q55" t="s">
-        <v>169</v>
+        <v>170</v>
       </c>
       <c r="R55" t="s">
-        <v>172</v>
+        <v>173</v>
       </c>
       <c r="S55" t="s">
-        <v>174</v>
+        <v>175</v>
       </c>
       <c r="T55" t="s">
         <v>180</v>
@@ -3724,7 +3854,7 @@
       <c r="U55" t="s">
         <v>183</v>
       </c>
-      <c r="V55" s="2">
+      <c r="V55" s="1">
         <v>46291</v>
       </c>
     </row>
@@ -3759,14 +3889,17 @@
       <c r="O56" t="s">
         <v>141</v>
       </c>
+      <c r="P56">
+        <v>1295422.28</v>
+      </c>
       <c r="Q56" t="s">
-        <v>169</v>
+        <v>170</v>
       </c>
       <c r="R56" t="s">
-        <v>172</v>
+        <v>173</v>
       </c>
       <c r="S56" t="s">
-        <v>174</v>
+        <v>175</v>
       </c>
       <c r="T56" t="s">
         <v>180</v>
@@ -3774,7 +3907,7 @@
       <c r="U56" t="s">
         <v>183</v>
       </c>
-      <c r="V56" s="2">
+      <c r="V56" s="1">
         <v>46352</v>
       </c>
     </row>
@@ -3809,14 +3942,17 @@
       <c r="O57" t="s">
         <v>142</v>
       </c>
+      <c r="P57">
+        <v>1962977.67</v>
+      </c>
       <c r="Q57" t="s">
-        <v>169</v>
+        <v>170</v>
       </c>
       <c r="R57" t="s">
-        <v>172</v>
+        <v>173</v>
       </c>
       <c r="S57" t="s">
-        <v>176</v>
+        <v>177</v>
       </c>
       <c r="T57" t="s">
         <v>181</v>
@@ -3824,7 +3960,7 @@
       <c r="U57" t="s">
         <v>183</v>
       </c>
-      <c r="V57" s="2">
+      <c r="V57" s="1">
         <v>46321</v>
       </c>
     </row>
@@ -3853,14 +3989,17 @@
       <c r="O58" t="s">
         <v>142</v>
       </c>
+      <c r="P58">
+        <v>2497091</v>
+      </c>
       <c r="Q58" t="s">
-        <v>169</v>
+        <v>170</v>
       </c>
       <c r="R58" t="s">
-        <v>172</v>
+        <v>173</v>
       </c>
       <c r="S58" t="s">
-        <v>176</v>
+        <v>177</v>
       </c>
       <c r="T58" t="s">
         <v>181</v>
@@ -3868,7 +4007,7 @@
       <c r="U58" t="s">
         <v>183</v>
       </c>
-      <c r="V58" s="2">
+      <c r="V58" s="1">
         <v>46321</v>
       </c>
     </row>
@@ -3898,13 +4037,13 @@
         <v>143</v>
       </c>
       <c r="Q59" t="s">
-        <v>169</v>
+        <v>170</v>
       </c>
       <c r="R59" t="s">
-        <v>172</v>
+        <v>173</v>
       </c>
       <c r="S59" t="s">
-        <v>176</v>
+        <v>177</v>
       </c>
       <c r="T59" t="s">
         <v>181</v>
@@ -3912,7 +4051,7 @@
       <c r="U59" t="s">
         <v>183</v>
       </c>
-      <c r="V59" s="2">
+      <c r="V59" s="1">
         <v>46049</v>
       </c>
     </row>
@@ -3942,13 +4081,13 @@
         <v>144</v>
       </c>
       <c r="Q60" t="s">
-        <v>169</v>
+        <v>170</v>
       </c>
       <c r="R60" t="s">
-        <v>172</v>
+        <v>173</v>
       </c>
       <c r="S60" t="s">
-        <v>176</v>
+        <v>177</v>
       </c>
       <c r="T60" t="s">
         <v>181</v>
@@ -3983,13 +4122,13 @@
         <v>145</v>
       </c>
       <c r="Q61" t="s">
-        <v>169</v>
+        <v>170</v>
       </c>
       <c r="R61" t="s">
-        <v>172</v>
+        <v>173</v>
       </c>
       <c r="S61" t="s">
-        <v>176</v>
+        <v>177</v>
       </c>
       <c r="T61" t="s">
         <v>181</v>
@@ -4020,14 +4159,17 @@
       <c r="O62" t="s">
         <v>146</v>
       </c>
+      <c r="P62">
+        <v>9389.959999999999</v>
+      </c>
       <c r="Q62" t="s">
-        <v>168</v>
+        <v>169</v>
       </c>
       <c r="R62" t="s">
-        <v>173</v>
+        <v>174</v>
       </c>
       <c r="S62" t="s">
-        <v>175</v>
+        <v>176</v>
       </c>
       <c r="T62" t="s">
         <v>178</v>
@@ -4035,7 +4177,7 @@
       <c r="U62" t="s">
         <v>183</v>
       </c>
-      <c r="V62" s="2">
+      <c r="V62" s="1">
         <v>46107</v>
       </c>
     </row>
@@ -4061,14 +4203,17 @@
       <c r="O63" t="s">
         <v>147</v>
       </c>
+      <c r="P63">
+        <v>7204.82</v>
+      </c>
       <c r="Q63" t="s">
-        <v>168</v>
+        <v>169</v>
       </c>
       <c r="R63" t="s">
-        <v>173</v>
+        <v>174</v>
       </c>
       <c r="S63" t="s">
-        <v>175</v>
+        <v>176</v>
       </c>
       <c r="T63" t="s">
         <v>178</v>
@@ -4076,7 +4221,7 @@
       <c r="U63" t="s">
         <v>183</v>
       </c>
-      <c r="V63" s="2">
+      <c r="V63" s="1">
         <v>46107</v>
       </c>
     </row>
@@ -4102,14 +4247,17 @@
       <c r="O64" t="s">
         <v>148</v>
       </c>
+      <c r="P64">
+        <v>4227.84</v>
+      </c>
       <c r="Q64" t="s">
-        <v>168</v>
+        <v>169</v>
       </c>
       <c r="R64" t="s">
-        <v>173</v>
+        <v>174</v>
       </c>
       <c r="S64" t="s">
-        <v>175</v>
+        <v>176</v>
       </c>
       <c r="T64" t="s">
         <v>178</v>
@@ -4117,7 +4265,7 @@
       <c r="U64" t="s">
         <v>183</v>
       </c>
-      <c r="V64" s="2">
+      <c r="V64" s="1">
         <v>46107</v>
       </c>
     </row>
@@ -4143,14 +4291,17 @@
       <c r="O65" t="s">
         <v>149</v>
       </c>
+      <c r="P65">
+        <v>4064.54</v>
+      </c>
       <c r="Q65" t="s">
-        <v>169</v>
+        <v>170</v>
       </c>
       <c r="R65" t="s">
-        <v>173</v>
+        <v>174</v>
       </c>
       <c r="S65" t="s">
-        <v>175</v>
+        <v>176</v>
       </c>
       <c r="T65" t="s">
         <v>178</v>
@@ -4158,7 +4309,7 @@
       <c r="U65" t="s">
         <v>183</v>
       </c>
-      <c r="V65" s="2">
+      <c r="V65" s="1">
         <v>46107</v>
       </c>
     </row>
@@ -4184,14 +4335,17 @@
       <c r="O66" t="s">
         <v>148</v>
       </c>
+      <c r="P66">
+        <v>3662.66</v>
+      </c>
       <c r="Q66" t="s">
-        <v>168</v>
+        <v>169</v>
       </c>
       <c r="R66" t="s">
-        <v>173</v>
+        <v>174</v>
       </c>
       <c r="S66" t="s">
-        <v>175</v>
+        <v>176</v>
       </c>
       <c r="T66" t="s">
         <v>178</v>
@@ -4199,7 +4353,7 @@
       <c r="U66" t="s">
         <v>183</v>
       </c>
-      <c r="V66" s="2">
+      <c r="V66" s="1">
         <v>46107</v>
       </c>
     </row>
@@ -4225,14 +4379,17 @@
       <c r="O67" t="s">
         <v>150</v>
       </c>
+      <c r="P67">
+        <v>1163.64</v>
+      </c>
       <c r="Q67" t="s">
-        <v>170</v>
+        <v>171</v>
       </c>
       <c r="R67" t="s">
-        <v>173</v>
+        <v>174</v>
       </c>
       <c r="S67" t="s">
-        <v>175</v>
+        <v>176</v>
       </c>
       <c r="T67" t="s">
         <v>178</v>
@@ -4240,7 +4397,7 @@
       <c r="U67" t="s">
         <v>183</v>
       </c>
-      <c r="V67" s="2">
+      <c r="V67" s="1">
         <v>46107</v>
       </c>
     </row>
@@ -4266,14 +4423,17 @@
       <c r="O68" t="s">
         <v>151</v>
       </c>
+      <c r="P68">
+        <v>120000</v>
+      </c>
       <c r="Q68" t="s">
-        <v>168</v>
+        <v>169</v>
       </c>
       <c r="R68" t="s">
-        <v>172</v>
+        <v>173</v>
       </c>
       <c r="S68" t="s">
-        <v>175</v>
+        <v>176</v>
       </c>
       <c r="T68" t="s">
         <v>178</v>
@@ -4281,7 +4441,7 @@
       <c r="U68" t="s">
         <v>28</v>
       </c>
-      <c r="V68" s="2">
+      <c r="V68" s="1">
         <v>46168</v>
       </c>
     </row>
@@ -4296,7 +4456,7 @@
         <v>22</v>
       </c>
       <c r="D69" t="s">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="E69" t="s">
         <v>28</v>
@@ -4304,6 +4464,9 @@
       <c r="F69" t="s">
         <v>30</v>
       </c>
+      <c r="G69" t="s">
+        <v>43</v>
+      </c>
       <c r="N69" t="s">
         <v>82</v>
       </c>
@@ -4311,13 +4474,13 @@
         <v>152</v>
       </c>
       <c r="Q69" t="s">
-        <v>168</v>
+        <v>169</v>
       </c>
       <c r="R69" t="s">
-        <v>171</v>
+        <v>172</v>
       </c>
       <c r="S69" t="s">
-        <v>174</v>
+        <v>175</v>
       </c>
       <c r="T69" t="s">
         <v>178</v>
@@ -4325,7 +4488,7 @@
       <c r="U69" t="s">
         <v>28</v>
       </c>
-      <c r="V69" s="2">
+      <c r="V69" s="1">
         <v>46291</v>
       </c>
     </row>
@@ -4360,14 +4523,17 @@
       <c r="O70" t="s">
         <v>153</v>
       </c>
+      <c r="P70">
+        <v>100000</v>
+      </c>
       <c r="Q70" t="s">
-        <v>170</v>
+        <v>171</v>
       </c>
       <c r="R70" t="s">
-        <v>171</v>
+        <v>172</v>
       </c>
       <c r="S70" t="s">
-        <v>174</v>
+        <v>175</v>
       </c>
       <c r="T70" t="s">
         <v>178</v>
@@ -4375,7 +4541,7 @@
       <c r="U70" t="s">
         <v>183</v>
       </c>
-      <c r="V70" s="2">
+      <c r="V70" s="1">
         <v>46229</v>
       </c>
     </row>
@@ -4401,14 +4567,17 @@
       <c r="O71" t="s">
         <v>154</v>
       </c>
+      <c r="P71">
+        <v>80000</v>
+      </c>
       <c r="Q71" t="s">
-        <v>168</v>
+        <v>169</v>
       </c>
       <c r="R71" t="s">
-        <v>172</v>
+        <v>173</v>
       </c>
       <c r="S71" t="s">
-        <v>175</v>
+        <v>176</v>
       </c>
       <c r="T71" t="s">
         <v>178</v>
@@ -4416,7 +4585,7 @@
       <c r="U71" t="s">
         <v>28</v>
       </c>
-      <c r="V71" s="2">
+      <c r="V71" s="1">
         <v>46260</v>
       </c>
     </row>
@@ -4442,14 +4611,17 @@
       <c r="O72" t="s">
         <v>155</v>
       </c>
+      <c r="P72">
+        <v>835000</v>
+      </c>
       <c r="Q72" t="s">
-        <v>168</v>
+        <v>169</v>
       </c>
       <c r="R72" t="s">
-        <v>171</v>
+        <v>172</v>
       </c>
       <c r="S72" t="s">
-        <v>175</v>
+        <v>176</v>
       </c>
       <c r="T72" t="s">
         <v>178</v>
@@ -4457,7 +4629,7 @@
       <c r="U72" t="s">
         <v>183</v>
       </c>
-      <c r="V72" s="2">
+      <c r="V72" s="1">
         <v>46291</v>
       </c>
     </row>
@@ -4483,14 +4655,17 @@
       <c r="O73" t="s">
         <v>155</v>
       </c>
+      <c r="P73">
+        <v>165000</v>
+      </c>
       <c r="Q73" t="s">
-        <v>168</v>
+        <v>169</v>
       </c>
       <c r="R73" t="s">
-        <v>171</v>
+        <v>172</v>
       </c>
       <c r="S73" t="s">
-        <v>175</v>
+        <v>176</v>
       </c>
       <c r="T73" t="s">
         <v>178</v>
@@ -4498,7 +4673,7 @@
       <c r="U73" t="s">
         <v>183</v>
       </c>
-      <c r="V73" s="2">
+      <c r="V73" s="1">
         <v>46168</v>
       </c>
     </row>
@@ -4524,14 +4699,17 @@
       <c r="O74" t="s">
         <v>156</v>
       </c>
+      <c r="P74">
+        <v>1000000</v>
+      </c>
       <c r="Q74" t="s">
-        <v>168</v>
+        <v>169</v>
       </c>
       <c r="R74" t="s">
-        <v>171</v>
+        <v>172</v>
       </c>
       <c r="S74" t="s">
-        <v>175</v>
+        <v>176</v>
       </c>
       <c r="T74" t="s">
         <v>178</v>
@@ -4539,7 +4717,7 @@
       <c r="U74" t="s">
         <v>183</v>
       </c>
-      <c r="V74" s="2">
+      <c r="V74" s="1">
         <v>46291</v>
       </c>
     </row>
@@ -4565,14 +4743,17 @@
       <c r="O75" t="s">
         <v>157</v>
       </c>
+      <c r="P75">
+        <v>1000000</v>
+      </c>
       <c r="Q75" t="s">
-        <v>168</v>
+        <v>169</v>
       </c>
       <c r="R75" t="s">
-        <v>171</v>
+        <v>172</v>
       </c>
       <c r="S75" t="s">
-        <v>175</v>
+        <v>176</v>
       </c>
       <c r="T75" t="s">
         <v>178</v>
@@ -4580,7 +4761,7 @@
       <c r="U75" t="s">
         <v>183</v>
       </c>
-      <c r="V75" s="2">
+      <c r="V75" s="1">
         <v>46291</v>
       </c>
     </row>
@@ -4606,14 +4787,17 @@
       <c r="O76" t="s">
         <v>158</v>
       </c>
+      <c r="P76">
+        <v>100000</v>
+      </c>
       <c r="Q76" t="s">
-        <v>170</v>
+        <v>171</v>
       </c>
       <c r="R76" t="s">
-        <v>171</v>
+        <v>172</v>
       </c>
       <c r="S76" t="s">
-        <v>175</v>
+        <v>176</v>
       </c>
       <c r="T76" t="s">
         <v>178</v>
@@ -4621,7 +4805,7 @@
       <c r="U76" t="s">
         <v>183</v>
       </c>
-      <c r="V76" s="2">
+      <c r="V76" s="1">
         <v>46291</v>
       </c>
     </row>
@@ -4650,14 +4834,17 @@
       <c r="O77" t="s">
         <v>159</v>
       </c>
+      <c r="P77">
+        <v>1000000</v>
+      </c>
       <c r="Q77" t="s">
-        <v>169</v>
+        <v>170</v>
       </c>
       <c r="R77" t="s">
-        <v>171</v>
+        <v>172</v>
       </c>
       <c r="S77" t="s">
-        <v>174</v>
+        <v>175</v>
       </c>
       <c r="T77" t="s">
         <v>179</v>
@@ -4665,7 +4852,7 @@
       <c r="U77" t="s">
         <v>28</v>
       </c>
-      <c r="V77" s="2">
+      <c r="V77" s="1">
         <v>46321</v>
       </c>
     </row>
@@ -4697,11 +4884,14 @@
       <c r="O78" t="s">
         <v>160</v>
       </c>
+      <c r="P78">
+        <v>1704503</v>
+      </c>
       <c r="Q78" t="s">
-        <v>169</v>
+        <v>170</v>
       </c>
       <c r="R78" t="s">
-        <v>172</v>
+        <v>173</v>
       </c>
       <c r="S78" t="s">
         <v>42</v>
@@ -4712,7 +4902,7 @@
       <c r="U78" t="s">
         <v>183</v>
       </c>
-      <c r="V78" s="2">
+      <c r="V78" s="1">
         <v>46381</v>
       </c>
     </row>
@@ -4744,11 +4934,14 @@
       <c r="O79" t="s">
         <v>161</v>
       </c>
+      <c r="P79">
+        <v>1638125.5</v>
+      </c>
       <c r="Q79" t="s">
-        <v>169</v>
+        <v>170</v>
       </c>
       <c r="R79" t="s">
-        <v>172</v>
+        <v>173</v>
       </c>
       <c r="S79" t="s">
         <v>42</v>
@@ -4759,7 +4952,7 @@
       <c r="U79" t="s">
         <v>183</v>
       </c>
-      <c r="V79" s="2">
+      <c r="V79" s="1">
         <v>46381</v>
       </c>
     </row>
@@ -4791,11 +4984,14 @@
       <c r="O80" t="s">
         <v>162</v>
       </c>
+      <c r="P80">
+        <v>3800000</v>
+      </c>
       <c r="Q80" t="s">
-        <v>169</v>
+        <v>170</v>
       </c>
       <c r="R80" t="s">
-        <v>172</v>
+        <v>173</v>
       </c>
       <c r="S80" t="s">
         <v>42</v>
@@ -4806,7 +5002,7 @@
       <c r="U80" t="s">
         <v>28</v>
       </c>
-      <c r="V80" s="2">
+      <c r="V80" s="1">
         <v>46381</v>
       </c>
     </row>
@@ -4838,11 +5034,14 @@
       <c r="O81" t="s">
         <v>163</v>
       </c>
+      <c r="P81">
+        <v>3800000</v>
+      </c>
       <c r="Q81" t="s">
-        <v>169</v>
+        <v>170</v>
       </c>
       <c r="R81" t="s">
-        <v>172</v>
+        <v>173</v>
       </c>
       <c r="S81" t="s">
         <v>42</v>
@@ -4853,7 +5052,7 @@
       <c r="U81" t="s">
         <v>28</v>
       </c>
-      <c r="V81" s="2">
+      <c r="V81" s="1">
         <v>46381</v>
       </c>
     </row>
@@ -4885,14 +5084,17 @@
       <c r="O82" t="s">
         <v>164</v>
       </c>
+      <c r="P82">
+        <v>3800000</v>
+      </c>
       <c r="Q82" t="s">
-        <v>169</v>
+        <v>170</v>
       </c>
       <c r="R82" t="s">
-        <v>172</v>
+        <v>173</v>
       </c>
       <c r="S82" t="s">
-        <v>175</v>
+        <v>176</v>
       </c>
       <c r="T82" t="s">
         <v>179</v>
@@ -4900,7 +5102,7 @@
       <c r="U82" t="s">
         <v>28</v>
       </c>
-      <c r="V82" s="2">
+      <c r="V82" s="1">
         <v>46382</v>
       </c>
     </row>
@@ -4926,14 +5128,17 @@
       <c r="O83" t="s">
         <v>99</v>
       </c>
+      <c r="P83">
+        <v>4394700</v>
+      </c>
       <c r="Q83" t="s">
-        <v>168</v>
+        <v>169</v>
       </c>
       <c r="R83" t="s">
-        <v>171</v>
+        <v>172</v>
       </c>
       <c r="S83" t="s">
-        <v>175</v>
+        <v>176</v>
       </c>
       <c r="T83" t="s">
         <v>179</v>
@@ -4941,7 +5146,7 @@
       <c r="U83" t="s">
         <v>28</v>
       </c>
-      <c r="V83" s="2">
+      <c r="V83" s="1">
         <v>46382</v>
       </c>
     </row>
@@ -4976,14 +5181,17 @@
       <c r="O84" t="s">
         <v>165</v>
       </c>
+      <c r="P84">
+        <v>528395.9300000001</v>
+      </c>
       <c r="Q84" t="s">
-        <v>169</v>
+        <v>170</v>
       </c>
       <c r="R84" t="s">
-        <v>172</v>
+        <v>173</v>
       </c>
       <c r="S84" t="s">
-        <v>174</v>
+        <v>175</v>
       </c>
       <c r="T84" t="s">
         <v>180</v>
@@ -4991,7 +5199,7 @@
       <c r="U84" t="s">
         <v>183</v>
       </c>
-      <c r="V84" s="2">
+      <c r="V84" s="1">
         <v>46382</v>
       </c>
     </row>
@@ -5006,10 +5214,13 @@
         <v>22</v>
       </c>
       <c r="D85" t="s">
-        <v>27</v>
+        <v>24</v>
       </c>
       <c r="E85" t="s">
-        <v>29</v>
+        <v>28</v>
+      </c>
+      <c r="F85" t="s">
+        <v>30</v>
       </c>
       <c r="N85" t="s">
         <v>89</v>
@@ -5017,14 +5228,17 @@
       <c r="O85" t="s">
         <v>166</v>
       </c>
+      <c r="P85">
+        <v>1000000</v>
+      </c>
       <c r="Q85" t="s">
-        <v>169</v>
+        <v>170</v>
       </c>
       <c r="R85" t="s">
-        <v>171</v>
+        <v>172</v>
       </c>
       <c r="S85" t="s">
-        <v>177</v>
+        <v>175</v>
       </c>
       <c r="T85" t="s">
         <v>179</v>
@@ -5032,7 +5246,7 @@
       <c r="U85" t="s">
         <v>28</v>
       </c>
-      <c r="V85" s="2">
+      <c r="V85" s="1">
         <v>46321</v>
       </c>
     </row>
@@ -5058,14 +5272,17 @@
       <c r="O86" t="s">
         <v>99</v>
       </c>
+      <c r="P86">
+        <v>4394700</v>
+      </c>
       <c r="Q86" t="s">
-        <v>168</v>
+        <v>169</v>
       </c>
       <c r="R86" t="s">
-        <v>171</v>
+        <v>172</v>
       </c>
       <c r="S86" t="s">
-        <v>175</v>
+        <v>176</v>
       </c>
       <c r="T86" t="s">
         <v>179</v>
@@ -5073,7 +5290,7 @@
       <c r="U86" t="s">
         <v>28</v>
       </c>
-      <c r="V86" s="2">
+      <c r="V86" s="1">
         <v>46382</v>
       </c>
     </row>
@@ -5105,11 +5322,14 @@
       <c r="O87" t="s">
         <v>99</v>
       </c>
+      <c r="P87">
+        <v>3306000</v>
+      </c>
       <c r="Q87" t="s">
-        <v>168</v>
+        <v>169</v>
       </c>
       <c r="R87" t="s">
-        <v>171</v>
+        <v>172</v>
       </c>
       <c r="S87" t="s">
         <v>42</v>
@@ -5149,11 +5369,14 @@
       <c r="O88" t="s">
         <v>99</v>
       </c>
+      <c r="P88">
+        <v>3306000</v>
+      </c>
       <c r="Q88" t="s">
-        <v>168</v>
+        <v>169</v>
       </c>
       <c r="R88" t="s">
-        <v>171</v>
+        <v>172</v>
       </c>
       <c r="S88" t="s">
         <v>42</v>
@@ -5190,14 +5413,17 @@
       <c r="O89" t="s">
         <v>167</v>
       </c>
+      <c r="P89">
+        <v>470820</v>
+      </c>
       <c r="Q89" t="s">
-        <v>168</v>
+        <v>169</v>
       </c>
       <c r="R89" t="s">
-        <v>171</v>
+        <v>172</v>
       </c>
       <c r="S89" t="s">
-        <v>174</v>
+        <v>175</v>
       </c>
       <c r="T89" t="s">
         <v>182</v>
@@ -5205,7 +5431,51 @@
       <c r="U89" t="s">
         <v>28</v>
       </c>
-      <c r="V89" s="2">
+      <c r="V89" s="1">
+        <v>46291</v>
+      </c>
+    </row>
+    <row r="90" spans="1:22">
+      <c r="A90">
+        <v>68160</v>
+      </c>
+      <c r="B90" t="s">
+        <v>22</v>
+      </c>
+      <c r="D90" t="s">
+        <v>24</v>
+      </c>
+      <c r="E90" t="s">
+        <v>28</v>
+      </c>
+      <c r="F90" t="s">
+        <v>30</v>
+      </c>
+      <c r="N90" t="s">
+        <v>90</v>
+      </c>
+      <c r="O90" t="s">
+        <v>168</v>
+      </c>
+      <c r="P90">
+        <v>2297180</v>
+      </c>
+      <c r="Q90" t="s">
+        <v>170</v>
+      </c>
+      <c r="R90" t="s">
+        <v>172</v>
+      </c>
+      <c r="S90" t="s">
+        <v>175</v>
+      </c>
+      <c r="T90" t="s">
+        <v>179</v>
+      </c>
+      <c r="U90" t="s">
+        <v>28</v>
+      </c>
+      <c r="V90" s="1">
         <v>46291</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Atualização automática: mta (23/09/2026 10:03)
</commit_message>
<xml_diff>
--- a/Projetos/02_Dados_Tratados/base_mta_tratada.xlsx
+++ b/Projetos/02_Dados_Tratados/base_mta_tratada.xlsx
@@ -14,7 +14,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1188" uniqueCount="184">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1188" uniqueCount="183">
   <si>
     <t>linha</t>
   </si>
@@ -232,7 +232,7 @@
     <t>e-mail 12/08</t>
   </si>
   <si>
-    <t>Atender; Alterar a tarefa para "Requisição Consumíveis". Alterar a ND para 339030</t>
+    <t>Atender</t>
   </si>
   <si>
     <t>ATENDER</t>
@@ -242,9 +242,6 @@
   </si>
   <si>
     <t>Atender SET</t>
-  </si>
-  <si>
-    <t>Atender</t>
   </si>
   <si>
     <t>Atender NOV</t>
@@ -575,8 +572,16 @@
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="YYYY-MM-DD HH:MM:SS"/>
   </numFmts>
-  <fonts count="1">
+  <fonts count="2">
     <font>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
       <sz val="11"/>
       <color theme="1"/>
       <name val="Calibri"/>
@@ -592,7 +597,7 @@
       <patternFill patternType="gray125"/>
     </fill>
   </fills>
-  <borders count="1">
+  <borders count="2">
     <border>
       <left/>
       <right/>
@@ -600,12 +605,30 @@
       <bottom/>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin">
+        <color auto="1"/>
+      </left>
+      <right style="thin">
+        <color auto="1"/>
+      </right>
+      <top style="thin">
+        <color auto="1"/>
+      </top>
+      <bottom style="thin">
+        <color auto="1"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="3">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
   </cellXfs>
   <cellStyles count="1">
@@ -905,70 +928,70 @@
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:22">
-      <c r="A1" t="s">
+      <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
-      <c r="B1" t="s">
+      <c r="B1" s="1" t="s">
         <v>1</v>
       </c>
-      <c r="C1" t="s">
+      <c r="C1" s="1" t="s">
         <v>2</v>
       </c>
-      <c r="D1" t="s">
+      <c r="D1" s="1" t="s">
         <v>3</v>
       </c>
-      <c r="E1" t="s">
+      <c r="E1" s="1" t="s">
         <v>4</v>
       </c>
-      <c r="F1" t="s">
+      <c r="F1" s="1" t="s">
         <v>5</v>
       </c>
-      <c r="G1" t="s">
+      <c r="G1" s="1" t="s">
         <v>6</v>
       </c>
-      <c r="H1" t="s">
+      <c r="H1" s="1" t="s">
         <v>7</v>
       </c>
-      <c r="I1" t="s">
+      <c r="I1" s="1" t="s">
         <v>8</v>
       </c>
-      <c r="J1" t="s">
+      <c r="J1" s="1" t="s">
         <v>9</v>
       </c>
-      <c r="K1" t="s">
+      <c r="K1" s="1" t="s">
         <v>10</v>
       </c>
-      <c r="L1" t="s">
+      <c r="L1" s="1" t="s">
         <v>11</v>
       </c>
-      <c r="M1" t="s">
+      <c r="M1" s="1" t="s">
         <v>12</v>
       </c>
-      <c r="N1" t="s">
+      <c r="N1" s="1" t="s">
         <v>13</v>
       </c>
-      <c r="O1" t="s">
+      <c r="O1" s="1" t="s">
         <v>14</v>
       </c>
-      <c r="P1" t="s">
+      <c r="P1" s="1" t="s">
         <v>15</v>
       </c>
-      <c r="Q1" t="s">
+      <c r="Q1" s="1" t="s">
         <v>16</v>
       </c>
-      <c r="R1" t="s">
+      <c r="R1" s="1" t="s">
         <v>17</v>
       </c>
-      <c r="S1" t="s">
+      <c r="S1" s="1" t="s">
         <v>18</v>
       </c>
-      <c r="T1" t="s">
+      <c r="T1" s="1" t="s">
         <v>19</v>
       </c>
-      <c r="U1" t="s">
+      <c r="U1" s="1" t="s">
         <v>20</v>
       </c>
-      <c r="V1" t="s">
+      <c r="V1" s="1" t="s">
         <v>21</v>
       </c>
     </row>
@@ -998,33 +1021,33 @@
         <v>72</v>
       </c>
       <c r="L2" t="s">
+        <v>80</v>
+      </c>
+      <c r="N2" t="s">
         <v>81</v>
       </c>
-      <c r="N2" t="s">
-        <v>82</v>
-      </c>
       <c r="O2" t="s">
-        <v>101</v>
+        <v>100</v>
       </c>
       <c r="P2">
         <v>135000</v>
       </c>
       <c r="Q2" t="s">
-        <v>169</v>
+        <v>168</v>
       </c>
       <c r="R2" t="s">
-        <v>172</v>
+        <v>171</v>
       </c>
       <c r="S2" t="s">
-        <v>175</v>
+        <v>174</v>
       </c>
       <c r="T2" t="s">
-        <v>178</v>
+        <v>177</v>
       </c>
       <c r="U2" t="s">
-        <v>183</v>
-      </c>
-      <c r="V2" s="1">
+        <v>182</v>
+      </c>
+      <c r="V2" s="2">
         <v>46229</v>
       </c>
     </row>
@@ -1051,27 +1074,27 @@
         <v>43</v>
       </c>
       <c r="N3" t="s">
-        <v>82</v>
+        <v>81</v>
       </c>
       <c r="O3" t="s">
-        <v>102</v>
+        <v>101</v>
       </c>
       <c r="Q3" t="s">
-        <v>169</v>
+        <v>168</v>
       </c>
       <c r="R3" t="s">
-        <v>172</v>
+        <v>171</v>
       </c>
       <c r="S3" t="s">
-        <v>175</v>
+        <v>174</v>
       </c>
       <c r="T3" t="s">
-        <v>178</v>
+        <v>177</v>
       </c>
       <c r="U3" t="s">
         <v>28</v>
       </c>
-      <c r="V3" s="1">
+      <c r="V3" s="2">
         <v>46291</v>
       </c>
     </row>
@@ -1098,27 +1121,27 @@
         <v>43</v>
       </c>
       <c r="N4" t="s">
-        <v>83</v>
+        <v>82</v>
       </c>
       <c r="O4" t="s">
-        <v>103</v>
+        <v>102</v>
       </c>
       <c r="Q4" t="s">
-        <v>169</v>
+        <v>168</v>
       </c>
       <c r="R4" t="s">
-        <v>173</v>
+        <v>172</v>
       </c>
       <c r="S4" t="s">
-        <v>175</v>
+        <v>174</v>
       </c>
       <c r="T4" t="s">
-        <v>178</v>
+        <v>177</v>
       </c>
       <c r="U4" t="s">
         <v>28</v>
       </c>
-      <c r="V4" s="1">
+      <c r="V4" s="2">
         <v>46321</v>
       </c>
     </row>
@@ -1145,27 +1168,27 @@
         <v>43</v>
       </c>
       <c r="N5" t="s">
-        <v>83</v>
+        <v>82</v>
       </c>
       <c r="O5" t="s">
-        <v>104</v>
+        <v>103</v>
       </c>
       <c r="Q5" t="s">
-        <v>169</v>
+        <v>168</v>
       </c>
       <c r="R5" t="s">
-        <v>173</v>
+        <v>172</v>
       </c>
       <c r="S5" t="s">
-        <v>175</v>
+        <v>174</v>
       </c>
       <c r="T5" t="s">
-        <v>178</v>
+        <v>177</v>
       </c>
       <c r="U5" t="s">
         <v>28</v>
       </c>
-      <c r="V5" s="1">
+      <c r="V5" s="2">
         <v>46321</v>
       </c>
     </row>
@@ -1192,30 +1215,30 @@
         <v>43</v>
       </c>
       <c r="L6" t="s">
-        <v>81</v>
+        <v>80</v>
       </c>
       <c r="N6" t="s">
-        <v>84</v>
+        <v>83</v>
       </c>
       <c r="O6" t="s">
-        <v>105</v>
+        <v>104</v>
       </c>
       <c r="Q6" t="s">
-        <v>169</v>
+        <v>168</v>
       </c>
       <c r="R6" t="s">
-        <v>173</v>
+        <v>172</v>
       </c>
       <c r="S6" t="s">
-        <v>175</v>
+        <v>174</v>
       </c>
       <c r="T6" t="s">
-        <v>178</v>
+        <v>177</v>
       </c>
       <c r="U6" t="s">
         <v>28</v>
       </c>
-      <c r="V6" s="1">
+      <c r="V6" s="2">
         <v>46291</v>
       </c>
     </row>
@@ -1241,37 +1264,37 @@
       <c r="G7" t="s">
         <v>44</v>
       </c>
-      <c r="H7" s="1">
+      <c r="H7" s="2">
         <v>46121</v>
       </c>
       <c r="I7" t="s">
         <v>47</v>
       </c>
       <c r="N7" t="s">
-        <v>85</v>
+        <v>84</v>
       </c>
       <c r="O7" t="s">
-        <v>106</v>
+        <v>105</v>
       </c>
       <c r="P7">
         <v>3799999.6</v>
       </c>
       <c r="Q7" t="s">
-        <v>170</v>
+        <v>169</v>
       </c>
       <c r="R7" t="s">
-        <v>173</v>
+        <v>172</v>
       </c>
       <c r="S7" t="s">
-        <v>175</v>
+        <v>174</v>
       </c>
       <c r="T7" t="s">
-        <v>179</v>
+        <v>178</v>
       </c>
       <c r="U7" t="s">
         <v>28</v>
       </c>
-      <c r="V7" s="1">
+      <c r="V7" s="2">
         <v>46138</v>
       </c>
     </row>
@@ -1298,27 +1321,27 @@
         <v>43</v>
       </c>
       <c r="N8" t="s">
-        <v>83</v>
+        <v>82</v>
       </c>
       <c r="O8" t="s">
-        <v>107</v>
+        <v>106</v>
       </c>
       <c r="Q8" t="s">
-        <v>169</v>
+        <v>168</v>
       </c>
       <c r="R8" t="s">
-        <v>173</v>
+        <v>172</v>
       </c>
       <c r="S8" t="s">
-        <v>175</v>
+        <v>174</v>
       </c>
       <c r="T8" t="s">
-        <v>178</v>
+        <v>177</v>
       </c>
       <c r="U8" t="s">
         <v>28</v>
       </c>
-      <c r="V8" s="1">
+      <c r="V8" s="2">
         <v>46291</v>
       </c>
     </row>
@@ -1342,30 +1365,30 @@
         <v>30</v>
       </c>
       <c r="N9" t="s">
-        <v>83</v>
+        <v>82</v>
       </c>
       <c r="O9" t="s">
-        <v>108</v>
+        <v>107</v>
       </c>
       <c r="P9">
         <v>60000</v>
       </c>
       <c r="Q9" t="s">
-        <v>169</v>
+        <v>168</v>
       </c>
       <c r="R9" t="s">
-        <v>173</v>
+        <v>172</v>
       </c>
       <c r="S9" t="s">
-        <v>175</v>
+        <v>174</v>
       </c>
       <c r="T9" t="s">
-        <v>178</v>
+        <v>177</v>
       </c>
       <c r="U9" t="s">
         <v>28</v>
       </c>
-      <c r="V9" s="1">
+      <c r="V9" s="2">
         <v>46291</v>
       </c>
     </row>
@@ -1392,27 +1415,27 @@
         <v>43</v>
       </c>
       <c r="N10" t="s">
-        <v>84</v>
+        <v>83</v>
       </c>
       <c r="O10" t="s">
-        <v>109</v>
+        <v>108</v>
       </c>
       <c r="Q10" t="s">
-        <v>169</v>
+        <v>168</v>
       </c>
       <c r="R10" t="s">
-        <v>173</v>
+        <v>172</v>
       </c>
       <c r="S10" t="s">
-        <v>175</v>
+        <v>174</v>
       </c>
       <c r="T10" t="s">
-        <v>178</v>
+        <v>177</v>
       </c>
       <c r="U10" t="s">
         <v>28</v>
       </c>
-      <c r="V10" s="1">
+      <c r="V10" s="2">
         <v>46291</v>
       </c>
     </row>
@@ -1439,27 +1462,27 @@
         <v>43</v>
       </c>
       <c r="N11" t="s">
-        <v>84</v>
+        <v>83</v>
       </c>
       <c r="O11" t="s">
-        <v>110</v>
+        <v>109</v>
       </c>
       <c r="Q11" t="s">
-        <v>169</v>
+        <v>168</v>
       </c>
       <c r="R11" t="s">
-        <v>173</v>
+        <v>172</v>
       </c>
       <c r="S11" t="s">
-        <v>175</v>
+        <v>174</v>
       </c>
       <c r="T11" t="s">
-        <v>178</v>
+        <v>177</v>
       </c>
       <c r="U11" t="s">
         <v>28</v>
       </c>
-      <c r="V11" s="1">
+      <c r="V11" s="2">
         <v>46291</v>
       </c>
     </row>
@@ -1485,7 +1508,7 @@
       <c r="G12" t="s">
         <v>44</v>
       </c>
-      <c r="H12" s="1">
+      <c r="H12" s="2">
         <v>46079</v>
       </c>
       <c r="I12" t="s">
@@ -1495,30 +1518,30 @@
         <v>65</v>
       </c>
       <c r="N12" t="s">
-        <v>82</v>
+        <v>81</v>
       </c>
       <c r="O12" t="s">
-        <v>111</v>
+        <v>110</v>
       </c>
       <c r="P12">
         <v>1187433.02</v>
       </c>
       <c r="Q12" t="s">
-        <v>169</v>
+        <v>168</v>
       </c>
       <c r="R12" t="s">
-        <v>172</v>
+        <v>171</v>
       </c>
       <c r="S12" t="s">
-        <v>175</v>
+        <v>174</v>
       </c>
       <c r="T12" t="s">
-        <v>178</v>
+        <v>177</v>
       </c>
       <c r="U12" t="s">
-        <v>183</v>
-      </c>
-      <c r="V12" s="1">
+        <v>182</v>
+      </c>
+      <c r="V12" s="2">
         <v>46079</v>
       </c>
     </row>
@@ -1548,30 +1571,30 @@
         <v>73</v>
       </c>
       <c r="N13" t="s">
-        <v>82</v>
+        <v>81</v>
       </c>
       <c r="O13" t="s">
-        <v>112</v>
+        <v>111</v>
       </c>
       <c r="P13">
         <v>1000000</v>
       </c>
       <c r="Q13" t="s">
-        <v>169</v>
+        <v>168</v>
       </c>
       <c r="R13" t="s">
-        <v>172</v>
+        <v>171</v>
       </c>
       <c r="S13" t="s">
-        <v>175</v>
+        <v>174</v>
       </c>
       <c r="T13" t="s">
-        <v>178</v>
+        <v>177</v>
       </c>
       <c r="U13" t="s">
-        <v>183</v>
-      </c>
-      <c r="V13" s="1">
+        <v>182</v>
+      </c>
+      <c r="V13" s="2">
         <v>46352</v>
       </c>
     </row>
@@ -1601,30 +1624,30 @@
         <v>73</v>
       </c>
       <c r="N14" t="s">
-        <v>82</v>
+        <v>81</v>
       </c>
       <c r="O14" t="s">
-        <v>113</v>
+        <v>112</v>
       </c>
       <c r="P14">
         <v>1000000</v>
       </c>
       <c r="Q14" t="s">
-        <v>169</v>
+        <v>168</v>
       </c>
       <c r="R14" t="s">
-        <v>172</v>
+        <v>171</v>
       </c>
       <c r="S14" t="s">
-        <v>175</v>
+        <v>174</v>
       </c>
       <c r="T14" t="s">
-        <v>178</v>
+        <v>177</v>
       </c>
       <c r="U14" t="s">
-        <v>183</v>
-      </c>
-      <c r="V14" s="1">
+        <v>182</v>
+      </c>
+      <c r="V14" s="2">
         <v>46352</v>
       </c>
     </row>
@@ -1654,30 +1677,30 @@
         <v>73</v>
       </c>
       <c r="N15" t="s">
-        <v>82</v>
+        <v>81</v>
       </c>
       <c r="O15" t="s">
-        <v>114</v>
+        <v>113</v>
       </c>
       <c r="P15">
         <v>1000000</v>
       </c>
       <c r="Q15" t="s">
-        <v>169</v>
+        <v>168</v>
       </c>
       <c r="R15" t="s">
-        <v>172</v>
+        <v>171</v>
       </c>
       <c r="S15" t="s">
-        <v>175</v>
+        <v>174</v>
       </c>
       <c r="T15" t="s">
-        <v>178</v>
+        <v>177</v>
       </c>
       <c r="U15" t="s">
-        <v>183</v>
-      </c>
-      <c r="V15" s="1">
+        <v>182</v>
+      </c>
+      <c r="V15" s="2">
         <v>46352</v>
       </c>
     </row>
@@ -1707,30 +1730,30 @@
         <v>73</v>
       </c>
       <c r="N16" t="s">
-        <v>86</v>
+        <v>85</v>
       </c>
       <c r="O16" t="s">
-        <v>115</v>
+        <v>114</v>
       </c>
       <c r="P16">
         <v>100000</v>
       </c>
       <c r="Q16" t="s">
+        <v>170</v>
+      </c>
+      <c r="R16" t="s">
         <v>171</v>
       </c>
-      <c r="R16" t="s">
-        <v>172</v>
-      </c>
       <c r="S16" t="s">
-        <v>175</v>
+        <v>174</v>
       </c>
       <c r="T16" t="s">
-        <v>178</v>
+        <v>177</v>
       </c>
       <c r="U16" t="s">
-        <v>183</v>
-      </c>
-      <c r="V16" s="1">
+        <v>182</v>
+      </c>
+      <c r="V16" s="2">
         <v>46229</v>
       </c>
     </row>
@@ -1756,7 +1779,7 @@
       <c r="G17" t="s">
         <v>44</v>
       </c>
-      <c r="H17" s="1">
+      <c r="H17" s="2">
         <v>46098</v>
       </c>
       <c r="I17" t="s">
@@ -1766,30 +1789,30 @@
         <v>65</v>
       </c>
       <c r="N17" t="s">
-        <v>87</v>
+        <v>86</v>
       </c>
       <c r="O17" t="s">
-        <v>116</v>
+        <v>115</v>
       </c>
       <c r="P17">
         <v>1770880.5</v>
       </c>
       <c r="Q17" t="s">
-        <v>170</v>
+        <v>169</v>
       </c>
       <c r="R17" t="s">
-        <v>173</v>
+        <v>172</v>
       </c>
       <c r="S17" t="s">
-        <v>175</v>
+        <v>174</v>
       </c>
       <c r="T17" t="s">
-        <v>180</v>
+        <v>179</v>
       </c>
       <c r="U17" t="s">
-        <v>183</v>
-      </c>
-      <c r="V17" s="1">
+        <v>182</v>
+      </c>
+      <c r="V17" s="2">
         <v>46107</v>
       </c>
     </row>
@@ -1815,37 +1838,37 @@
       <c r="G18" t="s">
         <v>44</v>
       </c>
-      <c r="H18" s="1">
+      <c r="H18" s="2">
         <v>46076</v>
       </c>
       <c r="I18" t="s">
         <v>50</v>
       </c>
       <c r="N18" t="s">
-        <v>88</v>
+        <v>87</v>
       </c>
       <c r="O18" t="s">
-        <v>117</v>
+        <v>116</v>
       </c>
       <c r="P18">
         <v>350000</v>
       </c>
       <c r="Q18" t="s">
-        <v>170</v>
+        <v>169</v>
       </c>
       <c r="R18" t="s">
-        <v>172</v>
+        <v>171</v>
       </c>
       <c r="S18" t="s">
-        <v>175</v>
+        <v>174</v>
       </c>
       <c r="T18" t="s">
-        <v>179</v>
+        <v>178</v>
       </c>
       <c r="U18" t="s">
         <v>28</v>
       </c>
-      <c r="V18" s="1">
+      <c r="V18" s="2">
         <v>46079</v>
       </c>
     </row>
@@ -1871,37 +1894,37 @@
       <c r="G19" t="s">
         <v>44</v>
       </c>
-      <c r="H19" s="1">
+      <c r="H19" s="2">
         <v>46076</v>
       </c>
       <c r="I19" t="s">
         <v>50</v>
       </c>
       <c r="N19" t="s">
-        <v>88</v>
+        <v>87</v>
       </c>
       <c r="O19" t="s">
-        <v>118</v>
+        <v>117</v>
       </c>
       <c r="P19">
         <v>350000</v>
       </c>
       <c r="Q19" t="s">
-        <v>170</v>
+        <v>169</v>
       </c>
       <c r="R19" t="s">
-        <v>172</v>
+        <v>171</v>
       </c>
       <c r="S19" t="s">
-        <v>175</v>
+        <v>174</v>
       </c>
       <c r="T19" t="s">
-        <v>179</v>
+        <v>178</v>
       </c>
       <c r="U19" t="s">
         <v>28</v>
       </c>
-      <c r="V19" s="1">
+      <c r="V19" s="2">
         <v>46079</v>
       </c>
     </row>
@@ -1925,30 +1948,30 @@
         <v>30</v>
       </c>
       <c r="N20" t="s">
-        <v>89</v>
+        <v>88</v>
       </c>
       <c r="O20" t="s">
-        <v>119</v>
+        <v>118</v>
       </c>
       <c r="P20">
         <v>1000000</v>
       </c>
       <c r="Q20" t="s">
-        <v>170</v>
+        <v>169</v>
       </c>
       <c r="R20" t="s">
-        <v>172</v>
+        <v>171</v>
       </c>
       <c r="S20" t="s">
-        <v>175</v>
+        <v>174</v>
       </c>
       <c r="T20" t="s">
-        <v>179</v>
+        <v>178</v>
       </c>
       <c r="U20" t="s">
         <v>28</v>
       </c>
-      <c r="V20" s="1">
+      <c r="V20" s="2">
         <v>46321</v>
       </c>
     </row>
@@ -1975,27 +1998,27 @@
         <v>43</v>
       </c>
       <c r="N21" t="s">
-        <v>82</v>
+        <v>81</v>
       </c>
       <c r="O21" t="s">
-        <v>120</v>
+        <v>119</v>
       </c>
       <c r="Q21" t="s">
-        <v>169</v>
+        <v>168</v>
       </c>
       <c r="R21" t="s">
-        <v>172</v>
+        <v>171</v>
       </c>
       <c r="S21" t="s">
-        <v>175</v>
+        <v>174</v>
       </c>
       <c r="T21" t="s">
-        <v>178</v>
+        <v>177</v>
       </c>
       <c r="U21" t="s">
         <v>28</v>
       </c>
-      <c r="V21" s="1">
+      <c r="V21" s="2">
         <v>46321</v>
       </c>
     </row>
@@ -2022,27 +2045,27 @@
         <v>43</v>
       </c>
       <c r="N22" t="s">
-        <v>83</v>
+        <v>82</v>
       </c>
       <c r="O22" t="s">
-        <v>121</v>
+        <v>120</v>
       </c>
       <c r="Q22" t="s">
-        <v>169</v>
+        <v>168</v>
       </c>
       <c r="R22" t="s">
-        <v>173</v>
+        <v>172</v>
       </c>
       <c r="S22" t="s">
-        <v>175</v>
+        <v>174</v>
       </c>
       <c r="T22" t="s">
-        <v>178</v>
+        <v>177</v>
       </c>
       <c r="U22" t="s">
         <v>28</v>
       </c>
-      <c r="V22" s="1">
+      <c r="V22" s="2">
         <v>46321</v>
       </c>
     </row>
@@ -2069,27 +2092,27 @@
         <v>43</v>
       </c>
       <c r="N23" t="s">
-        <v>83</v>
+        <v>82</v>
       </c>
       <c r="O23" t="s">
-        <v>122</v>
+        <v>121</v>
       </c>
       <c r="Q23" t="s">
-        <v>169</v>
+        <v>168</v>
       </c>
       <c r="R23" t="s">
-        <v>173</v>
+        <v>172</v>
       </c>
       <c r="S23" t="s">
-        <v>175</v>
+        <v>174</v>
       </c>
       <c r="T23" t="s">
-        <v>178</v>
+        <v>177</v>
       </c>
       <c r="U23" t="s">
         <v>28</v>
       </c>
-      <c r="V23" s="1">
+      <c r="V23" s="2">
         <v>46321</v>
       </c>
     </row>
@@ -2115,7 +2138,7 @@
       <c r="G24" t="s">
         <v>44</v>
       </c>
-      <c r="H24" s="1">
+      <c r="H24" s="2">
         <v>46119</v>
       </c>
       <c r="I24" t="s">
@@ -2125,30 +2148,30 @@
         <v>66</v>
       </c>
       <c r="N24" t="s">
-        <v>87</v>
+        <v>86</v>
       </c>
       <c r="O24" t="s">
-        <v>123</v>
+        <v>122</v>
       </c>
       <c r="P24">
         <v>1704503</v>
       </c>
       <c r="Q24" t="s">
-        <v>170</v>
+        <v>169</v>
       </c>
       <c r="R24" t="s">
-        <v>173</v>
+        <v>172</v>
       </c>
       <c r="S24" t="s">
-        <v>175</v>
+        <v>174</v>
       </c>
       <c r="T24" t="s">
-        <v>180</v>
+        <v>179</v>
       </c>
       <c r="U24" t="s">
-        <v>183</v>
-      </c>
-      <c r="V24" s="1">
+        <v>182</v>
+      </c>
+      <c r="V24" s="2">
         <v>46138</v>
       </c>
     </row>
@@ -2174,37 +2197,37 @@
       <c r="G25" t="s">
         <v>44</v>
       </c>
-      <c r="H25" s="1">
+      <c r="H25" s="2">
         <v>46121</v>
       </c>
       <c r="I25" t="s">
         <v>52</v>
       </c>
       <c r="N25" t="s">
-        <v>90</v>
+        <v>89</v>
       </c>
       <c r="O25" t="s">
-        <v>124</v>
+        <v>123</v>
       </c>
       <c r="P25">
         <v>3799000</v>
       </c>
       <c r="Q25" t="s">
-        <v>170</v>
+        <v>169</v>
       </c>
       <c r="R25" t="s">
-        <v>173</v>
+        <v>172</v>
       </c>
       <c r="S25" t="s">
-        <v>175</v>
+        <v>174</v>
       </c>
       <c r="T25" t="s">
-        <v>179</v>
+        <v>178</v>
       </c>
       <c r="U25" t="s">
         <v>28</v>
       </c>
-      <c r="V25" s="1">
+      <c r="V25" s="2">
         <v>46138</v>
       </c>
     </row>
@@ -2230,37 +2253,37 @@
       <c r="G26" t="s">
         <v>44</v>
       </c>
-      <c r="H26" s="1">
+      <c r="H26" s="2">
         <v>46076</v>
       </c>
       <c r="I26" t="s">
         <v>53</v>
       </c>
       <c r="N26" t="s">
-        <v>90</v>
+        <v>89</v>
       </c>
       <c r="O26" t="s">
-        <v>124</v>
+        <v>123</v>
       </c>
       <c r="P26">
         <v>1000</v>
       </c>
       <c r="Q26" t="s">
-        <v>170</v>
+        <v>169</v>
       </c>
       <c r="R26" t="s">
-        <v>172</v>
+        <v>171</v>
       </c>
       <c r="S26" t="s">
-        <v>175</v>
+        <v>174</v>
       </c>
       <c r="T26" t="s">
-        <v>179</v>
+        <v>178</v>
       </c>
       <c r="U26" t="s">
         <v>28</v>
       </c>
-      <c r="V26" s="1">
+      <c r="V26" s="2">
         <v>46079</v>
       </c>
     </row>
@@ -2290,30 +2313,30 @@
         <v>73</v>
       </c>
       <c r="N27" t="s">
-        <v>86</v>
+        <v>85</v>
       </c>
       <c r="O27" t="s">
-        <v>125</v>
+        <v>124</v>
       </c>
       <c r="P27">
         <v>100000</v>
       </c>
       <c r="Q27" t="s">
+        <v>170</v>
+      </c>
+      <c r="R27" t="s">
         <v>171</v>
       </c>
-      <c r="R27" t="s">
-        <v>172</v>
-      </c>
       <c r="S27" t="s">
-        <v>175</v>
+        <v>174</v>
       </c>
       <c r="T27" t="s">
-        <v>178</v>
+        <v>177</v>
       </c>
       <c r="U27" t="s">
-        <v>183</v>
-      </c>
-      <c r="V27" s="1">
+        <v>182</v>
+      </c>
+      <c r="V27" s="2">
         <v>46291</v>
       </c>
     </row>
@@ -2339,7 +2362,7 @@
       <c r="G28" t="s">
         <v>44</v>
       </c>
-      <c r="H28" s="1">
+      <c r="H28" s="2">
         <v>46199</v>
       </c>
       <c r="I28" t="s">
@@ -2349,30 +2372,30 @@
         <v>67</v>
       </c>
       <c r="N28" t="s">
-        <v>87</v>
+        <v>86</v>
       </c>
       <c r="O28" t="s">
-        <v>126</v>
+        <v>125</v>
       </c>
       <c r="P28">
         <v>150000</v>
       </c>
       <c r="Q28" t="s">
-        <v>170</v>
+        <v>169</v>
       </c>
       <c r="R28" t="s">
-        <v>173</v>
+        <v>172</v>
       </c>
       <c r="S28" t="s">
-        <v>175</v>
+        <v>174</v>
       </c>
       <c r="T28" t="s">
-        <v>179</v>
+        <v>178</v>
       </c>
       <c r="U28" t="s">
-        <v>183</v>
-      </c>
-      <c r="V28" s="1">
+        <v>182</v>
+      </c>
+      <c r="V28" s="2">
         <v>46199</v>
       </c>
     </row>
@@ -2398,7 +2421,7 @@
       <c r="G29" t="s">
         <v>44</v>
       </c>
-      <c r="H29" s="1">
+      <c r="H29" s="2">
         <v>46199</v>
       </c>
       <c r="I29" t="s">
@@ -2408,30 +2431,30 @@
         <v>67</v>
       </c>
       <c r="N29" t="s">
-        <v>87</v>
+        <v>86</v>
       </c>
       <c r="O29" t="s">
-        <v>127</v>
+        <v>126</v>
       </c>
       <c r="P29">
         <v>150000</v>
       </c>
       <c r="Q29" t="s">
-        <v>170</v>
+        <v>169</v>
       </c>
       <c r="R29" t="s">
-        <v>173</v>
+        <v>172</v>
       </c>
       <c r="S29" t="s">
-        <v>175</v>
+        <v>174</v>
       </c>
       <c r="T29" t="s">
-        <v>179</v>
+        <v>178</v>
       </c>
       <c r="U29" t="s">
-        <v>183</v>
-      </c>
-      <c r="V29" s="1">
+        <v>182</v>
+      </c>
+      <c r="V29" s="2">
         <v>46199</v>
       </c>
     </row>
@@ -2457,7 +2480,7 @@
       <c r="G30" t="s">
         <v>44</v>
       </c>
-      <c r="H30" s="1">
+      <c r="H30" s="2">
         <v>46199</v>
       </c>
       <c r="I30" t="s">
@@ -2467,30 +2490,30 @@
         <v>67</v>
       </c>
       <c r="N30" t="s">
-        <v>87</v>
+        <v>86</v>
       </c>
       <c r="O30" t="s">
-        <v>128</v>
+        <v>127</v>
       </c>
       <c r="P30">
         <v>18462.36</v>
       </c>
       <c r="Q30" t="s">
-        <v>170</v>
+        <v>169</v>
       </c>
       <c r="R30" t="s">
-        <v>173</v>
+        <v>172</v>
       </c>
       <c r="S30" t="s">
-        <v>175</v>
+        <v>174</v>
       </c>
       <c r="T30" t="s">
-        <v>179</v>
+        <v>178</v>
       </c>
       <c r="U30" t="s">
-        <v>183</v>
-      </c>
-      <c r="V30" s="1">
+        <v>182</v>
+      </c>
+      <c r="V30" s="2">
         <v>46199</v>
       </c>
     </row>
@@ -2516,7 +2539,7 @@
       <c r="G31" t="s">
         <v>44</v>
       </c>
-      <c r="H31" s="1">
+      <c r="H31" s="2">
         <v>46199</v>
       </c>
       <c r="I31" t="s">
@@ -2526,30 +2549,30 @@
         <v>67</v>
       </c>
       <c r="N31" t="s">
-        <v>87</v>
+        <v>86</v>
       </c>
       <c r="O31" t="s">
-        <v>128</v>
+        <v>127</v>
       </c>
       <c r="P31">
         <v>324166.14</v>
       </c>
       <c r="Q31" t="s">
-        <v>170</v>
+        <v>169</v>
       </c>
       <c r="R31" t="s">
-        <v>173</v>
+        <v>172</v>
       </c>
       <c r="S31" t="s">
-        <v>175</v>
+        <v>174</v>
       </c>
       <c r="T31" t="s">
-        <v>179</v>
+        <v>178</v>
       </c>
       <c r="U31" t="s">
-        <v>183</v>
-      </c>
-      <c r="V31" s="1">
+        <v>182</v>
+      </c>
+      <c r="V31" s="2">
         <v>46199</v>
       </c>
     </row>
@@ -2576,30 +2599,30 @@
         <v>74</v>
       </c>
       <c r="N32" t="s">
-        <v>87</v>
+        <v>86</v>
       </c>
       <c r="O32" t="s">
-        <v>129</v>
+        <v>128</v>
       </c>
       <c r="P32">
         <v>30000</v>
       </c>
       <c r="Q32" t="s">
-        <v>170</v>
+        <v>169</v>
       </c>
       <c r="R32" t="s">
-        <v>173</v>
+        <v>172</v>
       </c>
       <c r="S32" t="s">
-        <v>175</v>
+        <v>174</v>
       </c>
       <c r="T32" t="s">
-        <v>179</v>
+        <v>178</v>
       </c>
       <c r="U32" t="s">
-        <v>183</v>
-      </c>
-      <c r="V32" s="1">
+        <v>182</v>
+      </c>
+      <c r="V32" s="2">
         <v>46291</v>
       </c>
     </row>
@@ -2625,7 +2648,7 @@
       <c r="G33" t="s">
         <v>44</v>
       </c>
-      <c r="H33" s="1">
+      <c r="H33" s="2">
         <v>46191</v>
       </c>
       <c r="I33" t="s">
@@ -2635,30 +2658,30 @@
         <v>68</v>
       </c>
       <c r="N33" t="s">
-        <v>87</v>
+        <v>86</v>
       </c>
       <c r="O33" t="s">
-        <v>130</v>
+        <v>129</v>
       </c>
       <c r="P33">
         <v>1496713.48</v>
       </c>
       <c r="Q33" t="s">
-        <v>170</v>
+        <v>169</v>
       </c>
       <c r="R33" t="s">
-        <v>173</v>
+        <v>172</v>
       </c>
       <c r="S33" t="s">
-        <v>175</v>
+        <v>174</v>
       </c>
       <c r="T33" t="s">
-        <v>180</v>
+        <v>179</v>
       </c>
       <c r="U33" t="s">
-        <v>183</v>
-      </c>
-      <c r="V33" s="1">
+        <v>182</v>
+      </c>
+      <c r="V33" s="2">
         <v>46199</v>
       </c>
     </row>
@@ -2684,37 +2707,37 @@
       <c r="G34" t="s">
         <v>44</v>
       </c>
-      <c r="H34" s="1">
+      <c r="H34" s="2">
         <v>46119</v>
       </c>
       <c r="I34" t="s">
         <v>51</v>
       </c>
       <c r="N34" t="s">
-        <v>87</v>
+        <v>86</v>
       </c>
       <c r="O34" t="s">
-        <v>130</v>
+        <v>129</v>
       </c>
       <c r="P34">
         <v>207789.52</v>
       </c>
       <c r="Q34" t="s">
-        <v>170</v>
+        <v>169</v>
       </c>
       <c r="R34" t="s">
-        <v>173</v>
+        <v>172</v>
       </c>
       <c r="S34" t="s">
-        <v>175</v>
+        <v>174</v>
       </c>
       <c r="T34" t="s">
-        <v>180</v>
+        <v>179</v>
       </c>
       <c r="U34" t="s">
-        <v>183</v>
-      </c>
-      <c r="V34" s="1">
+        <v>182</v>
+      </c>
+      <c r="V34" s="2">
         <v>46138</v>
       </c>
     </row>
@@ -2740,37 +2763,37 @@
       <c r="G35" t="s">
         <v>44</v>
       </c>
-      <c r="H35" s="1">
+      <c r="H35" s="2">
         <v>46213</v>
       </c>
       <c r="I35" t="s">
         <v>57</v>
       </c>
       <c r="N35" t="s">
-        <v>90</v>
+        <v>89</v>
       </c>
       <c r="O35" t="s">
-        <v>131</v>
+        <v>130</v>
       </c>
       <c r="P35">
         <v>962290.8</v>
       </c>
       <c r="Q35" t="s">
-        <v>170</v>
+        <v>169</v>
       </c>
       <c r="R35" t="s">
-        <v>172</v>
+        <v>171</v>
       </c>
       <c r="S35" t="s">
-        <v>175</v>
+        <v>174</v>
       </c>
       <c r="T35" t="s">
-        <v>179</v>
+        <v>178</v>
       </c>
       <c r="U35" t="s">
         <v>28</v>
       </c>
-      <c r="V35" s="1">
+      <c r="V35" s="2">
         <v>46229</v>
       </c>
     </row>
@@ -2796,37 +2819,37 @@
       <c r="G36" t="s">
         <v>44</v>
       </c>
-      <c r="H36" s="1">
+      <c r="H36" s="2">
         <v>46175</v>
       </c>
       <c r="I36" t="s">
         <v>58</v>
       </c>
       <c r="N36" t="s">
-        <v>90</v>
+        <v>89</v>
       </c>
       <c r="O36" t="s">
-        <v>131</v>
+        <v>130</v>
       </c>
       <c r="P36">
         <v>798776.97</v>
       </c>
       <c r="Q36" t="s">
-        <v>170</v>
+        <v>169</v>
       </c>
       <c r="R36" t="s">
-        <v>173</v>
+        <v>172</v>
       </c>
       <c r="S36" t="s">
-        <v>175</v>
+        <v>174</v>
       </c>
       <c r="T36" t="s">
-        <v>179</v>
+        <v>178</v>
       </c>
       <c r="U36" t="s">
         <v>28</v>
       </c>
-      <c r="V36" s="1">
+      <c r="V36" s="2">
         <v>46199</v>
       </c>
     </row>
@@ -2852,37 +2875,37 @@
       <c r="G37" t="s">
         <v>44</v>
       </c>
-      <c r="H37" s="1">
+      <c r="H37" s="2">
         <v>46213</v>
       </c>
       <c r="I37" t="s">
         <v>57</v>
       </c>
       <c r="N37" t="s">
-        <v>90</v>
+        <v>89</v>
       </c>
       <c r="O37" t="s">
-        <v>131</v>
+        <v>130</v>
       </c>
       <c r="P37">
         <v>1530656.62</v>
       </c>
       <c r="Q37" t="s">
-        <v>170</v>
+        <v>169</v>
       </c>
       <c r="R37" t="s">
-        <v>172</v>
+        <v>171</v>
       </c>
       <c r="S37" t="s">
-        <v>175</v>
+        <v>174</v>
       </c>
       <c r="T37" t="s">
-        <v>179</v>
+        <v>178</v>
       </c>
       <c r="U37" t="s">
         <v>28</v>
       </c>
-      <c r="V37" s="1">
+      <c r="V37" s="2">
         <v>46229</v>
       </c>
     </row>
@@ -2908,37 +2931,37 @@
       <c r="G38" t="s">
         <v>44</v>
       </c>
-      <c r="H38" s="1">
+      <c r="H38" s="2">
         <v>46199</v>
       </c>
       <c r="I38" t="s">
         <v>59</v>
       </c>
       <c r="N38" t="s">
-        <v>90</v>
+        <v>89</v>
       </c>
       <c r="O38" t="s">
-        <v>131</v>
+        <v>130</v>
       </c>
       <c r="P38">
         <v>72958.08</v>
       </c>
       <c r="Q38" t="s">
-        <v>170</v>
+        <v>169</v>
       </c>
       <c r="R38" t="s">
-        <v>172</v>
+        <v>171</v>
       </c>
       <c r="S38" t="s">
-        <v>175</v>
+        <v>174</v>
       </c>
       <c r="T38" t="s">
-        <v>179</v>
+        <v>178</v>
       </c>
       <c r="U38" t="s">
         <v>28</v>
       </c>
-      <c r="V38" s="1">
+      <c r="V38" s="2">
         <v>46199</v>
       </c>
     </row>
@@ -2964,37 +2987,37 @@
       <c r="G39" t="s">
         <v>44</v>
       </c>
-      <c r="H39" s="1">
+      <c r="H39" s="2">
         <v>46199</v>
       </c>
       <c r="I39" t="s">
         <v>59</v>
       </c>
       <c r="N39" t="s">
-        <v>90</v>
+        <v>89</v>
       </c>
       <c r="O39" t="s">
-        <v>131</v>
+        <v>130</v>
       </c>
       <c r="P39">
         <v>8916</v>
       </c>
       <c r="Q39" t="s">
-        <v>170</v>
+        <v>169</v>
       </c>
       <c r="R39" t="s">
-        <v>172</v>
+        <v>171</v>
       </c>
       <c r="S39" t="s">
-        <v>175</v>
+        <v>174</v>
       </c>
       <c r="T39" t="s">
-        <v>179</v>
+        <v>178</v>
       </c>
       <c r="U39" t="s">
         <v>28</v>
       </c>
-      <c r="V39" s="1">
+      <c r="V39" s="2">
         <v>46199</v>
       </c>
     </row>
@@ -3020,37 +3043,37 @@
       <c r="G40" t="s">
         <v>44</v>
       </c>
-      <c r="H40" s="1">
+      <c r="H40" s="2">
         <v>46204</v>
       </c>
       <c r="I40" t="s">
         <v>59</v>
       </c>
       <c r="N40" t="s">
-        <v>90</v>
+        <v>89</v>
       </c>
       <c r="O40" t="s">
-        <v>131</v>
+        <v>130</v>
       </c>
       <c r="P40">
         <v>425178.5</v>
       </c>
       <c r="Q40" t="s">
-        <v>170</v>
+        <v>169</v>
       </c>
       <c r="R40" t="s">
-        <v>172</v>
+        <v>171</v>
       </c>
       <c r="S40" t="s">
-        <v>175</v>
+        <v>174</v>
       </c>
       <c r="T40" t="s">
-        <v>179</v>
+        <v>178</v>
       </c>
       <c r="U40" t="s">
         <v>28</v>
       </c>
-      <c r="V40" s="1">
+      <c r="V40" s="2">
         <v>46229</v>
       </c>
     </row>
@@ -3076,37 +3099,37 @@
       <c r="G41" t="s">
         <v>44</v>
       </c>
-      <c r="H41" s="1">
+      <c r="H41" s="2">
         <v>46244</v>
       </c>
       <c r="I41" t="s">
         <v>60</v>
       </c>
       <c r="N41" t="s">
-        <v>90</v>
+        <v>89</v>
       </c>
       <c r="O41" t="s">
-        <v>131</v>
+        <v>130</v>
       </c>
       <c r="P41">
         <v>1223.03</v>
       </c>
       <c r="Q41" t="s">
-        <v>170</v>
+        <v>169</v>
       </c>
       <c r="R41" t="s">
-        <v>172</v>
+        <v>171</v>
       </c>
       <c r="S41" t="s">
-        <v>175</v>
+        <v>174</v>
       </c>
       <c r="T41" t="s">
-        <v>179</v>
+        <v>178</v>
       </c>
       <c r="U41" t="s">
         <v>28</v>
       </c>
-      <c r="V41" s="1">
+      <c r="V41" s="2">
         <v>46199</v>
       </c>
     </row>
@@ -3130,27 +3153,27 @@
         <v>43</v>
       </c>
       <c r="N42" t="s">
-        <v>90</v>
+        <v>89</v>
       </c>
       <c r="O42" t="s">
-        <v>132</v>
+        <v>131</v>
       </c>
       <c r="Q42" t="s">
-        <v>170</v>
+        <v>169</v>
       </c>
       <c r="R42" t="s">
-        <v>172</v>
+        <v>171</v>
       </c>
       <c r="S42" t="s">
-        <v>176</v>
+        <v>175</v>
       </c>
       <c r="T42" t="s">
-        <v>179</v>
+        <v>178</v>
       </c>
       <c r="U42" t="s">
         <v>28</v>
       </c>
-      <c r="V42" s="1">
+      <c r="V42" s="2">
         <v>46260</v>
       </c>
     </row>
@@ -3176,37 +3199,37 @@
       <c r="G43" t="s">
         <v>44</v>
       </c>
-      <c r="H43" s="1">
+      <c r="H43" s="2">
         <v>46191</v>
       </c>
       <c r="I43" t="s">
         <v>61</v>
       </c>
       <c r="N43" t="s">
-        <v>88</v>
+        <v>87</v>
       </c>
       <c r="O43" t="s">
-        <v>133</v>
+        <v>132</v>
       </c>
       <c r="P43">
         <v>400000</v>
       </c>
       <c r="Q43" t="s">
-        <v>170</v>
+        <v>169</v>
       </c>
       <c r="R43" t="s">
-        <v>172</v>
+        <v>171</v>
       </c>
       <c r="S43" t="s">
-        <v>175</v>
+        <v>174</v>
       </c>
       <c r="T43" t="s">
-        <v>179</v>
+        <v>178</v>
       </c>
       <c r="U43" t="s">
         <v>28</v>
       </c>
-      <c r="V43" s="1">
+      <c r="V43" s="2">
         <v>46199</v>
       </c>
     </row>
@@ -3232,37 +3255,37 @@
       <c r="G44" t="s">
         <v>44</v>
       </c>
-      <c r="H44" s="1">
+      <c r="H44" s="2">
         <v>46191</v>
       </c>
       <c r="I44" t="s">
         <v>61</v>
       </c>
       <c r="N44" t="s">
-        <v>88</v>
+        <v>87</v>
       </c>
       <c r="O44" t="s">
-        <v>134</v>
+        <v>133</v>
       </c>
       <c r="P44">
         <v>400000</v>
       </c>
       <c r="Q44" t="s">
-        <v>170</v>
+        <v>169</v>
       </c>
       <c r="R44" t="s">
-        <v>172</v>
+        <v>171</v>
       </c>
       <c r="S44" t="s">
-        <v>175</v>
+        <v>174</v>
       </c>
       <c r="T44" t="s">
-        <v>179</v>
+        <v>178</v>
       </c>
       <c r="U44" t="s">
         <v>28</v>
       </c>
-      <c r="V44" s="1">
+      <c r="V44" s="2">
         <v>46199</v>
       </c>
     </row>
@@ -3288,7 +3311,7 @@
       <c r="G45" t="s">
         <v>44</v>
       </c>
-      <c r="H45" s="1">
+      <c r="H45" s="2">
         <v>46213</v>
       </c>
       <c r="I45" t="s">
@@ -3298,30 +3321,30 @@
         <v>69</v>
       </c>
       <c r="N45" t="s">
-        <v>87</v>
+        <v>86</v>
       </c>
       <c r="O45" t="s">
-        <v>135</v>
+        <v>134</v>
       </c>
       <c r="P45">
         <v>173846.38</v>
       </c>
       <c r="Q45" t="s">
-        <v>170</v>
+        <v>169</v>
       </c>
       <c r="R45" t="s">
-        <v>173</v>
+        <v>172</v>
       </c>
       <c r="S45" t="s">
-        <v>175</v>
+        <v>174</v>
       </c>
       <c r="T45" t="s">
-        <v>180</v>
+        <v>179</v>
       </c>
       <c r="U45" t="s">
-        <v>183</v>
-      </c>
-      <c r="V45" s="1">
+        <v>182</v>
+      </c>
+      <c r="V45" s="2">
         <v>46229</v>
       </c>
     </row>
@@ -3347,37 +3370,37 @@
       <c r="G46" t="s">
         <v>44</v>
       </c>
-      <c r="H46" s="1">
+      <c r="H46" s="2">
         <v>46210</v>
       </c>
       <c r="I46" t="s">
         <v>55</v>
       </c>
       <c r="N46" t="s">
-        <v>87</v>
+        <v>86</v>
       </c>
       <c r="O46" t="s">
-        <v>135</v>
+        <v>134</v>
       </c>
       <c r="P46">
         <v>1530656.62</v>
       </c>
       <c r="Q46" t="s">
-        <v>170</v>
+        <v>169</v>
       </c>
       <c r="R46" t="s">
-        <v>173</v>
+        <v>172</v>
       </c>
       <c r="S46" t="s">
-        <v>175</v>
+        <v>174</v>
       </c>
       <c r="T46" t="s">
-        <v>180</v>
+        <v>179</v>
       </c>
       <c r="U46" t="s">
-        <v>183</v>
-      </c>
-      <c r="V46" s="1">
+        <v>182</v>
+      </c>
+      <c r="V46" s="2">
         <v>46229</v>
       </c>
     </row>
@@ -3401,30 +3424,30 @@
         <v>30</v>
       </c>
       <c r="N47" t="s">
-        <v>89</v>
+        <v>88</v>
       </c>
       <c r="O47" t="s">
-        <v>136</v>
+        <v>135</v>
       </c>
       <c r="P47">
         <v>1000000</v>
       </c>
       <c r="Q47" t="s">
-        <v>170</v>
+        <v>169</v>
       </c>
       <c r="R47" t="s">
-        <v>172</v>
+        <v>171</v>
       </c>
       <c r="S47" t="s">
-        <v>175</v>
+        <v>174</v>
       </c>
       <c r="T47" t="s">
-        <v>179</v>
+        <v>178</v>
       </c>
       <c r="U47" t="s">
         <v>28</v>
       </c>
-      <c r="V47" s="1">
+      <c r="V47" s="2">
         <v>46321</v>
       </c>
     </row>
@@ -3454,30 +3477,30 @@
         <v>73</v>
       </c>
       <c r="N48" t="s">
-        <v>82</v>
+        <v>81</v>
       </c>
       <c r="O48" t="s">
-        <v>137</v>
+        <v>136</v>
       </c>
       <c r="P48">
         <v>958040</v>
       </c>
       <c r="Q48" t="s">
-        <v>169</v>
+        <v>168</v>
       </c>
       <c r="R48" t="s">
-        <v>172</v>
+        <v>171</v>
       </c>
       <c r="S48" t="s">
-        <v>175</v>
+        <v>174</v>
       </c>
       <c r="T48" t="s">
-        <v>178</v>
+        <v>177</v>
       </c>
       <c r="U48" t="s">
-        <v>183</v>
-      </c>
-      <c r="V48" s="1">
+        <v>182</v>
+      </c>
+      <c r="V48" s="2">
         <v>46291</v>
       </c>
     </row>
@@ -3503,7 +3526,7 @@
       <c r="G49" t="s">
         <v>44</v>
       </c>
-      <c r="H49" s="1">
+      <c r="H49" s="2">
         <v>46176</v>
       </c>
       <c r="I49" t="s">
@@ -3513,30 +3536,30 @@
         <v>70</v>
       </c>
       <c r="N49" t="s">
-        <v>82</v>
+        <v>81</v>
       </c>
       <c r="O49" t="s">
-        <v>137</v>
+        <v>136</v>
       </c>
       <c r="P49">
         <v>41730.64</v>
       </c>
       <c r="Q49" t="s">
-        <v>169</v>
+        <v>168</v>
       </c>
       <c r="R49" t="s">
-        <v>174</v>
+        <v>173</v>
       </c>
       <c r="S49" t="s">
-        <v>175</v>
+        <v>174</v>
       </c>
       <c r="T49" t="s">
-        <v>178</v>
+        <v>177</v>
       </c>
       <c r="U49" t="s">
-        <v>183</v>
-      </c>
-      <c r="V49" s="1">
+        <v>182</v>
+      </c>
+      <c r="V49" s="2">
         <v>46199</v>
       </c>
     </row>
@@ -3559,37 +3582,37 @@
       <c r="G50" t="s">
         <v>44</v>
       </c>
-      <c r="H50" s="1">
+      <c r="H50" s="2">
         <v>46280</v>
       </c>
       <c r="I50" t="s">
         <v>55</v>
       </c>
       <c r="N50" t="s">
-        <v>87</v>
+        <v>86</v>
       </c>
       <c r="O50" t="s">
-        <v>138</v>
+        <v>137</v>
       </c>
       <c r="P50">
         <v>859536.0699999999</v>
       </c>
       <c r="Q50" t="s">
-        <v>170</v>
+        <v>169</v>
       </c>
       <c r="R50" t="s">
-        <v>173</v>
+        <v>172</v>
       </c>
       <c r="S50" t="s">
-        <v>175</v>
+        <v>174</v>
       </c>
       <c r="T50" t="s">
-        <v>180</v>
+        <v>179</v>
       </c>
       <c r="U50" t="s">
-        <v>183</v>
-      </c>
-      <c r="V50" s="1">
+        <v>182</v>
+      </c>
+      <c r="V50" s="2">
         <v>46260</v>
       </c>
     </row>
@@ -3619,30 +3642,30 @@
         <v>75</v>
       </c>
       <c r="N51" t="s">
-        <v>87</v>
+        <v>86</v>
       </c>
       <c r="O51" t="s">
-        <v>138</v>
+        <v>137</v>
       </c>
       <c r="P51">
         <v>608623.25</v>
       </c>
       <c r="Q51" t="s">
-        <v>170</v>
+        <v>169</v>
       </c>
       <c r="R51" t="s">
-        <v>173</v>
+        <v>172</v>
       </c>
       <c r="S51" t="s">
-        <v>175</v>
+        <v>174</v>
       </c>
       <c r="T51" t="s">
-        <v>180</v>
+        <v>179</v>
       </c>
       <c r="U51" t="s">
-        <v>183</v>
-      </c>
-      <c r="V51" s="1">
+        <v>182</v>
+      </c>
+      <c r="V51" s="2">
         <v>46260</v>
       </c>
     </row>
@@ -3669,33 +3692,33 @@
         <v>69</v>
       </c>
       <c r="K52" t="s">
-        <v>76</v>
+        <v>72</v>
       </c>
       <c r="N52" t="s">
-        <v>87</v>
+        <v>86</v>
       </c>
       <c r="O52" t="s">
-        <v>139</v>
+        <v>138</v>
       </c>
       <c r="P52">
         <v>559040.0699999999</v>
       </c>
       <c r="Q52" t="s">
-        <v>170</v>
+        <v>169</v>
       </c>
       <c r="R52" t="s">
-        <v>173</v>
+        <v>172</v>
       </c>
       <c r="S52" t="s">
-        <v>175</v>
+        <v>174</v>
       </c>
       <c r="T52" t="s">
-        <v>180</v>
+        <v>179</v>
       </c>
       <c r="U52" t="s">
-        <v>183</v>
-      </c>
-      <c r="V52" s="1">
+        <v>182</v>
+      </c>
+      <c r="V52" s="2">
         <v>46291</v>
       </c>
     </row>
@@ -3722,30 +3745,30 @@
         <v>74</v>
       </c>
       <c r="N53" t="s">
-        <v>87</v>
+        <v>86</v>
       </c>
       <c r="O53" t="s">
-        <v>140</v>
+        <v>139</v>
       </c>
       <c r="P53">
         <v>1704503</v>
       </c>
       <c r="Q53" t="s">
-        <v>170</v>
+        <v>169</v>
       </c>
       <c r="R53" t="s">
-        <v>173</v>
+        <v>172</v>
       </c>
       <c r="S53" t="s">
-        <v>175</v>
+        <v>174</v>
       </c>
       <c r="T53" t="s">
-        <v>180</v>
+        <v>179</v>
       </c>
       <c r="U53" t="s">
-        <v>183</v>
-      </c>
-      <c r="V53" s="1">
+        <v>182</v>
+      </c>
+      <c r="V53" s="2">
         <v>46321</v>
       </c>
     </row>
@@ -3771,37 +3794,37 @@
       <c r="G54" t="s">
         <v>44</v>
       </c>
-      <c r="H54" s="1">
+      <c r="H54" s="2">
         <v>46227</v>
       </c>
       <c r="I54" t="s">
         <v>63</v>
       </c>
       <c r="N54" t="s">
-        <v>87</v>
+        <v>86</v>
       </c>
       <c r="O54" t="s">
-        <v>138</v>
+        <v>137</v>
       </c>
       <c r="P54">
         <v>236343.68</v>
       </c>
       <c r="Q54" t="s">
-        <v>170</v>
+        <v>169</v>
       </c>
       <c r="R54" t="s">
-        <v>173</v>
+        <v>172</v>
       </c>
       <c r="S54" t="s">
-        <v>175</v>
+        <v>174</v>
       </c>
       <c r="T54" t="s">
-        <v>180</v>
+        <v>179</v>
       </c>
       <c r="U54" t="s">
-        <v>183</v>
-      </c>
-      <c r="V54" s="1">
+        <v>182</v>
+      </c>
+      <c r="V54" s="2">
         <v>46229</v>
       </c>
     </row>
@@ -3824,37 +3847,37 @@
       <c r="G55" t="s">
         <v>44</v>
       </c>
-      <c r="H55" s="1">
+      <c r="H55" s="2">
         <v>46280</v>
       </c>
       <c r="I55" t="s">
         <v>55</v>
       </c>
       <c r="N55" t="s">
-        <v>87</v>
+        <v>86</v>
       </c>
       <c r="O55" t="s">
-        <v>139</v>
+        <v>138</v>
       </c>
       <c r="P55">
         <v>1145462.93</v>
       </c>
       <c r="Q55" t="s">
-        <v>170</v>
+        <v>169</v>
       </c>
       <c r="R55" t="s">
-        <v>173</v>
+        <v>172</v>
       </c>
       <c r="S55" t="s">
-        <v>175</v>
+        <v>174</v>
       </c>
       <c r="T55" t="s">
-        <v>180</v>
+        <v>179</v>
       </c>
       <c r="U55" t="s">
-        <v>183</v>
-      </c>
-      <c r="V55" s="1">
+        <v>182</v>
+      </c>
+      <c r="V55" s="2">
         <v>46291</v>
       </c>
     </row>
@@ -3881,33 +3904,33 @@
         <v>64</v>
       </c>
       <c r="K56" t="s">
-        <v>77</v>
+        <v>76</v>
       </c>
       <c r="N56" t="s">
-        <v>87</v>
+        <v>86</v>
       </c>
       <c r="O56" t="s">
-        <v>141</v>
+        <v>140</v>
       </c>
       <c r="P56">
         <v>1295422.28</v>
       </c>
       <c r="Q56" t="s">
-        <v>170</v>
+        <v>169</v>
       </c>
       <c r="R56" t="s">
-        <v>173</v>
+        <v>172</v>
       </c>
       <c r="S56" t="s">
-        <v>175</v>
+        <v>174</v>
       </c>
       <c r="T56" t="s">
-        <v>180</v>
+        <v>179</v>
       </c>
       <c r="U56" t="s">
-        <v>183</v>
-      </c>
-      <c r="V56" s="1">
+        <v>182</v>
+      </c>
+      <c r="V56" s="2">
         <v>46352</v>
       </c>
     </row>
@@ -3934,33 +3957,33 @@
         <v>64</v>
       </c>
       <c r="K57" t="s">
-        <v>78</v>
+        <v>77</v>
       </c>
       <c r="N57" t="s">
-        <v>91</v>
+        <v>90</v>
       </c>
       <c r="O57" t="s">
-        <v>142</v>
+        <v>141</v>
       </c>
       <c r="P57">
         <v>1962977.67</v>
       </c>
       <c r="Q57" t="s">
-        <v>170</v>
+        <v>169</v>
       </c>
       <c r="R57" t="s">
-        <v>173</v>
+        <v>172</v>
       </c>
       <c r="S57" t="s">
-        <v>177</v>
+        <v>176</v>
       </c>
       <c r="T57" t="s">
-        <v>181</v>
+        <v>180</v>
       </c>
       <c r="U57" t="s">
-        <v>183</v>
-      </c>
-      <c r="V57" s="1">
+        <v>182</v>
+      </c>
+      <c r="V57" s="2">
         <v>46321</v>
       </c>
     </row>
@@ -3984,30 +4007,30 @@
         <v>45</v>
       </c>
       <c r="N58" t="s">
-        <v>91</v>
+        <v>90</v>
       </c>
       <c r="O58" t="s">
-        <v>142</v>
+        <v>141</v>
       </c>
       <c r="P58">
         <v>2497091</v>
       </c>
       <c r="Q58" t="s">
-        <v>170</v>
+        <v>169</v>
       </c>
       <c r="R58" t="s">
-        <v>173</v>
+        <v>172</v>
       </c>
       <c r="S58" t="s">
-        <v>177</v>
+        <v>176</v>
       </c>
       <c r="T58" t="s">
-        <v>181</v>
+        <v>180</v>
       </c>
       <c r="U58" t="s">
-        <v>183</v>
-      </c>
-      <c r="V58" s="1">
+        <v>182</v>
+      </c>
+      <c r="V58" s="2">
         <v>46321</v>
       </c>
     </row>
@@ -4031,27 +4054,27 @@
         <v>43</v>
       </c>
       <c r="N59" t="s">
-        <v>91</v>
+        <v>90</v>
       </c>
       <c r="O59" t="s">
-        <v>143</v>
+        <v>142</v>
       </c>
       <c r="Q59" t="s">
-        <v>170</v>
+        <v>169</v>
       </c>
       <c r="R59" t="s">
-        <v>173</v>
+        <v>172</v>
       </c>
       <c r="S59" t="s">
-        <v>177</v>
+        <v>176</v>
       </c>
       <c r="T59" t="s">
-        <v>181</v>
+        <v>180</v>
       </c>
       <c r="U59" t="s">
-        <v>183</v>
-      </c>
-      <c r="V59" s="1">
+        <v>182</v>
+      </c>
+      <c r="V59" s="2">
         <v>46049</v>
       </c>
     </row>
@@ -4075,25 +4098,25 @@
         <v>43</v>
       </c>
       <c r="N60" t="s">
-        <v>91</v>
+        <v>90</v>
       </c>
       <c r="O60" t="s">
-        <v>144</v>
+        <v>143</v>
       </c>
       <c r="Q60" t="s">
-        <v>170</v>
+        <v>169</v>
       </c>
       <c r="R60" t="s">
-        <v>173</v>
+        <v>172</v>
       </c>
       <c r="S60" t="s">
-        <v>177</v>
+        <v>176</v>
       </c>
       <c r="T60" t="s">
-        <v>181</v>
+        <v>180</v>
       </c>
       <c r="U60" t="s">
-        <v>183</v>
+        <v>182</v>
       </c>
     </row>
     <row r="61" spans="1:22">
@@ -4116,25 +4139,25 @@
         <v>43</v>
       </c>
       <c r="N61" t="s">
-        <v>91</v>
+        <v>90</v>
       </c>
       <c r="O61" t="s">
-        <v>145</v>
+        <v>144</v>
       </c>
       <c r="Q61" t="s">
-        <v>170</v>
+        <v>169</v>
       </c>
       <c r="R61" t="s">
-        <v>173</v>
+        <v>172</v>
       </c>
       <c r="S61" t="s">
-        <v>177</v>
+        <v>176</v>
       </c>
       <c r="T61" t="s">
-        <v>181</v>
+        <v>180</v>
       </c>
       <c r="U61" t="s">
-        <v>183</v>
+        <v>182</v>
       </c>
     </row>
     <row r="62" spans="1:22">
@@ -4154,30 +4177,30 @@
         <v>29</v>
       </c>
       <c r="N62" t="s">
-        <v>92</v>
+        <v>91</v>
       </c>
       <c r="O62" t="s">
-        <v>146</v>
+        <v>145</v>
       </c>
       <c r="P62">
         <v>9389.959999999999</v>
       </c>
       <c r="Q62" t="s">
-        <v>169</v>
+        <v>168</v>
       </c>
       <c r="R62" t="s">
-        <v>174</v>
+        <v>173</v>
       </c>
       <c r="S62" t="s">
-        <v>176</v>
+        <v>175</v>
       </c>
       <c r="T62" t="s">
-        <v>178</v>
+        <v>177</v>
       </c>
       <c r="U62" t="s">
-        <v>183</v>
-      </c>
-      <c r="V62" s="1">
+        <v>182</v>
+      </c>
+      <c r="V62" s="2">
         <v>46107</v>
       </c>
     </row>
@@ -4198,30 +4221,30 @@
         <v>29</v>
       </c>
       <c r="N63" t="s">
-        <v>93</v>
+        <v>92</v>
       </c>
       <c r="O63" t="s">
-        <v>147</v>
+        <v>146</v>
       </c>
       <c r="P63">
         <v>7204.82</v>
       </c>
       <c r="Q63" t="s">
-        <v>169</v>
+        <v>168</v>
       </c>
       <c r="R63" t="s">
-        <v>174</v>
+        <v>173</v>
       </c>
       <c r="S63" t="s">
-        <v>176</v>
+        <v>175</v>
       </c>
       <c r="T63" t="s">
-        <v>178</v>
+        <v>177</v>
       </c>
       <c r="U63" t="s">
-        <v>183</v>
-      </c>
-      <c r="V63" s="1">
+        <v>182</v>
+      </c>
+      <c r="V63" s="2">
         <v>46107</v>
       </c>
     </row>
@@ -4242,30 +4265,30 @@
         <v>29</v>
       </c>
       <c r="N64" t="s">
-        <v>94</v>
+        <v>93</v>
       </c>
       <c r="O64" t="s">
-        <v>148</v>
+        <v>147</v>
       </c>
       <c r="P64">
         <v>4227.84</v>
       </c>
       <c r="Q64" t="s">
-        <v>169</v>
+        <v>168</v>
       </c>
       <c r="R64" t="s">
-        <v>174</v>
+        <v>173</v>
       </c>
       <c r="S64" t="s">
-        <v>176</v>
+        <v>175</v>
       </c>
       <c r="T64" t="s">
-        <v>178</v>
+        <v>177</v>
       </c>
       <c r="U64" t="s">
-        <v>183</v>
-      </c>
-      <c r="V64" s="1">
+        <v>182</v>
+      </c>
+      <c r="V64" s="2">
         <v>46107</v>
       </c>
     </row>
@@ -4286,30 +4309,30 @@
         <v>29</v>
       </c>
       <c r="N65" t="s">
-        <v>95</v>
+        <v>94</v>
       </c>
       <c r="O65" t="s">
-        <v>149</v>
+        <v>148</v>
       </c>
       <c r="P65">
         <v>4064.54</v>
       </c>
       <c r="Q65" t="s">
-        <v>170</v>
+        <v>169</v>
       </c>
       <c r="R65" t="s">
-        <v>174</v>
+        <v>173</v>
       </c>
       <c r="S65" t="s">
-        <v>176</v>
+        <v>175</v>
       </c>
       <c r="T65" t="s">
-        <v>178</v>
+        <v>177</v>
       </c>
       <c r="U65" t="s">
-        <v>183</v>
-      </c>
-      <c r="V65" s="1">
+        <v>182</v>
+      </c>
+      <c r="V65" s="2">
         <v>46107</v>
       </c>
     </row>
@@ -4330,30 +4353,30 @@
         <v>29</v>
       </c>
       <c r="N66" t="s">
-        <v>96</v>
+        <v>95</v>
       </c>
       <c r="O66" t="s">
-        <v>148</v>
+        <v>147</v>
       </c>
       <c r="P66">
         <v>3662.66</v>
       </c>
       <c r="Q66" t="s">
-        <v>169</v>
+        <v>168</v>
       </c>
       <c r="R66" t="s">
-        <v>174</v>
+        <v>173</v>
       </c>
       <c r="S66" t="s">
-        <v>176</v>
+        <v>175</v>
       </c>
       <c r="T66" t="s">
-        <v>178</v>
+        <v>177</v>
       </c>
       <c r="U66" t="s">
-        <v>183</v>
-      </c>
-      <c r="V66" s="1">
+        <v>182</v>
+      </c>
+      <c r="V66" s="2">
         <v>46107</v>
       </c>
     </row>
@@ -4374,30 +4397,30 @@
         <v>29</v>
       </c>
       <c r="N67" t="s">
-        <v>97</v>
+        <v>96</v>
       </c>
       <c r="O67" t="s">
-        <v>150</v>
+        <v>149</v>
       </c>
       <c r="P67">
         <v>1163.64</v>
       </c>
       <c r="Q67" t="s">
-        <v>171</v>
+        <v>170</v>
       </c>
       <c r="R67" t="s">
-        <v>174</v>
+        <v>173</v>
       </c>
       <c r="S67" t="s">
-        <v>176</v>
+        <v>175</v>
       </c>
       <c r="T67" t="s">
-        <v>178</v>
+        <v>177</v>
       </c>
       <c r="U67" t="s">
-        <v>183</v>
-      </c>
-      <c r="V67" s="1">
+        <v>182</v>
+      </c>
+      <c r="V67" s="2">
         <v>46107</v>
       </c>
     </row>
@@ -4418,30 +4441,30 @@
         <v>29</v>
       </c>
       <c r="N68" t="s">
-        <v>83</v>
+        <v>82</v>
       </c>
       <c r="O68" t="s">
-        <v>151</v>
+        <v>150</v>
       </c>
       <c r="P68">
         <v>120000</v>
       </c>
       <c r="Q68" t="s">
-        <v>169</v>
+        <v>168</v>
       </c>
       <c r="R68" t="s">
-        <v>173</v>
+        <v>172</v>
       </c>
       <c r="S68" t="s">
-        <v>176</v>
+        <v>175</v>
       </c>
       <c r="T68" t="s">
-        <v>178</v>
+        <v>177</v>
       </c>
       <c r="U68" t="s">
         <v>28</v>
       </c>
-      <c r="V68" s="1">
+      <c r="V68" s="2">
         <v>46168</v>
       </c>
     </row>
@@ -4468,27 +4491,27 @@
         <v>43</v>
       </c>
       <c r="N69" t="s">
-        <v>82</v>
+        <v>81</v>
       </c>
       <c r="O69" t="s">
-        <v>152</v>
+        <v>151</v>
       </c>
       <c r="Q69" t="s">
-        <v>169</v>
+        <v>168</v>
       </c>
       <c r="R69" t="s">
-        <v>172</v>
+        <v>171</v>
       </c>
       <c r="S69" t="s">
-        <v>175</v>
+        <v>174</v>
       </c>
       <c r="T69" t="s">
-        <v>178</v>
+        <v>177</v>
       </c>
       <c r="U69" t="s">
         <v>28</v>
       </c>
-      <c r="V69" s="1">
+      <c r="V69" s="2">
         <v>46291</v>
       </c>
     </row>
@@ -4518,30 +4541,30 @@
         <v>73</v>
       </c>
       <c r="N70" t="s">
-        <v>86</v>
+        <v>85</v>
       </c>
       <c r="O70" t="s">
-        <v>153</v>
+        <v>152</v>
       </c>
       <c r="P70">
         <v>100000</v>
       </c>
       <c r="Q70" t="s">
+        <v>170</v>
+      </c>
+      <c r="R70" t="s">
         <v>171</v>
       </c>
-      <c r="R70" t="s">
-        <v>172</v>
-      </c>
       <c r="S70" t="s">
-        <v>175</v>
+        <v>174</v>
       </c>
       <c r="T70" t="s">
-        <v>178</v>
+        <v>177</v>
       </c>
       <c r="U70" t="s">
-        <v>183</v>
-      </c>
-      <c r="V70" s="1">
+        <v>182</v>
+      </c>
+      <c r="V70" s="2">
         <v>46229</v>
       </c>
     </row>
@@ -4562,30 +4585,30 @@
         <v>29</v>
       </c>
       <c r="N71" t="s">
-        <v>83</v>
+        <v>82</v>
       </c>
       <c r="O71" t="s">
-        <v>154</v>
+        <v>153</v>
       </c>
       <c r="P71">
         <v>80000</v>
       </c>
       <c r="Q71" t="s">
-        <v>169</v>
+        <v>168</v>
       </c>
       <c r="R71" t="s">
-        <v>173</v>
+        <v>172</v>
       </c>
       <c r="S71" t="s">
-        <v>176</v>
+        <v>175</v>
       </c>
       <c r="T71" t="s">
-        <v>178</v>
+        <v>177</v>
       </c>
       <c r="U71" t="s">
         <v>28</v>
       </c>
-      <c r="V71" s="1">
+      <c r="V71" s="2">
         <v>46260</v>
       </c>
     </row>
@@ -4606,30 +4629,30 @@
         <v>29</v>
       </c>
       <c r="N72" t="s">
-        <v>82</v>
+        <v>81</v>
       </c>
       <c r="O72" t="s">
-        <v>155</v>
+        <v>154</v>
       </c>
       <c r="P72">
         <v>835000</v>
       </c>
       <c r="Q72" t="s">
-        <v>169</v>
+        <v>168</v>
       </c>
       <c r="R72" t="s">
-        <v>172</v>
+        <v>171</v>
       </c>
       <c r="S72" t="s">
-        <v>176</v>
+        <v>175</v>
       </c>
       <c r="T72" t="s">
-        <v>178</v>
+        <v>177</v>
       </c>
       <c r="U72" t="s">
-        <v>183</v>
-      </c>
-      <c r="V72" s="1">
+        <v>182</v>
+      </c>
+      <c r="V72" s="2">
         <v>46291</v>
       </c>
     </row>
@@ -4650,30 +4673,30 @@
         <v>29</v>
       </c>
       <c r="N73" t="s">
-        <v>82</v>
+        <v>81</v>
       </c>
       <c r="O73" t="s">
-        <v>155</v>
+        <v>154</v>
       </c>
       <c r="P73">
         <v>165000</v>
       </c>
       <c r="Q73" t="s">
-        <v>169</v>
+        <v>168</v>
       </c>
       <c r="R73" t="s">
-        <v>172</v>
+        <v>171</v>
       </c>
       <c r="S73" t="s">
-        <v>176</v>
+        <v>175</v>
       </c>
       <c r="T73" t="s">
-        <v>178</v>
+        <v>177</v>
       </c>
       <c r="U73" t="s">
-        <v>183</v>
-      </c>
-      <c r="V73" s="1">
+        <v>182</v>
+      </c>
+      <c r="V73" s="2">
         <v>46168</v>
       </c>
     </row>
@@ -4694,30 +4717,30 @@
         <v>29</v>
       </c>
       <c r="N74" t="s">
-        <v>82</v>
+        <v>81</v>
       </c>
       <c r="O74" t="s">
-        <v>156</v>
+        <v>155</v>
       </c>
       <c r="P74">
         <v>1000000</v>
       </c>
       <c r="Q74" t="s">
-        <v>169</v>
+        <v>168</v>
       </c>
       <c r="R74" t="s">
-        <v>172</v>
+        <v>171</v>
       </c>
       <c r="S74" t="s">
-        <v>176</v>
+        <v>175</v>
       </c>
       <c r="T74" t="s">
-        <v>178</v>
+        <v>177</v>
       </c>
       <c r="U74" t="s">
-        <v>183</v>
-      </c>
-      <c r="V74" s="1">
+        <v>182</v>
+      </c>
+      <c r="V74" s="2">
         <v>46291</v>
       </c>
     </row>
@@ -4738,30 +4761,30 @@
         <v>29</v>
       </c>
       <c r="N75" t="s">
-        <v>82</v>
+        <v>81</v>
       </c>
       <c r="O75" t="s">
-        <v>157</v>
+        <v>156</v>
       </c>
       <c r="P75">
         <v>1000000</v>
       </c>
       <c r="Q75" t="s">
-        <v>169</v>
+        <v>168</v>
       </c>
       <c r="R75" t="s">
-        <v>172</v>
+        <v>171</v>
       </c>
       <c r="S75" t="s">
-        <v>176</v>
+        <v>175</v>
       </c>
       <c r="T75" t="s">
-        <v>178</v>
+        <v>177</v>
       </c>
       <c r="U75" t="s">
-        <v>183</v>
-      </c>
-      <c r="V75" s="1">
+        <v>182</v>
+      </c>
+      <c r="V75" s="2">
         <v>46291</v>
       </c>
     </row>
@@ -4782,30 +4805,30 @@
         <v>29</v>
       </c>
       <c r="N76" t="s">
-        <v>86</v>
+        <v>85</v>
       </c>
       <c r="O76" t="s">
-        <v>158</v>
+        <v>157</v>
       </c>
       <c r="P76">
         <v>100000</v>
       </c>
       <c r="Q76" t="s">
+        <v>170</v>
+      </c>
+      <c r="R76" t="s">
         <v>171</v>
       </c>
-      <c r="R76" t="s">
-        <v>172</v>
-      </c>
       <c r="S76" t="s">
-        <v>176</v>
+        <v>175</v>
       </c>
       <c r="T76" t="s">
-        <v>178</v>
+        <v>177</v>
       </c>
       <c r="U76" t="s">
-        <v>183</v>
-      </c>
-      <c r="V76" s="1">
+        <v>182</v>
+      </c>
+      <c r="V76" s="2">
         <v>46291</v>
       </c>
     </row>
@@ -4829,30 +4852,30 @@
         <v>30</v>
       </c>
       <c r="N77" t="s">
-        <v>89</v>
+        <v>88</v>
       </c>
       <c r="O77" t="s">
-        <v>159</v>
+        <v>158</v>
       </c>
       <c r="P77">
         <v>1000000</v>
       </c>
       <c r="Q77" t="s">
-        <v>170</v>
+        <v>169</v>
       </c>
       <c r="R77" t="s">
-        <v>172</v>
+        <v>171</v>
       </c>
       <c r="S77" t="s">
-        <v>175</v>
+        <v>174</v>
       </c>
       <c r="T77" t="s">
-        <v>179</v>
+        <v>178</v>
       </c>
       <c r="U77" t="s">
         <v>28</v>
       </c>
-      <c r="V77" s="1">
+      <c r="V77" s="2">
         <v>46321</v>
       </c>
     </row>
@@ -4879,30 +4902,30 @@
         <v>46</v>
       </c>
       <c r="N78" t="s">
-        <v>87</v>
+        <v>86</v>
       </c>
       <c r="O78" t="s">
-        <v>160</v>
+        <v>159</v>
       </c>
       <c r="P78">
         <v>1704503</v>
       </c>
       <c r="Q78" t="s">
-        <v>170</v>
+        <v>169</v>
       </c>
       <c r="R78" t="s">
-        <v>173</v>
+        <v>172</v>
       </c>
       <c r="S78" t="s">
         <v>42</v>
       </c>
       <c r="T78" t="s">
-        <v>180</v>
+        <v>179</v>
       </c>
       <c r="U78" t="s">
-        <v>183</v>
-      </c>
-      <c r="V78" s="1">
+        <v>182</v>
+      </c>
+      <c r="V78" s="2">
         <v>46381</v>
       </c>
     </row>
@@ -4929,30 +4952,30 @@
         <v>46</v>
       </c>
       <c r="N79" t="s">
-        <v>87</v>
+        <v>86</v>
       </c>
       <c r="O79" t="s">
-        <v>161</v>
+        <v>160</v>
       </c>
       <c r="P79">
         <v>1638125.5</v>
       </c>
       <c r="Q79" t="s">
-        <v>170</v>
+        <v>169</v>
       </c>
       <c r="R79" t="s">
-        <v>173</v>
+        <v>172</v>
       </c>
       <c r="S79" t="s">
         <v>42</v>
       </c>
       <c r="T79" t="s">
-        <v>180</v>
+        <v>179</v>
       </c>
       <c r="U79" t="s">
-        <v>183</v>
-      </c>
-      <c r="V79" s="1">
+        <v>182</v>
+      </c>
+      <c r="V79" s="2">
         <v>46381</v>
       </c>
     </row>
@@ -4979,30 +5002,30 @@
         <v>46</v>
       </c>
       <c r="N80" t="s">
-        <v>85</v>
+        <v>84</v>
       </c>
       <c r="O80" t="s">
-        <v>162</v>
+        <v>161</v>
       </c>
       <c r="P80">
         <v>3800000</v>
       </c>
       <c r="Q80" t="s">
-        <v>170</v>
+        <v>169</v>
       </c>
       <c r="R80" t="s">
-        <v>173</v>
+        <v>172</v>
       </c>
       <c r="S80" t="s">
         <v>42</v>
       </c>
       <c r="T80" t="s">
-        <v>179</v>
+        <v>178</v>
       </c>
       <c r="U80" t="s">
         <v>28</v>
       </c>
-      <c r="V80" s="1">
+      <c r="V80" s="2">
         <v>46381</v>
       </c>
     </row>
@@ -5029,30 +5052,30 @@
         <v>46</v>
       </c>
       <c r="N81" t="s">
-        <v>85</v>
+        <v>84</v>
       </c>
       <c r="O81" t="s">
-        <v>163</v>
+        <v>162</v>
       </c>
       <c r="P81">
         <v>3800000</v>
       </c>
       <c r="Q81" t="s">
-        <v>170</v>
+        <v>169</v>
       </c>
       <c r="R81" t="s">
-        <v>173</v>
+        <v>172</v>
       </c>
       <c r="S81" t="s">
         <v>42</v>
       </c>
       <c r="T81" t="s">
-        <v>179</v>
+        <v>178</v>
       </c>
       <c r="U81" t="s">
         <v>28</v>
       </c>
-      <c r="V81" s="1">
+      <c r="V81" s="2">
         <v>46381</v>
       </c>
     </row>
@@ -5076,33 +5099,33 @@
         <v>71</v>
       </c>
       <c r="K82" t="s">
-        <v>79</v>
+        <v>78</v>
       </c>
       <c r="N82" t="s">
-        <v>90</v>
+        <v>89</v>
       </c>
       <c r="O82" t="s">
-        <v>164</v>
+        <v>163</v>
       </c>
       <c r="P82">
         <v>3800000</v>
       </c>
       <c r="Q82" t="s">
-        <v>170</v>
+        <v>169</v>
       </c>
       <c r="R82" t="s">
-        <v>173</v>
+        <v>172</v>
       </c>
       <c r="S82" t="s">
-        <v>176</v>
+        <v>175</v>
       </c>
       <c r="T82" t="s">
-        <v>179</v>
+        <v>178</v>
       </c>
       <c r="U82" t="s">
         <v>28</v>
       </c>
-      <c r="V82" s="1">
+      <c r="V82" s="2">
         <v>46382</v>
       </c>
     </row>
@@ -5123,30 +5146,30 @@
         <v>28</v>
       </c>
       <c r="N83" t="s">
+        <v>97</v>
+      </c>
+      <c r="O83" t="s">
         <v>98</v>
-      </c>
-      <c r="O83" t="s">
-        <v>99</v>
       </c>
       <c r="P83">
         <v>4394700</v>
       </c>
       <c r="Q83" t="s">
-        <v>169</v>
+        <v>168</v>
       </c>
       <c r="R83" t="s">
-        <v>172</v>
+        <v>171</v>
       </c>
       <c r="S83" t="s">
-        <v>176</v>
+        <v>175</v>
       </c>
       <c r="T83" t="s">
-        <v>179</v>
+        <v>178</v>
       </c>
       <c r="U83" t="s">
         <v>28</v>
       </c>
-      <c r="V83" s="1">
+      <c r="V83" s="2">
         <v>46382</v>
       </c>
     </row>
@@ -5173,33 +5196,33 @@
         <v>64</v>
       </c>
       <c r="K84" t="s">
-        <v>80</v>
+        <v>79</v>
       </c>
       <c r="N84" t="s">
-        <v>87</v>
+        <v>86</v>
       </c>
       <c r="O84" t="s">
-        <v>165</v>
+        <v>164</v>
       </c>
       <c r="P84">
         <v>528395.9300000001</v>
       </c>
       <c r="Q84" t="s">
-        <v>170</v>
+        <v>169</v>
       </c>
       <c r="R84" t="s">
-        <v>173</v>
+        <v>172</v>
       </c>
       <c r="S84" t="s">
-        <v>175</v>
+        <v>174</v>
       </c>
       <c r="T84" t="s">
-        <v>180</v>
+        <v>179</v>
       </c>
       <c r="U84" t="s">
-        <v>183</v>
-      </c>
-      <c r="V84" s="1">
+        <v>182</v>
+      </c>
+      <c r="V84" s="2">
         <v>46382</v>
       </c>
     </row>
@@ -5223,30 +5246,30 @@
         <v>30</v>
       </c>
       <c r="N85" t="s">
-        <v>89</v>
+        <v>88</v>
       </c>
       <c r="O85" t="s">
-        <v>166</v>
+        <v>165</v>
       </c>
       <c r="P85">
         <v>1000000</v>
       </c>
       <c r="Q85" t="s">
-        <v>170</v>
+        <v>169</v>
       </c>
       <c r="R85" t="s">
-        <v>172</v>
+        <v>171</v>
       </c>
       <c r="S85" t="s">
-        <v>175</v>
+        <v>174</v>
       </c>
       <c r="T85" t="s">
-        <v>179</v>
+        <v>178</v>
       </c>
       <c r="U85" t="s">
         <v>28</v>
       </c>
-      <c r="V85" s="1">
+      <c r="V85" s="2">
         <v>46321</v>
       </c>
     </row>
@@ -5267,30 +5290,30 @@
         <v>28</v>
       </c>
       <c r="N86" t="s">
+        <v>97</v>
+      </c>
+      <c r="O86" t="s">
         <v>98</v>
-      </c>
-      <c r="O86" t="s">
-        <v>99</v>
       </c>
       <c r="P86">
         <v>4394700</v>
       </c>
       <c r="Q86" t="s">
-        <v>169</v>
+        <v>168</v>
       </c>
       <c r="R86" t="s">
-        <v>172</v>
+        <v>171</v>
       </c>
       <c r="S86" t="s">
-        <v>176</v>
+        <v>175</v>
       </c>
       <c r="T86" t="s">
-        <v>179</v>
+        <v>178</v>
       </c>
       <c r="U86" t="s">
         <v>28</v>
       </c>
-      <c r="V86" s="1">
+      <c r="V86" s="2">
         <v>46382</v>
       </c>
     </row>
@@ -5317,25 +5340,25 @@
         <v>46</v>
       </c>
       <c r="N87" t="s">
-        <v>99</v>
+        <v>98</v>
       </c>
       <c r="O87" t="s">
-        <v>99</v>
+        <v>98</v>
       </c>
       <c r="P87">
         <v>3306000</v>
       </c>
       <c r="Q87" t="s">
-        <v>169</v>
+        <v>168</v>
       </c>
       <c r="R87" t="s">
-        <v>172</v>
+        <v>171</v>
       </c>
       <c r="S87" t="s">
         <v>42</v>
       </c>
       <c r="T87" t="s">
-        <v>179</v>
+        <v>178</v>
       </c>
       <c r="U87" t="s">
         <v>28</v>
@@ -5364,25 +5387,25 @@
         <v>46</v>
       </c>
       <c r="N88" t="s">
-        <v>99</v>
+        <v>98</v>
       </c>
       <c r="O88" t="s">
-        <v>99</v>
+        <v>98</v>
       </c>
       <c r="P88">
         <v>3306000</v>
       </c>
       <c r="Q88" t="s">
-        <v>169</v>
+        <v>168</v>
       </c>
       <c r="R88" t="s">
-        <v>172</v>
+        <v>171</v>
       </c>
       <c r="S88" t="s">
         <v>42</v>
       </c>
       <c r="T88" t="s">
-        <v>179</v>
+        <v>178</v>
       </c>
       <c r="U88" t="s">
         <v>28</v>
@@ -5408,30 +5431,30 @@
         <v>30</v>
       </c>
       <c r="N89" t="s">
-        <v>100</v>
+        <v>99</v>
       </c>
       <c r="O89" t="s">
-        <v>167</v>
+        <v>166</v>
       </c>
       <c r="P89">
         <v>470820</v>
       </c>
       <c r="Q89" t="s">
-        <v>169</v>
+        <v>168</v>
       </c>
       <c r="R89" t="s">
-        <v>172</v>
+        <v>171</v>
       </c>
       <c r="S89" t="s">
-        <v>175</v>
+        <v>174</v>
       </c>
       <c r="T89" t="s">
-        <v>182</v>
+        <v>181</v>
       </c>
       <c r="U89" t="s">
         <v>28</v>
       </c>
-      <c r="V89" s="1">
+      <c r="V89" s="2">
         <v>46291</v>
       </c>
     </row>
@@ -5452,30 +5475,30 @@
         <v>30</v>
       </c>
       <c r="N90" t="s">
-        <v>90</v>
+        <v>89</v>
       </c>
       <c r="O90" t="s">
-        <v>168</v>
+        <v>167</v>
       </c>
       <c r="P90">
         <v>2297180</v>
       </c>
       <c r="Q90" t="s">
-        <v>170</v>
+        <v>169</v>
       </c>
       <c r="R90" t="s">
-        <v>172</v>
+        <v>171</v>
       </c>
       <c r="S90" t="s">
-        <v>175</v>
+        <v>174</v>
       </c>
       <c r="T90" t="s">
-        <v>179</v>
+        <v>178</v>
       </c>
       <c r="U90" t="s">
         <v>28</v>
       </c>
-      <c r="V90" s="1">
+      <c r="V90" s="2">
         <v>46291</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Atualização automática: mta (23/09/2026 12:26)
</commit_message>
<xml_diff>
--- a/Projetos/02_Dados_Tratados/base_mta_tratada.xlsx
+++ b/Projetos/02_Dados_Tratados/base_mta_tratada.xlsx
@@ -572,16 +572,8 @@
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="YYYY-MM-DD HH:MM:SS"/>
   </numFmts>
-  <fonts count="2">
+  <fonts count="1">
     <font>
-      <sz val="11"/>
-      <color theme="1"/>
-      <name val="Calibri"/>
-      <family val="2"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <b/>
       <sz val="11"/>
       <color theme="1"/>
       <name val="Calibri"/>
@@ -597,7 +589,7 @@
       <patternFill patternType="gray125"/>
     </fill>
   </fills>
-  <borders count="2">
+  <borders count="1">
     <border>
       <left/>
       <right/>
@@ -605,30 +597,12 @@
       <bottom/>
       <diagonal/>
     </border>
-    <border>
-      <left style="thin">
-        <color auto="1"/>
-      </left>
-      <right style="thin">
-        <color auto="1"/>
-      </right>
-      <top style="thin">
-        <color auto="1"/>
-      </top>
-      <bottom style="thin">
-        <color auto="1"/>
-      </bottom>
-      <diagonal/>
-    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="3">
+  <cellXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top"/>
-    </xf>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
   </cellXfs>
   <cellStyles count="1">
@@ -928,70 +902,70 @@
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:22">
-      <c r="A1" s="1" t="s">
+      <c r="A1" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="1" t="s">
+      <c r="B1" t="s">
         <v>1</v>
       </c>
-      <c r="C1" s="1" t="s">
+      <c r="C1" t="s">
         <v>2</v>
       </c>
-      <c r="D1" s="1" t="s">
+      <c r="D1" t="s">
         <v>3</v>
       </c>
-      <c r="E1" s="1" t="s">
+      <c r="E1" t="s">
         <v>4</v>
       </c>
-      <c r="F1" s="1" t="s">
+      <c r="F1" t="s">
         <v>5</v>
       </c>
-      <c r="G1" s="1" t="s">
+      <c r="G1" t="s">
         <v>6</v>
       </c>
-      <c r="H1" s="1" t="s">
+      <c r="H1" t="s">
         <v>7</v>
       </c>
-      <c r="I1" s="1" t="s">
+      <c r="I1" t="s">
         <v>8</v>
       </c>
-      <c r="J1" s="1" t="s">
+      <c r="J1" t="s">
         <v>9</v>
       </c>
-      <c r="K1" s="1" t="s">
+      <c r="K1" t="s">
         <v>10</v>
       </c>
-      <c r="L1" s="1" t="s">
+      <c r="L1" t="s">
         <v>11</v>
       </c>
-      <c r="M1" s="1" t="s">
+      <c r="M1" t="s">
         <v>12</v>
       </c>
-      <c r="N1" s="1" t="s">
+      <c r="N1" t="s">
         <v>13</v>
       </c>
-      <c r="O1" s="1" t="s">
+      <c r="O1" t="s">
         <v>14</v>
       </c>
-      <c r="P1" s="1" t="s">
+      <c r="P1" t="s">
         <v>15</v>
       </c>
-      <c r="Q1" s="1" t="s">
+      <c r="Q1" t="s">
         <v>16</v>
       </c>
-      <c r="R1" s="1" t="s">
+      <c r="R1" t="s">
         <v>17</v>
       </c>
-      <c r="S1" s="1" t="s">
+      <c r="S1" t="s">
         <v>18</v>
       </c>
-      <c r="T1" s="1" t="s">
+      <c r="T1" t="s">
         <v>19</v>
       </c>
-      <c r="U1" s="1" t="s">
+      <c r="U1" t="s">
         <v>20</v>
       </c>
-      <c r="V1" s="1" t="s">
+      <c r="V1" t="s">
         <v>21</v>
       </c>
     </row>
@@ -1047,7 +1021,7 @@
       <c r="U2" t="s">
         <v>182</v>
       </c>
-      <c r="V2" s="2">
+      <c r="V2" s="1">
         <v>46229</v>
       </c>
     </row>
@@ -1094,7 +1068,7 @@
       <c r="U3" t="s">
         <v>28</v>
       </c>
-      <c r="V3" s="2">
+      <c r="V3" s="1">
         <v>46291</v>
       </c>
     </row>
@@ -1141,7 +1115,7 @@
       <c r="U4" t="s">
         <v>28</v>
       </c>
-      <c r="V4" s="2">
+      <c r="V4" s="1">
         <v>46321</v>
       </c>
     </row>
@@ -1188,7 +1162,7 @@
       <c r="U5" t="s">
         <v>28</v>
       </c>
-      <c r="V5" s="2">
+      <c r="V5" s="1">
         <v>46321</v>
       </c>
     </row>
@@ -1238,7 +1212,7 @@
       <c r="U6" t="s">
         <v>28</v>
       </c>
-      <c r="V6" s="2">
+      <c r="V6" s="1">
         <v>46291</v>
       </c>
     </row>
@@ -1264,7 +1238,7 @@
       <c r="G7" t="s">
         <v>44</v>
       </c>
-      <c r="H7" s="2">
+      <c r="H7" s="1">
         <v>46121</v>
       </c>
       <c r="I7" t="s">
@@ -1294,7 +1268,7 @@
       <c r="U7" t="s">
         <v>28</v>
       </c>
-      <c r="V7" s="2">
+      <c r="V7" s="1">
         <v>46138</v>
       </c>
     </row>
@@ -1341,7 +1315,7 @@
       <c r="U8" t="s">
         <v>28</v>
       </c>
-      <c r="V8" s="2">
+      <c r="V8" s="1">
         <v>46291</v>
       </c>
     </row>
@@ -1388,7 +1362,7 @@
       <c r="U9" t="s">
         <v>28</v>
       </c>
-      <c r="V9" s="2">
+      <c r="V9" s="1">
         <v>46291</v>
       </c>
     </row>
@@ -1435,7 +1409,7 @@
       <c r="U10" t="s">
         <v>28</v>
       </c>
-      <c r="V10" s="2">
+      <c r="V10" s="1">
         <v>46291</v>
       </c>
     </row>
@@ -1482,7 +1456,7 @@
       <c r="U11" t="s">
         <v>28</v>
       </c>
-      <c r="V11" s="2">
+      <c r="V11" s="1">
         <v>46291</v>
       </c>
     </row>
@@ -1508,7 +1482,7 @@
       <c r="G12" t="s">
         <v>44</v>
       </c>
-      <c r="H12" s="2">
+      <c r="H12" s="1">
         <v>46079</v>
       </c>
       <c r="I12" t="s">
@@ -1541,7 +1515,7 @@
       <c r="U12" t="s">
         <v>182</v>
       </c>
-      <c r="V12" s="2">
+      <c r="V12" s="1">
         <v>46079</v>
       </c>
     </row>
@@ -1594,7 +1568,7 @@
       <c r="U13" t="s">
         <v>182</v>
       </c>
-      <c r="V13" s="2">
+      <c r="V13" s="1">
         <v>46352</v>
       </c>
     </row>
@@ -1647,7 +1621,7 @@
       <c r="U14" t="s">
         <v>182</v>
       </c>
-      <c r="V14" s="2">
+      <c r="V14" s="1">
         <v>46352</v>
       </c>
     </row>
@@ -1700,7 +1674,7 @@
       <c r="U15" t="s">
         <v>182</v>
       </c>
-      <c r="V15" s="2">
+      <c r="V15" s="1">
         <v>46352</v>
       </c>
     </row>
@@ -1753,7 +1727,7 @@
       <c r="U16" t="s">
         <v>182</v>
       </c>
-      <c r="V16" s="2">
+      <c r="V16" s="1">
         <v>46229</v>
       </c>
     </row>
@@ -1779,7 +1753,7 @@
       <c r="G17" t="s">
         <v>44</v>
       </c>
-      <c r="H17" s="2">
+      <c r="H17" s="1">
         <v>46098</v>
       </c>
       <c r="I17" t="s">
@@ -1812,7 +1786,7 @@
       <c r="U17" t="s">
         <v>182</v>
       </c>
-      <c r="V17" s="2">
+      <c r="V17" s="1">
         <v>46107</v>
       </c>
     </row>
@@ -1838,7 +1812,7 @@
       <c r="G18" t="s">
         <v>44</v>
       </c>
-      <c r="H18" s="2">
+      <c r="H18" s="1">
         <v>46076</v>
       </c>
       <c r="I18" t="s">
@@ -1868,7 +1842,7 @@
       <c r="U18" t="s">
         <v>28</v>
       </c>
-      <c r="V18" s="2">
+      <c r="V18" s="1">
         <v>46079</v>
       </c>
     </row>
@@ -1894,7 +1868,7 @@
       <c r="G19" t="s">
         <v>44</v>
       </c>
-      <c r="H19" s="2">
+      <c r="H19" s="1">
         <v>46076</v>
       </c>
       <c r="I19" t="s">
@@ -1924,7 +1898,7 @@
       <c r="U19" t="s">
         <v>28</v>
       </c>
-      <c r="V19" s="2">
+      <c r="V19" s="1">
         <v>46079</v>
       </c>
     </row>
@@ -1971,7 +1945,7 @@
       <c r="U20" t="s">
         <v>28</v>
       </c>
-      <c r="V20" s="2">
+      <c r="V20" s="1">
         <v>46321</v>
       </c>
     </row>
@@ -2018,7 +1992,7 @@
       <c r="U21" t="s">
         <v>28</v>
       </c>
-      <c r="V21" s="2">
+      <c r="V21" s="1">
         <v>46321</v>
       </c>
     </row>
@@ -2065,7 +2039,7 @@
       <c r="U22" t="s">
         <v>28</v>
       </c>
-      <c r="V22" s="2">
+      <c r="V22" s="1">
         <v>46321</v>
       </c>
     </row>
@@ -2112,7 +2086,7 @@
       <c r="U23" t="s">
         <v>28</v>
       </c>
-      <c r="V23" s="2">
+      <c r="V23" s="1">
         <v>46321</v>
       </c>
     </row>
@@ -2138,7 +2112,7 @@
       <c r="G24" t="s">
         <v>44</v>
       </c>
-      <c r="H24" s="2">
+      <c r="H24" s="1">
         <v>46119</v>
       </c>
       <c r="I24" t="s">
@@ -2171,7 +2145,7 @@
       <c r="U24" t="s">
         <v>182</v>
       </c>
-      <c r="V24" s="2">
+      <c r="V24" s="1">
         <v>46138</v>
       </c>
     </row>
@@ -2197,7 +2171,7 @@
       <c r="G25" t="s">
         <v>44</v>
       </c>
-      <c r="H25" s="2">
+      <c r="H25" s="1">
         <v>46121</v>
       </c>
       <c r="I25" t="s">
@@ -2227,7 +2201,7 @@
       <c r="U25" t="s">
         <v>28</v>
       </c>
-      <c r="V25" s="2">
+      <c r="V25" s="1">
         <v>46138</v>
       </c>
     </row>
@@ -2253,7 +2227,7 @@
       <c r="G26" t="s">
         <v>44</v>
       </c>
-      <c r="H26" s="2">
+      <c r="H26" s="1">
         <v>46076</v>
       </c>
       <c r="I26" t="s">
@@ -2283,7 +2257,7 @@
       <c r="U26" t="s">
         <v>28</v>
       </c>
-      <c r="V26" s="2">
+      <c r="V26" s="1">
         <v>46079</v>
       </c>
     </row>
@@ -2336,7 +2310,7 @@
       <c r="U27" t="s">
         <v>182</v>
       </c>
-      <c r="V27" s="2">
+      <c r="V27" s="1">
         <v>46291</v>
       </c>
     </row>
@@ -2362,7 +2336,7 @@
       <c r="G28" t="s">
         <v>44</v>
       </c>
-      <c r="H28" s="2">
+      <c r="H28" s="1">
         <v>46199</v>
       </c>
       <c r="I28" t="s">
@@ -2395,7 +2369,7 @@
       <c r="U28" t="s">
         <v>182</v>
       </c>
-      <c r="V28" s="2">
+      <c r="V28" s="1">
         <v>46199</v>
       </c>
     </row>
@@ -2421,7 +2395,7 @@
       <c r="G29" t="s">
         <v>44</v>
       </c>
-      <c r="H29" s="2">
+      <c r="H29" s="1">
         <v>46199</v>
       </c>
       <c r="I29" t="s">
@@ -2454,7 +2428,7 @@
       <c r="U29" t="s">
         <v>182</v>
       </c>
-      <c r="V29" s="2">
+      <c r="V29" s="1">
         <v>46199</v>
       </c>
     </row>
@@ -2480,7 +2454,7 @@
       <c r="G30" t="s">
         <v>44</v>
       </c>
-      <c r="H30" s="2">
+      <c r="H30" s="1">
         <v>46199</v>
       </c>
       <c r="I30" t="s">
@@ -2513,7 +2487,7 @@
       <c r="U30" t="s">
         <v>182</v>
       </c>
-      <c r="V30" s="2">
+      <c r="V30" s="1">
         <v>46199</v>
       </c>
     </row>
@@ -2539,7 +2513,7 @@
       <c r="G31" t="s">
         <v>44</v>
       </c>
-      <c r="H31" s="2">
+      <c r="H31" s="1">
         <v>46199</v>
       </c>
       <c r="I31" t="s">
@@ -2572,7 +2546,7 @@
       <c r="U31" t="s">
         <v>182</v>
       </c>
-      <c r="V31" s="2">
+      <c r="V31" s="1">
         <v>46199</v>
       </c>
     </row>
@@ -2622,7 +2596,7 @@
       <c r="U32" t="s">
         <v>182</v>
       </c>
-      <c r="V32" s="2">
+      <c r="V32" s="1">
         <v>46291</v>
       </c>
     </row>
@@ -2648,7 +2622,7 @@
       <c r="G33" t="s">
         <v>44</v>
       </c>
-      <c r="H33" s="2">
+      <c r="H33" s="1">
         <v>46191</v>
       </c>
       <c r="I33" t="s">
@@ -2681,7 +2655,7 @@
       <c r="U33" t="s">
         <v>182</v>
       </c>
-      <c r="V33" s="2">
+      <c r="V33" s="1">
         <v>46199</v>
       </c>
     </row>
@@ -2707,7 +2681,7 @@
       <c r="G34" t="s">
         <v>44</v>
       </c>
-      <c r="H34" s="2">
+      <c r="H34" s="1">
         <v>46119</v>
       </c>
       <c r="I34" t="s">
@@ -2737,7 +2711,7 @@
       <c r="U34" t="s">
         <v>182</v>
       </c>
-      <c r="V34" s="2">
+      <c r="V34" s="1">
         <v>46138</v>
       </c>
     </row>
@@ -2763,7 +2737,7 @@
       <c r="G35" t="s">
         <v>44</v>
       </c>
-      <c r="H35" s="2">
+      <c r="H35" s="1">
         <v>46213</v>
       </c>
       <c r="I35" t="s">
@@ -2793,7 +2767,7 @@
       <c r="U35" t="s">
         <v>28</v>
       </c>
-      <c r="V35" s="2">
+      <c r="V35" s="1">
         <v>46229</v>
       </c>
     </row>
@@ -2819,7 +2793,7 @@
       <c r="G36" t="s">
         <v>44</v>
       </c>
-      <c r="H36" s="2">
+      <c r="H36" s="1">
         <v>46175</v>
       </c>
       <c r="I36" t="s">
@@ -2849,7 +2823,7 @@
       <c r="U36" t="s">
         <v>28</v>
       </c>
-      <c r="V36" s="2">
+      <c r="V36" s="1">
         <v>46199</v>
       </c>
     </row>
@@ -2875,7 +2849,7 @@
       <c r="G37" t="s">
         <v>44</v>
       </c>
-      <c r="H37" s="2">
+      <c r="H37" s="1">
         <v>46213</v>
       </c>
       <c r="I37" t="s">
@@ -2905,7 +2879,7 @@
       <c r="U37" t="s">
         <v>28</v>
       </c>
-      <c r="V37" s="2">
+      <c r="V37" s="1">
         <v>46229</v>
       </c>
     </row>
@@ -2931,7 +2905,7 @@
       <c r="G38" t="s">
         <v>44</v>
       </c>
-      <c r="H38" s="2">
+      <c r="H38" s="1">
         <v>46199</v>
       </c>
       <c r="I38" t="s">
@@ -2961,7 +2935,7 @@
       <c r="U38" t="s">
         <v>28</v>
       </c>
-      <c r="V38" s="2">
+      <c r="V38" s="1">
         <v>46199</v>
       </c>
     </row>
@@ -2987,7 +2961,7 @@
       <c r="G39" t="s">
         <v>44</v>
       </c>
-      <c r="H39" s="2">
+      <c r="H39" s="1">
         <v>46199</v>
       </c>
       <c r="I39" t="s">
@@ -3017,7 +2991,7 @@
       <c r="U39" t="s">
         <v>28</v>
       </c>
-      <c r="V39" s="2">
+      <c r="V39" s="1">
         <v>46199</v>
       </c>
     </row>
@@ -3043,7 +3017,7 @@
       <c r="G40" t="s">
         <v>44</v>
       </c>
-      <c r="H40" s="2">
+      <c r="H40" s="1">
         <v>46204</v>
       </c>
       <c r="I40" t="s">
@@ -3073,7 +3047,7 @@
       <c r="U40" t="s">
         <v>28</v>
       </c>
-      <c r="V40" s="2">
+      <c r="V40" s="1">
         <v>46229</v>
       </c>
     </row>
@@ -3099,7 +3073,7 @@
       <c r="G41" t="s">
         <v>44</v>
       </c>
-      <c r="H41" s="2">
+      <c r="H41" s="1">
         <v>46244</v>
       </c>
       <c r="I41" t="s">
@@ -3129,7 +3103,7 @@
       <c r="U41" t="s">
         <v>28</v>
       </c>
-      <c r="V41" s="2">
+      <c r="V41" s="1">
         <v>46199</v>
       </c>
     </row>
@@ -3173,7 +3147,7 @@
       <c r="U42" t="s">
         <v>28</v>
       </c>
-      <c r="V42" s="2">
+      <c r="V42" s="1">
         <v>46260</v>
       </c>
     </row>
@@ -3199,7 +3173,7 @@
       <c r="G43" t="s">
         <v>44</v>
       </c>
-      <c r="H43" s="2">
+      <c r="H43" s="1">
         <v>46191</v>
       </c>
       <c r="I43" t="s">
@@ -3229,7 +3203,7 @@
       <c r="U43" t="s">
         <v>28</v>
       </c>
-      <c r="V43" s="2">
+      <c r="V43" s="1">
         <v>46199</v>
       </c>
     </row>
@@ -3255,7 +3229,7 @@
       <c r="G44" t="s">
         <v>44</v>
       </c>
-      <c r="H44" s="2">
+      <c r="H44" s="1">
         <v>46191</v>
       </c>
       <c r="I44" t="s">
@@ -3285,7 +3259,7 @@
       <c r="U44" t="s">
         <v>28</v>
       </c>
-      <c r="V44" s="2">
+      <c r="V44" s="1">
         <v>46199</v>
       </c>
     </row>
@@ -3311,7 +3285,7 @@
       <c r="G45" t="s">
         <v>44</v>
       </c>
-      <c r="H45" s="2">
+      <c r="H45" s="1">
         <v>46213</v>
       </c>
       <c r="I45" t="s">
@@ -3344,7 +3318,7 @@
       <c r="U45" t="s">
         <v>182</v>
       </c>
-      <c r="V45" s="2">
+      <c r="V45" s="1">
         <v>46229</v>
       </c>
     </row>
@@ -3370,7 +3344,7 @@
       <c r="G46" t="s">
         <v>44</v>
       </c>
-      <c r="H46" s="2">
+      <c r="H46" s="1">
         <v>46210</v>
       </c>
       <c r="I46" t="s">
@@ -3400,7 +3374,7 @@
       <c r="U46" t="s">
         <v>182</v>
       </c>
-      <c r="V46" s="2">
+      <c r="V46" s="1">
         <v>46229</v>
       </c>
     </row>
@@ -3447,7 +3421,7 @@
       <c r="U47" t="s">
         <v>28</v>
       </c>
-      <c r="V47" s="2">
+      <c r="V47" s="1">
         <v>46321</v>
       </c>
     </row>
@@ -3500,7 +3474,7 @@
       <c r="U48" t="s">
         <v>182</v>
       </c>
-      <c r="V48" s="2">
+      <c r="V48" s="1">
         <v>46291</v>
       </c>
     </row>
@@ -3526,7 +3500,7 @@
       <c r="G49" t="s">
         <v>44</v>
       </c>
-      <c r="H49" s="2">
+      <c r="H49" s="1">
         <v>46176</v>
       </c>
       <c r="I49" t="s">
@@ -3559,7 +3533,7 @@
       <c r="U49" t="s">
         <v>182</v>
       </c>
-      <c r="V49" s="2">
+      <c r="V49" s="1">
         <v>46199</v>
       </c>
     </row>
@@ -3582,7 +3556,7 @@
       <c r="G50" t="s">
         <v>44</v>
       </c>
-      <c r="H50" s="2">
+      <c r="H50" s="1">
         <v>46280</v>
       </c>
       <c r="I50" t="s">
@@ -3612,7 +3586,7 @@
       <c r="U50" t="s">
         <v>182</v>
       </c>
-      <c r="V50" s="2">
+      <c r="V50" s="1">
         <v>46260</v>
       </c>
     </row>
@@ -3665,7 +3639,7 @@
       <c r="U51" t="s">
         <v>182</v>
       </c>
-      <c r="V51" s="2">
+      <c r="V51" s="1">
         <v>46260</v>
       </c>
     </row>
@@ -3718,7 +3692,7 @@
       <c r="U52" t="s">
         <v>182</v>
       </c>
-      <c r="V52" s="2">
+      <c r="V52" s="1">
         <v>46291</v>
       </c>
     </row>
@@ -3768,7 +3742,7 @@
       <c r="U53" t="s">
         <v>182</v>
       </c>
-      <c r="V53" s="2">
+      <c r="V53" s="1">
         <v>46321</v>
       </c>
     </row>
@@ -3794,7 +3768,7 @@
       <c r="G54" t="s">
         <v>44</v>
       </c>
-      <c r="H54" s="2">
+      <c r="H54" s="1">
         <v>46227</v>
       </c>
       <c r="I54" t="s">
@@ -3824,7 +3798,7 @@
       <c r="U54" t="s">
         <v>182</v>
       </c>
-      <c r="V54" s="2">
+      <c r="V54" s="1">
         <v>46229</v>
       </c>
     </row>
@@ -3847,7 +3821,7 @@
       <c r="G55" t="s">
         <v>44</v>
       </c>
-      <c r="H55" s="2">
+      <c r="H55" s="1">
         <v>46280</v>
       </c>
       <c r="I55" t="s">
@@ -3877,7 +3851,7 @@
       <c r="U55" t="s">
         <v>182</v>
       </c>
-      <c r="V55" s="2">
+      <c r="V55" s="1">
         <v>46291</v>
       </c>
     </row>
@@ -3930,7 +3904,7 @@
       <c r="U56" t="s">
         <v>182</v>
       </c>
-      <c r="V56" s="2">
+      <c r="V56" s="1">
         <v>46352</v>
       </c>
     </row>
@@ -3983,7 +3957,7 @@
       <c r="U57" t="s">
         <v>182</v>
       </c>
-      <c r="V57" s="2">
+      <c r="V57" s="1">
         <v>46321</v>
       </c>
     </row>
@@ -4030,7 +4004,7 @@
       <c r="U58" t="s">
         <v>182</v>
       </c>
-      <c r="V58" s="2">
+      <c r="V58" s="1">
         <v>46321</v>
       </c>
     </row>
@@ -4074,7 +4048,7 @@
       <c r="U59" t="s">
         <v>182</v>
       </c>
-      <c r="V59" s="2">
+      <c r="V59" s="1">
         <v>46049</v>
       </c>
     </row>
@@ -4200,7 +4174,7 @@
       <c r="U62" t="s">
         <v>182</v>
       </c>
-      <c r="V62" s="2">
+      <c r="V62" s="1">
         <v>46107</v>
       </c>
     </row>
@@ -4244,7 +4218,7 @@
       <c r="U63" t="s">
         <v>182</v>
       </c>
-      <c r="V63" s="2">
+      <c r="V63" s="1">
         <v>46107</v>
       </c>
     </row>
@@ -4288,7 +4262,7 @@
       <c r="U64" t="s">
         <v>182</v>
       </c>
-      <c r="V64" s="2">
+      <c r="V64" s="1">
         <v>46107</v>
       </c>
     </row>
@@ -4332,7 +4306,7 @@
       <c r="U65" t="s">
         <v>182</v>
       </c>
-      <c r="V65" s="2">
+      <c r="V65" s="1">
         <v>46107</v>
       </c>
     </row>
@@ -4376,7 +4350,7 @@
       <c r="U66" t="s">
         <v>182</v>
       </c>
-      <c r="V66" s="2">
+      <c r="V66" s="1">
         <v>46107</v>
       </c>
     </row>
@@ -4420,7 +4394,7 @@
       <c r="U67" t="s">
         <v>182</v>
       </c>
-      <c r="V67" s="2">
+      <c r="V67" s="1">
         <v>46107</v>
       </c>
     </row>
@@ -4464,7 +4438,7 @@
       <c r="U68" t="s">
         <v>28</v>
       </c>
-      <c r="V68" s="2">
+      <c r="V68" s="1">
         <v>46168</v>
       </c>
     </row>
@@ -4511,7 +4485,7 @@
       <c r="U69" t="s">
         <v>28</v>
       </c>
-      <c r="V69" s="2">
+      <c r="V69" s="1">
         <v>46291</v>
       </c>
     </row>
@@ -4564,7 +4538,7 @@
       <c r="U70" t="s">
         <v>182</v>
       </c>
-      <c r="V70" s="2">
+      <c r="V70" s="1">
         <v>46229</v>
       </c>
     </row>
@@ -4608,7 +4582,7 @@
       <c r="U71" t="s">
         <v>28</v>
       </c>
-      <c r="V71" s="2">
+      <c r="V71" s="1">
         <v>46260</v>
       </c>
     </row>
@@ -4652,7 +4626,7 @@
       <c r="U72" t="s">
         <v>182</v>
       </c>
-      <c r="V72" s="2">
+      <c r="V72" s="1">
         <v>46291</v>
       </c>
     </row>
@@ -4696,7 +4670,7 @@
       <c r="U73" t="s">
         <v>182</v>
       </c>
-      <c r="V73" s="2">
+      <c r="V73" s="1">
         <v>46168</v>
       </c>
     </row>
@@ -4740,7 +4714,7 @@
       <c r="U74" t="s">
         <v>182</v>
       </c>
-      <c r="V74" s="2">
+      <c r="V74" s="1">
         <v>46291</v>
       </c>
     </row>
@@ -4784,7 +4758,7 @@
       <c r="U75" t="s">
         <v>182</v>
       </c>
-      <c r="V75" s="2">
+      <c r="V75" s="1">
         <v>46291</v>
       </c>
     </row>
@@ -4828,7 +4802,7 @@
       <c r="U76" t="s">
         <v>182</v>
       </c>
-      <c r="V76" s="2">
+      <c r="V76" s="1">
         <v>46291</v>
       </c>
     </row>
@@ -4875,7 +4849,7 @@
       <c r="U77" t="s">
         <v>28</v>
       </c>
-      <c r="V77" s="2">
+      <c r="V77" s="1">
         <v>46321</v>
       </c>
     </row>
@@ -4925,7 +4899,7 @@
       <c r="U78" t="s">
         <v>182</v>
       </c>
-      <c r="V78" s="2">
+      <c r="V78" s="1">
         <v>46381</v>
       </c>
     </row>
@@ -4975,7 +4949,7 @@
       <c r="U79" t="s">
         <v>182</v>
       </c>
-      <c r="V79" s="2">
+      <c r="V79" s="1">
         <v>46381</v>
       </c>
     </row>
@@ -5025,7 +4999,7 @@
       <c r="U80" t="s">
         <v>28</v>
       </c>
-      <c r="V80" s="2">
+      <c r="V80" s="1">
         <v>46381</v>
       </c>
     </row>
@@ -5075,7 +5049,7 @@
       <c r="U81" t="s">
         <v>28</v>
       </c>
-      <c r="V81" s="2">
+      <c r="V81" s="1">
         <v>46381</v>
       </c>
     </row>
@@ -5125,7 +5099,7 @@
       <c r="U82" t="s">
         <v>28</v>
       </c>
-      <c r="V82" s="2">
+      <c r="V82" s="1">
         <v>46382</v>
       </c>
     </row>
@@ -5169,7 +5143,7 @@
       <c r="U83" t="s">
         <v>28</v>
       </c>
-      <c r="V83" s="2">
+      <c r="V83" s="1">
         <v>46382</v>
       </c>
     </row>
@@ -5222,7 +5196,7 @@
       <c r="U84" t="s">
         <v>182</v>
       </c>
-      <c r="V84" s="2">
+      <c r="V84" s="1">
         <v>46382</v>
       </c>
     </row>
@@ -5269,7 +5243,7 @@
       <c r="U85" t="s">
         <v>28</v>
       </c>
-      <c r="V85" s="2">
+      <c r="V85" s="1">
         <v>46321</v>
       </c>
     </row>
@@ -5313,7 +5287,7 @@
       <c r="U86" t="s">
         <v>28</v>
       </c>
-      <c r="V86" s="2">
+      <c r="V86" s="1">
         <v>46382</v>
       </c>
     </row>
@@ -5454,7 +5428,7 @@
       <c r="U89" t="s">
         <v>28</v>
       </c>
-      <c r="V89" s="2">
+      <c r="V89" s="1">
         <v>46291</v>
       </c>
     </row>
@@ -5498,7 +5472,7 @@
       <c r="U90" t="s">
         <v>28</v>
       </c>
-      <c r="V90" s="2">
+      <c r="V90" s="1">
         <v>46291</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Atualização automática: mta (25/09/2026 12:49)
</commit_message>
<xml_diff>
--- a/Projetos/02_Dados_Tratados/base_mta_tratada.xlsx
+++ b/Projetos/02_Dados_Tratados/base_mta_tratada.xlsx
@@ -14,7 +14,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1188" uniqueCount="183">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1188" uniqueCount="182">
   <si>
     <t>linha</t>
   </si>
@@ -130,15 +130,15 @@
     <t>DESTQ32</t>
   </si>
   <si>
+    <t>20XV</t>
+  </si>
+  <si>
+    <t>DESTQ50</t>
+  </si>
+  <si>
     <t>DESTQ51</t>
   </si>
   <si>
-    <t>20XV</t>
-  </si>
-  <si>
-    <t>DESTQ50</t>
-  </si>
-  <si>
     <t>20IH</t>
   </si>
   <si>
@@ -253,9 +253,6 @@
     <t>ATENDER com 20XV</t>
   </si>
   <si>
-    <t>Atender; Alterar a tarefa para "Módulo Extra - Sob demanda"</t>
-  </si>
-  <si>
     <t>LIVRE</t>
   </si>
   <si>
@@ -289,24 +286,24 @@
     <t>CNT XXX/CELOG-PAMALS/2026 - Modernização - C-98</t>
   </si>
   <si>
+    <t>2025-BABR-11</t>
+  </si>
+  <si>
+    <t>2025-BABR-13</t>
+  </si>
+  <si>
     <t>2025-BABR-24</t>
   </si>
   <si>
+    <t>2025-BABV-02</t>
+  </si>
+  <si>
     <t>2025-BABV-07</t>
   </si>
   <si>
-    <t>2025-BABR-13</t>
-  </si>
-  <si>
-    <t>2025-BABR-11</t>
-  </si>
-  <si>
     <t>2025-BABV-11</t>
   </si>
   <si>
-    <t>2025-BABV-02</t>
-  </si>
-  <si>
     <t>CNT XXX/CABW-PAMASP/2026 - XX- Exchange</t>
   </si>
   <si>
@@ -451,21 +448,21 @@
     <t>Modernização 4/4</t>
   </si>
   <si>
+    <t>PN 543-250 - RELÓGIO COMPARADOR</t>
+  </si>
+  <si>
+    <t>PN T2680003-10 - TEMPLATE/SCALE ASSEMBLY</t>
+  </si>
+  <si>
     <t>PN PS47699-3-4 - PITOT TEST, ADAPTOR</t>
   </si>
   <si>
+    <t>PN DBE4-0040 - GARFO DE REBOQUE COM TRATOR ANV C-98</t>
+  </si>
+  <si>
     <t>PN PS4769 - PITOT STATIC TEST ADAPTOR</t>
   </si>
   <si>
-    <t>PN T2680003-10 - TEMPLATE/SCALE ASSEMBLY</t>
-  </si>
-  <si>
-    <t>PN 543-250 - RELÓGIO COMPARADOR</t>
-  </si>
-  <si>
-    <t>PN DBE4-0040 - GARFO DE REBOQUE COM TRATOR ANV C-98</t>
-  </si>
-  <si>
     <t>Reparo de CTVR 2 EA (2/2)</t>
   </si>
   <si>
@@ -529,13 +526,10 @@
     <t>FMS</t>
   </si>
   <si>
-    <t>339030</t>
-  </si>
-  <si>
-    <t>339039</t>
-  </si>
-  <si>
-    <t>449052</t>
+    <t>DÓLAR</t>
+  </si>
+  <si>
+    <t>REAL</t>
   </si>
   <si>
     <t>A</t>
@@ -547,6 +541,12 @@
     <t>D</t>
   </si>
   <si>
+    <t>3</t>
+  </si>
+  <si>
+    <t>4</t>
+  </si>
+  <si>
     <t>REQUISIÇÃO</t>
   </si>
   <si>
@@ -560,9 +560,6 @@
   </si>
   <si>
     <t>CONTRATO</t>
-  </si>
-  <si>
-    <t>Não</t>
   </si>
 </sst>
 </file>
@@ -995,34 +992,34 @@
         <v>72</v>
       </c>
       <c r="L2" t="s">
+        <v>79</v>
+      </c>
+      <c r="N2" t="s">
         <v>80</v>
       </c>
-      <c r="N2" t="s">
-        <v>81</v>
-      </c>
       <c r="O2" t="s">
-        <v>100</v>
+        <v>99</v>
       </c>
       <c r="P2">
-        <v>135000</v>
+        <v>46229</v>
       </c>
       <c r="Q2" t="s">
-        <v>168</v>
+        <v>167</v>
       </c>
       <c r="R2" t="s">
-        <v>171</v>
+        <v>170</v>
       </c>
       <c r="S2" t="s">
-        <v>174</v>
+        <v>172</v>
       </c>
       <c r="T2" t="s">
+        <v>175</v>
+      </c>
+      <c r="U2" t="s">
         <v>177</v>
       </c>
-      <c r="U2" t="s">
-        <v>182</v>
-      </c>
       <c r="V2" s="1">
-        <v>46229</v>
+        <v>46291</v>
       </c>
     </row>
     <row r="3" spans="1:22">
@@ -1048,28 +1045,31 @@
         <v>43</v>
       </c>
       <c r="N3" t="s">
-        <v>81</v>
+        <v>80</v>
       </c>
       <c r="O3" t="s">
-        <v>101</v>
+        <v>100</v>
+      </c>
+      <c r="P3">
+        <v>46291</v>
       </c>
       <c r="Q3" t="s">
-        <v>168</v>
+        <v>167</v>
       </c>
       <c r="R3" t="s">
-        <v>171</v>
+        <v>170</v>
       </c>
       <c r="S3" t="s">
-        <v>174</v>
+        <v>172</v>
       </c>
       <c r="T3" t="s">
+        <v>175</v>
+      </c>
+      <c r="U3" t="s">
         <v>177</v>
       </c>
-      <c r="U3" t="s">
-        <v>28</v>
-      </c>
       <c r="V3" s="1">
-        <v>46291</v>
+        <v>46382</v>
       </c>
     </row>
     <row r="4" spans="1:22">
@@ -1095,28 +1095,31 @@
         <v>43</v>
       </c>
       <c r="N4" t="s">
-        <v>82</v>
+        <v>81</v>
       </c>
       <c r="O4" t="s">
-        <v>102</v>
+        <v>101</v>
+      </c>
+      <c r="P4">
+        <v>46321</v>
       </c>
       <c r="Q4" t="s">
-        <v>168</v>
+        <v>167</v>
       </c>
       <c r="R4" t="s">
-        <v>172</v>
+        <v>170</v>
       </c>
       <c r="S4" t="s">
-        <v>174</v>
+        <v>172</v>
       </c>
       <c r="T4" t="s">
+        <v>175</v>
+      </c>
+      <c r="U4" t="s">
         <v>177</v>
       </c>
-      <c r="U4" t="s">
-        <v>28</v>
-      </c>
       <c r="V4" s="1">
-        <v>46321</v>
+        <v>46169</v>
       </c>
     </row>
     <row r="5" spans="1:22">
@@ -1142,28 +1145,31 @@
         <v>43</v>
       </c>
       <c r="N5" t="s">
-        <v>82</v>
+        <v>81</v>
       </c>
       <c r="O5" t="s">
-        <v>103</v>
+        <v>102</v>
+      </c>
+      <c r="P5">
+        <v>46321</v>
       </c>
       <c r="Q5" t="s">
-        <v>168</v>
+        <v>167</v>
       </c>
       <c r="R5" t="s">
-        <v>172</v>
+        <v>170</v>
       </c>
       <c r="S5" t="s">
-        <v>174</v>
+        <v>172</v>
       </c>
       <c r="T5" t="s">
+        <v>175</v>
+      </c>
+      <c r="U5" t="s">
         <v>177</v>
       </c>
-      <c r="U5" t="s">
-        <v>28</v>
-      </c>
       <c r="V5" s="1">
-        <v>46321</v>
+        <v>46169</v>
       </c>
     </row>
     <row r="6" spans="1:22">
@@ -1189,31 +1195,34 @@
         <v>43</v>
       </c>
       <c r="L6" t="s">
-        <v>80</v>
+        <v>79</v>
       </c>
       <c r="N6" t="s">
-        <v>83</v>
+        <v>82</v>
       </c>
       <c r="O6" t="s">
-        <v>104</v>
+        <v>103</v>
+      </c>
+      <c r="P6">
+        <v>46291</v>
       </c>
       <c r="Q6" t="s">
-        <v>168</v>
+        <v>167</v>
       </c>
       <c r="R6" t="s">
-        <v>172</v>
+        <v>170</v>
       </c>
       <c r="S6" t="s">
-        <v>174</v>
+        <v>172</v>
       </c>
       <c r="T6" t="s">
+        <v>175</v>
+      </c>
+      <c r="U6" t="s">
         <v>177</v>
       </c>
-      <c r="U6" t="s">
-        <v>28</v>
-      </c>
       <c r="V6" s="1">
-        <v>46291</v>
+        <v>46352</v>
       </c>
     </row>
     <row r="7" spans="1:22">
@@ -1245,28 +1254,28 @@
         <v>47</v>
       </c>
       <c r="N7" t="s">
-        <v>84</v>
+        <v>83</v>
       </c>
       <c r="O7" t="s">
-        <v>105</v>
+        <v>104</v>
       </c>
       <c r="P7">
-        <v>3799999.6</v>
+        <v>46138</v>
       </c>
       <c r="Q7" t="s">
-        <v>169</v>
+        <v>168</v>
       </c>
       <c r="R7" t="s">
-        <v>172</v>
+        <v>171</v>
       </c>
       <c r="S7" t="s">
-        <v>174</v>
+        <v>172</v>
       </c>
       <c r="T7" t="s">
+        <v>175</v>
+      </c>
+      <c r="U7" t="s">
         <v>178</v>
-      </c>
-      <c r="U7" t="s">
-        <v>28</v>
       </c>
       <c r="V7" s="1">
         <v>46138</v>
@@ -1295,28 +1304,31 @@
         <v>43</v>
       </c>
       <c r="N8" t="s">
-        <v>82</v>
+        <v>81</v>
       </c>
       <c r="O8" t="s">
-        <v>106</v>
+        <v>105</v>
+      </c>
+      <c r="P8">
+        <v>46291</v>
       </c>
       <c r="Q8" t="s">
-        <v>168</v>
+        <v>167</v>
       </c>
       <c r="R8" t="s">
-        <v>172</v>
+        <v>170</v>
       </c>
       <c r="S8" t="s">
-        <v>174</v>
+        <v>172</v>
       </c>
       <c r="T8" t="s">
+        <v>175</v>
+      </c>
+      <c r="U8" t="s">
         <v>177</v>
       </c>
-      <c r="U8" t="s">
-        <v>28</v>
-      </c>
       <c r="V8" s="1">
-        <v>46291</v>
+        <v>46200</v>
       </c>
     </row>
     <row r="9" spans="1:22">
@@ -1339,31 +1351,31 @@
         <v>30</v>
       </c>
       <c r="N9" t="s">
-        <v>82</v>
+        <v>81</v>
       </c>
       <c r="O9" t="s">
-        <v>107</v>
+        <v>106</v>
       </c>
       <c r="P9">
-        <v>60000</v>
+        <v>46291</v>
       </c>
       <c r="Q9" t="s">
-        <v>168</v>
+        <v>167</v>
       </c>
       <c r="R9" t="s">
-        <v>172</v>
+        <v>170</v>
       </c>
       <c r="S9" t="s">
-        <v>174</v>
+        <v>172</v>
       </c>
       <c r="T9" t="s">
+        <v>175</v>
+      </c>
+      <c r="U9" t="s">
         <v>177</v>
       </c>
-      <c r="U9" t="s">
-        <v>28</v>
-      </c>
       <c r="V9" s="1">
-        <v>46291</v>
+        <v>46200</v>
       </c>
     </row>
     <row r="10" spans="1:22">
@@ -1389,28 +1401,31 @@
         <v>43</v>
       </c>
       <c r="N10" t="s">
-        <v>83</v>
+        <v>82</v>
       </c>
       <c r="O10" t="s">
-        <v>108</v>
+        <v>107</v>
+      </c>
+      <c r="P10">
+        <v>46291</v>
       </c>
       <c r="Q10" t="s">
-        <v>168</v>
+        <v>167</v>
       </c>
       <c r="R10" t="s">
-        <v>172</v>
+        <v>170</v>
       </c>
       <c r="S10" t="s">
-        <v>174</v>
+        <v>172</v>
       </c>
       <c r="T10" t="s">
+        <v>175</v>
+      </c>
+      <c r="U10" t="s">
         <v>177</v>
       </c>
-      <c r="U10" t="s">
-        <v>28</v>
-      </c>
       <c r="V10" s="1">
-        <v>46291</v>
+        <v>46352</v>
       </c>
     </row>
     <row r="11" spans="1:22">
@@ -1436,28 +1451,31 @@
         <v>43</v>
       </c>
       <c r="N11" t="s">
-        <v>83</v>
+        <v>82</v>
       </c>
       <c r="O11" t="s">
-        <v>109</v>
+        <v>108</v>
+      </c>
+      <c r="P11">
+        <v>46291</v>
       </c>
       <c r="Q11" t="s">
-        <v>168</v>
+        <v>167</v>
       </c>
       <c r="R11" t="s">
-        <v>172</v>
+        <v>170</v>
       </c>
       <c r="S11" t="s">
-        <v>174</v>
+        <v>172</v>
       </c>
       <c r="T11" t="s">
+        <v>175</v>
+      </c>
+      <c r="U11" t="s">
         <v>177</v>
       </c>
-      <c r="U11" t="s">
-        <v>28</v>
-      </c>
       <c r="V11" s="1">
-        <v>46291</v>
+        <v>46352</v>
       </c>
     </row>
     <row r="12" spans="1:22">
@@ -1492,31 +1510,31 @@
         <v>65</v>
       </c>
       <c r="N12" t="s">
-        <v>81</v>
+        <v>80</v>
       </c>
       <c r="O12" t="s">
-        <v>110</v>
+        <v>109</v>
       </c>
       <c r="P12">
-        <v>1187433.02</v>
+        <v>46079</v>
       </c>
       <c r="Q12" t="s">
-        <v>168</v>
+        <v>167</v>
       </c>
       <c r="R12" t="s">
-        <v>171</v>
+        <v>170</v>
       </c>
       <c r="S12" t="s">
-        <v>174</v>
+        <v>172</v>
       </c>
       <c r="T12" t="s">
+        <v>175</v>
+      </c>
+      <c r="U12" t="s">
         <v>177</v>
       </c>
-      <c r="U12" t="s">
-        <v>182</v>
-      </c>
       <c r="V12" s="1">
-        <v>46079</v>
+        <v>46168</v>
       </c>
     </row>
     <row r="13" spans="1:22">
@@ -1545,31 +1563,31 @@
         <v>73</v>
       </c>
       <c r="N13" t="s">
-        <v>81</v>
+        <v>80</v>
       </c>
       <c r="O13" t="s">
-        <v>111</v>
+        <v>110</v>
       </c>
       <c r="P13">
-        <v>1000000</v>
+        <v>46352</v>
       </c>
       <c r="Q13" t="s">
-        <v>168</v>
+        <v>167</v>
       </c>
       <c r="R13" t="s">
-        <v>171</v>
+        <v>170</v>
       </c>
       <c r="S13" t="s">
-        <v>174</v>
+        <v>172</v>
       </c>
       <c r="T13" t="s">
+        <v>175</v>
+      </c>
+      <c r="U13" t="s">
         <v>177</v>
       </c>
-      <c r="U13" t="s">
-        <v>182</v>
-      </c>
       <c r="V13" s="1">
-        <v>46352</v>
+        <v>46049</v>
       </c>
     </row>
     <row r="14" spans="1:22">
@@ -1598,31 +1616,31 @@
         <v>73</v>
       </c>
       <c r="N14" t="s">
-        <v>81</v>
+        <v>80</v>
       </c>
       <c r="O14" t="s">
-        <v>112</v>
+        <v>111</v>
       </c>
       <c r="P14">
-        <v>1000000</v>
+        <v>46352</v>
       </c>
       <c r="Q14" t="s">
-        <v>168</v>
+        <v>167</v>
       </c>
       <c r="R14" t="s">
-        <v>171</v>
+        <v>170</v>
       </c>
       <c r="S14" t="s">
-        <v>174</v>
+        <v>172</v>
       </c>
       <c r="T14" t="s">
+        <v>175</v>
+      </c>
+      <c r="U14" t="s">
         <v>177</v>
       </c>
-      <c r="U14" t="s">
-        <v>182</v>
-      </c>
       <c r="V14" s="1">
-        <v>46352</v>
+        <v>46049</v>
       </c>
     </row>
     <row r="15" spans="1:22">
@@ -1651,31 +1669,31 @@
         <v>73</v>
       </c>
       <c r="N15" t="s">
-        <v>81</v>
+        <v>80</v>
       </c>
       <c r="O15" t="s">
-        <v>113</v>
+        <v>112</v>
       </c>
       <c r="P15">
-        <v>1000000</v>
+        <v>46352</v>
       </c>
       <c r="Q15" t="s">
-        <v>168</v>
+        <v>167</v>
       </c>
       <c r="R15" t="s">
-        <v>171</v>
+        <v>170</v>
       </c>
       <c r="S15" t="s">
-        <v>174</v>
+        <v>172</v>
       </c>
       <c r="T15" t="s">
+        <v>175</v>
+      </c>
+      <c r="U15" t="s">
         <v>177</v>
       </c>
-      <c r="U15" t="s">
-        <v>182</v>
-      </c>
       <c r="V15" s="1">
-        <v>46352</v>
+        <v>46049</v>
       </c>
     </row>
     <row r="16" spans="1:22">
@@ -1704,31 +1722,31 @@
         <v>73</v>
       </c>
       <c r="N16" t="s">
-        <v>85</v>
+        <v>84</v>
       </c>
       <c r="O16" t="s">
-        <v>114</v>
+        <v>113</v>
       </c>
       <c r="P16">
-        <v>100000</v>
+        <v>46229</v>
       </c>
       <c r="Q16" t="s">
+        <v>169</v>
+      </c>
+      <c r="R16" t="s">
         <v>170</v>
       </c>
-      <c r="R16" t="s">
-        <v>171</v>
-      </c>
       <c r="S16" t="s">
-        <v>174</v>
+        <v>172</v>
       </c>
       <c r="T16" t="s">
+        <v>175</v>
+      </c>
+      <c r="U16" t="s">
         <v>177</v>
       </c>
-      <c r="U16" t="s">
-        <v>182</v>
-      </c>
       <c r="V16" s="1">
-        <v>46229</v>
+        <v>46291</v>
       </c>
     </row>
     <row r="17" spans="1:22">
@@ -1763,31 +1781,31 @@
         <v>65</v>
       </c>
       <c r="N17" t="s">
-        <v>86</v>
+        <v>85</v>
       </c>
       <c r="O17" t="s">
-        <v>115</v>
+        <v>114</v>
       </c>
       <c r="P17">
-        <v>1770880.5</v>
+        <v>46107</v>
       </c>
       <c r="Q17" t="s">
-        <v>169</v>
+        <v>168</v>
       </c>
       <c r="R17" t="s">
-        <v>172</v>
+        <v>171</v>
       </c>
       <c r="S17" t="s">
-        <v>174</v>
+        <v>172</v>
       </c>
       <c r="T17" t="s">
+        <v>175</v>
+      </c>
+      <c r="U17" t="s">
         <v>179</v>
       </c>
-      <c r="U17" t="s">
-        <v>182</v>
-      </c>
       <c r="V17" s="1">
-        <v>46107</v>
+        <v>46168</v>
       </c>
     </row>
     <row r="18" spans="1:22">
@@ -1819,31 +1837,31 @@
         <v>50</v>
       </c>
       <c r="N18" t="s">
-        <v>87</v>
+        <v>86</v>
       </c>
       <c r="O18" t="s">
-        <v>116</v>
+        <v>115</v>
       </c>
       <c r="P18">
-        <v>350000</v>
+        <v>46079</v>
       </c>
       <c r="Q18" t="s">
-        <v>169</v>
+        <v>168</v>
       </c>
       <c r="R18" t="s">
         <v>171</v>
       </c>
       <c r="S18" t="s">
-        <v>174</v>
+        <v>172</v>
       </c>
       <c r="T18" t="s">
+        <v>175</v>
+      </c>
+      <c r="U18" t="s">
         <v>178</v>
       </c>
-      <c r="U18" t="s">
-        <v>28</v>
-      </c>
       <c r="V18" s="1">
-        <v>46079</v>
+        <v>46260</v>
       </c>
     </row>
     <row r="19" spans="1:22">
@@ -1875,31 +1893,31 @@
         <v>50</v>
       </c>
       <c r="N19" t="s">
-        <v>87</v>
+        <v>86</v>
       </c>
       <c r="O19" t="s">
-        <v>117</v>
+        <v>116</v>
       </c>
       <c r="P19">
-        <v>350000</v>
+        <v>46079</v>
       </c>
       <c r="Q19" t="s">
-        <v>169</v>
+        <v>168</v>
       </c>
       <c r="R19" t="s">
         <v>171</v>
       </c>
       <c r="S19" t="s">
-        <v>174</v>
+        <v>172</v>
       </c>
       <c r="T19" t="s">
+        <v>175</v>
+      </c>
+      <c r="U19" t="s">
         <v>178</v>
       </c>
-      <c r="U19" t="s">
-        <v>28</v>
-      </c>
       <c r="V19" s="1">
-        <v>46079</v>
+        <v>46260</v>
       </c>
     </row>
     <row r="20" spans="1:22">
@@ -1922,31 +1940,31 @@
         <v>30</v>
       </c>
       <c r="N20" t="s">
-        <v>88</v>
+        <v>87</v>
       </c>
       <c r="O20" t="s">
-        <v>118</v>
+        <v>117</v>
       </c>
       <c r="P20">
-        <v>1000000</v>
+        <v>46321</v>
       </c>
       <c r="Q20" t="s">
-        <v>169</v>
+        <v>168</v>
       </c>
       <c r="R20" t="s">
         <v>171</v>
       </c>
       <c r="S20" t="s">
-        <v>174</v>
+        <v>172</v>
       </c>
       <c r="T20" t="s">
+        <v>175</v>
+      </c>
+      <c r="U20" t="s">
         <v>178</v>
       </c>
-      <c r="U20" t="s">
-        <v>28</v>
-      </c>
       <c r="V20" s="1">
-        <v>46321</v>
+        <v>46382</v>
       </c>
     </row>
     <row r="21" spans="1:22">
@@ -1972,28 +1990,31 @@
         <v>43</v>
       </c>
       <c r="N21" t="s">
-        <v>81</v>
+        <v>80</v>
       </c>
       <c r="O21" t="s">
-        <v>119</v>
+        <v>118</v>
+      </c>
+      <c r="P21">
+        <v>46321</v>
       </c>
       <c r="Q21" t="s">
-        <v>168</v>
+        <v>167</v>
       </c>
       <c r="R21" t="s">
-        <v>171</v>
+        <v>170</v>
       </c>
       <c r="S21" t="s">
-        <v>174</v>
+        <v>172</v>
       </c>
       <c r="T21" t="s">
+        <v>175</v>
+      </c>
+      <c r="U21" t="s">
         <v>177</v>
       </c>
-      <c r="U21" t="s">
-        <v>28</v>
-      </c>
       <c r="V21" s="1">
-        <v>46321</v>
+        <v>46382</v>
       </c>
     </row>
     <row r="22" spans="1:22">
@@ -2019,28 +2040,31 @@
         <v>43</v>
       </c>
       <c r="N22" t="s">
-        <v>82</v>
+        <v>81</v>
       </c>
       <c r="O22" t="s">
-        <v>120</v>
+        <v>119</v>
+      </c>
+      <c r="P22">
+        <v>46321</v>
       </c>
       <c r="Q22" t="s">
-        <v>168</v>
+        <v>167</v>
       </c>
       <c r="R22" t="s">
-        <v>172</v>
+        <v>170</v>
       </c>
       <c r="S22" t="s">
-        <v>174</v>
+        <v>172</v>
       </c>
       <c r="T22" t="s">
+        <v>175</v>
+      </c>
+      <c r="U22" t="s">
         <v>177</v>
       </c>
-      <c r="U22" t="s">
-        <v>28</v>
-      </c>
       <c r="V22" s="1">
-        <v>46321</v>
+        <v>46230</v>
       </c>
     </row>
     <row r="23" spans="1:22">
@@ -2066,28 +2090,31 @@
         <v>43</v>
       </c>
       <c r="N23" t="s">
-        <v>82</v>
+        <v>81</v>
       </c>
       <c r="O23" t="s">
-        <v>121</v>
+        <v>120</v>
+      </c>
+      <c r="P23">
+        <v>46321</v>
       </c>
       <c r="Q23" t="s">
-        <v>168</v>
+        <v>167</v>
       </c>
       <c r="R23" t="s">
-        <v>172</v>
+        <v>170</v>
       </c>
       <c r="S23" t="s">
-        <v>174</v>
+        <v>172</v>
       </c>
       <c r="T23" t="s">
+        <v>175</v>
+      </c>
+      <c r="U23" t="s">
         <v>177</v>
       </c>
-      <c r="U23" t="s">
-        <v>28</v>
-      </c>
       <c r="V23" s="1">
-        <v>46321</v>
+        <v>46230</v>
       </c>
     </row>
     <row r="24" spans="1:22">
@@ -2122,31 +2149,31 @@
         <v>66</v>
       </c>
       <c r="N24" t="s">
-        <v>86</v>
+        <v>85</v>
       </c>
       <c r="O24" t="s">
-        <v>122</v>
+        <v>121</v>
       </c>
       <c r="P24">
-        <v>1704503</v>
+        <v>46138</v>
       </c>
       <c r="Q24" t="s">
-        <v>169</v>
+        <v>168</v>
       </c>
       <c r="R24" t="s">
-        <v>172</v>
+        <v>171</v>
       </c>
       <c r="S24" t="s">
-        <v>174</v>
+        <v>172</v>
       </c>
       <c r="T24" t="s">
+        <v>175</v>
+      </c>
+      <c r="U24" t="s">
         <v>179</v>
       </c>
-      <c r="U24" t="s">
-        <v>182</v>
-      </c>
       <c r="V24" s="1">
-        <v>46138</v>
+        <v>46199</v>
       </c>
     </row>
     <row r="25" spans="1:22">
@@ -2178,31 +2205,31 @@
         <v>52</v>
       </c>
       <c r="N25" t="s">
-        <v>89</v>
+        <v>88</v>
       </c>
       <c r="O25" t="s">
-        <v>123</v>
+        <v>122</v>
       </c>
       <c r="P25">
-        <v>3799000</v>
+        <v>46138</v>
       </c>
       <c r="Q25" t="s">
-        <v>169</v>
+        <v>168</v>
       </c>
       <c r="R25" t="s">
-        <v>172</v>
+        <v>171</v>
       </c>
       <c r="S25" t="s">
-        <v>174</v>
+        <v>172</v>
       </c>
       <c r="T25" t="s">
+        <v>175</v>
+      </c>
+      <c r="U25" t="s">
         <v>178</v>
       </c>
-      <c r="U25" t="s">
-        <v>28</v>
-      </c>
       <c r="V25" s="1">
-        <v>46138</v>
+        <v>46199</v>
       </c>
     </row>
     <row r="26" spans="1:22">
@@ -2234,31 +2261,31 @@
         <v>53</v>
       </c>
       <c r="N26" t="s">
-        <v>89</v>
+        <v>88</v>
       </c>
       <c r="O26" t="s">
-        <v>123</v>
+        <v>122</v>
       </c>
       <c r="P26">
-        <v>1000</v>
+        <v>46079</v>
       </c>
       <c r="Q26" t="s">
-        <v>169</v>
+        <v>168</v>
       </c>
       <c r="R26" t="s">
         <v>171</v>
       </c>
       <c r="S26" t="s">
-        <v>174</v>
+        <v>172</v>
       </c>
       <c r="T26" t="s">
+        <v>175</v>
+      </c>
+      <c r="U26" t="s">
         <v>178</v>
       </c>
-      <c r="U26" t="s">
-        <v>28</v>
-      </c>
       <c r="V26" s="1">
-        <v>46079</v>
+        <v>46352</v>
       </c>
     </row>
     <row r="27" spans="1:22">
@@ -2287,31 +2314,31 @@
         <v>73</v>
       </c>
       <c r="N27" t="s">
-        <v>85</v>
+        <v>84</v>
       </c>
       <c r="O27" t="s">
-        <v>124</v>
+        <v>123</v>
       </c>
       <c r="P27">
-        <v>100000</v>
+        <v>46291</v>
       </c>
       <c r="Q27" t="s">
+        <v>169</v>
+      </c>
+      <c r="R27" t="s">
         <v>170</v>
       </c>
-      <c r="R27" t="s">
-        <v>171</v>
-      </c>
       <c r="S27" t="s">
-        <v>174</v>
+        <v>172</v>
       </c>
       <c r="T27" t="s">
+        <v>175</v>
+      </c>
+      <c r="U27" t="s">
         <v>177</v>
       </c>
-      <c r="U27" t="s">
-        <v>182</v>
-      </c>
       <c r="V27" s="1">
-        <v>46291</v>
+        <v>46352</v>
       </c>
     </row>
     <row r="28" spans="1:22">
@@ -2346,31 +2373,31 @@
         <v>67</v>
       </c>
       <c r="N28" t="s">
-        <v>86</v>
+        <v>85</v>
       </c>
       <c r="O28" t="s">
-        <v>125</v>
+        <v>124</v>
       </c>
       <c r="P28">
-        <v>150000</v>
+        <v>46199</v>
       </c>
       <c r="Q28" t="s">
-        <v>169</v>
+        <v>168</v>
       </c>
       <c r="R28" t="s">
-        <v>172</v>
+        <v>171</v>
       </c>
       <c r="S28" t="s">
-        <v>174</v>
+        <v>172</v>
       </c>
       <c r="T28" t="s">
+        <v>175</v>
+      </c>
+      <c r="U28" t="s">
         <v>178</v>
       </c>
-      <c r="U28" t="s">
-        <v>182</v>
-      </c>
       <c r="V28" s="1">
-        <v>46199</v>
+        <v>46260</v>
       </c>
     </row>
     <row r="29" spans="1:22">
@@ -2405,31 +2432,31 @@
         <v>67</v>
       </c>
       <c r="N29" t="s">
-        <v>86</v>
+        <v>85</v>
       </c>
       <c r="O29" t="s">
-        <v>126</v>
+        <v>125</v>
       </c>
       <c r="P29">
-        <v>150000</v>
+        <v>46199</v>
       </c>
       <c r="Q29" t="s">
-        <v>169</v>
+        <v>168</v>
       </c>
       <c r="R29" t="s">
-        <v>172</v>
+        <v>171</v>
       </c>
       <c r="S29" t="s">
-        <v>174</v>
+        <v>172</v>
       </c>
       <c r="T29" t="s">
+        <v>175</v>
+      </c>
+      <c r="U29" t="s">
         <v>178</v>
       </c>
-      <c r="U29" t="s">
-        <v>182</v>
-      </c>
       <c r="V29" s="1">
-        <v>46199</v>
+        <v>46260</v>
       </c>
     </row>
     <row r="30" spans="1:22">
@@ -2464,31 +2491,31 @@
         <v>67</v>
       </c>
       <c r="N30" t="s">
-        <v>86</v>
+        <v>85</v>
       </c>
       <c r="O30" t="s">
-        <v>127</v>
+        <v>126</v>
       </c>
       <c r="P30">
-        <v>18462.36</v>
+        <v>46199</v>
       </c>
       <c r="Q30" t="s">
-        <v>169</v>
+        <v>168</v>
       </c>
       <c r="R30" t="s">
-        <v>172</v>
+        <v>171</v>
       </c>
       <c r="S30" t="s">
-        <v>174</v>
+        <v>172</v>
       </c>
       <c r="T30" t="s">
+        <v>175</v>
+      </c>
+      <c r="U30" t="s">
         <v>178</v>
       </c>
-      <c r="U30" t="s">
-        <v>182</v>
-      </c>
       <c r="V30" s="1">
-        <v>46199</v>
+        <v>46260</v>
       </c>
     </row>
     <row r="31" spans="1:22">
@@ -2523,31 +2550,31 @@
         <v>67</v>
       </c>
       <c r="N31" t="s">
-        <v>86</v>
+        <v>85</v>
       </c>
       <c r="O31" t="s">
-        <v>127</v>
+        <v>126</v>
       </c>
       <c r="P31">
-        <v>324166.14</v>
+        <v>46199</v>
       </c>
       <c r="Q31" t="s">
-        <v>169</v>
+        <v>168</v>
       </c>
       <c r="R31" t="s">
-        <v>172</v>
+        <v>171</v>
       </c>
       <c r="S31" t="s">
-        <v>174</v>
+        <v>172</v>
       </c>
       <c r="T31" t="s">
+        <v>175</v>
+      </c>
+      <c r="U31" t="s">
         <v>178</v>
       </c>
-      <c r="U31" t="s">
-        <v>182</v>
-      </c>
       <c r="V31" s="1">
-        <v>46199</v>
+        <v>46260</v>
       </c>
     </row>
     <row r="32" spans="1:22">
@@ -2573,31 +2600,31 @@
         <v>74</v>
       </c>
       <c r="N32" t="s">
-        <v>86</v>
+        <v>85</v>
       </c>
       <c r="O32" t="s">
-        <v>128</v>
+        <v>127</v>
       </c>
       <c r="P32">
-        <v>30000</v>
+        <v>46291</v>
       </c>
       <c r="Q32" t="s">
-        <v>169</v>
+        <v>168</v>
       </c>
       <c r="R32" t="s">
-        <v>172</v>
+        <v>171</v>
       </c>
       <c r="S32" t="s">
-        <v>174</v>
+        <v>172</v>
       </c>
       <c r="T32" t="s">
+        <v>175</v>
+      </c>
+      <c r="U32" t="s">
         <v>178</v>
       </c>
-      <c r="U32" t="s">
-        <v>182</v>
-      </c>
       <c r="V32" s="1">
-        <v>46291</v>
+        <v>46352</v>
       </c>
     </row>
     <row r="33" spans="1:22">
@@ -2632,31 +2659,31 @@
         <v>68</v>
       </c>
       <c r="N33" t="s">
-        <v>86</v>
+        <v>85</v>
       </c>
       <c r="O33" t="s">
-        <v>129</v>
+        <v>128</v>
       </c>
       <c r="P33">
-        <v>1496713.48</v>
+        <v>46199</v>
       </c>
       <c r="Q33" t="s">
-        <v>169</v>
+        <v>168</v>
       </c>
       <c r="R33" t="s">
-        <v>172</v>
+        <v>171</v>
       </c>
       <c r="S33" t="s">
-        <v>174</v>
+        <v>172</v>
       </c>
       <c r="T33" t="s">
+        <v>175</v>
+      </c>
+      <c r="U33" t="s">
         <v>179</v>
       </c>
-      <c r="U33" t="s">
-        <v>182</v>
-      </c>
       <c r="V33" s="1">
-        <v>46199</v>
+        <v>46260</v>
       </c>
     </row>
     <row r="34" spans="1:22">
@@ -2688,31 +2715,31 @@
         <v>51</v>
       </c>
       <c r="N34" t="s">
-        <v>86</v>
+        <v>85</v>
       </c>
       <c r="O34" t="s">
-        <v>129</v>
+        <v>128</v>
       </c>
       <c r="P34">
-        <v>207789.52</v>
+        <v>46138</v>
       </c>
       <c r="Q34" t="s">
-        <v>169</v>
+        <v>168</v>
       </c>
       <c r="R34" t="s">
-        <v>172</v>
+        <v>171</v>
       </c>
       <c r="S34" t="s">
-        <v>174</v>
+        <v>172</v>
       </c>
       <c r="T34" t="s">
+        <v>175</v>
+      </c>
+      <c r="U34" t="s">
         <v>179</v>
       </c>
-      <c r="U34" t="s">
-        <v>182</v>
-      </c>
       <c r="V34" s="1">
-        <v>46138</v>
+        <v>46260</v>
       </c>
     </row>
     <row r="35" spans="1:22">
@@ -2744,31 +2771,31 @@
         <v>57</v>
       </c>
       <c r="N35" t="s">
-        <v>89</v>
+        <v>88</v>
       </c>
       <c r="O35" t="s">
-        <v>130</v>
+        <v>129</v>
       </c>
       <c r="P35">
-        <v>962290.8</v>
+        <v>46229</v>
       </c>
       <c r="Q35" t="s">
-        <v>169</v>
+        <v>168</v>
       </c>
       <c r="R35" t="s">
         <v>171</v>
       </c>
       <c r="S35" t="s">
-        <v>174</v>
+        <v>172</v>
       </c>
       <c r="T35" t="s">
+        <v>175</v>
+      </c>
+      <c r="U35" t="s">
         <v>178</v>
       </c>
-      <c r="U35" t="s">
-        <v>28</v>
-      </c>
       <c r="V35" s="1">
-        <v>46229</v>
+        <v>46352</v>
       </c>
     </row>
     <row r="36" spans="1:22">
@@ -2800,31 +2827,31 @@
         <v>58</v>
       </c>
       <c r="N36" t="s">
-        <v>89</v>
+        <v>88</v>
       </c>
       <c r="O36" t="s">
-        <v>130</v>
+        <v>129</v>
       </c>
       <c r="P36">
-        <v>798776.97</v>
+        <v>46199</v>
       </c>
       <c r="Q36" t="s">
-        <v>169</v>
+        <v>168</v>
       </c>
       <c r="R36" t="s">
-        <v>172</v>
+        <v>171</v>
       </c>
       <c r="S36" t="s">
-        <v>174</v>
+        <v>172</v>
       </c>
       <c r="T36" t="s">
+        <v>175</v>
+      </c>
+      <c r="U36" t="s">
         <v>178</v>
       </c>
-      <c r="U36" t="s">
-        <v>28</v>
-      </c>
       <c r="V36" s="1">
-        <v>46199</v>
+        <v>46260</v>
       </c>
     </row>
     <row r="37" spans="1:22">
@@ -2856,31 +2883,31 @@
         <v>57</v>
       </c>
       <c r="N37" t="s">
-        <v>89</v>
+        <v>88</v>
       </c>
       <c r="O37" t="s">
-        <v>130</v>
+        <v>129</v>
       </c>
       <c r="P37">
-        <v>1530656.62</v>
+        <v>46229</v>
       </c>
       <c r="Q37" t="s">
-        <v>169</v>
+        <v>168</v>
       </c>
       <c r="R37" t="s">
         <v>171</v>
       </c>
       <c r="S37" t="s">
-        <v>174</v>
+        <v>172</v>
       </c>
       <c r="T37" t="s">
+        <v>175</v>
+      </c>
+      <c r="U37" t="s">
         <v>178</v>
       </c>
-      <c r="U37" t="s">
-        <v>28</v>
-      </c>
       <c r="V37" s="1">
-        <v>46229</v>
+        <v>46352</v>
       </c>
     </row>
     <row r="38" spans="1:22">
@@ -2912,31 +2939,31 @@
         <v>59</v>
       </c>
       <c r="N38" t="s">
-        <v>89</v>
+        <v>88</v>
       </c>
       <c r="O38" t="s">
-        <v>130</v>
+        <v>129</v>
       </c>
       <c r="P38">
-        <v>72958.08</v>
+        <v>46199</v>
       </c>
       <c r="Q38" t="s">
-        <v>169</v>
+        <v>168</v>
       </c>
       <c r="R38" t="s">
         <v>171</v>
       </c>
       <c r="S38" t="s">
-        <v>174</v>
+        <v>172</v>
       </c>
       <c r="T38" t="s">
+        <v>175</v>
+      </c>
+      <c r="U38" t="s">
         <v>178</v>
       </c>
-      <c r="U38" t="s">
-        <v>28</v>
-      </c>
       <c r="V38" s="1">
-        <v>46199</v>
+        <v>46229</v>
       </c>
     </row>
     <row r="39" spans="1:22">
@@ -2968,31 +2995,31 @@
         <v>59</v>
       </c>
       <c r="N39" t="s">
-        <v>89</v>
+        <v>88</v>
       </c>
       <c r="O39" t="s">
-        <v>130</v>
+        <v>129</v>
       </c>
       <c r="P39">
-        <v>8916</v>
+        <v>46199</v>
       </c>
       <c r="Q39" t="s">
-        <v>169</v>
+        <v>168</v>
       </c>
       <c r="R39" t="s">
         <v>171</v>
       </c>
       <c r="S39" t="s">
-        <v>174</v>
+        <v>172</v>
       </c>
       <c r="T39" t="s">
+        <v>175</v>
+      </c>
+      <c r="U39" t="s">
         <v>178</v>
       </c>
-      <c r="U39" t="s">
-        <v>28</v>
-      </c>
       <c r="V39" s="1">
-        <v>46199</v>
+        <v>46229</v>
       </c>
     </row>
     <row r="40" spans="1:22">
@@ -3024,28 +3051,28 @@
         <v>59</v>
       </c>
       <c r="N40" t="s">
-        <v>89</v>
+        <v>88</v>
       </c>
       <c r="O40" t="s">
-        <v>130</v>
+        <v>129</v>
       </c>
       <c r="P40">
-        <v>425178.5</v>
+        <v>46229</v>
       </c>
       <c r="Q40" t="s">
-        <v>169</v>
+        <v>168</v>
       </c>
       <c r="R40" t="s">
         <v>171</v>
       </c>
       <c r="S40" t="s">
-        <v>174</v>
+        <v>172</v>
       </c>
       <c r="T40" t="s">
+        <v>175</v>
+      </c>
+      <c r="U40" t="s">
         <v>178</v>
-      </c>
-      <c r="U40" t="s">
-        <v>28</v>
       </c>
       <c r="V40" s="1">
         <v>46229</v>
@@ -3080,31 +3107,31 @@
         <v>60</v>
       </c>
       <c r="N41" t="s">
-        <v>89</v>
+        <v>88</v>
       </c>
       <c r="O41" t="s">
-        <v>130</v>
+        <v>129</v>
       </c>
       <c r="P41">
-        <v>1223.03</v>
+        <v>46199</v>
       </c>
       <c r="Q41" t="s">
-        <v>169</v>
+        <v>168</v>
       </c>
       <c r="R41" t="s">
         <v>171</v>
       </c>
       <c r="S41" t="s">
-        <v>174</v>
+        <v>172</v>
       </c>
       <c r="T41" t="s">
+        <v>175</v>
+      </c>
+      <c r="U41" t="s">
         <v>178</v>
       </c>
-      <c r="U41" t="s">
-        <v>28</v>
-      </c>
       <c r="V41" s="1">
-        <v>46199</v>
+        <v>46260</v>
       </c>
     </row>
     <row r="42" spans="1:22">
@@ -3127,28 +3154,31 @@
         <v>43</v>
       </c>
       <c r="N42" t="s">
-        <v>89</v>
+        <v>88</v>
       </c>
       <c r="O42" t="s">
-        <v>131</v>
+        <v>130</v>
+      </c>
+      <c r="P42">
+        <v>46260</v>
       </c>
       <c r="Q42" t="s">
-        <v>169</v>
+        <v>168</v>
       </c>
       <c r="R42" t="s">
         <v>171</v>
       </c>
       <c r="S42" t="s">
-        <v>175</v>
+        <v>173</v>
       </c>
       <c r="T42" t="s">
+        <v>175</v>
+      </c>
+      <c r="U42" t="s">
         <v>178</v>
       </c>
-      <c r="U42" t="s">
-        <v>28</v>
-      </c>
       <c r="V42" s="1">
-        <v>46260</v>
+        <v>46352</v>
       </c>
     </row>
     <row r="43" spans="1:22">
@@ -3180,31 +3210,31 @@
         <v>61</v>
       </c>
       <c r="N43" t="s">
-        <v>87</v>
+        <v>86</v>
       </c>
       <c r="O43" t="s">
-        <v>132</v>
+        <v>131</v>
       </c>
       <c r="P43">
-        <v>400000</v>
+        <v>46199</v>
       </c>
       <c r="Q43" t="s">
-        <v>169</v>
+        <v>168</v>
       </c>
       <c r="R43" t="s">
         <v>171</v>
       </c>
       <c r="S43" t="s">
-        <v>174</v>
+        <v>172</v>
       </c>
       <c r="T43" t="s">
+        <v>175</v>
+      </c>
+      <c r="U43" t="s">
         <v>178</v>
       </c>
-      <c r="U43" t="s">
-        <v>28</v>
-      </c>
       <c r="V43" s="1">
-        <v>46199</v>
+        <v>46229</v>
       </c>
     </row>
     <row r="44" spans="1:22">
@@ -3236,31 +3266,31 @@
         <v>61</v>
       </c>
       <c r="N44" t="s">
-        <v>87</v>
+        <v>86</v>
       </c>
       <c r="O44" t="s">
-        <v>133</v>
+        <v>132</v>
       </c>
       <c r="P44">
-        <v>400000</v>
+        <v>46199</v>
       </c>
       <c r="Q44" t="s">
-        <v>169</v>
+        <v>168</v>
       </c>
       <c r="R44" t="s">
         <v>171</v>
       </c>
       <c r="S44" t="s">
-        <v>174</v>
+        <v>172</v>
       </c>
       <c r="T44" t="s">
+        <v>175</v>
+      </c>
+      <c r="U44" t="s">
         <v>178</v>
       </c>
-      <c r="U44" t="s">
-        <v>28</v>
-      </c>
       <c r="V44" s="1">
-        <v>46199</v>
+        <v>46229</v>
       </c>
     </row>
     <row r="45" spans="1:22">
@@ -3295,31 +3325,31 @@
         <v>69</v>
       </c>
       <c r="N45" t="s">
-        <v>86</v>
+        <v>85</v>
       </c>
       <c r="O45" t="s">
-        <v>134</v>
+        <v>133</v>
       </c>
       <c r="P45">
-        <v>173846.38</v>
+        <v>46229</v>
       </c>
       <c r="Q45" t="s">
-        <v>169</v>
+        <v>168</v>
       </c>
       <c r="R45" t="s">
-        <v>172</v>
+        <v>171</v>
       </c>
       <c r="S45" t="s">
-        <v>174</v>
+        <v>172</v>
       </c>
       <c r="T45" t="s">
+        <v>175</v>
+      </c>
+      <c r="U45" t="s">
         <v>179</v>
       </c>
-      <c r="U45" t="s">
-        <v>182</v>
-      </c>
       <c r="V45" s="1">
-        <v>46229</v>
+        <v>46291</v>
       </c>
     </row>
     <row r="46" spans="1:22">
@@ -3351,31 +3381,31 @@
         <v>55</v>
       </c>
       <c r="N46" t="s">
-        <v>86</v>
+        <v>85</v>
       </c>
       <c r="O46" t="s">
-        <v>134</v>
+        <v>133</v>
       </c>
       <c r="P46">
-        <v>1530656.62</v>
+        <v>46229</v>
       </c>
       <c r="Q46" t="s">
-        <v>169</v>
+        <v>168</v>
       </c>
       <c r="R46" t="s">
-        <v>172</v>
+        <v>171</v>
       </c>
       <c r="S46" t="s">
-        <v>174</v>
+        <v>172</v>
       </c>
       <c r="T46" t="s">
+        <v>175</v>
+      </c>
+      <c r="U46" t="s">
         <v>179</v>
       </c>
-      <c r="U46" t="s">
-        <v>182</v>
-      </c>
       <c r="V46" s="1">
-        <v>46229</v>
+        <v>46291</v>
       </c>
     </row>
     <row r="47" spans="1:22">
@@ -3398,28 +3428,28 @@
         <v>30</v>
       </c>
       <c r="N47" t="s">
-        <v>88</v>
+        <v>87</v>
       </c>
       <c r="O47" t="s">
-        <v>135</v>
+        <v>134</v>
       </c>
       <c r="P47">
-        <v>1000000</v>
+        <v>46321</v>
       </c>
       <c r="Q47" t="s">
-        <v>169</v>
+        <v>168</v>
       </c>
       <c r="R47" t="s">
         <v>171</v>
       </c>
       <c r="S47" t="s">
-        <v>174</v>
+        <v>172</v>
       </c>
       <c r="T47" t="s">
+        <v>175</v>
+      </c>
+      <c r="U47" t="s">
         <v>178</v>
-      </c>
-      <c r="U47" t="s">
-        <v>28</v>
       </c>
       <c r="V47" s="1">
         <v>46321</v>
@@ -3451,31 +3481,31 @@
         <v>73</v>
       </c>
       <c r="N48" t="s">
-        <v>81</v>
+        <v>80</v>
       </c>
       <c r="O48" t="s">
-        <v>136</v>
+        <v>135</v>
       </c>
       <c r="P48">
-        <v>958040</v>
+        <v>46291</v>
       </c>
       <c r="Q48" t="s">
-        <v>168</v>
+        <v>167</v>
       </c>
       <c r="R48" t="s">
-        <v>171</v>
+        <v>170</v>
       </c>
       <c r="S48" t="s">
-        <v>174</v>
+        <v>172</v>
       </c>
       <c r="T48" t="s">
+        <v>175</v>
+      </c>
+      <c r="U48" t="s">
         <v>177</v>
       </c>
-      <c r="U48" t="s">
-        <v>182</v>
-      </c>
       <c r="V48" s="1">
-        <v>46291</v>
+        <v>46352</v>
       </c>
     </row>
     <row r="49" spans="1:22">
@@ -3510,89 +3540,89 @@
         <v>70</v>
       </c>
       <c r="N49" t="s">
-        <v>81</v>
+        <v>80</v>
       </c>
       <c r="O49" t="s">
-        <v>136</v>
+        <v>135</v>
       </c>
       <c r="P49">
-        <v>41730.64</v>
+        <v>46199</v>
       </c>
       <c r="Q49" t="s">
-        <v>168</v>
+        <v>167</v>
       </c>
       <c r="R49" t="s">
-        <v>173</v>
+        <v>170</v>
       </c>
       <c r="S49" t="s">
-        <v>174</v>
+        <v>172</v>
       </c>
       <c r="T49" t="s">
+        <v>176</v>
+      </c>
+      <c r="U49" t="s">
         <v>177</v>
       </c>
-      <c r="U49" t="s">
-        <v>182</v>
-      </c>
       <c r="V49" s="1">
-        <v>46199</v>
+        <v>46352</v>
       </c>
     </row>
     <row r="50" spans="1:22">
       <c r="A50">
-        <v>17765</v>
+        <v>17760</v>
       </c>
       <c r="B50" t="s">
         <v>22</v>
       </c>
+      <c r="C50" t="s">
+        <v>22</v>
+      </c>
       <c r="D50" t="s">
-        <v>26</v>
+        <v>24</v>
       </c>
       <c r="E50" t="s">
         <v>28</v>
       </c>
       <c r="F50" t="s">
-        <v>38</v>
-      </c>
-      <c r="G50" t="s">
-        <v>44</v>
-      </c>
-      <c r="H50" s="1">
-        <v>46280</v>
-      </c>
-      <c r="I50" t="s">
-        <v>55</v>
+        <v>30</v>
+      </c>
+      <c r="J50" t="s">
+        <v>69</v>
+      </c>
+      <c r="K50" t="s">
+        <v>75</v>
       </c>
       <c r="N50" t="s">
-        <v>86</v>
+        <v>85</v>
       </c>
       <c r="O50" t="s">
-        <v>137</v>
+        <v>136</v>
       </c>
       <c r="P50">
-        <v>859536.0699999999</v>
+        <v>46260</v>
       </c>
       <c r="Q50" t="s">
-        <v>169</v>
+        <v>168</v>
       </c>
       <c r="R50" t="s">
-        <v>172</v>
+        <v>171</v>
       </c>
       <c r="S50" t="s">
-        <v>174</v>
+        <v>172</v>
       </c>
       <c r="T50" t="s">
+        <v>175</v>
+      </c>
+      <c r="U50" t="s">
         <v>179</v>
       </c>
-      <c r="U50" t="s">
-        <v>182</v>
-      </c>
       <c r="V50" s="1">
-        <v>46260</v>
+        <v>46321</v>
       </c>
     </row>
     <row r="51" spans="1:22">
       <c r="A51">
-        <v>17760</v>
+        <v>17761</v>
       </c>
       <c r="B51" t="s">
         <v>22</v>
@@ -3613,39 +3643,39 @@
         <v>69</v>
       </c>
       <c r="K51" t="s">
-        <v>75</v>
+        <v>72</v>
       </c>
       <c r="N51" t="s">
-        <v>86</v>
+        <v>85</v>
       </c>
       <c r="O51" t="s">
         <v>137</v>
       </c>
       <c r="P51">
-        <v>608623.25</v>
+        <v>46291</v>
       </c>
       <c r="Q51" t="s">
-        <v>169</v>
+        <v>168</v>
       </c>
       <c r="R51" t="s">
-        <v>172</v>
+        <v>171</v>
       </c>
       <c r="S51" t="s">
-        <v>174</v>
+        <v>172</v>
       </c>
       <c r="T51" t="s">
+        <v>175</v>
+      </c>
+      <c r="U51" t="s">
         <v>179</v>
       </c>
-      <c r="U51" t="s">
-        <v>182</v>
-      </c>
       <c r="V51" s="1">
-        <v>46260</v>
+        <v>46352</v>
       </c>
     </row>
     <row r="52" spans="1:22">
       <c r="A52">
-        <v>17761</v>
+        <v>17762</v>
       </c>
       <c r="B52" t="s">
         <v>22</v>
@@ -3662,43 +3692,40 @@
       <c r="F52" t="s">
         <v>30</v>
       </c>
-      <c r="J52" t="s">
-        <v>69</v>
-      </c>
       <c r="K52" t="s">
-        <v>72</v>
+        <v>74</v>
       </c>
       <c r="N52" t="s">
-        <v>86</v>
+        <v>85</v>
       </c>
       <c r="O52" t="s">
         <v>138</v>
       </c>
       <c r="P52">
-        <v>559040.0699999999</v>
+        <v>46321</v>
       </c>
       <c r="Q52" t="s">
-        <v>169</v>
+        <v>168</v>
       </c>
       <c r="R52" t="s">
-        <v>172</v>
+        <v>171</v>
       </c>
       <c r="S52" t="s">
-        <v>174</v>
+        <v>172</v>
       </c>
       <c r="T52" t="s">
+        <v>175</v>
+      </c>
+      <c r="U52" t="s">
         <v>179</v>
       </c>
-      <c r="U52" t="s">
-        <v>182</v>
-      </c>
       <c r="V52" s="1">
-        <v>46291</v>
+        <v>46382</v>
       </c>
     </row>
     <row r="53" spans="1:22">
       <c r="A53">
-        <v>17762</v>
+        <v>17763</v>
       </c>
       <c r="B53" t="s">
         <v>22</v>
@@ -3707,40 +3734,46 @@
         <v>22</v>
       </c>
       <c r="D53" t="s">
-        <v>24</v>
+        <v>26</v>
       </c>
       <c r="E53" t="s">
         <v>28</v>
       </c>
       <c r="F53" t="s">
-        <v>30</v>
-      </c>
-      <c r="K53" t="s">
-        <v>74</v>
+        <v>38</v>
+      </c>
+      <c r="G53" t="s">
+        <v>44</v>
+      </c>
+      <c r="H53" s="1">
+        <v>46227</v>
+      </c>
+      <c r="I53" t="s">
+        <v>63</v>
       </c>
       <c r="N53" t="s">
-        <v>86</v>
+        <v>85</v>
       </c>
       <c r="O53" t="s">
-        <v>139</v>
+        <v>136</v>
       </c>
       <c r="P53">
-        <v>1704503</v>
+        <v>46229</v>
       </c>
       <c r="Q53" t="s">
-        <v>169</v>
+        <v>168</v>
       </c>
       <c r="R53" t="s">
-        <v>172</v>
+        <v>171</v>
       </c>
       <c r="S53" t="s">
-        <v>174</v>
+        <v>172</v>
       </c>
       <c r="T53" t="s">
+        <v>175</v>
+      </c>
+      <c r="U53" t="s">
         <v>179</v>
-      </c>
-      <c r="U53" t="s">
-        <v>182</v>
       </c>
       <c r="V53" s="1">
         <v>46321</v>
@@ -3748,12 +3781,9 @@
     </row>
     <row r="54" spans="1:22">
       <c r="A54">
-        <v>17763</v>
+        <v>17764</v>
       </c>
       <c r="B54" t="s">
-        <v>22</v>
-      </c>
-      <c r="C54" t="s">
         <v>22</v>
       </c>
       <c r="D54" t="s">
@@ -3769,42 +3799,42 @@
         <v>44</v>
       </c>
       <c r="H54" s="1">
-        <v>46227</v>
+        <v>46280</v>
       </c>
       <c r="I54" t="s">
-        <v>63</v>
+        <v>55</v>
       </c>
       <c r="N54" t="s">
-        <v>86</v>
+        <v>85</v>
       </c>
       <c r="O54" t="s">
         <v>137</v>
       </c>
       <c r="P54">
-        <v>236343.68</v>
+        <v>46291</v>
       </c>
       <c r="Q54" t="s">
-        <v>169</v>
+        <v>168</v>
       </c>
       <c r="R54" t="s">
-        <v>172</v>
+        <v>171</v>
       </c>
       <c r="S54" t="s">
-        <v>174</v>
+        <v>172</v>
       </c>
       <c r="T54" t="s">
+        <v>175</v>
+      </c>
+      <c r="U54" t="s">
         <v>179</v>
       </c>
-      <c r="U54" t="s">
-        <v>182</v>
-      </c>
       <c r="V54" s="1">
-        <v>46229</v>
+        <v>46352</v>
       </c>
     </row>
     <row r="55" spans="1:22">
       <c r="A55">
-        <v>17764</v>
+        <v>17765</v>
       </c>
       <c r="B55" t="s">
         <v>22</v>
@@ -3828,31 +3858,31 @@
         <v>55</v>
       </c>
       <c r="N55" t="s">
-        <v>86</v>
+        <v>85</v>
       </c>
       <c r="O55" t="s">
-        <v>138</v>
+        <v>136</v>
       </c>
       <c r="P55">
-        <v>1145462.93</v>
+        <v>46260</v>
       </c>
       <c r="Q55" t="s">
-        <v>169</v>
+        <v>168</v>
       </c>
       <c r="R55" t="s">
-        <v>172</v>
+        <v>171</v>
       </c>
       <c r="S55" t="s">
-        <v>174</v>
+        <v>172</v>
       </c>
       <c r="T55" t="s">
+        <v>175</v>
+      </c>
+      <c r="U55" t="s">
         <v>179</v>
       </c>
-      <c r="U55" t="s">
-        <v>182</v>
-      </c>
       <c r="V55" s="1">
-        <v>46291</v>
+        <v>46321</v>
       </c>
     </row>
     <row r="56" spans="1:22">
@@ -3881,31 +3911,31 @@
         <v>76</v>
       </c>
       <c r="N56" t="s">
-        <v>86</v>
+        <v>85</v>
       </c>
       <c r="O56" t="s">
-        <v>140</v>
+        <v>139</v>
       </c>
       <c r="P56">
-        <v>1295422.28</v>
+        <v>46352</v>
       </c>
       <c r="Q56" t="s">
-        <v>169</v>
+        <v>168</v>
       </c>
       <c r="R56" t="s">
-        <v>172</v>
+        <v>171</v>
       </c>
       <c r="S56" t="s">
-        <v>174</v>
+        <v>172</v>
       </c>
       <c r="T56" t="s">
+        <v>175</v>
+      </c>
+      <c r="U56" t="s">
         <v>179</v>
       </c>
-      <c r="U56" t="s">
-        <v>182</v>
-      </c>
       <c r="V56" s="1">
-        <v>46352</v>
+        <v>46049</v>
       </c>
     </row>
     <row r="57" spans="1:22">
@@ -3934,31 +3964,31 @@
         <v>77</v>
       </c>
       <c r="N57" t="s">
-        <v>90</v>
+        <v>89</v>
       </c>
       <c r="O57" t="s">
-        <v>141</v>
+        <v>140</v>
       </c>
       <c r="P57">
-        <v>1962977.67</v>
+        <v>46321</v>
       </c>
       <c r="Q57" t="s">
-        <v>169</v>
+        <v>168</v>
       </c>
       <c r="R57" t="s">
-        <v>172</v>
+        <v>171</v>
       </c>
       <c r="S57" t="s">
-        <v>176</v>
+        <v>174</v>
       </c>
       <c r="T57" t="s">
+        <v>175</v>
+      </c>
+      <c r="U57" t="s">
         <v>180</v>
       </c>
-      <c r="U57" t="s">
-        <v>182</v>
-      </c>
       <c r="V57" s="1">
-        <v>46321</v>
+        <v>46049</v>
       </c>
     </row>
     <row r="58" spans="1:22">
@@ -3981,31 +4011,31 @@
         <v>45</v>
       </c>
       <c r="N58" t="s">
-        <v>90</v>
+        <v>89</v>
       </c>
       <c r="O58" t="s">
-        <v>141</v>
+        <v>140</v>
       </c>
       <c r="P58">
-        <v>2497091</v>
+        <v>46321</v>
       </c>
       <c r="Q58" t="s">
-        <v>169</v>
+        <v>168</v>
       </c>
       <c r="R58" t="s">
-        <v>172</v>
+        <v>171</v>
       </c>
       <c r="S58" t="s">
-        <v>176</v>
+        <v>174</v>
       </c>
       <c r="T58" t="s">
+        <v>175</v>
+      </c>
+      <c r="U58" t="s">
         <v>180</v>
       </c>
-      <c r="U58" t="s">
-        <v>182</v>
-      </c>
       <c r="V58" s="1">
-        <v>46321</v>
+        <v>46049</v>
       </c>
     </row>
     <row r="59" spans="1:22">
@@ -4028,28 +4058,31 @@
         <v>43</v>
       </c>
       <c r="N59" t="s">
-        <v>90</v>
+        <v>89</v>
       </c>
       <c r="O59" t="s">
-        <v>142</v>
+        <v>141</v>
+      </c>
+      <c r="P59">
+        <v>46049</v>
       </c>
       <c r="Q59" t="s">
-        <v>169</v>
+        <v>168</v>
       </c>
       <c r="R59" t="s">
-        <v>172</v>
+        <v>171</v>
       </c>
       <c r="S59" t="s">
-        <v>176</v>
+        <v>174</v>
       </c>
       <c r="T59" t="s">
+        <v>175</v>
+      </c>
+      <c r="U59" t="s">
         <v>180</v>
       </c>
-      <c r="U59" t="s">
-        <v>182</v>
-      </c>
       <c r="V59" s="1">
-        <v>46049</v>
+        <v>46139</v>
       </c>
     </row>
     <row r="60" spans="1:22">
@@ -4072,25 +4105,25 @@
         <v>43</v>
       </c>
       <c r="N60" t="s">
-        <v>90</v>
+        <v>89</v>
       </c>
       <c r="O60" t="s">
-        <v>143</v>
+        <v>142</v>
       </c>
       <c r="Q60" t="s">
-        <v>169</v>
+        <v>168</v>
       </c>
       <c r="R60" t="s">
-        <v>172</v>
+        <v>171</v>
       </c>
       <c r="S60" t="s">
-        <v>176</v>
+        <v>174</v>
       </c>
       <c r="T60" t="s">
+        <v>175</v>
+      </c>
+      <c r="U60" t="s">
         <v>180</v>
-      </c>
-      <c r="U60" t="s">
-        <v>182</v>
       </c>
     </row>
     <row r="61" spans="1:22">
@@ -4113,30 +4146,30 @@
         <v>43</v>
       </c>
       <c r="N61" t="s">
-        <v>90</v>
+        <v>89</v>
       </c>
       <c r="O61" t="s">
-        <v>144</v>
+        <v>143</v>
       </c>
       <c r="Q61" t="s">
-        <v>169</v>
+        <v>168</v>
       </c>
       <c r="R61" t="s">
-        <v>172</v>
+        <v>171</v>
       </c>
       <c r="S61" t="s">
-        <v>176</v>
+        <v>174</v>
       </c>
       <c r="T61" t="s">
+        <v>175</v>
+      </c>
+      <c r="U61" t="s">
         <v>180</v>
-      </c>
-      <c r="U61" t="s">
-        <v>182</v>
       </c>
     </row>
     <row r="62" spans="1:22">
       <c r="A62">
-        <v>23120</v>
+        <v>23080</v>
       </c>
       <c r="B62" t="s">
         <v>22</v>
@@ -4151,36 +4184,36 @@
         <v>29</v>
       </c>
       <c r="N62" t="s">
-        <v>91</v>
+        <v>90</v>
       </c>
       <c r="O62" t="s">
-        <v>145</v>
+        <v>144</v>
       </c>
       <c r="P62">
-        <v>9389.959999999999</v>
+        <v>46107</v>
       </c>
       <c r="Q62" t="s">
         <v>168</v>
       </c>
       <c r="R62" t="s">
+        <v>171</v>
+      </c>
+      <c r="S62" t="s">
         <v>173</v>
       </c>
-      <c r="S62" t="s">
-        <v>175</v>
-      </c>
       <c r="T62" t="s">
+        <v>176</v>
+      </c>
+      <c r="U62" t="s">
         <v>177</v>
       </c>
-      <c r="U62" t="s">
-        <v>182</v>
-      </c>
       <c r="V62" s="1">
-        <v>46107</v>
+        <v>46168</v>
       </c>
     </row>
     <row r="63" spans="1:22">
       <c r="A63">
-        <v>23160</v>
+        <v>23100</v>
       </c>
       <c r="B63" t="s">
         <v>22</v>
@@ -4195,36 +4228,36 @@
         <v>29</v>
       </c>
       <c r="N63" t="s">
-        <v>92</v>
+        <v>91</v>
       </c>
       <c r="O63" t="s">
-        <v>146</v>
+        <v>145</v>
       </c>
       <c r="P63">
-        <v>7204.82</v>
+        <v>46107</v>
       </c>
       <c r="Q63" t="s">
-        <v>168</v>
+        <v>167</v>
       </c>
       <c r="R63" t="s">
+        <v>170</v>
+      </c>
+      <c r="S63" t="s">
         <v>173</v>
       </c>
-      <c r="S63" t="s">
-        <v>175</v>
-      </c>
       <c r="T63" t="s">
+        <v>176</v>
+      </c>
+      <c r="U63" t="s">
         <v>177</v>
       </c>
-      <c r="U63" t="s">
-        <v>182</v>
-      </c>
       <c r="V63" s="1">
-        <v>46107</v>
+        <v>46168</v>
       </c>
     </row>
     <row r="64" spans="1:22">
       <c r="A64">
-        <v>23100</v>
+        <v>23120</v>
       </c>
       <c r="B64" t="s">
         <v>22</v>
@@ -4239,36 +4272,36 @@
         <v>29</v>
       </c>
       <c r="N64" t="s">
-        <v>93</v>
+        <v>92</v>
       </c>
       <c r="O64" t="s">
-        <v>147</v>
+        <v>146</v>
       </c>
       <c r="P64">
-        <v>4227.84</v>
+        <v>46107</v>
       </c>
       <c r="Q64" t="s">
-        <v>168</v>
+        <v>167</v>
       </c>
       <c r="R64" t="s">
+        <v>170</v>
+      </c>
+      <c r="S64" t="s">
         <v>173</v>
       </c>
-      <c r="S64" t="s">
-        <v>175</v>
-      </c>
       <c r="T64" t="s">
+        <v>176</v>
+      </c>
+      <c r="U64" t="s">
         <v>177</v>
       </c>
-      <c r="U64" t="s">
-        <v>182</v>
-      </c>
       <c r="V64" s="1">
-        <v>46107</v>
+        <v>46168</v>
       </c>
     </row>
     <row r="65" spans="1:22">
       <c r="A65">
-        <v>23080</v>
+        <v>23140</v>
       </c>
       <c r="B65" t="s">
         <v>22</v>
@@ -4283,36 +4316,36 @@
         <v>29</v>
       </c>
       <c r="N65" t="s">
-        <v>94</v>
+        <v>93</v>
       </c>
       <c r="O65" t="s">
-        <v>148</v>
+        <v>147</v>
       </c>
       <c r="P65">
-        <v>4064.54</v>
+        <v>46107</v>
       </c>
       <c r="Q65" t="s">
         <v>169</v>
       </c>
       <c r="R65" t="s">
+        <v>170</v>
+      </c>
+      <c r="S65" t="s">
         <v>173</v>
       </c>
-      <c r="S65" t="s">
-        <v>175</v>
-      </c>
       <c r="T65" t="s">
+        <v>176</v>
+      </c>
+      <c r="U65" t="s">
         <v>177</v>
       </c>
-      <c r="U65" t="s">
-        <v>182</v>
-      </c>
       <c r="V65" s="1">
-        <v>46107</v>
+        <v>46168</v>
       </c>
     </row>
     <row r="66" spans="1:22">
       <c r="A66">
-        <v>23180</v>
+        <v>23160</v>
       </c>
       <c r="B66" t="s">
         <v>22</v>
@@ -4327,36 +4360,36 @@
         <v>29</v>
       </c>
       <c r="N66" t="s">
-        <v>95</v>
+        <v>94</v>
       </c>
       <c r="O66" t="s">
-        <v>147</v>
+        <v>148</v>
       </c>
       <c r="P66">
-        <v>3662.66</v>
+        <v>46107</v>
       </c>
       <c r="Q66" t="s">
-        <v>168</v>
+        <v>167</v>
       </c>
       <c r="R66" t="s">
+        <v>170</v>
+      </c>
+      <c r="S66" t="s">
         <v>173</v>
       </c>
-      <c r="S66" t="s">
-        <v>175</v>
-      </c>
       <c r="T66" t="s">
+        <v>176</v>
+      </c>
+      <c r="U66" t="s">
         <v>177</v>
       </c>
-      <c r="U66" t="s">
-        <v>182</v>
-      </c>
       <c r="V66" s="1">
-        <v>46107</v>
+        <v>46168</v>
       </c>
     </row>
     <row r="67" spans="1:22">
       <c r="A67">
-        <v>23140</v>
+        <v>23180</v>
       </c>
       <c r="B67" t="s">
         <v>22</v>
@@ -4371,31 +4404,31 @@
         <v>29</v>
       </c>
       <c r="N67" t="s">
-        <v>96</v>
+        <v>95</v>
       </c>
       <c r="O67" t="s">
-        <v>149</v>
+        <v>145</v>
       </c>
       <c r="P67">
-        <v>1163.64</v>
+        <v>46107</v>
       </c>
       <c r="Q67" t="s">
+        <v>167</v>
+      </c>
+      <c r="R67" t="s">
         <v>170</v>
       </c>
-      <c r="R67" t="s">
+      <c r="S67" t="s">
         <v>173</v>
       </c>
-      <c r="S67" t="s">
-        <v>175</v>
-      </c>
       <c r="T67" t="s">
+        <v>176</v>
+      </c>
+      <c r="U67" t="s">
         <v>177</v>
       </c>
-      <c r="U67" t="s">
-        <v>182</v>
-      </c>
       <c r="V67" s="1">
-        <v>46107</v>
+        <v>46168</v>
       </c>
     </row>
     <row r="68" spans="1:22">
@@ -4415,28 +4448,28 @@
         <v>29</v>
       </c>
       <c r="N68" t="s">
-        <v>82</v>
+        <v>81</v>
       </c>
       <c r="O68" t="s">
-        <v>150</v>
+        <v>149</v>
       </c>
       <c r="P68">
-        <v>120000</v>
+        <v>46168</v>
       </c>
       <c r="Q68" t="s">
-        <v>168</v>
+        <v>167</v>
       </c>
       <c r="R68" t="s">
-        <v>172</v>
+        <v>170</v>
       </c>
       <c r="S68" t="s">
-        <v>175</v>
+        <v>173</v>
       </c>
       <c r="T68" t="s">
+        <v>175</v>
+      </c>
+      <c r="U68" t="s">
         <v>177</v>
-      </c>
-      <c r="U68" t="s">
-        <v>28</v>
       </c>
       <c r="V68" s="1">
         <v>46168</v>
@@ -4465,28 +4498,31 @@
         <v>43</v>
       </c>
       <c r="N69" t="s">
-        <v>81</v>
+        <v>80</v>
       </c>
       <c r="O69" t="s">
-        <v>151</v>
+        <v>150</v>
+      </c>
+      <c r="P69">
+        <v>46291</v>
       </c>
       <c r="Q69" t="s">
-        <v>168</v>
+        <v>167</v>
       </c>
       <c r="R69" t="s">
-        <v>171</v>
+        <v>170</v>
       </c>
       <c r="S69" t="s">
-        <v>174</v>
+        <v>172</v>
       </c>
       <c r="T69" t="s">
+        <v>175</v>
+      </c>
+      <c r="U69" t="s">
         <v>177</v>
       </c>
-      <c r="U69" t="s">
-        <v>28</v>
-      </c>
       <c r="V69" s="1">
-        <v>46291</v>
+        <v>46382</v>
       </c>
     </row>
     <row r="70" spans="1:22">
@@ -4515,31 +4551,31 @@
         <v>73</v>
       </c>
       <c r="N70" t="s">
-        <v>85</v>
+        <v>84</v>
       </c>
       <c r="O70" t="s">
-        <v>152</v>
+        <v>151</v>
       </c>
       <c r="P70">
-        <v>100000</v>
+        <v>46229</v>
       </c>
       <c r="Q70" t="s">
+        <v>169</v>
+      </c>
+      <c r="R70" t="s">
         <v>170</v>
       </c>
-      <c r="R70" t="s">
-        <v>171</v>
-      </c>
       <c r="S70" t="s">
-        <v>174</v>
+        <v>172</v>
       </c>
       <c r="T70" t="s">
+        <v>175</v>
+      </c>
+      <c r="U70" t="s">
         <v>177</v>
       </c>
-      <c r="U70" t="s">
-        <v>182</v>
-      </c>
       <c r="V70" s="1">
-        <v>46229</v>
+        <v>46291</v>
       </c>
     </row>
     <row r="71" spans="1:22">
@@ -4559,28 +4595,28 @@
         <v>29</v>
       </c>
       <c r="N71" t="s">
-        <v>82</v>
+        <v>81</v>
       </c>
       <c r="O71" t="s">
-        <v>153</v>
+        <v>152</v>
       </c>
       <c r="P71">
-        <v>80000</v>
+        <v>46260</v>
       </c>
       <c r="Q71" t="s">
-        <v>168</v>
+        <v>167</v>
       </c>
       <c r="R71" t="s">
-        <v>172</v>
+        <v>170</v>
       </c>
       <c r="S71" t="s">
-        <v>175</v>
+        <v>173</v>
       </c>
       <c r="T71" t="s">
+        <v>175</v>
+      </c>
+      <c r="U71" t="s">
         <v>177</v>
-      </c>
-      <c r="U71" t="s">
-        <v>28</v>
       </c>
       <c r="V71" s="1">
         <v>46260</v>
@@ -4603,31 +4639,31 @@
         <v>29</v>
       </c>
       <c r="N72" t="s">
-        <v>81</v>
+        <v>80</v>
       </c>
       <c r="O72" t="s">
-        <v>154</v>
+        <v>153</v>
       </c>
       <c r="P72">
-        <v>835000</v>
+        <v>46291</v>
       </c>
       <c r="Q72" t="s">
-        <v>168</v>
+        <v>167</v>
       </c>
       <c r="R72" t="s">
-        <v>171</v>
+        <v>170</v>
       </c>
       <c r="S72" t="s">
-        <v>175</v>
+        <v>173</v>
       </c>
       <c r="T72" t="s">
+        <v>175</v>
+      </c>
+      <c r="U72" t="s">
         <v>177</v>
       </c>
-      <c r="U72" t="s">
-        <v>182</v>
-      </c>
       <c r="V72" s="1">
-        <v>46291</v>
+        <v>46352</v>
       </c>
     </row>
     <row r="73" spans="1:22">
@@ -4647,31 +4683,31 @@
         <v>29</v>
       </c>
       <c r="N73" t="s">
-        <v>81</v>
+        <v>80</v>
       </c>
       <c r="O73" t="s">
-        <v>154</v>
+        <v>153</v>
       </c>
       <c r="P73">
-        <v>165000</v>
+        <v>46168</v>
       </c>
       <c r="Q73" t="s">
-        <v>168</v>
+        <v>167</v>
       </c>
       <c r="R73" t="s">
-        <v>171</v>
+        <v>170</v>
       </c>
       <c r="S73" t="s">
-        <v>175</v>
+        <v>173</v>
       </c>
       <c r="T73" t="s">
+        <v>175</v>
+      </c>
+      <c r="U73" t="s">
         <v>177</v>
       </c>
-      <c r="U73" t="s">
-        <v>182</v>
-      </c>
       <c r="V73" s="1">
-        <v>46168</v>
+        <v>46229</v>
       </c>
     </row>
     <row r="74" spans="1:22">
@@ -4691,31 +4727,31 @@
         <v>29</v>
       </c>
       <c r="N74" t="s">
-        <v>81</v>
+        <v>80</v>
       </c>
       <c r="O74" t="s">
-        <v>155</v>
+        <v>154</v>
       </c>
       <c r="P74">
-        <v>1000000</v>
+        <v>46291</v>
       </c>
       <c r="Q74" t="s">
-        <v>168</v>
+        <v>167</v>
       </c>
       <c r="R74" t="s">
-        <v>171</v>
+        <v>170</v>
       </c>
       <c r="S74" t="s">
-        <v>175</v>
+        <v>173</v>
       </c>
       <c r="T74" t="s">
+        <v>175</v>
+      </c>
+      <c r="U74" t="s">
         <v>177</v>
       </c>
-      <c r="U74" t="s">
-        <v>182</v>
-      </c>
       <c r="V74" s="1">
-        <v>46291</v>
+        <v>46352</v>
       </c>
     </row>
     <row r="75" spans="1:22">
@@ -4735,31 +4771,31 @@
         <v>29</v>
       </c>
       <c r="N75" t="s">
-        <v>81</v>
+        <v>80</v>
       </c>
       <c r="O75" t="s">
-        <v>156</v>
+        <v>155</v>
       </c>
       <c r="P75">
-        <v>1000000</v>
+        <v>46291</v>
       </c>
       <c r="Q75" t="s">
-        <v>168</v>
+        <v>167</v>
       </c>
       <c r="R75" t="s">
-        <v>171</v>
+        <v>170</v>
       </c>
       <c r="S75" t="s">
-        <v>175</v>
+        <v>173</v>
       </c>
       <c r="T75" t="s">
+        <v>175</v>
+      </c>
+      <c r="U75" t="s">
         <v>177</v>
       </c>
-      <c r="U75" t="s">
-        <v>182</v>
-      </c>
       <c r="V75" s="1">
-        <v>46291</v>
+        <v>46352</v>
       </c>
     </row>
     <row r="76" spans="1:22">
@@ -4779,31 +4815,31 @@
         <v>29</v>
       </c>
       <c r="N76" t="s">
-        <v>85</v>
+        <v>84</v>
       </c>
       <c r="O76" t="s">
-        <v>157</v>
+        <v>156</v>
       </c>
       <c r="P76">
-        <v>100000</v>
+        <v>46291</v>
       </c>
       <c r="Q76" t="s">
+        <v>169</v>
+      </c>
+      <c r="R76" t="s">
         <v>170</v>
       </c>
-      <c r="R76" t="s">
-        <v>171</v>
-      </c>
       <c r="S76" t="s">
-        <v>175</v>
+        <v>173</v>
       </c>
       <c r="T76" t="s">
+        <v>175</v>
+      </c>
+      <c r="U76" t="s">
         <v>177</v>
       </c>
-      <c r="U76" t="s">
-        <v>182</v>
-      </c>
       <c r="V76" s="1">
-        <v>46291</v>
+        <v>46352</v>
       </c>
     </row>
     <row r="77" spans="1:22">
@@ -4826,31 +4862,31 @@
         <v>30</v>
       </c>
       <c r="N77" t="s">
-        <v>88</v>
+        <v>87</v>
       </c>
       <c r="O77" t="s">
-        <v>158</v>
+        <v>157</v>
       </c>
       <c r="P77">
-        <v>1000000</v>
+        <v>46321</v>
       </c>
       <c r="Q77" t="s">
-        <v>169</v>
+        <v>168</v>
       </c>
       <c r="R77" t="s">
         <v>171</v>
       </c>
       <c r="S77" t="s">
-        <v>174</v>
+        <v>172</v>
       </c>
       <c r="T77" t="s">
+        <v>175</v>
+      </c>
+      <c r="U77" t="s">
         <v>178</v>
       </c>
-      <c r="U77" t="s">
-        <v>28</v>
-      </c>
       <c r="V77" s="1">
-        <v>46321</v>
+        <v>46382</v>
       </c>
     </row>
     <row r="78" spans="1:22">
@@ -4876,31 +4912,31 @@
         <v>46</v>
       </c>
       <c r="N78" t="s">
-        <v>86</v>
+        <v>85</v>
       </c>
       <c r="O78" t="s">
-        <v>159</v>
+        <v>158</v>
       </c>
       <c r="P78">
-        <v>1704503</v>
+        <v>46381</v>
       </c>
       <c r="Q78" t="s">
-        <v>169</v>
+        <v>168</v>
       </c>
       <c r="R78" t="s">
-        <v>172</v>
+        <v>171</v>
       </c>
       <c r="S78" t="s">
         <v>42</v>
       </c>
       <c r="T78" t="s">
+        <v>175</v>
+      </c>
+      <c r="U78" t="s">
         <v>179</v>
       </c>
-      <c r="U78" t="s">
-        <v>182</v>
-      </c>
       <c r="V78" s="1">
-        <v>46381</v>
+        <v>46107</v>
       </c>
     </row>
     <row r="79" spans="1:22">
@@ -4926,31 +4962,31 @@
         <v>46</v>
       </c>
       <c r="N79" t="s">
-        <v>86</v>
+        <v>85</v>
       </c>
       <c r="O79" t="s">
-        <v>160</v>
+        <v>159</v>
       </c>
       <c r="P79">
-        <v>1638125.5</v>
+        <v>46381</v>
       </c>
       <c r="Q79" t="s">
-        <v>169</v>
+        <v>168</v>
       </c>
       <c r="R79" t="s">
-        <v>172</v>
+        <v>171</v>
       </c>
       <c r="S79" t="s">
         <v>42</v>
       </c>
       <c r="T79" t="s">
+        <v>175</v>
+      </c>
+      <c r="U79" t="s">
         <v>179</v>
       </c>
-      <c r="U79" t="s">
-        <v>182</v>
-      </c>
       <c r="V79" s="1">
-        <v>46381</v>
+        <v>46138</v>
       </c>
     </row>
     <row r="80" spans="1:22">
@@ -4976,31 +5012,31 @@
         <v>46</v>
       </c>
       <c r="N80" t="s">
-        <v>84</v>
+        <v>83</v>
       </c>
       <c r="O80" t="s">
-        <v>161</v>
+        <v>160</v>
       </c>
       <c r="P80">
-        <v>3800000</v>
+        <v>46381</v>
       </c>
       <c r="Q80" t="s">
-        <v>169</v>
+        <v>168</v>
       </c>
       <c r="R80" t="s">
-        <v>172</v>
+        <v>171</v>
       </c>
       <c r="S80" t="s">
         <v>42</v>
       </c>
       <c r="T80" t="s">
+        <v>175</v>
+      </c>
+      <c r="U80" t="s">
         <v>178</v>
       </c>
-      <c r="U80" t="s">
-        <v>28</v>
-      </c>
       <c r="V80" s="1">
-        <v>46381</v>
+        <v>46260</v>
       </c>
     </row>
     <row r="81" spans="1:22">
@@ -5026,31 +5062,31 @@
         <v>46</v>
       </c>
       <c r="N81" t="s">
-        <v>84</v>
+        <v>83</v>
       </c>
       <c r="O81" t="s">
-        <v>162</v>
+        <v>161</v>
       </c>
       <c r="P81">
-        <v>3800000</v>
+        <v>46381</v>
       </c>
       <c r="Q81" t="s">
-        <v>169</v>
+        <v>168</v>
       </c>
       <c r="R81" t="s">
-        <v>172</v>
+        <v>171</v>
       </c>
       <c r="S81" t="s">
         <v>42</v>
       </c>
       <c r="T81" t="s">
+        <v>175</v>
+      </c>
+      <c r="U81" t="s">
         <v>178</v>
       </c>
-      <c r="U81" t="s">
-        <v>28</v>
-      </c>
       <c r="V81" s="1">
-        <v>46381</v>
+        <v>46260</v>
       </c>
     </row>
     <row r="82" spans="1:22">
@@ -5076,31 +5112,31 @@
         <v>78</v>
       </c>
       <c r="N82" t="s">
-        <v>89</v>
+        <v>88</v>
       </c>
       <c r="O82" t="s">
-        <v>163</v>
+        <v>162</v>
       </c>
       <c r="P82">
-        <v>3800000</v>
+        <v>46382</v>
       </c>
       <c r="Q82" t="s">
-        <v>169</v>
+        <v>168</v>
       </c>
       <c r="R82" t="s">
-        <v>172</v>
+        <v>171</v>
       </c>
       <c r="S82" t="s">
-        <v>175</v>
+        <v>173</v>
       </c>
       <c r="T82" t="s">
+        <v>175</v>
+      </c>
+      <c r="U82" t="s">
         <v>178</v>
       </c>
-      <c r="U82" t="s">
-        <v>28</v>
-      </c>
       <c r="V82" s="1">
-        <v>46382</v>
+        <v>46108</v>
       </c>
     </row>
     <row r="83" spans="1:22">
@@ -5120,31 +5156,31 @@
         <v>28</v>
       </c>
       <c r="N83" t="s">
+        <v>96</v>
+      </c>
+      <c r="O83" t="s">
         <v>97</v>
       </c>
-      <c r="O83" t="s">
-        <v>98</v>
-      </c>
       <c r="P83">
-        <v>4394700</v>
+        <v>46382</v>
       </c>
       <c r="Q83" t="s">
-        <v>168</v>
+        <v>167</v>
       </c>
       <c r="R83" t="s">
-        <v>171</v>
+        <v>170</v>
       </c>
       <c r="S83" t="s">
-        <v>175</v>
+        <v>173</v>
       </c>
       <c r="T83" t="s">
+        <v>175</v>
+      </c>
+      <c r="U83" t="s">
         <v>178</v>
       </c>
-      <c r="U83" t="s">
-        <v>28</v>
-      </c>
       <c r="V83" s="1">
-        <v>46382</v>
+        <v>46108</v>
       </c>
     </row>
     <row r="84" spans="1:22">
@@ -5170,34 +5206,34 @@
         <v>64</v>
       </c>
       <c r="K84" t="s">
-        <v>79</v>
+        <v>72</v>
       </c>
       <c r="N84" t="s">
-        <v>86</v>
+        <v>85</v>
       </c>
       <c r="O84" t="s">
-        <v>164</v>
+        <v>163</v>
       </c>
       <c r="P84">
-        <v>528395.9300000001</v>
+        <v>46382</v>
       </c>
       <c r="Q84" t="s">
-        <v>169</v>
+        <v>168</v>
       </c>
       <c r="R84" t="s">
-        <v>172</v>
+        <v>171</v>
       </c>
       <c r="S84" t="s">
-        <v>174</v>
+        <v>172</v>
       </c>
       <c r="T84" t="s">
+        <v>175</v>
+      </c>
+      <c r="U84" t="s">
         <v>179</v>
       </c>
-      <c r="U84" t="s">
-        <v>182</v>
-      </c>
       <c r="V84" s="1">
-        <v>46382</v>
+        <v>46080</v>
       </c>
     </row>
     <row r="85" spans="1:22">
@@ -5220,31 +5256,31 @@
         <v>30</v>
       </c>
       <c r="N85" t="s">
-        <v>88</v>
+        <v>87</v>
       </c>
       <c r="O85" t="s">
-        <v>165</v>
+        <v>164</v>
       </c>
       <c r="P85">
-        <v>1000000</v>
+        <v>46321</v>
       </c>
       <c r="Q85" t="s">
-        <v>169</v>
+        <v>168</v>
       </c>
       <c r="R85" t="s">
         <v>171</v>
       </c>
       <c r="S85" t="s">
-        <v>174</v>
+        <v>172</v>
       </c>
       <c r="T85" t="s">
+        <v>175</v>
+      </c>
+      <c r="U85" t="s">
         <v>178</v>
       </c>
-      <c r="U85" t="s">
-        <v>28</v>
-      </c>
       <c r="V85" s="1">
-        <v>46321</v>
+        <v>46382</v>
       </c>
     </row>
     <row r="86" spans="1:22">
@@ -5264,31 +5300,31 @@
         <v>28</v>
       </c>
       <c r="N86" t="s">
+        <v>96</v>
+      </c>
+      <c r="O86" t="s">
         <v>97</v>
       </c>
-      <c r="O86" t="s">
-        <v>98</v>
-      </c>
       <c r="P86">
-        <v>4394700</v>
+        <v>46382</v>
       </c>
       <c r="Q86" t="s">
-        <v>168</v>
+        <v>167</v>
       </c>
       <c r="R86" t="s">
-        <v>171</v>
+        <v>170</v>
       </c>
       <c r="S86" t="s">
-        <v>175</v>
+        <v>173</v>
       </c>
       <c r="T86" t="s">
+        <v>175</v>
+      </c>
+      <c r="U86" t="s">
         <v>178</v>
       </c>
-      <c r="U86" t="s">
-        <v>28</v>
-      </c>
       <c r="V86" s="1">
-        <v>46382</v>
+        <v>46108</v>
       </c>
     </row>
     <row r="87" spans="1:22">
@@ -5314,28 +5350,25 @@
         <v>46</v>
       </c>
       <c r="N87" t="s">
-        <v>98</v>
+        <v>97</v>
       </c>
       <c r="O87" t="s">
-        <v>98</v>
-      </c>
-      <c r="P87">
-        <v>3306000</v>
+        <v>97</v>
       </c>
       <c r="Q87" t="s">
-        <v>168</v>
+        <v>167</v>
       </c>
       <c r="R87" t="s">
-        <v>171</v>
+        <v>170</v>
       </c>
       <c r="S87" t="s">
         <v>42</v>
       </c>
       <c r="T87" t="s">
+        <v>175</v>
+      </c>
+      <c r="U87" t="s">
         <v>178</v>
-      </c>
-      <c r="U87" t="s">
-        <v>28</v>
       </c>
     </row>
     <row r="88" spans="1:22">
@@ -5361,28 +5394,25 @@
         <v>46</v>
       </c>
       <c r="N88" t="s">
-        <v>98</v>
+        <v>97</v>
       </c>
       <c r="O88" t="s">
-        <v>98</v>
-      </c>
-      <c r="P88">
-        <v>3306000</v>
+        <v>97</v>
       </c>
       <c r="Q88" t="s">
-        <v>168</v>
+        <v>167</v>
       </c>
       <c r="R88" t="s">
-        <v>171</v>
+        <v>170</v>
       </c>
       <c r="S88" t="s">
         <v>42</v>
       </c>
       <c r="T88" t="s">
+        <v>175</v>
+      </c>
+      <c r="U88" t="s">
         <v>178</v>
-      </c>
-      <c r="U88" t="s">
-        <v>28</v>
       </c>
     </row>
     <row r="89" spans="1:22">
@@ -5405,31 +5435,31 @@
         <v>30</v>
       </c>
       <c r="N89" t="s">
-        <v>99</v>
+        <v>98</v>
       </c>
       <c r="O89" t="s">
-        <v>166</v>
+        <v>165</v>
       </c>
       <c r="P89">
-        <v>470820</v>
+        <v>46291</v>
       </c>
       <c r="Q89" t="s">
-        <v>168</v>
+        <v>167</v>
       </c>
       <c r="R89" t="s">
-        <v>171</v>
+        <v>170</v>
       </c>
       <c r="S89" t="s">
-        <v>174</v>
+        <v>172</v>
       </c>
       <c r="T89" t="s">
+        <v>175</v>
+      </c>
+      <c r="U89" t="s">
         <v>181</v>
       </c>
-      <c r="U89" t="s">
-        <v>28</v>
-      </c>
       <c r="V89" s="1">
-        <v>46291</v>
+        <v>46321</v>
       </c>
     </row>
     <row r="90" spans="1:22">
@@ -5449,31 +5479,31 @@
         <v>30</v>
       </c>
       <c r="N90" t="s">
-        <v>89</v>
+        <v>88</v>
       </c>
       <c r="O90" t="s">
-        <v>167</v>
+        <v>166</v>
       </c>
       <c r="P90">
-        <v>2297180</v>
+        <v>46291</v>
       </c>
       <c r="Q90" t="s">
-        <v>169</v>
+        <v>168</v>
       </c>
       <c r="R90" t="s">
         <v>171</v>
       </c>
       <c r="S90" t="s">
-        <v>174</v>
+        <v>172</v>
       </c>
       <c r="T90" t="s">
+        <v>175</v>
+      </c>
+      <c r="U90" t="s">
         <v>178</v>
       </c>
-      <c r="U90" t="s">
-        <v>28</v>
-      </c>
       <c r="V90" s="1">
-        <v>46291</v>
+        <v>46382</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Atualização automática: mta (28/09/2026 13:06)
</commit_message>
<xml_diff>
--- a/Projetos/02_Dados_Tratados/base_mta_tratada.xlsx
+++ b/Projetos/02_Dados_Tratados/base_mta_tratada.xlsx
@@ -14,7 +14,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1188" uniqueCount="182">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1188" uniqueCount="181">
   <si>
     <t>linha</t>
   </si>
@@ -541,12 +541,6 @@
     <t>D</t>
   </si>
   <si>
-    <t>3</t>
-  </si>
-  <si>
-    <t>4</t>
-  </si>
-  <si>
     <t>REQUISIÇÃO</t>
   </si>
   <si>
@@ -560,6 +554,9 @@
   </si>
   <si>
     <t>CONTRATO</t>
+  </si>
+  <si>
+    <t>Não</t>
   </si>
 </sst>
 </file>
@@ -569,8 +566,16 @@
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="YYYY-MM-DD HH:MM:SS"/>
   </numFmts>
-  <fonts count="1">
+  <fonts count="2">
     <font>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
       <sz val="11"/>
       <color theme="1"/>
       <name val="Calibri"/>
@@ -586,7 +591,7 @@
       <patternFill patternType="gray125"/>
     </fill>
   </fills>
-  <borders count="1">
+  <borders count="2">
     <border>
       <left/>
       <right/>
@@ -594,12 +599,30 @@
       <bottom/>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin">
+        <color auto="1"/>
+      </left>
+      <right style="thin">
+        <color auto="1"/>
+      </right>
+      <top style="thin">
+        <color auto="1"/>
+      </top>
+      <bottom style="thin">
+        <color auto="1"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="3">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
   </cellXfs>
   <cellStyles count="1">
@@ -899,70 +922,70 @@
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:22">
-      <c r="A1" t="s">
+      <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
-      <c r="B1" t="s">
+      <c r="B1" s="1" t="s">
         <v>1</v>
       </c>
-      <c r="C1" t="s">
+      <c r="C1" s="1" t="s">
         <v>2</v>
       </c>
-      <c r="D1" t="s">
+      <c r="D1" s="1" t="s">
         <v>3</v>
       </c>
-      <c r="E1" t="s">
+      <c r="E1" s="1" t="s">
         <v>4</v>
       </c>
-      <c r="F1" t="s">
+      <c r="F1" s="1" t="s">
         <v>5</v>
       </c>
-      <c r="G1" t="s">
+      <c r="G1" s="1" t="s">
         <v>6</v>
       </c>
-      <c r="H1" t="s">
+      <c r="H1" s="1" t="s">
         <v>7</v>
       </c>
-      <c r="I1" t="s">
+      <c r="I1" s="1" t="s">
         <v>8</v>
       </c>
-      <c r="J1" t="s">
+      <c r="J1" s="1" t="s">
         <v>9</v>
       </c>
-      <c r="K1" t="s">
+      <c r="K1" s="1" t="s">
         <v>10</v>
       </c>
-      <c r="L1" t="s">
+      <c r="L1" s="1" t="s">
         <v>11</v>
       </c>
-      <c r="M1" t="s">
+      <c r="M1" s="1" t="s">
         <v>12</v>
       </c>
-      <c r="N1" t="s">
+      <c r="N1" s="1" t="s">
         <v>13</v>
       </c>
-      <c r="O1" t="s">
+      <c r="O1" s="1" t="s">
         <v>14</v>
       </c>
-      <c r="P1" t="s">
+      <c r="P1" s="1" t="s">
         <v>15</v>
       </c>
-      <c r="Q1" t="s">
+      <c r="Q1" s="1" t="s">
         <v>16</v>
       </c>
-      <c r="R1" t="s">
+      <c r="R1" s="1" t="s">
         <v>17</v>
       </c>
-      <c r="S1" t="s">
+      <c r="S1" s="1" t="s">
         <v>18</v>
       </c>
-      <c r="T1" t="s">
+      <c r="T1" s="1" t="s">
         <v>19</v>
       </c>
-      <c r="U1" t="s">
+      <c r="U1" s="1" t="s">
         <v>20</v>
       </c>
-      <c r="V1" t="s">
+      <c r="V1" s="1" t="s">
         <v>21</v>
       </c>
     </row>
@@ -1001,7 +1024,7 @@
         <v>99</v>
       </c>
       <c r="P2">
-        <v>46229</v>
+        <v>135000</v>
       </c>
       <c r="Q2" t="s">
         <v>167</v>
@@ -1016,9 +1039,9 @@
         <v>175</v>
       </c>
       <c r="U2" t="s">
-        <v>177</v>
-      </c>
-      <c r="V2" s="1">
+        <v>180</v>
+      </c>
+      <c r="V2" s="2">
         <v>46291</v>
       </c>
     </row>
@@ -1050,9 +1073,6 @@
       <c r="O3" t="s">
         <v>100</v>
       </c>
-      <c r="P3">
-        <v>46291</v>
-      </c>
       <c r="Q3" t="s">
         <v>167</v>
       </c>
@@ -1066,9 +1086,9 @@
         <v>175</v>
       </c>
       <c r="U3" t="s">
-        <v>177</v>
-      </c>
-      <c r="V3" s="1">
+        <v>28</v>
+      </c>
+      <c r="V3" s="2">
         <v>46382</v>
       </c>
     </row>
@@ -1100,9 +1120,6 @@
       <c r="O4" t="s">
         <v>101</v>
       </c>
-      <c r="P4">
-        <v>46321</v>
-      </c>
       <c r="Q4" t="s">
         <v>167</v>
       </c>
@@ -1116,9 +1133,9 @@
         <v>175</v>
       </c>
       <c r="U4" t="s">
-        <v>177</v>
-      </c>
-      <c r="V4" s="1">
+        <v>28</v>
+      </c>
+      <c r="V4" s="2">
         <v>46169</v>
       </c>
     </row>
@@ -1150,9 +1167,6 @@
       <c r="O5" t="s">
         <v>102</v>
       </c>
-      <c r="P5">
-        <v>46321</v>
-      </c>
       <c r="Q5" t="s">
         <v>167</v>
       </c>
@@ -1166,9 +1180,9 @@
         <v>175</v>
       </c>
       <c r="U5" t="s">
-        <v>177</v>
-      </c>
-      <c r="V5" s="1">
+        <v>28</v>
+      </c>
+      <c r="V5" s="2">
         <v>46169</v>
       </c>
     </row>
@@ -1203,9 +1217,6 @@
       <c r="O6" t="s">
         <v>103</v>
       </c>
-      <c r="P6">
-        <v>46291</v>
-      </c>
       <c r="Q6" t="s">
         <v>167</v>
       </c>
@@ -1219,9 +1230,9 @@
         <v>175</v>
       </c>
       <c r="U6" t="s">
-        <v>177</v>
-      </c>
-      <c r="V6" s="1">
+        <v>28</v>
+      </c>
+      <c r="V6" s="2">
         <v>46352</v>
       </c>
     </row>
@@ -1247,7 +1258,7 @@
       <c r="G7" t="s">
         <v>44</v>
       </c>
-      <c r="H7" s="1">
+      <c r="H7" s="2">
         <v>46121</v>
       </c>
       <c r="I7" t="s">
@@ -1260,7 +1271,7 @@
         <v>104</v>
       </c>
       <c r="P7">
-        <v>46138</v>
+        <v>3799999.6</v>
       </c>
       <c r="Q7" t="s">
         <v>168</v>
@@ -1272,12 +1283,12 @@
         <v>172</v>
       </c>
       <c r="T7" t="s">
-        <v>175</v>
+        <v>176</v>
       </c>
       <c r="U7" t="s">
-        <v>178</v>
-      </c>
-      <c r="V7" s="1">
+        <v>28</v>
+      </c>
+      <c r="V7" s="2">
         <v>46138</v>
       </c>
     </row>
@@ -1309,9 +1320,6 @@
       <c r="O8" t="s">
         <v>105</v>
       </c>
-      <c r="P8">
-        <v>46291</v>
-      </c>
       <c r="Q8" t="s">
         <v>167</v>
       </c>
@@ -1325,9 +1333,9 @@
         <v>175</v>
       </c>
       <c r="U8" t="s">
-        <v>177</v>
-      </c>
-      <c r="V8" s="1">
+        <v>28</v>
+      </c>
+      <c r="V8" s="2">
         <v>46200</v>
       </c>
     </row>
@@ -1357,7 +1365,7 @@
         <v>106</v>
       </c>
       <c r="P9">
-        <v>46291</v>
+        <v>60000</v>
       </c>
       <c r="Q9" t="s">
         <v>167</v>
@@ -1372,9 +1380,9 @@
         <v>175</v>
       </c>
       <c r="U9" t="s">
-        <v>177</v>
-      </c>
-      <c r="V9" s="1">
+        <v>28</v>
+      </c>
+      <c r="V9" s="2">
         <v>46200</v>
       </c>
     </row>
@@ -1406,9 +1414,6 @@
       <c r="O10" t="s">
         <v>107</v>
       </c>
-      <c r="P10">
-        <v>46291</v>
-      </c>
       <c r="Q10" t="s">
         <v>167</v>
       </c>
@@ -1422,9 +1427,9 @@
         <v>175</v>
       </c>
       <c r="U10" t="s">
-        <v>177</v>
-      </c>
-      <c r="V10" s="1">
+        <v>28</v>
+      </c>
+      <c r="V10" s="2">
         <v>46352</v>
       </c>
     </row>
@@ -1456,9 +1461,6 @@
       <c r="O11" t="s">
         <v>108</v>
       </c>
-      <c r="P11">
-        <v>46291</v>
-      </c>
       <c r="Q11" t="s">
         <v>167</v>
       </c>
@@ -1472,9 +1474,9 @@
         <v>175</v>
       </c>
       <c r="U11" t="s">
-        <v>177</v>
-      </c>
-      <c r="V11" s="1">
+        <v>28</v>
+      </c>
+      <c r="V11" s="2">
         <v>46352</v>
       </c>
     </row>
@@ -1500,7 +1502,7 @@
       <c r="G12" t="s">
         <v>44</v>
       </c>
-      <c r="H12" s="1">
+      <c r="H12" s="2">
         <v>46079</v>
       </c>
       <c r="I12" t="s">
@@ -1516,7 +1518,7 @@
         <v>109</v>
       </c>
       <c r="P12">
-        <v>46079</v>
+        <v>1187433.02</v>
       </c>
       <c r="Q12" t="s">
         <v>167</v>
@@ -1531,9 +1533,9 @@
         <v>175</v>
       </c>
       <c r="U12" t="s">
-        <v>177</v>
-      </c>
-      <c r="V12" s="1">
+        <v>180</v>
+      </c>
+      <c r="V12" s="2">
         <v>46168</v>
       </c>
     </row>
@@ -1569,7 +1571,7 @@
         <v>110</v>
       </c>
       <c r="P13">
-        <v>46352</v>
+        <v>1000000</v>
       </c>
       <c r="Q13" t="s">
         <v>167</v>
@@ -1584,9 +1586,9 @@
         <v>175</v>
       </c>
       <c r="U13" t="s">
-        <v>177</v>
-      </c>
-      <c r="V13" s="1">
+        <v>180</v>
+      </c>
+      <c r="V13" s="2">
         <v>46049</v>
       </c>
     </row>
@@ -1622,7 +1624,7 @@
         <v>111</v>
       </c>
       <c r="P14">
-        <v>46352</v>
+        <v>1000000</v>
       </c>
       <c r="Q14" t="s">
         <v>167</v>
@@ -1637,9 +1639,9 @@
         <v>175</v>
       </c>
       <c r="U14" t="s">
-        <v>177</v>
-      </c>
-      <c r="V14" s="1">
+        <v>180</v>
+      </c>
+      <c r="V14" s="2">
         <v>46049</v>
       </c>
     </row>
@@ -1675,7 +1677,7 @@
         <v>112</v>
       </c>
       <c r="P15">
-        <v>46352</v>
+        <v>1000000</v>
       </c>
       <c r="Q15" t="s">
         <v>167</v>
@@ -1690,9 +1692,9 @@
         <v>175</v>
       </c>
       <c r="U15" t="s">
-        <v>177</v>
-      </c>
-      <c r="V15" s="1">
+        <v>180</v>
+      </c>
+      <c r="V15" s="2">
         <v>46049</v>
       </c>
     </row>
@@ -1728,7 +1730,7 @@
         <v>113</v>
       </c>
       <c r="P16">
-        <v>46229</v>
+        <v>100000</v>
       </c>
       <c r="Q16" t="s">
         <v>169</v>
@@ -1743,9 +1745,9 @@
         <v>175</v>
       </c>
       <c r="U16" t="s">
-        <v>177</v>
-      </c>
-      <c r="V16" s="1">
+        <v>180</v>
+      </c>
+      <c r="V16" s="2">
         <v>46291</v>
       </c>
     </row>
@@ -1771,7 +1773,7 @@
       <c r="G17" t="s">
         <v>44</v>
       </c>
-      <c r="H17" s="1">
+      <c r="H17" s="2">
         <v>46098</v>
       </c>
       <c r="I17" t="s">
@@ -1787,7 +1789,7 @@
         <v>114</v>
       </c>
       <c r="P17">
-        <v>46107</v>
+        <v>1770880.5</v>
       </c>
       <c r="Q17" t="s">
         <v>168</v>
@@ -1799,12 +1801,12 @@
         <v>172</v>
       </c>
       <c r="T17" t="s">
-        <v>175</v>
+        <v>177</v>
       </c>
       <c r="U17" t="s">
-        <v>179</v>
-      </c>
-      <c r="V17" s="1">
+        <v>180</v>
+      </c>
+      <c r="V17" s="2">
         <v>46168</v>
       </c>
     </row>
@@ -1830,7 +1832,7 @@
       <c r="G18" t="s">
         <v>44</v>
       </c>
-      <c r="H18" s="1">
+      <c r="H18" s="2">
         <v>46076</v>
       </c>
       <c r="I18" t="s">
@@ -1843,7 +1845,7 @@
         <v>115</v>
       </c>
       <c r="P18">
-        <v>46079</v>
+        <v>350000</v>
       </c>
       <c r="Q18" t="s">
         <v>168</v>
@@ -1855,12 +1857,12 @@
         <v>172</v>
       </c>
       <c r="T18" t="s">
-        <v>175</v>
+        <v>176</v>
       </c>
       <c r="U18" t="s">
-        <v>178</v>
-      </c>
-      <c r="V18" s="1">
+        <v>28</v>
+      </c>
+      <c r="V18" s="2">
         <v>46260</v>
       </c>
     </row>
@@ -1886,7 +1888,7 @@
       <c r="G19" t="s">
         <v>44</v>
       </c>
-      <c r="H19" s="1">
+      <c r="H19" s="2">
         <v>46076</v>
       </c>
       <c r="I19" t="s">
@@ -1899,7 +1901,7 @@
         <v>116</v>
       </c>
       <c r="P19">
-        <v>46079</v>
+        <v>350000</v>
       </c>
       <c r="Q19" t="s">
         <v>168</v>
@@ -1911,12 +1913,12 @@
         <v>172</v>
       </c>
       <c r="T19" t="s">
-        <v>175</v>
+        <v>176</v>
       </c>
       <c r="U19" t="s">
-        <v>178</v>
-      </c>
-      <c r="V19" s="1">
+        <v>28</v>
+      </c>
+      <c r="V19" s="2">
         <v>46260</v>
       </c>
     </row>
@@ -1946,7 +1948,7 @@
         <v>117</v>
       </c>
       <c r="P20">
-        <v>46321</v>
+        <v>1000000</v>
       </c>
       <c r="Q20" t="s">
         <v>168</v>
@@ -1958,12 +1960,12 @@
         <v>172</v>
       </c>
       <c r="T20" t="s">
-        <v>175</v>
+        <v>176</v>
       </c>
       <c r="U20" t="s">
-        <v>178</v>
-      </c>
-      <c r="V20" s="1">
+        <v>28</v>
+      </c>
+      <c r="V20" s="2">
         <v>46382</v>
       </c>
     </row>
@@ -1995,9 +1997,6 @@
       <c r="O21" t="s">
         <v>118</v>
       </c>
-      <c r="P21">
-        <v>46321</v>
-      </c>
       <c r="Q21" t="s">
         <v>167</v>
       </c>
@@ -2011,9 +2010,9 @@
         <v>175</v>
       </c>
       <c r="U21" t="s">
-        <v>177</v>
-      </c>
-      <c r="V21" s="1">
+        <v>28</v>
+      </c>
+      <c r="V21" s="2">
         <v>46382</v>
       </c>
     </row>
@@ -2045,9 +2044,6 @@
       <c r="O22" t="s">
         <v>119</v>
       </c>
-      <c r="P22">
-        <v>46321</v>
-      </c>
       <c r="Q22" t="s">
         <v>167</v>
       </c>
@@ -2061,9 +2057,9 @@
         <v>175</v>
       </c>
       <c r="U22" t="s">
-        <v>177</v>
-      </c>
-      <c r="V22" s="1">
+        <v>28</v>
+      </c>
+      <c r="V22" s="2">
         <v>46230</v>
       </c>
     </row>
@@ -2095,9 +2091,6 @@
       <c r="O23" t="s">
         <v>120</v>
       </c>
-      <c r="P23">
-        <v>46321</v>
-      </c>
       <c r="Q23" t="s">
         <v>167</v>
       </c>
@@ -2111,9 +2104,9 @@
         <v>175</v>
       </c>
       <c r="U23" t="s">
-        <v>177</v>
-      </c>
-      <c r="V23" s="1">
+        <v>28</v>
+      </c>
+      <c r="V23" s="2">
         <v>46230</v>
       </c>
     </row>
@@ -2139,7 +2132,7 @@
       <c r="G24" t="s">
         <v>44</v>
       </c>
-      <c r="H24" s="1">
+      <c r="H24" s="2">
         <v>46119</v>
       </c>
       <c r="I24" t="s">
@@ -2155,7 +2148,7 @@
         <v>121</v>
       </c>
       <c r="P24">
-        <v>46138</v>
+        <v>1704503</v>
       </c>
       <c r="Q24" t="s">
         <v>168</v>
@@ -2167,12 +2160,12 @@
         <v>172</v>
       </c>
       <c r="T24" t="s">
-        <v>175</v>
+        <v>177</v>
       </c>
       <c r="U24" t="s">
-        <v>179</v>
-      </c>
-      <c r="V24" s="1">
+        <v>180</v>
+      </c>
+      <c r="V24" s="2">
         <v>46199</v>
       </c>
     </row>
@@ -2198,7 +2191,7 @@
       <c r="G25" t="s">
         <v>44</v>
       </c>
-      <c r="H25" s="1">
+      <c r="H25" s="2">
         <v>46121</v>
       </c>
       <c r="I25" t="s">
@@ -2211,7 +2204,7 @@
         <v>122</v>
       </c>
       <c r="P25">
-        <v>46138</v>
+        <v>3799000</v>
       </c>
       <c r="Q25" t="s">
         <v>168</v>
@@ -2223,12 +2216,12 @@
         <v>172</v>
       </c>
       <c r="T25" t="s">
-        <v>175</v>
+        <v>176</v>
       </c>
       <c r="U25" t="s">
-        <v>178</v>
-      </c>
-      <c r="V25" s="1">
+        <v>28</v>
+      </c>
+      <c r="V25" s="2">
         <v>46199</v>
       </c>
     </row>
@@ -2254,7 +2247,7 @@
       <c r="G26" t="s">
         <v>44</v>
       </c>
-      <c r="H26" s="1">
+      <c r="H26" s="2">
         <v>46076</v>
       </c>
       <c r="I26" t="s">
@@ -2267,7 +2260,7 @@
         <v>122</v>
       </c>
       <c r="P26">
-        <v>46079</v>
+        <v>1000</v>
       </c>
       <c r="Q26" t="s">
         <v>168</v>
@@ -2279,12 +2272,12 @@
         <v>172</v>
       </c>
       <c r="T26" t="s">
-        <v>175</v>
+        <v>176</v>
       </c>
       <c r="U26" t="s">
-        <v>178</v>
-      </c>
-      <c r="V26" s="1">
+        <v>28</v>
+      </c>
+      <c r="V26" s="2">
         <v>46352</v>
       </c>
     </row>
@@ -2320,7 +2313,7 @@
         <v>123</v>
       </c>
       <c r="P27">
-        <v>46291</v>
+        <v>100000</v>
       </c>
       <c r="Q27" t="s">
         <v>169</v>
@@ -2335,9 +2328,9 @@
         <v>175</v>
       </c>
       <c r="U27" t="s">
-        <v>177</v>
-      </c>
-      <c r="V27" s="1">
+        <v>180</v>
+      </c>
+      <c r="V27" s="2">
         <v>46352</v>
       </c>
     </row>
@@ -2363,7 +2356,7 @@
       <c r="G28" t="s">
         <v>44</v>
       </c>
-      <c r="H28" s="1">
+      <c r="H28" s="2">
         <v>46199</v>
       </c>
       <c r="I28" t="s">
@@ -2379,7 +2372,7 @@
         <v>124</v>
       </c>
       <c r="P28">
-        <v>46199</v>
+        <v>150000</v>
       </c>
       <c r="Q28" t="s">
         <v>168</v>
@@ -2391,12 +2384,12 @@
         <v>172</v>
       </c>
       <c r="T28" t="s">
-        <v>175</v>
+        <v>176</v>
       </c>
       <c r="U28" t="s">
-        <v>178</v>
-      </c>
-      <c r="V28" s="1">
+        <v>180</v>
+      </c>
+      <c r="V28" s="2">
         <v>46260</v>
       </c>
     </row>
@@ -2422,7 +2415,7 @@
       <c r="G29" t="s">
         <v>44</v>
       </c>
-      <c r="H29" s="1">
+      <c r="H29" s="2">
         <v>46199</v>
       </c>
       <c r="I29" t="s">
@@ -2438,7 +2431,7 @@
         <v>125</v>
       </c>
       <c r="P29">
-        <v>46199</v>
+        <v>150000</v>
       </c>
       <c r="Q29" t="s">
         <v>168</v>
@@ -2450,12 +2443,12 @@
         <v>172</v>
       </c>
       <c r="T29" t="s">
-        <v>175</v>
+        <v>176</v>
       </c>
       <c r="U29" t="s">
-        <v>178</v>
-      </c>
-      <c r="V29" s="1">
+        <v>180</v>
+      </c>
+      <c r="V29" s="2">
         <v>46260</v>
       </c>
     </row>
@@ -2481,7 +2474,7 @@
       <c r="G30" t="s">
         <v>44</v>
       </c>
-      <c r="H30" s="1">
+      <c r="H30" s="2">
         <v>46199</v>
       </c>
       <c r="I30" t="s">
@@ -2497,7 +2490,7 @@
         <v>126</v>
       </c>
       <c r="P30">
-        <v>46199</v>
+        <v>18462.36</v>
       </c>
       <c r="Q30" t="s">
         <v>168</v>
@@ -2509,12 +2502,12 @@
         <v>172</v>
       </c>
       <c r="T30" t="s">
-        <v>175</v>
+        <v>176</v>
       </c>
       <c r="U30" t="s">
-        <v>178</v>
-      </c>
-      <c r="V30" s="1">
+        <v>180</v>
+      </c>
+      <c r="V30" s="2">
         <v>46260</v>
       </c>
     </row>
@@ -2540,7 +2533,7 @@
       <c r="G31" t="s">
         <v>44</v>
       </c>
-      <c r="H31" s="1">
+      <c r="H31" s="2">
         <v>46199</v>
       </c>
       <c r="I31" t="s">
@@ -2556,7 +2549,7 @@
         <v>126</v>
       </c>
       <c r="P31">
-        <v>46199</v>
+        <v>324166.14</v>
       </c>
       <c r="Q31" t="s">
         <v>168</v>
@@ -2568,12 +2561,12 @@
         <v>172</v>
       </c>
       <c r="T31" t="s">
-        <v>175</v>
+        <v>176</v>
       </c>
       <c r="U31" t="s">
-        <v>178</v>
-      </c>
-      <c r="V31" s="1">
+        <v>180</v>
+      </c>
+      <c r="V31" s="2">
         <v>46260</v>
       </c>
     </row>
@@ -2606,7 +2599,7 @@
         <v>127</v>
       </c>
       <c r="P32">
-        <v>46291</v>
+        <v>30000</v>
       </c>
       <c r="Q32" t="s">
         <v>168</v>
@@ -2618,12 +2611,12 @@
         <v>172</v>
       </c>
       <c r="T32" t="s">
-        <v>175</v>
+        <v>176</v>
       </c>
       <c r="U32" t="s">
-        <v>178</v>
-      </c>
-      <c r="V32" s="1">
+        <v>180</v>
+      </c>
+      <c r="V32" s="2">
         <v>46352</v>
       </c>
     </row>
@@ -2649,7 +2642,7 @@
       <c r="G33" t="s">
         <v>44</v>
       </c>
-      <c r="H33" s="1">
+      <c r="H33" s="2">
         <v>46191</v>
       </c>
       <c r="I33" t="s">
@@ -2665,7 +2658,7 @@
         <v>128</v>
       </c>
       <c r="P33">
-        <v>46199</v>
+        <v>1496713.48</v>
       </c>
       <c r="Q33" t="s">
         <v>168</v>
@@ -2677,12 +2670,12 @@
         <v>172</v>
       </c>
       <c r="T33" t="s">
-        <v>175</v>
+        <v>177</v>
       </c>
       <c r="U33" t="s">
-        <v>179</v>
-      </c>
-      <c r="V33" s="1">
+        <v>180</v>
+      </c>
+      <c r="V33" s="2">
         <v>46260</v>
       </c>
     </row>
@@ -2708,7 +2701,7 @@
       <c r="G34" t="s">
         <v>44</v>
       </c>
-      <c r="H34" s="1">
+      <c r="H34" s="2">
         <v>46119</v>
       </c>
       <c r="I34" t="s">
@@ -2721,7 +2714,7 @@
         <v>128</v>
       </c>
       <c r="P34">
-        <v>46138</v>
+        <v>207789.52</v>
       </c>
       <c r="Q34" t="s">
         <v>168</v>
@@ -2733,12 +2726,12 @@
         <v>172</v>
       </c>
       <c r="T34" t="s">
-        <v>175</v>
+        <v>177</v>
       </c>
       <c r="U34" t="s">
-        <v>179</v>
-      </c>
-      <c r="V34" s="1">
+        <v>180</v>
+      </c>
+      <c r="V34" s="2">
         <v>46260</v>
       </c>
     </row>
@@ -2764,7 +2757,7 @@
       <c r="G35" t="s">
         <v>44</v>
       </c>
-      <c r="H35" s="1">
+      <c r="H35" s="2">
         <v>46213</v>
       </c>
       <c r="I35" t="s">
@@ -2777,7 +2770,7 @@
         <v>129</v>
       </c>
       <c r="P35">
-        <v>46229</v>
+        <v>962290.8</v>
       </c>
       <c r="Q35" t="s">
         <v>168</v>
@@ -2789,12 +2782,12 @@
         <v>172</v>
       </c>
       <c r="T35" t="s">
-        <v>175</v>
+        <v>176</v>
       </c>
       <c r="U35" t="s">
-        <v>178</v>
-      </c>
-      <c r="V35" s="1">
+        <v>28</v>
+      </c>
+      <c r="V35" s="2">
         <v>46352</v>
       </c>
     </row>
@@ -2820,7 +2813,7 @@
       <c r="G36" t="s">
         <v>44</v>
       </c>
-      <c r="H36" s="1">
+      <c r="H36" s="2">
         <v>46175</v>
       </c>
       <c r="I36" t="s">
@@ -2833,7 +2826,7 @@
         <v>129</v>
       </c>
       <c r="P36">
-        <v>46199</v>
+        <v>798776.97</v>
       </c>
       <c r="Q36" t="s">
         <v>168</v>
@@ -2845,12 +2838,12 @@
         <v>172</v>
       </c>
       <c r="T36" t="s">
-        <v>175</v>
+        <v>176</v>
       </c>
       <c r="U36" t="s">
-        <v>178</v>
-      </c>
-      <c r="V36" s="1">
+        <v>28</v>
+      </c>
+      <c r="V36" s="2">
         <v>46260</v>
       </c>
     </row>
@@ -2876,7 +2869,7 @@
       <c r="G37" t="s">
         <v>44</v>
       </c>
-      <c r="H37" s="1">
+      <c r="H37" s="2">
         <v>46213</v>
       </c>
       <c r="I37" t="s">
@@ -2889,7 +2882,7 @@
         <v>129</v>
       </c>
       <c r="P37">
-        <v>46229</v>
+        <v>1530656.62</v>
       </c>
       <c r="Q37" t="s">
         <v>168</v>
@@ -2901,12 +2894,12 @@
         <v>172</v>
       </c>
       <c r="T37" t="s">
-        <v>175</v>
+        <v>176</v>
       </c>
       <c r="U37" t="s">
-        <v>178</v>
-      </c>
-      <c r="V37" s="1">
+        <v>28</v>
+      </c>
+      <c r="V37" s="2">
         <v>46352</v>
       </c>
     </row>
@@ -2932,7 +2925,7 @@
       <c r="G38" t="s">
         <v>44</v>
       </c>
-      <c r="H38" s="1">
+      <c r="H38" s="2">
         <v>46199</v>
       </c>
       <c r="I38" t="s">
@@ -2945,7 +2938,7 @@
         <v>129</v>
       </c>
       <c r="P38">
-        <v>46199</v>
+        <v>72958.08</v>
       </c>
       <c r="Q38" t="s">
         <v>168</v>
@@ -2957,12 +2950,12 @@
         <v>172</v>
       </c>
       <c r="T38" t="s">
-        <v>175</v>
+        <v>176</v>
       </c>
       <c r="U38" t="s">
-        <v>178</v>
-      </c>
-      <c r="V38" s="1">
+        <v>28</v>
+      </c>
+      <c r="V38" s="2">
         <v>46229</v>
       </c>
     </row>
@@ -2988,7 +2981,7 @@
       <c r="G39" t="s">
         <v>44</v>
       </c>
-      <c r="H39" s="1">
+      <c r="H39" s="2">
         <v>46199</v>
       </c>
       <c r="I39" t="s">
@@ -3001,7 +2994,7 @@
         <v>129</v>
       </c>
       <c r="P39">
-        <v>46199</v>
+        <v>8916</v>
       </c>
       <c r="Q39" t="s">
         <v>168</v>
@@ -3013,12 +3006,12 @@
         <v>172</v>
       </c>
       <c r="T39" t="s">
-        <v>175</v>
+        <v>176</v>
       </c>
       <c r="U39" t="s">
-        <v>178</v>
-      </c>
-      <c r="V39" s="1">
+        <v>28</v>
+      </c>
+      <c r="V39" s="2">
         <v>46229</v>
       </c>
     </row>
@@ -3044,7 +3037,7 @@
       <c r="G40" t="s">
         <v>44</v>
       </c>
-      <c r="H40" s="1">
+      <c r="H40" s="2">
         <v>46204</v>
       </c>
       <c r="I40" t="s">
@@ -3057,7 +3050,7 @@
         <v>129</v>
       </c>
       <c r="P40">
-        <v>46229</v>
+        <v>425178.5</v>
       </c>
       <c r="Q40" t="s">
         <v>168</v>
@@ -3069,12 +3062,12 @@
         <v>172</v>
       </c>
       <c r="T40" t="s">
-        <v>175</v>
+        <v>176</v>
       </c>
       <c r="U40" t="s">
-        <v>178</v>
-      </c>
-      <c r="V40" s="1">
+        <v>28</v>
+      </c>
+      <c r="V40" s="2">
         <v>46229</v>
       </c>
     </row>
@@ -3100,7 +3093,7 @@
       <c r="G41" t="s">
         <v>44</v>
       </c>
-      <c r="H41" s="1">
+      <c r="H41" s="2">
         <v>46244</v>
       </c>
       <c r="I41" t="s">
@@ -3113,7 +3106,7 @@
         <v>129</v>
       </c>
       <c r="P41">
-        <v>46199</v>
+        <v>1223.03</v>
       </c>
       <c r="Q41" t="s">
         <v>168</v>
@@ -3125,12 +3118,12 @@
         <v>172</v>
       </c>
       <c r="T41" t="s">
-        <v>175</v>
+        <v>176</v>
       </c>
       <c r="U41" t="s">
-        <v>178</v>
-      </c>
-      <c r="V41" s="1">
+        <v>28</v>
+      </c>
+      <c r="V41" s="2">
         <v>46260</v>
       </c>
     </row>
@@ -3159,9 +3152,6 @@
       <c r="O42" t="s">
         <v>130</v>
       </c>
-      <c r="P42">
-        <v>46260</v>
-      </c>
       <c r="Q42" t="s">
         <v>168</v>
       </c>
@@ -3172,12 +3162,12 @@
         <v>173</v>
       </c>
       <c r="T42" t="s">
-        <v>175</v>
+        <v>176</v>
       </c>
       <c r="U42" t="s">
-        <v>178</v>
-      </c>
-      <c r="V42" s="1">
+        <v>28</v>
+      </c>
+      <c r="V42" s="2">
         <v>46352</v>
       </c>
     </row>
@@ -3203,7 +3193,7 @@
       <c r="G43" t="s">
         <v>44</v>
       </c>
-      <c r="H43" s="1">
+      <c r="H43" s="2">
         <v>46191</v>
       </c>
       <c r="I43" t="s">
@@ -3216,7 +3206,7 @@
         <v>131</v>
       </c>
       <c r="P43">
-        <v>46199</v>
+        <v>400000</v>
       </c>
       <c r="Q43" t="s">
         <v>168</v>
@@ -3228,12 +3218,12 @@
         <v>172</v>
       </c>
       <c r="T43" t="s">
-        <v>175</v>
+        <v>176</v>
       </c>
       <c r="U43" t="s">
-        <v>178</v>
-      </c>
-      <c r="V43" s="1">
+        <v>28</v>
+      </c>
+      <c r="V43" s="2">
         <v>46229</v>
       </c>
     </row>
@@ -3259,7 +3249,7 @@
       <c r="G44" t="s">
         <v>44</v>
       </c>
-      <c r="H44" s="1">
+      <c r="H44" s="2">
         <v>46191</v>
       </c>
       <c r="I44" t="s">
@@ -3272,7 +3262,7 @@
         <v>132</v>
       </c>
       <c r="P44">
-        <v>46199</v>
+        <v>400000</v>
       </c>
       <c r="Q44" t="s">
         <v>168</v>
@@ -3284,12 +3274,12 @@
         <v>172</v>
       </c>
       <c r="T44" t="s">
-        <v>175</v>
+        <v>176</v>
       </c>
       <c r="U44" t="s">
-        <v>178</v>
-      </c>
-      <c r="V44" s="1">
+        <v>28</v>
+      </c>
+      <c r="V44" s="2">
         <v>46229</v>
       </c>
     </row>
@@ -3315,7 +3305,7 @@
       <c r="G45" t="s">
         <v>44</v>
       </c>
-      <c r="H45" s="1">
+      <c r="H45" s="2">
         <v>46213</v>
       </c>
       <c r="I45" t="s">
@@ -3331,7 +3321,7 @@
         <v>133</v>
       </c>
       <c r="P45">
-        <v>46229</v>
+        <v>173846.38</v>
       </c>
       <c r="Q45" t="s">
         <v>168</v>
@@ -3343,12 +3333,12 @@
         <v>172</v>
       </c>
       <c r="T45" t="s">
-        <v>175</v>
+        <v>177</v>
       </c>
       <c r="U45" t="s">
-        <v>179</v>
-      </c>
-      <c r="V45" s="1">
+        <v>180</v>
+      </c>
+      <c r="V45" s="2">
         <v>46291</v>
       </c>
     </row>
@@ -3374,7 +3364,7 @@
       <c r="G46" t="s">
         <v>44</v>
       </c>
-      <c r="H46" s="1">
+      <c r="H46" s="2">
         <v>46210</v>
       </c>
       <c r="I46" t="s">
@@ -3387,7 +3377,7 @@
         <v>133</v>
       </c>
       <c r="P46">
-        <v>46229</v>
+        <v>1530656.62</v>
       </c>
       <c r="Q46" t="s">
         <v>168</v>
@@ -3399,12 +3389,12 @@
         <v>172</v>
       </c>
       <c r="T46" t="s">
-        <v>175</v>
+        <v>177</v>
       </c>
       <c r="U46" t="s">
-        <v>179</v>
-      </c>
-      <c r="V46" s="1">
+        <v>180</v>
+      </c>
+      <c r="V46" s="2">
         <v>46291</v>
       </c>
     </row>
@@ -3434,7 +3424,7 @@
         <v>134</v>
       </c>
       <c r="P47">
-        <v>46321</v>
+        <v>1000000</v>
       </c>
       <c r="Q47" t="s">
         <v>168</v>
@@ -3446,12 +3436,12 @@
         <v>172</v>
       </c>
       <c r="T47" t="s">
-        <v>175</v>
+        <v>176</v>
       </c>
       <c r="U47" t="s">
-        <v>178</v>
-      </c>
-      <c r="V47" s="1">
+        <v>28</v>
+      </c>
+      <c r="V47" s="2">
         <v>46321</v>
       </c>
     </row>
@@ -3487,7 +3477,7 @@
         <v>135</v>
       </c>
       <c r="P48">
-        <v>46291</v>
+        <v>958040</v>
       </c>
       <c r="Q48" t="s">
         <v>167</v>
@@ -3502,9 +3492,9 @@
         <v>175</v>
       </c>
       <c r="U48" t="s">
-        <v>177</v>
-      </c>
-      <c r="V48" s="1">
+        <v>180</v>
+      </c>
+      <c r="V48" s="2">
         <v>46352</v>
       </c>
     </row>
@@ -3530,7 +3520,7 @@
       <c r="G49" t="s">
         <v>44</v>
       </c>
-      <c r="H49" s="1">
+      <c r="H49" s="2">
         <v>46176</v>
       </c>
       <c r="I49" t="s">
@@ -3546,7 +3536,7 @@
         <v>135</v>
       </c>
       <c r="P49">
-        <v>46199</v>
+        <v>41730.64</v>
       </c>
       <c r="Q49" t="s">
         <v>167</v>
@@ -3558,12 +3548,12 @@
         <v>172</v>
       </c>
       <c r="T49" t="s">
-        <v>176</v>
+        <v>175</v>
       </c>
       <c r="U49" t="s">
-        <v>177</v>
-      </c>
-      <c r="V49" s="1">
+        <v>180</v>
+      </c>
+      <c r="V49" s="2">
         <v>46352</v>
       </c>
     </row>
@@ -3599,7 +3589,7 @@
         <v>136</v>
       </c>
       <c r="P50">
-        <v>46260</v>
+        <v>608623.25</v>
       </c>
       <c r="Q50" t="s">
         <v>168</v>
@@ -3611,12 +3601,12 @@
         <v>172</v>
       </c>
       <c r="T50" t="s">
-        <v>175</v>
+        <v>177</v>
       </c>
       <c r="U50" t="s">
-        <v>179</v>
-      </c>
-      <c r="V50" s="1">
+        <v>180</v>
+      </c>
+      <c r="V50" s="2">
         <v>46321</v>
       </c>
     </row>
@@ -3652,7 +3642,7 @@
         <v>137</v>
       </c>
       <c r="P51">
-        <v>46291</v>
+        <v>559040.0699999999</v>
       </c>
       <c r="Q51" t="s">
         <v>168</v>
@@ -3664,12 +3654,12 @@
         <v>172</v>
       </c>
       <c r="T51" t="s">
-        <v>175</v>
+        <v>177</v>
       </c>
       <c r="U51" t="s">
-        <v>179</v>
-      </c>
-      <c r="V51" s="1">
+        <v>180</v>
+      </c>
+      <c r="V51" s="2">
         <v>46352</v>
       </c>
     </row>
@@ -3702,7 +3692,7 @@
         <v>138</v>
       </c>
       <c r="P52">
-        <v>46321</v>
+        <v>1704503</v>
       </c>
       <c r="Q52" t="s">
         <v>168</v>
@@ -3714,12 +3704,12 @@
         <v>172</v>
       </c>
       <c r="T52" t="s">
-        <v>175</v>
+        <v>177</v>
       </c>
       <c r="U52" t="s">
-        <v>179</v>
-      </c>
-      <c r="V52" s="1">
+        <v>180</v>
+      </c>
+      <c r="V52" s="2">
         <v>46382</v>
       </c>
     </row>
@@ -3745,7 +3735,7 @@
       <c r="G53" t="s">
         <v>44</v>
       </c>
-      <c r="H53" s="1">
+      <c r="H53" s="2">
         <v>46227</v>
       </c>
       <c r="I53" t="s">
@@ -3758,7 +3748,7 @@
         <v>136</v>
       </c>
       <c r="P53">
-        <v>46229</v>
+        <v>236343.68</v>
       </c>
       <c r="Q53" t="s">
         <v>168</v>
@@ -3770,12 +3760,12 @@
         <v>172</v>
       </c>
       <c r="T53" t="s">
-        <v>175</v>
+        <v>177</v>
       </c>
       <c r="U53" t="s">
-        <v>179</v>
-      </c>
-      <c r="V53" s="1">
+        <v>180</v>
+      </c>
+      <c r="V53" s="2">
         <v>46321</v>
       </c>
     </row>
@@ -3798,7 +3788,7 @@
       <c r="G54" t="s">
         <v>44</v>
       </c>
-      <c r="H54" s="1">
+      <c r="H54" s="2">
         <v>46280</v>
       </c>
       <c r="I54" t="s">
@@ -3811,7 +3801,7 @@
         <v>137</v>
       </c>
       <c r="P54">
-        <v>46291</v>
+        <v>1145462.93</v>
       </c>
       <c r="Q54" t="s">
         <v>168</v>
@@ -3823,12 +3813,12 @@
         <v>172</v>
       </c>
       <c r="T54" t="s">
-        <v>175</v>
+        <v>177</v>
       </c>
       <c r="U54" t="s">
-        <v>179</v>
-      </c>
-      <c r="V54" s="1">
+        <v>180</v>
+      </c>
+      <c r="V54" s="2">
         <v>46352</v>
       </c>
     </row>
@@ -3851,7 +3841,7 @@
       <c r="G55" t="s">
         <v>44</v>
       </c>
-      <c r="H55" s="1">
+      <c r="H55" s="2">
         <v>46280</v>
       </c>
       <c r="I55" t="s">
@@ -3864,7 +3854,7 @@
         <v>136</v>
       </c>
       <c r="P55">
-        <v>46260</v>
+        <v>859536.0699999999</v>
       </c>
       <c r="Q55" t="s">
         <v>168</v>
@@ -3876,12 +3866,12 @@
         <v>172</v>
       </c>
       <c r="T55" t="s">
-        <v>175</v>
+        <v>177</v>
       </c>
       <c r="U55" t="s">
-        <v>179</v>
-      </c>
-      <c r="V55" s="1">
+        <v>180</v>
+      </c>
+      <c r="V55" s="2">
         <v>46321</v>
       </c>
     </row>
@@ -3917,7 +3907,7 @@
         <v>139</v>
       </c>
       <c r="P56">
-        <v>46352</v>
+        <v>1295422.28</v>
       </c>
       <c r="Q56" t="s">
         <v>168</v>
@@ -3929,12 +3919,12 @@
         <v>172</v>
       </c>
       <c r="T56" t="s">
-        <v>175</v>
+        <v>177</v>
       </c>
       <c r="U56" t="s">
-        <v>179</v>
-      </c>
-      <c r="V56" s="1">
+        <v>180</v>
+      </c>
+      <c r="V56" s="2">
         <v>46049</v>
       </c>
     </row>
@@ -3970,7 +3960,7 @@
         <v>140</v>
       </c>
       <c r="P57">
-        <v>46321</v>
+        <v>1962977.67</v>
       </c>
       <c r="Q57" t="s">
         <v>168</v>
@@ -3982,12 +3972,12 @@
         <v>174</v>
       </c>
       <c r="T57" t="s">
-        <v>175</v>
+        <v>178</v>
       </c>
       <c r="U57" t="s">
         <v>180</v>
       </c>
-      <c r="V57" s="1">
+      <c r="V57" s="2">
         <v>46049</v>
       </c>
     </row>
@@ -4017,7 +4007,7 @@
         <v>140</v>
       </c>
       <c r="P58">
-        <v>46321</v>
+        <v>2497091</v>
       </c>
       <c r="Q58" t="s">
         <v>168</v>
@@ -4029,12 +4019,12 @@
         <v>174</v>
       </c>
       <c r="T58" t="s">
-        <v>175</v>
+        <v>178</v>
       </c>
       <c r="U58" t="s">
         <v>180</v>
       </c>
-      <c r="V58" s="1">
+      <c r="V58" s="2">
         <v>46049</v>
       </c>
     </row>
@@ -4063,9 +4053,6 @@
       <c r="O59" t="s">
         <v>141</v>
       </c>
-      <c r="P59">
-        <v>46049</v>
-      </c>
       <c r="Q59" t="s">
         <v>168</v>
       </c>
@@ -4076,12 +4063,12 @@
         <v>174</v>
       </c>
       <c r="T59" t="s">
-        <v>175</v>
+        <v>178</v>
       </c>
       <c r="U59" t="s">
         <v>180</v>
       </c>
-      <c r="V59" s="1">
+      <c r="V59" s="2">
         <v>46139</v>
       </c>
     </row>
@@ -4120,7 +4107,7 @@
         <v>174</v>
       </c>
       <c r="T60" t="s">
-        <v>175</v>
+        <v>178</v>
       </c>
       <c r="U60" t="s">
         <v>180</v>
@@ -4161,7 +4148,7 @@
         <v>174</v>
       </c>
       <c r="T61" t="s">
-        <v>175</v>
+        <v>178</v>
       </c>
       <c r="U61" t="s">
         <v>180</v>
@@ -4190,7 +4177,7 @@
         <v>144</v>
       </c>
       <c r="P62">
-        <v>46107</v>
+        <v>4064.54</v>
       </c>
       <c r="Q62" t="s">
         <v>168</v>
@@ -4202,12 +4189,12 @@
         <v>173</v>
       </c>
       <c r="T62" t="s">
-        <v>176</v>
+        <v>175</v>
       </c>
       <c r="U62" t="s">
-        <v>177</v>
-      </c>
-      <c r="V62" s="1">
+        <v>180</v>
+      </c>
+      <c r="V62" s="2">
         <v>46168</v>
       </c>
     </row>
@@ -4234,7 +4221,7 @@
         <v>145</v>
       </c>
       <c r="P63">
-        <v>46107</v>
+        <v>4227.84</v>
       </c>
       <c r="Q63" t="s">
         <v>167</v>
@@ -4246,12 +4233,12 @@
         <v>173</v>
       </c>
       <c r="T63" t="s">
-        <v>176</v>
+        <v>175</v>
       </c>
       <c r="U63" t="s">
-        <v>177</v>
-      </c>
-      <c r="V63" s="1">
+        <v>180</v>
+      </c>
+      <c r="V63" s="2">
         <v>46168</v>
       </c>
     </row>
@@ -4278,7 +4265,7 @@
         <v>146</v>
       </c>
       <c r="P64">
-        <v>46107</v>
+        <v>9389.959999999999</v>
       </c>
       <c r="Q64" t="s">
         <v>167</v>
@@ -4290,12 +4277,12 @@
         <v>173</v>
       </c>
       <c r="T64" t="s">
-        <v>176</v>
+        <v>175</v>
       </c>
       <c r="U64" t="s">
-        <v>177</v>
-      </c>
-      <c r="V64" s="1">
+        <v>180</v>
+      </c>
+      <c r="V64" s="2">
         <v>46168</v>
       </c>
     </row>
@@ -4322,7 +4309,7 @@
         <v>147</v>
       </c>
       <c r="P65">
-        <v>46107</v>
+        <v>1163.64</v>
       </c>
       <c r="Q65" t="s">
         <v>169</v>
@@ -4334,12 +4321,12 @@
         <v>173</v>
       </c>
       <c r="T65" t="s">
-        <v>176</v>
+        <v>175</v>
       </c>
       <c r="U65" t="s">
-        <v>177</v>
-      </c>
-      <c r="V65" s="1">
+        <v>180</v>
+      </c>
+      <c r="V65" s="2">
         <v>46168</v>
       </c>
     </row>
@@ -4366,7 +4353,7 @@
         <v>148</v>
       </c>
       <c r="P66">
-        <v>46107</v>
+        <v>7204.82</v>
       </c>
       <c r="Q66" t="s">
         <v>167</v>
@@ -4378,12 +4365,12 @@
         <v>173</v>
       </c>
       <c r="T66" t="s">
-        <v>176</v>
+        <v>175</v>
       </c>
       <c r="U66" t="s">
-        <v>177</v>
-      </c>
-      <c r="V66" s="1">
+        <v>180</v>
+      </c>
+      <c r="V66" s="2">
         <v>46168</v>
       </c>
     </row>
@@ -4410,7 +4397,7 @@
         <v>145</v>
       </c>
       <c r="P67">
-        <v>46107</v>
+        <v>3662.66</v>
       </c>
       <c r="Q67" t="s">
         <v>167</v>
@@ -4422,12 +4409,12 @@
         <v>173</v>
       </c>
       <c r="T67" t="s">
-        <v>176</v>
+        <v>175</v>
       </c>
       <c r="U67" t="s">
-        <v>177</v>
-      </c>
-      <c r="V67" s="1">
+        <v>180</v>
+      </c>
+      <c r="V67" s="2">
         <v>46168</v>
       </c>
     </row>
@@ -4454,7 +4441,7 @@
         <v>149</v>
       </c>
       <c r="P68">
-        <v>46168</v>
+        <v>120000</v>
       </c>
       <c r="Q68" t="s">
         <v>167</v>
@@ -4469,9 +4456,9 @@
         <v>175</v>
       </c>
       <c r="U68" t="s">
-        <v>177</v>
-      </c>
-      <c r="V68" s="1">
+        <v>28</v>
+      </c>
+      <c r="V68" s="2">
         <v>46168</v>
       </c>
     </row>
@@ -4503,9 +4490,6 @@
       <c r="O69" t="s">
         <v>150</v>
       </c>
-      <c r="P69">
-        <v>46291</v>
-      </c>
       <c r="Q69" t="s">
         <v>167</v>
       </c>
@@ -4519,9 +4503,9 @@
         <v>175</v>
       </c>
       <c r="U69" t="s">
-        <v>177</v>
-      </c>
-      <c r="V69" s="1">
+        <v>28</v>
+      </c>
+      <c r="V69" s="2">
         <v>46382</v>
       </c>
     </row>
@@ -4557,7 +4541,7 @@
         <v>151</v>
       </c>
       <c r="P70">
-        <v>46229</v>
+        <v>100000</v>
       </c>
       <c r="Q70" t="s">
         <v>169</v>
@@ -4572,9 +4556,9 @@
         <v>175</v>
       </c>
       <c r="U70" t="s">
-        <v>177</v>
-      </c>
-      <c r="V70" s="1">
+        <v>180</v>
+      </c>
+      <c r="V70" s="2">
         <v>46291</v>
       </c>
     </row>
@@ -4601,7 +4585,7 @@
         <v>152</v>
       </c>
       <c r="P71">
-        <v>46260</v>
+        <v>80000</v>
       </c>
       <c r="Q71" t="s">
         <v>167</v>
@@ -4616,9 +4600,9 @@
         <v>175</v>
       </c>
       <c r="U71" t="s">
-        <v>177</v>
-      </c>
-      <c r="V71" s="1">
+        <v>28</v>
+      </c>
+      <c r="V71" s="2">
         <v>46260</v>
       </c>
     </row>
@@ -4645,7 +4629,7 @@
         <v>153</v>
       </c>
       <c r="P72">
-        <v>46291</v>
+        <v>835000</v>
       </c>
       <c r="Q72" t="s">
         <v>167</v>
@@ -4660,9 +4644,9 @@
         <v>175</v>
       </c>
       <c r="U72" t="s">
-        <v>177</v>
-      </c>
-      <c r="V72" s="1">
+        <v>180</v>
+      </c>
+      <c r="V72" s="2">
         <v>46352</v>
       </c>
     </row>
@@ -4689,7 +4673,7 @@
         <v>153</v>
       </c>
       <c r="P73">
-        <v>46168</v>
+        <v>165000</v>
       </c>
       <c r="Q73" t="s">
         <v>167</v>
@@ -4704,9 +4688,9 @@
         <v>175</v>
       </c>
       <c r="U73" t="s">
-        <v>177</v>
-      </c>
-      <c r="V73" s="1">
+        <v>180</v>
+      </c>
+      <c r="V73" s="2">
         <v>46229</v>
       </c>
     </row>
@@ -4733,7 +4717,7 @@
         <v>154</v>
       </c>
       <c r="P74">
-        <v>46291</v>
+        <v>1000000</v>
       </c>
       <c r="Q74" t="s">
         <v>167</v>
@@ -4748,9 +4732,9 @@
         <v>175</v>
       </c>
       <c r="U74" t="s">
-        <v>177</v>
-      </c>
-      <c r="V74" s="1">
+        <v>180</v>
+      </c>
+      <c r="V74" s="2">
         <v>46352</v>
       </c>
     </row>
@@ -4777,7 +4761,7 @@
         <v>155</v>
       </c>
       <c r="P75">
-        <v>46291</v>
+        <v>1000000</v>
       </c>
       <c r="Q75" t="s">
         <v>167</v>
@@ -4792,9 +4776,9 @@
         <v>175</v>
       </c>
       <c r="U75" t="s">
-        <v>177</v>
-      </c>
-      <c r="V75" s="1">
+        <v>180</v>
+      </c>
+      <c r="V75" s="2">
         <v>46352</v>
       </c>
     </row>
@@ -4821,7 +4805,7 @@
         <v>156</v>
       </c>
       <c r="P76">
-        <v>46291</v>
+        <v>100000</v>
       </c>
       <c r="Q76" t="s">
         <v>169</v>
@@ -4836,9 +4820,9 @@
         <v>175</v>
       </c>
       <c r="U76" t="s">
-        <v>177</v>
-      </c>
-      <c r="V76" s="1">
+        <v>180</v>
+      </c>
+      <c r="V76" s="2">
         <v>46352</v>
       </c>
     </row>
@@ -4868,7 +4852,7 @@
         <v>157</v>
       </c>
       <c r="P77">
-        <v>46321</v>
+        <v>1000000</v>
       </c>
       <c r="Q77" t="s">
         <v>168</v>
@@ -4880,12 +4864,12 @@
         <v>172</v>
       </c>
       <c r="T77" t="s">
-        <v>175</v>
+        <v>176</v>
       </c>
       <c r="U77" t="s">
-        <v>178</v>
-      </c>
-      <c r="V77" s="1">
+        <v>28</v>
+      </c>
+      <c r="V77" s="2">
         <v>46382</v>
       </c>
     </row>
@@ -4918,7 +4902,7 @@
         <v>158</v>
       </c>
       <c r="P78">
-        <v>46381</v>
+        <v>1704503</v>
       </c>
       <c r="Q78" t="s">
         <v>168</v>
@@ -4930,12 +4914,12 @@
         <v>42</v>
       </c>
       <c r="T78" t="s">
-        <v>175</v>
+        <v>177</v>
       </c>
       <c r="U78" t="s">
-        <v>179</v>
-      </c>
-      <c r="V78" s="1">
+        <v>180</v>
+      </c>
+      <c r="V78" s="2">
         <v>46107</v>
       </c>
     </row>
@@ -4968,7 +4952,7 @@
         <v>159</v>
       </c>
       <c r="P79">
-        <v>46381</v>
+        <v>1638125.5</v>
       </c>
       <c r="Q79" t="s">
         <v>168</v>
@@ -4980,12 +4964,12 @@
         <v>42</v>
       </c>
       <c r="T79" t="s">
-        <v>175</v>
+        <v>177</v>
       </c>
       <c r="U79" t="s">
-        <v>179</v>
-      </c>
-      <c r="V79" s="1">
+        <v>180</v>
+      </c>
+      <c r="V79" s="2">
         <v>46138</v>
       </c>
     </row>
@@ -5018,7 +5002,7 @@
         <v>160</v>
       </c>
       <c r="P80">
-        <v>46381</v>
+        <v>3800000</v>
       </c>
       <c r="Q80" t="s">
         <v>168</v>
@@ -5030,12 +5014,12 @@
         <v>42</v>
       </c>
       <c r="T80" t="s">
-        <v>175</v>
+        <v>176</v>
       </c>
       <c r="U80" t="s">
-        <v>178</v>
-      </c>
-      <c r="V80" s="1">
+        <v>28</v>
+      </c>
+      <c r="V80" s="2">
         <v>46260</v>
       </c>
     </row>
@@ -5068,7 +5052,7 @@
         <v>161</v>
       </c>
       <c r="P81">
-        <v>46381</v>
+        <v>3800000</v>
       </c>
       <c r="Q81" t="s">
         <v>168</v>
@@ -5080,12 +5064,12 @@
         <v>42</v>
       </c>
       <c r="T81" t="s">
-        <v>175</v>
+        <v>176</v>
       </c>
       <c r="U81" t="s">
-        <v>178</v>
-      </c>
-      <c r="V81" s="1">
+        <v>28</v>
+      </c>
+      <c r="V81" s="2">
         <v>46260</v>
       </c>
     </row>
@@ -5118,7 +5102,7 @@
         <v>162</v>
       </c>
       <c r="P82">
-        <v>46382</v>
+        <v>3800000</v>
       </c>
       <c r="Q82" t="s">
         <v>168</v>
@@ -5130,12 +5114,12 @@
         <v>173</v>
       </c>
       <c r="T82" t="s">
-        <v>175</v>
+        <v>176</v>
       </c>
       <c r="U82" t="s">
-        <v>178</v>
-      </c>
-      <c r="V82" s="1">
+        <v>28</v>
+      </c>
+      <c r="V82" s="2">
         <v>46108</v>
       </c>
     </row>
@@ -5162,7 +5146,7 @@
         <v>97</v>
       </c>
       <c r="P83">
-        <v>46382</v>
+        <v>4394700</v>
       </c>
       <c r="Q83" t="s">
         <v>167</v>
@@ -5174,12 +5158,12 @@
         <v>173</v>
       </c>
       <c r="T83" t="s">
-        <v>175</v>
+        <v>176</v>
       </c>
       <c r="U83" t="s">
-        <v>178</v>
-      </c>
-      <c r="V83" s="1">
+        <v>28</v>
+      </c>
+      <c r="V83" s="2">
         <v>46108</v>
       </c>
     </row>
@@ -5215,7 +5199,7 @@
         <v>163</v>
       </c>
       <c r="P84">
-        <v>46382</v>
+        <v>528395.9300000001</v>
       </c>
       <c r="Q84" t="s">
         <v>168</v>
@@ -5227,12 +5211,12 @@
         <v>172</v>
       </c>
       <c r="T84" t="s">
-        <v>175</v>
+        <v>177</v>
       </c>
       <c r="U84" t="s">
-        <v>179</v>
-      </c>
-      <c r="V84" s="1">
+        <v>180</v>
+      </c>
+      <c r="V84" s="2">
         <v>46080</v>
       </c>
     </row>
@@ -5262,7 +5246,7 @@
         <v>164</v>
       </c>
       <c r="P85">
-        <v>46321</v>
+        <v>1000000</v>
       </c>
       <c r="Q85" t="s">
         <v>168</v>
@@ -5274,12 +5258,12 @@
         <v>172</v>
       </c>
       <c r="T85" t="s">
-        <v>175</v>
+        <v>176</v>
       </c>
       <c r="U85" t="s">
-        <v>178</v>
-      </c>
-      <c r="V85" s="1">
+        <v>28</v>
+      </c>
+      <c r="V85" s="2">
         <v>46382</v>
       </c>
     </row>
@@ -5306,7 +5290,7 @@
         <v>97</v>
       </c>
       <c r="P86">
-        <v>46382</v>
+        <v>4394700</v>
       </c>
       <c r="Q86" t="s">
         <v>167</v>
@@ -5318,12 +5302,12 @@
         <v>173</v>
       </c>
       <c r="T86" t="s">
-        <v>175</v>
+        <v>176</v>
       </c>
       <c r="U86" t="s">
-        <v>178</v>
-      </c>
-      <c r="V86" s="1">
+        <v>28</v>
+      </c>
+      <c r="V86" s="2">
         <v>46108</v>
       </c>
     </row>
@@ -5355,6 +5339,9 @@
       <c r="O87" t="s">
         <v>97</v>
       </c>
+      <c r="P87">
+        <v>3306000</v>
+      </c>
       <c r="Q87" t="s">
         <v>167</v>
       </c>
@@ -5365,10 +5352,10 @@
         <v>42</v>
       </c>
       <c r="T87" t="s">
-        <v>175</v>
+        <v>176</v>
       </c>
       <c r="U87" t="s">
-        <v>178</v>
+        <v>28</v>
       </c>
     </row>
     <row r="88" spans="1:22">
@@ -5399,6 +5386,9 @@
       <c r="O88" t="s">
         <v>97</v>
       </c>
+      <c r="P88">
+        <v>3306000</v>
+      </c>
       <c r="Q88" t="s">
         <v>167</v>
       </c>
@@ -5409,10 +5399,10 @@
         <v>42</v>
       </c>
       <c r="T88" t="s">
-        <v>175</v>
+        <v>176</v>
       </c>
       <c r="U88" t="s">
-        <v>178</v>
+        <v>28</v>
       </c>
     </row>
     <row r="89" spans="1:22">
@@ -5441,7 +5431,7 @@
         <v>165</v>
       </c>
       <c r="P89">
-        <v>46291</v>
+        <v>470820</v>
       </c>
       <c r="Q89" t="s">
         <v>167</v>
@@ -5453,12 +5443,12 @@
         <v>172</v>
       </c>
       <c r="T89" t="s">
-        <v>175</v>
+        <v>179</v>
       </c>
       <c r="U89" t="s">
-        <v>181</v>
-      </c>
-      <c r="V89" s="1">
+        <v>28</v>
+      </c>
+      <c r="V89" s="2">
         <v>46321</v>
       </c>
     </row>
@@ -5485,7 +5475,7 @@
         <v>166</v>
       </c>
       <c r="P90">
-        <v>46291</v>
+        <v>2297180</v>
       </c>
       <c r="Q90" t="s">
         <v>168</v>
@@ -5497,12 +5487,12 @@
         <v>172</v>
       </c>
       <c r="T90" t="s">
-        <v>175</v>
+        <v>176</v>
       </c>
       <c r="U90" t="s">
-        <v>178</v>
-      </c>
-      <c r="V90" s="1">
+        <v>28</v>
+      </c>
+      <c r="V90" s="2">
         <v>46382</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Atualização automática: mta (28/09/2026 15:35)
</commit_message>
<xml_diff>
--- a/Projetos/02_Dados_Tratados/base_mta_tratada.xlsx
+++ b/Projetos/02_Dados_Tratados/base_mta_tratada.xlsx
@@ -566,16 +566,8 @@
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="YYYY-MM-DD HH:MM:SS"/>
   </numFmts>
-  <fonts count="2">
+  <fonts count="1">
     <font>
-      <sz val="11"/>
-      <color theme="1"/>
-      <name val="Calibri"/>
-      <family val="2"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <b/>
       <sz val="11"/>
       <color theme="1"/>
       <name val="Calibri"/>
@@ -591,7 +583,7 @@
       <patternFill patternType="gray125"/>
     </fill>
   </fills>
-  <borders count="2">
+  <borders count="1">
     <border>
       <left/>
       <right/>
@@ -599,30 +591,12 @@
       <bottom/>
       <diagonal/>
     </border>
-    <border>
-      <left style="thin">
-        <color auto="1"/>
-      </left>
-      <right style="thin">
-        <color auto="1"/>
-      </right>
-      <top style="thin">
-        <color auto="1"/>
-      </top>
-      <bottom style="thin">
-        <color auto="1"/>
-      </bottom>
-      <diagonal/>
-    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="3">
+  <cellXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top"/>
-    </xf>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
   </cellXfs>
   <cellStyles count="1">
@@ -922,70 +896,70 @@
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:22">
-      <c r="A1" s="1" t="s">
+      <c r="A1" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="1" t="s">
+      <c r="B1" t="s">
         <v>1</v>
       </c>
-      <c r="C1" s="1" t="s">
+      <c r="C1" t="s">
         <v>2</v>
       </c>
-      <c r="D1" s="1" t="s">
+      <c r="D1" t="s">
         <v>3</v>
       </c>
-      <c r="E1" s="1" t="s">
+      <c r="E1" t="s">
         <v>4</v>
       </c>
-      <c r="F1" s="1" t="s">
+      <c r="F1" t="s">
         <v>5</v>
       </c>
-      <c r="G1" s="1" t="s">
+      <c r="G1" t="s">
         <v>6</v>
       </c>
-      <c r="H1" s="1" t="s">
+      <c r="H1" t="s">
         <v>7</v>
       </c>
-      <c r="I1" s="1" t="s">
+      <c r="I1" t="s">
         <v>8</v>
       </c>
-      <c r="J1" s="1" t="s">
+      <c r="J1" t="s">
         <v>9</v>
       </c>
-      <c r="K1" s="1" t="s">
+      <c r="K1" t="s">
         <v>10</v>
       </c>
-      <c r="L1" s="1" t="s">
+      <c r="L1" t="s">
         <v>11</v>
       </c>
-      <c r="M1" s="1" t="s">
+      <c r="M1" t="s">
         <v>12</v>
       </c>
-      <c r="N1" s="1" t="s">
+      <c r="N1" t="s">
         <v>13</v>
       </c>
-      <c r="O1" s="1" t="s">
+      <c r="O1" t="s">
         <v>14</v>
       </c>
-      <c r="P1" s="1" t="s">
+      <c r="P1" t="s">
         <v>15</v>
       </c>
-      <c r="Q1" s="1" t="s">
+      <c r="Q1" t="s">
         <v>16</v>
       </c>
-      <c r="R1" s="1" t="s">
+      <c r="R1" t="s">
         <v>17</v>
       </c>
-      <c r="S1" s="1" t="s">
+      <c r="S1" t="s">
         <v>18</v>
       </c>
-      <c r="T1" s="1" t="s">
+      <c r="T1" t="s">
         <v>19</v>
       </c>
-      <c r="U1" s="1" t="s">
+      <c r="U1" t="s">
         <v>20</v>
       </c>
-      <c r="V1" s="1" t="s">
+      <c r="V1" t="s">
         <v>21</v>
       </c>
     </row>
@@ -1041,7 +1015,7 @@
       <c r="U2" t="s">
         <v>180</v>
       </c>
-      <c r="V2" s="2">
+      <c r="V2" s="1">
         <v>46291</v>
       </c>
     </row>
@@ -1088,7 +1062,7 @@
       <c r="U3" t="s">
         <v>28</v>
       </c>
-      <c r="V3" s="2">
+      <c r="V3" s="1">
         <v>46382</v>
       </c>
     </row>
@@ -1135,7 +1109,7 @@
       <c r="U4" t="s">
         <v>28</v>
       </c>
-      <c r="V4" s="2">
+      <c r="V4" s="1">
         <v>46169</v>
       </c>
     </row>
@@ -1182,7 +1156,7 @@
       <c r="U5" t="s">
         <v>28</v>
       </c>
-      <c r="V5" s="2">
+      <c r="V5" s="1">
         <v>46169</v>
       </c>
     </row>
@@ -1232,7 +1206,7 @@
       <c r="U6" t="s">
         <v>28</v>
       </c>
-      <c r="V6" s="2">
+      <c r="V6" s="1">
         <v>46352</v>
       </c>
     </row>
@@ -1258,7 +1232,7 @@
       <c r="G7" t="s">
         <v>44</v>
       </c>
-      <c r="H7" s="2">
+      <c r="H7" s="1">
         <v>46121</v>
       </c>
       <c r="I7" t="s">
@@ -1288,7 +1262,7 @@
       <c r="U7" t="s">
         <v>28</v>
       </c>
-      <c r="V7" s="2">
+      <c r="V7" s="1">
         <v>46138</v>
       </c>
     </row>
@@ -1335,7 +1309,7 @@
       <c r="U8" t="s">
         <v>28</v>
       </c>
-      <c r="V8" s="2">
+      <c r="V8" s="1">
         <v>46200</v>
       </c>
     </row>
@@ -1382,7 +1356,7 @@
       <c r="U9" t="s">
         <v>28</v>
       </c>
-      <c r="V9" s="2">
+      <c r="V9" s="1">
         <v>46200</v>
       </c>
     </row>
@@ -1429,7 +1403,7 @@
       <c r="U10" t="s">
         <v>28</v>
       </c>
-      <c r="V10" s="2">
+      <c r="V10" s="1">
         <v>46352</v>
       </c>
     </row>
@@ -1476,7 +1450,7 @@
       <c r="U11" t="s">
         <v>28</v>
       </c>
-      <c r="V11" s="2">
+      <c r="V11" s="1">
         <v>46352</v>
       </c>
     </row>
@@ -1502,7 +1476,7 @@
       <c r="G12" t="s">
         <v>44</v>
       </c>
-      <c r="H12" s="2">
+      <c r="H12" s="1">
         <v>46079</v>
       </c>
       <c r="I12" t="s">
@@ -1535,7 +1509,7 @@
       <c r="U12" t="s">
         <v>180</v>
       </c>
-      <c r="V12" s="2">
+      <c r="V12" s="1">
         <v>46168</v>
       </c>
     </row>
@@ -1588,7 +1562,7 @@
       <c r="U13" t="s">
         <v>180</v>
       </c>
-      <c r="V13" s="2">
+      <c r="V13" s="1">
         <v>46049</v>
       </c>
     </row>
@@ -1641,7 +1615,7 @@
       <c r="U14" t="s">
         <v>180</v>
       </c>
-      <c r="V14" s="2">
+      <c r="V14" s="1">
         <v>46049</v>
       </c>
     </row>
@@ -1694,7 +1668,7 @@
       <c r="U15" t="s">
         <v>180</v>
       </c>
-      <c r="V15" s="2">
+      <c r="V15" s="1">
         <v>46049</v>
       </c>
     </row>
@@ -1747,7 +1721,7 @@
       <c r="U16" t="s">
         <v>180</v>
       </c>
-      <c r="V16" s="2">
+      <c r="V16" s="1">
         <v>46291</v>
       </c>
     </row>
@@ -1773,7 +1747,7 @@
       <c r="G17" t="s">
         <v>44</v>
       </c>
-      <c r="H17" s="2">
+      <c r="H17" s="1">
         <v>46098</v>
       </c>
       <c r="I17" t="s">
@@ -1806,7 +1780,7 @@
       <c r="U17" t="s">
         <v>180</v>
       </c>
-      <c r="V17" s="2">
+      <c r="V17" s="1">
         <v>46168</v>
       </c>
     </row>
@@ -1832,7 +1806,7 @@
       <c r="G18" t="s">
         <v>44</v>
       </c>
-      <c r="H18" s="2">
+      <c r="H18" s="1">
         <v>46076</v>
       </c>
       <c r="I18" t="s">
@@ -1862,7 +1836,7 @@
       <c r="U18" t="s">
         <v>28</v>
       </c>
-      <c r="V18" s="2">
+      <c r="V18" s="1">
         <v>46260</v>
       </c>
     </row>
@@ -1888,7 +1862,7 @@
       <c r="G19" t="s">
         <v>44</v>
       </c>
-      <c r="H19" s="2">
+      <c r="H19" s="1">
         <v>46076</v>
       </c>
       <c r="I19" t="s">
@@ -1918,7 +1892,7 @@
       <c r="U19" t="s">
         <v>28</v>
       </c>
-      <c r="V19" s="2">
+      <c r="V19" s="1">
         <v>46260</v>
       </c>
     </row>
@@ -1965,7 +1939,7 @@
       <c r="U20" t="s">
         <v>28</v>
       </c>
-      <c r="V20" s="2">
+      <c r="V20" s="1">
         <v>46382</v>
       </c>
     </row>
@@ -2012,7 +1986,7 @@
       <c r="U21" t="s">
         <v>28</v>
       </c>
-      <c r="V21" s="2">
+      <c r="V21" s="1">
         <v>46382</v>
       </c>
     </row>
@@ -2059,7 +2033,7 @@
       <c r="U22" t="s">
         <v>28</v>
       </c>
-      <c r="V22" s="2">
+      <c r="V22" s="1">
         <v>46230</v>
       </c>
     </row>
@@ -2106,7 +2080,7 @@
       <c r="U23" t="s">
         <v>28</v>
       </c>
-      <c r="V23" s="2">
+      <c r="V23" s="1">
         <v>46230</v>
       </c>
     </row>
@@ -2132,7 +2106,7 @@
       <c r="G24" t="s">
         <v>44</v>
       </c>
-      <c r="H24" s="2">
+      <c r="H24" s="1">
         <v>46119</v>
       </c>
       <c r="I24" t="s">
@@ -2165,7 +2139,7 @@
       <c r="U24" t="s">
         <v>180</v>
       </c>
-      <c r="V24" s="2">
+      <c r="V24" s="1">
         <v>46199</v>
       </c>
     </row>
@@ -2191,7 +2165,7 @@
       <c r="G25" t="s">
         <v>44</v>
       </c>
-      <c r="H25" s="2">
+      <c r="H25" s="1">
         <v>46121</v>
       </c>
       <c r="I25" t="s">
@@ -2221,7 +2195,7 @@
       <c r="U25" t="s">
         <v>28</v>
       </c>
-      <c r="V25" s="2">
+      <c r="V25" s="1">
         <v>46199</v>
       </c>
     </row>
@@ -2247,7 +2221,7 @@
       <c r="G26" t="s">
         <v>44</v>
       </c>
-      <c r="H26" s="2">
+      <c r="H26" s="1">
         <v>46076</v>
       </c>
       <c r="I26" t="s">
@@ -2277,7 +2251,7 @@
       <c r="U26" t="s">
         <v>28</v>
       </c>
-      <c r="V26" s="2">
+      <c r="V26" s="1">
         <v>46352</v>
       </c>
     </row>
@@ -2330,7 +2304,7 @@
       <c r="U27" t="s">
         <v>180</v>
       </c>
-      <c r="V27" s="2">
+      <c r="V27" s="1">
         <v>46352</v>
       </c>
     </row>
@@ -2356,7 +2330,7 @@
       <c r="G28" t="s">
         <v>44</v>
       </c>
-      <c r="H28" s="2">
+      <c r="H28" s="1">
         <v>46199</v>
       </c>
       <c r="I28" t="s">
@@ -2389,7 +2363,7 @@
       <c r="U28" t="s">
         <v>180</v>
       </c>
-      <c r="V28" s="2">
+      <c r="V28" s="1">
         <v>46260</v>
       </c>
     </row>
@@ -2415,7 +2389,7 @@
       <c r="G29" t="s">
         <v>44</v>
       </c>
-      <c r="H29" s="2">
+      <c r="H29" s="1">
         <v>46199</v>
       </c>
       <c r="I29" t="s">
@@ -2448,7 +2422,7 @@
       <c r="U29" t="s">
         <v>180</v>
       </c>
-      <c r="V29" s="2">
+      <c r="V29" s="1">
         <v>46260</v>
       </c>
     </row>
@@ -2474,7 +2448,7 @@
       <c r="G30" t="s">
         <v>44</v>
       </c>
-      <c r="H30" s="2">
+      <c r="H30" s="1">
         <v>46199</v>
       </c>
       <c r="I30" t="s">
@@ -2507,7 +2481,7 @@
       <c r="U30" t="s">
         <v>180</v>
       </c>
-      <c r="V30" s="2">
+      <c r="V30" s="1">
         <v>46260</v>
       </c>
     </row>
@@ -2533,7 +2507,7 @@
       <c r="G31" t="s">
         <v>44</v>
       </c>
-      <c r="H31" s="2">
+      <c r="H31" s="1">
         <v>46199</v>
       </c>
       <c r="I31" t="s">
@@ -2566,7 +2540,7 @@
       <c r="U31" t="s">
         <v>180</v>
       </c>
-      <c r="V31" s="2">
+      <c r="V31" s="1">
         <v>46260</v>
       </c>
     </row>
@@ -2616,7 +2590,7 @@
       <c r="U32" t="s">
         <v>180</v>
       </c>
-      <c r="V32" s="2">
+      <c r="V32" s="1">
         <v>46352</v>
       </c>
     </row>
@@ -2642,7 +2616,7 @@
       <c r="G33" t="s">
         <v>44</v>
       </c>
-      <c r="H33" s="2">
+      <c r="H33" s="1">
         <v>46191</v>
       </c>
       <c r="I33" t="s">
@@ -2675,7 +2649,7 @@
       <c r="U33" t="s">
         <v>180</v>
       </c>
-      <c r="V33" s="2">
+      <c r="V33" s="1">
         <v>46260</v>
       </c>
     </row>
@@ -2701,7 +2675,7 @@
       <c r="G34" t="s">
         <v>44</v>
       </c>
-      <c r="H34" s="2">
+      <c r="H34" s="1">
         <v>46119</v>
       </c>
       <c r="I34" t="s">
@@ -2731,7 +2705,7 @@
       <c r="U34" t="s">
         <v>180</v>
       </c>
-      <c r="V34" s="2">
+      <c r="V34" s="1">
         <v>46260</v>
       </c>
     </row>
@@ -2757,7 +2731,7 @@
       <c r="G35" t="s">
         <v>44</v>
       </c>
-      <c r="H35" s="2">
+      <c r="H35" s="1">
         <v>46213</v>
       </c>
       <c r="I35" t="s">
@@ -2787,7 +2761,7 @@
       <c r="U35" t="s">
         <v>28</v>
       </c>
-      <c r="V35" s="2">
+      <c r="V35" s="1">
         <v>46352</v>
       </c>
     </row>
@@ -2813,7 +2787,7 @@
       <c r="G36" t="s">
         <v>44</v>
       </c>
-      <c r="H36" s="2">
+      <c r="H36" s="1">
         <v>46175</v>
       </c>
       <c r="I36" t="s">
@@ -2843,7 +2817,7 @@
       <c r="U36" t="s">
         <v>28</v>
       </c>
-      <c r="V36" s="2">
+      <c r="V36" s="1">
         <v>46260</v>
       </c>
     </row>
@@ -2869,7 +2843,7 @@
       <c r="G37" t="s">
         <v>44</v>
       </c>
-      <c r="H37" s="2">
+      <c r="H37" s="1">
         <v>46213</v>
       </c>
       <c r="I37" t="s">
@@ -2899,7 +2873,7 @@
       <c r="U37" t="s">
         <v>28</v>
       </c>
-      <c r="V37" s="2">
+      <c r="V37" s="1">
         <v>46352</v>
       </c>
     </row>
@@ -2925,7 +2899,7 @@
       <c r="G38" t="s">
         <v>44</v>
       </c>
-      <c r="H38" s="2">
+      <c r="H38" s="1">
         <v>46199</v>
       </c>
       <c r="I38" t="s">
@@ -2955,7 +2929,7 @@
       <c r="U38" t="s">
         <v>28</v>
       </c>
-      <c r="V38" s="2">
+      <c r="V38" s="1">
         <v>46229</v>
       </c>
     </row>
@@ -2981,7 +2955,7 @@
       <c r="G39" t="s">
         <v>44</v>
       </c>
-      <c r="H39" s="2">
+      <c r="H39" s="1">
         <v>46199</v>
       </c>
       <c r="I39" t="s">
@@ -3011,7 +2985,7 @@
       <c r="U39" t="s">
         <v>28</v>
       </c>
-      <c r="V39" s="2">
+      <c r="V39" s="1">
         <v>46229</v>
       </c>
     </row>
@@ -3037,7 +3011,7 @@
       <c r="G40" t="s">
         <v>44</v>
       </c>
-      <c r="H40" s="2">
+      <c r="H40" s="1">
         <v>46204</v>
       </c>
       <c r="I40" t="s">
@@ -3067,7 +3041,7 @@
       <c r="U40" t="s">
         <v>28</v>
       </c>
-      <c r="V40" s="2">
+      <c r="V40" s="1">
         <v>46229</v>
       </c>
     </row>
@@ -3093,7 +3067,7 @@
       <c r="G41" t="s">
         <v>44</v>
       </c>
-      <c r="H41" s="2">
+      <c r="H41" s="1">
         <v>46244</v>
       </c>
       <c r="I41" t="s">
@@ -3123,7 +3097,7 @@
       <c r="U41" t="s">
         <v>28</v>
       </c>
-      <c r="V41" s="2">
+      <c r="V41" s="1">
         <v>46260</v>
       </c>
     </row>
@@ -3167,7 +3141,7 @@
       <c r="U42" t="s">
         <v>28</v>
       </c>
-      <c r="V42" s="2">
+      <c r="V42" s="1">
         <v>46352</v>
       </c>
     </row>
@@ -3193,7 +3167,7 @@
       <c r="G43" t="s">
         <v>44</v>
       </c>
-      <c r="H43" s="2">
+      <c r="H43" s="1">
         <v>46191</v>
       </c>
       <c r="I43" t="s">
@@ -3223,7 +3197,7 @@
       <c r="U43" t="s">
         <v>28</v>
       </c>
-      <c r="V43" s="2">
+      <c r="V43" s="1">
         <v>46229</v>
       </c>
     </row>
@@ -3249,7 +3223,7 @@
       <c r="G44" t="s">
         <v>44</v>
       </c>
-      <c r="H44" s="2">
+      <c r="H44" s="1">
         <v>46191</v>
       </c>
       <c r="I44" t="s">
@@ -3279,7 +3253,7 @@
       <c r="U44" t="s">
         <v>28</v>
       </c>
-      <c r="V44" s="2">
+      <c r="V44" s="1">
         <v>46229</v>
       </c>
     </row>
@@ -3305,7 +3279,7 @@
       <c r="G45" t="s">
         <v>44</v>
       </c>
-      <c r="H45" s="2">
+      <c r="H45" s="1">
         <v>46213</v>
       </c>
       <c r="I45" t="s">
@@ -3338,7 +3312,7 @@
       <c r="U45" t="s">
         <v>180</v>
       </c>
-      <c r="V45" s="2">
+      <c r="V45" s="1">
         <v>46291</v>
       </c>
     </row>
@@ -3364,7 +3338,7 @@
       <c r="G46" t="s">
         <v>44</v>
       </c>
-      <c r="H46" s="2">
+      <c r="H46" s="1">
         <v>46210</v>
       </c>
       <c r="I46" t="s">
@@ -3394,7 +3368,7 @@
       <c r="U46" t="s">
         <v>180</v>
       </c>
-      <c r="V46" s="2">
+      <c r="V46" s="1">
         <v>46291</v>
       </c>
     </row>
@@ -3441,7 +3415,7 @@
       <c r="U47" t="s">
         <v>28</v>
       </c>
-      <c r="V47" s="2">
+      <c r="V47" s="1">
         <v>46321</v>
       </c>
     </row>
@@ -3494,7 +3468,7 @@
       <c r="U48" t="s">
         <v>180</v>
       </c>
-      <c r="V48" s="2">
+      <c r="V48" s="1">
         <v>46352</v>
       </c>
     </row>
@@ -3520,7 +3494,7 @@
       <c r="G49" t="s">
         <v>44</v>
       </c>
-      <c r="H49" s="2">
+      <c r="H49" s="1">
         <v>46176</v>
       </c>
       <c r="I49" t="s">
@@ -3553,7 +3527,7 @@
       <c r="U49" t="s">
         <v>180</v>
       </c>
-      <c r="V49" s="2">
+      <c r="V49" s="1">
         <v>46352</v>
       </c>
     </row>
@@ -3606,7 +3580,7 @@
       <c r="U50" t="s">
         <v>180</v>
       </c>
-      <c r="V50" s="2">
+      <c r="V50" s="1">
         <v>46321</v>
       </c>
     </row>
@@ -3659,7 +3633,7 @@
       <c r="U51" t="s">
         <v>180</v>
       </c>
-      <c r="V51" s="2">
+      <c r="V51" s="1">
         <v>46352</v>
       </c>
     </row>
@@ -3709,7 +3683,7 @@
       <c r="U52" t="s">
         <v>180</v>
       </c>
-      <c r="V52" s="2">
+      <c r="V52" s="1">
         <v>46382</v>
       </c>
     </row>
@@ -3735,7 +3709,7 @@
       <c r="G53" t="s">
         <v>44</v>
       </c>
-      <c r="H53" s="2">
+      <c r="H53" s="1">
         <v>46227</v>
       </c>
       <c r="I53" t="s">
@@ -3765,7 +3739,7 @@
       <c r="U53" t="s">
         <v>180</v>
       </c>
-      <c r="V53" s="2">
+      <c r="V53" s="1">
         <v>46321</v>
       </c>
     </row>
@@ -3788,7 +3762,7 @@
       <c r="G54" t="s">
         <v>44</v>
       </c>
-      <c r="H54" s="2">
+      <c r="H54" s="1">
         <v>46280</v>
       </c>
       <c r="I54" t="s">
@@ -3818,7 +3792,7 @@
       <c r="U54" t="s">
         <v>180</v>
       </c>
-      <c r="V54" s="2">
+      <c r="V54" s="1">
         <v>46352</v>
       </c>
     </row>
@@ -3841,7 +3815,7 @@
       <c r="G55" t="s">
         <v>44</v>
       </c>
-      <c r="H55" s="2">
+      <c r="H55" s="1">
         <v>46280</v>
       </c>
       <c r="I55" t="s">
@@ -3871,7 +3845,7 @@
       <c r="U55" t="s">
         <v>180</v>
       </c>
-      <c r="V55" s="2">
+      <c r="V55" s="1">
         <v>46321</v>
       </c>
     </row>
@@ -3924,7 +3898,7 @@
       <c r="U56" t="s">
         <v>180</v>
       </c>
-      <c r="V56" s="2">
+      <c r="V56" s="1">
         <v>46049</v>
       </c>
     </row>
@@ -3977,7 +3951,7 @@
       <c r="U57" t="s">
         <v>180</v>
       </c>
-      <c r="V57" s="2">
+      <c r="V57" s="1">
         <v>46049</v>
       </c>
     </row>
@@ -4024,7 +3998,7 @@
       <c r="U58" t="s">
         <v>180</v>
       </c>
-      <c r="V58" s="2">
+      <c r="V58" s="1">
         <v>46049</v>
       </c>
     </row>
@@ -4068,7 +4042,7 @@
       <c r="U59" t="s">
         <v>180</v>
       </c>
-      <c r="V59" s="2">
+      <c r="V59" s="1">
         <v>46139</v>
       </c>
     </row>
@@ -4194,7 +4168,7 @@
       <c r="U62" t="s">
         <v>180</v>
       </c>
-      <c r="V62" s="2">
+      <c r="V62" s="1">
         <v>46168</v>
       </c>
     </row>
@@ -4238,7 +4212,7 @@
       <c r="U63" t="s">
         <v>180</v>
       </c>
-      <c r="V63" s="2">
+      <c r="V63" s="1">
         <v>46168</v>
       </c>
     </row>
@@ -4282,7 +4256,7 @@
       <c r="U64" t="s">
         <v>180</v>
       </c>
-      <c r="V64" s="2">
+      <c r="V64" s="1">
         <v>46168</v>
       </c>
     </row>
@@ -4326,7 +4300,7 @@
       <c r="U65" t="s">
         <v>180</v>
       </c>
-      <c r="V65" s="2">
+      <c r="V65" s="1">
         <v>46168</v>
       </c>
     </row>
@@ -4370,7 +4344,7 @@
       <c r="U66" t="s">
         <v>180</v>
       </c>
-      <c r="V66" s="2">
+      <c r="V66" s="1">
         <v>46168</v>
       </c>
     </row>
@@ -4414,7 +4388,7 @@
       <c r="U67" t="s">
         <v>180</v>
       </c>
-      <c r="V67" s="2">
+      <c r="V67" s="1">
         <v>46168</v>
       </c>
     </row>
@@ -4458,7 +4432,7 @@
       <c r="U68" t="s">
         <v>28</v>
       </c>
-      <c r="V68" s="2">
+      <c r="V68" s="1">
         <v>46168</v>
       </c>
     </row>
@@ -4505,7 +4479,7 @@
       <c r="U69" t="s">
         <v>28</v>
       </c>
-      <c r="V69" s="2">
+      <c r="V69" s="1">
         <v>46382</v>
       </c>
     </row>
@@ -4558,7 +4532,7 @@
       <c r="U70" t="s">
         <v>180</v>
       </c>
-      <c r="V70" s="2">
+      <c r="V70" s="1">
         <v>46291</v>
       </c>
     </row>
@@ -4602,7 +4576,7 @@
       <c r="U71" t="s">
         <v>28</v>
       </c>
-      <c r="V71" s="2">
+      <c r="V71" s="1">
         <v>46260</v>
       </c>
     </row>
@@ -4646,7 +4620,7 @@
       <c r="U72" t="s">
         <v>180</v>
       </c>
-      <c r="V72" s="2">
+      <c r="V72" s="1">
         <v>46352</v>
       </c>
     </row>
@@ -4690,7 +4664,7 @@
       <c r="U73" t="s">
         <v>180</v>
       </c>
-      <c r="V73" s="2">
+      <c r="V73" s="1">
         <v>46229</v>
       </c>
     </row>
@@ -4734,7 +4708,7 @@
       <c r="U74" t="s">
         <v>180</v>
       </c>
-      <c r="V74" s="2">
+      <c r="V74" s="1">
         <v>46352</v>
       </c>
     </row>
@@ -4778,7 +4752,7 @@
       <c r="U75" t="s">
         <v>180</v>
       </c>
-      <c r="V75" s="2">
+      <c r="V75" s="1">
         <v>46352</v>
       </c>
     </row>
@@ -4822,7 +4796,7 @@
       <c r="U76" t="s">
         <v>180</v>
       </c>
-      <c r="V76" s="2">
+      <c r="V76" s="1">
         <v>46352</v>
       </c>
     </row>
@@ -4869,7 +4843,7 @@
       <c r="U77" t="s">
         <v>28</v>
       </c>
-      <c r="V77" s="2">
+      <c r="V77" s="1">
         <v>46382</v>
       </c>
     </row>
@@ -4919,7 +4893,7 @@
       <c r="U78" t="s">
         <v>180</v>
       </c>
-      <c r="V78" s="2">
+      <c r="V78" s="1">
         <v>46107</v>
       </c>
     </row>
@@ -4969,7 +4943,7 @@
       <c r="U79" t="s">
         <v>180</v>
       </c>
-      <c r="V79" s="2">
+      <c r="V79" s="1">
         <v>46138</v>
       </c>
     </row>
@@ -5019,7 +4993,7 @@
       <c r="U80" t="s">
         <v>28</v>
       </c>
-      <c r="V80" s="2">
+      <c r="V80" s="1">
         <v>46260</v>
       </c>
     </row>
@@ -5069,7 +5043,7 @@
       <c r="U81" t="s">
         <v>28</v>
       </c>
-      <c r="V81" s="2">
+      <c r="V81" s="1">
         <v>46260</v>
       </c>
     </row>
@@ -5119,7 +5093,7 @@
       <c r="U82" t="s">
         <v>28</v>
       </c>
-      <c r="V82" s="2">
+      <c r="V82" s="1">
         <v>46108</v>
       </c>
     </row>
@@ -5163,7 +5137,7 @@
       <c r="U83" t="s">
         <v>28</v>
       </c>
-      <c r="V83" s="2">
+      <c r="V83" s="1">
         <v>46108</v>
       </c>
     </row>
@@ -5216,7 +5190,7 @@
       <c r="U84" t="s">
         <v>180</v>
       </c>
-      <c r="V84" s="2">
+      <c r="V84" s="1">
         <v>46080</v>
       </c>
     </row>
@@ -5263,7 +5237,7 @@
       <c r="U85" t="s">
         <v>28</v>
       </c>
-      <c r="V85" s="2">
+      <c r="V85" s="1">
         <v>46382</v>
       </c>
     </row>
@@ -5307,7 +5281,7 @@
       <c r="U86" t="s">
         <v>28</v>
       </c>
-      <c r="V86" s="2">
+      <c r="V86" s="1">
         <v>46108</v>
       </c>
     </row>
@@ -5448,7 +5422,7 @@
       <c r="U89" t="s">
         <v>28</v>
       </c>
-      <c r="V89" s="2">
+      <c r="V89" s="1">
         <v>46321</v>
       </c>
     </row>
@@ -5492,7 +5466,7 @@
       <c r="U90" t="s">
         <v>28</v>
       </c>
-      <c r="V90" s="2">
+      <c r="V90" s="1">
         <v>46382</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Atualização automática: mta (29/09/2026 13:53)
</commit_message>
<xml_diff>
--- a/Projetos/02_Dados_Tratados/base_mta_tratada.xlsx
+++ b/Projetos/02_Dados_Tratados/base_mta_tratada.xlsx
@@ -14,7 +14,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1188" uniqueCount="181">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1189" uniqueCount="182">
   <si>
     <t>linha</t>
   </si>
@@ -151,6 +151,9 @@
     <t>ATENDIDO</t>
   </si>
   <si>
+    <t>ATENDER</t>
+  </si>
+  <si>
     <t>BLOQUEIO</t>
   </si>
   <si>
@@ -235,9 +238,6 @@
     <t>Atender</t>
   </si>
   <si>
-    <t>ATENDER</t>
-  </si>
-  <si>
     <t>REMANEJAR</t>
   </si>
   <si>
@@ -526,10 +526,13 @@
     <t>FMS</t>
   </si>
   <si>
-    <t>DÓLAR</t>
-  </si>
-  <si>
-    <t>REAL</t>
+    <t>339030</t>
+  </si>
+  <si>
+    <t>339039</t>
+  </si>
+  <si>
+    <t>449052</t>
   </si>
   <si>
     <t>A</t>
@@ -983,10 +986,10 @@
         <v>30</v>
       </c>
       <c r="J2" t="s">
-        <v>64</v>
+        <v>65</v>
       </c>
       <c r="K2" t="s">
-        <v>72</v>
+        <v>73</v>
       </c>
       <c r="L2" t="s">
         <v>79</v>
@@ -1007,13 +1010,13 @@
         <v>170</v>
       </c>
       <c r="S2" t="s">
-        <v>172</v>
+        <v>173</v>
       </c>
       <c r="T2" t="s">
-        <v>175</v>
+        <v>176</v>
       </c>
       <c r="U2" t="s">
-        <v>180</v>
+        <v>181</v>
       </c>
       <c r="V2" s="1">
         <v>46291</v>
@@ -1054,10 +1057,10 @@
         <v>170</v>
       </c>
       <c r="S3" t="s">
-        <v>172</v>
+        <v>173</v>
       </c>
       <c r="T3" t="s">
-        <v>175</v>
+        <v>176</v>
       </c>
       <c r="U3" t="s">
         <v>28</v>
@@ -1098,13 +1101,13 @@
         <v>167</v>
       </c>
       <c r="R4" t="s">
-        <v>170</v>
+        <v>171</v>
       </c>
       <c r="S4" t="s">
-        <v>172</v>
+        <v>173</v>
       </c>
       <c r="T4" t="s">
-        <v>175</v>
+        <v>176</v>
       </c>
       <c r="U4" t="s">
         <v>28</v>
@@ -1145,13 +1148,13 @@
         <v>167</v>
       </c>
       <c r="R5" t="s">
-        <v>170</v>
+        <v>171</v>
       </c>
       <c r="S5" t="s">
-        <v>172</v>
+        <v>173</v>
       </c>
       <c r="T5" t="s">
-        <v>175</v>
+        <v>176</v>
       </c>
       <c r="U5" t="s">
         <v>28</v>
@@ -1195,13 +1198,13 @@
         <v>167</v>
       </c>
       <c r="R6" t="s">
-        <v>170</v>
+        <v>171</v>
       </c>
       <c r="S6" t="s">
-        <v>172</v>
+        <v>173</v>
       </c>
       <c r="T6" t="s">
-        <v>175</v>
+        <v>176</v>
       </c>
       <c r="U6" t="s">
         <v>28</v>
@@ -1236,7 +1239,7 @@
         <v>46121</v>
       </c>
       <c r="I7" t="s">
-        <v>47</v>
+        <v>48</v>
       </c>
       <c r="N7" t="s">
         <v>83</v>
@@ -1254,10 +1257,10 @@
         <v>171</v>
       </c>
       <c r="S7" t="s">
-        <v>172</v>
+        <v>173</v>
       </c>
       <c r="T7" t="s">
-        <v>176</v>
+        <v>177</v>
       </c>
       <c r="U7" t="s">
         <v>28</v>
@@ -1298,13 +1301,13 @@
         <v>167</v>
       </c>
       <c r="R8" t="s">
-        <v>170</v>
+        <v>171</v>
       </c>
       <c r="S8" t="s">
-        <v>172</v>
+        <v>173</v>
       </c>
       <c r="T8" t="s">
-        <v>175</v>
+        <v>176</v>
       </c>
       <c r="U8" t="s">
         <v>28</v>
@@ -1345,13 +1348,13 @@
         <v>167</v>
       </c>
       <c r="R9" t="s">
-        <v>170</v>
+        <v>171</v>
       </c>
       <c r="S9" t="s">
-        <v>172</v>
+        <v>173</v>
       </c>
       <c r="T9" t="s">
-        <v>175</v>
+        <v>176</v>
       </c>
       <c r="U9" t="s">
         <v>28</v>
@@ -1392,13 +1395,13 @@
         <v>167</v>
       </c>
       <c r="R10" t="s">
-        <v>170</v>
+        <v>171</v>
       </c>
       <c r="S10" t="s">
-        <v>172</v>
+        <v>173</v>
       </c>
       <c r="T10" t="s">
-        <v>175</v>
+        <v>176</v>
       </c>
       <c r="U10" t="s">
         <v>28</v>
@@ -1439,13 +1442,13 @@
         <v>167</v>
       </c>
       <c r="R11" t="s">
-        <v>170</v>
+        <v>171</v>
       </c>
       <c r="S11" t="s">
-        <v>172</v>
+        <v>173</v>
       </c>
       <c r="T11" t="s">
-        <v>175</v>
+        <v>176</v>
       </c>
       <c r="U11" t="s">
         <v>28</v>
@@ -1480,10 +1483,10 @@
         <v>46079</v>
       </c>
       <c r="I12" t="s">
-        <v>48</v>
+        <v>49</v>
       </c>
       <c r="J12" t="s">
-        <v>65</v>
+        <v>66</v>
       </c>
       <c r="N12" t="s">
         <v>80</v>
@@ -1501,13 +1504,13 @@
         <v>170</v>
       </c>
       <c r="S12" t="s">
-        <v>172</v>
+        <v>173</v>
       </c>
       <c r="T12" t="s">
-        <v>175</v>
+        <v>176</v>
       </c>
       <c r="U12" t="s">
-        <v>180</v>
+        <v>181</v>
       </c>
       <c r="V12" s="1">
         <v>46168</v>
@@ -1533,10 +1536,10 @@
         <v>30</v>
       </c>
       <c r="J13" t="s">
-        <v>64</v>
+        <v>65</v>
       </c>
       <c r="K13" t="s">
-        <v>73</v>
+        <v>45</v>
       </c>
       <c r="N13" t="s">
         <v>80</v>
@@ -1554,13 +1557,13 @@
         <v>170</v>
       </c>
       <c r="S13" t="s">
-        <v>172</v>
+        <v>173</v>
       </c>
       <c r="T13" t="s">
-        <v>175</v>
+        <v>176</v>
       </c>
       <c r="U13" t="s">
-        <v>180</v>
+        <v>181</v>
       </c>
       <c r="V13" s="1">
         <v>46049</v>
@@ -1586,10 +1589,10 @@
         <v>30</v>
       </c>
       <c r="J14" t="s">
-        <v>64</v>
+        <v>65</v>
       </c>
       <c r="K14" t="s">
-        <v>73</v>
+        <v>45</v>
       </c>
       <c r="N14" t="s">
         <v>80</v>
@@ -1607,13 +1610,13 @@
         <v>170</v>
       </c>
       <c r="S14" t="s">
-        <v>172</v>
+        <v>173</v>
       </c>
       <c r="T14" t="s">
-        <v>175</v>
+        <v>176</v>
       </c>
       <c r="U14" t="s">
-        <v>180</v>
+        <v>181</v>
       </c>
       <c r="V14" s="1">
         <v>46049</v>
@@ -1639,10 +1642,10 @@
         <v>30</v>
       </c>
       <c r="J15" t="s">
-        <v>64</v>
+        <v>65</v>
       </c>
       <c r="K15" t="s">
-        <v>73</v>
+        <v>45</v>
       </c>
       <c r="N15" t="s">
         <v>80</v>
@@ -1660,13 +1663,13 @@
         <v>170</v>
       </c>
       <c r="S15" t="s">
-        <v>172</v>
+        <v>173</v>
       </c>
       <c r="T15" t="s">
-        <v>175</v>
+        <v>176</v>
       </c>
       <c r="U15" t="s">
-        <v>180</v>
+        <v>181</v>
       </c>
       <c r="V15" s="1">
         <v>46049</v>
@@ -1692,10 +1695,10 @@
         <v>30</v>
       </c>
       <c r="J16" t="s">
-        <v>64</v>
+        <v>65</v>
       </c>
       <c r="K16" t="s">
-        <v>73</v>
+        <v>45</v>
       </c>
       <c r="N16" t="s">
         <v>84</v>
@@ -1713,13 +1716,13 @@
         <v>170</v>
       </c>
       <c r="S16" t="s">
-        <v>172</v>
+        <v>173</v>
       </c>
       <c r="T16" t="s">
-        <v>175</v>
+        <v>176</v>
       </c>
       <c r="U16" t="s">
-        <v>180</v>
+        <v>181</v>
       </c>
       <c r="V16" s="1">
         <v>46291</v>
@@ -1751,10 +1754,10 @@
         <v>46098</v>
       </c>
       <c r="I17" t="s">
-        <v>49</v>
+        <v>50</v>
       </c>
       <c r="J17" t="s">
-        <v>65</v>
+        <v>66</v>
       </c>
       <c r="N17" t="s">
         <v>85</v>
@@ -1772,13 +1775,13 @@
         <v>171</v>
       </c>
       <c r="S17" t="s">
-        <v>172</v>
+        <v>173</v>
       </c>
       <c r="T17" t="s">
-        <v>177</v>
+        <v>178</v>
       </c>
       <c r="U17" t="s">
-        <v>180</v>
+        <v>181</v>
       </c>
       <c r="V17" s="1">
         <v>46168</v>
@@ -1810,7 +1813,7 @@
         <v>46076</v>
       </c>
       <c r="I18" t="s">
-        <v>50</v>
+        <v>51</v>
       </c>
       <c r="N18" t="s">
         <v>86</v>
@@ -1825,13 +1828,13 @@
         <v>168</v>
       </c>
       <c r="R18" t="s">
-        <v>171</v>
+        <v>170</v>
       </c>
       <c r="S18" t="s">
-        <v>172</v>
+        <v>173</v>
       </c>
       <c r="T18" t="s">
-        <v>176</v>
+        <v>177</v>
       </c>
       <c r="U18" t="s">
         <v>28</v>
@@ -1866,7 +1869,7 @@
         <v>46076</v>
       </c>
       <c r="I19" t="s">
-        <v>50</v>
+        <v>51</v>
       </c>
       <c r="N19" t="s">
         <v>86</v>
@@ -1881,13 +1884,13 @@
         <v>168</v>
       </c>
       <c r="R19" t="s">
-        <v>171</v>
+        <v>170</v>
       </c>
       <c r="S19" t="s">
-        <v>172</v>
+        <v>173</v>
       </c>
       <c r="T19" t="s">
-        <v>176</v>
+        <v>177</v>
       </c>
       <c r="U19" t="s">
         <v>28</v>
@@ -1928,13 +1931,13 @@
         <v>168</v>
       </c>
       <c r="R20" t="s">
-        <v>171</v>
+        <v>170</v>
       </c>
       <c r="S20" t="s">
-        <v>172</v>
+        <v>173</v>
       </c>
       <c r="T20" t="s">
-        <v>176</v>
+        <v>177</v>
       </c>
       <c r="U20" t="s">
         <v>28</v>
@@ -1978,10 +1981,10 @@
         <v>170</v>
       </c>
       <c r="S21" t="s">
-        <v>172</v>
+        <v>173</v>
       </c>
       <c r="T21" t="s">
-        <v>175</v>
+        <v>176</v>
       </c>
       <c r="U21" t="s">
         <v>28</v>
@@ -2022,13 +2025,13 @@
         <v>167</v>
       </c>
       <c r="R22" t="s">
-        <v>170</v>
+        <v>171</v>
       </c>
       <c r="S22" t="s">
-        <v>172</v>
+        <v>173</v>
       </c>
       <c r="T22" t="s">
-        <v>175</v>
+        <v>176</v>
       </c>
       <c r="U22" t="s">
         <v>28</v>
@@ -2069,13 +2072,13 @@
         <v>167</v>
       </c>
       <c r="R23" t="s">
-        <v>170</v>
+        <v>171</v>
       </c>
       <c r="S23" t="s">
-        <v>172</v>
+        <v>173</v>
       </c>
       <c r="T23" t="s">
-        <v>175</v>
+        <v>176</v>
       </c>
       <c r="U23" t="s">
         <v>28</v>
@@ -2110,10 +2113,10 @@
         <v>46119</v>
       </c>
       <c r="I24" t="s">
-        <v>51</v>
+        <v>52</v>
       </c>
       <c r="J24" t="s">
-        <v>66</v>
+        <v>67</v>
       </c>
       <c r="N24" t="s">
         <v>85</v>
@@ -2131,13 +2134,13 @@
         <v>171</v>
       </c>
       <c r="S24" t="s">
-        <v>172</v>
+        <v>173</v>
       </c>
       <c r="T24" t="s">
-        <v>177</v>
+        <v>178</v>
       </c>
       <c r="U24" t="s">
-        <v>180</v>
+        <v>181</v>
       </c>
       <c r="V24" s="1">
         <v>46199</v>
@@ -2169,7 +2172,7 @@
         <v>46121</v>
       </c>
       <c r="I25" t="s">
-        <v>52</v>
+        <v>53</v>
       </c>
       <c r="N25" t="s">
         <v>88</v>
@@ -2187,10 +2190,10 @@
         <v>171</v>
       </c>
       <c r="S25" t="s">
-        <v>172</v>
+        <v>173</v>
       </c>
       <c r="T25" t="s">
-        <v>176</v>
+        <v>177</v>
       </c>
       <c r="U25" t="s">
         <v>28</v>
@@ -2225,7 +2228,7 @@
         <v>46076</v>
       </c>
       <c r="I26" t="s">
-        <v>53</v>
+        <v>54</v>
       </c>
       <c r="N26" t="s">
         <v>88</v>
@@ -2240,13 +2243,13 @@
         <v>168</v>
       </c>
       <c r="R26" t="s">
-        <v>171</v>
+        <v>170</v>
       </c>
       <c r="S26" t="s">
-        <v>172</v>
+        <v>173</v>
       </c>
       <c r="T26" t="s">
-        <v>176</v>
+        <v>177</v>
       </c>
       <c r="U26" t="s">
         <v>28</v>
@@ -2275,10 +2278,10 @@
         <v>30</v>
       </c>
       <c r="J27" t="s">
-        <v>64</v>
+        <v>65</v>
       </c>
       <c r="K27" t="s">
-        <v>73</v>
+        <v>45</v>
       </c>
       <c r="N27" t="s">
         <v>84</v>
@@ -2296,13 +2299,13 @@
         <v>170</v>
       </c>
       <c r="S27" t="s">
-        <v>172</v>
+        <v>173</v>
       </c>
       <c r="T27" t="s">
-        <v>175</v>
+        <v>176</v>
       </c>
       <c r="U27" t="s">
-        <v>180</v>
+        <v>181</v>
       </c>
       <c r="V27" s="1">
         <v>46352</v>
@@ -2334,10 +2337,10 @@
         <v>46199</v>
       </c>
       <c r="I28" t="s">
-        <v>54</v>
+        <v>55</v>
       </c>
       <c r="J28" t="s">
-        <v>67</v>
+        <v>68</v>
       </c>
       <c r="N28" t="s">
         <v>85</v>
@@ -2355,13 +2358,13 @@
         <v>171</v>
       </c>
       <c r="S28" t="s">
-        <v>172</v>
+        <v>173</v>
       </c>
       <c r="T28" t="s">
-        <v>176</v>
+        <v>177</v>
       </c>
       <c r="U28" t="s">
-        <v>180</v>
+        <v>181</v>
       </c>
       <c r="V28" s="1">
         <v>46260</v>
@@ -2393,10 +2396,10 @@
         <v>46199</v>
       </c>
       <c r="I29" t="s">
-        <v>54</v>
+        <v>55</v>
       </c>
       <c r="J29" t="s">
-        <v>67</v>
+        <v>68</v>
       </c>
       <c r="N29" t="s">
         <v>85</v>
@@ -2414,13 +2417,13 @@
         <v>171</v>
       </c>
       <c r="S29" t="s">
-        <v>172</v>
+        <v>173</v>
       </c>
       <c r="T29" t="s">
-        <v>176</v>
+        <v>177</v>
       </c>
       <c r="U29" t="s">
-        <v>180</v>
+        <v>181</v>
       </c>
       <c r="V29" s="1">
         <v>46260</v>
@@ -2452,10 +2455,10 @@
         <v>46199</v>
       </c>
       <c r="I30" t="s">
-        <v>55</v>
+        <v>56</v>
       </c>
       <c r="J30" t="s">
-        <v>67</v>
+        <v>68</v>
       </c>
       <c r="N30" t="s">
         <v>85</v>
@@ -2473,13 +2476,13 @@
         <v>171</v>
       </c>
       <c r="S30" t="s">
-        <v>172</v>
+        <v>173</v>
       </c>
       <c r="T30" t="s">
-        <v>176</v>
+        <v>177</v>
       </c>
       <c r="U30" t="s">
-        <v>180</v>
+        <v>181</v>
       </c>
       <c r="V30" s="1">
         <v>46260</v>
@@ -2511,10 +2514,10 @@
         <v>46199</v>
       </c>
       <c r="I31" t="s">
-        <v>54</v>
+        <v>55</v>
       </c>
       <c r="J31" t="s">
-        <v>67</v>
+        <v>68</v>
       </c>
       <c r="N31" t="s">
         <v>85</v>
@@ -2532,13 +2535,13 @@
         <v>171</v>
       </c>
       <c r="S31" t="s">
-        <v>172</v>
+        <v>173</v>
       </c>
       <c r="T31" t="s">
-        <v>176</v>
+        <v>177</v>
       </c>
       <c r="U31" t="s">
-        <v>180</v>
+        <v>181</v>
       </c>
       <c r="V31" s="1">
         <v>46260</v>
@@ -2582,13 +2585,13 @@
         <v>171</v>
       </c>
       <c r="S32" t="s">
-        <v>172</v>
+        <v>173</v>
       </c>
       <c r="T32" t="s">
-        <v>176</v>
+        <v>177</v>
       </c>
       <c r="U32" t="s">
-        <v>180</v>
+        <v>181</v>
       </c>
       <c r="V32" s="1">
         <v>46352</v>
@@ -2620,10 +2623,10 @@
         <v>46191</v>
       </c>
       <c r="I33" t="s">
-        <v>56</v>
+        <v>57</v>
       </c>
       <c r="J33" t="s">
-        <v>68</v>
+        <v>69</v>
       </c>
       <c r="N33" t="s">
         <v>85</v>
@@ -2641,13 +2644,13 @@
         <v>171</v>
       </c>
       <c r="S33" t="s">
-        <v>172</v>
+        <v>173</v>
       </c>
       <c r="T33" t="s">
-        <v>177</v>
+        <v>178</v>
       </c>
       <c r="U33" t="s">
-        <v>180</v>
+        <v>181</v>
       </c>
       <c r="V33" s="1">
         <v>46260</v>
@@ -2679,7 +2682,7 @@
         <v>46119</v>
       </c>
       <c r="I34" t="s">
-        <v>51</v>
+        <v>52</v>
       </c>
       <c r="N34" t="s">
         <v>85</v>
@@ -2697,13 +2700,13 @@
         <v>171</v>
       </c>
       <c r="S34" t="s">
-        <v>172</v>
+        <v>173</v>
       </c>
       <c r="T34" t="s">
-        <v>177</v>
+        <v>178</v>
       </c>
       <c r="U34" t="s">
-        <v>180</v>
+        <v>181</v>
       </c>
       <c r="V34" s="1">
         <v>46260</v>
@@ -2735,7 +2738,7 @@
         <v>46213</v>
       </c>
       <c r="I35" t="s">
-        <v>57</v>
+        <v>58</v>
       </c>
       <c r="N35" t="s">
         <v>88</v>
@@ -2750,13 +2753,13 @@
         <v>168</v>
       </c>
       <c r="R35" t="s">
-        <v>171</v>
+        <v>170</v>
       </c>
       <c r="S35" t="s">
-        <v>172</v>
+        <v>173</v>
       </c>
       <c r="T35" t="s">
-        <v>176</v>
+        <v>177</v>
       </c>
       <c r="U35" t="s">
         <v>28</v>
@@ -2791,7 +2794,7 @@
         <v>46175</v>
       </c>
       <c r="I36" t="s">
-        <v>58</v>
+        <v>59</v>
       </c>
       <c r="N36" t="s">
         <v>88</v>
@@ -2809,10 +2812,10 @@
         <v>171</v>
       </c>
       <c r="S36" t="s">
-        <v>172</v>
+        <v>173</v>
       </c>
       <c r="T36" t="s">
-        <v>176</v>
+        <v>177</v>
       </c>
       <c r="U36" t="s">
         <v>28</v>
@@ -2847,7 +2850,7 @@
         <v>46213</v>
       </c>
       <c r="I37" t="s">
-        <v>57</v>
+        <v>58</v>
       </c>
       <c r="N37" t="s">
         <v>88</v>
@@ -2862,13 +2865,13 @@
         <v>168</v>
       </c>
       <c r="R37" t="s">
-        <v>171</v>
+        <v>170</v>
       </c>
       <c r="S37" t="s">
-        <v>172</v>
+        <v>173</v>
       </c>
       <c r="T37" t="s">
-        <v>176</v>
+        <v>177</v>
       </c>
       <c r="U37" t="s">
         <v>28</v>
@@ -2903,7 +2906,7 @@
         <v>46199</v>
       </c>
       <c r="I38" t="s">
-        <v>59</v>
+        <v>60</v>
       </c>
       <c r="N38" t="s">
         <v>88</v>
@@ -2918,13 +2921,13 @@
         <v>168</v>
       </c>
       <c r="R38" t="s">
-        <v>171</v>
+        <v>170</v>
       </c>
       <c r="S38" t="s">
-        <v>172</v>
+        <v>173</v>
       </c>
       <c r="T38" t="s">
-        <v>176</v>
+        <v>177</v>
       </c>
       <c r="U38" t="s">
         <v>28</v>
@@ -2959,7 +2962,7 @@
         <v>46199</v>
       </c>
       <c r="I39" t="s">
-        <v>59</v>
+        <v>60</v>
       </c>
       <c r="N39" t="s">
         <v>88</v>
@@ -2974,13 +2977,13 @@
         <v>168</v>
       </c>
       <c r="R39" t="s">
-        <v>171</v>
+        <v>170</v>
       </c>
       <c r="S39" t="s">
-        <v>172</v>
+        <v>173</v>
       </c>
       <c r="T39" t="s">
-        <v>176</v>
+        <v>177</v>
       </c>
       <c r="U39" t="s">
         <v>28</v>
@@ -3015,7 +3018,7 @@
         <v>46204</v>
       </c>
       <c r="I40" t="s">
-        <v>59</v>
+        <v>60</v>
       </c>
       <c r="N40" t="s">
         <v>88</v>
@@ -3030,13 +3033,13 @@
         <v>168</v>
       </c>
       <c r="R40" t="s">
-        <v>171</v>
+        <v>170</v>
       </c>
       <c r="S40" t="s">
-        <v>172</v>
+        <v>173</v>
       </c>
       <c r="T40" t="s">
-        <v>176</v>
+        <v>177</v>
       </c>
       <c r="U40" t="s">
         <v>28</v>
@@ -3071,7 +3074,7 @@
         <v>46244</v>
       </c>
       <c r="I41" t="s">
-        <v>60</v>
+        <v>61</v>
       </c>
       <c r="N41" t="s">
         <v>88</v>
@@ -3086,13 +3089,13 @@
         <v>168</v>
       </c>
       <c r="R41" t="s">
-        <v>171</v>
+        <v>170</v>
       </c>
       <c r="S41" t="s">
-        <v>172</v>
+        <v>173</v>
       </c>
       <c r="T41" t="s">
-        <v>176</v>
+        <v>177</v>
       </c>
       <c r="U41" t="s">
         <v>28</v>
@@ -3130,13 +3133,13 @@
         <v>168</v>
       </c>
       <c r="R42" t="s">
-        <v>171</v>
+        <v>170</v>
       </c>
       <c r="S42" t="s">
-        <v>173</v>
+        <v>174</v>
       </c>
       <c r="T42" t="s">
-        <v>176</v>
+        <v>177</v>
       </c>
       <c r="U42" t="s">
         <v>28</v>
@@ -3171,7 +3174,7 @@
         <v>46191</v>
       </c>
       <c r="I43" t="s">
-        <v>61</v>
+        <v>62</v>
       </c>
       <c r="N43" t="s">
         <v>86</v>
@@ -3186,13 +3189,13 @@
         <v>168</v>
       </c>
       <c r="R43" t="s">
-        <v>171</v>
+        <v>170</v>
       </c>
       <c r="S43" t="s">
-        <v>172</v>
+        <v>173</v>
       </c>
       <c r="T43" t="s">
-        <v>176</v>
+        <v>177</v>
       </c>
       <c r="U43" t="s">
         <v>28</v>
@@ -3227,7 +3230,7 @@
         <v>46191</v>
       </c>
       <c r="I44" t="s">
-        <v>61</v>
+        <v>62</v>
       </c>
       <c r="N44" t="s">
         <v>86</v>
@@ -3242,13 +3245,13 @@
         <v>168</v>
       </c>
       <c r="R44" t="s">
-        <v>171</v>
+        <v>170</v>
       </c>
       <c r="S44" t="s">
-        <v>172</v>
+        <v>173</v>
       </c>
       <c r="T44" t="s">
-        <v>176</v>
+        <v>177</v>
       </c>
       <c r="U44" t="s">
         <v>28</v>
@@ -3283,10 +3286,10 @@
         <v>46213</v>
       </c>
       <c r="I45" t="s">
-        <v>56</v>
+        <v>57</v>
       </c>
       <c r="J45" t="s">
-        <v>69</v>
+        <v>70</v>
       </c>
       <c r="N45" t="s">
         <v>85</v>
@@ -3304,13 +3307,13 @@
         <v>171</v>
       </c>
       <c r="S45" t="s">
-        <v>172</v>
+        <v>173</v>
       </c>
       <c r="T45" t="s">
-        <v>177</v>
+        <v>178</v>
       </c>
       <c r="U45" t="s">
-        <v>180</v>
+        <v>181</v>
       </c>
       <c r="V45" s="1">
         <v>46291</v>
@@ -3342,7 +3345,7 @@
         <v>46210</v>
       </c>
       <c r="I46" t="s">
-        <v>55</v>
+        <v>56</v>
       </c>
       <c r="N46" t="s">
         <v>85</v>
@@ -3360,13 +3363,13 @@
         <v>171</v>
       </c>
       <c r="S46" t="s">
-        <v>172</v>
+        <v>173</v>
       </c>
       <c r="T46" t="s">
-        <v>177</v>
+        <v>178</v>
       </c>
       <c r="U46" t="s">
-        <v>180</v>
+        <v>181</v>
       </c>
       <c r="V46" s="1">
         <v>46291</v>
@@ -3404,13 +3407,13 @@
         <v>168</v>
       </c>
       <c r="R47" t="s">
-        <v>171</v>
+        <v>170</v>
       </c>
       <c r="S47" t="s">
-        <v>172</v>
+        <v>173</v>
       </c>
       <c r="T47" t="s">
-        <v>176</v>
+        <v>177</v>
       </c>
       <c r="U47" t="s">
         <v>28</v>
@@ -3439,10 +3442,10 @@
         <v>30</v>
       </c>
       <c r="J48" t="s">
-        <v>64</v>
+        <v>65</v>
       </c>
       <c r="K48" t="s">
-        <v>73</v>
+        <v>45</v>
       </c>
       <c r="N48" t="s">
         <v>80</v>
@@ -3460,13 +3463,13 @@
         <v>170</v>
       </c>
       <c r="S48" t="s">
-        <v>172</v>
+        <v>173</v>
       </c>
       <c r="T48" t="s">
-        <v>175</v>
+        <v>176</v>
       </c>
       <c r="U48" t="s">
-        <v>180</v>
+        <v>181</v>
       </c>
       <c r="V48" s="1">
         <v>46352</v>
@@ -3498,10 +3501,10 @@
         <v>46176</v>
       </c>
       <c r="I49" t="s">
-        <v>62</v>
+        <v>63</v>
       </c>
       <c r="J49" t="s">
-        <v>70</v>
+        <v>71</v>
       </c>
       <c r="N49" t="s">
         <v>80</v>
@@ -3516,16 +3519,16 @@
         <v>167</v>
       </c>
       <c r="R49" t="s">
-        <v>170</v>
+        <v>172</v>
       </c>
       <c r="S49" t="s">
-        <v>172</v>
+        <v>173</v>
       </c>
       <c r="T49" t="s">
-        <v>175</v>
+        <v>176</v>
       </c>
       <c r="U49" t="s">
-        <v>180</v>
+        <v>181</v>
       </c>
       <c r="V49" s="1">
         <v>46352</v>
@@ -3551,7 +3554,7 @@
         <v>30</v>
       </c>
       <c r="J50" t="s">
-        <v>69</v>
+        <v>70</v>
       </c>
       <c r="K50" t="s">
         <v>75</v>
@@ -3572,13 +3575,13 @@
         <v>171</v>
       </c>
       <c r="S50" t="s">
-        <v>172</v>
+        <v>173</v>
       </c>
       <c r="T50" t="s">
-        <v>177</v>
+        <v>178</v>
       </c>
       <c r="U50" t="s">
-        <v>180</v>
+        <v>181</v>
       </c>
       <c r="V50" s="1">
         <v>46321</v>
@@ -3595,7 +3598,7 @@
         <v>22</v>
       </c>
       <c r="D51" t="s">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="E51" t="s">
         <v>28</v>
@@ -3603,11 +3606,14 @@
       <c r="F51" t="s">
         <v>30</v>
       </c>
+      <c r="G51" t="s">
+        <v>45</v>
+      </c>
       <c r="J51" t="s">
-        <v>69</v>
+        <v>70</v>
       </c>
       <c r="K51" t="s">
-        <v>72</v>
+        <v>73</v>
       </c>
       <c r="N51" t="s">
         <v>85</v>
@@ -3625,13 +3631,13 @@
         <v>171</v>
       </c>
       <c r="S51" t="s">
-        <v>172</v>
+        <v>173</v>
       </c>
       <c r="T51" t="s">
-        <v>177</v>
+        <v>178</v>
       </c>
       <c r="U51" t="s">
-        <v>180</v>
+        <v>181</v>
       </c>
       <c r="V51" s="1">
         <v>46352</v>
@@ -3675,13 +3681,13 @@
         <v>171</v>
       </c>
       <c r="S52" t="s">
-        <v>172</v>
+        <v>173</v>
       </c>
       <c r="T52" t="s">
-        <v>177</v>
+        <v>178</v>
       </c>
       <c r="U52" t="s">
-        <v>180</v>
+        <v>181</v>
       </c>
       <c r="V52" s="1">
         <v>46382</v>
@@ -3713,7 +3719,7 @@
         <v>46227</v>
       </c>
       <c r="I53" t="s">
-        <v>63</v>
+        <v>64</v>
       </c>
       <c r="N53" t="s">
         <v>85</v>
@@ -3731,13 +3737,13 @@
         <v>171</v>
       </c>
       <c r="S53" t="s">
-        <v>172</v>
+        <v>173</v>
       </c>
       <c r="T53" t="s">
-        <v>177</v>
+        <v>178</v>
       </c>
       <c r="U53" t="s">
-        <v>180</v>
+        <v>181</v>
       </c>
       <c r="V53" s="1">
         <v>46321</v>
@@ -3766,7 +3772,7 @@
         <v>46280</v>
       </c>
       <c r="I54" t="s">
-        <v>55</v>
+        <v>56</v>
       </c>
       <c r="N54" t="s">
         <v>85</v>
@@ -3784,13 +3790,13 @@
         <v>171</v>
       </c>
       <c r="S54" t="s">
-        <v>172</v>
+        <v>173</v>
       </c>
       <c r="T54" t="s">
-        <v>177</v>
+        <v>178</v>
       </c>
       <c r="U54" t="s">
-        <v>180</v>
+        <v>181</v>
       </c>
       <c r="V54" s="1">
         <v>46352</v>
@@ -3819,7 +3825,7 @@
         <v>46280</v>
       </c>
       <c r="I55" t="s">
-        <v>55</v>
+        <v>56</v>
       </c>
       <c r="N55" t="s">
         <v>85</v>
@@ -3837,13 +3843,13 @@
         <v>171</v>
       </c>
       <c r="S55" t="s">
-        <v>172</v>
+        <v>173</v>
       </c>
       <c r="T55" t="s">
-        <v>177</v>
+        <v>178</v>
       </c>
       <c r="U55" t="s">
-        <v>180</v>
+        <v>181</v>
       </c>
       <c r="V55" s="1">
         <v>46321</v>
@@ -3869,7 +3875,7 @@
         <v>30</v>
       </c>
       <c r="J56" t="s">
-        <v>64</v>
+        <v>65</v>
       </c>
       <c r="K56" t="s">
         <v>76</v>
@@ -3890,13 +3896,13 @@
         <v>171</v>
       </c>
       <c r="S56" t="s">
-        <v>172</v>
+        <v>173</v>
       </c>
       <c r="T56" t="s">
-        <v>177</v>
+        <v>178</v>
       </c>
       <c r="U56" t="s">
-        <v>180</v>
+        <v>181</v>
       </c>
       <c r="V56" s="1">
         <v>46049</v>
@@ -3922,7 +3928,7 @@
         <v>41</v>
       </c>
       <c r="J57" t="s">
-        <v>64</v>
+        <v>65</v>
       </c>
       <c r="K57" t="s">
         <v>77</v>
@@ -3943,13 +3949,13 @@
         <v>171</v>
       </c>
       <c r="S57" t="s">
-        <v>174</v>
+        <v>175</v>
       </c>
       <c r="T57" t="s">
-        <v>178</v>
+        <v>179</v>
       </c>
       <c r="U57" t="s">
-        <v>180</v>
+        <v>181</v>
       </c>
       <c r="V57" s="1">
         <v>46049</v>
@@ -3972,7 +3978,7 @@
         <v>29</v>
       </c>
       <c r="G58" t="s">
-        <v>45</v>
+        <v>46</v>
       </c>
       <c r="N58" t="s">
         <v>89</v>
@@ -3990,13 +3996,13 @@
         <v>171</v>
       </c>
       <c r="S58" t="s">
-        <v>174</v>
+        <v>175</v>
       </c>
       <c r="T58" t="s">
-        <v>178</v>
+        <v>179</v>
       </c>
       <c r="U58" t="s">
-        <v>180</v>
+        <v>181</v>
       </c>
       <c r="V58" s="1">
         <v>46049</v>
@@ -4034,13 +4040,13 @@
         <v>171</v>
       </c>
       <c r="S59" t="s">
-        <v>174</v>
+        <v>175</v>
       </c>
       <c r="T59" t="s">
-        <v>178</v>
+        <v>179</v>
       </c>
       <c r="U59" t="s">
-        <v>180</v>
+        <v>181</v>
       </c>
       <c r="V59" s="1">
         <v>46139</v>
@@ -4078,13 +4084,13 @@
         <v>171</v>
       </c>
       <c r="S60" t="s">
-        <v>174</v>
+        <v>175</v>
       </c>
       <c r="T60" t="s">
-        <v>178</v>
+        <v>179</v>
       </c>
       <c r="U60" t="s">
-        <v>180</v>
+        <v>181</v>
       </c>
     </row>
     <row r="61" spans="1:22">
@@ -4119,13 +4125,13 @@
         <v>171</v>
       </c>
       <c r="S61" t="s">
-        <v>174</v>
+        <v>175</v>
       </c>
       <c r="T61" t="s">
-        <v>178</v>
+        <v>179</v>
       </c>
       <c r="U61" t="s">
-        <v>180</v>
+        <v>181</v>
       </c>
     </row>
     <row r="62" spans="1:22">
@@ -4157,16 +4163,16 @@
         <v>168</v>
       </c>
       <c r="R62" t="s">
-        <v>171</v>
+        <v>172</v>
       </c>
       <c r="S62" t="s">
-        <v>173</v>
+        <v>174</v>
       </c>
       <c r="T62" t="s">
-        <v>175</v>
+        <v>176</v>
       </c>
       <c r="U62" t="s">
-        <v>180</v>
+        <v>181</v>
       </c>
       <c r="V62" s="1">
         <v>46168</v>
@@ -4201,16 +4207,16 @@
         <v>167</v>
       </c>
       <c r="R63" t="s">
-        <v>170</v>
+        <v>172</v>
       </c>
       <c r="S63" t="s">
-        <v>173</v>
+        <v>174</v>
       </c>
       <c r="T63" t="s">
-        <v>175</v>
+        <v>176</v>
       </c>
       <c r="U63" t="s">
-        <v>180</v>
+        <v>181</v>
       </c>
       <c r="V63" s="1">
         <v>46168</v>
@@ -4245,16 +4251,16 @@
         <v>167</v>
       </c>
       <c r="R64" t="s">
-        <v>170</v>
+        <v>172</v>
       </c>
       <c r="S64" t="s">
-        <v>173</v>
+        <v>174</v>
       </c>
       <c r="T64" t="s">
-        <v>175</v>
+        <v>176</v>
       </c>
       <c r="U64" t="s">
-        <v>180</v>
+        <v>181</v>
       </c>
       <c r="V64" s="1">
         <v>46168</v>
@@ -4289,16 +4295,16 @@
         <v>169</v>
       </c>
       <c r="R65" t="s">
-        <v>170</v>
+        <v>172</v>
       </c>
       <c r="S65" t="s">
-        <v>173</v>
+        <v>174</v>
       </c>
       <c r="T65" t="s">
-        <v>175</v>
+        <v>176</v>
       </c>
       <c r="U65" t="s">
-        <v>180</v>
+        <v>181</v>
       </c>
       <c r="V65" s="1">
         <v>46168</v>
@@ -4333,16 +4339,16 @@
         <v>167</v>
       </c>
       <c r="R66" t="s">
-        <v>170</v>
+        <v>172</v>
       </c>
       <c r="S66" t="s">
-        <v>173</v>
+        <v>174</v>
       </c>
       <c r="T66" t="s">
-        <v>175</v>
+        <v>176</v>
       </c>
       <c r="U66" t="s">
-        <v>180</v>
+        <v>181</v>
       </c>
       <c r="V66" s="1">
         <v>46168</v>
@@ -4377,16 +4383,16 @@
         <v>167</v>
       </c>
       <c r="R67" t="s">
-        <v>170</v>
+        <v>172</v>
       </c>
       <c r="S67" t="s">
-        <v>173</v>
+        <v>174</v>
       </c>
       <c r="T67" t="s">
-        <v>175</v>
+        <v>176</v>
       </c>
       <c r="U67" t="s">
-        <v>180</v>
+        <v>181</v>
       </c>
       <c r="V67" s="1">
         <v>46168</v>
@@ -4421,13 +4427,13 @@
         <v>167</v>
       </c>
       <c r="R68" t="s">
-        <v>170</v>
+        <v>171</v>
       </c>
       <c r="S68" t="s">
-        <v>173</v>
+        <v>174</v>
       </c>
       <c r="T68" t="s">
-        <v>175</v>
+        <v>176</v>
       </c>
       <c r="U68" t="s">
         <v>28</v>
@@ -4471,10 +4477,10 @@
         <v>170</v>
       </c>
       <c r="S69" t="s">
-        <v>172</v>
+        <v>173</v>
       </c>
       <c r="T69" t="s">
-        <v>175</v>
+        <v>176</v>
       </c>
       <c r="U69" t="s">
         <v>28</v>
@@ -4503,10 +4509,10 @@
         <v>30</v>
       </c>
       <c r="J70" t="s">
-        <v>64</v>
+        <v>65</v>
       </c>
       <c r="K70" t="s">
-        <v>73</v>
+        <v>45</v>
       </c>
       <c r="N70" t="s">
         <v>84</v>
@@ -4524,13 +4530,13 @@
         <v>170</v>
       </c>
       <c r="S70" t="s">
-        <v>172</v>
+        <v>173</v>
       </c>
       <c r="T70" t="s">
-        <v>175</v>
+        <v>176</v>
       </c>
       <c r="U70" t="s">
-        <v>180</v>
+        <v>181</v>
       </c>
       <c r="V70" s="1">
         <v>46291</v>
@@ -4565,13 +4571,13 @@
         <v>167</v>
       </c>
       <c r="R71" t="s">
-        <v>170</v>
+        <v>171</v>
       </c>
       <c r="S71" t="s">
-        <v>173</v>
+        <v>174</v>
       </c>
       <c r="T71" t="s">
-        <v>175</v>
+        <v>176</v>
       </c>
       <c r="U71" t="s">
         <v>28</v>
@@ -4612,13 +4618,13 @@
         <v>170</v>
       </c>
       <c r="S72" t="s">
-        <v>173</v>
+        <v>174</v>
       </c>
       <c r="T72" t="s">
-        <v>175</v>
+        <v>176</v>
       </c>
       <c r="U72" t="s">
-        <v>180</v>
+        <v>181</v>
       </c>
       <c r="V72" s="1">
         <v>46352</v>
@@ -4656,13 +4662,13 @@
         <v>170</v>
       </c>
       <c r="S73" t="s">
-        <v>173</v>
+        <v>174</v>
       </c>
       <c r="T73" t="s">
-        <v>175</v>
+        <v>176</v>
       </c>
       <c r="U73" t="s">
-        <v>180</v>
+        <v>181</v>
       </c>
       <c r="V73" s="1">
         <v>46229</v>
@@ -4700,13 +4706,13 @@
         <v>170</v>
       </c>
       <c r="S74" t="s">
-        <v>173</v>
+        <v>174</v>
       </c>
       <c r="T74" t="s">
-        <v>175</v>
+        <v>176</v>
       </c>
       <c r="U74" t="s">
-        <v>180</v>
+        <v>181</v>
       </c>
       <c r="V74" s="1">
         <v>46352</v>
@@ -4744,13 +4750,13 @@
         <v>170</v>
       </c>
       <c r="S75" t="s">
-        <v>173</v>
+        <v>174</v>
       </c>
       <c r="T75" t="s">
-        <v>175</v>
+        <v>176</v>
       </c>
       <c r="U75" t="s">
-        <v>180</v>
+        <v>181</v>
       </c>
       <c r="V75" s="1">
         <v>46352</v>
@@ -4788,13 +4794,13 @@
         <v>170</v>
       </c>
       <c r="S76" t="s">
-        <v>173</v>
+        <v>174</v>
       </c>
       <c r="T76" t="s">
-        <v>175</v>
+        <v>176</v>
       </c>
       <c r="U76" t="s">
-        <v>180</v>
+        <v>181</v>
       </c>
       <c r="V76" s="1">
         <v>46352</v>
@@ -4832,13 +4838,13 @@
         <v>168</v>
       </c>
       <c r="R77" t="s">
-        <v>171</v>
+        <v>170</v>
       </c>
       <c r="S77" t="s">
-        <v>172</v>
+        <v>173</v>
       </c>
       <c r="T77" t="s">
-        <v>176</v>
+        <v>177</v>
       </c>
       <c r="U77" t="s">
         <v>28</v>
@@ -4867,7 +4873,7 @@
         <v>42</v>
       </c>
       <c r="G78" t="s">
-        <v>46</v>
+        <v>47</v>
       </c>
       <c r="N78" t="s">
         <v>85</v>
@@ -4888,10 +4894,10 @@
         <v>42</v>
       </c>
       <c r="T78" t="s">
-        <v>177</v>
+        <v>178</v>
       </c>
       <c r="U78" t="s">
-        <v>180</v>
+        <v>181</v>
       </c>
       <c r="V78" s="1">
         <v>46107</v>
@@ -4917,7 +4923,7 @@
         <v>42</v>
       </c>
       <c r="G79" t="s">
-        <v>46</v>
+        <v>47</v>
       </c>
       <c r="N79" t="s">
         <v>85</v>
@@ -4938,10 +4944,10 @@
         <v>42</v>
       </c>
       <c r="T79" t="s">
-        <v>177</v>
+        <v>178</v>
       </c>
       <c r="U79" t="s">
-        <v>180</v>
+        <v>181</v>
       </c>
       <c r="V79" s="1">
         <v>46138</v>
@@ -4967,7 +4973,7 @@
         <v>42</v>
       </c>
       <c r="G80" t="s">
-        <v>46</v>
+        <v>47</v>
       </c>
       <c r="N80" t="s">
         <v>83</v>
@@ -4988,7 +4994,7 @@
         <v>42</v>
       </c>
       <c r="T80" t="s">
-        <v>176</v>
+        <v>177</v>
       </c>
       <c r="U80" t="s">
         <v>28</v>
@@ -5017,7 +5023,7 @@
         <v>42</v>
       </c>
       <c r="G81" t="s">
-        <v>46</v>
+        <v>47</v>
       </c>
       <c r="N81" t="s">
         <v>83</v>
@@ -5038,7 +5044,7 @@
         <v>42</v>
       </c>
       <c r="T81" t="s">
-        <v>176</v>
+        <v>177</v>
       </c>
       <c r="U81" t="s">
         <v>28</v>
@@ -5064,7 +5070,7 @@
         <v>29</v>
       </c>
       <c r="J82" t="s">
-        <v>71</v>
+        <v>72</v>
       </c>
       <c r="K82" t="s">
         <v>78</v>
@@ -5085,10 +5091,10 @@
         <v>171</v>
       </c>
       <c r="S82" t="s">
-        <v>173</v>
+        <v>174</v>
       </c>
       <c r="T82" t="s">
-        <v>176</v>
+        <v>177</v>
       </c>
       <c r="U82" t="s">
         <v>28</v>
@@ -5129,10 +5135,10 @@
         <v>170</v>
       </c>
       <c r="S83" t="s">
-        <v>173</v>
+        <v>174</v>
       </c>
       <c r="T83" t="s">
-        <v>176</v>
+        <v>177</v>
       </c>
       <c r="U83" t="s">
         <v>28</v>
@@ -5161,10 +5167,10 @@
         <v>30</v>
       </c>
       <c r="J84" t="s">
-        <v>64</v>
+        <v>65</v>
       </c>
       <c r="K84" t="s">
-        <v>72</v>
+        <v>73</v>
       </c>
       <c r="N84" t="s">
         <v>85</v>
@@ -5182,13 +5188,13 @@
         <v>171</v>
       </c>
       <c r="S84" t="s">
-        <v>172</v>
+        <v>173</v>
       </c>
       <c r="T84" t="s">
-        <v>177</v>
+        <v>178</v>
       </c>
       <c r="U84" t="s">
-        <v>180</v>
+        <v>181</v>
       </c>
       <c r="V84" s="1">
         <v>46080</v>
@@ -5226,13 +5232,13 @@
         <v>168</v>
       </c>
       <c r="R85" t="s">
-        <v>171</v>
+        <v>170</v>
       </c>
       <c r="S85" t="s">
-        <v>172</v>
+        <v>173</v>
       </c>
       <c r="T85" t="s">
-        <v>176</v>
+        <v>177</v>
       </c>
       <c r="U85" t="s">
         <v>28</v>
@@ -5273,10 +5279,10 @@
         <v>170</v>
       </c>
       <c r="S86" t="s">
-        <v>173</v>
+        <v>174</v>
       </c>
       <c r="T86" t="s">
-        <v>176</v>
+        <v>177</v>
       </c>
       <c r="U86" t="s">
         <v>28</v>
@@ -5305,7 +5311,7 @@
         <v>42</v>
       </c>
       <c r="G87" t="s">
-        <v>46</v>
+        <v>47</v>
       </c>
       <c r="N87" t="s">
         <v>97</v>
@@ -5326,7 +5332,7 @@
         <v>42</v>
       </c>
       <c r="T87" t="s">
-        <v>176</v>
+        <v>177</v>
       </c>
       <c r="U87" t="s">
         <v>28</v>
@@ -5352,7 +5358,7 @@
         <v>42</v>
       </c>
       <c r="G88" t="s">
-        <v>46</v>
+        <v>47</v>
       </c>
       <c r="N88" t="s">
         <v>97</v>
@@ -5373,7 +5379,7 @@
         <v>42</v>
       </c>
       <c r="T88" t="s">
-        <v>176</v>
+        <v>177</v>
       </c>
       <c r="U88" t="s">
         <v>28</v>
@@ -5414,10 +5420,10 @@
         <v>170</v>
       </c>
       <c r="S89" t="s">
-        <v>172</v>
+        <v>173</v>
       </c>
       <c r="T89" t="s">
-        <v>179</v>
+        <v>180</v>
       </c>
       <c r="U89" t="s">
         <v>28</v>
@@ -5455,13 +5461,13 @@
         <v>168</v>
       </c>
       <c r="R90" t="s">
-        <v>171</v>
+        <v>170</v>
       </c>
       <c r="S90" t="s">
-        <v>172</v>
+        <v>173</v>
       </c>
       <c r="T90" t="s">
-        <v>176</v>
+        <v>177</v>
       </c>
       <c r="U90" t="s">
         <v>28</v>

</xml_diff>

<commit_message>
Atualização automática: mta (29/09/2026 19:54)
</commit_message>
<xml_diff>
--- a/Projetos/02_Dados_Tratados/base_mta_tratada.xlsx
+++ b/Projetos/02_Dados_Tratados/base_mta_tratada.xlsx
@@ -569,8 +569,16 @@
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="YYYY-MM-DD HH:MM:SS"/>
   </numFmts>
-  <fonts count="1">
+  <fonts count="2">
     <font>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
       <sz val="11"/>
       <color theme="1"/>
       <name val="Calibri"/>
@@ -586,7 +594,7 @@
       <patternFill patternType="gray125"/>
     </fill>
   </fills>
-  <borders count="1">
+  <borders count="2">
     <border>
       <left/>
       <right/>
@@ -594,12 +602,30 @@
       <bottom/>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin">
+        <color auto="1"/>
+      </left>
+      <right style="thin">
+        <color auto="1"/>
+      </right>
+      <top style="thin">
+        <color auto="1"/>
+      </top>
+      <bottom style="thin">
+        <color auto="1"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="3">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
   </cellXfs>
   <cellStyles count="1">
@@ -899,70 +925,70 @@
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:22">
-      <c r="A1" t="s">
+      <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
-      <c r="B1" t="s">
+      <c r="B1" s="1" t="s">
         <v>1</v>
       </c>
-      <c r="C1" t="s">
+      <c r="C1" s="1" t="s">
         <v>2</v>
       </c>
-      <c r="D1" t="s">
+      <c r="D1" s="1" t="s">
         <v>3</v>
       </c>
-      <c r="E1" t="s">
+      <c r="E1" s="1" t="s">
         <v>4</v>
       </c>
-      <c r="F1" t="s">
+      <c r="F1" s="1" t="s">
         <v>5</v>
       </c>
-      <c r="G1" t="s">
+      <c r="G1" s="1" t="s">
         <v>6</v>
       </c>
-      <c r="H1" t="s">
+      <c r="H1" s="1" t="s">
         <v>7</v>
       </c>
-      <c r="I1" t="s">
+      <c r="I1" s="1" t="s">
         <v>8</v>
       </c>
-      <c r="J1" t="s">
+      <c r="J1" s="1" t="s">
         <v>9</v>
       </c>
-      <c r="K1" t="s">
+      <c r="K1" s="1" t="s">
         <v>10</v>
       </c>
-      <c r="L1" t="s">
+      <c r="L1" s="1" t="s">
         <v>11</v>
       </c>
-      <c r="M1" t="s">
+      <c r="M1" s="1" t="s">
         <v>12</v>
       </c>
-      <c r="N1" t="s">
+      <c r="N1" s="1" t="s">
         <v>13</v>
       </c>
-      <c r="O1" t="s">
+      <c r="O1" s="1" t="s">
         <v>14</v>
       </c>
-      <c r="P1" t="s">
+      <c r="P1" s="1" t="s">
         <v>15</v>
       </c>
-      <c r="Q1" t="s">
+      <c r="Q1" s="1" t="s">
         <v>16</v>
       </c>
-      <c r="R1" t="s">
+      <c r="R1" s="1" t="s">
         <v>17</v>
       </c>
-      <c r="S1" t="s">
+      <c r="S1" s="1" t="s">
         <v>18</v>
       </c>
-      <c r="T1" t="s">
+      <c r="T1" s="1" t="s">
         <v>19</v>
       </c>
-      <c r="U1" t="s">
+      <c r="U1" s="1" t="s">
         <v>20</v>
       </c>
-      <c r="V1" t="s">
+      <c r="V1" s="1" t="s">
         <v>21</v>
       </c>
     </row>
@@ -1018,7 +1044,7 @@
       <c r="U2" t="s">
         <v>181</v>
       </c>
-      <c r="V2" s="1">
+      <c r="V2" s="2">
         <v>46291</v>
       </c>
     </row>
@@ -1065,7 +1091,7 @@
       <c r="U3" t="s">
         <v>28</v>
       </c>
-      <c r="V3" s="1">
+      <c r="V3" s="2">
         <v>46382</v>
       </c>
     </row>
@@ -1112,7 +1138,7 @@
       <c r="U4" t="s">
         <v>28</v>
       </c>
-      <c r="V4" s="1">
+      <c r="V4" s="2">
         <v>46169</v>
       </c>
     </row>
@@ -1159,7 +1185,7 @@
       <c r="U5" t="s">
         <v>28</v>
       </c>
-      <c r="V5" s="1">
+      <c r="V5" s="2">
         <v>46169</v>
       </c>
     </row>
@@ -1209,7 +1235,7 @@
       <c r="U6" t="s">
         <v>28</v>
       </c>
-      <c r="V6" s="1">
+      <c r="V6" s="2">
         <v>46352</v>
       </c>
     </row>
@@ -1235,7 +1261,7 @@
       <c r="G7" t="s">
         <v>44</v>
       </c>
-      <c r="H7" s="1">
+      <c r="H7" s="2">
         <v>46121</v>
       </c>
       <c r="I7" t="s">
@@ -1265,7 +1291,7 @@
       <c r="U7" t="s">
         <v>28</v>
       </c>
-      <c r="V7" s="1">
+      <c r="V7" s="2">
         <v>46138</v>
       </c>
     </row>
@@ -1312,7 +1338,7 @@
       <c r="U8" t="s">
         <v>28</v>
       </c>
-      <c r="V8" s="1">
+      <c r="V8" s="2">
         <v>46200</v>
       </c>
     </row>
@@ -1359,7 +1385,7 @@
       <c r="U9" t="s">
         <v>28</v>
       </c>
-      <c r="V9" s="1">
+      <c r="V9" s="2">
         <v>46200</v>
       </c>
     </row>
@@ -1406,7 +1432,7 @@
       <c r="U10" t="s">
         <v>28</v>
       </c>
-      <c r="V10" s="1">
+      <c r="V10" s="2">
         <v>46352</v>
       </c>
     </row>
@@ -1453,7 +1479,7 @@
       <c r="U11" t="s">
         <v>28</v>
       </c>
-      <c r="V11" s="1">
+      <c r="V11" s="2">
         <v>46352</v>
       </c>
     </row>
@@ -1479,7 +1505,7 @@
       <c r="G12" t="s">
         <v>44</v>
       </c>
-      <c r="H12" s="1">
+      <c r="H12" s="2">
         <v>46079</v>
       </c>
       <c r="I12" t="s">
@@ -1512,7 +1538,7 @@
       <c r="U12" t="s">
         <v>181</v>
       </c>
-      <c r="V12" s="1">
+      <c r="V12" s="2">
         <v>46168</v>
       </c>
     </row>
@@ -1565,7 +1591,7 @@
       <c r="U13" t="s">
         <v>181</v>
       </c>
-      <c r="V13" s="1">
+      <c r="V13" s="2">
         <v>46049</v>
       </c>
     </row>
@@ -1618,7 +1644,7 @@
       <c r="U14" t="s">
         <v>181</v>
       </c>
-      <c r="V14" s="1">
+      <c r="V14" s="2">
         <v>46049</v>
       </c>
     </row>
@@ -1671,7 +1697,7 @@
       <c r="U15" t="s">
         <v>181</v>
       </c>
-      <c r="V15" s="1">
+      <c r="V15" s="2">
         <v>46049</v>
       </c>
     </row>
@@ -1724,7 +1750,7 @@
       <c r="U16" t="s">
         <v>181</v>
       </c>
-      <c r="V16" s="1">
+      <c r="V16" s="2">
         <v>46291</v>
       </c>
     </row>
@@ -1750,7 +1776,7 @@
       <c r="G17" t="s">
         <v>44</v>
       </c>
-      <c r="H17" s="1">
+      <c r="H17" s="2">
         <v>46098</v>
       </c>
       <c r="I17" t="s">
@@ -1783,7 +1809,7 @@
       <c r="U17" t="s">
         <v>181</v>
       </c>
-      <c r="V17" s="1">
+      <c r="V17" s="2">
         <v>46168</v>
       </c>
     </row>
@@ -1809,7 +1835,7 @@
       <c r="G18" t="s">
         <v>44</v>
       </c>
-      <c r="H18" s="1">
+      <c r="H18" s="2">
         <v>46076</v>
       </c>
       <c r="I18" t="s">
@@ -1839,7 +1865,7 @@
       <c r="U18" t="s">
         <v>28</v>
       </c>
-      <c r="V18" s="1">
+      <c r="V18" s="2">
         <v>46260</v>
       </c>
     </row>
@@ -1865,7 +1891,7 @@
       <c r="G19" t="s">
         <v>44</v>
       </c>
-      <c r="H19" s="1">
+      <c r="H19" s="2">
         <v>46076</v>
       </c>
       <c r="I19" t="s">
@@ -1895,7 +1921,7 @@
       <c r="U19" t="s">
         <v>28</v>
       </c>
-      <c r="V19" s="1">
+      <c r="V19" s="2">
         <v>46260</v>
       </c>
     </row>
@@ -1942,7 +1968,7 @@
       <c r="U20" t="s">
         <v>28</v>
       </c>
-      <c r="V20" s="1">
+      <c r="V20" s="2">
         <v>46382</v>
       </c>
     </row>
@@ -1989,7 +2015,7 @@
       <c r="U21" t="s">
         <v>28</v>
       </c>
-      <c r="V21" s="1">
+      <c r="V21" s="2">
         <v>46382</v>
       </c>
     </row>
@@ -2036,7 +2062,7 @@
       <c r="U22" t="s">
         <v>28</v>
       </c>
-      <c r="V22" s="1">
+      <c r="V22" s="2">
         <v>46230</v>
       </c>
     </row>
@@ -2083,7 +2109,7 @@
       <c r="U23" t="s">
         <v>28</v>
       </c>
-      <c r="V23" s="1">
+      <c r="V23" s="2">
         <v>46230</v>
       </c>
     </row>
@@ -2109,7 +2135,7 @@
       <c r="G24" t="s">
         <v>44</v>
       </c>
-      <c r="H24" s="1">
+      <c r="H24" s="2">
         <v>46119</v>
       </c>
       <c r="I24" t="s">
@@ -2142,7 +2168,7 @@
       <c r="U24" t="s">
         <v>181</v>
       </c>
-      <c r="V24" s="1">
+      <c r="V24" s="2">
         <v>46199</v>
       </c>
     </row>
@@ -2168,7 +2194,7 @@
       <c r="G25" t="s">
         <v>44</v>
       </c>
-      <c r="H25" s="1">
+      <c r="H25" s="2">
         <v>46121</v>
       </c>
       <c r="I25" t="s">
@@ -2198,7 +2224,7 @@
       <c r="U25" t="s">
         <v>28</v>
       </c>
-      <c r="V25" s="1">
+      <c r="V25" s="2">
         <v>46199</v>
       </c>
     </row>
@@ -2224,7 +2250,7 @@
       <c r="G26" t="s">
         <v>44</v>
       </c>
-      <c r="H26" s="1">
+      <c r="H26" s="2">
         <v>46076</v>
       </c>
       <c r="I26" t="s">
@@ -2254,7 +2280,7 @@
       <c r="U26" t="s">
         <v>28</v>
       </c>
-      <c r="V26" s="1">
+      <c r="V26" s="2">
         <v>46352</v>
       </c>
     </row>
@@ -2307,7 +2333,7 @@
       <c r="U27" t="s">
         <v>181</v>
       </c>
-      <c r="V27" s="1">
+      <c r="V27" s="2">
         <v>46352</v>
       </c>
     </row>
@@ -2333,7 +2359,7 @@
       <c r="G28" t="s">
         <v>44</v>
       </c>
-      <c r="H28" s="1">
+      <c r="H28" s="2">
         <v>46199</v>
       </c>
       <c r="I28" t="s">
@@ -2366,7 +2392,7 @@
       <c r="U28" t="s">
         <v>181</v>
       </c>
-      <c r="V28" s="1">
+      <c r="V28" s="2">
         <v>46260</v>
       </c>
     </row>
@@ -2392,7 +2418,7 @@
       <c r="G29" t="s">
         <v>44</v>
       </c>
-      <c r="H29" s="1">
+      <c r="H29" s="2">
         <v>46199</v>
       </c>
       <c r="I29" t="s">
@@ -2425,7 +2451,7 @@
       <c r="U29" t="s">
         <v>181</v>
       </c>
-      <c r="V29" s="1">
+      <c r="V29" s="2">
         <v>46260</v>
       </c>
     </row>
@@ -2451,7 +2477,7 @@
       <c r="G30" t="s">
         <v>44</v>
       </c>
-      <c r="H30" s="1">
+      <c r="H30" s="2">
         <v>46199</v>
       </c>
       <c r="I30" t="s">
@@ -2484,7 +2510,7 @@
       <c r="U30" t="s">
         <v>181</v>
       </c>
-      <c r="V30" s="1">
+      <c r="V30" s="2">
         <v>46260</v>
       </c>
     </row>
@@ -2510,7 +2536,7 @@
       <c r="G31" t="s">
         <v>44</v>
       </c>
-      <c r="H31" s="1">
+      <c r="H31" s="2">
         <v>46199</v>
       </c>
       <c r="I31" t="s">
@@ -2543,7 +2569,7 @@
       <c r="U31" t="s">
         <v>181</v>
       </c>
-      <c r="V31" s="1">
+      <c r="V31" s="2">
         <v>46260</v>
       </c>
     </row>
@@ -2593,7 +2619,7 @@
       <c r="U32" t="s">
         <v>181</v>
       </c>
-      <c r="V32" s="1">
+      <c r="V32" s="2">
         <v>46352</v>
       </c>
     </row>
@@ -2619,7 +2645,7 @@
       <c r="G33" t="s">
         <v>44</v>
       </c>
-      <c r="H33" s="1">
+      <c r="H33" s="2">
         <v>46191</v>
       </c>
       <c r="I33" t="s">
@@ -2652,7 +2678,7 @@
       <c r="U33" t="s">
         <v>181</v>
       </c>
-      <c r="V33" s="1">
+      <c r="V33" s="2">
         <v>46260</v>
       </c>
     </row>
@@ -2678,7 +2704,7 @@
       <c r="G34" t="s">
         <v>44</v>
       </c>
-      <c r="H34" s="1">
+      <c r="H34" s="2">
         <v>46119</v>
       </c>
       <c r="I34" t="s">
@@ -2708,7 +2734,7 @@
       <c r="U34" t="s">
         <v>181</v>
       </c>
-      <c r="V34" s="1">
+      <c r="V34" s="2">
         <v>46260</v>
       </c>
     </row>
@@ -2734,7 +2760,7 @@
       <c r="G35" t="s">
         <v>44</v>
       </c>
-      <c r="H35" s="1">
+      <c r="H35" s="2">
         <v>46213</v>
       </c>
       <c r="I35" t="s">
@@ -2764,7 +2790,7 @@
       <c r="U35" t="s">
         <v>28</v>
       </c>
-      <c r="V35" s="1">
+      <c r="V35" s="2">
         <v>46352</v>
       </c>
     </row>
@@ -2790,7 +2816,7 @@
       <c r="G36" t="s">
         <v>44</v>
       </c>
-      <c r="H36" s="1">
+      <c r="H36" s="2">
         <v>46175</v>
       </c>
       <c r="I36" t="s">
@@ -2820,7 +2846,7 @@
       <c r="U36" t="s">
         <v>28</v>
       </c>
-      <c r="V36" s="1">
+      <c r="V36" s="2">
         <v>46260</v>
       </c>
     </row>
@@ -2846,7 +2872,7 @@
       <c r="G37" t="s">
         <v>44</v>
       </c>
-      <c r="H37" s="1">
+      <c r="H37" s="2">
         <v>46213</v>
       </c>
       <c r="I37" t="s">
@@ -2876,7 +2902,7 @@
       <c r="U37" t="s">
         <v>28</v>
       </c>
-      <c r="V37" s="1">
+      <c r="V37" s="2">
         <v>46352</v>
       </c>
     </row>
@@ -2902,7 +2928,7 @@
       <c r="G38" t="s">
         <v>44</v>
       </c>
-      <c r="H38" s="1">
+      <c r="H38" s="2">
         <v>46199</v>
       </c>
       <c r="I38" t="s">
@@ -2932,7 +2958,7 @@
       <c r="U38" t="s">
         <v>28</v>
       </c>
-      <c r="V38" s="1">
+      <c r="V38" s="2">
         <v>46229</v>
       </c>
     </row>
@@ -2958,7 +2984,7 @@
       <c r="G39" t="s">
         <v>44</v>
       </c>
-      <c r="H39" s="1">
+      <c r="H39" s="2">
         <v>46199</v>
       </c>
       <c r="I39" t="s">
@@ -2988,7 +3014,7 @@
       <c r="U39" t="s">
         <v>28</v>
       </c>
-      <c r="V39" s="1">
+      <c r="V39" s="2">
         <v>46229</v>
       </c>
     </row>
@@ -3014,7 +3040,7 @@
       <c r="G40" t="s">
         <v>44</v>
       </c>
-      <c r="H40" s="1">
+      <c r="H40" s="2">
         <v>46204</v>
       </c>
       <c r="I40" t="s">
@@ -3044,7 +3070,7 @@
       <c r="U40" t="s">
         <v>28</v>
       </c>
-      <c r="V40" s="1">
+      <c r="V40" s="2">
         <v>46229</v>
       </c>
     </row>
@@ -3070,7 +3096,7 @@
       <c r="G41" t="s">
         <v>44</v>
       </c>
-      <c r="H41" s="1">
+      <c r="H41" s="2">
         <v>46244</v>
       </c>
       <c r="I41" t="s">
@@ -3100,7 +3126,7 @@
       <c r="U41" t="s">
         <v>28</v>
       </c>
-      <c r="V41" s="1">
+      <c r="V41" s="2">
         <v>46260</v>
       </c>
     </row>
@@ -3144,7 +3170,7 @@
       <c r="U42" t="s">
         <v>28</v>
       </c>
-      <c r="V42" s="1">
+      <c r="V42" s="2">
         <v>46352</v>
       </c>
     </row>
@@ -3170,7 +3196,7 @@
       <c r="G43" t="s">
         <v>44</v>
       </c>
-      <c r="H43" s="1">
+      <c r="H43" s="2">
         <v>46191</v>
       </c>
       <c r="I43" t="s">
@@ -3200,7 +3226,7 @@
       <c r="U43" t="s">
         <v>28</v>
       </c>
-      <c r="V43" s="1">
+      <c r="V43" s="2">
         <v>46229</v>
       </c>
     </row>
@@ -3226,7 +3252,7 @@
       <c r="G44" t="s">
         <v>44</v>
       </c>
-      <c r="H44" s="1">
+      <c r="H44" s="2">
         <v>46191</v>
       </c>
       <c r="I44" t="s">
@@ -3256,7 +3282,7 @@
       <c r="U44" t="s">
         <v>28</v>
       </c>
-      <c r="V44" s="1">
+      <c r="V44" s="2">
         <v>46229</v>
       </c>
     </row>
@@ -3282,7 +3308,7 @@
       <c r="G45" t="s">
         <v>44</v>
       </c>
-      <c r="H45" s="1">
+      <c r="H45" s="2">
         <v>46213</v>
       </c>
       <c r="I45" t="s">
@@ -3315,7 +3341,7 @@
       <c r="U45" t="s">
         <v>181</v>
       </c>
-      <c r="V45" s="1">
+      <c r="V45" s="2">
         <v>46291</v>
       </c>
     </row>
@@ -3341,7 +3367,7 @@
       <c r="G46" t="s">
         <v>44</v>
       </c>
-      <c r="H46" s="1">
+      <c r="H46" s="2">
         <v>46210</v>
       </c>
       <c r="I46" t="s">
@@ -3371,7 +3397,7 @@
       <c r="U46" t="s">
         <v>181</v>
       </c>
-      <c r="V46" s="1">
+      <c r="V46" s="2">
         <v>46291</v>
       </c>
     </row>
@@ -3418,7 +3444,7 @@
       <c r="U47" t="s">
         <v>28</v>
       </c>
-      <c r="V47" s="1">
+      <c r="V47" s="2">
         <v>46321</v>
       </c>
     </row>
@@ -3471,7 +3497,7 @@
       <c r="U48" t="s">
         <v>181</v>
       </c>
-      <c r="V48" s="1">
+      <c r="V48" s="2">
         <v>46352</v>
       </c>
     </row>
@@ -3497,7 +3523,7 @@
       <c r="G49" t="s">
         <v>44</v>
       </c>
-      <c r="H49" s="1">
+      <c r="H49" s="2">
         <v>46176</v>
       </c>
       <c r="I49" t="s">
@@ -3530,7 +3556,7 @@
       <c r="U49" t="s">
         <v>181</v>
       </c>
-      <c r="V49" s="1">
+      <c r="V49" s="2">
         <v>46352</v>
       </c>
     </row>
@@ -3583,7 +3609,7 @@
       <c r="U50" t="s">
         <v>181</v>
       </c>
-      <c r="V50" s="1">
+      <c r="V50" s="2">
         <v>46321</v>
       </c>
     </row>
@@ -3639,7 +3665,7 @@
       <c r="U51" t="s">
         <v>181</v>
       </c>
-      <c r="V51" s="1">
+      <c r="V51" s="2">
         <v>46352</v>
       </c>
     </row>
@@ -3689,7 +3715,7 @@
       <c r="U52" t="s">
         <v>181</v>
       </c>
-      <c r="V52" s="1">
+      <c r="V52" s="2">
         <v>46382</v>
       </c>
     </row>
@@ -3715,7 +3741,7 @@
       <c r="G53" t="s">
         <v>44</v>
       </c>
-      <c r="H53" s="1">
+      <c r="H53" s="2">
         <v>46227</v>
       </c>
       <c r="I53" t="s">
@@ -3745,7 +3771,7 @@
       <c r="U53" t="s">
         <v>181</v>
       </c>
-      <c r="V53" s="1">
+      <c r="V53" s="2">
         <v>46321</v>
       </c>
     </row>
@@ -3768,7 +3794,7 @@
       <c r="G54" t="s">
         <v>44</v>
       </c>
-      <c r="H54" s="1">
+      <c r="H54" s="2">
         <v>46280</v>
       </c>
       <c r="I54" t="s">
@@ -3798,7 +3824,7 @@
       <c r="U54" t="s">
         <v>181</v>
       </c>
-      <c r="V54" s="1">
+      <c r="V54" s="2">
         <v>46352</v>
       </c>
     </row>
@@ -3821,7 +3847,7 @@
       <c r="G55" t="s">
         <v>44</v>
       </c>
-      <c r="H55" s="1">
+      <c r="H55" s="2">
         <v>46280</v>
       </c>
       <c r="I55" t="s">
@@ -3851,7 +3877,7 @@
       <c r="U55" t="s">
         <v>181</v>
       </c>
-      <c r="V55" s="1">
+      <c r="V55" s="2">
         <v>46321</v>
       </c>
     </row>
@@ -3904,7 +3930,7 @@
       <c r="U56" t="s">
         <v>181</v>
       </c>
-      <c r="V56" s="1">
+      <c r="V56" s="2">
         <v>46049</v>
       </c>
     </row>
@@ -3957,7 +3983,7 @@
       <c r="U57" t="s">
         <v>181</v>
       </c>
-      <c r="V57" s="1">
+      <c r="V57" s="2">
         <v>46049</v>
       </c>
     </row>
@@ -4004,7 +4030,7 @@
       <c r="U58" t="s">
         <v>181</v>
       </c>
-      <c r="V58" s="1">
+      <c r="V58" s="2">
         <v>46049</v>
       </c>
     </row>
@@ -4048,7 +4074,7 @@
       <c r="U59" t="s">
         <v>181</v>
       </c>
-      <c r="V59" s="1">
+      <c r="V59" s="2">
         <v>46139</v>
       </c>
     </row>
@@ -4174,7 +4200,7 @@
       <c r="U62" t="s">
         <v>181</v>
       </c>
-      <c r="V62" s="1">
+      <c r="V62" s="2">
         <v>46168</v>
       </c>
     </row>
@@ -4218,7 +4244,7 @@
       <c r="U63" t="s">
         <v>181</v>
       </c>
-      <c r="V63" s="1">
+      <c r="V63" s="2">
         <v>46168</v>
       </c>
     </row>
@@ -4262,7 +4288,7 @@
       <c r="U64" t="s">
         <v>181</v>
       </c>
-      <c r="V64" s="1">
+      <c r="V64" s="2">
         <v>46168</v>
       </c>
     </row>
@@ -4306,7 +4332,7 @@
       <c r="U65" t="s">
         <v>181</v>
       </c>
-      <c r="V65" s="1">
+      <c r="V65" s="2">
         <v>46168</v>
       </c>
     </row>
@@ -4350,7 +4376,7 @@
       <c r="U66" t="s">
         <v>181</v>
       </c>
-      <c r="V66" s="1">
+      <c r="V66" s="2">
         <v>46168</v>
       </c>
     </row>
@@ -4394,7 +4420,7 @@
       <c r="U67" t="s">
         <v>181</v>
       </c>
-      <c r="V67" s="1">
+      <c r="V67" s="2">
         <v>46168</v>
       </c>
     </row>
@@ -4438,7 +4464,7 @@
       <c r="U68" t="s">
         <v>28</v>
       </c>
-      <c r="V68" s="1">
+      <c r="V68" s="2">
         <v>46168</v>
       </c>
     </row>
@@ -4485,7 +4511,7 @@
       <c r="U69" t="s">
         <v>28</v>
       </c>
-      <c r="V69" s="1">
+      <c r="V69" s="2">
         <v>46382</v>
       </c>
     </row>
@@ -4538,7 +4564,7 @@
       <c r="U70" t="s">
         <v>181</v>
       </c>
-      <c r="V70" s="1">
+      <c r="V70" s="2">
         <v>46291</v>
       </c>
     </row>
@@ -4582,7 +4608,7 @@
       <c r="U71" t="s">
         <v>28</v>
       </c>
-      <c r="V71" s="1">
+      <c r="V71" s="2">
         <v>46260</v>
       </c>
     </row>
@@ -4626,7 +4652,7 @@
       <c r="U72" t="s">
         <v>181</v>
       </c>
-      <c r="V72" s="1">
+      <c r="V72" s="2">
         <v>46352</v>
       </c>
     </row>
@@ -4670,7 +4696,7 @@
       <c r="U73" t="s">
         <v>181</v>
       </c>
-      <c r="V73" s="1">
+      <c r="V73" s="2">
         <v>46229</v>
       </c>
     </row>
@@ -4714,7 +4740,7 @@
       <c r="U74" t="s">
         <v>181</v>
       </c>
-      <c r="V74" s="1">
+      <c r="V74" s="2">
         <v>46352</v>
       </c>
     </row>
@@ -4758,7 +4784,7 @@
       <c r="U75" t="s">
         <v>181</v>
       </c>
-      <c r="V75" s="1">
+      <c r="V75" s="2">
         <v>46352</v>
       </c>
     </row>
@@ -4802,7 +4828,7 @@
       <c r="U76" t="s">
         <v>181</v>
       </c>
-      <c r="V76" s="1">
+      <c r="V76" s="2">
         <v>46352</v>
       </c>
     </row>
@@ -4849,7 +4875,7 @@
       <c r="U77" t="s">
         <v>28</v>
       </c>
-      <c r="V77" s="1">
+      <c r="V77" s="2">
         <v>46382</v>
       </c>
     </row>
@@ -4899,7 +4925,7 @@
       <c r="U78" t="s">
         <v>181</v>
       </c>
-      <c r="V78" s="1">
+      <c r="V78" s="2">
         <v>46107</v>
       </c>
     </row>
@@ -4949,7 +4975,7 @@
       <c r="U79" t="s">
         <v>181</v>
       </c>
-      <c r="V79" s="1">
+      <c r="V79" s="2">
         <v>46138</v>
       </c>
     </row>
@@ -4999,7 +5025,7 @@
       <c r="U80" t="s">
         <v>28</v>
       </c>
-      <c r="V80" s="1">
+      <c r="V80" s="2">
         <v>46260</v>
       </c>
     </row>
@@ -5049,7 +5075,7 @@
       <c r="U81" t="s">
         <v>28</v>
       </c>
-      <c r="V81" s="1">
+      <c r="V81" s="2">
         <v>46260</v>
       </c>
     </row>
@@ -5099,7 +5125,7 @@
       <c r="U82" t="s">
         <v>28</v>
       </c>
-      <c r="V82" s="1">
+      <c r="V82" s="2">
         <v>46108</v>
       </c>
     </row>
@@ -5143,7 +5169,7 @@
       <c r="U83" t="s">
         <v>28</v>
       </c>
-      <c r="V83" s="1">
+      <c r="V83" s="2">
         <v>46108</v>
       </c>
     </row>
@@ -5196,7 +5222,7 @@
       <c r="U84" t="s">
         <v>181</v>
       </c>
-      <c r="V84" s="1">
+      <c r="V84" s="2">
         <v>46080</v>
       </c>
     </row>
@@ -5243,7 +5269,7 @@
       <c r="U85" t="s">
         <v>28</v>
       </c>
-      <c r="V85" s="1">
+      <c r="V85" s="2">
         <v>46382</v>
       </c>
     </row>
@@ -5287,7 +5313,7 @@
       <c r="U86" t="s">
         <v>28</v>
       </c>
-      <c r="V86" s="1">
+      <c r="V86" s="2">
         <v>46108</v>
       </c>
     </row>
@@ -5428,7 +5454,7 @@
       <c r="U89" t="s">
         <v>28</v>
       </c>
-      <c r="V89" s="1">
+      <c r="V89" s="2">
         <v>46321</v>
       </c>
     </row>
@@ -5472,7 +5498,7 @@
       <c r="U90" t="s">
         <v>28</v>
       </c>
-      <c r="V90" s="1">
+      <c r="V90" s="2">
         <v>46382</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Atualização automática: mta (30/09/2026 13:48)
</commit_message>
<xml_diff>
--- a/Projetos/02_Dados_Tratados/base_mta_tratada.xlsx
+++ b/Projetos/02_Dados_Tratados/base_mta_tratada.xlsx
@@ -569,16 +569,8 @@
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="YYYY-MM-DD HH:MM:SS"/>
   </numFmts>
-  <fonts count="2">
+  <fonts count="1">
     <font>
-      <sz val="11"/>
-      <color theme="1"/>
-      <name val="Calibri"/>
-      <family val="2"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <b/>
       <sz val="11"/>
       <color theme="1"/>
       <name val="Calibri"/>
@@ -594,7 +586,7 @@
       <patternFill patternType="gray125"/>
     </fill>
   </fills>
-  <borders count="2">
+  <borders count="1">
     <border>
       <left/>
       <right/>
@@ -602,30 +594,12 @@
       <bottom/>
       <diagonal/>
     </border>
-    <border>
-      <left style="thin">
-        <color auto="1"/>
-      </left>
-      <right style="thin">
-        <color auto="1"/>
-      </right>
-      <top style="thin">
-        <color auto="1"/>
-      </top>
-      <bottom style="thin">
-        <color auto="1"/>
-      </bottom>
-      <diagonal/>
-    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="3">
+  <cellXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top"/>
-    </xf>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
   </cellXfs>
   <cellStyles count="1">
@@ -925,70 +899,70 @@
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:22">
-      <c r="A1" s="1" t="s">
+      <c r="A1" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="1" t="s">
+      <c r="B1" t="s">
         <v>1</v>
       </c>
-      <c r="C1" s="1" t="s">
+      <c r="C1" t="s">
         <v>2</v>
       </c>
-      <c r="D1" s="1" t="s">
+      <c r="D1" t="s">
         <v>3</v>
       </c>
-      <c r="E1" s="1" t="s">
+      <c r="E1" t="s">
         <v>4</v>
       </c>
-      <c r="F1" s="1" t="s">
+      <c r="F1" t="s">
         <v>5</v>
       </c>
-      <c r="G1" s="1" t="s">
+      <c r="G1" t="s">
         <v>6</v>
       </c>
-      <c r="H1" s="1" t="s">
+      <c r="H1" t="s">
         <v>7</v>
       </c>
-      <c r="I1" s="1" t="s">
+      <c r="I1" t="s">
         <v>8</v>
       </c>
-      <c r="J1" s="1" t="s">
+      <c r="J1" t="s">
         <v>9</v>
       </c>
-      <c r="K1" s="1" t="s">
+      <c r="K1" t="s">
         <v>10</v>
       </c>
-      <c r="L1" s="1" t="s">
+      <c r="L1" t="s">
         <v>11</v>
       </c>
-      <c r="M1" s="1" t="s">
+      <c r="M1" t="s">
         <v>12</v>
       </c>
-      <c r="N1" s="1" t="s">
+      <c r="N1" t="s">
         <v>13</v>
       </c>
-      <c r="O1" s="1" t="s">
+      <c r="O1" t="s">
         <v>14</v>
       </c>
-      <c r="P1" s="1" t="s">
+      <c r="P1" t="s">
         <v>15</v>
       </c>
-      <c r="Q1" s="1" t="s">
+      <c r="Q1" t="s">
         <v>16</v>
       </c>
-      <c r="R1" s="1" t="s">
+      <c r="R1" t="s">
         <v>17</v>
       </c>
-      <c r="S1" s="1" t="s">
+      <c r="S1" t="s">
         <v>18</v>
       </c>
-      <c r="T1" s="1" t="s">
+      <c r="T1" t="s">
         <v>19</v>
       </c>
-      <c r="U1" s="1" t="s">
+      <c r="U1" t="s">
         <v>20</v>
       </c>
-      <c r="V1" s="1" t="s">
+      <c r="V1" t="s">
         <v>21</v>
       </c>
     </row>
@@ -1044,7 +1018,7 @@
       <c r="U2" t="s">
         <v>181</v>
       </c>
-      <c r="V2" s="2">
+      <c r="V2" s="1">
         <v>46291</v>
       </c>
     </row>
@@ -1091,7 +1065,7 @@
       <c r="U3" t="s">
         <v>28</v>
       </c>
-      <c r="V3" s="2">
+      <c r="V3" s="1">
         <v>46382</v>
       </c>
     </row>
@@ -1138,7 +1112,7 @@
       <c r="U4" t="s">
         <v>28</v>
       </c>
-      <c r="V4" s="2">
+      <c r="V4" s="1">
         <v>46169</v>
       </c>
     </row>
@@ -1185,7 +1159,7 @@
       <c r="U5" t="s">
         <v>28</v>
       </c>
-      <c r="V5" s="2">
+      <c r="V5" s="1">
         <v>46169</v>
       </c>
     </row>
@@ -1235,7 +1209,7 @@
       <c r="U6" t="s">
         <v>28</v>
       </c>
-      <c r="V6" s="2">
+      <c r="V6" s="1">
         <v>46352</v>
       </c>
     </row>
@@ -1261,7 +1235,7 @@
       <c r="G7" t="s">
         <v>44</v>
       </c>
-      <c r="H7" s="2">
+      <c r="H7" s="1">
         <v>46121</v>
       </c>
       <c r="I7" t="s">
@@ -1291,7 +1265,7 @@
       <c r="U7" t="s">
         <v>28</v>
       </c>
-      <c r="V7" s="2">
+      <c r="V7" s="1">
         <v>46138</v>
       </c>
     </row>
@@ -1338,7 +1312,7 @@
       <c r="U8" t="s">
         <v>28</v>
       </c>
-      <c r="V8" s="2">
+      <c r="V8" s="1">
         <v>46200</v>
       </c>
     </row>
@@ -1385,7 +1359,7 @@
       <c r="U9" t="s">
         <v>28</v>
       </c>
-      <c r="V9" s="2">
+      <c r="V9" s="1">
         <v>46200</v>
       </c>
     </row>
@@ -1432,7 +1406,7 @@
       <c r="U10" t="s">
         <v>28</v>
       </c>
-      <c r="V10" s="2">
+      <c r="V10" s="1">
         <v>46352</v>
       </c>
     </row>
@@ -1479,7 +1453,7 @@
       <c r="U11" t="s">
         <v>28</v>
       </c>
-      <c r="V11" s="2">
+      <c r="V11" s="1">
         <v>46352</v>
       </c>
     </row>
@@ -1505,7 +1479,7 @@
       <c r="G12" t="s">
         <v>44</v>
       </c>
-      <c r="H12" s="2">
+      <c r="H12" s="1">
         <v>46079</v>
       </c>
       <c r="I12" t="s">
@@ -1538,7 +1512,7 @@
       <c r="U12" t="s">
         <v>181</v>
       </c>
-      <c r="V12" s="2">
+      <c r="V12" s="1">
         <v>46168</v>
       </c>
     </row>
@@ -1591,7 +1565,7 @@
       <c r="U13" t="s">
         <v>181</v>
       </c>
-      <c r="V13" s="2">
+      <c r="V13" s="1">
         <v>46049</v>
       </c>
     </row>
@@ -1644,7 +1618,7 @@
       <c r="U14" t="s">
         <v>181</v>
       </c>
-      <c r="V14" s="2">
+      <c r="V14" s="1">
         <v>46049</v>
       </c>
     </row>
@@ -1697,7 +1671,7 @@
       <c r="U15" t="s">
         <v>181</v>
       </c>
-      <c r="V15" s="2">
+      <c r="V15" s="1">
         <v>46049</v>
       </c>
     </row>
@@ -1750,7 +1724,7 @@
       <c r="U16" t="s">
         <v>181</v>
       </c>
-      <c r="V16" s="2">
+      <c r="V16" s="1">
         <v>46291</v>
       </c>
     </row>
@@ -1776,7 +1750,7 @@
       <c r="G17" t="s">
         <v>44</v>
       </c>
-      <c r="H17" s="2">
+      <c r="H17" s="1">
         <v>46098</v>
       </c>
       <c r="I17" t="s">
@@ -1809,7 +1783,7 @@
       <c r="U17" t="s">
         <v>181</v>
       </c>
-      <c r="V17" s="2">
+      <c r="V17" s="1">
         <v>46168</v>
       </c>
     </row>
@@ -1835,7 +1809,7 @@
       <c r="G18" t="s">
         <v>44</v>
       </c>
-      <c r="H18" s="2">
+      <c r="H18" s="1">
         <v>46076</v>
       </c>
       <c r="I18" t="s">
@@ -1865,7 +1839,7 @@
       <c r="U18" t="s">
         <v>28</v>
       </c>
-      <c r="V18" s="2">
+      <c r="V18" s="1">
         <v>46260</v>
       </c>
     </row>
@@ -1891,7 +1865,7 @@
       <c r="G19" t="s">
         <v>44</v>
       </c>
-      <c r="H19" s="2">
+      <c r="H19" s="1">
         <v>46076</v>
       </c>
       <c r="I19" t="s">
@@ -1921,7 +1895,7 @@
       <c r="U19" t="s">
         <v>28</v>
       </c>
-      <c r="V19" s="2">
+      <c r="V19" s="1">
         <v>46260</v>
       </c>
     </row>
@@ -1968,7 +1942,7 @@
       <c r="U20" t="s">
         <v>28</v>
       </c>
-      <c r="V20" s="2">
+      <c r="V20" s="1">
         <v>46382</v>
       </c>
     </row>
@@ -2015,7 +1989,7 @@
       <c r="U21" t="s">
         <v>28</v>
       </c>
-      <c r="V21" s="2">
+      <c r="V21" s="1">
         <v>46382</v>
       </c>
     </row>
@@ -2062,7 +2036,7 @@
       <c r="U22" t="s">
         <v>28</v>
       </c>
-      <c r="V22" s="2">
+      <c r="V22" s="1">
         <v>46230</v>
       </c>
     </row>
@@ -2109,7 +2083,7 @@
       <c r="U23" t="s">
         <v>28</v>
       </c>
-      <c r="V23" s="2">
+      <c r="V23" s="1">
         <v>46230</v>
       </c>
     </row>
@@ -2135,7 +2109,7 @@
       <c r="G24" t="s">
         <v>44</v>
       </c>
-      <c r="H24" s="2">
+      <c r="H24" s="1">
         <v>46119</v>
       </c>
       <c r="I24" t="s">
@@ -2168,7 +2142,7 @@
       <c r="U24" t="s">
         <v>181</v>
       </c>
-      <c r="V24" s="2">
+      <c r="V24" s="1">
         <v>46199</v>
       </c>
     </row>
@@ -2194,7 +2168,7 @@
       <c r="G25" t="s">
         <v>44</v>
       </c>
-      <c r="H25" s="2">
+      <c r="H25" s="1">
         <v>46121</v>
       </c>
       <c r="I25" t="s">
@@ -2224,7 +2198,7 @@
       <c r="U25" t="s">
         <v>28</v>
       </c>
-      <c r="V25" s="2">
+      <c r="V25" s="1">
         <v>46199</v>
       </c>
     </row>
@@ -2250,7 +2224,7 @@
       <c r="G26" t="s">
         <v>44</v>
       </c>
-      <c r="H26" s="2">
+      <c r="H26" s="1">
         <v>46076</v>
       </c>
       <c r="I26" t="s">
@@ -2280,7 +2254,7 @@
       <c r="U26" t="s">
         <v>28</v>
       </c>
-      <c r="V26" s="2">
+      <c r="V26" s="1">
         <v>46352</v>
       </c>
     </row>
@@ -2333,7 +2307,7 @@
       <c r="U27" t="s">
         <v>181</v>
       </c>
-      <c r="V27" s="2">
+      <c r="V27" s="1">
         <v>46352</v>
       </c>
     </row>
@@ -2359,7 +2333,7 @@
       <c r="G28" t="s">
         <v>44</v>
       </c>
-      <c r="H28" s="2">
+      <c r="H28" s="1">
         <v>46199</v>
       </c>
       <c r="I28" t="s">
@@ -2392,7 +2366,7 @@
       <c r="U28" t="s">
         <v>181</v>
       </c>
-      <c r="V28" s="2">
+      <c r="V28" s="1">
         <v>46260</v>
       </c>
     </row>
@@ -2418,7 +2392,7 @@
       <c r="G29" t="s">
         <v>44</v>
       </c>
-      <c r="H29" s="2">
+      <c r="H29" s="1">
         <v>46199</v>
       </c>
       <c r="I29" t="s">
@@ -2451,7 +2425,7 @@
       <c r="U29" t="s">
         <v>181</v>
       </c>
-      <c r="V29" s="2">
+      <c r="V29" s="1">
         <v>46260</v>
       </c>
     </row>
@@ -2477,7 +2451,7 @@
       <c r="G30" t="s">
         <v>44</v>
       </c>
-      <c r="H30" s="2">
+      <c r="H30" s="1">
         <v>46199</v>
       </c>
       <c r="I30" t="s">
@@ -2510,7 +2484,7 @@
       <c r="U30" t="s">
         <v>181</v>
       </c>
-      <c r="V30" s="2">
+      <c r="V30" s="1">
         <v>46260</v>
       </c>
     </row>
@@ -2536,7 +2510,7 @@
       <c r="G31" t="s">
         <v>44</v>
       </c>
-      <c r="H31" s="2">
+      <c r="H31" s="1">
         <v>46199</v>
       </c>
       <c r="I31" t="s">
@@ -2569,7 +2543,7 @@
       <c r="U31" t="s">
         <v>181</v>
       </c>
-      <c r="V31" s="2">
+      <c r="V31" s="1">
         <v>46260</v>
       </c>
     </row>
@@ -2619,7 +2593,7 @@
       <c r="U32" t="s">
         <v>181</v>
       </c>
-      <c r="V32" s="2">
+      <c r="V32" s="1">
         <v>46352</v>
       </c>
     </row>
@@ -2645,7 +2619,7 @@
       <c r="G33" t="s">
         <v>44</v>
       </c>
-      <c r="H33" s="2">
+      <c r="H33" s="1">
         <v>46191</v>
       </c>
       <c r="I33" t="s">
@@ -2678,7 +2652,7 @@
       <c r="U33" t="s">
         <v>181</v>
       </c>
-      <c r="V33" s="2">
+      <c r="V33" s="1">
         <v>46260</v>
       </c>
     </row>
@@ -2704,7 +2678,7 @@
       <c r="G34" t="s">
         <v>44</v>
       </c>
-      <c r="H34" s="2">
+      <c r="H34" s="1">
         <v>46119</v>
       </c>
       <c r="I34" t="s">
@@ -2734,7 +2708,7 @@
       <c r="U34" t="s">
         <v>181</v>
       </c>
-      <c r="V34" s="2">
+      <c r="V34" s="1">
         <v>46260</v>
       </c>
     </row>
@@ -2760,7 +2734,7 @@
       <c r="G35" t="s">
         <v>44</v>
       </c>
-      <c r="H35" s="2">
+      <c r="H35" s="1">
         <v>46213</v>
       </c>
       <c r="I35" t="s">
@@ -2790,7 +2764,7 @@
       <c r="U35" t="s">
         <v>28</v>
       </c>
-      <c r="V35" s="2">
+      <c r="V35" s="1">
         <v>46352</v>
       </c>
     </row>
@@ -2816,7 +2790,7 @@
       <c r="G36" t="s">
         <v>44</v>
       </c>
-      <c r="H36" s="2">
+      <c r="H36" s="1">
         <v>46175</v>
       </c>
       <c r="I36" t="s">
@@ -2846,7 +2820,7 @@
       <c r="U36" t="s">
         <v>28</v>
       </c>
-      <c r="V36" s="2">
+      <c r="V36" s="1">
         <v>46260</v>
       </c>
     </row>
@@ -2872,7 +2846,7 @@
       <c r="G37" t="s">
         <v>44</v>
       </c>
-      <c r="H37" s="2">
+      <c r="H37" s="1">
         <v>46213</v>
       </c>
       <c r="I37" t="s">
@@ -2902,7 +2876,7 @@
       <c r="U37" t="s">
         <v>28</v>
       </c>
-      <c r="V37" s="2">
+      <c r="V37" s="1">
         <v>46352</v>
       </c>
     </row>
@@ -2928,7 +2902,7 @@
       <c r="G38" t="s">
         <v>44</v>
       </c>
-      <c r="H38" s="2">
+      <c r="H38" s="1">
         <v>46199</v>
       </c>
       <c r="I38" t="s">
@@ -2958,7 +2932,7 @@
       <c r="U38" t="s">
         <v>28</v>
       </c>
-      <c r="V38" s="2">
+      <c r="V38" s="1">
         <v>46229</v>
       </c>
     </row>
@@ -2984,7 +2958,7 @@
       <c r="G39" t="s">
         <v>44</v>
       </c>
-      <c r="H39" s="2">
+      <c r="H39" s="1">
         <v>46199</v>
       </c>
       <c r="I39" t="s">
@@ -3014,7 +2988,7 @@
       <c r="U39" t="s">
         <v>28</v>
       </c>
-      <c r="V39" s="2">
+      <c r="V39" s="1">
         <v>46229</v>
       </c>
     </row>
@@ -3040,7 +3014,7 @@
       <c r="G40" t="s">
         <v>44</v>
       </c>
-      <c r="H40" s="2">
+      <c r="H40" s="1">
         <v>46204</v>
       </c>
       <c r="I40" t="s">
@@ -3070,7 +3044,7 @@
       <c r="U40" t="s">
         <v>28</v>
       </c>
-      <c r="V40" s="2">
+      <c r="V40" s="1">
         <v>46229</v>
       </c>
     </row>
@@ -3096,7 +3070,7 @@
       <c r="G41" t="s">
         <v>44</v>
       </c>
-      <c r="H41" s="2">
+      <c r="H41" s="1">
         <v>46244</v>
       </c>
       <c r="I41" t="s">
@@ -3126,7 +3100,7 @@
       <c r="U41" t="s">
         <v>28</v>
       </c>
-      <c r="V41" s="2">
+      <c r="V41" s="1">
         <v>46260</v>
       </c>
     </row>
@@ -3170,7 +3144,7 @@
       <c r="U42" t="s">
         <v>28</v>
       </c>
-      <c r="V42" s="2">
+      <c r="V42" s="1">
         <v>46352</v>
       </c>
     </row>
@@ -3196,7 +3170,7 @@
       <c r="G43" t="s">
         <v>44</v>
       </c>
-      <c r="H43" s="2">
+      <c r="H43" s="1">
         <v>46191</v>
       </c>
       <c r="I43" t="s">
@@ -3226,7 +3200,7 @@
       <c r="U43" t="s">
         <v>28</v>
       </c>
-      <c r="V43" s="2">
+      <c r="V43" s="1">
         <v>46229</v>
       </c>
     </row>
@@ -3252,7 +3226,7 @@
       <c r="G44" t="s">
         <v>44</v>
       </c>
-      <c r="H44" s="2">
+      <c r="H44" s="1">
         <v>46191</v>
       </c>
       <c r="I44" t="s">
@@ -3282,7 +3256,7 @@
       <c r="U44" t="s">
         <v>28</v>
       </c>
-      <c r="V44" s="2">
+      <c r="V44" s="1">
         <v>46229</v>
       </c>
     </row>
@@ -3308,7 +3282,7 @@
       <c r="G45" t="s">
         <v>44</v>
       </c>
-      <c r="H45" s="2">
+      <c r="H45" s="1">
         <v>46213</v>
       </c>
       <c r="I45" t="s">
@@ -3341,7 +3315,7 @@
       <c r="U45" t="s">
         <v>181</v>
       </c>
-      <c r="V45" s="2">
+      <c r="V45" s="1">
         <v>46291</v>
       </c>
     </row>
@@ -3367,7 +3341,7 @@
       <c r="G46" t="s">
         <v>44</v>
       </c>
-      <c r="H46" s="2">
+      <c r="H46" s="1">
         <v>46210</v>
       </c>
       <c r="I46" t="s">
@@ -3397,7 +3371,7 @@
       <c r="U46" t="s">
         <v>181</v>
       </c>
-      <c r="V46" s="2">
+      <c r="V46" s="1">
         <v>46291</v>
       </c>
     </row>
@@ -3444,7 +3418,7 @@
       <c r="U47" t="s">
         <v>28</v>
       </c>
-      <c r="V47" s="2">
+      <c r="V47" s="1">
         <v>46321</v>
       </c>
     </row>
@@ -3497,7 +3471,7 @@
       <c r="U48" t="s">
         <v>181</v>
       </c>
-      <c r="V48" s="2">
+      <c r="V48" s="1">
         <v>46352</v>
       </c>
     </row>
@@ -3523,7 +3497,7 @@
       <c r="G49" t="s">
         <v>44</v>
       </c>
-      <c r="H49" s="2">
+      <c r="H49" s="1">
         <v>46176</v>
       </c>
       <c r="I49" t="s">
@@ -3556,7 +3530,7 @@
       <c r="U49" t="s">
         <v>181</v>
       </c>
-      <c r="V49" s="2">
+      <c r="V49" s="1">
         <v>46352</v>
       </c>
     </row>
@@ -3609,7 +3583,7 @@
       <c r="U50" t="s">
         <v>181</v>
       </c>
-      <c r="V50" s="2">
+      <c r="V50" s="1">
         <v>46321</v>
       </c>
     </row>
@@ -3665,7 +3639,7 @@
       <c r="U51" t="s">
         <v>181</v>
       </c>
-      <c r="V51" s="2">
+      <c r="V51" s="1">
         <v>46352</v>
       </c>
     </row>
@@ -3715,7 +3689,7 @@
       <c r="U52" t="s">
         <v>181</v>
       </c>
-      <c r="V52" s="2">
+      <c r="V52" s="1">
         <v>46382</v>
       </c>
     </row>
@@ -3741,7 +3715,7 @@
       <c r="G53" t="s">
         <v>44</v>
       </c>
-      <c r="H53" s="2">
+      <c r="H53" s="1">
         <v>46227</v>
       </c>
       <c r="I53" t="s">
@@ -3771,7 +3745,7 @@
       <c r="U53" t="s">
         <v>181</v>
       </c>
-      <c r="V53" s="2">
+      <c r="V53" s="1">
         <v>46321</v>
       </c>
     </row>
@@ -3794,7 +3768,7 @@
       <c r="G54" t="s">
         <v>44</v>
       </c>
-      <c r="H54" s="2">
+      <c r="H54" s="1">
         <v>46280</v>
       </c>
       <c r="I54" t="s">
@@ -3824,7 +3798,7 @@
       <c r="U54" t="s">
         <v>181</v>
       </c>
-      <c r="V54" s="2">
+      <c r="V54" s="1">
         <v>46352</v>
       </c>
     </row>
@@ -3847,7 +3821,7 @@
       <c r="G55" t="s">
         <v>44</v>
       </c>
-      <c r="H55" s="2">
+      <c r="H55" s="1">
         <v>46280</v>
       </c>
       <c r="I55" t="s">
@@ -3877,7 +3851,7 @@
       <c r="U55" t="s">
         <v>181</v>
       </c>
-      <c r="V55" s="2">
+      <c r="V55" s="1">
         <v>46321</v>
       </c>
     </row>
@@ -3930,7 +3904,7 @@
       <c r="U56" t="s">
         <v>181</v>
       </c>
-      <c r="V56" s="2">
+      <c r="V56" s="1">
         <v>46049</v>
       </c>
     </row>
@@ -3983,7 +3957,7 @@
       <c r="U57" t="s">
         <v>181</v>
       </c>
-      <c r="V57" s="2">
+      <c r="V57" s="1">
         <v>46049</v>
       </c>
     </row>
@@ -4030,7 +4004,7 @@
       <c r="U58" t="s">
         <v>181</v>
       </c>
-      <c r="V58" s="2">
+      <c r="V58" s="1">
         <v>46049</v>
       </c>
     </row>
@@ -4074,7 +4048,7 @@
       <c r="U59" t="s">
         <v>181</v>
       </c>
-      <c r="V59" s="2">
+      <c r="V59" s="1">
         <v>46139</v>
       </c>
     </row>
@@ -4200,7 +4174,7 @@
       <c r="U62" t="s">
         <v>181</v>
       </c>
-      <c r="V62" s="2">
+      <c r="V62" s="1">
         <v>46168</v>
       </c>
     </row>
@@ -4244,7 +4218,7 @@
       <c r="U63" t="s">
         <v>181</v>
       </c>
-      <c r="V63" s="2">
+      <c r="V63" s="1">
         <v>46168</v>
       </c>
     </row>
@@ -4288,7 +4262,7 @@
       <c r="U64" t="s">
         <v>181</v>
       </c>
-      <c r="V64" s="2">
+      <c r="V64" s="1">
         <v>46168</v>
       </c>
     </row>
@@ -4332,7 +4306,7 @@
       <c r="U65" t="s">
         <v>181</v>
       </c>
-      <c r="V65" s="2">
+      <c r="V65" s="1">
         <v>46168</v>
       </c>
     </row>
@@ -4376,7 +4350,7 @@
       <c r="U66" t="s">
         <v>181</v>
       </c>
-      <c r="V66" s="2">
+      <c r="V66" s="1">
         <v>46168</v>
       </c>
     </row>
@@ -4420,7 +4394,7 @@
       <c r="U67" t="s">
         <v>181</v>
       </c>
-      <c r="V67" s="2">
+      <c r="V67" s="1">
         <v>46168</v>
       </c>
     </row>
@@ -4464,7 +4438,7 @@
       <c r="U68" t="s">
         <v>28</v>
       </c>
-      <c r="V68" s="2">
+      <c r="V68" s="1">
         <v>46168</v>
       </c>
     </row>
@@ -4511,7 +4485,7 @@
       <c r="U69" t="s">
         <v>28</v>
       </c>
-      <c r="V69" s="2">
+      <c r="V69" s="1">
         <v>46382</v>
       </c>
     </row>
@@ -4564,7 +4538,7 @@
       <c r="U70" t="s">
         <v>181</v>
       </c>
-      <c r="V70" s="2">
+      <c r="V70" s="1">
         <v>46291</v>
       </c>
     </row>
@@ -4608,7 +4582,7 @@
       <c r="U71" t="s">
         <v>28</v>
       </c>
-      <c r="V71" s="2">
+      <c r="V71" s="1">
         <v>46260</v>
       </c>
     </row>
@@ -4652,7 +4626,7 @@
       <c r="U72" t="s">
         <v>181</v>
       </c>
-      <c r="V72" s="2">
+      <c r="V72" s="1">
         <v>46352</v>
       </c>
     </row>
@@ -4696,7 +4670,7 @@
       <c r="U73" t="s">
         <v>181</v>
       </c>
-      <c r="V73" s="2">
+      <c r="V73" s="1">
         <v>46229</v>
       </c>
     </row>
@@ -4740,7 +4714,7 @@
       <c r="U74" t="s">
         <v>181</v>
       </c>
-      <c r="V74" s="2">
+      <c r="V74" s="1">
         <v>46352</v>
       </c>
     </row>
@@ -4784,7 +4758,7 @@
       <c r="U75" t="s">
         <v>181</v>
       </c>
-      <c r="V75" s="2">
+      <c r="V75" s="1">
         <v>46352</v>
       </c>
     </row>
@@ -4828,7 +4802,7 @@
       <c r="U76" t="s">
         <v>181</v>
       </c>
-      <c r="V76" s="2">
+      <c r="V76" s="1">
         <v>46352</v>
       </c>
     </row>
@@ -4875,7 +4849,7 @@
       <c r="U77" t="s">
         <v>28</v>
       </c>
-      <c r="V77" s="2">
+      <c r="V77" s="1">
         <v>46382</v>
       </c>
     </row>
@@ -4925,7 +4899,7 @@
       <c r="U78" t="s">
         <v>181</v>
       </c>
-      <c r="V78" s="2">
+      <c r="V78" s="1">
         <v>46107</v>
       </c>
     </row>
@@ -4975,7 +4949,7 @@
       <c r="U79" t="s">
         <v>181</v>
       </c>
-      <c r="V79" s="2">
+      <c r="V79" s="1">
         <v>46138</v>
       </c>
     </row>
@@ -5025,7 +4999,7 @@
       <c r="U80" t="s">
         <v>28</v>
       </c>
-      <c r="V80" s="2">
+      <c r="V80" s="1">
         <v>46260</v>
       </c>
     </row>
@@ -5075,7 +5049,7 @@
       <c r="U81" t="s">
         <v>28</v>
       </c>
-      <c r="V81" s="2">
+      <c r="V81" s="1">
         <v>46260</v>
       </c>
     </row>
@@ -5125,7 +5099,7 @@
       <c r="U82" t="s">
         <v>28</v>
       </c>
-      <c r="V82" s="2">
+      <c r="V82" s="1">
         <v>46108</v>
       </c>
     </row>
@@ -5169,7 +5143,7 @@
       <c r="U83" t="s">
         <v>28</v>
       </c>
-      <c r="V83" s="2">
+      <c r="V83" s="1">
         <v>46108</v>
       </c>
     </row>
@@ -5222,7 +5196,7 @@
       <c r="U84" t="s">
         <v>181</v>
       </c>
-      <c r="V84" s="2">
+      <c r="V84" s="1">
         <v>46080</v>
       </c>
     </row>
@@ -5269,7 +5243,7 @@
       <c r="U85" t="s">
         <v>28</v>
       </c>
-      <c r="V85" s="2">
+      <c r="V85" s="1">
         <v>46382</v>
       </c>
     </row>
@@ -5313,7 +5287,7 @@
       <c r="U86" t="s">
         <v>28</v>
       </c>
-      <c r="V86" s="2">
+      <c r="V86" s="1">
         <v>46108</v>
       </c>
     </row>
@@ -5454,7 +5428,7 @@
       <c r="U89" t="s">
         <v>28</v>
       </c>
-      <c r="V89" s="2">
+      <c r="V89" s="1">
         <v>46321</v>
       </c>
     </row>
@@ -5498,7 +5472,7 @@
       <c r="U90" t="s">
         <v>28</v>
       </c>
-      <c r="V90" s="2">
+      <c r="V90" s="1">
         <v>46382</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Atualização automática: mta (02/10/2026 09:57)
</commit_message>
<xml_diff>
--- a/Projetos/02_Dados_Tratados/base_mta_tratada.xlsx
+++ b/Projetos/02_Dados_Tratados/base_mta_tratada.xlsx
@@ -533,8 +533,16 @@
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="YYYY-MM-DD HH:MM:SS"/>
   </numFmts>
-  <fonts count="1">
+  <fonts count="2">
     <font>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
       <sz val="11"/>
       <color theme="1"/>
       <name val="Calibri"/>
@@ -550,7 +558,7 @@
       <patternFill patternType="gray125"/>
     </fill>
   </fills>
-  <borders count="1">
+  <borders count="2">
     <border>
       <left/>
       <right/>
@@ -558,12 +566,30 @@
       <bottom/>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin">
+        <color auto="1"/>
+      </left>
+      <right style="thin">
+        <color auto="1"/>
+      </right>
+      <top style="thin">
+        <color auto="1"/>
+      </top>
+      <bottom style="thin">
+        <color auto="1"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="3">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
   </cellXfs>
   <cellStyles count="1">
@@ -863,70 +889,70 @@
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:22">
-      <c r="A1" t="s">
+      <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
-      <c r="B1" t="s">
+      <c r="B1" s="1" t="s">
         <v>1</v>
       </c>
-      <c r="C1" t="s">
+      <c r="C1" s="1" t="s">
         <v>2</v>
       </c>
-      <c r="D1" t="s">
+      <c r="D1" s="1" t="s">
         <v>3</v>
       </c>
-      <c r="E1" t="s">
+      <c r="E1" s="1" t="s">
         <v>4</v>
       </c>
-      <c r="F1" t="s">
+      <c r="F1" s="1" t="s">
         <v>5</v>
       </c>
-      <c r="G1" t="s">
+      <c r="G1" s="1" t="s">
         <v>6</v>
       </c>
-      <c r="H1" t="s">
+      <c r="H1" s="1" t="s">
         <v>7</v>
       </c>
-      <c r="I1" t="s">
+      <c r="I1" s="1" t="s">
         <v>8</v>
       </c>
-      <c r="J1" t="s">
+      <c r="J1" s="1" t="s">
         <v>9</v>
       </c>
-      <c r="K1" t="s">
+      <c r="K1" s="1" t="s">
         <v>10</v>
       </c>
-      <c r="L1" t="s">
+      <c r="L1" s="1" t="s">
         <v>11</v>
       </c>
-      <c r="M1" t="s">
+      <c r="M1" s="1" t="s">
         <v>12</v>
       </c>
-      <c r="N1" t="s">
+      <c r="N1" s="1" t="s">
         <v>13</v>
       </c>
-      <c r="O1" t="s">
+      <c r="O1" s="1" t="s">
         <v>14</v>
       </c>
-      <c r="P1" t="s">
+      <c r="P1" s="1" t="s">
         <v>15</v>
       </c>
-      <c r="Q1" t="s">
+      <c r="Q1" s="1" t="s">
         <v>16</v>
       </c>
-      <c r="R1" t="s">
+      <c r="R1" s="1" t="s">
         <v>17</v>
       </c>
-      <c r="S1" t="s">
+      <c r="S1" s="1" t="s">
         <v>18</v>
       </c>
-      <c r="T1" t="s">
+      <c r="T1" s="1" t="s">
         <v>19</v>
       </c>
-      <c r="U1" t="s">
+      <c r="U1" s="1" t="s">
         <v>20</v>
       </c>
-      <c r="V1" t="s">
+      <c r="V1" s="1" t="s">
         <v>21</v>
       </c>
     </row>
@@ -982,7 +1008,7 @@
       <c r="U2" t="s">
         <v>169</v>
       </c>
-      <c r="V2" s="1">
+      <c r="V2" s="2">
         <v>46229</v>
       </c>
     </row>
@@ -1029,7 +1055,7 @@
       <c r="U3" t="s">
         <v>91</v>
       </c>
-      <c r="V3" s="1">
+      <c r="V3" s="2">
         <v>46291</v>
       </c>
     </row>
@@ -1076,7 +1102,7 @@
       <c r="U4" t="s">
         <v>91</v>
       </c>
-      <c r="V4" s="1">
+      <c r="V4" s="2">
         <v>46321</v>
       </c>
     </row>
@@ -1123,7 +1149,7 @@
       <c r="U5" t="s">
         <v>91</v>
       </c>
-      <c r="V5" s="1">
+      <c r="V5" s="2">
         <v>46321</v>
       </c>
     </row>
@@ -1173,7 +1199,7 @@
       <c r="U6" t="s">
         <v>91</v>
       </c>
-      <c r="V6" s="1">
+      <c r="V6" s="2">
         <v>46291</v>
       </c>
     </row>
@@ -1199,7 +1225,7 @@
       <c r="G7" t="s">
         <v>105</v>
       </c>
-      <c r="H7" s="1">
+      <c r="H7" s="2">
         <v>46121</v>
       </c>
       <c r="I7" t="s">
@@ -1229,7 +1255,7 @@
       <c r="U7" t="s">
         <v>91</v>
       </c>
-      <c r="V7" s="1">
+      <c r="V7" s="2">
         <v>46138</v>
       </c>
     </row>
@@ -1276,7 +1302,7 @@
       <c r="U8" t="s">
         <v>91</v>
       </c>
-      <c r="V8" s="1">
+      <c r="V8" s="2">
         <v>46291</v>
       </c>
     </row>
@@ -1323,7 +1349,7 @@
       <c r="U9" t="s">
         <v>91</v>
       </c>
-      <c r="V9" s="1">
+      <c r="V9" s="2">
         <v>46291</v>
       </c>
     </row>
@@ -1370,7 +1396,7 @@
       <c r="U10" t="s">
         <v>91</v>
       </c>
-      <c r="V10" s="1">
+      <c r="V10" s="2">
         <v>46291</v>
       </c>
     </row>
@@ -1417,7 +1443,7 @@
       <c r="U11" t="s">
         <v>91</v>
       </c>
-      <c r="V11" s="1">
+      <c r="V11" s="2">
         <v>46291</v>
       </c>
     </row>
@@ -1443,7 +1469,7 @@
       <c r="G12" t="s">
         <v>105</v>
       </c>
-      <c r="H12" s="1">
+      <c r="H12" s="2">
         <v>46079</v>
       </c>
       <c r="I12" t="s">
@@ -1476,7 +1502,7 @@
       <c r="U12" t="s">
         <v>169</v>
       </c>
-      <c r="V12" s="1">
+      <c r="V12" s="2">
         <v>46079</v>
       </c>
     </row>
@@ -1529,7 +1555,7 @@
       <c r="U13" t="s">
         <v>169</v>
       </c>
-      <c r="V13" s="1">
+      <c r="V13" s="2">
         <v>46352</v>
       </c>
     </row>
@@ -1582,7 +1608,7 @@
       <c r="U14" t="s">
         <v>169</v>
       </c>
-      <c r="V14" s="1">
+      <c r="V14" s="2">
         <v>46352</v>
       </c>
     </row>
@@ -1635,7 +1661,7 @@
       <c r="U15" t="s">
         <v>169</v>
       </c>
-      <c r="V15" s="1">
+      <c r="V15" s="2">
         <v>46352</v>
       </c>
     </row>
@@ -1688,7 +1714,7 @@
       <c r="U16" t="s">
         <v>169</v>
       </c>
-      <c r="V16" s="1">
+      <c r="V16" s="2">
         <v>46229</v>
       </c>
     </row>
@@ -1714,7 +1740,7 @@
       <c r="G17" t="s">
         <v>105</v>
       </c>
-      <c r="H17" s="1">
+      <c r="H17" s="2">
         <v>46098</v>
       </c>
       <c r="I17" t="s">
@@ -1747,7 +1773,7 @@
       <c r="U17" t="s">
         <v>169</v>
       </c>
-      <c r="V17" s="1">
+      <c r="V17" s="2">
         <v>46107</v>
       </c>
     </row>
@@ -1773,7 +1799,7 @@
       <c r="G18" t="s">
         <v>105</v>
       </c>
-      <c r="H18" s="1">
+      <c r="H18" s="2">
         <v>46076</v>
       </c>
       <c r="I18" t="s">
@@ -1803,7 +1829,7 @@
       <c r="U18" t="s">
         <v>91</v>
       </c>
-      <c r="V18" s="1">
+      <c r="V18" s="2">
         <v>46079</v>
       </c>
     </row>
@@ -1829,7 +1855,7 @@
       <c r="G19" t="s">
         <v>105</v>
       </c>
-      <c r="H19" s="1">
+      <c r="H19" s="2">
         <v>46076</v>
       </c>
       <c r="I19" t="s">
@@ -1859,7 +1885,7 @@
       <c r="U19" t="s">
         <v>91</v>
       </c>
-      <c r="V19" s="1">
+      <c r="V19" s="2">
         <v>46079</v>
       </c>
     </row>
@@ -1906,7 +1932,7 @@
       <c r="U20" t="s">
         <v>91</v>
       </c>
-      <c r="V20" s="1">
+      <c r="V20" s="2">
         <v>46321</v>
       </c>
     </row>
@@ -1953,7 +1979,7 @@
       <c r="U21" t="s">
         <v>91</v>
       </c>
-      <c r="V21" s="1">
+      <c r="V21" s="2">
         <v>46321</v>
       </c>
     </row>
@@ -2000,7 +2026,7 @@
       <c r="U22" t="s">
         <v>91</v>
       </c>
-      <c r="V22" s="1">
+      <c r="V22" s="2">
         <v>46321</v>
       </c>
     </row>
@@ -2047,7 +2073,7 @@
       <c r="U23" t="s">
         <v>91</v>
       </c>
-      <c r="V23" s="1">
+      <c r="V23" s="2">
         <v>46321</v>
       </c>
     </row>
@@ -2073,7 +2099,7 @@
       <c r="G24" t="s">
         <v>105</v>
       </c>
-      <c r="H24" s="1">
+      <c r="H24" s="2">
         <v>46119</v>
       </c>
       <c r="I24" t="s">
@@ -2106,7 +2132,7 @@
       <c r="U24" t="s">
         <v>169</v>
       </c>
-      <c r="V24" s="1">
+      <c r="V24" s="2">
         <v>46138</v>
       </c>
     </row>
@@ -2132,7 +2158,7 @@
       <c r="G25" t="s">
         <v>105</v>
       </c>
-      <c r="H25" s="1">
+      <c r="H25" s="2">
         <v>46121</v>
       </c>
       <c r="I25" t="s">
@@ -2162,7 +2188,7 @@
       <c r="U25" t="s">
         <v>91</v>
       </c>
-      <c r="V25" s="1">
+      <c r="V25" s="2">
         <v>46138</v>
       </c>
     </row>
@@ -2188,7 +2214,7 @@
       <c r="G26" t="s">
         <v>105</v>
       </c>
-      <c r="H26" s="1">
+      <c r="H26" s="2">
         <v>46076</v>
       </c>
       <c r="I26" t="s">
@@ -2218,7 +2244,7 @@
       <c r="U26" t="s">
         <v>91</v>
       </c>
-      <c r="V26" s="1">
+      <c r="V26" s="2">
         <v>46079</v>
       </c>
     </row>
@@ -2271,7 +2297,7 @@
       <c r="U27" t="s">
         <v>169</v>
       </c>
-      <c r="V27" s="1">
+      <c r="V27" s="2">
         <v>46291</v>
       </c>
     </row>
@@ -2297,7 +2323,7 @@
       <c r="G28" t="s">
         <v>105</v>
       </c>
-      <c r="H28" s="1">
+      <c r="H28" s="2">
         <v>46199</v>
       </c>
       <c r="I28" t="s">
@@ -2330,7 +2356,7 @@
       <c r="U28" t="s">
         <v>169</v>
       </c>
-      <c r="V28" s="1">
+      <c r="V28" s="2">
         <v>46199</v>
       </c>
     </row>
@@ -2356,7 +2382,7 @@
       <c r="G29" t="s">
         <v>105</v>
       </c>
-      <c r="H29" s="1">
+      <c r="H29" s="2">
         <v>46199</v>
       </c>
       <c r="I29" t="s">
@@ -2389,7 +2415,7 @@
       <c r="U29" t="s">
         <v>169</v>
       </c>
-      <c r="V29" s="1">
+      <c r="V29" s="2">
         <v>46199</v>
       </c>
     </row>
@@ -2415,7 +2441,7 @@
       <c r="G30" t="s">
         <v>105</v>
       </c>
-      <c r="H30" s="1">
+      <c r="H30" s="2">
         <v>46199</v>
       </c>
       <c r="I30" t="s">
@@ -2448,7 +2474,7 @@
       <c r="U30" t="s">
         <v>169</v>
       </c>
-      <c r="V30" s="1">
+      <c r="V30" s="2">
         <v>46199</v>
       </c>
     </row>
@@ -2474,7 +2500,7 @@
       <c r="G31" t="s">
         <v>105</v>
       </c>
-      <c r="H31" s="1">
+      <c r="H31" s="2">
         <v>46199</v>
       </c>
       <c r="I31" t="s">
@@ -2507,7 +2533,7 @@
       <c r="U31" t="s">
         <v>169</v>
       </c>
-      <c r="V31" s="1">
+      <c r="V31" s="2">
         <v>46199</v>
       </c>
     </row>
@@ -2557,7 +2583,7 @@
       <c r="U32" t="s">
         <v>169</v>
       </c>
-      <c r="V32" s="1">
+      <c r="V32" s="2">
         <v>46291</v>
       </c>
     </row>
@@ -2583,7 +2609,7 @@
       <c r="G33" t="s">
         <v>105</v>
       </c>
-      <c r="H33" s="1">
+      <c r="H33" s="2">
         <v>46191</v>
       </c>
       <c r="I33" t="s">
@@ -2616,7 +2642,7 @@
       <c r="U33" t="s">
         <v>169</v>
       </c>
-      <c r="V33" s="1">
+      <c r="V33" s="2">
         <v>46199</v>
       </c>
     </row>
@@ -2642,7 +2668,7 @@
       <c r="G34" t="s">
         <v>105</v>
       </c>
-      <c r="H34" s="1">
+      <c r="H34" s="2">
         <v>46119</v>
       </c>
       <c r="I34" t="s">
@@ -2672,7 +2698,7 @@
       <c r="U34" t="s">
         <v>169</v>
       </c>
-      <c r="V34" s="1">
+      <c r="V34" s="2">
         <v>46138</v>
       </c>
     </row>
@@ -2698,7 +2724,7 @@
       <c r="G35" t="s">
         <v>105</v>
       </c>
-      <c r="H35" s="1">
+      <c r="H35" s="2">
         <v>46213</v>
       </c>
       <c r="I35" t="s">
@@ -2728,7 +2754,7 @@
       <c r="U35" t="s">
         <v>91</v>
       </c>
-      <c r="V35" s="1">
+      <c r="V35" s="2">
         <v>46229</v>
       </c>
     </row>
@@ -2754,7 +2780,7 @@
       <c r="G36" t="s">
         <v>105</v>
       </c>
-      <c r="H36" s="1">
+      <c r="H36" s="2">
         <v>46175</v>
       </c>
       <c r="I36" t="s">
@@ -2784,7 +2810,7 @@
       <c r="U36" t="s">
         <v>91</v>
       </c>
-      <c r="V36" s="1">
+      <c r="V36" s="2">
         <v>46199</v>
       </c>
     </row>
@@ -2810,7 +2836,7 @@
       <c r="G37" t="s">
         <v>105</v>
       </c>
-      <c r="H37" s="1">
+      <c r="H37" s="2">
         <v>46213</v>
       </c>
       <c r="I37" t="s">
@@ -2840,7 +2866,7 @@
       <c r="U37" t="s">
         <v>91</v>
       </c>
-      <c r="V37" s="1">
+      <c r="V37" s="2">
         <v>46229</v>
       </c>
     </row>
@@ -2866,7 +2892,7 @@
       <c r="G38" t="s">
         <v>105</v>
       </c>
-      <c r="H38" s="1">
+      <c r="H38" s="2">
         <v>46199</v>
       </c>
       <c r="I38" t="s">
@@ -2896,7 +2922,7 @@
       <c r="U38" t="s">
         <v>91</v>
       </c>
-      <c r="V38" s="1">
+      <c r="V38" s="2">
         <v>46199</v>
       </c>
     </row>
@@ -2922,7 +2948,7 @@
       <c r="G39" t="s">
         <v>105</v>
       </c>
-      <c r="H39" s="1">
+      <c r="H39" s="2">
         <v>46199</v>
       </c>
       <c r="I39" t="s">
@@ -2952,7 +2978,7 @@
       <c r="U39" t="s">
         <v>91</v>
       </c>
-      <c r="V39" s="1">
+      <c r="V39" s="2">
         <v>46199</v>
       </c>
     </row>
@@ -2978,7 +3004,7 @@
       <c r="G40" t="s">
         <v>105</v>
       </c>
-      <c r="H40" s="1">
+      <c r="H40" s="2">
         <v>46204</v>
       </c>
       <c r="I40" t="s">
@@ -3008,7 +3034,7 @@
       <c r="U40" t="s">
         <v>91</v>
       </c>
-      <c r="V40" s="1">
+      <c r="V40" s="2">
         <v>46229</v>
       </c>
     </row>
@@ -3034,7 +3060,7 @@
       <c r="G41" t="s">
         <v>105</v>
       </c>
-      <c r="H41" s="1">
+      <c r="H41" s="2">
         <v>46244</v>
       </c>
       <c r="I41" t="s">
@@ -3064,7 +3090,7 @@
       <c r="U41" t="s">
         <v>91</v>
       </c>
-      <c r="V41" s="1">
+      <c r="V41" s="2">
         <v>46199</v>
       </c>
     </row>
@@ -3108,7 +3134,7 @@
       <c r="U42" t="s">
         <v>91</v>
       </c>
-      <c r="V42" s="1">
+      <c r="V42" s="2">
         <v>46260</v>
       </c>
     </row>
@@ -3134,7 +3160,7 @@
       <c r="G43" t="s">
         <v>105</v>
       </c>
-      <c r="H43" s="1">
+      <c r="H43" s="2">
         <v>46191</v>
       </c>
       <c r="I43" t="s">
@@ -3164,7 +3190,7 @@
       <c r="U43" t="s">
         <v>91</v>
       </c>
-      <c r="V43" s="1">
+      <c r="V43" s="2">
         <v>46199</v>
       </c>
     </row>
@@ -3190,7 +3216,7 @@
       <c r="G44" t="s">
         <v>105</v>
       </c>
-      <c r="H44" s="1">
+      <c r="H44" s="2">
         <v>46191</v>
       </c>
       <c r="I44" t="s">
@@ -3220,7 +3246,7 @@
       <c r="U44" t="s">
         <v>91</v>
       </c>
-      <c r="V44" s="1">
+      <c r="V44" s="2">
         <v>46199</v>
       </c>
     </row>
@@ -3246,7 +3272,7 @@
       <c r="G45" t="s">
         <v>105</v>
       </c>
-      <c r="H45" s="1">
+      <c r="H45" s="2">
         <v>46213</v>
       </c>
       <c r="I45" t="s">
@@ -3279,7 +3305,7 @@
       <c r="U45" t="s">
         <v>169</v>
       </c>
-      <c r="V45" s="1">
+      <c r="V45" s="2">
         <v>46229</v>
       </c>
     </row>
@@ -3305,7 +3331,7 @@
       <c r="G46" t="s">
         <v>105</v>
       </c>
-      <c r="H46" s="1">
+      <c r="H46" s="2">
         <v>46210</v>
       </c>
       <c r="I46" t="s">
@@ -3335,7 +3361,7 @@
       <c r="U46" t="s">
         <v>169</v>
       </c>
-      <c r="V46" s="1">
+      <c r="V46" s="2">
         <v>46229</v>
       </c>
     </row>
@@ -3382,7 +3408,7 @@
       <c r="U47" t="s">
         <v>91</v>
       </c>
-      <c r="V47" s="1">
+      <c r="V47" s="2">
         <v>46321</v>
       </c>
     </row>
@@ -3435,7 +3461,7 @@
       <c r="U48" t="s">
         <v>169</v>
       </c>
-      <c r="V48" s="1">
+      <c r="V48" s="2">
         <v>46291</v>
       </c>
     </row>
@@ -3461,7 +3487,7 @@
       <c r="G49" t="s">
         <v>105</v>
       </c>
-      <c r="H49" s="1">
+      <c r="H49" s="2">
         <v>46176</v>
       </c>
       <c r="I49" t="s">
@@ -3494,7 +3520,7 @@
       <c r="U49" t="s">
         <v>169</v>
       </c>
-      <c r="V49" s="1">
+      <c r="V49" s="2">
         <v>46199</v>
       </c>
     </row>
@@ -3547,7 +3573,7 @@
       <c r="U50" t="s">
         <v>169</v>
       </c>
-      <c r="V50" s="1">
+      <c r="V50" s="2">
         <v>46260</v>
       </c>
     </row>
@@ -3573,7 +3599,7 @@
       <c r="G51" t="s">
         <v>106</v>
       </c>
-      <c r="H51" s="1">
+      <c r="H51" s="2">
         <v>46295</v>
       </c>
       <c r="J51" t="s">
@@ -3606,7 +3632,7 @@
       <c r="U51" t="s">
         <v>169</v>
       </c>
-      <c r="V51" s="1">
+      <c r="V51" s="2">
         <v>46291</v>
       </c>
     </row>
@@ -3632,7 +3658,7 @@
       <c r="G52" t="s">
         <v>106</v>
       </c>
-      <c r="H52" s="1">
+      <c r="H52" s="2">
         <v>46295</v>
       </c>
       <c r="K52" t="s">
@@ -3662,7 +3688,7 @@
       <c r="U52" t="s">
         <v>169</v>
       </c>
-      <c r="V52" s="1">
+      <c r="V52" s="2">
         <v>46291</v>
       </c>
     </row>
@@ -3688,7 +3714,7 @@
       <c r="G53" t="s">
         <v>106</v>
       </c>
-      <c r="H53" s="1">
+      <c r="H53" s="2">
         <v>46295</v>
       </c>
       <c r="N53" t="s">
@@ -3715,7 +3741,7 @@
       <c r="U53" t="s">
         <v>169</v>
       </c>
-      <c r="V53" s="1">
+      <c r="V53" s="2">
         <v>46291</v>
       </c>
     </row>
@@ -3738,7 +3764,7 @@
       <c r="G54" t="s">
         <v>105</v>
       </c>
-      <c r="H54" s="1">
+      <c r="H54" s="2">
         <v>46280</v>
       </c>
       <c r="I54" t="s">
@@ -3768,7 +3794,7 @@
       <c r="U54" t="s">
         <v>169</v>
       </c>
-      <c r="V54" s="1">
+      <c r="V54" s="2">
         <v>46291</v>
       </c>
     </row>
@@ -3791,7 +3817,7 @@
       <c r="G55" t="s">
         <v>105</v>
       </c>
-      <c r="H55" s="1">
+      <c r="H55" s="2">
         <v>46280</v>
       </c>
       <c r="I55" t="s">
@@ -3821,7 +3847,7 @@
       <c r="U55" t="s">
         <v>169</v>
       </c>
-      <c r="V55" s="1">
+      <c r="V55" s="2">
         <v>46260</v>
       </c>
     </row>
@@ -3874,7 +3900,7 @@
       <c r="U56" t="s">
         <v>169</v>
       </c>
-      <c r="V56" s="1">
+      <c r="V56" s="2">
         <v>46352</v>
       </c>
     </row>
@@ -3918,7 +3944,7 @@
       <c r="U57" t="s">
         <v>169</v>
       </c>
-      <c r="V57" s="1">
+      <c r="V57" s="2">
         <v>46107</v>
       </c>
     </row>
@@ -3962,7 +3988,7 @@
       <c r="U58" t="s">
         <v>169</v>
       </c>
-      <c r="V58" s="1">
+      <c r="V58" s="2">
         <v>46107</v>
       </c>
     </row>
@@ -4006,7 +4032,7 @@
       <c r="U59" t="s">
         <v>169</v>
       </c>
-      <c r="V59" s="1">
+      <c r="V59" s="2">
         <v>46107</v>
       </c>
     </row>
@@ -4050,7 +4076,7 @@
       <c r="U60" t="s">
         <v>169</v>
       </c>
-      <c r="V60" s="1">
+      <c r="V60" s="2">
         <v>46107</v>
       </c>
     </row>
@@ -4094,7 +4120,7 @@
       <c r="U61" t="s">
         <v>169</v>
       </c>
-      <c r="V61" s="1">
+      <c r="V61" s="2">
         <v>46107</v>
       </c>
     </row>
@@ -4138,7 +4164,7 @@
       <c r="U62" t="s">
         <v>169</v>
       </c>
-      <c r="V62" s="1">
+      <c r="V62" s="2">
         <v>46107</v>
       </c>
     </row>
@@ -4182,7 +4208,7 @@
       <c r="U63" t="s">
         <v>91</v>
       </c>
-      <c r="V63" s="1">
+      <c r="V63" s="2">
         <v>46168</v>
       </c>
     </row>
@@ -4229,7 +4255,7 @@
       <c r="U64" t="s">
         <v>91</v>
       </c>
-      <c r="V64" s="1">
+      <c r="V64" s="2">
         <v>46291</v>
       </c>
     </row>
@@ -4282,7 +4308,7 @@
       <c r="U65" t="s">
         <v>169</v>
       </c>
-      <c r="V65" s="1">
+      <c r="V65" s="2">
         <v>46229</v>
       </c>
     </row>
@@ -4326,7 +4352,7 @@
       <c r="U66" t="s">
         <v>91</v>
       </c>
-      <c r="V66" s="1">
+      <c r="V66" s="2">
         <v>46260</v>
       </c>
     </row>
@@ -4370,7 +4396,7 @@
       <c r="U67" t="s">
         <v>169</v>
       </c>
-      <c r="V67" s="1">
+      <c r="V67" s="2">
         <v>46291</v>
       </c>
     </row>
@@ -4414,7 +4440,7 @@
       <c r="U68" t="s">
         <v>169</v>
       </c>
-      <c r="V68" s="1">
+      <c r="V68" s="2">
         <v>46168</v>
       </c>
     </row>
@@ -4458,7 +4484,7 @@
       <c r="U69" t="s">
         <v>169</v>
       </c>
-      <c r="V69" s="1">
+      <c r="V69" s="2">
         <v>46291</v>
       </c>
     </row>
@@ -4502,7 +4528,7 @@
       <c r="U70" t="s">
         <v>169</v>
       </c>
-      <c r="V70" s="1">
+      <c r="V70" s="2">
         <v>46291</v>
       </c>
     </row>
@@ -4546,7 +4572,7 @@
       <c r="U71" t="s">
         <v>169</v>
       </c>
-      <c r="V71" s="1">
+      <c r="V71" s="2">
         <v>46291</v>
       </c>
     </row>
@@ -4593,7 +4619,7 @@
       <c r="U72" t="s">
         <v>91</v>
       </c>
-      <c r="V72" s="1">
+      <c r="V72" s="2">
         <v>46321</v>
       </c>
     </row>
@@ -4643,7 +4669,7 @@
       <c r="U73" t="s">
         <v>169</v>
       </c>
-      <c r="V73" s="1">
+      <c r="V73" s="2">
         <v>46381</v>
       </c>
     </row>
@@ -4693,7 +4719,7 @@
       <c r="U74" t="s">
         <v>169</v>
       </c>
-      <c r="V74" s="1">
+      <c r="V74" s="2">
         <v>46381</v>
       </c>
     </row>
@@ -4743,7 +4769,7 @@
       <c r="U75" t="s">
         <v>91</v>
       </c>
-      <c r="V75" s="1">
+      <c r="V75" s="2">
         <v>46381</v>
       </c>
     </row>
@@ -4793,7 +4819,7 @@
       <c r="U76" t="s">
         <v>91</v>
       </c>
-      <c r="V76" s="1">
+      <c r="V76" s="2">
         <v>46381</v>
       </c>
     </row>
@@ -4843,7 +4869,7 @@
       <c r="U77" t="s">
         <v>91</v>
       </c>
-      <c r="V77" s="1">
+      <c r="V77" s="2">
         <v>46382</v>
       </c>
     </row>
@@ -4887,7 +4913,7 @@
       <c r="U78" t="s">
         <v>91</v>
       </c>
-      <c r="V78" s="1">
+      <c r="V78" s="2">
         <v>46382</v>
       </c>
     </row>
@@ -4940,7 +4966,7 @@
       <c r="U79" t="s">
         <v>169</v>
       </c>
-      <c r="V79" s="1">
+      <c r="V79" s="2">
         <v>46382</v>
       </c>
     </row>
@@ -4987,7 +5013,7 @@
       <c r="U80" t="s">
         <v>91</v>
       </c>
-      <c r="V80" s="1">
+      <c r="V80" s="2">
         <v>46321</v>
       </c>
     </row>
@@ -5031,7 +5057,7 @@
       <c r="U81" t="s">
         <v>91</v>
       </c>
-      <c r="V81" s="1">
+      <c r="V81" s="2">
         <v>46382</v>
       </c>
     </row>
@@ -5172,7 +5198,7 @@
       <c r="U84" t="s">
         <v>91</v>
       </c>
-      <c r="V84" s="1">
+      <c r="V84" s="2">
         <v>46291</v>
       </c>
     </row>
@@ -5216,7 +5242,7 @@
       <c r="U85" t="s">
         <v>91</v>
       </c>
-      <c r="V85" s="1">
+      <c r="V85" s="2">
         <v>46291</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Atualização automática: mta (05/10/2026 08:40)
</commit_message>
<xml_diff>
--- a/Projetos/02_Dados_Tratados/base_mta_tratada.xlsx
+++ b/Projetos/02_Dados_Tratados/base_mta_tratada.xlsx
@@ -539,8 +539,16 @@
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="YYYY-MM-DD HH:MM:SS"/>
   </numFmts>
-  <fonts count="1">
+  <fonts count="2">
     <font>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
       <sz val="11"/>
       <color theme="1"/>
       <name val="Calibri"/>
@@ -556,7 +564,7 @@
       <patternFill patternType="gray125"/>
     </fill>
   </fills>
-  <borders count="1">
+  <borders count="2">
     <border>
       <left/>
       <right/>
@@ -564,12 +572,30 @@
       <bottom/>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin">
+        <color auto="1"/>
+      </left>
+      <right style="thin">
+        <color auto="1"/>
+      </right>
+      <top style="thin">
+        <color auto="1"/>
+      </top>
+      <bottom style="thin">
+        <color auto="1"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="3">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
   </cellXfs>
   <cellStyles count="1">
@@ -869,70 +895,70 @@
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:22">
-      <c r="A1" t="s">
+      <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
-      <c r="B1" t="s">
+      <c r="B1" s="1" t="s">
         <v>1</v>
       </c>
-      <c r="C1" t="s">
+      <c r="C1" s="1" t="s">
         <v>2</v>
       </c>
-      <c r="D1" t="s">
+      <c r="D1" s="1" t="s">
         <v>3</v>
       </c>
-      <c r="E1" t="s">
+      <c r="E1" s="1" t="s">
         <v>4</v>
       </c>
-      <c r="F1" t="s">
+      <c r="F1" s="1" t="s">
         <v>5</v>
       </c>
-      <c r="G1" t="s">
+      <c r="G1" s="1" t="s">
         <v>6</v>
       </c>
-      <c r="H1" t="s">
+      <c r="H1" s="1" t="s">
         <v>7</v>
       </c>
-      <c r="I1" t="s">
+      <c r="I1" s="1" t="s">
         <v>8</v>
       </c>
-      <c r="J1" t="s">
+      <c r="J1" s="1" t="s">
         <v>9</v>
       </c>
-      <c r="K1" t="s">
+      <c r="K1" s="1" t="s">
         <v>10</v>
       </c>
-      <c r="L1" t="s">
+      <c r="L1" s="1" t="s">
         <v>11</v>
       </c>
-      <c r="M1" t="s">
+      <c r="M1" s="1" t="s">
         <v>12</v>
       </c>
-      <c r="N1" t="s">
+      <c r="N1" s="1" t="s">
         <v>13</v>
       </c>
-      <c r="O1" t="s">
+      <c r="O1" s="1" t="s">
         <v>14</v>
       </c>
-      <c r="P1" t="s">
+      <c r="P1" s="1" t="s">
         <v>15</v>
       </c>
-      <c r="Q1" t="s">
+      <c r="Q1" s="1" t="s">
         <v>16</v>
       </c>
-      <c r="R1" t="s">
+      <c r="R1" s="1" t="s">
         <v>17</v>
       </c>
-      <c r="S1" t="s">
+      <c r="S1" s="1" t="s">
         <v>18</v>
       </c>
-      <c r="T1" t="s">
+      <c r="T1" s="1" t="s">
         <v>19</v>
       </c>
-      <c r="U1" t="s">
+      <c r="U1" s="1" t="s">
         <v>20</v>
       </c>
-      <c r="V1" t="s">
+      <c r="V1" s="1" t="s">
         <v>21</v>
       </c>
     </row>
@@ -988,7 +1014,7 @@
       <c r="U2" t="s">
         <v>171</v>
       </c>
-      <c r="V2" s="1">
+      <c r="V2" s="2">
         <v>46229</v>
       </c>
     </row>
@@ -1035,7 +1061,7 @@
       <c r="U3" t="s">
         <v>91</v>
       </c>
-      <c r="V3" s="1">
+      <c r="V3" s="2">
         <v>46291</v>
       </c>
     </row>
@@ -1082,7 +1108,7 @@
       <c r="U4" t="s">
         <v>91</v>
       </c>
-      <c r="V4" s="1">
+      <c r="V4" s="2">
         <v>46321</v>
       </c>
     </row>
@@ -1129,7 +1155,7 @@
       <c r="U5" t="s">
         <v>91</v>
       </c>
-      <c r="V5" s="1">
+      <c r="V5" s="2">
         <v>46321</v>
       </c>
     </row>
@@ -1179,7 +1205,7 @@
       <c r="U6" t="s">
         <v>91</v>
       </c>
-      <c r="V6" s="1">
+      <c r="V6" s="2">
         <v>46291</v>
       </c>
     </row>
@@ -1205,7 +1231,7 @@
       <c r="G7" t="s">
         <v>106</v>
       </c>
-      <c r="H7" s="1">
+      <c r="H7" s="2">
         <v>46121</v>
       </c>
       <c r="I7" t="s">
@@ -1235,7 +1261,7 @@
       <c r="U7" t="s">
         <v>91</v>
       </c>
-      <c r="V7" s="1">
+      <c r="V7" s="2">
         <v>46138</v>
       </c>
     </row>
@@ -1282,7 +1308,7 @@
       <c r="U8" t="s">
         <v>91</v>
       </c>
-      <c r="V8" s="1">
+      <c r="V8" s="2">
         <v>46291</v>
       </c>
     </row>
@@ -1329,7 +1355,7 @@
       <c r="U9" t="s">
         <v>91</v>
       </c>
-      <c r="V9" s="1">
+      <c r="V9" s="2">
         <v>46291</v>
       </c>
     </row>
@@ -1376,7 +1402,7 @@
       <c r="U10" t="s">
         <v>91</v>
       </c>
-      <c r="V10" s="1">
+      <c r="V10" s="2">
         <v>46291</v>
       </c>
     </row>
@@ -1423,7 +1449,7 @@
       <c r="U11" t="s">
         <v>91</v>
       </c>
-      <c r="V11" s="1">
+      <c r="V11" s="2">
         <v>46291</v>
       </c>
     </row>
@@ -1449,7 +1475,7 @@
       <c r="G12" t="s">
         <v>106</v>
       </c>
-      <c r="H12" s="1">
+      <c r="H12" s="2">
         <v>46079</v>
       </c>
       <c r="I12" t="s">
@@ -1482,7 +1508,7 @@
       <c r="U12" t="s">
         <v>171</v>
       </c>
-      <c r="V12" s="1">
+      <c r="V12" s="2">
         <v>46079</v>
       </c>
     </row>
@@ -1535,7 +1561,7 @@
       <c r="U13" t="s">
         <v>171</v>
       </c>
-      <c r="V13" s="1">
+      <c r="V13" s="2">
         <v>46352</v>
       </c>
     </row>
@@ -1588,7 +1614,7 @@
       <c r="U14" t="s">
         <v>171</v>
       </c>
-      <c r="V14" s="1">
+      <c r="V14" s="2">
         <v>46352</v>
       </c>
     </row>
@@ -1641,7 +1667,7 @@
       <c r="U15" t="s">
         <v>171</v>
       </c>
-      <c r="V15" s="1">
+      <c r="V15" s="2">
         <v>46352</v>
       </c>
     </row>
@@ -1694,7 +1720,7 @@
       <c r="U16" t="s">
         <v>171</v>
       </c>
-      <c r="V16" s="1">
+      <c r="V16" s="2">
         <v>46229</v>
       </c>
     </row>
@@ -1720,7 +1746,7 @@
       <c r="G17" t="s">
         <v>106</v>
       </c>
-      <c r="H17" s="1">
+      <c r="H17" s="2">
         <v>46098</v>
       </c>
       <c r="I17" t="s">
@@ -1753,7 +1779,7 @@
       <c r="U17" t="s">
         <v>171</v>
       </c>
-      <c r="V17" s="1">
+      <c r="V17" s="2">
         <v>46107</v>
       </c>
     </row>
@@ -1779,7 +1805,7 @@
       <c r="G18" t="s">
         <v>106</v>
       </c>
-      <c r="H18" s="1">
+      <c r="H18" s="2">
         <v>46076</v>
       </c>
       <c r="I18" t="s">
@@ -1809,7 +1835,7 @@
       <c r="U18" t="s">
         <v>91</v>
       </c>
-      <c r="V18" s="1">
+      <c r="V18" s="2">
         <v>46079</v>
       </c>
     </row>
@@ -1835,7 +1861,7 @@
       <c r="G19" t="s">
         <v>106</v>
       </c>
-      <c r="H19" s="1">
+      <c r="H19" s="2">
         <v>46076</v>
       </c>
       <c r="I19" t="s">
@@ -1865,7 +1891,7 @@
       <c r="U19" t="s">
         <v>91</v>
       </c>
-      <c r="V19" s="1">
+      <c r="V19" s="2">
         <v>46079</v>
       </c>
     </row>
@@ -1912,7 +1938,7 @@
       <c r="U20" t="s">
         <v>91</v>
       </c>
-      <c r="V20" s="1">
+      <c r="V20" s="2">
         <v>46321</v>
       </c>
     </row>
@@ -1959,7 +1985,7 @@
       <c r="U21" t="s">
         <v>91</v>
       </c>
-      <c r="V21" s="1">
+      <c r="V21" s="2">
         <v>46321</v>
       </c>
     </row>
@@ -2006,7 +2032,7 @@
       <c r="U22" t="s">
         <v>91</v>
       </c>
-      <c r="V22" s="1">
+      <c r="V22" s="2">
         <v>46321</v>
       </c>
     </row>
@@ -2053,7 +2079,7 @@
       <c r="U23" t="s">
         <v>91</v>
       </c>
-      <c r="V23" s="1">
+      <c r="V23" s="2">
         <v>46321</v>
       </c>
     </row>
@@ -2079,7 +2105,7 @@
       <c r="G24" t="s">
         <v>106</v>
       </c>
-      <c r="H24" s="1">
+      <c r="H24" s="2">
         <v>46119</v>
       </c>
       <c r="I24" t="s">
@@ -2112,7 +2138,7 @@
       <c r="U24" t="s">
         <v>171</v>
       </c>
-      <c r="V24" s="1">
+      <c r="V24" s="2">
         <v>46138</v>
       </c>
     </row>
@@ -2138,7 +2164,7 @@
       <c r="G25" t="s">
         <v>106</v>
       </c>
-      <c r="H25" s="1">
+      <c r="H25" s="2">
         <v>46121</v>
       </c>
       <c r="I25" t="s">
@@ -2168,7 +2194,7 @@
       <c r="U25" t="s">
         <v>91</v>
       </c>
-      <c r="V25" s="1">
+      <c r="V25" s="2">
         <v>46138</v>
       </c>
     </row>
@@ -2194,7 +2220,7 @@
       <c r="G26" t="s">
         <v>106</v>
       </c>
-      <c r="H26" s="1">
+      <c r="H26" s="2">
         <v>46076</v>
       </c>
       <c r="I26" t="s">
@@ -2224,7 +2250,7 @@
       <c r="U26" t="s">
         <v>91</v>
       </c>
-      <c r="V26" s="1">
+      <c r="V26" s="2">
         <v>46079</v>
       </c>
     </row>
@@ -2277,7 +2303,7 @@
       <c r="U27" t="s">
         <v>171</v>
       </c>
-      <c r="V27" s="1">
+      <c r="V27" s="2">
         <v>46291</v>
       </c>
     </row>
@@ -2303,7 +2329,7 @@
       <c r="G28" t="s">
         <v>106</v>
       </c>
-      <c r="H28" s="1">
+      <c r="H28" s="2">
         <v>46199</v>
       </c>
       <c r="I28" t="s">
@@ -2336,7 +2362,7 @@
       <c r="U28" t="s">
         <v>171</v>
       </c>
-      <c r="V28" s="1">
+      <c r="V28" s="2">
         <v>46199</v>
       </c>
     </row>
@@ -2362,7 +2388,7 @@
       <c r="G29" t="s">
         <v>106</v>
       </c>
-      <c r="H29" s="1">
+      <c r="H29" s="2">
         <v>46199</v>
       </c>
       <c r="I29" t="s">
@@ -2395,7 +2421,7 @@
       <c r="U29" t="s">
         <v>171</v>
       </c>
-      <c r="V29" s="1">
+      <c r="V29" s="2">
         <v>46199</v>
       </c>
     </row>
@@ -2421,7 +2447,7 @@
       <c r="G30" t="s">
         <v>106</v>
       </c>
-      <c r="H30" s="1">
+      <c r="H30" s="2">
         <v>46199</v>
       </c>
       <c r="I30" t="s">
@@ -2454,7 +2480,7 @@
       <c r="U30" t="s">
         <v>171</v>
       </c>
-      <c r="V30" s="1">
+      <c r="V30" s="2">
         <v>46199</v>
       </c>
     </row>
@@ -2480,7 +2506,7 @@
       <c r="G31" t="s">
         <v>106</v>
       </c>
-      <c r="H31" s="1">
+      <c r="H31" s="2">
         <v>46199</v>
       </c>
       <c r="I31" t="s">
@@ -2513,7 +2539,7 @@
       <c r="U31" t="s">
         <v>171</v>
       </c>
-      <c r="V31" s="1">
+      <c r="V31" s="2">
         <v>46199</v>
       </c>
     </row>
@@ -2563,7 +2589,7 @@
       <c r="U32" t="s">
         <v>171</v>
       </c>
-      <c r="V32" s="1">
+      <c r="V32" s="2">
         <v>46291</v>
       </c>
     </row>
@@ -2589,7 +2615,7 @@
       <c r="G33" t="s">
         <v>106</v>
       </c>
-      <c r="H33" s="1">
+      <c r="H33" s="2">
         <v>46191</v>
       </c>
       <c r="I33" t="s">
@@ -2622,7 +2648,7 @@
       <c r="U33" t="s">
         <v>171</v>
       </c>
-      <c r="V33" s="1">
+      <c r="V33" s="2">
         <v>46199</v>
       </c>
     </row>
@@ -2648,7 +2674,7 @@
       <c r="G34" t="s">
         <v>106</v>
       </c>
-      <c r="H34" s="1">
+      <c r="H34" s="2">
         <v>46119</v>
       </c>
       <c r="I34" t="s">
@@ -2678,7 +2704,7 @@
       <c r="U34" t="s">
         <v>171</v>
       </c>
-      <c r="V34" s="1">
+      <c r="V34" s="2">
         <v>46138</v>
       </c>
     </row>
@@ -2704,7 +2730,7 @@
       <c r="G35" t="s">
         <v>106</v>
       </c>
-      <c r="H35" s="1">
+      <c r="H35" s="2">
         <v>46213</v>
       </c>
       <c r="I35" t="s">
@@ -2734,7 +2760,7 @@
       <c r="U35" t="s">
         <v>91</v>
       </c>
-      <c r="V35" s="1">
+      <c r="V35" s="2">
         <v>46229</v>
       </c>
     </row>
@@ -2760,7 +2786,7 @@
       <c r="G36" t="s">
         <v>106</v>
       </c>
-      <c r="H36" s="1">
+      <c r="H36" s="2">
         <v>46175</v>
       </c>
       <c r="I36" t="s">
@@ -2790,7 +2816,7 @@
       <c r="U36" t="s">
         <v>91</v>
       </c>
-      <c r="V36" s="1">
+      <c r="V36" s="2">
         <v>46199</v>
       </c>
     </row>
@@ -2816,7 +2842,7 @@
       <c r="G37" t="s">
         <v>106</v>
       </c>
-      <c r="H37" s="1">
+      <c r="H37" s="2">
         <v>46213</v>
       </c>
       <c r="I37" t="s">
@@ -2846,7 +2872,7 @@
       <c r="U37" t="s">
         <v>91</v>
       </c>
-      <c r="V37" s="1">
+      <c r="V37" s="2">
         <v>46229</v>
       </c>
     </row>
@@ -2872,7 +2898,7 @@
       <c r="G38" t="s">
         <v>106</v>
       </c>
-      <c r="H38" s="1">
+      <c r="H38" s="2">
         <v>46199</v>
       </c>
       <c r="I38" t="s">
@@ -2902,7 +2928,7 @@
       <c r="U38" t="s">
         <v>91</v>
       </c>
-      <c r="V38" s="1">
+      <c r="V38" s="2">
         <v>46199</v>
       </c>
     </row>
@@ -2928,7 +2954,7 @@
       <c r="G39" t="s">
         <v>106</v>
       </c>
-      <c r="H39" s="1">
+      <c r="H39" s="2">
         <v>46199</v>
       </c>
       <c r="I39" t="s">
@@ -2958,7 +2984,7 @@
       <c r="U39" t="s">
         <v>91</v>
       </c>
-      <c r="V39" s="1">
+      <c r="V39" s="2">
         <v>46199</v>
       </c>
     </row>
@@ -2984,7 +3010,7 @@
       <c r="G40" t="s">
         <v>106</v>
       </c>
-      <c r="H40" s="1">
+      <c r="H40" s="2">
         <v>46204</v>
       </c>
       <c r="I40" t="s">
@@ -3014,7 +3040,7 @@
       <c r="U40" t="s">
         <v>91</v>
       </c>
-      <c r="V40" s="1">
+      <c r="V40" s="2">
         <v>46229</v>
       </c>
     </row>
@@ -3040,7 +3066,7 @@
       <c r="G41" t="s">
         <v>106</v>
       </c>
-      <c r="H41" s="1">
+      <c r="H41" s="2">
         <v>46244</v>
       </c>
       <c r="I41" t="s">
@@ -3070,7 +3096,7 @@
       <c r="U41" t="s">
         <v>91</v>
       </c>
-      <c r="V41" s="1">
+      <c r="V41" s="2">
         <v>46199</v>
       </c>
     </row>
@@ -3114,7 +3140,7 @@
       <c r="U42" t="s">
         <v>91</v>
       </c>
-      <c r="V42" s="1">
+      <c r="V42" s="2">
         <v>46260</v>
       </c>
     </row>
@@ -3140,7 +3166,7 @@
       <c r="G43" t="s">
         <v>106</v>
       </c>
-      <c r="H43" s="1">
+      <c r="H43" s="2">
         <v>46191</v>
       </c>
       <c r="I43" t="s">
@@ -3170,7 +3196,7 @@
       <c r="U43" t="s">
         <v>91</v>
       </c>
-      <c r="V43" s="1">
+      <c r="V43" s="2">
         <v>46199</v>
       </c>
     </row>
@@ -3196,7 +3222,7 @@
       <c r="G44" t="s">
         <v>106</v>
       </c>
-      <c r="H44" s="1">
+      <c r="H44" s="2">
         <v>46191</v>
       </c>
       <c r="I44" t="s">
@@ -3226,7 +3252,7 @@
       <c r="U44" t="s">
         <v>91</v>
       </c>
-      <c r="V44" s="1">
+      <c r="V44" s="2">
         <v>46199</v>
       </c>
     </row>
@@ -3252,7 +3278,7 @@
       <c r="G45" t="s">
         <v>106</v>
       </c>
-      <c r="H45" s="1">
+      <c r="H45" s="2">
         <v>46213</v>
       </c>
       <c r="I45" t="s">
@@ -3285,7 +3311,7 @@
       <c r="U45" t="s">
         <v>171</v>
       </c>
-      <c r="V45" s="1">
+      <c r="V45" s="2">
         <v>46229</v>
       </c>
     </row>
@@ -3311,7 +3337,7 @@
       <c r="G46" t="s">
         <v>106</v>
       </c>
-      <c r="H46" s="1">
+      <c r="H46" s="2">
         <v>46210</v>
       </c>
       <c r="I46" t="s">
@@ -3341,7 +3367,7 @@
       <c r="U46" t="s">
         <v>171</v>
       </c>
-      <c r="V46" s="1">
+      <c r="V46" s="2">
         <v>46229</v>
       </c>
     </row>
@@ -3388,7 +3414,7 @@
       <c r="U47" t="s">
         <v>91</v>
       </c>
-      <c r="V47" s="1">
+      <c r="V47" s="2">
         <v>46321</v>
       </c>
     </row>
@@ -3441,7 +3467,7 @@
       <c r="U48" t="s">
         <v>171</v>
       </c>
-      <c r="V48" s="1">
+      <c r="V48" s="2">
         <v>46291</v>
       </c>
     </row>
@@ -3467,7 +3493,7 @@
       <c r="G49" t="s">
         <v>106</v>
       </c>
-      <c r="H49" s="1">
+      <c r="H49" s="2">
         <v>46176</v>
       </c>
       <c r="I49" t="s">
@@ -3500,7 +3526,7 @@
       <c r="U49" t="s">
         <v>171</v>
       </c>
-      <c r="V49" s="1">
+      <c r="V49" s="2">
         <v>46199</v>
       </c>
     </row>
@@ -3553,7 +3579,7 @@
       <c r="U50" t="s">
         <v>171</v>
       </c>
-      <c r="V50" s="1">
+      <c r="V50" s="2">
         <v>46260</v>
       </c>
     </row>
@@ -3579,7 +3605,7 @@
       <c r="G51" t="s">
         <v>106</v>
       </c>
-      <c r="H51" s="1">
+      <c r="H51" s="2">
         <v>46295</v>
       </c>
       <c r="I51" t="s">
@@ -3615,7 +3641,7 @@
       <c r="U51" t="s">
         <v>171</v>
       </c>
-      <c r="V51" s="1">
+      <c r="V51" s="2">
         <v>46291</v>
       </c>
     </row>
@@ -3665,7 +3691,7 @@
       <c r="U52" t="s">
         <v>171</v>
       </c>
-      <c r="V52" s="1">
+      <c r="V52" s="2">
         <v>46321</v>
       </c>
     </row>
@@ -3691,7 +3717,7 @@
       <c r="G53" t="s">
         <v>106</v>
       </c>
-      <c r="H53" s="1">
+      <c r="H53" s="2">
         <v>46227</v>
       </c>
       <c r="I53" t="s">
@@ -3721,7 +3747,7 @@
       <c r="U53" t="s">
         <v>171</v>
       </c>
-      <c r="V53" s="1">
+      <c r="V53" s="2">
         <v>46229</v>
       </c>
     </row>
@@ -3744,7 +3770,7 @@
       <c r="G54" t="s">
         <v>106</v>
       </c>
-      <c r="H54" s="1">
+      <c r="H54" s="2">
         <v>46280</v>
       </c>
       <c r="I54" t="s">
@@ -3774,7 +3800,7 @@
       <c r="U54" t="s">
         <v>171</v>
       </c>
-      <c r="V54" s="1">
+      <c r="V54" s="2">
         <v>46291</v>
       </c>
     </row>
@@ -3797,7 +3823,7 @@
       <c r="G55" t="s">
         <v>106</v>
       </c>
-      <c r="H55" s="1">
+      <c r="H55" s="2">
         <v>46280</v>
       </c>
       <c r="I55" t="s">
@@ -3827,7 +3853,7 @@
       <c r="U55" t="s">
         <v>171</v>
       </c>
-      <c r="V55" s="1">
+      <c r="V55" s="2">
         <v>46260</v>
       </c>
     </row>
@@ -3850,7 +3876,7 @@
       <c r="G56" t="s">
         <v>106</v>
       </c>
-      <c r="H56" s="1">
+      <c r="H56" s="2">
         <v>46295</v>
       </c>
       <c r="I56" t="s">
@@ -3880,7 +3906,7 @@
       <c r="U56" t="s">
         <v>171</v>
       </c>
-      <c r="V56" s="1">
+      <c r="V56" s="2">
         <v>46291</v>
       </c>
     </row>
@@ -3903,7 +3929,7 @@
       <c r="G57" t="s">
         <v>106</v>
       </c>
-      <c r="H57" s="1">
+      <c r="H57" s="2">
         <v>46295</v>
       </c>
       <c r="I57" t="s">
@@ -3933,7 +3959,7 @@
       <c r="U57" t="s">
         <v>171</v>
       </c>
-      <c r="V57" s="1">
+      <c r="V57" s="2">
         <v>46291</v>
       </c>
     </row>
@@ -3986,7 +4012,7 @@
       <c r="U58" t="s">
         <v>171</v>
       </c>
-      <c r="V58" s="1">
+      <c r="V58" s="2">
         <v>46352</v>
       </c>
     </row>
@@ -4030,7 +4056,7 @@
       <c r="U59" t="s">
         <v>171</v>
       </c>
-      <c r="V59" s="1">
+      <c r="V59" s="2">
         <v>46107</v>
       </c>
     </row>
@@ -4074,7 +4100,7 @@
       <c r="U60" t="s">
         <v>171</v>
       </c>
-      <c r="V60" s="1">
+      <c r="V60" s="2">
         <v>46107</v>
       </c>
     </row>
@@ -4118,7 +4144,7 @@
       <c r="U61" t="s">
         <v>171</v>
       </c>
-      <c r="V61" s="1">
+      <c r="V61" s="2">
         <v>46107</v>
       </c>
     </row>
@@ -4162,7 +4188,7 @@
       <c r="U62" t="s">
         <v>171</v>
       </c>
-      <c r="V62" s="1">
+      <c r="V62" s="2">
         <v>46107</v>
       </c>
     </row>
@@ -4206,7 +4232,7 @@
       <c r="U63" t="s">
         <v>171</v>
       </c>
-      <c r="V63" s="1">
+      <c r="V63" s="2">
         <v>46107</v>
       </c>
     </row>
@@ -4250,7 +4276,7 @@
       <c r="U64" t="s">
         <v>171</v>
       </c>
-      <c r="V64" s="1">
+      <c r="V64" s="2">
         <v>46107</v>
       </c>
     </row>
@@ -4294,7 +4320,7 @@
       <c r="U65" t="s">
         <v>91</v>
       </c>
-      <c r="V65" s="1">
+      <c r="V65" s="2">
         <v>46168</v>
       </c>
     </row>
@@ -4341,7 +4367,7 @@
       <c r="U66" t="s">
         <v>91</v>
       </c>
-      <c r="V66" s="1">
+      <c r="V66" s="2">
         <v>46291</v>
       </c>
     </row>
@@ -4394,7 +4420,7 @@
       <c r="U67" t="s">
         <v>171</v>
       </c>
-      <c r="V67" s="1">
+      <c r="V67" s="2">
         <v>46229</v>
       </c>
     </row>
@@ -4438,7 +4464,7 @@
       <c r="U68" t="s">
         <v>91</v>
       </c>
-      <c r="V68" s="1">
+      <c r="V68" s="2">
         <v>46260</v>
       </c>
     </row>
@@ -4482,7 +4508,7 @@
       <c r="U69" t="s">
         <v>171</v>
       </c>
-      <c r="V69" s="1">
+      <c r="V69" s="2">
         <v>46291</v>
       </c>
     </row>
@@ -4526,7 +4552,7 @@
       <c r="U70" t="s">
         <v>171</v>
       </c>
-      <c r="V70" s="1">
+      <c r="V70" s="2">
         <v>46168</v>
       </c>
     </row>
@@ -4570,7 +4596,7 @@
       <c r="U71" t="s">
         <v>171</v>
       </c>
-      <c r="V71" s="1">
+      <c r="V71" s="2">
         <v>46291</v>
       </c>
     </row>
@@ -4614,7 +4640,7 @@
       <c r="U72" t="s">
         <v>171</v>
       </c>
-      <c r="V72" s="1">
+      <c r="V72" s="2">
         <v>46291</v>
       </c>
     </row>
@@ -4658,7 +4684,7 @@
       <c r="U73" t="s">
         <v>171</v>
       </c>
-      <c r="V73" s="1">
+      <c r="V73" s="2">
         <v>46291</v>
       </c>
     </row>
@@ -4705,7 +4731,7 @@
       <c r="U74" t="s">
         <v>91</v>
       </c>
-      <c r="V74" s="1">
+      <c r="V74" s="2">
         <v>46321</v>
       </c>
     </row>
@@ -4755,7 +4781,7 @@
       <c r="U75" t="s">
         <v>171</v>
       </c>
-      <c r="V75" s="1">
+      <c r="V75" s="2">
         <v>46381</v>
       </c>
     </row>
@@ -4805,7 +4831,7 @@
       <c r="U76" t="s">
         <v>171</v>
       </c>
-      <c r="V76" s="1">
+      <c r="V76" s="2">
         <v>46381</v>
       </c>
     </row>
@@ -4855,7 +4881,7 @@
       <c r="U77" t="s">
         <v>91</v>
       </c>
-      <c r="V77" s="1">
+      <c r="V77" s="2">
         <v>46381</v>
       </c>
     </row>
@@ -4905,7 +4931,7 @@
       <c r="U78" t="s">
         <v>91</v>
       </c>
-      <c r="V78" s="1">
+      <c r="V78" s="2">
         <v>46381</v>
       </c>
     </row>
@@ -4955,7 +4981,7 @@
       <c r="U79" t="s">
         <v>91</v>
       </c>
-      <c r="V79" s="1">
+      <c r="V79" s="2">
         <v>46382</v>
       </c>
     </row>
@@ -4999,7 +5025,7 @@
       <c r="U80" t="s">
         <v>91</v>
       </c>
-      <c r="V80" s="1">
+      <c r="V80" s="2">
         <v>46382</v>
       </c>
     </row>
@@ -5052,7 +5078,7 @@
       <c r="U81" t="s">
         <v>171</v>
       </c>
-      <c r="V81" s="1">
+      <c r="V81" s="2">
         <v>46382</v>
       </c>
     </row>
@@ -5099,7 +5125,7 @@
       <c r="U82" t="s">
         <v>91</v>
       </c>
-      <c r="V82" s="1">
+      <c r="V82" s="2">
         <v>46321</v>
       </c>
     </row>
@@ -5143,7 +5169,7 @@
       <c r="U83" t="s">
         <v>91</v>
       </c>
-      <c r="V83" s="1">
+      <c r="V83" s="2">
         <v>46382</v>
       </c>
     </row>
@@ -5284,7 +5310,7 @@
       <c r="U86" t="s">
         <v>91</v>
       </c>
-      <c r="V86" s="1">
+      <c r="V86" s="2">
         <v>46291</v>
       </c>
     </row>
@@ -5328,7 +5354,7 @@
       <c r="U87" t="s">
         <v>91</v>
       </c>
-      <c r="V87" s="1">
+      <c r="V87" s="2">
         <v>46291</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Atualização automática: mta (06/10/2026 13:46)
</commit_message>
<xml_diff>
--- a/Projetos/02_Dados_Tratados/base_mta_tratada.xlsx
+++ b/Projetos/02_Dados_Tratados/base_mta_tratada.xlsx
@@ -14,7 +14,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1154" uniqueCount="172">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1156" uniqueCount="173">
   <si>
     <t>linha</t>
   </si>
@@ -406,6 +406,9 @@
     <t>email do dia 19/06</t>
   </si>
   <si>
+    <t>2026-10-05 00:00:00</t>
+  </si>
+  <si>
     <t>email do dia 25/05</t>
   </si>
   <si>
@@ -424,7 +427,7 @@
     <t>ATENDER</t>
   </si>
   <si>
-    <t>REMANEJAR</t>
+    <t>Atender. Alterar a UGE para CABW. Alterar a atividade para "Requisição CABW". Alterar a tarefa para "Requisições Consumíveis". Alterar a ND para 339030.</t>
   </si>
   <si>
     <t>Atender SET</t>
@@ -985,13 +988,13 @@
         <v>126</v>
       </c>
       <c r="K2" t="s">
-        <v>134</v>
+        <v>135</v>
       </c>
       <c r="L2" t="s">
-        <v>140</v>
+        <v>141</v>
       </c>
       <c r="N2" t="s">
-        <v>141</v>
+        <v>142</v>
       </c>
       <c r="O2" t="s">
         <v>23</v>
@@ -1000,19 +1003,19 @@
         <v>135000</v>
       </c>
       <c r="Q2" t="s">
-        <v>159</v>
+        <v>160</v>
       </c>
       <c r="R2" t="s">
-        <v>162</v>
+        <v>163</v>
       </c>
       <c r="S2" t="s">
-        <v>165</v>
+        <v>166</v>
       </c>
       <c r="T2" t="s">
-        <v>167</v>
+        <v>168</v>
       </c>
       <c r="U2" t="s">
-        <v>171</v>
+        <v>172</v>
       </c>
       <c r="V2" s="2">
         <v>46229</v>
@@ -1041,22 +1044,22 @@
         <v>105</v>
       </c>
       <c r="N3" t="s">
-        <v>141</v>
+        <v>142</v>
       </c>
       <c r="O3" t="s">
         <v>24</v>
       </c>
       <c r="Q3" t="s">
-        <v>159</v>
+        <v>160</v>
       </c>
       <c r="R3" t="s">
-        <v>162</v>
+        <v>163</v>
       </c>
       <c r="S3" t="s">
-        <v>165</v>
+        <v>166</v>
       </c>
       <c r="T3" t="s">
-        <v>167</v>
+        <v>168</v>
       </c>
       <c r="U3" t="s">
         <v>91</v>
@@ -1088,22 +1091,22 @@
         <v>105</v>
       </c>
       <c r="N4" t="s">
-        <v>142</v>
+        <v>143</v>
       </c>
       <c r="O4" t="s">
         <v>25</v>
       </c>
       <c r="Q4" t="s">
-        <v>159</v>
+        <v>160</v>
       </c>
       <c r="R4" t="s">
-        <v>163</v>
+        <v>164</v>
       </c>
       <c r="S4" t="s">
-        <v>165</v>
+        <v>166</v>
       </c>
       <c r="T4" t="s">
-        <v>167</v>
+        <v>168</v>
       </c>
       <c r="U4" t="s">
         <v>91</v>
@@ -1135,22 +1138,22 @@
         <v>105</v>
       </c>
       <c r="N5" t="s">
-        <v>142</v>
+        <v>143</v>
       </c>
       <c r="O5" t="s">
         <v>26</v>
       </c>
       <c r="Q5" t="s">
-        <v>159</v>
+        <v>160</v>
       </c>
       <c r="R5" t="s">
-        <v>163</v>
+        <v>164</v>
       </c>
       <c r="S5" t="s">
-        <v>165</v>
+        <v>166</v>
       </c>
       <c r="T5" t="s">
-        <v>167</v>
+        <v>168</v>
       </c>
       <c r="U5" t="s">
         <v>91</v>
@@ -1182,25 +1185,25 @@
         <v>105</v>
       </c>
       <c r="L6" t="s">
-        <v>140</v>
+        <v>141</v>
       </c>
       <c r="N6" t="s">
-        <v>143</v>
+        <v>144</v>
       </c>
       <c r="O6" t="s">
         <v>27</v>
       </c>
       <c r="Q6" t="s">
-        <v>159</v>
+        <v>160</v>
       </c>
       <c r="R6" t="s">
-        <v>163</v>
+        <v>164</v>
       </c>
       <c r="S6" t="s">
-        <v>165</v>
+        <v>166</v>
       </c>
       <c r="T6" t="s">
-        <v>167</v>
+        <v>168</v>
       </c>
       <c r="U6" t="s">
         <v>91</v>
@@ -1238,7 +1241,7 @@
         <v>108</v>
       </c>
       <c r="N7" t="s">
-        <v>144</v>
+        <v>145</v>
       </c>
       <c r="O7" t="s">
         <v>28</v>
@@ -1247,16 +1250,16 @@
         <v>3799999.6</v>
       </c>
       <c r="Q7" t="s">
-        <v>160</v>
+        <v>161</v>
       </c>
       <c r="R7" t="s">
-        <v>163</v>
+        <v>164</v>
       </c>
       <c r="S7" t="s">
-        <v>165</v>
+        <v>166</v>
       </c>
       <c r="T7" t="s">
-        <v>168</v>
+        <v>169</v>
       </c>
       <c r="U7" t="s">
         <v>91</v>
@@ -1288,22 +1291,22 @@
         <v>105</v>
       </c>
       <c r="N8" t="s">
-        <v>142</v>
+        <v>143</v>
       </c>
       <c r="O8" t="s">
         <v>29</v>
       </c>
       <c r="Q8" t="s">
-        <v>159</v>
+        <v>160</v>
       </c>
       <c r="R8" t="s">
-        <v>163</v>
+        <v>164</v>
       </c>
       <c r="S8" t="s">
-        <v>165</v>
+        <v>166</v>
       </c>
       <c r="T8" t="s">
-        <v>167</v>
+        <v>168</v>
       </c>
       <c r="U8" t="s">
         <v>91</v>
@@ -1332,7 +1335,7 @@
         <v>93</v>
       </c>
       <c r="N9" t="s">
-        <v>142</v>
+        <v>143</v>
       </c>
       <c r="O9" t="s">
         <v>30</v>
@@ -1341,16 +1344,16 @@
         <v>60000</v>
       </c>
       <c r="Q9" t="s">
-        <v>159</v>
+        <v>160</v>
       </c>
       <c r="R9" t="s">
-        <v>163</v>
+        <v>164</v>
       </c>
       <c r="S9" t="s">
-        <v>165</v>
+        <v>166</v>
       </c>
       <c r="T9" t="s">
-        <v>167</v>
+        <v>168</v>
       </c>
       <c r="U9" t="s">
         <v>91</v>
@@ -1382,22 +1385,22 @@
         <v>105</v>
       </c>
       <c r="N10" t="s">
-        <v>143</v>
+        <v>144</v>
       </c>
       <c r="O10" t="s">
         <v>31</v>
       </c>
       <c r="Q10" t="s">
-        <v>159</v>
+        <v>160</v>
       </c>
       <c r="R10" t="s">
-        <v>163</v>
+        <v>164</v>
       </c>
       <c r="S10" t="s">
-        <v>165</v>
+        <v>166</v>
       </c>
       <c r="T10" t="s">
-        <v>167</v>
+        <v>168</v>
       </c>
       <c r="U10" t="s">
         <v>91</v>
@@ -1429,22 +1432,22 @@
         <v>105</v>
       </c>
       <c r="N11" t="s">
-        <v>143</v>
+        <v>144</v>
       </c>
       <c r="O11" t="s">
         <v>32</v>
       </c>
       <c r="Q11" t="s">
-        <v>159</v>
+        <v>160</v>
       </c>
       <c r="R11" t="s">
-        <v>163</v>
+        <v>164</v>
       </c>
       <c r="S11" t="s">
-        <v>165</v>
+        <v>166</v>
       </c>
       <c r="T11" t="s">
-        <v>167</v>
+        <v>168</v>
       </c>
       <c r="U11" t="s">
         <v>91</v>
@@ -1485,7 +1488,7 @@
         <v>127</v>
       </c>
       <c r="N12" t="s">
-        <v>141</v>
+        <v>142</v>
       </c>
       <c r="O12" t="s">
         <v>33</v>
@@ -1494,19 +1497,19 @@
         <v>1187433.02</v>
       </c>
       <c r="Q12" t="s">
-        <v>159</v>
+        <v>160</v>
       </c>
       <c r="R12" t="s">
-        <v>162</v>
+        <v>163</v>
       </c>
       <c r="S12" t="s">
-        <v>165</v>
+        <v>166</v>
       </c>
       <c r="T12" t="s">
-        <v>167</v>
+        <v>168</v>
       </c>
       <c r="U12" t="s">
-        <v>171</v>
+        <v>172</v>
       </c>
       <c r="V12" s="2">
         <v>46079</v>
@@ -1535,10 +1538,10 @@
         <v>126</v>
       </c>
       <c r="K13" t="s">
-        <v>135</v>
+        <v>136</v>
       </c>
       <c r="N13" t="s">
-        <v>141</v>
+        <v>142</v>
       </c>
       <c r="O13" t="s">
         <v>34</v>
@@ -1547,19 +1550,19 @@
         <v>1000000</v>
       </c>
       <c r="Q13" t="s">
-        <v>159</v>
+        <v>160</v>
       </c>
       <c r="R13" t="s">
-        <v>162</v>
+        <v>163</v>
       </c>
       <c r="S13" t="s">
-        <v>165</v>
+        <v>166</v>
       </c>
       <c r="T13" t="s">
-        <v>167</v>
+        <v>168</v>
       </c>
       <c r="U13" t="s">
-        <v>171</v>
+        <v>172</v>
       </c>
       <c r="V13" s="2">
         <v>46352</v>
@@ -1588,10 +1591,10 @@
         <v>126</v>
       </c>
       <c r="K14" t="s">
-        <v>135</v>
+        <v>136</v>
       </c>
       <c r="N14" t="s">
-        <v>141</v>
+        <v>142</v>
       </c>
       <c r="O14" t="s">
         <v>35</v>
@@ -1600,19 +1603,19 @@
         <v>1000000</v>
       </c>
       <c r="Q14" t="s">
-        <v>159</v>
+        <v>160</v>
       </c>
       <c r="R14" t="s">
-        <v>162</v>
+        <v>163</v>
       </c>
       <c r="S14" t="s">
-        <v>165</v>
+        <v>166</v>
       </c>
       <c r="T14" t="s">
-        <v>167</v>
+        <v>168</v>
       </c>
       <c r="U14" t="s">
-        <v>171</v>
+        <v>172</v>
       </c>
       <c r="V14" s="2">
         <v>46352</v>
@@ -1641,10 +1644,10 @@
         <v>126</v>
       </c>
       <c r="K15" t="s">
-        <v>135</v>
+        <v>136</v>
       </c>
       <c r="N15" t="s">
-        <v>141</v>
+        <v>142</v>
       </c>
       <c r="O15" t="s">
         <v>36</v>
@@ -1653,19 +1656,19 @@
         <v>1000000</v>
       </c>
       <c r="Q15" t="s">
-        <v>159</v>
+        <v>160</v>
       </c>
       <c r="R15" t="s">
-        <v>162</v>
+        <v>163</v>
       </c>
       <c r="S15" t="s">
-        <v>165</v>
+        <v>166</v>
       </c>
       <c r="T15" t="s">
-        <v>167</v>
+        <v>168</v>
       </c>
       <c r="U15" t="s">
-        <v>171</v>
+        <v>172</v>
       </c>
       <c r="V15" s="2">
         <v>46352</v>
@@ -1694,10 +1697,10 @@
         <v>126</v>
       </c>
       <c r="K16" t="s">
-        <v>135</v>
+        <v>136</v>
       </c>
       <c r="N16" t="s">
-        <v>145</v>
+        <v>146</v>
       </c>
       <c r="O16" t="s">
         <v>37</v>
@@ -1706,19 +1709,19 @@
         <v>100000</v>
       </c>
       <c r="Q16" t="s">
-        <v>161</v>
+        <v>162</v>
       </c>
       <c r="R16" t="s">
-        <v>162</v>
+        <v>163</v>
       </c>
       <c r="S16" t="s">
-        <v>165</v>
+        <v>166</v>
       </c>
       <c r="T16" t="s">
-        <v>167</v>
+        <v>168</v>
       </c>
       <c r="U16" t="s">
-        <v>171</v>
+        <v>172</v>
       </c>
       <c r="V16" s="2">
         <v>46229</v>
@@ -1756,7 +1759,7 @@
         <v>127</v>
       </c>
       <c r="N17" t="s">
-        <v>146</v>
+        <v>147</v>
       </c>
       <c r="O17" t="s">
         <v>38</v>
@@ -1765,19 +1768,19 @@
         <v>1770880.5</v>
       </c>
       <c r="Q17" t="s">
-        <v>160</v>
+        <v>161</v>
       </c>
       <c r="R17" t="s">
-        <v>163</v>
+        <v>164</v>
       </c>
       <c r="S17" t="s">
-        <v>165</v>
+        <v>166</v>
       </c>
       <c r="T17" t="s">
-        <v>169</v>
+        <v>170</v>
       </c>
       <c r="U17" t="s">
-        <v>171</v>
+        <v>172</v>
       </c>
       <c r="V17" s="2">
         <v>46107</v>
@@ -1812,7 +1815,7 @@
         <v>111</v>
       </c>
       <c r="N18" t="s">
-        <v>147</v>
+        <v>148</v>
       </c>
       <c r="O18" t="s">
         <v>39</v>
@@ -1821,16 +1824,16 @@
         <v>350000</v>
       </c>
       <c r="Q18" t="s">
-        <v>160</v>
+        <v>161</v>
       </c>
       <c r="R18" t="s">
-        <v>162</v>
+        <v>163</v>
       </c>
       <c r="S18" t="s">
-        <v>165</v>
+        <v>166</v>
       </c>
       <c r="T18" t="s">
-        <v>168</v>
+        <v>169</v>
       </c>
       <c r="U18" t="s">
         <v>91</v>
@@ -1868,7 +1871,7 @@
         <v>111</v>
       </c>
       <c r="N19" t="s">
-        <v>147</v>
+        <v>148</v>
       </c>
       <c r="O19" t="s">
         <v>40</v>
@@ -1877,16 +1880,16 @@
         <v>350000</v>
       </c>
       <c r="Q19" t="s">
-        <v>160</v>
+        <v>161</v>
       </c>
       <c r="R19" t="s">
-        <v>162</v>
+        <v>163</v>
       </c>
       <c r="S19" t="s">
-        <v>165</v>
+        <v>166</v>
       </c>
       <c r="T19" t="s">
-        <v>168</v>
+        <v>169</v>
       </c>
       <c r="U19" t="s">
         <v>91</v>
@@ -1915,7 +1918,7 @@
         <v>93</v>
       </c>
       <c r="N20" t="s">
-        <v>148</v>
+        <v>149</v>
       </c>
       <c r="O20" t="s">
         <v>41</v>
@@ -1924,16 +1927,16 @@
         <v>1000000</v>
       </c>
       <c r="Q20" t="s">
-        <v>160</v>
+        <v>161</v>
       </c>
       <c r="R20" t="s">
-        <v>162</v>
+        <v>163</v>
       </c>
       <c r="S20" t="s">
-        <v>165</v>
+        <v>166</v>
       </c>
       <c r="T20" t="s">
-        <v>168</v>
+        <v>169</v>
       </c>
       <c r="U20" t="s">
         <v>91</v>
@@ -1965,22 +1968,22 @@
         <v>105</v>
       </c>
       <c r="N21" t="s">
-        <v>141</v>
+        <v>142</v>
       </c>
       <c r="O21" t="s">
         <v>42</v>
       </c>
       <c r="Q21" t="s">
-        <v>159</v>
+        <v>160</v>
       </c>
       <c r="R21" t="s">
-        <v>162</v>
+        <v>163</v>
       </c>
       <c r="S21" t="s">
-        <v>165</v>
+        <v>166</v>
       </c>
       <c r="T21" t="s">
-        <v>167</v>
+        <v>168</v>
       </c>
       <c r="U21" t="s">
         <v>91</v>
@@ -2012,22 +2015,22 @@
         <v>105</v>
       </c>
       <c r="N22" t="s">
-        <v>142</v>
+        <v>143</v>
       </c>
       <c r="O22" t="s">
         <v>43</v>
       </c>
       <c r="Q22" t="s">
-        <v>159</v>
+        <v>160</v>
       </c>
       <c r="R22" t="s">
-        <v>163</v>
+        <v>164</v>
       </c>
       <c r="S22" t="s">
-        <v>165</v>
+        <v>166</v>
       </c>
       <c r="T22" t="s">
-        <v>167</v>
+        <v>168</v>
       </c>
       <c r="U22" t="s">
         <v>91</v>
@@ -2059,22 +2062,22 @@
         <v>105</v>
       </c>
       <c r="N23" t="s">
-        <v>142</v>
+        <v>143</v>
       </c>
       <c r="O23" t="s">
         <v>44</v>
       </c>
       <c r="Q23" t="s">
-        <v>159</v>
+        <v>160</v>
       </c>
       <c r="R23" t="s">
-        <v>163</v>
+        <v>164</v>
       </c>
       <c r="S23" t="s">
-        <v>165</v>
+        <v>166</v>
       </c>
       <c r="T23" t="s">
-        <v>167</v>
+        <v>168</v>
       </c>
       <c r="U23" t="s">
         <v>91</v>
@@ -2115,7 +2118,7 @@
         <v>128</v>
       </c>
       <c r="N24" t="s">
-        <v>146</v>
+        <v>147</v>
       </c>
       <c r="O24" t="s">
         <v>45</v>
@@ -2124,19 +2127,19 @@
         <v>1704503</v>
       </c>
       <c r="Q24" t="s">
-        <v>160</v>
+        <v>161</v>
       </c>
       <c r="R24" t="s">
-        <v>163</v>
+        <v>164</v>
       </c>
       <c r="S24" t="s">
-        <v>165</v>
+        <v>166</v>
       </c>
       <c r="T24" t="s">
-        <v>169</v>
+        <v>170</v>
       </c>
       <c r="U24" t="s">
-        <v>171</v>
+        <v>172</v>
       </c>
       <c r="V24" s="2">
         <v>46138</v>
@@ -2171,7 +2174,7 @@
         <v>113</v>
       </c>
       <c r="N25" t="s">
-        <v>149</v>
+        <v>150</v>
       </c>
       <c r="O25" t="s">
         <v>46</v>
@@ -2180,16 +2183,16 @@
         <v>3799000</v>
       </c>
       <c r="Q25" t="s">
-        <v>160</v>
+        <v>161</v>
       </c>
       <c r="R25" t="s">
-        <v>163</v>
+        <v>164</v>
       </c>
       <c r="S25" t="s">
-        <v>165</v>
+        <v>166</v>
       </c>
       <c r="T25" t="s">
-        <v>168</v>
+        <v>169</v>
       </c>
       <c r="U25" t="s">
         <v>91</v>
@@ -2227,7 +2230,7 @@
         <v>114</v>
       </c>
       <c r="N26" t="s">
-        <v>149</v>
+        <v>150</v>
       </c>
       <c r="O26" t="s">
         <v>46</v>
@@ -2236,16 +2239,16 @@
         <v>1000</v>
       </c>
       <c r="Q26" t="s">
-        <v>160</v>
+        <v>161</v>
       </c>
       <c r="R26" t="s">
-        <v>162</v>
+        <v>163</v>
       </c>
       <c r="S26" t="s">
-        <v>165</v>
+        <v>166</v>
       </c>
       <c r="T26" t="s">
-        <v>168</v>
+        <v>169</v>
       </c>
       <c r="U26" t="s">
         <v>91</v>
@@ -2277,10 +2280,10 @@
         <v>126</v>
       </c>
       <c r="K27" t="s">
-        <v>135</v>
+        <v>136</v>
       </c>
       <c r="N27" t="s">
-        <v>145</v>
+        <v>146</v>
       </c>
       <c r="O27" t="s">
         <v>47</v>
@@ -2289,19 +2292,19 @@
         <v>100000</v>
       </c>
       <c r="Q27" t="s">
-        <v>161</v>
+        <v>162</v>
       </c>
       <c r="R27" t="s">
-        <v>162</v>
+        <v>163</v>
       </c>
       <c r="S27" t="s">
-        <v>165</v>
+        <v>166</v>
       </c>
       <c r="T27" t="s">
-        <v>167</v>
+        <v>168</v>
       </c>
       <c r="U27" t="s">
-        <v>171</v>
+        <v>172</v>
       </c>
       <c r="V27" s="2">
         <v>46291</v>
@@ -2339,7 +2342,7 @@
         <v>129</v>
       </c>
       <c r="N28" t="s">
-        <v>146</v>
+        <v>147</v>
       </c>
       <c r="O28" t="s">
         <v>48</v>
@@ -2348,19 +2351,19 @@
         <v>150000</v>
       </c>
       <c r="Q28" t="s">
-        <v>160</v>
+        <v>161</v>
       </c>
       <c r="R28" t="s">
-        <v>163</v>
+        <v>164</v>
       </c>
       <c r="S28" t="s">
-        <v>165</v>
+        <v>166</v>
       </c>
       <c r="T28" t="s">
-        <v>168</v>
+        <v>169</v>
       </c>
       <c r="U28" t="s">
-        <v>171</v>
+        <v>172</v>
       </c>
       <c r="V28" s="2">
         <v>46199</v>
@@ -2398,7 +2401,7 @@
         <v>129</v>
       </c>
       <c r="N29" t="s">
-        <v>146</v>
+        <v>147</v>
       </c>
       <c r="O29" t="s">
         <v>49</v>
@@ -2407,19 +2410,19 @@
         <v>150000</v>
       </c>
       <c r="Q29" t="s">
-        <v>160</v>
+        <v>161</v>
       </c>
       <c r="R29" t="s">
-        <v>163</v>
+        <v>164</v>
       </c>
       <c r="S29" t="s">
-        <v>165</v>
+        <v>166</v>
       </c>
       <c r="T29" t="s">
-        <v>168</v>
+        <v>169</v>
       </c>
       <c r="U29" t="s">
-        <v>171</v>
+        <v>172</v>
       </c>
       <c r="V29" s="2">
         <v>46199</v>
@@ -2457,7 +2460,7 @@
         <v>129</v>
       </c>
       <c r="N30" t="s">
-        <v>146</v>
+        <v>147</v>
       </c>
       <c r="O30" t="s">
         <v>50</v>
@@ -2466,19 +2469,19 @@
         <v>18462.36</v>
       </c>
       <c r="Q30" t="s">
-        <v>160</v>
+        <v>161</v>
       </c>
       <c r="R30" t="s">
-        <v>163</v>
+        <v>164</v>
       </c>
       <c r="S30" t="s">
-        <v>165</v>
+        <v>166</v>
       </c>
       <c r="T30" t="s">
-        <v>168</v>
+        <v>169</v>
       </c>
       <c r="U30" t="s">
-        <v>171</v>
+        <v>172</v>
       </c>
       <c r="V30" s="2">
         <v>46199</v>
@@ -2516,7 +2519,7 @@
         <v>129</v>
       </c>
       <c r="N31" t="s">
-        <v>146</v>
+        <v>147</v>
       </c>
       <c r="O31" t="s">
         <v>50</v>
@@ -2525,19 +2528,19 @@
         <v>324166.14</v>
       </c>
       <c r="Q31" t="s">
-        <v>160</v>
+        <v>161</v>
       </c>
       <c r="R31" t="s">
-        <v>163</v>
+        <v>164</v>
       </c>
       <c r="S31" t="s">
-        <v>165</v>
+        <v>166</v>
       </c>
       <c r="T31" t="s">
-        <v>168</v>
+        <v>169</v>
       </c>
       <c r="U31" t="s">
-        <v>171</v>
+        <v>172</v>
       </c>
       <c r="V31" s="2">
         <v>46199</v>
@@ -2562,11 +2565,14 @@
       <c r="F32" t="s">
         <v>93</v>
       </c>
+      <c r="J32" t="s">
+        <v>130</v>
+      </c>
       <c r="K32" t="s">
-        <v>136</v>
+        <v>137</v>
       </c>
       <c r="N32" t="s">
-        <v>146</v>
+        <v>147</v>
       </c>
       <c r="O32" t="s">
         <v>51</v>
@@ -2575,19 +2581,19 @@
         <v>30000</v>
       </c>
       <c r="Q32" t="s">
-        <v>160</v>
+        <v>161</v>
       </c>
       <c r="R32" t="s">
-        <v>163</v>
+        <v>164</v>
       </c>
       <c r="S32" t="s">
-        <v>165</v>
+        <v>166</v>
       </c>
       <c r="T32" t="s">
-        <v>168</v>
+        <v>169</v>
       </c>
       <c r="U32" t="s">
-        <v>171</v>
+        <v>172</v>
       </c>
       <c r="V32" s="2">
         <v>46291</v>
@@ -2622,10 +2628,10 @@
         <v>117</v>
       </c>
       <c r="J33" t="s">
-        <v>130</v>
+        <v>131</v>
       </c>
       <c r="N33" t="s">
-        <v>146</v>
+        <v>147</v>
       </c>
       <c r="O33" t="s">
         <v>52</v>
@@ -2634,19 +2640,19 @@
         <v>1496713.48</v>
       </c>
       <c r="Q33" t="s">
-        <v>160</v>
+        <v>161</v>
       </c>
       <c r="R33" t="s">
-        <v>163</v>
+        <v>164</v>
       </c>
       <c r="S33" t="s">
-        <v>165</v>
+        <v>166</v>
       </c>
       <c r="T33" t="s">
-        <v>169</v>
+        <v>170</v>
       </c>
       <c r="U33" t="s">
-        <v>171</v>
+        <v>172</v>
       </c>
       <c r="V33" s="2">
         <v>46199</v>
@@ -2681,7 +2687,7 @@
         <v>112</v>
       </c>
       <c r="N34" t="s">
-        <v>146</v>
+        <v>147</v>
       </c>
       <c r="O34" t="s">
         <v>52</v>
@@ -2690,19 +2696,19 @@
         <v>207789.52</v>
       </c>
       <c r="Q34" t="s">
-        <v>160</v>
+        <v>161</v>
       </c>
       <c r="R34" t="s">
-        <v>163</v>
+        <v>164</v>
       </c>
       <c r="S34" t="s">
-        <v>165</v>
+        <v>166</v>
       </c>
       <c r="T34" t="s">
-        <v>169</v>
+        <v>170</v>
       </c>
       <c r="U34" t="s">
-        <v>171</v>
+        <v>172</v>
       </c>
       <c r="V34" s="2">
         <v>46138</v>
@@ -2737,7 +2743,7 @@
         <v>118</v>
       </c>
       <c r="N35" t="s">
-        <v>149</v>
+        <v>150</v>
       </c>
       <c r="O35" t="s">
         <v>53</v>
@@ -2746,16 +2752,16 @@
         <v>962290.8</v>
       </c>
       <c r="Q35" t="s">
-        <v>160</v>
+        <v>161</v>
       </c>
       <c r="R35" t="s">
-        <v>162</v>
+        <v>163</v>
       </c>
       <c r="S35" t="s">
-        <v>165</v>
+        <v>166</v>
       </c>
       <c r="T35" t="s">
-        <v>168</v>
+        <v>169</v>
       </c>
       <c r="U35" t="s">
         <v>91</v>
@@ -2793,7 +2799,7 @@
         <v>119</v>
       </c>
       <c r="N36" t="s">
-        <v>149</v>
+        <v>150</v>
       </c>
       <c r="O36" t="s">
         <v>53</v>
@@ -2802,16 +2808,16 @@
         <v>798776.97</v>
       </c>
       <c r="Q36" t="s">
-        <v>160</v>
+        <v>161</v>
       </c>
       <c r="R36" t="s">
-        <v>163</v>
+        <v>164</v>
       </c>
       <c r="S36" t="s">
-        <v>165</v>
+        <v>166</v>
       </c>
       <c r="T36" t="s">
-        <v>168</v>
+        <v>169</v>
       </c>
       <c r="U36" t="s">
         <v>91</v>
@@ -2849,7 +2855,7 @@
         <v>118</v>
       </c>
       <c r="N37" t="s">
-        <v>149</v>
+        <v>150</v>
       </c>
       <c r="O37" t="s">
         <v>53</v>
@@ -2858,16 +2864,16 @@
         <v>1530656.62</v>
       </c>
       <c r="Q37" t="s">
-        <v>160</v>
+        <v>161</v>
       </c>
       <c r="R37" t="s">
-        <v>162</v>
+        <v>163</v>
       </c>
       <c r="S37" t="s">
-        <v>165</v>
+        <v>166</v>
       </c>
       <c r="T37" t="s">
-        <v>168</v>
+        <v>169</v>
       </c>
       <c r="U37" t="s">
         <v>91</v>
@@ -2905,7 +2911,7 @@
         <v>120</v>
       </c>
       <c r="N38" t="s">
-        <v>149</v>
+        <v>150</v>
       </c>
       <c r="O38" t="s">
         <v>53</v>
@@ -2914,16 +2920,16 @@
         <v>72958.08</v>
       </c>
       <c r="Q38" t="s">
-        <v>160</v>
+        <v>161</v>
       </c>
       <c r="R38" t="s">
-        <v>162</v>
+        <v>163</v>
       </c>
       <c r="S38" t="s">
-        <v>165</v>
+        <v>166</v>
       </c>
       <c r="T38" t="s">
-        <v>168</v>
+        <v>169</v>
       </c>
       <c r="U38" t="s">
         <v>91</v>
@@ -2961,7 +2967,7 @@
         <v>120</v>
       </c>
       <c r="N39" t="s">
-        <v>149</v>
+        <v>150</v>
       </c>
       <c r="O39" t="s">
         <v>53</v>
@@ -2970,16 +2976,16 @@
         <v>8916</v>
       </c>
       <c r="Q39" t="s">
-        <v>160</v>
+        <v>161</v>
       </c>
       <c r="R39" t="s">
-        <v>162</v>
+        <v>163</v>
       </c>
       <c r="S39" t="s">
-        <v>165</v>
+        <v>166</v>
       </c>
       <c r="T39" t="s">
-        <v>168</v>
+        <v>169</v>
       </c>
       <c r="U39" t="s">
         <v>91</v>
@@ -3017,7 +3023,7 @@
         <v>120</v>
       </c>
       <c r="N40" t="s">
-        <v>149</v>
+        <v>150</v>
       </c>
       <c r="O40" t="s">
         <v>53</v>
@@ -3026,16 +3032,16 @@
         <v>425178.5</v>
       </c>
       <c r="Q40" t="s">
-        <v>160</v>
+        <v>161</v>
       </c>
       <c r="R40" t="s">
-        <v>162</v>
+        <v>163</v>
       </c>
       <c r="S40" t="s">
-        <v>165</v>
+        <v>166</v>
       </c>
       <c r="T40" t="s">
-        <v>168</v>
+        <v>169</v>
       </c>
       <c r="U40" t="s">
         <v>91</v>
@@ -3073,7 +3079,7 @@
         <v>121</v>
       </c>
       <c r="N41" t="s">
-        <v>149</v>
+        <v>150</v>
       </c>
       <c r="O41" t="s">
         <v>53</v>
@@ -3082,16 +3088,16 @@
         <v>1223.03</v>
       </c>
       <c r="Q41" t="s">
-        <v>160</v>
+        <v>161</v>
       </c>
       <c r="R41" t="s">
-        <v>162</v>
+        <v>163</v>
       </c>
       <c r="S41" t="s">
-        <v>165</v>
+        <v>166</v>
       </c>
       <c r="T41" t="s">
-        <v>168</v>
+        <v>169</v>
       </c>
       <c r="U41" t="s">
         <v>91</v>
@@ -3120,22 +3126,22 @@
         <v>105</v>
       </c>
       <c r="N42" t="s">
-        <v>149</v>
+        <v>150</v>
       </c>
       <c r="O42" t="s">
         <v>54</v>
       </c>
       <c r="Q42" t="s">
-        <v>160</v>
+        <v>161</v>
       </c>
       <c r="R42" t="s">
-        <v>162</v>
+        <v>163</v>
       </c>
       <c r="S42" t="s">
-        <v>166</v>
+        <v>167</v>
       </c>
       <c r="T42" t="s">
-        <v>168</v>
+        <v>169</v>
       </c>
       <c r="U42" t="s">
         <v>91</v>
@@ -3173,7 +3179,7 @@
         <v>122</v>
       </c>
       <c r="N43" t="s">
-        <v>147</v>
+        <v>148</v>
       </c>
       <c r="O43" t="s">
         <v>55</v>
@@ -3182,16 +3188,16 @@
         <v>400000</v>
       </c>
       <c r="Q43" t="s">
-        <v>160</v>
+        <v>161</v>
       </c>
       <c r="R43" t="s">
-        <v>162</v>
+        <v>163</v>
       </c>
       <c r="S43" t="s">
-        <v>165</v>
+        <v>166</v>
       </c>
       <c r="T43" t="s">
-        <v>168</v>
+        <v>169</v>
       </c>
       <c r="U43" t="s">
         <v>91</v>
@@ -3229,7 +3235,7 @@
         <v>122</v>
       </c>
       <c r="N44" t="s">
-        <v>147</v>
+        <v>148</v>
       </c>
       <c r="O44" t="s">
         <v>56</v>
@@ -3238,16 +3244,16 @@
         <v>400000</v>
       </c>
       <c r="Q44" t="s">
-        <v>160</v>
+        <v>161</v>
       </c>
       <c r="R44" t="s">
-        <v>162</v>
+        <v>163</v>
       </c>
       <c r="S44" t="s">
-        <v>165</v>
+        <v>166</v>
       </c>
       <c r="T44" t="s">
-        <v>168</v>
+        <v>169</v>
       </c>
       <c r="U44" t="s">
         <v>91</v>
@@ -3285,10 +3291,10 @@
         <v>117</v>
       </c>
       <c r="J45" t="s">
-        <v>131</v>
+        <v>132</v>
       </c>
       <c r="N45" t="s">
-        <v>146</v>
+        <v>147</v>
       </c>
       <c r="O45" t="s">
         <v>57</v>
@@ -3297,19 +3303,19 @@
         <v>173846.38</v>
       </c>
       <c r="Q45" t="s">
-        <v>160</v>
+        <v>161</v>
       </c>
       <c r="R45" t="s">
-        <v>163</v>
+        <v>164</v>
       </c>
       <c r="S45" t="s">
-        <v>165</v>
+        <v>166</v>
       </c>
       <c r="T45" t="s">
-        <v>169</v>
+        <v>170</v>
       </c>
       <c r="U45" t="s">
-        <v>171</v>
+        <v>172</v>
       </c>
       <c r="V45" s="2">
         <v>46229</v>
@@ -3344,7 +3350,7 @@
         <v>116</v>
       </c>
       <c r="N46" t="s">
-        <v>146</v>
+        <v>147</v>
       </c>
       <c r="O46" t="s">
         <v>57</v>
@@ -3353,19 +3359,19 @@
         <v>1530656.62</v>
       </c>
       <c r="Q46" t="s">
-        <v>160</v>
+        <v>161</v>
       </c>
       <c r="R46" t="s">
-        <v>163</v>
+        <v>164</v>
       </c>
       <c r="S46" t="s">
-        <v>165</v>
+        <v>166</v>
       </c>
       <c r="T46" t="s">
-        <v>169</v>
+        <v>170</v>
       </c>
       <c r="U46" t="s">
-        <v>171</v>
+        <v>172</v>
       </c>
       <c r="V46" s="2">
         <v>46229</v>
@@ -3391,7 +3397,7 @@
         <v>93</v>
       </c>
       <c r="N47" t="s">
-        <v>148</v>
+        <v>149</v>
       </c>
       <c r="O47" t="s">
         <v>58</v>
@@ -3400,16 +3406,16 @@
         <v>1000000</v>
       </c>
       <c r="Q47" t="s">
-        <v>160</v>
+        <v>161</v>
       </c>
       <c r="R47" t="s">
-        <v>162</v>
+        <v>163</v>
       </c>
       <c r="S47" t="s">
-        <v>165</v>
+        <v>166</v>
       </c>
       <c r="T47" t="s">
-        <v>168</v>
+        <v>169</v>
       </c>
       <c r="U47" t="s">
         <v>91</v>
@@ -3441,10 +3447,10 @@
         <v>126</v>
       </c>
       <c r="K48" t="s">
-        <v>135</v>
+        <v>136</v>
       </c>
       <c r="N48" t="s">
-        <v>141</v>
+        <v>142</v>
       </c>
       <c r="O48" t="s">
         <v>59</v>
@@ -3453,19 +3459,19 @@
         <v>958040</v>
       </c>
       <c r="Q48" t="s">
-        <v>159</v>
+        <v>160</v>
       </c>
       <c r="R48" t="s">
-        <v>162</v>
+        <v>163</v>
       </c>
       <c r="S48" t="s">
-        <v>165</v>
+        <v>166</v>
       </c>
       <c r="T48" t="s">
-        <v>167</v>
+        <v>168</v>
       </c>
       <c r="U48" t="s">
-        <v>171</v>
+        <v>172</v>
       </c>
       <c r="V48" s="2">
         <v>46291</v>
@@ -3500,10 +3506,10 @@
         <v>123</v>
       </c>
       <c r="J49" t="s">
-        <v>132</v>
+        <v>133</v>
       </c>
       <c r="N49" t="s">
-        <v>141</v>
+        <v>142</v>
       </c>
       <c r="O49" t="s">
         <v>59</v>
@@ -3512,19 +3518,19 @@
         <v>41730.64</v>
       </c>
       <c r="Q49" t="s">
-        <v>159</v>
+        <v>160</v>
       </c>
       <c r="R49" t="s">
-        <v>164</v>
+        <v>165</v>
       </c>
       <c r="S49" t="s">
-        <v>165</v>
+        <v>166</v>
       </c>
       <c r="T49" t="s">
-        <v>167</v>
+        <v>168</v>
       </c>
       <c r="U49" t="s">
-        <v>171</v>
+        <v>172</v>
       </c>
       <c r="V49" s="2">
         <v>46199</v>
@@ -3550,13 +3556,13 @@
         <v>93</v>
       </c>
       <c r="J50" t="s">
-        <v>131</v>
+        <v>132</v>
       </c>
       <c r="K50" t="s">
-        <v>137</v>
+        <v>138</v>
       </c>
       <c r="N50" t="s">
-        <v>146</v>
+        <v>147</v>
       </c>
       <c r="O50" t="s">
         <v>60</v>
@@ -3565,19 +3571,19 @@
         <v>608623.25</v>
       </c>
       <c r="Q50" t="s">
-        <v>160</v>
+        <v>161</v>
       </c>
       <c r="R50" t="s">
-        <v>163</v>
+        <v>164</v>
       </c>
       <c r="S50" t="s">
-        <v>165</v>
+        <v>166</v>
       </c>
       <c r="T50" t="s">
-        <v>169</v>
+        <v>170</v>
       </c>
       <c r="U50" t="s">
-        <v>171</v>
+        <v>172</v>
       </c>
       <c r="V50" s="2">
         <v>46260</v>
@@ -3612,13 +3618,13 @@
         <v>117</v>
       </c>
       <c r="J51" t="s">
-        <v>131</v>
+        <v>132</v>
       </c>
       <c r="K51" t="s">
-        <v>134</v>
+        <v>135</v>
       </c>
       <c r="N51" t="s">
-        <v>146</v>
+        <v>147</v>
       </c>
       <c r="O51" t="s">
         <v>61</v>
@@ -3627,19 +3633,19 @@
         <v>66366.75999999999</v>
       </c>
       <c r="Q51" t="s">
-        <v>160</v>
+        <v>161</v>
       </c>
       <c r="R51" t="s">
-        <v>163</v>
+        <v>164</v>
       </c>
       <c r="S51" t="s">
-        <v>165</v>
+        <v>166</v>
       </c>
       <c r="T51" t="s">
-        <v>169</v>
+        <v>170</v>
       </c>
       <c r="U51" t="s">
-        <v>171</v>
+        <v>172</v>
       </c>
       <c r="V51" s="2">
         <v>46291</v>
@@ -3664,11 +3670,14 @@
       <c r="F52" t="s">
         <v>93</v>
       </c>
+      <c r="J52" t="s">
+        <v>130</v>
+      </c>
       <c r="K52" t="s">
-        <v>136</v>
+        <v>137</v>
       </c>
       <c r="N52" t="s">
-        <v>146</v>
+        <v>147</v>
       </c>
       <c r="O52" t="s">
         <v>62</v>
@@ -3677,19 +3686,19 @@
         <v>1704503</v>
       </c>
       <c r="Q52" t="s">
-        <v>160</v>
+        <v>161</v>
       </c>
       <c r="R52" t="s">
-        <v>163</v>
+        <v>164</v>
       </c>
       <c r="S52" t="s">
-        <v>165</v>
+        <v>166</v>
       </c>
       <c r="T52" t="s">
-        <v>169</v>
+        <v>170</v>
       </c>
       <c r="U52" t="s">
-        <v>171</v>
+        <v>172</v>
       </c>
       <c r="V52" s="2">
         <v>46321</v>
@@ -3724,7 +3733,7 @@
         <v>124</v>
       </c>
       <c r="N53" t="s">
-        <v>146</v>
+        <v>147</v>
       </c>
       <c r="O53" t="s">
         <v>60</v>
@@ -3733,19 +3742,19 @@
         <v>236343.68</v>
       </c>
       <c r="Q53" t="s">
-        <v>160</v>
+        <v>161</v>
       </c>
       <c r="R53" t="s">
-        <v>163</v>
+        <v>164</v>
       </c>
       <c r="S53" t="s">
-        <v>165</v>
+        <v>166</v>
       </c>
       <c r="T53" t="s">
-        <v>169</v>
+        <v>170</v>
       </c>
       <c r="U53" t="s">
-        <v>171</v>
+        <v>172</v>
       </c>
       <c r="V53" s="2">
         <v>46229</v>
@@ -3777,7 +3786,7 @@
         <v>116</v>
       </c>
       <c r="N54" t="s">
-        <v>146</v>
+        <v>147</v>
       </c>
       <c r="O54" t="s">
         <v>61</v>
@@ -3786,19 +3795,19 @@
         <v>1145462.93</v>
       </c>
       <c r="Q54" t="s">
-        <v>160</v>
+        <v>161</v>
       </c>
       <c r="R54" t="s">
-        <v>163</v>
+        <v>164</v>
       </c>
       <c r="S54" t="s">
-        <v>165</v>
+        <v>166</v>
       </c>
       <c r="T54" t="s">
-        <v>169</v>
+        <v>170</v>
       </c>
       <c r="U54" t="s">
-        <v>171</v>
+        <v>172</v>
       </c>
       <c r="V54" s="2">
         <v>46291</v>
@@ -3830,7 +3839,7 @@
         <v>116</v>
       </c>
       <c r="N55" t="s">
-        <v>146</v>
+        <v>147</v>
       </c>
       <c r="O55" t="s">
         <v>60</v>
@@ -3839,19 +3848,19 @@
         <v>859536.0699999999</v>
       </c>
       <c r="Q55" t="s">
-        <v>160</v>
+        <v>161</v>
       </c>
       <c r="R55" t="s">
-        <v>163</v>
+        <v>164</v>
       </c>
       <c r="S55" t="s">
-        <v>165</v>
+        <v>166</v>
       </c>
       <c r="T55" t="s">
-        <v>169</v>
+        <v>170</v>
       </c>
       <c r="U55" t="s">
-        <v>171</v>
+        <v>172</v>
       </c>
       <c r="V55" s="2">
         <v>46260</v>
@@ -3883,7 +3892,7 @@
         <v>110</v>
       </c>
       <c r="N56" t="s">
-        <v>146</v>
+        <v>147</v>
       </c>
       <c r="O56" t="s">
         <v>61</v>
@@ -3892,19 +3901,19 @@
         <v>389619.06</v>
       </c>
       <c r="Q56" t="s">
-        <v>160</v>
+        <v>161</v>
       </c>
       <c r="R56" t="s">
-        <v>163</v>
+        <v>164</v>
       </c>
       <c r="S56" t="s">
-        <v>165</v>
+        <v>166</v>
       </c>
       <c r="T56" t="s">
-        <v>169</v>
+        <v>170</v>
       </c>
       <c r="U56" t="s">
-        <v>171</v>
+        <v>172</v>
       </c>
       <c r="V56" s="2">
         <v>46291</v>
@@ -3936,7 +3945,7 @@
         <v>125</v>
       </c>
       <c r="N57" t="s">
-        <v>146</v>
+        <v>147</v>
       </c>
       <c r="O57" t="s">
         <v>61</v>
@@ -3945,19 +3954,19 @@
         <v>103054.25</v>
       </c>
       <c r="Q57" t="s">
-        <v>160</v>
+        <v>161</v>
       </c>
       <c r="R57" t="s">
-        <v>163</v>
+        <v>164</v>
       </c>
       <c r="S57" t="s">
-        <v>165</v>
+        <v>166</v>
       </c>
       <c r="T57" t="s">
-        <v>169</v>
+        <v>170</v>
       </c>
       <c r="U57" t="s">
-        <v>171</v>
+        <v>172</v>
       </c>
       <c r="V57" s="2">
         <v>46291</v>
@@ -3986,10 +3995,10 @@
         <v>126</v>
       </c>
       <c r="K58" t="s">
-        <v>138</v>
+        <v>139</v>
       </c>
       <c r="N58" t="s">
-        <v>146</v>
+        <v>147</v>
       </c>
       <c r="O58" t="s">
         <v>63</v>
@@ -3998,19 +4007,19 @@
         <v>1295422.28</v>
       </c>
       <c r="Q58" t="s">
-        <v>160</v>
+        <v>161</v>
       </c>
       <c r="R58" t="s">
-        <v>163</v>
+        <v>164</v>
       </c>
       <c r="S58" t="s">
-        <v>165</v>
+        <v>166</v>
       </c>
       <c r="T58" t="s">
-        <v>169</v>
+        <v>170</v>
       </c>
       <c r="U58" t="s">
-        <v>171</v>
+        <v>172</v>
       </c>
       <c r="V58" s="2">
         <v>46352</v>
@@ -4033,7 +4042,7 @@
         <v>92</v>
       </c>
       <c r="N59" t="s">
-        <v>150</v>
+        <v>151</v>
       </c>
       <c r="O59" t="s">
         <v>64</v>
@@ -4042,19 +4051,19 @@
         <v>4064.54</v>
       </c>
       <c r="Q59" t="s">
-        <v>160</v>
+        <v>161</v>
       </c>
       <c r="R59" t="s">
-        <v>164</v>
+        <v>165</v>
       </c>
       <c r="S59" t="s">
-        <v>166</v>
+        <v>167</v>
       </c>
       <c r="T59" t="s">
-        <v>167</v>
+        <v>168</v>
       </c>
       <c r="U59" t="s">
-        <v>171</v>
+        <v>172</v>
       </c>
       <c r="V59" s="2">
         <v>46107</v>
@@ -4077,7 +4086,7 @@
         <v>92</v>
       </c>
       <c r="N60" t="s">
-        <v>151</v>
+        <v>152</v>
       </c>
       <c r="O60" t="s">
         <v>65</v>
@@ -4086,19 +4095,19 @@
         <v>4227.84</v>
       </c>
       <c r="Q60" t="s">
-        <v>159</v>
+        <v>160</v>
       </c>
       <c r="R60" t="s">
-        <v>164</v>
+        <v>165</v>
       </c>
       <c r="S60" t="s">
-        <v>166</v>
+        <v>167</v>
       </c>
       <c r="T60" t="s">
-        <v>167</v>
+        <v>168</v>
       </c>
       <c r="U60" t="s">
-        <v>171</v>
+        <v>172</v>
       </c>
       <c r="V60" s="2">
         <v>46107</v>
@@ -4121,7 +4130,7 @@
         <v>92</v>
       </c>
       <c r="N61" t="s">
-        <v>152</v>
+        <v>153</v>
       </c>
       <c r="O61" t="s">
         <v>66</v>
@@ -4130,19 +4139,19 @@
         <v>9389.959999999999</v>
       </c>
       <c r="Q61" t="s">
-        <v>159</v>
+        <v>160</v>
       </c>
       <c r="R61" t="s">
-        <v>164</v>
+        <v>165</v>
       </c>
       <c r="S61" t="s">
-        <v>166</v>
+        <v>167</v>
       </c>
       <c r="T61" t="s">
-        <v>167</v>
+        <v>168</v>
       </c>
       <c r="U61" t="s">
-        <v>171</v>
+        <v>172</v>
       </c>
       <c r="V61" s="2">
         <v>46107</v>
@@ -4165,7 +4174,7 @@
         <v>92</v>
       </c>
       <c r="N62" t="s">
-        <v>153</v>
+        <v>154</v>
       </c>
       <c r="O62" t="s">
         <v>67</v>
@@ -4174,19 +4183,19 @@
         <v>1163.64</v>
       </c>
       <c r="Q62" t="s">
-        <v>161</v>
+        <v>162</v>
       </c>
       <c r="R62" t="s">
-        <v>164</v>
+        <v>165</v>
       </c>
       <c r="S62" t="s">
-        <v>166</v>
+        <v>167</v>
       </c>
       <c r="T62" t="s">
-        <v>167</v>
+        <v>168</v>
       </c>
       <c r="U62" t="s">
-        <v>171</v>
+        <v>172</v>
       </c>
       <c r="V62" s="2">
         <v>46107</v>
@@ -4209,7 +4218,7 @@
         <v>92</v>
       </c>
       <c r="N63" t="s">
-        <v>154</v>
+        <v>155</v>
       </c>
       <c r="O63" t="s">
         <v>68</v>
@@ -4218,19 +4227,19 @@
         <v>7204.82</v>
       </c>
       <c r="Q63" t="s">
-        <v>159</v>
+        <v>160</v>
       </c>
       <c r="R63" t="s">
-        <v>164</v>
+        <v>165</v>
       </c>
       <c r="S63" t="s">
-        <v>166</v>
+        <v>167</v>
       </c>
       <c r="T63" t="s">
-        <v>167</v>
+        <v>168</v>
       </c>
       <c r="U63" t="s">
-        <v>171</v>
+        <v>172</v>
       </c>
       <c r="V63" s="2">
         <v>46107</v>
@@ -4253,7 +4262,7 @@
         <v>92</v>
       </c>
       <c r="N64" t="s">
-        <v>155</v>
+        <v>156</v>
       </c>
       <c r="O64" t="s">
         <v>65</v>
@@ -4262,19 +4271,19 @@
         <v>3662.66</v>
       </c>
       <c r="Q64" t="s">
-        <v>159</v>
+        <v>160</v>
       </c>
       <c r="R64" t="s">
-        <v>164</v>
+        <v>165</v>
       </c>
       <c r="S64" t="s">
-        <v>166</v>
+        <v>167</v>
       </c>
       <c r="T64" t="s">
-        <v>167</v>
+        <v>168</v>
       </c>
       <c r="U64" t="s">
-        <v>171</v>
+        <v>172</v>
       </c>
       <c r="V64" s="2">
         <v>46107</v>
@@ -4297,7 +4306,7 @@
         <v>92</v>
       </c>
       <c r="N65" t="s">
-        <v>142</v>
+        <v>143</v>
       </c>
       <c r="O65" t="s">
         <v>69</v>
@@ -4306,16 +4315,16 @@
         <v>120000</v>
       </c>
       <c r="Q65" t="s">
-        <v>159</v>
+        <v>160</v>
       </c>
       <c r="R65" t="s">
-        <v>163</v>
+        <v>164</v>
       </c>
       <c r="S65" t="s">
-        <v>166</v>
+        <v>167</v>
       </c>
       <c r="T65" t="s">
-        <v>167</v>
+        <v>168</v>
       </c>
       <c r="U65" t="s">
         <v>91</v>
@@ -4347,22 +4356,22 @@
         <v>105</v>
       </c>
       <c r="N66" t="s">
-        <v>141</v>
+        <v>142</v>
       </c>
       <c r="O66" t="s">
         <v>70</v>
       </c>
       <c r="Q66" t="s">
-        <v>159</v>
+        <v>160</v>
       </c>
       <c r="R66" t="s">
-        <v>162</v>
+        <v>163</v>
       </c>
       <c r="S66" t="s">
-        <v>165</v>
+        <v>166</v>
       </c>
       <c r="T66" t="s">
-        <v>167</v>
+        <v>168</v>
       </c>
       <c r="U66" t="s">
         <v>91</v>
@@ -4394,10 +4403,10 @@
         <v>126</v>
       </c>
       <c r="K67" t="s">
-        <v>135</v>
+        <v>136</v>
       </c>
       <c r="N67" t="s">
-        <v>145</v>
+        <v>146</v>
       </c>
       <c r="O67" t="s">
         <v>71</v>
@@ -4406,19 +4415,19 @@
         <v>100000</v>
       </c>
       <c r="Q67" t="s">
-        <v>161</v>
+        <v>162</v>
       </c>
       <c r="R67" t="s">
-        <v>162</v>
+        <v>163</v>
       </c>
       <c r="S67" t="s">
-        <v>165</v>
+        <v>166</v>
       </c>
       <c r="T67" t="s">
-        <v>167</v>
+        <v>168</v>
       </c>
       <c r="U67" t="s">
-        <v>171</v>
+        <v>172</v>
       </c>
       <c r="V67" s="2">
         <v>46229</v>
@@ -4441,7 +4450,7 @@
         <v>92</v>
       </c>
       <c r="N68" t="s">
-        <v>142</v>
+        <v>143</v>
       </c>
       <c r="O68" t="s">
         <v>72</v>
@@ -4450,16 +4459,16 @@
         <v>80000</v>
       </c>
       <c r="Q68" t="s">
-        <v>159</v>
+        <v>160</v>
       </c>
       <c r="R68" t="s">
-        <v>163</v>
+        <v>164</v>
       </c>
       <c r="S68" t="s">
-        <v>166</v>
+        <v>167</v>
       </c>
       <c r="T68" t="s">
-        <v>167</v>
+        <v>168</v>
       </c>
       <c r="U68" t="s">
         <v>91</v>
@@ -4485,7 +4494,7 @@
         <v>92</v>
       </c>
       <c r="N69" t="s">
-        <v>141</v>
+        <v>142</v>
       </c>
       <c r="O69" t="s">
         <v>73</v>
@@ -4494,19 +4503,19 @@
         <v>835000</v>
       </c>
       <c r="Q69" t="s">
-        <v>159</v>
+        <v>160</v>
       </c>
       <c r="R69" t="s">
-        <v>162</v>
+        <v>163</v>
       </c>
       <c r="S69" t="s">
-        <v>166</v>
+        <v>167</v>
       </c>
       <c r="T69" t="s">
-        <v>167</v>
+        <v>168</v>
       </c>
       <c r="U69" t="s">
-        <v>171</v>
+        <v>172</v>
       </c>
       <c r="V69" s="2">
         <v>46291</v>
@@ -4529,7 +4538,7 @@
         <v>92</v>
       </c>
       <c r="N70" t="s">
-        <v>141</v>
+        <v>142</v>
       </c>
       <c r="O70" t="s">
         <v>73</v>
@@ -4538,19 +4547,19 @@
         <v>165000</v>
       </c>
       <c r="Q70" t="s">
-        <v>159</v>
+        <v>160</v>
       </c>
       <c r="R70" t="s">
-        <v>162</v>
+        <v>163</v>
       </c>
       <c r="S70" t="s">
-        <v>166</v>
+        <v>167</v>
       </c>
       <c r="T70" t="s">
-        <v>167</v>
+        <v>168</v>
       </c>
       <c r="U70" t="s">
-        <v>171</v>
+        <v>172</v>
       </c>
       <c r="V70" s="2">
         <v>46168</v>
@@ -4573,7 +4582,7 @@
         <v>92</v>
       </c>
       <c r="N71" t="s">
-        <v>141</v>
+        <v>142</v>
       </c>
       <c r="O71" t="s">
         <v>74</v>
@@ -4582,19 +4591,19 @@
         <v>1000000</v>
       </c>
       <c r="Q71" t="s">
-        <v>159</v>
+        <v>160</v>
       </c>
       <c r="R71" t="s">
-        <v>162</v>
+        <v>163</v>
       </c>
       <c r="S71" t="s">
-        <v>166</v>
+        <v>167</v>
       </c>
       <c r="T71" t="s">
-        <v>167</v>
+        <v>168</v>
       </c>
       <c r="U71" t="s">
-        <v>171</v>
+        <v>172</v>
       </c>
       <c r="V71" s="2">
         <v>46291</v>
@@ -4617,7 +4626,7 @@
         <v>92</v>
       </c>
       <c r="N72" t="s">
-        <v>141</v>
+        <v>142</v>
       </c>
       <c r="O72" t="s">
         <v>75</v>
@@ -4626,19 +4635,19 @@
         <v>1000000</v>
       </c>
       <c r="Q72" t="s">
-        <v>159</v>
+        <v>160</v>
       </c>
       <c r="R72" t="s">
-        <v>162</v>
+        <v>163</v>
       </c>
       <c r="S72" t="s">
-        <v>166</v>
+        <v>167</v>
       </c>
       <c r="T72" t="s">
-        <v>167</v>
+        <v>168</v>
       </c>
       <c r="U72" t="s">
-        <v>171</v>
+        <v>172</v>
       </c>
       <c r="V72" s="2">
         <v>46291</v>
@@ -4661,7 +4670,7 @@
         <v>92</v>
       </c>
       <c r="N73" t="s">
-        <v>145</v>
+        <v>146</v>
       </c>
       <c r="O73" t="s">
         <v>76</v>
@@ -4670,19 +4679,19 @@
         <v>100000</v>
       </c>
       <c r="Q73" t="s">
-        <v>161</v>
+        <v>162</v>
       </c>
       <c r="R73" t="s">
-        <v>162</v>
+        <v>163</v>
       </c>
       <c r="S73" t="s">
-        <v>166</v>
+        <v>167</v>
       </c>
       <c r="T73" t="s">
-        <v>167</v>
+        <v>168</v>
       </c>
       <c r="U73" t="s">
-        <v>171</v>
+        <v>172</v>
       </c>
       <c r="V73" s="2">
         <v>46291</v>
@@ -4708,7 +4717,7 @@
         <v>93</v>
       </c>
       <c r="N74" t="s">
-        <v>148</v>
+        <v>149</v>
       </c>
       <c r="O74" t="s">
         <v>77</v>
@@ -4717,16 +4726,16 @@
         <v>1000000</v>
       </c>
       <c r="Q74" t="s">
-        <v>160</v>
+        <v>161</v>
       </c>
       <c r="R74" t="s">
-        <v>162</v>
+        <v>163</v>
       </c>
       <c r="S74" t="s">
-        <v>165</v>
+        <v>166</v>
       </c>
       <c r="T74" t="s">
-        <v>168</v>
+        <v>169</v>
       </c>
       <c r="U74" t="s">
         <v>91</v>
@@ -4758,7 +4767,7 @@
         <v>107</v>
       </c>
       <c r="N75" t="s">
-        <v>146</v>
+        <v>147</v>
       </c>
       <c r="O75" t="s">
         <v>78</v>
@@ -4767,19 +4776,19 @@
         <v>1704503</v>
       </c>
       <c r="Q75" t="s">
-        <v>160</v>
+        <v>161</v>
       </c>
       <c r="R75" t="s">
-        <v>163</v>
+        <v>164</v>
       </c>
       <c r="S75" t="s">
         <v>104</v>
       </c>
       <c r="T75" t="s">
-        <v>169</v>
+        <v>170</v>
       </c>
       <c r="U75" t="s">
-        <v>171</v>
+        <v>172</v>
       </c>
       <c r="V75" s="2">
         <v>46381</v>
@@ -4808,7 +4817,7 @@
         <v>107</v>
       </c>
       <c r="N76" t="s">
-        <v>146</v>
+        <v>147</v>
       </c>
       <c r="O76" t="s">
         <v>79</v>
@@ -4817,19 +4826,19 @@
         <v>1638125.5</v>
       </c>
       <c r="Q76" t="s">
-        <v>160</v>
+        <v>161</v>
       </c>
       <c r="R76" t="s">
-        <v>163</v>
+        <v>164</v>
       </c>
       <c r="S76" t="s">
         <v>104</v>
       </c>
       <c r="T76" t="s">
-        <v>169</v>
+        <v>170</v>
       </c>
       <c r="U76" t="s">
-        <v>171</v>
+        <v>172</v>
       </c>
       <c r="V76" s="2">
         <v>46381</v>
@@ -4858,7 +4867,7 @@
         <v>107</v>
       </c>
       <c r="N77" t="s">
-        <v>144</v>
+        <v>145</v>
       </c>
       <c r="O77" t="s">
         <v>80</v>
@@ -4867,16 +4876,16 @@
         <v>3800000</v>
       </c>
       <c r="Q77" t="s">
-        <v>160</v>
+        <v>161</v>
       </c>
       <c r="R77" t="s">
-        <v>163</v>
+        <v>164</v>
       </c>
       <c r="S77" t="s">
         <v>104</v>
       </c>
       <c r="T77" t="s">
-        <v>168</v>
+        <v>169</v>
       </c>
       <c r="U77" t="s">
         <v>91</v>
@@ -4908,7 +4917,7 @@
         <v>107</v>
       </c>
       <c r="N78" t="s">
-        <v>144</v>
+        <v>145</v>
       </c>
       <c r="O78" t="s">
         <v>81</v>
@@ -4917,16 +4926,16 @@
         <v>3800000</v>
       </c>
       <c r="Q78" t="s">
-        <v>160</v>
+        <v>161</v>
       </c>
       <c r="R78" t="s">
-        <v>163</v>
+        <v>164</v>
       </c>
       <c r="S78" t="s">
         <v>104</v>
       </c>
       <c r="T78" t="s">
-        <v>168</v>
+        <v>169</v>
       </c>
       <c r="U78" t="s">
         <v>91</v>
@@ -4952,13 +4961,13 @@
         <v>92</v>
       </c>
       <c r="J79" t="s">
-        <v>133</v>
+        <v>134</v>
       </c>
       <c r="K79" t="s">
-        <v>139</v>
+        <v>140</v>
       </c>
       <c r="N79" t="s">
-        <v>149</v>
+        <v>150</v>
       </c>
       <c r="O79" t="s">
         <v>82</v>
@@ -4967,16 +4976,16 @@
         <v>3800000</v>
       </c>
       <c r="Q79" t="s">
-        <v>160</v>
+        <v>161</v>
       </c>
       <c r="R79" t="s">
-        <v>163</v>
+        <v>164</v>
       </c>
       <c r="S79" t="s">
-        <v>166</v>
+        <v>167</v>
       </c>
       <c r="T79" t="s">
-        <v>168</v>
+        <v>169</v>
       </c>
       <c r="U79" t="s">
         <v>91</v>
@@ -5002,7 +5011,7 @@
         <v>91</v>
       </c>
       <c r="N80" t="s">
-        <v>156</v>
+        <v>157</v>
       </c>
       <c r="O80" t="s">
         <v>83</v>
@@ -5011,16 +5020,16 @@
         <v>4394700</v>
       </c>
       <c r="Q80" t="s">
-        <v>159</v>
+        <v>160</v>
       </c>
       <c r="R80" t="s">
-        <v>162</v>
+        <v>163</v>
       </c>
       <c r="S80" t="s">
-        <v>166</v>
+        <v>167</v>
       </c>
       <c r="T80" t="s">
-        <v>168</v>
+        <v>169</v>
       </c>
       <c r="U80" t="s">
         <v>91</v>
@@ -5052,10 +5061,10 @@
         <v>126</v>
       </c>
       <c r="K81" t="s">
-        <v>134</v>
+        <v>135</v>
       </c>
       <c r="N81" t="s">
-        <v>146</v>
+        <v>147</v>
       </c>
       <c r="O81" t="s">
         <v>84</v>
@@ -5064,19 +5073,19 @@
         <v>528395.9300000001</v>
       </c>
       <c r="Q81" t="s">
-        <v>160</v>
+        <v>161</v>
       </c>
       <c r="R81" t="s">
-        <v>163</v>
+        <v>164</v>
       </c>
       <c r="S81" t="s">
-        <v>165</v>
+        <v>166</v>
       </c>
       <c r="T81" t="s">
-        <v>169</v>
+        <v>170</v>
       </c>
       <c r="U81" t="s">
-        <v>171</v>
+        <v>172</v>
       </c>
       <c r="V81" s="2">
         <v>46382</v>
@@ -5102,7 +5111,7 @@
         <v>93</v>
       </c>
       <c r="N82" t="s">
-        <v>148</v>
+        <v>149</v>
       </c>
       <c r="O82" t="s">
         <v>85</v>
@@ -5111,16 +5120,16 @@
         <v>1000000</v>
       </c>
       <c r="Q82" t="s">
-        <v>160</v>
+        <v>161</v>
       </c>
       <c r="R82" t="s">
-        <v>162</v>
+        <v>163</v>
       </c>
       <c r="S82" t="s">
-        <v>165</v>
+        <v>166</v>
       </c>
       <c r="T82" t="s">
-        <v>168</v>
+        <v>169</v>
       </c>
       <c r="U82" t="s">
         <v>91</v>
@@ -5146,7 +5155,7 @@
         <v>91</v>
       </c>
       <c r="N83" t="s">
-        <v>156</v>
+        <v>157</v>
       </c>
       <c r="O83" t="s">
         <v>83</v>
@@ -5155,16 +5164,16 @@
         <v>4394700</v>
       </c>
       <c r="Q83" t="s">
-        <v>159</v>
+        <v>160</v>
       </c>
       <c r="R83" t="s">
-        <v>162</v>
+        <v>163</v>
       </c>
       <c r="S83" t="s">
-        <v>166</v>
+        <v>167</v>
       </c>
       <c r="T83" t="s">
-        <v>168</v>
+        <v>169</v>
       </c>
       <c r="U83" t="s">
         <v>91</v>
@@ -5205,16 +5214,16 @@
         <v>3306000</v>
       </c>
       <c r="Q84" t="s">
-        <v>159</v>
+        <v>160</v>
       </c>
       <c r="R84" t="s">
-        <v>162</v>
+        <v>163</v>
       </c>
       <c r="S84" t="s">
         <v>104</v>
       </c>
       <c r="T84" t="s">
-        <v>168</v>
+        <v>169</v>
       </c>
       <c r="U84" t="s">
         <v>91</v>
@@ -5252,16 +5261,16 @@
         <v>3306000</v>
       </c>
       <c r="Q85" t="s">
-        <v>159</v>
+        <v>160</v>
       </c>
       <c r="R85" t="s">
-        <v>162</v>
+        <v>163</v>
       </c>
       <c r="S85" t="s">
         <v>104</v>
       </c>
       <c r="T85" t="s">
-        <v>168</v>
+        <v>169</v>
       </c>
       <c r="U85" t="s">
         <v>91</v>
@@ -5287,7 +5296,7 @@
         <v>93</v>
       </c>
       <c r="N86" t="s">
-        <v>157</v>
+        <v>158</v>
       </c>
       <c r="O86" t="s">
         <v>86</v>
@@ -5296,16 +5305,16 @@
         <v>470820</v>
       </c>
       <c r="Q86" t="s">
-        <v>159</v>
+        <v>160</v>
       </c>
       <c r="R86" t="s">
-        <v>162</v>
+        <v>163</v>
       </c>
       <c r="S86" t="s">
-        <v>165</v>
+        <v>166</v>
       </c>
       <c r="T86" t="s">
-        <v>170</v>
+        <v>171</v>
       </c>
       <c r="U86" t="s">
         <v>91</v>
@@ -5331,25 +5340,25 @@
         <v>93</v>
       </c>
       <c r="N87" t="s">
-        <v>149</v>
+        <v>150</v>
       </c>
       <c r="O87" t="s">
-        <v>158</v>
+        <v>159</v>
       </c>
       <c r="P87">
         <v>2297180</v>
       </c>
       <c r="Q87" t="s">
-        <v>160</v>
+        <v>161</v>
       </c>
       <c r="R87" t="s">
-        <v>162</v>
+        <v>163</v>
       </c>
       <c r="S87" t="s">
-        <v>165</v>
+        <v>166</v>
       </c>
       <c r="T87" t="s">
-        <v>168</v>
+        <v>169</v>
       </c>
       <c r="U87" t="s">
         <v>91</v>

</xml_diff>

<commit_message>
Atualização automática: mta (06/10/2026 14:09)
</commit_message>
<xml_diff>
--- a/Projetos/02_Dados_Tratados/base_mta_tratada.xlsx
+++ b/Projetos/02_Dados_Tratados/base_mta_tratada.xlsx
@@ -542,16 +542,8 @@
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="YYYY-MM-DD HH:MM:SS"/>
   </numFmts>
-  <fonts count="2">
+  <fonts count="1">
     <font>
-      <sz val="11"/>
-      <color theme="1"/>
-      <name val="Calibri"/>
-      <family val="2"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <b/>
       <sz val="11"/>
       <color theme="1"/>
       <name val="Calibri"/>
@@ -567,7 +559,7 @@
       <patternFill patternType="gray125"/>
     </fill>
   </fills>
-  <borders count="2">
+  <borders count="1">
     <border>
       <left/>
       <right/>
@@ -575,30 +567,12 @@
       <bottom/>
       <diagonal/>
     </border>
-    <border>
-      <left style="thin">
-        <color auto="1"/>
-      </left>
-      <right style="thin">
-        <color auto="1"/>
-      </right>
-      <top style="thin">
-        <color auto="1"/>
-      </top>
-      <bottom style="thin">
-        <color auto="1"/>
-      </bottom>
-      <diagonal/>
-    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="3">
+  <cellXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top"/>
-    </xf>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
   </cellXfs>
   <cellStyles count="1">
@@ -898,70 +872,70 @@
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:22">
-      <c r="A1" s="1" t="s">
+      <c r="A1" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="1" t="s">
+      <c r="B1" t="s">
         <v>1</v>
       </c>
-      <c r="C1" s="1" t="s">
+      <c r="C1" t="s">
         <v>2</v>
       </c>
-      <c r="D1" s="1" t="s">
+      <c r="D1" t="s">
         <v>3</v>
       </c>
-      <c r="E1" s="1" t="s">
+      <c r="E1" t="s">
         <v>4</v>
       </c>
-      <c r="F1" s="1" t="s">
+      <c r="F1" t="s">
         <v>5</v>
       </c>
-      <c r="G1" s="1" t="s">
+      <c r="G1" t="s">
         <v>6</v>
       </c>
-      <c r="H1" s="1" t="s">
+      <c r="H1" t="s">
         <v>7</v>
       </c>
-      <c r="I1" s="1" t="s">
+      <c r="I1" t="s">
         <v>8</v>
       </c>
-      <c r="J1" s="1" t="s">
+      <c r="J1" t="s">
         <v>9</v>
       </c>
-      <c r="K1" s="1" t="s">
+      <c r="K1" t="s">
         <v>10</v>
       </c>
-      <c r="L1" s="1" t="s">
+      <c r="L1" t="s">
         <v>11</v>
       </c>
-      <c r="M1" s="1" t="s">
+      <c r="M1" t="s">
         <v>12</v>
       </c>
-      <c r="N1" s="1" t="s">
+      <c r="N1" t="s">
         <v>13</v>
       </c>
-      <c r="O1" s="1" t="s">
+      <c r="O1" t="s">
         <v>14</v>
       </c>
-      <c r="P1" s="1" t="s">
+      <c r="P1" t="s">
         <v>15</v>
       </c>
-      <c r="Q1" s="1" t="s">
+      <c r="Q1" t="s">
         <v>16</v>
       </c>
-      <c r="R1" s="1" t="s">
+      <c r="R1" t="s">
         <v>17</v>
       </c>
-      <c r="S1" s="1" t="s">
+      <c r="S1" t="s">
         <v>18</v>
       </c>
-      <c r="T1" s="1" t="s">
+      <c r="T1" t="s">
         <v>19</v>
       </c>
-      <c r="U1" s="1" t="s">
+      <c r="U1" t="s">
         <v>20</v>
       </c>
-      <c r="V1" s="1" t="s">
+      <c r="V1" t="s">
         <v>21</v>
       </c>
     </row>
@@ -1017,7 +991,7 @@
       <c r="U2" t="s">
         <v>172</v>
       </c>
-      <c r="V2" s="2">
+      <c r="V2" s="1">
         <v>46229</v>
       </c>
     </row>
@@ -1064,7 +1038,7 @@
       <c r="U3" t="s">
         <v>91</v>
       </c>
-      <c r="V3" s="2">
+      <c r="V3" s="1">
         <v>46291</v>
       </c>
     </row>
@@ -1111,7 +1085,7 @@
       <c r="U4" t="s">
         <v>91</v>
       </c>
-      <c r="V4" s="2">
+      <c r="V4" s="1">
         <v>46321</v>
       </c>
     </row>
@@ -1158,7 +1132,7 @@
       <c r="U5" t="s">
         <v>91</v>
       </c>
-      <c r="V5" s="2">
+      <c r="V5" s="1">
         <v>46321</v>
       </c>
     </row>
@@ -1208,7 +1182,7 @@
       <c r="U6" t="s">
         <v>91</v>
       </c>
-      <c r="V6" s="2">
+      <c r="V6" s="1">
         <v>46291</v>
       </c>
     </row>
@@ -1234,7 +1208,7 @@
       <c r="G7" t="s">
         <v>106</v>
       </c>
-      <c r="H7" s="2">
+      <c r="H7" s="1">
         <v>46121</v>
       </c>
       <c r="I7" t="s">
@@ -1264,7 +1238,7 @@
       <c r="U7" t="s">
         <v>91</v>
       </c>
-      <c r="V7" s="2">
+      <c r="V7" s="1">
         <v>46138</v>
       </c>
     </row>
@@ -1311,7 +1285,7 @@
       <c r="U8" t="s">
         <v>91</v>
       </c>
-      <c r="V8" s="2">
+      <c r="V8" s="1">
         <v>46291</v>
       </c>
     </row>
@@ -1358,7 +1332,7 @@
       <c r="U9" t="s">
         <v>91</v>
       </c>
-      <c r="V9" s="2">
+      <c r="V9" s="1">
         <v>46291</v>
       </c>
     </row>
@@ -1405,7 +1379,7 @@
       <c r="U10" t="s">
         <v>91</v>
       </c>
-      <c r="V10" s="2">
+      <c r="V10" s="1">
         <v>46291</v>
       </c>
     </row>
@@ -1452,7 +1426,7 @@
       <c r="U11" t="s">
         <v>91</v>
       </c>
-      <c r="V11" s="2">
+      <c r="V11" s="1">
         <v>46291</v>
       </c>
     </row>
@@ -1478,7 +1452,7 @@
       <c r="G12" t="s">
         <v>106</v>
       </c>
-      <c r="H12" s="2">
+      <c r="H12" s="1">
         <v>46079</v>
       </c>
       <c r="I12" t="s">
@@ -1511,7 +1485,7 @@
       <c r="U12" t="s">
         <v>172</v>
       </c>
-      <c r="V12" s="2">
+      <c r="V12" s="1">
         <v>46079</v>
       </c>
     </row>
@@ -1564,7 +1538,7 @@
       <c r="U13" t="s">
         <v>172</v>
       </c>
-      <c r="V13" s="2">
+      <c r="V13" s="1">
         <v>46352</v>
       </c>
     </row>
@@ -1617,7 +1591,7 @@
       <c r="U14" t="s">
         <v>172</v>
       </c>
-      <c r="V14" s="2">
+      <c r="V14" s="1">
         <v>46352</v>
       </c>
     </row>
@@ -1670,7 +1644,7 @@
       <c r="U15" t="s">
         <v>172</v>
       </c>
-      <c r="V15" s="2">
+      <c r="V15" s="1">
         <v>46352</v>
       </c>
     </row>
@@ -1723,7 +1697,7 @@
       <c r="U16" t="s">
         <v>172</v>
       </c>
-      <c r="V16" s="2">
+      <c r="V16" s="1">
         <v>46229</v>
       </c>
     </row>
@@ -1749,7 +1723,7 @@
       <c r="G17" t="s">
         <v>106</v>
       </c>
-      <c r="H17" s="2">
+      <c r="H17" s="1">
         <v>46098</v>
       </c>
       <c r="I17" t="s">
@@ -1782,7 +1756,7 @@
       <c r="U17" t="s">
         <v>172</v>
       </c>
-      <c r="V17" s="2">
+      <c r="V17" s="1">
         <v>46107</v>
       </c>
     </row>
@@ -1808,7 +1782,7 @@
       <c r="G18" t="s">
         <v>106</v>
       </c>
-      <c r="H18" s="2">
+      <c r="H18" s="1">
         <v>46076</v>
       </c>
       <c r="I18" t="s">
@@ -1838,7 +1812,7 @@
       <c r="U18" t="s">
         <v>91</v>
       </c>
-      <c r="V18" s="2">
+      <c r="V18" s="1">
         <v>46079</v>
       </c>
     </row>
@@ -1864,7 +1838,7 @@
       <c r="G19" t="s">
         <v>106</v>
       </c>
-      <c r="H19" s="2">
+      <c r="H19" s="1">
         <v>46076</v>
       </c>
       <c r="I19" t="s">
@@ -1894,7 +1868,7 @@
       <c r="U19" t="s">
         <v>91</v>
       </c>
-      <c r="V19" s="2">
+      <c r="V19" s="1">
         <v>46079</v>
       </c>
     </row>
@@ -1941,7 +1915,7 @@
       <c r="U20" t="s">
         <v>91</v>
       </c>
-      <c r="V20" s="2">
+      <c r="V20" s="1">
         <v>46321</v>
       </c>
     </row>
@@ -1988,7 +1962,7 @@
       <c r="U21" t="s">
         <v>91</v>
       </c>
-      <c r="V21" s="2">
+      <c r="V21" s="1">
         <v>46321</v>
       </c>
     </row>
@@ -2035,7 +2009,7 @@
       <c r="U22" t="s">
         <v>91</v>
       </c>
-      <c r="V22" s="2">
+      <c r="V22" s="1">
         <v>46321</v>
       </c>
     </row>
@@ -2082,7 +2056,7 @@
       <c r="U23" t="s">
         <v>91</v>
       </c>
-      <c r="V23" s="2">
+      <c r="V23" s="1">
         <v>46321</v>
       </c>
     </row>
@@ -2108,7 +2082,7 @@
       <c r="G24" t="s">
         <v>106</v>
       </c>
-      <c r="H24" s="2">
+      <c r="H24" s="1">
         <v>46119</v>
       </c>
       <c r="I24" t="s">
@@ -2141,7 +2115,7 @@
       <c r="U24" t="s">
         <v>172</v>
       </c>
-      <c r="V24" s="2">
+      <c r="V24" s="1">
         <v>46138</v>
       </c>
     </row>
@@ -2167,7 +2141,7 @@
       <c r="G25" t="s">
         <v>106</v>
       </c>
-      <c r="H25" s="2">
+      <c r="H25" s="1">
         <v>46121</v>
       </c>
       <c r="I25" t="s">
@@ -2197,7 +2171,7 @@
       <c r="U25" t="s">
         <v>91</v>
       </c>
-      <c r="V25" s="2">
+      <c r="V25" s="1">
         <v>46138</v>
       </c>
     </row>
@@ -2223,7 +2197,7 @@
       <c r="G26" t="s">
         <v>106</v>
       </c>
-      <c r="H26" s="2">
+      <c r="H26" s="1">
         <v>46076</v>
       </c>
       <c r="I26" t="s">
@@ -2253,7 +2227,7 @@
       <c r="U26" t="s">
         <v>91</v>
       </c>
-      <c r="V26" s="2">
+      <c r="V26" s="1">
         <v>46079</v>
       </c>
     </row>
@@ -2306,7 +2280,7 @@
       <c r="U27" t="s">
         <v>172</v>
       </c>
-      <c r="V27" s="2">
+      <c r="V27" s="1">
         <v>46291</v>
       </c>
     </row>
@@ -2332,7 +2306,7 @@
       <c r="G28" t="s">
         <v>106</v>
       </c>
-      <c r="H28" s="2">
+      <c r="H28" s="1">
         <v>46199</v>
       </c>
       <c r="I28" t="s">
@@ -2365,7 +2339,7 @@
       <c r="U28" t="s">
         <v>172</v>
       </c>
-      <c r="V28" s="2">
+      <c r="V28" s="1">
         <v>46199</v>
       </c>
     </row>
@@ -2391,7 +2365,7 @@
       <c r="G29" t="s">
         <v>106</v>
       </c>
-      <c r="H29" s="2">
+      <c r="H29" s="1">
         <v>46199</v>
       </c>
       <c r="I29" t="s">
@@ -2424,7 +2398,7 @@
       <c r="U29" t="s">
         <v>172</v>
       </c>
-      <c r="V29" s="2">
+      <c r="V29" s="1">
         <v>46199</v>
       </c>
     </row>
@@ -2450,7 +2424,7 @@
       <c r="G30" t="s">
         <v>106</v>
       </c>
-      <c r="H30" s="2">
+      <c r="H30" s="1">
         <v>46199</v>
       </c>
       <c r="I30" t="s">
@@ -2483,7 +2457,7 @@
       <c r="U30" t="s">
         <v>172</v>
       </c>
-      <c r="V30" s="2">
+      <c r="V30" s="1">
         <v>46199</v>
       </c>
     </row>
@@ -2509,7 +2483,7 @@
       <c r="G31" t="s">
         <v>106</v>
       </c>
-      <c r="H31" s="2">
+      <c r="H31" s="1">
         <v>46199</v>
       </c>
       <c r="I31" t="s">
@@ -2542,7 +2516,7 @@
       <c r="U31" t="s">
         <v>172</v>
       </c>
-      <c r="V31" s="2">
+      <c r="V31" s="1">
         <v>46199</v>
       </c>
     </row>
@@ -2595,7 +2569,7 @@
       <c r="U32" t="s">
         <v>172</v>
       </c>
-      <c r="V32" s="2">
+      <c r="V32" s="1">
         <v>46291</v>
       </c>
     </row>
@@ -2621,7 +2595,7 @@
       <c r="G33" t="s">
         <v>106</v>
       </c>
-      <c r="H33" s="2">
+      <c r="H33" s="1">
         <v>46191</v>
       </c>
       <c r="I33" t="s">
@@ -2654,7 +2628,7 @@
       <c r="U33" t="s">
         <v>172</v>
       </c>
-      <c r="V33" s="2">
+      <c r="V33" s="1">
         <v>46199</v>
       </c>
     </row>
@@ -2680,7 +2654,7 @@
       <c r="G34" t="s">
         <v>106</v>
       </c>
-      <c r="H34" s="2">
+      <c r="H34" s="1">
         <v>46119</v>
       </c>
       <c r="I34" t="s">
@@ -2710,7 +2684,7 @@
       <c r="U34" t="s">
         <v>172</v>
       </c>
-      <c r="V34" s="2">
+      <c r="V34" s="1">
         <v>46138</v>
       </c>
     </row>
@@ -2736,7 +2710,7 @@
       <c r="G35" t="s">
         <v>106</v>
       </c>
-      <c r="H35" s="2">
+      <c r="H35" s="1">
         <v>46213</v>
       </c>
       <c r="I35" t="s">
@@ -2766,7 +2740,7 @@
       <c r="U35" t="s">
         <v>91</v>
       </c>
-      <c r="V35" s="2">
+      <c r="V35" s="1">
         <v>46229</v>
       </c>
     </row>
@@ -2792,7 +2766,7 @@
       <c r="G36" t="s">
         <v>106</v>
       </c>
-      <c r="H36" s="2">
+      <c r="H36" s="1">
         <v>46175</v>
       </c>
       <c r="I36" t="s">
@@ -2822,7 +2796,7 @@
       <c r="U36" t="s">
         <v>91</v>
       </c>
-      <c r="V36" s="2">
+      <c r="V36" s="1">
         <v>46199</v>
       </c>
     </row>
@@ -2848,7 +2822,7 @@
       <c r="G37" t="s">
         <v>106</v>
       </c>
-      <c r="H37" s="2">
+      <c r="H37" s="1">
         <v>46213</v>
       </c>
       <c r="I37" t="s">
@@ -2878,7 +2852,7 @@
       <c r="U37" t="s">
         <v>91</v>
       </c>
-      <c r="V37" s="2">
+      <c r="V37" s="1">
         <v>46229</v>
       </c>
     </row>
@@ -2904,7 +2878,7 @@
       <c r="G38" t="s">
         <v>106</v>
       </c>
-      <c r="H38" s="2">
+      <c r="H38" s="1">
         <v>46199</v>
       </c>
       <c r="I38" t="s">
@@ -2934,7 +2908,7 @@
       <c r="U38" t="s">
         <v>91</v>
       </c>
-      <c r="V38" s="2">
+      <c r="V38" s="1">
         <v>46199</v>
       </c>
     </row>
@@ -2960,7 +2934,7 @@
       <c r="G39" t="s">
         <v>106</v>
       </c>
-      <c r="H39" s="2">
+      <c r="H39" s="1">
         <v>46199</v>
       </c>
       <c r="I39" t="s">
@@ -2990,7 +2964,7 @@
       <c r="U39" t="s">
         <v>91</v>
       </c>
-      <c r="V39" s="2">
+      <c r="V39" s="1">
         <v>46199</v>
       </c>
     </row>
@@ -3016,7 +2990,7 @@
       <c r="G40" t="s">
         <v>106</v>
       </c>
-      <c r="H40" s="2">
+      <c r="H40" s="1">
         <v>46204</v>
       </c>
       <c r="I40" t="s">
@@ -3046,7 +3020,7 @@
       <c r="U40" t="s">
         <v>91</v>
       </c>
-      <c r="V40" s="2">
+      <c r="V40" s="1">
         <v>46229</v>
       </c>
     </row>
@@ -3072,7 +3046,7 @@
       <c r="G41" t="s">
         <v>106</v>
       </c>
-      <c r="H41" s="2">
+      <c r="H41" s="1">
         <v>46244</v>
       </c>
       <c r="I41" t="s">
@@ -3102,7 +3076,7 @@
       <c r="U41" t="s">
         <v>91</v>
       </c>
-      <c r="V41" s="2">
+      <c r="V41" s="1">
         <v>46199</v>
       </c>
     </row>
@@ -3146,7 +3120,7 @@
       <c r="U42" t="s">
         <v>91</v>
       </c>
-      <c r="V42" s="2">
+      <c r="V42" s="1">
         <v>46260</v>
       </c>
     </row>
@@ -3172,7 +3146,7 @@
       <c r="G43" t="s">
         <v>106</v>
       </c>
-      <c r="H43" s="2">
+      <c r="H43" s="1">
         <v>46191</v>
       </c>
       <c r="I43" t="s">
@@ -3202,7 +3176,7 @@
       <c r="U43" t="s">
         <v>91</v>
       </c>
-      <c r="V43" s="2">
+      <c r="V43" s="1">
         <v>46199</v>
       </c>
     </row>
@@ -3228,7 +3202,7 @@
       <c r="G44" t="s">
         <v>106</v>
       </c>
-      <c r="H44" s="2">
+      <c r="H44" s="1">
         <v>46191</v>
       </c>
       <c r="I44" t="s">
@@ -3258,7 +3232,7 @@
       <c r="U44" t="s">
         <v>91</v>
       </c>
-      <c r="V44" s="2">
+      <c r="V44" s="1">
         <v>46199</v>
       </c>
     </row>
@@ -3284,7 +3258,7 @@
       <c r="G45" t="s">
         <v>106</v>
       </c>
-      <c r="H45" s="2">
+      <c r="H45" s="1">
         <v>46213</v>
       </c>
       <c r="I45" t="s">
@@ -3317,7 +3291,7 @@
       <c r="U45" t="s">
         <v>172</v>
       </c>
-      <c r="V45" s="2">
+      <c r="V45" s="1">
         <v>46229</v>
       </c>
     </row>
@@ -3343,7 +3317,7 @@
       <c r="G46" t="s">
         <v>106</v>
       </c>
-      <c r="H46" s="2">
+      <c r="H46" s="1">
         <v>46210</v>
       </c>
       <c r="I46" t="s">
@@ -3373,7 +3347,7 @@
       <c r="U46" t="s">
         <v>172</v>
       </c>
-      <c r="V46" s="2">
+      <c r="V46" s="1">
         <v>46229</v>
       </c>
     </row>
@@ -3420,7 +3394,7 @@
       <c r="U47" t="s">
         <v>91</v>
       </c>
-      <c r="V47" s="2">
+      <c r="V47" s="1">
         <v>46321</v>
       </c>
     </row>
@@ -3473,7 +3447,7 @@
       <c r="U48" t="s">
         <v>172</v>
       </c>
-      <c r="V48" s="2">
+      <c r="V48" s="1">
         <v>46291</v>
       </c>
     </row>
@@ -3499,7 +3473,7 @@
       <c r="G49" t="s">
         <v>106</v>
       </c>
-      <c r="H49" s="2">
+      <c r="H49" s="1">
         <v>46176</v>
       </c>
       <c r="I49" t="s">
@@ -3532,7 +3506,7 @@
       <c r="U49" t="s">
         <v>172</v>
       </c>
-      <c r="V49" s="2">
+      <c r="V49" s="1">
         <v>46199</v>
       </c>
     </row>
@@ -3585,7 +3559,7 @@
       <c r="U50" t="s">
         <v>172</v>
       </c>
-      <c r="V50" s="2">
+      <c r="V50" s="1">
         <v>46260</v>
       </c>
     </row>
@@ -3611,7 +3585,7 @@
       <c r="G51" t="s">
         <v>106</v>
       </c>
-      <c r="H51" s="2">
+      <c r="H51" s="1">
         <v>46295</v>
       </c>
       <c r="I51" t="s">
@@ -3647,7 +3621,7 @@
       <c r="U51" t="s">
         <v>172</v>
       </c>
-      <c r="V51" s="2">
+      <c r="V51" s="1">
         <v>46291</v>
       </c>
     </row>
@@ -3700,7 +3674,7 @@
       <c r="U52" t="s">
         <v>172</v>
       </c>
-      <c r="V52" s="2">
+      <c r="V52" s="1">
         <v>46321</v>
       </c>
     </row>
@@ -3726,7 +3700,7 @@
       <c r="G53" t="s">
         <v>106</v>
       </c>
-      <c r="H53" s="2">
+      <c r="H53" s="1">
         <v>46227</v>
       </c>
       <c r="I53" t="s">
@@ -3756,7 +3730,7 @@
       <c r="U53" t="s">
         <v>172</v>
       </c>
-      <c r="V53" s="2">
+      <c r="V53" s="1">
         <v>46229</v>
       </c>
     </row>
@@ -3779,7 +3753,7 @@
       <c r="G54" t="s">
         <v>106</v>
       </c>
-      <c r="H54" s="2">
+      <c r="H54" s="1">
         <v>46280</v>
       </c>
       <c r="I54" t="s">
@@ -3809,7 +3783,7 @@
       <c r="U54" t="s">
         <v>172</v>
       </c>
-      <c r="V54" s="2">
+      <c r="V54" s="1">
         <v>46291</v>
       </c>
     </row>
@@ -3832,7 +3806,7 @@
       <c r="G55" t="s">
         <v>106</v>
       </c>
-      <c r="H55" s="2">
+      <c r="H55" s="1">
         <v>46280</v>
       </c>
       <c r="I55" t="s">
@@ -3862,7 +3836,7 @@
       <c r="U55" t="s">
         <v>172</v>
       </c>
-      <c r="V55" s="2">
+      <c r="V55" s="1">
         <v>46260</v>
       </c>
     </row>
@@ -3885,7 +3859,7 @@
       <c r="G56" t="s">
         <v>106</v>
       </c>
-      <c r="H56" s="2">
+      <c r="H56" s="1">
         <v>46295</v>
       </c>
       <c r="I56" t="s">
@@ -3915,7 +3889,7 @@
       <c r="U56" t="s">
         <v>172</v>
       </c>
-      <c r="V56" s="2">
+      <c r="V56" s="1">
         <v>46291</v>
       </c>
     </row>
@@ -3938,7 +3912,7 @@
       <c r="G57" t="s">
         <v>106</v>
       </c>
-      <c r="H57" s="2">
+      <c r="H57" s="1">
         <v>46295</v>
       </c>
       <c r="I57" t="s">
@@ -3968,7 +3942,7 @@
       <c r="U57" t="s">
         <v>172</v>
       </c>
-      <c r="V57" s="2">
+      <c r="V57" s="1">
         <v>46291</v>
       </c>
     </row>
@@ -4021,7 +3995,7 @@
       <c r="U58" t="s">
         <v>172</v>
       </c>
-      <c r="V58" s="2">
+      <c r="V58" s="1">
         <v>46352</v>
       </c>
     </row>
@@ -4065,7 +4039,7 @@
       <c r="U59" t="s">
         <v>172</v>
       </c>
-      <c r="V59" s="2">
+      <c r="V59" s="1">
         <v>46107</v>
       </c>
     </row>
@@ -4109,7 +4083,7 @@
       <c r="U60" t="s">
         <v>172</v>
       </c>
-      <c r="V60" s="2">
+      <c r="V60" s="1">
         <v>46107</v>
       </c>
     </row>
@@ -4153,7 +4127,7 @@
       <c r="U61" t="s">
         <v>172</v>
       </c>
-      <c r="V61" s="2">
+      <c r="V61" s="1">
         <v>46107</v>
       </c>
     </row>
@@ -4197,7 +4171,7 @@
       <c r="U62" t="s">
         <v>172</v>
       </c>
-      <c r="V62" s="2">
+      <c r="V62" s="1">
         <v>46107</v>
       </c>
     </row>
@@ -4241,7 +4215,7 @@
       <c r="U63" t="s">
         <v>172</v>
       </c>
-      <c r="V63" s="2">
+      <c r="V63" s="1">
         <v>46107</v>
       </c>
     </row>
@@ -4285,7 +4259,7 @@
       <c r="U64" t="s">
         <v>172</v>
       </c>
-      <c r="V64" s="2">
+      <c r="V64" s="1">
         <v>46107</v>
       </c>
     </row>
@@ -4329,7 +4303,7 @@
       <c r="U65" t="s">
         <v>91</v>
       </c>
-      <c r="V65" s="2">
+      <c r="V65" s="1">
         <v>46168</v>
       </c>
     </row>
@@ -4376,7 +4350,7 @@
       <c r="U66" t="s">
         <v>91</v>
       </c>
-      <c r="V66" s="2">
+      <c r="V66" s="1">
         <v>46291</v>
       </c>
     </row>
@@ -4429,7 +4403,7 @@
       <c r="U67" t="s">
         <v>172</v>
       </c>
-      <c r="V67" s="2">
+      <c r="V67" s="1">
         <v>46229</v>
       </c>
     </row>
@@ -4473,7 +4447,7 @@
       <c r="U68" t="s">
         <v>91</v>
       </c>
-      <c r="V68" s="2">
+      <c r="V68" s="1">
         <v>46260</v>
       </c>
     </row>
@@ -4517,7 +4491,7 @@
       <c r="U69" t="s">
         <v>172</v>
       </c>
-      <c r="V69" s="2">
+      <c r="V69" s="1">
         <v>46291</v>
       </c>
     </row>
@@ -4561,7 +4535,7 @@
       <c r="U70" t="s">
         <v>172</v>
       </c>
-      <c r="V70" s="2">
+      <c r="V70" s="1">
         <v>46168</v>
       </c>
     </row>
@@ -4605,7 +4579,7 @@
       <c r="U71" t="s">
         <v>172</v>
       </c>
-      <c r="V71" s="2">
+      <c r="V71" s="1">
         <v>46291</v>
       </c>
     </row>
@@ -4649,7 +4623,7 @@
       <c r="U72" t="s">
         <v>172</v>
       </c>
-      <c r="V72" s="2">
+      <c r="V72" s="1">
         <v>46291</v>
       </c>
     </row>
@@ -4693,7 +4667,7 @@
       <c r="U73" t="s">
         <v>172</v>
       </c>
-      <c r="V73" s="2">
+      <c r="V73" s="1">
         <v>46291</v>
       </c>
     </row>
@@ -4740,7 +4714,7 @@
       <c r="U74" t="s">
         <v>91</v>
       </c>
-      <c r="V74" s="2">
+      <c r="V74" s="1">
         <v>46321</v>
       </c>
     </row>
@@ -4790,7 +4764,7 @@
       <c r="U75" t="s">
         <v>172</v>
       </c>
-      <c r="V75" s="2">
+      <c r="V75" s="1">
         <v>46381</v>
       </c>
     </row>
@@ -4840,7 +4814,7 @@
       <c r="U76" t="s">
         <v>172</v>
       </c>
-      <c r="V76" s="2">
+      <c r="V76" s="1">
         <v>46381</v>
       </c>
     </row>
@@ -4890,7 +4864,7 @@
       <c r="U77" t="s">
         <v>91</v>
       </c>
-      <c r="V77" s="2">
+      <c r="V77" s="1">
         <v>46381</v>
       </c>
     </row>
@@ -4940,7 +4914,7 @@
       <c r="U78" t="s">
         <v>91</v>
       </c>
-      <c r="V78" s="2">
+      <c r="V78" s="1">
         <v>46381</v>
       </c>
     </row>
@@ -4990,7 +4964,7 @@
       <c r="U79" t="s">
         <v>91</v>
       </c>
-      <c r="V79" s="2">
+      <c r="V79" s="1">
         <v>46382</v>
       </c>
     </row>
@@ -5034,7 +5008,7 @@
       <c r="U80" t="s">
         <v>91</v>
       </c>
-      <c r="V80" s="2">
+      <c r="V80" s="1">
         <v>46382</v>
       </c>
     </row>
@@ -5087,7 +5061,7 @@
       <c r="U81" t="s">
         <v>172</v>
       </c>
-      <c r="V81" s="2">
+      <c r="V81" s="1">
         <v>46382</v>
       </c>
     </row>
@@ -5134,7 +5108,7 @@
       <c r="U82" t="s">
         <v>91</v>
       </c>
-      <c r="V82" s="2">
+      <c r="V82" s="1">
         <v>46321</v>
       </c>
     </row>
@@ -5178,7 +5152,7 @@
       <c r="U83" t="s">
         <v>91</v>
       </c>
-      <c r="V83" s="2">
+      <c r="V83" s="1">
         <v>46382</v>
       </c>
     </row>
@@ -5319,7 +5293,7 @@
       <c r="U86" t="s">
         <v>91</v>
       </c>
-      <c r="V86" s="2">
+      <c r="V86" s="1">
         <v>46291</v>
       </c>
     </row>
@@ -5363,7 +5337,7 @@
       <c r="U87" t="s">
         <v>91</v>
       </c>
-      <c r="V87" s="2">
+      <c r="V87" s="1">
         <v>46291</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Atualização automática: mta (07/10/2026 14:47)
</commit_message>
<xml_diff>
--- a/Projetos/02_Dados_Tratados/base_mta_tratada.xlsx
+++ b/Projetos/02_Dados_Tratados/base_mta_tratada.xlsx
@@ -551,16 +551,8 @@
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="YYYY-MM-DD HH:MM:SS"/>
   </numFmts>
-  <fonts count="2">
+  <fonts count="1">
     <font>
-      <sz val="11"/>
-      <color theme="1"/>
-      <name val="Calibri"/>
-      <family val="2"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <b/>
       <sz val="11"/>
       <color theme="1"/>
       <name val="Calibri"/>
@@ -576,7 +568,7 @@
       <patternFill patternType="gray125"/>
     </fill>
   </fills>
-  <borders count="2">
+  <borders count="1">
     <border>
       <left/>
       <right/>
@@ -584,30 +576,12 @@
       <bottom/>
       <diagonal/>
     </border>
-    <border>
-      <left style="thin">
-        <color auto="1"/>
-      </left>
-      <right style="thin">
-        <color auto="1"/>
-      </right>
-      <top style="thin">
-        <color auto="1"/>
-      </top>
-      <bottom style="thin">
-        <color auto="1"/>
-      </bottom>
-      <diagonal/>
-    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="3">
+  <cellXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top"/>
-    </xf>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
   </cellXfs>
   <cellStyles count="1">
@@ -907,70 +881,70 @@
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:22">
-      <c r="A1" s="1" t="s">
+      <c r="A1" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="1" t="s">
+      <c r="B1" t="s">
         <v>1</v>
       </c>
-      <c r="C1" s="1" t="s">
+      <c r="C1" t="s">
         <v>2</v>
       </c>
-      <c r="D1" s="1" t="s">
+      <c r="D1" t="s">
         <v>3</v>
       </c>
-      <c r="E1" s="1" t="s">
+      <c r="E1" t="s">
         <v>4</v>
       </c>
-      <c r="F1" s="1" t="s">
+      <c r="F1" t="s">
         <v>5</v>
       </c>
-      <c r="G1" s="1" t="s">
+      <c r="G1" t="s">
         <v>6</v>
       </c>
-      <c r="H1" s="1" t="s">
+      <c r="H1" t="s">
         <v>7</v>
       </c>
-      <c r="I1" s="1" t="s">
+      <c r="I1" t="s">
         <v>8</v>
       </c>
-      <c r="J1" s="1" t="s">
+      <c r="J1" t="s">
         <v>9</v>
       </c>
-      <c r="K1" s="1" t="s">
+      <c r="K1" t="s">
         <v>10</v>
       </c>
-      <c r="L1" s="1" t="s">
+      <c r="L1" t="s">
         <v>11</v>
       </c>
-      <c r="M1" s="1" t="s">
+      <c r="M1" t="s">
         <v>12</v>
       </c>
-      <c r="N1" s="1" t="s">
+      <c r="N1" t="s">
         <v>13</v>
       </c>
-      <c r="O1" s="1" t="s">
+      <c r="O1" t="s">
         <v>14</v>
       </c>
-      <c r="P1" s="1" t="s">
+      <c r="P1" t="s">
         <v>15</v>
       </c>
-      <c r="Q1" s="1" t="s">
+      <c r="Q1" t="s">
         <v>16</v>
       </c>
-      <c r="R1" s="1" t="s">
+      <c r="R1" t="s">
         <v>17</v>
       </c>
-      <c r="S1" s="1" t="s">
+      <c r="S1" t="s">
         <v>18</v>
       </c>
-      <c r="T1" s="1" t="s">
+      <c r="T1" t="s">
         <v>19</v>
       </c>
-      <c r="U1" s="1" t="s">
+      <c r="U1" t="s">
         <v>20</v>
       </c>
-      <c r="V1" s="1" t="s">
+      <c r="V1" t="s">
         <v>21</v>
       </c>
     </row>
@@ -1029,7 +1003,7 @@
       <c r="U2" t="s">
         <v>175</v>
       </c>
-      <c r="V2" s="2">
+      <c r="V2" s="1">
         <v>46229</v>
       </c>
     </row>
@@ -1076,7 +1050,7 @@
       <c r="U3" t="s">
         <v>92</v>
       </c>
-      <c r="V3" s="2">
+      <c r="V3" s="1">
         <v>46291</v>
       </c>
     </row>
@@ -1123,7 +1097,7 @@
       <c r="U4" t="s">
         <v>92</v>
       </c>
-      <c r="V4" s="2">
+      <c r="V4" s="1">
         <v>46321</v>
       </c>
     </row>
@@ -1170,7 +1144,7 @@
       <c r="U5" t="s">
         <v>92</v>
       </c>
-      <c r="V5" s="2">
+      <c r="V5" s="1">
         <v>46321</v>
       </c>
     </row>
@@ -1220,7 +1194,7 @@
       <c r="U6" t="s">
         <v>92</v>
       </c>
-      <c r="V6" s="2">
+      <c r="V6" s="1">
         <v>46291</v>
       </c>
     </row>
@@ -1246,7 +1220,7 @@
       <c r="G7" t="s">
         <v>108</v>
       </c>
-      <c r="H7" s="2">
+      <c r="H7" s="1">
         <v>46121</v>
       </c>
       <c r="I7" t="s">
@@ -1273,7 +1247,7 @@
       <c r="U7" t="s">
         <v>92</v>
       </c>
-      <c r="V7" s="2">
+      <c r="V7" s="1">
         <v>46138</v>
       </c>
     </row>
@@ -1320,7 +1294,7 @@
       <c r="U8" t="s">
         <v>92</v>
       </c>
-      <c r="V8" s="2">
+      <c r="V8" s="1">
         <v>46291</v>
       </c>
     </row>
@@ -1364,7 +1338,7 @@
       <c r="U9" t="s">
         <v>92</v>
       </c>
-      <c r="V9" s="2">
+      <c r="V9" s="1">
         <v>46291</v>
       </c>
     </row>
@@ -1411,7 +1385,7 @@
       <c r="U10" t="s">
         <v>92</v>
       </c>
-      <c r="V10" s="2">
+      <c r="V10" s="1">
         <v>46291</v>
       </c>
     </row>
@@ -1458,7 +1432,7 @@
       <c r="U11" t="s">
         <v>92</v>
       </c>
-      <c r="V11" s="2">
+      <c r="V11" s="1">
         <v>46291</v>
       </c>
     </row>
@@ -1505,7 +1479,7 @@
       <c r="U12" t="s">
         <v>92</v>
       </c>
-      <c r="V12" s="2">
+      <c r="V12" s="1">
         <v>46291</v>
       </c>
     </row>
@@ -1531,7 +1505,7 @@
       <c r="G13" t="s">
         <v>108</v>
       </c>
-      <c r="H13" s="2">
+      <c r="H13" s="1">
         <v>46079</v>
       </c>
       <c r="I13" t="s">
@@ -1561,7 +1535,7 @@
       <c r="U13" t="s">
         <v>175</v>
       </c>
-      <c r="V13" s="2">
+      <c r="V13" s="1">
         <v>46079</v>
       </c>
     </row>
@@ -1617,7 +1591,7 @@
       <c r="U14" t="s">
         <v>175</v>
       </c>
-      <c r="V14" s="2">
+      <c r="V14" s="1">
         <v>46352</v>
       </c>
     </row>
@@ -1673,7 +1647,7 @@
       <c r="U15" t="s">
         <v>175</v>
       </c>
-      <c r="V15" s="2">
+      <c r="V15" s="1">
         <v>46352</v>
       </c>
     </row>
@@ -1729,7 +1703,7 @@
       <c r="U16" t="s">
         <v>175</v>
       </c>
-      <c r="V16" s="2">
+      <c r="V16" s="1">
         <v>46352</v>
       </c>
     </row>
@@ -1785,7 +1759,7 @@
       <c r="U17" t="s">
         <v>175</v>
       </c>
-      <c r="V17" s="2">
+      <c r="V17" s="1">
         <v>46229</v>
       </c>
     </row>
@@ -1811,7 +1785,7 @@
       <c r="G18" t="s">
         <v>108</v>
       </c>
-      <c r="H18" s="2">
+      <c r="H18" s="1">
         <v>46098</v>
       </c>
       <c r="I18" t="s">
@@ -1841,7 +1815,7 @@
       <c r="U18" t="s">
         <v>175</v>
       </c>
-      <c r="V18" s="2">
+      <c r="V18" s="1">
         <v>46107</v>
       </c>
     </row>
@@ -1867,7 +1841,7 @@
       <c r="G19" t="s">
         <v>108</v>
       </c>
-      <c r="H19" s="2">
+      <c r="H19" s="1">
         <v>46076</v>
       </c>
       <c r="I19" t="s">
@@ -1894,7 +1868,7 @@
       <c r="U19" t="s">
         <v>92</v>
       </c>
-      <c r="V19" s="2">
+      <c r="V19" s="1">
         <v>46079</v>
       </c>
     </row>
@@ -1920,7 +1894,7 @@
       <c r="G20" t="s">
         <v>108</v>
       </c>
-      <c r="H20" s="2">
+      <c r="H20" s="1">
         <v>46076</v>
       </c>
       <c r="I20" t="s">
@@ -1947,7 +1921,7 @@
       <c r="U20" t="s">
         <v>92</v>
       </c>
-      <c r="V20" s="2">
+      <c r="V20" s="1">
         <v>46079</v>
       </c>
     </row>
@@ -1991,7 +1965,7 @@
       <c r="U21" t="s">
         <v>92</v>
       </c>
-      <c r="V21" s="2">
+      <c r="V21" s="1">
         <v>46321</v>
       </c>
     </row>
@@ -2038,7 +2012,7 @@
       <c r="U22" t="s">
         <v>92</v>
       </c>
-      <c r="V22" s="2">
+      <c r="V22" s="1">
         <v>46321</v>
       </c>
     </row>
@@ -2085,7 +2059,7 @@
       <c r="U23" t="s">
         <v>92</v>
       </c>
-      <c r="V23" s="2">
+      <c r="V23" s="1">
         <v>46321</v>
       </c>
     </row>
@@ -2132,7 +2106,7 @@
       <c r="U24" t="s">
         <v>92</v>
       </c>
-      <c r="V24" s="2">
+      <c r="V24" s="1">
         <v>46321</v>
       </c>
     </row>
@@ -2158,7 +2132,7 @@
       <c r="G25" t="s">
         <v>108</v>
       </c>
-      <c r="H25" s="2">
+      <c r="H25" s="1">
         <v>46119</v>
       </c>
       <c r="I25" t="s">
@@ -2188,7 +2162,7 @@
       <c r="U25" t="s">
         <v>175</v>
       </c>
-      <c r="V25" s="2">
+      <c r="V25" s="1">
         <v>46138</v>
       </c>
     </row>
@@ -2214,7 +2188,7 @@
       <c r="G26" t="s">
         <v>108</v>
       </c>
-      <c r="H26" s="2">
+      <c r="H26" s="1">
         <v>46121</v>
       </c>
       <c r="I26" t="s">
@@ -2241,7 +2215,7 @@
       <c r="U26" t="s">
         <v>92</v>
       </c>
-      <c r="V26" s="2">
+      <c r="V26" s="1">
         <v>46138</v>
       </c>
     </row>
@@ -2267,7 +2241,7 @@
       <c r="G27" t="s">
         <v>108</v>
       </c>
-      <c r="H27" s="2">
+      <c r="H27" s="1">
         <v>46076</v>
       </c>
       <c r="I27" t="s">
@@ -2294,7 +2268,7 @@
       <c r="U27" t="s">
         <v>92</v>
       </c>
-      <c r="V27" s="2">
+      <c r="V27" s="1">
         <v>46079</v>
       </c>
     </row>
@@ -2350,7 +2324,7 @@
       <c r="U28" t="s">
         <v>175</v>
       </c>
-      <c r="V28" s="2">
+      <c r="V28" s="1">
         <v>46291</v>
       </c>
     </row>
@@ -2376,7 +2350,7 @@
       <c r="G29" t="s">
         <v>108</v>
       </c>
-      <c r="H29" s="2">
+      <c r="H29" s="1">
         <v>46199</v>
       </c>
       <c r="I29" t="s">
@@ -2406,7 +2380,7 @@
       <c r="U29" t="s">
         <v>175</v>
       </c>
-      <c r="V29" s="2">
+      <c r="V29" s="1">
         <v>46199</v>
       </c>
     </row>
@@ -2432,7 +2406,7 @@
       <c r="G30" t="s">
         <v>108</v>
       </c>
-      <c r="H30" s="2">
+      <c r="H30" s="1">
         <v>46199</v>
       </c>
       <c r="I30" t="s">
@@ -2462,7 +2436,7 @@
       <c r="U30" t="s">
         <v>175</v>
       </c>
-      <c r="V30" s="2">
+      <c r="V30" s="1">
         <v>46199</v>
       </c>
     </row>
@@ -2488,7 +2462,7 @@
       <c r="G31" t="s">
         <v>108</v>
       </c>
-      <c r="H31" s="2">
+      <c r="H31" s="1">
         <v>46199</v>
       </c>
       <c r="I31" t="s">
@@ -2518,7 +2492,7 @@
       <c r="U31" t="s">
         <v>175</v>
       </c>
-      <c r="V31" s="2">
+      <c r="V31" s="1">
         <v>46199</v>
       </c>
     </row>
@@ -2544,7 +2518,7 @@
       <c r="G32" t="s">
         <v>108</v>
       </c>
-      <c r="H32" s="2">
+      <c r="H32" s="1">
         <v>46199</v>
       </c>
       <c r="I32" t="s">
@@ -2574,7 +2548,7 @@
       <c r="U32" t="s">
         <v>175</v>
       </c>
-      <c r="V32" s="2">
+      <c r="V32" s="1">
         <v>46199</v>
       </c>
     </row>
@@ -2624,7 +2598,7 @@
       <c r="U33" t="s">
         <v>175</v>
       </c>
-      <c r="V33" s="2">
+      <c r="V33" s="1">
         <v>46291</v>
       </c>
     </row>
@@ -2650,7 +2624,7 @@
       <c r="G34" t="s">
         <v>108</v>
       </c>
-      <c r="H34" s="2">
+      <c r="H34" s="1">
         <v>46191</v>
       </c>
       <c r="I34" t="s">
@@ -2680,7 +2654,7 @@
       <c r="U34" t="s">
         <v>175</v>
       </c>
-      <c r="V34" s="2">
+      <c r="V34" s="1">
         <v>46199</v>
       </c>
     </row>
@@ -2706,7 +2680,7 @@
       <c r="G35" t="s">
         <v>108</v>
       </c>
-      <c r="H35" s="2">
+      <c r="H35" s="1">
         <v>46119</v>
       </c>
       <c r="I35" t="s">
@@ -2733,7 +2707,7 @@
       <c r="U35" t="s">
         <v>175</v>
       </c>
-      <c r="V35" s="2">
+      <c r="V35" s="1">
         <v>46138</v>
       </c>
     </row>
@@ -2759,7 +2733,7 @@
       <c r="G36" t="s">
         <v>108</v>
       </c>
-      <c r="H36" s="2">
+      <c r="H36" s="1">
         <v>46213</v>
       </c>
       <c r="I36" t="s">
@@ -2786,7 +2760,7 @@
       <c r="U36" t="s">
         <v>92</v>
       </c>
-      <c r="V36" s="2">
+      <c r="V36" s="1">
         <v>46229</v>
       </c>
     </row>
@@ -2812,7 +2786,7 @@
       <c r="G37" t="s">
         <v>108</v>
       </c>
-      <c r="H37" s="2">
+      <c r="H37" s="1">
         <v>46175</v>
       </c>
       <c r="I37" t="s">
@@ -2839,7 +2813,7 @@
       <c r="U37" t="s">
         <v>92</v>
       </c>
-      <c r="V37" s="2">
+      <c r="V37" s="1">
         <v>46199</v>
       </c>
     </row>
@@ -2865,7 +2839,7 @@
       <c r="G38" t="s">
         <v>108</v>
       </c>
-      <c r="H38" s="2">
+      <c r="H38" s="1">
         <v>46213</v>
       </c>
       <c r="I38" t="s">
@@ -2892,7 +2866,7 @@
       <c r="U38" t="s">
         <v>92</v>
       </c>
-      <c r="V38" s="2">
+      <c r="V38" s="1">
         <v>46229</v>
       </c>
     </row>
@@ -2918,7 +2892,7 @@
       <c r="G39" t="s">
         <v>108</v>
       </c>
-      <c r="H39" s="2">
+      <c r="H39" s="1">
         <v>46199</v>
       </c>
       <c r="I39" t="s">
@@ -2945,7 +2919,7 @@
       <c r="U39" t="s">
         <v>92</v>
       </c>
-      <c r="V39" s="2">
+      <c r="V39" s="1">
         <v>46199</v>
       </c>
     </row>
@@ -2971,7 +2945,7 @@
       <c r="G40" t="s">
         <v>108</v>
       </c>
-      <c r="H40" s="2">
+      <c r="H40" s="1">
         <v>46199</v>
       </c>
       <c r="I40" t="s">
@@ -2998,7 +2972,7 @@
       <c r="U40" t="s">
         <v>92</v>
       </c>
-      <c r="V40" s="2">
+      <c r="V40" s="1">
         <v>46199</v>
       </c>
     </row>
@@ -3024,7 +2998,7 @@
       <c r="G41" t="s">
         <v>108</v>
       </c>
-      <c r="H41" s="2">
+      <c r="H41" s="1">
         <v>46204</v>
       </c>
       <c r="I41" t="s">
@@ -3051,7 +3025,7 @@
       <c r="U41" t="s">
         <v>92</v>
       </c>
-      <c r="V41" s="2">
+      <c r="V41" s="1">
         <v>46229</v>
       </c>
     </row>
@@ -3077,7 +3051,7 @@
       <c r="G42" t="s">
         <v>108</v>
       </c>
-      <c r="H42" s="2">
+      <c r="H42" s="1">
         <v>46244</v>
       </c>
       <c r="I42" t="s">
@@ -3104,7 +3078,7 @@
       <c r="U42" t="s">
         <v>92</v>
       </c>
-      <c r="V42" s="2">
+      <c r="V42" s="1">
         <v>46199</v>
       </c>
     </row>
@@ -3148,7 +3122,7 @@
       <c r="U43" t="s">
         <v>92</v>
       </c>
-      <c r="V43" s="2">
+      <c r="V43" s="1">
         <v>46260</v>
       </c>
     </row>
@@ -3174,7 +3148,7 @@
       <c r="G44" t="s">
         <v>108</v>
       </c>
-      <c r="H44" s="2">
+      <c r="H44" s="1">
         <v>46191</v>
       </c>
       <c r="I44" t="s">
@@ -3201,7 +3175,7 @@
       <c r="U44" t="s">
         <v>92</v>
       </c>
-      <c r="V44" s="2">
+      <c r="V44" s="1">
         <v>46199</v>
       </c>
     </row>
@@ -3227,7 +3201,7 @@
       <c r="G45" t="s">
         <v>108</v>
       </c>
-      <c r="H45" s="2">
+      <c r="H45" s="1">
         <v>46191</v>
       </c>
       <c r="I45" t="s">
@@ -3254,7 +3228,7 @@
       <c r="U45" t="s">
         <v>92</v>
       </c>
-      <c r="V45" s="2">
+      <c r="V45" s="1">
         <v>46199</v>
       </c>
     </row>
@@ -3280,7 +3254,7 @@
       <c r="G46" t="s">
         <v>108</v>
       </c>
-      <c r="H46" s="2">
+      <c r="H46" s="1">
         <v>46213</v>
       </c>
       <c r="I46" t="s">
@@ -3310,7 +3284,7 @@
       <c r="U46" t="s">
         <v>175</v>
       </c>
-      <c r="V46" s="2">
+      <c r="V46" s="1">
         <v>46229</v>
       </c>
     </row>
@@ -3336,7 +3310,7 @@
       <c r="G47" t="s">
         <v>108</v>
       </c>
-      <c r="H47" s="2">
+      <c r="H47" s="1">
         <v>46210</v>
       </c>
       <c r="I47" t="s">
@@ -3363,7 +3337,7 @@
       <c r="U47" t="s">
         <v>175</v>
       </c>
-      <c r="V47" s="2">
+      <c r="V47" s="1">
         <v>46229</v>
       </c>
     </row>
@@ -3407,7 +3381,7 @@
       <c r="U48" t="s">
         <v>92</v>
       </c>
-      <c r="V48" s="2">
+      <c r="V48" s="1">
         <v>46321</v>
       </c>
     </row>
@@ -3463,7 +3437,7 @@
       <c r="U49" t="s">
         <v>175</v>
       </c>
-      <c r="V49" s="2">
+      <c r="V49" s="1">
         <v>46291</v>
       </c>
     </row>
@@ -3489,7 +3463,7 @@
       <c r="G50" t="s">
         <v>108</v>
       </c>
-      <c r="H50" s="2">
+      <c r="H50" s="1">
         <v>46176</v>
       </c>
       <c r="I50" t="s">
@@ -3519,7 +3493,7 @@
       <c r="U50" t="s">
         <v>175</v>
       </c>
-      <c r="V50" s="2">
+      <c r="V50" s="1">
         <v>46199</v>
       </c>
     </row>
@@ -3572,7 +3546,7 @@
       <c r="U51" t="s">
         <v>175</v>
       </c>
-      <c r="V51" s="2">
+      <c r="V51" s="1">
         <v>46260</v>
       </c>
     </row>
@@ -3598,7 +3572,7 @@
       <c r="G52" t="s">
         <v>108</v>
       </c>
-      <c r="H52" s="2">
+      <c r="H52" s="1">
         <v>46295</v>
       </c>
       <c r="I52" t="s">
@@ -3631,7 +3605,7 @@
       <c r="U52" t="s">
         <v>175</v>
       </c>
-      <c r="V52" s="2">
+      <c r="V52" s="1">
         <v>46291</v>
       </c>
     </row>
@@ -3681,7 +3655,7 @@
       <c r="U53" t="s">
         <v>175</v>
       </c>
-      <c r="V53" s="2">
+      <c r="V53" s="1">
         <v>46321</v>
       </c>
     </row>
@@ -3707,7 +3681,7 @@
       <c r="G54" t="s">
         <v>108</v>
       </c>
-      <c r="H54" s="2">
+      <c r="H54" s="1">
         <v>46227</v>
       </c>
       <c r="I54" t="s">
@@ -3734,7 +3708,7 @@
       <c r="U54" t="s">
         <v>175</v>
       </c>
-      <c r="V54" s="2">
+      <c r="V54" s="1">
         <v>46229</v>
       </c>
     </row>
@@ -3757,7 +3731,7 @@
       <c r="G55" t="s">
         <v>108</v>
       </c>
-      <c r="H55" s="2">
+      <c r="H55" s="1">
         <v>46280</v>
       </c>
       <c r="I55" t="s">
@@ -3784,7 +3758,7 @@
       <c r="U55" t="s">
         <v>175</v>
       </c>
-      <c r="V55" s="2">
+      <c r="V55" s="1">
         <v>46291</v>
       </c>
     </row>
@@ -3807,7 +3781,7 @@
       <c r="G56" t="s">
         <v>108</v>
       </c>
-      <c r="H56" s="2">
+      <c r="H56" s="1">
         <v>46280</v>
       </c>
       <c r="I56" t="s">
@@ -3834,7 +3808,7 @@
       <c r="U56" t="s">
         <v>175</v>
       </c>
-      <c r="V56" s="2">
+      <c r="V56" s="1">
         <v>46260</v>
       </c>
     </row>
@@ -3857,7 +3831,7 @@
       <c r="G57" t="s">
         <v>108</v>
       </c>
-      <c r="H57" s="2">
+      <c r="H57" s="1">
         <v>46295</v>
       </c>
       <c r="I57" t="s">
@@ -3884,7 +3858,7 @@
       <c r="U57" t="s">
         <v>175</v>
       </c>
-      <c r="V57" s="2">
+      <c r="V57" s="1">
         <v>46291</v>
       </c>
     </row>
@@ -3907,7 +3881,7 @@
       <c r="G58" t="s">
         <v>108</v>
       </c>
-      <c r="H58" s="2">
+      <c r="H58" s="1">
         <v>46295</v>
       </c>
       <c r="I58" t="s">
@@ -3934,7 +3908,7 @@
       <c r="U58" t="s">
         <v>175</v>
       </c>
-      <c r="V58" s="2">
+      <c r="V58" s="1">
         <v>46291</v>
       </c>
     </row>
@@ -3960,7 +3934,7 @@
       <c r="G59" t="s">
         <v>109</v>
       </c>
-      <c r="H59" s="2">
+      <c r="H59" s="1">
         <v>46301</v>
       </c>
       <c r="J59" t="s">
@@ -3990,7 +3964,7 @@
       <c r="U59" t="s">
         <v>175</v>
       </c>
-      <c r="V59" s="2">
+      <c r="V59" s="1">
         <v>46352</v>
       </c>
     </row>
@@ -4031,7 +4005,7 @@
       <c r="U60" t="s">
         <v>175</v>
       </c>
-      <c r="V60" s="2">
+      <c r="V60" s="1">
         <v>46107</v>
       </c>
     </row>
@@ -4072,7 +4046,7 @@
       <c r="U61" t="s">
         <v>175</v>
       </c>
-      <c r="V61" s="2">
+      <c r="V61" s="1">
         <v>46107</v>
       </c>
     </row>
@@ -4113,7 +4087,7 @@
       <c r="U62" t="s">
         <v>175</v>
       </c>
-      <c r="V62" s="2">
+      <c r="V62" s="1">
         <v>46107</v>
       </c>
     </row>
@@ -4154,7 +4128,7 @@
       <c r="U63" t="s">
         <v>175</v>
       </c>
-      <c r="V63" s="2">
+      <c r="V63" s="1">
         <v>46107</v>
       </c>
     </row>
@@ -4195,7 +4169,7 @@
       <c r="U64" t="s">
         <v>175</v>
       </c>
-      <c r="V64" s="2">
+      <c r="V64" s="1">
         <v>46107</v>
       </c>
     </row>
@@ -4236,7 +4210,7 @@
       <c r="U65" t="s">
         <v>175</v>
       </c>
-      <c r="V65" s="2">
+      <c r="V65" s="1">
         <v>46107</v>
       </c>
     </row>
@@ -4277,7 +4251,7 @@
       <c r="U66" t="s">
         <v>92</v>
       </c>
-      <c r="V66" s="2">
+      <c r="V66" s="1">
         <v>46168</v>
       </c>
     </row>
@@ -4324,7 +4298,7 @@
       <c r="U67" t="s">
         <v>92</v>
       </c>
-      <c r="V67" s="2">
+      <c r="V67" s="1">
         <v>46291</v>
       </c>
     </row>
@@ -4380,7 +4354,7 @@
       <c r="U68" t="s">
         <v>175</v>
       </c>
-      <c r="V68" s="2">
+      <c r="V68" s="1">
         <v>46229</v>
       </c>
     </row>
@@ -4421,7 +4395,7 @@
       <c r="U69" t="s">
         <v>92</v>
       </c>
-      <c r="V69" s="2">
+      <c r="V69" s="1">
         <v>46260</v>
       </c>
     </row>
@@ -4462,7 +4436,7 @@
       <c r="U70" t="s">
         <v>175</v>
       </c>
-      <c r="V70" s="2">
+      <c r="V70" s="1">
         <v>46291</v>
       </c>
     </row>
@@ -4503,7 +4477,7 @@
       <c r="U71" t="s">
         <v>175</v>
       </c>
-      <c r="V71" s="2">
+      <c r="V71" s="1">
         <v>46168</v>
       </c>
     </row>
@@ -4544,7 +4518,7 @@
       <c r="U72" t="s">
         <v>175</v>
       </c>
-      <c r="V72" s="2">
+      <c r="V72" s="1">
         <v>46291</v>
       </c>
     </row>
@@ -4585,7 +4559,7 @@
       <c r="U73" t="s">
         <v>175</v>
       </c>
-      <c r="V73" s="2">
+      <c r="V73" s="1">
         <v>46291</v>
       </c>
     </row>
@@ -4626,7 +4600,7 @@
       <c r="U74" t="s">
         <v>175</v>
       </c>
-      <c r="V74" s="2">
+      <c r="V74" s="1">
         <v>46291</v>
       </c>
     </row>
@@ -4670,7 +4644,7 @@
       <c r="U75" t="s">
         <v>92</v>
       </c>
-      <c r="V75" s="2">
+      <c r="V75" s="1">
         <v>46321</v>
       </c>
     </row>
@@ -4717,7 +4691,7 @@
       <c r="U76" t="s">
         <v>175</v>
       </c>
-      <c r="V76" s="2">
+      <c r="V76" s="1">
         <v>46381</v>
       </c>
     </row>
@@ -4764,7 +4738,7 @@
       <c r="U77" t="s">
         <v>175</v>
       </c>
-      <c r="V77" s="2">
+      <c r="V77" s="1">
         <v>46381</v>
       </c>
     </row>
@@ -4811,7 +4785,7 @@
       <c r="U78" t="s">
         <v>92</v>
       </c>
-      <c r="V78" s="2">
+      <c r="V78" s="1">
         <v>46381</v>
       </c>
     </row>
@@ -4858,7 +4832,7 @@
       <c r="U79" t="s">
         <v>92</v>
       </c>
-      <c r="V79" s="2">
+      <c r="V79" s="1">
         <v>46381</v>
       </c>
     </row>
@@ -4905,7 +4879,7 @@
       <c r="U80" t="s">
         <v>92</v>
       </c>
-      <c r="V80" s="2">
+      <c r="V80" s="1">
         <v>46382</v>
       </c>
     </row>
@@ -4946,7 +4920,7 @@
       <c r="U81" t="s">
         <v>92</v>
       </c>
-      <c r="V81" s="2">
+      <c r="V81" s="1">
         <v>46382</v>
       </c>
     </row>
@@ -4999,7 +4973,7 @@
       <c r="U82" t="s">
         <v>175</v>
       </c>
-      <c r="V82" s="2">
+      <c r="V82" s="1">
         <v>46382</v>
       </c>
     </row>
@@ -5046,7 +5020,7 @@
       <c r="U83" t="s">
         <v>92</v>
       </c>
-      <c r="V83" s="2">
+      <c r="V83" s="1">
         <v>46321</v>
       </c>
     </row>
@@ -5087,7 +5061,7 @@
       <c r="U84" t="s">
         <v>92</v>
       </c>
-      <c r="V84" s="2">
+      <c r="V84" s="1">
         <v>46382</v>
       </c>
     </row>
@@ -5225,7 +5199,7 @@
       <c r="U87" t="s">
         <v>92</v>
       </c>
-      <c r="V87" s="2">
+      <c r="V87" s="1">
         <v>46291</v>
       </c>
     </row>
@@ -5269,7 +5243,7 @@
       <c r="U88" t="s">
         <v>92</v>
       </c>
-      <c r="V88" s="2">
+      <c r="V88" s="1">
         <v>46291</v>
       </c>
     </row>

</xml_diff>

<commit_message>
MTA: corrige parser de valor monetário que zerava a soma — aceita agora string formatada ('R$ 135.000,00'), não só número puro. Achado pelo Wallace (10/10/26): coluna Valor da planilha passou a vir como texto e quase tudo (86 de 87 linhas) caía como 'inválido'/não somado; soma foi de ~0 para R$ 73.318.290,43
</commit_message>
<xml_diff>
--- a/Projetos/02_Dados_Tratados/base_mta_tratada.xlsx
+++ b/Projetos/02_Dados_Tratados/base_mta_tratada.xlsx
@@ -1014,6 +1014,9 @@
       <c r="O2" t="s">
         <v>23</v>
       </c>
+      <c r="P2">
+        <v>135000</v>
+      </c>
       <c r="Q2" t="s">
         <v>163</v>
       </c>
@@ -1258,6 +1261,9 @@
       <c r="O7" t="s">
         <v>28</v>
       </c>
+      <c r="P7">
+        <v>3799999.6</v>
+      </c>
       <c r="Q7" t="s">
         <v>164</v>
       </c>
@@ -1349,6 +1355,9 @@
       <c r="O9" t="s">
         <v>30</v>
       </c>
+      <c r="P9">
+        <v>36104.46</v>
+      </c>
       <c r="Q9" t="s">
         <v>163</v>
       </c>
@@ -1396,6 +1405,9 @@
       <c r="O10" t="s">
         <v>30</v>
       </c>
+      <c r="P10">
+        <v>23895.54</v>
+      </c>
       <c r="Q10" t="s">
         <v>163</v>
       </c>
@@ -1546,6 +1558,9 @@
       <c r="O13" t="s">
         <v>33</v>
       </c>
+      <c r="P13">
+        <v>1187433.02</v>
+      </c>
       <c r="Q13" t="s">
         <v>163</v>
       </c>
@@ -1602,6 +1617,9 @@
       <c r="O14" t="s">
         <v>34</v>
       </c>
+      <c r="P14">
+        <v>1000000</v>
+      </c>
       <c r="Q14" t="s">
         <v>163</v>
       </c>
@@ -1658,6 +1676,9 @@
       <c r="O15" t="s">
         <v>35</v>
       </c>
+      <c r="P15">
+        <v>1000000</v>
+      </c>
       <c r="Q15" t="s">
         <v>163</v>
       </c>
@@ -1714,6 +1735,9 @@
       <c r="O16" t="s">
         <v>36</v>
       </c>
+      <c r="P16">
+        <v>1000000</v>
+      </c>
       <c r="Q16" t="s">
         <v>163</v>
       </c>
@@ -1770,6 +1794,9 @@
       <c r="O17" t="s">
         <v>37</v>
       </c>
+      <c r="P17">
+        <v>100000</v>
+      </c>
       <c r="Q17" t="s">
         <v>165</v>
       </c>
@@ -1826,6 +1853,9 @@
       <c r="O18" t="s">
         <v>38</v>
       </c>
+      <c r="P18">
+        <v>1770880.5</v>
+      </c>
       <c r="Q18" t="s">
         <v>164</v>
       </c>
@@ -1879,6 +1909,9 @@
       <c r="O19" t="s">
         <v>39</v>
       </c>
+      <c r="P19">
+        <v>350000</v>
+      </c>
       <c r="Q19" t="s">
         <v>164</v>
       </c>
@@ -1932,6 +1965,9 @@
       <c r="O20" t="s">
         <v>40</v>
       </c>
+      <c r="P20">
+        <v>350000</v>
+      </c>
       <c r="Q20" t="s">
         <v>164</v>
       </c>
@@ -1976,6 +2012,9 @@
       <c r="O21" t="s">
         <v>41</v>
       </c>
+      <c r="P21">
+        <v>1000000</v>
+      </c>
       <c r="Q21" t="s">
         <v>164</v>
       </c>
@@ -2173,6 +2212,9 @@
       <c r="O25" t="s">
         <v>45</v>
       </c>
+      <c r="P25">
+        <v>1704503</v>
+      </c>
       <c r="Q25" t="s">
         <v>164</v>
       </c>
@@ -2226,6 +2268,9 @@
       <c r="O26" t="s">
         <v>46</v>
       </c>
+      <c r="P26">
+        <v>3799000</v>
+      </c>
       <c r="Q26" t="s">
         <v>164</v>
       </c>
@@ -2279,6 +2324,9 @@
       <c r="O27" t="s">
         <v>46</v>
       </c>
+      <c r="P27">
+        <v>1000</v>
+      </c>
       <c r="Q27" t="s">
         <v>164</v>
       </c>
@@ -2335,6 +2383,9 @@
       <c r="O28" t="s">
         <v>47</v>
       </c>
+      <c r="P28">
+        <v>100000</v>
+      </c>
       <c r="Q28" t="s">
         <v>165</v>
       </c>
@@ -2391,6 +2442,9 @@
       <c r="O29" t="s">
         <v>48</v>
       </c>
+      <c r="P29">
+        <v>150000</v>
+      </c>
       <c r="Q29" t="s">
         <v>164</v>
       </c>
@@ -2447,6 +2501,9 @@
       <c r="O30" t="s">
         <v>49</v>
       </c>
+      <c r="P30">
+        <v>150000</v>
+      </c>
       <c r="Q30" t="s">
         <v>164</v>
       </c>
@@ -2503,6 +2560,9 @@
       <c r="O31" t="s">
         <v>50</v>
       </c>
+      <c r="P31">
+        <v>18462.36</v>
+      </c>
       <c r="Q31" t="s">
         <v>164</v>
       </c>
@@ -2559,6 +2619,9 @@
       <c r="O32" t="s">
         <v>50</v>
       </c>
+      <c r="P32">
+        <v>324166.14</v>
+      </c>
       <c r="Q32" t="s">
         <v>164</v>
       </c>
@@ -2609,6 +2672,9 @@
       <c r="O33" t="s">
         <v>51</v>
       </c>
+      <c r="P33">
+        <v>30000</v>
+      </c>
       <c r="Q33" t="s">
         <v>164</v>
       </c>
@@ -2665,6 +2731,9 @@
       <c r="O34" t="s">
         <v>52</v>
       </c>
+      <c r="P34">
+        <v>1496713.48</v>
+      </c>
       <c r="Q34" t="s">
         <v>164</v>
       </c>
@@ -2718,6 +2787,9 @@
       <c r="O35" t="s">
         <v>52</v>
       </c>
+      <c r="P35">
+        <v>207789.52</v>
+      </c>
       <c r="Q35" t="s">
         <v>164</v>
       </c>
@@ -2771,6 +2843,9 @@
       <c r="O36" t="s">
         <v>53</v>
       </c>
+      <c r="P36">
+        <v>962290.8</v>
+      </c>
       <c r="Q36" t="s">
         <v>164</v>
       </c>
@@ -2824,6 +2899,9 @@
       <c r="O37" t="s">
         <v>53</v>
       </c>
+      <c r="P37">
+        <v>798776.97</v>
+      </c>
       <c r="Q37" t="s">
         <v>164</v>
       </c>
@@ -2877,6 +2955,9 @@
       <c r="O38" t="s">
         <v>53</v>
       </c>
+      <c r="P38">
+        <v>1530656.62</v>
+      </c>
       <c r="Q38" t="s">
         <v>164</v>
       </c>
@@ -2930,6 +3011,9 @@
       <c r="O39" t="s">
         <v>53</v>
       </c>
+      <c r="P39">
+        <v>72958.08</v>
+      </c>
       <c r="Q39" t="s">
         <v>164</v>
       </c>
@@ -2983,6 +3067,9 @@
       <c r="O40" t="s">
         <v>53</v>
       </c>
+      <c r="P40">
+        <v>8916</v>
+      </c>
       <c r="Q40" t="s">
         <v>164</v>
       </c>
@@ -3036,6 +3123,9 @@
       <c r="O41" t="s">
         <v>53</v>
       </c>
+      <c r="P41">
+        <v>425178.5</v>
+      </c>
       <c r="Q41" t="s">
         <v>164</v>
       </c>
@@ -3089,6 +3179,9 @@
       <c r="O42" t="s">
         <v>53</v>
       </c>
+      <c r="P42">
+        <v>1223.03</v>
+      </c>
       <c r="Q42" t="s">
         <v>164</v>
       </c>
@@ -3186,6 +3279,9 @@
       <c r="O44" t="s">
         <v>55</v>
       </c>
+      <c r="P44">
+        <v>400000</v>
+      </c>
       <c r="Q44" t="s">
         <v>164</v>
       </c>
@@ -3239,6 +3335,9 @@
       <c r="O45" t="s">
         <v>56</v>
       </c>
+      <c r="P45">
+        <v>400000</v>
+      </c>
       <c r="Q45" t="s">
         <v>164</v>
       </c>
@@ -3295,6 +3394,9 @@
       <c r="O46" t="s">
         <v>57</v>
       </c>
+      <c r="P46">
+        <v>173846.38</v>
+      </c>
       <c r="Q46" t="s">
         <v>164</v>
       </c>
@@ -3348,6 +3450,9 @@
       <c r="O47" t="s">
         <v>57</v>
       </c>
+      <c r="P47">
+        <v>1530656.62</v>
+      </c>
       <c r="Q47" t="s">
         <v>164</v>
       </c>
@@ -3392,6 +3497,9 @@
       <c r="O48" t="s">
         <v>58</v>
       </c>
+      <c r="P48">
+        <v>1000000</v>
+      </c>
       <c r="Q48" t="s">
         <v>164</v>
       </c>
@@ -3448,6 +3556,9 @@
       <c r="O49" t="s">
         <v>59</v>
       </c>
+      <c r="P49">
+        <v>958040</v>
+      </c>
       <c r="Q49" t="s">
         <v>163</v>
       </c>
@@ -3504,6 +3615,9 @@
       <c r="O50" t="s">
         <v>59</v>
       </c>
+      <c r="P50">
+        <v>41730.64</v>
+      </c>
       <c r="Q50" t="s">
         <v>163</v>
       </c>
@@ -3557,6 +3671,9 @@
       <c r="O51" t="s">
         <v>60</v>
       </c>
+      <c r="P51">
+        <v>608623.25</v>
+      </c>
       <c r="Q51" t="s">
         <v>164</v>
       </c>
@@ -3616,6 +3733,9 @@
       <c r="O52" t="s">
         <v>61</v>
       </c>
+      <c r="P52">
+        <v>66366.75999999999</v>
+      </c>
       <c r="Q52" t="s">
         <v>164</v>
       </c>
@@ -3666,6 +3786,9 @@
       <c r="O53" t="s">
         <v>62</v>
       </c>
+      <c r="P53">
+        <v>1704503</v>
+      </c>
       <c r="Q53" t="s">
         <v>164</v>
       </c>
@@ -3719,6 +3842,9 @@
       <c r="O54" t="s">
         <v>60</v>
       </c>
+      <c r="P54">
+        <v>236343.68</v>
+      </c>
       <c r="Q54" t="s">
         <v>164</v>
       </c>
@@ -3769,6 +3895,9 @@
       <c r="O55" t="s">
         <v>61</v>
       </c>
+      <c r="P55">
+        <v>1145462.93</v>
+      </c>
       <c r="Q55" t="s">
         <v>164</v>
       </c>
@@ -3819,6 +3948,9 @@
       <c r="O56" t="s">
         <v>60</v>
       </c>
+      <c r="P56">
+        <v>859536.0699999999</v>
+      </c>
       <c r="Q56" t="s">
         <v>164</v>
       </c>
@@ -3869,6 +4001,9 @@
       <c r="O57" t="s">
         <v>61</v>
       </c>
+      <c r="P57">
+        <v>389619.06</v>
+      </c>
       <c r="Q57" t="s">
         <v>164</v>
       </c>
@@ -3919,6 +4054,9 @@
       <c r="O58" t="s">
         <v>61</v>
       </c>
+      <c r="P58">
+        <v>103054.25</v>
+      </c>
       <c r="Q58" t="s">
         <v>164</v>
       </c>
@@ -3975,6 +4113,9 @@
       <c r="O59" t="s">
         <v>63</v>
       </c>
+      <c r="P59">
+        <v>1295422.28</v>
+      </c>
       <c r="Q59" t="s">
         <v>164</v>
       </c>
@@ -4016,6 +4157,9 @@
       <c r="O60" t="s">
         <v>64</v>
       </c>
+      <c r="P60">
+        <v>4064.54</v>
+      </c>
       <c r="Q60" t="s">
         <v>164</v>
       </c>
@@ -4057,6 +4201,9 @@
       <c r="O61" t="s">
         <v>65</v>
       </c>
+      <c r="P61">
+        <v>4227.84</v>
+      </c>
       <c r="Q61" t="s">
         <v>163</v>
       </c>
@@ -4098,6 +4245,9 @@
       <c r="O62" t="s">
         <v>66</v>
       </c>
+      <c r="P62">
+        <v>9389.959999999999</v>
+      </c>
       <c r="Q62" t="s">
         <v>163</v>
       </c>
@@ -4139,6 +4289,9 @@
       <c r="O63" t="s">
         <v>67</v>
       </c>
+      <c r="P63">
+        <v>1163.64</v>
+      </c>
       <c r="Q63" t="s">
         <v>165</v>
       </c>
@@ -4180,6 +4333,9 @@
       <c r="O64" t="s">
         <v>68</v>
       </c>
+      <c r="P64">
+        <v>7204.82</v>
+      </c>
       <c r="Q64" t="s">
         <v>163</v>
       </c>
@@ -4221,6 +4377,9 @@
       <c r="O65" t="s">
         <v>65</v>
       </c>
+      <c r="P65">
+        <v>3662.66</v>
+      </c>
       <c r="Q65" t="s">
         <v>163</v>
       </c>
@@ -4262,6 +4421,9 @@
       <c r="O66" t="s">
         <v>69</v>
       </c>
+      <c r="P66">
+        <v>120000</v>
+      </c>
       <c r="Q66" t="s">
         <v>163</v>
       </c>
@@ -4365,6 +4527,9 @@
       <c r="O68" t="s">
         <v>71</v>
       </c>
+      <c r="P68">
+        <v>100000</v>
+      </c>
       <c r="Q68" t="s">
         <v>165</v>
       </c>
@@ -4406,6 +4571,9 @@
       <c r="O69" t="s">
         <v>72</v>
       </c>
+      <c r="P69">
+        <v>80000</v>
+      </c>
       <c r="Q69" t="s">
         <v>163</v>
       </c>
@@ -4447,6 +4615,9 @@
       <c r="O70" t="s">
         <v>73</v>
       </c>
+      <c r="P70">
+        <v>835000</v>
+      </c>
       <c r="Q70" t="s">
         <v>163</v>
       </c>
@@ -4488,6 +4659,9 @@
       <c r="O71" t="s">
         <v>73</v>
       </c>
+      <c r="P71">
+        <v>165000</v>
+      </c>
       <c r="Q71" t="s">
         <v>163</v>
       </c>
@@ -4529,6 +4703,9 @@
       <c r="O72" t="s">
         <v>74</v>
       </c>
+      <c r="P72">
+        <v>1000000</v>
+      </c>
       <c r="Q72" t="s">
         <v>163</v>
       </c>
@@ -4570,6 +4747,9 @@
       <c r="O73" t="s">
         <v>75</v>
       </c>
+      <c r="P73">
+        <v>1000000</v>
+      </c>
       <c r="Q73" t="s">
         <v>163</v>
       </c>
@@ -4611,6 +4791,9 @@
       <c r="O74" t="s">
         <v>76</v>
       </c>
+      <c r="P74">
+        <v>100000</v>
+      </c>
       <c r="Q74" t="s">
         <v>165</v>
       </c>
@@ -4655,6 +4838,9 @@
       <c r="O75" t="s">
         <v>77</v>
       </c>
+      <c r="P75">
+        <v>1000000</v>
+      </c>
       <c r="Q75" t="s">
         <v>164</v>
       </c>
@@ -4702,6 +4888,9 @@
       <c r="O76" t="s">
         <v>78</v>
       </c>
+      <c r="P76">
+        <v>1704503</v>
+      </c>
       <c r="Q76" t="s">
         <v>164</v>
       </c>
@@ -4749,6 +4938,9 @@
       <c r="O77" t="s">
         <v>79</v>
       </c>
+      <c r="P77">
+        <v>1638125.5</v>
+      </c>
       <c r="Q77" t="s">
         <v>164</v>
       </c>
@@ -4796,6 +4988,9 @@
       <c r="O78" t="s">
         <v>80</v>
       </c>
+      <c r="P78">
+        <v>3800000</v>
+      </c>
       <c r="Q78" t="s">
         <v>164</v>
       </c>
@@ -4843,6 +5038,9 @@
       <c r="O79" t="s">
         <v>81</v>
       </c>
+      <c r="P79">
+        <v>3800000</v>
+      </c>
       <c r="Q79" t="s">
         <v>164</v>
       </c>
@@ -4890,6 +5088,9 @@
       <c r="O80" t="s">
         <v>82</v>
       </c>
+      <c r="P80">
+        <v>3800000</v>
+      </c>
       <c r="Q80" t="s">
         <v>164</v>
       </c>
@@ -4931,6 +5132,9 @@
       <c r="O81" t="s">
         <v>83</v>
       </c>
+      <c r="P81">
+        <v>4394700</v>
+      </c>
       <c r="Q81" t="s">
         <v>163</v>
       </c>
@@ -4984,6 +5188,9 @@
       <c r="O82" t="s">
         <v>84</v>
       </c>
+      <c r="P82">
+        <v>528395.9300000001</v>
+      </c>
       <c r="Q82" t="s">
         <v>164</v>
       </c>
@@ -5031,6 +5238,9 @@
       <c r="O83" t="s">
         <v>85</v>
       </c>
+      <c r="P83">
+        <v>1000000</v>
+      </c>
       <c r="Q83" t="s">
         <v>164</v>
       </c>
@@ -5072,6 +5282,9 @@
       <c r="O84" t="s">
         <v>83</v>
       </c>
+      <c r="P84">
+        <v>4394700</v>
+      </c>
       <c r="Q84" t="s">
         <v>163</v>
       </c>
@@ -5119,6 +5332,9 @@
       <c r="O85" t="s">
         <v>83</v>
       </c>
+      <c r="P85">
+        <v>3306000</v>
+      </c>
       <c r="Q85" t="s">
         <v>163</v>
       </c>
@@ -5163,6 +5379,9 @@
       <c r="O86" t="s">
         <v>83</v>
       </c>
+      <c r="P86">
+        <v>3306000</v>
+      </c>
       <c r="Q86" t="s">
         <v>163</v>
       </c>
@@ -5210,6 +5429,9 @@
       <c r="O87" t="s">
         <v>86</v>
       </c>
+      <c r="P87">
+        <v>470820</v>
+      </c>
       <c r="Q87" t="s">
         <v>163</v>
       </c>
@@ -5253,6 +5475,9 @@
       </c>
       <c r="O88" t="s">
         <v>162</v>
+      </c>
+      <c r="P88">
+        <v>2297180</v>
       </c>
       <c r="Q88" t="s">
         <v>164</v>

</xml_diff>

<commit_message>
Atualização automática: mta (08/10/2026 14:51)
</commit_message>
<xml_diff>
--- a/Projetos/02_Dados_Tratados/base_mta_tratada.xlsx
+++ b/Projetos/02_Dados_Tratados/base_mta_tratada.xlsx
@@ -551,16 +551,8 @@
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="YYYY-MM-DD HH:MM:SS"/>
   </numFmts>
-  <fonts count="2">
+  <fonts count="1">
     <font>
-      <sz val="11"/>
-      <color theme="1"/>
-      <name val="Calibri"/>
-      <family val="2"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <b/>
       <sz val="11"/>
       <color theme="1"/>
       <name val="Calibri"/>
@@ -576,7 +568,7 @@
       <patternFill patternType="gray125"/>
     </fill>
   </fills>
-  <borders count="2">
+  <borders count="1">
     <border>
       <left/>
       <right/>
@@ -584,30 +576,12 @@
       <bottom/>
       <diagonal/>
     </border>
-    <border>
-      <left style="thin">
-        <color auto="1"/>
-      </left>
-      <right style="thin">
-        <color auto="1"/>
-      </right>
-      <top style="thin">
-        <color auto="1"/>
-      </top>
-      <bottom style="thin">
-        <color auto="1"/>
-      </bottom>
-      <diagonal/>
-    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="3">
+  <cellXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top"/>
-    </xf>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
   </cellXfs>
   <cellStyles count="1">
@@ -907,70 +881,70 @@
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:22">
-      <c r="A1" s="1" t="s">
+      <c r="A1" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="1" t="s">
+      <c r="B1" t="s">
         <v>1</v>
       </c>
-      <c r="C1" s="1" t="s">
+      <c r="C1" t="s">
         <v>2</v>
       </c>
-      <c r="D1" s="1" t="s">
+      <c r="D1" t="s">
         <v>3</v>
       </c>
-      <c r="E1" s="1" t="s">
+      <c r="E1" t="s">
         <v>4</v>
       </c>
-      <c r="F1" s="1" t="s">
+      <c r="F1" t="s">
         <v>5</v>
       </c>
-      <c r="G1" s="1" t="s">
+      <c r="G1" t="s">
         <v>6</v>
       </c>
-      <c r="H1" s="1" t="s">
+      <c r="H1" t="s">
         <v>7</v>
       </c>
-      <c r="I1" s="1" t="s">
+      <c r="I1" t="s">
         <v>8</v>
       </c>
-      <c r="J1" s="1" t="s">
+      <c r="J1" t="s">
         <v>9</v>
       </c>
-      <c r="K1" s="1" t="s">
+      <c r="K1" t="s">
         <v>10</v>
       </c>
-      <c r="L1" s="1" t="s">
+      <c r="L1" t="s">
         <v>11</v>
       </c>
-      <c r="M1" s="1" t="s">
+      <c r="M1" t="s">
         <v>12</v>
       </c>
-      <c r="N1" s="1" t="s">
+      <c r="N1" t="s">
         <v>13</v>
       </c>
-      <c r="O1" s="1" t="s">
+      <c r="O1" t="s">
         <v>14</v>
       </c>
-      <c r="P1" s="1" t="s">
+      <c r="P1" t="s">
         <v>15</v>
       </c>
-      <c r="Q1" s="1" t="s">
+      <c r="Q1" t="s">
         <v>16</v>
       </c>
-      <c r="R1" s="1" t="s">
+      <c r="R1" t="s">
         <v>17</v>
       </c>
-      <c r="S1" s="1" t="s">
+      <c r="S1" t="s">
         <v>18</v>
       </c>
-      <c r="T1" s="1" t="s">
+      <c r="T1" t="s">
         <v>19</v>
       </c>
-      <c r="U1" s="1" t="s">
+      <c r="U1" t="s">
         <v>20</v>
       </c>
-      <c r="V1" s="1" t="s">
+      <c r="V1" t="s">
         <v>21</v>
       </c>
     </row>
@@ -1032,7 +1006,7 @@
       <c r="U2" t="s">
         <v>175</v>
       </c>
-      <c r="V2" s="2">
+      <c r="V2" s="1">
         <v>46229</v>
       </c>
     </row>
@@ -1079,7 +1053,7 @@
       <c r="U3" t="s">
         <v>92</v>
       </c>
-      <c r="V3" s="2">
+      <c r="V3" s="1">
         <v>46291</v>
       </c>
     </row>
@@ -1126,7 +1100,7 @@
       <c r="U4" t="s">
         <v>92</v>
       </c>
-      <c r="V4" s="2">
+      <c r="V4" s="1">
         <v>46321</v>
       </c>
     </row>
@@ -1173,7 +1147,7 @@
       <c r="U5" t="s">
         <v>92</v>
       </c>
-      <c r="V5" s="2">
+      <c r="V5" s="1">
         <v>46321</v>
       </c>
     </row>
@@ -1223,7 +1197,7 @@
       <c r="U6" t="s">
         <v>92</v>
       </c>
-      <c r="V6" s="2">
+      <c r="V6" s="1">
         <v>46291</v>
       </c>
     </row>
@@ -1249,7 +1223,7 @@
       <c r="G7" t="s">
         <v>108</v>
       </c>
-      <c r="H7" s="2">
+      <c r="H7" s="1">
         <v>46121</v>
       </c>
       <c r="I7" t="s">
@@ -1279,7 +1253,7 @@
       <c r="U7" t="s">
         <v>92</v>
       </c>
-      <c r="V7" s="2">
+      <c r="V7" s="1">
         <v>46138</v>
       </c>
     </row>
@@ -1326,7 +1300,7 @@
       <c r="U8" t="s">
         <v>92</v>
       </c>
-      <c r="V8" s="2">
+      <c r="V8" s="1">
         <v>46291</v>
       </c>
     </row>
@@ -1373,7 +1347,7 @@
       <c r="U9" t="s">
         <v>92</v>
       </c>
-      <c r="V9" s="2">
+      <c r="V9" s="1">
         <v>46291</v>
       </c>
     </row>
@@ -1423,7 +1397,7 @@
       <c r="U10" t="s">
         <v>92</v>
       </c>
-      <c r="V10" s="2">
+      <c r="V10" s="1">
         <v>46291</v>
       </c>
     </row>
@@ -1470,7 +1444,7 @@
       <c r="U11" t="s">
         <v>92</v>
       </c>
-      <c r="V11" s="2">
+      <c r="V11" s="1">
         <v>46291</v>
       </c>
     </row>
@@ -1517,7 +1491,7 @@
       <c r="U12" t="s">
         <v>92</v>
       </c>
-      <c r="V12" s="2">
+      <c r="V12" s="1">
         <v>46291</v>
       </c>
     </row>
@@ -1543,7 +1517,7 @@
       <c r="G13" t="s">
         <v>108</v>
       </c>
-      <c r="H13" s="2">
+      <c r="H13" s="1">
         <v>46079</v>
       </c>
       <c r="I13" t="s">
@@ -1576,7 +1550,7 @@
       <c r="U13" t="s">
         <v>175</v>
       </c>
-      <c r="V13" s="2">
+      <c r="V13" s="1">
         <v>46079</v>
       </c>
     </row>
@@ -1635,7 +1609,7 @@
       <c r="U14" t="s">
         <v>175</v>
       </c>
-      <c r="V14" s="2">
+      <c r="V14" s="1">
         <v>46352</v>
       </c>
     </row>
@@ -1694,7 +1668,7 @@
       <c r="U15" t="s">
         <v>175</v>
       </c>
-      <c r="V15" s="2">
+      <c r="V15" s="1">
         <v>46352</v>
       </c>
     </row>
@@ -1753,7 +1727,7 @@
       <c r="U16" t="s">
         <v>175</v>
       </c>
-      <c r="V16" s="2">
+      <c r="V16" s="1">
         <v>46352</v>
       </c>
     </row>
@@ -1812,7 +1786,7 @@
       <c r="U17" t="s">
         <v>175</v>
       </c>
-      <c r="V17" s="2">
+      <c r="V17" s="1">
         <v>46229</v>
       </c>
     </row>
@@ -1838,7 +1812,7 @@
       <c r="G18" t="s">
         <v>108</v>
       </c>
-      <c r="H18" s="2">
+      <c r="H18" s="1">
         <v>46098</v>
       </c>
       <c r="I18" t="s">
@@ -1871,7 +1845,7 @@
       <c r="U18" t="s">
         <v>175</v>
       </c>
-      <c r="V18" s="2">
+      <c r="V18" s="1">
         <v>46107</v>
       </c>
     </row>
@@ -1897,7 +1871,7 @@
       <c r="G19" t="s">
         <v>108</v>
       </c>
-      <c r="H19" s="2">
+      <c r="H19" s="1">
         <v>46076</v>
       </c>
       <c r="I19" t="s">
@@ -1927,7 +1901,7 @@
       <c r="U19" t="s">
         <v>92</v>
       </c>
-      <c r="V19" s="2">
+      <c r="V19" s="1">
         <v>46079</v>
       </c>
     </row>
@@ -1953,7 +1927,7 @@
       <c r="G20" t="s">
         <v>108</v>
       </c>
-      <c r="H20" s="2">
+      <c r="H20" s="1">
         <v>46076</v>
       </c>
       <c r="I20" t="s">
@@ -1983,7 +1957,7 @@
       <c r="U20" t="s">
         <v>92</v>
       </c>
-      <c r="V20" s="2">
+      <c r="V20" s="1">
         <v>46079</v>
       </c>
     </row>
@@ -2030,7 +2004,7 @@
       <c r="U21" t="s">
         <v>92</v>
       </c>
-      <c r="V21" s="2">
+      <c r="V21" s="1">
         <v>46321</v>
       </c>
     </row>
@@ -2077,7 +2051,7 @@
       <c r="U22" t="s">
         <v>92</v>
       </c>
-      <c r="V22" s="2">
+      <c r="V22" s="1">
         <v>46321</v>
       </c>
     </row>
@@ -2124,7 +2098,7 @@
       <c r="U23" t="s">
         <v>92</v>
       </c>
-      <c r="V23" s="2">
+      <c r="V23" s="1">
         <v>46321</v>
       </c>
     </row>
@@ -2171,7 +2145,7 @@
       <c r="U24" t="s">
         <v>92</v>
       </c>
-      <c r="V24" s="2">
+      <c r="V24" s="1">
         <v>46321</v>
       </c>
     </row>
@@ -2197,7 +2171,7 @@
       <c r="G25" t="s">
         <v>108</v>
       </c>
-      <c r="H25" s="2">
+      <c r="H25" s="1">
         <v>46119</v>
       </c>
       <c r="I25" t="s">
@@ -2230,7 +2204,7 @@
       <c r="U25" t="s">
         <v>175</v>
       </c>
-      <c r="V25" s="2">
+      <c r="V25" s="1">
         <v>46138</v>
       </c>
     </row>
@@ -2256,7 +2230,7 @@
       <c r="G26" t="s">
         <v>108</v>
       </c>
-      <c r="H26" s="2">
+      <c r="H26" s="1">
         <v>46121</v>
       </c>
       <c r="I26" t="s">
@@ -2286,7 +2260,7 @@
       <c r="U26" t="s">
         <v>92</v>
       </c>
-      <c r="V26" s="2">
+      <c r="V26" s="1">
         <v>46138</v>
       </c>
     </row>
@@ -2312,7 +2286,7 @@
       <c r="G27" t="s">
         <v>108</v>
       </c>
-      <c r="H27" s="2">
+      <c r="H27" s="1">
         <v>46076</v>
       </c>
       <c r="I27" t="s">
@@ -2342,7 +2316,7 @@
       <c r="U27" t="s">
         <v>92</v>
       </c>
-      <c r="V27" s="2">
+      <c r="V27" s="1">
         <v>46079</v>
       </c>
     </row>
@@ -2401,7 +2375,7 @@
       <c r="U28" t="s">
         <v>175</v>
       </c>
-      <c r="V28" s="2">
+      <c r="V28" s="1">
         <v>46291</v>
       </c>
     </row>
@@ -2427,7 +2401,7 @@
       <c r="G29" t="s">
         <v>108</v>
       </c>
-      <c r="H29" s="2">
+      <c r="H29" s="1">
         <v>46199</v>
       </c>
       <c r="I29" t="s">
@@ -2460,7 +2434,7 @@
       <c r="U29" t="s">
         <v>175</v>
       </c>
-      <c r="V29" s="2">
+      <c r="V29" s="1">
         <v>46199</v>
       </c>
     </row>
@@ -2486,7 +2460,7 @@
       <c r="G30" t="s">
         <v>108</v>
       </c>
-      <c r="H30" s="2">
+      <c r="H30" s="1">
         <v>46199</v>
       </c>
       <c r="I30" t="s">
@@ -2519,7 +2493,7 @@
       <c r="U30" t="s">
         <v>175</v>
       </c>
-      <c r="V30" s="2">
+      <c r="V30" s="1">
         <v>46199</v>
       </c>
     </row>
@@ -2545,7 +2519,7 @@
       <c r="G31" t="s">
         <v>108</v>
       </c>
-      <c r="H31" s="2">
+      <c r="H31" s="1">
         <v>46199</v>
       </c>
       <c r="I31" t="s">
@@ -2578,7 +2552,7 @@
       <c r="U31" t="s">
         <v>175</v>
       </c>
-      <c r="V31" s="2">
+      <c r="V31" s="1">
         <v>46199</v>
       </c>
     </row>
@@ -2604,7 +2578,7 @@
       <c r="G32" t="s">
         <v>108</v>
       </c>
-      <c r="H32" s="2">
+      <c r="H32" s="1">
         <v>46199</v>
       </c>
       <c r="I32" t="s">
@@ -2637,7 +2611,7 @@
       <c r="U32" t="s">
         <v>175</v>
       </c>
-      <c r="V32" s="2">
+      <c r="V32" s="1">
         <v>46199</v>
       </c>
     </row>
@@ -2690,7 +2664,7 @@
       <c r="U33" t="s">
         <v>175</v>
       </c>
-      <c r="V33" s="2">
+      <c r="V33" s="1">
         <v>46291</v>
       </c>
     </row>
@@ -2716,7 +2690,7 @@
       <c r="G34" t="s">
         <v>108</v>
       </c>
-      <c r="H34" s="2">
+      <c r="H34" s="1">
         <v>46191</v>
       </c>
       <c r="I34" t="s">
@@ -2749,7 +2723,7 @@
       <c r="U34" t="s">
         <v>175</v>
       </c>
-      <c r="V34" s="2">
+      <c r="V34" s="1">
         <v>46199</v>
       </c>
     </row>
@@ -2775,7 +2749,7 @@
       <c r="G35" t="s">
         <v>108</v>
       </c>
-      <c r="H35" s="2">
+      <c r="H35" s="1">
         <v>46119</v>
       </c>
       <c r="I35" t="s">
@@ -2805,7 +2779,7 @@
       <c r="U35" t="s">
         <v>175</v>
       </c>
-      <c r="V35" s="2">
+      <c r="V35" s="1">
         <v>46138</v>
       </c>
     </row>
@@ -2831,7 +2805,7 @@
       <c r="G36" t="s">
         <v>108</v>
       </c>
-      <c r="H36" s="2">
+      <c r="H36" s="1">
         <v>46213</v>
       </c>
       <c r="I36" t="s">
@@ -2861,7 +2835,7 @@
       <c r="U36" t="s">
         <v>92</v>
       </c>
-      <c r="V36" s="2">
+      <c r="V36" s="1">
         <v>46229</v>
       </c>
     </row>
@@ -2887,7 +2861,7 @@
       <c r="G37" t="s">
         <v>108</v>
       </c>
-      <c r="H37" s="2">
+      <c r="H37" s="1">
         <v>46175</v>
       </c>
       <c r="I37" t="s">
@@ -2917,7 +2891,7 @@
       <c r="U37" t="s">
         <v>92</v>
       </c>
-      <c r="V37" s="2">
+      <c r="V37" s="1">
         <v>46199</v>
       </c>
     </row>
@@ -2943,7 +2917,7 @@
       <c r="G38" t="s">
         <v>108</v>
       </c>
-      <c r="H38" s="2">
+      <c r="H38" s="1">
         <v>46213</v>
       </c>
       <c r="I38" t="s">
@@ -2973,7 +2947,7 @@
       <c r="U38" t="s">
         <v>92</v>
       </c>
-      <c r="V38" s="2">
+      <c r="V38" s="1">
         <v>46229</v>
       </c>
     </row>
@@ -2999,7 +2973,7 @@
       <c r="G39" t="s">
         <v>108</v>
       </c>
-      <c r="H39" s="2">
+      <c r="H39" s="1">
         <v>46199</v>
       </c>
       <c r="I39" t="s">
@@ -3029,7 +3003,7 @@
       <c r="U39" t="s">
         <v>92</v>
       </c>
-      <c r="V39" s="2">
+      <c r="V39" s="1">
         <v>46199</v>
       </c>
     </row>
@@ -3055,7 +3029,7 @@
       <c r="G40" t="s">
         <v>108</v>
       </c>
-      <c r="H40" s="2">
+      <c r="H40" s="1">
         <v>46199</v>
       </c>
       <c r="I40" t="s">
@@ -3085,7 +3059,7 @@
       <c r="U40" t="s">
         <v>92</v>
       </c>
-      <c r="V40" s="2">
+      <c r="V40" s="1">
         <v>46199</v>
       </c>
     </row>
@@ -3111,7 +3085,7 @@
       <c r="G41" t="s">
         <v>108</v>
       </c>
-      <c r="H41" s="2">
+      <c r="H41" s="1">
         <v>46204</v>
       </c>
       <c r="I41" t="s">
@@ -3141,7 +3115,7 @@
       <c r="U41" t="s">
         <v>92</v>
       </c>
-      <c r="V41" s="2">
+      <c r="V41" s="1">
         <v>46229</v>
       </c>
     </row>
@@ -3167,7 +3141,7 @@
       <c r="G42" t="s">
         <v>108</v>
       </c>
-      <c r="H42" s="2">
+      <c r="H42" s="1">
         <v>46244</v>
       </c>
       <c r="I42" t="s">
@@ -3197,7 +3171,7 @@
       <c r="U42" t="s">
         <v>92</v>
       </c>
-      <c r="V42" s="2">
+      <c r="V42" s="1">
         <v>46199</v>
       </c>
     </row>
@@ -3241,7 +3215,7 @@
       <c r="U43" t="s">
         <v>92</v>
       </c>
-      <c r="V43" s="2">
+      <c r="V43" s="1">
         <v>46260</v>
       </c>
     </row>
@@ -3267,7 +3241,7 @@
       <c r="G44" t="s">
         <v>108</v>
       </c>
-      <c r="H44" s="2">
+      <c r="H44" s="1">
         <v>46191</v>
       </c>
       <c r="I44" t="s">
@@ -3297,7 +3271,7 @@
       <c r="U44" t="s">
         <v>92</v>
       </c>
-      <c r="V44" s="2">
+      <c r="V44" s="1">
         <v>46199</v>
       </c>
     </row>
@@ -3323,7 +3297,7 @@
       <c r="G45" t="s">
         <v>108</v>
       </c>
-      <c r="H45" s="2">
+      <c r="H45" s="1">
         <v>46191</v>
       </c>
       <c r="I45" t="s">
@@ -3353,7 +3327,7 @@
       <c r="U45" t="s">
         <v>92</v>
       </c>
-      <c r="V45" s="2">
+      <c r="V45" s="1">
         <v>46199</v>
       </c>
     </row>
@@ -3379,7 +3353,7 @@
       <c r="G46" t="s">
         <v>108</v>
       </c>
-      <c r="H46" s="2">
+      <c r="H46" s="1">
         <v>46213</v>
       </c>
       <c r="I46" t="s">
@@ -3412,7 +3386,7 @@
       <c r="U46" t="s">
         <v>175</v>
       </c>
-      <c r="V46" s="2">
+      <c r="V46" s="1">
         <v>46229</v>
       </c>
     </row>
@@ -3438,7 +3412,7 @@
       <c r="G47" t="s">
         <v>108</v>
       </c>
-      <c r="H47" s="2">
+      <c r="H47" s="1">
         <v>46210</v>
       </c>
       <c r="I47" t="s">
@@ -3468,7 +3442,7 @@
       <c r="U47" t="s">
         <v>175</v>
       </c>
-      <c r="V47" s="2">
+      <c r="V47" s="1">
         <v>46229</v>
       </c>
     </row>
@@ -3515,7 +3489,7 @@
       <c r="U48" t="s">
         <v>92</v>
       </c>
-      <c r="V48" s="2">
+      <c r="V48" s="1">
         <v>46321</v>
       </c>
     </row>
@@ -3574,7 +3548,7 @@
       <c r="U49" t="s">
         <v>175</v>
       </c>
-      <c r="V49" s="2">
+      <c r="V49" s="1">
         <v>46291</v>
       </c>
     </row>
@@ -3600,7 +3574,7 @@
       <c r="G50" t="s">
         <v>108</v>
       </c>
-      <c r="H50" s="2">
+      <c r="H50" s="1">
         <v>46176</v>
       </c>
       <c r="I50" t="s">
@@ -3633,7 +3607,7 @@
       <c r="U50" t="s">
         <v>175</v>
       </c>
-      <c r="V50" s="2">
+      <c r="V50" s="1">
         <v>46199</v>
       </c>
     </row>
@@ -3689,7 +3663,7 @@
       <c r="U51" t="s">
         <v>175</v>
       </c>
-      <c r="V51" s="2">
+      <c r="V51" s="1">
         <v>46260</v>
       </c>
     </row>
@@ -3715,7 +3689,7 @@
       <c r="G52" t="s">
         <v>108</v>
       </c>
-      <c r="H52" s="2">
+      <c r="H52" s="1">
         <v>46295</v>
       </c>
       <c r="I52" t="s">
@@ -3751,7 +3725,7 @@
       <c r="U52" t="s">
         <v>175</v>
       </c>
-      <c r="V52" s="2">
+      <c r="V52" s="1">
         <v>46291</v>
       </c>
     </row>
@@ -3804,7 +3778,7 @@
       <c r="U53" t="s">
         <v>175</v>
       </c>
-      <c r="V53" s="2">
+      <c r="V53" s="1">
         <v>46321</v>
       </c>
     </row>
@@ -3830,7 +3804,7 @@
       <c r="G54" t="s">
         <v>108</v>
       </c>
-      <c r="H54" s="2">
+      <c r="H54" s="1">
         <v>46227</v>
       </c>
       <c r="I54" t="s">
@@ -3860,7 +3834,7 @@
       <c r="U54" t="s">
         <v>175</v>
       </c>
-      <c r="V54" s="2">
+      <c r="V54" s="1">
         <v>46229</v>
       </c>
     </row>
@@ -3883,7 +3857,7 @@
       <c r="G55" t="s">
         <v>108</v>
       </c>
-      <c r="H55" s="2">
+      <c r="H55" s="1">
         <v>46280</v>
       </c>
       <c r="I55" t="s">
@@ -3913,7 +3887,7 @@
       <c r="U55" t="s">
         <v>175</v>
       </c>
-      <c r="V55" s="2">
+      <c r="V55" s="1">
         <v>46291</v>
       </c>
     </row>
@@ -3936,7 +3910,7 @@
       <c r="G56" t="s">
         <v>108</v>
       </c>
-      <c r="H56" s="2">
+      <c r="H56" s="1">
         <v>46280</v>
       </c>
       <c r="I56" t="s">
@@ -3966,7 +3940,7 @@
       <c r="U56" t="s">
         <v>175</v>
       </c>
-      <c r="V56" s="2">
+      <c r="V56" s="1">
         <v>46260</v>
       </c>
     </row>
@@ -3989,7 +3963,7 @@
       <c r="G57" t="s">
         <v>108</v>
       </c>
-      <c r="H57" s="2">
+      <c r="H57" s="1">
         <v>46295</v>
       </c>
       <c r="I57" t="s">
@@ -4019,7 +3993,7 @@
       <c r="U57" t="s">
         <v>175</v>
       </c>
-      <c r="V57" s="2">
+      <c r="V57" s="1">
         <v>46291</v>
       </c>
     </row>
@@ -4042,7 +4016,7 @@
       <c r="G58" t="s">
         <v>108</v>
       </c>
-      <c r="H58" s="2">
+      <c r="H58" s="1">
         <v>46295</v>
       </c>
       <c r="I58" t="s">
@@ -4072,7 +4046,7 @@
       <c r="U58" t="s">
         <v>175</v>
       </c>
-      <c r="V58" s="2">
+      <c r="V58" s="1">
         <v>46291</v>
       </c>
     </row>
@@ -4098,7 +4072,7 @@
       <c r="G59" t="s">
         <v>109</v>
       </c>
-      <c r="H59" s="2">
+      <c r="H59" s="1">
         <v>46301</v>
       </c>
       <c r="J59" t="s">
@@ -4131,7 +4105,7 @@
       <c r="U59" t="s">
         <v>175</v>
       </c>
-      <c r="V59" s="2">
+      <c r="V59" s="1">
         <v>46352</v>
       </c>
     </row>
@@ -4175,7 +4149,7 @@
       <c r="U60" t="s">
         <v>175</v>
       </c>
-      <c r="V60" s="2">
+      <c r="V60" s="1">
         <v>46107</v>
       </c>
     </row>
@@ -4219,7 +4193,7 @@
       <c r="U61" t="s">
         <v>175</v>
       </c>
-      <c r="V61" s="2">
+      <c r="V61" s="1">
         <v>46107</v>
       </c>
     </row>
@@ -4263,7 +4237,7 @@
       <c r="U62" t="s">
         <v>175</v>
       </c>
-      <c r="V62" s="2">
+      <c r="V62" s="1">
         <v>46107</v>
       </c>
     </row>
@@ -4307,7 +4281,7 @@
       <c r="U63" t="s">
         <v>175</v>
       </c>
-      <c r="V63" s="2">
+      <c r="V63" s="1">
         <v>46107</v>
       </c>
     </row>
@@ -4351,7 +4325,7 @@
       <c r="U64" t="s">
         <v>175</v>
       </c>
-      <c r="V64" s="2">
+      <c r="V64" s="1">
         <v>46107</v>
       </c>
     </row>
@@ -4395,7 +4369,7 @@
       <c r="U65" t="s">
         <v>175</v>
       </c>
-      <c r="V65" s="2">
+      <c r="V65" s="1">
         <v>46107</v>
       </c>
     </row>
@@ -4439,7 +4413,7 @@
       <c r="U66" t="s">
         <v>92</v>
       </c>
-      <c r="V66" s="2">
+      <c r="V66" s="1">
         <v>46168</v>
       </c>
     </row>
@@ -4486,7 +4460,7 @@
       <c r="U67" t="s">
         <v>92</v>
       </c>
-      <c r="V67" s="2">
+      <c r="V67" s="1">
         <v>46291</v>
       </c>
     </row>
@@ -4545,7 +4519,7 @@
       <c r="U68" t="s">
         <v>175</v>
       </c>
-      <c r="V68" s="2">
+      <c r="V68" s="1">
         <v>46229</v>
       </c>
     </row>
@@ -4589,7 +4563,7 @@
       <c r="U69" t="s">
         <v>92</v>
       </c>
-      <c r="V69" s="2">
+      <c r="V69" s="1">
         <v>46260</v>
       </c>
     </row>
@@ -4633,7 +4607,7 @@
       <c r="U70" t="s">
         <v>175</v>
       </c>
-      <c r="V70" s="2">
+      <c r="V70" s="1">
         <v>46291</v>
       </c>
     </row>
@@ -4677,7 +4651,7 @@
       <c r="U71" t="s">
         <v>175</v>
       </c>
-      <c r="V71" s="2">
+      <c r="V71" s="1">
         <v>46168</v>
       </c>
     </row>
@@ -4721,7 +4695,7 @@
       <c r="U72" t="s">
         <v>175</v>
       </c>
-      <c r="V72" s="2">
+      <c r="V72" s="1">
         <v>46291</v>
       </c>
     </row>
@@ -4765,7 +4739,7 @@
       <c r="U73" t="s">
         <v>175</v>
       </c>
-      <c r="V73" s="2">
+      <c r="V73" s="1">
         <v>46291</v>
       </c>
     </row>
@@ -4809,7 +4783,7 @@
       <c r="U74" t="s">
         <v>175</v>
       </c>
-      <c r="V74" s="2">
+      <c r="V74" s="1">
         <v>46291</v>
       </c>
     </row>
@@ -4856,7 +4830,7 @@
       <c r="U75" t="s">
         <v>92</v>
       </c>
-      <c r="V75" s="2">
+      <c r="V75" s="1">
         <v>46321</v>
       </c>
     </row>
@@ -4906,7 +4880,7 @@
       <c r="U76" t="s">
         <v>175</v>
       </c>
-      <c r="V76" s="2">
+      <c r="V76" s="1">
         <v>46381</v>
       </c>
     </row>
@@ -4956,7 +4930,7 @@
       <c r="U77" t="s">
         <v>175</v>
       </c>
-      <c r="V77" s="2">
+      <c r="V77" s="1">
         <v>46381</v>
       </c>
     </row>
@@ -5006,7 +4980,7 @@
       <c r="U78" t="s">
         <v>92</v>
       </c>
-      <c r="V78" s="2">
+      <c r="V78" s="1">
         <v>46381</v>
       </c>
     </row>
@@ -5056,7 +5030,7 @@
       <c r="U79" t="s">
         <v>92</v>
       </c>
-      <c r="V79" s="2">
+      <c r="V79" s="1">
         <v>46381</v>
       </c>
     </row>
@@ -5106,7 +5080,7 @@
       <c r="U80" t="s">
         <v>92</v>
       </c>
-      <c r="V80" s="2">
+      <c r="V80" s="1">
         <v>46382</v>
       </c>
     </row>
@@ -5150,7 +5124,7 @@
       <c r="U81" t="s">
         <v>92</v>
       </c>
-      <c r="V81" s="2">
+      <c r="V81" s="1">
         <v>46382</v>
       </c>
     </row>
@@ -5206,7 +5180,7 @@
       <c r="U82" t="s">
         <v>175</v>
       </c>
-      <c r="V82" s="2">
+      <c r="V82" s="1">
         <v>46382</v>
       </c>
     </row>
@@ -5256,7 +5230,7 @@
       <c r="U83" t="s">
         <v>92</v>
       </c>
-      <c r="V83" s="2">
+      <c r="V83" s="1">
         <v>46321</v>
       </c>
     </row>
@@ -5300,7 +5274,7 @@
       <c r="U84" t="s">
         <v>92</v>
       </c>
-      <c r="V84" s="2">
+      <c r="V84" s="1">
         <v>46382</v>
       </c>
     </row>
@@ -5447,7 +5421,7 @@
       <c r="U87" t="s">
         <v>92</v>
       </c>
-      <c r="V87" s="2">
+      <c r="V87" s="1">
         <v>46291</v>
       </c>
     </row>
@@ -5494,7 +5468,7 @@
       <c r="U88" t="s">
         <v>92</v>
       </c>
-      <c r="V88" s="2">
+      <c r="V88" s="1">
         <v>46291</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Atualização automática: mta (09/10/2026 14:26)
</commit_message>
<xml_diff>
--- a/Projetos/02_Dados_Tratados/base_mta_tratada.xlsx
+++ b/Projetos/02_Dados_Tratados/base_mta_tratada.xlsx
@@ -14,7 +14,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1192" uniqueCount="176">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1205" uniqueCount="177">
   <si>
     <t>linha</t>
   </si>
@@ -277,6 +277,9 @@
     <t>Pagar avaliação dos cores</t>
   </si>
   <si>
+    <t>Em trâmite</t>
+  </si>
+  <si>
     <t>Sem informação</t>
   </si>
   <si>
@@ -289,9 +292,6 @@
     <t>Não aprovado</t>
   </si>
   <si>
-    <t>Em trâmite</t>
-  </si>
-  <si>
     <t>SIM</t>
   </si>
   <si>
@@ -331,19 +331,22 @@
     <t>DESTQ51</t>
   </si>
   <si>
+    <t>DESTQ53</t>
+  </si>
+  <si>
     <t>RAP</t>
   </si>
   <si>
+    <t>EM TRÂMITE</t>
+  </si>
+  <si>
+    <t>CANCELADO</t>
+  </si>
+  <si>
+    <t>ATENDIDO</t>
+  </si>
+  <si>
     <t>ATENDER</t>
-  </si>
-  <si>
-    <t>CANCELADO</t>
-  </si>
-  <si>
-    <t>ATENDIDO</t>
-  </si>
-  <si>
-    <t>EM TRÂMITE</t>
   </si>
   <si>
     <t>PROCESSADO</t>
@@ -877,7 +880,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:V88"/>
+  <dimension ref="A1:V89"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:22">
@@ -968,22 +971,25 @@
         <v>94</v>
       </c>
       <c r="G2" t="s">
-        <v>106</v>
+        <v>107</v>
+      </c>
+      <c r="H2" s="1">
+        <v>46303</v>
       </c>
       <c r="I2" t="s">
-        <v>111</v>
+        <v>112</v>
       </c>
       <c r="J2" t="s">
-        <v>130</v>
+        <v>131</v>
       </c>
       <c r="K2" t="s">
-        <v>139</v>
+        <v>140</v>
       </c>
       <c r="L2" t="s">
-        <v>144</v>
+        <v>145</v>
       </c>
       <c r="N2" t="s">
-        <v>145</v>
+        <v>146</v>
       </c>
       <c r="O2" t="s">
         <v>23</v>
@@ -992,19 +998,19 @@
         <v>135000</v>
       </c>
       <c r="Q2" t="s">
-        <v>163</v>
+        <v>164</v>
       </c>
       <c r="R2" t="s">
-        <v>166</v>
+        <v>167</v>
       </c>
       <c r="S2" t="s">
-        <v>169</v>
+        <v>170</v>
       </c>
       <c r="T2" t="s">
-        <v>171</v>
+        <v>172</v>
       </c>
       <c r="U2" t="s">
-        <v>175</v>
+        <v>176</v>
       </c>
       <c r="V2" s="1">
         <v>46229</v>
@@ -1021,7 +1027,7 @@
         <v>24</v>
       </c>
       <c r="D3" t="s">
-        <v>87</v>
+        <v>88</v>
       </c>
       <c r="E3" t="s">
         <v>92</v>
@@ -1030,25 +1036,25 @@
         <v>94</v>
       </c>
       <c r="G3" t="s">
-        <v>107</v>
+        <v>108</v>
       </c>
       <c r="N3" t="s">
-        <v>145</v>
+        <v>146</v>
       </c>
       <c r="O3" t="s">
         <v>24</v>
       </c>
       <c r="Q3" t="s">
-        <v>163</v>
+        <v>164</v>
       </c>
       <c r="R3" t="s">
-        <v>166</v>
+        <v>167</v>
       </c>
       <c r="S3" t="s">
-        <v>169</v>
+        <v>170</v>
       </c>
       <c r="T3" t="s">
-        <v>171</v>
+        <v>172</v>
       </c>
       <c r="U3" t="s">
         <v>92</v>
@@ -1068,7 +1074,7 @@
         <v>25</v>
       </c>
       <c r="D4" t="s">
-        <v>87</v>
+        <v>88</v>
       </c>
       <c r="E4" t="s">
         <v>92</v>
@@ -1077,25 +1083,25 @@
         <v>94</v>
       </c>
       <c r="G4" t="s">
-        <v>107</v>
+        <v>108</v>
       </c>
       <c r="N4" t="s">
-        <v>146</v>
+        <v>147</v>
       </c>
       <c r="O4" t="s">
         <v>25</v>
       </c>
       <c r="Q4" t="s">
-        <v>163</v>
+        <v>164</v>
       </c>
       <c r="R4" t="s">
-        <v>167</v>
+        <v>168</v>
       </c>
       <c r="S4" t="s">
-        <v>169</v>
+        <v>170</v>
       </c>
       <c r="T4" t="s">
-        <v>171</v>
+        <v>172</v>
       </c>
       <c r="U4" t="s">
         <v>92</v>
@@ -1115,7 +1121,7 @@
         <v>26</v>
       </c>
       <c r="D5" t="s">
-        <v>87</v>
+        <v>88</v>
       </c>
       <c r="E5" t="s">
         <v>92</v>
@@ -1124,25 +1130,25 @@
         <v>94</v>
       </c>
       <c r="G5" t="s">
-        <v>107</v>
+        <v>108</v>
       </c>
       <c r="N5" t="s">
-        <v>146</v>
+        <v>147</v>
       </c>
       <c r="O5" t="s">
         <v>26</v>
       </c>
       <c r="Q5" t="s">
-        <v>163</v>
+        <v>164</v>
       </c>
       <c r="R5" t="s">
-        <v>167</v>
+        <v>168</v>
       </c>
       <c r="S5" t="s">
-        <v>169</v>
+        <v>170</v>
       </c>
       <c r="T5" t="s">
-        <v>171</v>
+        <v>172</v>
       </c>
       <c r="U5" t="s">
         <v>92</v>
@@ -1162,7 +1168,7 @@
         <v>27</v>
       </c>
       <c r="D6" t="s">
-        <v>87</v>
+        <v>88</v>
       </c>
       <c r="E6" t="s">
         <v>92</v>
@@ -1171,28 +1177,28 @@
         <v>94</v>
       </c>
       <c r="G6" t="s">
-        <v>107</v>
+        <v>108</v>
       </c>
       <c r="L6" t="s">
-        <v>144</v>
+        <v>145</v>
       </c>
       <c r="N6" t="s">
-        <v>147</v>
+        <v>148</v>
       </c>
       <c r="O6" t="s">
         <v>27</v>
       </c>
       <c r="Q6" t="s">
-        <v>163</v>
+        <v>164</v>
       </c>
       <c r="R6" t="s">
-        <v>167</v>
+        <v>168</v>
       </c>
       <c r="S6" t="s">
-        <v>169</v>
+        <v>170</v>
       </c>
       <c r="T6" t="s">
-        <v>171</v>
+        <v>172</v>
       </c>
       <c r="U6" t="s">
         <v>92</v>
@@ -1212,7 +1218,7 @@
         <v>28</v>
       </c>
       <c r="D7" t="s">
-        <v>88</v>
+        <v>89</v>
       </c>
       <c r="E7" t="s">
         <v>92</v>
@@ -1221,16 +1227,16 @@
         <v>94</v>
       </c>
       <c r="G7" t="s">
-        <v>108</v>
+        <v>109</v>
       </c>
       <c r="H7" s="1">
         <v>46121</v>
       </c>
       <c r="I7" t="s">
-        <v>112</v>
+        <v>113</v>
       </c>
       <c r="N7" t="s">
-        <v>148</v>
+        <v>149</v>
       </c>
       <c r="O7" t="s">
         <v>28</v>
@@ -1239,16 +1245,16 @@
         <v>3799999.6</v>
       </c>
       <c r="Q7" t="s">
-        <v>164</v>
+        <v>165</v>
       </c>
       <c r="R7" t="s">
-        <v>167</v>
+        <v>168</v>
       </c>
       <c r="S7" t="s">
-        <v>169</v>
+        <v>170</v>
       </c>
       <c r="T7" t="s">
-        <v>172</v>
+        <v>173</v>
       </c>
       <c r="U7" t="s">
         <v>92</v>
@@ -1268,7 +1274,7 @@
         <v>29</v>
       </c>
       <c r="D8" t="s">
-        <v>87</v>
+        <v>88</v>
       </c>
       <c r="E8" t="s">
         <v>92</v>
@@ -1277,25 +1283,25 @@
         <v>94</v>
       </c>
       <c r="G8" t="s">
-        <v>107</v>
+        <v>108</v>
       </c>
       <c r="N8" t="s">
-        <v>146</v>
+        <v>147</v>
       </c>
       <c r="O8" t="s">
         <v>29</v>
       </c>
       <c r="Q8" t="s">
-        <v>163</v>
+        <v>164</v>
       </c>
       <c r="R8" t="s">
-        <v>167</v>
+        <v>168</v>
       </c>
       <c r="S8" t="s">
-        <v>169</v>
+        <v>170</v>
       </c>
       <c r="T8" t="s">
-        <v>171</v>
+        <v>172</v>
       </c>
       <c r="U8" t="s">
         <v>92</v>
@@ -1315,7 +1321,7 @@
         <v>30</v>
       </c>
       <c r="D9" t="s">
-        <v>89</v>
+        <v>90</v>
       </c>
       <c r="E9" t="s">
         <v>92</v>
@@ -1324,25 +1330,25 @@
         <v>94</v>
       </c>
       <c r="N9" t="s">
-        <v>146</v>
+        <v>147</v>
       </c>
       <c r="O9" t="s">
         <v>30</v>
       </c>
       <c r="P9">
-        <v>36104.46</v>
+        <v>23895.54</v>
       </c>
       <c r="Q9" t="s">
-        <v>163</v>
+        <v>164</v>
       </c>
       <c r="R9" t="s">
-        <v>167</v>
+        <v>168</v>
       </c>
       <c r="S9" t="s">
-        <v>169</v>
+        <v>170</v>
       </c>
       <c r="T9" t="s">
-        <v>171</v>
+        <v>172</v>
       </c>
       <c r="U9" t="s">
         <v>92</v>
@@ -1368,13 +1374,16 @@
         <v>94</v>
       </c>
       <c r="G10" t="s">
-        <v>106</v>
+        <v>107</v>
+      </c>
+      <c r="H10" s="1">
+        <v>46303</v>
       </c>
       <c r="I10" t="s">
-        <v>111</v>
+        <v>112</v>
       </c>
       <c r="N10" t="s">
-        <v>146</v>
+        <v>147</v>
       </c>
       <c r="O10" t="s">
         <v>30</v>
@@ -1383,16 +1392,16 @@
         <v>23895.54</v>
       </c>
       <c r="Q10" t="s">
-        <v>163</v>
+        <v>164</v>
       </c>
       <c r="R10" t="s">
-        <v>167</v>
+        <v>168</v>
       </c>
       <c r="S10" t="s">
-        <v>169</v>
+        <v>170</v>
       </c>
       <c r="T10" t="s">
-        <v>171</v>
+        <v>172</v>
       </c>
       <c r="U10" t="s">
         <v>92</v>
@@ -1412,7 +1421,7 @@
         <v>31</v>
       </c>
       <c r="D11" t="s">
-        <v>87</v>
+        <v>88</v>
       </c>
       <c r="E11" t="s">
         <v>92</v>
@@ -1421,25 +1430,25 @@
         <v>94</v>
       </c>
       <c r="G11" t="s">
-        <v>107</v>
+        <v>108</v>
       </c>
       <c r="N11" t="s">
-        <v>147</v>
+        <v>148</v>
       </c>
       <c r="O11" t="s">
         <v>31</v>
       </c>
       <c r="Q11" t="s">
-        <v>163</v>
+        <v>164</v>
       </c>
       <c r="R11" t="s">
-        <v>167</v>
+        <v>168</v>
       </c>
       <c r="S11" t="s">
-        <v>169</v>
+        <v>170</v>
       </c>
       <c r="T11" t="s">
-        <v>171</v>
+        <v>172</v>
       </c>
       <c r="U11" t="s">
         <v>92</v>
@@ -1459,7 +1468,7 @@
         <v>32</v>
       </c>
       <c r="D12" t="s">
-        <v>87</v>
+        <v>88</v>
       </c>
       <c r="E12" t="s">
         <v>92</v>
@@ -1468,25 +1477,25 @@
         <v>94</v>
       </c>
       <c r="G12" t="s">
-        <v>107</v>
+        <v>108</v>
       </c>
       <c r="N12" t="s">
-        <v>147</v>
+        <v>148</v>
       </c>
       <c r="O12" t="s">
         <v>32</v>
       </c>
       <c r="Q12" t="s">
-        <v>163</v>
+        <v>164</v>
       </c>
       <c r="R12" t="s">
-        <v>167</v>
+        <v>168</v>
       </c>
       <c r="S12" t="s">
-        <v>169</v>
+        <v>170</v>
       </c>
       <c r="T12" t="s">
-        <v>171</v>
+        <v>172</v>
       </c>
       <c r="U12" t="s">
         <v>92</v>
@@ -1506,7 +1515,7 @@
         <v>33</v>
       </c>
       <c r="D13" t="s">
-        <v>88</v>
+        <v>89</v>
       </c>
       <c r="E13" t="s">
         <v>92</v>
@@ -1515,19 +1524,19 @@
         <v>94</v>
       </c>
       <c r="G13" t="s">
-        <v>108</v>
+        <v>109</v>
       </c>
       <c r="H13" s="1">
         <v>46079</v>
       </c>
       <c r="I13" t="s">
-        <v>113</v>
+        <v>114</v>
       </c>
       <c r="J13" t="s">
-        <v>131</v>
+        <v>132</v>
       </c>
       <c r="N13" t="s">
-        <v>145</v>
+        <v>146</v>
       </c>
       <c r="O13" t="s">
         <v>33</v>
@@ -1536,19 +1545,19 @@
         <v>1187433.02</v>
       </c>
       <c r="Q13" t="s">
-        <v>163</v>
+        <v>164</v>
       </c>
       <c r="R13" t="s">
-        <v>166</v>
+        <v>167</v>
       </c>
       <c r="S13" t="s">
-        <v>169</v>
+        <v>170</v>
       </c>
       <c r="T13" t="s">
-        <v>171</v>
+        <v>172</v>
       </c>
       <c r="U13" t="s">
-        <v>175</v>
+        <v>176</v>
       </c>
       <c r="V13" s="1">
         <v>46079</v>
@@ -1574,19 +1583,22 @@
         <v>94</v>
       </c>
       <c r="G14" t="s">
-        <v>106</v>
+        <v>107</v>
+      </c>
+      <c r="H14" s="1">
+        <v>46303</v>
       </c>
       <c r="I14" t="s">
-        <v>111</v>
+        <v>112</v>
       </c>
       <c r="J14" t="s">
-        <v>130</v>
+        <v>131</v>
       </c>
       <c r="K14" t="s">
-        <v>106</v>
+        <v>110</v>
       </c>
       <c r="N14" t="s">
-        <v>145</v>
+        <v>146</v>
       </c>
       <c r="O14" t="s">
         <v>34</v>
@@ -1595,19 +1607,19 @@
         <v>1000000</v>
       </c>
       <c r="Q14" t="s">
-        <v>163</v>
+        <v>164</v>
       </c>
       <c r="R14" t="s">
-        <v>166</v>
+        <v>167</v>
       </c>
       <c r="S14" t="s">
-        <v>169</v>
+        <v>170</v>
       </c>
       <c r="T14" t="s">
-        <v>171</v>
+        <v>172</v>
       </c>
       <c r="U14" t="s">
-        <v>175</v>
+        <v>176</v>
       </c>
       <c r="V14" s="1">
         <v>46352</v>
@@ -1633,19 +1645,22 @@
         <v>94</v>
       </c>
       <c r="G15" t="s">
-        <v>106</v>
+        <v>107</v>
+      </c>
+      <c r="H15" s="1">
+        <v>46303</v>
       </c>
       <c r="I15" t="s">
-        <v>111</v>
+        <v>112</v>
       </c>
       <c r="J15" t="s">
-        <v>130</v>
+        <v>131</v>
       </c>
       <c r="K15" t="s">
-        <v>106</v>
+        <v>110</v>
       </c>
       <c r="N15" t="s">
-        <v>145</v>
+        <v>146</v>
       </c>
       <c r="O15" t="s">
         <v>35</v>
@@ -1654,19 +1669,19 @@
         <v>1000000</v>
       </c>
       <c r="Q15" t="s">
-        <v>163</v>
+        <v>164</v>
       </c>
       <c r="R15" t="s">
-        <v>166</v>
+        <v>167</v>
       </c>
       <c r="S15" t="s">
-        <v>169</v>
+        <v>170</v>
       </c>
       <c r="T15" t="s">
-        <v>171</v>
+        <v>172</v>
       </c>
       <c r="U15" t="s">
-        <v>175</v>
+        <v>176</v>
       </c>
       <c r="V15" s="1">
         <v>46352</v>
@@ -1692,19 +1707,22 @@
         <v>94</v>
       </c>
       <c r="G16" t="s">
-        <v>106</v>
+        <v>107</v>
+      </c>
+      <c r="H16" s="1">
+        <v>46303</v>
       </c>
       <c r="I16" t="s">
-        <v>111</v>
+        <v>112</v>
       </c>
       <c r="J16" t="s">
-        <v>130</v>
+        <v>131</v>
       </c>
       <c r="K16" t="s">
-        <v>106</v>
+        <v>110</v>
       </c>
       <c r="N16" t="s">
-        <v>145</v>
+        <v>146</v>
       </c>
       <c r="O16" t="s">
         <v>36</v>
@@ -1713,19 +1731,19 @@
         <v>1000000</v>
       </c>
       <c r="Q16" t="s">
-        <v>163</v>
+        <v>164</v>
       </c>
       <c r="R16" t="s">
-        <v>166</v>
+        <v>167</v>
       </c>
       <c r="S16" t="s">
-        <v>169</v>
+        <v>170</v>
       </c>
       <c r="T16" t="s">
-        <v>171</v>
+        <v>172</v>
       </c>
       <c r="U16" t="s">
-        <v>175</v>
+        <v>176</v>
       </c>
       <c r="V16" s="1">
         <v>46352</v>
@@ -1751,19 +1769,22 @@
         <v>94</v>
       </c>
       <c r="G17" t="s">
-        <v>106</v>
+        <v>107</v>
+      </c>
+      <c r="H17" s="1">
+        <v>46303</v>
       </c>
       <c r="I17" t="s">
-        <v>111</v>
+        <v>112</v>
       </c>
       <c r="J17" t="s">
-        <v>130</v>
+        <v>131</v>
       </c>
       <c r="K17" t="s">
-        <v>106</v>
+        <v>110</v>
       </c>
       <c r="N17" t="s">
-        <v>149</v>
+        <v>150</v>
       </c>
       <c r="O17" t="s">
         <v>37</v>
@@ -1772,19 +1793,19 @@
         <v>100000</v>
       </c>
       <c r="Q17" t="s">
-        <v>165</v>
+        <v>166</v>
       </c>
       <c r="R17" t="s">
-        <v>166</v>
+        <v>167</v>
       </c>
       <c r="S17" t="s">
-        <v>169</v>
+        <v>170</v>
       </c>
       <c r="T17" t="s">
-        <v>171</v>
+        <v>172</v>
       </c>
       <c r="U17" t="s">
-        <v>175</v>
+        <v>176</v>
       </c>
       <c r="V17" s="1">
         <v>46229</v>
@@ -1801,7 +1822,7 @@
         <v>38</v>
       </c>
       <c r="D18" t="s">
-        <v>88</v>
+        <v>89</v>
       </c>
       <c r="E18" t="s">
         <v>92</v>
@@ -1810,19 +1831,19 @@
         <v>94</v>
       </c>
       <c r="G18" t="s">
-        <v>108</v>
+        <v>109</v>
       </c>
       <c r="H18" s="1">
         <v>46098</v>
       </c>
       <c r="I18" t="s">
-        <v>114</v>
+        <v>115</v>
       </c>
       <c r="J18" t="s">
-        <v>131</v>
+        <v>132</v>
       </c>
       <c r="N18" t="s">
-        <v>150</v>
+        <v>151</v>
       </c>
       <c r="O18" t="s">
         <v>38</v>
@@ -1831,19 +1852,19 @@
         <v>1770880.5</v>
       </c>
       <c r="Q18" t="s">
-        <v>164</v>
+        <v>165</v>
       </c>
       <c r="R18" t="s">
-        <v>167</v>
+        <v>168</v>
       </c>
       <c r="S18" t="s">
-        <v>169</v>
+        <v>170</v>
       </c>
       <c r="T18" t="s">
-        <v>173</v>
+        <v>174</v>
       </c>
       <c r="U18" t="s">
-        <v>175</v>
+        <v>176</v>
       </c>
       <c r="V18" s="1">
         <v>46107</v>
@@ -1860,7 +1881,7 @@
         <v>39</v>
       </c>
       <c r="D19" t="s">
-        <v>88</v>
+        <v>89</v>
       </c>
       <c r="E19" t="s">
         <v>92</v>
@@ -1869,16 +1890,16 @@
         <v>94</v>
       </c>
       <c r="G19" t="s">
-        <v>108</v>
+        <v>109</v>
       </c>
       <c r="H19" s="1">
         <v>46076</v>
       </c>
       <c r="I19" t="s">
-        <v>115</v>
+        <v>116</v>
       </c>
       <c r="N19" t="s">
-        <v>151</v>
+        <v>152</v>
       </c>
       <c r="O19" t="s">
         <v>39</v>
@@ -1887,16 +1908,16 @@
         <v>350000</v>
       </c>
       <c r="Q19" t="s">
-        <v>164</v>
+        <v>165</v>
       </c>
       <c r="R19" t="s">
-        <v>166</v>
+        <v>167</v>
       </c>
       <c r="S19" t="s">
-        <v>169</v>
+        <v>170</v>
       </c>
       <c r="T19" t="s">
-        <v>172</v>
+        <v>173</v>
       </c>
       <c r="U19" t="s">
         <v>92</v>
@@ -1916,7 +1937,7 @@
         <v>40</v>
       </c>
       <c r="D20" t="s">
-        <v>88</v>
+        <v>89</v>
       </c>
       <c r="E20" t="s">
         <v>92</v>
@@ -1925,16 +1946,16 @@
         <v>94</v>
       </c>
       <c r="G20" t="s">
-        <v>108</v>
+        <v>109</v>
       </c>
       <c r="H20" s="1">
         <v>46076</v>
       </c>
       <c r="I20" t="s">
-        <v>115</v>
+        <v>116</v>
       </c>
       <c r="N20" t="s">
-        <v>151</v>
+        <v>152</v>
       </c>
       <c r="O20" t="s">
         <v>40</v>
@@ -1943,16 +1964,16 @@
         <v>350000</v>
       </c>
       <c r="Q20" t="s">
-        <v>164</v>
+        <v>165</v>
       </c>
       <c r="R20" t="s">
-        <v>166</v>
+        <v>167</v>
       </c>
       <c r="S20" t="s">
-        <v>169</v>
+        <v>170</v>
       </c>
       <c r="T20" t="s">
-        <v>172</v>
+        <v>173</v>
       </c>
       <c r="U20" t="s">
         <v>92</v>
@@ -1972,7 +1993,7 @@
         <v>41</v>
       </c>
       <c r="D21" t="s">
-        <v>89</v>
+        <v>90</v>
       </c>
       <c r="E21" t="s">
         <v>92</v>
@@ -1981,7 +2002,7 @@
         <v>94</v>
       </c>
       <c r="N21" t="s">
-        <v>152</v>
+        <v>153</v>
       </c>
       <c r="O21" t="s">
         <v>41</v>
@@ -1990,16 +2011,16 @@
         <v>1000000</v>
       </c>
       <c r="Q21" t="s">
-        <v>164</v>
+        <v>165</v>
       </c>
       <c r="R21" t="s">
-        <v>166</v>
+        <v>167</v>
       </c>
       <c r="S21" t="s">
-        <v>169</v>
+        <v>170</v>
       </c>
       <c r="T21" t="s">
-        <v>172</v>
+        <v>173</v>
       </c>
       <c r="U21" t="s">
         <v>92</v>
@@ -2019,7 +2040,7 @@
         <v>42</v>
       </c>
       <c r="D22" t="s">
-        <v>87</v>
+        <v>88</v>
       </c>
       <c r="E22" t="s">
         <v>92</v>
@@ -2028,25 +2049,25 @@
         <v>94</v>
       </c>
       <c r="G22" t="s">
-        <v>107</v>
+        <v>108</v>
       </c>
       <c r="N22" t="s">
-        <v>145</v>
+        <v>146</v>
       </c>
       <c r="O22" t="s">
         <v>42</v>
       </c>
       <c r="Q22" t="s">
-        <v>163</v>
+        <v>164</v>
       </c>
       <c r="R22" t="s">
-        <v>166</v>
+        <v>167</v>
       </c>
       <c r="S22" t="s">
-        <v>169</v>
+        <v>170</v>
       </c>
       <c r="T22" t="s">
-        <v>171</v>
+        <v>172</v>
       </c>
       <c r="U22" t="s">
         <v>92</v>
@@ -2066,7 +2087,7 @@
         <v>43</v>
       </c>
       <c r="D23" t="s">
-        <v>87</v>
+        <v>88</v>
       </c>
       <c r="E23" t="s">
         <v>92</v>
@@ -2075,25 +2096,25 @@
         <v>94</v>
       </c>
       <c r="G23" t="s">
-        <v>107</v>
+        <v>108</v>
       </c>
       <c r="N23" t="s">
-        <v>146</v>
+        <v>147</v>
       </c>
       <c r="O23" t="s">
         <v>43</v>
       </c>
       <c r="Q23" t="s">
-        <v>163</v>
+        <v>164</v>
       </c>
       <c r="R23" t="s">
-        <v>167</v>
+        <v>168</v>
       </c>
       <c r="S23" t="s">
-        <v>169</v>
+        <v>170</v>
       </c>
       <c r="T23" t="s">
-        <v>171</v>
+        <v>172</v>
       </c>
       <c r="U23" t="s">
         <v>92</v>
@@ -2113,7 +2134,7 @@
         <v>44</v>
       </c>
       <c r="D24" t="s">
-        <v>87</v>
+        <v>88</v>
       </c>
       <c r="E24" t="s">
         <v>92</v>
@@ -2122,25 +2143,25 @@
         <v>94</v>
       </c>
       <c r="G24" t="s">
-        <v>107</v>
+        <v>108</v>
       </c>
       <c r="N24" t="s">
-        <v>146</v>
+        <v>147</v>
       </c>
       <c r="O24" t="s">
         <v>44</v>
       </c>
       <c r="Q24" t="s">
-        <v>163</v>
+        <v>164</v>
       </c>
       <c r="R24" t="s">
-        <v>167</v>
+        <v>168</v>
       </c>
       <c r="S24" t="s">
-        <v>169</v>
+        <v>170</v>
       </c>
       <c r="T24" t="s">
-        <v>171</v>
+        <v>172</v>
       </c>
       <c r="U24" t="s">
         <v>92</v>
@@ -2160,7 +2181,7 @@
         <v>45</v>
       </c>
       <c r="D25" t="s">
-        <v>88</v>
+        <v>89</v>
       </c>
       <c r="E25" t="s">
         <v>92</v>
@@ -2169,19 +2190,19 @@
         <v>95</v>
       </c>
       <c r="G25" t="s">
-        <v>108</v>
+        <v>109</v>
       </c>
       <c r="H25" s="1">
         <v>46119</v>
       </c>
       <c r="I25" t="s">
-        <v>116</v>
+        <v>117</v>
       </c>
       <c r="J25" t="s">
-        <v>132</v>
+        <v>133</v>
       </c>
       <c r="N25" t="s">
-        <v>150</v>
+        <v>151</v>
       </c>
       <c r="O25" t="s">
         <v>45</v>
@@ -2190,19 +2211,19 @@
         <v>1704503</v>
       </c>
       <c r="Q25" t="s">
-        <v>164</v>
+        <v>165</v>
       </c>
       <c r="R25" t="s">
-        <v>167</v>
+        <v>168</v>
       </c>
       <c r="S25" t="s">
-        <v>169</v>
+        <v>170</v>
       </c>
       <c r="T25" t="s">
-        <v>173</v>
+        <v>174</v>
       </c>
       <c r="U25" t="s">
-        <v>175</v>
+        <v>176</v>
       </c>
       <c r="V25" s="1">
         <v>46138</v>
@@ -2219,7 +2240,7 @@
         <v>46</v>
       </c>
       <c r="D26" t="s">
-        <v>88</v>
+        <v>89</v>
       </c>
       <c r="E26" t="s">
         <v>92</v>
@@ -2228,16 +2249,16 @@
         <v>94</v>
       </c>
       <c r="G26" t="s">
-        <v>108</v>
+        <v>109</v>
       </c>
       <c r="H26" s="1">
         <v>46121</v>
       </c>
       <c r="I26" t="s">
-        <v>117</v>
+        <v>118</v>
       </c>
       <c r="N26" t="s">
-        <v>153</v>
+        <v>154</v>
       </c>
       <c r="O26" t="s">
         <v>46</v>
@@ -2246,16 +2267,16 @@
         <v>3799000</v>
       </c>
       <c r="Q26" t="s">
-        <v>164</v>
+        <v>165</v>
       </c>
       <c r="R26" t="s">
-        <v>167</v>
+        <v>168</v>
       </c>
       <c r="S26" t="s">
-        <v>169</v>
+        <v>170</v>
       </c>
       <c r="T26" t="s">
-        <v>172</v>
+        <v>173</v>
       </c>
       <c r="U26" t="s">
         <v>92</v>
@@ -2275,7 +2296,7 @@
         <v>46</v>
       </c>
       <c r="D27" t="s">
-        <v>88</v>
+        <v>89</v>
       </c>
       <c r="E27" t="s">
         <v>92</v>
@@ -2284,16 +2305,16 @@
         <v>94</v>
       </c>
       <c r="G27" t="s">
-        <v>108</v>
+        <v>109</v>
       </c>
       <c r="H27" s="1">
         <v>46076</v>
       </c>
       <c r="I27" t="s">
-        <v>118</v>
+        <v>119</v>
       </c>
       <c r="N27" t="s">
-        <v>153</v>
+        <v>154</v>
       </c>
       <c r="O27" t="s">
         <v>46</v>
@@ -2302,16 +2323,16 @@
         <v>1000</v>
       </c>
       <c r="Q27" t="s">
-        <v>164</v>
+        <v>165</v>
       </c>
       <c r="R27" t="s">
-        <v>166</v>
+        <v>167</v>
       </c>
       <c r="S27" t="s">
-        <v>169</v>
+        <v>170</v>
       </c>
       <c r="T27" t="s">
-        <v>172</v>
+        <v>173</v>
       </c>
       <c r="U27" t="s">
         <v>92</v>
@@ -2340,19 +2361,22 @@
         <v>94</v>
       </c>
       <c r="G28" t="s">
-        <v>106</v>
+        <v>107</v>
+      </c>
+      <c r="H28" s="1">
+        <v>46303</v>
       </c>
       <c r="I28" t="s">
-        <v>111</v>
+        <v>112</v>
       </c>
       <c r="J28" t="s">
-        <v>130</v>
+        <v>131</v>
       </c>
       <c r="K28" t="s">
-        <v>106</v>
+        <v>110</v>
       </c>
       <c r="N28" t="s">
-        <v>149</v>
+        <v>150</v>
       </c>
       <c r="O28" t="s">
         <v>47</v>
@@ -2361,19 +2385,19 @@
         <v>100000</v>
       </c>
       <c r="Q28" t="s">
-        <v>165</v>
+        <v>166</v>
       </c>
       <c r="R28" t="s">
-        <v>166</v>
+        <v>167</v>
       </c>
       <c r="S28" t="s">
-        <v>169</v>
+        <v>170</v>
       </c>
       <c r="T28" t="s">
-        <v>171</v>
+        <v>172</v>
       </c>
       <c r="U28" t="s">
-        <v>175</v>
+        <v>176</v>
       </c>
       <c r="V28" s="1">
         <v>46291</v>
@@ -2390,7 +2414,7 @@
         <v>48</v>
       </c>
       <c r="D29" t="s">
-        <v>88</v>
+        <v>89</v>
       </c>
       <c r="E29" t="s">
         <v>92</v>
@@ -2399,19 +2423,19 @@
         <v>96</v>
       </c>
       <c r="G29" t="s">
-        <v>108</v>
+        <v>109</v>
       </c>
       <c r="H29" s="1">
         <v>46199</v>
       </c>
       <c r="I29" t="s">
-        <v>119</v>
+        <v>120</v>
       </c>
       <c r="J29" t="s">
-        <v>133</v>
+        <v>134</v>
       </c>
       <c r="N29" t="s">
-        <v>150</v>
+        <v>151</v>
       </c>
       <c r="O29" t="s">
         <v>48</v>
@@ -2420,19 +2444,19 @@
         <v>150000</v>
       </c>
       <c r="Q29" t="s">
-        <v>164</v>
+        <v>165</v>
       </c>
       <c r="R29" t="s">
-        <v>167</v>
+        <v>168</v>
       </c>
       <c r="S29" t="s">
-        <v>169</v>
+        <v>170</v>
       </c>
       <c r="T29" t="s">
-        <v>172</v>
+        <v>173</v>
       </c>
       <c r="U29" t="s">
-        <v>175</v>
+        <v>176</v>
       </c>
       <c r="V29" s="1">
         <v>46199</v>
@@ -2449,7 +2473,7 @@
         <v>49</v>
       </c>
       <c r="D30" t="s">
-        <v>88</v>
+        <v>89</v>
       </c>
       <c r="E30" t="s">
         <v>92</v>
@@ -2458,19 +2482,19 @@
         <v>96</v>
       </c>
       <c r="G30" t="s">
-        <v>108</v>
+        <v>109</v>
       </c>
       <c r="H30" s="1">
         <v>46199</v>
       </c>
       <c r="I30" t="s">
-        <v>119</v>
+        <v>120</v>
       </c>
       <c r="J30" t="s">
-        <v>133</v>
+        <v>134</v>
       </c>
       <c r="N30" t="s">
-        <v>150</v>
+        <v>151</v>
       </c>
       <c r="O30" t="s">
         <v>49</v>
@@ -2479,19 +2503,19 @@
         <v>150000</v>
       </c>
       <c r="Q30" t="s">
-        <v>164</v>
+        <v>165</v>
       </c>
       <c r="R30" t="s">
-        <v>167</v>
+        <v>168</v>
       </c>
       <c r="S30" t="s">
-        <v>169</v>
+        <v>170</v>
       </c>
       <c r="T30" t="s">
-        <v>172</v>
+        <v>173</v>
       </c>
       <c r="U30" t="s">
-        <v>175</v>
+        <v>176</v>
       </c>
       <c r="V30" s="1">
         <v>46199</v>
@@ -2508,7 +2532,7 @@
         <v>50</v>
       </c>
       <c r="D31" t="s">
-        <v>88</v>
+        <v>89</v>
       </c>
       <c r="E31" t="s">
         <v>92</v>
@@ -2517,19 +2541,19 @@
         <v>97</v>
       </c>
       <c r="G31" t="s">
-        <v>108</v>
+        <v>109</v>
       </c>
       <c r="H31" s="1">
         <v>46199</v>
       </c>
       <c r="I31" t="s">
-        <v>120</v>
+        <v>121</v>
       </c>
       <c r="J31" t="s">
-        <v>133</v>
+        <v>134</v>
       </c>
       <c r="N31" t="s">
-        <v>150</v>
+        <v>151</v>
       </c>
       <c r="O31" t="s">
         <v>50</v>
@@ -2538,19 +2562,19 @@
         <v>18462.36</v>
       </c>
       <c r="Q31" t="s">
-        <v>164</v>
+        <v>165</v>
       </c>
       <c r="R31" t="s">
-        <v>167</v>
+        <v>168</v>
       </c>
       <c r="S31" t="s">
-        <v>169</v>
+        <v>170</v>
       </c>
       <c r="T31" t="s">
-        <v>172</v>
+        <v>173</v>
       </c>
       <c r="U31" t="s">
-        <v>175</v>
+        <v>176</v>
       </c>
       <c r="V31" s="1">
         <v>46199</v>
@@ -2567,7 +2591,7 @@
         <v>50</v>
       </c>
       <c r="D32" t="s">
-        <v>88</v>
+        <v>89</v>
       </c>
       <c r="E32" t="s">
         <v>92</v>
@@ -2576,19 +2600,19 @@
         <v>96</v>
       </c>
       <c r="G32" t="s">
-        <v>108</v>
+        <v>109</v>
       </c>
       <c r="H32" s="1">
         <v>46199</v>
       </c>
       <c r="I32" t="s">
-        <v>119</v>
+        <v>120</v>
       </c>
       <c r="J32" t="s">
-        <v>133</v>
+        <v>134</v>
       </c>
       <c r="N32" t="s">
-        <v>150</v>
+        <v>151</v>
       </c>
       <c r="O32" t="s">
         <v>50</v>
@@ -2597,19 +2621,19 @@
         <v>324166.14</v>
       </c>
       <c r="Q32" t="s">
-        <v>164</v>
+        <v>165</v>
       </c>
       <c r="R32" t="s">
-        <v>167</v>
+        <v>168</v>
       </c>
       <c r="S32" t="s">
-        <v>169</v>
+        <v>170</v>
       </c>
       <c r="T32" t="s">
-        <v>172</v>
+        <v>173</v>
       </c>
       <c r="U32" t="s">
-        <v>175</v>
+        <v>176</v>
       </c>
       <c r="V32" s="1">
         <v>46199</v>
@@ -2626,7 +2650,7 @@
         <v>51</v>
       </c>
       <c r="D33" t="s">
-        <v>89</v>
+        <v>90</v>
       </c>
       <c r="E33" t="s">
         <v>92</v>
@@ -2635,13 +2659,13 @@
         <v>94</v>
       </c>
       <c r="J33" t="s">
-        <v>134</v>
+        <v>135</v>
       </c>
       <c r="K33" t="s">
-        <v>140</v>
+        <v>141</v>
       </c>
       <c r="N33" t="s">
-        <v>150</v>
+        <v>151</v>
       </c>
       <c r="O33" t="s">
         <v>51</v>
@@ -2650,19 +2674,19 @@
         <v>30000</v>
       </c>
       <c r="Q33" t="s">
-        <v>164</v>
+        <v>165</v>
       </c>
       <c r="R33" t="s">
-        <v>167</v>
+        <v>168</v>
       </c>
       <c r="S33" t="s">
-        <v>169</v>
+        <v>170</v>
       </c>
       <c r="T33" t="s">
-        <v>172</v>
+        <v>173</v>
       </c>
       <c r="U33" t="s">
-        <v>175</v>
+        <v>176</v>
       </c>
       <c r="V33" s="1">
         <v>46291</v>
@@ -2679,7 +2703,7 @@
         <v>52</v>
       </c>
       <c r="D34" t="s">
-        <v>88</v>
+        <v>89</v>
       </c>
       <c r="E34" t="s">
         <v>92</v>
@@ -2688,19 +2712,19 @@
         <v>94</v>
       </c>
       <c r="G34" t="s">
-        <v>108</v>
+        <v>109</v>
       </c>
       <c r="H34" s="1">
         <v>46191</v>
       </c>
       <c r="I34" t="s">
-        <v>121</v>
+        <v>122</v>
       </c>
       <c r="J34" t="s">
-        <v>135</v>
+        <v>136</v>
       </c>
       <c r="N34" t="s">
-        <v>150</v>
+        <v>151</v>
       </c>
       <c r="O34" t="s">
         <v>52</v>
@@ -2709,19 +2733,19 @@
         <v>1496713.48</v>
       </c>
       <c r="Q34" t="s">
-        <v>164</v>
+        <v>165</v>
       </c>
       <c r="R34" t="s">
-        <v>167</v>
+        <v>168</v>
       </c>
       <c r="S34" t="s">
-        <v>169</v>
+        <v>170</v>
       </c>
       <c r="T34" t="s">
-        <v>173</v>
+        <v>174</v>
       </c>
       <c r="U34" t="s">
-        <v>175</v>
+        <v>176</v>
       </c>
       <c r="V34" s="1">
         <v>46199</v>
@@ -2738,7 +2762,7 @@
         <v>52</v>
       </c>
       <c r="D35" t="s">
-        <v>88</v>
+        <v>89</v>
       </c>
       <c r="E35" t="s">
         <v>92</v>
@@ -2747,16 +2771,16 @@
         <v>95</v>
       </c>
       <c r="G35" t="s">
-        <v>108</v>
+        <v>109</v>
       </c>
       <c r="H35" s="1">
         <v>46119</v>
       </c>
       <c r="I35" t="s">
-        <v>116</v>
+        <v>117</v>
       </c>
       <c r="N35" t="s">
-        <v>150</v>
+        <v>151</v>
       </c>
       <c r="O35" t="s">
         <v>52</v>
@@ -2765,19 +2789,19 @@
         <v>207789.52</v>
       </c>
       <c r="Q35" t="s">
-        <v>164</v>
+        <v>165</v>
       </c>
       <c r="R35" t="s">
-        <v>167</v>
+        <v>168</v>
       </c>
       <c r="S35" t="s">
-        <v>169</v>
+        <v>170</v>
       </c>
       <c r="T35" t="s">
-        <v>173</v>
+        <v>174</v>
       </c>
       <c r="U35" t="s">
-        <v>175</v>
+        <v>176</v>
       </c>
       <c r="V35" s="1">
         <v>46138</v>
@@ -2794,7 +2818,7 @@
         <v>53</v>
       </c>
       <c r="D36" t="s">
-        <v>88</v>
+        <v>89</v>
       </c>
       <c r="E36" t="s">
         <v>92</v>
@@ -2803,16 +2827,16 @@
         <v>94</v>
       </c>
       <c r="G36" t="s">
-        <v>108</v>
+        <v>109</v>
       </c>
       <c r="H36" s="1">
         <v>46213</v>
       </c>
       <c r="I36" t="s">
-        <v>122</v>
+        <v>123</v>
       </c>
       <c r="N36" t="s">
-        <v>153</v>
+        <v>154</v>
       </c>
       <c r="O36" t="s">
         <v>53</v>
@@ -2821,16 +2845,16 @@
         <v>962290.8</v>
       </c>
       <c r="Q36" t="s">
-        <v>164</v>
+        <v>165</v>
       </c>
       <c r="R36" t="s">
-        <v>166</v>
+        <v>167</v>
       </c>
       <c r="S36" t="s">
-        <v>169</v>
+        <v>170</v>
       </c>
       <c r="T36" t="s">
-        <v>172</v>
+        <v>173</v>
       </c>
       <c r="U36" t="s">
         <v>92</v>
@@ -2850,7 +2874,7 @@
         <v>53</v>
       </c>
       <c r="D37" t="s">
-        <v>88</v>
+        <v>89</v>
       </c>
       <c r="E37" t="s">
         <v>92</v>
@@ -2859,16 +2883,16 @@
         <v>98</v>
       </c>
       <c r="G37" t="s">
-        <v>108</v>
+        <v>109</v>
       </c>
       <c r="H37" s="1">
         <v>46175</v>
       </c>
       <c r="I37" t="s">
-        <v>123</v>
+        <v>124</v>
       </c>
       <c r="N37" t="s">
-        <v>153</v>
+        <v>154</v>
       </c>
       <c r="O37" t="s">
         <v>53</v>
@@ -2877,16 +2901,16 @@
         <v>798776.97</v>
       </c>
       <c r="Q37" t="s">
-        <v>164</v>
+        <v>165</v>
       </c>
       <c r="R37" t="s">
-        <v>167</v>
+        <v>168</v>
       </c>
       <c r="S37" t="s">
-        <v>169</v>
+        <v>170</v>
       </c>
       <c r="T37" t="s">
-        <v>172</v>
+        <v>173</v>
       </c>
       <c r="U37" t="s">
         <v>92</v>
@@ -2906,7 +2930,7 @@
         <v>53</v>
       </c>
       <c r="D38" t="s">
-        <v>88</v>
+        <v>89</v>
       </c>
       <c r="E38" t="s">
         <v>92</v>
@@ -2915,16 +2939,16 @@
         <v>94</v>
       </c>
       <c r="G38" t="s">
-        <v>108</v>
+        <v>109</v>
       </c>
       <c r="H38" s="1">
         <v>46213</v>
       </c>
       <c r="I38" t="s">
-        <v>122</v>
+        <v>123</v>
       </c>
       <c r="N38" t="s">
-        <v>153</v>
+        <v>154</v>
       </c>
       <c r="O38" t="s">
         <v>53</v>
@@ -2933,16 +2957,16 @@
         <v>1530656.62</v>
       </c>
       <c r="Q38" t="s">
-        <v>164</v>
+        <v>165</v>
       </c>
       <c r="R38" t="s">
-        <v>166</v>
+        <v>167</v>
       </c>
       <c r="S38" t="s">
-        <v>169</v>
+        <v>170</v>
       </c>
       <c r="T38" t="s">
-        <v>172</v>
+        <v>173</v>
       </c>
       <c r="U38" t="s">
         <v>92</v>
@@ -2962,7 +2986,7 @@
         <v>53</v>
       </c>
       <c r="D39" t="s">
-        <v>88</v>
+        <v>89</v>
       </c>
       <c r="E39" t="s">
         <v>92</v>
@@ -2971,16 +2995,16 @@
         <v>99</v>
       </c>
       <c r="G39" t="s">
-        <v>108</v>
+        <v>109</v>
       </c>
       <c r="H39" s="1">
         <v>46199</v>
       </c>
       <c r="I39" t="s">
-        <v>124</v>
+        <v>125</v>
       </c>
       <c r="N39" t="s">
-        <v>153</v>
+        <v>154</v>
       </c>
       <c r="O39" t="s">
         <v>53</v>
@@ -2989,16 +3013,16 @@
         <v>72958.08</v>
       </c>
       <c r="Q39" t="s">
-        <v>164</v>
+        <v>165</v>
       </c>
       <c r="R39" t="s">
-        <v>166</v>
+        <v>167</v>
       </c>
       <c r="S39" t="s">
-        <v>169</v>
+        <v>170</v>
       </c>
       <c r="T39" t="s">
-        <v>172</v>
+        <v>173</v>
       </c>
       <c r="U39" t="s">
         <v>92</v>
@@ -3018,7 +3042,7 @@
         <v>53</v>
       </c>
       <c r="D40" t="s">
-        <v>88</v>
+        <v>89</v>
       </c>
       <c r="E40" t="s">
         <v>92</v>
@@ -3027,16 +3051,16 @@
         <v>100</v>
       </c>
       <c r="G40" t="s">
-        <v>108</v>
+        <v>109</v>
       </c>
       <c r="H40" s="1">
         <v>46199</v>
       </c>
       <c r="I40" t="s">
-        <v>124</v>
+        <v>125</v>
       </c>
       <c r="N40" t="s">
-        <v>153</v>
+        <v>154</v>
       </c>
       <c r="O40" t="s">
         <v>53</v>
@@ -3045,16 +3069,16 @@
         <v>8916</v>
       </c>
       <c r="Q40" t="s">
-        <v>164</v>
+        <v>165</v>
       </c>
       <c r="R40" t="s">
-        <v>166</v>
+        <v>167</v>
       </c>
       <c r="S40" t="s">
-        <v>169</v>
+        <v>170</v>
       </c>
       <c r="T40" t="s">
-        <v>172</v>
+        <v>173</v>
       </c>
       <c r="U40" t="s">
         <v>92</v>
@@ -3074,7 +3098,7 @@
         <v>53</v>
       </c>
       <c r="D41" t="s">
-        <v>88</v>
+        <v>89</v>
       </c>
       <c r="E41" t="s">
         <v>92</v>
@@ -3083,16 +3107,16 @@
         <v>101</v>
       </c>
       <c r="G41" t="s">
-        <v>108</v>
+        <v>109</v>
       </c>
       <c r="H41" s="1">
         <v>46204</v>
       </c>
       <c r="I41" t="s">
-        <v>124</v>
+        <v>125</v>
       </c>
       <c r="N41" t="s">
-        <v>153</v>
+        <v>154</v>
       </c>
       <c r="O41" t="s">
         <v>53</v>
@@ -3101,16 +3125,16 @@
         <v>425178.5</v>
       </c>
       <c r="Q41" t="s">
-        <v>164</v>
+        <v>165</v>
       </c>
       <c r="R41" t="s">
-        <v>166</v>
+        <v>167</v>
       </c>
       <c r="S41" t="s">
-        <v>169</v>
+        <v>170</v>
       </c>
       <c r="T41" t="s">
-        <v>172</v>
+        <v>173</v>
       </c>
       <c r="U41" t="s">
         <v>92</v>
@@ -3130,7 +3154,7 @@
         <v>53</v>
       </c>
       <c r="D42" t="s">
-        <v>88</v>
+        <v>89</v>
       </c>
       <c r="E42" t="s">
         <v>92</v>
@@ -3139,16 +3163,16 @@
         <v>98</v>
       </c>
       <c r="G42" t="s">
-        <v>108</v>
+        <v>109</v>
       </c>
       <c r="H42" s="1">
         <v>46244</v>
       </c>
       <c r="I42" t="s">
-        <v>125</v>
+        <v>126</v>
       </c>
       <c r="N42" t="s">
-        <v>153</v>
+        <v>154</v>
       </c>
       <c r="O42" t="s">
         <v>53</v>
@@ -3157,16 +3181,16 @@
         <v>1223.03</v>
       </c>
       <c r="Q42" t="s">
-        <v>164</v>
+        <v>165</v>
       </c>
       <c r="R42" t="s">
-        <v>166</v>
+        <v>167</v>
       </c>
       <c r="S42" t="s">
-        <v>169</v>
+        <v>170</v>
       </c>
       <c r="T42" t="s">
-        <v>172</v>
+        <v>173</v>
       </c>
       <c r="U42" t="s">
         <v>92</v>
@@ -3186,31 +3210,31 @@
         <v>54</v>
       </c>
       <c r="D43" t="s">
-        <v>90</v>
+        <v>91</v>
       </c>
       <c r="E43" t="s">
         <v>93</v>
       </c>
       <c r="G43" t="s">
-        <v>107</v>
+        <v>108</v>
       </c>
       <c r="N43" t="s">
-        <v>153</v>
+        <v>154</v>
       </c>
       <c r="O43" t="s">
         <v>54</v>
       </c>
       <c r="Q43" t="s">
-        <v>164</v>
+        <v>165</v>
       </c>
       <c r="R43" t="s">
-        <v>166</v>
+        <v>167</v>
       </c>
       <c r="S43" t="s">
-        <v>170</v>
+        <v>171</v>
       </c>
       <c r="T43" t="s">
-        <v>172</v>
+        <v>173</v>
       </c>
       <c r="U43" t="s">
         <v>92</v>
@@ -3230,7 +3254,7 @@
         <v>55</v>
       </c>
       <c r="D44" t="s">
-        <v>88</v>
+        <v>89</v>
       </c>
       <c r="E44" t="s">
         <v>92</v>
@@ -3239,16 +3263,16 @@
         <v>94</v>
       </c>
       <c r="G44" t="s">
-        <v>108</v>
+        <v>109</v>
       </c>
       <c r="H44" s="1">
         <v>46191</v>
       </c>
       <c r="I44" t="s">
-        <v>126</v>
+        <v>127</v>
       </c>
       <c r="N44" t="s">
-        <v>151</v>
+        <v>152</v>
       </c>
       <c r="O44" t="s">
         <v>55</v>
@@ -3257,16 +3281,16 @@
         <v>400000</v>
       </c>
       <c r="Q44" t="s">
-        <v>164</v>
+        <v>165</v>
       </c>
       <c r="R44" t="s">
-        <v>166</v>
+        <v>167</v>
       </c>
       <c r="S44" t="s">
-        <v>169</v>
+        <v>170</v>
       </c>
       <c r="T44" t="s">
-        <v>172</v>
+        <v>173</v>
       </c>
       <c r="U44" t="s">
         <v>92</v>
@@ -3286,7 +3310,7 @@
         <v>56</v>
       </c>
       <c r="D45" t="s">
-        <v>88</v>
+        <v>89</v>
       </c>
       <c r="E45" t="s">
         <v>92</v>
@@ -3295,16 +3319,16 @@
         <v>94</v>
       </c>
       <c r="G45" t="s">
-        <v>108</v>
+        <v>109</v>
       </c>
       <c r="H45" s="1">
         <v>46191</v>
       </c>
       <c r="I45" t="s">
-        <v>126</v>
+        <v>127</v>
       </c>
       <c r="N45" t="s">
-        <v>151</v>
+        <v>152</v>
       </c>
       <c r="O45" t="s">
         <v>56</v>
@@ -3313,16 +3337,16 @@
         <v>400000</v>
       </c>
       <c r="Q45" t="s">
-        <v>164</v>
+        <v>165</v>
       </c>
       <c r="R45" t="s">
-        <v>166</v>
+        <v>167</v>
       </c>
       <c r="S45" t="s">
-        <v>169</v>
+        <v>170</v>
       </c>
       <c r="T45" t="s">
-        <v>172</v>
+        <v>173</v>
       </c>
       <c r="U45" t="s">
         <v>92</v>
@@ -3342,7 +3366,7 @@
         <v>57</v>
       </c>
       <c r="D46" t="s">
-        <v>88</v>
+        <v>89</v>
       </c>
       <c r="E46" t="s">
         <v>92</v>
@@ -3351,19 +3375,19 @@
         <v>94</v>
       </c>
       <c r="G46" t="s">
-        <v>108</v>
+        <v>109</v>
       </c>
       <c r="H46" s="1">
         <v>46213</v>
       </c>
       <c r="I46" t="s">
-        <v>121</v>
+        <v>122</v>
       </c>
       <c r="J46" t="s">
-        <v>136</v>
+        <v>137</v>
       </c>
       <c r="N46" t="s">
-        <v>150</v>
+        <v>151</v>
       </c>
       <c r="O46" t="s">
         <v>57</v>
@@ -3372,19 +3396,19 @@
         <v>173846.38</v>
       </c>
       <c r="Q46" t="s">
-        <v>164</v>
+        <v>165</v>
       </c>
       <c r="R46" t="s">
-        <v>167</v>
+        <v>168</v>
       </c>
       <c r="S46" t="s">
-        <v>169</v>
+        <v>170</v>
       </c>
       <c r="T46" t="s">
-        <v>173</v>
+        <v>174</v>
       </c>
       <c r="U46" t="s">
-        <v>175</v>
+        <v>176</v>
       </c>
       <c r="V46" s="1">
         <v>46229</v>
@@ -3401,7 +3425,7 @@
         <v>57</v>
       </c>
       <c r="D47" t="s">
-        <v>88</v>
+        <v>89</v>
       </c>
       <c r="E47" t="s">
         <v>92</v>
@@ -3410,16 +3434,16 @@
         <v>97</v>
       </c>
       <c r="G47" t="s">
-        <v>108</v>
+        <v>109</v>
       </c>
       <c r="H47" s="1">
         <v>46210</v>
       </c>
       <c r="I47" t="s">
-        <v>120</v>
+        <v>121</v>
       </c>
       <c r="N47" t="s">
-        <v>150</v>
+        <v>151</v>
       </c>
       <c r="O47" t="s">
         <v>57</v>
@@ -3428,19 +3452,19 @@
         <v>1530656.62</v>
       </c>
       <c r="Q47" t="s">
-        <v>164</v>
+        <v>165</v>
       </c>
       <c r="R47" t="s">
-        <v>167</v>
+        <v>168</v>
       </c>
       <c r="S47" t="s">
-        <v>169</v>
+        <v>170</v>
       </c>
       <c r="T47" t="s">
-        <v>173</v>
+        <v>174</v>
       </c>
       <c r="U47" t="s">
-        <v>175</v>
+        <v>176</v>
       </c>
       <c r="V47" s="1">
         <v>46229</v>
@@ -3457,7 +3481,7 @@
         <v>58</v>
       </c>
       <c r="D48" t="s">
-        <v>89</v>
+        <v>90</v>
       </c>
       <c r="E48" t="s">
         <v>92</v>
@@ -3466,7 +3490,7 @@
         <v>94</v>
       </c>
       <c r="N48" t="s">
-        <v>152</v>
+        <v>153</v>
       </c>
       <c r="O48" t="s">
         <v>58</v>
@@ -3475,16 +3499,16 @@
         <v>1000000</v>
       </c>
       <c r="Q48" t="s">
-        <v>164</v>
+        <v>165</v>
       </c>
       <c r="R48" t="s">
-        <v>166</v>
+        <v>167</v>
       </c>
       <c r="S48" t="s">
-        <v>169</v>
+        <v>170</v>
       </c>
       <c r="T48" t="s">
-        <v>172</v>
+        <v>173</v>
       </c>
       <c r="U48" t="s">
         <v>92</v>
@@ -3513,19 +3537,22 @@
         <v>94</v>
       </c>
       <c r="G49" t="s">
-        <v>106</v>
+        <v>107</v>
+      </c>
+      <c r="H49" s="1">
+        <v>46303</v>
       </c>
       <c r="I49" t="s">
-        <v>111</v>
+        <v>112</v>
       </c>
       <c r="J49" t="s">
-        <v>130</v>
+        <v>131</v>
       </c>
       <c r="K49" t="s">
-        <v>106</v>
+        <v>110</v>
       </c>
       <c r="N49" t="s">
-        <v>145</v>
+        <v>146</v>
       </c>
       <c r="O49" t="s">
         <v>59</v>
@@ -3534,19 +3561,19 @@
         <v>958040</v>
       </c>
       <c r="Q49" t="s">
-        <v>163</v>
+        <v>164</v>
       </c>
       <c r="R49" t="s">
-        <v>166</v>
+        <v>167</v>
       </c>
       <c r="S49" t="s">
-        <v>169</v>
+        <v>170</v>
       </c>
       <c r="T49" t="s">
-        <v>171</v>
+        <v>172</v>
       </c>
       <c r="U49" t="s">
-        <v>175</v>
+        <v>176</v>
       </c>
       <c r="V49" s="1">
         <v>46291</v>
@@ -3563,7 +3590,7 @@
         <v>59</v>
       </c>
       <c r="D50" t="s">
-        <v>88</v>
+        <v>89</v>
       </c>
       <c r="E50" t="s">
         <v>92</v>
@@ -3572,19 +3599,19 @@
         <v>94</v>
       </c>
       <c r="G50" t="s">
-        <v>108</v>
+        <v>109</v>
       </c>
       <c r="H50" s="1">
         <v>46176</v>
       </c>
       <c r="I50" t="s">
-        <v>127</v>
+        <v>128</v>
       </c>
       <c r="J50" t="s">
-        <v>137</v>
+        <v>138</v>
       </c>
       <c r="N50" t="s">
-        <v>145</v>
+        <v>146</v>
       </c>
       <c r="O50" t="s">
         <v>59</v>
@@ -3593,19 +3620,19 @@
         <v>41730.64</v>
       </c>
       <c r="Q50" t="s">
-        <v>163</v>
+        <v>164</v>
       </c>
       <c r="R50" t="s">
-        <v>168</v>
+        <v>169</v>
       </c>
       <c r="S50" t="s">
-        <v>169</v>
+        <v>170</v>
       </c>
       <c r="T50" t="s">
-        <v>171</v>
+        <v>172</v>
       </c>
       <c r="U50" t="s">
-        <v>175</v>
+        <v>176</v>
       </c>
       <c r="V50" s="1">
         <v>46199</v>
@@ -3622,7 +3649,7 @@
         <v>60</v>
       </c>
       <c r="D51" t="s">
-        <v>87</v>
+        <v>88</v>
       </c>
       <c r="E51" t="s">
         <v>92</v>
@@ -3631,16 +3658,16 @@
         <v>94</v>
       </c>
       <c r="G51" t="s">
-        <v>106</v>
+        <v>110</v>
       </c>
       <c r="J51" t="s">
-        <v>136</v>
+        <v>137</v>
       </c>
       <c r="K51" t="s">
-        <v>141</v>
+        <v>142</v>
       </c>
       <c r="N51" t="s">
-        <v>150</v>
+        <v>151</v>
       </c>
       <c r="O51" t="s">
         <v>60</v>
@@ -3649,19 +3676,19 @@
         <v>608623.25</v>
       </c>
       <c r="Q51" t="s">
-        <v>164</v>
+        <v>165</v>
       </c>
       <c r="R51" t="s">
-        <v>167</v>
+        <v>168</v>
       </c>
       <c r="S51" t="s">
-        <v>169</v>
+        <v>170</v>
       </c>
       <c r="T51" t="s">
-        <v>173</v>
+        <v>174</v>
       </c>
       <c r="U51" t="s">
-        <v>175</v>
+        <v>176</v>
       </c>
       <c r="V51" s="1">
         <v>46260</v>
@@ -3678,7 +3705,7 @@
         <v>61</v>
       </c>
       <c r="D52" t="s">
-        <v>88</v>
+        <v>89</v>
       </c>
       <c r="E52" t="s">
         <v>92</v>
@@ -3687,22 +3714,22 @@
         <v>94</v>
       </c>
       <c r="G52" t="s">
-        <v>108</v>
+        <v>109</v>
       </c>
       <c r="H52" s="1">
         <v>46295</v>
       </c>
       <c r="I52" t="s">
-        <v>121</v>
+        <v>122</v>
       </c>
       <c r="J52" t="s">
-        <v>136</v>
+        <v>137</v>
       </c>
       <c r="K52" t="s">
-        <v>139</v>
+        <v>140</v>
       </c>
       <c r="N52" t="s">
-        <v>150</v>
+        <v>151</v>
       </c>
       <c r="O52" t="s">
         <v>61</v>
@@ -3711,19 +3738,19 @@
         <v>66366.75999999999</v>
       </c>
       <c r="Q52" t="s">
-        <v>164</v>
+        <v>165</v>
       </c>
       <c r="R52" t="s">
-        <v>167</v>
+        <v>168</v>
       </c>
       <c r="S52" t="s">
-        <v>169</v>
+        <v>170</v>
       </c>
       <c r="T52" t="s">
-        <v>173</v>
+        <v>174</v>
       </c>
       <c r="U52" t="s">
-        <v>175</v>
+        <v>176</v>
       </c>
       <c r="V52" s="1">
         <v>46291</v>
@@ -3740,7 +3767,7 @@
         <v>62</v>
       </c>
       <c r="D53" t="s">
-        <v>89</v>
+        <v>90</v>
       </c>
       <c r="E53" t="s">
         <v>92</v>
@@ -3749,34 +3776,34 @@
         <v>94</v>
       </c>
       <c r="J53" t="s">
-        <v>134</v>
+        <v>135</v>
       </c>
       <c r="K53" t="s">
-        <v>140</v>
+        <v>141</v>
       </c>
       <c r="N53" t="s">
-        <v>150</v>
+        <v>151</v>
       </c>
       <c r="O53" t="s">
         <v>62</v>
       </c>
       <c r="P53">
-        <v>1704503</v>
+        <v>1586760.42</v>
       </c>
       <c r="Q53" t="s">
-        <v>164</v>
+        <v>165</v>
       </c>
       <c r="R53" t="s">
-        <v>167</v>
+        <v>168</v>
       </c>
       <c r="S53" t="s">
-        <v>169</v>
+        <v>170</v>
       </c>
       <c r="T53" t="s">
-        <v>173</v>
+        <v>174</v>
       </c>
       <c r="U53" t="s">
-        <v>175</v>
+        <v>176</v>
       </c>
       <c r="V53" s="1">
         <v>46321</v>
@@ -3793,7 +3820,7 @@
         <v>60</v>
       </c>
       <c r="D54" t="s">
-        <v>88</v>
+        <v>89</v>
       </c>
       <c r="E54" t="s">
         <v>92</v>
@@ -3802,16 +3829,16 @@
         <v>102</v>
       </c>
       <c r="G54" t="s">
-        <v>108</v>
+        <v>109</v>
       </c>
       <c r="H54" s="1">
         <v>46227</v>
       </c>
       <c r="I54" t="s">
-        <v>128</v>
+        <v>129</v>
       </c>
       <c r="N54" t="s">
-        <v>150</v>
+        <v>151</v>
       </c>
       <c r="O54" t="s">
         <v>60</v>
@@ -3820,19 +3847,19 @@
         <v>236343.68</v>
       </c>
       <c r="Q54" t="s">
-        <v>164</v>
+        <v>165</v>
       </c>
       <c r="R54" t="s">
-        <v>167</v>
+        <v>168</v>
       </c>
       <c r="S54" t="s">
-        <v>169</v>
+        <v>170</v>
       </c>
       <c r="T54" t="s">
-        <v>173</v>
+        <v>174</v>
       </c>
       <c r="U54" t="s">
-        <v>175</v>
+        <v>176</v>
       </c>
       <c r="V54" s="1">
         <v>46229</v>
@@ -3846,7 +3873,7 @@
         <v>22</v>
       </c>
       <c r="D55" t="s">
-        <v>88</v>
+        <v>89</v>
       </c>
       <c r="E55" t="s">
         <v>92</v>
@@ -3855,16 +3882,16 @@
         <v>103</v>
       </c>
       <c r="G55" t="s">
-        <v>108</v>
+        <v>109</v>
       </c>
       <c r="H55" s="1">
         <v>46280</v>
       </c>
       <c r="I55" t="s">
-        <v>120</v>
+        <v>121</v>
       </c>
       <c r="N55" t="s">
-        <v>150</v>
+        <v>151</v>
       </c>
       <c r="O55" t="s">
         <v>61</v>
@@ -3873,19 +3900,19 @@
         <v>1145462.93</v>
       </c>
       <c r="Q55" t="s">
-        <v>164</v>
+        <v>165</v>
       </c>
       <c r="R55" t="s">
-        <v>167</v>
+        <v>168</v>
       </c>
       <c r="S55" t="s">
-        <v>169</v>
+        <v>170</v>
       </c>
       <c r="T55" t="s">
-        <v>173</v>
+        <v>174</v>
       </c>
       <c r="U55" t="s">
-        <v>175</v>
+        <v>176</v>
       </c>
       <c r="V55" s="1">
         <v>46291</v>
@@ -3899,7 +3926,7 @@
         <v>22</v>
       </c>
       <c r="D56" t="s">
-        <v>88</v>
+        <v>89</v>
       </c>
       <c r="E56" t="s">
         <v>92</v>
@@ -3908,16 +3935,16 @@
         <v>104</v>
       </c>
       <c r="G56" t="s">
-        <v>108</v>
+        <v>109</v>
       </c>
       <c r="H56" s="1">
         <v>46280</v>
       </c>
       <c r="I56" t="s">
-        <v>120</v>
+        <v>121</v>
       </c>
       <c r="N56" t="s">
-        <v>150</v>
+        <v>151</v>
       </c>
       <c r="O56" t="s">
         <v>60</v>
@@ -3926,19 +3953,19 @@
         <v>859536.0699999999</v>
       </c>
       <c r="Q56" t="s">
-        <v>164</v>
+        <v>165</v>
       </c>
       <c r="R56" t="s">
-        <v>167</v>
+        <v>168</v>
       </c>
       <c r="S56" t="s">
-        <v>169</v>
+        <v>170</v>
       </c>
       <c r="T56" t="s">
-        <v>173</v>
+        <v>174</v>
       </c>
       <c r="U56" t="s">
-        <v>175</v>
+        <v>176</v>
       </c>
       <c r="V56" s="1">
         <v>46260</v>
@@ -3952,7 +3979,7 @@
         <v>22</v>
       </c>
       <c r="D57" t="s">
-        <v>88</v>
+        <v>89</v>
       </c>
       <c r="E57" t="s">
         <v>92</v>
@@ -3961,16 +3988,16 @@
         <v>94</v>
       </c>
       <c r="G57" t="s">
-        <v>108</v>
+        <v>109</v>
       </c>
       <c r="H57" s="1">
         <v>46295</v>
       </c>
       <c r="I57" t="s">
-        <v>114</v>
+        <v>115</v>
       </c>
       <c r="N57" t="s">
-        <v>150</v>
+        <v>151</v>
       </c>
       <c r="O57" t="s">
         <v>61</v>
@@ -3979,19 +4006,19 @@
         <v>389619.06</v>
       </c>
       <c r="Q57" t="s">
-        <v>164</v>
+        <v>165</v>
       </c>
       <c r="R57" t="s">
-        <v>167</v>
+        <v>168</v>
       </c>
       <c r="S57" t="s">
-        <v>169</v>
+        <v>170</v>
       </c>
       <c r="T57" t="s">
-        <v>173</v>
+        <v>174</v>
       </c>
       <c r="U57" t="s">
-        <v>175</v>
+        <v>176</v>
       </c>
       <c r="V57" s="1">
         <v>46291</v>
@@ -4005,7 +4032,7 @@
         <v>22</v>
       </c>
       <c r="D58" t="s">
-        <v>88</v>
+        <v>89</v>
       </c>
       <c r="E58" t="s">
         <v>92</v>
@@ -4014,16 +4041,16 @@
         <v>94</v>
       </c>
       <c r="G58" t="s">
-        <v>108</v>
+        <v>109</v>
       </c>
       <c r="H58" s="1">
         <v>46295</v>
       </c>
       <c r="I58" t="s">
-        <v>129</v>
+        <v>130</v>
       </c>
       <c r="N58" t="s">
-        <v>150</v>
+        <v>151</v>
       </c>
       <c r="O58" t="s">
         <v>61</v>
@@ -4032,19 +4059,19 @@
         <v>103054.25</v>
       </c>
       <c r="Q58" t="s">
-        <v>164</v>
+        <v>165</v>
       </c>
       <c r="R58" t="s">
-        <v>167</v>
+        <v>168</v>
       </c>
       <c r="S58" t="s">
-        <v>169</v>
+        <v>170</v>
       </c>
       <c r="T58" t="s">
-        <v>173</v>
+        <v>174</v>
       </c>
       <c r="U58" t="s">
-        <v>175</v>
+        <v>176</v>
       </c>
       <c r="V58" s="1">
         <v>46291</v>
@@ -4052,90 +4079,96 @@
     </row>
     <row r="59" spans="1:22">
       <c r="A59">
-        <v>18140</v>
+        <v>17768</v>
       </c>
       <c r="B59" t="s">
         <v>22</v>
       </c>
-      <c r="C59" t="s">
-        <v>63</v>
-      </c>
       <c r="D59" t="s">
-        <v>91</v>
+        <v>88</v>
       </c>
       <c r="E59" t="s">
         <v>92</v>
       </c>
       <c r="F59" t="s">
-        <v>94</v>
+        <v>105</v>
       </c>
       <c r="G59" t="s">
-        <v>109</v>
-      </c>
-      <c r="H59" s="1">
-        <v>46301</v>
-      </c>
-      <c r="J59" t="s">
-        <v>130</v>
-      </c>
-      <c r="K59" t="s">
-        <v>142</v>
+        <v>110</v>
       </c>
       <c r="N59" t="s">
-        <v>150</v>
+        <v>151</v>
       </c>
       <c r="O59" t="s">
-        <v>63</v>
+        <v>62</v>
       </c>
       <c r="P59">
-        <v>1295422.28</v>
+        <v>117742.58</v>
       </c>
       <c r="Q59" t="s">
-        <v>164</v>
+        <v>165</v>
       </c>
       <c r="R59" t="s">
-        <v>167</v>
+        <v>168</v>
       </c>
       <c r="S59" t="s">
-        <v>169</v>
+        <v>170</v>
       </c>
       <c r="T59" t="s">
-        <v>173</v>
+        <v>174</v>
       </c>
       <c r="U59" t="s">
-        <v>175</v>
+        <v>176</v>
       </c>
       <c r="V59" s="1">
-        <v>46352</v>
+        <v>46321</v>
       </c>
     </row>
     <row r="60" spans="1:22">
       <c r="A60">
-        <v>23080</v>
+        <v>18140</v>
       </c>
       <c r="B60" t="s">
         <v>22</v>
       </c>
       <c r="C60" t="s">
-        <v>64</v>
+        <v>63</v>
       </c>
       <c r="D60" t="s">
-        <v>90</v>
+        <v>89</v>
       </c>
       <c r="E60" t="s">
-        <v>93</v>
+        <v>92</v>
+      </c>
+      <c r="F60" t="s">
+        <v>94</v>
+      </c>
+      <c r="G60" t="s">
+        <v>109</v>
+      </c>
+      <c r="H60" s="1">
+        <v>46301</v>
+      </c>
+      <c r="I60" t="s">
+        <v>115</v>
+      </c>
+      <c r="J60" t="s">
+        <v>131</v>
+      </c>
+      <c r="K60" t="s">
+        <v>143</v>
       </c>
       <c r="N60" t="s">
-        <v>154</v>
+        <v>151</v>
       </c>
       <c r="O60" t="s">
-        <v>64</v>
+        <v>63</v>
       </c>
       <c r="P60">
-        <v>4064.54</v>
+        <v>1295422.28</v>
       </c>
       <c r="Q60" t="s">
-        <v>164</v>
+        <v>165</v>
       </c>
       <c r="R60" t="s">
         <v>168</v>
@@ -4144,27 +4177,27 @@
         <v>170</v>
       </c>
       <c r="T60" t="s">
-        <v>171</v>
+        <v>174</v>
       </c>
       <c r="U60" t="s">
-        <v>175</v>
+        <v>176</v>
       </c>
       <c r="V60" s="1">
-        <v>46107</v>
+        <v>46352</v>
       </c>
     </row>
     <row r="61" spans="1:22">
       <c r="A61">
-        <v>23100</v>
+        <v>23080</v>
       </c>
       <c r="B61" t="s">
         <v>22</v>
       </c>
       <c r="C61" t="s">
-        <v>65</v>
+        <v>64</v>
       </c>
       <c r="D61" t="s">
-        <v>90</v>
+        <v>91</v>
       </c>
       <c r="E61" t="s">
         <v>93</v>
@@ -4173,25 +4206,25 @@
         <v>155</v>
       </c>
       <c r="O61" t="s">
-        <v>65</v>
+        <v>64</v>
       </c>
       <c r="P61">
-        <v>4227.84</v>
+        <v>4064.54</v>
       </c>
       <c r="Q61" t="s">
-        <v>163</v>
+        <v>165</v>
       </c>
       <c r="R61" t="s">
-        <v>168</v>
+        <v>169</v>
       </c>
       <c r="S61" t="s">
-        <v>170</v>
+        <v>171</v>
       </c>
       <c r="T61" t="s">
-        <v>171</v>
+        <v>172</v>
       </c>
       <c r="U61" t="s">
-        <v>175</v>
+        <v>176</v>
       </c>
       <c r="V61" s="1">
         <v>46107</v>
@@ -4199,16 +4232,16 @@
     </row>
     <row r="62" spans="1:22">
       <c r="A62">
-        <v>23120</v>
+        <v>23100</v>
       </c>
       <c r="B62" t="s">
         <v>22</v>
       </c>
       <c r="C62" t="s">
-        <v>66</v>
+        <v>65</v>
       </c>
       <c r="D62" t="s">
-        <v>90</v>
+        <v>91</v>
       </c>
       <c r="E62" t="s">
         <v>93</v>
@@ -4217,25 +4250,25 @@
         <v>156</v>
       </c>
       <c r="O62" t="s">
-        <v>66</v>
+        <v>65</v>
       </c>
       <c r="P62">
-        <v>9389.959999999999</v>
+        <v>4227.84</v>
       </c>
       <c r="Q62" t="s">
-        <v>163</v>
+        <v>164</v>
       </c>
       <c r="R62" t="s">
-        <v>168</v>
+        <v>169</v>
       </c>
       <c r="S62" t="s">
-        <v>170</v>
+        <v>171</v>
       </c>
       <c r="T62" t="s">
-        <v>171</v>
+        <v>172</v>
       </c>
       <c r="U62" t="s">
-        <v>175</v>
+        <v>176</v>
       </c>
       <c r="V62" s="1">
         <v>46107</v>
@@ -4243,16 +4276,16 @@
     </row>
     <row r="63" spans="1:22">
       <c r="A63">
-        <v>23140</v>
+        <v>23120</v>
       </c>
       <c r="B63" t="s">
         <v>22</v>
       </c>
       <c r="C63" t="s">
-        <v>67</v>
+        <v>66</v>
       </c>
       <c r="D63" t="s">
-        <v>90</v>
+        <v>91</v>
       </c>
       <c r="E63" t="s">
         <v>93</v>
@@ -4261,25 +4294,25 @@
         <v>157</v>
       </c>
       <c r="O63" t="s">
-        <v>67</v>
+        <v>66</v>
       </c>
       <c r="P63">
-        <v>1163.64</v>
+        <v>9389.959999999999</v>
       </c>
       <c r="Q63" t="s">
-        <v>165</v>
+        <v>164</v>
       </c>
       <c r="R63" t="s">
-        <v>168</v>
+        <v>169</v>
       </c>
       <c r="S63" t="s">
-        <v>170</v>
+        <v>171</v>
       </c>
       <c r="T63" t="s">
-        <v>171</v>
+        <v>172</v>
       </c>
       <c r="U63" t="s">
-        <v>175</v>
+        <v>176</v>
       </c>
       <c r="V63" s="1">
         <v>46107</v>
@@ -4287,16 +4320,16 @@
     </row>
     <row r="64" spans="1:22">
       <c r="A64">
-        <v>23160</v>
+        <v>23140</v>
       </c>
       <c r="B64" t="s">
         <v>22</v>
       </c>
       <c r="C64" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
       <c r="D64" t="s">
-        <v>90</v>
+        <v>91</v>
       </c>
       <c r="E64" t="s">
         <v>93</v>
@@ -4305,25 +4338,25 @@
         <v>158</v>
       </c>
       <c r="O64" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
       <c r="P64">
-        <v>7204.82</v>
+        <v>1163.64</v>
       </c>
       <c r="Q64" t="s">
-        <v>163</v>
+        <v>166</v>
       </c>
       <c r="R64" t="s">
-        <v>168</v>
+        <v>169</v>
       </c>
       <c r="S64" t="s">
-        <v>170</v>
+        <v>171</v>
       </c>
       <c r="T64" t="s">
-        <v>171</v>
+        <v>172</v>
       </c>
       <c r="U64" t="s">
-        <v>175</v>
+        <v>176</v>
       </c>
       <c r="V64" s="1">
         <v>46107</v>
@@ -4331,16 +4364,16 @@
     </row>
     <row r="65" spans="1:22">
       <c r="A65">
-        <v>23180</v>
+        <v>23160</v>
       </c>
       <c r="B65" t="s">
         <v>22</v>
       </c>
       <c r="C65" t="s">
-        <v>65</v>
+        <v>68</v>
       </c>
       <c r="D65" t="s">
-        <v>90</v>
+        <v>91</v>
       </c>
       <c r="E65" t="s">
         <v>93</v>
@@ -4349,25 +4382,25 @@
         <v>159</v>
       </c>
       <c r="O65" t="s">
-        <v>65</v>
+        <v>68</v>
       </c>
       <c r="P65">
-        <v>3662.66</v>
+        <v>7204.82</v>
       </c>
       <c r="Q65" t="s">
-        <v>163</v>
+        <v>164</v>
       </c>
       <c r="R65" t="s">
-        <v>168</v>
+        <v>169</v>
       </c>
       <c r="S65" t="s">
-        <v>170</v>
+        <v>171</v>
       </c>
       <c r="T65" t="s">
-        <v>171</v>
+        <v>172</v>
       </c>
       <c r="U65" t="s">
-        <v>175</v>
+        <v>176</v>
       </c>
       <c r="V65" s="1">
         <v>46107</v>
@@ -4375,107 +4408,104 @@
     </row>
     <row r="66" spans="1:22">
       <c r="A66">
-        <v>23640</v>
+        <v>23180</v>
       </c>
       <c r="B66" t="s">
         <v>22</v>
       </c>
       <c r="C66" t="s">
-        <v>69</v>
+        <v>65</v>
       </c>
       <c r="D66" t="s">
-        <v>90</v>
+        <v>91</v>
       </c>
       <c r="E66" t="s">
         <v>93</v>
       </c>
       <c r="N66" t="s">
-        <v>146</v>
+        <v>160</v>
       </c>
       <c r="O66" t="s">
-        <v>69</v>
+        <v>65</v>
       </c>
       <c r="P66">
-        <v>120000</v>
+        <v>3662.66</v>
       </c>
       <c r="Q66" t="s">
-        <v>163</v>
+        <v>164</v>
       </c>
       <c r="R66" t="s">
-        <v>167</v>
+        <v>169</v>
       </c>
       <c r="S66" t="s">
-        <v>170</v>
+        <v>171</v>
       </c>
       <c r="T66" t="s">
-        <v>171</v>
+        <v>172</v>
       </c>
       <c r="U66" t="s">
-        <v>92</v>
+        <v>176</v>
       </c>
       <c r="V66" s="1">
-        <v>46168</v>
+        <v>46107</v>
       </c>
     </row>
     <row r="67" spans="1:22">
       <c r="A67">
-        <v>23740</v>
+        <v>23640</v>
       </c>
       <c r="B67" t="s">
         <v>22</v>
       </c>
       <c r="C67" t="s">
-        <v>70</v>
+        <v>69</v>
       </c>
       <c r="D67" t="s">
-        <v>87</v>
+        <v>91</v>
       </c>
       <c r="E67" t="s">
-        <v>92</v>
-      </c>
-      <c r="F67" t="s">
-        <v>94</v>
-      </c>
-      <c r="G67" t="s">
-        <v>107</v>
+        <v>93</v>
       </c>
       <c r="N67" t="s">
-        <v>145</v>
+        <v>147</v>
       </c>
       <c r="O67" t="s">
-        <v>70</v>
+        <v>69</v>
+      </c>
+      <c r="P67">
+        <v>120000</v>
       </c>
       <c r="Q67" t="s">
-        <v>163</v>
+        <v>164</v>
       </c>
       <c r="R67" t="s">
-        <v>166</v>
+        <v>168</v>
       </c>
       <c r="S67" t="s">
-        <v>169</v>
+        <v>171</v>
       </c>
       <c r="T67" t="s">
-        <v>171</v>
+        <v>172</v>
       </c>
       <c r="U67" t="s">
         <v>92</v>
       </c>
       <c r="V67" s="1">
-        <v>46291</v>
+        <v>46168</v>
       </c>
     </row>
     <row r="68" spans="1:22">
       <c r="A68">
-        <v>24180</v>
+        <v>23740</v>
       </c>
       <c r="B68" t="s">
         <v>22</v>
       </c>
       <c r="C68" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
       <c r="D68" t="s">
-        <v>87</v>
+        <v>88</v>
       </c>
       <c r="E68" t="s">
         <v>92</v>
@@ -4484,72 +4514,78 @@
         <v>94</v>
       </c>
       <c r="G68" t="s">
-        <v>106</v>
-      </c>
-      <c r="I68" t="s">
-        <v>111</v>
-      </c>
-      <c r="J68" t="s">
-        <v>130</v>
-      </c>
-      <c r="K68" t="s">
-        <v>106</v>
+        <v>108</v>
       </c>
       <c r="N68" t="s">
-        <v>149</v>
+        <v>146</v>
       </c>
       <c r="O68" t="s">
-        <v>71</v>
-      </c>
-      <c r="P68">
-        <v>100000</v>
+        <v>70</v>
       </c>
       <c r="Q68" t="s">
-        <v>165</v>
+        <v>164</v>
       </c>
       <c r="R68" t="s">
-        <v>166</v>
+        <v>167</v>
       </c>
       <c r="S68" t="s">
-        <v>169</v>
+        <v>170</v>
       </c>
       <c r="T68" t="s">
-        <v>171</v>
+        <v>172</v>
       </c>
       <c r="U68" t="s">
-        <v>175</v>
+        <v>92</v>
       </c>
       <c r="V68" s="1">
-        <v>46229</v>
+        <v>46291</v>
       </c>
     </row>
     <row r="69" spans="1:22">
       <c r="A69">
-        <v>24380</v>
+        <v>24180</v>
       </c>
       <c r="B69" t="s">
         <v>22</v>
       </c>
       <c r="C69" t="s">
-        <v>72</v>
+        <v>71</v>
       </c>
       <c r="D69" t="s">
-        <v>90</v>
+        <v>87</v>
       </c>
       <c r="E69" t="s">
-        <v>93</v>
+        <v>92</v>
+      </c>
+      <c r="F69" t="s">
+        <v>94</v>
+      </c>
+      <c r="G69" t="s">
+        <v>107</v>
+      </c>
+      <c r="H69" s="1">
+        <v>46303</v>
+      </c>
+      <c r="I69" t="s">
+        <v>112</v>
+      </c>
+      <c r="J69" t="s">
+        <v>131</v>
+      </c>
+      <c r="K69" t="s">
+        <v>110</v>
       </c>
       <c r="N69" t="s">
-        <v>146</v>
+        <v>150</v>
       </c>
       <c r="O69" t="s">
-        <v>72</v>
+        <v>71</v>
       </c>
       <c r="P69">
-        <v>80000</v>
+        <v>100000</v>
       </c>
       <c r="Q69" t="s">
-        <v>163</v>
+        <v>166</v>
       </c>
       <c r="R69" t="s">
         <v>167</v>
@@ -4558,62 +4594,62 @@
         <v>170</v>
       </c>
       <c r="T69" t="s">
-        <v>171</v>
+        <v>172</v>
       </c>
       <c r="U69" t="s">
-        <v>92</v>
+        <v>176</v>
       </c>
       <c r="V69" s="1">
-        <v>46260</v>
+        <v>46229</v>
       </c>
     </row>
     <row r="70" spans="1:22">
       <c r="A70">
-        <v>24660</v>
+        <v>24380</v>
       </c>
       <c r="B70" t="s">
         <v>22</v>
       </c>
       <c r="C70" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
       <c r="D70" t="s">
-        <v>90</v>
+        <v>91</v>
       </c>
       <c r="E70" t="s">
         <v>93</v>
       </c>
       <c r="N70" t="s">
-        <v>145</v>
+        <v>147</v>
       </c>
       <c r="O70" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
       <c r="P70">
-        <v>835000</v>
+        <v>80000</v>
       </c>
       <c r="Q70" t="s">
-        <v>163</v>
+        <v>164</v>
       </c>
       <c r="R70" t="s">
-        <v>166</v>
+        <v>168</v>
       </c>
       <c r="S70" t="s">
-        <v>170</v>
+        <v>171</v>
       </c>
       <c r="T70" t="s">
-        <v>171</v>
+        <v>172</v>
       </c>
       <c r="U70" t="s">
-        <v>175</v>
+        <v>92</v>
       </c>
       <c r="V70" s="1">
-        <v>46291</v>
+        <v>46260</v>
       </c>
     </row>
     <row r="71" spans="1:22">
       <c r="A71">
-        <v>24661</v>
+        <v>24660</v>
       </c>
       <c r="B71" t="s">
         <v>22</v>
@@ -4622,122 +4658,122 @@
         <v>73</v>
       </c>
       <c r="D71" t="s">
-        <v>90</v>
+        <v>91</v>
       </c>
       <c r="E71" t="s">
         <v>93</v>
       </c>
       <c r="N71" t="s">
-        <v>145</v>
+        <v>146</v>
       </c>
       <c r="O71" t="s">
         <v>73</v>
       </c>
       <c r="P71">
-        <v>165000</v>
+        <v>835000</v>
       </c>
       <c r="Q71" t="s">
-        <v>163</v>
+        <v>164</v>
       </c>
       <c r="R71" t="s">
-        <v>166</v>
+        <v>167</v>
       </c>
       <c r="S71" t="s">
-        <v>170</v>
+        <v>171</v>
       </c>
       <c r="T71" t="s">
-        <v>171</v>
+        <v>172</v>
       </c>
       <c r="U71" t="s">
-        <v>175</v>
+        <v>176</v>
       </c>
       <c r="V71" s="1">
-        <v>46168</v>
+        <v>46291</v>
       </c>
     </row>
     <row r="72" spans="1:22">
       <c r="A72">
-        <v>24680</v>
+        <v>24661</v>
       </c>
       <c r="B72" t="s">
         <v>22</v>
       </c>
       <c r="C72" t="s">
-        <v>74</v>
+        <v>73</v>
       </c>
       <c r="D72" t="s">
-        <v>90</v>
+        <v>91</v>
       </c>
       <c r="E72" t="s">
         <v>93</v>
       </c>
       <c r="N72" t="s">
-        <v>145</v>
+        <v>146</v>
       </c>
       <c r="O72" t="s">
-        <v>74</v>
+        <v>73</v>
       </c>
       <c r="P72">
-        <v>1000000</v>
+        <v>165000</v>
       </c>
       <c r="Q72" t="s">
-        <v>163</v>
+        <v>164</v>
       </c>
       <c r="R72" t="s">
-        <v>166</v>
+        <v>167</v>
       </c>
       <c r="S72" t="s">
-        <v>170</v>
+        <v>171</v>
       </c>
       <c r="T72" t="s">
-        <v>171</v>
+        <v>172</v>
       </c>
       <c r="U72" t="s">
-        <v>175</v>
+        <v>176</v>
       </c>
       <c r="V72" s="1">
-        <v>46291</v>
+        <v>46168</v>
       </c>
     </row>
     <row r="73" spans="1:22">
       <c r="A73">
-        <v>24700</v>
+        <v>24680</v>
       </c>
       <c r="B73" t="s">
         <v>22</v>
       </c>
       <c r="C73" t="s">
-        <v>75</v>
+        <v>74</v>
       </c>
       <c r="D73" t="s">
-        <v>90</v>
+        <v>91</v>
       </c>
       <c r="E73" t="s">
         <v>93</v>
       </c>
       <c r="N73" t="s">
-        <v>145</v>
+        <v>146</v>
       </c>
       <c r="O73" t="s">
-        <v>75</v>
+        <v>74</v>
       </c>
       <c r="P73">
         <v>1000000</v>
       </c>
       <c r="Q73" t="s">
-        <v>163</v>
+        <v>164</v>
       </c>
       <c r="R73" t="s">
-        <v>166</v>
+        <v>167</v>
       </c>
       <c r="S73" t="s">
-        <v>170</v>
+        <v>171</v>
       </c>
       <c r="T73" t="s">
-        <v>171</v>
+        <v>172</v>
       </c>
       <c r="U73" t="s">
-        <v>175</v>
+        <v>176</v>
       </c>
       <c r="V73" s="1">
         <v>46291</v>
@@ -4745,43 +4781,43 @@
     </row>
     <row r="74" spans="1:22">
       <c r="A74">
-        <v>24720</v>
+        <v>24700</v>
       </c>
       <c r="B74" t="s">
         <v>22</v>
       </c>
       <c r="C74" t="s">
-        <v>76</v>
+        <v>75</v>
       </c>
       <c r="D74" t="s">
-        <v>90</v>
+        <v>91</v>
       </c>
       <c r="E74" t="s">
         <v>93</v>
       </c>
       <c r="N74" t="s">
-        <v>149</v>
+        <v>146</v>
       </c>
       <c r="O74" t="s">
-        <v>76</v>
+        <v>75</v>
       </c>
       <c r="P74">
-        <v>100000</v>
+        <v>1000000</v>
       </c>
       <c r="Q74" t="s">
-        <v>165</v>
+        <v>164</v>
       </c>
       <c r="R74" t="s">
-        <v>166</v>
+        <v>167</v>
       </c>
       <c r="S74" t="s">
-        <v>170</v>
+        <v>171</v>
       </c>
       <c r="T74" t="s">
-        <v>171</v>
+        <v>172</v>
       </c>
       <c r="U74" t="s">
-        <v>175</v>
+        <v>176</v>
       </c>
       <c r="V74" s="1">
         <v>46291</v>
@@ -4789,146 +4825,140 @@
     </row>
     <row r="75" spans="1:22">
       <c r="A75">
-        <v>25180</v>
+        <v>24720</v>
       </c>
       <c r="B75" t="s">
         <v>22</v>
       </c>
       <c r="C75" t="s">
-        <v>77</v>
+        <v>76</v>
       </c>
       <c r="D75" t="s">
-        <v>89</v>
+        <v>91</v>
       </c>
       <c r="E75" t="s">
-        <v>92</v>
-      </c>
-      <c r="F75" t="s">
-        <v>94</v>
+        <v>93</v>
       </c>
       <c r="N75" t="s">
-        <v>152</v>
+        <v>150</v>
       </c>
       <c r="O75" t="s">
-        <v>77</v>
+        <v>76</v>
       </c>
       <c r="P75">
-        <v>1000000</v>
+        <v>100000</v>
       </c>
       <c r="Q75" t="s">
-        <v>164</v>
+        <v>166</v>
       </c>
       <c r="R75" t="s">
-        <v>166</v>
+        <v>167</v>
       </c>
       <c r="S75" t="s">
-        <v>169</v>
+        <v>171</v>
       </c>
       <c r="T75" t="s">
         <v>172</v>
       </c>
       <c r="U75" t="s">
-        <v>92</v>
+        <v>176</v>
       </c>
       <c r="V75" s="1">
-        <v>46321</v>
+        <v>46291</v>
       </c>
     </row>
     <row r="76" spans="1:22">
       <c r="A76">
-        <v>25900</v>
+        <v>25180</v>
       </c>
       <c r="B76" t="s">
         <v>22</v>
       </c>
       <c r="C76" t="s">
-        <v>78</v>
+        <v>77</v>
       </c>
       <c r="D76" t="s">
-        <v>87</v>
+        <v>90</v>
       </c>
       <c r="E76" t="s">
         <v>92</v>
       </c>
       <c r="F76" t="s">
-        <v>105</v>
-      </c>
-      <c r="G76" t="s">
-        <v>110</v>
+        <v>94</v>
       </c>
       <c r="N76" t="s">
-        <v>150</v>
+        <v>153</v>
       </c>
       <c r="O76" t="s">
-        <v>78</v>
+        <v>77</v>
       </c>
       <c r="P76">
-        <v>1704503</v>
+        <v>1000000</v>
       </c>
       <c r="Q76" t="s">
-        <v>164</v>
+        <v>165</v>
       </c>
       <c r="R76" t="s">
         <v>167</v>
       </c>
       <c r="S76" t="s">
-        <v>105</v>
+        <v>170</v>
       </c>
       <c r="T76" t="s">
         <v>173</v>
       </c>
       <c r="U76" t="s">
-        <v>175</v>
+        <v>92</v>
       </c>
       <c r="V76" s="1">
-        <v>46381</v>
+        <v>46321</v>
       </c>
     </row>
     <row r="77" spans="1:22">
       <c r="A77">
-        <v>25920</v>
+        <v>25900</v>
       </c>
       <c r="B77" t="s">
         <v>22</v>
       </c>
       <c r="C77" t="s">
-        <v>79</v>
+        <v>78</v>
       </c>
       <c r="D77" t="s">
-        <v>87</v>
+        <v>88</v>
       </c>
       <c r="E77" t="s">
         <v>92</v>
       </c>
       <c r="F77" t="s">
-        <v>105</v>
+        <v>106</v>
       </c>
       <c r="G77" t="s">
-        <v>110</v>
+        <v>111</v>
       </c>
       <c r="N77" t="s">
-        <v>150</v>
+        <v>151</v>
       </c>
       <c r="O77" t="s">
-        <v>79</v>
+        <v>78</v>
       </c>
       <c r="P77">
-        <v>1638125.5</v>
+        <v>1704503</v>
       </c>
       <c r="Q77" t="s">
-        <v>164</v>
+        <v>165</v>
       </c>
       <c r="R77" t="s">
-        <v>167</v>
+        <v>168</v>
       </c>
       <c r="S77" t="s">
-        <v>105</v>
+        <v>106</v>
       </c>
       <c r="T77" t="s">
-        <v>173</v>
+        <v>174</v>
       </c>
       <c r="U77" t="s">
-        <v>175</v>
+        <v>176</v>
       </c>
       <c r="V77" s="1">
         <v>46381</v>
@@ -4936,49 +4966,49 @@
     </row>
     <row r="78" spans="1:22">
       <c r="A78">
-        <v>25940</v>
+        <v>25920</v>
       </c>
       <c r="B78" t="s">
         <v>22</v>
       </c>
       <c r="C78" t="s">
-        <v>80</v>
+        <v>79</v>
       </c>
       <c r="D78" t="s">
-        <v>87</v>
+        <v>88</v>
       </c>
       <c r="E78" t="s">
         <v>92</v>
       </c>
       <c r="F78" t="s">
-        <v>105</v>
+        <v>106</v>
       </c>
       <c r="G78" t="s">
-        <v>110</v>
+        <v>111</v>
       </c>
       <c r="N78" t="s">
-        <v>148</v>
+        <v>151</v>
       </c>
       <c r="O78" t="s">
-        <v>80</v>
+        <v>79</v>
       </c>
       <c r="P78">
-        <v>3800000</v>
+        <v>1638125.5</v>
       </c>
       <c r="Q78" t="s">
-        <v>164</v>
+        <v>165</v>
       </c>
       <c r="R78" t="s">
-        <v>167</v>
+        <v>168</v>
       </c>
       <c r="S78" t="s">
-        <v>105</v>
+        <v>106</v>
       </c>
       <c r="T78" t="s">
-        <v>172</v>
+        <v>174</v>
       </c>
       <c r="U78" t="s">
-        <v>92</v>
+        <v>176</v>
       </c>
       <c r="V78" s="1">
         <v>46381</v>
@@ -4986,46 +5016,46 @@
     </row>
     <row r="79" spans="1:22">
       <c r="A79">
-        <v>25960</v>
+        <v>25940</v>
       </c>
       <c r="B79" t="s">
         <v>22</v>
       </c>
       <c r="C79" t="s">
-        <v>81</v>
+        <v>80</v>
       </c>
       <c r="D79" t="s">
-        <v>87</v>
+        <v>88</v>
       </c>
       <c r="E79" t="s">
         <v>92</v>
       </c>
       <c r="F79" t="s">
-        <v>105</v>
+        <v>106</v>
       </c>
       <c r="G79" t="s">
-        <v>110</v>
+        <v>111</v>
       </c>
       <c r="N79" t="s">
-        <v>148</v>
+        <v>149</v>
       </c>
       <c r="O79" t="s">
-        <v>81</v>
+        <v>80</v>
       </c>
       <c r="P79">
         <v>3800000</v>
       </c>
       <c r="Q79" t="s">
-        <v>164</v>
+        <v>165</v>
       </c>
       <c r="R79" t="s">
-        <v>167</v>
+        <v>168</v>
       </c>
       <c r="S79" t="s">
-        <v>105</v>
+        <v>106</v>
       </c>
       <c r="T79" t="s">
-        <v>172</v>
+        <v>173</v>
       </c>
       <c r="U79" t="s">
         <v>92</v>
@@ -5036,90 +5066,96 @@
     </row>
     <row r="80" spans="1:22">
       <c r="A80">
-        <v>63120</v>
+        <v>25960</v>
       </c>
       <c r="B80" t="s">
         <v>22</v>
       </c>
       <c r="C80" t="s">
-        <v>82</v>
+        <v>81</v>
       </c>
       <c r="D80" t="s">
-        <v>90</v>
+        <v>88</v>
       </c>
       <c r="E80" t="s">
-        <v>93</v>
-      </c>
-      <c r="J80" t="s">
-        <v>138</v>
-      </c>
-      <c r="K80" t="s">
-        <v>143</v>
+        <v>92</v>
+      </c>
+      <c r="F80" t="s">
+        <v>106</v>
+      </c>
+      <c r="G80" t="s">
+        <v>111</v>
       </c>
       <c r="N80" t="s">
-        <v>153</v>
+        <v>149</v>
       </c>
       <c r="O80" t="s">
-        <v>82</v>
+        <v>81</v>
       </c>
       <c r="P80">
         <v>3800000</v>
       </c>
       <c r="Q80" t="s">
-        <v>164</v>
+        <v>165</v>
       </c>
       <c r="R80" t="s">
-        <v>167</v>
+        <v>168</v>
       </c>
       <c r="S80" t="s">
-        <v>170</v>
+        <v>106</v>
       </c>
       <c r="T80" t="s">
-        <v>172</v>
+        <v>173</v>
       </c>
       <c r="U80" t="s">
         <v>92</v>
       </c>
       <c r="V80" s="1">
-        <v>46382</v>
+        <v>46381</v>
       </c>
     </row>
     <row r="81" spans="1:22">
       <c r="A81">
-        <v>63140</v>
+        <v>63120</v>
       </c>
       <c r="B81" t="s">
         <v>22</v>
       </c>
       <c r="C81" t="s">
-        <v>83</v>
+        <v>82</v>
       </c>
       <c r="D81" t="s">
-        <v>89</v>
+        <v>91</v>
       </c>
       <c r="E81" t="s">
-        <v>92</v>
+        <v>93</v>
+      </c>
+      <c r="J81" t="s">
+        <v>139</v>
+      </c>
+      <c r="K81" t="s">
+        <v>144</v>
       </c>
       <c r="N81" t="s">
-        <v>160</v>
+        <v>154</v>
       </c>
       <c r="O81" t="s">
-        <v>83</v>
+        <v>82</v>
       </c>
       <c r="P81">
-        <v>4394700</v>
+        <v>3800000</v>
       </c>
       <c r="Q81" t="s">
-        <v>163</v>
+        <v>165</v>
       </c>
       <c r="R81" t="s">
-        <v>166</v>
+        <v>168</v>
       </c>
       <c r="S81" t="s">
-        <v>170</v>
+        <v>171</v>
       </c>
       <c r="T81" t="s">
-        <v>172</v>
+        <v>173</v>
       </c>
       <c r="U81" t="s">
         <v>92</v>
@@ -5130,40 +5166,28 @@
     </row>
     <row r="82" spans="1:22">
       <c r="A82">
-        <v>63940</v>
+        <v>63140</v>
       </c>
       <c r="B82" t="s">
         <v>22</v>
       </c>
       <c r="C82" t="s">
-        <v>84</v>
+        <v>83</v>
       </c>
       <c r="D82" t="s">
-        <v>87</v>
+        <v>90</v>
       </c>
       <c r="E82" t="s">
         <v>92</v>
       </c>
-      <c r="F82" t="s">
-        <v>94</v>
-      </c>
-      <c r="G82" t="s">
-        <v>106</v>
-      </c>
-      <c r="J82" t="s">
-        <v>130</v>
-      </c>
-      <c r="K82" t="s">
-        <v>139</v>
-      </c>
       <c r="N82" t="s">
-        <v>150</v>
+        <v>161</v>
       </c>
       <c r="O82" t="s">
-        <v>84</v>
+        <v>83</v>
       </c>
       <c r="P82">
-        <v>528395.9300000001</v>
+        <v>4394700</v>
       </c>
       <c r="Q82" t="s">
         <v>164</v>
@@ -5172,13 +5196,13 @@
         <v>167</v>
       </c>
       <c r="S82" t="s">
-        <v>169</v>
+        <v>171</v>
       </c>
       <c r="T82" t="s">
         <v>173</v>
       </c>
       <c r="U82" t="s">
-        <v>175</v>
+        <v>92</v>
       </c>
       <c r="V82" s="1">
         <v>46382</v>
@@ -5186,16 +5210,16 @@
     </row>
     <row r="83" spans="1:22">
       <c r="A83">
-        <v>63960</v>
+        <v>63940</v>
       </c>
       <c r="B83" t="s">
         <v>22</v>
       </c>
       <c r="C83" t="s">
-        <v>85</v>
+        <v>84</v>
       </c>
       <c r="D83" t="s">
-        <v>87</v>
+        <v>88</v>
       </c>
       <c r="E83" t="s">
         <v>92</v>
@@ -5204,83 +5228,95 @@
         <v>94</v>
       </c>
       <c r="G83" t="s">
-        <v>106</v>
+        <v>110</v>
+      </c>
+      <c r="J83" t="s">
+        <v>131</v>
+      </c>
+      <c r="K83" t="s">
+        <v>140</v>
       </c>
       <c r="N83" t="s">
-        <v>152</v>
+        <v>151</v>
       </c>
       <c r="O83" t="s">
-        <v>85</v>
+        <v>84</v>
       </c>
       <c r="P83">
-        <v>1000000</v>
+        <v>528395.9300000001</v>
       </c>
       <c r="Q83" t="s">
-        <v>164</v>
+        <v>165</v>
       </c>
       <c r="R83" t="s">
-        <v>166</v>
+        <v>168</v>
       </c>
       <c r="S83" t="s">
-        <v>169</v>
+        <v>170</v>
       </c>
       <c r="T83" t="s">
-        <v>172</v>
+        <v>174</v>
       </c>
       <c r="U83" t="s">
-        <v>92</v>
+        <v>176</v>
       </c>
       <c r="V83" s="1">
-        <v>46321</v>
+        <v>46382</v>
       </c>
     </row>
     <row r="84" spans="1:22">
       <c r="A84">
-        <v>64340</v>
+        <v>63960</v>
       </c>
       <c r="B84" t="s">
         <v>22</v>
       </c>
       <c r="C84" t="s">
-        <v>83</v>
+        <v>85</v>
       </c>
       <c r="D84" t="s">
-        <v>89</v>
+        <v>88</v>
       </c>
       <c r="E84" t="s">
         <v>92</v>
       </c>
+      <c r="F84" t="s">
+        <v>94</v>
+      </c>
+      <c r="G84" t="s">
+        <v>110</v>
+      </c>
       <c r="N84" t="s">
-        <v>160</v>
+        <v>153</v>
       </c>
       <c r="O84" t="s">
-        <v>83</v>
+        <v>85</v>
       </c>
       <c r="P84">
-        <v>4394700</v>
+        <v>1000000</v>
       </c>
       <c r="Q84" t="s">
-        <v>163</v>
+        <v>165</v>
       </c>
       <c r="R84" t="s">
-        <v>166</v>
+        <v>167</v>
       </c>
       <c r="S84" t="s">
         <v>170</v>
       </c>
       <c r="T84" t="s">
-        <v>172</v>
+        <v>173</v>
       </c>
       <c r="U84" t="s">
         <v>92</v>
       </c>
       <c r="V84" s="1">
-        <v>46382</v>
+        <v>46321</v>
       </c>
     </row>
     <row r="85" spans="1:22">
       <c r="A85">
-        <v>64760</v>
+        <v>64340</v>
       </c>
       <c r="B85" t="s">
         <v>22</v>
@@ -5289,45 +5325,42 @@
         <v>83</v>
       </c>
       <c r="D85" t="s">
-        <v>87</v>
+        <v>90</v>
       </c>
       <c r="E85" t="s">
         <v>92</v>
       </c>
-      <c r="F85" t="s">
-        <v>105</v>
-      </c>
-      <c r="G85" t="s">
-        <v>110</v>
-      </c>
       <c r="N85" t="s">
-        <v>83</v>
+        <v>161</v>
       </c>
       <c r="O85" t="s">
         <v>83</v>
       </c>
       <c r="P85">
-        <v>3306000</v>
+        <v>4394700</v>
       </c>
       <c r="Q85" t="s">
-        <v>163</v>
+        <v>164</v>
       </c>
       <c r="R85" t="s">
-        <v>166</v>
+        <v>167</v>
       </c>
       <c r="S85" t="s">
-        <v>105</v>
+        <v>171</v>
       </c>
       <c r="T85" t="s">
-        <v>172</v>
+        <v>173</v>
       </c>
       <c r="U85" t="s">
         <v>92</v>
+      </c>
+      <c r="V85" s="1">
+        <v>46382</v>
       </c>
     </row>
     <row r="86" spans="1:22">
       <c r="A86">
-        <v>64780</v>
+        <v>64760</v>
       </c>
       <c r="B86" t="s">
         <v>22</v>
@@ -5336,16 +5369,16 @@
         <v>83</v>
       </c>
       <c r="D86" t="s">
-        <v>87</v>
+        <v>88</v>
       </c>
       <c r="E86" t="s">
         <v>92</v>
       </c>
       <c r="F86" t="s">
-        <v>105</v>
+        <v>106</v>
       </c>
       <c r="G86" t="s">
-        <v>110</v>
+        <v>111</v>
       </c>
       <c r="N86" t="s">
         <v>83</v>
@@ -5357,16 +5390,16 @@
         <v>3306000</v>
       </c>
       <c r="Q86" t="s">
-        <v>163</v>
+        <v>164</v>
       </c>
       <c r="R86" t="s">
-        <v>166</v>
+        <v>167</v>
       </c>
       <c r="S86" t="s">
-        <v>105</v>
+        <v>106</v>
       </c>
       <c r="T86" t="s">
-        <v>172</v>
+        <v>173</v>
       </c>
       <c r="U86" t="s">
         <v>92</v>
@@ -5374,63 +5407,60 @@
     </row>
     <row r="87" spans="1:22">
       <c r="A87">
-        <v>64840</v>
+        <v>64780</v>
       </c>
       <c r="B87" t="s">
         <v>22</v>
       </c>
       <c r="C87" t="s">
-        <v>86</v>
+        <v>83</v>
       </c>
       <c r="D87" t="s">
-        <v>87</v>
+        <v>88</v>
       </c>
       <c r="E87" t="s">
         <v>92</v>
       </c>
       <c r="F87" t="s">
-        <v>94</v>
+        <v>106</v>
       </c>
       <c r="G87" t="s">
+        <v>111</v>
+      </c>
+      <c r="N87" t="s">
+        <v>83</v>
+      </c>
+      <c r="O87" t="s">
+        <v>83</v>
+      </c>
+      <c r="P87">
+        <v>3306000</v>
+      </c>
+      <c r="Q87" t="s">
+        <v>164</v>
+      </c>
+      <c r="R87" t="s">
+        <v>167</v>
+      </c>
+      <c r="S87" t="s">
         <v>106</v>
       </c>
-      <c r="I87" t="s">
-        <v>111</v>
-      </c>
-      <c r="N87" t="s">
-        <v>161</v>
-      </c>
-      <c r="O87" t="s">
-        <v>86</v>
-      </c>
-      <c r="P87">
-        <v>470820</v>
-      </c>
-      <c r="Q87" t="s">
-        <v>163</v>
-      </c>
-      <c r="R87" t="s">
-        <v>166</v>
-      </c>
-      <c r="S87" t="s">
-        <v>169</v>
-      </c>
       <c r="T87" t="s">
-        <v>174</v>
+        <v>173</v>
       </c>
       <c r="U87" t="s">
         <v>92</v>
-      </c>
-      <c r="V87" s="1">
-        <v>46291</v>
       </c>
     </row>
     <row r="88" spans="1:22">
       <c r="A88">
-        <v>68160</v>
+        <v>64840</v>
       </c>
       <c r="B88" t="s">
         <v>22</v>
+      </c>
+      <c r="C88" t="s">
+        <v>86</v>
       </c>
       <c r="D88" t="s">
         <v>87</v>
@@ -5442,33 +5472,86 @@
         <v>94</v>
       </c>
       <c r="G88" t="s">
-        <v>106</v>
+        <v>107</v>
+      </c>
+      <c r="H88" s="1">
+        <v>46303</v>
+      </c>
+      <c r="I88" t="s">
+        <v>112</v>
       </c>
       <c r="N88" t="s">
-        <v>153</v>
+        <v>162</v>
       </c>
       <c r="O88" t="s">
-        <v>162</v>
+        <v>86</v>
       </c>
       <c r="P88">
-        <v>2297180</v>
+        <v>470820</v>
       </c>
       <c r="Q88" t="s">
         <v>164</v>
       </c>
       <c r="R88" t="s">
-        <v>166</v>
+        <v>167</v>
       </c>
       <c r="S88" t="s">
-        <v>169</v>
+        <v>170</v>
       </c>
       <c r="T88" t="s">
-        <v>172</v>
+        <v>175</v>
       </c>
       <c r="U88" t="s">
         <v>92</v>
       </c>
       <c r="V88" s="1">
+        <v>46291</v>
+      </c>
+    </row>
+    <row r="89" spans="1:22">
+      <c r="A89">
+        <v>68160</v>
+      </c>
+      <c r="B89" t="s">
+        <v>22</v>
+      </c>
+      <c r="D89" t="s">
+        <v>88</v>
+      </c>
+      <c r="E89" t="s">
+        <v>92</v>
+      </c>
+      <c r="F89" t="s">
+        <v>94</v>
+      </c>
+      <c r="G89" t="s">
+        <v>110</v>
+      </c>
+      <c r="N89" t="s">
+        <v>154</v>
+      </c>
+      <c r="O89" t="s">
+        <v>163</v>
+      </c>
+      <c r="P89">
+        <v>2297180</v>
+      </c>
+      <c r="Q89" t="s">
+        <v>165</v>
+      </c>
+      <c r="R89" t="s">
+        <v>167</v>
+      </c>
+      <c r="S89" t="s">
+        <v>170</v>
+      </c>
+      <c r="T89" t="s">
+        <v>173</v>
+      </c>
+      <c r="U89" t="s">
+        <v>92</v>
+      </c>
+      <c r="V89" s="1">
         <v>46291</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Atualização automática: mta (13/10/2026 10:14)
</commit_message>
<xml_diff>
--- a/Projetos/02_Dados_Tratados/base_mta_tratada.xlsx
+++ b/Projetos/02_Dados_Tratados/base_mta_tratada.xlsx
@@ -554,8 +554,16 @@
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="YYYY-MM-DD HH:MM:SS"/>
   </numFmts>
-  <fonts count="1">
+  <fonts count="2">
     <font>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
       <sz val="11"/>
       <color theme="1"/>
       <name val="Calibri"/>
@@ -571,7 +579,7 @@
       <patternFill patternType="gray125"/>
     </fill>
   </fills>
-  <borders count="1">
+  <borders count="2">
     <border>
       <left/>
       <right/>
@@ -579,12 +587,30 @@
       <bottom/>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin">
+        <color auto="1"/>
+      </left>
+      <right style="thin">
+        <color auto="1"/>
+      </right>
+      <top style="thin">
+        <color auto="1"/>
+      </top>
+      <bottom style="thin">
+        <color auto="1"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="3">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
   </cellXfs>
   <cellStyles count="1">
@@ -884,70 +910,70 @@
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:22">
-      <c r="A1" t="s">
+      <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
-      <c r="B1" t="s">
+      <c r="B1" s="1" t="s">
         <v>1</v>
       </c>
-      <c r="C1" t="s">
+      <c r="C1" s="1" t="s">
         <v>2</v>
       </c>
-      <c r="D1" t="s">
+      <c r="D1" s="1" t="s">
         <v>3</v>
       </c>
-      <c r="E1" t="s">
+      <c r="E1" s="1" t="s">
         <v>4</v>
       </c>
-      <c r="F1" t="s">
+      <c r="F1" s="1" t="s">
         <v>5</v>
       </c>
-      <c r="G1" t="s">
+      <c r="G1" s="1" t="s">
         <v>6</v>
       </c>
-      <c r="H1" t="s">
+      <c r="H1" s="1" t="s">
         <v>7</v>
       </c>
-      <c r="I1" t="s">
+      <c r="I1" s="1" t="s">
         <v>8</v>
       </c>
-      <c r="J1" t="s">
+      <c r="J1" s="1" t="s">
         <v>9</v>
       </c>
-      <c r="K1" t="s">
+      <c r="K1" s="1" t="s">
         <v>10</v>
       </c>
-      <c r="L1" t="s">
+      <c r="L1" s="1" t="s">
         <v>11</v>
       </c>
-      <c r="M1" t="s">
+      <c r="M1" s="1" t="s">
         <v>12</v>
       </c>
-      <c r="N1" t="s">
+      <c r="N1" s="1" t="s">
         <v>13</v>
       </c>
-      <c r="O1" t="s">
+      <c r="O1" s="1" t="s">
         <v>14</v>
       </c>
-      <c r="P1" t="s">
+      <c r="P1" s="1" t="s">
         <v>15</v>
       </c>
-      <c r="Q1" t="s">
+      <c r="Q1" s="1" t="s">
         <v>16</v>
       </c>
-      <c r="R1" t="s">
+      <c r="R1" s="1" t="s">
         <v>17</v>
       </c>
-      <c r="S1" t="s">
+      <c r="S1" s="1" t="s">
         <v>18</v>
       </c>
-      <c r="T1" t="s">
+      <c r="T1" s="1" t="s">
         <v>19</v>
       </c>
-      <c r="U1" t="s">
+      <c r="U1" s="1" t="s">
         <v>20</v>
       </c>
-      <c r="V1" t="s">
+      <c r="V1" s="1" t="s">
         <v>21</v>
       </c>
     </row>
@@ -973,7 +999,7 @@
       <c r="G2" t="s">
         <v>107</v>
       </c>
-      <c r="H2" s="1">
+      <c r="H2" s="2">
         <v>46303</v>
       </c>
       <c r="I2" t="s">
@@ -1012,7 +1038,7 @@
       <c r="U2" t="s">
         <v>176</v>
       </c>
-      <c r="V2" s="1">
+      <c r="V2" s="2">
         <v>46229</v>
       </c>
     </row>
@@ -1059,7 +1085,7 @@
       <c r="U3" t="s">
         <v>92</v>
       </c>
-      <c r="V3" s="1">
+      <c r="V3" s="2">
         <v>46291</v>
       </c>
     </row>
@@ -1106,7 +1132,7 @@
       <c r="U4" t="s">
         <v>92</v>
       </c>
-      <c r="V4" s="1">
+      <c r="V4" s="2">
         <v>46321</v>
       </c>
     </row>
@@ -1153,7 +1179,7 @@
       <c r="U5" t="s">
         <v>92</v>
       </c>
-      <c r="V5" s="1">
+      <c r="V5" s="2">
         <v>46321</v>
       </c>
     </row>
@@ -1203,7 +1229,7 @@
       <c r="U6" t="s">
         <v>92</v>
       </c>
-      <c r="V6" s="1">
+      <c r="V6" s="2">
         <v>46291</v>
       </c>
     </row>
@@ -1229,7 +1255,7 @@
       <c r="G7" t="s">
         <v>109</v>
       </c>
-      <c r="H7" s="1">
+      <c r="H7" s="2">
         <v>46121</v>
       </c>
       <c r="I7" t="s">
@@ -1259,7 +1285,7 @@
       <c r="U7" t="s">
         <v>92</v>
       </c>
-      <c r="V7" s="1">
+      <c r="V7" s="2">
         <v>46138</v>
       </c>
     </row>
@@ -1306,7 +1332,7 @@
       <c r="U8" t="s">
         <v>92</v>
       </c>
-      <c r="V8" s="1">
+      <c r="V8" s="2">
         <v>46291</v>
       </c>
     </row>
@@ -1353,7 +1379,7 @@
       <c r="U9" t="s">
         <v>92</v>
       </c>
-      <c r="V9" s="1">
+      <c r="V9" s="2">
         <v>46291</v>
       </c>
     </row>
@@ -1376,7 +1402,7 @@
       <c r="G10" t="s">
         <v>107</v>
       </c>
-      <c r="H10" s="1">
+      <c r="H10" s="2">
         <v>46303</v>
       </c>
       <c r="I10" t="s">
@@ -1406,7 +1432,7 @@
       <c r="U10" t="s">
         <v>92</v>
       </c>
-      <c r="V10" s="1">
+      <c r="V10" s="2">
         <v>46291</v>
       </c>
     </row>
@@ -1453,7 +1479,7 @@
       <c r="U11" t="s">
         <v>92</v>
       </c>
-      <c r="V11" s="1">
+      <c r="V11" s="2">
         <v>46291</v>
       </c>
     </row>
@@ -1500,7 +1526,7 @@
       <c r="U12" t="s">
         <v>92</v>
       </c>
-      <c r="V12" s="1">
+      <c r="V12" s="2">
         <v>46291</v>
       </c>
     </row>
@@ -1526,7 +1552,7 @@
       <c r="G13" t="s">
         <v>109</v>
       </c>
-      <c r="H13" s="1">
+      <c r="H13" s="2">
         <v>46079</v>
       </c>
       <c r="I13" t="s">
@@ -1559,7 +1585,7 @@
       <c r="U13" t="s">
         <v>176</v>
       </c>
-      <c r="V13" s="1">
+      <c r="V13" s="2">
         <v>46079</v>
       </c>
     </row>
@@ -1585,7 +1611,7 @@
       <c r="G14" t="s">
         <v>107</v>
       </c>
-      <c r="H14" s="1">
+      <c r="H14" s="2">
         <v>46303</v>
       </c>
       <c r="I14" t="s">
@@ -1621,7 +1647,7 @@
       <c r="U14" t="s">
         <v>176</v>
       </c>
-      <c r="V14" s="1">
+      <c r="V14" s="2">
         <v>46352</v>
       </c>
     </row>
@@ -1647,7 +1673,7 @@
       <c r="G15" t="s">
         <v>107</v>
       </c>
-      <c r="H15" s="1">
+      <c r="H15" s="2">
         <v>46303</v>
       </c>
       <c r="I15" t="s">
@@ -1683,7 +1709,7 @@
       <c r="U15" t="s">
         <v>176</v>
       </c>
-      <c r="V15" s="1">
+      <c r="V15" s="2">
         <v>46352</v>
       </c>
     </row>
@@ -1709,7 +1735,7 @@
       <c r="G16" t="s">
         <v>107</v>
       </c>
-      <c r="H16" s="1">
+      <c r="H16" s="2">
         <v>46303</v>
       </c>
       <c r="I16" t="s">
@@ -1745,7 +1771,7 @@
       <c r="U16" t="s">
         <v>176</v>
       </c>
-      <c r="V16" s="1">
+      <c r="V16" s="2">
         <v>46352</v>
       </c>
     </row>
@@ -1771,7 +1797,7 @@
       <c r="G17" t="s">
         <v>107</v>
       </c>
-      <c r="H17" s="1">
+      <c r="H17" s="2">
         <v>46303</v>
       </c>
       <c r="I17" t="s">
@@ -1807,7 +1833,7 @@
       <c r="U17" t="s">
         <v>176</v>
       </c>
-      <c r="V17" s="1">
+      <c r="V17" s="2">
         <v>46229</v>
       </c>
     </row>
@@ -1833,7 +1859,7 @@
       <c r="G18" t="s">
         <v>109</v>
       </c>
-      <c r="H18" s="1">
+      <c r="H18" s="2">
         <v>46098</v>
       </c>
       <c r="I18" t="s">
@@ -1866,7 +1892,7 @@
       <c r="U18" t="s">
         <v>176</v>
       </c>
-      <c r="V18" s="1">
+      <c r="V18" s="2">
         <v>46107</v>
       </c>
     </row>
@@ -1892,7 +1918,7 @@
       <c r="G19" t="s">
         <v>109</v>
       </c>
-      <c r="H19" s="1">
+      <c r="H19" s="2">
         <v>46076</v>
       </c>
       <c r="I19" t="s">
@@ -1922,7 +1948,7 @@
       <c r="U19" t="s">
         <v>92</v>
       </c>
-      <c r="V19" s="1">
+      <c r="V19" s="2">
         <v>46079</v>
       </c>
     </row>
@@ -1948,7 +1974,7 @@
       <c r="G20" t="s">
         <v>109</v>
       </c>
-      <c r="H20" s="1">
+      <c r="H20" s="2">
         <v>46076</v>
       </c>
       <c r="I20" t="s">
@@ -1978,7 +2004,7 @@
       <c r="U20" t="s">
         <v>92</v>
       </c>
-      <c r="V20" s="1">
+      <c r="V20" s="2">
         <v>46079</v>
       </c>
     </row>
@@ -2025,7 +2051,7 @@
       <c r="U21" t="s">
         <v>92</v>
       </c>
-      <c r="V21" s="1">
+      <c r="V21" s="2">
         <v>46321</v>
       </c>
     </row>
@@ -2072,7 +2098,7 @@
       <c r="U22" t="s">
         <v>92</v>
       </c>
-      <c r="V22" s="1">
+      <c r="V22" s="2">
         <v>46321</v>
       </c>
     </row>
@@ -2119,7 +2145,7 @@
       <c r="U23" t="s">
         <v>92</v>
       </c>
-      <c r="V23" s="1">
+      <c r="V23" s="2">
         <v>46321</v>
       </c>
     </row>
@@ -2166,7 +2192,7 @@
       <c r="U24" t="s">
         <v>92</v>
       </c>
-      <c r="V24" s="1">
+      <c r="V24" s="2">
         <v>46321</v>
       </c>
     </row>
@@ -2192,7 +2218,7 @@
       <c r="G25" t="s">
         <v>109</v>
       </c>
-      <c r="H25" s="1">
+      <c r="H25" s="2">
         <v>46119</v>
       </c>
       <c r="I25" t="s">
@@ -2225,7 +2251,7 @@
       <c r="U25" t="s">
         <v>176</v>
       </c>
-      <c r="V25" s="1">
+      <c r="V25" s="2">
         <v>46138</v>
       </c>
     </row>
@@ -2251,7 +2277,7 @@
       <c r="G26" t="s">
         <v>109</v>
       </c>
-      <c r="H26" s="1">
+      <c r="H26" s="2">
         <v>46121</v>
       </c>
       <c r="I26" t="s">
@@ -2281,7 +2307,7 @@
       <c r="U26" t="s">
         <v>92</v>
       </c>
-      <c r="V26" s="1">
+      <c r="V26" s="2">
         <v>46138</v>
       </c>
     </row>
@@ -2307,7 +2333,7 @@
       <c r="G27" t="s">
         <v>109</v>
       </c>
-      <c r="H27" s="1">
+      <c r="H27" s="2">
         <v>46076</v>
       </c>
       <c r="I27" t="s">
@@ -2337,7 +2363,7 @@
       <c r="U27" t="s">
         <v>92</v>
       </c>
-      <c r="V27" s="1">
+      <c r="V27" s="2">
         <v>46079</v>
       </c>
     </row>
@@ -2363,7 +2389,7 @@
       <c r="G28" t="s">
         <v>107</v>
       </c>
-      <c r="H28" s="1">
+      <c r="H28" s="2">
         <v>46303</v>
       </c>
       <c r="I28" t="s">
@@ -2399,7 +2425,7 @@
       <c r="U28" t="s">
         <v>176</v>
       </c>
-      <c r="V28" s="1">
+      <c r="V28" s="2">
         <v>46291</v>
       </c>
     </row>
@@ -2425,7 +2451,7 @@
       <c r="G29" t="s">
         <v>109</v>
       </c>
-      <c r="H29" s="1">
+      <c r="H29" s="2">
         <v>46199</v>
       </c>
       <c r="I29" t="s">
@@ -2458,7 +2484,7 @@
       <c r="U29" t="s">
         <v>176</v>
       </c>
-      <c r="V29" s="1">
+      <c r="V29" s="2">
         <v>46199</v>
       </c>
     </row>
@@ -2484,7 +2510,7 @@
       <c r="G30" t="s">
         <v>109</v>
       </c>
-      <c r="H30" s="1">
+      <c r="H30" s="2">
         <v>46199</v>
       </c>
       <c r="I30" t="s">
@@ -2517,7 +2543,7 @@
       <c r="U30" t="s">
         <v>176</v>
       </c>
-      <c r="V30" s="1">
+      <c r="V30" s="2">
         <v>46199</v>
       </c>
     </row>
@@ -2543,7 +2569,7 @@
       <c r="G31" t="s">
         <v>109</v>
       </c>
-      <c r="H31" s="1">
+      <c r="H31" s="2">
         <v>46199</v>
       </c>
       <c r="I31" t="s">
@@ -2576,7 +2602,7 @@
       <c r="U31" t="s">
         <v>176</v>
       </c>
-      <c r="V31" s="1">
+      <c r="V31" s="2">
         <v>46199</v>
       </c>
     </row>
@@ -2602,7 +2628,7 @@
       <c r="G32" t="s">
         <v>109</v>
       </c>
-      <c r="H32" s="1">
+      <c r="H32" s="2">
         <v>46199</v>
       </c>
       <c r="I32" t="s">
@@ -2635,7 +2661,7 @@
       <c r="U32" t="s">
         <v>176</v>
       </c>
-      <c r="V32" s="1">
+      <c r="V32" s="2">
         <v>46199</v>
       </c>
     </row>
@@ -2688,7 +2714,7 @@
       <c r="U33" t="s">
         <v>176</v>
       </c>
-      <c r="V33" s="1">
+      <c r="V33" s="2">
         <v>46291</v>
       </c>
     </row>
@@ -2714,7 +2740,7 @@
       <c r="G34" t="s">
         <v>109</v>
       </c>
-      <c r="H34" s="1">
+      <c r="H34" s="2">
         <v>46191</v>
       </c>
       <c r="I34" t="s">
@@ -2747,7 +2773,7 @@
       <c r="U34" t="s">
         <v>176</v>
       </c>
-      <c r="V34" s="1">
+      <c r="V34" s="2">
         <v>46199</v>
       </c>
     </row>
@@ -2773,7 +2799,7 @@
       <c r="G35" t="s">
         <v>109</v>
       </c>
-      <c r="H35" s="1">
+      <c r="H35" s="2">
         <v>46119</v>
       </c>
       <c r="I35" t="s">
@@ -2803,7 +2829,7 @@
       <c r="U35" t="s">
         <v>176</v>
       </c>
-      <c r="V35" s="1">
+      <c r="V35" s="2">
         <v>46138</v>
       </c>
     </row>
@@ -2829,7 +2855,7 @@
       <c r="G36" t="s">
         <v>109</v>
       </c>
-      <c r="H36" s="1">
+      <c r="H36" s="2">
         <v>46213</v>
       </c>
       <c r="I36" t="s">
@@ -2859,7 +2885,7 @@
       <c r="U36" t="s">
         <v>92</v>
       </c>
-      <c r="V36" s="1">
+      <c r="V36" s="2">
         <v>46229</v>
       </c>
     </row>
@@ -2885,7 +2911,7 @@
       <c r="G37" t="s">
         <v>109</v>
       </c>
-      <c r="H37" s="1">
+      <c r="H37" s="2">
         <v>46175</v>
       </c>
       <c r="I37" t="s">
@@ -2915,7 +2941,7 @@
       <c r="U37" t="s">
         <v>92</v>
       </c>
-      <c r="V37" s="1">
+      <c r="V37" s="2">
         <v>46199</v>
       </c>
     </row>
@@ -2941,7 +2967,7 @@
       <c r="G38" t="s">
         <v>109</v>
       </c>
-      <c r="H38" s="1">
+      <c r="H38" s="2">
         <v>46213</v>
       </c>
       <c r="I38" t="s">
@@ -2971,7 +2997,7 @@
       <c r="U38" t="s">
         <v>92</v>
       </c>
-      <c r="V38" s="1">
+      <c r="V38" s="2">
         <v>46229</v>
       </c>
     </row>
@@ -2997,7 +3023,7 @@
       <c r="G39" t="s">
         <v>109</v>
       </c>
-      <c r="H39" s="1">
+      <c r="H39" s="2">
         <v>46199</v>
       </c>
       <c r="I39" t="s">
@@ -3027,7 +3053,7 @@
       <c r="U39" t="s">
         <v>92</v>
       </c>
-      <c r="V39" s="1">
+      <c r="V39" s="2">
         <v>46199</v>
       </c>
     </row>
@@ -3053,7 +3079,7 @@
       <c r="G40" t="s">
         <v>109</v>
       </c>
-      <c r="H40" s="1">
+      <c r="H40" s="2">
         <v>46199</v>
       </c>
       <c r="I40" t="s">
@@ -3083,7 +3109,7 @@
       <c r="U40" t="s">
         <v>92</v>
       </c>
-      <c r="V40" s="1">
+      <c r="V40" s="2">
         <v>46199</v>
       </c>
     </row>
@@ -3109,7 +3135,7 @@
       <c r="G41" t="s">
         <v>109</v>
       </c>
-      <c r="H41" s="1">
+      <c r="H41" s="2">
         <v>46204</v>
       </c>
       <c r="I41" t="s">
@@ -3139,7 +3165,7 @@
       <c r="U41" t="s">
         <v>92</v>
       </c>
-      <c r="V41" s="1">
+      <c r="V41" s="2">
         <v>46229</v>
       </c>
     </row>
@@ -3165,7 +3191,7 @@
       <c r="G42" t="s">
         <v>109</v>
       </c>
-      <c r="H42" s="1">
+      <c r="H42" s="2">
         <v>46244</v>
       </c>
       <c r="I42" t="s">
@@ -3195,7 +3221,7 @@
       <c r="U42" t="s">
         <v>92</v>
       </c>
-      <c r="V42" s="1">
+      <c r="V42" s="2">
         <v>46199</v>
       </c>
     </row>
@@ -3239,7 +3265,7 @@
       <c r="U43" t="s">
         <v>92</v>
       </c>
-      <c r="V43" s="1">
+      <c r="V43" s="2">
         <v>46260</v>
       </c>
     </row>
@@ -3265,7 +3291,7 @@
       <c r="G44" t="s">
         <v>109</v>
       </c>
-      <c r="H44" s="1">
+      <c r="H44" s="2">
         <v>46191</v>
       </c>
       <c r="I44" t="s">
@@ -3295,7 +3321,7 @@
       <c r="U44" t="s">
         <v>92</v>
       </c>
-      <c r="V44" s="1">
+      <c r="V44" s="2">
         <v>46199</v>
       </c>
     </row>
@@ -3321,7 +3347,7 @@
       <c r="G45" t="s">
         <v>109</v>
       </c>
-      <c r="H45" s="1">
+      <c r="H45" s="2">
         <v>46191</v>
       </c>
       <c r="I45" t="s">
@@ -3351,7 +3377,7 @@
       <c r="U45" t="s">
         <v>92</v>
       </c>
-      <c r="V45" s="1">
+      <c r="V45" s="2">
         <v>46199</v>
       </c>
     </row>
@@ -3377,7 +3403,7 @@
       <c r="G46" t="s">
         <v>109</v>
       </c>
-      <c r="H46" s="1">
+      <c r="H46" s="2">
         <v>46213</v>
       </c>
       <c r="I46" t="s">
@@ -3410,7 +3436,7 @@
       <c r="U46" t="s">
         <v>176</v>
       </c>
-      <c r="V46" s="1">
+      <c r="V46" s="2">
         <v>46229</v>
       </c>
     </row>
@@ -3436,7 +3462,7 @@
       <c r="G47" t="s">
         <v>109</v>
       </c>
-      <c r="H47" s="1">
+      <c r="H47" s="2">
         <v>46210</v>
       </c>
       <c r="I47" t="s">
@@ -3466,7 +3492,7 @@
       <c r="U47" t="s">
         <v>176</v>
       </c>
-      <c r="V47" s="1">
+      <c r="V47" s="2">
         <v>46229</v>
       </c>
     </row>
@@ -3513,7 +3539,7 @@
       <c r="U48" t="s">
         <v>92</v>
       </c>
-      <c r="V48" s="1">
+      <c r="V48" s="2">
         <v>46321</v>
       </c>
     </row>
@@ -3539,7 +3565,7 @@
       <c r="G49" t="s">
         <v>107</v>
       </c>
-      <c r="H49" s="1">
+      <c r="H49" s="2">
         <v>46303</v>
       </c>
       <c r="I49" t="s">
@@ -3575,7 +3601,7 @@
       <c r="U49" t="s">
         <v>176</v>
       </c>
-      <c r="V49" s="1">
+      <c r="V49" s="2">
         <v>46291</v>
       </c>
     </row>
@@ -3601,7 +3627,7 @@
       <c r="G50" t="s">
         <v>109</v>
       </c>
-      <c r="H50" s="1">
+      <c r="H50" s="2">
         <v>46176</v>
       </c>
       <c r="I50" t="s">
@@ -3634,7 +3660,7 @@
       <c r="U50" t="s">
         <v>176</v>
       </c>
-      <c r="V50" s="1">
+      <c r="V50" s="2">
         <v>46199</v>
       </c>
     </row>
@@ -3690,7 +3716,7 @@
       <c r="U51" t="s">
         <v>176</v>
       </c>
-      <c r="V51" s="1">
+      <c r="V51" s="2">
         <v>46260</v>
       </c>
     </row>
@@ -3716,7 +3742,7 @@
       <c r="G52" t="s">
         <v>109</v>
       </c>
-      <c r="H52" s="1">
+      <c r="H52" s="2">
         <v>46295</v>
       </c>
       <c r="I52" t="s">
@@ -3752,7 +3778,7 @@
       <c r="U52" t="s">
         <v>176</v>
       </c>
-      <c r="V52" s="1">
+      <c r="V52" s="2">
         <v>46291</v>
       </c>
     </row>
@@ -3805,7 +3831,7 @@
       <c r="U53" t="s">
         <v>176</v>
       </c>
-      <c r="V53" s="1">
+      <c r="V53" s="2">
         <v>46321</v>
       </c>
     </row>
@@ -3831,7 +3857,7 @@
       <c r="G54" t="s">
         <v>109</v>
       </c>
-      <c r="H54" s="1">
+      <c r="H54" s="2">
         <v>46227</v>
       </c>
       <c r="I54" t="s">
@@ -3861,7 +3887,7 @@
       <c r="U54" t="s">
         <v>176</v>
       </c>
-      <c r="V54" s="1">
+      <c r="V54" s="2">
         <v>46229</v>
       </c>
     </row>
@@ -3884,7 +3910,7 @@
       <c r="G55" t="s">
         <v>109</v>
       </c>
-      <c r="H55" s="1">
+      <c r="H55" s="2">
         <v>46280</v>
       </c>
       <c r="I55" t="s">
@@ -3914,7 +3940,7 @@
       <c r="U55" t="s">
         <v>176</v>
       </c>
-      <c r="V55" s="1">
+      <c r="V55" s="2">
         <v>46291</v>
       </c>
     </row>
@@ -3937,7 +3963,7 @@
       <c r="G56" t="s">
         <v>109</v>
       </c>
-      <c r="H56" s="1">
+      <c r="H56" s="2">
         <v>46280</v>
       </c>
       <c r="I56" t="s">
@@ -3967,7 +3993,7 @@
       <c r="U56" t="s">
         <v>176</v>
       </c>
-      <c r="V56" s="1">
+      <c r="V56" s="2">
         <v>46260</v>
       </c>
     </row>
@@ -3990,7 +4016,7 @@
       <c r="G57" t="s">
         <v>109</v>
       </c>
-      <c r="H57" s="1">
+      <c r="H57" s="2">
         <v>46295</v>
       </c>
       <c r="I57" t="s">
@@ -4020,7 +4046,7 @@
       <c r="U57" t="s">
         <v>176</v>
       </c>
-      <c r="V57" s="1">
+      <c r="V57" s="2">
         <v>46291</v>
       </c>
     </row>
@@ -4043,7 +4069,7 @@
       <c r="G58" t="s">
         <v>109</v>
       </c>
-      <c r="H58" s="1">
+      <c r="H58" s="2">
         <v>46295</v>
       </c>
       <c r="I58" t="s">
@@ -4073,7 +4099,7 @@
       <c r="U58" t="s">
         <v>176</v>
       </c>
-      <c r="V58" s="1">
+      <c r="V58" s="2">
         <v>46291</v>
       </c>
     </row>
@@ -4120,7 +4146,7 @@
       <c r="U59" t="s">
         <v>176</v>
       </c>
-      <c r="V59" s="1">
+      <c r="V59" s="2">
         <v>46321</v>
       </c>
     </row>
@@ -4146,7 +4172,7 @@
       <c r="G60" t="s">
         <v>109</v>
       </c>
-      <c r="H60" s="1">
+      <c r="H60" s="2">
         <v>46301</v>
       </c>
       <c r="I60" t="s">
@@ -4182,7 +4208,7 @@
       <c r="U60" t="s">
         <v>176</v>
       </c>
-      <c r="V60" s="1">
+      <c r="V60" s="2">
         <v>46352</v>
       </c>
     </row>
@@ -4226,7 +4252,7 @@
       <c r="U61" t="s">
         <v>176</v>
       </c>
-      <c r="V61" s="1">
+      <c r="V61" s="2">
         <v>46107</v>
       </c>
     </row>
@@ -4270,7 +4296,7 @@
       <c r="U62" t="s">
         <v>176</v>
       </c>
-      <c r="V62" s="1">
+      <c r="V62" s="2">
         <v>46107</v>
       </c>
     </row>
@@ -4314,7 +4340,7 @@
       <c r="U63" t="s">
         <v>176</v>
       </c>
-      <c r="V63" s="1">
+      <c r="V63" s="2">
         <v>46107</v>
       </c>
     </row>
@@ -4358,7 +4384,7 @@
       <c r="U64" t="s">
         <v>176</v>
       </c>
-      <c r="V64" s="1">
+      <c r="V64" s="2">
         <v>46107</v>
       </c>
     </row>
@@ -4402,7 +4428,7 @@
       <c r="U65" t="s">
         <v>176</v>
       </c>
-      <c r="V65" s="1">
+      <c r="V65" s="2">
         <v>46107</v>
       </c>
     </row>
@@ -4446,7 +4472,7 @@
       <c r="U66" t="s">
         <v>176</v>
       </c>
-      <c r="V66" s="1">
+      <c r="V66" s="2">
         <v>46107</v>
       </c>
     </row>
@@ -4490,7 +4516,7 @@
       <c r="U67" t="s">
         <v>92</v>
       </c>
-      <c r="V67" s="1">
+      <c r="V67" s="2">
         <v>46168</v>
       </c>
     </row>
@@ -4537,7 +4563,7 @@
       <c r="U68" t="s">
         <v>92</v>
       </c>
-      <c r="V68" s="1">
+      <c r="V68" s="2">
         <v>46291</v>
       </c>
     </row>
@@ -4563,7 +4589,7 @@
       <c r="G69" t="s">
         <v>107</v>
       </c>
-      <c r="H69" s="1">
+      <c r="H69" s="2">
         <v>46303</v>
       </c>
       <c r="I69" t="s">
@@ -4599,7 +4625,7 @@
       <c r="U69" t="s">
         <v>176</v>
       </c>
-      <c r="V69" s="1">
+      <c r="V69" s="2">
         <v>46229</v>
       </c>
     </row>
@@ -4643,7 +4669,7 @@
       <c r="U70" t="s">
         <v>92</v>
       </c>
-      <c r="V70" s="1">
+      <c r="V70" s="2">
         <v>46260</v>
       </c>
     </row>
@@ -4687,7 +4713,7 @@
       <c r="U71" t="s">
         <v>176</v>
       </c>
-      <c r="V71" s="1">
+      <c r="V71" s="2">
         <v>46291</v>
       </c>
     </row>
@@ -4731,7 +4757,7 @@
       <c r="U72" t="s">
         <v>176</v>
       </c>
-      <c r="V72" s="1">
+      <c r="V72" s="2">
         <v>46168</v>
       </c>
     </row>
@@ -4775,7 +4801,7 @@
       <c r="U73" t="s">
         <v>176</v>
       </c>
-      <c r="V73" s="1">
+      <c r="V73" s="2">
         <v>46291</v>
       </c>
     </row>
@@ -4819,7 +4845,7 @@
       <c r="U74" t="s">
         <v>176</v>
       </c>
-      <c r="V74" s="1">
+      <c r="V74" s="2">
         <v>46291</v>
       </c>
     </row>
@@ -4863,7 +4889,7 @@
       <c r="U75" t="s">
         <v>176</v>
       </c>
-      <c r="V75" s="1">
+      <c r="V75" s="2">
         <v>46291</v>
       </c>
     </row>
@@ -4910,7 +4936,7 @@
       <c r="U76" t="s">
         <v>92</v>
       </c>
-      <c r="V76" s="1">
+      <c r="V76" s="2">
         <v>46321</v>
       </c>
     </row>
@@ -4960,7 +4986,7 @@
       <c r="U77" t="s">
         <v>176</v>
       </c>
-      <c r="V77" s="1">
+      <c r="V77" s="2">
         <v>46381</v>
       </c>
     </row>
@@ -5010,7 +5036,7 @@
       <c r="U78" t="s">
         <v>176</v>
       </c>
-      <c r="V78" s="1">
+      <c r="V78" s="2">
         <v>46381</v>
       </c>
     </row>
@@ -5060,7 +5086,7 @@
       <c r="U79" t="s">
         <v>92</v>
       </c>
-      <c r="V79" s="1">
+      <c r="V79" s="2">
         <v>46381</v>
       </c>
     </row>
@@ -5110,7 +5136,7 @@
       <c r="U80" t="s">
         <v>92</v>
       </c>
-      <c r="V80" s="1">
+      <c r="V80" s="2">
         <v>46381</v>
       </c>
     </row>
@@ -5160,7 +5186,7 @@
       <c r="U81" t="s">
         <v>92</v>
       </c>
-      <c r="V81" s="1">
+      <c r="V81" s="2">
         <v>46382</v>
       </c>
     </row>
@@ -5204,7 +5230,7 @@
       <c r="U82" t="s">
         <v>92</v>
       </c>
-      <c r="V82" s="1">
+      <c r="V82" s="2">
         <v>46382</v>
       </c>
     </row>
@@ -5260,7 +5286,7 @@
       <c r="U83" t="s">
         <v>176</v>
       </c>
-      <c r="V83" s="1">
+      <c r="V83" s="2">
         <v>46382</v>
       </c>
     </row>
@@ -5310,7 +5336,7 @@
       <c r="U84" t="s">
         <v>92</v>
       </c>
-      <c r="V84" s="1">
+      <c r="V84" s="2">
         <v>46321</v>
       </c>
     </row>
@@ -5354,7 +5380,7 @@
       <c r="U85" t="s">
         <v>92</v>
       </c>
-      <c r="V85" s="1">
+      <c r="V85" s="2">
         <v>46382</v>
       </c>
     </row>
@@ -5474,7 +5500,7 @@
       <c r="G88" t="s">
         <v>107</v>
       </c>
-      <c r="H88" s="1">
+      <c r="H88" s="2">
         <v>46303</v>
       </c>
       <c r="I88" t="s">
@@ -5504,7 +5530,7 @@
       <c r="U88" t="s">
         <v>92</v>
       </c>
-      <c r="V88" s="1">
+      <c r="V88" s="2">
         <v>46291</v>
       </c>
     </row>
@@ -5551,7 +5577,7 @@
       <c r="U89" t="s">
         <v>92</v>
       </c>
-      <c r="V89" s="1">
+      <c r="V89" s="2">
         <v>46291</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Atualização automática: mta (13/10/2026 15:08)
</commit_message>
<xml_diff>
--- a/Projetos/02_Dados_Tratados/base_mta_tratada.xlsx
+++ b/Projetos/02_Dados_Tratados/base_mta_tratada.xlsx
@@ -554,16 +554,8 @@
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="YYYY-MM-DD HH:MM:SS"/>
   </numFmts>
-  <fonts count="2">
+  <fonts count="1">
     <font>
-      <sz val="11"/>
-      <color theme="1"/>
-      <name val="Calibri"/>
-      <family val="2"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <b/>
       <sz val="11"/>
       <color theme="1"/>
       <name val="Calibri"/>
@@ -579,7 +571,7 @@
       <patternFill patternType="gray125"/>
     </fill>
   </fills>
-  <borders count="2">
+  <borders count="1">
     <border>
       <left/>
       <right/>
@@ -587,30 +579,12 @@
       <bottom/>
       <diagonal/>
     </border>
-    <border>
-      <left style="thin">
-        <color auto="1"/>
-      </left>
-      <right style="thin">
-        <color auto="1"/>
-      </right>
-      <top style="thin">
-        <color auto="1"/>
-      </top>
-      <bottom style="thin">
-        <color auto="1"/>
-      </bottom>
-      <diagonal/>
-    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="3">
+  <cellXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top"/>
-    </xf>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
   </cellXfs>
   <cellStyles count="1">
@@ -910,70 +884,70 @@
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:22">
-      <c r="A1" s="1" t="s">
+      <c r="A1" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="1" t="s">
+      <c r="B1" t="s">
         <v>1</v>
       </c>
-      <c r="C1" s="1" t="s">
+      <c r="C1" t="s">
         <v>2</v>
       </c>
-      <c r="D1" s="1" t="s">
+      <c r="D1" t="s">
         <v>3</v>
       </c>
-      <c r="E1" s="1" t="s">
+      <c r="E1" t="s">
         <v>4</v>
       </c>
-      <c r="F1" s="1" t="s">
+      <c r="F1" t="s">
         <v>5</v>
       </c>
-      <c r="G1" s="1" t="s">
+      <c r="G1" t="s">
         <v>6</v>
       </c>
-      <c r="H1" s="1" t="s">
+      <c r="H1" t="s">
         <v>7</v>
       </c>
-      <c r="I1" s="1" t="s">
+      <c r="I1" t="s">
         <v>8</v>
       </c>
-      <c r="J1" s="1" t="s">
+      <c r="J1" t="s">
         <v>9</v>
       </c>
-      <c r="K1" s="1" t="s">
+      <c r="K1" t="s">
         <v>10</v>
       </c>
-      <c r="L1" s="1" t="s">
+      <c r="L1" t="s">
         <v>11</v>
       </c>
-      <c r="M1" s="1" t="s">
+      <c r="M1" t="s">
         <v>12</v>
       </c>
-      <c r="N1" s="1" t="s">
+      <c r="N1" t="s">
         <v>13</v>
       </c>
-      <c r="O1" s="1" t="s">
+      <c r="O1" t="s">
         <v>14</v>
       </c>
-      <c r="P1" s="1" t="s">
+      <c r="P1" t="s">
         <v>15</v>
       </c>
-      <c r="Q1" s="1" t="s">
+      <c r="Q1" t="s">
         <v>16</v>
       </c>
-      <c r="R1" s="1" t="s">
+      <c r="R1" t="s">
         <v>17</v>
       </c>
-      <c r="S1" s="1" t="s">
+      <c r="S1" t="s">
         <v>18</v>
       </c>
-      <c r="T1" s="1" t="s">
+      <c r="T1" t="s">
         <v>19</v>
       </c>
-      <c r="U1" s="1" t="s">
+      <c r="U1" t="s">
         <v>20</v>
       </c>
-      <c r="V1" s="1" t="s">
+      <c r="V1" t="s">
         <v>21</v>
       </c>
     </row>
@@ -999,7 +973,7 @@
       <c r="G2" t="s">
         <v>107</v>
       </c>
-      <c r="H2" s="2">
+      <c r="H2" s="1">
         <v>46303</v>
       </c>
       <c r="I2" t="s">
@@ -1038,7 +1012,7 @@
       <c r="U2" t="s">
         <v>176</v>
       </c>
-      <c r="V2" s="2">
+      <c r="V2" s="1">
         <v>46229</v>
       </c>
     </row>
@@ -1085,7 +1059,7 @@
       <c r="U3" t="s">
         <v>92</v>
       </c>
-      <c r="V3" s="2">
+      <c r="V3" s="1">
         <v>46291</v>
       </c>
     </row>
@@ -1132,7 +1106,7 @@
       <c r="U4" t="s">
         <v>92</v>
       </c>
-      <c r="V4" s="2">
+      <c r="V4" s="1">
         <v>46321</v>
       </c>
     </row>
@@ -1179,7 +1153,7 @@
       <c r="U5" t="s">
         <v>92</v>
       </c>
-      <c r="V5" s="2">
+      <c r="V5" s="1">
         <v>46321</v>
       </c>
     </row>
@@ -1229,7 +1203,7 @@
       <c r="U6" t="s">
         <v>92</v>
       </c>
-      <c r="V6" s="2">
+      <c r="V6" s="1">
         <v>46291</v>
       </c>
     </row>
@@ -1255,7 +1229,7 @@
       <c r="G7" t="s">
         <v>109</v>
       </c>
-      <c r="H7" s="2">
+      <c r="H7" s="1">
         <v>46121</v>
       </c>
       <c r="I7" t="s">
@@ -1285,7 +1259,7 @@
       <c r="U7" t="s">
         <v>92</v>
       </c>
-      <c r="V7" s="2">
+      <c r="V7" s="1">
         <v>46138</v>
       </c>
     </row>
@@ -1332,7 +1306,7 @@
       <c r="U8" t="s">
         <v>92</v>
       </c>
-      <c r="V8" s="2">
+      <c r="V8" s="1">
         <v>46291</v>
       </c>
     </row>
@@ -1379,7 +1353,7 @@
       <c r="U9" t="s">
         <v>92</v>
       </c>
-      <c r="V9" s="2">
+      <c r="V9" s="1">
         <v>46291</v>
       </c>
     </row>
@@ -1402,7 +1376,7 @@
       <c r="G10" t="s">
         <v>107</v>
       </c>
-      <c r="H10" s="2">
+      <c r="H10" s="1">
         <v>46303</v>
       </c>
       <c r="I10" t="s">
@@ -1432,7 +1406,7 @@
       <c r="U10" t="s">
         <v>92</v>
       </c>
-      <c r="V10" s="2">
+      <c r="V10" s="1">
         <v>46291</v>
       </c>
     </row>
@@ -1479,7 +1453,7 @@
       <c r="U11" t="s">
         <v>92</v>
       </c>
-      <c r="V11" s="2">
+      <c r="V11" s="1">
         <v>46291</v>
       </c>
     </row>
@@ -1526,7 +1500,7 @@
       <c r="U12" t="s">
         <v>92</v>
       </c>
-      <c r="V12" s="2">
+      <c r="V12" s="1">
         <v>46291</v>
       </c>
     </row>
@@ -1552,7 +1526,7 @@
       <c r="G13" t="s">
         <v>109</v>
       </c>
-      <c r="H13" s="2">
+      <c r="H13" s="1">
         <v>46079</v>
       </c>
       <c r="I13" t="s">
@@ -1585,7 +1559,7 @@
       <c r="U13" t="s">
         <v>176</v>
       </c>
-      <c r="V13" s="2">
+      <c r="V13" s="1">
         <v>46079</v>
       </c>
     </row>
@@ -1611,7 +1585,7 @@
       <c r="G14" t="s">
         <v>107</v>
       </c>
-      <c r="H14" s="2">
+      <c r="H14" s="1">
         <v>46303</v>
       </c>
       <c r="I14" t="s">
@@ -1647,7 +1621,7 @@
       <c r="U14" t="s">
         <v>176</v>
       </c>
-      <c r="V14" s="2">
+      <c r="V14" s="1">
         <v>46352</v>
       </c>
     </row>
@@ -1673,7 +1647,7 @@
       <c r="G15" t="s">
         <v>107</v>
       </c>
-      <c r="H15" s="2">
+      <c r="H15" s="1">
         <v>46303</v>
       </c>
       <c r="I15" t="s">
@@ -1709,7 +1683,7 @@
       <c r="U15" t="s">
         <v>176</v>
       </c>
-      <c r="V15" s="2">
+      <c r="V15" s="1">
         <v>46352</v>
       </c>
     </row>
@@ -1735,7 +1709,7 @@
       <c r="G16" t="s">
         <v>107</v>
       </c>
-      <c r="H16" s="2">
+      <c r="H16" s="1">
         <v>46303</v>
       </c>
       <c r="I16" t="s">
@@ -1771,7 +1745,7 @@
       <c r="U16" t="s">
         <v>176</v>
       </c>
-      <c r="V16" s="2">
+      <c r="V16" s="1">
         <v>46352</v>
       </c>
     </row>
@@ -1797,7 +1771,7 @@
       <c r="G17" t="s">
         <v>107</v>
       </c>
-      <c r="H17" s="2">
+      <c r="H17" s="1">
         <v>46303</v>
       </c>
       <c r="I17" t="s">
@@ -1833,7 +1807,7 @@
       <c r="U17" t="s">
         <v>176</v>
       </c>
-      <c r="V17" s="2">
+      <c r="V17" s="1">
         <v>46229</v>
       </c>
     </row>
@@ -1859,7 +1833,7 @@
       <c r="G18" t="s">
         <v>109</v>
       </c>
-      <c r="H18" s="2">
+      <c r="H18" s="1">
         <v>46098</v>
       </c>
       <c r="I18" t="s">
@@ -1892,7 +1866,7 @@
       <c r="U18" t="s">
         <v>176</v>
       </c>
-      <c r="V18" s="2">
+      <c r="V18" s="1">
         <v>46107</v>
       </c>
     </row>
@@ -1918,7 +1892,7 @@
       <c r="G19" t="s">
         <v>109</v>
       </c>
-      <c r="H19" s="2">
+      <c r="H19" s="1">
         <v>46076</v>
       </c>
       <c r="I19" t="s">
@@ -1948,7 +1922,7 @@
       <c r="U19" t="s">
         <v>92</v>
       </c>
-      <c r="V19" s="2">
+      <c r="V19" s="1">
         <v>46079</v>
       </c>
     </row>
@@ -1974,7 +1948,7 @@
       <c r="G20" t="s">
         <v>109</v>
       </c>
-      <c r="H20" s="2">
+      <c r="H20" s="1">
         <v>46076</v>
       </c>
       <c r="I20" t="s">
@@ -2004,7 +1978,7 @@
       <c r="U20" t="s">
         <v>92</v>
       </c>
-      <c r="V20" s="2">
+      <c r="V20" s="1">
         <v>46079</v>
       </c>
     </row>
@@ -2051,7 +2025,7 @@
       <c r="U21" t="s">
         <v>92</v>
       </c>
-      <c r="V21" s="2">
+      <c r="V21" s="1">
         <v>46321</v>
       </c>
     </row>
@@ -2098,7 +2072,7 @@
       <c r="U22" t="s">
         <v>92</v>
       </c>
-      <c r="V22" s="2">
+      <c r="V22" s="1">
         <v>46321</v>
       </c>
     </row>
@@ -2145,7 +2119,7 @@
       <c r="U23" t="s">
         <v>92</v>
       </c>
-      <c r="V23" s="2">
+      <c r="V23" s="1">
         <v>46321</v>
       </c>
     </row>
@@ -2192,7 +2166,7 @@
       <c r="U24" t="s">
         <v>92</v>
       </c>
-      <c r="V24" s="2">
+      <c r="V24" s="1">
         <v>46321</v>
       </c>
     </row>
@@ -2218,7 +2192,7 @@
       <c r="G25" t="s">
         <v>109</v>
       </c>
-      <c r="H25" s="2">
+      <c r="H25" s="1">
         <v>46119</v>
       </c>
       <c r="I25" t="s">
@@ -2251,7 +2225,7 @@
       <c r="U25" t="s">
         <v>176</v>
       </c>
-      <c r="V25" s="2">
+      <c r="V25" s="1">
         <v>46138</v>
       </c>
     </row>
@@ -2277,7 +2251,7 @@
       <c r="G26" t="s">
         <v>109</v>
       </c>
-      <c r="H26" s="2">
+      <c r="H26" s="1">
         <v>46121</v>
       </c>
       <c r="I26" t="s">
@@ -2307,7 +2281,7 @@
       <c r="U26" t="s">
         <v>92</v>
       </c>
-      <c r="V26" s="2">
+      <c r="V26" s="1">
         <v>46138</v>
       </c>
     </row>
@@ -2333,7 +2307,7 @@
       <c r="G27" t="s">
         <v>109</v>
       </c>
-      <c r="H27" s="2">
+      <c r="H27" s="1">
         <v>46076</v>
       </c>
       <c r="I27" t="s">
@@ -2363,7 +2337,7 @@
       <c r="U27" t="s">
         <v>92</v>
       </c>
-      <c r="V27" s="2">
+      <c r="V27" s="1">
         <v>46079</v>
       </c>
     </row>
@@ -2389,7 +2363,7 @@
       <c r="G28" t="s">
         <v>107</v>
       </c>
-      <c r="H28" s="2">
+      <c r="H28" s="1">
         <v>46303</v>
       </c>
       <c r="I28" t="s">
@@ -2425,7 +2399,7 @@
       <c r="U28" t="s">
         <v>176</v>
       </c>
-      <c r="V28" s="2">
+      <c r="V28" s="1">
         <v>46291</v>
       </c>
     </row>
@@ -2451,7 +2425,7 @@
       <c r="G29" t="s">
         <v>109</v>
       </c>
-      <c r="H29" s="2">
+      <c r="H29" s="1">
         <v>46199</v>
       </c>
       <c r="I29" t="s">
@@ -2484,7 +2458,7 @@
       <c r="U29" t="s">
         <v>176</v>
       </c>
-      <c r="V29" s="2">
+      <c r="V29" s="1">
         <v>46199</v>
       </c>
     </row>
@@ -2510,7 +2484,7 @@
       <c r="G30" t="s">
         <v>109</v>
       </c>
-      <c r="H30" s="2">
+      <c r="H30" s="1">
         <v>46199</v>
       </c>
       <c r="I30" t="s">
@@ -2543,7 +2517,7 @@
       <c r="U30" t="s">
         <v>176</v>
       </c>
-      <c r="V30" s="2">
+      <c r="V30" s="1">
         <v>46199</v>
       </c>
     </row>
@@ -2569,7 +2543,7 @@
       <c r="G31" t="s">
         <v>109</v>
       </c>
-      <c r="H31" s="2">
+      <c r="H31" s="1">
         <v>46199</v>
       </c>
       <c r="I31" t="s">
@@ -2602,7 +2576,7 @@
       <c r="U31" t="s">
         <v>176</v>
       </c>
-      <c r="V31" s="2">
+      <c r="V31" s="1">
         <v>46199</v>
       </c>
     </row>
@@ -2628,7 +2602,7 @@
       <c r="G32" t="s">
         <v>109</v>
       </c>
-      <c r="H32" s="2">
+      <c r="H32" s="1">
         <v>46199</v>
       </c>
       <c r="I32" t="s">
@@ -2661,7 +2635,7 @@
       <c r="U32" t="s">
         <v>176</v>
       </c>
-      <c r="V32" s="2">
+      <c r="V32" s="1">
         <v>46199</v>
       </c>
     </row>
@@ -2714,7 +2688,7 @@
       <c r="U33" t="s">
         <v>176</v>
       </c>
-      <c r="V33" s="2">
+      <c r="V33" s="1">
         <v>46291</v>
       </c>
     </row>
@@ -2740,7 +2714,7 @@
       <c r="G34" t="s">
         <v>109</v>
       </c>
-      <c r="H34" s="2">
+      <c r="H34" s="1">
         <v>46191</v>
       </c>
       <c r="I34" t="s">
@@ -2773,7 +2747,7 @@
       <c r="U34" t="s">
         <v>176</v>
       </c>
-      <c r="V34" s="2">
+      <c r="V34" s="1">
         <v>46199</v>
       </c>
     </row>
@@ -2799,7 +2773,7 @@
       <c r="G35" t="s">
         <v>109</v>
       </c>
-      <c r="H35" s="2">
+      <c r="H35" s="1">
         <v>46119</v>
       </c>
       <c r="I35" t="s">
@@ -2829,7 +2803,7 @@
       <c r="U35" t="s">
         <v>176</v>
       </c>
-      <c r="V35" s="2">
+      <c r="V35" s="1">
         <v>46138</v>
       </c>
     </row>
@@ -2855,7 +2829,7 @@
       <c r="G36" t="s">
         <v>109</v>
       </c>
-      <c r="H36" s="2">
+      <c r="H36" s="1">
         <v>46213</v>
       </c>
       <c r="I36" t="s">
@@ -2885,7 +2859,7 @@
       <c r="U36" t="s">
         <v>92</v>
       </c>
-      <c r="V36" s="2">
+      <c r="V36" s="1">
         <v>46229</v>
       </c>
     </row>
@@ -2911,7 +2885,7 @@
       <c r="G37" t="s">
         <v>109</v>
       </c>
-      <c r="H37" s="2">
+      <c r="H37" s="1">
         <v>46175</v>
       </c>
       <c r="I37" t="s">
@@ -2941,7 +2915,7 @@
       <c r="U37" t="s">
         <v>92</v>
       </c>
-      <c r="V37" s="2">
+      <c r="V37" s="1">
         <v>46199</v>
       </c>
     </row>
@@ -2967,7 +2941,7 @@
       <c r="G38" t="s">
         <v>109</v>
       </c>
-      <c r="H38" s="2">
+      <c r="H38" s="1">
         <v>46213</v>
       </c>
       <c r="I38" t="s">
@@ -2997,7 +2971,7 @@
       <c r="U38" t="s">
         <v>92</v>
       </c>
-      <c r="V38" s="2">
+      <c r="V38" s="1">
         <v>46229</v>
       </c>
     </row>
@@ -3023,7 +2997,7 @@
       <c r="G39" t="s">
         <v>109</v>
       </c>
-      <c r="H39" s="2">
+      <c r="H39" s="1">
         <v>46199</v>
       </c>
       <c r="I39" t="s">
@@ -3053,7 +3027,7 @@
       <c r="U39" t="s">
         <v>92</v>
       </c>
-      <c r="V39" s="2">
+      <c r="V39" s="1">
         <v>46199</v>
       </c>
     </row>
@@ -3079,7 +3053,7 @@
       <c r="G40" t="s">
         <v>109</v>
       </c>
-      <c r="H40" s="2">
+      <c r="H40" s="1">
         <v>46199</v>
       </c>
       <c r="I40" t="s">
@@ -3109,7 +3083,7 @@
       <c r="U40" t="s">
         <v>92</v>
       </c>
-      <c r="V40" s="2">
+      <c r="V40" s="1">
         <v>46199</v>
       </c>
     </row>
@@ -3135,7 +3109,7 @@
       <c r="G41" t="s">
         <v>109</v>
       </c>
-      <c r="H41" s="2">
+      <c r="H41" s="1">
         <v>46204</v>
       </c>
       <c r="I41" t="s">
@@ -3165,7 +3139,7 @@
       <c r="U41" t="s">
         <v>92</v>
       </c>
-      <c r="V41" s="2">
+      <c r="V41" s="1">
         <v>46229</v>
       </c>
     </row>
@@ -3191,7 +3165,7 @@
       <c r="G42" t="s">
         <v>109</v>
       </c>
-      <c r="H42" s="2">
+      <c r="H42" s="1">
         <v>46244</v>
       </c>
       <c r="I42" t="s">
@@ -3221,7 +3195,7 @@
       <c r="U42" t="s">
         <v>92</v>
       </c>
-      <c r="V42" s="2">
+      <c r="V42" s="1">
         <v>46199</v>
       </c>
     </row>
@@ -3265,7 +3239,7 @@
       <c r="U43" t="s">
         <v>92</v>
       </c>
-      <c r="V43" s="2">
+      <c r="V43" s="1">
         <v>46260</v>
       </c>
     </row>
@@ -3291,7 +3265,7 @@
       <c r="G44" t="s">
         <v>109</v>
       </c>
-      <c r="H44" s="2">
+      <c r="H44" s="1">
         <v>46191</v>
       </c>
       <c r="I44" t="s">
@@ -3321,7 +3295,7 @@
       <c r="U44" t="s">
         <v>92</v>
       </c>
-      <c r="V44" s="2">
+      <c r="V44" s="1">
         <v>46199</v>
       </c>
     </row>
@@ -3347,7 +3321,7 @@
       <c r="G45" t="s">
         <v>109</v>
       </c>
-      <c r="H45" s="2">
+      <c r="H45" s="1">
         <v>46191</v>
       </c>
       <c r="I45" t="s">
@@ -3377,7 +3351,7 @@
       <c r="U45" t="s">
         <v>92</v>
       </c>
-      <c r="V45" s="2">
+      <c r="V45" s="1">
         <v>46199</v>
       </c>
     </row>
@@ -3403,7 +3377,7 @@
       <c r="G46" t="s">
         <v>109</v>
       </c>
-      <c r="H46" s="2">
+      <c r="H46" s="1">
         <v>46213</v>
       </c>
       <c r="I46" t="s">
@@ -3436,7 +3410,7 @@
       <c r="U46" t="s">
         <v>176</v>
       </c>
-      <c r="V46" s="2">
+      <c r="V46" s="1">
         <v>46229</v>
       </c>
     </row>
@@ -3462,7 +3436,7 @@
       <c r="G47" t="s">
         <v>109</v>
       </c>
-      <c r="H47" s="2">
+      <c r="H47" s="1">
         <v>46210</v>
       </c>
       <c r="I47" t="s">
@@ -3492,7 +3466,7 @@
       <c r="U47" t="s">
         <v>176</v>
       </c>
-      <c r="V47" s="2">
+      <c r="V47" s="1">
         <v>46229</v>
       </c>
     </row>
@@ -3539,7 +3513,7 @@
       <c r="U48" t="s">
         <v>92</v>
       </c>
-      <c r="V48" s="2">
+      <c r="V48" s="1">
         <v>46321</v>
       </c>
     </row>
@@ -3565,7 +3539,7 @@
       <c r="G49" t="s">
         <v>107</v>
       </c>
-      <c r="H49" s="2">
+      <c r="H49" s="1">
         <v>46303</v>
       </c>
       <c r="I49" t="s">
@@ -3601,7 +3575,7 @@
       <c r="U49" t="s">
         <v>176</v>
       </c>
-      <c r="V49" s="2">
+      <c r="V49" s="1">
         <v>46291</v>
       </c>
     </row>
@@ -3627,7 +3601,7 @@
       <c r="G50" t="s">
         <v>109</v>
       </c>
-      <c r="H50" s="2">
+      <c r="H50" s="1">
         <v>46176</v>
       </c>
       <c r="I50" t="s">
@@ -3660,7 +3634,7 @@
       <c r="U50" t="s">
         <v>176</v>
       </c>
-      <c r="V50" s="2">
+      <c r="V50" s="1">
         <v>46199</v>
       </c>
     </row>
@@ -3716,7 +3690,7 @@
       <c r="U51" t="s">
         <v>176</v>
       </c>
-      <c r="V51" s="2">
+      <c r="V51" s="1">
         <v>46260</v>
       </c>
     </row>
@@ -3742,7 +3716,7 @@
       <c r="G52" t="s">
         <v>109</v>
       </c>
-      <c r="H52" s="2">
+      <c r="H52" s="1">
         <v>46295</v>
       </c>
       <c r="I52" t="s">
@@ -3778,7 +3752,7 @@
       <c r="U52" t="s">
         <v>176</v>
       </c>
-      <c r="V52" s="2">
+      <c r="V52" s="1">
         <v>46291</v>
       </c>
     </row>
@@ -3831,7 +3805,7 @@
       <c r="U53" t="s">
         <v>176</v>
       </c>
-      <c r="V53" s="2">
+      <c r="V53" s="1">
         <v>46321</v>
       </c>
     </row>
@@ -3857,7 +3831,7 @@
       <c r="G54" t="s">
         <v>109</v>
       </c>
-      <c r="H54" s="2">
+      <c r="H54" s="1">
         <v>46227</v>
       </c>
       <c r="I54" t="s">
@@ -3887,7 +3861,7 @@
       <c r="U54" t="s">
         <v>176</v>
       </c>
-      <c r="V54" s="2">
+      <c r="V54" s="1">
         <v>46229</v>
       </c>
     </row>
@@ -3910,7 +3884,7 @@
       <c r="G55" t="s">
         <v>109</v>
       </c>
-      <c r="H55" s="2">
+      <c r="H55" s="1">
         <v>46280</v>
       </c>
       <c r="I55" t="s">
@@ -3940,7 +3914,7 @@
       <c r="U55" t="s">
         <v>176</v>
       </c>
-      <c r="V55" s="2">
+      <c r="V55" s="1">
         <v>46291</v>
       </c>
     </row>
@@ -3963,7 +3937,7 @@
       <c r="G56" t="s">
         <v>109</v>
       </c>
-      <c r="H56" s="2">
+      <c r="H56" s="1">
         <v>46280</v>
       </c>
       <c r="I56" t="s">
@@ -3993,7 +3967,7 @@
       <c r="U56" t="s">
         <v>176</v>
       </c>
-      <c r="V56" s="2">
+      <c r="V56" s="1">
         <v>46260</v>
       </c>
     </row>
@@ -4016,7 +3990,7 @@
       <c r="G57" t="s">
         <v>109</v>
       </c>
-      <c r="H57" s="2">
+      <c r="H57" s="1">
         <v>46295</v>
       </c>
       <c r="I57" t="s">
@@ -4046,7 +4020,7 @@
       <c r="U57" t="s">
         <v>176</v>
       </c>
-      <c r="V57" s="2">
+      <c r="V57" s="1">
         <v>46291</v>
       </c>
     </row>
@@ -4069,7 +4043,7 @@
       <c r="G58" t="s">
         <v>109</v>
       </c>
-      <c r="H58" s="2">
+      <c r="H58" s="1">
         <v>46295</v>
       </c>
       <c r="I58" t="s">
@@ -4099,7 +4073,7 @@
       <c r="U58" t="s">
         <v>176</v>
       </c>
-      <c r="V58" s="2">
+      <c r="V58" s="1">
         <v>46291</v>
       </c>
     </row>
@@ -4146,7 +4120,7 @@
       <c r="U59" t="s">
         <v>176</v>
       </c>
-      <c r="V59" s="2">
+      <c r="V59" s="1">
         <v>46321</v>
       </c>
     </row>
@@ -4172,7 +4146,7 @@
       <c r="G60" t="s">
         <v>109</v>
       </c>
-      <c r="H60" s="2">
+      <c r="H60" s="1">
         <v>46301</v>
       </c>
       <c r="I60" t="s">
@@ -4208,7 +4182,7 @@
       <c r="U60" t="s">
         <v>176</v>
       </c>
-      <c r="V60" s="2">
+      <c r="V60" s="1">
         <v>46352</v>
       </c>
     </row>
@@ -4252,7 +4226,7 @@
       <c r="U61" t="s">
         <v>176</v>
       </c>
-      <c r="V61" s="2">
+      <c r="V61" s="1">
         <v>46107</v>
       </c>
     </row>
@@ -4296,7 +4270,7 @@
       <c r="U62" t="s">
         <v>176</v>
       </c>
-      <c r="V62" s="2">
+      <c r="V62" s="1">
         <v>46107</v>
       </c>
     </row>
@@ -4340,7 +4314,7 @@
       <c r="U63" t="s">
         <v>176</v>
       </c>
-      <c r="V63" s="2">
+      <c r="V63" s="1">
         <v>46107</v>
       </c>
     </row>
@@ -4384,7 +4358,7 @@
       <c r="U64" t="s">
         <v>176</v>
       </c>
-      <c r="V64" s="2">
+      <c r="V64" s="1">
         <v>46107</v>
       </c>
     </row>
@@ -4428,7 +4402,7 @@
       <c r="U65" t="s">
         <v>176</v>
       </c>
-      <c r="V65" s="2">
+      <c r="V65" s="1">
         <v>46107</v>
       </c>
     </row>
@@ -4472,7 +4446,7 @@
       <c r="U66" t="s">
         <v>176</v>
       </c>
-      <c r="V66" s="2">
+      <c r="V66" s="1">
         <v>46107</v>
       </c>
     </row>
@@ -4516,7 +4490,7 @@
       <c r="U67" t="s">
         <v>92</v>
       </c>
-      <c r="V67" s="2">
+      <c r="V67" s="1">
         <v>46168</v>
       </c>
     </row>
@@ -4563,7 +4537,7 @@
       <c r="U68" t="s">
         <v>92</v>
       </c>
-      <c r="V68" s="2">
+      <c r="V68" s="1">
         <v>46291</v>
       </c>
     </row>
@@ -4589,7 +4563,7 @@
       <c r="G69" t="s">
         <v>107</v>
       </c>
-      <c r="H69" s="2">
+      <c r="H69" s="1">
         <v>46303</v>
       </c>
       <c r="I69" t="s">
@@ -4625,7 +4599,7 @@
       <c r="U69" t="s">
         <v>176</v>
       </c>
-      <c r="V69" s="2">
+      <c r="V69" s="1">
         <v>46229</v>
       </c>
     </row>
@@ -4669,7 +4643,7 @@
       <c r="U70" t="s">
         <v>92</v>
       </c>
-      <c r="V70" s="2">
+      <c r="V70" s="1">
         <v>46260</v>
       </c>
     </row>
@@ -4713,7 +4687,7 @@
       <c r="U71" t="s">
         <v>176</v>
       </c>
-      <c r="V71" s="2">
+      <c r="V71" s="1">
         <v>46291</v>
       </c>
     </row>
@@ -4757,7 +4731,7 @@
       <c r="U72" t="s">
         <v>176</v>
       </c>
-      <c r="V72" s="2">
+      <c r="V72" s="1">
         <v>46168</v>
       </c>
     </row>
@@ -4801,7 +4775,7 @@
       <c r="U73" t="s">
         <v>176</v>
       </c>
-      <c r="V73" s="2">
+      <c r="V73" s="1">
         <v>46291</v>
       </c>
     </row>
@@ -4845,7 +4819,7 @@
       <c r="U74" t="s">
         <v>176</v>
       </c>
-      <c r="V74" s="2">
+      <c r="V74" s="1">
         <v>46291</v>
       </c>
     </row>
@@ -4889,7 +4863,7 @@
       <c r="U75" t="s">
         <v>176</v>
       </c>
-      <c r="V75" s="2">
+      <c r="V75" s="1">
         <v>46291</v>
       </c>
     </row>
@@ -4936,7 +4910,7 @@
       <c r="U76" t="s">
         <v>92</v>
       </c>
-      <c r="V76" s="2">
+      <c r="V76" s="1">
         <v>46321</v>
       </c>
     </row>
@@ -4986,7 +4960,7 @@
       <c r="U77" t="s">
         <v>176</v>
       </c>
-      <c r="V77" s="2">
+      <c r="V77" s="1">
         <v>46381</v>
       </c>
     </row>
@@ -5036,7 +5010,7 @@
       <c r="U78" t="s">
         <v>176</v>
       </c>
-      <c r="V78" s="2">
+      <c r="V78" s="1">
         <v>46381</v>
       </c>
     </row>
@@ -5086,7 +5060,7 @@
       <c r="U79" t="s">
         <v>92</v>
       </c>
-      <c r="V79" s="2">
+      <c r="V79" s="1">
         <v>46381</v>
       </c>
     </row>
@@ -5136,7 +5110,7 @@
       <c r="U80" t="s">
         <v>92</v>
       </c>
-      <c r="V80" s="2">
+      <c r="V80" s="1">
         <v>46381</v>
       </c>
     </row>
@@ -5186,7 +5160,7 @@
       <c r="U81" t="s">
         <v>92</v>
       </c>
-      <c r="V81" s="2">
+      <c r="V81" s="1">
         <v>46382</v>
       </c>
     </row>
@@ -5230,7 +5204,7 @@
       <c r="U82" t="s">
         <v>92</v>
       </c>
-      <c r="V82" s="2">
+      <c r="V82" s="1">
         <v>46382</v>
       </c>
     </row>
@@ -5286,7 +5260,7 @@
       <c r="U83" t="s">
         <v>176</v>
       </c>
-      <c r="V83" s="2">
+      <c r="V83" s="1">
         <v>46382</v>
       </c>
     </row>
@@ -5336,7 +5310,7 @@
       <c r="U84" t="s">
         <v>92</v>
       </c>
-      <c r="V84" s="2">
+      <c r="V84" s="1">
         <v>46321</v>
       </c>
     </row>
@@ -5380,7 +5354,7 @@
       <c r="U85" t="s">
         <v>92</v>
       </c>
-      <c r="V85" s="2">
+      <c r="V85" s="1">
         <v>46382</v>
       </c>
     </row>
@@ -5500,7 +5474,7 @@
       <c r="G88" t="s">
         <v>107</v>
       </c>
-      <c r="H88" s="2">
+      <c r="H88" s="1">
         <v>46303</v>
       </c>
       <c r="I88" t="s">
@@ -5530,7 +5504,7 @@
       <c r="U88" t="s">
         <v>92</v>
       </c>
-      <c r="V88" s="2">
+      <c r="V88" s="1">
         <v>46291</v>
       </c>
     </row>
@@ -5577,7 +5551,7 @@
       <c r="U89" t="s">
         <v>92</v>
       </c>
-      <c r="V89" s="2">
+      <c r="V89" s="1">
         <v>46291</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Atualização automática: mta (14/10/2026 12:48)
</commit_message>
<xml_diff>
--- a/Projetos/02_Dados_Tratados/base_mta_tratada.xlsx
+++ b/Projetos/02_Dados_Tratados/base_mta_tratada.xlsx
@@ -14,7 +14,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1205" uniqueCount="177">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1206" uniqueCount="181">
   <si>
     <t>linha</t>
   </si>
@@ -358,6 +358,9 @@
     <t>C26216</t>
   </si>
   <si>
+    <t>C26245</t>
+  </si>
+  <si>
     <t>C26042</t>
   </si>
   <si>
@@ -409,6 +412,12 @@
     <t>C26485</t>
   </si>
   <si>
+    <t>C26526</t>
+  </si>
+  <si>
+    <t>C26243</t>
+  </si>
+  <si>
     <t>2026-09-11 00:00:00</t>
   </si>
   <si>
@@ -439,6 +448,9 @@
     <t>Atender</t>
   </si>
   <si>
+    <t>ATENDER CABW 30</t>
+  </si>
+  <si>
     <t>Atender. Alterar a UGE para CABW. Alterar a atividade para "Requisição CABW". Alterar a tarefa para "Requisições Consumíveis". Alterar a ND para 339030.</t>
   </si>
   <si>
@@ -466,37 +478,37 @@
     <t>CNT 031/CELOG-PAMASP/2022 - PW - RG</t>
   </si>
   <si>
+    <t>CNT 005/CELOG-PAMALS/2025 - VEE ONE</t>
+  </si>
+  <si>
+    <t>CNT 048/CELOG-PAMASP/2022 - PW - Material</t>
+  </si>
+  <si>
+    <t>CNT XXX/CELOG-PAMASP/2026 - Material</t>
+  </si>
+  <si>
+    <t>CNT 006/CELOG-PAMASP/2026 - PW - RG</t>
+  </si>
+  <si>
+    <t>2025-BABR-11</t>
+  </si>
+  <si>
+    <t>2025-BABR-13</t>
+  </si>
+  <si>
+    <t>2025-BABR-24</t>
+  </si>
+  <si>
+    <t>2025-BABV-02</t>
+  </si>
+  <si>
+    <t>2025-BABV-07</t>
+  </si>
+  <si>
+    <t>2025-BABV-11</t>
+  </si>
+  <si>
     <t>Requisição FMS</t>
-  </si>
-  <si>
-    <t>CNT 005/CELOG-PAMALS/2025 - VEE ONE</t>
-  </si>
-  <si>
-    <t>CNT 048/CELOG-PAMASP/2022 - PW - Material</t>
-  </si>
-  <si>
-    <t>CNT XXX/CELOG-PAMASP/2026 - Material</t>
-  </si>
-  <si>
-    <t>CNT 006/CELOG-PAMASP/2026 - PW - RG</t>
-  </si>
-  <si>
-    <t>2025-BABR-11</t>
-  </si>
-  <si>
-    <t>2025-BABR-13</t>
-  </si>
-  <si>
-    <t>2025-BABR-24</t>
-  </si>
-  <si>
-    <t>2025-BABV-02</t>
-  </si>
-  <si>
-    <t>2025-BABV-07</t>
-  </si>
-  <si>
-    <t>2025-BABV-11</t>
   </si>
   <si>
     <t>CNT XXX/CABW-PAMASP/2026 - XX- Exchange</t>
@@ -980,16 +992,16 @@
         <v>112</v>
       </c>
       <c r="J2" t="s">
-        <v>131</v>
+        <v>134</v>
       </c>
       <c r="K2" t="s">
-        <v>140</v>
+        <v>143</v>
       </c>
       <c r="L2" t="s">
-        <v>145</v>
+        <v>149</v>
       </c>
       <c r="N2" t="s">
-        <v>146</v>
+        <v>150</v>
       </c>
       <c r="O2" t="s">
         <v>23</v>
@@ -998,19 +1010,19 @@
         <v>135000</v>
       </c>
       <c r="Q2" t="s">
-        <v>164</v>
+        <v>168</v>
       </c>
       <c r="R2" t="s">
-        <v>167</v>
+        <v>171</v>
       </c>
       <c r="S2" t="s">
-        <v>170</v>
+        <v>174</v>
       </c>
       <c r="T2" t="s">
-        <v>172</v>
+        <v>176</v>
       </c>
       <c r="U2" t="s">
-        <v>176</v>
+        <v>180</v>
       </c>
       <c r="V2" s="1">
         <v>46229</v>
@@ -1039,22 +1051,22 @@
         <v>108</v>
       </c>
       <c r="N3" t="s">
-        <v>146</v>
+        <v>150</v>
       </c>
       <c r="O3" t="s">
         <v>24</v>
       </c>
       <c r="Q3" t="s">
-        <v>164</v>
+        <v>168</v>
       </c>
       <c r="R3" t="s">
-        <v>167</v>
+        <v>171</v>
       </c>
       <c r="S3" t="s">
-        <v>170</v>
+        <v>174</v>
       </c>
       <c r="T3" t="s">
-        <v>172</v>
+        <v>176</v>
       </c>
       <c r="U3" t="s">
         <v>92</v>
@@ -1086,22 +1098,22 @@
         <v>108</v>
       </c>
       <c r="N4" t="s">
-        <v>147</v>
+        <v>151</v>
       </c>
       <c r="O4" t="s">
         <v>25</v>
       </c>
       <c r="Q4" t="s">
-        <v>164</v>
+        <v>168</v>
       </c>
       <c r="R4" t="s">
-        <v>168</v>
+        <v>172</v>
       </c>
       <c r="S4" t="s">
-        <v>170</v>
+        <v>174</v>
       </c>
       <c r="T4" t="s">
-        <v>172</v>
+        <v>176</v>
       </c>
       <c r="U4" t="s">
         <v>92</v>
@@ -1133,22 +1145,22 @@
         <v>108</v>
       </c>
       <c r="N5" t="s">
-        <v>147</v>
+        <v>151</v>
       </c>
       <c r="O5" t="s">
         <v>26</v>
       </c>
       <c r="Q5" t="s">
-        <v>164</v>
+        <v>168</v>
       </c>
       <c r="R5" t="s">
-        <v>168</v>
+        <v>172</v>
       </c>
       <c r="S5" t="s">
-        <v>170</v>
+        <v>174</v>
       </c>
       <c r="T5" t="s">
-        <v>172</v>
+        <v>176</v>
       </c>
       <c r="U5" t="s">
         <v>92</v>
@@ -1180,25 +1192,25 @@
         <v>108</v>
       </c>
       <c r="L6" t="s">
-        <v>145</v>
+        <v>149</v>
       </c>
       <c r="N6" t="s">
-        <v>148</v>
+        <v>152</v>
       </c>
       <c r="O6" t="s">
         <v>27</v>
       </c>
       <c r="Q6" t="s">
-        <v>164</v>
+        <v>168</v>
       </c>
       <c r="R6" t="s">
-        <v>168</v>
+        <v>172</v>
       </c>
       <c r="S6" t="s">
-        <v>170</v>
+        <v>174</v>
       </c>
       <c r="T6" t="s">
-        <v>172</v>
+        <v>176</v>
       </c>
       <c r="U6" t="s">
         <v>92</v>
@@ -1236,7 +1248,7 @@
         <v>113</v>
       </c>
       <c r="N7" t="s">
-        <v>149</v>
+        <v>153</v>
       </c>
       <c r="O7" t="s">
         <v>28</v>
@@ -1245,16 +1257,16 @@
         <v>3799999.6</v>
       </c>
       <c r="Q7" t="s">
-        <v>165</v>
+        <v>169</v>
       </c>
       <c r="R7" t="s">
-        <v>168</v>
+        <v>172</v>
       </c>
       <c r="S7" t="s">
-        <v>170</v>
+        <v>174</v>
       </c>
       <c r="T7" t="s">
-        <v>173</v>
+        <v>177</v>
       </c>
       <c r="U7" t="s">
         <v>92</v>
@@ -1286,22 +1298,22 @@
         <v>108</v>
       </c>
       <c r="N8" t="s">
-        <v>147</v>
+        <v>151</v>
       </c>
       <c r="O8" t="s">
         <v>29</v>
       </c>
       <c r="Q8" t="s">
-        <v>164</v>
+        <v>168</v>
       </c>
       <c r="R8" t="s">
-        <v>168</v>
+        <v>172</v>
       </c>
       <c r="S8" t="s">
-        <v>170</v>
+        <v>174</v>
       </c>
       <c r="T8" t="s">
-        <v>172</v>
+        <v>176</v>
       </c>
       <c r="U8" t="s">
         <v>92</v>
@@ -1330,7 +1342,7 @@
         <v>94</v>
       </c>
       <c r="N9" t="s">
-        <v>147</v>
+        <v>151</v>
       </c>
       <c r="O9" t="s">
         <v>30</v>
@@ -1339,16 +1351,16 @@
         <v>23895.54</v>
       </c>
       <c r="Q9" t="s">
-        <v>164</v>
+        <v>168</v>
       </c>
       <c r="R9" t="s">
-        <v>168</v>
+        <v>172</v>
       </c>
       <c r="S9" t="s">
-        <v>170</v>
+        <v>174</v>
       </c>
       <c r="T9" t="s">
-        <v>172</v>
+        <v>176</v>
       </c>
       <c r="U9" t="s">
         <v>92</v>
@@ -1365,7 +1377,7 @@
         <v>22</v>
       </c>
       <c r="D10" t="s">
-        <v>87</v>
+        <v>89</v>
       </c>
       <c r="E10" t="s">
         <v>92</v>
@@ -1374,16 +1386,16 @@
         <v>94</v>
       </c>
       <c r="G10" t="s">
-        <v>107</v>
+        <v>109</v>
       </c>
       <c r="H10" s="1">
         <v>46303</v>
       </c>
       <c r="I10" t="s">
-        <v>112</v>
+        <v>114</v>
       </c>
       <c r="N10" t="s">
-        <v>147</v>
+        <v>151</v>
       </c>
       <c r="O10" t="s">
         <v>30</v>
@@ -1392,16 +1404,16 @@
         <v>23895.54</v>
       </c>
       <c r="Q10" t="s">
-        <v>164</v>
+        <v>168</v>
       </c>
       <c r="R10" t="s">
-        <v>168</v>
+        <v>172</v>
       </c>
       <c r="S10" t="s">
-        <v>170</v>
+        <v>174</v>
       </c>
       <c r="T10" t="s">
-        <v>172</v>
+        <v>176</v>
       </c>
       <c r="U10" t="s">
         <v>92</v>
@@ -1433,22 +1445,22 @@
         <v>108</v>
       </c>
       <c r="N11" t="s">
-        <v>148</v>
+        <v>152</v>
       </c>
       <c r="O11" t="s">
         <v>31</v>
       </c>
       <c r="Q11" t="s">
-        <v>164</v>
+        <v>168</v>
       </c>
       <c r="R11" t="s">
-        <v>168</v>
+        <v>172</v>
       </c>
       <c r="S11" t="s">
-        <v>170</v>
+        <v>174</v>
       </c>
       <c r="T11" t="s">
-        <v>172</v>
+        <v>176</v>
       </c>
       <c r="U11" t="s">
         <v>92</v>
@@ -1480,22 +1492,22 @@
         <v>108</v>
       </c>
       <c r="N12" t="s">
-        <v>148</v>
+        <v>152</v>
       </c>
       <c r="O12" t="s">
         <v>32</v>
       </c>
       <c r="Q12" t="s">
-        <v>164</v>
+        <v>168</v>
       </c>
       <c r="R12" t="s">
-        <v>168</v>
+        <v>172</v>
       </c>
       <c r="S12" t="s">
-        <v>170</v>
+        <v>174</v>
       </c>
       <c r="T12" t="s">
-        <v>172</v>
+        <v>176</v>
       </c>
       <c r="U12" t="s">
         <v>92</v>
@@ -1530,13 +1542,13 @@
         <v>46079</v>
       </c>
       <c r="I13" t="s">
-        <v>114</v>
+        <v>115</v>
       </c>
       <c r="J13" t="s">
-        <v>132</v>
+        <v>135</v>
       </c>
       <c r="N13" t="s">
-        <v>146</v>
+        <v>150</v>
       </c>
       <c r="O13" t="s">
         <v>33</v>
@@ -1545,19 +1557,19 @@
         <v>1187433.02</v>
       </c>
       <c r="Q13" t="s">
-        <v>164</v>
+        <v>168</v>
       </c>
       <c r="R13" t="s">
-        <v>167</v>
+        <v>171</v>
       </c>
       <c r="S13" t="s">
-        <v>170</v>
+        <v>174</v>
       </c>
       <c r="T13" t="s">
-        <v>172</v>
+        <v>176</v>
       </c>
       <c r="U13" t="s">
-        <v>176</v>
+        <v>180</v>
       </c>
       <c r="V13" s="1">
         <v>46079</v>
@@ -1592,13 +1604,13 @@
         <v>112</v>
       </c>
       <c r="J14" t="s">
-        <v>131</v>
+        <v>134</v>
       </c>
       <c r="K14" t="s">
         <v>110</v>
       </c>
       <c r="N14" t="s">
-        <v>146</v>
+        <v>150</v>
       </c>
       <c r="O14" t="s">
         <v>34</v>
@@ -1607,19 +1619,19 @@
         <v>1000000</v>
       </c>
       <c r="Q14" t="s">
-        <v>164</v>
+        <v>168</v>
       </c>
       <c r="R14" t="s">
-        <v>167</v>
+        <v>171</v>
       </c>
       <c r="S14" t="s">
-        <v>170</v>
+        <v>174</v>
       </c>
       <c r="T14" t="s">
-        <v>172</v>
+        <v>176</v>
       </c>
       <c r="U14" t="s">
-        <v>176</v>
+        <v>180</v>
       </c>
       <c r="V14" s="1">
         <v>46352</v>
@@ -1654,13 +1666,13 @@
         <v>112</v>
       </c>
       <c r="J15" t="s">
-        <v>131</v>
+        <v>134</v>
       </c>
       <c r="K15" t="s">
         <v>110</v>
       </c>
       <c r="N15" t="s">
-        <v>146</v>
+        <v>150</v>
       </c>
       <c r="O15" t="s">
         <v>35</v>
@@ -1669,19 +1681,19 @@
         <v>1000000</v>
       </c>
       <c r="Q15" t="s">
-        <v>164</v>
+        <v>168</v>
       </c>
       <c r="R15" t="s">
-        <v>167</v>
+        <v>171</v>
       </c>
       <c r="S15" t="s">
-        <v>170</v>
+        <v>174</v>
       </c>
       <c r="T15" t="s">
-        <v>172</v>
+        <v>176</v>
       </c>
       <c r="U15" t="s">
-        <v>176</v>
+        <v>180</v>
       </c>
       <c r="V15" s="1">
         <v>46352</v>
@@ -1716,13 +1728,13 @@
         <v>112</v>
       </c>
       <c r="J16" t="s">
-        <v>131</v>
+        <v>134</v>
       </c>
       <c r="K16" t="s">
         <v>110</v>
       </c>
       <c r="N16" t="s">
-        <v>146</v>
+        <v>150</v>
       </c>
       <c r="O16" t="s">
         <v>36</v>
@@ -1731,19 +1743,19 @@
         <v>1000000</v>
       </c>
       <c r="Q16" t="s">
-        <v>164</v>
+        <v>168</v>
       </c>
       <c r="R16" t="s">
-        <v>167</v>
+        <v>171</v>
       </c>
       <c r="S16" t="s">
-        <v>170</v>
+        <v>174</v>
       </c>
       <c r="T16" t="s">
-        <v>172</v>
+        <v>176</v>
       </c>
       <c r="U16" t="s">
-        <v>176</v>
+        <v>180</v>
       </c>
       <c r="V16" s="1">
         <v>46352</v>
@@ -1778,7 +1790,7 @@
         <v>112</v>
       </c>
       <c r="J17" t="s">
-        <v>131</v>
+        <v>134</v>
       </c>
       <c r="K17" t="s">
         <v>110</v>
@@ -1793,19 +1805,19 @@
         <v>100000</v>
       </c>
       <c r="Q17" t="s">
-        <v>166</v>
+        <v>168</v>
       </c>
       <c r="R17" t="s">
-        <v>167</v>
+        <v>171</v>
       </c>
       <c r="S17" t="s">
-        <v>170</v>
+        <v>174</v>
       </c>
       <c r="T17" t="s">
-        <v>172</v>
+        <v>176</v>
       </c>
       <c r="U17" t="s">
-        <v>176</v>
+        <v>180</v>
       </c>
       <c r="V17" s="1">
         <v>46229</v>
@@ -1837,13 +1849,13 @@
         <v>46098</v>
       </c>
       <c r="I18" t="s">
-        <v>115</v>
+        <v>116</v>
       </c>
       <c r="J18" t="s">
-        <v>132</v>
+        <v>135</v>
       </c>
       <c r="N18" t="s">
-        <v>151</v>
+        <v>154</v>
       </c>
       <c r="O18" t="s">
         <v>38</v>
@@ -1852,19 +1864,19 @@
         <v>1770880.5</v>
       </c>
       <c r="Q18" t="s">
-        <v>165</v>
+        <v>169</v>
       </c>
       <c r="R18" t="s">
-        <v>168</v>
+        <v>172</v>
       </c>
       <c r="S18" t="s">
-        <v>170</v>
+        <v>174</v>
       </c>
       <c r="T18" t="s">
-        <v>174</v>
+        <v>178</v>
       </c>
       <c r="U18" t="s">
-        <v>176</v>
+        <v>180</v>
       </c>
       <c r="V18" s="1">
         <v>46107</v>
@@ -1896,10 +1908,10 @@
         <v>46076</v>
       </c>
       <c r="I19" t="s">
-        <v>116</v>
+        <v>117</v>
       </c>
       <c r="N19" t="s">
-        <v>152</v>
+        <v>155</v>
       </c>
       <c r="O19" t="s">
         <v>39</v>
@@ -1908,16 +1920,16 @@
         <v>350000</v>
       </c>
       <c r="Q19" t="s">
-        <v>165</v>
+        <v>169</v>
       </c>
       <c r="R19" t="s">
-        <v>167</v>
+        <v>171</v>
       </c>
       <c r="S19" t="s">
-        <v>170</v>
+        <v>174</v>
       </c>
       <c r="T19" t="s">
-        <v>173</v>
+        <v>177</v>
       </c>
       <c r="U19" t="s">
         <v>92</v>
@@ -1952,10 +1964,10 @@
         <v>46076</v>
       </c>
       <c r="I20" t="s">
-        <v>116</v>
+        <v>117</v>
       </c>
       <c r="N20" t="s">
-        <v>152</v>
+        <v>155</v>
       </c>
       <c r="O20" t="s">
         <v>40</v>
@@ -1964,16 +1976,16 @@
         <v>350000</v>
       </c>
       <c r="Q20" t="s">
-        <v>165</v>
+        <v>169</v>
       </c>
       <c r="R20" t="s">
-        <v>167</v>
+        <v>171</v>
       </c>
       <c r="S20" t="s">
-        <v>170</v>
+        <v>174</v>
       </c>
       <c r="T20" t="s">
-        <v>173</v>
+        <v>177</v>
       </c>
       <c r="U20" t="s">
         <v>92</v>
@@ -2002,7 +2014,7 @@
         <v>94</v>
       </c>
       <c r="N21" t="s">
-        <v>153</v>
+        <v>156</v>
       </c>
       <c r="O21" t="s">
         <v>41</v>
@@ -2011,16 +2023,16 @@
         <v>1000000</v>
       </c>
       <c r="Q21" t="s">
-        <v>165</v>
+        <v>169</v>
       </c>
       <c r="R21" t="s">
-        <v>167</v>
+        <v>171</v>
       </c>
       <c r="S21" t="s">
-        <v>170</v>
+        <v>174</v>
       </c>
       <c r="T21" t="s">
-        <v>173</v>
+        <v>177</v>
       </c>
       <c r="U21" t="s">
         <v>92</v>
@@ -2052,22 +2064,22 @@
         <v>108</v>
       </c>
       <c r="N22" t="s">
-        <v>146</v>
+        <v>150</v>
       </c>
       <c r="O22" t="s">
         <v>42</v>
       </c>
       <c r="Q22" t="s">
-        <v>164</v>
+        <v>168</v>
       </c>
       <c r="R22" t="s">
-        <v>167</v>
+        <v>171</v>
       </c>
       <c r="S22" t="s">
-        <v>170</v>
+        <v>174</v>
       </c>
       <c r="T22" t="s">
-        <v>172</v>
+        <v>176</v>
       </c>
       <c r="U22" t="s">
         <v>92</v>
@@ -2099,22 +2111,22 @@
         <v>108</v>
       </c>
       <c r="N23" t="s">
-        <v>147</v>
+        <v>151</v>
       </c>
       <c r="O23" t="s">
         <v>43</v>
       </c>
       <c r="Q23" t="s">
-        <v>164</v>
+        <v>168</v>
       </c>
       <c r="R23" t="s">
-        <v>168</v>
+        <v>172</v>
       </c>
       <c r="S23" t="s">
-        <v>170</v>
+        <v>174</v>
       </c>
       <c r="T23" t="s">
-        <v>172</v>
+        <v>176</v>
       </c>
       <c r="U23" t="s">
         <v>92</v>
@@ -2146,22 +2158,22 @@
         <v>108</v>
       </c>
       <c r="N24" t="s">
-        <v>147</v>
+        <v>151</v>
       </c>
       <c r="O24" t="s">
         <v>44</v>
       </c>
       <c r="Q24" t="s">
-        <v>164</v>
+        <v>168</v>
       </c>
       <c r="R24" t="s">
-        <v>168</v>
+        <v>172</v>
       </c>
       <c r="S24" t="s">
-        <v>170</v>
+        <v>174</v>
       </c>
       <c r="T24" t="s">
-        <v>172</v>
+        <v>176</v>
       </c>
       <c r="U24" t="s">
         <v>92</v>
@@ -2196,13 +2208,13 @@
         <v>46119</v>
       </c>
       <c r="I25" t="s">
-        <v>117</v>
+        <v>118</v>
       </c>
       <c r="J25" t="s">
-        <v>133</v>
+        <v>136</v>
       </c>
       <c r="N25" t="s">
-        <v>151</v>
+        <v>154</v>
       </c>
       <c r="O25" t="s">
         <v>45</v>
@@ -2211,19 +2223,19 @@
         <v>1704503</v>
       </c>
       <c r="Q25" t="s">
-        <v>165</v>
+        <v>169</v>
       </c>
       <c r="R25" t="s">
-        <v>168</v>
+        <v>172</v>
       </c>
       <c r="S25" t="s">
-        <v>170</v>
+        <v>174</v>
       </c>
       <c r="T25" t="s">
-        <v>174</v>
+        <v>178</v>
       </c>
       <c r="U25" t="s">
-        <v>176</v>
+        <v>180</v>
       </c>
       <c r="V25" s="1">
         <v>46138</v>
@@ -2255,10 +2267,10 @@
         <v>46121</v>
       </c>
       <c r="I26" t="s">
-        <v>118</v>
+        <v>119</v>
       </c>
       <c r="N26" t="s">
-        <v>154</v>
+        <v>157</v>
       </c>
       <c r="O26" t="s">
         <v>46</v>
@@ -2267,16 +2279,16 @@
         <v>3799000</v>
       </c>
       <c r="Q26" t="s">
-        <v>165</v>
+        <v>169</v>
       </c>
       <c r="R26" t="s">
-        <v>168</v>
+        <v>172</v>
       </c>
       <c r="S26" t="s">
-        <v>170</v>
+        <v>174</v>
       </c>
       <c r="T26" t="s">
-        <v>173</v>
+        <v>177</v>
       </c>
       <c r="U26" t="s">
         <v>92</v>
@@ -2311,10 +2323,10 @@
         <v>46076</v>
       </c>
       <c r="I27" t="s">
-        <v>119</v>
+        <v>120</v>
       </c>
       <c r="N27" t="s">
-        <v>154</v>
+        <v>157</v>
       </c>
       <c r="O27" t="s">
         <v>46</v>
@@ -2323,16 +2335,16 @@
         <v>1000</v>
       </c>
       <c r="Q27" t="s">
-        <v>165</v>
+        <v>169</v>
       </c>
       <c r="R27" t="s">
-        <v>167</v>
+        <v>171</v>
       </c>
       <c r="S27" t="s">
-        <v>170</v>
+        <v>174</v>
       </c>
       <c r="T27" t="s">
-        <v>173</v>
+        <v>177</v>
       </c>
       <c r="U27" t="s">
         <v>92</v>
@@ -2370,10 +2382,10 @@
         <v>112</v>
       </c>
       <c r="J28" t="s">
-        <v>131</v>
+        <v>134</v>
       </c>
       <c r="K28" t="s">
-        <v>110</v>
+        <v>144</v>
       </c>
       <c r="N28" t="s">
         <v>150</v>
@@ -2385,19 +2397,19 @@
         <v>100000</v>
       </c>
       <c r="Q28" t="s">
-        <v>166</v>
+        <v>168</v>
       </c>
       <c r="R28" t="s">
-        <v>167</v>
+        <v>171</v>
       </c>
       <c r="S28" t="s">
-        <v>170</v>
+        <v>174</v>
       </c>
       <c r="T28" t="s">
-        <v>172</v>
+        <v>176</v>
       </c>
       <c r="U28" t="s">
-        <v>176</v>
+        <v>180</v>
       </c>
       <c r="V28" s="1">
         <v>46291</v>
@@ -2429,13 +2441,13 @@
         <v>46199</v>
       </c>
       <c r="I29" t="s">
-        <v>120</v>
+        <v>121</v>
       </c>
       <c r="J29" t="s">
-        <v>134</v>
+        <v>137</v>
       </c>
       <c r="N29" t="s">
-        <v>151</v>
+        <v>154</v>
       </c>
       <c r="O29" t="s">
         <v>48</v>
@@ -2444,19 +2456,19 @@
         <v>150000</v>
       </c>
       <c r="Q29" t="s">
-        <v>165</v>
+        <v>169</v>
       </c>
       <c r="R29" t="s">
-        <v>168</v>
+        <v>172</v>
       </c>
       <c r="S29" t="s">
-        <v>170</v>
+        <v>174</v>
       </c>
       <c r="T29" t="s">
-        <v>173</v>
+        <v>177</v>
       </c>
       <c r="U29" t="s">
-        <v>176</v>
+        <v>180</v>
       </c>
       <c r="V29" s="1">
         <v>46199</v>
@@ -2488,13 +2500,13 @@
         <v>46199</v>
       </c>
       <c r="I30" t="s">
-        <v>120</v>
+        <v>121</v>
       </c>
       <c r="J30" t="s">
-        <v>134</v>
+        <v>137</v>
       </c>
       <c r="N30" t="s">
-        <v>151</v>
+        <v>154</v>
       </c>
       <c r="O30" t="s">
         <v>49</v>
@@ -2503,19 +2515,19 @@
         <v>150000</v>
       </c>
       <c r="Q30" t="s">
-        <v>165</v>
+        <v>169</v>
       </c>
       <c r="R30" t="s">
-        <v>168</v>
+        <v>172</v>
       </c>
       <c r="S30" t="s">
-        <v>170</v>
+        <v>174</v>
       </c>
       <c r="T30" t="s">
-        <v>173</v>
+        <v>177</v>
       </c>
       <c r="U30" t="s">
-        <v>176</v>
+        <v>180</v>
       </c>
       <c r="V30" s="1">
         <v>46199</v>
@@ -2547,13 +2559,13 @@
         <v>46199</v>
       </c>
       <c r="I31" t="s">
-        <v>121</v>
+        <v>122</v>
       </c>
       <c r="J31" t="s">
-        <v>134</v>
+        <v>137</v>
       </c>
       <c r="N31" t="s">
-        <v>151</v>
+        <v>154</v>
       </c>
       <c r="O31" t="s">
         <v>50</v>
@@ -2562,19 +2574,19 @@
         <v>18462.36</v>
       </c>
       <c r="Q31" t="s">
-        <v>165</v>
+        <v>169</v>
       </c>
       <c r="R31" t="s">
-        <v>168</v>
+        <v>172</v>
       </c>
       <c r="S31" t="s">
-        <v>170</v>
+        <v>174</v>
       </c>
       <c r="T31" t="s">
-        <v>173</v>
+        <v>177</v>
       </c>
       <c r="U31" t="s">
-        <v>176</v>
+        <v>180</v>
       </c>
       <c r="V31" s="1">
         <v>46199</v>
@@ -2606,13 +2618,13 @@
         <v>46199</v>
       </c>
       <c r="I32" t="s">
-        <v>120</v>
+        <v>121</v>
       </c>
       <c r="J32" t="s">
-        <v>134</v>
+        <v>137</v>
       </c>
       <c r="N32" t="s">
-        <v>151</v>
+        <v>154</v>
       </c>
       <c r="O32" t="s">
         <v>50</v>
@@ -2621,19 +2633,19 @@
         <v>324166.14</v>
       </c>
       <c r="Q32" t="s">
-        <v>165</v>
+        <v>169</v>
       </c>
       <c r="R32" t="s">
-        <v>168</v>
+        <v>172</v>
       </c>
       <c r="S32" t="s">
-        <v>170</v>
+        <v>174</v>
       </c>
       <c r="T32" t="s">
-        <v>173</v>
+        <v>177</v>
       </c>
       <c r="U32" t="s">
-        <v>176</v>
+        <v>180</v>
       </c>
       <c r="V32" s="1">
         <v>46199</v>
@@ -2659,13 +2671,13 @@
         <v>94</v>
       </c>
       <c r="J33" t="s">
-        <v>135</v>
+        <v>138</v>
       </c>
       <c r="K33" t="s">
-        <v>141</v>
+        <v>145</v>
       </c>
       <c r="N33" t="s">
-        <v>151</v>
+        <v>154</v>
       </c>
       <c r="O33" t="s">
         <v>51</v>
@@ -2674,19 +2686,19 @@
         <v>30000</v>
       </c>
       <c r="Q33" t="s">
-        <v>165</v>
+        <v>169</v>
       </c>
       <c r="R33" t="s">
-        <v>168</v>
+        <v>172</v>
       </c>
       <c r="S33" t="s">
-        <v>170</v>
+        <v>174</v>
       </c>
       <c r="T33" t="s">
-        <v>173</v>
+        <v>177</v>
       </c>
       <c r="U33" t="s">
-        <v>176</v>
+        <v>180</v>
       </c>
       <c r="V33" s="1">
         <v>46291</v>
@@ -2718,13 +2730,13 @@
         <v>46191</v>
       </c>
       <c r="I34" t="s">
-        <v>122</v>
+        <v>123</v>
       </c>
       <c r="J34" t="s">
-        <v>136</v>
+        <v>139</v>
       </c>
       <c r="N34" t="s">
-        <v>151</v>
+        <v>154</v>
       </c>
       <c r="O34" t="s">
         <v>52</v>
@@ -2733,19 +2745,19 @@
         <v>1496713.48</v>
       </c>
       <c r="Q34" t="s">
-        <v>165</v>
+        <v>169</v>
       </c>
       <c r="R34" t="s">
-        <v>168</v>
+        <v>172</v>
       </c>
       <c r="S34" t="s">
-        <v>170</v>
+        <v>174</v>
       </c>
       <c r="T34" t="s">
-        <v>174</v>
+        <v>178</v>
       </c>
       <c r="U34" t="s">
-        <v>176</v>
+        <v>180</v>
       </c>
       <c r="V34" s="1">
         <v>46199</v>
@@ -2777,10 +2789,10 @@
         <v>46119</v>
       </c>
       <c r="I35" t="s">
-        <v>117</v>
+        <v>118</v>
       </c>
       <c r="N35" t="s">
-        <v>151</v>
+        <v>154</v>
       </c>
       <c r="O35" t="s">
         <v>52</v>
@@ -2789,19 +2801,19 @@
         <v>207789.52</v>
       </c>
       <c r="Q35" t="s">
-        <v>165</v>
+        <v>169</v>
       </c>
       <c r="R35" t="s">
-        <v>168</v>
+        <v>172</v>
       </c>
       <c r="S35" t="s">
-        <v>170</v>
+        <v>174</v>
       </c>
       <c r="T35" t="s">
-        <v>174</v>
+        <v>178</v>
       </c>
       <c r="U35" t="s">
-        <v>176</v>
+        <v>180</v>
       </c>
       <c r="V35" s="1">
         <v>46138</v>
@@ -2833,10 +2845,10 @@
         <v>46213</v>
       </c>
       <c r="I36" t="s">
-        <v>123</v>
+        <v>124</v>
       </c>
       <c r="N36" t="s">
-        <v>154</v>
+        <v>157</v>
       </c>
       <c r="O36" t="s">
         <v>53</v>
@@ -2845,16 +2857,16 @@
         <v>962290.8</v>
       </c>
       <c r="Q36" t="s">
-        <v>165</v>
+        <v>169</v>
       </c>
       <c r="R36" t="s">
-        <v>167</v>
+        <v>171</v>
       </c>
       <c r="S36" t="s">
-        <v>170</v>
+        <v>174</v>
       </c>
       <c r="T36" t="s">
-        <v>173</v>
+        <v>177</v>
       </c>
       <c r="U36" t="s">
         <v>92</v>
@@ -2889,10 +2901,10 @@
         <v>46175</v>
       </c>
       <c r="I37" t="s">
-        <v>124</v>
+        <v>125</v>
       </c>
       <c r="N37" t="s">
-        <v>154</v>
+        <v>157</v>
       </c>
       <c r="O37" t="s">
         <v>53</v>
@@ -2901,16 +2913,16 @@
         <v>798776.97</v>
       </c>
       <c r="Q37" t="s">
-        <v>165</v>
+        <v>169</v>
       </c>
       <c r="R37" t="s">
-        <v>168</v>
+        <v>172</v>
       </c>
       <c r="S37" t="s">
-        <v>170</v>
+        <v>174</v>
       </c>
       <c r="T37" t="s">
-        <v>173</v>
+        <v>177</v>
       </c>
       <c r="U37" t="s">
         <v>92</v>
@@ -2945,10 +2957,10 @@
         <v>46213</v>
       </c>
       <c r="I38" t="s">
-        <v>123</v>
+        <v>124</v>
       </c>
       <c r="N38" t="s">
-        <v>154</v>
+        <v>157</v>
       </c>
       <c r="O38" t="s">
         <v>53</v>
@@ -2957,16 +2969,16 @@
         <v>1530656.62</v>
       </c>
       <c r="Q38" t="s">
-        <v>165</v>
+        <v>169</v>
       </c>
       <c r="R38" t="s">
-        <v>167</v>
+        <v>171</v>
       </c>
       <c r="S38" t="s">
-        <v>170</v>
+        <v>174</v>
       </c>
       <c r="T38" t="s">
-        <v>173</v>
+        <v>177</v>
       </c>
       <c r="U38" t="s">
         <v>92</v>
@@ -3001,10 +3013,10 @@
         <v>46199</v>
       </c>
       <c r="I39" t="s">
-        <v>125</v>
+        <v>126</v>
       </c>
       <c r="N39" t="s">
-        <v>154</v>
+        <v>157</v>
       </c>
       <c r="O39" t="s">
         <v>53</v>
@@ -3013,16 +3025,16 @@
         <v>72958.08</v>
       </c>
       <c r="Q39" t="s">
-        <v>165</v>
+        <v>169</v>
       </c>
       <c r="R39" t="s">
-        <v>167</v>
+        <v>171</v>
       </c>
       <c r="S39" t="s">
-        <v>170</v>
+        <v>174</v>
       </c>
       <c r="T39" t="s">
-        <v>173</v>
+        <v>177</v>
       </c>
       <c r="U39" t="s">
         <v>92</v>
@@ -3057,10 +3069,10 @@
         <v>46199</v>
       </c>
       <c r="I40" t="s">
-        <v>125</v>
+        <v>126</v>
       </c>
       <c r="N40" t="s">
-        <v>154</v>
+        <v>157</v>
       </c>
       <c r="O40" t="s">
         <v>53</v>
@@ -3069,16 +3081,16 @@
         <v>8916</v>
       </c>
       <c r="Q40" t="s">
-        <v>165</v>
+        <v>169</v>
       </c>
       <c r="R40" t="s">
-        <v>167</v>
+        <v>171</v>
       </c>
       <c r="S40" t="s">
-        <v>170</v>
+        <v>174</v>
       </c>
       <c r="T40" t="s">
-        <v>173</v>
+        <v>177</v>
       </c>
       <c r="U40" t="s">
         <v>92</v>
@@ -3113,10 +3125,10 @@
         <v>46204</v>
       </c>
       <c r="I41" t="s">
-        <v>125</v>
+        <v>126</v>
       </c>
       <c r="N41" t="s">
-        <v>154</v>
+        <v>157</v>
       </c>
       <c r="O41" t="s">
         <v>53</v>
@@ -3125,16 +3137,16 @@
         <v>425178.5</v>
       </c>
       <c r="Q41" t="s">
-        <v>165</v>
+        <v>169</v>
       </c>
       <c r="R41" t="s">
-        <v>167</v>
+        <v>171</v>
       </c>
       <c r="S41" t="s">
-        <v>170</v>
+        <v>174</v>
       </c>
       <c r="T41" t="s">
-        <v>173</v>
+        <v>177</v>
       </c>
       <c r="U41" t="s">
         <v>92</v>
@@ -3169,10 +3181,10 @@
         <v>46244</v>
       </c>
       <c r="I42" t="s">
-        <v>126</v>
+        <v>127</v>
       </c>
       <c r="N42" t="s">
-        <v>154</v>
+        <v>157</v>
       </c>
       <c r="O42" t="s">
         <v>53</v>
@@ -3181,16 +3193,16 @@
         <v>1223.03</v>
       </c>
       <c r="Q42" t="s">
-        <v>165</v>
+        <v>169</v>
       </c>
       <c r="R42" t="s">
-        <v>167</v>
+        <v>171</v>
       </c>
       <c r="S42" t="s">
-        <v>170</v>
+        <v>174</v>
       </c>
       <c r="T42" t="s">
-        <v>173</v>
+        <v>177</v>
       </c>
       <c r="U42" t="s">
         <v>92</v>
@@ -3219,22 +3231,22 @@
         <v>108</v>
       </c>
       <c r="N43" t="s">
-        <v>154</v>
+        <v>157</v>
       </c>
       <c r="O43" t="s">
         <v>54</v>
       </c>
       <c r="Q43" t="s">
-        <v>165</v>
+        <v>169</v>
       </c>
       <c r="R43" t="s">
-        <v>167</v>
+        <v>171</v>
       </c>
       <c r="S43" t="s">
-        <v>171</v>
+        <v>175</v>
       </c>
       <c r="T43" t="s">
-        <v>173</v>
+        <v>177</v>
       </c>
       <c r="U43" t="s">
         <v>92</v>
@@ -3269,10 +3281,10 @@
         <v>46191</v>
       </c>
       <c r="I44" t="s">
-        <v>127</v>
+        <v>128</v>
       </c>
       <c r="N44" t="s">
-        <v>152</v>
+        <v>155</v>
       </c>
       <c r="O44" t="s">
         <v>55</v>
@@ -3281,16 +3293,16 @@
         <v>400000</v>
       </c>
       <c r="Q44" t="s">
-        <v>165</v>
+        <v>169</v>
       </c>
       <c r="R44" t="s">
-        <v>167</v>
+        <v>171</v>
       </c>
       <c r="S44" t="s">
-        <v>170</v>
+        <v>174</v>
       </c>
       <c r="T44" t="s">
-        <v>173</v>
+        <v>177</v>
       </c>
       <c r="U44" t="s">
         <v>92</v>
@@ -3325,10 +3337,10 @@
         <v>46191</v>
       </c>
       <c r="I45" t="s">
-        <v>127</v>
+        <v>128</v>
       </c>
       <c r="N45" t="s">
-        <v>152</v>
+        <v>155</v>
       </c>
       <c r="O45" t="s">
         <v>56</v>
@@ -3337,16 +3349,16 @@
         <v>400000</v>
       </c>
       <c r="Q45" t="s">
-        <v>165</v>
+        <v>169</v>
       </c>
       <c r="R45" t="s">
-        <v>167</v>
+        <v>171</v>
       </c>
       <c r="S45" t="s">
-        <v>170</v>
+        <v>174</v>
       </c>
       <c r="T45" t="s">
-        <v>173</v>
+        <v>177</v>
       </c>
       <c r="U45" t="s">
         <v>92</v>
@@ -3381,13 +3393,13 @@
         <v>46213</v>
       </c>
       <c r="I46" t="s">
-        <v>122</v>
+        <v>123</v>
       </c>
       <c r="J46" t="s">
-        <v>137</v>
+        <v>140</v>
       </c>
       <c r="N46" t="s">
-        <v>151</v>
+        <v>154</v>
       </c>
       <c r="O46" t="s">
         <v>57</v>
@@ -3396,19 +3408,19 @@
         <v>173846.38</v>
       </c>
       <c r="Q46" t="s">
-        <v>165</v>
+        <v>169</v>
       </c>
       <c r="R46" t="s">
-        <v>168</v>
+        <v>172</v>
       </c>
       <c r="S46" t="s">
-        <v>170</v>
+        <v>174</v>
       </c>
       <c r="T46" t="s">
-        <v>174</v>
+        <v>178</v>
       </c>
       <c r="U46" t="s">
-        <v>176</v>
+        <v>180</v>
       </c>
       <c r="V46" s="1">
         <v>46229</v>
@@ -3440,10 +3452,10 @@
         <v>46210</v>
       </c>
       <c r="I47" t="s">
-        <v>121</v>
+        <v>122</v>
       </c>
       <c r="N47" t="s">
-        <v>151</v>
+        <v>154</v>
       </c>
       <c r="O47" t="s">
         <v>57</v>
@@ -3452,19 +3464,19 @@
         <v>1530656.62</v>
       </c>
       <c r="Q47" t="s">
-        <v>165</v>
+        <v>169</v>
       </c>
       <c r="R47" t="s">
-        <v>168</v>
+        <v>172</v>
       </c>
       <c r="S47" t="s">
-        <v>170</v>
+        <v>174</v>
       </c>
       <c r="T47" t="s">
-        <v>174</v>
+        <v>178</v>
       </c>
       <c r="U47" t="s">
-        <v>176</v>
+        <v>180</v>
       </c>
       <c r="V47" s="1">
         <v>46229</v>
@@ -3490,7 +3502,7 @@
         <v>94</v>
       </c>
       <c r="N48" t="s">
-        <v>153</v>
+        <v>156</v>
       </c>
       <c r="O48" t="s">
         <v>58</v>
@@ -3499,16 +3511,16 @@
         <v>1000000</v>
       </c>
       <c r="Q48" t="s">
-        <v>165</v>
+        <v>169</v>
       </c>
       <c r="R48" t="s">
-        <v>167</v>
+        <v>171</v>
       </c>
       <c r="S48" t="s">
-        <v>170</v>
+        <v>174</v>
       </c>
       <c r="T48" t="s">
-        <v>173</v>
+        <v>177</v>
       </c>
       <c r="U48" t="s">
         <v>92</v>
@@ -3546,13 +3558,13 @@
         <v>112</v>
       </c>
       <c r="J49" t="s">
-        <v>131</v>
+        <v>134</v>
       </c>
       <c r="K49" t="s">
         <v>110</v>
       </c>
       <c r="N49" t="s">
-        <v>146</v>
+        <v>150</v>
       </c>
       <c r="O49" t="s">
         <v>59</v>
@@ -3561,19 +3573,19 @@
         <v>958040</v>
       </c>
       <c r="Q49" t="s">
-        <v>164</v>
+        <v>168</v>
       </c>
       <c r="R49" t="s">
-        <v>167</v>
+        <v>171</v>
       </c>
       <c r="S49" t="s">
-        <v>170</v>
+        <v>174</v>
       </c>
       <c r="T49" t="s">
-        <v>172</v>
+        <v>176</v>
       </c>
       <c r="U49" t="s">
-        <v>176</v>
+        <v>180</v>
       </c>
       <c r="V49" s="1">
         <v>46291</v>
@@ -3605,13 +3617,13 @@
         <v>46176</v>
       </c>
       <c r="I50" t="s">
-        <v>128</v>
+        <v>129</v>
       </c>
       <c r="J50" t="s">
-        <v>138</v>
+        <v>141</v>
       </c>
       <c r="N50" t="s">
-        <v>146</v>
+        <v>150</v>
       </c>
       <c r="O50" t="s">
         <v>59</v>
@@ -3620,19 +3632,19 @@
         <v>41730.64</v>
       </c>
       <c r="Q50" t="s">
-        <v>164</v>
+        <v>168</v>
       </c>
       <c r="R50" t="s">
-        <v>169</v>
+        <v>173</v>
       </c>
       <c r="S50" t="s">
-        <v>170</v>
+        <v>174</v>
       </c>
       <c r="T50" t="s">
-        <v>172</v>
+        <v>176</v>
       </c>
       <c r="U50" t="s">
-        <v>176</v>
+        <v>180</v>
       </c>
       <c r="V50" s="1">
         <v>46199</v>
@@ -3661,13 +3673,13 @@
         <v>110</v>
       </c>
       <c r="J51" t="s">
-        <v>137</v>
+        <v>140</v>
       </c>
       <c r="K51" t="s">
-        <v>142</v>
+        <v>146</v>
       </c>
       <c r="N51" t="s">
-        <v>151</v>
+        <v>154</v>
       </c>
       <c r="O51" t="s">
         <v>60</v>
@@ -3676,19 +3688,19 @@
         <v>608623.25</v>
       </c>
       <c r="Q51" t="s">
-        <v>165</v>
+        <v>169</v>
       </c>
       <c r="R51" t="s">
-        <v>168</v>
+        <v>172</v>
       </c>
       <c r="S51" t="s">
-        <v>170</v>
+        <v>174</v>
       </c>
       <c r="T51" t="s">
-        <v>174</v>
+        <v>178</v>
       </c>
       <c r="U51" t="s">
-        <v>176</v>
+        <v>180</v>
       </c>
       <c r="V51" s="1">
         <v>46260</v>
@@ -3720,16 +3732,16 @@
         <v>46295</v>
       </c>
       <c r="I52" t="s">
-        <v>122</v>
+        <v>123</v>
       </c>
       <c r="J52" t="s">
-        <v>137</v>
+        <v>140</v>
       </c>
       <c r="K52" t="s">
-        <v>140</v>
+        <v>143</v>
       </c>
       <c r="N52" t="s">
-        <v>151</v>
+        <v>154</v>
       </c>
       <c r="O52" t="s">
         <v>61</v>
@@ -3738,19 +3750,19 @@
         <v>66366.75999999999</v>
       </c>
       <c r="Q52" t="s">
-        <v>165</v>
+        <v>169</v>
       </c>
       <c r="R52" t="s">
-        <v>168</v>
+        <v>172</v>
       </c>
       <c r="S52" t="s">
-        <v>170</v>
+        <v>174</v>
       </c>
       <c r="T52" t="s">
-        <v>174</v>
+        <v>178</v>
       </c>
       <c r="U52" t="s">
-        <v>176</v>
+        <v>180</v>
       </c>
       <c r="V52" s="1">
         <v>46291</v>
@@ -3776,13 +3788,13 @@
         <v>94</v>
       </c>
       <c r="J53" t="s">
-        <v>135</v>
+        <v>138</v>
       </c>
       <c r="K53" t="s">
-        <v>141</v>
+        <v>145</v>
       </c>
       <c r="N53" t="s">
-        <v>151</v>
+        <v>154</v>
       </c>
       <c r="O53" t="s">
         <v>62</v>
@@ -3791,19 +3803,19 @@
         <v>1586760.42</v>
       </c>
       <c r="Q53" t="s">
-        <v>165</v>
+        <v>169</v>
       </c>
       <c r="R53" t="s">
-        <v>168</v>
+        <v>172</v>
       </c>
       <c r="S53" t="s">
-        <v>170</v>
+        <v>174</v>
       </c>
       <c r="T53" t="s">
-        <v>174</v>
+        <v>178</v>
       </c>
       <c r="U53" t="s">
-        <v>176</v>
+        <v>180</v>
       </c>
       <c r="V53" s="1">
         <v>46321</v>
@@ -3835,10 +3847,10 @@
         <v>46227</v>
       </c>
       <c r="I54" t="s">
-        <v>129</v>
+        <v>130</v>
       </c>
       <c r="N54" t="s">
-        <v>151</v>
+        <v>154</v>
       </c>
       <c r="O54" t="s">
         <v>60</v>
@@ -3847,19 +3859,19 @@
         <v>236343.68</v>
       </c>
       <c r="Q54" t="s">
-        <v>165</v>
+        <v>169</v>
       </c>
       <c r="R54" t="s">
-        <v>168</v>
+        <v>172</v>
       </c>
       <c r="S54" t="s">
-        <v>170</v>
+        <v>174</v>
       </c>
       <c r="T54" t="s">
-        <v>174</v>
+        <v>178</v>
       </c>
       <c r="U54" t="s">
-        <v>176</v>
+        <v>180</v>
       </c>
       <c r="V54" s="1">
         <v>46229</v>
@@ -3888,10 +3900,10 @@
         <v>46280</v>
       </c>
       <c r="I55" t="s">
-        <v>121</v>
+        <v>122</v>
       </c>
       <c r="N55" t="s">
-        <v>151</v>
+        <v>154</v>
       </c>
       <c r="O55" t="s">
         <v>61</v>
@@ -3900,19 +3912,19 @@
         <v>1145462.93</v>
       </c>
       <c r="Q55" t="s">
-        <v>165</v>
+        <v>169</v>
       </c>
       <c r="R55" t="s">
-        <v>168</v>
+        <v>172</v>
       </c>
       <c r="S55" t="s">
-        <v>170</v>
+        <v>174</v>
       </c>
       <c r="T55" t="s">
-        <v>174</v>
+        <v>178</v>
       </c>
       <c r="U55" t="s">
-        <v>176</v>
+        <v>180</v>
       </c>
       <c r="V55" s="1">
         <v>46291</v>
@@ -3941,10 +3953,10 @@
         <v>46280</v>
       </c>
       <c r="I56" t="s">
-        <v>121</v>
+        <v>122</v>
       </c>
       <c r="N56" t="s">
-        <v>151</v>
+        <v>154</v>
       </c>
       <c r="O56" t="s">
         <v>60</v>
@@ -3953,19 +3965,19 @@
         <v>859536.0699999999</v>
       </c>
       <c r="Q56" t="s">
-        <v>165</v>
+        <v>169</v>
       </c>
       <c r="R56" t="s">
-        <v>168</v>
+        <v>172</v>
       </c>
       <c r="S56" t="s">
-        <v>170</v>
+        <v>174</v>
       </c>
       <c r="T56" t="s">
-        <v>174</v>
+        <v>178</v>
       </c>
       <c r="U56" t="s">
-        <v>176</v>
+        <v>180</v>
       </c>
       <c r="V56" s="1">
         <v>46260</v>
@@ -3994,10 +4006,10 @@
         <v>46295</v>
       </c>
       <c r="I57" t="s">
-        <v>115</v>
+        <v>116</v>
       </c>
       <c r="N57" t="s">
-        <v>151</v>
+        <v>154</v>
       </c>
       <c r="O57" t="s">
         <v>61</v>
@@ -4006,19 +4018,19 @@
         <v>389619.06</v>
       </c>
       <c r="Q57" t="s">
-        <v>165</v>
+        <v>169</v>
       </c>
       <c r="R57" t="s">
-        <v>168</v>
+        <v>172</v>
       </c>
       <c r="S57" t="s">
-        <v>170</v>
+        <v>174</v>
       </c>
       <c r="T57" t="s">
-        <v>174</v>
+        <v>178</v>
       </c>
       <c r="U57" t="s">
-        <v>176</v>
+        <v>180</v>
       </c>
       <c r="V57" s="1">
         <v>46291</v>
@@ -4047,10 +4059,10 @@
         <v>46295</v>
       </c>
       <c r="I58" t="s">
-        <v>130</v>
+        <v>131</v>
       </c>
       <c r="N58" t="s">
-        <v>151</v>
+        <v>154</v>
       </c>
       <c r="O58" t="s">
         <v>61</v>
@@ -4059,19 +4071,19 @@
         <v>103054.25</v>
       </c>
       <c r="Q58" t="s">
-        <v>165</v>
+        <v>169</v>
       </c>
       <c r="R58" t="s">
-        <v>168</v>
+        <v>172</v>
       </c>
       <c r="S58" t="s">
-        <v>170</v>
+        <v>174</v>
       </c>
       <c r="T58" t="s">
-        <v>174</v>
+        <v>178</v>
       </c>
       <c r="U58" t="s">
-        <v>176</v>
+        <v>180</v>
       </c>
       <c r="V58" s="1">
         <v>46291</v>
@@ -4085,7 +4097,7 @@
         <v>22</v>
       </c>
       <c r="D59" t="s">
-        <v>88</v>
+        <v>89</v>
       </c>
       <c r="E59" t="s">
         <v>92</v>
@@ -4094,10 +4106,16 @@
         <v>105</v>
       </c>
       <c r="G59" t="s">
-        <v>110</v>
+        <v>109</v>
+      </c>
+      <c r="H59" s="1">
+        <v>46304</v>
+      </c>
+      <c r="I59" t="s">
+        <v>132</v>
       </c>
       <c r="N59" t="s">
-        <v>151</v>
+        <v>154</v>
       </c>
       <c r="O59" t="s">
         <v>62</v>
@@ -4106,19 +4124,19 @@
         <v>117742.58</v>
       </c>
       <c r="Q59" t="s">
-        <v>165</v>
+        <v>169</v>
       </c>
       <c r="R59" t="s">
-        <v>168</v>
+        <v>172</v>
       </c>
       <c r="S59" t="s">
-        <v>170</v>
+        <v>174</v>
       </c>
       <c r="T59" t="s">
-        <v>174</v>
+        <v>178</v>
       </c>
       <c r="U59" t="s">
-        <v>176</v>
+        <v>180</v>
       </c>
       <c r="V59" s="1">
         <v>46321</v>
@@ -4150,16 +4168,16 @@
         <v>46301</v>
       </c>
       <c r="I60" t="s">
-        <v>115</v>
+        <v>116</v>
       </c>
       <c r="J60" t="s">
-        <v>131</v>
+        <v>134</v>
       </c>
       <c r="K60" t="s">
-        <v>143</v>
+        <v>147</v>
       </c>
       <c r="N60" t="s">
-        <v>151</v>
+        <v>154</v>
       </c>
       <c r="O60" t="s">
         <v>63</v>
@@ -4168,19 +4186,19 @@
         <v>1295422.28</v>
       </c>
       <c r="Q60" t="s">
-        <v>165</v>
+        <v>169</v>
       </c>
       <c r="R60" t="s">
-        <v>168</v>
+        <v>172</v>
       </c>
       <c r="S60" t="s">
-        <v>170</v>
+        <v>174</v>
       </c>
       <c r="T60" t="s">
-        <v>174</v>
+        <v>178</v>
       </c>
       <c r="U60" t="s">
-        <v>176</v>
+        <v>180</v>
       </c>
       <c r="V60" s="1">
         <v>46352</v>
@@ -4203,7 +4221,7 @@
         <v>93</v>
       </c>
       <c r="N61" t="s">
-        <v>155</v>
+        <v>158</v>
       </c>
       <c r="O61" t="s">
         <v>64</v>
@@ -4212,19 +4230,19 @@
         <v>4064.54</v>
       </c>
       <c r="Q61" t="s">
-        <v>165</v>
+        <v>169</v>
       </c>
       <c r="R61" t="s">
-        <v>169</v>
+        <v>173</v>
       </c>
       <c r="S61" t="s">
-        <v>171</v>
+        <v>175</v>
       </c>
       <c r="T61" t="s">
-        <v>172</v>
+        <v>176</v>
       </c>
       <c r="U61" t="s">
-        <v>176</v>
+        <v>180</v>
       </c>
       <c r="V61" s="1">
         <v>46107</v>
@@ -4247,7 +4265,7 @@
         <v>93</v>
       </c>
       <c r="N62" t="s">
-        <v>156</v>
+        <v>159</v>
       </c>
       <c r="O62" t="s">
         <v>65</v>
@@ -4256,19 +4274,19 @@
         <v>4227.84</v>
       </c>
       <c r="Q62" t="s">
-        <v>164</v>
+        <v>168</v>
       </c>
       <c r="R62" t="s">
-        <v>169</v>
+        <v>173</v>
       </c>
       <c r="S62" t="s">
-        <v>171</v>
+        <v>175</v>
       </c>
       <c r="T62" t="s">
-        <v>172</v>
+        <v>176</v>
       </c>
       <c r="U62" t="s">
-        <v>176</v>
+        <v>180</v>
       </c>
       <c r="V62" s="1">
         <v>46107</v>
@@ -4291,7 +4309,7 @@
         <v>93</v>
       </c>
       <c r="N63" t="s">
-        <v>157</v>
+        <v>160</v>
       </c>
       <c r="O63" t="s">
         <v>66</v>
@@ -4300,19 +4318,19 @@
         <v>9389.959999999999</v>
       </c>
       <c r="Q63" t="s">
-        <v>164</v>
+        <v>168</v>
       </c>
       <c r="R63" t="s">
-        <v>169</v>
+        <v>173</v>
       </c>
       <c r="S63" t="s">
-        <v>171</v>
+        <v>175</v>
       </c>
       <c r="T63" t="s">
-        <v>172</v>
+        <v>176</v>
       </c>
       <c r="U63" t="s">
-        <v>176</v>
+        <v>180</v>
       </c>
       <c r="V63" s="1">
         <v>46107</v>
@@ -4335,7 +4353,7 @@
         <v>93</v>
       </c>
       <c r="N64" t="s">
-        <v>158</v>
+        <v>161</v>
       </c>
       <c r="O64" t="s">
         <v>67</v>
@@ -4344,19 +4362,19 @@
         <v>1163.64</v>
       </c>
       <c r="Q64" t="s">
-        <v>166</v>
+        <v>170</v>
       </c>
       <c r="R64" t="s">
-        <v>169</v>
+        <v>173</v>
       </c>
       <c r="S64" t="s">
-        <v>171</v>
+        <v>175</v>
       </c>
       <c r="T64" t="s">
-        <v>172</v>
+        <v>176</v>
       </c>
       <c r="U64" t="s">
-        <v>176</v>
+        <v>180</v>
       </c>
       <c r="V64" s="1">
         <v>46107</v>
@@ -4379,7 +4397,7 @@
         <v>93</v>
       </c>
       <c r="N65" t="s">
-        <v>159</v>
+        <v>162</v>
       </c>
       <c r="O65" t="s">
         <v>68</v>
@@ -4388,19 +4406,19 @@
         <v>7204.82</v>
       </c>
       <c r="Q65" t="s">
-        <v>164</v>
+        <v>168</v>
       </c>
       <c r="R65" t="s">
-        <v>169</v>
+        <v>173</v>
       </c>
       <c r="S65" t="s">
-        <v>171</v>
+        <v>175</v>
       </c>
       <c r="T65" t="s">
-        <v>172</v>
+        <v>176</v>
       </c>
       <c r="U65" t="s">
-        <v>176</v>
+        <v>180</v>
       </c>
       <c r="V65" s="1">
         <v>46107</v>
@@ -4423,7 +4441,7 @@
         <v>93</v>
       </c>
       <c r="N66" t="s">
-        <v>160</v>
+        <v>163</v>
       </c>
       <c r="O66" t="s">
         <v>65</v>
@@ -4432,19 +4450,19 @@
         <v>3662.66</v>
       </c>
       <c r="Q66" t="s">
-        <v>164</v>
+        <v>168</v>
       </c>
       <c r="R66" t="s">
-        <v>169</v>
+        <v>173</v>
       </c>
       <c r="S66" t="s">
-        <v>171</v>
+        <v>175</v>
       </c>
       <c r="T66" t="s">
-        <v>172</v>
+        <v>176</v>
       </c>
       <c r="U66" t="s">
-        <v>176</v>
+        <v>180</v>
       </c>
       <c r="V66" s="1">
         <v>46107</v>
@@ -4467,7 +4485,7 @@
         <v>93</v>
       </c>
       <c r="N67" t="s">
-        <v>147</v>
+        <v>151</v>
       </c>
       <c r="O67" t="s">
         <v>69</v>
@@ -4476,16 +4494,16 @@
         <v>120000</v>
       </c>
       <c r="Q67" t="s">
-        <v>164</v>
+        <v>168</v>
       </c>
       <c r="R67" t="s">
-        <v>168</v>
+        <v>172</v>
       </c>
       <c r="S67" t="s">
-        <v>171</v>
+        <v>175</v>
       </c>
       <c r="T67" t="s">
-        <v>172</v>
+        <v>176</v>
       </c>
       <c r="U67" t="s">
         <v>92</v>
@@ -4517,22 +4535,22 @@
         <v>108</v>
       </c>
       <c r="N68" t="s">
-        <v>146</v>
+        <v>150</v>
       </c>
       <c r="O68" t="s">
         <v>70</v>
       </c>
       <c r="Q68" t="s">
-        <v>164</v>
+        <v>168</v>
       </c>
       <c r="R68" t="s">
-        <v>167</v>
+        <v>171</v>
       </c>
       <c r="S68" t="s">
-        <v>170</v>
+        <v>174</v>
       </c>
       <c r="T68" t="s">
-        <v>172</v>
+        <v>176</v>
       </c>
       <c r="U68" t="s">
         <v>92</v>
@@ -4570,7 +4588,7 @@
         <v>112</v>
       </c>
       <c r="J69" t="s">
-        <v>131</v>
+        <v>134</v>
       </c>
       <c r="K69" t="s">
         <v>110</v>
@@ -4585,19 +4603,19 @@
         <v>100000</v>
       </c>
       <c r="Q69" t="s">
-        <v>166</v>
+        <v>168</v>
       </c>
       <c r="R69" t="s">
-        <v>167</v>
+        <v>171</v>
       </c>
       <c r="S69" t="s">
-        <v>170</v>
+        <v>174</v>
       </c>
       <c r="T69" t="s">
-        <v>172</v>
+        <v>176</v>
       </c>
       <c r="U69" t="s">
-        <v>176</v>
+        <v>180</v>
       </c>
       <c r="V69" s="1">
         <v>46229</v>
@@ -4620,7 +4638,7 @@
         <v>93</v>
       </c>
       <c r="N70" t="s">
-        <v>147</v>
+        <v>151</v>
       </c>
       <c r="O70" t="s">
         <v>72</v>
@@ -4629,16 +4647,16 @@
         <v>80000</v>
       </c>
       <c r="Q70" t="s">
-        <v>164</v>
+        <v>168</v>
       </c>
       <c r="R70" t="s">
-        <v>168</v>
+        <v>172</v>
       </c>
       <c r="S70" t="s">
-        <v>171</v>
+        <v>175</v>
       </c>
       <c r="T70" t="s">
-        <v>172</v>
+        <v>176</v>
       </c>
       <c r="U70" t="s">
         <v>92</v>
@@ -4664,7 +4682,7 @@
         <v>93</v>
       </c>
       <c r="N71" t="s">
-        <v>146</v>
+        <v>150</v>
       </c>
       <c r="O71" t="s">
         <v>73</v>
@@ -4673,19 +4691,19 @@
         <v>835000</v>
       </c>
       <c r="Q71" t="s">
-        <v>164</v>
+        <v>168</v>
       </c>
       <c r="R71" t="s">
-        <v>167</v>
+        <v>171</v>
       </c>
       <c r="S71" t="s">
-        <v>171</v>
+        <v>175</v>
       </c>
       <c r="T71" t="s">
-        <v>172</v>
+        <v>176</v>
       </c>
       <c r="U71" t="s">
-        <v>176</v>
+        <v>180</v>
       </c>
       <c r="V71" s="1">
         <v>46291</v>
@@ -4708,7 +4726,7 @@
         <v>93</v>
       </c>
       <c r="N72" t="s">
-        <v>146</v>
+        <v>150</v>
       </c>
       <c r="O72" t="s">
         <v>73</v>
@@ -4717,19 +4735,19 @@
         <v>165000</v>
       </c>
       <c r="Q72" t="s">
-        <v>164</v>
+        <v>168</v>
       </c>
       <c r="R72" t="s">
-        <v>167</v>
+        <v>171</v>
       </c>
       <c r="S72" t="s">
-        <v>171</v>
+        <v>175</v>
       </c>
       <c r="T72" t="s">
-        <v>172</v>
+        <v>176</v>
       </c>
       <c r="U72" t="s">
-        <v>176</v>
+        <v>180</v>
       </c>
       <c r="V72" s="1">
         <v>46168</v>
@@ -4752,7 +4770,7 @@
         <v>93</v>
       </c>
       <c r="N73" t="s">
-        <v>146</v>
+        <v>150</v>
       </c>
       <c r="O73" t="s">
         <v>74</v>
@@ -4761,19 +4779,19 @@
         <v>1000000</v>
       </c>
       <c r="Q73" t="s">
-        <v>164</v>
+        <v>168</v>
       </c>
       <c r="R73" t="s">
-        <v>167</v>
+        <v>171</v>
       </c>
       <c r="S73" t="s">
-        <v>171</v>
+        <v>175</v>
       </c>
       <c r="T73" t="s">
-        <v>172</v>
+        <v>176</v>
       </c>
       <c r="U73" t="s">
-        <v>176</v>
+        <v>180</v>
       </c>
       <c r="V73" s="1">
         <v>46291</v>
@@ -4796,7 +4814,7 @@
         <v>93</v>
       </c>
       <c r="N74" t="s">
-        <v>146</v>
+        <v>150</v>
       </c>
       <c r="O74" t="s">
         <v>75</v>
@@ -4805,19 +4823,19 @@
         <v>1000000</v>
       </c>
       <c r="Q74" t="s">
-        <v>164</v>
+        <v>168</v>
       </c>
       <c r="R74" t="s">
-        <v>167</v>
+        <v>171</v>
       </c>
       <c r="S74" t="s">
-        <v>171</v>
+        <v>175</v>
       </c>
       <c r="T74" t="s">
-        <v>172</v>
+        <v>176</v>
       </c>
       <c r="U74" t="s">
-        <v>176</v>
+        <v>180</v>
       </c>
       <c r="V74" s="1">
         <v>46291</v>
@@ -4840,7 +4858,7 @@
         <v>93</v>
       </c>
       <c r="N75" t="s">
-        <v>150</v>
+        <v>164</v>
       </c>
       <c r="O75" t="s">
         <v>76</v>
@@ -4849,19 +4867,19 @@
         <v>100000</v>
       </c>
       <c r="Q75" t="s">
-        <v>166</v>
+        <v>170</v>
       </c>
       <c r="R75" t="s">
-        <v>167</v>
+        <v>171</v>
       </c>
       <c r="S75" t="s">
-        <v>171</v>
+        <v>175</v>
       </c>
       <c r="T75" t="s">
-        <v>172</v>
+        <v>176</v>
       </c>
       <c r="U75" t="s">
-        <v>176</v>
+        <v>180</v>
       </c>
       <c r="V75" s="1">
         <v>46291</v>
@@ -4887,7 +4905,7 @@
         <v>94</v>
       </c>
       <c r="N76" t="s">
-        <v>153</v>
+        <v>156</v>
       </c>
       <c r="O76" t="s">
         <v>77</v>
@@ -4896,16 +4914,16 @@
         <v>1000000</v>
       </c>
       <c r="Q76" t="s">
-        <v>165</v>
+        <v>169</v>
       </c>
       <c r="R76" t="s">
-        <v>167</v>
+        <v>171</v>
       </c>
       <c r="S76" t="s">
-        <v>170</v>
+        <v>174</v>
       </c>
       <c r="T76" t="s">
-        <v>173</v>
+        <v>177</v>
       </c>
       <c r="U76" t="s">
         <v>92</v>
@@ -4937,7 +4955,7 @@
         <v>111</v>
       </c>
       <c r="N77" t="s">
-        <v>151</v>
+        <v>154</v>
       </c>
       <c r="O77" t="s">
         <v>78</v>
@@ -4946,19 +4964,19 @@
         <v>1704503</v>
       </c>
       <c r="Q77" t="s">
-        <v>165</v>
+        <v>169</v>
       </c>
       <c r="R77" t="s">
-        <v>168</v>
+        <v>172</v>
       </c>
       <c r="S77" t="s">
         <v>106</v>
       </c>
       <c r="T77" t="s">
-        <v>174</v>
+        <v>178</v>
       </c>
       <c r="U77" t="s">
-        <v>176</v>
+        <v>180</v>
       </c>
       <c r="V77" s="1">
         <v>46381</v>
@@ -4987,7 +5005,7 @@
         <v>111</v>
       </c>
       <c r="N78" t="s">
-        <v>151</v>
+        <v>154</v>
       </c>
       <c r="O78" t="s">
         <v>79</v>
@@ -4996,19 +5014,19 @@
         <v>1638125.5</v>
       </c>
       <c r="Q78" t="s">
-        <v>165</v>
+        <v>169</v>
       </c>
       <c r="R78" t="s">
-        <v>168</v>
+        <v>172</v>
       </c>
       <c r="S78" t="s">
         <v>106</v>
       </c>
       <c r="T78" t="s">
-        <v>174</v>
+        <v>178</v>
       </c>
       <c r="U78" t="s">
-        <v>176</v>
+        <v>180</v>
       </c>
       <c r="V78" s="1">
         <v>46381</v>
@@ -5037,7 +5055,7 @@
         <v>111</v>
       </c>
       <c r="N79" t="s">
-        <v>149</v>
+        <v>153</v>
       </c>
       <c r="O79" t="s">
         <v>80</v>
@@ -5046,16 +5064,16 @@
         <v>3800000</v>
       </c>
       <c r="Q79" t="s">
-        <v>165</v>
+        <v>169</v>
       </c>
       <c r="R79" t="s">
-        <v>168</v>
+        <v>172</v>
       </c>
       <c r="S79" t="s">
         <v>106</v>
       </c>
       <c r="T79" t="s">
-        <v>173</v>
+        <v>177</v>
       </c>
       <c r="U79" t="s">
         <v>92</v>
@@ -5087,7 +5105,7 @@
         <v>111</v>
       </c>
       <c r="N80" t="s">
-        <v>149</v>
+        <v>153</v>
       </c>
       <c r="O80" t="s">
         <v>81</v>
@@ -5096,16 +5114,16 @@
         <v>3800000</v>
       </c>
       <c r="Q80" t="s">
-        <v>165</v>
+        <v>169</v>
       </c>
       <c r="R80" t="s">
-        <v>168</v>
+        <v>172</v>
       </c>
       <c r="S80" t="s">
         <v>106</v>
       </c>
       <c r="T80" t="s">
-        <v>173</v>
+        <v>177</v>
       </c>
       <c r="U80" t="s">
         <v>92</v>
@@ -5131,13 +5149,13 @@
         <v>93</v>
       </c>
       <c r="J81" t="s">
-        <v>139</v>
+        <v>142</v>
       </c>
       <c r="K81" t="s">
-        <v>144</v>
+        <v>148</v>
       </c>
       <c r="N81" t="s">
-        <v>154</v>
+        <v>157</v>
       </c>
       <c r="O81" t="s">
         <v>82</v>
@@ -5146,16 +5164,16 @@
         <v>3800000</v>
       </c>
       <c r="Q81" t="s">
-        <v>165</v>
+        <v>169</v>
       </c>
       <c r="R81" t="s">
-        <v>168</v>
+        <v>172</v>
       </c>
       <c r="S81" t="s">
-        <v>171</v>
+        <v>175</v>
       </c>
       <c r="T81" t="s">
-        <v>173</v>
+        <v>177</v>
       </c>
       <c r="U81" t="s">
         <v>92</v>
@@ -5181,7 +5199,7 @@
         <v>92</v>
       </c>
       <c r="N82" t="s">
-        <v>161</v>
+        <v>165</v>
       </c>
       <c r="O82" t="s">
         <v>83</v>
@@ -5190,16 +5208,16 @@
         <v>4394700</v>
       </c>
       <c r="Q82" t="s">
-        <v>164</v>
+        <v>168</v>
       </c>
       <c r="R82" t="s">
-        <v>167</v>
+        <v>171</v>
       </c>
       <c r="S82" t="s">
-        <v>171</v>
+        <v>175</v>
       </c>
       <c r="T82" t="s">
-        <v>173</v>
+        <v>177</v>
       </c>
       <c r="U82" t="s">
         <v>92</v>
@@ -5231,13 +5249,13 @@
         <v>110</v>
       </c>
       <c r="J83" t="s">
-        <v>131</v>
+        <v>134</v>
       </c>
       <c r="K83" t="s">
-        <v>140</v>
+        <v>143</v>
       </c>
       <c r="N83" t="s">
-        <v>151</v>
+        <v>154</v>
       </c>
       <c r="O83" t="s">
         <v>84</v>
@@ -5246,19 +5264,19 @@
         <v>528395.9300000001</v>
       </c>
       <c r="Q83" t="s">
-        <v>165</v>
+        <v>169</v>
       </c>
       <c r="R83" t="s">
-        <v>168</v>
+        <v>172</v>
       </c>
       <c r="S83" t="s">
-        <v>170</v>
+        <v>174</v>
       </c>
       <c r="T83" t="s">
-        <v>174</v>
+        <v>178</v>
       </c>
       <c r="U83" t="s">
-        <v>176</v>
+        <v>180</v>
       </c>
       <c r="V83" s="1">
         <v>46382</v>
@@ -5287,7 +5305,7 @@
         <v>110</v>
       </c>
       <c r="N84" t="s">
-        <v>153</v>
+        <v>156</v>
       </c>
       <c r="O84" t="s">
         <v>85</v>
@@ -5296,16 +5314,16 @@
         <v>1000000</v>
       </c>
       <c r="Q84" t="s">
-        <v>165</v>
+        <v>169</v>
       </c>
       <c r="R84" t="s">
-        <v>167</v>
+        <v>171</v>
       </c>
       <c r="S84" t="s">
-        <v>170</v>
+        <v>174</v>
       </c>
       <c r="T84" t="s">
-        <v>173</v>
+        <v>177</v>
       </c>
       <c r="U84" t="s">
         <v>92</v>
@@ -5331,7 +5349,7 @@
         <v>92</v>
       </c>
       <c r="N85" t="s">
-        <v>161</v>
+        <v>165</v>
       </c>
       <c r="O85" t="s">
         <v>83</v>
@@ -5340,16 +5358,16 @@
         <v>4394700</v>
       </c>
       <c r="Q85" t="s">
-        <v>164</v>
+        <v>168</v>
       </c>
       <c r="R85" t="s">
-        <v>167</v>
+        <v>171</v>
       </c>
       <c r="S85" t="s">
-        <v>171</v>
+        <v>175</v>
       </c>
       <c r="T85" t="s">
-        <v>173</v>
+        <v>177</v>
       </c>
       <c r="U85" t="s">
         <v>92</v>
@@ -5390,16 +5408,16 @@
         <v>3306000</v>
       </c>
       <c r="Q86" t="s">
-        <v>164</v>
+        <v>168</v>
       </c>
       <c r="R86" t="s">
-        <v>167</v>
+        <v>171</v>
       </c>
       <c r="S86" t="s">
         <v>106</v>
       </c>
       <c r="T86" t="s">
-        <v>173</v>
+        <v>177</v>
       </c>
       <c r="U86" t="s">
         <v>92</v>
@@ -5437,16 +5455,16 @@
         <v>3306000</v>
       </c>
       <c r="Q87" t="s">
-        <v>164</v>
+        <v>168</v>
       </c>
       <c r="R87" t="s">
-        <v>167</v>
+        <v>171</v>
       </c>
       <c r="S87" t="s">
         <v>106</v>
       </c>
       <c r="T87" t="s">
-        <v>173</v>
+        <v>177</v>
       </c>
       <c r="U87" t="s">
         <v>92</v>
@@ -5463,7 +5481,7 @@
         <v>86</v>
       </c>
       <c r="D88" t="s">
-        <v>87</v>
+        <v>89</v>
       </c>
       <c r="E88" t="s">
         <v>92</v>
@@ -5472,34 +5490,34 @@
         <v>94</v>
       </c>
       <c r="G88" t="s">
-        <v>107</v>
+        <v>109</v>
       </c>
       <c r="H88" s="1">
         <v>46303</v>
       </c>
       <c r="I88" t="s">
-        <v>112</v>
+        <v>133</v>
       </c>
       <c r="N88" t="s">
-        <v>162</v>
+        <v>166</v>
       </c>
       <c r="O88" t="s">
         <v>86</v>
       </c>
       <c r="P88">
-        <v>470820</v>
+        <v>412107.92</v>
       </c>
       <c r="Q88" t="s">
-        <v>164</v>
+        <v>168</v>
       </c>
       <c r="R88" t="s">
-        <v>167</v>
+        <v>171</v>
       </c>
       <c r="S88" t="s">
-        <v>170</v>
+        <v>174</v>
       </c>
       <c r="T88" t="s">
-        <v>175</v>
+        <v>179</v>
       </c>
       <c r="U88" t="s">
         <v>92</v>
@@ -5528,25 +5546,25 @@
         <v>110</v>
       </c>
       <c r="N89" t="s">
-        <v>154</v>
+        <v>157</v>
       </c>
       <c r="O89" t="s">
-        <v>163</v>
+        <v>167</v>
       </c>
       <c r="P89">
         <v>2297180</v>
       </c>
       <c r="Q89" t="s">
-        <v>165</v>
+        <v>169</v>
       </c>
       <c r="R89" t="s">
-        <v>167</v>
+        <v>171</v>
       </c>
       <c r="S89" t="s">
-        <v>170</v>
+        <v>174</v>
       </c>
       <c r="T89" t="s">
-        <v>173</v>
+        <v>177</v>
       </c>
       <c r="U89" t="s">
         <v>92</v>

</xml_diff>

<commit_message>
Atualização automática: mta (14/10/2026 13:34)
</commit_message>
<xml_diff>
--- a/Projetos/02_Dados_Tratados/base_mta_tratada.xlsx
+++ b/Projetos/02_Dados_Tratados/base_mta_tratada.xlsx
@@ -566,8 +566,16 @@
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="YYYY-MM-DD HH:MM:SS"/>
   </numFmts>
-  <fonts count="1">
+  <fonts count="2">
     <font>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
       <sz val="11"/>
       <color theme="1"/>
       <name val="Calibri"/>
@@ -583,7 +591,7 @@
       <patternFill patternType="gray125"/>
     </fill>
   </fills>
-  <borders count="1">
+  <borders count="2">
     <border>
       <left/>
       <right/>
@@ -591,12 +599,30 @@
       <bottom/>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin">
+        <color auto="1"/>
+      </left>
+      <right style="thin">
+        <color auto="1"/>
+      </right>
+      <top style="thin">
+        <color auto="1"/>
+      </top>
+      <bottom style="thin">
+        <color auto="1"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="3">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
   </cellXfs>
   <cellStyles count="1">
@@ -896,70 +922,70 @@
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:22">
-      <c r="A1" t="s">
+      <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
-      <c r="B1" t="s">
+      <c r="B1" s="1" t="s">
         <v>1</v>
       </c>
-      <c r="C1" t="s">
+      <c r="C1" s="1" t="s">
         <v>2</v>
       </c>
-      <c r="D1" t="s">
+      <c r="D1" s="1" t="s">
         <v>3</v>
       </c>
-      <c r="E1" t="s">
+      <c r="E1" s="1" t="s">
         <v>4</v>
       </c>
-      <c r="F1" t="s">
+      <c r="F1" s="1" t="s">
         <v>5</v>
       </c>
-      <c r="G1" t="s">
+      <c r="G1" s="1" t="s">
         <v>6</v>
       </c>
-      <c r="H1" t="s">
+      <c r="H1" s="1" t="s">
         <v>7</v>
       </c>
-      <c r="I1" t="s">
+      <c r="I1" s="1" t="s">
         <v>8</v>
       </c>
-      <c r="J1" t="s">
+      <c r="J1" s="1" t="s">
         <v>9</v>
       </c>
-      <c r="K1" t="s">
+      <c r="K1" s="1" t="s">
         <v>10</v>
       </c>
-      <c r="L1" t="s">
+      <c r="L1" s="1" t="s">
         <v>11</v>
       </c>
-      <c r="M1" t="s">
+      <c r="M1" s="1" t="s">
         <v>12</v>
       </c>
-      <c r="N1" t="s">
+      <c r="N1" s="1" t="s">
         <v>13</v>
       </c>
-      <c r="O1" t="s">
+      <c r="O1" s="1" t="s">
         <v>14</v>
       </c>
-      <c r="P1" t="s">
+      <c r="P1" s="1" t="s">
         <v>15</v>
       </c>
-      <c r="Q1" t="s">
+      <c r="Q1" s="1" t="s">
         <v>16</v>
       </c>
-      <c r="R1" t="s">
+      <c r="R1" s="1" t="s">
         <v>17</v>
       </c>
-      <c r="S1" t="s">
+      <c r="S1" s="1" t="s">
         <v>18</v>
       </c>
-      <c r="T1" t="s">
+      <c r="T1" s="1" t="s">
         <v>19</v>
       </c>
-      <c r="U1" t="s">
+      <c r="U1" s="1" t="s">
         <v>20</v>
       </c>
-      <c r="V1" t="s">
+      <c r="V1" s="1" t="s">
         <v>21</v>
       </c>
     </row>
@@ -985,7 +1011,7 @@
       <c r="G2" t="s">
         <v>107</v>
       </c>
-      <c r="H2" s="1">
+      <c r="H2" s="2">
         <v>46303</v>
       </c>
       <c r="I2" t="s">
@@ -1024,7 +1050,7 @@
       <c r="U2" t="s">
         <v>180</v>
       </c>
-      <c r="V2" s="1">
+      <c r="V2" s="2">
         <v>46229</v>
       </c>
     </row>
@@ -1071,7 +1097,7 @@
       <c r="U3" t="s">
         <v>92</v>
       </c>
-      <c r="V3" s="1">
+      <c r="V3" s="2">
         <v>46291</v>
       </c>
     </row>
@@ -1118,7 +1144,7 @@
       <c r="U4" t="s">
         <v>92</v>
       </c>
-      <c r="V4" s="1">
+      <c r="V4" s="2">
         <v>46321</v>
       </c>
     </row>
@@ -1165,7 +1191,7 @@
       <c r="U5" t="s">
         <v>92</v>
       </c>
-      <c r="V5" s="1">
+      <c r="V5" s="2">
         <v>46321</v>
       </c>
     </row>
@@ -1215,7 +1241,7 @@
       <c r="U6" t="s">
         <v>92</v>
       </c>
-      <c r="V6" s="1">
+      <c r="V6" s="2">
         <v>46291</v>
       </c>
     </row>
@@ -1241,7 +1267,7 @@
       <c r="G7" t="s">
         <v>109</v>
       </c>
-      <c r="H7" s="1">
+      <c r="H7" s="2">
         <v>46121</v>
       </c>
       <c r="I7" t="s">
@@ -1271,7 +1297,7 @@
       <c r="U7" t="s">
         <v>92</v>
       </c>
-      <c r="V7" s="1">
+      <c r="V7" s="2">
         <v>46138</v>
       </c>
     </row>
@@ -1318,7 +1344,7 @@
       <c r="U8" t="s">
         <v>92</v>
       </c>
-      <c r="V8" s="1">
+      <c r="V8" s="2">
         <v>46291</v>
       </c>
     </row>
@@ -1365,7 +1391,7 @@
       <c r="U9" t="s">
         <v>92</v>
       </c>
-      <c r="V9" s="1">
+      <c r="V9" s="2">
         <v>46291</v>
       </c>
     </row>
@@ -1388,7 +1414,7 @@
       <c r="G10" t="s">
         <v>109</v>
       </c>
-      <c r="H10" s="1">
+      <c r="H10" s="2">
         <v>46303</v>
       </c>
       <c r="I10" t="s">
@@ -1418,7 +1444,7 @@
       <c r="U10" t="s">
         <v>92</v>
       </c>
-      <c r="V10" s="1">
+      <c r="V10" s="2">
         <v>46291</v>
       </c>
     </row>
@@ -1465,7 +1491,7 @@
       <c r="U11" t="s">
         <v>92</v>
       </c>
-      <c r="V11" s="1">
+      <c r="V11" s="2">
         <v>46291</v>
       </c>
     </row>
@@ -1512,7 +1538,7 @@
       <c r="U12" t="s">
         <v>92</v>
       </c>
-      <c r="V12" s="1">
+      <c r="V12" s="2">
         <v>46291</v>
       </c>
     </row>
@@ -1538,7 +1564,7 @@
       <c r="G13" t="s">
         <v>109</v>
       </c>
-      <c r="H13" s="1">
+      <c r="H13" s="2">
         <v>46079</v>
       </c>
       <c r="I13" t="s">
@@ -1571,7 +1597,7 @@
       <c r="U13" t="s">
         <v>180</v>
       </c>
-      <c r="V13" s="1">
+      <c r="V13" s="2">
         <v>46079</v>
       </c>
     </row>
@@ -1597,7 +1623,7 @@
       <c r="G14" t="s">
         <v>107</v>
       </c>
-      <c r="H14" s="1">
+      <c r="H14" s="2">
         <v>46303</v>
       </c>
       <c r="I14" t="s">
@@ -1633,7 +1659,7 @@
       <c r="U14" t="s">
         <v>180</v>
       </c>
-      <c r="V14" s="1">
+      <c r="V14" s="2">
         <v>46352</v>
       </c>
     </row>
@@ -1659,7 +1685,7 @@
       <c r="G15" t="s">
         <v>107</v>
       </c>
-      <c r="H15" s="1">
+      <c r="H15" s="2">
         <v>46303</v>
       </c>
       <c r="I15" t="s">
@@ -1695,7 +1721,7 @@
       <c r="U15" t="s">
         <v>180</v>
       </c>
-      <c r="V15" s="1">
+      <c r="V15" s="2">
         <v>46352</v>
       </c>
     </row>
@@ -1721,7 +1747,7 @@
       <c r="G16" t="s">
         <v>107</v>
       </c>
-      <c r="H16" s="1">
+      <c r="H16" s="2">
         <v>46303</v>
       </c>
       <c r="I16" t="s">
@@ -1757,7 +1783,7 @@
       <c r="U16" t="s">
         <v>180</v>
       </c>
-      <c r="V16" s="1">
+      <c r="V16" s="2">
         <v>46352</v>
       </c>
     </row>
@@ -1783,7 +1809,7 @@
       <c r="G17" t="s">
         <v>107</v>
       </c>
-      <c r="H17" s="1">
+      <c r="H17" s="2">
         <v>46303</v>
       </c>
       <c r="I17" t="s">
@@ -1819,7 +1845,7 @@
       <c r="U17" t="s">
         <v>180</v>
       </c>
-      <c r="V17" s="1">
+      <c r="V17" s="2">
         <v>46229</v>
       </c>
     </row>
@@ -1845,7 +1871,7 @@
       <c r="G18" t="s">
         <v>109</v>
       </c>
-      <c r="H18" s="1">
+      <c r="H18" s="2">
         <v>46098</v>
       </c>
       <c r="I18" t="s">
@@ -1878,7 +1904,7 @@
       <c r="U18" t="s">
         <v>180</v>
       </c>
-      <c r="V18" s="1">
+      <c r="V18" s="2">
         <v>46107</v>
       </c>
     </row>
@@ -1904,7 +1930,7 @@
       <c r="G19" t="s">
         <v>109</v>
       </c>
-      <c r="H19" s="1">
+      <c r="H19" s="2">
         <v>46076</v>
       </c>
       <c r="I19" t="s">
@@ -1934,7 +1960,7 @@
       <c r="U19" t="s">
         <v>92</v>
       </c>
-      <c r="V19" s="1">
+      <c r="V19" s="2">
         <v>46079</v>
       </c>
     </row>
@@ -1960,7 +1986,7 @@
       <c r="G20" t="s">
         <v>109</v>
       </c>
-      <c r="H20" s="1">
+      <c r="H20" s="2">
         <v>46076</v>
       </c>
       <c r="I20" t="s">
@@ -1990,7 +2016,7 @@
       <c r="U20" t="s">
         <v>92</v>
       </c>
-      <c r="V20" s="1">
+      <c r="V20" s="2">
         <v>46079</v>
       </c>
     </row>
@@ -2037,7 +2063,7 @@
       <c r="U21" t="s">
         <v>92</v>
       </c>
-      <c r="V21" s="1">
+      <c r="V21" s="2">
         <v>46321</v>
       </c>
     </row>
@@ -2084,7 +2110,7 @@
       <c r="U22" t="s">
         <v>92</v>
       </c>
-      <c r="V22" s="1">
+      <c r="V22" s="2">
         <v>46321</v>
       </c>
     </row>
@@ -2131,7 +2157,7 @@
       <c r="U23" t="s">
         <v>92</v>
       </c>
-      <c r="V23" s="1">
+      <c r="V23" s="2">
         <v>46321</v>
       </c>
     </row>
@@ -2178,7 +2204,7 @@
       <c r="U24" t="s">
         <v>92</v>
       </c>
-      <c r="V24" s="1">
+      <c r="V24" s="2">
         <v>46321</v>
       </c>
     </row>
@@ -2204,7 +2230,7 @@
       <c r="G25" t="s">
         <v>109</v>
       </c>
-      <c r="H25" s="1">
+      <c r="H25" s="2">
         <v>46119</v>
       </c>
       <c r="I25" t="s">
@@ -2237,7 +2263,7 @@
       <c r="U25" t="s">
         <v>180</v>
       </c>
-      <c r="V25" s="1">
+      <c r="V25" s="2">
         <v>46138</v>
       </c>
     </row>
@@ -2263,7 +2289,7 @@
       <c r="G26" t="s">
         <v>109</v>
       </c>
-      <c r="H26" s="1">
+      <c r="H26" s="2">
         <v>46121</v>
       </c>
       <c r="I26" t="s">
@@ -2293,7 +2319,7 @@
       <c r="U26" t="s">
         <v>92</v>
       </c>
-      <c r="V26" s="1">
+      <c r="V26" s="2">
         <v>46138</v>
       </c>
     </row>
@@ -2319,7 +2345,7 @@
       <c r="G27" t="s">
         <v>109</v>
       </c>
-      <c r="H27" s="1">
+      <c r="H27" s="2">
         <v>46076</v>
       </c>
       <c r="I27" t="s">
@@ -2349,7 +2375,7 @@
       <c r="U27" t="s">
         <v>92</v>
       </c>
-      <c r="V27" s="1">
+      <c r="V27" s="2">
         <v>46079</v>
       </c>
     </row>
@@ -2375,7 +2401,7 @@
       <c r="G28" t="s">
         <v>107</v>
       </c>
-      <c r="H28" s="1">
+      <c r="H28" s="2">
         <v>46303</v>
       </c>
       <c r="I28" t="s">
@@ -2411,7 +2437,7 @@
       <c r="U28" t="s">
         <v>180</v>
       </c>
-      <c r="V28" s="1">
+      <c r="V28" s="2">
         <v>46291</v>
       </c>
     </row>
@@ -2437,7 +2463,7 @@
       <c r="G29" t="s">
         <v>109</v>
       </c>
-      <c r="H29" s="1">
+      <c r="H29" s="2">
         <v>46199</v>
       </c>
       <c r="I29" t="s">
@@ -2470,7 +2496,7 @@
       <c r="U29" t="s">
         <v>180</v>
       </c>
-      <c r="V29" s="1">
+      <c r="V29" s="2">
         <v>46199</v>
       </c>
     </row>
@@ -2496,7 +2522,7 @@
       <c r="G30" t="s">
         <v>109</v>
       </c>
-      <c r="H30" s="1">
+      <c r="H30" s="2">
         <v>46199</v>
       </c>
       <c r="I30" t="s">
@@ -2529,7 +2555,7 @@
       <c r="U30" t="s">
         <v>180</v>
       </c>
-      <c r="V30" s="1">
+      <c r="V30" s="2">
         <v>46199</v>
       </c>
     </row>
@@ -2555,7 +2581,7 @@
       <c r="G31" t="s">
         <v>109</v>
       </c>
-      <c r="H31" s="1">
+      <c r="H31" s="2">
         <v>46199</v>
       </c>
       <c r="I31" t="s">
@@ -2588,7 +2614,7 @@
       <c r="U31" t="s">
         <v>180</v>
       </c>
-      <c r="V31" s="1">
+      <c r="V31" s="2">
         <v>46199</v>
       </c>
     </row>
@@ -2614,7 +2640,7 @@
       <c r="G32" t="s">
         <v>109</v>
       </c>
-      <c r="H32" s="1">
+      <c r="H32" s="2">
         <v>46199</v>
       </c>
       <c r="I32" t="s">
@@ -2647,7 +2673,7 @@
       <c r="U32" t="s">
         <v>180</v>
       </c>
-      <c r="V32" s="1">
+      <c r="V32" s="2">
         <v>46199</v>
       </c>
     </row>
@@ -2700,7 +2726,7 @@
       <c r="U33" t="s">
         <v>180</v>
       </c>
-      <c r="V33" s="1">
+      <c r="V33" s="2">
         <v>46291</v>
       </c>
     </row>
@@ -2726,7 +2752,7 @@
       <c r="G34" t="s">
         <v>109</v>
       </c>
-      <c r="H34" s="1">
+      <c r="H34" s="2">
         <v>46191</v>
       </c>
       <c r="I34" t="s">
@@ -2759,7 +2785,7 @@
       <c r="U34" t="s">
         <v>180</v>
       </c>
-      <c r="V34" s="1">
+      <c r="V34" s="2">
         <v>46199</v>
       </c>
     </row>
@@ -2785,7 +2811,7 @@
       <c r="G35" t="s">
         <v>109</v>
       </c>
-      <c r="H35" s="1">
+      <c r="H35" s="2">
         <v>46119</v>
       </c>
       <c r="I35" t="s">
@@ -2815,7 +2841,7 @@
       <c r="U35" t="s">
         <v>180</v>
       </c>
-      <c r="V35" s="1">
+      <c r="V35" s="2">
         <v>46138</v>
       </c>
     </row>
@@ -2841,7 +2867,7 @@
       <c r="G36" t="s">
         <v>109</v>
       </c>
-      <c r="H36" s="1">
+      <c r="H36" s="2">
         <v>46213</v>
       </c>
       <c r="I36" t="s">
@@ -2871,7 +2897,7 @@
       <c r="U36" t="s">
         <v>92</v>
       </c>
-      <c r="V36" s="1">
+      <c r="V36" s="2">
         <v>46229</v>
       </c>
     </row>
@@ -2897,7 +2923,7 @@
       <c r="G37" t="s">
         <v>109</v>
       </c>
-      <c r="H37" s="1">
+      <c r="H37" s="2">
         <v>46175</v>
       </c>
       <c r="I37" t="s">
@@ -2927,7 +2953,7 @@
       <c r="U37" t="s">
         <v>92</v>
       </c>
-      <c r="V37" s="1">
+      <c r="V37" s="2">
         <v>46199</v>
       </c>
     </row>
@@ -2953,7 +2979,7 @@
       <c r="G38" t="s">
         <v>109</v>
       </c>
-      <c r="H38" s="1">
+      <c r="H38" s="2">
         <v>46213</v>
       </c>
       <c r="I38" t="s">
@@ -2983,7 +3009,7 @@
       <c r="U38" t="s">
         <v>92</v>
       </c>
-      <c r="V38" s="1">
+      <c r="V38" s="2">
         <v>46229</v>
       </c>
     </row>
@@ -3009,7 +3035,7 @@
       <c r="G39" t="s">
         <v>109</v>
       </c>
-      <c r="H39" s="1">
+      <c r="H39" s="2">
         <v>46199</v>
       </c>
       <c r="I39" t="s">
@@ -3039,7 +3065,7 @@
       <c r="U39" t="s">
         <v>92</v>
       </c>
-      <c r="V39" s="1">
+      <c r="V39" s="2">
         <v>46199</v>
       </c>
     </row>
@@ -3065,7 +3091,7 @@
       <c r="G40" t="s">
         <v>109</v>
       </c>
-      <c r="H40" s="1">
+      <c r="H40" s="2">
         <v>46199</v>
       </c>
       <c r="I40" t="s">
@@ -3095,7 +3121,7 @@
       <c r="U40" t="s">
         <v>92</v>
       </c>
-      <c r="V40" s="1">
+      <c r="V40" s="2">
         <v>46199</v>
       </c>
     </row>
@@ -3121,7 +3147,7 @@
       <c r="G41" t="s">
         <v>109</v>
       </c>
-      <c r="H41" s="1">
+      <c r="H41" s="2">
         <v>46204</v>
       </c>
       <c r="I41" t="s">
@@ -3151,7 +3177,7 @@
       <c r="U41" t="s">
         <v>92</v>
       </c>
-      <c r="V41" s="1">
+      <c r="V41" s="2">
         <v>46229</v>
       </c>
     </row>
@@ -3177,7 +3203,7 @@
       <c r="G42" t="s">
         <v>109</v>
       </c>
-      <c r="H42" s="1">
+      <c r="H42" s="2">
         <v>46244</v>
       </c>
       <c r="I42" t="s">
@@ -3207,7 +3233,7 @@
       <c r="U42" t="s">
         <v>92</v>
       </c>
-      <c r="V42" s="1">
+      <c r="V42" s="2">
         <v>46199</v>
       </c>
     </row>
@@ -3251,7 +3277,7 @@
       <c r="U43" t="s">
         <v>92</v>
       </c>
-      <c r="V43" s="1">
+      <c r="V43" s="2">
         <v>46260</v>
       </c>
     </row>
@@ -3277,7 +3303,7 @@
       <c r="G44" t="s">
         <v>109</v>
       </c>
-      <c r="H44" s="1">
+      <c r="H44" s="2">
         <v>46191</v>
       </c>
       <c r="I44" t="s">
@@ -3307,7 +3333,7 @@
       <c r="U44" t="s">
         <v>92</v>
       </c>
-      <c r="V44" s="1">
+      <c r="V44" s="2">
         <v>46199</v>
       </c>
     </row>
@@ -3333,7 +3359,7 @@
       <c r="G45" t="s">
         <v>109</v>
       </c>
-      <c r="H45" s="1">
+      <c r="H45" s="2">
         <v>46191</v>
       </c>
       <c r="I45" t="s">
@@ -3363,7 +3389,7 @@
       <c r="U45" t="s">
         <v>92</v>
       </c>
-      <c r="V45" s="1">
+      <c r="V45" s="2">
         <v>46199</v>
       </c>
     </row>
@@ -3389,7 +3415,7 @@
       <c r="G46" t="s">
         <v>109</v>
       </c>
-      <c r="H46" s="1">
+      <c r="H46" s="2">
         <v>46213</v>
       </c>
       <c r="I46" t="s">
@@ -3422,7 +3448,7 @@
       <c r="U46" t="s">
         <v>180</v>
       </c>
-      <c r="V46" s="1">
+      <c r="V46" s="2">
         <v>46229</v>
       </c>
     </row>
@@ -3448,7 +3474,7 @@
       <c r="G47" t="s">
         <v>109</v>
       </c>
-      <c r="H47" s="1">
+      <c r="H47" s="2">
         <v>46210</v>
       </c>
       <c r="I47" t="s">
@@ -3478,7 +3504,7 @@
       <c r="U47" t="s">
         <v>180</v>
       </c>
-      <c r="V47" s="1">
+      <c r="V47" s="2">
         <v>46229</v>
       </c>
     </row>
@@ -3525,7 +3551,7 @@
       <c r="U48" t="s">
         <v>92</v>
       </c>
-      <c r="V48" s="1">
+      <c r="V48" s="2">
         <v>46321</v>
       </c>
     </row>
@@ -3551,7 +3577,7 @@
       <c r="G49" t="s">
         <v>107</v>
       </c>
-      <c r="H49" s="1">
+      <c r="H49" s="2">
         <v>46303</v>
       </c>
       <c r="I49" t="s">
@@ -3587,7 +3613,7 @@
       <c r="U49" t="s">
         <v>180</v>
       </c>
-      <c r="V49" s="1">
+      <c r="V49" s="2">
         <v>46291</v>
       </c>
     </row>
@@ -3613,7 +3639,7 @@
       <c r="G50" t="s">
         <v>109</v>
       </c>
-      <c r="H50" s="1">
+      <c r="H50" s="2">
         <v>46176</v>
       </c>
       <c r="I50" t="s">
@@ -3646,7 +3672,7 @@
       <c r="U50" t="s">
         <v>180</v>
       </c>
-      <c r="V50" s="1">
+      <c r="V50" s="2">
         <v>46199</v>
       </c>
     </row>
@@ -3702,7 +3728,7 @@
       <c r="U51" t="s">
         <v>180</v>
       </c>
-      <c r="V51" s="1">
+      <c r="V51" s="2">
         <v>46260</v>
       </c>
     </row>
@@ -3728,7 +3754,7 @@
       <c r="G52" t="s">
         <v>109</v>
       </c>
-      <c r="H52" s="1">
+      <c r="H52" s="2">
         <v>46295</v>
       </c>
       <c r="I52" t="s">
@@ -3764,7 +3790,7 @@
       <c r="U52" t="s">
         <v>180</v>
       </c>
-      <c r="V52" s="1">
+      <c r="V52" s="2">
         <v>46291</v>
       </c>
     </row>
@@ -3817,7 +3843,7 @@
       <c r="U53" t="s">
         <v>180</v>
       </c>
-      <c r="V53" s="1">
+      <c r="V53" s="2">
         <v>46321</v>
       </c>
     </row>
@@ -3843,7 +3869,7 @@
       <c r="G54" t="s">
         <v>109</v>
       </c>
-      <c r="H54" s="1">
+      <c r="H54" s="2">
         <v>46227</v>
       </c>
       <c r="I54" t="s">
@@ -3873,7 +3899,7 @@
       <c r="U54" t="s">
         <v>180</v>
       </c>
-      <c r="V54" s="1">
+      <c r="V54" s="2">
         <v>46229</v>
       </c>
     </row>
@@ -3896,7 +3922,7 @@
       <c r="G55" t="s">
         <v>109</v>
       </c>
-      <c r="H55" s="1">
+      <c r="H55" s="2">
         <v>46280</v>
       </c>
       <c r="I55" t="s">
@@ -3926,7 +3952,7 @@
       <c r="U55" t="s">
         <v>180</v>
       </c>
-      <c r="V55" s="1">
+      <c r="V55" s="2">
         <v>46291</v>
       </c>
     </row>
@@ -3949,7 +3975,7 @@
       <c r="G56" t="s">
         <v>109</v>
       </c>
-      <c r="H56" s="1">
+      <c r="H56" s="2">
         <v>46280</v>
       </c>
       <c r="I56" t="s">
@@ -3979,7 +4005,7 @@
       <c r="U56" t="s">
         <v>180</v>
       </c>
-      <c r="V56" s="1">
+      <c r="V56" s="2">
         <v>46260</v>
       </c>
     </row>
@@ -4002,7 +4028,7 @@
       <c r="G57" t="s">
         <v>109</v>
       </c>
-      <c r="H57" s="1">
+      <c r="H57" s="2">
         <v>46295</v>
       </c>
       <c r="I57" t="s">
@@ -4032,7 +4058,7 @@
       <c r="U57" t="s">
         <v>180</v>
       </c>
-      <c r="V57" s="1">
+      <c r="V57" s="2">
         <v>46291</v>
       </c>
     </row>
@@ -4055,7 +4081,7 @@
       <c r="G58" t="s">
         <v>109</v>
       </c>
-      <c r="H58" s="1">
+      <c r="H58" s="2">
         <v>46295</v>
       </c>
       <c r="I58" t="s">
@@ -4085,7 +4111,7 @@
       <c r="U58" t="s">
         <v>180</v>
       </c>
-      <c r="V58" s="1">
+      <c r="V58" s="2">
         <v>46291</v>
       </c>
     </row>
@@ -4108,7 +4134,7 @@
       <c r="G59" t="s">
         <v>109</v>
       </c>
-      <c r="H59" s="1">
+      <c r="H59" s="2">
         <v>46304</v>
       </c>
       <c r="I59" t="s">
@@ -4138,7 +4164,7 @@
       <c r="U59" t="s">
         <v>180</v>
       </c>
-      <c r="V59" s="1">
+      <c r="V59" s="2">
         <v>46321</v>
       </c>
     </row>
@@ -4164,7 +4190,7 @@
       <c r="G60" t="s">
         <v>109</v>
       </c>
-      <c r="H60" s="1">
+      <c r="H60" s="2">
         <v>46301</v>
       </c>
       <c r="I60" t="s">
@@ -4200,7 +4226,7 @@
       <c r="U60" t="s">
         <v>180</v>
       </c>
-      <c r="V60" s="1">
+      <c r="V60" s="2">
         <v>46352</v>
       </c>
     </row>
@@ -4244,7 +4270,7 @@
       <c r="U61" t="s">
         <v>180</v>
       </c>
-      <c r="V61" s="1">
+      <c r="V61" s="2">
         <v>46107</v>
       </c>
     </row>
@@ -4288,7 +4314,7 @@
       <c r="U62" t="s">
         <v>180</v>
       </c>
-      <c r="V62" s="1">
+      <c r="V62" s="2">
         <v>46107</v>
       </c>
     </row>
@@ -4332,7 +4358,7 @@
       <c r="U63" t="s">
         <v>180</v>
       </c>
-      <c r="V63" s="1">
+      <c r="V63" s="2">
         <v>46107</v>
       </c>
     </row>
@@ -4376,7 +4402,7 @@
       <c r="U64" t="s">
         <v>180</v>
       </c>
-      <c r="V64" s="1">
+      <c r="V64" s="2">
         <v>46107</v>
       </c>
     </row>
@@ -4420,7 +4446,7 @@
       <c r="U65" t="s">
         <v>180</v>
       </c>
-      <c r="V65" s="1">
+      <c r="V65" s="2">
         <v>46107</v>
       </c>
     </row>
@@ -4464,7 +4490,7 @@
       <c r="U66" t="s">
         <v>180</v>
       </c>
-      <c r="V66" s="1">
+      <c r="V66" s="2">
         <v>46107</v>
       </c>
     </row>
@@ -4508,7 +4534,7 @@
       <c r="U67" t="s">
         <v>92</v>
       </c>
-      <c r="V67" s="1">
+      <c r="V67" s="2">
         <v>46168</v>
       </c>
     </row>
@@ -4555,7 +4581,7 @@
       <c r="U68" t="s">
         <v>92</v>
       </c>
-      <c r="V68" s="1">
+      <c r="V68" s="2">
         <v>46291</v>
       </c>
     </row>
@@ -4581,7 +4607,7 @@
       <c r="G69" t="s">
         <v>107</v>
       </c>
-      <c r="H69" s="1">
+      <c r="H69" s="2">
         <v>46303</v>
       </c>
       <c r="I69" t="s">
@@ -4617,7 +4643,7 @@
       <c r="U69" t="s">
         <v>180</v>
       </c>
-      <c r="V69" s="1">
+      <c r="V69" s="2">
         <v>46229</v>
       </c>
     </row>
@@ -4661,7 +4687,7 @@
       <c r="U70" t="s">
         <v>92</v>
       </c>
-      <c r="V70" s="1">
+      <c r="V70" s="2">
         <v>46260</v>
       </c>
     </row>
@@ -4705,7 +4731,7 @@
       <c r="U71" t="s">
         <v>180</v>
       </c>
-      <c r="V71" s="1">
+      <c r="V71" s="2">
         <v>46291</v>
       </c>
     </row>
@@ -4749,7 +4775,7 @@
       <c r="U72" t="s">
         <v>180</v>
       </c>
-      <c r="V72" s="1">
+      <c r="V72" s="2">
         <v>46168</v>
       </c>
     </row>
@@ -4793,7 +4819,7 @@
       <c r="U73" t="s">
         <v>180</v>
       </c>
-      <c r="V73" s="1">
+      <c r="V73" s="2">
         <v>46291</v>
       </c>
     </row>
@@ -4837,7 +4863,7 @@
       <c r="U74" t="s">
         <v>180</v>
       </c>
-      <c r="V74" s="1">
+      <c r="V74" s="2">
         <v>46291</v>
       </c>
     </row>
@@ -4881,7 +4907,7 @@
       <c r="U75" t="s">
         <v>180</v>
       </c>
-      <c r="V75" s="1">
+      <c r="V75" s="2">
         <v>46291</v>
       </c>
     </row>
@@ -4928,7 +4954,7 @@
       <c r="U76" t="s">
         <v>92</v>
       </c>
-      <c r="V76" s="1">
+      <c r="V76" s="2">
         <v>46321</v>
       </c>
     </row>
@@ -4978,7 +5004,7 @@
       <c r="U77" t="s">
         <v>180</v>
       </c>
-      <c r="V77" s="1">
+      <c r="V77" s="2">
         <v>46381</v>
       </c>
     </row>
@@ -5028,7 +5054,7 @@
       <c r="U78" t="s">
         <v>180</v>
       </c>
-      <c r="V78" s="1">
+      <c r="V78" s="2">
         <v>46381</v>
       </c>
     </row>
@@ -5078,7 +5104,7 @@
       <c r="U79" t="s">
         <v>92</v>
       </c>
-      <c r="V79" s="1">
+      <c r="V79" s="2">
         <v>46381</v>
       </c>
     </row>
@@ -5128,7 +5154,7 @@
       <c r="U80" t="s">
         <v>92</v>
       </c>
-      <c r="V80" s="1">
+      <c r="V80" s="2">
         <v>46381</v>
       </c>
     </row>
@@ -5178,7 +5204,7 @@
       <c r="U81" t="s">
         <v>92</v>
       </c>
-      <c r="V81" s="1">
+      <c r="V81" s="2">
         <v>46382</v>
       </c>
     </row>
@@ -5222,7 +5248,7 @@
       <c r="U82" t="s">
         <v>92</v>
       </c>
-      <c r="V82" s="1">
+      <c r="V82" s="2">
         <v>46382</v>
       </c>
     </row>
@@ -5278,7 +5304,7 @@
       <c r="U83" t="s">
         <v>180</v>
       </c>
-      <c r="V83" s="1">
+      <c r="V83" s="2">
         <v>46382</v>
       </c>
     </row>
@@ -5328,7 +5354,7 @@
       <c r="U84" t="s">
         <v>92</v>
       </c>
-      <c r="V84" s="1">
+      <c r="V84" s="2">
         <v>46321</v>
       </c>
     </row>
@@ -5372,7 +5398,7 @@
       <c r="U85" t="s">
         <v>92</v>
       </c>
-      <c r="V85" s="1">
+      <c r="V85" s="2">
         <v>46382</v>
       </c>
     </row>
@@ -5492,7 +5518,7 @@
       <c r="G88" t="s">
         <v>109</v>
       </c>
-      <c r="H88" s="1">
+      <c r="H88" s="2">
         <v>46303</v>
       </c>
       <c r="I88" t="s">
@@ -5522,7 +5548,7 @@
       <c r="U88" t="s">
         <v>92</v>
       </c>
-      <c r="V88" s="1">
+      <c r="V88" s="2">
         <v>46291</v>
       </c>
     </row>
@@ -5569,7 +5595,7 @@
       <c r="U89" t="s">
         <v>92</v>
       </c>
-      <c r="V89" s="1">
+      <c r="V89" s="2">
         <v>46291</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Atualização automática: mta (15/10/2026 12:35)
</commit_message>
<xml_diff>
--- a/Projetos/02_Dados_Tratados/base_mta_tratada.xlsx
+++ b/Projetos/02_Dados_Tratados/base_mta_tratada.xlsx
@@ -566,16 +566,8 @@
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="YYYY-MM-DD HH:MM:SS"/>
   </numFmts>
-  <fonts count="2">
+  <fonts count="1">
     <font>
-      <sz val="11"/>
-      <color theme="1"/>
-      <name val="Calibri"/>
-      <family val="2"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <b/>
       <sz val="11"/>
       <color theme="1"/>
       <name val="Calibri"/>
@@ -591,7 +583,7 @@
       <patternFill patternType="gray125"/>
     </fill>
   </fills>
-  <borders count="2">
+  <borders count="1">
     <border>
       <left/>
       <right/>
@@ -599,30 +591,12 @@
       <bottom/>
       <diagonal/>
     </border>
-    <border>
-      <left style="thin">
-        <color auto="1"/>
-      </left>
-      <right style="thin">
-        <color auto="1"/>
-      </right>
-      <top style="thin">
-        <color auto="1"/>
-      </top>
-      <bottom style="thin">
-        <color auto="1"/>
-      </bottom>
-      <diagonal/>
-    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="3">
+  <cellXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top"/>
-    </xf>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
   </cellXfs>
   <cellStyles count="1">
@@ -922,70 +896,70 @@
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:22">
-      <c r="A1" s="1" t="s">
+      <c r="A1" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="1" t="s">
+      <c r="B1" t="s">
         <v>1</v>
       </c>
-      <c r="C1" s="1" t="s">
+      <c r="C1" t="s">
         <v>2</v>
       </c>
-      <c r="D1" s="1" t="s">
+      <c r="D1" t="s">
         <v>3</v>
       </c>
-      <c r="E1" s="1" t="s">
+      <c r="E1" t="s">
         <v>4</v>
       </c>
-      <c r="F1" s="1" t="s">
+      <c r="F1" t="s">
         <v>5</v>
       </c>
-      <c r="G1" s="1" t="s">
+      <c r="G1" t="s">
         <v>6</v>
       </c>
-      <c r="H1" s="1" t="s">
+      <c r="H1" t="s">
         <v>7</v>
       </c>
-      <c r="I1" s="1" t="s">
+      <c r="I1" t="s">
         <v>8</v>
       </c>
-      <c r="J1" s="1" t="s">
+      <c r="J1" t="s">
         <v>9</v>
       </c>
-      <c r="K1" s="1" t="s">
+      <c r="K1" t="s">
         <v>10</v>
       </c>
-      <c r="L1" s="1" t="s">
+      <c r="L1" t="s">
         <v>11</v>
       </c>
-      <c r="M1" s="1" t="s">
+      <c r="M1" t="s">
         <v>12</v>
       </c>
-      <c r="N1" s="1" t="s">
+      <c r="N1" t="s">
         <v>13</v>
       </c>
-      <c r="O1" s="1" t="s">
+      <c r="O1" t="s">
         <v>14</v>
       </c>
-      <c r="P1" s="1" t="s">
+      <c r="P1" t="s">
         <v>15</v>
       </c>
-      <c r="Q1" s="1" t="s">
+      <c r="Q1" t="s">
         <v>16</v>
       </c>
-      <c r="R1" s="1" t="s">
+      <c r="R1" t="s">
         <v>17</v>
       </c>
-      <c r="S1" s="1" t="s">
+      <c r="S1" t="s">
         <v>18</v>
       </c>
-      <c r="T1" s="1" t="s">
+      <c r="T1" t="s">
         <v>19</v>
       </c>
-      <c r="U1" s="1" t="s">
+      <c r="U1" t="s">
         <v>20</v>
       </c>
-      <c r="V1" s="1" t="s">
+      <c r="V1" t="s">
         <v>21</v>
       </c>
     </row>
@@ -1011,7 +985,7 @@
       <c r="G2" t="s">
         <v>107</v>
       </c>
-      <c r="H2" s="2">
+      <c r="H2" s="1">
         <v>46303</v>
       </c>
       <c r="I2" t="s">
@@ -1050,7 +1024,7 @@
       <c r="U2" t="s">
         <v>180</v>
       </c>
-      <c r="V2" s="2">
+      <c r="V2" s="1">
         <v>46229</v>
       </c>
     </row>
@@ -1097,7 +1071,7 @@
       <c r="U3" t="s">
         <v>92</v>
       </c>
-      <c r="V3" s="2">
+      <c r="V3" s="1">
         <v>46291</v>
       </c>
     </row>
@@ -1144,7 +1118,7 @@
       <c r="U4" t="s">
         <v>92</v>
       </c>
-      <c r="V4" s="2">
+      <c r="V4" s="1">
         <v>46321</v>
       </c>
     </row>
@@ -1191,7 +1165,7 @@
       <c r="U5" t="s">
         <v>92</v>
       </c>
-      <c r="V5" s="2">
+      <c r="V5" s="1">
         <v>46321</v>
       </c>
     </row>
@@ -1241,7 +1215,7 @@
       <c r="U6" t="s">
         <v>92</v>
       </c>
-      <c r="V6" s="2">
+      <c r="V6" s="1">
         <v>46291</v>
       </c>
     </row>
@@ -1267,7 +1241,7 @@
       <c r="G7" t="s">
         <v>109</v>
       </c>
-      <c r="H7" s="2">
+      <c r="H7" s="1">
         <v>46121</v>
       </c>
       <c r="I7" t="s">
@@ -1297,7 +1271,7 @@
       <c r="U7" t="s">
         <v>92</v>
       </c>
-      <c r="V7" s="2">
+      <c r="V7" s="1">
         <v>46138</v>
       </c>
     </row>
@@ -1344,7 +1318,7 @@
       <c r="U8" t="s">
         <v>92</v>
       </c>
-      <c r="V8" s="2">
+      <c r="V8" s="1">
         <v>46291</v>
       </c>
     </row>
@@ -1391,7 +1365,7 @@
       <c r="U9" t="s">
         <v>92</v>
       </c>
-      <c r="V9" s="2">
+      <c r="V9" s="1">
         <v>46291</v>
       </c>
     </row>
@@ -1414,7 +1388,7 @@
       <c r="G10" t="s">
         <v>109</v>
       </c>
-      <c r="H10" s="2">
+      <c r="H10" s="1">
         <v>46303</v>
       </c>
       <c r="I10" t="s">
@@ -1444,7 +1418,7 @@
       <c r="U10" t="s">
         <v>92</v>
       </c>
-      <c r="V10" s="2">
+      <c r="V10" s="1">
         <v>46291</v>
       </c>
     </row>
@@ -1491,7 +1465,7 @@
       <c r="U11" t="s">
         <v>92</v>
       </c>
-      <c r="V11" s="2">
+      <c r="V11" s="1">
         <v>46291</v>
       </c>
     </row>
@@ -1538,7 +1512,7 @@
       <c r="U12" t="s">
         <v>92</v>
       </c>
-      <c r="V12" s="2">
+      <c r="V12" s="1">
         <v>46291</v>
       </c>
     </row>
@@ -1564,7 +1538,7 @@
       <c r="G13" t="s">
         <v>109</v>
       </c>
-      <c r="H13" s="2">
+      <c r="H13" s="1">
         <v>46079</v>
       </c>
       <c r="I13" t="s">
@@ -1597,7 +1571,7 @@
       <c r="U13" t="s">
         <v>180</v>
       </c>
-      <c r="V13" s="2">
+      <c r="V13" s="1">
         <v>46079</v>
       </c>
     </row>
@@ -1623,7 +1597,7 @@
       <c r="G14" t="s">
         <v>107</v>
       </c>
-      <c r="H14" s="2">
+      <c r="H14" s="1">
         <v>46303</v>
       </c>
       <c r="I14" t="s">
@@ -1659,7 +1633,7 @@
       <c r="U14" t="s">
         <v>180</v>
       </c>
-      <c r="V14" s="2">
+      <c r="V14" s="1">
         <v>46352</v>
       </c>
     </row>
@@ -1685,7 +1659,7 @@
       <c r="G15" t="s">
         <v>107</v>
       </c>
-      <c r="H15" s="2">
+      <c r="H15" s="1">
         <v>46303</v>
       </c>
       <c r="I15" t="s">
@@ -1721,7 +1695,7 @@
       <c r="U15" t="s">
         <v>180</v>
       </c>
-      <c r="V15" s="2">
+      <c r="V15" s="1">
         <v>46352</v>
       </c>
     </row>
@@ -1747,7 +1721,7 @@
       <c r="G16" t="s">
         <v>107</v>
       </c>
-      <c r="H16" s="2">
+      <c r="H16" s="1">
         <v>46303</v>
       </c>
       <c r="I16" t="s">
@@ -1783,7 +1757,7 @@
       <c r="U16" t="s">
         <v>180</v>
       </c>
-      <c r="V16" s="2">
+      <c r="V16" s="1">
         <v>46352</v>
       </c>
     </row>
@@ -1809,7 +1783,7 @@
       <c r="G17" t="s">
         <v>107</v>
       </c>
-      <c r="H17" s="2">
+      <c r="H17" s="1">
         <v>46303</v>
       </c>
       <c r="I17" t="s">
@@ -1845,7 +1819,7 @@
       <c r="U17" t="s">
         <v>180</v>
       </c>
-      <c r="V17" s="2">
+      <c r="V17" s="1">
         <v>46229</v>
       </c>
     </row>
@@ -1871,7 +1845,7 @@
       <c r="G18" t="s">
         <v>109</v>
       </c>
-      <c r="H18" s="2">
+      <c r="H18" s="1">
         <v>46098</v>
       </c>
       <c r="I18" t="s">
@@ -1904,7 +1878,7 @@
       <c r="U18" t="s">
         <v>180</v>
       </c>
-      <c r="V18" s="2">
+      <c r="V18" s="1">
         <v>46107</v>
       </c>
     </row>
@@ -1930,7 +1904,7 @@
       <c r="G19" t="s">
         <v>109</v>
       </c>
-      <c r="H19" s="2">
+      <c r="H19" s="1">
         <v>46076</v>
       </c>
       <c r="I19" t="s">
@@ -1960,7 +1934,7 @@
       <c r="U19" t="s">
         <v>92</v>
       </c>
-      <c r="V19" s="2">
+      <c r="V19" s="1">
         <v>46079</v>
       </c>
     </row>
@@ -1986,7 +1960,7 @@
       <c r="G20" t="s">
         <v>109</v>
       </c>
-      <c r="H20" s="2">
+      <c r="H20" s="1">
         <v>46076</v>
       </c>
       <c r="I20" t="s">
@@ -2016,7 +1990,7 @@
       <c r="U20" t="s">
         <v>92</v>
       </c>
-      <c r="V20" s="2">
+      <c r="V20" s="1">
         <v>46079</v>
       </c>
     </row>
@@ -2063,7 +2037,7 @@
       <c r="U21" t="s">
         <v>92</v>
       </c>
-      <c r="V21" s="2">
+      <c r="V21" s="1">
         <v>46321</v>
       </c>
     </row>
@@ -2110,7 +2084,7 @@
       <c r="U22" t="s">
         <v>92</v>
       </c>
-      <c r="V22" s="2">
+      <c r="V22" s="1">
         <v>46321</v>
       </c>
     </row>
@@ -2157,7 +2131,7 @@
       <c r="U23" t="s">
         <v>92</v>
       </c>
-      <c r="V23" s="2">
+      <c r="V23" s="1">
         <v>46321</v>
       </c>
     </row>
@@ -2204,7 +2178,7 @@
       <c r="U24" t="s">
         <v>92</v>
       </c>
-      <c r="V24" s="2">
+      <c r="V24" s="1">
         <v>46321</v>
       </c>
     </row>
@@ -2230,7 +2204,7 @@
       <c r="G25" t="s">
         <v>109</v>
       </c>
-      <c r="H25" s="2">
+      <c r="H25" s="1">
         <v>46119</v>
       </c>
       <c r="I25" t="s">
@@ -2263,7 +2237,7 @@
       <c r="U25" t="s">
         <v>180</v>
       </c>
-      <c r="V25" s="2">
+      <c r="V25" s="1">
         <v>46138</v>
       </c>
     </row>
@@ -2289,7 +2263,7 @@
       <c r="G26" t="s">
         <v>109</v>
       </c>
-      <c r="H26" s="2">
+      <c r="H26" s="1">
         <v>46121</v>
       </c>
       <c r="I26" t="s">
@@ -2319,7 +2293,7 @@
       <c r="U26" t="s">
         <v>92</v>
       </c>
-      <c r="V26" s="2">
+      <c r="V26" s="1">
         <v>46138</v>
       </c>
     </row>
@@ -2345,7 +2319,7 @@
       <c r="G27" t="s">
         <v>109</v>
       </c>
-      <c r="H27" s="2">
+      <c r="H27" s="1">
         <v>46076</v>
       </c>
       <c r="I27" t="s">
@@ -2375,7 +2349,7 @@
       <c r="U27" t="s">
         <v>92</v>
       </c>
-      <c r="V27" s="2">
+      <c r="V27" s="1">
         <v>46079</v>
       </c>
     </row>
@@ -2401,7 +2375,7 @@
       <c r="G28" t="s">
         <v>107</v>
       </c>
-      <c r="H28" s="2">
+      <c r="H28" s="1">
         <v>46303</v>
       </c>
       <c r="I28" t="s">
@@ -2437,7 +2411,7 @@
       <c r="U28" t="s">
         <v>180</v>
       </c>
-      <c r="V28" s="2">
+      <c r="V28" s="1">
         <v>46291</v>
       </c>
     </row>
@@ -2463,7 +2437,7 @@
       <c r="G29" t="s">
         <v>109</v>
       </c>
-      <c r="H29" s="2">
+      <c r="H29" s="1">
         <v>46199</v>
       </c>
       <c r="I29" t="s">
@@ -2496,7 +2470,7 @@
       <c r="U29" t="s">
         <v>180</v>
       </c>
-      <c r="V29" s="2">
+      <c r="V29" s="1">
         <v>46199</v>
       </c>
     </row>
@@ -2522,7 +2496,7 @@
       <c r="G30" t="s">
         <v>109</v>
       </c>
-      <c r="H30" s="2">
+      <c r="H30" s="1">
         <v>46199</v>
       </c>
       <c r="I30" t="s">
@@ -2555,7 +2529,7 @@
       <c r="U30" t="s">
         <v>180</v>
       </c>
-      <c r="V30" s="2">
+      <c r="V30" s="1">
         <v>46199</v>
       </c>
     </row>
@@ -2581,7 +2555,7 @@
       <c r="G31" t="s">
         <v>109</v>
       </c>
-      <c r="H31" s="2">
+      <c r="H31" s="1">
         <v>46199</v>
       </c>
       <c r="I31" t="s">
@@ -2614,7 +2588,7 @@
       <c r="U31" t="s">
         <v>180</v>
       </c>
-      <c r="V31" s="2">
+      <c r="V31" s="1">
         <v>46199</v>
       </c>
     </row>
@@ -2640,7 +2614,7 @@
       <c r="G32" t="s">
         <v>109</v>
       </c>
-      <c r="H32" s="2">
+      <c r="H32" s="1">
         <v>46199</v>
       </c>
       <c r="I32" t="s">
@@ -2673,7 +2647,7 @@
       <c r="U32" t="s">
         <v>180</v>
       </c>
-      <c r="V32" s="2">
+      <c r="V32" s="1">
         <v>46199</v>
       </c>
     </row>
@@ -2726,7 +2700,7 @@
       <c r="U33" t="s">
         <v>180</v>
       </c>
-      <c r="V33" s="2">
+      <c r="V33" s="1">
         <v>46291</v>
       </c>
     </row>
@@ -2752,7 +2726,7 @@
       <c r="G34" t="s">
         <v>109</v>
       </c>
-      <c r="H34" s="2">
+      <c r="H34" s="1">
         <v>46191</v>
       </c>
       <c r="I34" t="s">
@@ -2785,7 +2759,7 @@
       <c r="U34" t="s">
         <v>180</v>
       </c>
-      <c r="V34" s="2">
+      <c r="V34" s="1">
         <v>46199</v>
       </c>
     </row>
@@ -2811,7 +2785,7 @@
       <c r="G35" t="s">
         <v>109</v>
       </c>
-      <c r="H35" s="2">
+      <c r="H35" s="1">
         <v>46119</v>
       </c>
       <c r="I35" t="s">
@@ -2841,7 +2815,7 @@
       <c r="U35" t="s">
         <v>180</v>
       </c>
-      <c r="V35" s="2">
+      <c r="V35" s="1">
         <v>46138</v>
       </c>
     </row>
@@ -2867,7 +2841,7 @@
       <c r="G36" t="s">
         <v>109</v>
       </c>
-      <c r="H36" s="2">
+      <c r="H36" s="1">
         <v>46213</v>
       </c>
       <c r="I36" t="s">
@@ -2897,7 +2871,7 @@
       <c r="U36" t="s">
         <v>92</v>
       </c>
-      <c r="V36" s="2">
+      <c r="V36" s="1">
         <v>46229</v>
       </c>
     </row>
@@ -2923,7 +2897,7 @@
       <c r="G37" t="s">
         <v>109</v>
       </c>
-      <c r="H37" s="2">
+      <c r="H37" s="1">
         <v>46175</v>
       </c>
       <c r="I37" t="s">
@@ -2953,7 +2927,7 @@
       <c r="U37" t="s">
         <v>92</v>
       </c>
-      <c r="V37" s="2">
+      <c r="V37" s="1">
         <v>46199</v>
       </c>
     </row>
@@ -2979,7 +2953,7 @@
       <c r="G38" t="s">
         <v>109</v>
       </c>
-      <c r="H38" s="2">
+      <c r="H38" s="1">
         <v>46213</v>
       </c>
       <c r="I38" t="s">
@@ -3009,7 +2983,7 @@
       <c r="U38" t="s">
         <v>92</v>
       </c>
-      <c r="V38" s="2">
+      <c r="V38" s="1">
         <v>46229</v>
       </c>
     </row>
@@ -3035,7 +3009,7 @@
       <c r="G39" t="s">
         <v>109</v>
       </c>
-      <c r="H39" s="2">
+      <c r="H39" s="1">
         <v>46199</v>
       </c>
       <c r="I39" t="s">
@@ -3065,7 +3039,7 @@
       <c r="U39" t="s">
         <v>92</v>
       </c>
-      <c r="V39" s="2">
+      <c r="V39" s="1">
         <v>46199</v>
       </c>
     </row>
@@ -3091,7 +3065,7 @@
       <c r="G40" t="s">
         <v>109</v>
       </c>
-      <c r="H40" s="2">
+      <c r="H40" s="1">
         <v>46199</v>
       </c>
       <c r="I40" t="s">
@@ -3121,7 +3095,7 @@
       <c r="U40" t="s">
         <v>92</v>
       </c>
-      <c r="V40" s="2">
+      <c r="V40" s="1">
         <v>46199</v>
       </c>
     </row>
@@ -3147,7 +3121,7 @@
       <c r="G41" t="s">
         <v>109</v>
       </c>
-      <c r="H41" s="2">
+      <c r="H41" s="1">
         <v>46204</v>
       </c>
       <c r="I41" t="s">
@@ -3177,7 +3151,7 @@
       <c r="U41" t="s">
         <v>92</v>
       </c>
-      <c r="V41" s="2">
+      <c r="V41" s="1">
         <v>46229</v>
       </c>
     </row>
@@ -3203,7 +3177,7 @@
       <c r="G42" t="s">
         <v>109</v>
       </c>
-      <c r="H42" s="2">
+      <c r="H42" s="1">
         <v>46244</v>
       </c>
       <c r="I42" t="s">
@@ -3233,7 +3207,7 @@
       <c r="U42" t="s">
         <v>92</v>
       </c>
-      <c r="V42" s="2">
+      <c r="V42" s="1">
         <v>46199</v>
       </c>
     </row>
@@ -3277,7 +3251,7 @@
       <c r="U43" t="s">
         <v>92</v>
       </c>
-      <c r="V43" s="2">
+      <c r="V43" s="1">
         <v>46260</v>
       </c>
     </row>
@@ -3303,7 +3277,7 @@
       <c r="G44" t="s">
         <v>109</v>
       </c>
-      <c r="H44" s="2">
+      <c r="H44" s="1">
         <v>46191</v>
       </c>
       <c r="I44" t="s">
@@ -3333,7 +3307,7 @@
       <c r="U44" t="s">
         <v>92</v>
       </c>
-      <c r="V44" s="2">
+      <c r="V44" s="1">
         <v>46199</v>
       </c>
     </row>
@@ -3359,7 +3333,7 @@
       <c r="G45" t="s">
         <v>109</v>
       </c>
-      <c r="H45" s="2">
+      <c r="H45" s="1">
         <v>46191</v>
       </c>
       <c r="I45" t="s">
@@ -3389,7 +3363,7 @@
       <c r="U45" t="s">
         <v>92</v>
       </c>
-      <c r="V45" s="2">
+      <c r="V45" s="1">
         <v>46199</v>
       </c>
     </row>
@@ -3415,7 +3389,7 @@
       <c r="G46" t="s">
         <v>109</v>
       </c>
-      <c r="H46" s="2">
+      <c r="H46" s="1">
         <v>46213</v>
       </c>
       <c r="I46" t="s">
@@ -3448,7 +3422,7 @@
       <c r="U46" t="s">
         <v>180</v>
       </c>
-      <c r="V46" s="2">
+      <c r="V46" s="1">
         <v>46229</v>
       </c>
     </row>
@@ -3474,7 +3448,7 @@
       <c r="G47" t="s">
         <v>109</v>
       </c>
-      <c r="H47" s="2">
+      <c r="H47" s="1">
         <v>46210</v>
       </c>
       <c r="I47" t="s">
@@ -3504,7 +3478,7 @@
       <c r="U47" t="s">
         <v>180</v>
       </c>
-      <c r="V47" s="2">
+      <c r="V47" s="1">
         <v>46229</v>
       </c>
     </row>
@@ -3551,7 +3525,7 @@
       <c r="U48" t="s">
         <v>92</v>
       </c>
-      <c r="V48" s="2">
+      <c r="V48" s="1">
         <v>46321</v>
       </c>
     </row>
@@ -3577,7 +3551,7 @@
       <c r="G49" t="s">
         <v>107</v>
       </c>
-      <c r="H49" s="2">
+      <c r="H49" s="1">
         <v>46303</v>
       </c>
       <c r="I49" t="s">
@@ -3613,7 +3587,7 @@
       <c r="U49" t="s">
         <v>180</v>
       </c>
-      <c r="V49" s="2">
+      <c r="V49" s="1">
         <v>46291</v>
       </c>
     </row>
@@ -3639,7 +3613,7 @@
       <c r="G50" t="s">
         <v>109</v>
       </c>
-      <c r="H50" s="2">
+      <c r="H50" s="1">
         <v>46176</v>
       </c>
       <c r="I50" t="s">
@@ -3672,7 +3646,7 @@
       <c r="U50" t="s">
         <v>180</v>
       </c>
-      <c r="V50" s="2">
+      <c r="V50" s="1">
         <v>46199</v>
       </c>
     </row>
@@ -3728,7 +3702,7 @@
       <c r="U51" t="s">
         <v>180</v>
       </c>
-      <c r="V51" s="2">
+      <c r="V51" s="1">
         <v>46260</v>
       </c>
     </row>
@@ -3754,7 +3728,7 @@
       <c r="G52" t="s">
         <v>109</v>
       </c>
-      <c r="H52" s="2">
+      <c r="H52" s="1">
         <v>46295</v>
       </c>
       <c r="I52" t="s">
@@ -3790,7 +3764,7 @@
       <c r="U52" t="s">
         <v>180</v>
       </c>
-      <c r="V52" s="2">
+      <c r="V52" s="1">
         <v>46291</v>
       </c>
     </row>
@@ -3843,7 +3817,7 @@
       <c r="U53" t="s">
         <v>180</v>
       </c>
-      <c r="V53" s="2">
+      <c r="V53" s="1">
         <v>46321</v>
       </c>
     </row>
@@ -3869,7 +3843,7 @@
       <c r="G54" t="s">
         <v>109</v>
       </c>
-      <c r="H54" s="2">
+      <c r="H54" s="1">
         <v>46227</v>
       </c>
       <c r="I54" t="s">
@@ -3899,7 +3873,7 @@
       <c r="U54" t="s">
         <v>180</v>
       </c>
-      <c r="V54" s="2">
+      <c r="V54" s="1">
         <v>46229</v>
       </c>
     </row>
@@ -3922,7 +3896,7 @@
       <c r="G55" t="s">
         <v>109</v>
       </c>
-      <c r="H55" s="2">
+      <c r="H55" s="1">
         <v>46280</v>
       </c>
       <c r="I55" t="s">
@@ -3952,7 +3926,7 @@
       <c r="U55" t="s">
         <v>180</v>
       </c>
-      <c r="V55" s="2">
+      <c r="V55" s="1">
         <v>46291</v>
       </c>
     </row>
@@ -3975,7 +3949,7 @@
       <c r="G56" t="s">
         <v>109</v>
       </c>
-      <c r="H56" s="2">
+      <c r="H56" s="1">
         <v>46280</v>
       </c>
       <c r="I56" t="s">
@@ -4005,7 +3979,7 @@
       <c r="U56" t="s">
         <v>180</v>
       </c>
-      <c r="V56" s="2">
+      <c r="V56" s="1">
         <v>46260</v>
       </c>
     </row>
@@ -4028,7 +4002,7 @@
       <c r="G57" t="s">
         <v>109</v>
       </c>
-      <c r="H57" s="2">
+      <c r="H57" s="1">
         <v>46295</v>
       </c>
       <c r="I57" t="s">
@@ -4058,7 +4032,7 @@
       <c r="U57" t="s">
         <v>180</v>
       </c>
-      <c r="V57" s="2">
+      <c r="V57" s="1">
         <v>46291</v>
       </c>
     </row>
@@ -4081,7 +4055,7 @@
       <c r="G58" t="s">
         <v>109</v>
       </c>
-      <c r="H58" s="2">
+      <c r="H58" s="1">
         <v>46295</v>
       </c>
       <c r="I58" t="s">
@@ -4111,7 +4085,7 @@
       <c r="U58" t="s">
         <v>180</v>
       </c>
-      <c r="V58" s="2">
+      <c r="V58" s="1">
         <v>46291</v>
       </c>
     </row>
@@ -4134,7 +4108,7 @@
       <c r="G59" t="s">
         <v>109</v>
       </c>
-      <c r="H59" s="2">
+      <c r="H59" s="1">
         <v>46304</v>
       </c>
       <c r="I59" t="s">
@@ -4164,7 +4138,7 @@
       <c r="U59" t="s">
         <v>180</v>
       </c>
-      <c r="V59" s="2">
+      <c r="V59" s="1">
         <v>46321</v>
       </c>
     </row>
@@ -4190,7 +4164,7 @@
       <c r="G60" t="s">
         <v>109</v>
       </c>
-      <c r="H60" s="2">
+      <c r="H60" s="1">
         <v>46301</v>
       </c>
       <c r="I60" t="s">
@@ -4226,7 +4200,7 @@
       <c r="U60" t="s">
         <v>180</v>
       </c>
-      <c r="V60" s="2">
+      <c r="V60" s="1">
         <v>46352</v>
       </c>
     </row>
@@ -4270,7 +4244,7 @@
       <c r="U61" t="s">
         <v>180</v>
       </c>
-      <c r="V61" s="2">
+      <c r="V61" s="1">
         <v>46107</v>
       </c>
     </row>
@@ -4314,7 +4288,7 @@
       <c r="U62" t="s">
         <v>180</v>
       </c>
-      <c r="V62" s="2">
+      <c r="V62" s="1">
         <v>46107</v>
       </c>
     </row>
@@ -4358,7 +4332,7 @@
       <c r="U63" t="s">
         <v>180</v>
       </c>
-      <c r="V63" s="2">
+      <c r="V63" s="1">
         <v>46107</v>
       </c>
     </row>
@@ -4402,7 +4376,7 @@
       <c r="U64" t="s">
         <v>180</v>
       </c>
-      <c r="V64" s="2">
+      <c r="V64" s="1">
         <v>46107</v>
       </c>
     </row>
@@ -4446,7 +4420,7 @@
       <c r="U65" t="s">
         <v>180</v>
       </c>
-      <c r="V65" s="2">
+      <c r="V65" s="1">
         <v>46107</v>
       </c>
     </row>
@@ -4490,7 +4464,7 @@
       <c r="U66" t="s">
         <v>180</v>
       </c>
-      <c r="V66" s="2">
+      <c r="V66" s="1">
         <v>46107</v>
       </c>
     </row>
@@ -4534,7 +4508,7 @@
       <c r="U67" t="s">
         <v>92</v>
       </c>
-      <c r="V67" s="2">
+      <c r="V67" s="1">
         <v>46168</v>
       </c>
     </row>
@@ -4581,7 +4555,7 @@
       <c r="U68" t="s">
         <v>92</v>
       </c>
-      <c r="V68" s="2">
+      <c r="V68" s="1">
         <v>46291</v>
       </c>
     </row>
@@ -4607,7 +4581,7 @@
       <c r="G69" t="s">
         <v>107</v>
       </c>
-      <c r="H69" s="2">
+      <c r="H69" s="1">
         <v>46303</v>
       </c>
       <c r="I69" t="s">
@@ -4643,7 +4617,7 @@
       <c r="U69" t="s">
         <v>180</v>
       </c>
-      <c r="V69" s="2">
+      <c r="V69" s="1">
         <v>46229</v>
       </c>
     </row>
@@ -4687,7 +4661,7 @@
       <c r="U70" t="s">
         <v>92</v>
       </c>
-      <c r="V70" s="2">
+      <c r="V70" s="1">
         <v>46260</v>
       </c>
     </row>
@@ -4731,7 +4705,7 @@
       <c r="U71" t="s">
         <v>180</v>
       </c>
-      <c r="V71" s="2">
+      <c r="V71" s="1">
         <v>46291</v>
       </c>
     </row>
@@ -4775,7 +4749,7 @@
       <c r="U72" t="s">
         <v>180</v>
       </c>
-      <c r="V72" s="2">
+      <c r="V72" s="1">
         <v>46168</v>
       </c>
     </row>
@@ -4819,7 +4793,7 @@
       <c r="U73" t="s">
         <v>180</v>
       </c>
-      <c r="V73" s="2">
+      <c r="V73" s="1">
         <v>46291</v>
       </c>
     </row>
@@ -4863,7 +4837,7 @@
       <c r="U74" t="s">
         <v>180</v>
       </c>
-      <c r="V74" s="2">
+      <c r="V74" s="1">
         <v>46291</v>
       </c>
     </row>
@@ -4907,7 +4881,7 @@
       <c r="U75" t="s">
         <v>180</v>
       </c>
-      <c r="V75" s="2">
+      <c r="V75" s="1">
         <v>46291</v>
       </c>
     </row>
@@ -4954,7 +4928,7 @@
       <c r="U76" t="s">
         <v>92</v>
       </c>
-      <c r="V76" s="2">
+      <c r="V76" s="1">
         <v>46321</v>
       </c>
     </row>
@@ -5004,7 +4978,7 @@
       <c r="U77" t="s">
         <v>180</v>
       </c>
-      <c r="V77" s="2">
+      <c r="V77" s="1">
         <v>46381</v>
       </c>
     </row>
@@ -5054,7 +5028,7 @@
       <c r="U78" t="s">
         <v>180</v>
       </c>
-      <c r="V78" s="2">
+      <c r="V78" s="1">
         <v>46381</v>
       </c>
     </row>
@@ -5104,7 +5078,7 @@
       <c r="U79" t="s">
         <v>92</v>
       </c>
-      <c r="V79" s="2">
+      <c r="V79" s="1">
         <v>46381</v>
       </c>
     </row>
@@ -5154,7 +5128,7 @@
       <c r="U80" t="s">
         <v>92</v>
       </c>
-      <c r="V80" s="2">
+      <c r="V80" s="1">
         <v>46381</v>
       </c>
     </row>
@@ -5204,7 +5178,7 @@
       <c r="U81" t="s">
         <v>92</v>
       </c>
-      <c r="V81" s="2">
+      <c r="V81" s="1">
         <v>46382</v>
       </c>
     </row>
@@ -5248,7 +5222,7 @@
       <c r="U82" t="s">
         <v>92</v>
       </c>
-      <c r="V82" s="2">
+      <c r="V82" s="1">
         <v>46382</v>
       </c>
     </row>
@@ -5304,7 +5278,7 @@
       <c r="U83" t="s">
         <v>180</v>
       </c>
-      <c r="V83" s="2">
+      <c r="V83" s="1">
         <v>46382</v>
       </c>
     </row>
@@ -5354,7 +5328,7 @@
       <c r="U84" t="s">
         <v>92</v>
       </c>
-      <c r="V84" s="2">
+      <c r="V84" s="1">
         <v>46321</v>
       </c>
     </row>
@@ -5398,7 +5372,7 @@
       <c r="U85" t="s">
         <v>92</v>
       </c>
-      <c r="V85" s="2">
+      <c r="V85" s="1">
         <v>46382</v>
       </c>
     </row>
@@ -5518,7 +5492,7 @@
       <c r="G88" t="s">
         <v>109</v>
       </c>
-      <c r="H88" s="2">
+      <c r="H88" s="1">
         <v>46303</v>
       </c>
       <c r="I88" t="s">
@@ -5548,7 +5522,7 @@
       <c r="U88" t="s">
         <v>92</v>
       </c>
-      <c r="V88" s="2">
+      <c r="V88" s="1">
         <v>46291</v>
       </c>
     </row>
@@ -5595,7 +5569,7 @@
       <c r="U89" t="s">
         <v>92</v>
       </c>
-      <c r="V89" s="2">
+      <c r="V89" s="1">
         <v>46291</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Atualização automática: mta (16/10/2026 12:02)
</commit_message>
<xml_diff>
--- a/Projetos/02_Dados_Tratados/base_mta_tratada.xlsx
+++ b/Projetos/02_Dados_Tratados/base_mta_tratada.xlsx
@@ -566,8 +566,16 @@
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="YYYY-MM-DD HH:MM:SS"/>
   </numFmts>
-  <fonts count="1">
+  <fonts count="2">
     <font>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
       <sz val="11"/>
       <color theme="1"/>
       <name val="Calibri"/>
@@ -583,7 +591,7 @@
       <patternFill patternType="gray125"/>
     </fill>
   </fills>
-  <borders count="1">
+  <borders count="2">
     <border>
       <left/>
       <right/>
@@ -591,12 +599,30 @@
       <bottom/>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin">
+        <color auto="1"/>
+      </left>
+      <right style="thin">
+        <color auto="1"/>
+      </right>
+      <top style="thin">
+        <color auto="1"/>
+      </top>
+      <bottom style="thin">
+        <color auto="1"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="3">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
   </cellXfs>
   <cellStyles count="1">
@@ -896,70 +922,70 @@
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:22">
-      <c r="A1" t="s">
+      <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
-      <c r="B1" t="s">
+      <c r="B1" s="1" t="s">
         <v>1</v>
       </c>
-      <c r="C1" t="s">
+      <c r="C1" s="1" t="s">
         <v>2</v>
       </c>
-      <c r="D1" t="s">
+      <c r="D1" s="1" t="s">
         <v>3</v>
       </c>
-      <c r="E1" t="s">
+      <c r="E1" s="1" t="s">
         <v>4</v>
       </c>
-      <c r="F1" t="s">
+      <c r="F1" s="1" t="s">
         <v>5</v>
       </c>
-      <c r="G1" t="s">
+      <c r="G1" s="1" t="s">
         <v>6</v>
       </c>
-      <c r="H1" t="s">
+      <c r="H1" s="1" t="s">
         <v>7</v>
       </c>
-      <c r="I1" t="s">
+      <c r="I1" s="1" t="s">
         <v>8</v>
       </c>
-      <c r="J1" t="s">
+      <c r="J1" s="1" t="s">
         <v>9</v>
       </c>
-      <c r="K1" t="s">
+      <c r="K1" s="1" t="s">
         <v>10</v>
       </c>
-      <c r="L1" t="s">
+      <c r="L1" s="1" t="s">
         <v>11</v>
       </c>
-      <c r="M1" t="s">
+      <c r="M1" s="1" t="s">
         <v>12</v>
       </c>
-      <c r="N1" t="s">
+      <c r="N1" s="1" t="s">
         <v>13</v>
       </c>
-      <c r="O1" t="s">
+      <c r="O1" s="1" t="s">
         <v>14</v>
       </c>
-      <c r="P1" t="s">
+      <c r="P1" s="1" t="s">
         <v>15</v>
       </c>
-      <c r="Q1" t="s">
+      <c r="Q1" s="1" t="s">
         <v>16</v>
       </c>
-      <c r="R1" t="s">
+      <c r="R1" s="1" t="s">
         <v>17</v>
       </c>
-      <c r="S1" t="s">
+      <c r="S1" s="1" t="s">
         <v>18</v>
       </c>
-      <c r="T1" t="s">
+      <c r="T1" s="1" t="s">
         <v>19</v>
       </c>
-      <c r="U1" t="s">
+      <c r="U1" s="1" t="s">
         <v>20</v>
       </c>
-      <c r="V1" t="s">
+      <c r="V1" s="1" t="s">
         <v>21</v>
       </c>
     </row>
@@ -985,7 +1011,7 @@
       <c r="G2" t="s">
         <v>107</v>
       </c>
-      <c r="H2" s="1">
+      <c r="H2" s="2">
         <v>46303</v>
       </c>
       <c r="I2" t="s">
@@ -1024,7 +1050,7 @@
       <c r="U2" t="s">
         <v>180</v>
       </c>
-      <c r="V2" s="1">
+      <c r="V2" s="2">
         <v>46229</v>
       </c>
     </row>
@@ -1071,7 +1097,7 @@
       <c r="U3" t="s">
         <v>92</v>
       </c>
-      <c r="V3" s="1">
+      <c r="V3" s="2">
         <v>46291</v>
       </c>
     </row>
@@ -1118,7 +1144,7 @@
       <c r="U4" t="s">
         <v>92</v>
       </c>
-      <c r="V4" s="1">
+      <c r="V4" s="2">
         <v>46321</v>
       </c>
     </row>
@@ -1165,7 +1191,7 @@
       <c r="U5" t="s">
         <v>92</v>
       </c>
-      <c r="V5" s="1">
+      <c r="V5" s="2">
         <v>46321</v>
       </c>
     </row>
@@ -1215,7 +1241,7 @@
       <c r="U6" t="s">
         <v>92</v>
       </c>
-      <c r="V6" s="1">
+      <c r="V6" s="2">
         <v>46291</v>
       </c>
     </row>
@@ -1241,7 +1267,7 @@
       <c r="G7" t="s">
         <v>109</v>
       </c>
-      <c r="H7" s="1">
+      <c r="H7" s="2">
         <v>46121</v>
       </c>
       <c r="I7" t="s">
@@ -1271,7 +1297,7 @@
       <c r="U7" t="s">
         <v>92</v>
       </c>
-      <c r="V7" s="1">
+      <c r="V7" s="2">
         <v>46138</v>
       </c>
     </row>
@@ -1318,7 +1344,7 @@
       <c r="U8" t="s">
         <v>92</v>
       </c>
-      <c r="V8" s="1">
+      <c r="V8" s="2">
         <v>46291</v>
       </c>
     </row>
@@ -1365,7 +1391,7 @@
       <c r="U9" t="s">
         <v>92</v>
       </c>
-      <c r="V9" s="1">
+      <c r="V9" s="2">
         <v>46291</v>
       </c>
     </row>
@@ -1388,7 +1414,7 @@
       <c r="G10" t="s">
         <v>109</v>
       </c>
-      <c r="H10" s="1">
+      <c r="H10" s="2">
         <v>46303</v>
       </c>
       <c r="I10" t="s">
@@ -1418,7 +1444,7 @@
       <c r="U10" t="s">
         <v>92</v>
       </c>
-      <c r="V10" s="1">
+      <c r="V10" s="2">
         <v>46291</v>
       </c>
     </row>
@@ -1465,7 +1491,7 @@
       <c r="U11" t="s">
         <v>92</v>
       </c>
-      <c r="V11" s="1">
+      <c r="V11" s="2">
         <v>46291</v>
       </c>
     </row>
@@ -1512,7 +1538,7 @@
       <c r="U12" t="s">
         <v>92</v>
       </c>
-      <c r="V12" s="1">
+      <c r="V12" s="2">
         <v>46291</v>
       </c>
     </row>
@@ -1538,7 +1564,7 @@
       <c r="G13" t="s">
         <v>109</v>
       </c>
-      <c r="H13" s="1">
+      <c r="H13" s="2">
         <v>46079</v>
       </c>
       <c r="I13" t="s">
@@ -1571,7 +1597,7 @@
       <c r="U13" t="s">
         <v>180</v>
       </c>
-      <c r="V13" s="1">
+      <c r="V13" s="2">
         <v>46079</v>
       </c>
     </row>
@@ -1597,7 +1623,7 @@
       <c r="G14" t="s">
         <v>107</v>
       </c>
-      <c r="H14" s="1">
+      <c r="H14" s="2">
         <v>46303</v>
       </c>
       <c r="I14" t="s">
@@ -1633,7 +1659,7 @@
       <c r="U14" t="s">
         <v>180</v>
       </c>
-      <c r="V14" s="1">
+      <c r="V14" s="2">
         <v>46352</v>
       </c>
     </row>
@@ -1659,7 +1685,7 @@
       <c r="G15" t="s">
         <v>107</v>
       </c>
-      <c r="H15" s="1">
+      <c r="H15" s="2">
         <v>46303</v>
       </c>
       <c r="I15" t="s">
@@ -1695,7 +1721,7 @@
       <c r="U15" t="s">
         <v>180</v>
       </c>
-      <c r="V15" s="1">
+      <c r="V15" s="2">
         <v>46352</v>
       </c>
     </row>
@@ -1721,7 +1747,7 @@
       <c r="G16" t="s">
         <v>107</v>
       </c>
-      <c r="H16" s="1">
+      <c r="H16" s="2">
         <v>46303</v>
       </c>
       <c r="I16" t="s">
@@ -1757,7 +1783,7 @@
       <c r="U16" t="s">
         <v>180</v>
       </c>
-      <c r="V16" s="1">
+      <c r="V16" s="2">
         <v>46352</v>
       </c>
     </row>
@@ -1783,7 +1809,7 @@
       <c r="G17" t="s">
         <v>107</v>
       </c>
-      <c r="H17" s="1">
+      <c r="H17" s="2">
         <v>46303</v>
       </c>
       <c r="I17" t="s">
@@ -1819,7 +1845,7 @@
       <c r="U17" t="s">
         <v>180</v>
       </c>
-      <c r="V17" s="1">
+      <c r="V17" s="2">
         <v>46229</v>
       </c>
     </row>
@@ -1845,7 +1871,7 @@
       <c r="G18" t="s">
         <v>109</v>
       </c>
-      <c r="H18" s="1">
+      <c r="H18" s="2">
         <v>46098</v>
       </c>
       <c r="I18" t="s">
@@ -1878,7 +1904,7 @@
       <c r="U18" t="s">
         <v>180</v>
       </c>
-      <c r="V18" s="1">
+      <c r="V18" s="2">
         <v>46107</v>
       </c>
     </row>
@@ -1904,7 +1930,7 @@
       <c r="G19" t="s">
         <v>109</v>
       </c>
-      <c r="H19" s="1">
+      <c r="H19" s="2">
         <v>46076</v>
       </c>
       <c r="I19" t="s">
@@ -1934,7 +1960,7 @@
       <c r="U19" t="s">
         <v>92</v>
       </c>
-      <c r="V19" s="1">
+      <c r="V19" s="2">
         <v>46079</v>
       </c>
     </row>
@@ -1960,7 +1986,7 @@
       <c r="G20" t="s">
         <v>109</v>
       </c>
-      <c r="H20" s="1">
+      <c r="H20" s="2">
         <v>46076</v>
       </c>
       <c r="I20" t="s">
@@ -1990,7 +2016,7 @@
       <c r="U20" t="s">
         <v>92</v>
       </c>
-      <c r="V20" s="1">
+      <c r="V20" s="2">
         <v>46079</v>
       </c>
     </row>
@@ -2037,7 +2063,7 @@
       <c r="U21" t="s">
         <v>92</v>
       </c>
-      <c r="V21" s="1">
+      <c r="V21" s="2">
         <v>46321</v>
       </c>
     </row>
@@ -2084,7 +2110,7 @@
       <c r="U22" t="s">
         <v>92</v>
       </c>
-      <c r="V22" s="1">
+      <c r="V22" s="2">
         <v>46321</v>
       </c>
     </row>
@@ -2131,7 +2157,7 @@
       <c r="U23" t="s">
         <v>92</v>
       </c>
-      <c r="V23" s="1">
+      <c r="V23" s="2">
         <v>46321</v>
       </c>
     </row>
@@ -2178,7 +2204,7 @@
       <c r="U24" t="s">
         <v>92</v>
       </c>
-      <c r="V24" s="1">
+      <c r="V24" s="2">
         <v>46321</v>
       </c>
     </row>
@@ -2204,7 +2230,7 @@
       <c r="G25" t="s">
         <v>109</v>
       </c>
-      <c r="H25" s="1">
+      <c r="H25" s="2">
         <v>46119</v>
       </c>
       <c r="I25" t="s">
@@ -2237,7 +2263,7 @@
       <c r="U25" t="s">
         <v>180</v>
       </c>
-      <c r="V25" s="1">
+      <c r="V25" s="2">
         <v>46138</v>
       </c>
     </row>
@@ -2263,7 +2289,7 @@
       <c r="G26" t="s">
         <v>109</v>
       </c>
-      <c r="H26" s="1">
+      <c r="H26" s="2">
         <v>46121</v>
       </c>
       <c r="I26" t="s">
@@ -2293,7 +2319,7 @@
       <c r="U26" t="s">
         <v>92</v>
       </c>
-      <c r="V26" s="1">
+      <c r="V26" s="2">
         <v>46138</v>
       </c>
     </row>
@@ -2319,7 +2345,7 @@
       <c r="G27" t="s">
         <v>109</v>
       </c>
-      <c r="H27" s="1">
+      <c r="H27" s="2">
         <v>46076</v>
       </c>
       <c r="I27" t="s">
@@ -2349,7 +2375,7 @@
       <c r="U27" t="s">
         <v>92</v>
       </c>
-      <c r="V27" s="1">
+      <c r="V27" s="2">
         <v>46079</v>
       </c>
     </row>
@@ -2375,7 +2401,7 @@
       <c r="G28" t="s">
         <v>107</v>
       </c>
-      <c r="H28" s="1">
+      <c r="H28" s="2">
         <v>46303</v>
       </c>
       <c r="I28" t="s">
@@ -2411,7 +2437,7 @@
       <c r="U28" t="s">
         <v>180</v>
       </c>
-      <c r="V28" s="1">
+      <c r="V28" s="2">
         <v>46291</v>
       </c>
     </row>
@@ -2437,7 +2463,7 @@
       <c r="G29" t="s">
         <v>109</v>
       </c>
-      <c r="H29" s="1">
+      <c r="H29" s="2">
         <v>46199</v>
       </c>
       <c r="I29" t="s">
@@ -2470,7 +2496,7 @@
       <c r="U29" t="s">
         <v>180</v>
       </c>
-      <c r="V29" s="1">
+      <c r="V29" s="2">
         <v>46199</v>
       </c>
     </row>
@@ -2496,7 +2522,7 @@
       <c r="G30" t="s">
         <v>109</v>
       </c>
-      <c r="H30" s="1">
+      <c r="H30" s="2">
         <v>46199</v>
       </c>
       <c r="I30" t="s">
@@ -2529,7 +2555,7 @@
       <c r="U30" t="s">
         <v>180</v>
       </c>
-      <c r="V30" s="1">
+      <c r="V30" s="2">
         <v>46199</v>
       </c>
     </row>
@@ -2555,7 +2581,7 @@
       <c r="G31" t="s">
         <v>109</v>
       </c>
-      <c r="H31" s="1">
+      <c r="H31" s="2">
         <v>46199</v>
       </c>
       <c r="I31" t="s">
@@ -2588,7 +2614,7 @@
       <c r="U31" t="s">
         <v>180</v>
       </c>
-      <c r="V31" s="1">
+      <c r="V31" s="2">
         <v>46199</v>
       </c>
     </row>
@@ -2614,7 +2640,7 @@
       <c r="G32" t="s">
         <v>109</v>
       </c>
-      <c r="H32" s="1">
+      <c r="H32" s="2">
         <v>46199</v>
       </c>
       <c r="I32" t="s">
@@ -2647,7 +2673,7 @@
       <c r="U32" t="s">
         <v>180</v>
       </c>
-      <c r="V32" s="1">
+      <c r="V32" s="2">
         <v>46199</v>
       </c>
     </row>
@@ -2700,7 +2726,7 @@
       <c r="U33" t="s">
         <v>180</v>
       </c>
-      <c r="V33" s="1">
+      <c r="V33" s="2">
         <v>46291</v>
       </c>
     </row>
@@ -2726,7 +2752,7 @@
       <c r="G34" t="s">
         <v>109</v>
       </c>
-      <c r="H34" s="1">
+      <c r="H34" s="2">
         <v>46191</v>
       </c>
       <c r="I34" t="s">
@@ -2759,7 +2785,7 @@
       <c r="U34" t="s">
         <v>180</v>
       </c>
-      <c r="V34" s="1">
+      <c r="V34" s="2">
         <v>46199</v>
       </c>
     </row>
@@ -2785,7 +2811,7 @@
       <c r="G35" t="s">
         <v>109</v>
       </c>
-      <c r="H35" s="1">
+      <c r="H35" s="2">
         <v>46119</v>
       </c>
       <c r="I35" t="s">
@@ -2815,7 +2841,7 @@
       <c r="U35" t="s">
         <v>180</v>
       </c>
-      <c r="V35" s="1">
+      <c r="V35" s="2">
         <v>46138</v>
       </c>
     </row>
@@ -2841,7 +2867,7 @@
       <c r="G36" t="s">
         <v>109</v>
       </c>
-      <c r="H36" s="1">
+      <c r="H36" s="2">
         <v>46213</v>
       </c>
       <c r="I36" t="s">
@@ -2871,7 +2897,7 @@
       <c r="U36" t="s">
         <v>92</v>
       </c>
-      <c r="V36" s="1">
+      <c r="V36" s="2">
         <v>46229</v>
       </c>
     </row>
@@ -2897,7 +2923,7 @@
       <c r="G37" t="s">
         <v>109</v>
       </c>
-      <c r="H37" s="1">
+      <c r="H37" s="2">
         <v>46175</v>
       </c>
       <c r="I37" t="s">
@@ -2927,7 +2953,7 @@
       <c r="U37" t="s">
         <v>92</v>
       </c>
-      <c r="V37" s="1">
+      <c r="V37" s="2">
         <v>46199</v>
       </c>
     </row>
@@ -2953,7 +2979,7 @@
       <c r="G38" t="s">
         <v>109</v>
       </c>
-      <c r="H38" s="1">
+      <c r="H38" s="2">
         <v>46213</v>
       </c>
       <c r="I38" t="s">
@@ -2983,7 +3009,7 @@
       <c r="U38" t="s">
         <v>92</v>
       </c>
-      <c r="V38" s="1">
+      <c r="V38" s="2">
         <v>46229</v>
       </c>
     </row>
@@ -3009,7 +3035,7 @@
       <c r="G39" t="s">
         <v>109</v>
       </c>
-      <c r="H39" s="1">
+      <c r="H39" s="2">
         <v>46199</v>
       </c>
       <c r="I39" t="s">
@@ -3039,7 +3065,7 @@
       <c r="U39" t="s">
         <v>92</v>
       </c>
-      <c r="V39" s="1">
+      <c r="V39" s="2">
         <v>46199</v>
       </c>
     </row>
@@ -3065,7 +3091,7 @@
       <c r="G40" t="s">
         <v>109</v>
       </c>
-      <c r="H40" s="1">
+      <c r="H40" s="2">
         <v>46199</v>
       </c>
       <c r="I40" t="s">
@@ -3095,7 +3121,7 @@
       <c r="U40" t="s">
         <v>92</v>
       </c>
-      <c r="V40" s="1">
+      <c r="V40" s="2">
         <v>46199</v>
       </c>
     </row>
@@ -3121,7 +3147,7 @@
       <c r="G41" t="s">
         <v>109</v>
       </c>
-      <c r="H41" s="1">
+      <c r="H41" s="2">
         <v>46204</v>
       </c>
       <c r="I41" t="s">
@@ -3151,7 +3177,7 @@
       <c r="U41" t="s">
         <v>92</v>
       </c>
-      <c r="V41" s="1">
+      <c r="V41" s="2">
         <v>46229</v>
       </c>
     </row>
@@ -3177,7 +3203,7 @@
       <c r="G42" t="s">
         <v>109</v>
       </c>
-      <c r="H42" s="1">
+      <c r="H42" s="2">
         <v>46244</v>
       </c>
       <c r="I42" t="s">
@@ -3207,7 +3233,7 @@
       <c r="U42" t="s">
         <v>92</v>
       </c>
-      <c r="V42" s="1">
+      <c r="V42" s="2">
         <v>46199</v>
       </c>
     </row>
@@ -3251,7 +3277,7 @@
       <c r="U43" t="s">
         <v>92</v>
       </c>
-      <c r="V43" s="1">
+      <c r="V43" s="2">
         <v>46260</v>
       </c>
     </row>
@@ -3277,7 +3303,7 @@
       <c r="G44" t="s">
         <v>109</v>
       </c>
-      <c r="H44" s="1">
+      <c r="H44" s="2">
         <v>46191</v>
       </c>
       <c r="I44" t="s">
@@ -3307,7 +3333,7 @@
       <c r="U44" t="s">
         <v>92</v>
       </c>
-      <c r="V44" s="1">
+      <c r="V44" s="2">
         <v>46199</v>
       </c>
     </row>
@@ -3333,7 +3359,7 @@
       <c r="G45" t="s">
         <v>109</v>
       </c>
-      <c r="H45" s="1">
+      <c r="H45" s="2">
         <v>46191</v>
       </c>
       <c r="I45" t="s">
@@ -3363,7 +3389,7 @@
       <c r="U45" t="s">
         <v>92</v>
       </c>
-      <c r="V45" s="1">
+      <c r="V45" s="2">
         <v>46199</v>
       </c>
     </row>
@@ -3389,7 +3415,7 @@
       <c r="G46" t="s">
         <v>109</v>
       </c>
-      <c r="H46" s="1">
+      <c r="H46" s="2">
         <v>46213</v>
       </c>
       <c r="I46" t="s">
@@ -3422,7 +3448,7 @@
       <c r="U46" t="s">
         <v>180</v>
       </c>
-      <c r="V46" s="1">
+      <c r="V46" s="2">
         <v>46229</v>
       </c>
     </row>
@@ -3448,7 +3474,7 @@
       <c r="G47" t="s">
         <v>109</v>
       </c>
-      <c r="H47" s="1">
+      <c r="H47" s="2">
         <v>46210</v>
       </c>
       <c r="I47" t="s">
@@ -3478,7 +3504,7 @@
       <c r="U47" t="s">
         <v>180</v>
       </c>
-      <c r="V47" s="1">
+      <c r="V47" s="2">
         <v>46229</v>
       </c>
     </row>
@@ -3525,7 +3551,7 @@
       <c r="U48" t="s">
         <v>92</v>
       </c>
-      <c r="V48" s="1">
+      <c r="V48" s="2">
         <v>46321</v>
       </c>
     </row>
@@ -3551,7 +3577,7 @@
       <c r="G49" t="s">
         <v>107</v>
       </c>
-      <c r="H49" s="1">
+      <c r="H49" s="2">
         <v>46303</v>
       </c>
       <c r="I49" t="s">
@@ -3587,7 +3613,7 @@
       <c r="U49" t="s">
         <v>180</v>
       </c>
-      <c r="V49" s="1">
+      <c r="V49" s="2">
         <v>46291</v>
       </c>
     </row>
@@ -3613,7 +3639,7 @@
       <c r="G50" t="s">
         <v>109</v>
       </c>
-      <c r="H50" s="1">
+      <c r="H50" s="2">
         <v>46176</v>
       </c>
       <c r="I50" t="s">
@@ -3646,7 +3672,7 @@
       <c r="U50" t="s">
         <v>180</v>
       </c>
-      <c r="V50" s="1">
+      <c r="V50" s="2">
         <v>46199</v>
       </c>
     </row>
@@ -3702,7 +3728,7 @@
       <c r="U51" t="s">
         <v>180</v>
       </c>
-      <c r="V51" s="1">
+      <c r="V51" s="2">
         <v>46260</v>
       </c>
     </row>
@@ -3728,7 +3754,7 @@
       <c r="G52" t="s">
         <v>109</v>
       </c>
-      <c r="H52" s="1">
+      <c r="H52" s="2">
         <v>46295</v>
       </c>
       <c r="I52" t="s">
@@ -3764,7 +3790,7 @@
       <c r="U52" t="s">
         <v>180</v>
       </c>
-      <c r="V52" s="1">
+      <c r="V52" s="2">
         <v>46291</v>
       </c>
     </row>
@@ -3817,7 +3843,7 @@
       <c r="U53" t="s">
         <v>180</v>
       </c>
-      <c r="V53" s="1">
+      <c r="V53" s="2">
         <v>46321</v>
       </c>
     </row>
@@ -3843,7 +3869,7 @@
       <c r="G54" t="s">
         <v>109</v>
       </c>
-      <c r="H54" s="1">
+      <c r="H54" s="2">
         <v>46227</v>
       </c>
       <c r="I54" t="s">
@@ -3873,7 +3899,7 @@
       <c r="U54" t="s">
         <v>180</v>
       </c>
-      <c r="V54" s="1">
+      <c r="V54" s="2">
         <v>46229</v>
       </c>
     </row>
@@ -3896,7 +3922,7 @@
       <c r="G55" t="s">
         <v>109</v>
       </c>
-      <c r="H55" s="1">
+      <c r="H55" s="2">
         <v>46280</v>
       </c>
       <c r="I55" t="s">
@@ -3926,7 +3952,7 @@
       <c r="U55" t="s">
         <v>180</v>
       </c>
-      <c r="V55" s="1">
+      <c r="V55" s="2">
         <v>46291</v>
       </c>
     </row>
@@ -3949,7 +3975,7 @@
       <c r="G56" t="s">
         <v>109</v>
       </c>
-      <c r="H56" s="1">
+      <c r="H56" s="2">
         <v>46280</v>
       </c>
       <c r="I56" t="s">
@@ -3979,7 +4005,7 @@
       <c r="U56" t="s">
         <v>180</v>
       </c>
-      <c r="V56" s="1">
+      <c r="V56" s="2">
         <v>46260</v>
       </c>
     </row>
@@ -4002,7 +4028,7 @@
       <c r="G57" t="s">
         <v>109</v>
       </c>
-      <c r="H57" s="1">
+      <c r="H57" s="2">
         <v>46295</v>
       </c>
       <c r="I57" t="s">
@@ -4032,7 +4058,7 @@
       <c r="U57" t="s">
         <v>180</v>
       </c>
-      <c r="V57" s="1">
+      <c r="V57" s="2">
         <v>46291</v>
       </c>
     </row>
@@ -4055,7 +4081,7 @@
       <c r="G58" t="s">
         <v>109</v>
       </c>
-      <c r="H58" s="1">
+      <c r="H58" s="2">
         <v>46295</v>
       </c>
       <c r="I58" t="s">
@@ -4085,7 +4111,7 @@
       <c r="U58" t="s">
         <v>180</v>
       </c>
-      <c r="V58" s="1">
+      <c r="V58" s="2">
         <v>46291</v>
       </c>
     </row>
@@ -4108,7 +4134,7 @@
       <c r="G59" t="s">
         <v>109</v>
       </c>
-      <c r="H59" s="1">
+      <c r="H59" s="2">
         <v>46304</v>
       </c>
       <c r="I59" t="s">
@@ -4138,7 +4164,7 @@
       <c r="U59" t="s">
         <v>180</v>
       </c>
-      <c r="V59" s="1">
+      <c r="V59" s="2">
         <v>46321</v>
       </c>
     </row>
@@ -4164,7 +4190,7 @@
       <c r="G60" t="s">
         <v>109</v>
       </c>
-      <c r="H60" s="1">
+      <c r="H60" s="2">
         <v>46301</v>
       </c>
       <c r="I60" t="s">
@@ -4200,7 +4226,7 @@
       <c r="U60" t="s">
         <v>180</v>
       </c>
-      <c r="V60" s="1">
+      <c r="V60" s="2">
         <v>46352</v>
       </c>
     </row>
@@ -4244,7 +4270,7 @@
       <c r="U61" t="s">
         <v>180</v>
       </c>
-      <c r="V61" s="1">
+      <c r="V61" s="2">
         <v>46107</v>
       </c>
     </row>
@@ -4288,7 +4314,7 @@
       <c r="U62" t="s">
         <v>180</v>
       </c>
-      <c r="V62" s="1">
+      <c r="V62" s="2">
         <v>46107</v>
       </c>
     </row>
@@ -4332,7 +4358,7 @@
       <c r="U63" t="s">
         <v>180</v>
       </c>
-      <c r="V63" s="1">
+      <c r="V63" s="2">
         <v>46107</v>
       </c>
     </row>
@@ -4376,7 +4402,7 @@
       <c r="U64" t="s">
         <v>180</v>
       </c>
-      <c r="V64" s="1">
+      <c r="V64" s="2">
         <v>46107</v>
       </c>
     </row>
@@ -4420,7 +4446,7 @@
       <c r="U65" t="s">
         <v>180</v>
       </c>
-      <c r="V65" s="1">
+      <c r="V65" s="2">
         <v>46107</v>
       </c>
     </row>
@@ -4464,7 +4490,7 @@
       <c r="U66" t="s">
         <v>180</v>
       </c>
-      <c r="V66" s="1">
+      <c r="V66" s="2">
         <v>46107</v>
       </c>
     </row>
@@ -4508,7 +4534,7 @@
       <c r="U67" t="s">
         <v>92</v>
       </c>
-      <c r="V67" s="1">
+      <c r="V67" s="2">
         <v>46168</v>
       </c>
     </row>
@@ -4555,7 +4581,7 @@
       <c r="U68" t="s">
         <v>92</v>
       </c>
-      <c r="V68" s="1">
+      <c r="V68" s="2">
         <v>46291</v>
       </c>
     </row>
@@ -4581,7 +4607,7 @@
       <c r="G69" t="s">
         <v>107</v>
       </c>
-      <c r="H69" s="1">
+      <c r="H69" s="2">
         <v>46303</v>
       </c>
       <c r="I69" t="s">
@@ -4617,7 +4643,7 @@
       <c r="U69" t="s">
         <v>180</v>
       </c>
-      <c r="V69" s="1">
+      <c r="V69" s="2">
         <v>46229</v>
       </c>
     </row>
@@ -4661,7 +4687,7 @@
       <c r="U70" t="s">
         <v>92</v>
       </c>
-      <c r="V70" s="1">
+      <c r="V70" s="2">
         <v>46260</v>
       </c>
     </row>
@@ -4705,7 +4731,7 @@
       <c r="U71" t="s">
         <v>180</v>
       </c>
-      <c r="V71" s="1">
+      <c r="V71" s="2">
         <v>46291</v>
       </c>
     </row>
@@ -4749,7 +4775,7 @@
       <c r="U72" t="s">
         <v>180</v>
       </c>
-      <c r="V72" s="1">
+      <c r="V72" s="2">
         <v>46168</v>
       </c>
     </row>
@@ -4793,7 +4819,7 @@
       <c r="U73" t="s">
         <v>180</v>
       </c>
-      <c r="V73" s="1">
+      <c r="V73" s="2">
         <v>46291</v>
       </c>
     </row>
@@ -4837,7 +4863,7 @@
       <c r="U74" t="s">
         <v>180</v>
       </c>
-      <c r="V74" s="1">
+      <c r="V74" s="2">
         <v>46291</v>
       </c>
     </row>
@@ -4881,7 +4907,7 @@
       <c r="U75" t="s">
         <v>180</v>
       </c>
-      <c r="V75" s="1">
+      <c r="V75" s="2">
         <v>46291</v>
       </c>
     </row>
@@ -4928,7 +4954,7 @@
       <c r="U76" t="s">
         <v>92</v>
       </c>
-      <c r="V76" s="1">
+      <c r="V76" s="2">
         <v>46321</v>
       </c>
     </row>
@@ -4978,7 +5004,7 @@
       <c r="U77" t="s">
         <v>180</v>
       </c>
-      <c r="V77" s="1">
+      <c r="V77" s="2">
         <v>46381</v>
       </c>
     </row>
@@ -5028,7 +5054,7 @@
       <c r="U78" t="s">
         <v>180</v>
       </c>
-      <c r="V78" s="1">
+      <c r="V78" s="2">
         <v>46381</v>
       </c>
     </row>
@@ -5078,7 +5104,7 @@
       <c r="U79" t="s">
         <v>92</v>
       </c>
-      <c r="V79" s="1">
+      <c r="V79" s="2">
         <v>46381</v>
       </c>
     </row>
@@ -5128,7 +5154,7 @@
       <c r="U80" t="s">
         <v>92</v>
       </c>
-      <c r="V80" s="1">
+      <c r="V80" s="2">
         <v>46381</v>
       </c>
     </row>
@@ -5178,7 +5204,7 @@
       <c r="U81" t="s">
         <v>92</v>
       </c>
-      <c r="V81" s="1">
+      <c r="V81" s="2">
         <v>46382</v>
       </c>
     </row>
@@ -5222,7 +5248,7 @@
       <c r="U82" t="s">
         <v>92</v>
       </c>
-      <c r="V82" s="1">
+      <c r="V82" s="2">
         <v>46382</v>
       </c>
     </row>
@@ -5278,7 +5304,7 @@
       <c r="U83" t="s">
         <v>180</v>
       </c>
-      <c r="V83" s="1">
+      <c r="V83" s="2">
         <v>46382</v>
       </c>
     </row>
@@ -5328,7 +5354,7 @@
       <c r="U84" t="s">
         <v>92</v>
       </c>
-      <c r="V84" s="1">
+      <c r="V84" s="2">
         <v>46321</v>
       </c>
     </row>
@@ -5372,7 +5398,7 @@
       <c r="U85" t="s">
         <v>92</v>
       </c>
-      <c r="V85" s="1">
+      <c r="V85" s="2">
         <v>46382</v>
       </c>
     </row>
@@ -5492,7 +5518,7 @@
       <c r="G88" t="s">
         <v>109</v>
       </c>
-      <c r="H88" s="1">
+      <c r="H88" s="2">
         <v>46303</v>
       </c>
       <c r="I88" t="s">
@@ -5522,7 +5548,7 @@
       <c r="U88" t="s">
         <v>92</v>
       </c>
-      <c r="V88" s="1">
+      <c r="V88" s="2">
         <v>46291</v>
       </c>
     </row>
@@ -5569,7 +5595,7 @@
       <c r="U89" t="s">
         <v>92</v>
       </c>
-      <c r="V89" s="1">
+      <c r="V89" s="2">
         <v>46291</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Atualização automática: mta (16/10/2026 12:21)
</commit_message>
<xml_diff>
--- a/Projetos/02_Dados_Tratados/base_mta_tratada.xlsx
+++ b/Projetos/02_Dados_Tratados/base_mta_tratada.xlsx
@@ -566,16 +566,8 @@
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="YYYY-MM-DD HH:MM:SS"/>
   </numFmts>
-  <fonts count="2">
+  <fonts count="1">
     <font>
-      <sz val="11"/>
-      <color theme="1"/>
-      <name val="Calibri"/>
-      <family val="2"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <b/>
       <sz val="11"/>
       <color theme="1"/>
       <name val="Calibri"/>
@@ -591,7 +583,7 @@
       <patternFill patternType="gray125"/>
     </fill>
   </fills>
-  <borders count="2">
+  <borders count="1">
     <border>
       <left/>
       <right/>
@@ -599,30 +591,12 @@
       <bottom/>
       <diagonal/>
     </border>
-    <border>
-      <left style="thin">
-        <color auto="1"/>
-      </left>
-      <right style="thin">
-        <color auto="1"/>
-      </right>
-      <top style="thin">
-        <color auto="1"/>
-      </top>
-      <bottom style="thin">
-        <color auto="1"/>
-      </bottom>
-      <diagonal/>
-    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="3">
+  <cellXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top"/>
-    </xf>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
   </cellXfs>
   <cellStyles count="1">
@@ -922,70 +896,70 @@
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:22">
-      <c r="A1" s="1" t="s">
+      <c r="A1" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="1" t="s">
+      <c r="B1" t="s">
         <v>1</v>
       </c>
-      <c r="C1" s="1" t="s">
+      <c r="C1" t="s">
         <v>2</v>
       </c>
-      <c r="D1" s="1" t="s">
+      <c r="D1" t="s">
         <v>3</v>
       </c>
-      <c r="E1" s="1" t="s">
+      <c r="E1" t="s">
         <v>4</v>
       </c>
-      <c r="F1" s="1" t="s">
+      <c r="F1" t="s">
         <v>5</v>
       </c>
-      <c r="G1" s="1" t="s">
+      <c r="G1" t="s">
         <v>6</v>
       </c>
-      <c r="H1" s="1" t="s">
+      <c r="H1" t="s">
         <v>7</v>
       </c>
-      <c r="I1" s="1" t="s">
+      <c r="I1" t="s">
         <v>8</v>
       </c>
-      <c r="J1" s="1" t="s">
+      <c r="J1" t="s">
         <v>9</v>
       </c>
-      <c r="K1" s="1" t="s">
+      <c r="K1" t="s">
         <v>10</v>
       </c>
-      <c r="L1" s="1" t="s">
+      <c r="L1" t="s">
         <v>11</v>
       </c>
-      <c r="M1" s="1" t="s">
+      <c r="M1" t="s">
         <v>12</v>
       </c>
-      <c r="N1" s="1" t="s">
+      <c r="N1" t="s">
         <v>13</v>
       </c>
-      <c r="O1" s="1" t="s">
+      <c r="O1" t="s">
         <v>14</v>
       </c>
-      <c r="P1" s="1" t="s">
+      <c r="P1" t="s">
         <v>15</v>
       </c>
-      <c r="Q1" s="1" t="s">
+      <c r="Q1" t="s">
         <v>16</v>
       </c>
-      <c r="R1" s="1" t="s">
+      <c r="R1" t="s">
         <v>17</v>
       </c>
-      <c r="S1" s="1" t="s">
+      <c r="S1" t="s">
         <v>18</v>
       </c>
-      <c r="T1" s="1" t="s">
+      <c r="T1" t="s">
         <v>19</v>
       </c>
-      <c r="U1" s="1" t="s">
+      <c r="U1" t="s">
         <v>20</v>
       </c>
-      <c r="V1" s="1" t="s">
+      <c r="V1" t="s">
         <v>21</v>
       </c>
     </row>
@@ -1011,7 +985,7 @@
       <c r="G2" t="s">
         <v>107</v>
       </c>
-      <c r="H2" s="2">
+      <c r="H2" s="1">
         <v>46303</v>
       </c>
       <c r="I2" t="s">
@@ -1050,7 +1024,7 @@
       <c r="U2" t="s">
         <v>180</v>
       </c>
-      <c r="V2" s="2">
+      <c r="V2" s="1">
         <v>46229</v>
       </c>
     </row>
@@ -1097,7 +1071,7 @@
       <c r="U3" t="s">
         <v>92</v>
       </c>
-      <c r="V3" s="2">
+      <c r="V3" s="1">
         <v>46291</v>
       </c>
     </row>
@@ -1144,7 +1118,7 @@
       <c r="U4" t="s">
         <v>92</v>
       </c>
-      <c r="V4" s="2">
+      <c r="V4" s="1">
         <v>46321</v>
       </c>
     </row>
@@ -1191,7 +1165,7 @@
       <c r="U5" t="s">
         <v>92</v>
       </c>
-      <c r="V5" s="2">
+      <c r="V5" s="1">
         <v>46321</v>
       </c>
     </row>
@@ -1241,7 +1215,7 @@
       <c r="U6" t="s">
         <v>92</v>
       </c>
-      <c r="V6" s="2">
+      <c r="V6" s="1">
         <v>46291</v>
       </c>
     </row>
@@ -1267,7 +1241,7 @@
       <c r="G7" t="s">
         <v>109</v>
       </c>
-      <c r="H7" s="2">
+      <c r="H7" s="1">
         <v>46121</v>
       </c>
       <c r="I7" t="s">
@@ -1297,7 +1271,7 @@
       <c r="U7" t="s">
         <v>92</v>
       </c>
-      <c r="V7" s="2">
+      <c r="V7" s="1">
         <v>46138</v>
       </c>
     </row>
@@ -1344,7 +1318,7 @@
       <c r="U8" t="s">
         <v>92</v>
       </c>
-      <c r="V8" s="2">
+      <c r="V8" s="1">
         <v>46291</v>
       </c>
     </row>
@@ -1391,7 +1365,7 @@
       <c r="U9" t="s">
         <v>92</v>
       </c>
-      <c r="V9" s="2">
+      <c r="V9" s="1">
         <v>46291</v>
       </c>
     </row>
@@ -1414,7 +1388,7 @@
       <c r="G10" t="s">
         <v>109</v>
       </c>
-      <c r="H10" s="2">
+      <c r="H10" s="1">
         <v>46303</v>
       </c>
       <c r="I10" t="s">
@@ -1444,7 +1418,7 @@
       <c r="U10" t="s">
         <v>92</v>
       </c>
-      <c r="V10" s="2">
+      <c r="V10" s="1">
         <v>46291</v>
       </c>
     </row>
@@ -1491,7 +1465,7 @@
       <c r="U11" t="s">
         <v>92</v>
       </c>
-      <c r="V11" s="2">
+      <c r="V11" s="1">
         <v>46291</v>
       </c>
     </row>
@@ -1538,7 +1512,7 @@
       <c r="U12" t="s">
         <v>92</v>
       </c>
-      <c r="V12" s="2">
+      <c r="V12" s="1">
         <v>46291</v>
       </c>
     </row>
@@ -1564,7 +1538,7 @@
       <c r="G13" t="s">
         <v>109</v>
       </c>
-      <c r="H13" s="2">
+      <c r="H13" s="1">
         <v>46079</v>
       </c>
       <c r="I13" t="s">
@@ -1597,7 +1571,7 @@
       <c r="U13" t="s">
         <v>180</v>
       </c>
-      <c r="V13" s="2">
+      <c r="V13" s="1">
         <v>46079</v>
       </c>
     </row>
@@ -1623,7 +1597,7 @@
       <c r="G14" t="s">
         <v>107</v>
       </c>
-      <c r="H14" s="2">
+      <c r="H14" s="1">
         <v>46303</v>
       </c>
       <c r="I14" t="s">
@@ -1659,7 +1633,7 @@
       <c r="U14" t="s">
         <v>180</v>
       </c>
-      <c r="V14" s="2">
+      <c r="V14" s="1">
         <v>46352</v>
       </c>
     </row>
@@ -1685,7 +1659,7 @@
       <c r="G15" t="s">
         <v>107</v>
       </c>
-      <c r="H15" s="2">
+      <c r="H15" s="1">
         <v>46303</v>
       </c>
       <c r="I15" t="s">
@@ -1721,7 +1695,7 @@
       <c r="U15" t="s">
         <v>180</v>
       </c>
-      <c r="V15" s="2">
+      <c r="V15" s="1">
         <v>46352</v>
       </c>
     </row>
@@ -1747,7 +1721,7 @@
       <c r="G16" t="s">
         <v>107</v>
       </c>
-      <c r="H16" s="2">
+      <c r="H16" s="1">
         <v>46303</v>
       </c>
       <c r="I16" t="s">
@@ -1783,7 +1757,7 @@
       <c r="U16" t="s">
         <v>180</v>
       </c>
-      <c r="V16" s="2">
+      <c r="V16" s="1">
         <v>46352</v>
       </c>
     </row>
@@ -1809,7 +1783,7 @@
       <c r="G17" t="s">
         <v>107</v>
       </c>
-      <c r="H17" s="2">
+      <c r="H17" s="1">
         <v>46303</v>
       </c>
       <c r="I17" t="s">
@@ -1845,7 +1819,7 @@
       <c r="U17" t="s">
         <v>180</v>
       </c>
-      <c r="V17" s="2">
+      <c r="V17" s="1">
         <v>46229</v>
       </c>
     </row>
@@ -1871,7 +1845,7 @@
       <c r="G18" t="s">
         <v>109</v>
       </c>
-      <c r="H18" s="2">
+      <c r="H18" s="1">
         <v>46098</v>
       </c>
       <c r="I18" t="s">
@@ -1904,7 +1878,7 @@
       <c r="U18" t="s">
         <v>180</v>
       </c>
-      <c r="V18" s="2">
+      <c r="V18" s="1">
         <v>46107</v>
       </c>
     </row>
@@ -1930,7 +1904,7 @@
       <c r="G19" t="s">
         <v>109</v>
       </c>
-      <c r="H19" s="2">
+      <c r="H19" s="1">
         <v>46076</v>
       </c>
       <c r="I19" t="s">
@@ -1960,7 +1934,7 @@
       <c r="U19" t="s">
         <v>92</v>
       </c>
-      <c r="V19" s="2">
+      <c r="V19" s="1">
         <v>46079</v>
       </c>
     </row>
@@ -1986,7 +1960,7 @@
       <c r="G20" t="s">
         <v>109</v>
       </c>
-      <c r="H20" s="2">
+      <c r="H20" s="1">
         <v>46076</v>
       </c>
       <c r="I20" t="s">
@@ -2016,7 +1990,7 @@
       <c r="U20" t="s">
         <v>92</v>
       </c>
-      <c r="V20" s="2">
+      <c r="V20" s="1">
         <v>46079</v>
       </c>
     </row>
@@ -2063,7 +2037,7 @@
       <c r="U21" t="s">
         <v>92</v>
       </c>
-      <c r="V21" s="2">
+      <c r="V21" s="1">
         <v>46321</v>
       </c>
     </row>
@@ -2110,7 +2084,7 @@
       <c r="U22" t="s">
         <v>92</v>
       </c>
-      <c r="V22" s="2">
+      <c r="V22" s="1">
         <v>46321</v>
       </c>
     </row>
@@ -2157,7 +2131,7 @@
       <c r="U23" t="s">
         <v>92</v>
       </c>
-      <c r="V23" s="2">
+      <c r="V23" s="1">
         <v>46321</v>
       </c>
     </row>
@@ -2204,7 +2178,7 @@
       <c r="U24" t="s">
         <v>92</v>
       </c>
-      <c r="V24" s="2">
+      <c r="V24" s="1">
         <v>46321</v>
       </c>
     </row>
@@ -2230,7 +2204,7 @@
       <c r="G25" t="s">
         <v>109</v>
       </c>
-      <c r="H25" s="2">
+      <c r="H25" s="1">
         <v>46119</v>
       </c>
       <c r="I25" t="s">
@@ -2263,7 +2237,7 @@
       <c r="U25" t="s">
         <v>180</v>
       </c>
-      <c r="V25" s="2">
+      <c r="V25" s="1">
         <v>46138</v>
       </c>
     </row>
@@ -2289,7 +2263,7 @@
       <c r="G26" t="s">
         <v>109</v>
       </c>
-      <c r="H26" s="2">
+      <c r="H26" s="1">
         <v>46121</v>
       </c>
       <c r="I26" t="s">
@@ -2319,7 +2293,7 @@
       <c r="U26" t="s">
         <v>92</v>
       </c>
-      <c r="V26" s="2">
+      <c r="V26" s="1">
         <v>46138</v>
       </c>
     </row>
@@ -2345,7 +2319,7 @@
       <c r="G27" t="s">
         <v>109</v>
       </c>
-      <c r="H27" s="2">
+      <c r="H27" s="1">
         <v>46076</v>
       </c>
       <c r="I27" t="s">
@@ -2375,7 +2349,7 @@
       <c r="U27" t="s">
         <v>92</v>
       </c>
-      <c r="V27" s="2">
+      <c r="V27" s="1">
         <v>46079</v>
       </c>
     </row>
@@ -2401,7 +2375,7 @@
       <c r="G28" t="s">
         <v>107</v>
       </c>
-      <c r="H28" s="2">
+      <c r="H28" s="1">
         <v>46303</v>
       </c>
       <c r="I28" t="s">
@@ -2437,7 +2411,7 @@
       <c r="U28" t="s">
         <v>180</v>
       </c>
-      <c r="V28" s="2">
+      <c r="V28" s="1">
         <v>46291</v>
       </c>
     </row>
@@ -2463,7 +2437,7 @@
       <c r="G29" t="s">
         <v>109</v>
       </c>
-      <c r="H29" s="2">
+      <c r="H29" s="1">
         <v>46199</v>
       </c>
       <c r="I29" t="s">
@@ -2496,7 +2470,7 @@
       <c r="U29" t="s">
         <v>180</v>
       </c>
-      <c r="V29" s="2">
+      <c r="V29" s="1">
         <v>46199</v>
       </c>
     </row>
@@ -2522,7 +2496,7 @@
       <c r="G30" t="s">
         <v>109</v>
       </c>
-      <c r="H30" s="2">
+      <c r="H30" s="1">
         <v>46199</v>
       </c>
       <c r="I30" t="s">
@@ -2555,7 +2529,7 @@
       <c r="U30" t="s">
         <v>180</v>
       </c>
-      <c r="V30" s="2">
+      <c r="V30" s="1">
         <v>46199</v>
       </c>
     </row>
@@ -2581,7 +2555,7 @@
       <c r="G31" t="s">
         <v>109</v>
       </c>
-      <c r="H31" s="2">
+      <c r="H31" s="1">
         <v>46199</v>
       </c>
       <c r="I31" t="s">
@@ -2614,7 +2588,7 @@
       <c r="U31" t="s">
         <v>180</v>
       </c>
-      <c r="V31" s="2">
+      <c r="V31" s="1">
         <v>46199</v>
       </c>
     </row>
@@ -2640,7 +2614,7 @@
       <c r="G32" t="s">
         <v>109</v>
       </c>
-      <c r="H32" s="2">
+      <c r="H32" s="1">
         <v>46199</v>
       </c>
       <c r="I32" t="s">
@@ -2673,7 +2647,7 @@
       <c r="U32" t="s">
         <v>180</v>
       </c>
-      <c r="V32" s="2">
+      <c r="V32" s="1">
         <v>46199</v>
       </c>
     </row>
@@ -2726,7 +2700,7 @@
       <c r="U33" t="s">
         <v>180</v>
       </c>
-      <c r="V33" s="2">
+      <c r="V33" s="1">
         <v>46291</v>
       </c>
     </row>
@@ -2752,7 +2726,7 @@
       <c r="G34" t="s">
         <v>109</v>
       </c>
-      <c r="H34" s="2">
+      <c r="H34" s="1">
         <v>46191</v>
       </c>
       <c r="I34" t="s">
@@ -2785,7 +2759,7 @@
       <c r="U34" t="s">
         <v>180</v>
       </c>
-      <c r="V34" s="2">
+      <c r="V34" s="1">
         <v>46199</v>
       </c>
     </row>
@@ -2811,7 +2785,7 @@
       <c r="G35" t="s">
         <v>109</v>
       </c>
-      <c r="H35" s="2">
+      <c r="H35" s="1">
         <v>46119</v>
       </c>
       <c r="I35" t="s">
@@ -2841,7 +2815,7 @@
       <c r="U35" t="s">
         <v>180</v>
       </c>
-      <c r="V35" s="2">
+      <c r="V35" s="1">
         <v>46138</v>
       </c>
     </row>
@@ -2867,7 +2841,7 @@
       <c r="G36" t="s">
         <v>109</v>
       </c>
-      <c r="H36" s="2">
+      <c r="H36" s="1">
         <v>46213</v>
       </c>
       <c r="I36" t="s">
@@ -2897,7 +2871,7 @@
       <c r="U36" t="s">
         <v>92</v>
       </c>
-      <c r="V36" s="2">
+      <c r="V36" s="1">
         <v>46229</v>
       </c>
     </row>
@@ -2923,7 +2897,7 @@
       <c r="G37" t="s">
         <v>109</v>
       </c>
-      <c r="H37" s="2">
+      <c r="H37" s="1">
         <v>46175</v>
       </c>
       <c r="I37" t="s">
@@ -2953,7 +2927,7 @@
       <c r="U37" t="s">
         <v>92</v>
       </c>
-      <c r="V37" s="2">
+      <c r="V37" s="1">
         <v>46199</v>
       </c>
     </row>
@@ -2979,7 +2953,7 @@
       <c r="G38" t="s">
         <v>109</v>
       </c>
-      <c r="H38" s="2">
+      <c r="H38" s="1">
         <v>46213</v>
       </c>
       <c r="I38" t="s">
@@ -3009,7 +2983,7 @@
       <c r="U38" t="s">
         <v>92</v>
       </c>
-      <c r="V38" s="2">
+      <c r="V38" s="1">
         <v>46229</v>
       </c>
     </row>
@@ -3035,7 +3009,7 @@
       <c r="G39" t="s">
         <v>109</v>
       </c>
-      <c r="H39" s="2">
+      <c r="H39" s="1">
         <v>46199</v>
       </c>
       <c r="I39" t="s">
@@ -3065,7 +3039,7 @@
       <c r="U39" t="s">
         <v>92</v>
       </c>
-      <c r="V39" s="2">
+      <c r="V39" s="1">
         <v>46199</v>
       </c>
     </row>
@@ -3091,7 +3065,7 @@
       <c r="G40" t="s">
         <v>109</v>
       </c>
-      <c r="H40" s="2">
+      <c r="H40" s="1">
         <v>46199</v>
       </c>
       <c r="I40" t="s">
@@ -3121,7 +3095,7 @@
       <c r="U40" t="s">
         <v>92</v>
       </c>
-      <c r="V40" s="2">
+      <c r="V40" s="1">
         <v>46199</v>
       </c>
     </row>
@@ -3147,7 +3121,7 @@
       <c r="G41" t="s">
         <v>109</v>
       </c>
-      <c r="H41" s="2">
+      <c r="H41" s="1">
         <v>46204</v>
       </c>
       <c r="I41" t="s">
@@ -3177,7 +3151,7 @@
       <c r="U41" t="s">
         <v>92</v>
       </c>
-      <c r="V41" s="2">
+      <c r="V41" s="1">
         <v>46229</v>
       </c>
     </row>
@@ -3203,7 +3177,7 @@
       <c r="G42" t="s">
         <v>109</v>
       </c>
-      <c r="H42" s="2">
+      <c r="H42" s="1">
         <v>46244</v>
       </c>
       <c r="I42" t="s">
@@ -3233,7 +3207,7 @@
       <c r="U42" t="s">
         <v>92</v>
       </c>
-      <c r="V42" s="2">
+      <c r="V42" s="1">
         <v>46199</v>
       </c>
     </row>
@@ -3277,7 +3251,7 @@
       <c r="U43" t="s">
         <v>92</v>
       </c>
-      <c r="V43" s="2">
+      <c r="V43" s="1">
         <v>46260</v>
       </c>
     </row>
@@ -3303,7 +3277,7 @@
       <c r="G44" t="s">
         <v>109</v>
       </c>
-      <c r="H44" s="2">
+      <c r="H44" s="1">
         <v>46191</v>
       </c>
       <c r="I44" t="s">
@@ -3333,7 +3307,7 @@
       <c r="U44" t="s">
         <v>92</v>
       </c>
-      <c r="V44" s="2">
+      <c r="V44" s="1">
         <v>46199</v>
       </c>
     </row>
@@ -3359,7 +3333,7 @@
       <c r="G45" t="s">
         <v>109</v>
       </c>
-      <c r="H45" s="2">
+      <c r="H45" s="1">
         <v>46191</v>
       </c>
       <c r="I45" t="s">
@@ -3389,7 +3363,7 @@
       <c r="U45" t="s">
         <v>92</v>
       </c>
-      <c r="V45" s="2">
+      <c r="V45" s="1">
         <v>46199</v>
       </c>
     </row>
@@ -3415,7 +3389,7 @@
       <c r="G46" t="s">
         <v>109</v>
       </c>
-      <c r="H46" s="2">
+      <c r="H46" s="1">
         <v>46213</v>
       </c>
       <c r="I46" t="s">
@@ -3448,7 +3422,7 @@
       <c r="U46" t="s">
         <v>180</v>
       </c>
-      <c r="V46" s="2">
+      <c r="V46" s="1">
         <v>46229</v>
       </c>
     </row>
@@ -3474,7 +3448,7 @@
       <c r="G47" t="s">
         <v>109</v>
       </c>
-      <c r="H47" s="2">
+      <c r="H47" s="1">
         <v>46210</v>
       </c>
       <c r="I47" t="s">
@@ -3504,7 +3478,7 @@
       <c r="U47" t="s">
         <v>180</v>
       </c>
-      <c r="V47" s="2">
+      <c r="V47" s="1">
         <v>46229</v>
       </c>
     </row>
@@ -3551,7 +3525,7 @@
       <c r="U48" t="s">
         <v>92</v>
       </c>
-      <c r="V48" s="2">
+      <c r="V48" s="1">
         <v>46321</v>
       </c>
     </row>
@@ -3577,7 +3551,7 @@
       <c r="G49" t="s">
         <v>107</v>
       </c>
-      <c r="H49" s="2">
+      <c r="H49" s="1">
         <v>46303</v>
       </c>
       <c r="I49" t="s">
@@ -3613,7 +3587,7 @@
       <c r="U49" t="s">
         <v>180</v>
       </c>
-      <c r="V49" s="2">
+      <c r="V49" s="1">
         <v>46291</v>
       </c>
     </row>
@@ -3639,7 +3613,7 @@
       <c r="G50" t="s">
         <v>109</v>
       </c>
-      <c r="H50" s="2">
+      <c r="H50" s="1">
         <v>46176</v>
       </c>
       <c r="I50" t="s">
@@ -3672,7 +3646,7 @@
       <c r="U50" t="s">
         <v>180</v>
       </c>
-      <c r="V50" s="2">
+      <c r="V50" s="1">
         <v>46199</v>
       </c>
     </row>
@@ -3728,7 +3702,7 @@
       <c r="U51" t="s">
         <v>180</v>
       </c>
-      <c r="V51" s="2">
+      <c r="V51" s="1">
         <v>46260</v>
       </c>
     </row>
@@ -3754,7 +3728,7 @@
       <c r="G52" t="s">
         <v>109</v>
       </c>
-      <c r="H52" s="2">
+      <c r="H52" s="1">
         <v>46295</v>
       </c>
       <c r="I52" t="s">
@@ -3790,7 +3764,7 @@
       <c r="U52" t="s">
         <v>180</v>
       </c>
-      <c r="V52" s="2">
+      <c r="V52" s="1">
         <v>46291</v>
       </c>
     </row>
@@ -3843,7 +3817,7 @@
       <c r="U53" t="s">
         <v>180</v>
       </c>
-      <c r="V53" s="2">
+      <c r="V53" s="1">
         <v>46321</v>
       </c>
     </row>
@@ -3869,7 +3843,7 @@
       <c r="G54" t="s">
         <v>109</v>
       </c>
-      <c r="H54" s="2">
+      <c r="H54" s="1">
         <v>46227</v>
       </c>
       <c r="I54" t="s">
@@ -3899,7 +3873,7 @@
       <c r="U54" t="s">
         <v>180</v>
       </c>
-      <c r="V54" s="2">
+      <c r="V54" s="1">
         <v>46229</v>
       </c>
     </row>
@@ -3922,7 +3896,7 @@
       <c r="G55" t="s">
         <v>109</v>
       </c>
-      <c r="H55" s="2">
+      <c r="H55" s="1">
         <v>46280</v>
       </c>
       <c r="I55" t="s">
@@ -3952,7 +3926,7 @@
       <c r="U55" t="s">
         <v>180</v>
       </c>
-      <c r="V55" s="2">
+      <c r="V55" s="1">
         <v>46291</v>
       </c>
     </row>
@@ -3975,7 +3949,7 @@
       <c r="G56" t="s">
         <v>109</v>
       </c>
-      <c r="H56" s="2">
+      <c r="H56" s="1">
         <v>46280</v>
       </c>
       <c r="I56" t="s">
@@ -4005,7 +3979,7 @@
       <c r="U56" t="s">
         <v>180</v>
       </c>
-      <c r="V56" s="2">
+      <c r="V56" s="1">
         <v>46260</v>
       </c>
     </row>
@@ -4028,7 +4002,7 @@
       <c r="G57" t="s">
         <v>109</v>
       </c>
-      <c r="H57" s="2">
+      <c r="H57" s="1">
         <v>46295</v>
       </c>
       <c r="I57" t="s">
@@ -4058,7 +4032,7 @@
       <c r="U57" t="s">
         <v>180</v>
       </c>
-      <c r="V57" s="2">
+      <c r="V57" s="1">
         <v>46291</v>
       </c>
     </row>
@@ -4081,7 +4055,7 @@
       <c r="G58" t="s">
         <v>109</v>
       </c>
-      <c r="H58" s="2">
+      <c r="H58" s="1">
         <v>46295</v>
       </c>
       <c r="I58" t="s">
@@ -4111,7 +4085,7 @@
       <c r="U58" t="s">
         <v>180</v>
       </c>
-      <c r="V58" s="2">
+      <c r="V58" s="1">
         <v>46291</v>
       </c>
     </row>
@@ -4134,7 +4108,7 @@
       <c r="G59" t="s">
         <v>109</v>
       </c>
-      <c r="H59" s="2">
+      <c r="H59" s="1">
         <v>46304</v>
       </c>
       <c r="I59" t="s">
@@ -4164,7 +4138,7 @@
       <c r="U59" t="s">
         <v>180</v>
       </c>
-      <c r="V59" s="2">
+      <c r="V59" s="1">
         <v>46321</v>
       </c>
     </row>
@@ -4190,7 +4164,7 @@
       <c r="G60" t="s">
         <v>109</v>
       </c>
-      <c r="H60" s="2">
+      <c r="H60" s="1">
         <v>46301</v>
       </c>
       <c r="I60" t="s">
@@ -4226,7 +4200,7 @@
       <c r="U60" t="s">
         <v>180</v>
       </c>
-      <c r="V60" s="2">
+      <c r="V60" s="1">
         <v>46352</v>
       </c>
     </row>
@@ -4270,7 +4244,7 @@
       <c r="U61" t="s">
         <v>180</v>
       </c>
-      <c r="V61" s="2">
+      <c r="V61" s="1">
         <v>46107</v>
       </c>
     </row>
@@ -4314,7 +4288,7 @@
       <c r="U62" t="s">
         <v>180</v>
       </c>
-      <c r="V62" s="2">
+      <c r="V62" s="1">
         <v>46107</v>
       </c>
     </row>
@@ -4358,7 +4332,7 @@
       <c r="U63" t="s">
         <v>180</v>
       </c>
-      <c r="V63" s="2">
+      <c r="V63" s="1">
         <v>46107</v>
       </c>
     </row>
@@ -4402,7 +4376,7 @@
       <c r="U64" t="s">
         <v>180</v>
       </c>
-      <c r="V64" s="2">
+      <c r="V64" s="1">
         <v>46107</v>
       </c>
     </row>
@@ -4446,7 +4420,7 @@
       <c r="U65" t="s">
         <v>180</v>
       </c>
-      <c r="V65" s="2">
+      <c r="V65" s="1">
         <v>46107</v>
       </c>
     </row>
@@ -4490,7 +4464,7 @@
       <c r="U66" t="s">
         <v>180</v>
       </c>
-      <c r="V66" s="2">
+      <c r="V66" s="1">
         <v>46107</v>
       </c>
     </row>
@@ -4534,7 +4508,7 @@
       <c r="U67" t="s">
         <v>92</v>
       </c>
-      <c r="V67" s="2">
+      <c r="V67" s="1">
         <v>46168</v>
       </c>
     </row>
@@ -4581,7 +4555,7 @@
       <c r="U68" t="s">
         <v>92</v>
       </c>
-      <c r="V68" s="2">
+      <c r="V68" s="1">
         <v>46291</v>
       </c>
     </row>
@@ -4607,7 +4581,7 @@
       <c r="G69" t="s">
         <v>107</v>
       </c>
-      <c r="H69" s="2">
+      <c r="H69" s="1">
         <v>46303</v>
       </c>
       <c r="I69" t="s">
@@ -4643,7 +4617,7 @@
       <c r="U69" t="s">
         <v>180</v>
       </c>
-      <c r="V69" s="2">
+      <c r="V69" s="1">
         <v>46229</v>
       </c>
     </row>
@@ -4687,7 +4661,7 @@
       <c r="U70" t="s">
         <v>92</v>
       </c>
-      <c r="V70" s="2">
+      <c r="V70" s="1">
         <v>46260</v>
       </c>
     </row>
@@ -4731,7 +4705,7 @@
       <c r="U71" t="s">
         <v>180</v>
       </c>
-      <c r="V71" s="2">
+      <c r="V71" s="1">
         <v>46291</v>
       </c>
     </row>
@@ -4775,7 +4749,7 @@
       <c r="U72" t="s">
         <v>180</v>
       </c>
-      <c r="V72" s="2">
+      <c r="V72" s="1">
         <v>46168</v>
       </c>
     </row>
@@ -4819,7 +4793,7 @@
       <c r="U73" t="s">
         <v>180</v>
       </c>
-      <c r="V73" s="2">
+      <c r="V73" s="1">
         <v>46291</v>
       </c>
     </row>
@@ -4863,7 +4837,7 @@
       <c r="U74" t="s">
         <v>180</v>
       </c>
-      <c r="V74" s="2">
+      <c r="V74" s="1">
         <v>46291</v>
       </c>
     </row>
@@ -4907,7 +4881,7 @@
       <c r="U75" t="s">
         <v>180</v>
       </c>
-      <c r="V75" s="2">
+      <c r="V75" s="1">
         <v>46291</v>
       </c>
     </row>
@@ -4954,7 +4928,7 @@
       <c r="U76" t="s">
         <v>92</v>
       </c>
-      <c r="V76" s="2">
+      <c r="V76" s="1">
         <v>46321</v>
       </c>
     </row>
@@ -5004,7 +4978,7 @@
       <c r="U77" t="s">
         <v>180</v>
       </c>
-      <c r="V77" s="2">
+      <c r="V77" s="1">
         <v>46381</v>
       </c>
     </row>
@@ -5054,7 +5028,7 @@
       <c r="U78" t="s">
         <v>180</v>
       </c>
-      <c r="V78" s="2">
+      <c r="V78" s="1">
         <v>46381</v>
       </c>
     </row>
@@ -5104,7 +5078,7 @@
       <c r="U79" t="s">
         <v>92</v>
       </c>
-      <c r="V79" s="2">
+      <c r="V79" s="1">
         <v>46381</v>
       </c>
     </row>
@@ -5154,7 +5128,7 @@
       <c r="U80" t="s">
         <v>92</v>
       </c>
-      <c r="V80" s="2">
+      <c r="V80" s="1">
         <v>46381</v>
       </c>
     </row>
@@ -5204,7 +5178,7 @@
       <c r="U81" t="s">
         <v>92</v>
       </c>
-      <c r="V81" s="2">
+      <c r="V81" s="1">
         <v>46382</v>
       </c>
     </row>
@@ -5248,7 +5222,7 @@
       <c r="U82" t="s">
         <v>92</v>
       </c>
-      <c r="V82" s="2">
+      <c r="V82" s="1">
         <v>46382</v>
       </c>
     </row>
@@ -5304,7 +5278,7 @@
       <c r="U83" t="s">
         <v>180</v>
       </c>
-      <c r="V83" s="2">
+      <c r="V83" s="1">
         <v>46382</v>
       </c>
     </row>
@@ -5354,7 +5328,7 @@
       <c r="U84" t="s">
         <v>92</v>
       </c>
-      <c r="V84" s="2">
+      <c r="V84" s="1">
         <v>46321</v>
       </c>
     </row>
@@ -5398,7 +5372,7 @@
       <c r="U85" t="s">
         <v>92</v>
       </c>
-      <c r="V85" s="2">
+      <c r="V85" s="1">
         <v>46382</v>
       </c>
     </row>
@@ -5518,7 +5492,7 @@
       <c r="G88" t="s">
         <v>109</v>
       </c>
-      <c r="H88" s="2">
+      <c r="H88" s="1">
         <v>46303</v>
       </c>
       <c r="I88" t="s">
@@ -5548,7 +5522,7 @@
       <c r="U88" t="s">
         <v>92</v>
       </c>
-      <c r="V88" s="2">
+      <c r="V88" s="1">
         <v>46291</v>
       </c>
     </row>
@@ -5595,7 +5569,7 @@
       <c r="U89" t="s">
         <v>92</v>
       </c>
-      <c r="V89" s="2">
+      <c r="V89" s="1">
         <v>46291</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Atualização automática: mta (19/10/2026 13:33)
</commit_message>
<xml_diff>
--- a/Projetos/02_Dados_Tratados/base_mta_tratada.xlsx
+++ b/Projetos/02_Dados_Tratados/base_mta_tratada.xlsx
@@ -566,8 +566,16 @@
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="YYYY-MM-DD HH:MM:SS"/>
   </numFmts>
-  <fonts count="1">
+  <fonts count="2">
     <font>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
       <sz val="11"/>
       <color theme="1"/>
       <name val="Calibri"/>
@@ -583,7 +591,7 @@
       <patternFill patternType="gray125"/>
     </fill>
   </fills>
-  <borders count="1">
+  <borders count="2">
     <border>
       <left/>
       <right/>
@@ -591,12 +599,30 @@
       <bottom/>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin">
+        <color auto="1"/>
+      </left>
+      <right style="thin">
+        <color auto="1"/>
+      </right>
+      <top style="thin">
+        <color auto="1"/>
+      </top>
+      <bottom style="thin">
+        <color auto="1"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="3">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
   </cellXfs>
   <cellStyles count="1">
@@ -896,70 +922,70 @@
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:22">
-      <c r="A1" t="s">
+      <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
-      <c r="B1" t="s">
+      <c r="B1" s="1" t="s">
         <v>1</v>
       </c>
-      <c r="C1" t="s">
+      <c r="C1" s="1" t="s">
         <v>2</v>
       </c>
-      <c r="D1" t="s">
+      <c r="D1" s="1" t="s">
         <v>3</v>
       </c>
-      <c r="E1" t="s">
+      <c r="E1" s="1" t="s">
         <v>4</v>
       </c>
-      <c r="F1" t="s">
+      <c r="F1" s="1" t="s">
         <v>5</v>
       </c>
-      <c r="G1" t="s">
+      <c r="G1" s="1" t="s">
         <v>6</v>
       </c>
-      <c r="H1" t="s">
+      <c r="H1" s="1" t="s">
         <v>7</v>
       </c>
-      <c r="I1" t="s">
+      <c r="I1" s="1" t="s">
         <v>8</v>
       </c>
-      <c r="J1" t="s">
+      <c r="J1" s="1" t="s">
         <v>9</v>
       </c>
-      <c r="K1" t="s">
+      <c r="K1" s="1" t="s">
         <v>10</v>
       </c>
-      <c r="L1" t="s">
+      <c r="L1" s="1" t="s">
         <v>11</v>
       </c>
-      <c r="M1" t="s">
+      <c r="M1" s="1" t="s">
         <v>12</v>
       </c>
-      <c r="N1" t="s">
+      <c r="N1" s="1" t="s">
         <v>13</v>
       </c>
-      <c r="O1" t="s">
+      <c r="O1" s="1" t="s">
         <v>14</v>
       </c>
-      <c r="P1" t="s">
+      <c r="P1" s="1" t="s">
         <v>15</v>
       </c>
-      <c r="Q1" t="s">
+      <c r="Q1" s="1" t="s">
         <v>16</v>
       </c>
-      <c r="R1" t="s">
+      <c r="R1" s="1" t="s">
         <v>17</v>
       </c>
-      <c r="S1" t="s">
+      <c r="S1" s="1" t="s">
         <v>18</v>
       </c>
-      <c r="T1" t="s">
+      <c r="T1" s="1" t="s">
         <v>19</v>
       </c>
-      <c r="U1" t="s">
+      <c r="U1" s="1" t="s">
         <v>20</v>
       </c>
-      <c r="V1" t="s">
+      <c r="V1" s="1" t="s">
         <v>21</v>
       </c>
     </row>
@@ -985,7 +1011,7 @@
       <c r="G2" t="s">
         <v>107</v>
       </c>
-      <c r="H2" s="1">
+      <c r="H2" s="2">
         <v>46303</v>
       </c>
       <c r="I2" t="s">
@@ -1024,7 +1050,7 @@
       <c r="U2" t="s">
         <v>180</v>
       </c>
-      <c r="V2" s="1">
+      <c r="V2" s="2">
         <v>46229</v>
       </c>
     </row>
@@ -1071,7 +1097,7 @@
       <c r="U3" t="s">
         <v>92</v>
       </c>
-      <c r="V3" s="1">
+      <c r="V3" s="2">
         <v>46291</v>
       </c>
     </row>
@@ -1118,7 +1144,7 @@
       <c r="U4" t="s">
         <v>92</v>
       </c>
-      <c r="V4" s="1">
+      <c r="V4" s="2">
         <v>46321</v>
       </c>
     </row>
@@ -1165,7 +1191,7 @@
       <c r="U5" t="s">
         <v>92</v>
       </c>
-      <c r="V5" s="1">
+      <c r="V5" s="2">
         <v>46321</v>
       </c>
     </row>
@@ -1215,7 +1241,7 @@
       <c r="U6" t="s">
         <v>92</v>
       </c>
-      <c r="V6" s="1">
+      <c r="V6" s="2">
         <v>46291</v>
       </c>
     </row>
@@ -1241,7 +1267,7 @@
       <c r="G7" t="s">
         <v>109</v>
       </c>
-      <c r="H7" s="1">
+      <c r="H7" s="2">
         <v>46121</v>
       </c>
       <c r="I7" t="s">
@@ -1271,7 +1297,7 @@
       <c r="U7" t="s">
         <v>92</v>
       </c>
-      <c r="V7" s="1">
+      <c r="V7" s="2">
         <v>46138</v>
       </c>
     </row>
@@ -1318,7 +1344,7 @@
       <c r="U8" t="s">
         <v>92</v>
       </c>
-      <c r="V8" s="1">
+      <c r="V8" s="2">
         <v>46291</v>
       </c>
     </row>
@@ -1365,7 +1391,7 @@
       <c r="U9" t="s">
         <v>92</v>
       </c>
-      <c r="V9" s="1">
+      <c r="V9" s="2">
         <v>46291</v>
       </c>
     </row>
@@ -1388,7 +1414,7 @@
       <c r="G10" t="s">
         <v>109</v>
       </c>
-      <c r="H10" s="1">
+      <c r="H10" s="2">
         <v>46303</v>
       </c>
       <c r="I10" t="s">
@@ -1418,7 +1444,7 @@
       <c r="U10" t="s">
         <v>92</v>
       </c>
-      <c r="V10" s="1">
+      <c r="V10" s="2">
         <v>46291</v>
       </c>
     </row>
@@ -1465,7 +1491,7 @@
       <c r="U11" t="s">
         <v>92</v>
       </c>
-      <c r="V11" s="1">
+      <c r="V11" s="2">
         <v>46291</v>
       </c>
     </row>
@@ -1512,7 +1538,7 @@
       <c r="U12" t="s">
         <v>92</v>
       </c>
-      <c r="V12" s="1">
+      <c r="V12" s="2">
         <v>46291</v>
       </c>
     </row>
@@ -1538,7 +1564,7 @@
       <c r="G13" t="s">
         <v>109</v>
       </c>
-      <c r="H13" s="1">
+      <c r="H13" s="2">
         <v>46079</v>
       </c>
       <c r="I13" t="s">
@@ -1571,7 +1597,7 @@
       <c r="U13" t="s">
         <v>180</v>
       </c>
-      <c r="V13" s="1">
+      <c r="V13" s="2">
         <v>46079</v>
       </c>
     </row>
@@ -1597,7 +1623,7 @@
       <c r="G14" t="s">
         <v>107</v>
       </c>
-      <c r="H14" s="1">
+      <c r="H14" s="2">
         <v>46303</v>
       </c>
       <c r="I14" t="s">
@@ -1633,7 +1659,7 @@
       <c r="U14" t="s">
         <v>180</v>
       </c>
-      <c r="V14" s="1">
+      <c r="V14" s="2">
         <v>46352</v>
       </c>
     </row>
@@ -1659,7 +1685,7 @@
       <c r="G15" t="s">
         <v>107</v>
       </c>
-      <c r="H15" s="1">
+      <c r="H15" s="2">
         <v>46303</v>
       </c>
       <c r="I15" t="s">
@@ -1695,7 +1721,7 @@
       <c r="U15" t="s">
         <v>180</v>
       </c>
-      <c r="V15" s="1">
+      <c r="V15" s="2">
         <v>46352</v>
       </c>
     </row>
@@ -1721,7 +1747,7 @@
       <c r="G16" t="s">
         <v>107</v>
       </c>
-      <c r="H16" s="1">
+      <c r="H16" s="2">
         <v>46303</v>
       </c>
       <c r="I16" t="s">
@@ -1757,7 +1783,7 @@
       <c r="U16" t="s">
         <v>180</v>
       </c>
-      <c r="V16" s="1">
+      <c r="V16" s="2">
         <v>46352</v>
       </c>
     </row>
@@ -1783,7 +1809,7 @@
       <c r="G17" t="s">
         <v>107</v>
       </c>
-      <c r="H17" s="1">
+      <c r="H17" s="2">
         <v>46303</v>
       </c>
       <c r="I17" t="s">
@@ -1819,7 +1845,7 @@
       <c r="U17" t="s">
         <v>180</v>
       </c>
-      <c r="V17" s="1">
+      <c r="V17" s="2">
         <v>46229</v>
       </c>
     </row>
@@ -1845,7 +1871,7 @@
       <c r="G18" t="s">
         <v>109</v>
       </c>
-      <c r="H18" s="1">
+      <c r="H18" s="2">
         <v>46098</v>
       </c>
       <c r="I18" t="s">
@@ -1878,7 +1904,7 @@
       <c r="U18" t="s">
         <v>180</v>
       </c>
-      <c r="V18" s="1">
+      <c r="V18" s="2">
         <v>46107</v>
       </c>
     </row>
@@ -1904,7 +1930,7 @@
       <c r="G19" t="s">
         <v>109</v>
       </c>
-      <c r="H19" s="1">
+      <c r="H19" s="2">
         <v>46076</v>
       </c>
       <c r="I19" t="s">
@@ -1934,7 +1960,7 @@
       <c r="U19" t="s">
         <v>92</v>
       </c>
-      <c r="V19" s="1">
+      <c r="V19" s="2">
         <v>46079</v>
       </c>
     </row>
@@ -1960,7 +1986,7 @@
       <c r="G20" t="s">
         <v>109</v>
       </c>
-      <c r="H20" s="1">
+      <c r="H20" s="2">
         <v>46076</v>
       </c>
       <c r="I20" t="s">
@@ -1990,7 +2016,7 @@
       <c r="U20" t="s">
         <v>92</v>
       </c>
-      <c r="V20" s="1">
+      <c r="V20" s="2">
         <v>46079</v>
       </c>
     </row>
@@ -2037,7 +2063,7 @@
       <c r="U21" t="s">
         <v>92</v>
       </c>
-      <c r="V21" s="1">
+      <c r="V21" s="2">
         <v>46321</v>
       </c>
     </row>
@@ -2084,7 +2110,7 @@
       <c r="U22" t="s">
         <v>92</v>
       </c>
-      <c r="V22" s="1">
+      <c r="V22" s="2">
         <v>46321</v>
       </c>
     </row>
@@ -2131,7 +2157,7 @@
       <c r="U23" t="s">
         <v>92</v>
       </c>
-      <c r="V23" s="1">
+      <c r="V23" s="2">
         <v>46321</v>
       </c>
     </row>
@@ -2178,7 +2204,7 @@
       <c r="U24" t="s">
         <v>92</v>
       </c>
-      <c r="V24" s="1">
+      <c r="V24" s="2">
         <v>46321</v>
       </c>
     </row>
@@ -2204,7 +2230,7 @@
       <c r="G25" t="s">
         <v>109</v>
       </c>
-      <c r="H25" s="1">
+      <c r="H25" s="2">
         <v>46119</v>
       </c>
       <c r="I25" t="s">
@@ -2237,7 +2263,7 @@
       <c r="U25" t="s">
         <v>180</v>
       </c>
-      <c r="V25" s="1">
+      <c r="V25" s="2">
         <v>46138</v>
       </c>
     </row>
@@ -2263,7 +2289,7 @@
       <c r="G26" t="s">
         <v>109</v>
       </c>
-      <c r="H26" s="1">
+      <c r="H26" s="2">
         <v>46121</v>
       </c>
       <c r="I26" t="s">
@@ -2293,7 +2319,7 @@
       <c r="U26" t="s">
         <v>92</v>
       </c>
-      <c r="V26" s="1">
+      <c r="V26" s="2">
         <v>46138</v>
       </c>
     </row>
@@ -2319,7 +2345,7 @@
       <c r="G27" t="s">
         <v>109</v>
       </c>
-      <c r="H27" s="1">
+      <c r="H27" s="2">
         <v>46076</v>
       </c>
       <c r="I27" t="s">
@@ -2349,7 +2375,7 @@
       <c r="U27" t="s">
         <v>92</v>
       </c>
-      <c r="V27" s="1">
+      <c r="V27" s="2">
         <v>46079</v>
       </c>
     </row>
@@ -2375,7 +2401,7 @@
       <c r="G28" t="s">
         <v>107</v>
       </c>
-      <c r="H28" s="1">
+      <c r="H28" s="2">
         <v>46303</v>
       </c>
       <c r="I28" t="s">
@@ -2411,7 +2437,7 @@
       <c r="U28" t="s">
         <v>180</v>
       </c>
-      <c r="V28" s="1">
+      <c r="V28" s="2">
         <v>46291</v>
       </c>
     </row>
@@ -2437,7 +2463,7 @@
       <c r="G29" t="s">
         <v>109</v>
       </c>
-      <c r="H29" s="1">
+      <c r="H29" s="2">
         <v>46199</v>
       </c>
       <c r="I29" t="s">
@@ -2470,7 +2496,7 @@
       <c r="U29" t="s">
         <v>180</v>
       </c>
-      <c r="V29" s="1">
+      <c r="V29" s="2">
         <v>46199</v>
       </c>
     </row>
@@ -2496,7 +2522,7 @@
       <c r="G30" t="s">
         <v>109</v>
       </c>
-      <c r="H30" s="1">
+      <c r="H30" s="2">
         <v>46199</v>
       </c>
       <c r="I30" t="s">
@@ -2529,7 +2555,7 @@
       <c r="U30" t="s">
         <v>180</v>
       </c>
-      <c r="V30" s="1">
+      <c r="V30" s="2">
         <v>46199</v>
       </c>
     </row>
@@ -2555,7 +2581,7 @@
       <c r="G31" t="s">
         <v>109</v>
       </c>
-      <c r="H31" s="1">
+      <c r="H31" s="2">
         <v>46199</v>
       </c>
       <c r="I31" t="s">
@@ -2588,7 +2614,7 @@
       <c r="U31" t="s">
         <v>180</v>
       </c>
-      <c r="V31" s="1">
+      <c r="V31" s="2">
         <v>46199</v>
       </c>
     </row>
@@ -2614,7 +2640,7 @@
       <c r="G32" t="s">
         <v>109</v>
       </c>
-      <c r="H32" s="1">
+      <c r="H32" s="2">
         <v>46199</v>
       </c>
       <c r="I32" t="s">
@@ -2647,7 +2673,7 @@
       <c r="U32" t="s">
         <v>180</v>
       </c>
-      <c r="V32" s="1">
+      <c r="V32" s="2">
         <v>46199</v>
       </c>
     </row>
@@ -2700,7 +2726,7 @@
       <c r="U33" t="s">
         <v>180</v>
       </c>
-      <c r="V33" s="1">
+      <c r="V33" s="2">
         <v>46291</v>
       </c>
     </row>
@@ -2726,7 +2752,7 @@
       <c r="G34" t="s">
         <v>109</v>
       </c>
-      <c r="H34" s="1">
+      <c r="H34" s="2">
         <v>46191</v>
       </c>
       <c r="I34" t="s">
@@ -2759,7 +2785,7 @@
       <c r="U34" t="s">
         <v>180</v>
       </c>
-      <c r="V34" s="1">
+      <c r="V34" s="2">
         <v>46199</v>
       </c>
     </row>
@@ -2785,7 +2811,7 @@
       <c r="G35" t="s">
         <v>109</v>
       </c>
-      <c r="H35" s="1">
+      <c r="H35" s="2">
         <v>46119</v>
       </c>
       <c r="I35" t="s">
@@ -2815,7 +2841,7 @@
       <c r="U35" t="s">
         <v>180</v>
       </c>
-      <c r="V35" s="1">
+      <c r="V35" s="2">
         <v>46138</v>
       </c>
     </row>
@@ -2841,7 +2867,7 @@
       <c r="G36" t="s">
         <v>109</v>
       </c>
-      <c r="H36" s="1">
+      <c r="H36" s="2">
         <v>46213</v>
       </c>
       <c r="I36" t="s">
@@ -2871,7 +2897,7 @@
       <c r="U36" t="s">
         <v>92</v>
       </c>
-      <c r="V36" s="1">
+      <c r="V36" s="2">
         <v>46229</v>
       </c>
     </row>
@@ -2897,7 +2923,7 @@
       <c r="G37" t="s">
         <v>109</v>
       </c>
-      <c r="H37" s="1">
+      <c r="H37" s="2">
         <v>46175</v>
       </c>
       <c r="I37" t="s">
@@ -2927,7 +2953,7 @@
       <c r="U37" t="s">
         <v>92</v>
       </c>
-      <c r="V37" s="1">
+      <c r="V37" s="2">
         <v>46199</v>
       </c>
     </row>
@@ -2953,7 +2979,7 @@
       <c r="G38" t="s">
         <v>109</v>
       </c>
-      <c r="H38" s="1">
+      <c r="H38" s="2">
         <v>46213</v>
       </c>
       <c r="I38" t="s">
@@ -2983,7 +3009,7 @@
       <c r="U38" t="s">
         <v>92</v>
       </c>
-      <c r="V38" s="1">
+      <c r="V38" s="2">
         <v>46229</v>
       </c>
     </row>
@@ -3009,7 +3035,7 @@
       <c r="G39" t="s">
         <v>109</v>
       </c>
-      <c r="H39" s="1">
+      <c r="H39" s="2">
         <v>46199</v>
       </c>
       <c r="I39" t="s">
@@ -3039,7 +3065,7 @@
       <c r="U39" t="s">
         <v>92</v>
       </c>
-      <c r="V39" s="1">
+      <c r="V39" s="2">
         <v>46199</v>
       </c>
     </row>
@@ -3065,7 +3091,7 @@
       <c r="G40" t="s">
         <v>109</v>
       </c>
-      <c r="H40" s="1">
+      <c r="H40" s="2">
         <v>46199</v>
       </c>
       <c r="I40" t="s">
@@ -3095,7 +3121,7 @@
       <c r="U40" t="s">
         <v>92</v>
       </c>
-      <c r="V40" s="1">
+      <c r="V40" s="2">
         <v>46199</v>
       </c>
     </row>
@@ -3121,7 +3147,7 @@
       <c r="G41" t="s">
         <v>109</v>
       </c>
-      <c r="H41" s="1">
+      <c r="H41" s="2">
         <v>46204</v>
       </c>
       <c r="I41" t="s">
@@ -3151,7 +3177,7 @@
       <c r="U41" t="s">
         <v>92</v>
       </c>
-      <c r="V41" s="1">
+      <c r="V41" s="2">
         <v>46229</v>
       </c>
     </row>
@@ -3177,7 +3203,7 @@
       <c r="G42" t="s">
         <v>109</v>
       </c>
-      <c r="H42" s="1">
+      <c r="H42" s="2">
         <v>46244</v>
       </c>
       <c r="I42" t="s">
@@ -3207,7 +3233,7 @@
       <c r="U42" t="s">
         <v>92</v>
       </c>
-      <c r="V42" s="1">
+      <c r="V42" s="2">
         <v>46199</v>
       </c>
     </row>
@@ -3251,7 +3277,7 @@
       <c r="U43" t="s">
         <v>92</v>
       </c>
-      <c r="V43" s="1">
+      <c r="V43" s="2">
         <v>46260</v>
       </c>
     </row>
@@ -3277,7 +3303,7 @@
       <c r="G44" t="s">
         <v>109</v>
       </c>
-      <c r="H44" s="1">
+      <c r="H44" s="2">
         <v>46191</v>
       </c>
       <c r="I44" t="s">
@@ -3307,7 +3333,7 @@
       <c r="U44" t="s">
         <v>92</v>
       </c>
-      <c r="V44" s="1">
+      <c r="V44" s="2">
         <v>46199</v>
       </c>
     </row>
@@ -3333,7 +3359,7 @@
       <c r="G45" t="s">
         <v>109</v>
       </c>
-      <c r="H45" s="1">
+      <c r="H45" s="2">
         <v>46191</v>
       </c>
       <c r="I45" t="s">
@@ -3363,7 +3389,7 @@
       <c r="U45" t="s">
         <v>92</v>
       </c>
-      <c r="V45" s="1">
+      <c r="V45" s="2">
         <v>46199</v>
       </c>
     </row>
@@ -3389,7 +3415,7 @@
       <c r="G46" t="s">
         <v>109</v>
       </c>
-      <c r="H46" s="1">
+      <c r="H46" s="2">
         <v>46213</v>
       </c>
       <c r="I46" t="s">
@@ -3422,7 +3448,7 @@
       <c r="U46" t="s">
         <v>180</v>
       </c>
-      <c r="V46" s="1">
+      <c r="V46" s="2">
         <v>46229</v>
       </c>
     </row>
@@ -3448,7 +3474,7 @@
       <c r="G47" t="s">
         <v>109</v>
       </c>
-      <c r="H47" s="1">
+      <c r="H47" s="2">
         <v>46210</v>
       </c>
       <c r="I47" t="s">
@@ -3478,7 +3504,7 @@
       <c r="U47" t="s">
         <v>180</v>
       </c>
-      <c r="V47" s="1">
+      <c r="V47" s="2">
         <v>46229</v>
       </c>
     </row>
@@ -3525,7 +3551,7 @@
       <c r="U48" t="s">
         <v>92</v>
       </c>
-      <c r="V48" s="1">
+      <c r="V48" s="2">
         <v>46321</v>
       </c>
     </row>
@@ -3551,7 +3577,7 @@
       <c r="G49" t="s">
         <v>107</v>
       </c>
-      <c r="H49" s="1">
+      <c r="H49" s="2">
         <v>46303</v>
       </c>
       <c r="I49" t="s">
@@ -3587,7 +3613,7 @@
       <c r="U49" t="s">
         <v>180</v>
       </c>
-      <c r="V49" s="1">
+      <c r="V49" s="2">
         <v>46291</v>
       </c>
     </row>
@@ -3613,7 +3639,7 @@
       <c r="G50" t="s">
         <v>109</v>
       </c>
-      <c r="H50" s="1">
+      <c r="H50" s="2">
         <v>46176</v>
       </c>
       <c r="I50" t="s">
@@ -3646,7 +3672,7 @@
       <c r="U50" t="s">
         <v>180</v>
       </c>
-      <c r="V50" s="1">
+      <c r="V50" s="2">
         <v>46199</v>
       </c>
     </row>
@@ -3702,7 +3728,7 @@
       <c r="U51" t="s">
         <v>180</v>
       </c>
-      <c r="V51" s="1">
+      <c r="V51" s="2">
         <v>46260</v>
       </c>
     </row>
@@ -3728,7 +3754,7 @@
       <c r="G52" t="s">
         <v>109</v>
       </c>
-      <c r="H52" s="1">
+      <c r="H52" s="2">
         <v>46295</v>
       </c>
       <c r="I52" t="s">
@@ -3764,7 +3790,7 @@
       <c r="U52" t="s">
         <v>180</v>
       </c>
-      <c r="V52" s="1">
+      <c r="V52" s="2">
         <v>46291</v>
       </c>
     </row>
@@ -3817,7 +3843,7 @@
       <c r="U53" t="s">
         <v>180</v>
       </c>
-      <c r="V53" s="1">
+      <c r="V53" s="2">
         <v>46321</v>
       </c>
     </row>
@@ -3843,7 +3869,7 @@
       <c r="G54" t="s">
         <v>109</v>
       </c>
-      <c r="H54" s="1">
+      <c r="H54" s="2">
         <v>46227</v>
       </c>
       <c r="I54" t="s">
@@ -3873,7 +3899,7 @@
       <c r="U54" t="s">
         <v>180</v>
       </c>
-      <c r="V54" s="1">
+      <c r="V54" s="2">
         <v>46229</v>
       </c>
     </row>
@@ -3896,7 +3922,7 @@
       <c r="G55" t="s">
         <v>109</v>
       </c>
-      <c r="H55" s="1">
+      <c r="H55" s="2">
         <v>46280</v>
       </c>
       <c r="I55" t="s">
@@ -3926,7 +3952,7 @@
       <c r="U55" t="s">
         <v>180</v>
       </c>
-      <c r="V55" s="1">
+      <c r="V55" s="2">
         <v>46291</v>
       </c>
     </row>
@@ -3949,7 +3975,7 @@
       <c r="G56" t="s">
         <v>109</v>
       </c>
-      <c r="H56" s="1">
+      <c r="H56" s="2">
         <v>46280</v>
       </c>
       <c r="I56" t="s">
@@ -3979,7 +4005,7 @@
       <c r="U56" t="s">
         <v>180</v>
       </c>
-      <c r="V56" s="1">
+      <c r="V56" s="2">
         <v>46260</v>
       </c>
     </row>
@@ -4002,7 +4028,7 @@
       <c r="G57" t="s">
         <v>109</v>
       </c>
-      <c r="H57" s="1">
+      <c r="H57" s="2">
         <v>46295</v>
       </c>
       <c r="I57" t="s">
@@ -4032,7 +4058,7 @@
       <c r="U57" t="s">
         <v>180</v>
       </c>
-      <c r="V57" s="1">
+      <c r="V57" s="2">
         <v>46291</v>
       </c>
     </row>
@@ -4055,7 +4081,7 @@
       <c r="G58" t="s">
         <v>109</v>
       </c>
-      <c r="H58" s="1">
+      <c r="H58" s="2">
         <v>46295</v>
       </c>
       <c r="I58" t="s">
@@ -4085,7 +4111,7 @@
       <c r="U58" t="s">
         <v>180</v>
       </c>
-      <c r="V58" s="1">
+      <c r="V58" s="2">
         <v>46291</v>
       </c>
     </row>
@@ -4108,7 +4134,7 @@
       <c r="G59" t="s">
         <v>109</v>
       </c>
-      <c r="H59" s="1">
+      <c r="H59" s="2">
         <v>46304</v>
       </c>
       <c r="I59" t="s">
@@ -4138,7 +4164,7 @@
       <c r="U59" t="s">
         <v>180</v>
       </c>
-      <c r="V59" s="1">
+      <c r="V59" s="2">
         <v>46321</v>
       </c>
     </row>
@@ -4164,7 +4190,7 @@
       <c r="G60" t="s">
         <v>109</v>
       </c>
-      <c r="H60" s="1">
+      <c r="H60" s="2">
         <v>46301</v>
       </c>
       <c r="I60" t="s">
@@ -4200,7 +4226,7 @@
       <c r="U60" t="s">
         <v>180</v>
       </c>
-      <c r="V60" s="1">
+      <c r="V60" s="2">
         <v>46352</v>
       </c>
     </row>
@@ -4244,7 +4270,7 @@
       <c r="U61" t="s">
         <v>180</v>
       </c>
-      <c r="V61" s="1">
+      <c r="V61" s="2">
         <v>46107</v>
       </c>
     </row>
@@ -4288,7 +4314,7 @@
       <c r="U62" t="s">
         <v>180</v>
       </c>
-      <c r="V62" s="1">
+      <c r="V62" s="2">
         <v>46107</v>
       </c>
     </row>
@@ -4332,7 +4358,7 @@
       <c r="U63" t="s">
         <v>180</v>
       </c>
-      <c r="V63" s="1">
+      <c r="V63" s="2">
         <v>46107</v>
       </c>
     </row>
@@ -4376,7 +4402,7 @@
       <c r="U64" t="s">
         <v>180</v>
       </c>
-      <c r="V64" s="1">
+      <c r="V64" s="2">
         <v>46107</v>
       </c>
     </row>
@@ -4420,7 +4446,7 @@
       <c r="U65" t="s">
         <v>180</v>
       </c>
-      <c r="V65" s="1">
+      <c r="V65" s="2">
         <v>46107</v>
       </c>
     </row>
@@ -4464,7 +4490,7 @@
       <c r="U66" t="s">
         <v>180</v>
       </c>
-      <c r="V66" s="1">
+      <c r="V66" s="2">
         <v>46107</v>
       </c>
     </row>
@@ -4508,7 +4534,7 @@
       <c r="U67" t="s">
         <v>92</v>
       </c>
-      <c r="V67" s="1">
+      <c r="V67" s="2">
         <v>46168</v>
       </c>
     </row>
@@ -4555,7 +4581,7 @@
       <c r="U68" t="s">
         <v>92</v>
       </c>
-      <c r="V68" s="1">
+      <c r="V68" s="2">
         <v>46291</v>
       </c>
     </row>
@@ -4581,7 +4607,7 @@
       <c r="G69" t="s">
         <v>107</v>
       </c>
-      <c r="H69" s="1">
+      <c r="H69" s="2">
         <v>46303</v>
       </c>
       <c r="I69" t="s">
@@ -4617,7 +4643,7 @@
       <c r="U69" t="s">
         <v>180</v>
       </c>
-      <c r="V69" s="1">
+      <c r="V69" s="2">
         <v>46229</v>
       </c>
     </row>
@@ -4661,7 +4687,7 @@
       <c r="U70" t="s">
         <v>92</v>
       </c>
-      <c r="V70" s="1">
+      <c r="V70" s="2">
         <v>46260</v>
       </c>
     </row>
@@ -4705,7 +4731,7 @@
       <c r="U71" t="s">
         <v>180</v>
       </c>
-      <c r="V71" s="1">
+      <c r="V71" s="2">
         <v>46291</v>
       </c>
     </row>
@@ -4749,7 +4775,7 @@
       <c r="U72" t="s">
         <v>180</v>
       </c>
-      <c r="V72" s="1">
+      <c r="V72" s="2">
         <v>46168</v>
       </c>
     </row>
@@ -4793,7 +4819,7 @@
       <c r="U73" t="s">
         <v>180</v>
       </c>
-      <c r="V73" s="1">
+      <c r="V73" s="2">
         <v>46291</v>
       </c>
     </row>
@@ -4837,7 +4863,7 @@
       <c r="U74" t="s">
         <v>180</v>
       </c>
-      <c r="V74" s="1">
+      <c r="V74" s="2">
         <v>46291</v>
       </c>
     </row>
@@ -4881,7 +4907,7 @@
       <c r="U75" t="s">
         <v>180</v>
       </c>
-      <c r="V75" s="1">
+      <c r="V75" s="2">
         <v>46291</v>
       </c>
     </row>
@@ -4928,7 +4954,7 @@
       <c r="U76" t="s">
         <v>92</v>
       </c>
-      <c r="V76" s="1">
+      <c r="V76" s="2">
         <v>46321</v>
       </c>
     </row>
@@ -4978,7 +5004,7 @@
       <c r="U77" t="s">
         <v>180</v>
       </c>
-      <c r="V77" s="1">
+      <c r="V77" s="2">
         <v>46381</v>
       </c>
     </row>
@@ -5028,7 +5054,7 @@
       <c r="U78" t="s">
         <v>180</v>
       </c>
-      <c r="V78" s="1">
+      <c r="V78" s="2">
         <v>46381</v>
       </c>
     </row>
@@ -5078,7 +5104,7 @@
       <c r="U79" t="s">
         <v>92</v>
       </c>
-      <c r="V79" s="1">
+      <c r="V79" s="2">
         <v>46381</v>
       </c>
     </row>
@@ -5128,7 +5154,7 @@
       <c r="U80" t="s">
         <v>92</v>
       </c>
-      <c r="V80" s="1">
+      <c r="V80" s="2">
         <v>46381</v>
       </c>
     </row>
@@ -5178,7 +5204,7 @@
       <c r="U81" t="s">
         <v>92</v>
       </c>
-      <c r="V81" s="1">
+      <c r="V81" s="2">
         <v>46382</v>
       </c>
     </row>
@@ -5222,7 +5248,7 @@
       <c r="U82" t="s">
         <v>92</v>
       </c>
-      <c r="V82" s="1">
+      <c r="V82" s="2">
         <v>46382</v>
       </c>
     </row>
@@ -5278,7 +5304,7 @@
       <c r="U83" t="s">
         <v>180</v>
       </c>
-      <c r="V83" s="1">
+      <c r="V83" s="2">
         <v>46382</v>
       </c>
     </row>
@@ -5328,7 +5354,7 @@
       <c r="U84" t="s">
         <v>92</v>
       </c>
-      <c r="V84" s="1">
+      <c r="V84" s="2">
         <v>46321</v>
       </c>
     </row>
@@ -5372,7 +5398,7 @@
       <c r="U85" t="s">
         <v>92</v>
       </c>
-      <c r="V85" s="1">
+      <c r="V85" s="2">
         <v>46382</v>
       </c>
     </row>
@@ -5492,7 +5518,7 @@
       <c r="G88" t="s">
         <v>109</v>
       </c>
-      <c r="H88" s="1">
+      <c r="H88" s="2">
         <v>46303</v>
       </c>
       <c r="I88" t="s">
@@ -5522,7 +5548,7 @@
       <c r="U88" t="s">
         <v>92</v>
       </c>
-      <c r="V88" s="1">
+      <c r="V88" s="2">
         <v>46291</v>
       </c>
     </row>
@@ -5569,7 +5595,7 @@
       <c r="U89" t="s">
         <v>92</v>
       </c>
-      <c r="V89" s="1">
+      <c r="V89" s="2">
         <v>46291</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Atualização automática: mta (19/10/2026 14:26)
</commit_message>
<xml_diff>
--- a/Projetos/02_Dados_Tratados/base_mta_tratada.xlsx
+++ b/Projetos/02_Dados_Tratados/base_mta_tratada.xlsx
@@ -566,16 +566,8 @@
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="YYYY-MM-DD HH:MM:SS"/>
   </numFmts>
-  <fonts count="2">
+  <fonts count="1">
     <font>
-      <sz val="11"/>
-      <color theme="1"/>
-      <name val="Calibri"/>
-      <family val="2"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <b/>
       <sz val="11"/>
       <color theme="1"/>
       <name val="Calibri"/>
@@ -591,7 +583,7 @@
       <patternFill patternType="gray125"/>
     </fill>
   </fills>
-  <borders count="2">
+  <borders count="1">
     <border>
       <left/>
       <right/>
@@ -599,30 +591,12 @@
       <bottom/>
       <diagonal/>
     </border>
-    <border>
-      <left style="thin">
-        <color auto="1"/>
-      </left>
-      <right style="thin">
-        <color auto="1"/>
-      </right>
-      <top style="thin">
-        <color auto="1"/>
-      </top>
-      <bottom style="thin">
-        <color auto="1"/>
-      </bottom>
-      <diagonal/>
-    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="3">
+  <cellXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top"/>
-    </xf>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
   </cellXfs>
   <cellStyles count="1">
@@ -922,70 +896,70 @@
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:22">
-      <c r="A1" s="1" t="s">
+      <c r="A1" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="1" t="s">
+      <c r="B1" t="s">
         <v>1</v>
       </c>
-      <c r="C1" s="1" t="s">
+      <c r="C1" t="s">
         <v>2</v>
       </c>
-      <c r="D1" s="1" t="s">
+      <c r="D1" t="s">
         <v>3</v>
       </c>
-      <c r="E1" s="1" t="s">
+      <c r="E1" t="s">
         <v>4</v>
       </c>
-      <c r="F1" s="1" t="s">
+      <c r="F1" t="s">
         <v>5</v>
       </c>
-      <c r="G1" s="1" t="s">
+      <c r="G1" t="s">
         <v>6</v>
       </c>
-      <c r="H1" s="1" t="s">
+      <c r="H1" t="s">
         <v>7</v>
       </c>
-      <c r="I1" s="1" t="s">
+      <c r="I1" t="s">
         <v>8</v>
       </c>
-      <c r="J1" s="1" t="s">
+      <c r="J1" t="s">
         <v>9</v>
       </c>
-      <c r="K1" s="1" t="s">
+      <c r="K1" t="s">
         <v>10</v>
       </c>
-      <c r="L1" s="1" t="s">
+      <c r="L1" t="s">
         <v>11</v>
       </c>
-      <c r="M1" s="1" t="s">
+      <c r="M1" t="s">
         <v>12</v>
       </c>
-      <c r="N1" s="1" t="s">
+      <c r="N1" t="s">
         <v>13</v>
       </c>
-      <c r="O1" s="1" t="s">
+      <c r="O1" t="s">
         <v>14</v>
       </c>
-      <c r="P1" s="1" t="s">
+      <c r="P1" t="s">
         <v>15</v>
       </c>
-      <c r="Q1" s="1" t="s">
+      <c r="Q1" t="s">
         <v>16</v>
       </c>
-      <c r="R1" s="1" t="s">
+      <c r="R1" t="s">
         <v>17</v>
       </c>
-      <c r="S1" s="1" t="s">
+      <c r="S1" t="s">
         <v>18</v>
       </c>
-      <c r="T1" s="1" t="s">
+      <c r="T1" t="s">
         <v>19</v>
       </c>
-      <c r="U1" s="1" t="s">
+      <c r="U1" t="s">
         <v>20</v>
       </c>
-      <c r="V1" s="1" t="s">
+      <c r="V1" t="s">
         <v>21</v>
       </c>
     </row>
@@ -1011,7 +985,7 @@
       <c r="G2" t="s">
         <v>107</v>
       </c>
-      <c r="H2" s="2">
+      <c r="H2" s="1">
         <v>46303</v>
       </c>
       <c r="I2" t="s">
@@ -1050,7 +1024,7 @@
       <c r="U2" t="s">
         <v>180</v>
       </c>
-      <c r="V2" s="2">
+      <c r="V2" s="1">
         <v>46229</v>
       </c>
     </row>
@@ -1097,7 +1071,7 @@
       <c r="U3" t="s">
         <v>92</v>
       </c>
-      <c r="V3" s="2">
+      <c r="V3" s="1">
         <v>46291</v>
       </c>
     </row>
@@ -1144,7 +1118,7 @@
       <c r="U4" t="s">
         <v>92</v>
       </c>
-      <c r="V4" s="2">
+      <c r="V4" s="1">
         <v>46321</v>
       </c>
     </row>
@@ -1191,7 +1165,7 @@
       <c r="U5" t="s">
         <v>92</v>
       </c>
-      <c r="V5" s="2">
+      <c r="V5" s="1">
         <v>46321</v>
       </c>
     </row>
@@ -1241,7 +1215,7 @@
       <c r="U6" t="s">
         <v>92</v>
       </c>
-      <c r="V6" s="2">
+      <c r="V6" s="1">
         <v>46291</v>
       </c>
     </row>
@@ -1267,7 +1241,7 @@
       <c r="G7" t="s">
         <v>109</v>
       </c>
-      <c r="H7" s="2">
+      <c r="H7" s="1">
         <v>46121</v>
       </c>
       <c r="I7" t="s">
@@ -1297,7 +1271,7 @@
       <c r="U7" t="s">
         <v>92</v>
       </c>
-      <c r="V7" s="2">
+      <c r="V7" s="1">
         <v>46138</v>
       </c>
     </row>
@@ -1344,7 +1318,7 @@
       <c r="U8" t="s">
         <v>92</v>
       </c>
-      <c r="V8" s="2">
+      <c r="V8" s="1">
         <v>46291</v>
       </c>
     </row>
@@ -1391,7 +1365,7 @@
       <c r="U9" t="s">
         <v>92</v>
       </c>
-      <c r="V9" s="2">
+      <c r="V9" s="1">
         <v>46291</v>
       </c>
     </row>
@@ -1414,7 +1388,7 @@
       <c r="G10" t="s">
         <v>109</v>
       </c>
-      <c r="H10" s="2">
+      <c r="H10" s="1">
         <v>46303</v>
       </c>
       <c r="I10" t="s">
@@ -1444,7 +1418,7 @@
       <c r="U10" t="s">
         <v>92</v>
       </c>
-      <c r="V10" s="2">
+      <c r="V10" s="1">
         <v>46291</v>
       </c>
     </row>
@@ -1491,7 +1465,7 @@
       <c r="U11" t="s">
         <v>92</v>
       </c>
-      <c r="V11" s="2">
+      <c r="V11" s="1">
         <v>46291</v>
       </c>
     </row>
@@ -1538,7 +1512,7 @@
       <c r="U12" t="s">
         <v>92</v>
       </c>
-      <c r="V12" s="2">
+      <c r="V12" s="1">
         <v>46291</v>
       </c>
     </row>
@@ -1564,7 +1538,7 @@
       <c r="G13" t="s">
         <v>109</v>
       </c>
-      <c r="H13" s="2">
+      <c r="H13" s="1">
         <v>46079</v>
       </c>
       <c r="I13" t="s">
@@ -1597,7 +1571,7 @@
       <c r="U13" t="s">
         <v>180</v>
       </c>
-      <c r="V13" s="2">
+      <c r="V13" s="1">
         <v>46079</v>
       </c>
     </row>
@@ -1623,7 +1597,7 @@
       <c r="G14" t="s">
         <v>107</v>
       </c>
-      <c r="H14" s="2">
+      <c r="H14" s="1">
         <v>46303</v>
       </c>
       <c r="I14" t="s">
@@ -1659,7 +1633,7 @@
       <c r="U14" t="s">
         <v>180</v>
       </c>
-      <c r="V14" s="2">
+      <c r="V14" s="1">
         <v>46352</v>
       </c>
     </row>
@@ -1685,7 +1659,7 @@
       <c r="G15" t="s">
         <v>107</v>
       </c>
-      <c r="H15" s="2">
+      <c r="H15" s="1">
         <v>46303</v>
       </c>
       <c r="I15" t="s">
@@ -1721,7 +1695,7 @@
       <c r="U15" t="s">
         <v>180</v>
       </c>
-      <c r="V15" s="2">
+      <c r="V15" s="1">
         <v>46352</v>
       </c>
     </row>
@@ -1747,7 +1721,7 @@
       <c r="G16" t="s">
         <v>107</v>
       </c>
-      <c r="H16" s="2">
+      <c r="H16" s="1">
         <v>46303</v>
       </c>
       <c r="I16" t="s">
@@ -1783,7 +1757,7 @@
       <c r="U16" t="s">
         <v>180</v>
       </c>
-      <c r="V16" s="2">
+      <c r="V16" s="1">
         <v>46352</v>
       </c>
     </row>
@@ -1809,7 +1783,7 @@
       <c r="G17" t="s">
         <v>107</v>
       </c>
-      <c r="H17" s="2">
+      <c r="H17" s="1">
         <v>46303</v>
       </c>
       <c r="I17" t="s">
@@ -1845,7 +1819,7 @@
       <c r="U17" t="s">
         <v>180</v>
       </c>
-      <c r="V17" s="2">
+      <c r="V17" s="1">
         <v>46229</v>
       </c>
     </row>
@@ -1871,7 +1845,7 @@
       <c r="G18" t="s">
         <v>109</v>
       </c>
-      <c r="H18" s="2">
+      <c r="H18" s="1">
         <v>46098</v>
       </c>
       <c r="I18" t="s">
@@ -1904,7 +1878,7 @@
       <c r="U18" t="s">
         <v>180</v>
       </c>
-      <c r="V18" s="2">
+      <c r="V18" s="1">
         <v>46107</v>
       </c>
     </row>
@@ -1930,7 +1904,7 @@
       <c r="G19" t="s">
         <v>109</v>
       </c>
-      <c r="H19" s="2">
+      <c r="H19" s="1">
         <v>46076</v>
       </c>
       <c r="I19" t="s">
@@ -1960,7 +1934,7 @@
       <c r="U19" t="s">
         <v>92</v>
       </c>
-      <c r="V19" s="2">
+      <c r="V19" s="1">
         <v>46079</v>
       </c>
     </row>
@@ -1986,7 +1960,7 @@
       <c r="G20" t="s">
         <v>109</v>
       </c>
-      <c r="H20" s="2">
+      <c r="H20" s="1">
         <v>46076</v>
       </c>
       <c r="I20" t="s">
@@ -2016,7 +1990,7 @@
       <c r="U20" t="s">
         <v>92</v>
       </c>
-      <c r="V20" s="2">
+      <c r="V20" s="1">
         <v>46079</v>
       </c>
     </row>
@@ -2063,7 +2037,7 @@
       <c r="U21" t="s">
         <v>92</v>
       </c>
-      <c r="V21" s="2">
+      <c r="V21" s="1">
         <v>46321</v>
       </c>
     </row>
@@ -2110,7 +2084,7 @@
       <c r="U22" t="s">
         <v>92</v>
       </c>
-      <c r="V22" s="2">
+      <c r="V22" s="1">
         <v>46321</v>
       </c>
     </row>
@@ -2157,7 +2131,7 @@
       <c r="U23" t="s">
         <v>92</v>
       </c>
-      <c r="V23" s="2">
+      <c r="V23" s="1">
         <v>46321</v>
       </c>
     </row>
@@ -2204,7 +2178,7 @@
       <c r="U24" t="s">
         <v>92</v>
       </c>
-      <c r="V24" s="2">
+      <c r="V24" s="1">
         <v>46321</v>
       </c>
     </row>
@@ -2230,7 +2204,7 @@
       <c r="G25" t="s">
         <v>109</v>
       </c>
-      <c r="H25" s="2">
+      <c r="H25" s="1">
         <v>46119</v>
       </c>
       <c r="I25" t="s">
@@ -2263,7 +2237,7 @@
       <c r="U25" t="s">
         <v>180</v>
       </c>
-      <c r="V25" s="2">
+      <c r="V25" s="1">
         <v>46138</v>
       </c>
     </row>
@@ -2289,7 +2263,7 @@
       <c r="G26" t="s">
         <v>109</v>
       </c>
-      <c r="H26" s="2">
+      <c r="H26" s="1">
         <v>46121</v>
       </c>
       <c r="I26" t="s">
@@ -2319,7 +2293,7 @@
       <c r="U26" t="s">
         <v>92</v>
       </c>
-      <c r="V26" s="2">
+      <c r="V26" s="1">
         <v>46138</v>
       </c>
     </row>
@@ -2345,7 +2319,7 @@
       <c r="G27" t="s">
         <v>109</v>
       </c>
-      <c r="H27" s="2">
+      <c r="H27" s="1">
         <v>46076</v>
       </c>
       <c r="I27" t="s">
@@ -2375,7 +2349,7 @@
       <c r="U27" t="s">
         <v>92</v>
       </c>
-      <c r="V27" s="2">
+      <c r="V27" s="1">
         <v>46079</v>
       </c>
     </row>
@@ -2401,7 +2375,7 @@
       <c r="G28" t="s">
         <v>107</v>
       </c>
-      <c r="H28" s="2">
+      <c r="H28" s="1">
         <v>46303</v>
       </c>
       <c r="I28" t="s">
@@ -2437,7 +2411,7 @@
       <c r="U28" t="s">
         <v>180</v>
       </c>
-      <c r="V28" s="2">
+      <c r="V28" s="1">
         <v>46291</v>
       </c>
     </row>
@@ -2463,7 +2437,7 @@
       <c r="G29" t="s">
         <v>109</v>
       </c>
-      <c r="H29" s="2">
+      <c r="H29" s="1">
         <v>46199</v>
       </c>
       <c r="I29" t="s">
@@ -2496,7 +2470,7 @@
       <c r="U29" t="s">
         <v>180</v>
       </c>
-      <c r="V29" s="2">
+      <c r="V29" s="1">
         <v>46199</v>
       </c>
     </row>
@@ -2522,7 +2496,7 @@
       <c r="G30" t="s">
         <v>109</v>
       </c>
-      <c r="H30" s="2">
+      <c r="H30" s="1">
         <v>46199</v>
       </c>
       <c r="I30" t="s">
@@ -2555,7 +2529,7 @@
       <c r="U30" t="s">
         <v>180</v>
       </c>
-      <c r="V30" s="2">
+      <c r="V30" s="1">
         <v>46199</v>
       </c>
     </row>
@@ -2581,7 +2555,7 @@
       <c r="G31" t="s">
         <v>109</v>
       </c>
-      <c r="H31" s="2">
+      <c r="H31" s="1">
         <v>46199</v>
       </c>
       <c r="I31" t="s">
@@ -2614,7 +2588,7 @@
       <c r="U31" t="s">
         <v>180</v>
       </c>
-      <c r="V31" s="2">
+      <c r="V31" s="1">
         <v>46199</v>
       </c>
     </row>
@@ -2640,7 +2614,7 @@
       <c r="G32" t="s">
         <v>109</v>
       </c>
-      <c r="H32" s="2">
+      <c r="H32" s="1">
         <v>46199</v>
       </c>
       <c r="I32" t="s">
@@ -2673,7 +2647,7 @@
       <c r="U32" t="s">
         <v>180</v>
       </c>
-      <c r="V32" s="2">
+      <c r="V32" s="1">
         <v>46199</v>
       </c>
     </row>
@@ -2726,7 +2700,7 @@
       <c r="U33" t="s">
         <v>180</v>
       </c>
-      <c r="V33" s="2">
+      <c r="V33" s="1">
         <v>46291</v>
       </c>
     </row>
@@ -2752,7 +2726,7 @@
       <c r="G34" t="s">
         <v>109</v>
       </c>
-      <c r="H34" s="2">
+      <c r="H34" s="1">
         <v>46191</v>
       </c>
       <c r="I34" t="s">
@@ -2785,7 +2759,7 @@
       <c r="U34" t="s">
         <v>180</v>
       </c>
-      <c r="V34" s="2">
+      <c r="V34" s="1">
         <v>46199</v>
       </c>
     </row>
@@ -2811,7 +2785,7 @@
       <c r="G35" t="s">
         <v>109</v>
       </c>
-      <c r="H35" s="2">
+      <c r="H35" s="1">
         <v>46119</v>
       </c>
       <c r="I35" t="s">
@@ -2841,7 +2815,7 @@
       <c r="U35" t="s">
         <v>180</v>
       </c>
-      <c r="V35" s="2">
+      <c r="V35" s="1">
         <v>46138</v>
       </c>
     </row>
@@ -2867,7 +2841,7 @@
       <c r="G36" t="s">
         <v>109</v>
       </c>
-      <c r="H36" s="2">
+      <c r="H36" s="1">
         <v>46213</v>
       </c>
       <c r="I36" t="s">
@@ -2897,7 +2871,7 @@
       <c r="U36" t="s">
         <v>92</v>
       </c>
-      <c r="V36" s="2">
+      <c r="V36" s="1">
         <v>46229</v>
       </c>
     </row>
@@ -2923,7 +2897,7 @@
       <c r="G37" t="s">
         <v>109</v>
       </c>
-      <c r="H37" s="2">
+      <c r="H37" s="1">
         <v>46175</v>
       </c>
       <c r="I37" t="s">
@@ -2953,7 +2927,7 @@
       <c r="U37" t="s">
         <v>92</v>
       </c>
-      <c r="V37" s="2">
+      <c r="V37" s="1">
         <v>46199</v>
       </c>
     </row>
@@ -2979,7 +2953,7 @@
       <c r="G38" t="s">
         <v>109</v>
       </c>
-      <c r="H38" s="2">
+      <c r="H38" s="1">
         <v>46213</v>
       </c>
       <c r="I38" t="s">
@@ -3009,7 +2983,7 @@
       <c r="U38" t="s">
         <v>92</v>
       </c>
-      <c r="V38" s="2">
+      <c r="V38" s="1">
         <v>46229</v>
       </c>
     </row>
@@ -3035,7 +3009,7 @@
       <c r="G39" t="s">
         <v>109</v>
       </c>
-      <c r="H39" s="2">
+      <c r="H39" s="1">
         <v>46199</v>
       </c>
       <c r="I39" t="s">
@@ -3065,7 +3039,7 @@
       <c r="U39" t="s">
         <v>92</v>
       </c>
-      <c r="V39" s="2">
+      <c r="V39" s="1">
         <v>46199</v>
       </c>
     </row>
@@ -3091,7 +3065,7 @@
       <c r="G40" t="s">
         <v>109</v>
       </c>
-      <c r="H40" s="2">
+      <c r="H40" s="1">
         <v>46199</v>
       </c>
       <c r="I40" t="s">
@@ -3121,7 +3095,7 @@
       <c r="U40" t="s">
         <v>92</v>
       </c>
-      <c r="V40" s="2">
+      <c r="V40" s="1">
         <v>46199</v>
       </c>
     </row>
@@ -3147,7 +3121,7 @@
       <c r="G41" t="s">
         <v>109</v>
       </c>
-      <c r="H41" s="2">
+      <c r="H41" s="1">
         <v>46204</v>
       </c>
       <c r="I41" t="s">
@@ -3177,7 +3151,7 @@
       <c r="U41" t="s">
         <v>92</v>
       </c>
-      <c r="V41" s="2">
+      <c r="V41" s="1">
         <v>46229</v>
       </c>
     </row>
@@ -3203,7 +3177,7 @@
       <c r="G42" t="s">
         <v>109</v>
       </c>
-      <c r="H42" s="2">
+      <c r="H42" s="1">
         <v>46244</v>
       </c>
       <c r="I42" t="s">
@@ -3233,7 +3207,7 @@
       <c r="U42" t="s">
         <v>92</v>
       </c>
-      <c r="V42" s="2">
+      <c r="V42" s="1">
         <v>46199</v>
       </c>
     </row>
@@ -3277,7 +3251,7 @@
       <c r="U43" t="s">
         <v>92</v>
       </c>
-      <c r="V43" s="2">
+      <c r="V43" s="1">
         <v>46260</v>
       </c>
     </row>
@@ -3303,7 +3277,7 @@
       <c r="G44" t="s">
         <v>109</v>
       </c>
-      <c r="H44" s="2">
+      <c r="H44" s="1">
         <v>46191</v>
       </c>
       <c r="I44" t="s">
@@ -3333,7 +3307,7 @@
       <c r="U44" t="s">
         <v>92</v>
       </c>
-      <c r="V44" s="2">
+      <c r="V44" s="1">
         <v>46199</v>
       </c>
     </row>
@@ -3359,7 +3333,7 @@
       <c r="G45" t="s">
         <v>109</v>
       </c>
-      <c r="H45" s="2">
+      <c r="H45" s="1">
         <v>46191</v>
       </c>
       <c r="I45" t="s">
@@ -3389,7 +3363,7 @@
       <c r="U45" t="s">
         <v>92</v>
       </c>
-      <c r="V45" s="2">
+      <c r="V45" s="1">
         <v>46199</v>
       </c>
     </row>
@@ -3415,7 +3389,7 @@
       <c r="G46" t="s">
         <v>109</v>
       </c>
-      <c r="H46" s="2">
+      <c r="H46" s="1">
         <v>46213</v>
       </c>
       <c r="I46" t="s">
@@ -3448,7 +3422,7 @@
       <c r="U46" t="s">
         <v>180</v>
       </c>
-      <c r="V46" s="2">
+      <c r="V46" s="1">
         <v>46229</v>
       </c>
     </row>
@@ -3474,7 +3448,7 @@
       <c r="G47" t="s">
         <v>109</v>
       </c>
-      <c r="H47" s="2">
+      <c r="H47" s="1">
         <v>46210</v>
       </c>
       <c r="I47" t="s">
@@ -3504,7 +3478,7 @@
       <c r="U47" t="s">
         <v>180</v>
       </c>
-      <c r="V47" s="2">
+      <c r="V47" s="1">
         <v>46229</v>
       </c>
     </row>
@@ -3551,7 +3525,7 @@
       <c r="U48" t="s">
         <v>92</v>
       </c>
-      <c r="V48" s="2">
+      <c r="V48" s="1">
         <v>46321</v>
       </c>
     </row>
@@ -3577,7 +3551,7 @@
       <c r="G49" t="s">
         <v>107</v>
       </c>
-      <c r="H49" s="2">
+      <c r="H49" s="1">
         <v>46303</v>
       </c>
       <c r="I49" t="s">
@@ -3613,7 +3587,7 @@
       <c r="U49" t="s">
         <v>180</v>
       </c>
-      <c r="V49" s="2">
+      <c r="V49" s="1">
         <v>46291</v>
       </c>
     </row>
@@ -3639,7 +3613,7 @@
       <c r="G50" t="s">
         <v>109</v>
       </c>
-      <c r="H50" s="2">
+      <c r="H50" s="1">
         <v>46176</v>
       </c>
       <c r="I50" t="s">
@@ -3672,7 +3646,7 @@
       <c r="U50" t="s">
         <v>180</v>
       </c>
-      <c r="V50" s="2">
+      <c r="V50" s="1">
         <v>46199</v>
       </c>
     </row>
@@ -3728,7 +3702,7 @@
       <c r="U51" t="s">
         <v>180</v>
       </c>
-      <c r="V51" s="2">
+      <c r="V51" s="1">
         <v>46260</v>
       </c>
     </row>
@@ -3754,7 +3728,7 @@
       <c r="G52" t="s">
         <v>109</v>
       </c>
-      <c r="H52" s="2">
+      <c r="H52" s="1">
         <v>46295</v>
       </c>
       <c r="I52" t="s">
@@ -3790,7 +3764,7 @@
       <c r="U52" t="s">
         <v>180</v>
       </c>
-      <c r="V52" s="2">
+      <c r="V52" s="1">
         <v>46291</v>
       </c>
     </row>
@@ -3843,7 +3817,7 @@
       <c r="U53" t="s">
         <v>180</v>
       </c>
-      <c r="V53" s="2">
+      <c r="V53" s="1">
         <v>46321</v>
       </c>
     </row>
@@ -3869,7 +3843,7 @@
       <c r="G54" t="s">
         <v>109</v>
       </c>
-      <c r="H54" s="2">
+      <c r="H54" s="1">
         <v>46227</v>
       </c>
       <c r="I54" t="s">
@@ -3899,7 +3873,7 @@
       <c r="U54" t="s">
         <v>180</v>
       </c>
-      <c r="V54" s="2">
+      <c r="V54" s="1">
         <v>46229</v>
       </c>
     </row>
@@ -3922,7 +3896,7 @@
       <c r="G55" t="s">
         <v>109</v>
       </c>
-      <c r="H55" s="2">
+      <c r="H55" s="1">
         <v>46280</v>
       </c>
       <c r="I55" t="s">
@@ -3952,7 +3926,7 @@
       <c r="U55" t="s">
         <v>180</v>
       </c>
-      <c r="V55" s="2">
+      <c r="V55" s="1">
         <v>46291</v>
       </c>
     </row>
@@ -3975,7 +3949,7 @@
       <c r="G56" t="s">
         <v>109</v>
       </c>
-      <c r="H56" s="2">
+      <c r="H56" s="1">
         <v>46280</v>
       </c>
       <c r="I56" t="s">
@@ -4005,7 +3979,7 @@
       <c r="U56" t="s">
         <v>180</v>
       </c>
-      <c r="V56" s="2">
+      <c r="V56" s="1">
         <v>46260</v>
       </c>
     </row>
@@ -4028,7 +4002,7 @@
       <c r="G57" t="s">
         <v>109</v>
       </c>
-      <c r="H57" s="2">
+      <c r="H57" s="1">
         <v>46295</v>
       </c>
       <c r="I57" t="s">
@@ -4058,7 +4032,7 @@
       <c r="U57" t="s">
         <v>180</v>
       </c>
-      <c r="V57" s="2">
+      <c r="V57" s="1">
         <v>46291</v>
       </c>
     </row>
@@ -4081,7 +4055,7 @@
       <c r="G58" t="s">
         <v>109</v>
       </c>
-      <c r="H58" s="2">
+      <c r="H58" s="1">
         <v>46295</v>
       </c>
       <c r="I58" t="s">
@@ -4111,7 +4085,7 @@
       <c r="U58" t="s">
         <v>180</v>
       </c>
-      <c r="V58" s="2">
+      <c r="V58" s="1">
         <v>46291</v>
       </c>
     </row>
@@ -4134,7 +4108,7 @@
       <c r="G59" t="s">
         <v>109</v>
       </c>
-      <c r="H59" s="2">
+      <c r="H59" s="1">
         <v>46304</v>
       </c>
       <c r="I59" t="s">
@@ -4164,7 +4138,7 @@
       <c r="U59" t="s">
         <v>180</v>
       </c>
-      <c r="V59" s="2">
+      <c r="V59" s="1">
         <v>46321</v>
       </c>
     </row>
@@ -4190,7 +4164,7 @@
       <c r="G60" t="s">
         <v>109</v>
       </c>
-      <c r="H60" s="2">
+      <c r="H60" s="1">
         <v>46301</v>
       </c>
       <c r="I60" t="s">
@@ -4226,7 +4200,7 @@
       <c r="U60" t="s">
         <v>180</v>
       </c>
-      <c r="V60" s="2">
+      <c r="V60" s="1">
         <v>46352</v>
       </c>
     </row>
@@ -4270,7 +4244,7 @@
       <c r="U61" t="s">
         <v>180</v>
       </c>
-      <c r="V61" s="2">
+      <c r="V61" s="1">
         <v>46107</v>
       </c>
     </row>
@@ -4314,7 +4288,7 @@
       <c r="U62" t="s">
         <v>180</v>
       </c>
-      <c r="V62" s="2">
+      <c r="V62" s="1">
         <v>46107</v>
       </c>
     </row>
@@ -4358,7 +4332,7 @@
       <c r="U63" t="s">
         <v>180</v>
       </c>
-      <c r="V63" s="2">
+      <c r="V63" s="1">
         <v>46107</v>
       </c>
     </row>
@@ -4402,7 +4376,7 @@
       <c r="U64" t="s">
         <v>180</v>
       </c>
-      <c r="V64" s="2">
+      <c r="V64" s="1">
         <v>46107</v>
       </c>
     </row>
@@ -4446,7 +4420,7 @@
       <c r="U65" t="s">
         <v>180</v>
       </c>
-      <c r="V65" s="2">
+      <c r="V65" s="1">
         <v>46107</v>
       </c>
     </row>
@@ -4490,7 +4464,7 @@
       <c r="U66" t="s">
         <v>180</v>
       </c>
-      <c r="V66" s="2">
+      <c r="V66" s="1">
         <v>46107</v>
       </c>
     </row>
@@ -4534,7 +4508,7 @@
       <c r="U67" t="s">
         <v>92</v>
       </c>
-      <c r="V67" s="2">
+      <c r="V67" s="1">
         <v>46168</v>
       </c>
     </row>
@@ -4581,7 +4555,7 @@
       <c r="U68" t="s">
         <v>92</v>
       </c>
-      <c r="V68" s="2">
+      <c r="V68" s="1">
         <v>46291</v>
       </c>
     </row>
@@ -4607,7 +4581,7 @@
       <c r="G69" t="s">
         <v>107</v>
       </c>
-      <c r="H69" s="2">
+      <c r="H69" s="1">
         <v>46303</v>
       </c>
       <c r="I69" t="s">
@@ -4643,7 +4617,7 @@
       <c r="U69" t="s">
         <v>180</v>
       </c>
-      <c r="V69" s="2">
+      <c r="V69" s="1">
         <v>46229</v>
       </c>
     </row>
@@ -4687,7 +4661,7 @@
       <c r="U70" t="s">
         <v>92</v>
       </c>
-      <c r="V70" s="2">
+      <c r="V70" s="1">
         <v>46260</v>
       </c>
     </row>
@@ -4731,7 +4705,7 @@
       <c r="U71" t="s">
         <v>180</v>
       </c>
-      <c r="V71" s="2">
+      <c r="V71" s="1">
         <v>46291</v>
       </c>
     </row>
@@ -4775,7 +4749,7 @@
       <c r="U72" t="s">
         <v>180</v>
       </c>
-      <c r="V72" s="2">
+      <c r="V72" s="1">
         <v>46168</v>
       </c>
     </row>
@@ -4819,7 +4793,7 @@
       <c r="U73" t="s">
         <v>180</v>
       </c>
-      <c r="V73" s="2">
+      <c r="V73" s="1">
         <v>46291</v>
       </c>
     </row>
@@ -4863,7 +4837,7 @@
       <c r="U74" t="s">
         <v>180</v>
       </c>
-      <c r="V74" s="2">
+      <c r="V74" s="1">
         <v>46291</v>
       </c>
     </row>
@@ -4907,7 +4881,7 @@
       <c r="U75" t="s">
         <v>180</v>
       </c>
-      <c r="V75" s="2">
+      <c r="V75" s="1">
         <v>46291</v>
       </c>
     </row>
@@ -4954,7 +4928,7 @@
       <c r="U76" t="s">
         <v>92</v>
       </c>
-      <c r="V76" s="2">
+      <c r="V76" s="1">
         <v>46321</v>
       </c>
     </row>
@@ -5004,7 +4978,7 @@
       <c r="U77" t="s">
         <v>180</v>
       </c>
-      <c r="V77" s="2">
+      <c r="V77" s="1">
         <v>46381</v>
       </c>
     </row>
@@ -5054,7 +5028,7 @@
       <c r="U78" t="s">
         <v>180</v>
       </c>
-      <c r="V78" s="2">
+      <c r="V78" s="1">
         <v>46381</v>
       </c>
     </row>
@@ -5104,7 +5078,7 @@
       <c r="U79" t="s">
         <v>92</v>
       </c>
-      <c r="V79" s="2">
+      <c r="V79" s="1">
         <v>46381</v>
       </c>
     </row>
@@ -5154,7 +5128,7 @@
       <c r="U80" t="s">
         <v>92</v>
       </c>
-      <c r="V80" s="2">
+      <c r="V80" s="1">
         <v>46381</v>
       </c>
     </row>
@@ -5204,7 +5178,7 @@
       <c r="U81" t="s">
         <v>92</v>
       </c>
-      <c r="V81" s="2">
+      <c r="V81" s="1">
         <v>46382</v>
       </c>
     </row>
@@ -5248,7 +5222,7 @@
       <c r="U82" t="s">
         <v>92</v>
       </c>
-      <c r="V82" s="2">
+      <c r="V82" s="1">
         <v>46382</v>
       </c>
     </row>
@@ -5304,7 +5278,7 @@
       <c r="U83" t="s">
         <v>180</v>
       </c>
-      <c r="V83" s="2">
+      <c r="V83" s="1">
         <v>46382</v>
       </c>
     </row>
@@ -5354,7 +5328,7 @@
       <c r="U84" t="s">
         <v>92</v>
       </c>
-      <c r="V84" s="2">
+      <c r="V84" s="1">
         <v>46321</v>
       </c>
     </row>
@@ -5398,7 +5372,7 @@
       <c r="U85" t="s">
         <v>92</v>
       </c>
-      <c r="V85" s="2">
+      <c r="V85" s="1">
         <v>46382</v>
       </c>
     </row>
@@ -5518,7 +5492,7 @@
       <c r="G88" t="s">
         <v>109</v>
       </c>
-      <c r="H88" s="2">
+      <c r="H88" s="1">
         <v>46303</v>
       </c>
       <c r="I88" t="s">
@@ -5548,7 +5522,7 @@
       <c r="U88" t="s">
         <v>92</v>
       </c>
-      <c r="V88" s="2">
+      <c r="V88" s="1">
         <v>46291</v>
       </c>
     </row>
@@ -5595,7 +5569,7 @@
       <c r="U89" t="s">
         <v>92</v>
       </c>
-      <c r="V89" s="2">
+      <c r="V89" s="1">
         <v>46291</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Atualização automática: mta (20/10/2026 12:38)
</commit_message>
<xml_diff>
--- a/Projetos/02_Dados_Tratados/base_mta_tratada.xlsx
+++ b/Projetos/02_Dados_Tratados/base_mta_tratada.xlsx
@@ -560,16 +560,8 @@
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="YYYY-MM-DD HH:MM:SS"/>
   </numFmts>
-  <fonts count="2">
+  <fonts count="1">
     <font>
-      <sz val="11"/>
-      <color theme="1"/>
-      <name val="Calibri"/>
-      <family val="2"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <b/>
       <sz val="11"/>
       <color theme="1"/>
       <name val="Calibri"/>
@@ -585,7 +577,7 @@
       <patternFill patternType="gray125"/>
     </fill>
   </fills>
-  <borders count="2">
+  <borders count="1">
     <border>
       <left/>
       <right/>
@@ -593,30 +585,12 @@
       <bottom/>
       <diagonal/>
     </border>
-    <border>
-      <left style="thin">
-        <color auto="1"/>
-      </left>
-      <right style="thin">
-        <color auto="1"/>
-      </right>
-      <top style="thin">
-        <color auto="1"/>
-      </top>
-      <bottom style="thin">
-        <color auto="1"/>
-      </bottom>
-      <diagonal/>
-    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="3">
+  <cellXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top"/>
-    </xf>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
   </cellXfs>
   <cellStyles count="1">
@@ -916,70 +890,70 @@
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:22">
-      <c r="A1" s="1" t="s">
+      <c r="A1" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="1" t="s">
+      <c r="B1" t="s">
         <v>1</v>
       </c>
-      <c r="C1" s="1" t="s">
+      <c r="C1" t="s">
         <v>2</v>
       </c>
-      <c r="D1" s="1" t="s">
+      <c r="D1" t="s">
         <v>3</v>
       </c>
-      <c r="E1" s="1" t="s">
+      <c r="E1" t="s">
         <v>4</v>
       </c>
-      <c r="F1" s="1" t="s">
+      <c r="F1" t="s">
         <v>5</v>
       </c>
-      <c r="G1" s="1" t="s">
+      <c r="G1" t="s">
         <v>6</v>
       </c>
-      <c r="H1" s="1" t="s">
+      <c r="H1" t="s">
         <v>7</v>
       </c>
-      <c r="I1" s="1" t="s">
+      <c r="I1" t="s">
         <v>8</v>
       </c>
-      <c r="J1" s="1" t="s">
+      <c r="J1" t="s">
         <v>9</v>
       </c>
-      <c r="K1" s="1" t="s">
+      <c r="K1" t="s">
         <v>10</v>
       </c>
-      <c r="L1" s="1" t="s">
+      <c r="L1" t="s">
         <v>11</v>
       </c>
-      <c r="M1" s="1" t="s">
+      <c r="M1" t="s">
         <v>12</v>
       </c>
-      <c r="N1" s="1" t="s">
+      <c r="N1" t="s">
         <v>13</v>
       </c>
-      <c r="O1" s="1" t="s">
+      <c r="O1" t="s">
         <v>14</v>
       </c>
-      <c r="P1" s="1" t="s">
+      <c r="P1" t="s">
         <v>15</v>
       </c>
-      <c r="Q1" s="1" t="s">
+      <c r="Q1" t="s">
         <v>16</v>
       </c>
-      <c r="R1" s="1" t="s">
+      <c r="R1" t="s">
         <v>17</v>
       </c>
-      <c r="S1" s="1" t="s">
+      <c r="S1" t="s">
         <v>18</v>
       </c>
-      <c r="T1" s="1" t="s">
+      <c r="T1" t="s">
         <v>19</v>
       </c>
-      <c r="U1" s="1" t="s">
+      <c r="U1" t="s">
         <v>20</v>
       </c>
-      <c r="V1" s="1" t="s">
+      <c r="V1" t="s">
         <v>21</v>
       </c>
     </row>
@@ -1005,7 +979,7 @@
       <c r="G2" t="s">
         <v>106</v>
       </c>
-      <c r="H2" s="2">
+      <c r="H2" s="1">
         <v>46303</v>
       </c>
       <c r="I2" t="s">
@@ -1044,7 +1018,7 @@
       <c r="U2" t="s">
         <v>178</v>
       </c>
-      <c r="V2" s="2">
+      <c r="V2" s="1">
         <v>46229</v>
       </c>
     </row>
@@ -1091,7 +1065,7 @@
       <c r="U3" t="s">
         <v>91</v>
       </c>
-      <c r="V3" s="2">
+      <c r="V3" s="1">
         <v>46291</v>
       </c>
     </row>
@@ -1138,7 +1112,7 @@
       <c r="U4" t="s">
         <v>91</v>
       </c>
-      <c r="V4" s="2">
+      <c r="V4" s="1">
         <v>46321</v>
       </c>
     </row>
@@ -1185,7 +1159,7 @@
       <c r="U5" t="s">
         <v>91</v>
       </c>
-      <c r="V5" s="2">
+      <c r="V5" s="1">
         <v>46321</v>
       </c>
     </row>
@@ -1235,7 +1209,7 @@
       <c r="U6" t="s">
         <v>91</v>
       </c>
-      <c r="V6" s="2">
+      <c r="V6" s="1">
         <v>46291</v>
       </c>
     </row>
@@ -1261,7 +1235,7 @@
       <c r="G7" t="s">
         <v>106</v>
       </c>
-      <c r="H7" s="2">
+      <c r="H7" s="1">
         <v>46121</v>
       </c>
       <c r="I7" t="s">
@@ -1291,7 +1265,7 @@
       <c r="U7" t="s">
         <v>91</v>
       </c>
-      <c r="V7" s="2">
+      <c r="V7" s="1">
         <v>46138</v>
       </c>
     </row>
@@ -1338,7 +1312,7 @@
       <c r="U8" t="s">
         <v>91</v>
       </c>
-      <c r="V8" s="2">
+      <c r="V8" s="1">
         <v>46291</v>
       </c>
     </row>
@@ -1385,7 +1359,7 @@
       <c r="U9" t="s">
         <v>91</v>
       </c>
-      <c r="V9" s="2">
+      <c r="V9" s="1">
         <v>46291</v>
       </c>
     </row>
@@ -1408,7 +1382,7 @@
       <c r="G10" t="s">
         <v>106</v>
       </c>
-      <c r="H10" s="2">
+      <c r="H10" s="1">
         <v>46303</v>
       </c>
       <c r="I10" t="s">
@@ -1438,7 +1412,7 @@
       <c r="U10" t="s">
         <v>91</v>
       </c>
-      <c r="V10" s="2">
+      <c r="V10" s="1">
         <v>46291</v>
       </c>
     </row>
@@ -1485,7 +1459,7 @@
       <c r="U11" t="s">
         <v>91</v>
       </c>
-      <c r="V11" s="2">
+      <c r="V11" s="1">
         <v>46291</v>
       </c>
     </row>
@@ -1532,7 +1506,7 @@
       <c r="U12" t="s">
         <v>91</v>
       </c>
-      <c r="V12" s="2">
+      <c r="V12" s="1">
         <v>46291</v>
       </c>
     </row>
@@ -1558,7 +1532,7 @@
       <c r="G13" t="s">
         <v>106</v>
       </c>
-      <c r="H13" s="2">
+      <c r="H13" s="1">
         <v>46079</v>
       </c>
       <c r="I13" t="s">
@@ -1591,7 +1565,7 @@
       <c r="U13" t="s">
         <v>178</v>
       </c>
-      <c r="V13" s="2">
+      <c r="V13" s="1">
         <v>46079</v>
       </c>
     </row>
@@ -1617,7 +1591,7 @@
       <c r="G14" t="s">
         <v>106</v>
       </c>
-      <c r="H14" s="2">
+      <c r="H14" s="1">
         <v>46303</v>
       </c>
       <c r="I14" t="s">
@@ -1653,7 +1627,7 @@
       <c r="U14" t="s">
         <v>178</v>
       </c>
-      <c r="V14" s="2">
+      <c r="V14" s="1">
         <v>46352</v>
       </c>
     </row>
@@ -1679,7 +1653,7 @@
       <c r="G15" t="s">
         <v>106</v>
       </c>
-      <c r="H15" s="2">
+      <c r="H15" s="1">
         <v>46303</v>
       </c>
       <c r="I15" t="s">
@@ -1715,7 +1689,7 @@
       <c r="U15" t="s">
         <v>178</v>
       </c>
-      <c r="V15" s="2">
+      <c r="V15" s="1">
         <v>46352</v>
       </c>
     </row>
@@ -1741,7 +1715,7 @@
       <c r="G16" t="s">
         <v>106</v>
       </c>
-      <c r="H16" s="2">
+      <c r="H16" s="1">
         <v>46303</v>
       </c>
       <c r="I16" t="s">
@@ -1777,7 +1751,7 @@
       <c r="U16" t="s">
         <v>178</v>
       </c>
-      <c r="V16" s="2">
+      <c r="V16" s="1">
         <v>46352</v>
       </c>
     </row>
@@ -1803,7 +1777,7 @@
       <c r="G17" t="s">
         <v>106</v>
       </c>
-      <c r="H17" s="2">
+      <c r="H17" s="1">
         <v>46303</v>
       </c>
       <c r="I17" t="s">
@@ -1839,7 +1813,7 @@
       <c r="U17" t="s">
         <v>178</v>
       </c>
-      <c r="V17" s="2">
+      <c r="V17" s="1">
         <v>46229</v>
       </c>
     </row>
@@ -1865,7 +1839,7 @@
       <c r="G18" t="s">
         <v>106</v>
       </c>
-      <c r="H18" s="2">
+      <c r="H18" s="1">
         <v>46098</v>
       </c>
       <c r="I18" t="s">
@@ -1898,7 +1872,7 @@
       <c r="U18" t="s">
         <v>178</v>
       </c>
-      <c r="V18" s="2">
+      <c r="V18" s="1">
         <v>46107</v>
       </c>
     </row>
@@ -1924,7 +1898,7 @@
       <c r="G19" t="s">
         <v>106</v>
       </c>
-      <c r="H19" s="2">
+      <c r="H19" s="1">
         <v>46076</v>
       </c>
       <c r="I19" t="s">
@@ -1954,7 +1928,7 @@
       <c r="U19" t="s">
         <v>91</v>
       </c>
-      <c r="V19" s="2">
+      <c r="V19" s="1">
         <v>46079</v>
       </c>
     </row>
@@ -1980,7 +1954,7 @@
       <c r="G20" t="s">
         <v>106</v>
       </c>
-      <c r="H20" s="2">
+      <c r="H20" s="1">
         <v>46076</v>
       </c>
       <c r="I20" t="s">
@@ -2010,7 +1984,7 @@
       <c r="U20" t="s">
         <v>91</v>
       </c>
-      <c r="V20" s="2">
+      <c r="V20" s="1">
         <v>46079</v>
       </c>
     </row>
@@ -2057,7 +2031,7 @@
       <c r="U21" t="s">
         <v>91</v>
       </c>
-      <c r="V21" s="2">
+      <c r="V21" s="1">
         <v>46321</v>
       </c>
     </row>
@@ -2104,7 +2078,7 @@
       <c r="U22" t="s">
         <v>91</v>
       </c>
-      <c r="V22" s="2">
+      <c r="V22" s="1">
         <v>46321</v>
       </c>
     </row>
@@ -2151,7 +2125,7 @@
       <c r="U23" t="s">
         <v>91</v>
       </c>
-      <c r="V23" s="2">
+      <c r="V23" s="1">
         <v>46321</v>
       </c>
     </row>
@@ -2198,7 +2172,7 @@
       <c r="U24" t="s">
         <v>91</v>
       </c>
-      <c r="V24" s="2">
+      <c r="V24" s="1">
         <v>46321</v>
       </c>
     </row>
@@ -2224,7 +2198,7 @@
       <c r="G25" t="s">
         <v>106</v>
       </c>
-      <c r="H25" s="2">
+      <c r="H25" s="1">
         <v>46119</v>
       </c>
       <c r="I25" t="s">
@@ -2257,7 +2231,7 @@
       <c r="U25" t="s">
         <v>178</v>
       </c>
-      <c r="V25" s="2">
+      <c r="V25" s="1">
         <v>46138</v>
       </c>
     </row>
@@ -2283,7 +2257,7 @@
       <c r="G26" t="s">
         <v>106</v>
       </c>
-      <c r="H26" s="2">
+      <c r="H26" s="1">
         <v>46121</v>
       </c>
       <c r="I26" t="s">
@@ -2313,7 +2287,7 @@
       <c r="U26" t="s">
         <v>91</v>
       </c>
-      <c r="V26" s="2">
+      <c r="V26" s="1">
         <v>46138</v>
       </c>
     </row>
@@ -2339,7 +2313,7 @@
       <c r="G27" t="s">
         <v>106</v>
       </c>
-      <c r="H27" s="2">
+      <c r="H27" s="1">
         <v>46076</v>
       </c>
       <c r="I27" t="s">
@@ -2369,7 +2343,7 @@
       <c r="U27" t="s">
         <v>91</v>
       </c>
-      <c r="V27" s="2">
+      <c r="V27" s="1">
         <v>46079</v>
       </c>
     </row>
@@ -2395,7 +2369,7 @@
       <c r="G28" t="s">
         <v>106</v>
       </c>
-      <c r="H28" s="2">
+      <c r="H28" s="1">
         <v>46303</v>
       </c>
       <c r="I28" t="s">
@@ -2431,7 +2405,7 @@
       <c r="U28" t="s">
         <v>178</v>
       </c>
-      <c r="V28" s="2">
+      <c r="V28" s="1">
         <v>46291</v>
       </c>
     </row>
@@ -2457,7 +2431,7 @@
       <c r="G29" t="s">
         <v>106</v>
       </c>
-      <c r="H29" s="2">
+      <c r="H29" s="1">
         <v>46199</v>
       </c>
       <c r="I29" t="s">
@@ -2490,7 +2464,7 @@
       <c r="U29" t="s">
         <v>178</v>
       </c>
-      <c r="V29" s="2">
+      <c r="V29" s="1">
         <v>46199</v>
       </c>
     </row>
@@ -2516,7 +2490,7 @@
       <c r="G30" t="s">
         <v>106</v>
       </c>
-      <c r="H30" s="2">
+      <c r="H30" s="1">
         <v>46199</v>
       </c>
       <c r="I30" t="s">
@@ -2549,7 +2523,7 @@
       <c r="U30" t="s">
         <v>178</v>
       </c>
-      <c r="V30" s="2">
+      <c r="V30" s="1">
         <v>46199</v>
       </c>
     </row>
@@ -2575,7 +2549,7 @@
       <c r="G31" t="s">
         <v>106</v>
       </c>
-      <c r="H31" s="2">
+      <c r="H31" s="1">
         <v>46199</v>
       </c>
       <c r="I31" t="s">
@@ -2608,7 +2582,7 @@
       <c r="U31" t="s">
         <v>178</v>
       </c>
-      <c r="V31" s="2">
+      <c r="V31" s="1">
         <v>46199</v>
       </c>
     </row>
@@ -2634,7 +2608,7 @@
       <c r="G32" t="s">
         <v>106</v>
       </c>
-      <c r="H32" s="2">
+      <c r="H32" s="1">
         <v>46199</v>
       </c>
       <c r="I32" t="s">
@@ -2667,7 +2641,7 @@
       <c r="U32" t="s">
         <v>178</v>
       </c>
-      <c r="V32" s="2">
+      <c r="V32" s="1">
         <v>46199</v>
       </c>
     </row>
@@ -2720,7 +2694,7 @@
       <c r="U33" t="s">
         <v>178</v>
       </c>
-      <c r="V33" s="2">
+      <c r="V33" s="1">
         <v>46291</v>
       </c>
     </row>
@@ -2746,7 +2720,7 @@
       <c r="G34" t="s">
         <v>106</v>
       </c>
-      <c r="H34" s="2">
+      <c r="H34" s="1">
         <v>46191</v>
       </c>
       <c r="I34" t="s">
@@ -2779,7 +2753,7 @@
       <c r="U34" t="s">
         <v>178</v>
       </c>
-      <c r="V34" s="2">
+      <c r="V34" s="1">
         <v>46199</v>
       </c>
     </row>
@@ -2805,7 +2779,7 @@
       <c r="G35" t="s">
         <v>106</v>
       </c>
-      <c r="H35" s="2">
+      <c r="H35" s="1">
         <v>46119</v>
       </c>
       <c r="I35" t="s">
@@ -2835,7 +2809,7 @@
       <c r="U35" t="s">
         <v>178</v>
       </c>
-      <c r="V35" s="2">
+      <c r="V35" s="1">
         <v>46138</v>
       </c>
     </row>
@@ -2861,7 +2835,7 @@
       <c r="G36" t="s">
         <v>106</v>
       </c>
-      <c r="H36" s="2">
+      <c r="H36" s="1">
         <v>46213</v>
       </c>
       <c r="I36" t="s">
@@ -2891,7 +2865,7 @@
       <c r="U36" t="s">
         <v>91</v>
       </c>
-      <c r="V36" s="2">
+      <c r="V36" s="1">
         <v>46229</v>
       </c>
     </row>
@@ -2917,7 +2891,7 @@
       <c r="G37" t="s">
         <v>106</v>
       </c>
-      <c r="H37" s="2">
+      <c r="H37" s="1">
         <v>46175</v>
       </c>
       <c r="I37" t="s">
@@ -2947,7 +2921,7 @@
       <c r="U37" t="s">
         <v>91</v>
       </c>
-      <c r="V37" s="2">
+      <c r="V37" s="1">
         <v>46199</v>
       </c>
     </row>
@@ -2973,7 +2947,7 @@
       <c r="G38" t="s">
         <v>106</v>
       </c>
-      <c r="H38" s="2">
+      <c r="H38" s="1">
         <v>46213</v>
       </c>
       <c r="I38" t="s">
@@ -3003,7 +2977,7 @@
       <c r="U38" t="s">
         <v>91</v>
       </c>
-      <c r="V38" s="2">
+      <c r="V38" s="1">
         <v>46229</v>
       </c>
     </row>
@@ -3029,7 +3003,7 @@
       <c r="G39" t="s">
         <v>106</v>
       </c>
-      <c r="H39" s="2">
+      <c r="H39" s="1">
         <v>46199</v>
       </c>
       <c r="I39" t="s">
@@ -3059,7 +3033,7 @@
       <c r="U39" t="s">
         <v>91</v>
       </c>
-      <c r="V39" s="2">
+      <c r="V39" s="1">
         <v>46199</v>
       </c>
     </row>
@@ -3085,7 +3059,7 @@
       <c r="G40" t="s">
         <v>106</v>
       </c>
-      <c r="H40" s="2">
+      <c r="H40" s="1">
         <v>46199</v>
       </c>
       <c r="I40" t="s">
@@ -3115,7 +3089,7 @@
       <c r="U40" t="s">
         <v>91</v>
       </c>
-      <c r="V40" s="2">
+      <c r="V40" s="1">
         <v>46199</v>
       </c>
     </row>
@@ -3141,7 +3115,7 @@
       <c r="G41" t="s">
         <v>106</v>
       </c>
-      <c r="H41" s="2">
+      <c r="H41" s="1">
         <v>46204</v>
       </c>
       <c r="I41" t="s">
@@ -3171,7 +3145,7 @@
       <c r="U41" t="s">
         <v>91</v>
       </c>
-      <c r="V41" s="2">
+      <c r="V41" s="1">
         <v>46229</v>
       </c>
     </row>
@@ -3197,7 +3171,7 @@
       <c r="G42" t="s">
         <v>106</v>
       </c>
-      <c r="H42" s="2">
+      <c r="H42" s="1">
         <v>46244</v>
       </c>
       <c r="I42" t="s">
@@ -3227,7 +3201,7 @@
       <c r="U42" t="s">
         <v>91</v>
       </c>
-      <c r="V42" s="2">
+      <c r="V42" s="1">
         <v>46199</v>
       </c>
     </row>
@@ -3271,7 +3245,7 @@
       <c r="U43" t="s">
         <v>91</v>
       </c>
-      <c r="V43" s="2">
+      <c r="V43" s="1">
         <v>46260</v>
       </c>
     </row>
@@ -3297,7 +3271,7 @@
       <c r="G44" t="s">
         <v>106</v>
       </c>
-      <c r="H44" s="2">
+      <c r="H44" s="1">
         <v>46191</v>
       </c>
       <c r="I44" t="s">
@@ -3327,7 +3301,7 @@
       <c r="U44" t="s">
         <v>91</v>
       </c>
-      <c r="V44" s="2">
+      <c r="V44" s="1">
         <v>46199</v>
       </c>
     </row>
@@ -3353,7 +3327,7 @@
       <c r="G45" t="s">
         <v>106</v>
       </c>
-      <c r="H45" s="2">
+      <c r="H45" s="1">
         <v>46191</v>
       </c>
       <c r="I45" t="s">
@@ -3383,7 +3357,7 @@
       <c r="U45" t="s">
         <v>91</v>
       </c>
-      <c r="V45" s="2">
+      <c r="V45" s="1">
         <v>46199</v>
       </c>
     </row>
@@ -3409,7 +3383,7 @@
       <c r="G46" t="s">
         <v>106</v>
       </c>
-      <c r="H46" s="2">
+      <c r="H46" s="1">
         <v>46213</v>
       </c>
       <c r="I46" t="s">
@@ -3442,7 +3416,7 @@
       <c r="U46" t="s">
         <v>178</v>
       </c>
-      <c r="V46" s="2">
+      <c r="V46" s="1">
         <v>46229</v>
       </c>
     </row>
@@ -3468,7 +3442,7 @@
       <c r="G47" t="s">
         <v>106</v>
       </c>
-      <c r="H47" s="2">
+      <c r="H47" s="1">
         <v>46210</v>
       </c>
       <c r="I47" t="s">
@@ -3498,7 +3472,7 @@
       <c r="U47" t="s">
         <v>178</v>
       </c>
-      <c r="V47" s="2">
+      <c r="V47" s="1">
         <v>46229</v>
       </c>
     </row>
@@ -3545,7 +3519,7 @@
       <c r="U48" t="s">
         <v>91</v>
       </c>
-      <c r="V48" s="2">
+      <c r="V48" s="1">
         <v>46321</v>
       </c>
     </row>
@@ -3571,7 +3545,7 @@
       <c r="G49" t="s">
         <v>106</v>
       </c>
-      <c r="H49" s="2">
+      <c r="H49" s="1">
         <v>46303</v>
       </c>
       <c r="I49" t="s">
@@ -3607,7 +3581,7 @@
       <c r="U49" t="s">
         <v>178</v>
       </c>
-      <c r="V49" s="2">
+      <c r="V49" s="1">
         <v>46291</v>
       </c>
     </row>
@@ -3633,7 +3607,7 @@
       <c r="G50" t="s">
         <v>106</v>
       </c>
-      <c r="H50" s="2">
+      <c r="H50" s="1">
         <v>46176</v>
       </c>
       <c r="I50" t="s">
@@ -3666,7 +3640,7 @@
       <c r="U50" t="s">
         <v>178</v>
       </c>
-      <c r="V50" s="2">
+      <c r="V50" s="1">
         <v>46199</v>
       </c>
     </row>
@@ -3722,7 +3696,7 @@
       <c r="U51" t="s">
         <v>178</v>
       </c>
-      <c r="V51" s="2">
+      <c r="V51" s="1">
         <v>46260</v>
       </c>
     </row>
@@ -3748,7 +3722,7 @@
       <c r="G52" t="s">
         <v>106</v>
       </c>
-      <c r="H52" s="2">
+      <c r="H52" s="1">
         <v>46295</v>
       </c>
       <c r="I52" t="s">
@@ -3784,7 +3758,7 @@
       <c r="U52" t="s">
         <v>178</v>
       </c>
-      <c r="V52" s="2">
+      <c r="V52" s="1">
         <v>46291</v>
       </c>
     </row>
@@ -3837,7 +3811,7 @@
       <c r="U53" t="s">
         <v>178</v>
       </c>
-      <c r="V53" s="2">
+      <c r="V53" s="1">
         <v>46321</v>
       </c>
     </row>
@@ -3863,7 +3837,7 @@
       <c r="G54" t="s">
         <v>106</v>
       </c>
-      <c r="H54" s="2">
+      <c r="H54" s="1">
         <v>46227</v>
       </c>
       <c r="I54" t="s">
@@ -3893,7 +3867,7 @@
       <c r="U54" t="s">
         <v>178</v>
       </c>
-      <c r="V54" s="2">
+      <c r="V54" s="1">
         <v>46229</v>
       </c>
     </row>
@@ -3916,7 +3890,7 @@
       <c r="G55" t="s">
         <v>106</v>
       </c>
-      <c r="H55" s="2">
+      <c r="H55" s="1">
         <v>46280</v>
       </c>
       <c r="I55" t="s">
@@ -3946,7 +3920,7 @@
       <c r="U55" t="s">
         <v>178</v>
       </c>
-      <c r="V55" s="2">
+      <c r="V55" s="1">
         <v>46291</v>
       </c>
     </row>
@@ -3969,7 +3943,7 @@
       <c r="G56" t="s">
         <v>106</v>
       </c>
-      <c r="H56" s="2">
+      <c r="H56" s="1">
         <v>46280</v>
       </c>
       <c r="I56" t="s">
@@ -3999,7 +3973,7 @@
       <c r="U56" t="s">
         <v>178</v>
       </c>
-      <c r="V56" s="2">
+      <c r="V56" s="1">
         <v>46260</v>
       </c>
     </row>
@@ -4022,7 +3996,7 @@
       <c r="G57" t="s">
         <v>106</v>
       </c>
-      <c r="H57" s="2">
+      <c r="H57" s="1">
         <v>46295</v>
       </c>
       <c r="I57" t="s">
@@ -4052,7 +4026,7 @@
       <c r="U57" t="s">
         <v>178</v>
       </c>
-      <c r="V57" s="2">
+      <c r="V57" s="1">
         <v>46291</v>
       </c>
     </row>
@@ -4075,7 +4049,7 @@
       <c r="G58" t="s">
         <v>106</v>
       </c>
-      <c r="H58" s="2">
+      <c r="H58" s="1">
         <v>46295</v>
       </c>
       <c r="I58" t="s">
@@ -4105,7 +4079,7 @@
       <c r="U58" t="s">
         <v>178</v>
       </c>
-      <c r="V58" s="2">
+      <c r="V58" s="1">
         <v>46291</v>
       </c>
     </row>
@@ -4128,7 +4102,7 @@
       <c r="G59" t="s">
         <v>106</v>
       </c>
-      <c r="H59" s="2">
+      <c r="H59" s="1">
         <v>46304</v>
       </c>
       <c r="I59" t="s">
@@ -4158,7 +4132,7 @@
       <c r="U59" t="s">
         <v>178</v>
       </c>
-      <c r="V59" s="2">
+      <c r="V59" s="1">
         <v>46321</v>
       </c>
     </row>
@@ -4184,7 +4158,7 @@
       <c r="G60" t="s">
         <v>106</v>
       </c>
-      <c r="H60" s="2">
+      <c r="H60" s="1">
         <v>46301</v>
       </c>
       <c r="I60" t="s">
@@ -4220,7 +4194,7 @@
       <c r="U60" t="s">
         <v>178</v>
       </c>
-      <c r="V60" s="2">
+      <c r="V60" s="1">
         <v>46352</v>
       </c>
     </row>
@@ -4264,7 +4238,7 @@
       <c r="U61" t="s">
         <v>178</v>
       </c>
-      <c r="V61" s="2">
+      <c r="V61" s="1">
         <v>46107</v>
       </c>
     </row>
@@ -4308,7 +4282,7 @@
       <c r="U62" t="s">
         <v>178</v>
       </c>
-      <c r="V62" s="2">
+      <c r="V62" s="1">
         <v>46107</v>
       </c>
     </row>
@@ -4352,7 +4326,7 @@
       <c r="U63" t="s">
         <v>178</v>
       </c>
-      <c r="V63" s="2">
+      <c r="V63" s="1">
         <v>46107</v>
       </c>
     </row>
@@ -4396,7 +4370,7 @@
       <c r="U64" t="s">
         <v>178</v>
       </c>
-      <c r="V64" s="2">
+      <c r="V64" s="1">
         <v>46107</v>
       </c>
     </row>
@@ -4440,7 +4414,7 @@
       <c r="U65" t="s">
         <v>178</v>
       </c>
-      <c r="V65" s="2">
+      <c r="V65" s="1">
         <v>46107</v>
       </c>
     </row>
@@ -4484,7 +4458,7 @@
       <c r="U66" t="s">
         <v>178</v>
       </c>
-      <c r="V66" s="2">
+      <c r="V66" s="1">
         <v>46107</v>
       </c>
     </row>
@@ -4528,7 +4502,7 @@
       <c r="U67" t="s">
         <v>91</v>
       </c>
-      <c r="V67" s="2">
+      <c r="V67" s="1">
         <v>46168</v>
       </c>
     </row>
@@ -4575,7 +4549,7 @@
       <c r="U68" t="s">
         <v>91</v>
       </c>
-      <c r="V68" s="2">
+      <c r="V68" s="1">
         <v>46291</v>
       </c>
     </row>
@@ -4601,7 +4575,7 @@
       <c r="G69" t="s">
         <v>106</v>
       </c>
-      <c r="H69" s="2">
+      <c r="H69" s="1">
         <v>46303</v>
       </c>
       <c r="I69" t="s">
@@ -4637,7 +4611,7 @@
       <c r="U69" t="s">
         <v>178</v>
       </c>
-      <c r="V69" s="2">
+      <c r="V69" s="1">
         <v>46229</v>
       </c>
     </row>
@@ -4681,7 +4655,7 @@
       <c r="U70" t="s">
         <v>91</v>
       </c>
-      <c r="V70" s="2">
+      <c r="V70" s="1">
         <v>46260</v>
       </c>
     </row>
@@ -4725,7 +4699,7 @@
       <c r="U71" t="s">
         <v>178</v>
       </c>
-      <c r="V71" s="2">
+      <c r="V71" s="1">
         <v>46291</v>
       </c>
     </row>
@@ -4769,7 +4743,7 @@
       <c r="U72" t="s">
         <v>178</v>
       </c>
-      <c r="V72" s="2">
+      <c r="V72" s="1">
         <v>46168</v>
       </c>
     </row>
@@ -4813,7 +4787,7 @@
       <c r="U73" t="s">
         <v>178</v>
       </c>
-      <c r="V73" s="2">
+      <c r="V73" s="1">
         <v>46291</v>
       </c>
     </row>
@@ -4857,7 +4831,7 @@
       <c r="U74" t="s">
         <v>178</v>
       </c>
-      <c r="V74" s="2">
+      <c r="V74" s="1">
         <v>46291</v>
       </c>
     </row>
@@ -4901,7 +4875,7 @@
       <c r="U75" t="s">
         <v>178</v>
       </c>
-      <c r="V75" s="2">
+      <c r="V75" s="1">
         <v>46291</v>
       </c>
     </row>
@@ -4948,7 +4922,7 @@
       <c r="U76" t="s">
         <v>91</v>
       </c>
-      <c r="V76" s="2">
+      <c r="V76" s="1">
         <v>46321</v>
       </c>
     </row>
@@ -4998,7 +4972,7 @@
       <c r="U77" t="s">
         <v>178</v>
       </c>
-      <c r="V77" s="2">
+      <c r="V77" s="1">
         <v>46381</v>
       </c>
     </row>
@@ -5048,7 +5022,7 @@
       <c r="U78" t="s">
         <v>178</v>
       </c>
-      <c r="V78" s="2">
+      <c r="V78" s="1">
         <v>46381</v>
       </c>
     </row>
@@ -5098,7 +5072,7 @@
       <c r="U79" t="s">
         <v>91</v>
       </c>
-      <c r="V79" s="2">
+      <c r="V79" s="1">
         <v>46381</v>
       </c>
     </row>
@@ -5148,7 +5122,7 @@
       <c r="U80" t="s">
         <v>91</v>
       </c>
-      <c r="V80" s="2">
+      <c r="V80" s="1">
         <v>46381</v>
       </c>
     </row>
@@ -5198,7 +5172,7 @@
       <c r="U81" t="s">
         <v>91</v>
       </c>
-      <c r="V81" s="2">
+      <c r="V81" s="1">
         <v>46382</v>
       </c>
     </row>
@@ -5242,7 +5216,7 @@
       <c r="U82" t="s">
         <v>91</v>
       </c>
-      <c r="V82" s="2">
+      <c r="V82" s="1">
         <v>46382</v>
       </c>
     </row>
@@ -5298,7 +5272,7 @@
       <c r="U83" t="s">
         <v>178</v>
       </c>
-      <c r="V83" s="2">
+      <c r="V83" s="1">
         <v>46382</v>
       </c>
     </row>
@@ -5348,7 +5322,7 @@
       <c r="U84" t="s">
         <v>91</v>
       </c>
-      <c r="V84" s="2">
+      <c r="V84" s="1">
         <v>46321</v>
       </c>
     </row>
@@ -5392,7 +5366,7 @@
       <c r="U85" t="s">
         <v>91</v>
       </c>
-      <c r="V85" s="2">
+      <c r="V85" s="1">
         <v>46382</v>
       </c>
     </row>
@@ -5512,7 +5486,7 @@
       <c r="G88" t="s">
         <v>106</v>
       </c>
-      <c r="H88" s="2">
+      <c r="H88" s="1">
         <v>46303</v>
       </c>
       <c r="I88" t="s">
@@ -5542,7 +5516,7 @@
       <c r="U88" t="s">
         <v>91</v>
       </c>
-      <c r="V88" s="2">
+      <c r="V88" s="1">
         <v>46291</v>
       </c>
     </row>
@@ -5589,7 +5563,7 @@
       <c r="U89" t="s">
         <v>91</v>
       </c>
-      <c r="V89" s="2">
+      <c r="V89" s="1">
         <v>46291</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Atualização automática: mta (21/10/2026 12:56)
</commit_message>
<xml_diff>
--- a/Projetos/02_Dados_Tratados/base_mta_tratada.xlsx
+++ b/Projetos/02_Dados_Tratados/base_mta_tratada.xlsx
@@ -14,7 +14,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1206" uniqueCount="179">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1208" uniqueCount="179">
   <si>
     <t>linha</t>
   </si>
@@ -340,10 +340,10 @@
     <t>CANCELADO</t>
   </si>
   <si>
+    <t>PROCESSADO</t>
+  </si>
+  <si>
     <t>ATENDER</t>
-  </si>
-  <si>
-    <t>PROCESSADO</t>
   </si>
   <si>
     <t>C26249</t>
@@ -1601,7 +1601,7 @@
         <v>132</v>
       </c>
       <c r="K14" t="s">
-        <v>108</v>
+        <v>109</v>
       </c>
       <c r="N14" t="s">
         <v>148</v>
@@ -1663,7 +1663,7 @@
         <v>132</v>
       </c>
       <c r="K15" t="s">
-        <v>108</v>
+        <v>109</v>
       </c>
       <c r="N15" t="s">
         <v>148</v>
@@ -1725,7 +1725,7 @@
         <v>132</v>
       </c>
       <c r="K16" t="s">
-        <v>108</v>
+        <v>109</v>
       </c>
       <c r="N16" t="s">
         <v>148</v>
@@ -1787,7 +1787,7 @@
         <v>132</v>
       </c>
       <c r="K17" t="s">
-        <v>108</v>
+        <v>109</v>
       </c>
       <c r="N17" t="s">
         <v>148</v>
@@ -3555,7 +3555,7 @@
         <v>132</v>
       </c>
       <c r="K49" t="s">
-        <v>108</v>
+        <v>109</v>
       </c>
       <c r="N49" t="s">
         <v>148</v>
@@ -3655,7 +3655,7 @@
         <v>60</v>
       </c>
       <c r="D51" t="s">
-        <v>88</v>
+        <v>87</v>
       </c>
       <c r="E51" t="s">
         <v>91</v>
@@ -3664,7 +3664,13 @@
         <v>93</v>
       </c>
       <c r="G51" t="s">
-        <v>108</v>
+        <v>106</v>
+      </c>
+      <c r="H51" s="1">
+        <v>46314</v>
+      </c>
+      <c r="I51" t="s">
+        <v>121</v>
       </c>
       <c r="J51" t="s">
         <v>138</v>
@@ -4585,7 +4591,7 @@
         <v>132</v>
       </c>
       <c r="K69" t="s">
-        <v>108</v>
+        <v>109</v>
       </c>
       <c r="N69" t="s">
         <v>148</v>
@@ -4946,7 +4952,7 @@
         <v>105</v>
       </c>
       <c r="G77" t="s">
-        <v>109</v>
+        <v>108</v>
       </c>
       <c r="N77" t="s">
         <v>152</v>
@@ -4996,7 +5002,7 @@
         <v>105</v>
       </c>
       <c r="G78" t="s">
-        <v>109</v>
+        <v>108</v>
       </c>
       <c r="N78" t="s">
         <v>152</v>
@@ -5046,7 +5052,7 @@
         <v>105</v>
       </c>
       <c r="G79" t="s">
-        <v>109</v>
+        <v>108</v>
       </c>
       <c r="N79" t="s">
         <v>151</v>
@@ -5096,7 +5102,7 @@
         <v>105</v>
       </c>
       <c r="G80" t="s">
-        <v>109</v>
+        <v>108</v>
       </c>
       <c r="N80" t="s">
         <v>151</v>
@@ -5231,7 +5237,7 @@
         <v>84</v>
       </c>
       <c r="D83" t="s">
-        <v>88</v>
+        <v>87</v>
       </c>
       <c r="E83" t="s">
         <v>91</v>
@@ -5240,7 +5246,13 @@
         <v>93</v>
       </c>
       <c r="G83" t="s">
-        <v>108</v>
+        <v>106</v>
+      </c>
+      <c r="H83" s="1">
+        <v>46314</v>
+      </c>
+      <c r="I83" t="s">
+        <v>121</v>
       </c>
       <c r="J83" t="s">
         <v>132</v>
@@ -5296,7 +5308,7 @@
         <v>93</v>
       </c>
       <c r="G84" t="s">
-        <v>108</v>
+        <v>109</v>
       </c>
       <c r="N84" t="s">
         <v>154</v>
@@ -5390,7 +5402,7 @@
         <v>105</v>
       </c>
       <c r="G86" t="s">
-        <v>109</v>
+        <v>108</v>
       </c>
       <c r="N86" t="s">
         <v>83</v>
@@ -5437,7 +5449,7 @@
         <v>105</v>
       </c>
       <c r="G87" t="s">
-        <v>109</v>
+        <v>108</v>
       </c>
       <c r="N87" t="s">
         <v>83</v>
@@ -5537,7 +5549,7 @@
         <v>93</v>
       </c>
       <c r="G89" t="s">
-        <v>108</v>
+        <v>109</v>
       </c>
       <c r="N89" t="s">
         <v>155</v>

</xml_diff>

<commit_message>
Atualização automática: mta (21/10/2026 14:22)
</commit_message>
<xml_diff>
--- a/Projetos/02_Dados_Tratados/base_mta_tratada.xlsx
+++ b/Projetos/02_Dados_Tratados/base_mta_tratada.xlsx
@@ -560,8 +560,16 @@
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="YYYY-MM-DD HH:MM:SS"/>
   </numFmts>
-  <fonts count="1">
+  <fonts count="2">
     <font>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
       <sz val="11"/>
       <color theme="1"/>
       <name val="Calibri"/>
@@ -577,7 +585,7 @@
       <patternFill patternType="gray125"/>
     </fill>
   </fills>
-  <borders count="1">
+  <borders count="2">
     <border>
       <left/>
       <right/>
@@ -585,12 +593,30 @@
       <bottom/>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin">
+        <color auto="1"/>
+      </left>
+      <right style="thin">
+        <color auto="1"/>
+      </right>
+      <top style="thin">
+        <color auto="1"/>
+      </top>
+      <bottom style="thin">
+        <color auto="1"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="3">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
   </cellXfs>
   <cellStyles count="1">
@@ -890,70 +916,70 @@
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:22">
-      <c r="A1" t="s">
+      <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
-      <c r="B1" t="s">
+      <c r="B1" s="1" t="s">
         <v>1</v>
       </c>
-      <c r="C1" t="s">
+      <c r="C1" s="1" t="s">
         <v>2</v>
       </c>
-      <c r="D1" t="s">
+      <c r="D1" s="1" t="s">
         <v>3</v>
       </c>
-      <c r="E1" t="s">
+      <c r="E1" s="1" t="s">
         <v>4</v>
       </c>
-      <c r="F1" t="s">
+      <c r="F1" s="1" t="s">
         <v>5</v>
       </c>
-      <c r="G1" t="s">
+      <c r="G1" s="1" t="s">
         <v>6</v>
       </c>
-      <c r="H1" t="s">
+      <c r="H1" s="1" t="s">
         <v>7</v>
       </c>
-      <c r="I1" t="s">
+      <c r="I1" s="1" t="s">
         <v>8</v>
       </c>
-      <c r="J1" t="s">
+      <c r="J1" s="1" t="s">
         <v>9</v>
       </c>
-      <c r="K1" t="s">
+      <c r="K1" s="1" t="s">
         <v>10</v>
       </c>
-      <c r="L1" t="s">
+      <c r="L1" s="1" t="s">
         <v>11</v>
       </c>
-      <c r="M1" t="s">
+      <c r="M1" s="1" t="s">
         <v>12</v>
       </c>
-      <c r="N1" t="s">
+      <c r="N1" s="1" t="s">
         <v>13</v>
       </c>
-      <c r="O1" t="s">
+      <c r="O1" s="1" t="s">
         <v>14</v>
       </c>
-      <c r="P1" t="s">
+      <c r="P1" s="1" t="s">
         <v>15</v>
       </c>
-      <c r="Q1" t="s">
+      <c r="Q1" s="1" t="s">
         <v>16</v>
       </c>
-      <c r="R1" t="s">
+      <c r="R1" s="1" t="s">
         <v>17</v>
       </c>
-      <c r="S1" t="s">
+      <c r="S1" s="1" t="s">
         <v>18</v>
       </c>
-      <c r="T1" t="s">
+      <c r="T1" s="1" t="s">
         <v>19</v>
       </c>
-      <c r="U1" t="s">
+      <c r="U1" s="1" t="s">
         <v>20</v>
       </c>
-      <c r="V1" t="s">
+      <c r="V1" s="1" t="s">
         <v>21</v>
       </c>
     </row>
@@ -979,7 +1005,7 @@
       <c r="G2" t="s">
         <v>106</v>
       </c>
-      <c r="H2" s="1">
+      <c r="H2" s="2">
         <v>46303</v>
       </c>
       <c r="I2" t="s">
@@ -1018,7 +1044,7 @@
       <c r="U2" t="s">
         <v>178</v>
       </c>
-      <c r="V2" s="1">
+      <c r="V2" s="2">
         <v>46229</v>
       </c>
     </row>
@@ -1065,7 +1091,7 @@
       <c r="U3" t="s">
         <v>91</v>
       </c>
-      <c r="V3" s="1">
+      <c r="V3" s="2">
         <v>46291</v>
       </c>
     </row>
@@ -1112,7 +1138,7 @@
       <c r="U4" t="s">
         <v>91</v>
       </c>
-      <c r="V4" s="1">
+      <c r="V4" s="2">
         <v>46321</v>
       </c>
     </row>
@@ -1159,7 +1185,7 @@
       <c r="U5" t="s">
         <v>91</v>
       </c>
-      <c r="V5" s="1">
+      <c r="V5" s="2">
         <v>46321</v>
       </c>
     </row>
@@ -1209,7 +1235,7 @@
       <c r="U6" t="s">
         <v>91</v>
       </c>
-      <c r="V6" s="1">
+      <c r="V6" s="2">
         <v>46291</v>
       </c>
     </row>
@@ -1235,7 +1261,7 @@
       <c r="G7" t="s">
         <v>106</v>
       </c>
-      <c r="H7" s="1">
+      <c r="H7" s="2">
         <v>46121</v>
       </c>
       <c r="I7" t="s">
@@ -1265,7 +1291,7 @@
       <c r="U7" t="s">
         <v>91</v>
       </c>
-      <c r="V7" s="1">
+      <c r="V7" s="2">
         <v>46138</v>
       </c>
     </row>
@@ -1312,7 +1338,7 @@
       <c r="U8" t="s">
         <v>91</v>
       </c>
-      <c r="V8" s="1">
+      <c r="V8" s="2">
         <v>46291</v>
       </c>
     </row>
@@ -1359,7 +1385,7 @@
       <c r="U9" t="s">
         <v>91</v>
       </c>
-      <c r="V9" s="1">
+      <c r="V9" s="2">
         <v>46291</v>
       </c>
     </row>
@@ -1382,7 +1408,7 @@
       <c r="G10" t="s">
         <v>106</v>
       </c>
-      <c r="H10" s="1">
+      <c r="H10" s="2">
         <v>46303</v>
       </c>
       <c r="I10" t="s">
@@ -1412,7 +1438,7 @@
       <c r="U10" t="s">
         <v>91</v>
       </c>
-      <c r="V10" s="1">
+      <c r="V10" s="2">
         <v>46291</v>
       </c>
     </row>
@@ -1459,7 +1485,7 @@
       <c r="U11" t="s">
         <v>91</v>
       </c>
-      <c r="V11" s="1">
+      <c r="V11" s="2">
         <v>46291</v>
       </c>
     </row>
@@ -1506,7 +1532,7 @@
       <c r="U12" t="s">
         <v>91</v>
       </c>
-      <c r="V12" s="1">
+      <c r="V12" s="2">
         <v>46291</v>
       </c>
     </row>
@@ -1532,7 +1558,7 @@
       <c r="G13" t="s">
         <v>106</v>
       </c>
-      <c r="H13" s="1">
+      <c r="H13" s="2">
         <v>46079</v>
       </c>
       <c r="I13" t="s">
@@ -1565,7 +1591,7 @@
       <c r="U13" t="s">
         <v>178</v>
       </c>
-      <c r="V13" s="1">
+      <c r="V13" s="2">
         <v>46079</v>
       </c>
     </row>
@@ -1591,7 +1617,7 @@
       <c r="G14" t="s">
         <v>106</v>
       </c>
-      <c r="H14" s="1">
+      <c r="H14" s="2">
         <v>46303</v>
       </c>
       <c r="I14" t="s">
@@ -1627,7 +1653,7 @@
       <c r="U14" t="s">
         <v>178</v>
       </c>
-      <c r="V14" s="1">
+      <c r="V14" s="2">
         <v>46352</v>
       </c>
     </row>
@@ -1653,7 +1679,7 @@
       <c r="G15" t="s">
         <v>106</v>
       </c>
-      <c r="H15" s="1">
+      <c r="H15" s="2">
         <v>46303</v>
       </c>
       <c r="I15" t="s">
@@ -1689,7 +1715,7 @@
       <c r="U15" t="s">
         <v>178</v>
       </c>
-      <c r="V15" s="1">
+      <c r="V15" s="2">
         <v>46352</v>
       </c>
     </row>
@@ -1715,7 +1741,7 @@
       <c r="G16" t="s">
         <v>106</v>
       </c>
-      <c r="H16" s="1">
+      <c r="H16" s="2">
         <v>46303</v>
       </c>
       <c r="I16" t="s">
@@ -1751,7 +1777,7 @@
       <c r="U16" t="s">
         <v>178</v>
       </c>
-      <c r="V16" s="1">
+      <c r="V16" s="2">
         <v>46352</v>
       </c>
     </row>
@@ -1777,7 +1803,7 @@
       <c r="G17" t="s">
         <v>106</v>
       </c>
-      <c r="H17" s="1">
+      <c r="H17" s="2">
         <v>46303</v>
       </c>
       <c r="I17" t="s">
@@ -1813,7 +1839,7 @@
       <c r="U17" t="s">
         <v>178</v>
       </c>
-      <c r="V17" s="1">
+      <c r="V17" s="2">
         <v>46229</v>
       </c>
     </row>
@@ -1839,7 +1865,7 @@
       <c r="G18" t="s">
         <v>106</v>
       </c>
-      <c r="H18" s="1">
+      <c r="H18" s="2">
         <v>46098</v>
       </c>
       <c r="I18" t="s">
@@ -1872,7 +1898,7 @@
       <c r="U18" t="s">
         <v>178</v>
       </c>
-      <c r="V18" s="1">
+      <c r="V18" s="2">
         <v>46107</v>
       </c>
     </row>
@@ -1898,7 +1924,7 @@
       <c r="G19" t="s">
         <v>106</v>
       </c>
-      <c r="H19" s="1">
+      <c r="H19" s="2">
         <v>46076</v>
       </c>
       <c r="I19" t="s">
@@ -1928,7 +1954,7 @@
       <c r="U19" t="s">
         <v>91</v>
       </c>
-      <c r="V19" s="1">
+      <c r="V19" s="2">
         <v>46079</v>
       </c>
     </row>
@@ -1954,7 +1980,7 @@
       <c r="G20" t="s">
         <v>106</v>
       </c>
-      <c r="H20" s="1">
+      <c r="H20" s="2">
         <v>46076</v>
       </c>
       <c r="I20" t="s">
@@ -1984,7 +2010,7 @@
       <c r="U20" t="s">
         <v>91</v>
       </c>
-      <c r="V20" s="1">
+      <c r="V20" s="2">
         <v>46079</v>
       </c>
     </row>
@@ -2031,7 +2057,7 @@
       <c r="U21" t="s">
         <v>91</v>
       </c>
-      <c r="V21" s="1">
+      <c r="V21" s="2">
         <v>46321</v>
       </c>
     </row>
@@ -2078,7 +2104,7 @@
       <c r="U22" t="s">
         <v>91</v>
       </c>
-      <c r="V22" s="1">
+      <c r="V22" s="2">
         <v>46321</v>
       </c>
     </row>
@@ -2125,7 +2151,7 @@
       <c r="U23" t="s">
         <v>91</v>
       </c>
-      <c r="V23" s="1">
+      <c r="V23" s="2">
         <v>46321</v>
       </c>
     </row>
@@ -2172,7 +2198,7 @@
       <c r="U24" t="s">
         <v>91</v>
       </c>
-      <c r="V24" s="1">
+      <c r="V24" s="2">
         <v>46321</v>
       </c>
     </row>
@@ -2198,7 +2224,7 @@
       <c r="G25" t="s">
         <v>106</v>
       </c>
-      <c r="H25" s="1">
+      <c r="H25" s="2">
         <v>46119</v>
       </c>
       <c r="I25" t="s">
@@ -2231,7 +2257,7 @@
       <c r="U25" t="s">
         <v>178</v>
       </c>
-      <c r="V25" s="1">
+      <c r="V25" s="2">
         <v>46138</v>
       </c>
     </row>
@@ -2257,7 +2283,7 @@
       <c r="G26" t="s">
         <v>106</v>
       </c>
-      <c r="H26" s="1">
+      <c r="H26" s="2">
         <v>46121</v>
       </c>
       <c r="I26" t="s">
@@ -2287,7 +2313,7 @@
       <c r="U26" t="s">
         <v>91</v>
       </c>
-      <c r="V26" s="1">
+      <c r="V26" s="2">
         <v>46138</v>
       </c>
     </row>
@@ -2313,7 +2339,7 @@
       <c r="G27" t="s">
         <v>106</v>
       </c>
-      <c r="H27" s="1">
+      <c r="H27" s="2">
         <v>46076</v>
       </c>
       <c r="I27" t="s">
@@ -2343,7 +2369,7 @@
       <c r="U27" t="s">
         <v>91</v>
       </c>
-      <c r="V27" s="1">
+      <c r="V27" s="2">
         <v>46079</v>
       </c>
     </row>
@@ -2369,7 +2395,7 @@
       <c r="G28" t="s">
         <v>106</v>
       </c>
-      <c r="H28" s="1">
+      <c r="H28" s="2">
         <v>46303</v>
       </c>
       <c r="I28" t="s">
@@ -2405,7 +2431,7 @@
       <c r="U28" t="s">
         <v>178</v>
       </c>
-      <c r="V28" s="1">
+      <c r="V28" s="2">
         <v>46291</v>
       </c>
     </row>
@@ -2431,7 +2457,7 @@
       <c r="G29" t="s">
         <v>106</v>
       </c>
-      <c r="H29" s="1">
+      <c r="H29" s="2">
         <v>46199</v>
       </c>
       <c r="I29" t="s">
@@ -2464,7 +2490,7 @@
       <c r="U29" t="s">
         <v>178</v>
       </c>
-      <c r="V29" s="1">
+      <c r="V29" s="2">
         <v>46199</v>
       </c>
     </row>
@@ -2490,7 +2516,7 @@
       <c r="G30" t="s">
         <v>106</v>
       </c>
-      <c r="H30" s="1">
+      <c r="H30" s="2">
         <v>46199</v>
       </c>
       <c r="I30" t="s">
@@ -2523,7 +2549,7 @@
       <c r="U30" t="s">
         <v>178</v>
       </c>
-      <c r="V30" s="1">
+      <c r="V30" s="2">
         <v>46199</v>
       </c>
     </row>
@@ -2549,7 +2575,7 @@
       <c r="G31" t="s">
         <v>106</v>
       </c>
-      <c r="H31" s="1">
+      <c r="H31" s="2">
         <v>46199</v>
       </c>
       <c r="I31" t="s">
@@ -2582,7 +2608,7 @@
       <c r="U31" t="s">
         <v>178</v>
       </c>
-      <c r="V31" s="1">
+      <c r="V31" s="2">
         <v>46199</v>
       </c>
     </row>
@@ -2608,7 +2634,7 @@
       <c r="G32" t="s">
         <v>106</v>
       </c>
-      <c r="H32" s="1">
+      <c r="H32" s="2">
         <v>46199</v>
       </c>
       <c r="I32" t="s">
@@ -2641,7 +2667,7 @@
       <c r="U32" t="s">
         <v>178</v>
       </c>
-      <c r="V32" s="1">
+      <c r="V32" s="2">
         <v>46199</v>
       </c>
     </row>
@@ -2694,7 +2720,7 @@
       <c r="U33" t="s">
         <v>178</v>
       </c>
-      <c r="V33" s="1">
+      <c r="V33" s="2">
         <v>46291</v>
       </c>
     </row>
@@ -2720,7 +2746,7 @@
       <c r="G34" t="s">
         <v>106</v>
       </c>
-      <c r="H34" s="1">
+      <c r="H34" s="2">
         <v>46191</v>
       </c>
       <c r="I34" t="s">
@@ -2753,7 +2779,7 @@
       <c r="U34" t="s">
         <v>178</v>
       </c>
-      <c r="V34" s="1">
+      <c r="V34" s="2">
         <v>46199</v>
       </c>
     </row>
@@ -2779,7 +2805,7 @@
       <c r="G35" t="s">
         <v>106</v>
       </c>
-      <c r="H35" s="1">
+      <c r="H35" s="2">
         <v>46119</v>
       </c>
       <c r="I35" t="s">
@@ -2809,7 +2835,7 @@
       <c r="U35" t="s">
         <v>178</v>
       </c>
-      <c r="V35" s="1">
+      <c r="V35" s="2">
         <v>46138</v>
       </c>
     </row>
@@ -2835,7 +2861,7 @@
       <c r="G36" t="s">
         <v>106</v>
       </c>
-      <c r="H36" s="1">
+      <c r="H36" s="2">
         <v>46213</v>
       </c>
       <c r="I36" t="s">
@@ -2865,7 +2891,7 @@
       <c r="U36" t="s">
         <v>91</v>
       </c>
-      <c r="V36" s="1">
+      <c r="V36" s="2">
         <v>46229</v>
       </c>
     </row>
@@ -2891,7 +2917,7 @@
       <c r="G37" t="s">
         <v>106</v>
       </c>
-      <c r="H37" s="1">
+      <c r="H37" s="2">
         <v>46175</v>
       </c>
       <c r="I37" t="s">
@@ -2921,7 +2947,7 @@
       <c r="U37" t="s">
         <v>91</v>
       </c>
-      <c r="V37" s="1">
+      <c r="V37" s="2">
         <v>46199</v>
       </c>
     </row>
@@ -2947,7 +2973,7 @@
       <c r="G38" t="s">
         <v>106</v>
       </c>
-      <c r="H38" s="1">
+      <c r="H38" s="2">
         <v>46213</v>
       </c>
       <c r="I38" t="s">
@@ -2977,7 +3003,7 @@
       <c r="U38" t="s">
         <v>91</v>
       </c>
-      <c r="V38" s="1">
+      <c r="V38" s="2">
         <v>46229</v>
       </c>
     </row>
@@ -3003,7 +3029,7 @@
       <c r="G39" t="s">
         <v>106</v>
       </c>
-      <c r="H39" s="1">
+      <c r="H39" s="2">
         <v>46199</v>
       </c>
       <c r="I39" t="s">
@@ -3033,7 +3059,7 @@
       <c r="U39" t="s">
         <v>91</v>
       </c>
-      <c r="V39" s="1">
+      <c r="V39" s="2">
         <v>46199</v>
       </c>
     </row>
@@ -3059,7 +3085,7 @@
       <c r="G40" t="s">
         <v>106</v>
       </c>
-      <c r="H40" s="1">
+      <c r="H40" s="2">
         <v>46199</v>
       </c>
       <c r="I40" t="s">
@@ -3089,7 +3115,7 @@
       <c r="U40" t="s">
         <v>91</v>
       </c>
-      <c r="V40" s="1">
+      <c r="V40" s="2">
         <v>46199</v>
       </c>
     </row>
@@ -3115,7 +3141,7 @@
       <c r="G41" t="s">
         <v>106</v>
       </c>
-      <c r="H41" s="1">
+      <c r="H41" s="2">
         <v>46204</v>
       </c>
       <c r="I41" t="s">
@@ -3145,7 +3171,7 @@
       <c r="U41" t="s">
         <v>91</v>
       </c>
-      <c r="V41" s="1">
+      <c r="V41" s="2">
         <v>46229</v>
       </c>
     </row>
@@ -3171,7 +3197,7 @@
       <c r="G42" t="s">
         <v>106</v>
       </c>
-      <c r="H42" s="1">
+      <c r="H42" s="2">
         <v>46244</v>
       </c>
       <c r="I42" t="s">
@@ -3201,7 +3227,7 @@
       <c r="U42" t="s">
         <v>91</v>
       </c>
-      <c r="V42" s="1">
+      <c r="V42" s="2">
         <v>46199</v>
       </c>
     </row>
@@ -3245,7 +3271,7 @@
       <c r="U43" t="s">
         <v>91</v>
       </c>
-      <c r="V43" s="1">
+      <c r="V43" s="2">
         <v>46260</v>
       </c>
     </row>
@@ -3271,7 +3297,7 @@
       <c r="G44" t="s">
         <v>106</v>
       </c>
-      <c r="H44" s="1">
+      <c r="H44" s="2">
         <v>46191</v>
       </c>
       <c r="I44" t="s">
@@ -3301,7 +3327,7 @@
       <c r="U44" t="s">
         <v>91</v>
       </c>
-      <c r="V44" s="1">
+      <c r="V44" s="2">
         <v>46199</v>
       </c>
     </row>
@@ -3327,7 +3353,7 @@
       <c r="G45" t="s">
         <v>106</v>
       </c>
-      <c r="H45" s="1">
+      <c r="H45" s="2">
         <v>46191</v>
       </c>
       <c r="I45" t="s">
@@ -3357,7 +3383,7 @@
       <c r="U45" t="s">
         <v>91</v>
       </c>
-      <c r="V45" s="1">
+      <c r="V45" s="2">
         <v>46199</v>
       </c>
     </row>
@@ -3383,7 +3409,7 @@
       <c r="G46" t="s">
         <v>106</v>
       </c>
-      <c r="H46" s="1">
+      <c r="H46" s="2">
         <v>46213</v>
       </c>
       <c r="I46" t="s">
@@ -3416,7 +3442,7 @@
       <c r="U46" t="s">
         <v>178</v>
       </c>
-      <c r="V46" s="1">
+      <c r="V46" s="2">
         <v>46229</v>
       </c>
     </row>
@@ -3442,7 +3468,7 @@
       <c r="G47" t="s">
         <v>106</v>
       </c>
-      <c r="H47" s="1">
+      <c r="H47" s="2">
         <v>46210</v>
       </c>
       <c r="I47" t="s">
@@ -3472,7 +3498,7 @@
       <c r="U47" t="s">
         <v>178</v>
       </c>
-      <c r="V47" s="1">
+      <c r="V47" s="2">
         <v>46229</v>
       </c>
     </row>
@@ -3519,7 +3545,7 @@
       <c r="U48" t="s">
         <v>91</v>
       </c>
-      <c r="V48" s="1">
+      <c r="V48" s="2">
         <v>46321</v>
       </c>
     </row>
@@ -3545,7 +3571,7 @@
       <c r="G49" t="s">
         <v>106</v>
       </c>
-      <c r="H49" s="1">
+      <c r="H49" s="2">
         <v>46303</v>
       </c>
       <c r="I49" t="s">
@@ -3581,7 +3607,7 @@
       <c r="U49" t="s">
         <v>178</v>
       </c>
-      <c r="V49" s="1">
+      <c r="V49" s="2">
         <v>46291</v>
       </c>
     </row>
@@ -3607,7 +3633,7 @@
       <c r="G50" t="s">
         <v>106</v>
       </c>
-      <c r="H50" s="1">
+      <c r="H50" s="2">
         <v>46176</v>
       </c>
       <c r="I50" t="s">
@@ -3640,7 +3666,7 @@
       <c r="U50" t="s">
         <v>178</v>
       </c>
-      <c r="V50" s="1">
+      <c r="V50" s="2">
         <v>46199</v>
       </c>
     </row>
@@ -3666,7 +3692,7 @@
       <c r="G51" t="s">
         <v>106</v>
       </c>
-      <c r="H51" s="1">
+      <c r="H51" s="2">
         <v>46314</v>
       </c>
       <c r="I51" t="s">
@@ -3702,7 +3728,7 @@
       <c r="U51" t="s">
         <v>178</v>
       </c>
-      <c r="V51" s="1">
+      <c r="V51" s="2">
         <v>46260</v>
       </c>
     </row>
@@ -3728,7 +3754,7 @@
       <c r="G52" t="s">
         <v>106</v>
       </c>
-      <c r="H52" s="1">
+      <c r="H52" s="2">
         <v>46295</v>
       </c>
       <c r="I52" t="s">
@@ -3764,7 +3790,7 @@
       <c r="U52" t="s">
         <v>178</v>
       </c>
-      <c r="V52" s="1">
+      <c r="V52" s="2">
         <v>46291</v>
       </c>
     </row>
@@ -3817,7 +3843,7 @@
       <c r="U53" t="s">
         <v>178</v>
       </c>
-      <c r="V53" s="1">
+      <c r="V53" s="2">
         <v>46321</v>
       </c>
     </row>
@@ -3843,7 +3869,7 @@
       <c r="G54" t="s">
         <v>106</v>
       </c>
-      <c r="H54" s="1">
+      <c r="H54" s="2">
         <v>46227</v>
       </c>
       <c r="I54" t="s">
@@ -3873,7 +3899,7 @@
       <c r="U54" t="s">
         <v>178</v>
       </c>
-      <c r="V54" s="1">
+      <c r="V54" s="2">
         <v>46229</v>
       </c>
     </row>
@@ -3896,7 +3922,7 @@
       <c r="G55" t="s">
         <v>106</v>
       </c>
-      <c r="H55" s="1">
+      <c r="H55" s="2">
         <v>46280</v>
       </c>
       <c r="I55" t="s">
@@ -3926,7 +3952,7 @@
       <c r="U55" t="s">
         <v>178</v>
       </c>
-      <c r="V55" s="1">
+      <c r="V55" s="2">
         <v>46291</v>
       </c>
     </row>
@@ -3949,7 +3975,7 @@
       <c r="G56" t="s">
         <v>106</v>
       </c>
-      <c r="H56" s="1">
+      <c r="H56" s="2">
         <v>46280</v>
       </c>
       <c r="I56" t="s">
@@ -3979,7 +4005,7 @@
       <c r="U56" t="s">
         <v>178</v>
       </c>
-      <c r="V56" s="1">
+      <c r="V56" s="2">
         <v>46260</v>
       </c>
     </row>
@@ -4002,7 +4028,7 @@
       <c r="G57" t="s">
         <v>106</v>
       </c>
-      <c r="H57" s="1">
+      <c r="H57" s="2">
         <v>46295</v>
       </c>
       <c r="I57" t="s">
@@ -4032,7 +4058,7 @@
       <c r="U57" t="s">
         <v>178</v>
       </c>
-      <c r="V57" s="1">
+      <c r="V57" s="2">
         <v>46291</v>
       </c>
     </row>
@@ -4055,7 +4081,7 @@
       <c r="G58" t="s">
         <v>106</v>
       </c>
-      <c r="H58" s="1">
+      <c r="H58" s="2">
         <v>46295</v>
       </c>
       <c r="I58" t="s">
@@ -4085,7 +4111,7 @@
       <c r="U58" t="s">
         <v>178</v>
       </c>
-      <c r="V58" s="1">
+      <c r="V58" s="2">
         <v>46291</v>
       </c>
     </row>
@@ -4108,7 +4134,7 @@
       <c r="G59" t="s">
         <v>106</v>
       </c>
-      <c r="H59" s="1">
+      <c r="H59" s="2">
         <v>46304</v>
       </c>
       <c r="I59" t="s">
@@ -4138,7 +4164,7 @@
       <c r="U59" t="s">
         <v>178</v>
       </c>
-      <c r="V59" s="1">
+      <c r="V59" s="2">
         <v>46321</v>
       </c>
     </row>
@@ -4164,7 +4190,7 @@
       <c r="G60" t="s">
         <v>106</v>
       </c>
-      <c r="H60" s="1">
+      <c r="H60" s="2">
         <v>46301</v>
       </c>
       <c r="I60" t="s">
@@ -4200,7 +4226,7 @@
       <c r="U60" t="s">
         <v>178</v>
       </c>
-      <c r="V60" s="1">
+      <c r="V60" s="2">
         <v>46352</v>
       </c>
     </row>
@@ -4244,7 +4270,7 @@
       <c r="U61" t="s">
         <v>178</v>
       </c>
-      <c r="V61" s="1">
+      <c r="V61" s="2">
         <v>46107</v>
       </c>
     </row>
@@ -4288,7 +4314,7 @@
       <c r="U62" t="s">
         <v>178</v>
       </c>
-      <c r="V62" s="1">
+      <c r="V62" s="2">
         <v>46107</v>
       </c>
     </row>
@@ -4332,7 +4358,7 @@
       <c r="U63" t="s">
         <v>178</v>
       </c>
-      <c r="V63" s="1">
+      <c r="V63" s="2">
         <v>46107</v>
       </c>
     </row>
@@ -4376,7 +4402,7 @@
       <c r="U64" t="s">
         <v>178</v>
       </c>
-      <c r="V64" s="1">
+      <c r="V64" s="2">
         <v>46107</v>
       </c>
     </row>
@@ -4420,7 +4446,7 @@
       <c r="U65" t="s">
         <v>178</v>
       </c>
-      <c r="V65" s="1">
+      <c r="V65" s="2">
         <v>46107</v>
       </c>
     </row>
@@ -4464,7 +4490,7 @@
       <c r="U66" t="s">
         <v>178</v>
       </c>
-      <c r="V66" s="1">
+      <c r="V66" s="2">
         <v>46107</v>
       </c>
     </row>
@@ -4508,7 +4534,7 @@
       <c r="U67" t="s">
         <v>91</v>
       </c>
-      <c r="V67" s="1">
+      <c r="V67" s="2">
         <v>46168</v>
       </c>
     </row>
@@ -4555,7 +4581,7 @@
       <c r="U68" t="s">
         <v>91</v>
       </c>
-      <c r="V68" s="1">
+      <c r="V68" s="2">
         <v>46291</v>
       </c>
     </row>
@@ -4581,7 +4607,7 @@
       <c r="G69" t="s">
         <v>106</v>
       </c>
-      <c r="H69" s="1">
+      <c r="H69" s="2">
         <v>46303</v>
       </c>
       <c r="I69" t="s">
@@ -4617,7 +4643,7 @@
       <c r="U69" t="s">
         <v>178</v>
       </c>
-      <c r="V69" s="1">
+      <c r="V69" s="2">
         <v>46229</v>
       </c>
     </row>
@@ -4661,7 +4687,7 @@
       <c r="U70" t="s">
         <v>91</v>
       </c>
-      <c r="V70" s="1">
+      <c r="V70" s="2">
         <v>46260</v>
       </c>
     </row>
@@ -4705,7 +4731,7 @@
       <c r="U71" t="s">
         <v>178</v>
       </c>
-      <c r="V71" s="1">
+      <c r="V71" s="2">
         <v>46291</v>
       </c>
     </row>
@@ -4749,7 +4775,7 @@
       <c r="U72" t="s">
         <v>178</v>
       </c>
-      <c r="V72" s="1">
+      <c r="V72" s="2">
         <v>46168</v>
       </c>
     </row>
@@ -4793,7 +4819,7 @@
       <c r="U73" t="s">
         <v>178</v>
       </c>
-      <c r="V73" s="1">
+      <c r="V73" s="2">
         <v>46291</v>
       </c>
     </row>
@@ -4837,7 +4863,7 @@
       <c r="U74" t="s">
         <v>178</v>
       </c>
-      <c r="V74" s="1">
+      <c r="V74" s="2">
         <v>46291</v>
       </c>
     </row>
@@ -4881,7 +4907,7 @@
       <c r="U75" t="s">
         <v>178</v>
       </c>
-      <c r="V75" s="1">
+      <c r="V75" s="2">
         <v>46291</v>
       </c>
     </row>
@@ -4928,7 +4954,7 @@
       <c r="U76" t="s">
         <v>91</v>
       </c>
-      <c r="V76" s="1">
+      <c r="V76" s="2">
         <v>46321</v>
       </c>
     </row>
@@ -4978,7 +5004,7 @@
       <c r="U77" t="s">
         <v>178</v>
       </c>
-      <c r="V77" s="1">
+      <c r="V77" s="2">
         <v>46381</v>
       </c>
     </row>
@@ -5028,7 +5054,7 @@
       <c r="U78" t="s">
         <v>178</v>
       </c>
-      <c r="V78" s="1">
+      <c r="V78" s="2">
         <v>46381</v>
       </c>
     </row>
@@ -5078,7 +5104,7 @@
       <c r="U79" t="s">
         <v>91</v>
       </c>
-      <c r="V79" s="1">
+      <c r="V79" s="2">
         <v>46381</v>
       </c>
     </row>
@@ -5128,7 +5154,7 @@
       <c r="U80" t="s">
         <v>91</v>
       </c>
-      <c r="V80" s="1">
+      <c r="V80" s="2">
         <v>46381</v>
       </c>
     </row>
@@ -5178,7 +5204,7 @@
       <c r="U81" t="s">
         <v>91</v>
       </c>
-      <c r="V81" s="1">
+      <c r="V81" s="2">
         <v>46382</v>
       </c>
     </row>
@@ -5222,7 +5248,7 @@
       <c r="U82" t="s">
         <v>91</v>
       </c>
-      <c r="V82" s="1">
+      <c r="V82" s="2">
         <v>46382</v>
       </c>
     </row>
@@ -5248,7 +5274,7 @@
       <c r="G83" t="s">
         <v>106</v>
       </c>
-      <c r="H83" s="1">
+      <c r="H83" s="2">
         <v>46314</v>
       </c>
       <c r="I83" t="s">
@@ -5284,7 +5310,7 @@
       <c r="U83" t="s">
         <v>178</v>
       </c>
-      <c r="V83" s="1">
+      <c r="V83" s="2">
         <v>46382</v>
       </c>
     </row>
@@ -5334,7 +5360,7 @@
       <c r="U84" t="s">
         <v>91</v>
       </c>
-      <c r="V84" s="1">
+      <c r="V84" s="2">
         <v>46321</v>
       </c>
     </row>
@@ -5378,7 +5404,7 @@
       <c r="U85" t="s">
         <v>91</v>
       </c>
-      <c r="V85" s="1">
+      <c r="V85" s="2">
         <v>46382</v>
       </c>
     </row>
@@ -5498,7 +5524,7 @@
       <c r="G88" t="s">
         <v>106</v>
       </c>
-      <c r="H88" s="1">
+      <c r="H88" s="2">
         <v>46303</v>
       </c>
       <c r="I88" t="s">
@@ -5528,7 +5554,7 @@
       <c r="U88" t="s">
         <v>91</v>
       </c>
-      <c r="V88" s="1">
+      <c r="V88" s="2">
         <v>46291</v>
       </c>
     </row>
@@ -5575,7 +5601,7 @@
       <c r="U89" t="s">
         <v>91</v>
       </c>
-      <c r="V89" s="1">
+      <c r="V89" s="2">
         <v>46291</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Atualização automática: mta (22/10/2026 12:52)
</commit_message>
<xml_diff>
--- a/Projetos/02_Dados_Tratados/base_mta_tratada.xlsx
+++ b/Projetos/02_Dados_Tratados/base_mta_tratada.xlsx
@@ -560,16 +560,8 @@
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="YYYY-MM-DD HH:MM:SS"/>
   </numFmts>
-  <fonts count="2">
+  <fonts count="1">
     <font>
-      <sz val="11"/>
-      <color theme="1"/>
-      <name val="Calibri"/>
-      <family val="2"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <b/>
       <sz val="11"/>
       <color theme="1"/>
       <name val="Calibri"/>
@@ -585,7 +577,7 @@
       <patternFill patternType="gray125"/>
     </fill>
   </fills>
-  <borders count="2">
+  <borders count="1">
     <border>
       <left/>
       <right/>
@@ -593,30 +585,12 @@
       <bottom/>
       <diagonal/>
     </border>
-    <border>
-      <left style="thin">
-        <color auto="1"/>
-      </left>
-      <right style="thin">
-        <color auto="1"/>
-      </right>
-      <top style="thin">
-        <color auto="1"/>
-      </top>
-      <bottom style="thin">
-        <color auto="1"/>
-      </bottom>
-      <diagonal/>
-    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="3">
+  <cellXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top"/>
-    </xf>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
   </cellXfs>
   <cellStyles count="1">
@@ -916,70 +890,70 @@
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:22">
-      <c r="A1" s="1" t="s">
+      <c r="A1" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="1" t="s">
+      <c r="B1" t="s">
         <v>1</v>
       </c>
-      <c r="C1" s="1" t="s">
+      <c r="C1" t="s">
         <v>2</v>
       </c>
-      <c r="D1" s="1" t="s">
+      <c r="D1" t="s">
         <v>3</v>
       </c>
-      <c r="E1" s="1" t="s">
+      <c r="E1" t="s">
         <v>4</v>
       </c>
-      <c r="F1" s="1" t="s">
+      <c r="F1" t="s">
         <v>5</v>
       </c>
-      <c r="G1" s="1" t="s">
+      <c r="G1" t="s">
         <v>6</v>
       </c>
-      <c r="H1" s="1" t="s">
+      <c r="H1" t="s">
         <v>7</v>
       </c>
-      <c r="I1" s="1" t="s">
+      <c r="I1" t="s">
         <v>8</v>
       </c>
-      <c r="J1" s="1" t="s">
+      <c r="J1" t="s">
         <v>9</v>
       </c>
-      <c r="K1" s="1" t="s">
+      <c r="K1" t="s">
         <v>10</v>
       </c>
-      <c r="L1" s="1" t="s">
+      <c r="L1" t="s">
         <v>11</v>
       </c>
-      <c r="M1" s="1" t="s">
+      <c r="M1" t="s">
         <v>12</v>
       </c>
-      <c r="N1" s="1" t="s">
+      <c r="N1" t="s">
         <v>13</v>
       </c>
-      <c r="O1" s="1" t="s">
+      <c r="O1" t="s">
         <v>14</v>
       </c>
-      <c r="P1" s="1" t="s">
+      <c r="P1" t="s">
         <v>15</v>
       </c>
-      <c r="Q1" s="1" t="s">
+      <c r="Q1" t="s">
         <v>16</v>
       </c>
-      <c r="R1" s="1" t="s">
+      <c r="R1" t="s">
         <v>17</v>
       </c>
-      <c r="S1" s="1" t="s">
+      <c r="S1" t="s">
         <v>18</v>
       </c>
-      <c r="T1" s="1" t="s">
+      <c r="T1" t="s">
         <v>19</v>
       </c>
-      <c r="U1" s="1" t="s">
+      <c r="U1" t="s">
         <v>20</v>
       </c>
-      <c r="V1" s="1" t="s">
+      <c r="V1" t="s">
         <v>21</v>
       </c>
     </row>
@@ -1005,7 +979,7 @@
       <c r="G2" t="s">
         <v>106</v>
       </c>
-      <c r="H2" s="2">
+      <c r="H2" s="1">
         <v>46303</v>
       </c>
       <c r="I2" t="s">
@@ -1044,7 +1018,7 @@
       <c r="U2" t="s">
         <v>178</v>
       </c>
-      <c r="V2" s="2">
+      <c r="V2" s="1">
         <v>46229</v>
       </c>
     </row>
@@ -1091,7 +1065,7 @@
       <c r="U3" t="s">
         <v>91</v>
       </c>
-      <c r="V3" s="2">
+      <c r="V3" s="1">
         <v>46291</v>
       </c>
     </row>
@@ -1138,7 +1112,7 @@
       <c r="U4" t="s">
         <v>91</v>
       </c>
-      <c r="V4" s="2">
+      <c r="V4" s="1">
         <v>46321</v>
       </c>
     </row>
@@ -1185,7 +1159,7 @@
       <c r="U5" t="s">
         <v>91</v>
       </c>
-      <c r="V5" s="2">
+      <c r="V5" s="1">
         <v>46321</v>
       </c>
     </row>
@@ -1235,7 +1209,7 @@
       <c r="U6" t="s">
         <v>91</v>
       </c>
-      <c r="V6" s="2">
+      <c r="V6" s="1">
         <v>46291</v>
       </c>
     </row>
@@ -1261,7 +1235,7 @@
       <c r="G7" t="s">
         <v>106</v>
       </c>
-      <c r="H7" s="2">
+      <c r="H7" s="1">
         <v>46121</v>
       </c>
       <c r="I7" t="s">
@@ -1291,7 +1265,7 @@
       <c r="U7" t="s">
         <v>91</v>
       </c>
-      <c r="V7" s="2">
+      <c r="V7" s="1">
         <v>46138</v>
       </c>
     </row>
@@ -1338,7 +1312,7 @@
       <c r="U8" t="s">
         <v>91</v>
       </c>
-      <c r="V8" s="2">
+      <c r="V8" s="1">
         <v>46291</v>
       </c>
     </row>
@@ -1385,7 +1359,7 @@
       <c r="U9" t="s">
         <v>91</v>
       </c>
-      <c r="V9" s="2">
+      <c r="V9" s="1">
         <v>46291</v>
       </c>
     </row>
@@ -1408,7 +1382,7 @@
       <c r="G10" t="s">
         <v>106</v>
       </c>
-      <c r="H10" s="2">
+      <c r="H10" s="1">
         <v>46303</v>
       </c>
       <c r="I10" t="s">
@@ -1438,7 +1412,7 @@
       <c r="U10" t="s">
         <v>91</v>
       </c>
-      <c r="V10" s="2">
+      <c r="V10" s="1">
         <v>46291</v>
       </c>
     </row>
@@ -1485,7 +1459,7 @@
       <c r="U11" t="s">
         <v>91</v>
       </c>
-      <c r="V11" s="2">
+      <c r="V11" s="1">
         <v>46291</v>
       </c>
     </row>
@@ -1532,7 +1506,7 @@
       <c r="U12" t="s">
         <v>91</v>
       </c>
-      <c r="V12" s="2">
+      <c r="V12" s="1">
         <v>46291</v>
       </c>
     </row>
@@ -1558,7 +1532,7 @@
       <c r="G13" t="s">
         <v>106</v>
       </c>
-      <c r="H13" s="2">
+      <c r="H13" s="1">
         <v>46079</v>
       </c>
       <c r="I13" t="s">
@@ -1591,7 +1565,7 @@
       <c r="U13" t="s">
         <v>178</v>
       </c>
-      <c r="V13" s="2">
+      <c r="V13" s="1">
         <v>46079</v>
       </c>
     </row>
@@ -1617,7 +1591,7 @@
       <c r="G14" t="s">
         <v>106</v>
       </c>
-      <c r="H14" s="2">
+      <c r="H14" s="1">
         <v>46303</v>
       </c>
       <c r="I14" t="s">
@@ -1653,7 +1627,7 @@
       <c r="U14" t="s">
         <v>178</v>
       </c>
-      <c r="V14" s="2">
+      <c r="V14" s="1">
         <v>46352</v>
       </c>
     </row>
@@ -1679,7 +1653,7 @@
       <c r="G15" t="s">
         <v>106</v>
       </c>
-      <c r="H15" s="2">
+      <c r="H15" s="1">
         <v>46303</v>
       </c>
       <c r="I15" t="s">
@@ -1715,7 +1689,7 @@
       <c r="U15" t="s">
         <v>178</v>
       </c>
-      <c r="V15" s="2">
+      <c r="V15" s="1">
         <v>46352</v>
       </c>
     </row>
@@ -1741,7 +1715,7 @@
       <c r="G16" t="s">
         <v>106</v>
       </c>
-      <c r="H16" s="2">
+      <c r="H16" s="1">
         <v>46303</v>
       </c>
       <c r="I16" t="s">
@@ -1777,7 +1751,7 @@
       <c r="U16" t="s">
         <v>178</v>
       </c>
-      <c r="V16" s="2">
+      <c r="V16" s="1">
         <v>46352</v>
       </c>
     </row>
@@ -1803,7 +1777,7 @@
       <c r="G17" t="s">
         <v>106</v>
       </c>
-      <c r="H17" s="2">
+      <c r="H17" s="1">
         <v>46303</v>
       </c>
       <c r="I17" t="s">
@@ -1839,7 +1813,7 @@
       <c r="U17" t="s">
         <v>178</v>
       </c>
-      <c r="V17" s="2">
+      <c r="V17" s="1">
         <v>46229</v>
       </c>
     </row>
@@ -1865,7 +1839,7 @@
       <c r="G18" t="s">
         <v>106</v>
       </c>
-      <c r="H18" s="2">
+      <c r="H18" s="1">
         <v>46098</v>
       </c>
       <c r="I18" t="s">
@@ -1898,7 +1872,7 @@
       <c r="U18" t="s">
         <v>178</v>
       </c>
-      <c r="V18" s="2">
+      <c r="V18" s="1">
         <v>46107</v>
       </c>
     </row>
@@ -1924,7 +1898,7 @@
       <c r="G19" t="s">
         <v>106</v>
       </c>
-      <c r="H19" s="2">
+      <c r="H19" s="1">
         <v>46076</v>
       </c>
       <c r="I19" t="s">
@@ -1954,7 +1928,7 @@
       <c r="U19" t="s">
         <v>91</v>
       </c>
-      <c r="V19" s="2">
+      <c r="V19" s="1">
         <v>46079</v>
       </c>
     </row>
@@ -1980,7 +1954,7 @@
       <c r="G20" t="s">
         <v>106</v>
       </c>
-      <c r="H20" s="2">
+      <c r="H20" s="1">
         <v>46076</v>
       </c>
       <c r="I20" t="s">
@@ -2010,7 +1984,7 @@
       <c r="U20" t="s">
         <v>91</v>
       </c>
-      <c r="V20" s="2">
+      <c r="V20" s="1">
         <v>46079</v>
       </c>
     </row>
@@ -2057,7 +2031,7 @@
       <c r="U21" t="s">
         <v>91</v>
       </c>
-      <c r="V21" s="2">
+      <c r="V21" s="1">
         <v>46321</v>
       </c>
     </row>
@@ -2104,7 +2078,7 @@
       <c r="U22" t="s">
         <v>91</v>
       </c>
-      <c r="V22" s="2">
+      <c r="V22" s="1">
         <v>46321</v>
       </c>
     </row>
@@ -2151,7 +2125,7 @@
       <c r="U23" t="s">
         <v>91</v>
       </c>
-      <c r="V23" s="2">
+      <c r="V23" s="1">
         <v>46321</v>
       </c>
     </row>
@@ -2198,7 +2172,7 @@
       <c r="U24" t="s">
         <v>91</v>
       </c>
-      <c r="V24" s="2">
+      <c r="V24" s="1">
         <v>46321</v>
       </c>
     </row>
@@ -2224,7 +2198,7 @@
       <c r="G25" t="s">
         <v>106</v>
       </c>
-      <c r="H25" s="2">
+      <c r="H25" s="1">
         <v>46119</v>
       </c>
       <c r="I25" t="s">
@@ -2257,7 +2231,7 @@
       <c r="U25" t="s">
         <v>178</v>
       </c>
-      <c r="V25" s="2">
+      <c r="V25" s="1">
         <v>46138</v>
       </c>
     </row>
@@ -2283,7 +2257,7 @@
       <c r="G26" t="s">
         <v>106</v>
       </c>
-      <c r="H26" s="2">
+      <c r="H26" s="1">
         <v>46121</v>
       </c>
       <c r="I26" t="s">
@@ -2313,7 +2287,7 @@
       <c r="U26" t="s">
         <v>91</v>
       </c>
-      <c r="V26" s="2">
+      <c r="V26" s="1">
         <v>46138</v>
       </c>
     </row>
@@ -2339,7 +2313,7 @@
       <c r="G27" t="s">
         <v>106</v>
       </c>
-      <c r="H27" s="2">
+      <c r="H27" s="1">
         <v>46076</v>
       </c>
       <c r="I27" t="s">
@@ -2369,7 +2343,7 @@
       <c r="U27" t="s">
         <v>91</v>
       </c>
-      <c r="V27" s="2">
+      <c r="V27" s="1">
         <v>46079</v>
       </c>
     </row>
@@ -2395,7 +2369,7 @@
       <c r="G28" t="s">
         <v>106</v>
       </c>
-      <c r="H28" s="2">
+      <c r="H28" s="1">
         <v>46303</v>
       </c>
       <c r="I28" t="s">
@@ -2431,7 +2405,7 @@
       <c r="U28" t="s">
         <v>178</v>
       </c>
-      <c r="V28" s="2">
+      <c r="V28" s="1">
         <v>46291</v>
       </c>
     </row>
@@ -2457,7 +2431,7 @@
       <c r="G29" t="s">
         <v>106</v>
       </c>
-      <c r="H29" s="2">
+      <c r="H29" s="1">
         <v>46199</v>
       </c>
       <c r="I29" t="s">
@@ -2490,7 +2464,7 @@
       <c r="U29" t="s">
         <v>178</v>
       </c>
-      <c r="V29" s="2">
+      <c r="V29" s="1">
         <v>46199</v>
       </c>
     </row>
@@ -2516,7 +2490,7 @@
       <c r="G30" t="s">
         <v>106</v>
       </c>
-      <c r="H30" s="2">
+      <c r="H30" s="1">
         <v>46199</v>
       </c>
       <c r="I30" t="s">
@@ -2549,7 +2523,7 @@
       <c r="U30" t="s">
         <v>178</v>
       </c>
-      <c r="V30" s="2">
+      <c r="V30" s="1">
         <v>46199</v>
       </c>
     </row>
@@ -2575,7 +2549,7 @@
       <c r="G31" t="s">
         <v>106</v>
       </c>
-      <c r="H31" s="2">
+      <c r="H31" s="1">
         <v>46199</v>
       </c>
       <c r="I31" t="s">
@@ -2608,7 +2582,7 @@
       <c r="U31" t="s">
         <v>178</v>
       </c>
-      <c r="V31" s="2">
+      <c r="V31" s="1">
         <v>46199</v>
       </c>
     </row>
@@ -2634,7 +2608,7 @@
       <c r="G32" t="s">
         <v>106</v>
       </c>
-      <c r="H32" s="2">
+      <c r="H32" s="1">
         <v>46199</v>
       </c>
       <c r="I32" t="s">
@@ -2667,7 +2641,7 @@
       <c r="U32" t="s">
         <v>178</v>
       </c>
-      <c r="V32" s="2">
+      <c r="V32" s="1">
         <v>46199</v>
       </c>
     </row>
@@ -2720,7 +2694,7 @@
       <c r="U33" t="s">
         <v>178</v>
       </c>
-      <c r="V33" s="2">
+      <c r="V33" s="1">
         <v>46291</v>
       </c>
     </row>
@@ -2746,7 +2720,7 @@
       <c r="G34" t="s">
         <v>106</v>
       </c>
-      <c r="H34" s="2">
+      <c r="H34" s="1">
         <v>46191</v>
       </c>
       <c r="I34" t="s">
@@ -2779,7 +2753,7 @@
       <c r="U34" t="s">
         <v>178</v>
       </c>
-      <c r="V34" s="2">
+      <c r="V34" s="1">
         <v>46199</v>
       </c>
     </row>
@@ -2805,7 +2779,7 @@
       <c r="G35" t="s">
         <v>106</v>
       </c>
-      <c r="H35" s="2">
+      <c r="H35" s="1">
         <v>46119</v>
       </c>
       <c r="I35" t="s">
@@ -2835,7 +2809,7 @@
       <c r="U35" t="s">
         <v>178</v>
       </c>
-      <c r="V35" s="2">
+      <c r="V35" s="1">
         <v>46138</v>
       </c>
     </row>
@@ -2861,7 +2835,7 @@
       <c r="G36" t="s">
         <v>106</v>
       </c>
-      <c r="H36" s="2">
+      <c r="H36" s="1">
         <v>46213</v>
       </c>
       <c r="I36" t="s">
@@ -2891,7 +2865,7 @@
       <c r="U36" t="s">
         <v>91</v>
       </c>
-      <c r="V36" s="2">
+      <c r="V36" s="1">
         <v>46229</v>
       </c>
     </row>
@@ -2917,7 +2891,7 @@
       <c r="G37" t="s">
         <v>106</v>
       </c>
-      <c r="H37" s="2">
+      <c r="H37" s="1">
         <v>46175</v>
       </c>
       <c r="I37" t="s">
@@ -2947,7 +2921,7 @@
       <c r="U37" t="s">
         <v>91</v>
       </c>
-      <c r="V37" s="2">
+      <c r="V37" s="1">
         <v>46199</v>
       </c>
     </row>
@@ -2973,7 +2947,7 @@
       <c r="G38" t="s">
         <v>106</v>
       </c>
-      <c r="H38" s="2">
+      <c r="H38" s="1">
         <v>46213</v>
       </c>
       <c r="I38" t="s">
@@ -3003,7 +2977,7 @@
       <c r="U38" t="s">
         <v>91</v>
       </c>
-      <c r="V38" s="2">
+      <c r="V38" s="1">
         <v>46229</v>
       </c>
     </row>
@@ -3029,7 +3003,7 @@
       <c r="G39" t="s">
         <v>106</v>
       </c>
-      <c r="H39" s="2">
+      <c r="H39" s="1">
         <v>46199</v>
       </c>
       <c r="I39" t="s">
@@ -3059,7 +3033,7 @@
       <c r="U39" t="s">
         <v>91</v>
       </c>
-      <c r="V39" s="2">
+      <c r="V39" s="1">
         <v>46199</v>
       </c>
     </row>
@@ -3085,7 +3059,7 @@
       <c r="G40" t="s">
         <v>106</v>
       </c>
-      <c r="H40" s="2">
+      <c r="H40" s="1">
         <v>46199</v>
       </c>
       <c r="I40" t="s">
@@ -3115,7 +3089,7 @@
       <c r="U40" t="s">
         <v>91</v>
       </c>
-      <c r="V40" s="2">
+      <c r="V40" s="1">
         <v>46199</v>
       </c>
     </row>
@@ -3141,7 +3115,7 @@
       <c r="G41" t="s">
         <v>106</v>
       </c>
-      <c r="H41" s="2">
+      <c r="H41" s="1">
         <v>46204</v>
       </c>
       <c r="I41" t="s">
@@ -3171,7 +3145,7 @@
       <c r="U41" t="s">
         <v>91</v>
       </c>
-      <c r="V41" s="2">
+      <c r="V41" s="1">
         <v>46229</v>
       </c>
     </row>
@@ -3197,7 +3171,7 @@
       <c r="G42" t="s">
         <v>106</v>
       </c>
-      <c r="H42" s="2">
+      <c r="H42" s="1">
         <v>46244</v>
       </c>
       <c r="I42" t="s">
@@ -3227,7 +3201,7 @@
       <c r="U42" t="s">
         <v>91</v>
       </c>
-      <c r="V42" s="2">
+      <c r="V42" s="1">
         <v>46199</v>
       </c>
     </row>
@@ -3271,7 +3245,7 @@
       <c r="U43" t="s">
         <v>91</v>
       </c>
-      <c r="V43" s="2">
+      <c r="V43" s="1">
         <v>46260</v>
       </c>
     </row>
@@ -3297,7 +3271,7 @@
       <c r="G44" t="s">
         <v>106</v>
       </c>
-      <c r="H44" s="2">
+      <c r="H44" s="1">
         <v>46191</v>
       </c>
       <c r="I44" t="s">
@@ -3327,7 +3301,7 @@
       <c r="U44" t="s">
         <v>91</v>
       </c>
-      <c r="V44" s="2">
+      <c r="V44" s="1">
         <v>46199</v>
       </c>
     </row>
@@ -3353,7 +3327,7 @@
       <c r="G45" t="s">
         <v>106</v>
       </c>
-      <c r="H45" s="2">
+      <c r="H45" s="1">
         <v>46191</v>
       </c>
       <c r="I45" t="s">
@@ -3383,7 +3357,7 @@
       <c r="U45" t="s">
         <v>91</v>
       </c>
-      <c r="V45" s="2">
+      <c r="V45" s="1">
         <v>46199</v>
       </c>
     </row>
@@ -3409,7 +3383,7 @@
       <c r="G46" t="s">
         <v>106</v>
       </c>
-      <c r="H46" s="2">
+      <c r="H46" s="1">
         <v>46213</v>
       </c>
       <c r="I46" t="s">
@@ -3442,7 +3416,7 @@
       <c r="U46" t="s">
         <v>178</v>
       </c>
-      <c r="V46" s="2">
+      <c r="V46" s="1">
         <v>46229</v>
       </c>
     </row>
@@ -3468,7 +3442,7 @@
       <c r="G47" t="s">
         <v>106</v>
       </c>
-      <c r="H47" s="2">
+      <c r="H47" s="1">
         <v>46210</v>
       </c>
       <c r="I47" t="s">
@@ -3498,7 +3472,7 @@
       <c r="U47" t="s">
         <v>178</v>
       </c>
-      <c r="V47" s="2">
+      <c r="V47" s="1">
         <v>46229</v>
       </c>
     </row>
@@ -3545,7 +3519,7 @@
       <c r="U48" t="s">
         <v>91</v>
       </c>
-      <c r="V48" s="2">
+      <c r="V48" s="1">
         <v>46321</v>
       </c>
     </row>
@@ -3571,7 +3545,7 @@
       <c r="G49" t="s">
         <v>106</v>
       </c>
-      <c r="H49" s="2">
+      <c r="H49" s="1">
         <v>46303</v>
       </c>
       <c r="I49" t="s">
@@ -3607,7 +3581,7 @@
       <c r="U49" t="s">
         <v>178</v>
       </c>
-      <c r="V49" s="2">
+      <c r="V49" s="1">
         <v>46291</v>
       </c>
     </row>
@@ -3633,7 +3607,7 @@
       <c r="G50" t="s">
         <v>106</v>
       </c>
-      <c r="H50" s="2">
+      <c r="H50" s="1">
         <v>46176</v>
       </c>
       <c r="I50" t="s">
@@ -3666,7 +3640,7 @@
       <c r="U50" t="s">
         <v>178</v>
       </c>
-      <c r="V50" s="2">
+      <c r="V50" s="1">
         <v>46199</v>
       </c>
     </row>
@@ -3692,7 +3666,7 @@
       <c r="G51" t="s">
         <v>106</v>
       </c>
-      <c r="H51" s="2">
+      <c r="H51" s="1">
         <v>46314</v>
       </c>
       <c r="I51" t="s">
@@ -3728,7 +3702,7 @@
       <c r="U51" t="s">
         <v>178</v>
       </c>
-      <c r="V51" s="2">
+      <c r="V51" s="1">
         <v>46260</v>
       </c>
     </row>
@@ -3754,7 +3728,7 @@
       <c r="G52" t="s">
         <v>106</v>
       </c>
-      <c r="H52" s="2">
+      <c r="H52" s="1">
         <v>46295</v>
       </c>
       <c r="I52" t="s">
@@ -3790,7 +3764,7 @@
       <c r="U52" t="s">
         <v>178</v>
       </c>
-      <c r="V52" s="2">
+      <c r="V52" s="1">
         <v>46291</v>
       </c>
     </row>
@@ -3843,7 +3817,7 @@
       <c r="U53" t="s">
         <v>178</v>
       </c>
-      <c r="V53" s="2">
+      <c r="V53" s="1">
         <v>46321</v>
       </c>
     </row>
@@ -3869,7 +3843,7 @@
       <c r="G54" t="s">
         <v>106</v>
       </c>
-      <c r="H54" s="2">
+      <c r="H54" s="1">
         <v>46227</v>
       </c>
       <c r="I54" t="s">
@@ -3899,7 +3873,7 @@
       <c r="U54" t="s">
         <v>178</v>
       </c>
-      <c r="V54" s="2">
+      <c r="V54" s="1">
         <v>46229</v>
       </c>
     </row>
@@ -3922,7 +3896,7 @@
       <c r="G55" t="s">
         <v>106</v>
       </c>
-      <c r="H55" s="2">
+      <c r="H55" s="1">
         <v>46280</v>
       </c>
       <c r="I55" t="s">
@@ -3952,7 +3926,7 @@
       <c r="U55" t="s">
         <v>178</v>
       </c>
-      <c r="V55" s="2">
+      <c r="V55" s="1">
         <v>46291</v>
       </c>
     </row>
@@ -3975,7 +3949,7 @@
       <c r="G56" t="s">
         <v>106</v>
       </c>
-      <c r="H56" s="2">
+      <c r="H56" s="1">
         <v>46280</v>
       </c>
       <c r="I56" t="s">
@@ -4005,7 +3979,7 @@
       <c r="U56" t="s">
         <v>178</v>
       </c>
-      <c r="V56" s="2">
+      <c r="V56" s="1">
         <v>46260</v>
       </c>
     </row>
@@ -4028,7 +4002,7 @@
       <c r="G57" t="s">
         <v>106</v>
       </c>
-      <c r="H57" s="2">
+      <c r="H57" s="1">
         <v>46295</v>
       </c>
       <c r="I57" t="s">
@@ -4058,7 +4032,7 @@
       <c r="U57" t="s">
         <v>178</v>
       </c>
-      <c r="V57" s="2">
+      <c r="V57" s="1">
         <v>46291</v>
       </c>
     </row>
@@ -4081,7 +4055,7 @@
       <c r="G58" t="s">
         <v>106</v>
       </c>
-      <c r="H58" s="2">
+      <c r="H58" s="1">
         <v>46295</v>
       </c>
       <c r="I58" t="s">
@@ -4111,7 +4085,7 @@
       <c r="U58" t="s">
         <v>178</v>
       </c>
-      <c r="V58" s="2">
+      <c r="V58" s="1">
         <v>46291</v>
       </c>
     </row>
@@ -4134,7 +4108,7 @@
       <c r="G59" t="s">
         <v>106</v>
       </c>
-      <c r="H59" s="2">
+      <c r="H59" s="1">
         <v>46304</v>
       </c>
       <c r="I59" t="s">
@@ -4164,7 +4138,7 @@
       <c r="U59" t="s">
         <v>178</v>
       </c>
-      <c r="V59" s="2">
+      <c r="V59" s="1">
         <v>46321</v>
       </c>
     </row>
@@ -4190,7 +4164,7 @@
       <c r="G60" t="s">
         <v>106</v>
       </c>
-      <c r="H60" s="2">
+      <c r="H60" s="1">
         <v>46301</v>
       </c>
       <c r="I60" t="s">
@@ -4226,7 +4200,7 @@
       <c r="U60" t="s">
         <v>178</v>
       </c>
-      <c r="V60" s="2">
+      <c r="V60" s="1">
         <v>46352</v>
       </c>
     </row>
@@ -4270,7 +4244,7 @@
       <c r="U61" t="s">
         <v>178</v>
       </c>
-      <c r="V61" s="2">
+      <c r="V61" s="1">
         <v>46107</v>
       </c>
     </row>
@@ -4314,7 +4288,7 @@
       <c r="U62" t="s">
         <v>178</v>
       </c>
-      <c r="V62" s="2">
+      <c r="V62" s="1">
         <v>46107</v>
       </c>
     </row>
@@ -4358,7 +4332,7 @@
       <c r="U63" t="s">
         <v>178</v>
       </c>
-      <c r="V63" s="2">
+      <c r="V63" s="1">
         <v>46107</v>
       </c>
     </row>
@@ -4402,7 +4376,7 @@
       <c r="U64" t="s">
         <v>178</v>
       </c>
-      <c r="V64" s="2">
+      <c r="V64" s="1">
         <v>46107</v>
       </c>
     </row>
@@ -4446,7 +4420,7 @@
       <c r="U65" t="s">
         <v>178</v>
       </c>
-      <c r="V65" s="2">
+      <c r="V65" s="1">
         <v>46107</v>
       </c>
     </row>
@@ -4490,7 +4464,7 @@
       <c r="U66" t="s">
         <v>178</v>
       </c>
-      <c r="V66" s="2">
+      <c r="V66" s="1">
         <v>46107</v>
       </c>
     </row>
@@ -4534,7 +4508,7 @@
       <c r="U67" t="s">
         <v>91</v>
       </c>
-      <c r="V67" s="2">
+      <c r="V67" s="1">
         <v>46168</v>
       </c>
     </row>
@@ -4581,7 +4555,7 @@
       <c r="U68" t="s">
         <v>91</v>
       </c>
-      <c r="V68" s="2">
+      <c r="V68" s="1">
         <v>46291</v>
       </c>
     </row>
@@ -4607,7 +4581,7 @@
       <c r="G69" t="s">
         <v>106</v>
       </c>
-      <c r="H69" s="2">
+      <c r="H69" s="1">
         <v>46303</v>
       </c>
       <c r="I69" t="s">
@@ -4643,7 +4617,7 @@
       <c r="U69" t="s">
         <v>178</v>
       </c>
-      <c r="V69" s="2">
+      <c r="V69" s="1">
         <v>46229</v>
       </c>
     </row>
@@ -4687,7 +4661,7 @@
       <c r="U70" t="s">
         <v>91</v>
       </c>
-      <c r="V70" s="2">
+      <c r="V70" s="1">
         <v>46260</v>
       </c>
     </row>
@@ -4731,7 +4705,7 @@
       <c r="U71" t="s">
         <v>178</v>
       </c>
-      <c r="V71" s="2">
+      <c r="V71" s="1">
         <v>46291</v>
       </c>
     </row>
@@ -4775,7 +4749,7 @@
       <c r="U72" t="s">
         <v>178</v>
       </c>
-      <c r="V72" s="2">
+      <c r="V72" s="1">
         <v>46168</v>
       </c>
     </row>
@@ -4819,7 +4793,7 @@
       <c r="U73" t="s">
         <v>178</v>
       </c>
-      <c r="V73" s="2">
+      <c r="V73" s="1">
         <v>46291</v>
       </c>
     </row>
@@ -4863,7 +4837,7 @@
       <c r="U74" t="s">
         <v>178</v>
       </c>
-      <c r="V74" s="2">
+      <c r="V74" s="1">
         <v>46291</v>
       </c>
     </row>
@@ -4907,7 +4881,7 @@
       <c r="U75" t="s">
         <v>178</v>
       </c>
-      <c r="V75" s="2">
+      <c r="V75" s="1">
         <v>46291</v>
       </c>
     </row>
@@ -4954,7 +4928,7 @@
       <c r="U76" t="s">
         <v>91</v>
       </c>
-      <c r="V76" s="2">
+      <c r="V76" s="1">
         <v>46321</v>
       </c>
     </row>
@@ -5004,7 +4978,7 @@
       <c r="U77" t="s">
         <v>178</v>
       </c>
-      <c r="V77" s="2">
+      <c r="V77" s="1">
         <v>46381</v>
       </c>
     </row>
@@ -5054,7 +5028,7 @@
       <c r="U78" t="s">
         <v>178</v>
       </c>
-      <c r="V78" s="2">
+      <c r="V78" s="1">
         <v>46381</v>
       </c>
     </row>
@@ -5104,7 +5078,7 @@
       <c r="U79" t="s">
         <v>91</v>
       </c>
-      <c r="V79" s="2">
+      <c r="V79" s="1">
         <v>46381</v>
       </c>
     </row>
@@ -5154,7 +5128,7 @@
       <c r="U80" t="s">
         <v>91</v>
       </c>
-      <c r="V80" s="2">
+      <c r="V80" s="1">
         <v>46381</v>
       </c>
     </row>
@@ -5204,7 +5178,7 @@
       <c r="U81" t="s">
         <v>91</v>
       </c>
-      <c r="V81" s="2">
+      <c r="V81" s="1">
         <v>46382</v>
       </c>
     </row>
@@ -5248,7 +5222,7 @@
       <c r="U82" t="s">
         <v>91</v>
       </c>
-      <c r="V82" s="2">
+      <c r="V82" s="1">
         <v>46382</v>
       </c>
     </row>
@@ -5274,7 +5248,7 @@
       <c r="G83" t="s">
         <v>106</v>
       </c>
-      <c r="H83" s="2">
+      <c r="H83" s="1">
         <v>46314</v>
       </c>
       <c r="I83" t="s">
@@ -5310,7 +5284,7 @@
       <c r="U83" t="s">
         <v>178</v>
       </c>
-      <c r="V83" s="2">
+      <c r="V83" s="1">
         <v>46382</v>
       </c>
     </row>
@@ -5360,7 +5334,7 @@
       <c r="U84" t="s">
         <v>91</v>
       </c>
-      <c r="V84" s="2">
+      <c r="V84" s="1">
         <v>46321</v>
       </c>
     </row>
@@ -5404,7 +5378,7 @@
       <c r="U85" t="s">
         <v>91</v>
       </c>
-      <c r="V85" s="2">
+      <c r="V85" s="1">
         <v>46382</v>
       </c>
     </row>
@@ -5524,7 +5498,7 @@
       <c r="G88" t="s">
         <v>106</v>
       </c>
-      <c r="H88" s="2">
+      <c r="H88" s="1">
         <v>46303</v>
       </c>
       <c r="I88" t="s">
@@ -5554,7 +5528,7 @@
       <c r="U88" t="s">
         <v>91</v>
       </c>
-      <c r="V88" s="2">
+      <c r="V88" s="1">
         <v>46291</v>
       </c>
     </row>
@@ -5601,7 +5575,7 @@
       <c r="U89" t="s">
         <v>91</v>
       </c>
-      <c r="V89" s="2">
+      <c r="V89" s="1">
         <v>46291</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Atualização automática: mta (23/10/2026 14:21)
</commit_message>
<xml_diff>
--- a/Projetos/02_Dados_Tratados/base_mta_tratada.xlsx
+++ b/Projetos/02_Dados_Tratados/base_mta_tratada.xlsx
@@ -560,8 +560,16 @@
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="YYYY-MM-DD HH:MM:SS"/>
   </numFmts>
-  <fonts count="1">
+  <fonts count="2">
     <font>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
       <sz val="11"/>
       <color theme="1"/>
       <name val="Calibri"/>
@@ -577,7 +585,7 @@
       <patternFill patternType="gray125"/>
     </fill>
   </fills>
-  <borders count="1">
+  <borders count="2">
     <border>
       <left/>
       <right/>
@@ -585,12 +593,30 @@
       <bottom/>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin">
+        <color auto="1"/>
+      </left>
+      <right style="thin">
+        <color auto="1"/>
+      </right>
+      <top style="thin">
+        <color auto="1"/>
+      </top>
+      <bottom style="thin">
+        <color auto="1"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="3">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
   </cellXfs>
   <cellStyles count="1">
@@ -890,70 +916,70 @@
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:22">
-      <c r="A1" t="s">
+      <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
-      <c r="B1" t="s">
+      <c r="B1" s="1" t="s">
         <v>1</v>
       </c>
-      <c r="C1" t="s">
+      <c r="C1" s="1" t="s">
         <v>2</v>
       </c>
-      <c r="D1" t="s">
+      <c r="D1" s="1" t="s">
         <v>3</v>
       </c>
-      <c r="E1" t="s">
+      <c r="E1" s="1" t="s">
         <v>4</v>
       </c>
-      <c r="F1" t="s">
+      <c r="F1" s="1" t="s">
         <v>5</v>
       </c>
-      <c r="G1" t="s">
+      <c r="G1" s="1" t="s">
         <v>6</v>
       </c>
-      <c r="H1" t="s">
+      <c r="H1" s="1" t="s">
         <v>7</v>
       </c>
-      <c r="I1" t="s">
+      <c r="I1" s="1" t="s">
         <v>8</v>
       </c>
-      <c r="J1" t="s">
+      <c r="J1" s="1" t="s">
         <v>9</v>
       </c>
-      <c r="K1" t="s">
+      <c r="K1" s="1" t="s">
         <v>10</v>
       </c>
-      <c r="L1" t="s">
+      <c r="L1" s="1" t="s">
         <v>11</v>
       </c>
-      <c r="M1" t="s">
+      <c r="M1" s="1" t="s">
         <v>12</v>
       </c>
-      <c r="N1" t="s">
+      <c r="N1" s="1" t="s">
         <v>13</v>
       </c>
-      <c r="O1" t="s">
+      <c r="O1" s="1" t="s">
         <v>14</v>
       </c>
-      <c r="P1" t="s">
+      <c r="P1" s="1" t="s">
         <v>15</v>
       </c>
-      <c r="Q1" t="s">
+      <c r="Q1" s="1" t="s">
         <v>16</v>
       </c>
-      <c r="R1" t="s">
+      <c r="R1" s="1" t="s">
         <v>17</v>
       </c>
-      <c r="S1" t="s">
+      <c r="S1" s="1" t="s">
         <v>18</v>
       </c>
-      <c r="T1" t="s">
+      <c r="T1" s="1" t="s">
         <v>19</v>
       </c>
-      <c r="U1" t="s">
+      <c r="U1" s="1" t="s">
         <v>20</v>
       </c>
-      <c r="V1" t="s">
+      <c r="V1" s="1" t="s">
         <v>21</v>
       </c>
     </row>
@@ -979,7 +1005,7 @@
       <c r="G2" t="s">
         <v>106</v>
       </c>
-      <c r="H2" s="1">
+      <c r="H2" s="2">
         <v>46303</v>
       </c>
       <c r="I2" t="s">
@@ -1018,7 +1044,7 @@
       <c r="U2" t="s">
         <v>178</v>
       </c>
-      <c r="V2" s="1">
+      <c r="V2" s="2">
         <v>46229</v>
       </c>
     </row>
@@ -1065,7 +1091,7 @@
       <c r="U3" t="s">
         <v>91</v>
       </c>
-      <c r="V3" s="1">
+      <c r="V3" s="2">
         <v>46291</v>
       </c>
     </row>
@@ -1112,7 +1138,7 @@
       <c r="U4" t="s">
         <v>91</v>
       </c>
-      <c r="V4" s="1">
+      <c r="V4" s="2">
         <v>46321</v>
       </c>
     </row>
@@ -1159,7 +1185,7 @@
       <c r="U5" t="s">
         <v>91</v>
       </c>
-      <c r="V5" s="1">
+      <c r="V5" s="2">
         <v>46321</v>
       </c>
     </row>
@@ -1209,7 +1235,7 @@
       <c r="U6" t="s">
         <v>91</v>
       </c>
-      <c r="V6" s="1">
+      <c r="V6" s="2">
         <v>46291</v>
       </c>
     </row>
@@ -1235,7 +1261,7 @@
       <c r="G7" t="s">
         <v>106</v>
       </c>
-      <c r="H7" s="1">
+      <c r="H7" s="2">
         <v>46121</v>
       </c>
       <c r="I7" t="s">
@@ -1265,7 +1291,7 @@
       <c r="U7" t="s">
         <v>91</v>
       </c>
-      <c r="V7" s="1">
+      <c r="V7" s="2">
         <v>46138</v>
       </c>
     </row>
@@ -1312,7 +1338,7 @@
       <c r="U8" t="s">
         <v>91</v>
       </c>
-      <c r="V8" s="1">
+      <c r="V8" s="2">
         <v>46291</v>
       </c>
     </row>
@@ -1359,7 +1385,7 @@
       <c r="U9" t="s">
         <v>91</v>
       </c>
-      <c r="V9" s="1">
+      <c r="V9" s="2">
         <v>46291</v>
       </c>
     </row>
@@ -1382,7 +1408,7 @@
       <c r="G10" t="s">
         <v>106</v>
       </c>
-      <c r="H10" s="1">
+      <c r="H10" s="2">
         <v>46303</v>
       </c>
       <c r="I10" t="s">
@@ -1412,7 +1438,7 @@
       <c r="U10" t="s">
         <v>91</v>
       </c>
-      <c r="V10" s="1">
+      <c r="V10" s="2">
         <v>46291</v>
       </c>
     </row>
@@ -1459,7 +1485,7 @@
       <c r="U11" t="s">
         <v>91</v>
       </c>
-      <c r="V11" s="1">
+      <c r="V11" s="2">
         <v>46291</v>
       </c>
     </row>
@@ -1506,7 +1532,7 @@
       <c r="U12" t="s">
         <v>91</v>
       </c>
-      <c r="V12" s="1">
+      <c r="V12" s="2">
         <v>46291</v>
       </c>
     </row>
@@ -1532,7 +1558,7 @@
       <c r="G13" t="s">
         <v>106</v>
       </c>
-      <c r="H13" s="1">
+      <c r="H13" s="2">
         <v>46079</v>
       </c>
       <c r="I13" t="s">
@@ -1565,7 +1591,7 @@
       <c r="U13" t="s">
         <v>178</v>
       </c>
-      <c r="V13" s="1">
+      <c r="V13" s="2">
         <v>46079</v>
       </c>
     </row>
@@ -1591,7 +1617,7 @@
       <c r="G14" t="s">
         <v>106</v>
       </c>
-      <c r="H14" s="1">
+      <c r="H14" s="2">
         <v>46303</v>
       </c>
       <c r="I14" t="s">
@@ -1627,7 +1653,7 @@
       <c r="U14" t="s">
         <v>178</v>
       </c>
-      <c r="V14" s="1">
+      <c r="V14" s="2">
         <v>46352</v>
       </c>
     </row>
@@ -1653,7 +1679,7 @@
       <c r="G15" t="s">
         <v>106</v>
       </c>
-      <c r="H15" s="1">
+      <c r="H15" s="2">
         <v>46303</v>
       </c>
       <c r="I15" t="s">
@@ -1689,7 +1715,7 @@
       <c r="U15" t="s">
         <v>178</v>
       </c>
-      <c r="V15" s="1">
+      <c r="V15" s="2">
         <v>46352</v>
       </c>
     </row>
@@ -1715,7 +1741,7 @@
       <c r="G16" t="s">
         <v>106</v>
       </c>
-      <c r="H16" s="1">
+      <c r="H16" s="2">
         <v>46303</v>
       </c>
       <c r="I16" t="s">
@@ -1751,7 +1777,7 @@
       <c r="U16" t="s">
         <v>178</v>
       </c>
-      <c r="V16" s="1">
+      <c r="V16" s="2">
         <v>46352</v>
       </c>
     </row>
@@ -1777,7 +1803,7 @@
       <c r="G17" t="s">
         <v>106</v>
       </c>
-      <c r="H17" s="1">
+      <c r="H17" s="2">
         <v>46303</v>
       </c>
       <c r="I17" t="s">
@@ -1813,7 +1839,7 @@
       <c r="U17" t="s">
         <v>178</v>
       </c>
-      <c r="V17" s="1">
+      <c r="V17" s="2">
         <v>46229</v>
       </c>
     </row>
@@ -1839,7 +1865,7 @@
       <c r="G18" t="s">
         <v>106</v>
       </c>
-      <c r="H18" s="1">
+      <c r="H18" s="2">
         <v>46098</v>
       </c>
       <c r="I18" t="s">
@@ -1872,7 +1898,7 @@
       <c r="U18" t="s">
         <v>178</v>
       </c>
-      <c r="V18" s="1">
+      <c r="V18" s="2">
         <v>46107</v>
       </c>
     </row>
@@ -1898,7 +1924,7 @@
       <c r="G19" t="s">
         <v>106</v>
       </c>
-      <c r="H19" s="1">
+      <c r="H19" s="2">
         <v>46076</v>
       </c>
       <c r="I19" t="s">
@@ -1928,7 +1954,7 @@
       <c r="U19" t="s">
         <v>91</v>
       </c>
-      <c r="V19" s="1">
+      <c r="V19" s="2">
         <v>46079</v>
       </c>
     </row>
@@ -1954,7 +1980,7 @@
       <c r="G20" t="s">
         <v>106</v>
       </c>
-      <c r="H20" s="1">
+      <c r="H20" s="2">
         <v>46076</v>
       </c>
       <c r="I20" t="s">
@@ -1984,7 +2010,7 @@
       <c r="U20" t="s">
         <v>91</v>
       </c>
-      <c r="V20" s="1">
+      <c r="V20" s="2">
         <v>46079</v>
       </c>
     </row>
@@ -2031,7 +2057,7 @@
       <c r="U21" t="s">
         <v>91</v>
       </c>
-      <c r="V21" s="1">
+      <c r="V21" s="2">
         <v>46321</v>
       </c>
     </row>
@@ -2078,7 +2104,7 @@
       <c r="U22" t="s">
         <v>91</v>
       </c>
-      <c r="V22" s="1">
+      <c r="V22" s="2">
         <v>46321</v>
       </c>
     </row>
@@ -2125,7 +2151,7 @@
       <c r="U23" t="s">
         <v>91</v>
       </c>
-      <c r="V23" s="1">
+      <c r="V23" s="2">
         <v>46321</v>
       </c>
     </row>
@@ -2172,7 +2198,7 @@
       <c r="U24" t="s">
         <v>91</v>
       </c>
-      <c r="V24" s="1">
+      <c r="V24" s="2">
         <v>46321</v>
       </c>
     </row>
@@ -2198,7 +2224,7 @@
       <c r="G25" t="s">
         <v>106</v>
       </c>
-      <c r="H25" s="1">
+      <c r="H25" s="2">
         <v>46119</v>
       </c>
       <c r="I25" t="s">
@@ -2231,7 +2257,7 @@
       <c r="U25" t="s">
         <v>178</v>
       </c>
-      <c r="V25" s="1">
+      <c r="V25" s="2">
         <v>46138</v>
       </c>
     </row>
@@ -2257,7 +2283,7 @@
       <c r="G26" t="s">
         <v>106</v>
       </c>
-      <c r="H26" s="1">
+      <c r="H26" s="2">
         <v>46121</v>
       </c>
       <c r="I26" t="s">
@@ -2287,7 +2313,7 @@
       <c r="U26" t="s">
         <v>91</v>
       </c>
-      <c r="V26" s="1">
+      <c r="V26" s="2">
         <v>46138</v>
       </c>
     </row>
@@ -2313,7 +2339,7 @@
       <c r="G27" t="s">
         <v>106</v>
       </c>
-      <c r="H27" s="1">
+      <c r="H27" s="2">
         <v>46076</v>
       </c>
       <c r="I27" t="s">
@@ -2343,7 +2369,7 @@
       <c r="U27" t="s">
         <v>91</v>
       </c>
-      <c r="V27" s="1">
+      <c r="V27" s="2">
         <v>46079</v>
       </c>
     </row>
@@ -2369,7 +2395,7 @@
       <c r="G28" t="s">
         <v>106</v>
       </c>
-      <c r="H28" s="1">
+      <c r="H28" s="2">
         <v>46303</v>
       </c>
       <c r="I28" t="s">
@@ -2405,7 +2431,7 @@
       <c r="U28" t="s">
         <v>178</v>
       </c>
-      <c r="V28" s="1">
+      <c r="V28" s="2">
         <v>46291</v>
       </c>
     </row>
@@ -2431,7 +2457,7 @@
       <c r="G29" t="s">
         <v>106</v>
       </c>
-      <c r="H29" s="1">
+      <c r="H29" s="2">
         <v>46199</v>
       </c>
       <c r="I29" t="s">
@@ -2464,7 +2490,7 @@
       <c r="U29" t="s">
         <v>178</v>
       </c>
-      <c r="V29" s="1">
+      <c r="V29" s="2">
         <v>46199</v>
       </c>
     </row>
@@ -2490,7 +2516,7 @@
       <c r="G30" t="s">
         <v>106</v>
       </c>
-      <c r="H30" s="1">
+      <c r="H30" s="2">
         <v>46199</v>
       </c>
       <c r="I30" t="s">
@@ -2523,7 +2549,7 @@
       <c r="U30" t="s">
         <v>178</v>
       </c>
-      <c r="V30" s="1">
+      <c r="V30" s="2">
         <v>46199</v>
       </c>
     </row>
@@ -2549,7 +2575,7 @@
       <c r="G31" t="s">
         <v>106</v>
       </c>
-      <c r="H31" s="1">
+      <c r="H31" s="2">
         <v>46199</v>
       </c>
       <c r="I31" t="s">
@@ -2582,7 +2608,7 @@
       <c r="U31" t="s">
         <v>178</v>
       </c>
-      <c r="V31" s="1">
+      <c r="V31" s="2">
         <v>46199</v>
       </c>
     </row>
@@ -2608,7 +2634,7 @@
       <c r="G32" t="s">
         <v>106</v>
       </c>
-      <c r="H32" s="1">
+      <c r="H32" s="2">
         <v>46199</v>
       </c>
       <c r="I32" t="s">
@@ -2641,7 +2667,7 @@
       <c r="U32" t="s">
         <v>178</v>
       </c>
-      <c r="V32" s="1">
+      <c r="V32" s="2">
         <v>46199</v>
       </c>
     </row>
@@ -2694,7 +2720,7 @@
       <c r="U33" t="s">
         <v>178</v>
       </c>
-      <c r="V33" s="1">
+      <c r="V33" s="2">
         <v>46291</v>
       </c>
     </row>
@@ -2720,7 +2746,7 @@
       <c r="G34" t="s">
         <v>106</v>
       </c>
-      <c r="H34" s="1">
+      <c r="H34" s="2">
         <v>46191</v>
       </c>
       <c r="I34" t="s">
@@ -2753,7 +2779,7 @@
       <c r="U34" t="s">
         <v>178</v>
       </c>
-      <c r="V34" s="1">
+      <c r="V34" s="2">
         <v>46199</v>
       </c>
     </row>
@@ -2779,7 +2805,7 @@
       <c r="G35" t="s">
         <v>106</v>
       </c>
-      <c r="H35" s="1">
+      <c r="H35" s="2">
         <v>46119</v>
       </c>
       <c r="I35" t="s">
@@ -2809,7 +2835,7 @@
       <c r="U35" t="s">
         <v>178</v>
       </c>
-      <c r="V35" s="1">
+      <c r="V35" s="2">
         <v>46138</v>
       </c>
     </row>
@@ -2835,7 +2861,7 @@
       <c r="G36" t="s">
         <v>106</v>
       </c>
-      <c r="H36" s="1">
+      <c r="H36" s="2">
         <v>46213</v>
       </c>
       <c r="I36" t="s">
@@ -2865,7 +2891,7 @@
       <c r="U36" t="s">
         <v>91</v>
       </c>
-      <c r="V36" s="1">
+      <c r="V36" s="2">
         <v>46229</v>
       </c>
     </row>
@@ -2891,7 +2917,7 @@
       <c r="G37" t="s">
         <v>106</v>
       </c>
-      <c r="H37" s="1">
+      <c r="H37" s="2">
         <v>46175</v>
       </c>
       <c r="I37" t="s">
@@ -2921,7 +2947,7 @@
       <c r="U37" t="s">
         <v>91</v>
       </c>
-      <c r="V37" s="1">
+      <c r="V37" s="2">
         <v>46199</v>
       </c>
     </row>
@@ -2947,7 +2973,7 @@
       <c r="G38" t="s">
         <v>106</v>
       </c>
-      <c r="H38" s="1">
+      <c r="H38" s="2">
         <v>46213</v>
       </c>
       <c r="I38" t="s">
@@ -2977,7 +3003,7 @@
       <c r="U38" t="s">
         <v>91</v>
       </c>
-      <c r="V38" s="1">
+      <c r="V38" s="2">
         <v>46229</v>
       </c>
     </row>
@@ -3003,7 +3029,7 @@
       <c r="G39" t="s">
         <v>106</v>
       </c>
-      <c r="H39" s="1">
+      <c r="H39" s="2">
         <v>46199</v>
       </c>
       <c r="I39" t="s">
@@ -3033,7 +3059,7 @@
       <c r="U39" t="s">
         <v>91</v>
       </c>
-      <c r="V39" s="1">
+      <c r="V39" s="2">
         <v>46199</v>
       </c>
     </row>
@@ -3059,7 +3085,7 @@
       <c r="G40" t="s">
         <v>106</v>
       </c>
-      <c r="H40" s="1">
+      <c r="H40" s="2">
         <v>46199</v>
       </c>
       <c r="I40" t="s">
@@ -3089,7 +3115,7 @@
       <c r="U40" t="s">
         <v>91</v>
       </c>
-      <c r="V40" s="1">
+      <c r="V40" s="2">
         <v>46199</v>
       </c>
     </row>
@@ -3115,7 +3141,7 @@
       <c r="G41" t="s">
         <v>106</v>
       </c>
-      <c r="H41" s="1">
+      <c r="H41" s="2">
         <v>46204</v>
       </c>
       <c r="I41" t="s">
@@ -3145,7 +3171,7 @@
       <c r="U41" t="s">
         <v>91</v>
       </c>
-      <c r="V41" s="1">
+      <c r="V41" s="2">
         <v>46229</v>
       </c>
     </row>
@@ -3171,7 +3197,7 @@
       <c r="G42" t="s">
         <v>106</v>
       </c>
-      <c r="H42" s="1">
+      <c r="H42" s="2">
         <v>46244</v>
       </c>
       <c r="I42" t="s">
@@ -3201,7 +3227,7 @@
       <c r="U42" t="s">
         <v>91</v>
       </c>
-      <c r="V42" s="1">
+      <c r="V42" s="2">
         <v>46199</v>
       </c>
     </row>
@@ -3245,7 +3271,7 @@
       <c r="U43" t="s">
         <v>91</v>
       </c>
-      <c r="V43" s="1">
+      <c r="V43" s="2">
         <v>46260</v>
       </c>
     </row>
@@ -3271,7 +3297,7 @@
       <c r="G44" t="s">
         <v>106</v>
       </c>
-      <c r="H44" s="1">
+      <c r="H44" s="2">
         <v>46191</v>
       </c>
       <c r="I44" t="s">
@@ -3301,7 +3327,7 @@
       <c r="U44" t="s">
         <v>91</v>
       </c>
-      <c r="V44" s="1">
+      <c r="V44" s="2">
         <v>46199</v>
       </c>
     </row>
@@ -3327,7 +3353,7 @@
       <c r="G45" t="s">
         <v>106</v>
       </c>
-      <c r="H45" s="1">
+      <c r="H45" s="2">
         <v>46191</v>
       </c>
       <c r="I45" t="s">
@@ -3357,7 +3383,7 @@
       <c r="U45" t="s">
         <v>91</v>
       </c>
-      <c r="V45" s="1">
+      <c r="V45" s="2">
         <v>46199</v>
       </c>
     </row>
@@ -3383,7 +3409,7 @@
       <c r="G46" t="s">
         <v>106</v>
       </c>
-      <c r="H46" s="1">
+      <c r="H46" s="2">
         <v>46213</v>
       </c>
       <c r="I46" t="s">
@@ -3416,7 +3442,7 @@
       <c r="U46" t="s">
         <v>178</v>
       </c>
-      <c r="V46" s="1">
+      <c r="V46" s="2">
         <v>46229</v>
       </c>
     </row>
@@ -3442,7 +3468,7 @@
       <c r="G47" t="s">
         <v>106</v>
       </c>
-      <c r="H47" s="1">
+      <c r="H47" s="2">
         <v>46210</v>
       </c>
       <c r="I47" t="s">
@@ -3472,7 +3498,7 @@
       <c r="U47" t="s">
         <v>178</v>
       </c>
-      <c r="V47" s="1">
+      <c r="V47" s="2">
         <v>46229</v>
       </c>
     </row>
@@ -3519,7 +3545,7 @@
       <c r="U48" t="s">
         <v>91</v>
       </c>
-      <c r="V48" s="1">
+      <c r="V48" s="2">
         <v>46321</v>
       </c>
     </row>
@@ -3545,7 +3571,7 @@
       <c r="G49" t="s">
         <v>106</v>
       </c>
-      <c r="H49" s="1">
+      <c r="H49" s="2">
         <v>46303</v>
       </c>
       <c r="I49" t="s">
@@ -3581,7 +3607,7 @@
       <c r="U49" t="s">
         <v>178</v>
       </c>
-      <c r="V49" s="1">
+      <c r="V49" s="2">
         <v>46291</v>
       </c>
     </row>
@@ -3607,7 +3633,7 @@
       <c r="G50" t="s">
         <v>106</v>
       </c>
-      <c r="H50" s="1">
+      <c r="H50" s="2">
         <v>46176</v>
       </c>
       <c r="I50" t="s">
@@ -3640,7 +3666,7 @@
       <c r="U50" t="s">
         <v>178</v>
       </c>
-      <c r="V50" s="1">
+      <c r="V50" s="2">
         <v>46199</v>
       </c>
     </row>
@@ -3666,7 +3692,7 @@
       <c r="G51" t="s">
         <v>106</v>
       </c>
-      <c r="H51" s="1">
+      <c r="H51" s="2">
         <v>46314</v>
       </c>
       <c r="I51" t="s">
@@ -3702,7 +3728,7 @@
       <c r="U51" t="s">
         <v>178</v>
       </c>
-      <c r="V51" s="1">
+      <c r="V51" s="2">
         <v>46260</v>
       </c>
     </row>
@@ -3728,7 +3754,7 @@
       <c r="G52" t="s">
         <v>106</v>
       </c>
-      <c r="H52" s="1">
+      <c r="H52" s="2">
         <v>46295</v>
       </c>
       <c r="I52" t="s">
@@ -3764,7 +3790,7 @@
       <c r="U52" t="s">
         <v>178</v>
       </c>
-      <c r="V52" s="1">
+      <c r="V52" s="2">
         <v>46291</v>
       </c>
     </row>
@@ -3817,7 +3843,7 @@
       <c r="U53" t="s">
         <v>178</v>
       </c>
-      <c r="V53" s="1">
+      <c r="V53" s="2">
         <v>46321</v>
       </c>
     </row>
@@ -3843,7 +3869,7 @@
       <c r="G54" t="s">
         <v>106</v>
       </c>
-      <c r="H54" s="1">
+      <c r="H54" s="2">
         <v>46227</v>
       </c>
       <c r="I54" t="s">
@@ -3873,7 +3899,7 @@
       <c r="U54" t="s">
         <v>178</v>
       </c>
-      <c r="V54" s="1">
+      <c r="V54" s="2">
         <v>46229</v>
       </c>
     </row>
@@ -3896,7 +3922,7 @@
       <c r="G55" t="s">
         <v>106</v>
       </c>
-      <c r="H55" s="1">
+      <c r="H55" s="2">
         <v>46280</v>
       </c>
       <c r="I55" t="s">
@@ -3926,7 +3952,7 @@
       <c r="U55" t="s">
         <v>178</v>
       </c>
-      <c r="V55" s="1">
+      <c r="V55" s="2">
         <v>46291</v>
       </c>
     </row>
@@ -3949,7 +3975,7 @@
       <c r="G56" t="s">
         <v>106</v>
       </c>
-      <c r="H56" s="1">
+      <c r="H56" s="2">
         <v>46280</v>
       </c>
       <c r="I56" t="s">
@@ -3979,7 +4005,7 @@
       <c r="U56" t="s">
         <v>178</v>
       </c>
-      <c r="V56" s="1">
+      <c r="V56" s="2">
         <v>46260</v>
       </c>
     </row>
@@ -4002,7 +4028,7 @@
       <c r="G57" t="s">
         <v>106</v>
       </c>
-      <c r="H57" s="1">
+      <c r="H57" s="2">
         <v>46295</v>
       </c>
       <c r="I57" t="s">
@@ -4032,7 +4058,7 @@
       <c r="U57" t="s">
         <v>178</v>
       </c>
-      <c r="V57" s="1">
+      <c r="V57" s="2">
         <v>46291</v>
       </c>
     </row>
@@ -4055,7 +4081,7 @@
       <c r="G58" t="s">
         <v>106</v>
       </c>
-      <c r="H58" s="1">
+      <c r="H58" s="2">
         <v>46295</v>
       </c>
       <c r="I58" t="s">
@@ -4085,7 +4111,7 @@
       <c r="U58" t="s">
         <v>178</v>
       </c>
-      <c r="V58" s="1">
+      <c r="V58" s="2">
         <v>46291</v>
       </c>
     </row>
@@ -4108,7 +4134,7 @@
       <c r="G59" t="s">
         <v>106</v>
       </c>
-      <c r="H59" s="1">
+      <c r="H59" s="2">
         <v>46304</v>
       </c>
       <c r="I59" t="s">
@@ -4138,7 +4164,7 @@
       <c r="U59" t="s">
         <v>178</v>
       </c>
-      <c r="V59" s="1">
+      <c r="V59" s="2">
         <v>46321</v>
       </c>
     </row>
@@ -4164,7 +4190,7 @@
       <c r="G60" t="s">
         <v>106</v>
       </c>
-      <c r="H60" s="1">
+      <c r="H60" s="2">
         <v>46301</v>
       </c>
       <c r="I60" t="s">
@@ -4200,7 +4226,7 @@
       <c r="U60" t="s">
         <v>178</v>
       </c>
-      <c r="V60" s="1">
+      <c r="V60" s="2">
         <v>46352</v>
       </c>
     </row>
@@ -4244,7 +4270,7 @@
       <c r="U61" t="s">
         <v>178</v>
       </c>
-      <c r="V61" s="1">
+      <c r="V61" s="2">
         <v>46107</v>
       </c>
     </row>
@@ -4288,7 +4314,7 @@
       <c r="U62" t="s">
         <v>178</v>
       </c>
-      <c r="V62" s="1">
+      <c r="V62" s="2">
         <v>46107</v>
       </c>
     </row>
@@ -4332,7 +4358,7 @@
       <c r="U63" t="s">
         <v>178</v>
       </c>
-      <c r="V63" s="1">
+      <c r="V63" s="2">
         <v>46107</v>
       </c>
     </row>
@@ -4376,7 +4402,7 @@
       <c r="U64" t="s">
         <v>178</v>
       </c>
-      <c r="V64" s="1">
+      <c r="V64" s="2">
         <v>46107</v>
       </c>
     </row>
@@ -4420,7 +4446,7 @@
       <c r="U65" t="s">
         <v>178</v>
       </c>
-      <c r="V65" s="1">
+      <c r="V65" s="2">
         <v>46107</v>
       </c>
     </row>
@@ -4464,7 +4490,7 @@
       <c r="U66" t="s">
         <v>178</v>
       </c>
-      <c r="V66" s="1">
+      <c r="V66" s="2">
         <v>46107</v>
       </c>
     </row>
@@ -4508,7 +4534,7 @@
       <c r="U67" t="s">
         <v>91</v>
       </c>
-      <c r="V67" s="1">
+      <c r="V67" s="2">
         <v>46168</v>
       </c>
     </row>
@@ -4555,7 +4581,7 @@
       <c r="U68" t="s">
         <v>91</v>
       </c>
-      <c r="V68" s="1">
+      <c r="V68" s="2">
         <v>46291</v>
       </c>
     </row>
@@ -4581,7 +4607,7 @@
       <c r="G69" t="s">
         <v>106</v>
       </c>
-      <c r="H69" s="1">
+      <c r="H69" s="2">
         <v>46303</v>
       </c>
       <c r="I69" t="s">
@@ -4617,7 +4643,7 @@
       <c r="U69" t="s">
         <v>178</v>
       </c>
-      <c r="V69" s="1">
+      <c r="V69" s="2">
         <v>46229</v>
       </c>
     </row>
@@ -4661,7 +4687,7 @@
       <c r="U70" t="s">
         <v>91</v>
       </c>
-      <c r="V70" s="1">
+      <c r="V70" s="2">
         <v>46260</v>
       </c>
     </row>
@@ -4705,7 +4731,7 @@
       <c r="U71" t="s">
         <v>178</v>
       </c>
-      <c r="V71" s="1">
+      <c r="V71" s="2">
         <v>46291</v>
       </c>
     </row>
@@ -4749,7 +4775,7 @@
       <c r="U72" t="s">
         <v>178</v>
       </c>
-      <c r="V72" s="1">
+      <c r="V72" s="2">
         <v>46168</v>
       </c>
     </row>
@@ -4793,7 +4819,7 @@
       <c r="U73" t="s">
         <v>178</v>
       </c>
-      <c r="V73" s="1">
+      <c r="V73" s="2">
         <v>46291</v>
       </c>
     </row>
@@ -4837,7 +4863,7 @@
       <c r="U74" t="s">
         <v>178</v>
       </c>
-      <c r="V74" s="1">
+      <c r="V74" s="2">
         <v>46291</v>
       </c>
     </row>
@@ -4881,7 +4907,7 @@
       <c r="U75" t="s">
         <v>178</v>
       </c>
-      <c r="V75" s="1">
+      <c r="V75" s="2">
         <v>46291</v>
       </c>
     </row>
@@ -4928,7 +4954,7 @@
       <c r="U76" t="s">
         <v>91</v>
       </c>
-      <c r="V76" s="1">
+      <c r="V76" s="2">
         <v>46321</v>
       </c>
     </row>
@@ -4978,7 +5004,7 @@
       <c r="U77" t="s">
         <v>178</v>
       </c>
-      <c r="V77" s="1">
+      <c r="V77" s="2">
         <v>46381</v>
       </c>
     </row>
@@ -5028,7 +5054,7 @@
       <c r="U78" t="s">
         <v>178</v>
       </c>
-      <c r="V78" s="1">
+      <c r="V78" s="2">
         <v>46381</v>
       </c>
     </row>
@@ -5078,7 +5104,7 @@
       <c r="U79" t="s">
         <v>91</v>
       </c>
-      <c r="V79" s="1">
+      <c r="V79" s="2">
         <v>46381</v>
       </c>
     </row>
@@ -5128,7 +5154,7 @@
       <c r="U80" t="s">
         <v>91</v>
       </c>
-      <c r="V80" s="1">
+      <c r="V80" s="2">
         <v>46381</v>
       </c>
     </row>
@@ -5178,7 +5204,7 @@
       <c r="U81" t="s">
         <v>91</v>
       </c>
-      <c r="V81" s="1">
+      <c r="V81" s="2">
         <v>46382</v>
       </c>
     </row>
@@ -5222,7 +5248,7 @@
       <c r="U82" t="s">
         <v>91</v>
       </c>
-      <c r="V82" s="1">
+      <c r="V82" s="2">
         <v>46382</v>
       </c>
     </row>
@@ -5248,7 +5274,7 @@
       <c r="G83" t="s">
         <v>106</v>
       </c>
-      <c r="H83" s="1">
+      <c r="H83" s="2">
         <v>46314</v>
       </c>
       <c r="I83" t="s">
@@ -5284,7 +5310,7 @@
       <c r="U83" t="s">
         <v>178</v>
       </c>
-      <c r="V83" s="1">
+      <c r="V83" s="2">
         <v>46382</v>
       </c>
     </row>
@@ -5334,7 +5360,7 @@
       <c r="U84" t="s">
         <v>91</v>
       </c>
-      <c r="V84" s="1">
+      <c r="V84" s="2">
         <v>46321</v>
       </c>
     </row>
@@ -5378,7 +5404,7 @@
       <c r="U85" t="s">
         <v>91</v>
       </c>
-      <c r="V85" s="1">
+      <c r="V85" s="2">
         <v>46382</v>
       </c>
     </row>
@@ -5498,7 +5524,7 @@
       <c r="G88" t="s">
         <v>106</v>
       </c>
-      <c r="H88" s="1">
+      <c r="H88" s="2">
         <v>46303</v>
       </c>
       <c r="I88" t="s">
@@ -5528,7 +5554,7 @@
       <c r="U88" t="s">
         <v>91</v>
       </c>
-      <c r="V88" s="1">
+      <c r="V88" s="2">
         <v>46291</v>
       </c>
     </row>
@@ -5575,7 +5601,7 @@
       <c r="U89" t="s">
         <v>91</v>
       </c>
-      <c r="V89" s="1">
+      <c r="V89" s="2">
         <v>46291</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Atualização automática: mta (26/10/2026 14:17)
</commit_message>
<xml_diff>
--- a/Projetos/02_Dados_Tratados/base_mta_tratada.xlsx
+++ b/Projetos/02_Dados_Tratados/base_mta_tratada.xlsx
@@ -560,16 +560,8 @@
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="YYYY-MM-DD HH:MM:SS"/>
   </numFmts>
-  <fonts count="2">
+  <fonts count="1">
     <font>
-      <sz val="11"/>
-      <color theme="1"/>
-      <name val="Calibri"/>
-      <family val="2"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <b/>
       <sz val="11"/>
       <color theme="1"/>
       <name val="Calibri"/>
@@ -585,7 +577,7 @@
       <patternFill patternType="gray125"/>
     </fill>
   </fills>
-  <borders count="2">
+  <borders count="1">
     <border>
       <left/>
       <right/>
@@ -593,30 +585,12 @@
       <bottom/>
       <diagonal/>
     </border>
-    <border>
-      <left style="thin">
-        <color auto="1"/>
-      </left>
-      <right style="thin">
-        <color auto="1"/>
-      </right>
-      <top style="thin">
-        <color auto="1"/>
-      </top>
-      <bottom style="thin">
-        <color auto="1"/>
-      </bottom>
-      <diagonal/>
-    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="3">
+  <cellXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top"/>
-    </xf>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
   </cellXfs>
   <cellStyles count="1">
@@ -916,70 +890,70 @@
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:22">
-      <c r="A1" s="1" t="s">
+      <c r="A1" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="1" t="s">
+      <c r="B1" t="s">
         <v>1</v>
       </c>
-      <c r="C1" s="1" t="s">
+      <c r="C1" t="s">
         <v>2</v>
       </c>
-      <c r="D1" s="1" t="s">
+      <c r="D1" t="s">
         <v>3</v>
       </c>
-      <c r="E1" s="1" t="s">
+      <c r="E1" t="s">
         <v>4</v>
       </c>
-      <c r="F1" s="1" t="s">
+      <c r="F1" t="s">
         <v>5</v>
       </c>
-      <c r="G1" s="1" t="s">
+      <c r="G1" t="s">
         <v>6</v>
       </c>
-      <c r="H1" s="1" t="s">
+      <c r="H1" t="s">
         <v>7</v>
       </c>
-      <c r="I1" s="1" t="s">
+      <c r="I1" t="s">
         <v>8</v>
       </c>
-      <c r="J1" s="1" t="s">
+      <c r="J1" t="s">
         <v>9</v>
       </c>
-      <c r="K1" s="1" t="s">
+      <c r="K1" t="s">
         <v>10</v>
       </c>
-      <c r="L1" s="1" t="s">
+      <c r="L1" t="s">
         <v>11</v>
       </c>
-      <c r="M1" s="1" t="s">
+      <c r="M1" t="s">
         <v>12</v>
       </c>
-      <c r="N1" s="1" t="s">
+      <c r="N1" t="s">
         <v>13</v>
       </c>
-      <c r="O1" s="1" t="s">
+      <c r="O1" t="s">
         <v>14</v>
       </c>
-      <c r="P1" s="1" t="s">
+      <c r="P1" t="s">
         <v>15</v>
       </c>
-      <c r="Q1" s="1" t="s">
+      <c r="Q1" t="s">
         <v>16</v>
       </c>
-      <c r="R1" s="1" t="s">
+      <c r="R1" t="s">
         <v>17</v>
       </c>
-      <c r="S1" s="1" t="s">
+      <c r="S1" t="s">
         <v>18</v>
       </c>
-      <c r="T1" s="1" t="s">
+      <c r="T1" t="s">
         <v>19</v>
       </c>
-      <c r="U1" s="1" t="s">
+      <c r="U1" t="s">
         <v>20</v>
       </c>
-      <c r="V1" s="1" t="s">
+      <c r="V1" t="s">
         <v>21</v>
       </c>
     </row>
@@ -1005,7 +979,7 @@
       <c r="G2" t="s">
         <v>106</v>
       </c>
-      <c r="H2" s="2">
+      <c r="H2" s="1">
         <v>46303</v>
       </c>
       <c r="I2" t="s">
@@ -1044,7 +1018,7 @@
       <c r="U2" t="s">
         <v>178</v>
       </c>
-      <c r="V2" s="2">
+      <c r="V2" s="1">
         <v>46229</v>
       </c>
     </row>
@@ -1091,7 +1065,7 @@
       <c r="U3" t="s">
         <v>91</v>
       </c>
-      <c r="V3" s="2">
+      <c r="V3" s="1">
         <v>46291</v>
       </c>
     </row>
@@ -1138,7 +1112,7 @@
       <c r="U4" t="s">
         <v>91</v>
       </c>
-      <c r="V4" s="2">
+      <c r="V4" s="1">
         <v>46321</v>
       </c>
     </row>
@@ -1185,7 +1159,7 @@
       <c r="U5" t="s">
         <v>91</v>
       </c>
-      <c r="V5" s="2">
+      <c r="V5" s="1">
         <v>46321</v>
       </c>
     </row>
@@ -1235,7 +1209,7 @@
       <c r="U6" t="s">
         <v>91</v>
       </c>
-      <c r="V6" s="2">
+      <c r="V6" s="1">
         <v>46291</v>
       </c>
     </row>
@@ -1261,7 +1235,7 @@
       <c r="G7" t="s">
         <v>106</v>
       </c>
-      <c r="H7" s="2">
+      <c r="H7" s="1">
         <v>46121</v>
       </c>
       <c r="I7" t="s">
@@ -1291,7 +1265,7 @@
       <c r="U7" t="s">
         <v>91</v>
       </c>
-      <c r="V7" s="2">
+      <c r="V7" s="1">
         <v>46138</v>
       </c>
     </row>
@@ -1338,7 +1312,7 @@
       <c r="U8" t="s">
         <v>91</v>
       </c>
-      <c r="V8" s="2">
+      <c r="V8" s="1">
         <v>46291</v>
       </c>
     </row>
@@ -1385,7 +1359,7 @@
       <c r="U9" t="s">
         <v>91</v>
       </c>
-      <c r="V9" s="2">
+      <c r="V9" s="1">
         <v>46291</v>
       </c>
     </row>
@@ -1408,7 +1382,7 @@
       <c r="G10" t="s">
         <v>106</v>
       </c>
-      <c r="H10" s="2">
+      <c r="H10" s="1">
         <v>46303</v>
       </c>
       <c r="I10" t="s">
@@ -1438,7 +1412,7 @@
       <c r="U10" t="s">
         <v>91</v>
       </c>
-      <c r="V10" s="2">
+      <c r="V10" s="1">
         <v>46291</v>
       </c>
     </row>
@@ -1485,7 +1459,7 @@
       <c r="U11" t="s">
         <v>91</v>
       </c>
-      <c r="V11" s="2">
+      <c r="V11" s="1">
         <v>46291</v>
       </c>
     </row>
@@ -1532,7 +1506,7 @@
       <c r="U12" t="s">
         <v>91</v>
       </c>
-      <c r="V12" s="2">
+      <c r="V12" s="1">
         <v>46291</v>
       </c>
     </row>
@@ -1558,7 +1532,7 @@
       <c r="G13" t="s">
         <v>106</v>
       </c>
-      <c r="H13" s="2">
+      <c r="H13" s="1">
         <v>46079</v>
       </c>
       <c r="I13" t="s">
@@ -1591,7 +1565,7 @@
       <c r="U13" t="s">
         <v>178</v>
       </c>
-      <c r="V13" s="2">
+      <c r="V13" s="1">
         <v>46079</v>
       </c>
     </row>
@@ -1617,7 +1591,7 @@
       <c r="G14" t="s">
         <v>106</v>
       </c>
-      <c r="H14" s="2">
+      <c r="H14" s="1">
         <v>46303</v>
       </c>
       <c r="I14" t="s">
@@ -1653,7 +1627,7 @@
       <c r="U14" t="s">
         <v>178</v>
       </c>
-      <c r="V14" s="2">
+      <c r="V14" s="1">
         <v>46352</v>
       </c>
     </row>
@@ -1679,7 +1653,7 @@
       <c r="G15" t="s">
         <v>106</v>
       </c>
-      <c r="H15" s="2">
+      <c r="H15" s="1">
         <v>46303</v>
       </c>
       <c r="I15" t="s">
@@ -1715,7 +1689,7 @@
       <c r="U15" t="s">
         <v>178</v>
       </c>
-      <c r="V15" s="2">
+      <c r="V15" s="1">
         <v>46352</v>
       </c>
     </row>
@@ -1741,7 +1715,7 @@
       <c r="G16" t="s">
         <v>106</v>
       </c>
-      <c r="H16" s="2">
+      <c r="H16" s="1">
         <v>46303</v>
       </c>
       <c r="I16" t="s">
@@ -1777,7 +1751,7 @@
       <c r="U16" t="s">
         <v>178</v>
       </c>
-      <c r="V16" s="2">
+      <c r="V16" s="1">
         <v>46352</v>
       </c>
     </row>
@@ -1803,7 +1777,7 @@
       <c r="G17" t="s">
         <v>106</v>
       </c>
-      <c r="H17" s="2">
+      <c r="H17" s="1">
         <v>46303</v>
       </c>
       <c r="I17" t="s">
@@ -1839,7 +1813,7 @@
       <c r="U17" t="s">
         <v>178</v>
       </c>
-      <c r="V17" s="2">
+      <c r="V17" s="1">
         <v>46229</v>
       </c>
     </row>
@@ -1865,7 +1839,7 @@
       <c r="G18" t="s">
         <v>106</v>
       </c>
-      <c r="H18" s="2">
+      <c r="H18" s="1">
         <v>46098</v>
       </c>
       <c r="I18" t="s">
@@ -1898,7 +1872,7 @@
       <c r="U18" t="s">
         <v>178</v>
       </c>
-      <c r="V18" s="2">
+      <c r="V18" s="1">
         <v>46107</v>
       </c>
     </row>
@@ -1924,7 +1898,7 @@
       <c r="G19" t="s">
         <v>106</v>
       </c>
-      <c r="H19" s="2">
+      <c r="H19" s="1">
         <v>46076</v>
       </c>
       <c r="I19" t="s">
@@ -1954,7 +1928,7 @@
       <c r="U19" t="s">
         <v>91</v>
       </c>
-      <c r="V19" s="2">
+      <c r="V19" s="1">
         <v>46079</v>
       </c>
     </row>
@@ -1980,7 +1954,7 @@
       <c r="G20" t="s">
         <v>106</v>
       </c>
-      <c r="H20" s="2">
+      <c r="H20" s="1">
         <v>46076</v>
       </c>
       <c r="I20" t="s">
@@ -2010,7 +1984,7 @@
       <c r="U20" t="s">
         <v>91</v>
       </c>
-      <c r="V20" s="2">
+      <c r="V20" s="1">
         <v>46079</v>
       </c>
     </row>
@@ -2057,7 +2031,7 @@
       <c r="U21" t="s">
         <v>91</v>
       </c>
-      <c r="V21" s="2">
+      <c r="V21" s="1">
         <v>46321</v>
       </c>
     </row>
@@ -2104,7 +2078,7 @@
       <c r="U22" t="s">
         <v>91</v>
       </c>
-      <c r="V22" s="2">
+      <c r="V22" s="1">
         <v>46321</v>
       </c>
     </row>
@@ -2151,7 +2125,7 @@
       <c r="U23" t="s">
         <v>91</v>
       </c>
-      <c r="V23" s="2">
+      <c r="V23" s="1">
         <v>46321</v>
       </c>
     </row>
@@ -2198,7 +2172,7 @@
       <c r="U24" t="s">
         <v>91</v>
       </c>
-      <c r="V24" s="2">
+      <c r="V24" s="1">
         <v>46321</v>
       </c>
     </row>
@@ -2224,7 +2198,7 @@
       <c r="G25" t="s">
         <v>106</v>
       </c>
-      <c r="H25" s="2">
+      <c r="H25" s="1">
         <v>46119</v>
       </c>
       <c r="I25" t="s">
@@ -2257,7 +2231,7 @@
       <c r="U25" t="s">
         <v>178</v>
       </c>
-      <c r="V25" s="2">
+      <c r="V25" s="1">
         <v>46138</v>
       </c>
     </row>
@@ -2283,7 +2257,7 @@
       <c r="G26" t="s">
         <v>106</v>
       </c>
-      <c r="H26" s="2">
+      <c r="H26" s="1">
         <v>46121</v>
       </c>
       <c r="I26" t="s">
@@ -2313,7 +2287,7 @@
       <c r="U26" t="s">
         <v>91</v>
       </c>
-      <c r="V26" s="2">
+      <c r="V26" s="1">
         <v>46138</v>
       </c>
     </row>
@@ -2339,7 +2313,7 @@
       <c r="G27" t="s">
         <v>106</v>
       </c>
-      <c r="H27" s="2">
+      <c r="H27" s="1">
         <v>46076</v>
       </c>
       <c r="I27" t="s">
@@ -2369,7 +2343,7 @@
       <c r="U27" t="s">
         <v>91</v>
       </c>
-      <c r="V27" s="2">
+      <c r="V27" s="1">
         <v>46079</v>
       </c>
     </row>
@@ -2395,7 +2369,7 @@
       <c r="G28" t="s">
         <v>106</v>
       </c>
-      <c r="H28" s="2">
+      <c r="H28" s="1">
         <v>46303</v>
       </c>
       <c r="I28" t="s">
@@ -2431,7 +2405,7 @@
       <c r="U28" t="s">
         <v>178</v>
       </c>
-      <c r="V28" s="2">
+      <c r="V28" s="1">
         <v>46291</v>
       </c>
     </row>
@@ -2457,7 +2431,7 @@
       <c r="G29" t="s">
         <v>106</v>
       </c>
-      <c r="H29" s="2">
+      <c r="H29" s="1">
         <v>46199</v>
       </c>
       <c r="I29" t="s">
@@ -2490,7 +2464,7 @@
       <c r="U29" t="s">
         <v>178</v>
       </c>
-      <c r="V29" s="2">
+      <c r="V29" s="1">
         <v>46199</v>
       </c>
     </row>
@@ -2516,7 +2490,7 @@
       <c r="G30" t="s">
         <v>106</v>
       </c>
-      <c r="H30" s="2">
+      <c r="H30" s="1">
         <v>46199</v>
       </c>
       <c r="I30" t="s">
@@ -2549,7 +2523,7 @@
       <c r="U30" t="s">
         <v>178</v>
       </c>
-      <c r="V30" s="2">
+      <c r="V30" s="1">
         <v>46199</v>
       </c>
     </row>
@@ -2575,7 +2549,7 @@
       <c r="G31" t="s">
         <v>106</v>
       </c>
-      <c r="H31" s="2">
+      <c r="H31" s="1">
         <v>46199</v>
       </c>
       <c r="I31" t="s">
@@ -2608,7 +2582,7 @@
       <c r="U31" t="s">
         <v>178</v>
       </c>
-      <c r="V31" s="2">
+      <c r="V31" s="1">
         <v>46199</v>
       </c>
     </row>
@@ -2634,7 +2608,7 @@
       <c r="G32" t="s">
         <v>106</v>
       </c>
-      <c r="H32" s="2">
+      <c r="H32" s="1">
         <v>46199</v>
       </c>
       <c r="I32" t="s">
@@ -2667,7 +2641,7 @@
       <c r="U32" t="s">
         <v>178</v>
       </c>
-      <c r="V32" s="2">
+      <c r="V32" s="1">
         <v>46199</v>
       </c>
     </row>
@@ -2720,7 +2694,7 @@
       <c r="U33" t="s">
         <v>178</v>
       </c>
-      <c r="V33" s="2">
+      <c r="V33" s="1">
         <v>46291</v>
       </c>
     </row>
@@ -2746,7 +2720,7 @@
       <c r="G34" t="s">
         <v>106</v>
       </c>
-      <c r="H34" s="2">
+      <c r="H34" s="1">
         <v>46191</v>
       </c>
       <c r="I34" t="s">
@@ -2779,7 +2753,7 @@
       <c r="U34" t="s">
         <v>178</v>
       </c>
-      <c r="V34" s="2">
+      <c r="V34" s="1">
         <v>46199</v>
       </c>
     </row>
@@ -2805,7 +2779,7 @@
       <c r="G35" t="s">
         <v>106</v>
       </c>
-      <c r="H35" s="2">
+      <c r="H35" s="1">
         <v>46119</v>
       </c>
       <c r="I35" t="s">
@@ -2835,7 +2809,7 @@
       <c r="U35" t="s">
         <v>178</v>
       </c>
-      <c r="V35" s="2">
+      <c r="V35" s="1">
         <v>46138</v>
       </c>
     </row>
@@ -2861,7 +2835,7 @@
       <c r="G36" t="s">
         <v>106</v>
       </c>
-      <c r="H36" s="2">
+      <c r="H36" s="1">
         <v>46213</v>
       </c>
       <c r="I36" t="s">
@@ -2891,7 +2865,7 @@
       <c r="U36" t="s">
         <v>91</v>
       </c>
-      <c r="V36" s="2">
+      <c r="V36" s="1">
         <v>46229</v>
       </c>
     </row>
@@ -2917,7 +2891,7 @@
       <c r="G37" t="s">
         <v>106</v>
       </c>
-      <c r="H37" s="2">
+      <c r="H37" s="1">
         <v>46175</v>
       </c>
       <c r="I37" t="s">
@@ -2947,7 +2921,7 @@
       <c r="U37" t="s">
         <v>91</v>
       </c>
-      <c r="V37" s="2">
+      <c r="V37" s="1">
         <v>46199</v>
       </c>
     </row>
@@ -2973,7 +2947,7 @@
       <c r="G38" t="s">
         <v>106</v>
       </c>
-      <c r="H38" s="2">
+      <c r="H38" s="1">
         <v>46213</v>
       </c>
       <c r="I38" t="s">
@@ -3003,7 +2977,7 @@
       <c r="U38" t="s">
         <v>91</v>
       </c>
-      <c r="V38" s="2">
+      <c r="V38" s="1">
         <v>46229</v>
       </c>
     </row>
@@ -3029,7 +3003,7 @@
       <c r="G39" t="s">
         <v>106</v>
       </c>
-      <c r="H39" s="2">
+      <c r="H39" s="1">
         <v>46199</v>
       </c>
       <c r="I39" t="s">
@@ -3059,7 +3033,7 @@
       <c r="U39" t="s">
         <v>91</v>
       </c>
-      <c r="V39" s="2">
+      <c r="V39" s="1">
         <v>46199</v>
       </c>
     </row>
@@ -3085,7 +3059,7 @@
       <c r="G40" t="s">
         <v>106</v>
       </c>
-      <c r="H40" s="2">
+      <c r="H40" s="1">
         <v>46199</v>
       </c>
       <c r="I40" t="s">
@@ -3115,7 +3089,7 @@
       <c r="U40" t="s">
         <v>91</v>
       </c>
-      <c r="V40" s="2">
+      <c r="V40" s="1">
         <v>46199</v>
       </c>
     </row>
@@ -3141,7 +3115,7 @@
       <c r="G41" t="s">
         <v>106</v>
       </c>
-      <c r="H41" s="2">
+      <c r="H41" s="1">
         <v>46204</v>
       </c>
       <c r="I41" t="s">
@@ -3171,7 +3145,7 @@
       <c r="U41" t="s">
         <v>91</v>
       </c>
-      <c r="V41" s="2">
+      <c r="V41" s="1">
         <v>46229</v>
       </c>
     </row>
@@ -3197,7 +3171,7 @@
       <c r="G42" t="s">
         <v>106</v>
       </c>
-      <c r="H42" s="2">
+      <c r="H42" s="1">
         <v>46244</v>
       </c>
       <c r="I42" t="s">
@@ -3227,7 +3201,7 @@
       <c r="U42" t="s">
         <v>91</v>
       </c>
-      <c r="V42" s="2">
+      <c r="V42" s="1">
         <v>46199</v>
       </c>
     </row>
@@ -3271,7 +3245,7 @@
       <c r="U43" t="s">
         <v>91</v>
       </c>
-      <c r="V43" s="2">
+      <c r="V43" s="1">
         <v>46260</v>
       </c>
     </row>
@@ -3297,7 +3271,7 @@
       <c r="G44" t="s">
         <v>106</v>
       </c>
-      <c r="H44" s="2">
+      <c r="H44" s="1">
         <v>46191</v>
       </c>
       <c r="I44" t="s">
@@ -3327,7 +3301,7 @@
       <c r="U44" t="s">
         <v>91</v>
       </c>
-      <c r="V44" s="2">
+      <c r="V44" s="1">
         <v>46199</v>
       </c>
     </row>
@@ -3353,7 +3327,7 @@
       <c r="G45" t="s">
         <v>106</v>
       </c>
-      <c r="H45" s="2">
+      <c r="H45" s="1">
         <v>46191</v>
       </c>
       <c r="I45" t="s">
@@ -3383,7 +3357,7 @@
       <c r="U45" t="s">
         <v>91</v>
       </c>
-      <c r="V45" s="2">
+      <c r="V45" s="1">
         <v>46199</v>
       </c>
     </row>
@@ -3409,7 +3383,7 @@
       <c r="G46" t="s">
         <v>106</v>
       </c>
-      <c r="H46" s="2">
+      <c r="H46" s="1">
         <v>46213</v>
       </c>
       <c r="I46" t="s">
@@ -3442,7 +3416,7 @@
       <c r="U46" t="s">
         <v>178</v>
       </c>
-      <c r="V46" s="2">
+      <c r="V46" s="1">
         <v>46229</v>
       </c>
     </row>
@@ -3468,7 +3442,7 @@
       <c r="G47" t="s">
         <v>106</v>
       </c>
-      <c r="H47" s="2">
+      <c r="H47" s="1">
         <v>46210</v>
       </c>
       <c r="I47" t="s">
@@ -3498,7 +3472,7 @@
       <c r="U47" t="s">
         <v>178</v>
       </c>
-      <c r="V47" s="2">
+      <c r="V47" s="1">
         <v>46229</v>
       </c>
     </row>
@@ -3545,7 +3519,7 @@
       <c r="U48" t="s">
         <v>91</v>
       </c>
-      <c r="V48" s="2">
+      <c r="V48" s="1">
         <v>46321</v>
       </c>
     </row>
@@ -3571,7 +3545,7 @@
       <c r="G49" t="s">
         <v>106</v>
       </c>
-      <c r="H49" s="2">
+      <c r="H49" s="1">
         <v>46303</v>
       </c>
       <c r="I49" t="s">
@@ -3607,7 +3581,7 @@
       <c r="U49" t="s">
         <v>178</v>
       </c>
-      <c r="V49" s="2">
+      <c r="V49" s="1">
         <v>46291</v>
       </c>
     </row>
@@ -3633,7 +3607,7 @@
       <c r="G50" t="s">
         <v>106</v>
       </c>
-      <c r="H50" s="2">
+      <c r="H50" s="1">
         <v>46176</v>
       </c>
       <c r="I50" t="s">
@@ -3666,7 +3640,7 @@
       <c r="U50" t="s">
         <v>178</v>
       </c>
-      <c r="V50" s="2">
+      <c r="V50" s="1">
         <v>46199</v>
       </c>
     </row>
@@ -3692,7 +3666,7 @@
       <c r="G51" t="s">
         <v>106</v>
       </c>
-      <c r="H51" s="2">
+      <c r="H51" s="1">
         <v>46314</v>
       </c>
       <c r="I51" t="s">
@@ -3728,7 +3702,7 @@
       <c r="U51" t="s">
         <v>178</v>
       </c>
-      <c r="V51" s="2">
+      <c r="V51" s="1">
         <v>46260</v>
       </c>
     </row>
@@ -3754,7 +3728,7 @@
       <c r="G52" t="s">
         <v>106</v>
       </c>
-      <c r="H52" s="2">
+      <c r="H52" s="1">
         <v>46295</v>
       </c>
       <c r="I52" t="s">
@@ -3790,7 +3764,7 @@
       <c r="U52" t="s">
         <v>178</v>
       </c>
-      <c r="V52" s="2">
+      <c r="V52" s="1">
         <v>46291</v>
       </c>
     </row>
@@ -3843,7 +3817,7 @@
       <c r="U53" t="s">
         <v>178</v>
       </c>
-      <c r="V53" s="2">
+      <c r="V53" s="1">
         <v>46321</v>
       </c>
     </row>
@@ -3869,7 +3843,7 @@
       <c r="G54" t="s">
         <v>106</v>
       </c>
-      <c r="H54" s="2">
+      <c r="H54" s="1">
         <v>46227</v>
       </c>
       <c r="I54" t="s">
@@ -3899,7 +3873,7 @@
       <c r="U54" t="s">
         <v>178</v>
       </c>
-      <c r="V54" s="2">
+      <c r="V54" s="1">
         <v>46229</v>
       </c>
     </row>
@@ -3922,7 +3896,7 @@
       <c r="G55" t="s">
         <v>106</v>
       </c>
-      <c r="H55" s="2">
+      <c r="H55" s="1">
         <v>46280</v>
       </c>
       <c r="I55" t="s">
@@ -3952,7 +3926,7 @@
       <c r="U55" t="s">
         <v>178</v>
       </c>
-      <c r="V55" s="2">
+      <c r="V55" s="1">
         <v>46291</v>
       </c>
     </row>
@@ -3975,7 +3949,7 @@
       <c r="G56" t="s">
         <v>106</v>
       </c>
-      <c r="H56" s="2">
+      <c r="H56" s="1">
         <v>46280</v>
       </c>
       <c r="I56" t="s">
@@ -4005,7 +3979,7 @@
       <c r="U56" t="s">
         <v>178</v>
       </c>
-      <c r="V56" s="2">
+      <c r="V56" s="1">
         <v>46260</v>
       </c>
     </row>
@@ -4028,7 +4002,7 @@
       <c r="G57" t="s">
         <v>106</v>
       </c>
-      <c r="H57" s="2">
+      <c r="H57" s="1">
         <v>46295</v>
       </c>
       <c r="I57" t="s">
@@ -4058,7 +4032,7 @@
       <c r="U57" t="s">
         <v>178</v>
       </c>
-      <c r="V57" s="2">
+      <c r="V57" s="1">
         <v>46291</v>
       </c>
     </row>
@@ -4081,7 +4055,7 @@
       <c r="G58" t="s">
         <v>106</v>
       </c>
-      <c r="H58" s="2">
+      <c r="H58" s="1">
         <v>46295</v>
       </c>
       <c r="I58" t="s">
@@ -4111,7 +4085,7 @@
       <c r="U58" t="s">
         <v>178</v>
       </c>
-      <c r="V58" s="2">
+      <c r="V58" s="1">
         <v>46291</v>
       </c>
     </row>
@@ -4134,7 +4108,7 @@
       <c r="G59" t="s">
         <v>106</v>
       </c>
-      <c r="H59" s="2">
+      <c r="H59" s="1">
         <v>46304</v>
       </c>
       <c r="I59" t="s">
@@ -4164,7 +4138,7 @@
       <c r="U59" t="s">
         <v>178</v>
       </c>
-      <c r="V59" s="2">
+      <c r="V59" s="1">
         <v>46321</v>
       </c>
     </row>
@@ -4190,7 +4164,7 @@
       <c r="G60" t="s">
         <v>106</v>
       </c>
-      <c r="H60" s="2">
+      <c r="H60" s="1">
         <v>46301</v>
       </c>
       <c r="I60" t="s">
@@ -4226,7 +4200,7 @@
       <c r="U60" t="s">
         <v>178</v>
       </c>
-      <c r="V60" s="2">
+      <c r="V60" s="1">
         <v>46352</v>
       </c>
     </row>
@@ -4270,7 +4244,7 @@
       <c r="U61" t="s">
         <v>178</v>
       </c>
-      <c r="V61" s="2">
+      <c r="V61" s="1">
         <v>46107</v>
       </c>
     </row>
@@ -4314,7 +4288,7 @@
       <c r="U62" t="s">
         <v>178</v>
       </c>
-      <c r="V62" s="2">
+      <c r="V62" s="1">
         <v>46107</v>
       </c>
     </row>
@@ -4358,7 +4332,7 @@
       <c r="U63" t="s">
         <v>178</v>
       </c>
-      <c r="V63" s="2">
+      <c r="V63" s="1">
         <v>46107</v>
       </c>
     </row>
@@ -4402,7 +4376,7 @@
       <c r="U64" t="s">
         <v>178</v>
       </c>
-      <c r="V64" s="2">
+      <c r="V64" s="1">
         <v>46107</v>
       </c>
     </row>
@@ -4446,7 +4420,7 @@
       <c r="U65" t="s">
         <v>178</v>
       </c>
-      <c r="V65" s="2">
+      <c r="V65" s="1">
         <v>46107</v>
       </c>
     </row>
@@ -4490,7 +4464,7 @@
       <c r="U66" t="s">
         <v>178</v>
       </c>
-      <c r="V66" s="2">
+      <c r="V66" s="1">
         <v>46107</v>
       </c>
     </row>
@@ -4534,7 +4508,7 @@
       <c r="U67" t="s">
         <v>91</v>
       </c>
-      <c r="V67" s="2">
+      <c r="V67" s="1">
         <v>46168</v>
       </c>
     </row>
@@ -4581,7 +4555,7 @@
       <c r="U68" t="s">
         <v>91</v>
       </c>
-      <c r="V68" s="2">
+      <c r="V68" s="1">
         <v>46291</v>
       </c>
     </row>
@@ -4607,7 +4581,7 @@
       <c r="G69" t="s">
         <v>106</v>
       </c>
-      <c r="H69" s="2">
+      <c r="H69" s="1">
         <v>46303</v>
       </c>
       <c r="I69" t="s">
@@ -4643,7 +4617,7 @@
       <c r="U69" t="s">
         <v>178</v>
       </c>
-      <c r="V69" s="2">
+      <c r="V69" s="1">
         <v>46229</v>
       </c>
     </row>
@@ -4687,7 +4661,7 @@
       <c r="U70" t="s">
         <v>91</v>
       </c>
-      <c r="V70" s="2">
+      <c r="V70" s="1">
         <v>46260</v>
       </c>
     </row>
@@ -4731,7 +4705,7 @@
       <c r="U71" t="s">
         <v>178</v>
       </c>
-      <c r="V71" s="2">
+      <c r="V71" s="1">
         <v>46291</v>
       </c>
     </row>
@@ -4775,7 +4749,7 @@
       <c r="U72" t="s">
         <v>178</v>
       </c>
-      <c r="V72" s="2">
+      <c r="V72" s="1">
         <v>46168</v>
       </c>
     </row>
@@ -4819,7 +4793,7 @@
       <c r="U73" t="s">
         <v>178</v>
       </c>
-      <c r="V73" s="2">
+      <c r="V73" s="1">
         <v>46291</v>
       </c>
     </row>
@@ -4863,7 +4837,7 @@
       <c r="U74" t="s">
         <v>178</v>
       </c>
-      <c r="V74" s="2">
+      <c r="V74" s="1">
         <v>46291</v>
       </c>
     </row>
@@ -4907,7 +4881,7 @@
       <c r="U75" t="s">
         <v>178</v>
       </c>
-      <c r="V75" s="2">
+      <c r="V75" s="1">
         <v>46291</v>
       </c>
     </row>
@@ -4954,7 +4928,7 @@
       <c r="U76" t="s">
         <v>91</v>
       </c>
-      <c r="V76" s="2">
+      <c r="V76" s="1">
         <v>46321</v>
       </c>
     </row>
@@ -5004,7 +4978,7 @@
       <c r="U77" t="s">
         <v>178</v>
       </c>
-      <c r="V77" s="2">
+      <c r="V77" s="1">
         <v>46381</v>
       </c>
     </row>
@@ -5054,7 +5028,7 @@
       <c r="U78" t="s">
         <v>178</v>
       </c>
-      <c r="V78" s="2">
+      <c r="V78" s="1">
         <v>46381</v>
       </c>
     </row>
@@ -5104,7 +5078,7 @@
       <c r="U79" t="s">
         <v>91</v>
       </c>
-      <c r="V79" s="2">
+      <c r="V79" s="1">
         <v>46381</v>
       </c>
     </row>
@@ -5154,7 +5128,7 @@
       <c r="U80" t="s">
         <v>91</v>
       </c>
-      <c r="V80" s="2">
+      <c r="V80" s="1">
         <v>46381</v>
       </c>
     </row>
@@ -5204,7 +5178,7 @@
       <c r="U81" t="s">
         <v>91</v>
       </c>
-      <c r="V81" s="2">
+      <c r="V81" s="1">
         <v>46382</v>
       </c>
     </row>
@@ -5248,7 +5222,7 @@
       <c r="U82" t="s">
         <v>91</v>
       </c>
-      <c r="V82" s="2">
+      <c r="V82" s="1">
         <v>46382</v>
       </c>
     </row>
@@ -5274,7 +5248,7 @@
       <c r="G83" t="s">
         <v>106</v>
       </c>
-      <c r="H83" s="2">
+      <c r="H83" s="1">
         <v>46314</v>
       </c>
       <c r="I83" t="s">
@@ -5310,7 +5284,7 @@
       <c r="U83" t="s">
         <v>178</v>
       </c>
-      <c r="V83" s="2">
+      <c r="V83" s="1">
         <v>46382</v>
       </c>
     </row>
@@ -5360,7 +5334,7 @@
       <c r="U84" t="s">
         <v>91</v>
       </c>
-      <c r="V84" s="2">
+      <c r="V84" s="1">
         <v>46321</v>
       </c>
     </row>
@@ -5404,7 +5378,7 @@
       <c r="U85" t="s">
         <v>91</v>
       </c>
-      <c r="V85" s="2">
+      <c r="V85" s="1">
         <v>46382</v>
       </c>
     </row>
@@ -5524,7 +5498,7 @@
       <c r="G88" t="s">
         <v>106</v>
       </c>
-      <c r="H88" s="2">
+      <c r="H88" s="1">
         <v>46303</v>
       </c>
       <c r="I88" t="s">
@@ -5554,7 +5528,7 @@
       <c r="U88" t="s">
         <v>91</v>
       </c>
-      <c r="V88" s="2">
+      <c r="V88" s="1">
         <v>46291</v>
       </c>
     </row>
@@ -5601,7 +5575,7 @@
       <c r="U89" t="s">
         <v>91</v>
       </c>
-      <c r="V89" s="2">
+      <c r="V89" s="1">
         <v>46291</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Atualização automática: mta (27/10/2026 13:26)
</commit_message>
<xml_diff>
--- a/Projetos/02_Dados_Tratados/base_mta_tratada.xlsx
+++ b/Projetos/02_Dados_Tratados/base_mta_tratada.xlsx
@@ -14,7 +14,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1208" uniqueCount="179">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1202" uniqueCount="177">
   <si>
     <t>linha</t>
   </si>
@@ -439,22 +439,16 @@
     <t>e-mail 12/08</t>
   </si>
   <si>
-    <t>Atender</t>
-  </si>
-  <si>
-    <t>ATENDER CABW 30</t>
+    <t>Agd Cp Camacho checar processo</t>
   </si>
   <si>
     <t>Atender. Alterar a UGE para CABW. Alterar a atividade para "Requisição CABW". Alterar a tarefa para "Requisições Consumíveis". Alterar a ND para 339030.</t>
   </si>
   <si>
-    <t>Atender SET</t>
-  </si>
-  <si>
-    <t>Atender NOV</t>
-  </si>
-  <si>
     <t>ATENDER com 20XV</t>
+  </si>
+  <si>
+    <t>Remanejar</t>
   </si>
   <si>
     <t>LIVRE</t>
@@ -988,14 +982,11 @@
       <c r="J2" t="s">
         <v>132</v>
       </c>
-      <c r="K2" t="s">
-        <v>141</v>
-      </c>
       <c r="L2" t="s">
-        <v>147</v>
+        <v>145</v>
       </c>
       <c r="N2" t="s">
-        <v>148</v>
+        <v>146</v>
       </c>
       <c r="O2" t="s">
         <v>23</v>
@@ -1004,19 +995,19 @@
         <v>135000</v>
       </c>
       <c r="Q2" t="s">
-        <v>166</v>
+        <v>164</v>
       </c>
       <c r="R2" t="s">
-        <v>169</v>
+        <v>167</v>
       </c>
       <c r="S2" t="s">
+        <v>170</v>
+      </c>
+      <c r="T2" t="s">
         <v>172</v>
       </c>
-      <c r="T2" t="s">
-        <v>174</v>
-      </c>
       <c r="U2" t="s">
-        <v>178</v>
+        <v>176</v>
       </c>
       <c r="V2" s="1">
         <v>46229</v>
@@ -1045,22 +1036,22 @@
         <v>107</v>
       </c>
       <c r="N3" t="s">
-        <v>148</v>
+        <v>146</v>
       </c>
       <c r="O3" t="s">
         <v>24</v>
       </c>
       <c r="Q3" t="s">
-        <v>166</v>
+        <v>164</v>
       </c>
       <c r="R3" t="s">
-        <v>169</v>
+        <v>167</v>
       </c>
       <c r="S3" t="s">
+        <v>170</v>
+      </c>
+      <c r="T3" t="s">
         <v>172</v>
-      </c>
-      <c r="T3" t="s">
-        <v>174</v>
       </c>
       <c r="U3" t="s">
         <v>91</v>
@@ -1092,22 +1083,22 @@
         <v>107</v>
       </c>
       <c r="N4" t="s">
-        <v>149</v>
+        <v>147</v>
       </c>
       <c r="O4" t="s">
         <v>25</v>
       </c>
       <c r="Q4" t="s">
-        <v>166</v>
+        <v>164</v>
       </c>
       <c r="R4" t="s">
-        <v>170</v>
+        <v>168</v>
       </c>
       <c r="S4" t="s">
+        <v>170</v>
+      </c>
+      <c r="T4" t="s">
         <v>172</v>
-      </c>
-      <c r="T4" t="s">
-        <v>174</v>
       </c>
       <c r="U4" t="s">
         <v>91</v>
@@ -1139,22 +1130,22 @@
         <v>107</v>
       </c>
       <c r="N5" t="s">
-        <v>149</v>
+        <v>147</v>
       </c>
       <c r="O5" t="s">
         <v>26</v>
       </c>
       <c r="Q5" t="s">
-        <v>166</v>
+        <v>164</v>
       </c>
       <c r="R5" t="s">
-        <v>170</v>
+        <v>168</v>
       </c>
       <c r="S5" t="s">
+        <v>170</v>
+      </c>
+      <c r="T5" t="s">
         <v>172</v>
-      </c>
-      <c r="T5" t="s">
-        <v>174</v>
       </c>
       <c r="U5" t="s">
         <v>91</v>
@@ -1186,25 +1177,25 @@
         <v>107</v>
       </c>
       <c r="L6" t="s">
-        <v>147</v>
+        <v>145</v>
       </c>
       <c r="N6" t="s">
-        <v>150</v>
+        <v>148</v>
       </c>
       <c r="O6" t="s">
         <v>27</v>
       </c>
       <c r="Q6" t="s">
-        <v>166</v>
+        <v>164</v>
       </c>
       <c r="R6" t="s">
-        <v>170</v>
+        <v>168</v>
       </c>
       <c r="S6" t="s">
+        <v>170</v>
+      </c>
+      <c r="T6" t="s">
         <v>172</v>
-      </c>
-      <c r="T6" t="s">
-        <v>174</v>
       </c>
       <c r="U6" t="s">
         <v>91</v>
@@ -1242,7 +1233,7 @@
         <v>111</v>
       </c>
       <c r="N7" t="s">
-        <v>151</v>
+        <v>149</v>
       </c>
       <c r="O7" t="s">
         <v>28</v>
@@ -1251,16 +1242,16 @@
         <v>3799999.6</v>
       </c>
       <c r="Q7" t="s">
-        <v>167</v>
+        <v>165</v>
       </c>
       <c r="R7" t="s">
-        <v>170</v>
+        <v>168</v>
       </c>
       <c r="S7" t="s">
-        <v>172</v>
+        <v>170</v>
       </c>
       <c r="T7" t="s">
-        <v>175</v>
+        <v>173</v>
       </c>
       <c r="U7" t="s">
         <v>91</v>
@@ -1292,22 +1283,22 @@
         <v>107</v>
       </c>
       <c r="N8" t="s">
-        <v>149</v>
+        <v>147</v>
       </c>
       <c r="O8" t="s">
         <v>29</v>
       </c>
       <c r="Q8" t="s">
-        <v>166</v>
+        <v>164</v>
       </c>
       <c r="R8" t="s">
-        <v>170</v>
+        <v>168</v>
       </c>
       <c r="S8" t="s">
+        <v>170</v>
+      </c>
+      <c r="T8" t="s">
         <v>172</v>
-      </c>
-      <c r="T8" t="s">
-        <v>174</v>
       </c>
       <c r="U8" t="s">
         <v>91</v>
@@ -1336,7 +1327,7 @@
         <v>93</v>
       </c>
       <c r="N9" t="s">
-        <v>149</v>
+        <v>147</v>
       </c>
       <c r="O9" t="s">
         <v>30</v>
@@ -1345,16 +1336,16 @@
         <v>23895.54</v>
       </c>
       <c r="Q9" t="s">
-        <v>166</v>
+        <v>164</v>
       </c>
       <c r="R9" t="s">
-        <v>170</v>
+        <v>168</v>
       </c>
       <c r="S9" t="s">
+        <v>170</v>
+      </c>
+      <c r="T9" t="s">
         <v>172</v>
-      </c>
-      <c r="T9" t="s">
-        <v>174</v>
       </c>
       <c r="U9" t="s">
         <v>91</v>
@@ -1389,7 +1380,7 @@
         <v>112</v>
       </c>
       <c r="N10" t="s">
-        <v>149</v>
+        <v>147</v>
       </c>
       <c r="O10" t="s">
         <v>30</v>
@@ -1398,16 +1389,16 @@
         <v>23895.54</v>
       </c>
       <c r="Q10" t="s">
-        <v>166</v>
+        <v>164</v>
       </c>
       <c r="R10" t="s">
-        <v>170</v>
+        <v>168</v>
       </c>
       <c r="S10" t="s">
+        <v>170</v>
+      </c>
+      <c r="T10" t="s">
         <v>172</v>
-      </c>
-      <c r="T10" t="s">
-        <v>174</v>
       </c>
       <c r="U10" t="s">
         <v>91</v>
@@ -1439,22 +1430,22 @@
         <v>107</v>
       </c>
       <c r="N11" t="s">
-        <v>150</v>
+        <v>148</v>
       </c>
       <c r="O11" t="s">
         <v>31</v>
       </c>
       <c r="Q11" t="s">
-        <v>166</v>
+        <v>164</v>
       </c>
       <c r="R11" t="s">
-        <v>170</v>
+        <v>168</v>
       </c>
       <c r="S11" t="s">
+        <v>170</v>
+      </c>
+      <c r="T11" t="s">
         <v>172</v>
-      </c>
-      <c r="T11" t="s">
-        <v>174</v>
       </c>
       <c r="U11" t="s">
         <v>91</v>
@@ -1486,22 +1477,22 @@
         <v>107</v>
       </c>
       <c r="N12" t="s">
-        <v>150</v>
+        <v>148</v>
       </c>
       <c r="O12" t="s">
         <v>32</v>
       </c>
       <c r="Q12" t="s">
-        <v>166</v>
+        <v>164</v>
       </c>
       <c r="R12" t="s">
-        <v>170</v>
+        <v>168</v>
       </c>
       <c r="S12" t="s">
+        <v>170</v>
+      </c>
+      <c r="T12" t="s">
         <v>172</v>
-      </c>
-      <c r="T12" t="s">
-        <v>174</v>
       </c>
       <c r="U12" t="s">
         <v>91</v>
@@ -1542,7 +1533,7 @@
         <v>133</v>
       </c>
       <c r="N13" t="s">
-        <v>148</v>
+        <v>146</v>
       </c>
       <c r="O13" t="s">
         <v>33</v>
@@ -1551,19 +1542,19 @@
         <v>1187433.02</v>
       </c>
       <c r="Q13" t="s">
-        <v>166</v>
+        <v>164</v>
       </c>
       <c r="R13" t="s">
-        <v>169</v>
+        <v>167</v>
       </c>
       <c r="S13" t="s">
+        <v>170</v>
+      </c>
+      <c r="T13" t="s">
         <v>172</v>
       </c>
-      <c r="T13" t="s">
-        <v>174</v>
-      </c>
       <c r="U13" t="s">
-        <v>178</v>
+        <v>176</v>
       </c>
       <c r="V13" s="1">
         <v>46079</v>
@@ -1600,11 +1591,8 @@
       <c r="J14" t="s">
         <v>132</v>
       </c>
-      <c r="K14" t="s">
-        <v>109</v>
-      </c>
       <c r="N14" t="s">
-        <v>148</v>
+        <v>146</v>
       </c>
       <c r="O14" t="s">
         <v>34</v>
@@ -1613,19 +1601,19 @@
         <v>1000000</v>
       </c>
       <c r="Q14" t="s">
-        <v>166</v>
+        <v>164</v>
       </c>
       <c r="R14" t="s">
-        <v>169</v>
+        <v>167</v>
       </c>
       <c r="S14" t="s">
+        <v>170</v>
+      </c>
+      <c r="T14" t="s">
         <v>172</v>
       </c>
-      <c r="T14" t="s">
-        <v>174</v>
-      </c>
       <c r="U14" t="s">
-        <v>178</v>
+        <v>176</v>
       </c>
       <c r="V14" s="1">
         <v>46352</v>
@@ -1662,11 +1650,8 @@
       <c r="J15" t="s">
         <v>132</v>
       </c>
-      <c r="K15" t="s">
-        <v>109</v>
-      </c>
       <c r="N15" t="s">
-        <v>148</v>
+        <v>146</v>
       </c>
       <c r="O15" t="s">
         <v>35</v>
@@ -1675,19 +1660,19 @@
         <v>1000000</v>
       </c>
       <c r="Q15" t="s">
-        <v>166</v>
+        <v>164</v>
       </c>
       <c r="R15" t="s">
-        <v>169</v>
+        <v>167</v>
       </c>
       <c r="S15" t="s">
+        <v>170</v>
+      </c>
+      <c r="T15" t="s">
         <v>172</v>
       </c>
-      <c r="T15" t="s">
-        <v>174</v>
-      </c>
       <c r="U15" t="s">
-        <v>178</v>
+        <v>176</v>
       </c>
       <c r="V15" s="1">
         <v>46352</v>
@@ -1724,11 +1709,8 @@
       <c r="J16" t="s">
         <v>132</v>
       </c>
-      <c r="K16" t="s">
-        <v>109</v>
-      </c>
       <c r="N16" t="s">
-        <v>148</v>
+        <v>146</v>
       </c>
       <c r="O16" t="s">
         <v>36</v>
@@ -1737,19 +1719,19 @@
         <v>1000000</v>
       </c>
       <c r="Q16" t="s">
-        <v>166</v>
+        <v>164</v>
       </c>
       <c r="R16" t="s">
-        <v>169</v>
+        <v>167</v>
       </c>
       <c r="S16" t="s">
+        <v>170</v>
+      </c>
+      <c r="T16" t="s">
         <v>172</v>
       </c>
-      <c r="T16" t="s">
-        <v>174</v>
-      </c>
       <c r="U16" t="s">
-        <v>178</v>
+        <v>176</v>
       </c>
       <c r="V16" s="1">
         <v>46352</v>
@@ -1786,11 +1768,8 @@
       <c r="J17" t="s">
         <v>132</v>
       </c>
-      <c r="K17" t="s">
-        <v>109</v>
-      </c>
       <c r="N17" t="s">
-        <v>148</v>
+        <v>146</v>
       </c>
       <c r="O17" t="s">
         <v>37</v>
@@ -1799,19 +1778,19 @@
         <v>100000</v>
       </c>
       <c r="Q17" t="s">
-        <v>166</v>
+        <v>164</v>
       </c>
       <c r="R17" t="s">
-        <v>169</v>
+        <v>167</v>
       </c>
       <c r="S17" t="s">
+        <v>170</v>
+      </c>
+      <c r="T17" t="s">
         <v>172</v>
       </c>
-      <c r="T17" t="s">
-        <v>174</v>
-      </c>
       <c r="U17" t="s">
-        <v>178</v>
+        <v>176</v>
       </c>
       <c r="V17" s="1">
         <v>46229</v>
@@ -1849,7 +1828,7 @@
         <v>133</v>
       </c>
       <c r="N18" t="s">
-        <v>152</v>
+        <v>150</v>
       </c>
       <c r="O18" t="s">
         <v>38</v>
@@ -1858,19 +1837,19 @@
         <v>1770880.5</v>
       </c>
       <c r="Q18" t="s">
-        <v>167</v>
+        <v>165</v>
       </c>
       <c r="R18" t="s">
-        <v>170</v>
+        <v>168</v>
       </c>
       <c r="S18" t="s">
-        <v>172</v>
+        <v>170</v>
       </c>
       <c r="T18" t="s">
+        <v>174</v>
+      </c>
+      <c r="U18" t="s">
         <v>176</v>
-      </c>
-      <c r="U18" t="s">
-        <v>178</v>
       </c>
       <c r="V18" s="1">
         <v>46107</v>
@@ -1905,7 +1884,7 @@
         <v>115</v>
       </c>
       <c r="N19" t="s">
-        <v>153</v>
+        <v>151</v>
       </c>
       <c r="O19" t="s">
         <v>39</v>
@@ -1914,16 +1893,16 @@
         <v>350000</v>
       </c>
       <c r="Q19" t="s">
+        <v>165</v>
+      </c>
+      <c r="R19" t="s">
         <v>167</v>
       </c>
-      <c r="R19" t="s">
-        <v>169</v>
-      </c>
       <c r="S19" t="s">
-        <v>172</v>
+        <v>170</v>
       </c>
       <c r="T19" t="s">
-        <v>175</v>
+        <v>173</v>
       </c>
       <c r="U19" t="s">
         <v>91</v>
@@ -1961,7 +1940,7 @@
         <v>115</v>
       </c>
       <c r="N20" t="s">
-        <v>153</v>
+        <v>151</v>
       </c>
       <c r="O20" t="s">
         <v>40</v>
@@ -1970,16 +1949,16 @@
         <v>350000</v>
       </c>
       <c r="Q20" t="s">
+        <v>165</v>
+      </c>
+      <c r="R20" t="s">
         <v>167</v>
       </c>
-      <c r="R20" t="s">
-        <v>169</v>
-      </c>
       <c r="S20" t="s">
-        <v>172</v>
+        <v>170</v>
       </c>
       <c r="T20" t="s">
-        <v>175</v>
+        <v>173</v>
       </c>
       <c r="U20" t="s">
         <v>91</v>
@@ -2007,8 +1986,11 @@
       <c r="F21" t="s">
         <v>93</v>
       </c>
+      <c r="K21" t="s">
+        <v>141</v>
+      </c>
       <c r="N21" t="s">
-        <v>154</v>
+        <v>152</v>
       </c>
       <c r="O21" t="s">
         <v>41</v>
@@ -2017,16 +1999,16 @@
         <v>1000000</v>
       </c>
       <c r="Q21" t="s">
+        <v>165</v>
+      </c>
+      <c r="R21" t="s">
         <v>167</v>
       </c>
-      <c r="R21" t="s">
-        <v>169</v>
-      </c>
       <c r="S21" t="s">
-        <v>172</v>
+        <v>170</v>
       </c>
       <c r="T21" t="s">
-        <v>175</v>
+        <v>173</v>
       </c>
       <c r="U21" t="s">
         <v>91</v>
@@ -2058,22 +2040,22 @@
         <v>107</v>
       </c>
       <c r="N22" t="s">
-        <v>148</v>
+        <v>146</v>
       </c>
       <c r="O22" t="s">
         <v>42</v>
       </c>
       <c r="Q22" t="s">
-        <v>166</v>
+        <v>164</v>
       </c>
       <c r="R22" t="s">
-        <v>169</v>
+        <v>167</v>
       </c>
       <c r="S22" t="s">
+        <v>170</v>
+      </c>
+      <c r="T22" t="s">
         <v>172</v>
-      </c>
-      <c r="T22" t="s">
-        <v>174</v>
       </c>
       <c r="U22" t="s">
         <v>91</v>
@@ -2105,22 +2087,22 @@
         <v>107</v>
       </c>
       <c r="N23" t="s">
-        <v>149</v>
+        <v>147</v>
       </c>
       <c r="O23" t="s">
         <v>43</v>
       </c>
       <c r="Q23" t="s">
-        <v>166</v>
+        <v>164</v>
       </c>
       <c r="R23" t="s">
-        <v>170</v>
+        <v>168</v>
       </c>
       <c r="S23" t="s">
+        <v>170</v>
+      </c>
+      <c r="T23" t="s">
         <v>172</v>
-      </c>
-      <c r="T23" t="s">
-        <v>174</v>
       </c>
       <c r="U23" t="s">
         <v>91</v>
@@ -2152,22 +2134,22 @@
         <v>107</v>
       </c>
       <c r="N24" t="s">
-        <v>149</v>
+        <v>147</v>
       </c>
       <c r="O24" t="s">
         <v>44</v>
       </c>
       <c r="Q24" t="s">
-        <v>166</v>
+        <v>164</v>
       </c>
       <c r="R24" t="s">
-        <v>170</v>
+        <v>168</v>
       </c>
       <c r="S24" t="s">
+        <v>170</v>
+      </c>
+      <c r="T24" t="s">
         <v>172</v>
-      </c>
-      <c r="T24" t="s">
-        <v>174</v>
       </c>
       <c r="U24" t="s">
         <v>91</v>
@@ -2208,7 +2190,7 @@
         <v>134</v>
       </c>
       <c r="N25" t="s">
-        <v>152</v>
+        <v>150</v>
       </c>
       <c r="O25" t="s">
         <v>45</v>
@@ -2217,19 +2199,19 @@
         <v>1704503</v>
       </c>
       <c r="Q25" t="s">
-        <v>167</v>
+        <v>165</v>
       </c>
       <c r="R25" t="s">
-        <v>170</v>
+        <v>168</v>
       </c>
       <c r="S25" t="s">
-        <v>172</v>
+        <v>170</v>
       </c>
       <c r="T25" t="s">
+        <v>174</v>
+      </c>
+      <c r="U25" t="s">
         <v>176</v>
-      </c>
-      <c r="U25" t="s">
-        <v>178</v>
       </c>
       <c r="V25" s="1">
         <v>46138</v>
@@ -2264,7 +2246,7 @@
         <v>117</v>
       </c>
       <c r="N26" t="s">
-        <v>155</v>
+        <v>153</v>
       </c>
       <c r="O26" t="s">
         <v>46</v>
@@ -2273,16 +2255,16 @@
         <v>3799000</v>
       </c>
       <c r="Q26" t="s">
-        <v>167</v>
+        <v>165</v>
       </c>
       <c r="R26" t="s">
-        <v>170</v>
+        <v>168</v>
       </c>
       <c r="S26" t="s">
-        <v>172</v>
+        <v>170</v>
       </c>
       <c r="T26" t="s">
-        <v>175</v>
+        <v>173</v>
       </c>
       <c r="U26" t="s">
         <v>91</v>
@@ -2320,7 +2302,7 @@
         <v>118</v>
       </c>
       <c r="N27" t="s">
-        <v>155</v>
+        <v>153</v>
       </c>
       <c r="O27" t="s">
         <v>46</v>
@@ -2329,16 +2311,16 @@
         <v>1000</v>
       </c>
       <c r="Q27" t="s">
+        <v>165</v>
+      </c>
+      <c r="R27" t="s">
         <v>167</v>
       </c>
-      <c r="R27" t="s">
-        <v>169</v>
-      </c>
       <c r="S27" t="s">
-        <v>172</v>
+        <v>170</v>
       </c>
       <c r="T27" t="s">
-        <v>175</v>
+        <v>173</v>
       </c>
       <c r="U27" t="s">
         <v>91</v>
@@ -2378,11 +2360,8 @@
       <c r="J28" t="s">
         <v>132</v>
       </c>
-      <c r="K28" t="s">
-        <v>142</v>
-      </c>
       <c r="N28" t="s">
-        <v>148</v>
+        <v>146</v>
       </c>
       <c r="O28" t="s">
         <v>47</v>
@@ -2391,19 +2370,19 @@
         <v>100000</v>
       </c>
       <c r="Q28" t="s">
-        <v>166</v>
+        <v>164</v>
       </c>
       <c r="R28" t="s">
-        <v>169</v>
+        <v>167</v>
       </c>
       <c r="S28" t="s">
+        <v>170</v>
+      </c>
+      <c r="T28" t="s">
         <v>172</v>
       </c>
-      <c r="T28" t="s">
-        <v>174</v>
-      </c>
       <c r="U28" t="s">
-        <v>178</v>
+        <v>176</v>
       </c>
       <c r="V28" s="1">
         <v>46291</v>
@@ -2441,7 +2420,7 @@
         <v>135</v>
       </c>
       <c r="N29" t="s">
-        <v>152</v>
+        <v>150</v>
       </c>
       <c r="O29" t="s">
         <v>48</v>
@@ -2450,19 +2429,19 @@
         <v>150000</v>
       </c>
       <c r="Q29" t="s">
-        <v>167</v>
+        <v>165</v>
       </c>
       <c r="R29" t="s">
-        <v>170</v>
+        <v>168</v>
       </c>
       <c r="S29" t="s">
-        <v>172</v>
+        <v>170</v>
       </c>
       <c r="T29" t="s">
-        <v>175</v>
+        <v>173</v>
       </c>
       <c r="U29" t="s">
-        <v>178</v>
+        <v>176</v>
       </c>
       <c r="V29" s="1">
         <v>46199</v>
@@ -2500,7 +2479,7 @@
         <v>135</v>
       </c>
       <c r="N30" t="s">
-        <v>152</v>
+        <v>150</v>
       </c>
       <c r="O30" t="s">
         <v>49</v>
@@ -2509,19 +2488,19 @@
         <v>150000</v>
       </c>
       <c r="Q30" t="s">
-        <v>167</v>
+        <v>165</v>
       </c>
       <c r="R30" t="s">
-        <v>170</v>
+        <v>168</v>
       </c>
       <c r="S30" t="s">
-        <v>172</v>
+        <v>170</v>
       </c>
       <c r="T30" t="s">
-        <v>175</v>
+        <v>173</v>
       </c>
       <c r="U30" t="s">
-        <v>178</v>
+        <v>176</v>
       </c>
       <c r="V30" s="1">
         <v>46199</v>
@@ -2559,7 +2538,7 @@
         <v>135</v>
       </c>
       <c r="N31" t="s">
-        <v>152</v>
+        <v>150</v>
       </c>
       <c r="O31" t="s">
         <v>50</v>
@@ -2568,19 +2547,19 @@
         <v>18462.36</v>
       </c>
       <c r="Q31" t="s">
-        <v>167</v>
+        <v>165</v>
       </c>
       <c r="R31" t="s">
-        <v>170</v>
+        <v>168</v>
       </c>
       <c r="S31" t="s">
-        <v>172</v>
+        <v>170</v>
       </c>
       <c r="T31" t="s">
-        <v>175</v>
+        <v>173</v>
       </c>
       <c r="U31" t="s">
-        <v>178</v>
+        <v>176</v>
       </c>
       <c r="V31" s="1">
         <v>46199</v>
@@ -2618,7 +2597,7 @@
         <v>135</v>
       </c>
       <c r="N32" t="s">
-        <v>152</v>
+        <v>150</v>
       </c>
       <c r="O32" t="s">
         <v>50</v>
@@ -2627,19 +2606,19 @@
         <v>324166.14</v>
       </c>
       <c r="Q32" t="s">
-        <v>167</v>
+        <v>165</v>
       </c>
       <c r="R32" t="s">
-        <v>170</v>
+        <v>168</v>
       </c>
       <c r="S32" t="s">
-        <v>172</v>
+        <v>170</v>
       </c>
       <c r="T32" t="s">
-        <v>175</v>
+        <v>173</v>
       </c>
       <c r="U32" t="s">
-        <v>178</v>
+        <v>176</v>
       </c>
       <c r="V32" s="1">
         <v>46199</v>
@@ -2668,10 +2647,10 @@
         <v>136</v>
       </c>
       <c r="K33" t="s">
-        <v>143</v>
+        <v>142</v>
       </c>
       <c r="N33" t="s">
-        <v>152</v>
+        <v>150</v>
       </c>
       <c r="O33" t="s">
         <v>51</v>
@@ -2680,19 +2659,19 @@
         <v>30000</v>
       </c>
       <c r="Q33" t="s">
-        <v>167</v>
+        <v>165</v>
       </c>
       <c r="R33" t="s">
-        <v>170</v>
+        <v>168</v>
       </c>
       <c r="S33" t="s">
-        <v>172</v>
+        <v>170</v>
       </c>
       <c r="T33" t="s">
-        <v>175</v>
+        <v>173</v>
       </c>
       <c r="U33" t="s">
-        <v>178</v>
+        <v>176</v>
       </c>
       <c r="V33" s="1">
         <v>46291</v>
@@ -2730,7 +2709,7 @@
         <v>137</v>
       </c>
       <c r="N34" t="s">
-        <v>152</v>
+        <v>150</v>
       </c>
       <c r="O34" t="s">
         <v>52</v>
@@ -2739,19 +2718,19 @@
         <v>1496713.48</v>
       </c>
       <c r="Q34" t="s">
-        <v>167</v>
+        <v>165</v>
       </c>
       <c r="R34" t="s">
-        <v>170</v>
+        <v>168</v>
       </c>
       <c r="S34" t="s">
-        <v>172</v>
+        <v>170</v>
       </c>
       <c r="T34" t="s">
+        <v>174</v>
+      </c>
+      <c r="U34" t="s">
         <v>176</v>
-      </c>
-      <c r="U34" t="s">
-        <v>178</v>
       </c>
       <c r="V34" s="1">
         <v>46199</v>
@@ -2786,7 +2765,7 @@
         <v>116</v>
       </c>
       <c r="N35" t="s">
-        <v>152</v>
+        <v>150</v>
       </c>
       <c r="O35" t="s">
         <v>52</v>
@@ -2795,19 +2774,19 @@
         <v>207789.52</v>
       </c>
       <c r="Q35" t="s">
-        <v>167</v>
+        <v>165</v>
       </c>
       <c r="R35" t="s">
-        <v>170</v>
+        <v>168</v>
       </c>
       <c r="S35" t="s">
-        <v>172</v>
+        <v>170</v>
       </c>
       <c r="T35" t="s">
+        <v>174</v>
+      </c>
+      <c r="U35" t="s">
         <v>176</v>
-      </c>
-      <c r="U35" t="s">
-        <v>178</v>
       </c>
       <c r="V35" s="1">
         <v>46138</v>
@@ -2842,7 +2821,7 @@
         <v>122</v>
       </c>
       <c r="N36" t="s">
-        <v>155</v>
+        <v>153</v>
       </c>
       <c r="O36" t="s">
         <v>53</v>
@@ -2851,16 +2830,16 @@
         <v>962290.8</v>
       </c>
       <c r="Q36" t="s">
+        <v>165</v>
+      </c>
+      <c r="R36" t="s">
         <v>167</v>
       </c>
-      <c r="R36" t="s">
-        <v>169</v>
-      </c>
       <c r="S36" t="s">
-        <v>172</v>
+        <v>170</v>
       </c>
       <c r="T36" t="s">
-        <v>175</v>
+        <v>173</v>
       </c>
       <c r="U36" t="s">
         <v>91</v>
@@ -2898,7 +2877,7 @@
         <v>123</v>
       </c>
       <c r="N37" t="s">
-        <v>155</v>
+        <v>153</v>
       </c>
       <c r="O37" t="s">
         <v>53</v>
@@ -2907,16 +2886,16 @@
         <v>798776.97</v>
       </c>
       <c r="Q37" t="s">
-        <v>167</v>
+        <v>165</v>
       </c>
       <c r="R37" t="s">
-        <v>170</v>
+        <v>168</v>
       </c>
       <c r="S37" t="s">
-        <v>172</v>
+        <v>170</v>
       </c>
       <c r="T37" t="s">
-        <v>175</v>
+        <v>173</v>
       </c>
       <c r="U37" t="s">
         <v>91</v>
@@ -2954,7 +2933,7 @@
         <v>122</v>
       </c>
       <c r="N38" t="s">
-        <v>155</v>
+        <v>153</v>
       </c>
       <c r="O38" t="s">
         <v>53</v>
@@ -2963,16 +2942,16 @@
         <v>1530656.62</v>
       </c>
       <c r="Q38" t="s">
+        <v>165</v>
+      </c>
+      <c r="R38" t="s">
         <v>167</v>
       </c>
-      <c r="R38" t="s">
-        <v>169</v>
-      </c>
       <c r="S38" t="s">
-        <v>172</v>
+        <v>170</v>
       </c>
       <c r="T38" t="s">
-        <v>175</v>
+        <v>173</v>
       </c>
       <c r="U38" t="s">
         <v>91</v>
@@ -3010,7 +2989,7 @@
         <v>124</v>
       </c>
       <c r="N39" t="s">
-        <v>155</v>
+        <v>153</v>
       </c>
       <c r="O39" t="s">
         <v>53</v>
@@ -3019,16 +2998,16 @@
         <v>72958.08</v>
       </c>
       <c r="Q39" t="s">
+        <v>165</v>
+      </c>
+      <c r="R39" t="s">
         <v>167</v>
       </c>
-      <c r="R39" t="s">
-        <v>169</v>
-      </c>
       <c r="S39" t="s">
-        <v>172</v>
+        <v>170</v>
       </c>
       <c r="T39" t="s">
-        <v>175</v>
+        <v>173</v>
       </c>
       <c r="U39" t="s">
         <v>91</v>
@@ -3066,7 +3045,7 @@
         <v>124</v>
       </c>
       <c r="N40" t="s">
-        <v>155</v>
+        <v>153</v>
       </c>
       <c r="O40" t="s">
         <v>53</v>
@@ -3075,16 +3054,16 @@
         <v>8916</v>
       </c>
       <c r="Q40" t="s">
+        <v>165</v>
+      </c>
+      <c r="R40" t="s">
         <v>167</v>
       </c>
-      <c r="R40" t="s">
-        <v>169</v>
-      </c>
       <c r="S40" t="s">
-        <v>172</v>
+        <v>170</v>
       </c>
       <c r="T40" t="s">
-        <v>175</v>
+        <v>173</v>
       </c>
       <c r="U40" t="s">
         <v>91</v>
@@ -3122,7 +3101,7 @@
         <v>124</v>
       </c>
       <c r="N41" t="s">
-        <v>155</v>
+        <v>153</v>
       </c>
       <c r="O41" t="s">
         <v>53</v>
@@ -3131,16 +3110,16 @@
         <v>425178.5</v>
       </c>
       <c r="Q41" t="s">
+        <v>165</v>
+      </c>
+      <c r="R41" t="s">
         <v>167</v>
       </c>
-      <c r="R41" t="s">
-        <v>169</v>
-      </c>
       <c r="S41" t="s">
-        <v>172</v>
+        <v>170</v>
       </c>
       <c r="T41" t="s">
-        <v>175</v>
+        <v>173</v>
       </c>
       <c r="U41" t="s">
         <v>91</v>
@@ -3178,7 +3157,7 @@
         <v>125</v>
       </c>
       <c r="N42" t="s">
-        <v>155</v>
+        <v>153</v>
       </c>
       <c r="O42" t="s">
         <v>53</v>
@@ -3187,16 +3166,16 @@
         <v>1223.03</v>
       </c>
       <c r="Q42" t="s">
+        <v>165</v>
+      </c>
+      <c r="R42" t="s">
         <v>167</v>
       </c>
-      <c r="R42" t="s">
-        <v>169</v>
-      </c>
       <c r="S42" t="s">
-        <v>172</v>
+        <v>170</v>
       </c>
       <c r="T42" t="s">
-        <v>175</v>
+        <v>173</v>
       </c>
       <c r="U42" t="s">
         <v>91</v>
@@ -3225,22 +3204,22 @@
         <v>107</v>
       </c>
       <c r="N43" t="s">
-        <v>155</v>
+        <v>153</v>
       </c>
       <c r="O43" t="s">
         <v>54</v>
       </c>
       <c r="Q43" t="s">
+        <v>165</v>
+      </c>
+      <c r="R43" t="s">
         <v>167</v>
       </c>
-      <c r="R43" t="s">
-        <v>169</v>
-      </c>
       <c r="S43" t="s">
+        <v>171</v>
+      </c>
+      <c r="T43" t="s">
         <v>173</v>
-      </c>
-      <c r="T43" t="s">
-        <v>175</v>
       </c>
       <c r="U43" t="s">
         <v>91</v>
@@ -3278,7 +3257,7 @@
         <v>126</v>
       </c>
       <c r="N44" t="s">
-        <v>153</v>
+        <v>151</v>
       </c>
       <c r="O44" t="s">
         <v>55</v>
@@ -3287,16 +3266,16 @@
         <v>400000</v>
       </c>
       <c r="Q44" t="s">
+        <v>165</v>
+      </c>
+      <c r="R44" t="s">
         <v>167</v>
       </c>
-      <c r="R44" t="s">
-        <v>169</v>
-      </c>
       <c r="S44" t="s">
-        <v>172</v>
+        <v>170</v>
       </c>
       <c r="T44" t="s">
-        <v>175</v>
+        <v>173</v>
       </c>
       <c r="U44" t="s">
         <v>91</v>
@@ -3334,7 +3313,7 @@
         <v>126</v>
       </c>
       <c r="N45" t="s">
-        <v>153</v>
+        <v>151</v>
       </c>
       <c r="O45" t="s">
         <v>56</v>
@@ -3343,16 +3322,16 @@
         <v>400000</v>
       </c>
       <c r="Q45" t="s">
+        <v>165</v>
+      </c>
+      <c r="R45" t="s">
         <v>167</v>
       </c>
-      <c r="R45" t="s">
-        <v>169</v>
-      </c>
       <c r="S45" t="s">
-        <v>172</v>
+        <v>170</v>
       </c>
       <c r="T45" t="s">
-        <v>175</v>
+        <v>173</v>
       </c>
       <c r="U45" t="s">
         <v>91</v>
@@ -3393,7 +3372,7 @@
         <v>138</v>
       </c>
       <c r="N46" t="s">
-        <v>152</v>
+        <v>150</v>
       </c>
       <c r="O46" t="s">
         <v>57</v>
@@ -3402,19 +3381,19 @@
         <v>173846.38</v>
       </c>
       <c r="Q46" t="s">
-        <v>167</v>
+        <v>165</v>
       </c>
       <c r="R46" t="s">
-        <v>170</v>
+        <v>168</v>
       </c>
       <c r="S46" t="s">
-        <v>172</v>
+        <v>170</v>
       </c>
       <c r="T46" t="s">
+        <v>174</v>
+      </c>
+      <c r="U46" t="s">
         <v>176</v>
-      </c>
-      <c r="U46" t="s">
-        <v>178</v>
       </c>
       <c r="V46" s="1">
         <v>46229</v>
@@ -3449,7 +3428,7 @@
         <v>120</v>
       </c>
       <c r="N47" t="s">
-        <v>152</v>
+        <v>150</v>
       </c>
       <c r="O47" t="s">
         <v>57</v>
@@ -3458,19 +3437,19 @@
         <v>1530656.62</v>
       </c>
       <c r="Q47" t="s">
-        <v>167</v>
+        <v>165</v>
       </c>
       <c r="R47" t="s">
-        <v>170</v>
+        <v>168</v>
       </c>
       <c r="S47" t="s">
-        <v>172</v>
+        <v>170</v>
       </c>
       <c r="T47" t="s">
+        <v>174</v>
+      </c>
+      <c r="U47" t="s">
         <v>176</v>
-      </c>
-      <c r="U47" t="s">
-        <v>178</v>
       </c>
       <c r="V47" s="1">
         <v>46229</v>
@@ -3495,8 +3474,11 @@
       <c r="F48" t="s">
         <v>93</v>
       </c>
+      <c r="K48" t="s">
+        <v>141</v>
+      </c>
       <c r="N48" t="s">
-        <v>154</v>
+        <v>152</v>
       </c>
       <c r="O48" t="s">
         <v>58</v>
@@ -3505,16 +3487,16 @@
         <v>1000000</v>
       </c>
       <c r="Q48" t="s">
+        <v>165</v>
+      </c>
+      <c r="R48" t="s">
         <v>167</v>
       </c>
-      <c r="R48" t="s">
-        <v>169</v>
-      </c>
       <c r="S48" t="s">
-        <v>172</v>
+        <v>170</v>
       </c>
       <c r="T48" t="s">
-        <v>175</v>
+        <v>173</v>
       </c>
       <c r="U48" t="s">
         <v>91</v>
@@ -3554,11 +3536,8 @@
       <c r="J49" t="s">
         <v>132</v>
       </c>
-      <c r="K49" t="s">
-        <v>109</v>
-      </c>
       <c r="N49" t="s">
-        <v>148</v>
+        <v>146</v>
       </c>
       <c r="O49" t="s">
         <v>59</v>
@@ -3567,19 +3546,19 @@
         <v>958040</v>
       </c>
       <c r="Q49" t="s">
-        <v>166</v>
+        <v>164</v>
       </c>
       <c r="R49" t="s">
-        <v>169</v>
+        <v>167</v>
       </c>
       <c r="S49" t="s">
+        <v>170</v>
+      </c>
+      <c r="T49" t="s">
         <v>172</v>
       </c>
-      <c r="T49" t="s">
-        <v>174</v>
-      </c>
       <c r="U49" t="s">
-        <v>178</v>
+        <v>176</v>
       </c>
       <c r="V49" s="1">
         <v>46291</v>
@@ -3617,7 +3596,7 @@
         <v>139</v>
       </c>
       <c r="N50" t="s">
-        <v>148</v>
+        <v>146</v>
       </c>
       <c r="O50" t="s">
         <v>59</v>
@@ -3626,19 +3605,19 @@
         <v>41730.64</v>
       </c>
       <c r="Q50" t="s">
-        <v>166</v>
+        <v>164</v>
       </c>
       <c r="R50" t="s">
-        <v>171</v>
+        <v>169</v>
       </c>
       <c r="S50" t="s">
+        <v>170</v>
+      </c>
+      <c r="T50" t="s">
         <v>172</v>
       </c>
-      <c r="T50" t="s">
-        <v>174</v>
-      </c>
       <c r="U50" t="s">
-        <v>178</v>
+        <v>176</v>
       </c>
       <c r="V50" s="1">
         <v>46199</v>
@@ -3675,11 +3654,8 @@
       <c r="J51" t="s">
         <v>138</v>
       </c>
-      <c r="K51" t="s">
-        <v>144</v>
-      </c>
       <c r="N51" t="s">
-        <v>152</v>
+        <v>150</v>
       </c>
       <c r="O51" t="s">
         <v>60</v>
@@ -3688,19 +3664,19 @@
         <v>608623.25</v>
       </c>
       <c r="Q51" t="s">
-        <v>167</v>
+        <v>165</v>
       </c>
       <c r="R51" t="s">
-        <v>170</v>
+        <v>168</v>
       </c>
       <c r="S51" t="s">
-        <v>172</v>
+        <v>170</v>
       </c>
       <c r="T51" t="s">
+        <v>174</v>
+      </c>
+      <c r="U51" t="s">
         <v>176</v>
-      </c>
-      <c r="U51" t="s">
-        <v>178</v>
       </c>
       <c r="V51" s="1">
         <v>46260</v>
@@ -3737,11 +3713,8 @@
       <c r="J52" t="s">
         <v>138</v>
       </c>
-      <c r="K52" t="s">
-        <v>141</v>
-      </c>
       <c r="N52" t="s">
-        <v>152</v>
+        <v>150</v>
       </c>
       <c r="O52" t="s">
         <v>61</v>
@@ -3750,19 +3723,19 @@
         <v>66366.75999999999</v>
       </c>
       <c r="Q52" t="s">
-        <v>167</v>
+        <v>165</v>
       </c>
       <c r="R52" t="s">
-        <v>170</v>
+        <v>168</v>
       </c>
       <c r="S52" t="s">
-        <v>172</v>
+        <v>170</v>
       </c>
       <c r="T52" t="s">
+        <v>174</v>
+      </c>
+      <c r="U52" t="s">
         <v>176</v>
-      </c>
-      <c r="U52" t="s">
-        <v>178</v>
       </c>
       <c r="V52" s="1">
         <v>46291</v>
@@ -3791,10 +3764,10 @@
         <v>136</v>
       </c>
       <c r="K53" t="s">
-        <v>143</v>
+        <v>142</v>
       </c>
       <c r="N53" t="s">
-        <v>152</v>
+        <v>150</v>
       </c>
       <c r="O53" t="s">
         <v>62</v>
@@ -3803,19 +3776,19 @@
         <v>1586760.42</v>
       </c>
       <c r="Q53" t="s">
-        <v>167</v>
+        <v>165</v>
       </c>
       <c r="R53" t="s">
-        <v>170</v>
+        <v>168</v>
       </c>
       <c r="S53" t="s">
-        <v>172</v>
+        <v>170</v>
       </c>
       <c r="T53" t="s">
+        <v>174</v>
+      </c>
+      <c r="U53" t="s">
         <v>176</v>
-      </c>
-      <c r="U53" t="s">
-        <v>178</v>
       </c>
       <c r="V53" s="1">
         <v>46321</v>
@@ -3850,7 +3823,7 @@
         <v>128</v>
       </c>
       <c r="N54" t="s">
-        <v>152</v>
+        <v>150</v>
       </c>
       <c r="O54" t="s">
         <v>60</v>
@@ -3859,19 +3832,19 @@
         <v>236343.68</v>
       </c>
       <c r="Q54" t="s">
-        <v>167</v>
+        <v>165</v>
       </c>
       <c r="R54" t="s">
-        <v>170</v>
+        <v>168</v>
       </c>
       <c r="S54" t="s">
-        <v>172</v>
+        <v>170</v>
       </c>
       <c r="T54" t="s">
+        <v>174</v>
+      </c>
+      <c r="U54" t="s">
         <v>176</v>
-      </c>
-      <c r="U54" t="s">
-        <v>178</v>
       </c>
       <c r="V54" s="1">
         <v>46229</v>
@@ -3903,7 +3876,7 @@
         <v>120</v>
       </c>
       <c r="N55" t="s">
-        <v>152</v>
+        <v>150</v>
       </c>
       <c r="O55" t="s">
         <v>61</v>
@@ -3912,19 +3885,19 @@
         <v>1145462.93</v>
       </c>
       <c r="Q55" t="s">
-        <v>167</v>
+        <v>165</v>
       </c>
       <c r="R55" t="s">
-        <v>170</v>
+        <v>168</v>
       </c>
       <c r="S55" t="s">
-        <v>172</v>
+        <v>170</v>
       </c>
       <c r="T55" t="s">
+        <v>174</v>
+      </c>
+      <c r="U55" t="s">
         <v>176</v>
-      </c>
-      <c r="U55" t="s">
-        <v>178</v>
       </c>
       <c r="V55" s="1">
         <v>46291</v>
@@ -3956,7 +3929,7 @@
         <v>120</v>
       </c>
       <c r="N56" t="s">
-        <v>152</v>
+        <v>150</v>
       </c>
       <c r="O56" t="s">
         <v>60</v>
@@ -3965,19 +3938,19 @@
         <v>859536.0699999999</v>
       </c>
       <c r="Q56" t="s">
-        <v>167</v>
+        <v>165</v>
       </c>
       <c r="R56" t="s">
-        <v>170</v>
+        <v>168</v>
       </c>
       <c r="S56" t="s">
-        <v>172</v>
+        <v>170</v>
       </c>
       <c r="T56" t="s">
+        <v>174</v>
+      </c>
+      <c r="U56" t="s">
         <v>176</v>
-      </c>
-      <c r="U56" t="s">
-        <v>178</v>
       </c>
       <c r="V56" s="1">
         <v>46260</v>
@@ -4009,7 +3982,7 @@
         <v>114</v>
       </c>
       <c r="N57" t="s">
-        <v>152</v>
+        <v>150</v>
       </c>
       <c r="O57" t="s">
         <v>61</v>
@@ -4018,19 +3991,19 @@
         <v>389619.06</v>
       </c>
       <c r="Q57" t="s">
-        <v>167</v>
+        <v>165</v>
       </c>
       <c r="R57" t="s">
-        <v>170</v>
+        <v>168</v>
       </c>
       <c r="S57" t="s">
-        <v>172</v>
+        <v>170</v>
       </c>
       <c r="T57" t="s">
+        <v>174</v>
+      </c>
+      <c r="U57" t="s">
         <v>176</v>
-      </c>
-      <c r="U57" t="s">
-        <v>178</v>
       </c>
       <c r="V57" s="1">
         <v>46291</v>
@@ -4062,7 +4035,7 @@
         <v>129</v>
       </c>
       <c r="N58" t="s">
-        <v>152</v>
+        <v>150</v>
       </c>
       <c r="O58" t="s">
         <v>61</v>
@@ -4071,19 +4044,19 @@
         <v>103054.25</v>
       </c>
       <c r="Q58" t="s">
-        <v>167</v>
+        <v>165</v>
       </c>
       <c r="R58" t="s">
-        <v>170</v>
+        <v>168</v>
       </c>
       <c r="S58" t="s">
-        <v>172</v>
+        <v>170</v>
       </c>
       <c r="T58" t="s">
+        <v>174</v>
+      </c>
+      <c r="U58" t="s">
         <v>176</v>
-      </c>
-      <c r="U58" t="s">
-        <v>178</v>
       </c>
       <c r="V58" s="1">
         <v>46291</v>
@@ -4115,7 +4088,7 @@
         <v>130</v>
       </c>
       <c r="N59" t="s">
-        <v>152</v>
+        <v>150</v>
       </c>
       <c r="O59" t="s">
         <v>62</v>
@@ -4124,19 +4097,19 @@
         <v>117742.58</v>
       </c>
       <c r="Q59" t="s">
-        <v>167</v>
+        <v>165</v>
       </c>
       <c r="R59" t="s">
-        <v>170</v>
+        <v>168</v>
       </c>
       <c r="S59" t="s">
-        <v>172</v>
+        <v>170</v>
       </c>
       <c r="T59" t="s">
+        <v>174</v>
+      </c>
+      <c r="U59" t="s">
         <v>176</v>
-      </c>
-      <c r="U59" t="s">
-        <v>178</v>
       </c>
       <c r="V59" s="1">
         <v>46321</v>
@@ -4173,11 +4146,8 @@
       <c r="J60" t="s">
         <v>132</v>
       </c>
-      <c r="K60" t="s">
-        <v>145</v>
-      </c>
       <c r="N60" t="s">
-        <v>152</v>
+        <v>150</v>
       </c>
       <c r="O60" t="s">
         <v>63</v>
@@ -4186,19 +4156,19 @@
         <v>1295422.28</v>
       </c>
       <c r="Q60" t="s">
-        <v>167</v>
+        <v>165</v>
       </c>
       <c r="R60" t="s">
-        <v>170</v>
+        <v>168</v>
       </c>
       <c r="S60" t="s">
-        <v>172</v>
+        <v>170</v>
       </c>
       <c r="T60" t="s">
+        <v>174</v>
+      </c>
+      <c r="U60" t="s">
         <v>176</v>
-      </c>
-      <c r="U60" t="s">
-        <v>178</v>
       </c>
       <c r="V60" s="1">
         <v>46352</v>
@@ -4221,7 +4191,7 @@
         <v>92</v>
       </c>
       <c r="N61" t="s">
-        <v>156</v>
+        <v>154</v>
       </c>
       <c r="O61" t="s">
         <v>64</v>
@@ -4230,19 +4200,19 @@
         <v>4064.54</v>
       </c>
       <c r="Q61" t="s">
-        <v>167</v>
+        <v>165</v>
       </c>
       <c r="R61" t="s">
+        <v>169</v>
+      </c>
+      <c r="S61" t="s">
         <v>171</v>
       </c>
-      <c r="S61" t="s">
-        <v>173</v>
-      </c>
       <c r="T61" t="s">
-        <v>174</v>
+        <v>172</v>
       </c>
       <c r="U61" t="s">
-        <v>178</v>
+        <v>176</v>
       </c>
       <c r="V61" s="1">
         <v>46107</v>
@@ -4265,7 +4235,7 @@
         <v>92</v>
       </c>
       <c r="N62" t="s">
-        <v>157</v>
+        <v>155</v>
       </c>
       <c r="O62" t="s">
         <v>65</v>
@@ -4274,19 +4244,19 @@
         <v>4227.84</v>
       </c>
       <c r="Q62" t="s">
-        <v>166</v>
+        <v>164</v>
       </c>
       <c r="R62" t="s">
+        <v>169</v>
+      </c>
+      <c r="S62" t="s">
         <v>171</v>
       </c>
-      <c r="S62" t="s">
-        <v>173</v>
-      </c>
       <c r="T62" t="s">
-        <v>174</v>
+        <v>172</v>
       </c>
       <c r="U62" t="s">
-        <v>178</v>
+        <v>176</v>
       </c>
       <c r="V62" s="1">
         <v>46107</v>
@@ -4309,7 +4279,7 @@
         <v>92</v>
       </c>
       <c r="N63" t="s">
-        <v>158</v>
+        <v>156</v>
       </c>
       <c r="O63" t="s">
         <v>66</v>
@@ -4318,19 +4288,19 @@
         <v>9389.959999999999</v>
       </c>
       <c r="Q63" t="s">
-        <v>166</v>
+        <v>164</v>
       </c>
       <c r="R63" t="s">
+        <v>169</v>
+      </c>
+      <c r="S63" t="s">
         <v>171</v>
       </c>
-      <c r="S63" t="s">
-        <v>173</v>
-      </c>
       <c r="T63" t="s">
-        <v>174</v>
+        <v>172</v>
       </c>
       <c r="U63" t="s">
-        <v>178</v>
+        <v>176</v>
       </c>
       <c r="V63" s="1">
         <v>46107</v>
@@ -4353,7 +4323,7 @@
         <v>92</v>
       </c>
       <c r="N64" t="s">
-        <v>159</v>
+        <v>157</v>
       </c>
       <c r="O64" t="s">
         <v>67</v>
@@ -4362,19 +4332,19 @@
         <v>1163.64</v>
       </c>
       <c r="Q64" t="s">
-        <v>168</v>
+        <v>166</v>
       </c>
       <c r="R64" t="s">
+        <v>169</v>
+      </c>
+      <c r="S64" t="s">
         <v>171</v>
       </c>
-      <c r="S64" t="s">
-        <v>173</v>
-      </c>
       <c r="T64" t="s">
-        <v>174</v>
+        <v>172</v>
       </c>
       <c r="U64" t="s">
-        <v>178</v>
+        <v>176</v>
       </c>
       <c r="V64" s="1">
         <v>46107</v>
@@ -4397,7 +4367,7 @@
         <v>92</v>
       </c>
       <c r="N65" t="s">
-        <v>160</v>
+        <v>158</v>
       </c>
       <c r="O65" t="s">
         <v>68</v>
@@ -4406,19 +4376,19 @@
         <v>7204.82</v>
       </c>
       <c r="Q65" t="s">
-        <v>166</v>
+        <v>164</v>
       </c>
       <c r="R65" t="s">
+        <v>169</v>
+      </c>
+      <c r="S65" t="s">
         <v>171</v>
       </c>
-      <c r="S65" t="s">
-        <v>173</v>
-      </c>
       <c r="T65" t="s">
-        <v>174</v>
+        <v>172</v>
       </c>
       <c r="U65" t="s">
-        <v>178</v>
+        <v>176</v>
       </c>
       <c r="V65" s="1">
         <v>46107</v>
@@ -4441,7 +4411,7 @@
         <v>92</v>
       </c>
       <c r="N66" t="s">
-        <v>161</v>
+        <v>159</v>
       </c>
       <c r="O66" t="s">
         <v>65</v>
@@ -4450,19 +4420,19 @@
         <v>3662.66</v>
       </c>
       <c r="Q66" t="s">
-        <v>166</v>
+        <v>164</v>
       </c>
       <c r="R66" t="s">
+        <v>169</v>
+      </c>
+      <c r="S66" t="s">
         <v>171</v>
       </c>
-      <c r="S66" t="s">
-        <v>173</v>
-      </c>
       <c r="T66" t="s">
-        <v>174</v>
+        <v>172</v>
       </c>
       <c r="U66" t="s">
-        <v>178</v>
+        <v>176</v>
       </c>
       <c r="V66" s="1">
         <v>46107</v>
@@ -4485,7 +4455,7 @@
         <v>92</v>
       </c>
       <c r="N67" t="s">
-        <v>149</v>
+        <v>147</v>
       </c>
       <c r="O67" t="s">
         <v>69</v>
@@ -4494,16 +4464,16 @@
         <v>120000</v>
       </c>
       <c r="Q67" t="s">
-        <v>166</v>
+        <v>164</v>
       </c>
       <c r="R67" t="s">
-        <v>170</v>
+        <v>168</v>
       </c>
       <c r="S67" t="s">
-        <v>173</v>
+        <v>171</v>
       </c>
       <c r="T67" t="s">
-        <v>174</v>
+        <v>172</v>
       </c>
       <c r="U67" t="s">
         <v>91</v>
@@ -4535,22 +4505,22 @@
         <v>107</v>
       </c>
       <c r="N68" t="s">
-        <v>148</v>
+        <v>146</v>
       </c>
       <c r="O68" t="s">
         <v>70</v>
       </c>
       <c r="Q68" t="s">
-        <v>166</v>
+        <v>164</v>
       </c>
       <c r="R68" t="s">
-        <v>169</v>
+        <v>167</v>
       </c>
       <c r="S68" t="s">
+        <v>170</v>
+      </c>
+      <c r="T68" t="s">
         <v>172</v>
-      </c>
-      <c r="T68" t="s">
-        <v>174</v>
       </c>
       <c r="U68" t="s">
         <v>91</v>
@@ -4590,11 +4560,8 @@
       <c r="J69" t="s">
         <v>132</v>
       </c>
-      <c r="K69" t="s">
-        <v>109</v>
-      </c>
       <c r="N69" t="s">
-        <v>148</v>
+        <v>146</v>
       </c>
       <c r="O69" t="s">
         <v>71</v>
@@ -4603,19 +4570,19 @@
         <v>100000</v>
       </c>
       <c r="Q69" t="s">
-        <v>166</v>
+        <v>164</v>
       </c>
       <c r="R69" t="s">
-        <v>169</v>
+        <v>167</v>
       </c>
       <c r="S69" t="s">
+        <v>170</v>
+      </c>
+      <c r="T69" t="s">
         <v>172</v>
       </c>
-      <c r="T69" t="s">
-        <v>174</v>
-      </c>
       <c r="U69" t="s">
-        <v>178</v>
+        <v>176</v>
       </c>
       <c r="V69" s="1">
         <v>46229</v>
@@ -4638,7 +4605,7 @@
         <v>92</v>
       </c>
       <c r="N70" t="s">
-        <v>149</v>
+        <v>147</v>
       </c>
       <c r="O70" t="s">
         <v>72</v>
@@ -4647,16 +4614,16 @@
         <v>80000</v>
       </c>
       <c r="Q70" t="s">
-        <v>166</v>
+        <v>164</v>
       </c>
       <c r="R70" t="s">
-        <v>170</v>
+        <v>168</v>
       </c>
       <c r="S70" t="s">
-        <v>173</v>
+        <v>171</v>
       </c>
       <c r="T70" t="s">
-        <v>174</v>
+        <v>172</v>
       </c>
       <c r="U70" t="s">
         <v>91</v>
@@ -4682,7 +4649,7 @@
         <v>92</v>
       </c>
       <c r="N71" t="s">
-        <v>148</v>
+        <v>146</v>
       </c>
       <c r="O71" t="s">
         <v>73</v>
@@ -4691,19 +4658,19 @@
         <v>835000</v>
       </c>
       <c r="Q71" t="s">
-        <v>166</v>
+        <v>164</v>
       </c>
       <c r="R71" t="s">
-        <v>169</v>
+        <v>167</v>
       </c>
       <c r="S71" t="s">
-        <v>173</v>
+        <v>171</v>
       </c>
       <c r="T71" t="s">
-        <v>174</v>
+        <v>172</v>
       </c>
       <c r="U71" t="s">
-        <v>178</v>
+        <v>176</v>
       </c>
       <c r="V71" s="1">
         <v>46291</v>
@@ -4726,7 +4693,7 @@
         <v>92</v>
       </c>
       <c r="N72" t="s">
-        <v>148</v>
+        <v>146</v>
       </c>
       <c r="O72" t="s">
         <v>73</v>
@@ -4735,19 +4702,19 @@
         <v>165000</v>
       </c>
       <c r="Q72" t="s">
-        <v>166</v>
+        <v>164</v>
       </c>
       <c r="R72" t="s">
-        <v>169</v>
+        <v>167</v>
       </c>
       <c r="S72" t="s">
-        <v>173</v>
+        <v>171</v>
       </c>
       <c r="T72" t="s">
-        <v>174</v>
+        <v>172</v>
       </c>
       <c r="U72" t="s">
-        <v>178</v>
+        <v>176</v>
       </c>
       <c r="V72" s="1">
         <v>46168</v>
@@ -4770,7 +4737,7 @@
         <v>92</v>
       </c>
       <c r="N73" t="s">
-        <v>148</v>
+        <v>146</v>
       </c>
       <c r="O73" t="s">
         <v>74</v>
@@ -4779,19 +4746,19 @@
         <v>1000000</v>
       </c>
       <c r="Q73" t="s">
-        <v>166</v>
+        <v>164</v>
       </c>
       <c r="R73" t="s">
-        <v>169</v>
+        <v>167</v>
       </c>
       <c r="S73" t="s">
-        <v>173</v>
+        <v>171</v>
       </c>
       <c r="T73" t="s">
-        <v>174</v>
+        <v>172</v>
       </c>
       <c r="U73" t="s">
-        <v>178</v>
+        <v>176</v>
       </c>
       <c r="V73" s="1">
         <v>46291</v>
@@ -4814,7 +4781,7 @@
         <v>92</v>
       </c>
       <c r="N74" t="s">
-        <v>148</v>
+        <v>146</v>
       </c>
       <c r="O74" t="s">
         <v>75</v>
@@ -4823,19 +4790,19 @@
         <v>1000000</v>
       </c>
       <c r="Q74" t="s">
-        <v>166</v>
+        <v>164</v>
       </c>
       <c r="R74" t="s">
-        <v>169</v>
+        <v>167</v>
       </c>
       <c r="S74" t="s">
-        <v>173</v>
+        <v>171</v>
       </c>
       <c r="T74" t="s">
-        <v>174</v>
+        <v>172</v>
       </c>
       <c r="U74" t="s">
-        <v>178</v>
+        <v>176</v>
       </c>
       <c r="V74" s="1">
         <v>46291</v>
@@ -4858,7 +4825,7 @@
         <v>92</v>
       </c>
       <c r="N75" t="s">
-        <v>162</v>
+        <v>160</v>
       </c>
       <c r="O75" t="s">
         <v>76</v>
@@ -4867,19 +4834,19 @@
         <v>100000</v>
       </c>
       <c r="Q75" t="s">
-        <v>168</v>
+        <v>166</v>
       </c>
       <c r="R75" t="s">
-        <v>169</v>
+        <v>167</v>
       </c>
       <c r="S75" t="s">
-        <v>173</v>
+        <v>171</v>
       </c>
       <c r="T75" t="s">
-        <v>174</v>
+        <v>172</v>
       </c>
       <c r="U75" t="s">
-        <v>178</v>
+        <v>176</v>
       </c>
       <c r="V75" s="1">
         <v>46291</v>
@@ -4904,8 +4871,11 @@
       <c r="F76" t="s">
         <v>93</v>
       </c>
+      <c r="K76" t="s">
+        <v>141</v>
+      </c>
       <c r="N76" t="s">
-        <v>154</v>
+        <v>152</v>
       </c>
       <c r="O76" t="s">
         <v>77</v>
@@ -4914,16 +4884,16 @@
         <v>1000000</v>
       </c>
       <c r="Q76" t="s">
+        <v>165</v>
+      </c>
+      <c r="R76" t="s">
         <v>167</v>
       </c>
-      <c r="R76" t="s">
-        <v>169</v>
-      </c>
       <c r="S76" t="s">
-        <v>172</v>
+        <v>170</v>
       </c>
       <c r="T76" t="s">
-        <v>175</v>
+        <v>173</v>
       </c>
       <c r="U76" t="s">
         <v>91</v>
@@ -4955,7 +4925,7 @@
         <v>108</v>
       </c>
       <c r="N77" t="s">
-        <v>152</v>
+        <v>150</v>
       </c>
       <c r="O77" t="s">
         <v>78</v>
@@ -4964,19 +4934,19 @@
         <v>1704503</v>
       </c>
       <c r="Q77" t="s">
-        <v>167</v>
+        <v>165</v>
       </c>
       <c r="R77" t="s">
-        <v>170</v>
+        <v>168</v>
       </c>
       <c r="S77" t="s">
         <v>105</v>
       </c>
       <c r="T77" t="s">
+        <v>174</v>
+      </c>
+      <c r="U77" t="s">
         <v>176</v>
-      </c>
-      <c r="U77" t="s">
-        <v>178</v>
       </c>
       <c r="V77" s="1">
         <v>46381</v>
@@ -5005,7 +4975,7 @@
         <v>108</v>
       </c>
       <c r="N78" t="s">
-        <v>152</v>
+        <v>150</v>
       </c>
       <c r="O78" t="s">
         <v>79</v>
@@ -5014,19 +4984,19 @@
         <v>1638125.5</v>
       </c>
       <c r="Q78" t="s">
-        <v>167</v>
+        <v>165</v>
       </c>
       <c r="R78" t="s">
-        <v>170</v>
+        <v>168</v>
       </c>
       <c r="S78" t="s">
         <v>105</v>
       </c>
       <c r="T78" t="s">
+        <v>174</v>
+      </c>
+      <c r="U78" t="s">
         <v>176</v>
-      </c>
-      <c r="U78" t="s">
-        <v>178</v>
       </c>
       <c r="V78" s="1">
         <v>46381</v>
@@ -5055,7 +5025,7 @@
         <v>108</v>
       </c>
       <c r="N79" t="s">
-        <v>151</v>
+        <v>149</v>
       </c>
       <c r="O79" t="s">
         <v>80</v>
@@ -5064,16 +5034,16 @@
         <v>3800000</v>
       </c>
       <c r="Q79" t="s">
-        <v>167</v>
+        <v>165</v>
       </c>
       <c r="R79" t="s">
-        <v>170</v>
+        <v>168</v>
       </c>
       <c r="S79" t="s">
         <v>105</v>
       </c>
       <c r="T79" t="s">
-        <v>175</v>
+        <v>173</v>
       </c>
       <c r="U79" t="s">
         <v>91</v>
@@ -5105,7 +5075,7 @@
         <v>108</v>
       </c>
       <c r="N80" t="s">
-        <v>151</v>
+        <v>149</v>
       </c>
       <c r="O80" t="s">
         <v>81</v>
@@ -5114,16 +5084,16 @@
         <v>3800000</v>
       </c>
       <c r="Q80" t="s">
-        <v>167</v>
+        <v>165</v>
       </c>
       <c r="R80" t="s">
-        <v>170</v>
+        <v>168</v>
       </c>
       <c r="S80" t="s">
         <v>105</v>
       </c>
       <c r="T80" t="s">
-        <v>175</v>
+        <v>173</v>
       </c>
       <c r="U80" t="s">
         <v>91</v>
@@ -5152,10 +5122,10 @@
         <v>140</v>
       </c>
       <c r="K81" t="s">
-        <v>146</v>
+        <v>143</v>
       </c>
       <c r="N81" t="s">
-        <v>155</v>
+        <v>153</v>
       </c>
       <c r="O81" t="s">
         <v>82</v>
@@ -5164,16 +5134,16 @@
         <v>3800000</v>
       </c>
       <c r="Q81" t="s">
-        <v>167</v>
+        <v>165</v>
       </c>
       <c r="R81" t="s">
-        <v>170</v>
+        <v>168</v>
       </c>
       <c r="S81" t="s">
+        <v>171</v>
+      </c>
+      <c r="T81" t="s">
         <v>173</v>
-      </c>
-      <c r="T81" t="s">
-        <v>175</v>
       </c>
       <c r="U81" t="s">
         <v>91</v>
@@ -5198,8 +5168,11 @@
       <c r="E82" t="s">
         <v>91</v>
       </c>
+      <c r="K82" t="s">
+        <v>144</v>
+      </c>
       <c r="N82" t="s">
-        <v>163</v>
+        <v>161</v>
       </c>
       <c r="O82" t="s">
         <v>83</v>
@@ -5208,16 +5181,16 @@
         <v>4394700</v>
       </c>
       <c r="Q82" t="s">
-        <v>166</v>
+        <v>164</v>
       </c>
       <c r="R82" t="s">
-        <v>169</v>
+        <v>167</v>
       </c>
       <c r="S82" t="s">
+        <v>171</v>
+      </c>
+      <c r="T82" t="s">
         <v>173</v>
-      </c>
-      <c r="T82" t="s">
-        <v>175</v>
       </c>
       <c r="U82" t="s">
         <v>91</v>
@@ -5257,11 +5230,8 @@
       <c r="J83" t="s">
         <v>132</v>
       </c>
-      <c r="K83" t="s">
-        <v>141</v>
-      </c>
       <c r="N83" t="s">
-        <v>152</v>
+        <v>150</v>
       </c>
       <c r="O83" t="s">
         <v>84</v>
@@ -5270,19 +5240,19 @@
         <v>528395.9300000001</v>
       </c>
       <c r="Q83" t="s">
-        <v>167</v>
+        <v>165</v>
       </c>
       <c r="R83" t="s">
-        <v>170</v>
+        <v>168</v>
       </c>
       <c r="S83" t="s">
-        <v>172</v>
+        <v>170</v>
       </c>
       <c r="T83" t="s">
+        <v>174</v>
+      </c>
+      <c r="U83" t="s">
         <v>176</v>
-      </c>
-      <c r="U83" t="s">
-        <v>178</v>
       </c>
       <c r="V83" s="1">
         <v>46382</v>
@@ -5310,8 +5280,11 @@
       <c r="G84" t="s">
         <v>109</v>
       </c>
+      <c r="K84" t="s">
+        <v>141</v>
+      </c>
       <c r="N84" t="s">
-        <v>154</v>
+        <v>152</v>
       </c>
       <c r="O84" t="s">
         <v>85</v>
@@ -5320,16 +5293,16 @@
         <v>1000000</v>
       </c>
       <c r="Q84" t="s">
+        <v>165</v>
+      </c>
+      <c r="R84" t="s">
         <v>167</v>
       </c>
-      <c r="R84" t="s">
-        <v>169</v>
-      </c>
       <c r="S84" t="s">
-        <v>172</v>
+        <v>170</v>
       </c>
       <c r="T84" t="s">
-        <v>175</v>
+        <v>173</v>
       </c>
       <c r="U84" t="s">
         <v>91</v>
@@ -5354,8 +5327,11 @@
       <c r="E85" t="s">
         <v>91</v>
       </c>
+      <c r="K85" t="s">
+        <v>144</v>
+      </c>
       <c r="N85" t="s">
-        <v>163</v>
+        <v>161</v>
       </c>
       <c r="O85" t="s">
         <v>83</v>
@@ -5364,16 +5340,16 @@
         <v>4394700</v>
       </c>
       <c r="Q85" t="s">
-        <v>166</v>
+        <v>164</v>
       </c>
       <c r="R85" t="s">
-        <v>169</v>
+        <v>167</v>
       </c>
       <c r="S85" t="s">
+        <v>171</v>
+      </c>
+      <c r="T85" t="s">
         <v>173</v>
-      </c>
-      <c r="T85" t="s">
-        <v>175</v>
       </c>
       <c r="U85" t="s">
         <v>91</v>
@@ -5414,16 +5390,16 @@
         <v>3306000</v>
       </c>
       <c r="Q86" t="s">
-        <v>166</v>
+        <v>164</v>
       </c>
       <c r="R86" t="s">
-        <v>169</v>
+        <v>167</v>
       </c>
       <c r="S86" t="s">
         <v>105</v>
       </c>
       <c r="T86" t="s">
-        <v>175</v>
+        <v>173</v>
       </c>
       <c r="U86" t="s">
         <v>91</v>
@@ -5461,16 +5437,16 @@
         <v>3306000</v>
       </c>
       <c r="Q87" t="s">
-        <v>166</v>
+        <v>164</v>
       </c>
       <c r="R87" t="s">
-        <v>169</v>
+        <v>167</v>
       </c>
       <c r="S87" t="s">
         <v>105</v>
       </c>
       <c r="T87" t="s">
-        <v>175</v>
+        <v>173</v>
       </c>
       <c r="U87" t="s">
         <v>91</v>
@@ -5505,7 +5481,7 @@
         <v>131</v>
       </c>
       <c r="N88" t="s">
-        <v>164</v>
+        <v>162</v>
       </c>
       <c r="O88" t="s">
         <v>86</v>
@@ -5514,16 +5490,16 @@
         <v>412107.92</v>
       </c>
       <c r="Q88" t="s">
-        <v>166</v>
+        <v>164</v>
       </c>
       <c r="R88" t="s">
-        <v>169</v>
+        <v>167</v>
       </c>
       <c r="S88" t="s">
-        <v>172</v>
+        <v>170</v>
       </c>
       <c r="T88" t="s">
-        <v>177</v>
+        <v>175</v>
       </c>
       <c r="U88" t="s">
         <v>91</v>
@@ -5552,25 +5528,25 @@
         <v>109</v>
       </c>
       <c r="N89" t="s">
-        <v>155</v>
+        <v>153</v>
       </c>
       <c r="O89" t="s">
-        <v>165</v>
+        <v>163</v>
       </c>
       <c r="P89">
         <v>2297180</v>
       </c>
       <c r="Q89" t="s">
+        <v>165</v>
+      </c>
+      <c r="R89" t="s">
         <v>167</v>
       </c>
-      <c r="R89" t="s">
-        <v>169</v>
-      </c>
       <c r="S89" t="s">
-        <v>172</v>
+        <v>170</v>
       </c>
       <c r="T89" t="s">
-        <v>175</v>
+        <v>173</v>
       </c>
       <c r="U89" t="s">
         <v>91</v>

</xml_diff>